<commit_message>
Update results of bets
</commit_message>
<xml_diff>
--- a/data/predicciones.xlsx
+++ b/data/predicciones.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AG10"/>
+  <dimension ref="A1:AG9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -602,78 +602,78 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>tYjCfe2E</t>
+          <t>6sP22LDL</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>45514.45833333334</v>
+        <v>45515.54166666666</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>manchester city</t>
+          <t>brescia</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>manchester utd</t>
+          <t>venezia</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>48</v>
+        <v>77</v>
       </c>
       <c r="F2" t="n">
-        <v>482</v>
+        <v>773</v>
       </c>
       <c r="G2" t="n">
-        <v>1.57</v>
+        <v>2.88</v>
       </c>
       <c r="H2" t="n">
-        <v>4.5</v>
+        <v>3.2</v>
       </c>
       <c r="I2" t="n">
-        <v>5</v>
+        <v>2.45</v>
       </c>
       <c r="J2" t="n">
-        <v>0.6013630896699185</v>
+        <v>0.325149303251493</v>
       </c>
       <c r="K2" t="n">
-        <v>0.2098089001737271</v>
+        <v>0.2926343729263438</v>
       </c>
       <c r="L2" t="n">
-        <v>0.1888280101563544</v>
+        <v>0.3822163238221633</v>
       </c>
       <c r="M2" t="n">
-        <v>0.0591648973814578</v>
+        <v>0.06788548752834456</v>
       </c>
       <c r="N2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O2" t="n">
-        <v>0.631817708239324</v>
+        <v>0.3392938152055931</v>
       </c>
       <c r="P2" t="n">
-        <v>0.2258488301524321</v>
+        <v>0.3561153239435523</v>
       </c>
       <c r="Q2" t="n">
-        <v>0.1423334616082436</v>
+        <v>0.3045908608508545</v>
       </c>
       <c r="R2" t="n">
         <v>1</v>
       </c>
       <c r="S2" t="n">
-        <v>0.03045461856940557</v>
+        <v>0.06348095101720852</v>
       </c>
       <c r="T2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U2" t="n">
-        <v>0.03045461856940557</v>
+        <v>0.06348095101720852</v>
       </c>
       <c r="V2" t="n">
-        <v>0.631817708239324</v>
+        <v>0.3561153239435523</v>
       </c>
       <c r="W2" t="n">
-        <v>1.57</v>
+        <v>3.2</v>
       </c>
       <c r="X2" t="inlineStr">
         <is>
@@ -681,25 +681,25 @@
         </is>
       </c>
       <c r="Y2" t="n">
-        <v>7.947567290584082</v>
+        <v>4.258461309133468</v>
       </c>
       <c r="Z2" t="n">
-        <v>7.947567290584082</v>
+        <v>4.258461309133468</v>
       </c>
       <c r="AA2" t="inlineStr">
         <is>
-          <t>england</t>
+          <t>italy</t>
         </is>
       </c>
       <c r="AB2" t="inlineStr">
         <is>
-          <t>fa community shield</t>
+          <t>coppa italia</t>
         </is>
       </c>
       <c r="AC2" t="inlineStr"/>
       <c r="AD2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="AE2" t="inlineStr">
@@ -711,26 +711,26 @@
         <v>1</v>
       </c>
       <c r="AG2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>bs5ow5pA</t>
+          <t>bepKi4a3</t>
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>45514.54166666666</v>
+        <v>45515.5625</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>cremonese</t>
+          <t>parma</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>bari</t>
+          <t>palermo</t>
         </is>
       </c>
       <c r="E3" t="n">
@@ -740,55 +740,55 @@
         <v>773</v>
       </c>
       <c r="G3" t="n">
-        <v>1.85</v>
+        <v>1.9</v>
       </c>
       <c r="H3" t="n">
-        <v>3.3</v>
+        <v>3.4</v>
       </c>
       <c r="I3" t="n">
-        <v>4.5</v>
+        <v>4.1</v>
       </c>
       <c r="J3" t="n">
-        <v>0.5071721311475409</v>
+        <v>0.4945015963107485</v>
       </c>
       <c r="K3" t="n">
-        <v>0.2843237704918032</v>
+        <v>0.2763391273501242</v>
       </c>
       <c r="L3" t="n">
-        <v>0.2085040983606557</v>
+        <v>0.2291592763391274</v>
       </c>
       <c r="M3" t="n">
-        <v>0.06579306579306587</v>
+        <v>0.0643358755568979</v>
       </c>
       <c r="N3" t="n">
         <v>1</v>
       </c>
       <c r="O3" t="n">
-        <v>0.4008732509736669</v>
+        <v>0.4035638632982509</v>
       </c>
       <c r="P3" t="n">
-        <v>0.3715855311020828</v>
+        <v>0.3642107603159362</v>
       </c>
       <c r="Q3" t="n">
-        <v>0.2275412179242504</v>
+        <v>0.2322253763858128</v>
       </c>
       <c r="R3" t="n">
         <v>1</v>
       </c>
       <c r="S3" t="n">
-        <v>-0.106298880173874</v>
+        <v>-0.09093773301249763</v>
       </c>
       <c r="T3" t="n">
         <v>1</v>
       </c>
       <c r="U3" t="n">
-        <v>-0.106298880173874</v>
+        <v>-0.09093773301249763</v>
       </c>
       <c r="V3" t="n">
-        <v>0.4008732509736669</v>
+        <v>0.4035638632982509</v>
       </c>
       <c r="W3" t="n">
-        <v>1.85</v>
+        <v>1.9</v>
       </c>
       <c r="X3" t="inlineStr">
         <is>
@@ -796,10 +796,10 @@
         </is>
       </c>
       <c r="Y3" t="n">
-        <v>4.793680907167317</v>
+        <v>4.825855508235411</v>
       </c>
       <c r="Z3" t="n">
-        <v>4.793680907167317</v>
+        <v>4.825855508235411</v>
       </c>
       <c r="AA3" t="inlineStr">
         <is>
@@ -814,7 +814,7 @@
       <c r="AC3" t="inlineStr"/>
       <c r="AD3" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AE3" t="inlineStr">
@@ -823,29 +823,29 @@
         </is>
       </c>
       <c r="AF3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AG3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>02s0k9od</t>
+          <t>ILr8tvi2</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>45514.5625</v>
+        <v>45515.65625</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>verona</t>
+          <t>sampdoria</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>cesena</t>
+          <t>como</t>
         </is>
       </c>
       <c r="E4" t="n">
@@ -855,49 +855,67 @@
         <v>773</v>
       </c>
       <c r="G4" t="n">
-        <v>1.57</v>
+        <v>3</v>
       </c>
       <c r="H4" t="n">
-        <v>3.8</v>
+        <v>3.3</v>
       </c>
       <c r="I4" t="n">
-        <v>6</v>
+        <v>2.3</v>
       </c>
       <c r="J4" t="n">
-        <v>0.5970774629445346</v>
+        <v>0.3111931119311193</v>
       </c>
       <c r="K4" t="n">
-        <v>0.2466872675849787</v>
+        <v>0.2829028290282903</v>
       </c>
       <c r="L4" t="n">
-        <v>0.1562352694704865</v>
+        <v>0.4059040590405905</v>
       </c>
       <c r="M4" t="n">
-        <v>0.06676723656274453</v>
-      </c>
-      <c r="N4" t="inlineStr"/>
-      <c r="O4" t="inlineStr"/>
-      <c r="P4" t="inlineStr"/>
-      <c r="Q4" t="inlineStr"/>
+        <v>0.07114624505928857</v>
+      </c>
+      <c r="N4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O4" t="n">
+        <v>0.3733539654536731</v>
+      </c>
+      <c r="P4" t="n">
+        <v>0.3753850775205632</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>0.2512609570257635</v>
+      </c>
       <c r="R4" t="n">
         <v>1</v>
       </c>
-      <c r="S4" t="inlineStr"/>
+      <c r="S4" t="n">
+        <v>0.09248224849227293</v>
+      </c>
       <c r="T4" t="n">
         <v>0</v>
       </c>
-      <c r="U4" t="inlineStr"/>
-      <c r="V4" t="inlineStr"/>
+      <c r="U4" t="n">
+        <v>0.09248224849227293</v>
+      </c>
+      <c r="V4" t="n">
+        <v>0.3753850775205632</v>
+      </c>
       <c r="W4" t="n">
-        <v>1.244385733157199</v>
+        <v>3.3</v>
       </c>
       <c r="X4" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &lt; -0.5</t>
-        </is>
-      </c>
-      <c r="Y4" t="inlineStr"/>
-      <c r="Z4" t="inlineStr"/>
+          <t>dif_prob_mod_bm &gt; -0.5</t>
+        </is>
+      </c>
+      <c r="Y4" t="n">
+        <v>4.488890876543054</v>
+      </c>
+      <c r="Z4" t="n">
+        <v>4.488890876543054</v>
+      </c>
       <c r="AA4" t="inlineStr">
         <is>
           <t>italy</t>
@@ -911,16 +929,16 @@
       <c r="AC4" t="inlineStr"/>
       <c r="AD4" t="inlineStr">
         <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AE4" t="inlineStr">
+        <is>
           <t>1</t>
         </is>
       </c>
-      <c r="AE4" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
       <c r="AF4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AG4" t="n">
         <v>0</v>
@@ -929,20 +947,20 @@
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>Ob5Zdayq</t>
+          <t>ALOjHNNj</t>
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>45514.65625</v>
+        <v>45515.67708333334</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>empoli</t>
+          <t>torino</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>catanzaro</t>
+          <t>cosenza</t>
         </is>
       </c>
       <c r="E5" t="n">
@@ -952,55 +970,55 @@
         <v>773</v>
       </c>
       <c r="G5" t="n">
-        <v>1.5</v>
+        <v>1.3</v>
       </c>
       <c r="H5" t="n">
-        <v>4.1</v>
+        <v>5.5</v>
       </c>
       <c r="I5" t="n">
-        <v>6.5</v>
+        <v>8.5</v>
       </c>
       <c r="J5" t="n">
-        <v>0.6263219741480611</v>
+        <v>0.7197844495765973</v>
       </c>
       <c r="K5" t="n">
-        <v>0.2291421856639248</v>
+        <v>0.170130869899923</v>
       </c>
       <c r="L5" t="n">
-        <v>0.1445358401880141</v>
+        <v>0.1100846805234796</v>
       </c>
       <c r="M5" t="n">
-        <v>0.06441525953721072</v>
+        <v>0.06869600987248048</v>
       </c>
       <c r="N5" t="n">
         <v>1</v>
       </c>
       <c r="O5" t="n">
-        <v>0.4402219831272048</v>
+        <v>0.4739078815334473</v>
       </c>
       <c r="P5" t="n">
-        <v>0.3643307535591714</v>
+        <v>0.4223234754116265</v>
       </c>
       <c r="Q5" t="n">
-        <v>0.1954472633136242</v>
+        <v>0.1037686430549261</v>
       </c>
       <c r="R5" t="n">
         <v>1</v>
       </c>
       <c r="S5" t="n">
-        <v>-0.1860999910208563</v>
+        <v>-0.2458765680431499</v>
       </c>
       <c r="T5" t="n">
         <v>1</v>
       </c>
       <c r="U5" t="n">
-        <v>-0.1860999910208563</v>
+        <v>-0.2458765680431499</v>
       </c>
       <c r="V5" t="n">
-        <v>0.4402219831272048</v>
+        <v>0.4739078815334473</v>
       </c>
       <c r="W5" t="n">
-        <v>1.5</v>
+        <v>1.3</v>
       </c>
       <c r="X5" t="inlineStr">
         <is>
@@ -1008,10 +1026,10 @@
         </is>
       </c>
       <c r="Y5" t="n">
-        <v>5.264216832394331</v>
+        <v>5.667036046793324</v>
       </c>
       <c r="Z5" t="n">
-        <v>5.264216832394331</v>
+        <v>5.667036046793324</v>
       </c>
       <c r="AA5" t="inlineStr">
         <is>
@@ -1026,12 +1044,12 @@
       <c r="AC5" t="inlineStr"/>
       <c r="AD5" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="AE5" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AF5" t="n">
@@ -1044,20 +1062,20 @@
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>dC3sew6e</t>
+          <t>Aeu0r0Mk</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>45514.67708333334</v>
+        <v>45516.54166666666</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>napoli</t>
+          <t>frosinone</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>modena</t>
+          <t>pisa</t>
         </is>
       </c>
       <c r="E6" t="n">
@@ -1067,55 +1085,55 @@
         <v>773</v>
       </c>
       <c r="G6" t="n">
-        <v>1.17</v>
+        <v>1.8</v>
       </c>
       <c r="H6" t="n">
-        <v>7.5</v>
+        <v>3.4</v>
       </c>
       <c r="I6" t="n">
-        <v>13</v>
+        <v>4.75</v>
       </c>
       <c r="J6" t="n">
-        <v>0.8025682182985554</v>
+        <v>0.5240103828682673</v>
       </c>
       <c r="K6" t="n">
-        <v>0.1252006420545747</v>
+        <v>0.2774172615184945</v>
       </c>
       <c r="L6" t="n">
-        <v>0.07223113964686999</v>
+        <v>0.1985723556132381</v>
       </c>
       <c r="M6" t="n">
-        <v>0.06495726495726495</v>
+        <v>0.06019951840385285</v>
       </c>
       <c r="N6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O6" t="n">
-        <v>0.4763906586701594</v>
+        <v>0.4203876243472635</v>
       </c>
       <c r="P6" t="n">
-        <v>0.4799440635934727</v>
+        <v>0.382093697401959</v>
       </c>
       <c r="Q6" t="n">
-        <v>0.04366527773636795</v>
+        <v>0.1975186782507776</v>
       </c>
       <c r="R6" t="n">
         <v>1</v>
       </c>
       <c r="S6" t="n">
-        <v>0.354743421538898</v>
+        <v>-0.1036227585210038</v>
       </c>
       <c r="T6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U6" t="n">
-        <v>0.354743421538898</v>
+        <v>-0.1036227585210038</v>
       </c>
       <c r="V6" t="n">
-        <v>0.4799440635934727</v>
+        <v>0.4203876243472635</v>
       </c>
       <c r="W6" t="n">
-        <v>7.5</v>
+        <v>1.8</v>
       </c>
       <c r="X6" t="inlineStr">
         <is>
@@ -1123,10 +1141,10 @@
         </is>
       </c>
       <c r="Y6" t="n">
-        <v>5.739217292668545</v>
+        <v>5.027035661641791</v>
       </c>
       <c r="Z6" t="n">
-        <v>5.739217292668545</v>
+        <v>5.027035661641791</v>
       </c>
       <c r="AA6" t="inlineStr">
         <is>
@@ -1141,16 +1159,16 @@
       <c r="AC6" t="inlineStr"/>
       <c r="AD6" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AE6" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>3</t>
         </is>
       </c>
       <c r="AF6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AG6" t="n">
         <v>0</v>
@@ -1159,20 +1177,20 @@
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>6sP22LDL</t>
+          <t>42SH31wI</t>
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>45515.54166666666</v>
+        <v>45516.5625</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>brescia</t>
+          <t>lecce</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>venezia</t>
+          <t>mantova</t>
         </is>
       </c>
       <c r="E7" t="n">
@@ -1182,55 +1200,55 @@
         <v>773</v>
       </c>
       <c r="G7" t="n">
-        <v>2.88</v>
+        <v>1.44</v>
       </c>
       <c r="H7" t="n">
-        <v>3.2</v>
+        <v>4</v>
       </c>
       <c r="I7" t="n">
-        <v>2.45</v>
+        <v>8.5</v>
       </c>
       <c r="J7" t="n">
-        <v>0.325149303251493</v>
+        <v>0.6538461538461539</v>
       </c>
       <c r="K7" t="n">
-        <v>0.2926343729263438</v>
+        <v>0.2353846153846154</v>
       </c>
       <c r="L7" t="n">
-        <v>0.3822163238221633</v>
+        <v>0.1107692307692308</v>
       </c>
       <c r="M7" t="n">
-        <v>0.06788548752834456</v>
+        <v>0.06209150326797386</v>
       </c>
       <c r="N7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O7" t="n">
-        <v>0.3392938152055931</v>
+        <v>0.388304129198316</v>
       </c>
       <c r="P7" t="n">
-        <v>0.3561153239435523</v>
+        <v>0.3675779794257129</v>
       </c>
       <c r="Q7" t="n">
-        <v>0.3045908608508545</v>
+        <v>0.244117891375971</v>
       </c>
       <c r="R7" t="n">
         <v>1</v>
       </c>
       <c r="S7" t="n">
-        <v>0.06348095101720852</v>
+        <v>-0.2655420246478378</v>
       </c>
       <c r="T7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U7" t="n">
-        <v>0.06348095101720852</v>
+        <v>-0.2655420246478378</v>
       </c>
       <c r="V7" t="n">
-        <v>0.3561153239435523</v>
+        <v>0.388304129198316</v>
       </c>
       <c r="W7" t="n">
-        <v>3.2</v>
+        <v>1.44</v>
       </c>
       <c r="X7" t="inlineStr">
         <is>
@@ -1238,10 +1256,10 @@
         </is>
       </c>
       <c r="Y7" t="n">
-        <v>4.258461309133468</v>
+        <v>4.643378139576774</v>
       </c>
       <c r="Z7" t="n">
-        <v>4.258461309133468</v>
+        <v>4.643378139576774</v>
       </c>
       <c r="AA7" t="inlineStr">
         <is>
@@ -1256,7 +1274,7 @@
       <c r="AC7" t="inlineStr"/>
       <c r="AD7" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="AE7" t="inlineStr">
@@ -1268,26 +1286,26 @@
         <v>1</v>
       </c>
       <c r="AG7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
         <is>
-          <t>bepKi4a3</t>
+          <t>fNwTkrUF</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>45515.5625</v>
+        <v>45516.65625</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>parma</t>
+          <t>salernitana</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>palermo</t>
+          <t>spezia</t>
         </is>
       </c>
       <c r="E8" t="n">
@@ -1297,55 +1315,55 @@
         <v>773</v>
       </c>
       <c r="G8" t="n">
-        <v>1.9</v>
+        <v>2.15</v>
       </c>
       <c r="H8" t="n">
-        <v>3.4</v>
+        <v>3.2</v>
       </c>
       <c r="I8" t="n">
-        <v>4.1</v>
+        <v>3.6</v>
       </c>
       <c r="J8" t="n">
-        <v>0.4945015963107485</v>
+        <v>0.4407039020657996</v>
       </c>
       <c r="K8" t="n">
-        <v>0.2763391273501242</v>
+        <v>0.2960979342004591</v>
       </c>
       <c r="L8" t="n">
-        <v>0.2291592763391274</v>
+        <v>0.2631981637337414</v>
       </c>
       <c r="M8" t="n">
-        <v>0.0643358755568979</v>
+        <v>0.05539405684754506</v>
       </c>
       <c r="N8" t="n">
         <v>1</v>
       </c>
       <c r="O8" t="n">
-        <v>0.4035638632982509</v>
+        <v>0.4440924956845937</v>
       </c>
       <c r="P8" t="n">
-        <v>0.3642107603159362</v>
+        <v>0.3844438367580742</v>
       </c>
       <c r="Q8" t="n">
-        <v>0.2322253763858128</v>
+        <v>0.1714636675573318</v>
       </c>
       <c r="R8" t="n">
         <v>1</v>
       </c>
       <c r="S8" t="n">
-        <v>-0.09093773301249763</v>
+        <v>0.003388593618794067</v>
       </c>
       <c r="T8" t="n">
         <v>1</v>
       </c>
       <c r="U8" t="n">
-        <v>-0.09093773301249763</v>
+        <v>0.003388593618794067</v>
       </c>
       <c r="V8" t="n">
-        <v>0.4035638632982509</v>
+        <v>0.4440924956845937</v>
       </c>
       <c r="W8" t="n">
-        <v>1.9</v>
+        <v>2.15</v>
       </c>
       <c r="X8" t="inlineStr">
         <is>
@@ -1353,10 +1371,10 @@
         </is>
       </c>
       <c r="Y8" t="n">
-        <v>4.825855508235411</v>
+        <v>5.310500793976306</v>
       </c>
       <c r="Z8" t="n">
-        <v>4.825855508235411</v>
+        <v>5.310500793976306</v>
       </c>
       <c r="AA8" t="inlineStr">
         <is>
@@ -1371,38 +1389,38 @@
       <c r="AC8" t="inlineStr"/>
       <c r="AD8" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>4</t>
         </is>
       </c>
       <c r="AE8" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="AF8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AG8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
         <is>
-          <t>ILr8tvi2</t>
+          <t>8KIdPmPc</t>
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>45515.65625</v>
+        <v>45516.67708333334</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>sampdoria</t>
+          <t>cagliari</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>como</t>
+          <t>carrarese</t>
         </is>
       </c>
       <c r="E9" t="n">
@@ -1412,55 +1430,55 @@
         <v>773</v>
       </c>
       <c r="G9" t="n">
-        <v>3</v>
+        <v>1.42</v>
       </c>
       <c r="H9" t="n">
-        <v>3.3</v>
+        <v>4.5</v>
       </c>
       <c r="I9" t="n">
-        <v>2.3</v>
+        <v>7.5</v>
       </c>
       <c r="J9" t="n">
-        <v>0.3111931119311193</v>
+        <v>0.6645008860011814</v>
       </c>
       <c r="K9" t="n">
-        <v>0.2829028290282903</v>
+        <v>0.2096869462492617</v>
       </c>
       <c r="L9" t="n">
-        <v>0.4059040590405905</v>
+        <v>0.125812167749557</v>
       </c>
       <c r="M9" t="n">
-        <v>0.07114624505928857</v>
+        <v>0.05978090766823163</v>
       </c>
       <c r="N9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O9" t="n">
-        <v>0.3733539654536731</v>
+        <v>0.4464358758202748</v>
       </c>
       <c r="P9" t="n">
-        <v>0.3753850775205632</v>
+        <v>0.3612273568598673</v>
       </c>
       <c r="Q9" t="n">
-        <v>0.2512609570257635</v>
+        <v>0.1923367673198579</v>
       </c>
       <c r="R9" t="n">
         <v>1</v>
       </c>
       <c r="S9" t="n">
-        <v>0.09248224849227293</v>
+        <v>-0.2180650101809066</v>
       </c>
       <c r="T9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U9" t="n">
-        <v>0.09248224849227293</v>
+        <v>-0.2180650101809066</v>
       </c>
       <c r="V9" t="n">
-        <v>0.3753850775205632</v>
+        <v>0.4464358758202748</v>
       </c>
       <c r="W9" t="n">
-        <v>3.3</v>
+        <v>1.42</v>
       </c>
       <c r="X9" t="inlineStr">
         <is>
@@ -1468,10 +1486,10 @@
         </is>
       </c>
       <c r="Y9" t="n">
-        <v>4.488890876543054</v>
+        <v>5.338523159118818</v>
       </c>
       <c r="Z9" t="n">
-        <v>4.488890876543054</v>
+        <v>5.338523159118818</v>
       </c>
       <c r="AA9" t="inlineStr">
         <is>
@@ -1486,7 +1504,7 @@
       <c r="AC9" t="inlineStr"/>
       <c r="AD9" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="AE9" t="inlineStr">
@@ -1498,121 +1516,6 @@
         <v>1</v>
       </c>
       <c r="AG9" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="1" t="inlineStr">
-        <is>
-          <t>ALOjHNNj</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="n">
-        <v>45515.67708333334</v>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>torino</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>cosenza</t>
-        </is>
-      </c>
-      <c r="E10" t="n">
-        <v>77</v>
-      </c>
-      <c r="F10" t="n">
-        <v>773</v>
-      </c>
-      <c r="G10" t="n">
-        <v>1.3</v>
-      </c>
-      <c r="H10" t="n">
-        <v>5.5</v>
-      </c>
-      <c r="I10" t="n">
-        <v>8.5</v>
-      </c>
-      <c r="J10" t="n">
-        <v>0.7197844495765973</v>
-      </c>
-      <c r="K10" t="n">
-        <v>0.170130869899923</v>
-      </c>
-      <c r="L10" t="n">
-        <v>0.1100846805234796</v>
-      </c>
-      <c r="M10" t="n">
-        <v>0.06869600987248048</v>
-      </c>
-      <c r="N10" t="n">
-        <v>1</v>
-      </c>
-      <c r="O10" t="n">
-        <v>0.4739078815334473</v>
-      </c>
-      <c r="P10" t="n">
-        <v>0.4223234754116265</v>
-      </c>
-      <c r="Q10" t="n">
-        <v>0.1037686430549261</v>
-      </c>
-      <c r="R10" t="n">
-        <v>1</v>
-      </c>
-      <c r="S10" t="n">
-        <v>-0.2458765680431499</v>
-      </c>
-      <c r="T10" t="n">
-        <v>1</v>
-      </c>
-      <c r="U10" t="n">
-        <v>-0.2458765680431499</v>
-      </c>
-      <c r="V10" t="n">
-        <v>0.4739078815334473</v>
-      </c>
-      <c r="W10" t="n">
-        <v>1.3</v>
-      </c>
-      <c r="X10" t="inlineStr">
-        <is>
-          <t>dif_prob_mod_bm &gt; -0.5</t>
-        </is>
-      </c>
-      <c r="Y10" t="n">
-        <v>5.667036046793324</v>
-      </c>
-      <c r="Z10" t="n">
-        <v>5.667036046793324</v>
-      </c>
-      <c r="AA10" t="inlineStr">
-        <is>
-          <t>italy</t>
-        </is>
-      </c>
-      <c r="AB10" t="inlineStr">
-        <is>
-          <t>coppa italia</t>
-        </is>
-      </c>
-      <c r="AC10" t="inlineStr"/>
-      <c r="AD10" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="AE10" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AF10" t="n">
-        <v>1</v>
-      </c>
-      <c r="AG10" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
DATA. Cambio de modelo en SPA (me arrepenti del 52, vuelvo al 75)
</commit_message>
<xml_diff>
--- a/data/predicciones.xlsx
+++ b/data/predicciones.xlsx
@@ -634,13 +634,13 @@
         <v>1</v>
       </c>
       <c r="Q2" t="n">
-        <v>0.5040312631960935</v>
+        <v>0.4832340351862966</v>
       </c>
       <c r="R2" t="n">
-        <v>0.3062966000045459</v>
+        <v>0.3055226080408455</v>
       </c>
       <c r="S2" t="n">
-        <v>0.1896721367993606</v>
+        <v>0.2112433567728581</v>
       </c>
       <c r="T2" t="n">
         <v>1</v>
@@ -649,16 +649,16 @@
         <v>0</v>
       </c>
       <c r="V2" t="n">
-        <v>-0.006510282897333575</v>
+        <v>-0.02730751090713046</v>
       </c>
       <c r="W2" t="n">
         <v>1</v>
       </c>
       <c r="X2" t="n">
-        <v>-0.006510282897333575</v>
+        <v>-0.02730751090713046</v>
       </c>
       <c r="Y2" t="n">
-        <v>0.5040312631960935</v>
+        <v>0.4832340351862966</v>
       </c>
       <c r="Z2" t="n">
         <v>1.85</v>
@@ -669,7 +669,7 @@
         </is>
       </c>
       <c r="AB2" t="n">
-        <v>5.970251763585119</v>
+        <v>5.984063864924396</v>
       </c>
     </row>
     <row r="3">
@@ -732,13 +732,13 @@
         <v>1</v>
       </c>
       <c r="Q3" t="n">
-        <v>0.5753202418193056</v>
+        <v>0.4536655896075555</v>
       </c>
       <c r="R3" t="n">
-        <v>0.264894884600652</v>
+        <v>0.3180504880757256</v>
       </c>
       <c r="S3" t="n">
-        <v>0.1597848735800425</v>
+        <v>0.2282839223167188</v>
       </c>
       <c r="T3" t="n">
         <v>1</v>
@@ -747,16 +747,16 @@
         <v>0</v>
       </c>
       <c r="V3" t="n">
-        <v>0.06746050784107105</v>
+        <v>-0.05419414437067904</v>
       </c>
       <c r="W3" t="n">
         <v>1</v>
       </c>
       <c r="X3" t="n">
-        <v>0.06746050784107105</v>
+        <v>-0.05419414437067904</v>
       </c>
       <c r="Y3" t="n">
-        <v>0.5753202418193056</v>
+        <v>0.4536655896075555</v>
       </c>
       <c r="Z3" t="n">
         <v>1.85</v>
@@ -767,26 +767,26 @@
         </is>
       </c>
       <c r="AB3" t="n">
-        <v>6.903842901831667</v>
+        <v>3.79022419399743</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>rciODVxp</t>
+          <t>CE0hJiFM</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>45675.60416666666</v>
+        <v>45676.51041666666</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>betis</t>
+          <t>real madrid</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>alaves</t>
+          <t>las palmas</t>
         </is>
       </c>
       <c r="E4" t="n">
@@ -806,37 +806,37 @@
         </is>
       </c>
       <c r="I4" t="n">
-        <v>1.7</v>
+        <v>1.14</v>
       </c>
       <c r="J4" t="n">
-        <v>3.5</v>
+        <v>8</v>
       </c>
       <c r="K4" t="n">
-        <v>5.5</v>
+        <v>15</v>
       </c>
       <c r="L4" t="n">
-        <v>0.557163531114327</v>
+        <v>0.8206811653672549</v>
       </c>
       <c r="M4" t="n">
-        <v>0.2706222865412445</v>
+        <v>0.1169470660648338</v>
       </c>
       <c r="N4" t="n">
-        <v>0.1722141823444284</v>
+        <v>0.06237176856791136</v>
       </c>
       <c r="O4" t="n">
-        <v>0.05576776165011466</v>
+        <v>0.06885964912280707</v>
       </c>
       <c r="P4" t="n">
         <v>1</v>
       </c>
       <c r="Q4" t="n">
-        <v>0.4782121506166395</v>
+        <v>0.6960880515797752</v>
       </c>
       <c r="R4" t="n">
-        <v>0.3985360113319936</v>
+        <v>0.2604734092648778</v>
       </c>
       <c r="S4" t="n">
-        <v>0.1232518380513669</v>
+        <v>0.043438539155347</v>
       </c>
       <c r="T4" t="n">
         <v>1</v>
@@ -845,19 +845,19 @@
         <v>0</v>
       </c>
       <c r="V4" t="n">
-        <v>-0.07895138049768752</v>
+        <v>-0.1245931137874797</v>
       </c>
       <c r="W4" t="n">
         <v>1</v>
       </c>
       <c r="X4" t="n">
-        <v>-0.07895138049768752</v>
+        <v>-0.1245931137874797</v>
       </c>
       <c r="Y4" t="n">
-        <v>0.4782121506166395</v>
+        <v>0.6960880515797752</v>
       </c>
       <c r="Z4" t="n">
-        <v>1.7</v>
+        <v>1.14</v>
       </c>
       <c r="AA4" t="inlineStr">
         <is>
@@ -865,26 +865,26 @@
         </is>
       </c>
       <c r="AB4" t="n">
-        <v>4.791129241427424</v>
+        <v>3.1634495428777</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>CE0hJiFM</t>
+          <t>6eM98z14</t>
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>45676.51041666666</v>
+        <v>45676.60416666666</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>real madrid</t>
+          <t>osasuna</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>las palmas</t>
+          <t>rayo vallecano</t>
         </is>
       </c>
       <c r="E5" t="n">
@@ -904,37 +904,37 @@
         </is>
       </c>
       <c r="I5" t="n">
-        <v>1.14</v>
+        <v>2.25</v>
       </c>
       <c r="J5" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="K5" t="n">
-        <v>15</v>
+        <v>3.5</v>
       </c>
       <c r="L5" t="n">
-        <v>0.8206811653672549</v>
+        <v>0.4179104477611941</v>
       </c>
       <c r="M5" t="n">
-        <v>0.1169470660648338</v>
+        <v>0.3134328358208956</v>
       </c>
       <c r="N5" t="n">
-        <v>0.06237176856791136</v>
+        <v>0.2686567164179105</v>
       </c>
       <c r="O5" t="n">
-        <v>0.06885964912280707</v>
+        <v>0.06349206349206327</v>
       </c>
       <c r="P5" t="n">
         <v>1</v>
       </c>
       <c r="Q5" t="n">
-        <v>0.6705696565488336</v>
+        <v>0.3825798416000299</v>
       </c>
       <c r="R5" t="n">
-        <v>0.3002447137331953</v>
+        <v>0.3071215190896318</v>
       </c>
       <c r="S5" t="n">
-        <v>0.02918562971797116</v>
+        <v>0.3102986393103384</v>
       </c>
       <c r="T5" t="n">
         <v>1</v>
@@ -943,19 +943,19 @@
         <v>0</v>
       </c>
       <c r="V5" t="n">
-        <v>-0.1501115088184213</v>
+        <v>-0.03533060616116418</v>
       </c>
       <c r="W5" t="n">
         <v>1</v>
       </c>
       <c r="X5" t="n">
-        <v>-0.1501115088184213</v>
+        <v>-0.03533060616116418</v>
       </c>
       <c r="Y5" t="n">
-        <v>0.6705696565488336</v>
+        <v>0.3825798416000299</v>
       </c>
       <c r="Z5" t="n">
-        <v>1.14</v>
+        <v>2.25</v>
       </c>
       <c r="AA5" t="inlineStr">
         <is>
@@ -963,26 +963,26 @@
         </is>
       </c>
       <c r="AB5" t="n">
-        <v>6.245497772764948</v>
+        <v>3.860118671285971</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>6eM98z14</t>
+          <t>KbnqNZFc</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>45676.60416666666</v>
+        <v>45677.70833333334</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>osasuna</t>
+          <t>villarreal</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>rayo vallecano</t>
+          <t>mallorca</t>
         </is>
       </c>
       <c r="E6" t="n">
@@ -1002,37 +1002,37 @@
         </is>
       </c>
       <c r="I6" t="n">
-        <v>2.25</v>
+        <v>1.65</v>
       </c>
       <c r="J6" t="n">
-        <v>3</v>
+        <v>3.6</v>
       </c>
       <c r="K6" t="n">
-        <v>3.5</v>
+        <v>5.75</v>
       </c>
       <c r="L6" t="n">
-        <v>0.4179104477611941</v>
+        <v>0.5729707286692962</v>
       </c>
       <c r="M6" t="n">
-        <v>0.3134328358208956</v>
+        <v>0.2626115839734274</v>
       </c>
       <c r="N6" t="n">
-        <v>0.2686567164179105</v>
+        <v>0.1644176873572763</v>
       </c>
       <c r="O6" t="n">
-        <v>0.06349206349206327</v>
+        <v>0.05775142731664484</v>
       </c>
       <c r="P6" t="n">
         <v>1</v>
       </c>
       <c r="Q6" t="n">
-        <v>0.4254843466991549</v>
+        <v>0.4720095339252821</v>
       </c>
       <c r="R6" t="n">
-        <v>0.3189353250199098</v>
+        <v>0.301995190755136</v>
       </c>
       <c r="S6" t="n">
-        <v>0.2555803282809353</v>
+        <v>0.2259952753195818</v>
       </c>
       <c r="T6" t="n">
         <v>1</v>
@@ -1041,19 +1041,19 @@
         <v>0</v>
       </c>
       <c r="V6" t="n">
-        <v>0.007573898937960788</v>
+        <v>-0.1009611947440141</v>
       </c>
       <c r="W6" t="n">
         <v>1</v>
       </c>
       <c r="X6" t="n">
-        <v>0.007573898937960788</v>
+        <v>-0.1009611947440141</v>
       </c>
       <c r="Y6" t="n">
-        <v>0.4254843466991549</v>
+        <v>0.4720095339252821</v>
       </c>
       <c r="Z6" t="n">
-        <v>2.25</v>
+        <v>1.65</v>
       </c>
       <c r="AA6" t="inlineStr">
         <is>
@@ -1061,26 +1061,26 @@
         </is>
       </c>
       <c r="AB6" t="n">
-        <v>5.105812160389858</v>
+        <v>1.090636079187611</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>KbnqNZFc</t>
+          <t>WIXIZCa3</t>
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>45677.70833333334</v>
+        <v>45682.51041666666</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
+          <t>atl  madrid</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
           <t>villarreal</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>mallorca</t>
         </is>
       </c>
       <c r="E7" t="n">
@@ -1100,37 +1100,37 @@
         </is>
       </c>
       <c r="I7" t="n">
-        <v>1.65</v>
+        <v>1.53</v>
       </c>
       <c r="J7" t="n">
-        <v>3.6</v>
+        <v>4.2</v>
       </c>
       <c r="K7" t="n">
-        <v>5.75</v>
+        <v>6.25</v>
       </c>
       <c r="L7" t="n">
-        <v>0.5729707286692962</v>
+        <v>0.621470932916652</v>
       </c>
       <c r="M7" t="n">
-        <v>0.2626115839734274</v>
+        <v>0.2263929827053518</v>
       </c>
       <c r="N7" t="n">
-        <v>0.1644176873572763</v>
+        <v>0.1521360843779964</v>
       </c>
       <c r="O7" t="n">
-        <v>0.05775142731664484</v>
+        <v>0.05169000933706802</v>
       </c>
       <c r="P7" t="n">
         <v>1</v>
       </c>
       <c r="Q7" t="n">
-        <v>0.4394407526910414</v>
+        <v>0.456039922617096</v>
       </c>
       <c r="R7" t="n">
-        <v>0.317374530435741</v>
+        <v>0.2760070196241792</v>
       </c>
       <c r="S7" t="n">
-        <v>0.2431847168732174</v>
+        <v>0.2679530577587248</v>
       </c>
       <c r="T7" t="n">
         <v>1</v>
@@ -1139,19 +1139,19 @@
         <v>0</v>
       </c>
       <c r="V7" t="n">
-        <v>-0.1335299759782548</v>
+        <v>-0.165431010299556</v>
       </c>
       <c r="W7" t="n">
         <v>1</v>
       </c>
       <c r="X7" t="n">
-        <v>-0.1335299759782548</v>
+        <v>-0.165431010299556</v>
       </c>
       <c r="Y7" t="n">
-        <v>0.4394407526910414</v>
+        <v>0.456039922617096</v>
       </c>
       <c r="Z7" t="n">
-        <v>1.65</v>
+        <v>1.53</v>
       </c>
       <c r="AA7" t="inlineStr">
         <is>
@@ -1159,26 +1159,26 @@
         </is>
       </c>
       <c r="AB7" t="n">
-        <v>3.670929320553438</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
         <is>
-          <t>WIXIZCa3</t>
+          <t>4CuXB97d</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>45682.51041666666</v>
+        <v>45683.60416666666</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>atl  madrid</t>
+          <t>ath bilbao</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>villarreal</t>
+          <t>leganes</t>
         </is>
       </c>
       <c r="E8" t="n">
@@ -1198,37 +1198,37 @@
         </is>
       </c>
       <c r="I8" t="n">
-        <v>1.53</v>
+        <v>1.33</v>
       </c>
       <c r="J8" t="n">
-        <v>4.2</v>
+        <v>5.25</v>
       </c>
       <c r="K8" t="n">
-        <v>6.25</v>
+        <v>8</v>
       </c>
       <c r="L8" t="n">
-        <v>0.621470932916652</v>
+        <v>0.7044320516583504</v>
       </c>
       <c r="M8" t="n">
-        <v>0.2263929827053518</v>
+        <v>0.1784561197534488</v>
       </c>
       <c r="N8" t="n">
-        <v>0.1521360843779964</v>
+        <v>0.1171118285882008</v>
       </c>
       <c r="O8" t="n">
-        <v>0.05169000933706802</v>
+        <v>0.06735588972431072</v>
       </c>
       <c r="P8" t="n">
         <v>1</v>
       </c>
       <c r="Q8" t="n">
-        <v>0.443983477562666</v>
+        <v>0.4627684606049773</v>
       </c>
       <c r="R8" t="n">
-        <v>0.3978199419067835</v>
+        <v>0.4027016613764486</v>
       </c>
       <c r="S8" t="n">
-        <v>0.1581965805305504</v>
+        <v>0.1345298780185741</v>
       </c>
       <c r="T8" t="n">
         <v>1</v>
@@ -1237,19 +1237,19 @@
         <v>0</v>
       </c>
       <c r="V8" t="n">
-        <v>-0.177487455353986</v>
+        <v>-0.2416635910533731</v>
       </c>
       <c r="W8" t="n">
         <v>1</v>
       </c>
       <c r="X8" t="n">
-        <v>-0.177487455353986</v>
+        <v>-0.2416635910533731</v>
       </c>
       <c r="Y8" t="n">
-        <v>0.443983477562666</v>
+        <v>0.4627684606049773</v>
       </c>
       <c r="Z8" t="n">
-        <v>1.53</v>
+        <v>1.33</v>
       </c>
       <c r="AA8" t="inlineStr">
         <is>
@@ -1257,26 +1257,26 @@
         </is>
       </c>
       <c r="AB8" t="n">
-        <v>3.197952266504159</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
         <is>
-          <t>hn10njq9</t>
+          <t>CSuRXjUF</t>
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>45683.51041666666</v>
+        <v>45683.70833333334</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>real sociedad</t>
+          <t>barcelona</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>getafe</t>
+          <t>valencia</t>
         </is>
       </c>
       <c r="E9" t="n">
@@ -1296,37 +1296,37 @@
         </is>
       </c>
       <c r="I9" t="n">
-        <v>1.65</v>
+        <v>1.27</v>
       </c>
       <c r="J9" t="n">
-        <v>3.6</v>
+        <v>6.5</v>
       </c>
       <c r="K9" t="n">
-        <v>5.5</v>
+        <v>8.5</v>
       </c>
       <c r="L9" t="n">
-        <v>0.5687203791469194</v>
+        <v>0.7436069986541051</v>
       </c>
       <c r="M9" t="n">
-        <v>0.2606635071090047</v>
+        <v>0.1452893674293405</v>
       </c>
       <c r="N9" t="n">
-        <v>0.1706161137440758</v>
+        <v>0.1111036339165545</v>
       </c>
       <c r="O9" t="n">
-        <v>0.06565656565656575</v>
+        <v>0.05889478747283272</v>
       </c>
       <c r="P9" t="n">
         <v>1</v>
       </c>
       <c r="Q9" t="n">
-        <v>0.5109610885677233</v>
+        <v>0.6084439736577477</v>
       </c>
       <c r="R9" t="n">
-        <v>0.3288357702439992</v>
+        <v>0.3200100405348513</v>
       </c>
       <c r="S9" t="n">
-        <v>0.1602031411882775</v>
+        <v>0.07154598580740112</v>
       </c>
       <c r="T9" t="n">
         <v>1</v>
@@ -1335,19 +1335,19 @@
         <v>0</v>
       </c>
       <c r="V9" t="n">
-        <v>-0.05775929057919615</v>
+        <v>-0.1351630249963574</v>
       </c>
       <c r="W9" t="n">
         <v>1</v>
       </c>
       <c r="X9" t="n">
-        <v>-0.05775929057919615</v>
+        <v>-0.1351630249963574</v>
       </c>
       <c r="Y9" t="n">
-        <v>0.5109610885677233</v>
+        <v>0.6084439736577477</v>
       </c>
       <c r="Z9" t="n">
-        <v>1.65</v>
+        <v>1.27</v>
       </c>
       <c r="AA9" t="inlineStr">
         <is>
@@ -1355,26 +1355,26 @@
         </is>
       </c>
       <c r="AB9" t="n">
-        <v>5.438421575862326</v>
+        <v>1.084669978757093</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
         <is>
-          <t>CSuRXjUF</t>
+          <t>rciODVxp</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
-        <v>45683.70833333334</v>
+        <v>45675.60416666666</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>barcelona</t>
+          <t>betis</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>valencia</t>
+          <t>alaves</t>
         </is>
       </c>
       <c r="E10" t="n">
@@ -1394,37 +1394,37 @@
         </is>
       </c>
       <c r="I10" t="n">
-        <v>1.27</v>
+        <v>1.7</v>
       </c>
       <c r="J10" t="n">
-        <v>6.5</v>
+        <v>3.5</v>
       </c>
       <c r="K10" t="n">
-        <v>8.5</v>
+        <v>5.5</v>
       </c>
       <c r="L10" t="n">
-        <v>0.7436069986541051</v>
+        <v>0.557163531114327</v>
       </c>
       <c r="M10" t="n">
-        <v>0.1452893674293405</v>
+        <v>0.2706222865412445</v>
       </c>
       <c r="N10" t="n">
-        <v>0.1111036339165545</v>
+        <v>0.1722141823444284</v>
       </c>
       <c r="O10" t="n">
-        <v>0.05889478747283272</v>
+        <v>0.05576776165011466</v>
       </c>
       <c r="P10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q10" t="n">
-        <v>0.5994720811319718</v>
+        <v>0.3995271685663001</v>
       </c>
       <c r="R10" t="n">
-        <v>0.3442018005186119</v>
+        <v>0.5055025467375889</v>
       </c>
       <c r="S10" t="n">
-        <v>0.05632611834941616</v>
+        <v>0.09497028469611105</v>
       </c>
       <c r="T10" t="n">
         <v>1</v>
@@ -1433,19 +1433,19 @@
         <v>0</v>
       </c>
       <c r="V10" t="n">
-        <v>-0.1441349175221333</v>
+        <v>0.2348802601963443</v>
       </c>
       <c r="W10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X10" t="n">
-        <v>-0.1441349175221333</v>
+        <v>0.2348802601963443</v>
       </c>
       <c r="Y10" t="n">
-        <v>0.5994720811319718</v>
+        <v>0.5055025467375889</v>
       </c>
       <c r="Z10" t="n">
-        <v>1.27</v>
+        <v>3.5</v>
       </c>
       <c r="AA10" t="inlineStr">
         <is>
@@ -1453,26 +1453,26 @@
         </is>
       </c>
       <c r="AB10" t="n">
-        <v>5.464045963318063</v>
+        <v>2.527512733687944</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
         <is>
-          <t>Amk0hOA6</t>
+          <t>ChPH6EVG</t>
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>45670.70833333334</v>
+        <v>45676.41666666666</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>real sociedad</t>
+          <t>celta vigo</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>villarreal</t>
+          <t>ath bilbao</t>
         </is>
       </c>
       <c r="E11" t="n">
@@ -1492,37 +1492,37 @@
         </is>
       </c>
       <c r="I11" t="n">
-        <v>2.05</v>
+        <v>2.7</v>
       </c>
       <c r="J11" t="n">
-        <v>3.3</v>
+        <v>3.1</v>
       </c>
       <c r="K11" t="n">
-        <v>3.8</v>
+        <v>2.75</v>
       </c>
       <c r="L11" t="n">
-        <v>0.4628160177154457</v>
+        <v>0.3505345394736841</v>
       </c>
       <c r="M11" t="n">
-        <v>0.2875069200959586</v>
+        <v>0.3053042763157894</v>
       </c>
       <c r="N11" t="n">
-        <v>0.2496770621885956</v>
+        <v>0.3441611842105263</v>
       </c>
       <c r="O11" t="n">
-        <v>0.05399307581592572</v>
+        <v>0.05658737916802448</v>
       </c>
       <c r="P11" t="n">
         <v>0</v>
       </c>
       <c r="Q11" t="n">
-        <v>0.2500013229951756</v>
+        <v>0.2274458940289709</v>
       </c>
       <c r="R11" t="n">
-        <v>0.4785774234524267</v>
+        <v>0.4384156620196354</v>
       </c>
       <c r="S11" t="n">
-        <v>0.2714212535523977</v>
+        <v>0.3341384439513938</v>
       </c>
       <c r="T11" t="n">
         <v>1</v>
@@ -1531,19 +1531,19 @@
         <v>0</v>
       </c>
       <c r="V11" t="n">
-        <v>0.1910705033564681</v>
+        <v>0.133111385703846</v>
       </c>
       <c r="W11" t="n">
         <v>0</v>
       </c>
       <c r="X11" t="n">
-        <v>0.1910705033564681</v>
+        <v>0.133111385703846</v>
       </c>
       <c r="Y11" t="n">
-        <v>0.4785774234524267</v>
+        <v>0.4384156620196354</v>
       </c>
       <c r="Z11" t="n">
-        <v>3.3</v>
+        <v>3.1</v>
       </c>
       <c r="AA11" t="inlineStr">
         <is>
@@ -1551,26 +1551,26 @@
         </is>
       </c>
       <c r="AB11" t="n">
-        <v>5.74292908142912</v>
+        <v>2.192078310098177</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
         <is>
-          <t>ChPH6EVG</t>
+          <t>hCpiLDpA</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
-        <v>45676.41666666666</v>
+        <v>45676.70833333334</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>celta vigo</t>
+          <t>valencia</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>ath bilbao</t>
+          <t>real sociedad</t>
         </is>
       </c>
       <c r="E12" t="n">
@@ -1590,37 +1590,37 @@
         </is>
       </c>
       <c r="I12" t="n">
-        <v>2.7</v>
+        <v>3.4</v>
       </c>
       <c r="J12" t="n">
         <v>3.1</v>
       </c>
       <c r="K12" t="n">
-        <v>2.75</v>
+        <v>2.25</v>
       </c>
       <c r="L12" t="n">
-        <v>0.3505345394736841</v>
+        <v>0.2771706735545401</v>
       </c>
       <c r="M12" t="n">
-        <v>0.3053042763157894</v>
+        <v>0.3039936419630439</v>
       </c>
       <c r="N12" t="n">
-        <v>0.3441611842105263</v>
+        <v>0.418835684482416</v>
       </c>
       <c r="O12" t="n">
-        <v>0.05658737916802448</v>
+        <v>0.06114273666455827</v>
       </c>
       <c r="P12" t="n">
         <v>0</v>
       </c>
       <c r="Q12" t="n">
-        <v>0.2430174202809387</v>
+        <v>0.2252237365664616</v>
       </c>
       <c r="R12" t="n">
-        <v>0.3900929263669987</v>
+        <v>0.4701496602568991</v>
       </c>
       <c r="S12" t="n">
-        <v>0.3668896533520626</v>
+        <v>0.3046266031766393</v>
       </c>
       <c r="T12" t="n">
         <v>1</v>
@@ -1629,16 +1629,16 @@
         <v>0</v>
       </c>
       <c r="V12" t="n">
-        <v>0.08478865005120928</v>
+        <v>0.1661560182938552</v>
       </c>
       <c r="W12" t="n">
         <v>0</v>
       </c>
       <c r="X12" t="n">
-        <v>0.08478865005120928</v>
+        <v>0.1661560182938552</v>
       </c>
       <c r="Y12" t="n">
-        <v>0.3900929263669987</v>
+        <v>0.4701496602568991</v>
       </c>
       <c r="Z12" t="n">
         <v>3.1</v>
@@ -1649,26 +1649,26 @@
         </is>
       </c>
       <c r="AB12" t="n">
-        <v>4.681115116403984</v>
+        <v>2.350748301284496</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
-          <t>hCpiLDpA</t>
+          <t>ptvZVUbS</t>
         </is>
       </c>
       <c r="B13" s="2" t="n">
-        <v>45676.70833333334</v>
+        <v>45681.70833333334</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>valencia</t>
+          <t>las palmas</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>real sociedad</t>
+          <t>osasuna</t>
         </is>
       </c>
       <c r="E13" t="n">
@@ -1688,37 +1688,37 @@
         </is>
       </c>
       <c r="I13" t="n">
-        <v>3.4</v>
+        <v>2.45</v>
       </c>
       <c r="J13" t="n">
         <v>3.1</v>
       </c>
       <c r="K13" t="n">
-        <v>2.25</v>
+        <v>3</v>
       </c>
       <c r="L13" t="n">
-        <v>0.2771706735545401</v>
+        <v>0.3835842441740565</v>
       </c>
       <c r="M13" t="n">
-        <v>0.3039936419630439</v>
+        <v>0.303155289750464</v>
       </c>
       <c r="N13" t="n">
-        <v>0.418835684482416</v>
+        <v>0.3132604660754795</v>
       </c>
       <c r="O13" t="n">
-        <v>0.06114273666455827</v>
+        <v>0.06407724380074598</v>
       </c>
       <c r="P13" t="n">
         <v>0</v>
       </c>
       <c r="Q13" t="n">
-        <v>0.1927735960192002</v>
+        <v>0.1820507129935932</v>
       </c>
       <c r="R13" t="n">
-        <v>0.4441116943642978</v>
+        <v>0.4925312724904186</v>
       </c>
       <c r="S13" t="n">
-        <v>0.3631147096165021</v>
+        <v>0.3254180145159881</v>
       </c>
       <c r="T13" t="n">
         <v>1</v>
@@ -1727,16 +1727,16 @@
         <v>0</v>
       </c>
       <c r="V13" t="n">
-        <v>0.1401180524012539</v>
+        <v>0.1893759827399546</v>
       </c>
       <c r="W13" t="n">
         <v>0</v>
       </c>
       <c r="X13" t="n">
-        <v>0.1401180524012539</v>
+        <v>0.1893759827399546</v>
       </c>
       <c r="Y13" t="n">
-        <v>0.4441116943642978</v>
+        <v>0.4925312724904186</v>
       </c>
       <c r="Z13" t="n">
         <v>3.1</v>
@@ -1747,26 +1747,26 @@
         </is>
       </c>
       <c r="AB13" t="n">
-        <v>5.329340332371573</v>
+        <v>2.462656362452093</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="inlineStr">
         <is>
-          <t>ptvZVUbS</t>
+          <t>CjODOni2</t>
         </is>
       </c>
       <c r="B14" s="2" t="n">
-        <v>45681.70833333334</v>
+        <v>45682.41666666666</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>las palmas</t>
+          <t>mallorca</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>osasuna</t>
+          <t>betis</t>
         </is>
       </c>
       <c r="E14" t="n">
@@ -1786,7 +1786,7 @@
         </is>
       </c>
       <c r="I14" t="n">
-        <v>2.45</v>
+        <v>2.5</v>
       </c>
       <c r="J14" t="n">
         <v>3.1</v>
@@ -1795,28 +1795,28 @@
         <v>3</v>
       </c>
       <c r="L14" t="n">
-        <v>0.3835842441740565</v>
+        <v>0.3788187372708758</v>
       </c>
       <c r="M14" t="n">
-        <v>0.303155289750464</v>
+        <v>0.3054989816700611</v>
       </c>
       <c r="N14" t="n">
-        <v>0.3132604660754795</v>
+        <v>0.3156822810590631</v>
       </c>
       <c r="O14" t="n">
-        <v>0.06407724380074598</v>
+        <v>0.05591397849462365</v>
       </c>
       <c r="P14" t="n">
         <v>0</v>
       </c>
       <c r="Q14" t="n">
-        <v>0.2306258630685199</v>
+        <v>0.2936297286600816</v>
       </c>
       <c r="R14" t="n">
-        <v>0.489051242883132</v>
+        <v>0.3676433843476864</v>
       </c>
       <c r="S14" t="n">
-        <v>0.280322894048348</v>
+        <v>0.3387268869922321</v>
       </c>
       <c r="T14" t="n">
         <v>1</v>
@@ -1825,16 +1825,16 @@
         <v>0</v>
       </c>
       <c r="V14" t="n">
-        <v>0.185895953132668</v>
+        <v>0.06214440267762528</v>
       </c>
       <c r="W14" t="n">
         <v>0</v>
       </c>
       <c r="X14" t="n">
-        <v>0.185895953132668</v>
+        <v>0.06214440267762528</v>
       </c>
       <c r="Y14" t="n">
-        <v>0.489051242883132</v>
+        <v>0.3676433843476864</v>
       </c>
       <c r="Z14" t="n">
         <v>3.1</v>
@@ -1845,26 +1845,26 @@
         </is>
       </c>
       <c r="AB14" t="n">
-        <v>5.868614914597583</v>
+        <v>1.838216921738432</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="inlineStr">
         <is>
-          <t>CjODOni2</t>
+          <t>tSapoxPp</t>
         </is>
       </c>
       <c r="B15" s="2" t="n">
-        <v>45682.41666666666</v>
+        <v>45682.60416666666</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>mallorca</t>
+          <t>sevilla</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>betis</t>
+          <t>espanyol</t>
         </is>
       </c>
       <c r="E15" t="n">
@@ -1884,37 +1884,37 @@
         </is>
       </c>
       <c r="I15" t="n">
-        <v>2.5</v>
+        <v>1.83</v>
       </c>
       <c r="J15" t="n">
-        <v>3.1</v>
+        <v>3.6</v>
       </c>
       <c r="K15" t="n">
-        <v>3</v>
+        <v>4.2</v>
       </c>
       <c r="L15" t="n">
-        <v>0.3788187372708758</v>
+        <v>0.5143906919779547</v>
       </c>
       <c r="M15" t="n">
-        <v>0.3054989816700611</v>
+        <v>0.2614819350887937</v>
       </c>
       <c r="N15" t="n">
-        <v>0.3156822810590631</v>
+        <v>0.2241273729332517</v>
       </c>
       <c r="O15" t="n">
-        <v>0.05591397849462365</v>
+        <v>0.06232110330470975</v>
       </c>
       <c r="P15" t="n">
         <v>0</v>
       </c>
       <c r="Q15" t="n">
-        <v>0.2953522565831334</v>
+        <v>0.3937618820808784</v>
       </c>
       <c r="R15" t="n">
-        <v>0.3558948893268954</v>
+        <v>0.4029033599397874</v>
       </c>
       <c r="S15" t="n">
-        <v>0.3487528540899714</v>
+        <v>0.2033347579793342</v>
       </c>
       <c r="T15" t="n">
         <v>1</v>
@@ -1923,19 +1923,19 @@
         <v>0</v>
       </c>
       <c r="V15" t="n">
-        <v>0.05039590765683427</v>
+        <v>0.1414214248509937</v>
       </c>
       <c r="W15" t="n">
         <v>0</v>
       </c>
       <c r="X15" t="n">
-        <v>0.05039590765683427</v>
+        <v>0.1414214248509937</v>
       </c>
       <c r="Y15" t="n">
-        <v>0.3558948893268954</v>
+        <v>0.4029033599397874</v>
       </c>
       <c r="Z15" t="n">
-        <v>3.1</v>
+        <v>3.6</v>
       </c>
       <c r="AA15" t="inlineStr">
         <is>
@@ -1943,26 +1943,26 @@
         </is>
       </c>
       <c r="AB15" t="n">
-        <v>4.270738671922745</v>
+        <v>2.014516799698937</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="inlineStr">
         <is>
-          <t>tSapoxPp</t>
+          <t>hn10njq9</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
-        <v>45682.60416666666</v>
+        <v>45683.51041666666</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>sevilla</t>
+          <t>real sociedad</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>espanyol</t>
+          <t>getafe</t>
         </is>
       </c>
       <c r="E16" t="n">
@@ -1982,37 +1982,37 @@
         </is>
       </c>
       <c r="I16" t="n">
-        <v>1.83</v>
+        <v>1.65</v>
       </c>
       <c r="J16" t="n">
         <v>3.6</v>
       </c>
       <c r="K16" t="n">
-        <v>4.2</v>
+        <v>5.5</v>
       </c>
       <c r="L16" t="n">
-        <v>0.5143906919779547</v>
+        <v>0.5687203791469194</v>
       </c>
       <c r="M16" t="n">
-        <v>0.2614819350887937</v>
+        <v>0.2606635071090047</v>
       </c>
       <c r="N16" t="n">
-        <v>0.2241273729332517</v>
+        <v>0.1706161137440758</v>
       </c>
       <c r="O16" t="n">
-        <v>0.06232110330470975</v>
+        <v>0.06565656565656575</v>
       </c>
       <c r="P16" t="n">
         <v>0</v>
       </c>
       <c r="Q16" t="n">
-        <v>0.2687104111812759</v>
+        <v>0.3155680897676792</v>
       </c>
       <c r="R16" t="n">
-        <v>0.5011285964452017</v>
+        <v>0.4772716339323213</v>
       </c>
       <c r="S16" t="n">
-        <v>0.2301609923735224</v>
+        <v>0.2071602762999995</v>
       </c>
       <c r="T16" t="n">
         <v>1</v>
@@ -2021,16 +2021,16 @@
         <v>0</v>
       </c>
       <c r="V16" t="n">
-        <v>0.239646661356408</v>
+        <v>0.2166081268233166</v>
       </c>
       <c r="W16" t="n">
         <v>0</v>
       </c>
       <c r="X16" t="n">
-        <v>0.239646661356408</v>
+        <v>0.2166081268233166</v>
       </c>
       <c r="Y16" t="n">
-        <v>0.5011285964452017</v>
+        <v>0.4772716339323213</v>
       </c>
       <c r="Z16" t="n">
         <v>3.6</v>
@@ -2041,26 +2041,26 @@
         </is>
       </c>
       <c r="AB16" t="n">
-        <v>6.01354315734242</v>
+        <v>2.386358169661607</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="inlineStr">
         <is>
-          <t>xxOXTsTs</t>
+          <t>Amk0hOA6</t>
         </is>
       </c>
       <c r="B17" s="2" t="n">
-        <v>45683.41666666666</v>
+        <v>45670.70833333334</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>rayo vallecano</t>
+          <t>real sociedad</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>girona</t>
+          <t>villarreal</t>
         </is>
       </c>
       <c r="E17" t="n">
@@ -2080,37 +2080,37 @@
         </is>
       </c>
       <c r="I17" t="n">
-        <v>2.88</v>
+        <v>2.05</v>
       </c>
       <c r="J17" t="n">
-        <v>2.88</v>
+        <v>3.3</v>
       </c>
       <c r="K17" t="n">
-        <v>2.7</v>
+        <v>3.8</v>
       </c>
       <c r="L17" t="n">
-        <v>0.3260869565217391</v>
+        <v>0.4628160177154457</v>
       </c>
       <c r="M17" t="n">
-        <v>0.3260869565217391</v>
+        <v>0.2875069200959586</v>
       </c>
       <c r="N17" t="n">
-        <v>0.3478260869565217</v>
+        <v>0.2496770621885956</v>
       </c>
       <c r="O17" t="n">
-        <v>0.06481481481481488</v>
+        <v>0.05399307581592572</v>
       </c>
       <c r="P17" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="Q17" t="n">
-        <v>0.1851331597482263</v>
+        <v>0.1630696751213538</v>
       </c>
       <c r="R17" t="n">
-        <v>0.4267001277686934</v>
+        <v>0.3874683618063422</v>
       </c>
       <c r="S17" t="n">
-        <v>0.3881667124830803</v>
+        <v>0.4494619630723039</v>
       </c>
       <c r="T17" t="n">
         <v>1</v>
@@ -2119,19 +2119,19 @@
         <v>0</v>
       </c>
       <c r="V17" t="n">
-        <v>0.1006131712469543</v>
+        <v>0.1997849008837083</v>
       </c>
       <c r="W17" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="X17" t="n">
-        <v>0.1006131712469543</v>
+        <v>0.1997849008837083</v>
       </c>
       <c r="Y17" t="n">
-        <v>0.4267001277686934</v>
+        <v>0.4494619630723039</v>
       </c>
       <c r="Z17" t="n">
-        <v>2.88</v>
+        <v>3.8</v>
       </c>
       <c r="AA17" t="inlineStr">
         <is>
@@ -2139,26 +2139,26 @@
         </is>
       </c>
       <c r="AB17" t="n">
-        <v>5.120401533224321</v>
+        <v>3.595695704578432</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="inlineStr">
         <is>
-          <t>4CuXB97d</t>
+          <t>Y7DQ4h0T</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
-        <v>45683.60416666666</v>
+        <v>45675.51041666666</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>ath bilbao</t>
+          <t>leganes</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>leganes</t>
+          <t>atl  madrid</t>
         </is>
       </c>
       <c r="E18" t="n">
@@ -2178,37 +2178,37 @@
         </is>
       </c>
       <c r="I18" t="n">
-        <v>1.33</v>
+        <v>7.5</v>
       </c>
       <c r="J18" t="n">
-        <v>5.25</v>
+        <v>4.2</v>
       </c>
       <c r="K18" t="n">
-        <v>8</v>
+        <v>1.45</v>
       </c>
       <c r="L18" t="n">
-        <v>0.7044320516583504</v>
+        <v>0.1256576911173011</v>
       </c>
       <c r="M18" t="n">
-        <v>0.1784561197534488</v>
+        <v>0.2243887341380377</v>
       </c>
       <c r="N18" t="n">
-        <v>0.1171118285882008</v>
+        <v>0.6499535747446611</v>
       </c>
       <c r="O18" t="n">
-        <v>0.06735588972431072</v>
+        <v>0.06108374384236459</v>
       </c>
       <c r="P18" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="Q18" t="n">
-        <v>0.3254920369107678</v>
+        <v>0.08019541629752157</v>
       </c>
       <c r="R18" t="n">
-        <v>0.5230131486973156</v>
+        <v>0.4212402436411409</v>
       </c>
       <c r="S18" t="n">
-        <v>0.1514948143919167</v>
+        <v>0.4985643400613377</v>
       </c>
       <c r="T18" t="n">
         <v>1</v>
@@ -2217,19 +2217,19 @@
         <v>0</v>
       </c>
       <c r="V18" t="n">
-        <v>0.3445570289438669</v>
+        <v>-0.1513892346833234</v>
       </c>
       <c r="W18" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="X18" t="n">
-        <v>0.3445570289438669</v>
+        <v>-0.1513892346833234</v>
       </c>
       <c r="Y18" t="n">
-        <v>0.5230131486973156</v>
+        <v>0.4985643400613377</v>
       </c>
       <c r="Z18" t="n">
-        <v>5.25</v>
+        <v>1.45</v>
       </c>
       <c r="AA18" t="inlineStr">
         <is>
@@ -2237,26 +2237,26 @@
         </is>
       </c>
       <c r="AB18" t="n">
-        <v>6.276157784367787</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="inlineStr">
         <is>
-          <t>Y7DQ4h0T</t>
+          <t>4j4daWNj</t>
         </is>
       </c>
       <c r="B19" s="2" t="n">
-        <v>45675.51041666666</v>
+        <v>45675.70833333334</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>leganes</t>
+          <t>getafe</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>atl  madrid</t>
+          <t>barcelona</t>
         </is>
       </c>
       <c r="E19" t="n">
@@ -2276,37 +2276,37 @@
         </is>
       </c>
       <c r="I19" t="n">
-        <v>7.5</v>
+        <v>7</v>
       </c>
       <c r="J19" t="n">
-        <v>4.2</v>
+        <v>4.1</v>
       </c>
       <c r="K19" t="n">
-        <v>1.45</v>
+        <v>1.48</v>
       </c>
       <c r="L19" t="n">
-        <v>0.1256576911173011</v>
+        <v>0.1344619748271583</v>
       </c>
       <c r="M19" t="n">
-        <v>0.2243887341380377</v>
+        <v>0.2295692253146606</v>
       </c>
       <c r="N19" t="n">
-        <v>0.6499535747446611</v>
+        <v>0.6359687998581812</v>
       </c>
       <c r="O19" t="n">
-        <v>0.06108374384236459</v>
+        <v>0.06243525755720869</v>
       </c>
       <c r="P19" t="n">
         <v>2</v>
       </c>
       <c r="Q19" t="n">
-        <v>0.09210975963731143</v>
+        <v>0.04637280531647024</v>
       </c>
       <c r="R19" t="n">
-        <v>0.3782419131789316</v>
+        <v>0.1541339932826796</v>
       </c>
       <c r="S19" t="n">
-        <v>0.529648327183757</v>
+        <v>0.7994932014008501</v>
       </c>
       <c r="T19" t="n">
         <v>1</v>
@@ -2315,19 +2315,19 @@
         <v>0</v>
       </c>
       <c r="V19" t="n">
-        <v>-0.1203052475609041</v>
+        <v>0.1635244015426689</v>
       </c>
       <c r="W19" t="n">
         <v>2</v>
       </c>
       <c r="X19" t="n">
-        <v>-0.1203052475609041</v>
+        <v>0.1635244015426689</v>
       </c>
       <c r="Y19" t="n">
-        <v>0.529648327183757</v>
+        <v>0.7994932014008501</v>
       </c>
       <c r="Z19" t="n">
-        <v>1.45</v>
+        <v>1.48</v>
       </c>
       <c r="AA19" t="inlineStr">
         <is>
@@ -2335,26 +2335,26 @@
         </is>
       </c>
       <c r="AB19" t="n">
-        <v>0.5811280432816868</v>
+        <v>6.395945611206802</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="inlineStr">
         <is>
-          <t>4j4daWNj</t>
+          <t>Y3HtSLcf</t>
         </is>
       </c>
       <c r="B20" s="2" t="n">
-        <v>45675.70833333334</v>
+        <v>45682.70833333334</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>getafe</t>
+          <t>valladolid</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>barcelona</t>
+          <t>real madrid</t>
         </is>
       </c>
       <c r="E20" t="n">
@@ -2374,37 +2374,37 @@
         </is>
       </c>
       <c r="I20" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="J20" t="n">
-        <v>4.1</v>
+        <v>5.25</v>
       </c>
       <c r="K20" t="n">
-        <v>1.48</v>
+        <v>1.33</v>
       </c>
       <c r="L20" t="n">
-        <v>0.1344619748271583</v>
+        <v>0.105471847739889</v>
       </c>
       <c r="M20" t="n">
-        <v>0.2295692253146606</v>
+        <v>0.1808088818398097</v>
       </c>
       <c r="N20" t="n">
-        <v>0.6359687998581812</v>
+        <v>0.7137192704203014</v>
       </c>
       <c r="O20" t="n">
-        <v>0.06243525755720869</v>
+        <v>0.05346700083542189</v>
       </c>
       <c r="P20" t="n">
         <v>2</v>
       </c>
       <c r="Q20" t="n">
-        <v>0.1382151566107977</v>
+        <v>0.05536201709256244</v>
       </c>
       <c r="R20" t="n">
-        <v>0.1964759705777878</v>
+        <v>0.1764308588225157</v>
       </c>
       <c r="S20" t="n">
-        <v>0.6653088728114145</v>
+        <v>0.7682071240849219</v>
       </c>
       <c r="T20" t="n">
         <v>1</v>
@@ -2413,19 +2413,19 @@
         <v>0</v>
       </c>
       <c r="V20" t="n">
-        <v>0.02934007295323326</v>
+        <v>0.0544878536646205</v>
       </c>
       <c r="W20" t="n">
         <v>2</v>
       </c>
       <c r="X20" t="n">
-        <v>0.02934007295323326</v>
+        <v>0.0544878536646205</v>
       </c>
       <c r="Y20" t="n">
-        <v>0.6653088728114145</v>
+        <v>0.7682071240849219</v>
       </c>
       <c r="Z20" t="n">
-        <v>1.48</v>
+        <v>1.33</v>
       </c>
       <c r="AA20" t="inlineStr">
         <is>
@@ -2433,26 +2433,26 @@
         </is>
       </c>
       <c r="AB20" t="n">
-        <v>7.983706473736974</v>
+        <v>6.145656992679375</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="inlineStr">
         <is>
-          <t>Y3HtSLcf</t>
+          <t>xxOXTsTs</t>
         </is>
       </c>
       <c r="B21" s="2" t="n">
-        <v>45682.70833333334</v>
+        <v>45683.41666666666</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>valladolid</t>
+          <t>rayo vallecano</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>real madrid</t>
+          <t>girona</t>
         </is>
       </c>
       <c r="E21" t="n">
@@ -2472,37 +2472,37 @@
         </is>
       </c>
       <c r="I21" t="n">
-        <v>9</v>
+        <v>2.88</v>
       </c>
       <c r="J21" t="n">
-        <v>5.25</v>
+        <v>2.88</v>
       </c>
       <c r="K21" t="n">
-        <v>1.33</v>
+        <v>2.7</v>
       </c>
       <c r="L21" t="n">
-        <v>0.105471847739889</v>
+        <v>0.3260869565217391</v>
       </c>
       <c r="M21" t="n">
-        <v>0.1808088818398097</v>
+        <v>0.3260869565217391</v>
       </c>
       <c r="N21" t="n">
-        <v>0.7137192704203014</v>
+        <v>0.3478260869565217</v>
       </c>
       <c r="O21" t="n">
-        <v>0.05346700083542189</v>
+        <v>0.06481481481481488</v>
       </c>
       <c r="P21" t="n">
         <v>2</v>
       </c>
       <c r="Q21" t="n">
-        <v>0.03756016662428575</v>
+        <v>0.1760890462195282</v>
       </c>
       <c r="R21" t="n">
-        <v>0.2855909604340587</v>
+        <v>0.4081263905874344</v>
       </c>
       <c r="S21" t="n">
-        <v>0.6768488729416556</v>
+        <v>0.4157845631930372</v>
       </c>
       <c r="T21" t="n">
         <v>1</v>
@@ -2511,19 +2511,19 @@
         <v>0</v>
       </c>
       <c r="V21" t="n">
-        <v>-0.03687039747864573</v>
+        <v>0.06795847623651557</v>
       </c>
       <c r="W21" t="n">
         <v>2</v>
       </c>
       <c r="X21" t="n">
-        <v>-0.03687039747864573</v>
+        <v>0.06795847623651557</v>
       </c>
       <c r="Y21" t="n">
-        <v>0.6768488729416556</v>
+        <v>0.4157845631930372</v>
       </c>
       <c r="Z21" t="n">
-        <v>1.33</v>
+        <v>2.7</v>
       </c>
       <c r="AA21" t="inlineStr">
         <is>
@@ -2531,7 +2531,7 @@
         </is>
       </c>
       <c r="AB21" t="n">
-        <v>6.352407396324872</v>
+        <v>3.326276505544298</v>
       </c>
     </row>
     <row r="22">
@@ -2594,13 +2594,13 @@
         <v>2</v>
       </c>
       <c r="Q22" t="n">
-        <v>0.1266422402886511</v>
+        <v>0.1527852016672188</v>
       </c>
       <c r="R22" t="n">
-        <v>0.4187807165387002</v>
+        <v>0.3602924143906949</v>
       </c>
       <c r="S22" t="n">
-        <v>0.4545770431726487</v>
+        <v>0.4869223839420863</v>
       </c>
       <c r="T22" t="n">
         <v>1</v>
@@ -2609,16 +2609,16 @@
         <v>0</v>
       </c>
       <c r="V22" t="n">
-        <v>0.1059669755543166</v>
+        <v>0.1383123163237542</v>
       </c>
       <c r="W22" t="n">
         <v>2</v>
       </c>
       <c r="X22" t="n">
-        <v>0.1059669755543166</v>
+        <v>0.1383123163237542</v>
       </c>
       <c r="Y22" t="n">
-        <v>0.4545770431726487</v>
+        <v>0.4869223839420863</v>
       </c>
       <c r="Z22" t="n">
         <v>2.7</v>
@@ -2629,7 +2629,7 @@
         </is>
       </c>
       <c r="AB22" t="n">
-        <v>5.454924518071784</v>
+        <v>3.89537907153669</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
DATA. Actualizo predicciones tras cambio en betting strategy (b ≠ por resultado)
</commit_message>
<xml_diff>
--- a/data/predicciones.xlsx
+++ b/data/predicciones.xlsx
@@ -677,7 +677,7 @@
         </is>
       </c>
       <c r="AC2" t="n">
-        <v>2.212865364295014</v>
+        <v>1.852911555386943</v>
       </c>
     </row>
     <row r="3">
@@ -879,7 +879,7 @@
         </is>
       </c>
       <c r="AC4" t="n">
-        <v>1.289069572918791</v>
+        <v>2.025350820818737</v>
       </c>
     </row>
     <row r="5">
@@ -980,7 +980,7 @@
         </is>
       </c>
       <c r="AC5" t="n">
-        <v>1.18538321269683</v>
+        <v>1.021640326178215</v>
       </c>
     </row>
     <row r="6">
@@ -1081,7 +1081,7 @@
         </is>
       </c>
       <c r="AC6" t="n">
-        <v>5.322809868342301</v>
+        <v>3.462237781793743</v>
       </c>
     </row>
     <row r="7">
@@ -1182,7 +1182,7 @@
         </is>
       </c>
       <c r="AC7" t="n">
-        <v>0</v>
+        <v>0.604161136239777</v>
       </c>
     </row>
     <row r="8">
@@ -2519,7 +2519,7 @@
         </is>
       </c>
       <c r="AC22" t="n">
-        <v>0</v>
+        <v>0.7604136691603824</v>
       </c>
     </row>
     <row r="23">
@@ -2620,7 +2620,7 @@
         </is>
       </c>
       <c r="AC23" t="n">
-        <v>1.227643351944434</v>
+        <v>2.681612749560419</v>
       </c>
     </row>
     <row r="24">
@@ -2822,7 +2822,7 @@
         </is>
       </c>
       <c r="AC25" t="n">
-        <v>2.358542469525512</v>
+        <v>3.316845252541551</v>
       </c>
     </row>
     <row r="26">
@@ -2923,7 +2923,7 @@
         </is>
       </c>
       <c r="AC26" t="n">
-        <v>0</v>
+        <v>1.816528771201623</v>
       </c>
     </row>
     <row r="27">
@@ -3024,7 +3024,7 @@
         </is>
       </c>
       <c r="AC27" t="n">
-        <v>0.7733816287629811</v>
+        <v>2.059488276366756</v>
       </c>
     </row>
     <row r="28">
@@ -3226,7 +3226,7 @@
         </is>
       </c>
       <c r="AC29" t="n">
-        <v>1.730395029496366</v>
+        <v>3.428374917913574</v>
       </c>
     </row>
     <row r="30">
@@ -4572,7 +4572,7 @@
         </is>
       </c>
       <c r="AC43" t="n">
-        <v>2.505169654090739</v>
+        <v>1.645076890305358</v>
       </c>
     </row>
     <row r="44">
@@ -4671,7 +4671,7 @@
         </is>
       </c>
       <c r="AC44" t="n">
-        <v>2.966515191997904</v>
+        <v>1.966515191997905</v>
       </c>
     </row>
     <row r="45">
@@ -4770,7 +4770,7 @@
         </is>
       </c>
       <c r="AC45" t="n">
-        <v>2.265607066758001</v>
+        <v>1.265607066758001</v>
       </c>
     </row>
     <row r="46">
@@ -4869,7 +4869,7 @@
         </is>
       </c>
       <c r="AC46" t="n">
-        <v>2.401059920258104</v>
+        <v>1.401059920258104</v>
       </c>
     </row>
     <row r="47">
@@ -4968,7 +4968,7 @@
         </is>
       </c>
       <c r="AC47" t="n">
-        <v>2.352783988829092</v>
+        <v>1.352783988829092</v>
       </c>
     </row>
     <row r="48">
@@ -5067,7 +5067,7 @@
         </is>
       </c>
       <c r="AC48" t="n">
-        <v>2.484203354874458</v>
+        <v>1.484203354874458</v>
       </c>
     </row>
     <row r="49">
@@ -5166,7 +5166,7 @@
         </is>
       </c>
       <c r="AC49" t="n">
-        <v>2.261488872492219</v>
+        <v>1.26148887249222</v>
       </c>
     </row>
     <row r="50">
@@ -7637,7 +7637,7 @@
         </is>
       </c>
       <c r="AC76" t="n">
-        <v>7.265510037650245</v>
+        <v>1.265510037650245</v>
       </c>
     </row>
     <row r="77">
@@ -7738,7 +7738,7 @@
         </is>
       </c>
       <c r="AC77" t="n">
-        <v>7.532184514172696</v>
+        <v>1.532184514172697</v>
       </c>
     </row>
     <row r="78">
@@ -7839,7 +7839,7 @@
         </is>
       </c>
       <c r="AC78" t="n">
-        <v>12.29034546967975</v>
+        <v>6.290345469679751</v>
       </c>
     </row>
     <row r="79">
@@ -7940,7 +7940,7 @@
         </is>
       </c>
       <c r="AC79" t="n">
-        <v>9.710385231374911</v>
+        <v>3.710385231374911</v>
       </c>
     </row>
     <row r="80">
@@ -8041,7 +8041,7 @@
         </is>
       </c>
       <c r="AC80" t="n">
-        <v>6.089313071082018</v>
+        <v>0.08931307108201877</v>
       </c>
     </row>
     <row r="81">
@@ -8142,7 +8142,7 @@
         </is>
       </c>
       <c r="AC81" t="n">
-        <v>9.760957332184347</v>
+        <v>3.760957332184347</v>
       </c>
     </row>
     <row r="82">
@@ -8243,7 +8243,7 @@
         </is>
       </c>
       <c r="AC82" t="n">
-        <v>6.20408316119806</v>
+        <v>0.20408316119806</v>
       </c>
     </row>
     <row r="83">
@@ -8344,7 +8344,7 @@
         </is>
       </c>
       <c r="AC83" t="n">
-        <v>12.79541592816042</v>
+        <v>6.795415928160416</v>
       </c>
     </row>
     <row r="84">
@@ -8445,7 +8445,7 @@
         </is>
       </c>
       <c r="AC84" t="n">
-        <v>10.67859267352226</v>
+        <v>4.678592673522261</v>
       </c>
     </row>
     <row r="85">
@@ -8546,7 +8546,7 @@
         </is>
       </c>
       <c r="AC85" t="n">
-        <v>7.718784068028782</v>
+        <v>1.718784068028782</v>
       </c>
     </row>
     <row r="86">
@@ -8647,7 +8647,7 @@
         </is>
       </c>
       <c r="AC86" t="n">
-        <v>6.242338935086154</v>
+        <v>0.2423389350861545</v>
       </c>
     </row>
     <row r="87">
@@ -8748,7 +8748,7 @@
         </is>
       </c>
       <c r="AC87" t="n">
-        <v>6.879662951380382</v>
+        <v>0.8796629513803822</v>
       </c>
     </row>
     <row r="88">
@@ -9657,7 +9657,7 @@
         </is>
       </c>
       <c r="AC96" t="n">
-        <v>9.110537544545624</v>
+        <v>6.527174353470441</v>
       </c>
     </row>
     <row r="97">
@@ -9756,7 +9756,7 @@
         </is>
       </c>
       <c r="AC97" t="n">
-        <v>3.611803522184147</v>
+        <v>4.349106316676669</v>
       </c>
     </row>
     <row r="98">
@@ -9855,7 +9855,7 @@
         </is>
       </c>
       <c r="AC98" t="n">
-        <v>2.218260699220416</v>
+        <v>3.982618379158188</v>
       </c>
     </row>
     <row r="99">
@@ -9954,7 +9954,7 @@
         </is>
       </c>
       <c r="AC99" t="n">
-        <v>2.893064175215955</v>
+        <v>6.193282251259419</v>
       </c>
     </row>
     <row r="100">
@@ -10053,7 +10053,7 @@
         </is>
       </c>
       <c r="AC100" t="n">
-        <v>2.381799121981961</v>
+        <v>3.41634530288355</v>
       </c>
     </row>
     <row r="101">
@@ -10152,7 +10152,7 @@
         </is>
       </c>
       <c r="AC101" t="n">
-        <v>1.990066537840891</v>
+        <v>4.255802096236626</v>
       </c>
     </row>
     <row r="102">
@@ -10251,7 +10251,7 @@
         </is>
       </c>
       <c r="AC102" t="n">
-        <v>1.084208070814662</v>
+        <v>4.465980814891067</v>
       </c>
     </row>
     <row r="103">
@@ -10350,7 +10350,7 @@
         </is>
       </c>
       <c r="AC103" t="n">
-        <v>0</v>
+        <v>4.154353041060308</v>
       </c>
     </row>
     <row r="104">
@@ -10449,7 +10449,7 @@
         </is>
       </c>
       <c r="AC104" t="n">
-        <v>1.826594088018081</v>
+        <v>5.475995762919729</v>
       </c>
     </row>
     <row r="105">
@@ -10716,7 +10716,7 @@
         <v>0.4712129007212892</v>
       </c>
       <c r="S107" t="n">
-        <v>0.305391910675529</v>
+        <v>0.3053919106755289</v>
       </c>
       <c r="T107" t="n">
         <v>1</v>
@@ -11112,7 +11112,7 @@
         <v>0.5197697644699125</v>
       </c>
       <c r="S111" t="n">
-        <v>0.1978719678240424</v>
+        <v>0.1978719678240425</v>
       </c>
       <c r="T111" t="n">
         <v>1</v>
@@ -11241,7 +11241,7 @@
         </is>
       </c>
       <c r="AC112" t="n">
-        <v>0.2975476788144791</v>
+        <v>1.677596327746554</v>
       </c>
     </row>
     <row r="113">

</xml_diff>

<commit_message>
Data. Actualizo data con nueva estrategia
</commit_message>
<xml_diff>
--- a/data/predicciones.xlsx
+++ b/data/predicciones.xlsx
@@ -677,7 +677,7 @@
         </is>
       </c>
       <c r="AC2" t="n">
-        <v>0.9771152823397535</v>
+        <v>0.5271152823397536</v>
       </c>
     </row>
     <row r="3">
@@ -778,7 +778,7 @@
         </is>
       </c>
       <c r="AC3" t="n">
-        <v>2.093852733892531</v>
+        <v>1.643852733892531</v>
       </c>
     </row>
     <row r="4">
@@ -980,7 +980,7 @@
         </is>
       </c>
       <c r="AC5" t="n">
-        <v>3.713392207954464</v>
+        <v>3.263392207954464</v>
       </c>
     </row>
     <row r="6">
@@ -1081,7 +1081,7 @@
         </is>
       </c>
       <c r="AC6" t="n">
-        <v>4.598540078293374</v>
+        <v>4.148540078293374</v>
       </c>
     </row>
     <row r="7">
@@ -1182,7 +1182,7 @@
         </is>
       </c>
       <c r="AC7" t="n">
-        <v>3.815121939346301</v>
+        <v>8.3151219393463</v>
       </c>
     </row>
     <row r="8">
@@ -1887,7 +1887,7 @@
         </is>
       </c>
       <c r="AC14" t="n">
-        <v>2.617019598995019</v>
+        <v>4.530512787196848</v>
       </c>
     </row>
     <row r="15">
@@ -1986,7 +1986,7 @@
         </is>
       </c>
       <c r="AC15" t="n">
-        <v>2.963176061268277</v>
+        <v>5.06125930297017</v>
       </c>
     </row>
     <row r="16">
@@ -2085,7 +2085,7 @@
         </is>
       </c>
       <c r="AC16" t="n">
-        <v>2.13196713044545</v>
+        <v>3.728534196674211</v>
       </c>
     </row>
     <row r="17">
@@ -2184,7 +2184,7 @@
         </is>
       </c>
       <c r="AC17" t="n">
-        <v>1.86424338893615</v>
+        <v>3.090913584851023</v>
       </c>
     </row>
     <row r="18">
@@ -2283,7 +2283,7 @@
         </is>
       </c>
       <c r="AC18" t="n">
-        <v>2.173805001186003</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19">
@@ -2382,7 +2382,7 @@
         </is>
       </c>
       <c r="AC19" t="n">
-        <v>2.160035546966248</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20">
@@ -3372,7 +3372,7 @@
         </is>
       </c>
       <c r="AC29" t="n">
-        <v>4.264222391183198</v>
+        <v>3.664222391183198</v>
       </c>
     </row>
     <row r="30">
@@ -3471,7 +3471,7 @@
         </is>
       </c>
       <c r="AC30" t="n">
-        <v>3.739107548780254</v>
+        <v>3.139107548780254</v>
       </c>
     </row>
     <row r="31">
@@ -3570,7 +3570,7 @@
         </is>
       </c>
       <c r="AC31" t="n">
-        <v>5.277550944897574</v>
+        <v>4.677550944897575</v>
       </c>
     </row>
     <row r="32">
@@ -5075,7 +5075,7 @@
         </is>
       </c>
       <c r="AC46" t="n">
-        <v>5.166862790561393</v>
+        <v>12.66686279056139</v>
       </c>
     </row>
     <row r="47">
@@ -5174,7 +5174,7 @@
         </is>
       </c>
       <c r="AC47" t="n">
-        <v>5.417434482523507</v>
+        <v>12.91743448252351</v>
       </c>
     </row>
     <row r="48">
@@ -5273,7 +5273,7 @@
         </is>
       </c>
       <c r="AC48" t="n">
-        <v>8.160855635124749</v>
+        <v>9.660855635124749</v>
       </c>
     </row>
     <row r="49">
@@ -5372,7 +5372,7 @@
         </is>
       </c>
       <c r="AC49" t="n">
-        <v>6.916292438649586</v>
+        <v>8.416292438649586</v>
       </c>
     </row>
     <row r="50">
@@ -5471,7 +5471,7 @@
         </is>
       </c>
       <c r="AC50" t="n">
-        <v>4.556513843712848</v>
+        <v>6.056513843712848</v>
       </c>
     </row>
     <row r="51">
@@ -5570,7 +5570,7 @@
         </is>
       </c>
       <c r="AC51" t="n">
-        <v>3.108747899479221</v>
+        <v>4.608747899479221</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
DATA. Actualizo predicciones tras cambiar modelo en ENG y arreglar formato de missing en ultimos partidos.
</commit_message>
<xml_diff>
--- a/data/predicciones.xlsx
+++ b/data/predicciones.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC49"/>
+  <dimension ref="A1:AC48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -615,37 +615,37 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>1.62</v>
+        <v>1.6</v>
       </c>
       <c r="J2" t="n">
-        <v>4.2</v>
+        <v>4.33</v>
       </c>
       <c r="K2" t="n">
         <v>5</v>
       </c>
       <c r="L2" t="n">
-        <v>0.5848930481283423</v>
+        <v>0.5918858330143802</v>
       </c>
       <c r="M2" t="n">
-        <v>0.2256016042780749</v>
+        <v>0.2187107004210181</v>
       </c>
       <c r="N2" t="n">
-        <v>0.1895053475935829</v>
+        <v>0.1894034665646017</v>
       </c>
       <c r="O2" t="n">
-        <v>0.0553791887125219</v>
+        <v>0.0559468822170901</v>
       </c>
       <c r="P2" t="n">
         <v>1</v>
       </c>
       <c r="Q2" t="n">
-        <v>0.6326741178897731</v>
+        <v>0.5114076458506506</v>
       </c>
       <c r="R2" t="n">
-        <v>0.1758420997675452</v>
+        <v>0.3278921041229221</v>
       </c>
       <c r="S2" t="n">
-        <v>0.1914837823426818</v>
+        <v>0.1607002500264273</v>
       </c>
       <c r="T2" t="n">
         <v>1</v>
@@ -657,19 +657,19 @@
         <v>0</v>
       </c>
       <c r="W2" t="n">
-        <v>0.04778106976143082</v>
+        <v>-0.08047818716372968</v>
       </c>
       <c r="X2" t="n">
         <v>1</v>
       </c>
       <c r="Y2" t="n">
-        <v>0.04778106976143082</v>
+        <v>-0.08047818716372968</v>
       </c>
       <c r="Z2" t="n">
-        <v>0.6326741178897731</v>
+        <v>0.5114076458506506</v>
       </c>
       <c r="AA2" t="n">
-        <v>1.62</v>
+        <v>1.6</v>
       </c>
       <c r="AB2" t="inlineStr">
         <is>
@@ -677,26 +677,26 @@
         </is>
       </c>
       <c r="AC2" t="n">
-        <v>0</v>
+        <v>1.354061443708721</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>hMkFPYKG</t>
+          <t>CQMutf5c</t>
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>45675.60416666666</v>
+        <v>45676.45833333334</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>arsenal</t>
+          <t>everton</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>aston villa</t>
+          <t>tottenham</t>
         </is>
       </c>
       <c r="E3" t="n">
@@ -716,37 +716,37 @@
         </is>
       </c>
       <c r="I3" t="n">
-        <v>1.48</v>
+        <v>2.8</v>
       </c>
       <c r="J3" t="n">
-        <v>4.1</v>
+        <v>3.5</v>
       </c>
       <c r="K3" t="n">
-        <v>7</v>
+        <v>2.45</v>
       </c>
       <c r="L3" t="n">
-        <v>0.6359687998581812</v>
+        <v>0.3398058252427185</v>
       </c>
       <c r="M3" t="n">
-        <v>0.2295692253146606</v>
+        <v>0.2718446601941747</v>
       </c>
       <c r="N3" t="n">
-        <v>0.1344619748271583</v>
+        <v>0.3883495145631068</v>
       </c>
       <c r="O3" t="n">
-        <v>0.06243525755720869</v>
+        <v>0.05102040816326525</v>
       </c>
       <c r="P3" t="n">
         <v>1</v>
       </c>
       <c r="Q3" t="n">
-        <v>0.4600253226596581</v>
+        <v>0.3984480646195233</v>
       </c>
       <c r="R3" t="n">
-        <v>0.3265115660047451</v>
+        <v>0.2917962523932104</v>
       </c>
       <c r="S3" t="n">
-        <v>0.2134631113355968</v>
+        <v>0.3097556829872662</v>
       </c>
       <c r="T3" t="n">
         <v>1</v>
@@ -758,19 +758,19 @@
         <v>0</v>
       </c>
       <c r="W3" t="n">
-        <v>-0.1759434771985231</v>
+        <v>0.05864223937680485</v>
       </c>
       <c r="X3" t="n">
         <v>1</v>
       </c>
       <c r="Y3" t="n">
-        <v>-0.1759434771985231</v>
+        <v>0.05864223937680485</v>
       </c>
       <c r="Z3" t="n">
-        <v>0.4600253226596581</v>
+        <v>0.3984480646195233</v>
       </c>
       <c r="AA3" t="n">
-        <v>1.48</v>
+        <v>2.8</v>
       </c>
       <c r="AB3" t="inlineStr">
         <is>
@@ -778,7 +778,7 @@
         </is>
       </c>
       <c r="AC3" t="n">
-        <v>0</v>
+        <v>1.78603258157571</v>
       </c>
     </row>
     <row r="4">
@@ -817,37 +817,37 @@
         </is>
       </c>
       <c r="I4" t="n">
-        <v>2.05</v>
+        <v>2.1</v>
       </c>
       <c r="J4" t="n">
         <v>3.6</v>
       </c>
       <c r="K4" t="n">
-        <v>3.4</v>
+        <v>3.3</v>
       </c>
       <c r="L4" t="n">
-        <v>0.4603234298608499</v>
+        <v>0.4505119453924915</v>
       </c>
       <c r="M4" t="n">
-        <v>0.2621286197818729</v>
+        <v>0.2627986348122867</v>
       </c>
       <c r="N4" t="n">
-        <v>0.2775479503572771</v>
+        <v>0.2866894197952219</v>
       </c>
       <c r="O4" t="n">
-        <v>0.05970030288538197</v>
+        <v>0.05699855699855694</v>
       </c>
       <c r="P4" t="n">
         <v>1</v>
       </c>
       <c r="Q4" t="n">
-        <v>0.6219963769927466</v>
+        <v>0.6982467434109429</v>
       </c>
       <c r="R4" t="n">
-        <v>0.3138934003294714</v>
+        <v>0.08187118821184748</v>
       </c>
       <c r="S4" t="n">
-        <v>0.06411022267778203</v>
+        <v>0.2198820683772096</v>
       </c>
       <c r="T4" t="n">
         <v>1</v>
@@ -859,19 +859,19 @@
         <v>0</v>
       </c>
       <c r="W4" t="n">
-        <v>0.1616729471318967</v>
+        <v>0.2477347980184515</v>
       </c>
       <c r="X4" t="n">
         <v>1</v>
       </c>
       <c r="Y4" t="n">
-        <v>0.1616729471318967</v>
+        <v>0.2477347980184515</v>
       </c>
       <c r="Z4" t="n">
-        <v>0.6219963769927466</v>
+        <v>0.6982467434109429</v>
       </c>
       <c r="AA4" t="n">
-        <v>2.05</v>
+        <v>2.1</v>
       </c>
       <c r="AB4" t="inlineStr">
         <is>
@@ -879,26 +879,26 @@
         </is>
       </c>
       <c r="AC4" t="n">
-        <v>0</v>
+        <v>4.484220690698487</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>WtIFhXl3</t>
+          <t>KWZgIjDj</t>
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>45676.45833333334</v>
+        <v>45677.70833333334</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>nottingham</t>
+          <t>chelsea</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>southampton</t>
+          <t>wolves</t>
         </is>
       </c>
       <c r="E5" t="n">
@@ -918,37 +918,37 @@
         </is>
       </c>
       <c r="I5" t="n">
-        <v>1.42</v>
+        <v>1.36</v>
       </c>
       <c r="J5" t="n">
-        <v>4.75</v>
+        <v>5.75</v>
       </c>
       <c r="K5" t="n">
-        <v>7.5</v>
+        <v>6.5</v>
       </c>
       <c r="L5" t="n">
-        <v>0.6719162580158431</v>
+        <v>0.6916813176644768</v>
       </c>
       <c r="M5" t="n">
-        <v>0.2008675971331573</v>
+        <v>0.1635976681780328</v>
       </c>
       <c r="N5" t="n">
-        <v>0.1272161448509996</v>
+        <v>0.1447210141574906</v>
       </c>
       <c r="O5" t="n">
-        <v>0.0480850012354832</v>
+        <v>0.06305331497147337</v>
       </c>
       <c r="P5" t="n">
         <v>1</v>
       </c>
       <c r="Q5" t="n">
-        <v>0.467758289691255</v>
+        <v>0.7093270030604</v>
       </c>
       <c r="R5" t="n">
-        <v>0.4418630144542261</v>
+        <v>0.1414551179088045</v>
       </c>
       <c r="S5" t="n">
-        <v>0.09037869585451891</v>
+        <v>0.1492178790307955</v>
       </c>
       <c r="T5" t="n">
         <v>1</v>
@@ -960,19 +960,19 @@
         <v>0</v>
       </c>
       <c r="W5" t="n">
-        <v>-0.2041579683245881</v>
+        <v>0.01764568539592315</v>
       </c>
       <c r="X5" t="n">
         <v>1</v>
       </c>
       <c r="Y5" t="n">
-        <v>-0.2041579683245881</v>
+        <v>0.01764568539592315</v>
       </c>
       <c r="Z5" t="n">
-        <v>0.467758289691255</v>
+        <v>0.7093270030604</v>
       </c>
       <c r="AA5" t="n">
-        <v>1.42</v>
+        <v>1.36</v>
       </c>
       <c r="AB5" t="inlineStr">
         <is>
@@ -980,26 +980,26 @@
         </is>
       </c>
       <c r="AC5" t="n">
-        <v>0</v>
+        <v>4.5839430275436</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>KWZgIjDj</t>
+          <t>vgtkxC4M</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>45677.70833333334</v>
+        <v>45675.5</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>chelsea</t>
+          <t>leicester</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>wolves</t>
+          <t>fulham</t>
         </is>
       </c>
       <c r="E6" t="n">
@@ -1019,37 +1019,37 @@
         </is>
       </c>
       <c r="I6" t="n">
-        <v>1.33</v>
+        <v>4.33</v>
       </c>
       <c r="J6" t="n">
-        <v>6</v>
+        <v>3.7</v>
       </c>
       <c r="K6" t="n">
-        <v>7</v>
+        <v>1.8</v>
       </c>
       <c r="L6" t="n">
-        <v>0.7083825265643447</v>
+        <v>0.2185397867104184</v>
       </c>
       <c r="M6" t="n">
-        <v>0.1570247933884298</v>
+        <v>0.2557506152584085</v>
       </c>
       <c r="N6" t="n">
-        <v>0.1345926800472255</v>
+        <v>0.5257095980311731</v>
       </c>
       <c r="O6" t="n">
-        <v>0.06140350877192979</v>
+        <v>0.0567727080429159</v>
       </c>
       <c r="P6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q6" t="n">
-        <v>0.481804720237996</v>
+        <v>0.1869333597957384</v>
       </c>
       <c r="R6" t="n">
-        <v>0.4149935099620544</v>
+        <v>0.4282632081078129</v>
       </c>
       <c r="S6" t="n">
-        <v>0.1032017697999496</v>
+        <v>0.3848034320964487</v>
       </c>
       <c r="T6" t="n">
         <v>1</v>
@@ -1061,19 +1061,19 @@
         <v>0</v>
       </c>
       <c r="W6" t="n">
-        <v>-0.2265778063263488</v>
+        <v>0.1725125928494045</v>
       </c>
       <c r="X6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Y6" t="n">
-        <v>-0.2265778063263488</v>
+        <v>0.1725125928494045</v>
       </c>
       <c r="Z6" t="n">
-        <v>0.481804720237996</v>
+        <v>0.4282632081078129</v>
       </c>
       <c r="AA6" t="n">
-        <v>1.33</v>
+        <v>3.7</v>
       </c>
       <c r="AB6" t="inlineStr">
         <is>
@@ -1081,26 +1081,26 @@
         </is>
       </c>
       <c r="AC6" t="n">
-        <v>0</v>
+        <v>4.754368872970316</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>4fGNjBJF</t>
+          <t>hMkFPYKG</t>
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>45675.5</v>
+        <v>45675.60416666666</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>west ham</t>
+          <t>arsenal</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>crystal palace</t>
+          <t>aston villa</t>
         </is>
       </c>
       <c r="E7" t="n">
@@ -1120,37 +1120,37 @@
         </is>
       </c>
       <c r="I7" t="n">
-        <v>2.7</v>
+        <v>1.5</v>
       </c>
       <c r="J7" t="n">
-        <v>3.25</v>
+        <v>4.1</v>
       </c>
       <c r="K7" t="n">
-        <v>2.7</v>
+        <v>7</v>
       </c>
       <c r="L7" t="n">
-        <v>0.3532608695652174</v>
+        <v>0.6328555678059536</v>
       </c>
       <c r="M7" t="n">
-        <v>0.2934782608695652</v>
+        <v>0.2315325248070562</v>
       </c>
       <c r="N7" t="n">
-        <v>0.3532608695652174</v>
+        <v>0.1356119073869901</v>
       </c>
       <c r="O7" t="n">
-        <v>0.04843304843304841</v>
+        <v>0.05342624854819977</v>
       </c>
       <c r="P7" t="n">
         <v>0</v>
       </c>
       <c r="Q7" t="n">
-        <v>0.3522049242986355</v>
+        <v>0.3433664173152183</v>
       </c>
       <c r="R7" t="n">
-        <v>0.3688488547905101</v>
+        <v>0.4469060169409866</v>
       </c>
       <c r="S7" t="n">
-        <v>0.2789462209108544</v>
+        <v>0.2097275657437951</v>
       </c>
       <c r="T7" t="n">
         <v>1</v>
@@ -1162,19 +1162,19 @@
         <v>0</v>
       </c>
       <c r="W7" t="n">
-        <v>0.07537059392094486</v>
+        <v>0.2153734921339304</v>
       </c>
       <c r="X7" t="n">
         <v>0</v>
       </c>
       <c r="Y7" t="n">
-        <v>0.07537059392094486</v>
+        <v>0.2153734921339304</v>
       </c>
       <c r="Z7" t="n">
-        <v>0.3688488547905101</v>
+        <v>0.4469060169409866</v>
       </c>
       <c r="AA7" t="n">
-        <v>3.25</v>
+        <v>4.1</v>
       </c>
       <c r="AB7" t="inlineStr">
         <is>
@@ -1182,7 +1182,7 @@
         </is>
       </c>
       <c r="AC7" t="n">
-        <v>4.219639693114591</v>
+        <v>4.92215415246888</v>
       </c>
     </row>
     <row r="8">
@@ -1221,37 +1221,37 @@
         </is>
       </c>
       <c r="I8" t="n">
-        <v>6.25</v>
+        <v>6.5</v>
       </c>
       <c r="J8" t="n">
-        <v>4.75</v>
+        <v>5</v>
       </c>
       <c r="K8" t="n">
-        <v>1.45</v>
+        <v>1.42</v>
       </c>
       <c r="L8" t="n">
-        <v>0.1509175568337442</v>
+        <v>0.1454024165472046</v>
       </c>
       <c r="M8" t="n">
-        <v>0.1985757326759792</v>
+        <v>0.189023141511366</v>
       </c>
       <c r="N8" t="n">
-        <v>0.6505067104902768</v>
+        <v>0.6655744419414295</v>
       </c>
       <c r="O8" t="n">
-        <v>0.06018148820326674</v>
+        <v>0.05807150595882993</v>
       </c>
       <c r="P8" t="n">
         <v>2</v>
       </c>
       <c r="Q8" t="n">
-        <v>0.03161872639411436</v>
+        <v>0.0676682026702463</v>
       </c>
       <c r="R8" t="n">
-        <v>0.1577132081774078</v>
+        <v>0.2632735041608344</v>
       </c>
       <c r="S8" t="n">
-        <v>0.8106680654284778</v>
+        <v>0.6690582931689193</v>
       </c>
       <c r="T8" t="n">
         <v>1</v>
@@ -1263,19 +1263,19 @@
         <v>0</v>
       </c>
       <c r="W8" t="n">
-        <v>0.1601613549382011</v>
+        <v>0.003483851227489843</v>
       </c>
       <c r="X8" t="n">
         <v>2</v>
       </c>
       <c r="Y8" t="n">
-        <v>0.1601613549382011</v>
+        <v>0.003483851227489843</v>
       </c>
       <c r="Z8" t="n">
-        <v>0.8106680654284778</v>
+        <v>0.6690582931689193</v>
       </c>
       <c r="AA8" t="n">
-        <v>1.45</v>
+        <v>1.42</v>
       </c>
       <c r="AB8" t="inlineStr">
         <is>
@@ -1283,13 +1283,13 @@
         </is>
       </c>
       <c r="AC8" t="n">
-        <v>8.1960125888563</v>
+        <v>6.921524638520273</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
         <is>
-          <t>vgtkxC4M</t>
+          <t>4fGNjBJF</t>
         </is>
       </c>
       <c r="B9" s="2" t="n">
@@ -1297,12 +1297,12 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>leicester</t>
+          <t>west ham</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>fulham</t>
+          <t>crystal palace</t>
         </is>
       </c>
       <c r="E9" t="n">
@@ -1322,37 +1322,37 @@
         </is>
       </c>
       <c r="I9" t="n">
-        <v>4</v>
+        <v>2.63</v>
       </c>
       <c r="J9" t="n">
-        <v>3.6</v>
+        <v>3.5</v>
       </c>
       <c r="K9" t="n">
-        <v>1.9</v>
+        <v>2.6</v>
       </c>
       <c r="L9" t="n">
-        <v>0.2371705963938974</v>
+        <v>0.3619297617627173</v>
       </c>
       <c r="M9" t="n">
-        <v>0.2635228848821082</v>
+        <v>0.2719643638388418</v>
       </c>
       <c r="N9" t="n">
-        <v>0.4993065187239945</v>
+        <v>0.3661058743984409</v>
       </c>
       <c r="O9" t="n">
-        <v>0.05409356725146197</v>
+        <v>0.05055780721179959</v>
       </c>
       <c r="P9" t="n">
         <v>2</v>
       </c>
       <c r="Q9" t="n">
-        <v>0.1670761994545134</v>
+        <v>0.3387342820447961</v>
       </c>
       <c r="R9" t="n">
-        <v>0.3021970842180285</v>
+        <v>0.2984022651693051</v>
       </c>
       <c r="S9" t="n">
-        <v>0.5307267163274582</v>
+        <v>0.3628634527858988</v>
       </c>
       <c r="T9" t="n">
         <v>1</v>
@@ -1364,19 +1364,19 @@
         <v>0</v>
       </c>
       <c r="W9" t="n">
-        <v>0.03142019760346371</v>
+        <v>-0.003242421612542123</v>
       </c>
       <c r="X9" t="n">
         <v>2</v>
       </c>
       <c r="Y9" t="n">
-        <v>0.03142019760346371</v>
+        <v>-0.003242421612542123</v>
       </c>
       <c r="Z9" t="n">
-        <v>0.5307267163274582</v>
+        <v>0.3628634527858988</v>
       </c>
       <c r="AA9" t="n">
-        <v>1.9</v>
+        <v>2.6</v>
       </c>
       <c r="AB9" t="inlineStr">
         <is>
@@ -1384,13 +1384,13 @@
         </is>
       </c>
       <c r="AC9" t="n">
-        <v>5.676540446947123</v>
+        <v>4.165771075073089</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
         <is>
-          <t>CQMutf5c</t>
+          <t>WtIFhXl3</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
@@ -1398,12 +1398,12 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>everton</t>
+          <t>nottingham</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>tottenham</t>
+          <t>southampton</t>
         </is>
       </c>
       <c r="E10" t="n">
@@ -1423,37 +1423,37 @@
         </is>
       </c>
       <c r="I10" t="n">
-        <v>2.8</v>
+        <v>1.38</v>
       </c>
       <c r="J10" t="n">
-        <v>3.5</v>
+        <v>4.75</v>
       </c>
       <c r="K10" t="n">
-        <v>2.4</v>
+        <v>8</v>
       </c>
       <c r="L10" t="n">
-        <v>0.3370786516853932</v>
+        <v>0.6835147045597626</v>
       </c>
       <c r="M10" t="n">
-        <v>0.2696629213483146</v>
+        <v>0.1985790089036784</v>
       </c>
       <c r="N10" t="n">
-        <v>0.3932584269662922</v>
+        <v>0.117906286536559</v>
       </c>
       <c r="O10" t="n">
-        <v>0.05952380952380953</v>
+        <v>0.06016399694889407</v>
       </c>
       <c r="P10" t="n">
         <v>2</v>
       </c>
       <c r="Q10" t="n">
-        <v>0.2878570412158478</v>
+        <v>0.356019562817172</v>
       </c>
       <c r="R10" t="n">
-        <v>0.2024165581770267</v>
+        <v>0.05582212895481122</v>
       </c>
       <c r="S10" t="n">
-        <v>0.5097264006071256</v>
+        <v>0.5881583082280168</v>
       </c>
       <c r="T10" t="n">
         <v>1</v>
@@ -1465,19 +1465,19 @@
         <v>0</v>
       </c>
       <c r="W10" t="n">
-        <v>0.1164679736408334</v>
+        <v>0.4702520216914578</v>
       </c>
       <c r="X10" t="n">
         <v>2</v>
       </c>
       <c r="Y10" t="n">
-        <v>0.1164679736408334</v>
+        <v>0.4702520216914578</v>
       </c>
       <c r="Z10" t="n">
-        <v>0.5097264006071256</v>
+        <v>0.5881583082280168</v>
       </c>
       <c r="AA10" t="n">
-        <v>2.4</v>
+        <v>8</v>
       </c>
       <c r="AB10" t="inlineStr">
         <is>
@@ -1485,7 +1485,7 @@
         </is>
       </c>
       <c r="AC10" t="n">
-        <v>5.487537605464131</v>
+        <v>6.193424774052152</v>
       </c>
     </row>
     <row r="11">
@@ -1524,37 +1524,37 @@
         </is>
       </c>
       <c r="I11" t="n">
-        <v>8</v>
+        <v>7.5</v>
       </c>
       <c r="J11" t="n">
-        <v>5.5</v>
+        <v>5.25</v>
       </c>
       <c r="K11" t="n">
-        <v>1.33</v>
+        <v>1.36</v>
       </c>
       <c r="L11" t="n">
-        <v>0.1180695666209345</v>
+        <v>0.1258926209997356</v>
       </c>
       <c r="M11" t="n">
-        <v>0.1717375514486321</v>
+        <v>0.1798466014281936</v>
       </c>
       <c r="N11" t="n">
-        <v>0.7101928819304333</v>
+        <v>0.6942607775720709</v>
       </c>
       <c r="O11" t="n">
-        <v>0.05869788106630214</v>
+        <v>0.05910364145658242</v>
       </c>
       <c r="P11" t="n">
         <v>2</v>
       </c>
       <c r="Q11" t="n">
-        <v>0.05776827111272127</v>
+        <v>0.11957244334075</v>
       </c>
       <c r="R11" t="n">
-        <v>0.1155968338440626</v>
+        <v>0.1248982848704146</v>
       </c>
       <c r="S11" t="n">
-        <v>0.8266348950432161</v>
+        <v>0.7555292717888353</v>
       </c>
       <c r="T11" t="n">
         <v>1</v>
@@ -1566,19 +1566,19 @@
         <v>0</v>
       </c>
       <c r="W11" t="n">
-        <v>0.1164420131127828</v>
+        <v>0.06126849421676439</v>
       </c>
       <c r="X11" t="n">
         <v>2</v>
       </c>
       <c r="Y11" t="n">
-        <v>0.1164420131127828</v>
+        <v>0.06126849421676439</v>
       </c>
       <c r="Z11" t="n">
-        <v>0.8266348950432161</v>
+        <v>0.7555292717888353</v>
       </c>
       <c r="AA11" t="n">
-        <v>1.33</v>
+        <v>1.36</v>
       </c>
       <c r="AB11" t="inlineStr">
         <is>
@@ -1586,7 +1586,7 @@
         </is>
       </c>
       <c r="AC11" t="n">
-        <v>8.339714055388944</v>
+        <v>7.699763446099517</v>
       </c>
     </row>
     <row r="12">
@@ -1625,37 +1625,37 @@
         </is>
       </c>
       <c r="I12" t="n">
-        <v>1.95</v>
+        <v>2.15</v>
       </c>
       <c r="J12" t="n">
-        <v>3.75</v>
+        <v>3.4</v>
       </c>
       <c r="K12" t="n">
-        <v>3.5</v>
+        <v>3.4</v>
       </c>
       <c r="L12" t="n">
-        <v>0.4814305364511692</v>
+        <v>0.4415584415584415</v>
       </c>
       <c r="M12" t="n">
-        <v>0.2503438789546079</v>
+        <v>0.2792207792207792</v>
       </c>
       <c r="N12" t="n">
-        <v>0.2682255845942227</v>
+        <v>0.2792207792207792</v>
       </c>
       <c r="O12" t="n">
-        <v>0.06520146520146541</v>
+        <v>0.05335157318741457</v>
       </c>
       <c r="P12" t="n">
         <v>1</v>
       </c>
       <c r="Q12" t="n">
-        <v>0.4172544017988651</v>
+        <v>0.4137335399498263</v>
       </c>
       <c r="R12" t="n">
-        <v>0.2906643598066308</v>
+        <v>0.2936952084550549</v>
       </c>
       <c r="S12" t="n">
-        <v>0.292081238394504</v>
+        <v>0.2925712515951189</v>
       </c>
       <c r="T12" t="n">
         <v>1</v>
@@ -1665,19 +1665,19 @@
       </c>
       <c r="V12" t="inlineStr"/>
       <c r="W12" t="n">
-        <v>-0.06417613465230404</v>
+        <v>-0.02782490160861528</v>
       </c>
       <c r="X12" t="n">
         <v>1</v>
       </c>
       <c r="Y12" t="n">
-        <v>-0.06417613465230404</v>
+        <v>-0.02782490160861528</v>
       </c>
       <c r="Z12" t="n">
-        <v>0.4172544017988651</v>
+        <v>0.4137335399498263</v>
       </c>
       <c r="AA12" t="n">
-        <v>1.95</v>
+        <v>2.15</v>
       </c>
       <c r="AB12" t="inlineStr">
         <is>
@@ -1685,7 +1685,7 @@
         </is>
       </c>
       <c r="AC12" t="n">
-        <v>4.733412794965542</v>
+        <v>5.148502420395574</v>
       </c>
     </row>
     <row r="13">
@@ -1823,7 +1823,7 @@
         </is>
       </c>
       <c r="I14" t="n">
-        <v>1.83</v>
+        <v>1.85</v>
       </c>
       <c r="J14" t="n">
         <v>3.9</v>
@@ -1832,16 +1832,16 @@
         <v>4</v>
       </c>
       <c r="L14" t="n">
-        <v>0.5190138736400838</v>
+        <v>0.5162998510673505</v>
       </c>
       <c r="M14" t="n">
-        <v>0.2435372791695778</v>
+        <v>0.2449114678139997</v>
       </c>
       <c r="N14" t="n">
-        <v>0.2374488471903384</v>
+        <v>0.2387886811186497</v>
       </c>
       <c r="O14" t="n">
-        <v>0.05285834384195032</v>
+        <v>0.04695079695079696</v>
       </c>
       <c r="P14" t="n">
         <v>1</v>
@@ -1863,19 +1863,19 @@
       </c>
       <c r="V14" t="inlineStr"/>
       <c r="W14" t="n">
-        <v>-0.129780529603969</v>
+        <v>-0.1270665070312357</v>
       </c>
       <c r="X14" t="n">
         <v>1</v>
       </c>
       <c r="Y14" t="n">
-        <v>-0.129780529603969</v>
+        <v>-0.1270665070312357</v>
       </c>
       <c r="Z14" t="n">
         <v>0.3892333440361148</v>
       </c>
       <c r="AA14" t="n">
-        <v>1.83</v>
+        <v>1.85</v>
       </c>
       <c r="AB14" t="inlineStr">
         <is>
@@ -1883,7 +1883,7 @@
         </is>
       </c>
       <c r="AC14" t="n">
-        <v>3.778033708969061</v>
+        <v>3.81060197984186</v>
       </c>
     </row>
     <row r="15">
@@ -1946,13 +1946,13 @@
         <v>1</v>
       </c>
       <c r="Q15" t="n">
-        <v>0.3938726932531847</v>
+        <v>0.397646042709287</v>
       </c>
       <c r="R15" t="n">
-        <v>0.343162863005007</v>
+        <v>0.3390616858705089</v>
       </c>
       <c r="S15" t="n">
-        <v>0.2629644437418081</v>
+        <v>0.2632922714202039</v>
       </c>
       <c r="T15" t="n">
         <v>1</v>
@@ -1962,16 +1962,16 @@
       </c>
       <c r="V15" t="inlineStr"/>
       <c r="W15" t="n">
-        <v>-0.2079444729312163</v>
+        <v>-0.2041711234751141</v>
       </c>
       <c r="X15" t="n">
         <v>1</v>
       </c>
       <c r="Y15" t="n">
-        <v>-0.2079444729312163</v>
+        <v>-0.2041711234751141</v>
       </c>
       <c r="Z15" t="n">
-        <v>0.3938726932531847</v>
+        <v>0.397646042709287</v>
       </c>
       <c r="AA15" t="n">
         <v>1.57</v>
@@ -1982,7 +1982,7 @@
         </is>
       </c>
       <c r="AC15" t="n">
-        <v>2.867902484344512</v>
+        <v>2.935822774554353</v>
       </c>
     </row>
     <row r="16">
@@ -2045,13 +2045,13 @@
         <v>0</v>
       </c>
       <c r="Q16" t="n">
-        <v>0.3113130005865305</v>
+        <v>0.3004328746570458</v>
       </c>
       <c r="R16" t="n">
-        <v>0.3587579939966317</v>
+        <v>0.3641164746936828</v>
       </c>
       <c r="S16" t="n">
-        <v>0.3299290054168378</v>
+        <v>0.3354506506492714</v>
       </c>
       <c r="T16" t="n">
         <v>1</v>
@@ -2061,16 +2061,16 @@
       </c>
       <c r="V16" t="inlineStr"/>
       <c r="W16" t="n">
-        <v>0.06866919130192922</v>
+        <v>0.07402767199898036</v>
       </c>
       <c r="X16" t="n">
         <v>0</v>
       </c>
       <c r="Y16" t="n">
-        <v>0.06866919130192922</v>
+        <v>0.07402767199898036</v>
       </c>
       <c r="Z16" t="n">
-        <v>0.3587579939966317</v>
+        <v>0.3641164746936828</v>
       </c>
       <c r="AA16" t="n">
         <v>3.25</v>
@@ -2120,37 +2120,37 @@
         </is>
       </c>
       <c r="I17" t="n">
-        <v>1.65</v>
+        <v>1.62</v>
       </c>
       <c r="J17" t="n">
-        <v>3.9</v>
+        <v>4</v>
       </c>
       <c r="K17" t="n">
         <v>5.25</v>
       </c>
       <c r="L17" t="n">
-        <v>0.5755850727387729</v>
+        <v>0.5835764902042518</v>
       </c>
       <c r="M17" t="n">
-        <v>0.243516761543327</v>
+        <v>0.236348478532722</v>
       </c>
       <c r="N17" t="n">
-        <v>0.1808981657179</v>
+        <v>0.1800750312630263</v>
       </c>
       <c r="O17" t="n">
-        <v>0.05294705294705304</v>
+        <v>0.05776014109347427</v>
       </c>
       <c r="P17" t="n">
         <v>0</v>
       </c>
       <c r="Q17" t="n">
-        <v>0.3256125263669397</v>
+        <v>0.3208821878196372</v>
       </c>
       <c r="R17" t="n">
-        <v>0.3600059244943746</v>
+        <v>0.3616990171979568</v>
       </c>
       <c r="S17" t="n">
-        <v>0.3143815491386857</v>
+        <v>0.3174187949824059</v>
       </c>
       <c r="T17" t="n">
         <v>1</v>
@@ -2160,19 +2160,19 @@
       </c>
       <c r="V17" t="inlineStr"/>
       <c r="W17" t="n">
-        <v>0.1164891629510476</v>
+        <v>0.1253505386652348</v>
       </c>
       <c r="X17" t="n">
         <v>0</v>
       </c>
       <c r="Y17" t="n">
-        <v>0.1164891629510476</v>
+        <v>0.1253505386652348</v>
       </c>
       <c r="Z17" t="n">
-        <v>0.3600059244943746</v>
+        <v>0.3616990171979568</v>
       </c>
       <c r="AA17" t="n">
-        <v>3.9</v>
+        <v>4</v>
       </c>
       <c r="AB17" t="inlineStr">
         <is>
@@ -2186,20 +2186,20 @@
     <row r="18">
       <c r="A18" s="1" t="inlineStr">
         <is>
-          <t>jgXCVB9F</t>
+          <t>xj7wHCfM</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
-        <v>45674.625</v>
+        <v>45675.54166666666</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>montpellier</t>
+          <t>lens</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>monaco</t>
+          <t>psg</t>
         </is>
       </c>
       <c r="E18" t="n">
@@ -2219,37 +2219,37 @@
         </is>
       </c>
       <c r="I18" t="n">
-        <v>5</v>
+        <v>4.5</v>
       </c>
       <c r="J18" t="n">
-        <v>4.75</v>
+        <v>4</v>
       </c>
       <c r="K18" t="n">
-        <v>1.57</v>
+        <v>1.7</v>
       </c>
       <c r="L18" t="n">
-        <v>0.1909364398643026</v>
+        <v>0.2095531587057011</v>
       </c>
       <c r="M18" t="n">
-        <v>0.2009857261729501</v>
+        <v>0.2357473035439137</v>
       </c>
       <c r="N18" t="n">
-        <v>0.6080778339627472</v>
+        <v>0.5546995377503853</v>
       </c>
       <c r="O18" t="n">
-        <v>0.04746899094870938</v>
+        <v>0.06045751633986929</v>
       </c>
       <c r="P18" t="n">
         <v>2</v>
       </c>
       <c r="Q18" t="n">
-        <v>0.1541132090310229</v>
+        <v>0.09658747436562415</v>
       </c>
       <c r="R18" t="n">
-        <v>0.3014249007768399</v>
+        <v>0.294214214041345</v>
       </c>
       <c r="S18" t="n">
-        <v>0.5444618901921372</v>
+        <v>0.6091983115930308</v>
       </c>
       <c r="T18" t="n">
         <v>1</v>
@@ -2259,19 +2259,19 @@
       </c>
       <c r="V18" t="inlineStr"/>
       <c r="W18" t="n">
-        <v>-0.06361594377060997</v>
+        <v>0.05449877384264556</v>
       </c>
       <c r="X18" t="n">
         <v>2</v>
       </c>
       <c r="Y18" t="n">
-        <v>-0.06361594377060997</v>
+        <v>0.05449877384264556</v>
       </c>
       <c r="Z18" t="n">
-        <v>0.5444618901921372</v>
+        <v>0.6091983115930308</v>
       </c>
       <c r="AA18" t="n">
-        <v>1.57</v>
+        <v>1.7</v>
       </c>
       <c r="AB18" t="inlineStr">
         <is>
@@ -2279,26 +2279,26 @@
         </is>
       </c>
       <c r="AC18" t="n">
-        <v>3.103380015905503</v>
+        <v>4.255189869558184</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="inlineStr">
         <is>
-          <t>xj7wHCfM</t>
+          <t>riCiOT1k</t>
         </is>
       </c>
       <c r="B19" s="2" t="n">
-        <v>45675.54166666666</v>
+        <v>45676.55208333334</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>lens</t>
+          <t>angers</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>psg</t>
+          <t>auxerre</t>
         </is>
       </c>
       <c r="E19" t="n">
@@ -2318,37 +2318,37 @@
         </is>
       </c>
       <c r="I19" t="n">
-        <v>4.33</v>
+        <v>2.4</v>
       </c>
       <c r="J19" t="n">
-        <v>3.9</v>
+        <v>3.2</v>
       </c>
       <c r="K19" t="n">
-        <v>1.75</v>
+        <v>3</v>
       </c>
       <c r="L19" t="n">
-        <v>0.2181242908963071</v>
+        <v>0.392156862745098</v>
       </c>
       <c r="M19" t="n">
-        <v>0.2421738922002589</v>
+        <v>0.2941176470588235</v>
       </c>
       <c r="N19" t="n">
-        <v>0.539701816903434</v>
+        <v>0.3137254901960784</v>
       </c>
       <c r="O19" t="n">
-        <v>0.05878571005591793</v>
+        <v>0.0625</v>
       </c>
       <c r="P19" t="n">
         <v>2</v>
       </c>
       <c r="Q19" t="n">
-        <v>0.1005799308040856</v>
+        <v>0.2966974546613351</v>
       </c>
       <c r="R19" t="n">
-        <v>0.2925517421501925</v>
+        <v>0.3259418900680082</v>
       </c>
       <c r="S19" t="n">
-        <v>0.6068683270457219</v>
+        <v>0.3773606552706568</v>
       </c>
       <c r="T19" t="n">
         <v>1</v>
@@ -2358,19 +2358,19 @@
       </c>
       <c r="V19" t="inlineStr"/>
       <c r="W19" t="n">
-        <v>0.06716651014228792</v>
+        <v>0.06363516507457839</v>
       </c>
       <c r="X19" t="n">
         <v>2</v>
       </c>
       <c r="Y19" t="n">
-        <v>0.06716651014228792</v>
+        <v>0.06363516507457839</v>
       </c>
       <c r="Z19" t="n">
-        <v>0.6068683270457219</v>
+        <v>0.3773606552706568</v>
       </c>
       <c r="AA19" t="n">
-        <v>1.75</v>
+        <v>3</v>
       </c>
       <c r="AB19" t="inlineStr">
         <is>
@@ -2378,76 +2378,76 @@
         </is>
       </c>
       <c r="AC19" t="n">
-        <v>4.241209962274331</v>
+        <v>2.864163931623941</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="inlineStr">
         <is>
-          <t>riCiOT1k</t>
+          <t>GOve9IPO</t>
         </is>
       </c>
       <c r="B20" s="2" t="n">
-        <v>45676.55208333334</v>
+        <v>45675.47916666666</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>angers</t>
+          <t>bayern munich</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>auxerre</t>
+          <t>wolfsburg</t>
         </is>
       </c>
       <c r="E20" t="n">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="F20" t="n">
-        <v>551</v>
+        <v>591</v>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>france</t>
+          <t>germany</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>ligue 1</t>
+          <t>bundesliga</t>
         </is>
       </c>
       <c r="I20" t="n">
-        <v>2.4</v>
+        <v>1.17</v>
       </c>
       <c r="J20" t="n">
-        <v>3.25</v>
+        <v>7.5</v>
       </c>
       <c r="K20" t="n">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="L20" t="n">
-        <v>0.393939393939394</v>
+        <v>0.8103727714748785</v>
       </c>
       <c r="M20" t="n">
-        <v>0.2909090909090909</v>
+        <v>0.126418152350081</v>
       </c>
       <c r="N20" t="n">
-        <v>0.3151515151515151</v>
+        <v>0.06320907617504051</v>
       </c>
       <c r="O20" t="n">
-        <v>0.05769230769230771</v>
+        <v>0.05470085470085473</v>
       </c>
       <c r="P20" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q20" t="n">
-        <v>0.2966974546613351</v>
+        <v>0.6787465742725992</v>
       </c>
       <c r="R20" t="n">
-        <v>0.3259418900680082</v>
+        <v>0.2315661113221025</v>
       </c>
       <c r="S20" t="n">
-        <v>0.3773606552706568</v>
+        <v>0.08968731440529824</v>
       </c>
       <c r="T20" t="n">
         <v>1</v>
@@ -2457,19 +2457,19 @@
       </c>
       <c r="V20" t="inlineStr"/>
       <c r="W20" t="n">
-        <v>0.06220914011914169</v>
+        <v>-0.1316261972022793</v>
       </c>
       <c r="X20" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Y20" t="n">
-        <v>0.06220914011914169</v>
+        <v>-0.1316261972022793</v>
       </c>
       <c r="Z20" t="n">
-        <v>0.3773606552706568</v>
+        <v>0.6787465742725992</v>
       </c>
       <c r="AA20" t="n">
-        <v>3</v>
+        <v>1.17</v>
       </c>
       <c r="AB20" t="inlineStr">
         <is>
@@ -2477,13 +2477,13 @@
         </is>
       </c>
       <c r="AC20" t="n">
-        <v>2.864163931623941</v>
+        <v>5.492965079208243</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="inlineStr">
         <is>
-          <t>GOve9IPO</t>
+          <t>S28DRaug</t>
         </is>
       </c>
       <c r="B21" s="2" t="n">
@@ -2491,12 +2491,12 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>bayern munich</t>
+          <t>heidenheim</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>wolfsburg</t>
+          <t>st  pauli</t>
         </is>
       </c>
       <c r="E21" t="n">
@@ -2516,37 +2516,37 @@
         </is>
       </c>
       <c r="I21" t="n">
-        <v>1.17</v>
+        <v>2.38</v>
       </c>
       <c r="J21" t="n">
-        <v>7.5</v>
+        <v>3.5</v>
       </c>
       <c r="K21" t="n">
-        <v>15</v>
+        <v>2.8</v>
       </c>
       <c r="L21" t="n">
-        <v>0.8103727714748785</v>
+        <v>0.3952569169960474</v>
       </c>
       <c r="M21" t="n">
-        <v>0.126418152350081</v>
+        <v>0.2687747035573123</v>
       </c>
       <c r="N21" t="n">
-        <v>0.06320907617504051</v>
+        <v>0.3359683794466403</v>
       </c>
       <c r="O21" t="n">
-        <v>0.05470085470085473</v>
+        <v>0.06302521008403361</v>
       </c>
       <c r="P21" t="n">
         <v>1</v>
       </c>
       <c r="Q21" t="n">
-        <v>0.6695936358057532</v>
+        <v>0.5578992423794036</v>
       </c>
       <c r="R21" t="n">
-        <v>0.243173602449389</v>
+        <v>0.3368674404475523</v>
       </c>
       <c r="S21" t="n">
-        <v>0.08723276174485786</v>
+        <v>0.1052333171730441</v>
       </c>
       <c r="T21" t="n">
         <v>1</v>
@@ -2556,19 +2556,19 @@
       </c>
       <c r="V21" t="inlineStr"/>
       <c r="W21" t="n">
-        <v>-0.1407791356691254</v>
+        <v>0.1626423253833562</v>
       </c>
       <c r="X21" t="n">
         <v>1</v>
       </c>
       <c r="Y21" t="n">
-        <v>-0.1407791356691254</v>
+        <v>0.1626423253833562</v>
       </c>
       <c r="Z21" t="n">
-        <v>0.6695936358057532</v>
+        <v>0.5578992423794036</v>
       </c>
       <c r="AA21" t="n">
-        <v>1.17</v>
+        <v>2.38</v>
       </c>
       <c r="AB21" t="inlineStr">
         <is>
@@ -2576,13 +2576,13 @@
         </is>
       </c>
       <c r="AC21" t="n">
-        <v>5.328212186805014</v>
+        <v>6.347395454276421</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="inlineStr">
         <is>
-          <t>S28DRaug</t>
+          <t>8bymBveC</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
@@ -2590,12 +2590,12 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>heidenheim</t>
+          <t>stuttgart</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>st  pauli</t>
+          <t>freiburg</t>
         </is>
       </c>
       <c r="E22" t="n">
@@ -2615,37 +2615,37 @@
         </is>
       </c>
       <c r="I22" t="n">
-        <v>2.38</v>
+        <v>1.65</v>
       </c>
       <c r="J22" t="n">
-        <v>3.5</v>
+        <v>4.5</v>
       </c>
       <c r="K22" t="n">
-        <v>2.8</v>
+        <v>4.5</v>
       </c>
       <c r="L22" t="n">
-        <v>0.3952569169960474</v>
+        <v>0.5769230769230769</v>
       </c>
       <c r="M22" t="n">
-        <v>0.2687747035573123</v>
+        <v>0.2115384615384615</v>
       </c>
       <c r="N22" t="n">
-        <v>0.3359683794466403</v>
+        <v>0.2115384615384615</v>
       </c>
       <c r="O22" t="n">
-        <v>0.06302521008403361</v>
+        <v>0.05050505050505061</v>
       </c>
       <c r="P22" t="n">
         <v>1</v>
       </c>
       <c r="Q22" t="n">
-        <v>0.5635331531949277</v>
+        <v>0.4008005900541703</v>
       </c>
       <c r="R22" t="n">
-        <v>0.3444318150154728</v>
+        <v>0.3976788801741771</v>
       </c>
       <c r="S22" t="n">
-        <v>0.09203503178959961</v>
+        <v>0.2015205297716524</v>
       </c>
       <c r="T22" t="n">
         <v>1</v>
@@ -2655,19 +2655,19 @@
       </c>
       <c r="V22" t="inlineStr"/>
       <c r="W22" t="n">
-        <v>0.1682762361988803</v>
+        <v>-0.1761224868689065</v>
       </c>
       <c r="X22" t="n">
         <v>1</v>
       </c>
       <c r="Y22" t="n">
-        <v>0.1682762361988803</v>
+        <v>-0.1761224868689065</v>
       </c>
       <c r="Z22" t="n">
-        <v>0.5635331531949277</v>
+        <v>0.4008005900541703</v>
       </c>
       <c r="AA22" t="n">
-        <v>2.38</v>
+        <v>1.65</v>
       </c>
       <c r="AB22" t="inlineStr">
         <is>
@@ -2675,7 +2675,7 @@
         </is>
       </c>
       <c r="AC22" t="n">
-        <v>6.381198919169566</v>
+        <v>3.291333697898144</v>
       </c>
     </row>
     <row r="23">
@@ -2720,19 +2720,19 @@
         <v>5.75</v>
       </c>
       <c r="K23" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="L23" t="n">
-        <v>0.7419115512402826</v>
+        <v>0.7483214528675796</v>
       </c>
       <c r="M23" t="n">
-        <v>0.1638656817522016</v>
+        <v>0.1652814339377089</v>
       </c>
       <c r="N23" t="n">
-        <v>0.0942227670075159</v>
+        <v>0.08639711319471147</v>
       </c>
       <c r="O23" t="n">
-        <v>0.06131461828141038</v>
+        <v>0.05222370919050134</v>
       </c>
       <c r="P23" t="n">
         <v>1</v>
@@ -2754,13 +2754,13 @@
       </c>
       <c r="V23" t="inlineStr"/>
       <c r="W23" t="n">
-        <v>-0.02347067314521478</v>
+        <v>-0.02988057477251171</v>
       </c>
       <c r="X23" t="n">
         <v>1</v>
       </c>
       <c r="Y23" t="n">
-        <v>-0.02347067314521478</v>
+        <v>-0.02988057477251171</v>
       </c>
       <c r="Z23" t="n">
         <v>0.7184408780950678</v>
@@ -2774,7 +2774,7 @@
         </is>
       </c>
       <c r="AC23" t="n">
-        <v>7.02899719082783</v>
+        <v>6.952078371300267</v>
       </c>
     </row>
     <row r="24">
@@ -2837,13 +2837,13 @@
         <v>1</v>
       </c>
       <c r="Q24" t="n">
-        <v>0.5523228021287199</v>
+        <v>0.5441698177103385</v>
       </c>
       <c r="R24" t="n">
-        <v>0.2959396058862702</v>
+        <v>0.2985304841096286</v>
       </c>
       <c r="S24" t="n">
-        <v>0.1517375919850098</v>
+        <v>0.1572996981800329</v>
       </c>
       <c r="T24" t="n">
         <v>1</v>
@@ -2853,16 +2853,16 @@
       </c>
       <c r="V24" t="inlineStr"/>
       <c r="W24" t="n">
-        <v>0.1795072681481373</v>
+        <v>0.1713542837297559</v>
       </c>
       <c r="X24" t="n">
         <v>1</v>
       </c>
       <c r="Y24" t="n">
-        <v>0.1795072681481373</v>
+        <v>0.1713542837297559</v>
       </c>
       <c r="Z24" t="n">
-        <v>0.5523228021287199</v>
+        <v>0.5441698177103385</v>
       </c>
       <c r="AA24" t="n">
         <v>2.55</v>
@@ -2873,7 +2873,7 @@
         </is>
       </c>
       <c r="AC24" t="n">
-        <v>6.31393681277232</v>
+        <v>6.265018906262031</v>
       </c>
     </row>
     <row r="25">
@@ -2936,13 +2936,13 @@
         <v>1</v>
       </c>
       <c r="Q25" t="n">
-        <v>0.4588581665612719</v>
+        <v>0.4752308506649044</v>
       </c>
       <c r="R25" t="n">
-        <v>0.4046096958411554</v>
+        <v>0.3879902566190263</v>
       </c>
       <c r="S25" t="n">
-        <v>0.1365321375975728</v>
+        <v>0.1367788927160693</v>
       </c>
       <c r="T25" t="n">
         <v>1</v>
@@ -2952,16 +2952,16 @@
       </c>
       <c r="V25" t="inlineStr"/>
       <c r="W25" t="n">
-        <v>-0.0541354210188833</v>
+        <v>-0.03776273691525078</v>
       </c>
       <c r="X25" t="n">
         <v>1</v>
       </c>
       <c r="Y25" t="n">
-        <v>-0.0541354210188833</v>
+        <v>-0.03776273691525078</v>
       </c>
       <c r="Z25" t="n">
-        <v>0.4588581665612719</v>
+        <v>0.4752308506649044</v>
       </c>
       <c r="AA25" t="n">
         <v>1.85</v>
@@ -2972,26 +2972,26 @@
         </is>
       </c>
       <c r="AC25" t="n">
-        <v>5.103523947141031</v>
+        <v>5.398232261006417</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="1" t="inlineStr">
         <is>
-          <t>8bymBveC</t>
+          <t>Kx55TLAt</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
-        <v>45675.47916666666</v>
+        <v>45674.6875</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>stuttgart</t>
+          <t>eintracht frankfurt</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>freiburg</t>
+          <t>dortmund</t>
         </is>
       </c>
       <c r="E26" t="n">
@@ -3011,59 +3011,57 @@
         </is>
       </c>
       <c r="I26" t="n">
-        <v>1.62</v>
+        <v>2.63</v>
       </c>
       <c r="J26" t="n">
-        <v>4.5</v>
+        <v>3.6</v>
       </c>
       <c r="K26" t="n">
-        <v>4.75</v>
+        <v>2.55</v>
       </c>
       <c r="L26" t="n">
-        <v>0.5878712871287128</v>
+        <v>0.3620659054605692</v>
       </c>
       <c r="M26" t="n">
-        <v>0.2116336633663366</v>
+        <v>0.2645092587114714</v>
       </c>
       <c r="N26" t="n">
-        <v>0.2004950495049505</v>
+        <v>0.3734248358279596</v>
       </c>
       <c r="O26" t="n">
-        <v>0.0500324886289798</v>
+        <v>0.05016277740500508</v>
       </c>
       <c r="P26" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="Q26" t="n">
-        <v>0.4039313812642942</v>
+        <v>0.1121637536304423</v>
       </c>
       <c r="R26" t="n">
-        <v>0.4060773338696998</v>
+        <v>0.2706266185782136</v>
       </c>
       <c r="S26" t="n">
-        <v>0.1899912848660061</v>
-      </c>
-      <c r="T26" t="n">
-        <v>1</v>
-      </c>
+        <v>0.6172096277913441</v>
+      </c>
+      <c r="T26" t="inlineStr"/>
       <c r="U26" t="n">
         <v>0</v>
       </c>
       <c r="V26" t="inlineStr"/>
       <c r="W26" t="n">
-        <v>0.1944436705033632</v>
+        <v>0.2437847919633845</v>
       </c>
       <c r="X26" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="Y26" t="n">
-        <v>0.1944436705033632</v>
+        <v>0.2437847919633845</v>
       </c>
       <c r="Z26" t="n">
-        <v>0.4060773338696998</v>
+        <v>0.6172096277913441</v>
       </c>
       <c r="AA26" t="n">
-        <v>4.5</v>
+        <v>2.55</v>
       </c>
       <c r="AB26" t="inlineStr">
         <is>
@@ -3071,26 +3069,26 @@
         </is>
       </c>
       <c r="AC26" t="n">
-        <v>2.436464003218199</v>
+        <v>2.503257766748065</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="1" t="inlineStr">
         <is>
-          <t>Kx55TLAt</t>
+          <t>xh8xMe9U</t>
         </is>
       </c>
       <c r="B27" s="2" t="n">
-        <v>45674.6875</v>
+        <v>45675.47916666666</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>eintracht frankfurt</t>
+          <t>bochum</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>dortmund</t>
+          <t>rb leipzig</t>
         </is>
       </c>
       <c r="E27" t="n">
@@ -3110,37 +3108,37 @@
         </is>
       </c>
       <c r="I27" t="n">
-        <v>2.4</v>
+        <v>3.7</v>
       </c>
       <c r="J27" t="n">
-        <v>3.7</v>
+        <v>3.6</v>
       </c>
       <c r="K27" t="n">
-        <v>2.75</v>
+        <v>2</v>
       </c>
       <c r="L27" t="n">
-        <v>0.3966088481777432</v>
+        <v>0.2578796561604584</v>
       </c>
       <c r="M27" t="n">
-        <v>0.2572597934125901</v>
+        <v>0.2650429799426934</v>
       </c>
       <c r="N27" t="n">
-        <v>0.3461313584096668</v>
+        <v>0.4770773638968481</v>
       </c>
       <c r="O27" t="n">
-        <v>0.05057330057330045</v>
+        <v>0.04804804804804808</v>
       </c>
       <c r="P27" t="n">
         <v>2</v>
       </c>
       <c r="Q27" t="n">
-        <v>0.141502202835892</v>
+        <v>0.2460401455508437</v>
       </c>
       <c r="R27" t="n">
-        <v>0.3031459312321747</v>
+        <v>0.2603028704889312</v>
       </c>
       <c r="S27" t="n">
-        <v>0.5553518659319332</v>
+        <v>0.4936569839602251</v>
       </c>
       <c r="T27" t="n">
         <v>1</v>
@@ -3150,19 +3148,19 @@
       </c>
       <c r="V27" t="inlineStr"/>
       <c r="W27" t="n">
-        <v>0.2092205075222664</v>
+        <v>0.01657962006337699</v>
       </c>
       <c r="X27" t="n">
         <v>2</v>
       </c>
       <c r="Y27" t="n">
-        <v>0.2092205075222664</v>
+        <v>0.01657962006337699</v>
       </c>
       <c r="Z27" t="n">
-        <v>0.5553518659319332</v>
+        <v>0.4936569839602251</v>
       </c>
       <c r="AA27" t="n">
-        <v>2.75</v>
+        <v>2</v>
       </c>
       <c r="AB27" t="inlineStr">
         <is>
@@ -3170,13 +3168,13 @@
         </is>
       </c>
       <c r="AC27" t="n">
-        <v>2.132111195591599</v>
+        <v>1.761941903761351</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="1" t="inlineStr">
         <is>
-          <t>xh8xMe9U</t>
+          <t>SGmntafn</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
@@ -3184,12 +3182,12 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>bochum</t>
+          <t>holstein kiel</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>rb leipzig</t>
+          <t>hoffenheim</t>
         </is>
       </c>
       <c r="E28" t="n">
@@ -3209,37 +3207,37 @@
         </is>
       </c>
       <c r="I28" t="n">
-        <v>3.7</v>
+        <v>3</v>
       </c>
       <c r="J28" t="n">
-        <v>3.6</v>
+        <v>3.4</v>
       </c>
       <c r="K28" t="n">
-        <v>2</v>
+        <v>2.35</v>
       </c>
       <c r="L28" t="n">
-        <v>0.2578796561604584</v>
+        <v>0.3165610142630745</v>
       </c>
       <c r="M28" t="n">
-        <v>0.2650429799426934</v>
+        <v>0.2793185419968304</v>
       </c>
       <c r="N28" t="n">
-        <v>0.4770773638968481</v>
+        <v>0.4041204437400951</v>
       </c>
       <c r="O28" t="n">
-        <v>0.04804804804804808</v>
+        <v>0.05298289528577382</v>
       </c>
       <c r="P28" t="n">
         <v>2</v>
       </c>
       <c r="Q28" t="n">
-        <v>0.2223883515599566</v>
+        <v>0.08354123669379669</v>
       </c>
       <c r="R28" t="n">
-        <v>0.2660193527083555</v>
+        <v>0.3282321609610204</v>
       </c>
       <c r="S28" t="n">
-        <v>0.5115922957316879</v>
+        <v>0.588226602345183</v>
       </c>
       <c r="T28" t="n">
         <v>1</v>
@@ -3249,19 +3247,19 @@
       </c>
       <c r="V28" t="inlineStr"/>
       <c r="W28" t="n">
-        <v>0.03451493183483972</v>
+        <v>0.1841061586050879</v>
       </c>
       <c r="X28" t="n">
         <v>2</v>
       </c>
       <c r="Y28" t="n">
-        <v>0.03451493183483972</v>
+        <v>0.1841061586050879</v>
       </c>
       <c r="Z28" t="n">
-        <v>0.5115922957316879</v>
+        <v>0.588226602345183</v>
       </c>
       <c r="AA28" t="n">
-        <v>2</v>
+        <v>2.35</v>
       </c>
       <c r="AB28" t="inlineStr">
         <is>
@@ -3269,76 +3267,76 @@
         </is>
       </c>
       <c r="AC28" t="n">
-        <v>1.869553774390127</v>
+        <v>2.329359614071098</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="1" t="inlineStr">
         <is>
-          <t>SGmntafn</t>
+          <t>2P2WQCin</t>
         </is>
       </c>
       <c r="B29" s="2" t="n">
-        <v>45675.47916666666</v>
+        <v>45674.69791666666</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>holstein kiel</t>
+          <t>as roma</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>hoffenheim</t>
+          <t>genoa</t>
         </is>
       </c>
       <c r="E29" t="n">
-        <v>59</v>
+        <v>77</v>
       </c>
       <c r="F29" t="n">
-        <v>591</v>
+        <v>771</v>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>germany</t>
+          <t>italy</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>bundesliga</t>
+          <t>serie a</t>
         </is>
       </c>
       <c r="I29" t="n">
-        <v>3</v>
+        <v>1.48</v>
       </c>
       <c r="J29" t="n">
-        <v>3.4</v>
+        <v>4.2</v>
       </c>
       <c r="K29" t="n">
-        <v>2.35</v>
+        <v>7</v>
       </c>
       <c r="L29" t="n">
-        <v>0.3165610142630745</v>
+        <v>0.6394640682095006</v>
       </c>
       <c r="M29" t="n">
-        <v>0.2793185419968304</v>
+        <v>0.2253349573690621</v>
       </c>
       <c r="N29" t="n">
-        <v>0.4041204437400951</v>
+        <v>0.1352009744214373</v>
       </c>
       <c r="O29" t="n">
-        <v>0.05298289528577382</v>
+        <v>0.05662805662805659</v>
       </c>
       <c r="P29" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q29" t="n">
-        <v>0.07380469808814408</v>
+        <v>0.8542784923832019</v>
       </c>
       <c r="R29" t="n">
-        <v>0.2863993898370581</v>
+        <v>0.1130494914543739</v>
       </c>
       <c r="S29" t="n">
-        <v>0.6397959120747979</v>
+        <v>0.03267201616242433</v>
       </c>
       <c r="T29" t="n">
         <v>1</v>
@@ -3346,21 +3344,23 @@
       <c r="U29" t="n">
         <v>0</v>
       </c>
-      <c r="V29" t="inlineStr"/>
+      <c r="V29" t="n">
+        <v>0</v>
+      </c>
       <c r="W29" t="n">
-        <v>0.2356754683347028</v>
+        <v>0.2148144241737012</v>
       </c>
       <c r="X29" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Y29" t="n">
-        <v>0.2356754683347028</v>
+        <v>0.2148144241737012</v>
       </c>
       <c r="Z29" t="n">
-        <v>0.6397959120747979</v>
+        <v>0.8542784923832019</v>
       </c>
       <c r="AA29" t="n">
-        <v>2.35</v>
+        <v>1.48</v>
       </c>
       <c r="AB29" t="inlineStr">
         <is>
@@ -3368,26 +3368,26 @@
         </is>
       </c>
       <c r="AC29" t="n">
-        <v>2.638775472448787</v>
+        <v>2.777012862897634</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="1" t="inlineStr">
         <is>
-          <t>2P2WQCin</t>
+          <t>O4zWcENa</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
-        <v>45674.69791666666</v>
+        <v>45675.45833333334</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>as roma</t>
+          <t>bologna</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>genoa</t>
+          <t>monza</t>
         </is>
       </c>
       <c r="E30" t="n">
@@ -3407,37 +3407,37 @@
         </is>
       </c>
       <c r="I30" t="n">
-        <v>1.53</v>
+        <v>1.6</v>
       </c>
       <c r="J30" t="n">
-        <v>4.2</v>
+        <v>3.75</v>
       </c>
       <c r="K30" t="n">
-        <v>6.25</v>
+        <v>6</v>
       </c>
       <c r="L30" t="n">
-        <v>0.621470932916652</v>
+        <v>0.5905511811023622</v>
       </c>
       <c r="M30" t="n">
-        <v>0.2263929827053518</v>
+        <v>0.2519685039370079</v>
       </c>
       <c r="N30" t="n">
-        <v>0.1521360843779964</v>
+        <v>0.1574803149606299</v>
       </c>
       <c r="O30" t="n">
-        <v>0.05169000933706802</v>
+        <v>0.05833333333333335</v>
       </c>
       <c r="P30" t="n">
         <v>1</v>
       </c>
       <c r="Q30" t="n">
-        <v>0.847266012749617</v>
+        <v>0.6681648631553461</v>
       </c>
       <c r="R30" t="n">
-        <v>0.1176157890866706</v>
+        <v>0.2467502430742633</v>
       </c>
       <c r="S30" t="n">
-        <v>0.03511819816371234</v>
+        <v>0.08508489377039057</v>
       </c>
       <c r="T30" t="n">
         <v>1</v>
@@ -3449,19 +3449,19 @@
         <v>0</v>
       </c>
       <c r="W30" t="n">
-        <v>0.225795079832965</v>
+        <v>0.07761368205298391</v>
       </c>
       <c r="X30" t="n">
         <v>1</v>
       </c>
       <c r="Y30" t="n">
-        <v>0.225795079832965</v>
+        <v>0.07761368205298391</v>
       </c>
       <c r="Z30" t="n">
-        <v>0.847266012749617</v>
+        <v>0.6681648631553461</v>
       </c>
       <c r="AA30" t="n">
-        <v>1.53</v>
+        <v>1.6</v>
       </c>
       <c r="AB30" t="inlineStr">
         <is>
@@ -3469,26 +3469,26 @@
         </is>
       </c>
       <c r="AC30" t="n">
-        <v>2.650788229493105</v>
+        <v>0</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="1" t="inlineStr">
         <is>
-          <t>O4zWcENa</t>
+          <t>2knNazgm</t>
         </is>
       </c>
       <c r="B31" s="2" t="n">
-        <v>45675.45833333334</v>
+        <v>45675.69791666666</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>bologna</t>
+          <t>atalanta</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>monza</t>
+          <t>napoli</t>
         </is>
       </c>
       <c r="E31" t="n">
@@ -3508,37 +3508,37 @@
         </is>
       </c>
       <c r="I31" t="n">
-        <v>1.6</v>
+        <v>2.25</v>
       </c>
       <c r="J31" t="n">
-        <v>3.7</v>
+        <v>3.25</v>
       </c>
       <c r="K31" t="n">
-        <v>6</v>
+        <v>3.25</v>
       </c>
       <c r="L31" t="n">
-        <v>0.5885471898197243</v>
+        <v>0.4193548387096774</v>
       </c>
       <c r="M31" t="n">
-        <v>0.2545068928950159</v>
+        <v>0.2903225806451613</v>
       </c>
       <c r="N31" t="n">
-        <v>0.1569459172852598</v>
+        <v>0.2903225806451613</v>
       </c>
       <c r="O31" t="n">
-        <v>0.06193693693693691</v>
+        <v>0.05982905982905984</v>
       </c>
       <c r="P31" t="n">
         <v>1</v>
       </c>
       <c r="Q31" t="n">
-        <v>0.6637345380379597</v>
+        <v>0.380034330542821</v>
       </c>
       <c r="R31" t="n">
-        <v>0.2492334732365229</v>
+        <v>0.291572028203385</v>
       </c>
       <c r="S31" t="n">
-        <v>0.08703198872551746</v>
+        <v>0.3283936412537941</v>
       </c>
       <c r="T31" t="n">
         <v>1</v>
@@ -3550,19 +3550,19 @@
         <v>0</v>
       </c>
       <c r="W31" t="n">
-        <v>0.07518734821823536</v>
+        <v>-0.03932050816685639</v>
       </c>
       <c r="X31" t="n">
         <v>1</v>
       </c>
       <c r="Y31" t="n">
-        <v>0.07518734821823536</v>
+        <v>-0.03932050816685639</v>
       </c>
       <c r="Z31" t="n">
-        <v>0.6637345380379597</v>
+        <v>0.380034330542821</v>
       </c>
       <c r="AA31" t="n">
-        <v>1.6</v>
+        <v>2.25</v>
       </c>
       <c r="AB31" t="inlineStr">
         <is>
@@ -3576,20 +3576,20 @@
     <row r="32">
       <c r="A32" s="1" t="inlineStr">
         <is>
-          <t>2knNazgm</t>
+          <t>r97dEZ7t</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
-        <v>45675.69791666666</v>
+        <v>45676.35416666666</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>atalanta</t>
+          <t>fiorentina</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>napoli</t>
+          <t>torino</t>
         </is>
       </c>
       <c r="E32" t="n">
@@ -3609,37 +3609,37 @@
         </is>
       </c>
       <c r="I32" t="n">
-        <v>2.25</v>
+        <v>1.73</v>
       </c>
       <c r="J32" t="n">
-        <v>3.25</v>
+        <v>3.4</v>
       </c>
       <c r="K32" t="n">
-        <v>3.25</v>
+        <v>5.5</v>
       </c>
       <c r="L32" t="n">
-        <v>0.4193548387096774</v>
+        <v>0.5484353462181424</v>
       </c>
       <c r="M32" t="n">
-        <v>0.2903225806451613</v>
+        <v>0.2790568085168783</v>
       </c>
       <c r="N32" t="n">
-        <v>0.2903225806451613</v>
+        <v>0.1725078452649793</v>
       </c>
       <c r="O32" t="n">
-        <v>0.05982905982905984</v>
+        <v>0.05397051095793026</v>
       </c>
       <c r="P32" t="n">
         <v>1</v>
       </c>
       <c r="Q32" t="n">
-        <v>0.3664620343929892</v>
+        <v>0.5738043721160205</v>
       </c>
       <c r="R32" t="n">
-        <v>0.2930233628344416</v>
+        <v>0.3099249756430049</v>
       </c>
       <c r="S32" t="n">
-        <v>0.3405146027725691</v>
+        <v>0.1162706522409748</v>
       </c>
       <c r="T32" t="n">
         <v>1</v>
@@ -3651,19 +3651,19 @@
         <v>0</v>
       </c>
       <c r="W32" t="n">
-        <v>-0.05289280431668819</v>
+        <v>0.02536902589787815</v>
       </c>
       <c r="X32" t="n">
         <v>1</v>
       </c>
       <c r="Y32" t="n">
-        <v>-0.05289280431668819</v>
+        <v>0.02536902589787815</v>
       </c>
       <c r="Z32" t="n">
-        <v>0.3664620343929892</v>
+        <v>0.5738043721160205</v>
       </c>
       <c r="AA32" t="n">
-        <v>2.25</v>
+        <v>1.73</v>
       </c>
       <c r="AB32" t="inlineStr">
         <is>
@@ -3677,20 +3677,20 @@
     <row r="33">
       <c r="A33" s="1" t="inlineStr">
         <is>
-          <t>r97dEZ7t</t>
+          <t>AyR5Ai75</t>
         </is>
       </c>
       <c r="B33" s="2" t="n">
-        <v>45676.35416666666</v>
+        <v>45676.69791666666</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>fiorentina</t>
+          <t>inter</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>torino</t>
+          <t>empoli</t>
         </is>
       </c>
       <c r="E33" t="n">
@@ -3710,37 +3710,37 @@
         </is>
       </c>
       <c r="I33" t="n">
-        <v>1.73</v>
+        <v>1.25</v>
       </c>
       <c r="J33" t="n">
-        <v>3.4</v>
+        <v>5.75</v>
       </c>
       <c r="K33" t="n">
-        <v>5.5</v>
+        <v>13</v>
       </c>
       <c r="L33" t="n">
-        <v>0.5484353462181424</v>
+        <v>0.7612985359643539</v>
       </c>
       <c r="M33" t="n">
-        <v>0.2790568085168783</v>
+        <v>0.1654996817313813</v>
       </c>
       <c r="N33" t="n">
-        <v>0.1725078452649793</v>
+        <v>0.0732017823042648</v>
       </c>
       <c r="O33" t="n">
-        <v>0.05397051095793026</v>
+        <v>0.05083612040133789</v>
       </c>
       <c r="P33" t="n">
         <v>1</v>
       </c>
       <c r="Q33" t="n">
-        <v>0.5738043721160205</v>
+        <v>0.8179683161623547</v>
       </c>
       <c r="R33" t="n">
-        <v>0.3099249756430049</v>
+        <v>0.1645990978182047</v>
       </c>
       <c r="S33" t="n">
-        <v>0.1162706522409748</v>
+        <v>0.0174325860194408</v>
       </c>
       <c r="T33" t="n">
         <v>1</v>
@@ -3752,19 +3752,19 @@
         <v>0</v>
       </c>
       <c r="W33" t="n">
-        <v>0.02536902589787815</v>
+        <v>0.05666978019800073</v>
       </c>
       <c r="X33" t="n">
         <v>1</v>
       </c>
       <c r="Y33" t="n">
-        <v>0.02536902589787815</v>
+        <v>0.05666978019800073</v>
       </c>
       <c r="Z33" t="n">
-        <v>0.5738043721160205</v>
+        <v>0.8179683161623547</v>
       </c>
       <c r="AA33" t="n">
-        <v>1.73</v>
+        <v>1.25</v>
       </c>
       <c r="AB33" t="inlineStr">
         <is>
@@ -3772,26 +3772,26 @@
         </is>
       </c>
       <c r="AC33" t="n">
-        <v>0</v>
+        <v>2.123429690922383</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="1" t="inlineStr">
         <is>
-          <t>AyR5Ai75</t>
+          <t>SdXnfWMO</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
-        <v>45676.69791666666</v>
+        <v>45677.69791666666</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>inter</t>
+          <t>como</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>empoli</t>
+          <t>udinese</t>
         </is>
       </c>
       <c r="E34" t="n">
@@ -3811,37 +3811,37 @@
         </is>
       </c>
       <c r="I34" t="n">
-        <v>1.25</v>
+        <v>2.15</v>
       </c>
       <c r="J34" t="n">
-        <v>5.75</v>
+        <v>3.4</v>
       </c>
       <c r="K34" t="n">
-        <v>13</v>
+        <v>3.4</v>
       </c>
       <c r="L34" t="n">
-        <v>0.7612985359643539</v>
+        <v>0.4415584415584415</v>
       </c>
       <c r="M34" t="n">
-        <v>0.1654996817313813</v>
+        <v>0.2792207792207792</v>
       </c>
       <c r="N34" t="n">
-        <v>0.0732017823042648</v>
+        <v>0.2792207792207792</v>
       </c>
       <c r="O34" t="n">
-        <v>0.05083612040133789</v>
+        <v>0.05335157318741457</v>
       </c>
       <c r="P34" t="n">
         <v>1</v>
       </c>
       <c r="Q34" t="n">
-        <v>0.8183055467643469</v>
+        <v>0.6836304049197356</v>
       </c>
       <c r="R34" t="n">
-        <v>0.1643060216778468</v>
+        <v>0.1994769377371045</v>
       </c>
       <c r="S34" t="n">
-        <v>0.01738843155780633</v>
+        <v>0.1168926573431598</v>
       </c>
       <c r="T34" t="n">
         <v>1</v>
@@ -3853,19 +3853,19 @@
         <v>0</v>
       </c>
       <c r="W34" t="n">
-        <v>0.05700701079999293</v>
+        <v>0.2420719633612941</v>
       </c>
       <c r="X34" t="n">
         <v>1</v>
       </c>
       <c r="Y34" t="n">
-        <v>0.05700701079999293</v>
+        <v>0.2420719633612941</v>
       </c>
       <c r="Z34" t="n">
-        <v>0.8183055467643469</v>
+        <v>0.6836304049197356</v>
       </c>
       <c r="AA34" t="n">
-        <v>1.25</v>
+        <v>2.15</v>
       </c>
       <c r="AB34" t="inlineStr">
         <is>
@@ -3873,26 +3873,26 @@
         </is>
       </c>
       <c r="AC34" t="n">
-        <v>2.129499841758244</v>
+        <v>0</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="1" t="inlineStr">
         <is>
-          <t>SdXnfWMO</t>
+          <t>vHIM696U</t>
         </is>
       </c>
       <c r="B35" s="2" t="n">
-        <v>45677.69791666666</v>
+        <v>45676.45833333334</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>como</t>
+          <t>parma</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>udinese</t>
+          <t>venezia</t>
         </is>
       </c>
       <c r="E35" t="n">
@@ -3912,37 +3912,37 @@
         </is>
       </c>
       <c r="I35" t="n">
-        <v>2.1</v>
+        <v>2.15</v>
       </c>
       <c r="J35" t="n">
-        <v>3.4</v>
+        <v>3.7</v>
       </c>
       <c r="K35" t="n">
-        <v>3.6</v>
+        <v>3.1</v>
       </c>
       <c r="L35" t="n">
-        <v>0.4543429844097996</v>
+        <v>0.439632042928325</v>
       </c>
       <c r="M35" t="n">
-        <v>0.2806236080178174</v>
+        <v>0.2554618627826753</v>
       </c>
       <c r="N35" t="n">
-        <v>0.2650334075723831</v>
+        <v>0.3049060942889996</v>
       </c>
       <c r="O35" t="n">
-        <v>0.04808590102707733</v>
+        <v>0.05796719450132803</v>
       </c>
       <c r="P35" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q35" t="n">
-        <v>0.6847454663719253</v>
+        <v>0.3261836109870547</v>
       </c>
       <c r="R35" t="n">
-        <v>0.1988894069901252</v>
+        <v>0.4169344799204003</v>
       </c>
       <c r="S35" t="n">
-        <v>0.1163651266379496</v>
+        <v>0.2568819090925449</v>
       </c>
       <c r="T35" t="n">
         <v>1</v>
@@ -3954,19 +3954,19 @@
         <v>0</v>
       </c>
       <c r="W35" t="n">
-        <v>0.2304024819621258</v>
+        <v>0.161472617137725</v>
       </c>
       <c r="X35" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Y35" t="n">
-        <v>0.2304024819621258</v>
+        <v>0.161472617137725</v>
       </c>
       <c r="Z35" t="n">
-        <v>0.6847454663719253</v>
+        <v>0.4169344799204003</v>
       </c>
       <c r="AA35" t="n">
-        <v>2.1</v>
+        <v>3.7</v>
       </c>
       <c r="AB35" t="inlineStr">
         <is>
@@ -3974,26 +3974,26 @@
         </is>
       </c>
       <c r="AC35" t="n">
-        <v>0</v>
+        <v>16.5048206385672</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="1" t="inlineStr">
         <is>
-          <t>vHIM696U</t>
+          <t>WjFE8VyI</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
-        <v>45676.45833333334</v>
+        <v>45675.58333333334</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>parma</t>
+          <t>juventus</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>venezia</t>
+          <t>ac milan</t>
         </is>
       </c>
       <c r="E36" t="n">
@@ -4016,34 +4016,34 @@
         <v>2.15</v>
       </c>
       <c r="J36" t="n">
-        <v>3.7</v>
+        <v>3.3</v>
       </c>
       <c r="K36" t="n">
-        <v>3.1</v>
+        <v>3.4</v>
       </c>
       <c r="L36" t="n">
-        <v>0.439632042928325</v>
+        <v>0.4378536585365854</v>
       </c>
       <c r="M36" t="n">
-        <v>0.2554618627826753</v>
+        <v>0.2852682926829269</v>
       </c>
       <c r="N36" t="n">
-        <v>0.3049060942889996</v>
+        <v>0.2768780487804878</v>
       </c>
       <c r="O36" t="n">
-        <v>0.05796719450132803</v>
+        <v>0.06226422915889396</v>
       </c>
       <c r="P36" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="Q36" t="n">
-        <v>0.3261836109870547</v>
+        <v>0.2285649651351678</v>
       </c>
       <c r="R36" t="n">
-        <v>0.4169344799204003</v>
+        <v>0.2354135391350798</v>
       </c>
       <c r="S36" t="n">
-        <v>0.2568819090925449</v>
+        <v>0.5360214957297524</v>
       </c>
       <c r="T36" t="n">
         <v>1</v>
@@ -4055,19 +4055,19 @@
         <v>0</v>
       </c>
       <c r="W36" t="n">
-        <v>0.161472617137725</v>
+        <v>0.2591434469492646</v>
       </c>
       <c r="X36" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="Y36" t="n">
-        <v>0.161472617137725</v>
+        <v>0.2591434469492646</v>
       </c>
       <c r="Z36" t="n">
-        <v>0.4169344799204003</v>
+        <v>0.5360214957297524</v>
       </c>
       <c r="AA36" t="n">
-        <v>3.7</v>
+        <v>3.4</v>
       </c>
       <c r="AB36" t="inlineStr">
         <is>
@@ -4075,26 +4075,26 @@
         </is>
       </c>
       <c r="AC36" t="n">
-        <v>16.5048206385672</v>
+        <v>11.44838692313554</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="1" t="inlineStr">
         <is>
-          <t>WjFE8VyI</t>
+          <t>WUwvdhhC</t>
         </is>
       </c>
       <c r="B37" s="2" t="n">
-        <v>45675.58333333334</v>
+        <v>45676.45833333334</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>juventus</t>
+          <t>cagliari</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>ac milan</t>
+          <t>lecce</t>
         </is>
       </c>
       <c r="E37" t="n">
@@ -4114,37 +4114,37 @@
         </is>
       </c>
       <c r="I37" t="n">
-        <v>2.15</v>
+        <v>1.95</v>
       </c>
       <c r="J37" t="n">
         <v>3.3</v>
       </c>
       <c r="K37" t="n">
-        <v>3.4</v>
+        <v>4.1</v>
       </c>
       <c r="L37" t="n">
-        <v>0.4378536585365854</v>
+        <v>0.4839055793991416</v>
       </c>
       <c r="M37" t="n">
-        <v>0.2852682926829269</v>
+        <v>0.2859442060085837</v>
       </c>
       <c r="N37" t="n">
-        <v>0.2768780487804878</v>
+        <v>0.2301502145922747</v>
       </c>
       <c r="O37" t="n">
-        <v>0.06226422915889396</v>
+        <v>0.05975325487520622</v>
       </c>
       <c r="P37" t="n">
         <v>2</v>
       </c>
       <c r="Q37" t="n">
-        <v>0.1846780307188483</v>
+        <v>0.2950293145178599</v>
       </c>
       <c r="R37" t="n">
-        <v>0.2250219312311089</v>
+        <v>0.2914187522133488</v>
       </c>
       <c r="S37" t="n">
-        <v>0.5903000380500428</v>
+        <v>0.4135519332687914</v>
       </c>
       <c r="T37" t="n">
         <v>1</v>
@@ -4156,19 +4156,19 @@
         <v>0</v>
       </c>
       <c r="W37" t="n">
-        <v>0.313421989269555</v>
+        <v>0.1834017186765167</v>
       </c>
       <c r="X37" t="n">
         <v>2</v>
       </c>
       <c r="Y37" t="n">
-        <v>0.313421989269555</v>
+        <v>0.1834017186765167</v>
       </c>
       <c r="Z37" t="n">
-        <v>0.5903000380500428</v>
+        <v>0.4135519332687914</v>
       </c>
       <c r="AA37" t="n">
-        <v>3.4</v>
+        <v>4.1</v>
       </c>
       <c r="AB37" t="inlineStr">
         <is>
@@ -4176,26 +4176,26 @@
         </is>
       </c>
       <c r="AC37" t="n">
-        <v>12.42540068490077</v>
+        <v>9.243934798838245</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="1" t="inlineStr">
         <is>
-          <t>WUwvdhhC</t>
+          <t>2BNcCDxg</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
-        <v>45676.45833333334</v>
+        <v>45676.58333333334</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>cagliari</t>
+          <t>verona</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>lecce</t>
+          <t>lazio</t>
         </is>
       </c>
       <c r="E38" t="n">
@@ -4215,37 +4215,37 @@
         </is>
       </c>
       <c r="I38" t="n">
-        <v>1.95</v>
+        <v>5</v>
       </c>
       <c r="J38" t="n">
-        <v>3.3</v>
+        <v>3.5</v>
       </c>
       <c r="K38" t="n">
-        <v>4.1</v>
+        <v>1.75</v>
       </c>
       <c r="L38" t="n">
-        <v>0.4839055793991416</v>
+        <v>0.1891891891891892</v>
       </c>
       <c r="M38" t="n">
-        <v>0.2859442060085837</v>
+        <v>0.2702702702702702</v>
       </c>
       <c r="N38" t="n">
-        <v>0.2301502145922747</v>
+        <v>0.5405405405405405</v>
       </c>
       <c r="O38" t="n">
-        <v>0.05975325487520622</v>
+        <v>0.05714285714285716</v>
       </c>
       <c r="P38" t="n">
         <v>2</v>
       </c>
       <c r="Q38" t="n">
-        <v>0.2950293145178599</v>
+        <v>0.04256680280030593</v>
       </c>
       <c r="R38" t="n">
-        <v>0.2914187522133488</v>
+        <v>0.2436564508187101</v>
       </c>
       <c r="S38" t="n">
-        <v>0.4135519332687914</v>
+        <v>0.713776746380984</v>
       </c>
       <c r="T38" t="n">
         <v>1</v>
@@ -4257,19 +4257,19 @@
         <v>0</v>
       </c>
       <c r="W38" t="n">
-        <v>0.1834017186765167</v>
+        <v>0.1732362058404435</v>
       </c>
       <c r="X38" t="n">
         <v>2</v>
       </c>
       <c r="Y38" t="n">
-        <v>0.1834017186765167</v>
+        <v>0.1732362058404435</v>
       </c>
       <c r="Z38" t="n">
-        <v>0.4135519332687914</v>
+        <v>0.713776746380984</v>
       </c>
       <c r="AA38" t="n">
-        <v>4.1</v>
+        <v>1.75</v>
       </c>
       <c r="AB38" t="inlineStr">
         <is>
@@ -4277,76 +4277,76 @@
         </is>
       </c>
       <c r="AC38" t="n">
-        <v>9.243934798838245</v>
+        <v>14.64798143485771</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="1" t="inlineStr">
         <is>
-          <t>2BNcCDxg</t>
+          <t>MsJDjb1N</t>
         </is>
       </c>
       <c r="B39" s="2" t="n">
-        <v>45676.58333333334</v>
+        <v>45674.70833333334</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>verona</t>
+          <t>espanyol</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>lazio</t>
+          <t>valladolid</t>
         </is>
       </c>
       <c r="E39" t="n">
-        <v>77</v>
+        <v>148</v>
       </c>
       <c r="F39" t="n">
-        <v>771</v>
+        <v>1481</v>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>italy</t>
+          <t>spain</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>serie a</t>
+          <t>laliga</t>
         </is>
       </c>
       <c r="I39" t="n">
-        <v>5</v>
+        <v>1.73</v>
       </c>
       <c r="J39" t="n">
         <v>3.5</v>
       </c>
       <c r="K39" t="n">
-        <v>1.75</v>
+        <v>5.5</v>
       </c>
       <c r="L39" t="n">
-        <v>0.1891891891891892</v>
+        <v>0.5528431935669156</v>
       </c>
       <c r="M39" t="n">
-        <v>0.2702702702702702</v>
+        <v>0.2732624928202183</v>
       </c>
       <c r="N39" t="n">
-        <v>0.5405405405405405</v>
+        <v>0.1738943136128662</v>
       </c>
       <c r="O39" t="n">
-        <v>0.05714285714285716</v>
+        <v>0.04556714961339248</v>
       </c>
       <c r="P39" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q39" t="n">
-        <v>0.04256680280030593</v>
+        <v>0.4082163112105208</v>
       </c>
       <c r="R39" t="n">
-        <v>0.2436564508187101</v>
+        <v>0.3447177082743725</v>
       </c>
       <c r="S39" t="n">
-        <v>0.713776746380984</v>
+        <v>0.2470659805151066</v>
       </c>
       <c r="T39" t="n">
         <v>1</v>
@@ -4354,23 +4354,21 @@
       <c r="U39" t="n">
         <v>0</v>
       </c>
-      <c r="V39" t="n">
-        <v>0</v>
-      </c>
+      <c r="V39" t="inlineStr"/>
       <c r="W39" t="n">
-        <v>0.1732362058404435</v>
+        <v>-0.1446268823563948</v>
       </c>
       <c r="X39" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Y39" t="n">
-        <v>0.1732362058404435</v>
+        <v>-0.1446268823563948</v>
       </c>
       <c r="Z39" t="n">
-        <v>0.713776746380984</v>
+        <v>0.4082163112105208</v>
       </c>
       <c r="AA39" t="n">
-        <v>1.75</v>
+        <v>1.73</v>
       </c>
       <c r="AB39" t="inlineStr">
         <is>
@@ -4378,26 +4376,26 @@
         </is>
       </c>
       <c r="AC39" t="n">
-        <v>14.64798143485771</v>
+        <v>3.28443819746597</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="1" t="inlineStr">
         <is>
-          <t>MsJDjb1N</t>
+          <t>ATS0AdWi</t>
         </is>
       </c>
       <c r="B40" s="2" t="n">
-        <v>45674.70833333334</v>
+        <v>45675.41666666666</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>espanyol</t>
+          <t>girona</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>valladolid</t>
+          <t>sevilla</t>
         </is>
       </c>
       <c r="E40" t="n">
@@ -4417,37 +4415,37 @@
         </is>
       </c>
       <c r="I40" t="n">
-        <v>1.9</v>
+        <v>1.91</v>
       </c>
       <c r="J40" t="n">
-        <v>3.25</v>
+        <v>3.5</v>
       </c>
       <c r="K40" t="n">
-        <v>4.5</v>
+        <v>4</v>
       </c>
       <c r="L40" t="n">
-        <v>0.4982964224872232</v>
+        <v>0.4942630185348632</v>
       </c>
       <c r="M40" t="n">
-        <v>0.2913117546848382</v>
+        <v>0.2697263901147396</v>
       </c>
       <c r="N40" t="n">
-        <v>0.2103918228279387</v>
+        <v>0.2360105913503972</v>
       </c>
       <c r="O40" t="n">
-        <v>0.0562303193882141</v>
+        <v>0.05927449513836947</v>
       </c>
       <c r="P40" t="n">
         <v>1</v>
       </c>
       <c r="Q40" t="n">
-        <v>0.4082163112105208</v>
+        <v>0.4811713192483967</v>
       </c>
       <c r="R40" t="n">
-        <v>0.3447177082743725</v>
+        <v>0.3204136257977307</v>
       </c>
       <c r="S40" t="n">
-        <v>0.2470659805151066</v>
+        <v>0.1984150549538725</v>
       </c>
       <c r="T40" t="n">
         <v>1</v>
@@ -4457,19 +4455,19 @@
       </c>
       <c r="V40" t="inlineStr"/>
       <c r="W40" t="n">
-        <v>-0.09008011127670235</v>
+        <v>-0.01309169928646647</v>
       </c>
       <c r="X40" t="n">
         <v>1</v>
       </c>
       <c r="Y40" t="n">
-        <v>-0.09008011127670235</v>
+        <v>-0.01309169928646647</v>
       </c>
       <c r="Z40" t="n">
-        <v>0.4082163112105208</v>
+        <v>0.4811713192483967</v>
       </c>
       <c r="AA40" t="n">
-        <v>1.9</v>
+        <v>1.91</v>
       </c>
       <c r="AB40" t="inlineStr">
         <is>
@@ -4477,26 +4475,26 @@
         </is>
       </c>
       <c r="AC40" t="n">
-        <v>4.920841329856741</v>
+        <v>8.324818810131957</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="1" t="inlineStr">
         <is>
-          <t>ATS0AdWi</t>
+          <t>rciODVxp</t>
         </is>
       </c>
       <c r="B41" s="2" t="n">
-        <v>45675.41666666666</v>
+        <v>45675.60416666666</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>girona</t>
+          <t>betis</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>sevilla</t>
+          <t>alaves</t>
         </is>
       </c>
       <c r="E41" t="n">
@@ -4516,37 +4514,37 @@
         </is>
       </c>
       <c r="I41" t="n">
-        <v>1.91</v>
+        <v>1.75</v>
       </c>
       <c r="J41" t="n">
-        <v>3.5</v>
+        <v>3.6</v>
       </c>
       <c r="K41" t="n">
-        <v>4</v>
+        <v>4.75</v>
       </c>
       <c r="L41" t="n">
-        <v>0.4942630185348632</v>
+        <v>0.5392195506503745</v>
       </c>
       <c r="M41" t="n">
-        <v>0.2697263901147396</v>
+        <v>0.2621206148994876</v>
       </c>
       <c r="N41" t="n">
-        <v>0.2360105913503972</v>
+        <v>0.198659834450138</v>
       </c>
       <c r="O41" t="n">
-        <v>0.05927449513836947</v>
+        <v>0.05973266499582275</v>
       </c>
       <c r="P41" t="n">
         <v>1</v>
       </c>
       <c r="Q41" t="n">
-        <v>0.4811713192483967</v>
+        <v>0.4714159361151539</v>
       </c>
       <c r="R41" t="n">
-        <v>0.3204136257977307</v>
+        <v>0.3398291918567071</v>
       </c>
       <c r="S41" t="n">
-        <v>0.1984150549538725</v>
+        <v>0.188754872028139</v>
       </c>
       <c r="T41" t="n">
         <v>1</v>
@@ -4556,19 +4554,19 @@
       </c>
       <c r="V41" t="inlineStr"/>
       <c r="W41" t="n">
-        <v>-0.01309169928646647</v>
+        <v>-0.06780361453522066</v>
       </c>
       <c r="X41" t="n">
         <v>1</v>
       </c>
       <c r="Y41" t="n">
-        <v>-0.01309169928646647</v>
+        <v>-0.06780361453522066</v>
       </c>
       <c r="Z41" t="n">
-        <v>0.4811713192483967</v>
+        <v>0.4714159361151539</v>
       </c>
       <c r="AA41" t="n">
-        <v>1.91</v>
+        <v>1.75</v>
       </c>
       <c r="AB41" t="inlineStr">
         <is>
@@ -4576,26 +4574,26 @@
         </is>
       </c>
       <c r="AC41" t="n">
-        <v>8.324818810131957</v>
+        <v>6.537130605670687</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="1" t="inlineStr">
         <is>
-          <t>rciODVxp</t>
+          <t>CE0hJiFM</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
-        <v>45675.60416666666</v>
+        <v>45676.51041666666</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>betis</t>
+          <t>real madrid</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>alaves</t>
+          <t>las palmas</t>
         </is>
       </c>
       <c r="E42" t="n">
@@ -4615,37 +4613,37 @@
         </is>
       </c>
       <c r="I42" t="n">
-        <v>1.75</v>
+        <v>1.14</v>
       </c>
       <c r="J42" t="n">
-        <v>3.75</v>
+        <v>7.5</v>
       </c>
       <c r="K42" t="n">
-        <v>4.75</v>
+        <v>17</v>
       </c>
       <c r="L42" t="n">
-        <v>0.5449330783938815</v>
+        <v>0.820304960432349</v>
       </c>
       <c r="M42" t="n">
-        <v>0.254302103250478</v>
+        <v>0.124686353985717</v>
       </c>
       <c r="N42" t="n">
-        <v>0.2007648183556406</v>
+        <v>0.05500868558193399</v>
       </c>
       <c r="O42" t="n">
-        <v>0.04862155388471168</v>
+        <v>0.06934984520123844</v>
       </c>
       <c r="P42" t="n">
         <v>1</v>
       </c>
       <c r="Q42" t="n">
-        <v>0.4714159361151539</v>
+        <v>0.7276693411101831</v>
       </c>
       <c r="R42" t="n">
-        <v>0.3398291918567071</v>
+        <v>0.2226244325162247</v>
       </c>
       <c r="S42" t="n">
-        <v>0.188754872028139</v>
+        <v>0.04970622637359232</v>
       </c>
       <c r="T42" t="n">
         <v>1</v>
@@ -4655,19 +4653,19 @@
       </c>
       <c r="V42" t="inlineStr"/>
       <c r="W42" t="n">
-        <v>-0.07351714227872763</v>
+        <v>-0.09263561932216591</v>
       </c>
       <c r="X42" t="n">
         <v>1</v>
       </c>
       <c r="Y42" t="n">
-        <v>-0.07351714227872763</v>
+        <v>-0.09263561932216591</v>
       </c>
       <c r="Z42" t="n">
-        <v>0.4714159361151539</v>
+        <v>0.7276693411101831</v>
       </c>
       <c r="AA42" t="n">
-        <v>1.75</v>
+        <v>1.14</v>
       </c>
       <c r="AB42" t="inlineStr">
         <is>
@@ -4675,26 +4673,26 @@
         </is>
       </c>
       <c r="AC42" t="n">
-        <v>6.365724773365478</v>
+        <v>9.635971536987769</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="1" t="inlineStr">
         <is>
-          <t>CE0hJiFM</t>
+          <t>6eM98z14</t>
         </is>
       </c>
       <c r="B43" s="2" t="n">
-        <v>45676.51041666666</v>
+        <v>45676.60416666666</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>real madrid</t>
+          <t>osasuna</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>las palmas</t>
+          <t>rayo vallecano</t>
         </is>
       </c>
       <c r="E43" t="n">
@@ -4714,37 +4712,37 @@
         </is>
       </c>
       <c r="I43" t="n">
-        <v>1.14</v>
+        <v>2.15</v>
       </c>
       <c r="J43" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="K43" t="n">
-        <v>17</v>
+        <v>3.8</v>
       </c>
       <c r="L43" t="n">
-        <v>0.8267477203647416</v>
+        <v>0.4381245196003075</v>
       </c>
       <c r="M43" t="n">
-        <v>0.1178115501519757</v>
+        <v>0.313989239046887</v>
       </c>
       <c r="N43" t="n">
-        <v>0.05544072948328267</v>
+        <v>0.2478862413528055</v>
       </c>
       <c r="O43" t="n">
-        <v>0.06101651186790513</v>
+        <v>0.0616075071399429</v>
       </c>
       <c r="P43" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q43" t="n">
-        <v>0.7276693411101831</v>
+        <v>0.3212474655210754</v>
       </c>
       <c r="R43" t="n">
-        <v>0.2226244325162247</v>
+        <v>0.3456437490563224</v>
       </c>
       <c r="S43" t="n">
-        <v>0.04970622637359232</v>
+        <v>0.3331087854226021</v>
       </c>
       <c r="T43" t="n">
         <v>1</v>
@@ -4754,19 +4752,19 @@
       </c>
       <c r="V43" t="inlineStr"/>
       <c r="W43" t="n">
-        <v>-0.09907837925455854</v>
+        <v>0.03165451000943548</v>
       </c>
       <c r="X43" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Y43" t="n">
-        <v>-0.09907837925455854</v>
+        <v>0.03165451000943548</v>
       </c>
       <c r="Z43" t="n">
-        <v>0.7276693411101831</v>
+        <v>0.3456437490563224</v>
       </c>
       <c r="AA43" t="n">
-        <v>1.14</v>
+        <v>3</v>
       </c>
       <c r="AB43" t="inlineStr">
         <is>
@@ -4774,26 +4772,26 @@
         </is>
       </c>
       <c r="AC43" t="n">
-        <v>9.44268873901599</v>
+        <v>12.68465623584484</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="1" t="inlineStr">
         <is>
-          <t>6eM98z14</t>
+          <t>KbnqNZFc</t>
         </is>
       </c>
       <c r="B44" s="2" t="n">
-        <v>45676.60416666666</v>
+        <v>45677.70833333334</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>osasuna</t>
+          <t>villarreal</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>rayo vallecano</t>
+          <t>mallorca</t>
         </is>
       </c>
       <c r="E44" t="n">
@@ -4813,37 +4811,37 @@
         </is>
       </c>
       <c r="I44" t="n">
-        <v>2.15</v>
+        <v>1.73</v>
       </c>
       <c r="J44" t="n">
-        <v>3</v>
+        <v>3.5</v>
       </c>
       <c r="K44" t="n">
-        <v>3.8</v>
+        <v>5.25</v>
       </c>
       <c r="L44" t="n">
-        <v>0.4381245196003075</v>
+        <v>0.5483028720626633</v>
       </c>
       <c r="M44" t="n">
-        <v>0.313989239046887</v>
+        <v>0.2710182767624021</v>
       </c>
       <c r="N44" t="n">
-        <v>0.2478862413528055</v>
+        <v>0.1806788511749347</v>
       </c>
       <c r="O44" t="n">
-        <v>0.0616075071399429</v>
+        <v>0.05422515827140106</v>
       </c>
       <c r="P44" t="n">
         <v>0</v>
       </c>
       <c r="Q44" t="n">
-        <v>0.3212474655210754</v>
+        <v>0.3426133713638728</v>
       </c>
       <c r="R44" t="n">
-        <v>0.3456437490563224</v>
+        <v>0.3611622988349005</v>
       </c>
       <c r="S44" t="n">
-        <v>0.3331087854226021</v>
+        <v>0.2962243298012267</v>
       </c>
       <c r="T44" t="n">
         <v>1</v>
@@ -4853,19 +4851,19 @@
       </c>
       <c r="V44" t="inlineStr"/>
       <c r="W44" t="n">
-        <v>0.03165451000943548</v>
+        <v>0.09014402207249839</v>
       </c>
       <c r="X44" t="n">
         <v>0</v>
       </c>
       <c r="Y44" t="n">
-        <v>0.03165451000943548</v>
+        <v>0.09014402207249839</v>
       </c>
       <c r="Z44" t="n">
-        <v>0.3456437490563224</v>
+        <v>0.3611622988349005</v>
       </c>
       <c r="AA44" t="n">
-        <v>3</v>
+        <v>3.5</v>
       </c>
       <c r="AB44" t="inlineStr">
         <is>
@@ -4873,26 +4871,26 @@
         </is>
       </c>
       <c r="AC44" t="n">
-        <v>12.68465623584484</v>
+        <v>12.91743448252351</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="1" t="inlineStr">
         <is>
-          <t>KbnqNZFc</t>
+          <t>Y7DQ4h0T</t>
         </is>
       </c>
       <c r="B45" s="2" t="n">
-        <v>45677.70833333334</v>
+        <v>45675.51041666666</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>villarreal</t>
+          <t>leganes</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>mallorca</t>
+          <t>atl  madrid</t>
         </is>
       </c>
       <c r="E45" t="n">
@@ -4912,37 +4910,37 @@
         </is>
       </c>
       <c r="I45" t="n">
-        <v>1.73</v>
+        <v>7</v>
       </c>
       <c r="J45" t="n">
-        <v>3.5</v>
+        <v>4</v>
       </c>
       <c r="K45" t="n">
-        <v>5.25</v>
+        <v>1.5</v>
       </c>
       <c r="L45" t="n">
-        <v>0.5483028720626633</v>
+        <v>0.1348314606741573</v>
       </c>
       <c r="M45" t="n">
-        <v>0.2710182767624021</v>
+        <v>0.2359550561797753</v>
       </c>
       <c r="N45" t="n">
-        <v>0.1806788511749347</v>
+        <v>0.6292134831460674</v>
       </c>
       <c r="O45" t="n">
-        <v>0.05422515827140106</v>
+        <v>0.05952380952380953</v>
       </c>
       <c r="P45" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="Q45" t="n">
-        <v>0.3426133713638728</v>
+        <v>0.05227173949272378</v>
       </c>
       <c r="R45" t="n">
-        <v>0.3611622988349005</v>
+        <v>0.1945286339595058</v>
       </c>
       <c r="S45" t="n">
-        <v>0.2962243298012267</v>
+        <v>0.7531996265477705</v>
       </c>
       <c r="T45" t="n">
         <v>1</v>
@@ -4952,19 +4950,19 @@
       </c>
       <c r="V45" t="inlineStr"/>
       <c r="W45" t="n">
-        <v>0.09014402207249839</v>
+        <v>0.1239861434017031</v>
       </c>
       <c r="X45" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="Y45" t="n">
-        <v>0.09014402207249839</v>
+        <v>0.1239861434017031</v>
       </c>
       <c r="Z45" t="n">
-        <v>0.3611622988349005</v>
+        <v>0.7531996265477705</v>
       </c>
       <c r="AA45" t="n">
-        <v>3.5</v>
+        <v>1.5</v>
       </c>
       <c r="AB45" t="inlineStr">
         <is>
@@ -4972,26 +4970,26 @@
         </is>
       </c>
       <c r="AC45" t="n">
-        <v>12.91743448252351</v>
+        <v>9.797994398216556</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="1" t="inlineStr">
         <is>
-          <t>Y7DQ4h0T</t>
+          <t>4j4daWNj</t>
         </is>
       </c>
       <c r="B46" s="2" t="n">
-        <v>45675.51041666666</v>
+        <v>45675.70833333334</v>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>leganes</t>
+          <t>getafe</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>atl  madrid</t>
+          <t>barcelona</t>
         </is>
       </c>
       <c r="E46" t="n">
@@ -5011,37 +5009,37 @@
         </is>
       </c>
       <c r="I46" t="n">
-        <v>7</v>
+        <v>6.5</v>
       </c>
       <c r="J46" t="n">
-        <v>4</v>
+        <v>4.2</v>
       </c>
       <c r="K46" t="n">
-        <v>1.53</v>
+        <v>1.5</v>
       </c>
       <c r="L46" t="n">
-        <v>0.1365157260762882</v>
+        <v>0.1453287197231834</v>
       </c>
       <c r="M46" t="n">
-        <v>0.2389025206335043</v>
+        <v>0.2249134948096886</v>
       </c>
       <c r="N46" t="n">
-        <v>0.6245817532902074</v>
+        <v>0.629757785467128</v>
       </c>
       <c r="O46" t="n">
-        <v>0.04645191409897298</v>
+        <v>0.05860805860805862</v>
       </c>
       <c r="P46" t="n">
         <v>2</v>
       </c>
       <c r="Q46" t="n">
-        <v>0.05227173949272378</v>
+        <v>0.09066022859148465</v>
       </c>
       <c r="R46" t="n">
-        <v>0.1945286339595058</v>
+        <v>0.2482536088318762</v>
       </c>
       <c r="S46" t="n">
-        <v>0.7531996265477705</v>
+        <v>0.6610861625766391</v>
       </c>
       <c r="T46" t="n">
         <v>1</v>
@@ -5051,19 +5049,19 @@
       </c>
       <c r="V46" t="inlineStr"/>
       <c r="W46" t="n">
-        <v>0.1286178732575631</v>
+        <v>0.03132837710951109</v>
       </c>
       <c r="X46" t="n">
         <v>2</v>
       </c>
       <c r="Y46" t="n">
-        <v>0.1286178732575631</v>
+        <v>0.03132837710951109</v>
       </c>
       <c r="Z46" t="n">
-        <v>0.7531996265477705</v>
+        <v>0.6610861625766391</v>
       </c>
       <c r="AA46" t="n">
-        <v>1.53</v>
+        <v>1.5</v>
       </c>
       <c r="AB46" t="inlineStr">
         <is>
@@ -5071,26 +5069,26 @@
         </is>
       </c>
       <c r="AC46" t="n">
-        <v>9.797994398216556</v>
+        <v>8.416292438649586</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="1" t="inlineStr">
         <is>
-          <t>4j4daWNj</t>
+          <t>ChPH6EVG</t>
         </is>
       </c>
       <c r="B47" s="2" t="n">
-        <v>45675.70833333334</v>
+        <v>45676.41666666666</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>getafe</t>
+          <t>celta vigo</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>barcelona</t>
+          <t>ath bilbao</t>
         </is>
       </c>
       <c r="E47" t="n">
@@ -5110,37 +5108,37 @@
         </is>
       </c>
       <c r="I47" t="n">
-        <v>6.25</v>
+        <v>2.8</v>
       </c>
       <c r="J47" t="n">
-        <v>4.2</v>
+        <v>3.2</v>
       </c>
       <c r="K47" t="n">
-        <v>1.5</v>
+        <v>2.6</v>
       </c>
       <c r="L47" t="n">
-        <v>0.1502683363148479</v>
+        <v>0.3387622149837133</v>
       </c>
       <c r="M47" t="n">
-        <v>0.223613595706619</v>
+        <v>0.2964169381107492</v>
       </c>
       <c r="N47" t="n">
-        <v>0.6261180679785331</v>
+        <v>0.3648208469055374</v>
       </c>
       <c r="O47" t="n">
-        <v>0.0647619047619048</v>
+        <v>0.05425824175824179</v>
       </c>
       <c r="P47" t="n">
         <v>2</v>
       </c>
       <c r="Q47" t="n">
-        <v>0.09066022859148465</v>
+        <v>0.173590741010381</v>
       </c>
       <c r="R47" t="n">
-        <v>0.2482536088318762</v>
+        <v>0.3226416694087625</v>
       </c>
       <c r="S47" t="n">
-        <v>0.6610861625766391</v>
+        <v>0.5037675895808565</v>
       </c>
       <c r="T47" t="n">
         <v>1</v>
@@ -5150,19 +5148,19 @@
       </c>
       <c r="V47" t="inlineStr"/>
       <c r="W47" t="n">
-        <v>0.03496809459810601</v>
+        <v>0.1389467426753191</v>
       </c>
       <c r="X47" t="n">
         <v>2</v>
       </c>
       <c r="Y47" t="n">
-        <v>0.03496809459810601</v>
+        <v>0.1389467426753191</v>
       </c>
       <c r="Z47" t="n">
-        <v>0.6610861625766391</v>
+        <v>0.5037675895808565</v>
       </c>
       <c r="AA47" t="n">
-        <v>1.5</v>
+        <v>2.6</v>
       </c>
       <c r="AB47" t="inlineStr">
         <is>
@@ -5170,26 +5168,26 @@
         </is>
       </c>
       <c r="AC47" t="n">
-        <v>8.416292438649586</v>
+        <v>6.056513843712848</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="1" t="inlineStr">
         <is>
-          <t>ChPH6EVG</t>
+          <t>hCpiLDpA</t>
         </is>
       </c>
       <c r="B48" s="2" t="n">
-        <v>45676.41666666666</v>
+        <v>45676.70833333334</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>celta vigo</t>
+          <t>valencia</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>ath bilbao</t>
+          <t>real sociedad</t>
         </is>
       </c>
       <c r="E48" t="n">
@@ -5209,37 +5207,37 @@
         </is>
       </c>
       <c r="I48" t="n">
-        <v>2.75</v>
+        <v>3.1</v>
       </c>
       <c r="J48" t="n">
-        <v>3.2</v>
+        <v>3</v>
       </c>
       <c r="K48" t="n">
-        <v>2.63</v>
+        <v>2.55</v>
       </c>
       <c r="L48" t="n">
-        <v>0.3442337975744933</v>
+        <v>0.3077851538925769</v>
       </c>
       <c r="M48" t="n">
-        <v>0.2958259197905802</v>
+        <v>0.3180446590223295</v>
       </c>
       <c r="N48" t="n">
-        <v>0.3599402826349265</v>
+        <v>0.3741701870850936</v>
       </c>
       <c r="O48" t="n">
-        <v>0.05636450051849295</v>
+        <v>0.04807084123972172</v>
       </c>
       <c r="P48" t="n">
         <v>2</v>
       </c>
       <c r="Q48" t="n">
-        <v>0.173590741010381</v>
+        <v>0.2533140525360198</v>
       </c>
       <c r="R48" t="n">
-        <v>0.3226416694087625</v>
+        <v>0.3394360874986988</v>
       </c>
       <c r="S48" t="n">
-        <v>0.5037675895808565</v>
+        <v>0.4072498599652814</v>
       </c>
       <c r="T48" t="n">
         <v>1</v>
@@ -5249,19 +5247,19 @@
       </c>
       <c r="V48" t="inlineStr"/>
       <c r="W48" t="n">
-        <v>0.14382730694593</v>
+        <v>0.03307967288018782</v>
       </c>
       <c r="X48" t="n">
         <v>2</v>
       </c>
       <c r="Y48" t="n">
-        <v>0.14382730694593</v>
+        <v>0.03307967288018782</v>
       </c>
       <c r="Z48" t="n">
-        <v>0.5037675895808565</v>
+        <v>0.4072498599652814</v>
       </c>
       <c r="AA48" t="n">
-        <v>2.63</v>
+        <v>2.55</v>
       </c>
       <c r="AB48" t="inlineStr">
         <is>
@@ -5269,105 +5267,6 @@
         </is>
       </c>
       <c r="AC48" t="n">
-        <v>6.056513843712848</v>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="1" t="inlineStr">
-        <is>
-          <t>hCpiLDpA</t>
-        </is>
-      </c>
-      <c r="B49" s="2" t="n">
-        <v>45676.70833333334</v>
-      </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>valencia</t>
-        </is>
-      </c>
-      <c r="D49" t="inlineStr">
-        <is>
-          <t>real sociedad</t>
-        </is>
-      </c>
-      <c r="E49" t="n">
-        <v>148</v>
-      </c>
-      <c r="F49" t="n">
-        <v>1481</v>
-      </c>
-      <c r="G49" t="inlineStr">
-        <is>
-          <t>spain</t>
-        </is>
-      </c>
-      <c r="H49" t="inlineStr">
-        <is>
-          <t>laliga</t>
-        </is>
-      </c>
-      <c r="I49" t="n">
-        <v>3.1</v>
-      </c>
-      <c r="J49" t="n">
-        <v>3</v>
-      </c>
-      <c r="K49" t="n">
-        <v>2.55</v>
-      </c>
-      <c r="L49" t="n">
-        <v>0.3077851538925769</v>
-      </c>
-      <c r="M49" t="n">
-        <v>0.3180446590223295</v>
-      </c>
-      <c r="N49" t="n">
-        <v>0.3741701870850936</v>
-      </c>
-      <c r="O49" t="n">
-        <v>0.04807084123972172</v>
-      </c>
-      <c r="P49" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q49" t="n">
-        <v>0.2533140525360198</v>
-      </c>
-      <c r="R49" t="n">
-        <v>0.3394360874986988</v>
-      </c>
-      <c r="S49" t="n">
-        <v>0.4072498599652814</v>
-      </c>
-      <c r="T49" t="n">
-        <v>1</v>
-      </c>
-      <c r="U49" t="n">
-        <v>0</v>
-      </c>
-      <c r="V49" t="inlineStr"/>
-      <c r="W49" t="n">
-        <v>0.03307967288018782</v>
-      </c>
-      <c r="X49" t="n">
-        <v>2</v>
-      </c>
-      <c r="Y49" t="n">
-        <v>0.03307967288018782</v>
-      </c>
-      <c r="Z49" t="n">
-        <v>0.4072498599652814</v>
-      </c>
-      <c r="AA49" t="n">
-        <v>2.55</v>
-      </c>
-      <c r="AB49" t="inlineStr">
-        <is>
-          <t>dif_prob_mod_bm &gt; -1</t>
-        </is>
-      </c>
-      <c r="AC49" t="n">
         <v>4.608747899479221</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualizo predicciones tras cambio de modelos + reduccion de b
</commit_message>
<xml_diff>
--- a/data/predicciones.xlsx
+++ b/data/predicciones.xlsx
@@ -774,7 +774,7 @@
         </is>
       </c>
       <c r="AC3" t="n">
-        <v>2.549248910009322</v>
+        <v>4.349248910009321</v>
       </c>
     </row>
     <row r="4">
@@ -871,7 +871,7 @@
         </is>
       </c>
       <c r="AC4" t="n">
-        <v>0.4721208760505936</v>
+        <v>2.272120876050594</v>
       </c>
     </row>
     <row r="5">
@@ -968,7 +968,7 @@
         </is>
       </c>
       <c r="AC5" t="n">
-        <v>0.2413190845932696</v>
+        <v>2.041319084593269</v>
       </c>
     </row>
     <row r="6">
@@ -1065,7 +1065,7 @@
         </is>
       </c>
       <c r="AC6" t="n">
-        <v>0.6269404378829311</v>
+        <v>2.426940437882931</v>
       </c>
     </row>
     <row r="7">
@@ -1263,7 +1263,7 @@
         </is>
       </c>
       <c r="AC8" t="n">
-        <v>8.318121778493961</v>
+        <v>7.41812177849396</v>
       </c>
     </row>
     <row r="9">
@@ -1360,7 +1360,7 @@
         </is>
       </c>
       <c r="AC9" t="n">
-        <v>6.496352487988231</v>
+        <v>5.596352487988231</v>
       </c>
     </row>
     <row r="10">
@@ -1457,7 +1457,7 @@
         </is>
       </c>
       <c r="AC10" t="n">
-        <v>7.514926808304434</v>
+        <v>6.614926808304434</v>
       </c>
     </row>
     <row r="11">
@@ -1558,7 +1558,7 @@
         </is>
       </c>
       <c r="AC11" t="n">
-        <v>7.980301790843282</v>
+        <v>7.080301790843282</v>
       </c>
     </row>
     <row r="12">
@@ -1659,7 +1659,7 @@
         </is>
       </c>
       <c r="AC12" t="n">
-        <v>5.338504608877666</v>
+        <v>4.438504608877666</v>
       </c>
     </row>
     <row r="13">
@@ -1756,7 +1756,7 @@
         </is>
       </c>
       <c r="AC13" t="n">
-        <v>7.196243262041671</v>
+        <v>6.296243262041672</v>
       </c>
     </row>
     <row r="14">
@@ -1853,7 +1853,7 @@
         </is>
       </c>
       <c r="AC14" t="n">
-        <v>5.715164668902383</v>
+        <v>4.815164668902383</v>
       </c>
     </row>
     <row r="15">
@@ -2635,7 +2635,7 @@
         </is>
       </c>
       <c r="AC22" t="n">
-        <v>8.312335051052184</v>
+        <v>7.412335051052183</v>
       </c>
     </row>
     <row r="23">
@@ -2734,7 +2734,7 @@
         </is>
       </c>
       <c r="AC23" t="n">
-        <v>3.678491822977588</v>
+        <v>4.347897732132791</v>
       </c>
     </row>
     <row r="24">
@@ -2833,7 +2833,7 @@
         </is>
       </c>
       <c r="AC24" t="n">
-        <v>6.83053435896676</v>
+        <v>6.782281312629124</v>
       </c>
     </row>
     <row r="25">
@@ -2932,7 +2932,7 @@
         </is>
       </c>
       <c r="AC25" t="n">
-        <v>5.838231326602215</v>
+        <v>5.545209869220241</v>
       </c>
     </row>
     <row r="26">
@@ -3031,7 +3031,7 @@
         </is>
       </c>
       <c r="AC26" t="n">
-        <v>8.189730408427765</v>
+        <v>7.289730408427765</v>
       </c>
     </row>
     <row r="27">
@@ -3130,7 +3130,7 @@
         </is>
       </c>
       <c r="AC27" t="n">
-        <v>8.379253464493518</v>
+        <v>7.479253464493518</v>
       </c>
     </row>
     <row r="28">
@@ -4419,7 +4419,7 @@
         </is>
       </c>
       <c r="AC40" t="n">
-        <v>4.569469418159906</v>
+        <v>4.788613734363567</v>
       </c>
     </row>
     <row r="41">
@@ -4516,7 +4516,7 @@
         </is>
       </c>
       <c r="AC41" t="n">
-        <v>5.79720524846678</v>
+        <v>5.106908984155707</v>
       </c>
     </row>
     <row r="42">
@@ -4613,7 +4613,7 @@
         </is>
       </c>
       <c r="AC42" t="n">
-        <v>3.679976991751182</v>
+        <v>3.903893097618444</v>
       </c>
     </row>
     <row r="43">
@@ -4710,7 +4710,7 @@
         </is>
       </c>
       <c r="AC43" t="n">
-        <v>4.112059012979431</v>
+        <v>3.626663323298775</v>
       </c>
     </row>
     <row r="44">
@@ -4811,7 +4811,7 @@
         </is>
       </c>
       <c r="AC44" t="n">
-        <v>7.153857102290909</v>
+        <v>6.966891144661663</v>
       </c>
     </row>
     <row r="45">
@@ -4908,7 +4908,7 @@
         </is>
       </c>
       <c r="AC45" t="n">
-        <v>4.630522184161555</v>
+        <v>4.739417599027191</v>
       </c>
     </row>
     <row r="46">
@@ -5005,7 +5005,7 @@
         </is>
       </c>
       <c r="AC46" t="n">
-        <v>4.53722316669907</v>
+        <v>4.273076236464505</v>
       </c>
     </row>
     <row r="47">
@@ -5102,7 +5102,7 @@
         </is>
       </c>
       <c r="AC47" t="n">
-        <v>5.78340163796699</v>
+        <v>5.708715265211424</v>
       </c>
     </row>
     <row r="48">
@@ -5199,7 +5199,7 @@
         </is>
       </c>
       <c r="AC48" t="n">
-        <v>4.509014213855417</v>
+        <v>3.759014213855417</v>
       </c>
     </row>
     <row r="49">
@@ -5300,7 +5300,7 @@
         </is>
       </c>
       <c r="AC49" t="n">
-        <v>4.393205169327538</v>
+        <v>3.643205169327538</v>
       </c>
     </row>
     <row r="50">
@@ -5397,7 +5397,7 @@
         </is>
       </c>
       <c r="AC50" t="n">
-        <v>5.117977433131697</v>
+        <v>4.367977433131697</v>
       </c>
     </row>
     <row r="51">
@@ -5494,7 +5494,7 @@
         </is>
       </c>
       <c r="AC51" t="n">
-        <v>0.06080868836915929</v>
+        <v>1.560808688369159</v>
       </c>
     </row>
     <row r="52">
@@ -5595,7 +5595,7 @@
         </is>
       </c>
       <c r="AC52" t="n">
-        <v>2.375828127940919</v>
+        <v>3.875828127940919</v>
       </c>
     </row>
     <row r="53">
@@ -5692,7 +5692,7 @@
         </is>
       </c>
       <c r="AC53" t="n">
-        <v>0.3918547915764282</v>
+        <v>1.891854791576428</v>
       </c>
     </row>
     <row r="54">
@@ -5789,7 +5789,7 @@
         </is>
       </c>
       <c r="AC54" t="n">
-        <v>1.045649912643785</v>
+        <v>2.545649912643785</v>
       </c>
     </row>
     <row r="55">
@@ -5886,7 +5886,7 @@
         </is>
       </c>
       <c r="AC55" t="n">
-        <v>0.9695542369029204</v>
+        <v>2.46955423690292</v>
       </c>
     </row>
     <row r="56">
@@ -5987,7 +5987,7 @@
         </is>
       </c>
       <c r="AC56" t="n">
-        <v>0.3627308368640056</v>
+        <v>1.862730836864006</v>
       </c>
     </row>
     <row r="57">
@@ -6084,7 +6084,7 @@
         </is>
       </c>
       <c r="AC57" t="n">
-        <v>1.825349049484263</v>
+        <v>3.325349049484263</v>
       </c>
     </row>
     <row r="58">
@@ -6147,13 +6147,13 @@
         <v>1</v>
       </c>
       <c r="Q58" t="n">
-        <v>0.371715301152454</v>
+        <v>0.4563497107132452</v>
       </c>
       <c r="R58" t="n">
-        <v>0.5762191378898942</v>
+        <v>0.4914932469238735</v>
       </c>
       <c r="S58" t="n">
-        <v>0.05206556095765168</v>
+        <v>0.05215704236288122</v>
       </c>
       <c r="T58" t="n">
         <v>1</v>
@@ -6161,16 +6161,16 @@
       <c r="U58" t="inlineStr"/>
       <c r="V58" t="inlineStr"/>
       <c r="W58" t="n">
-        <v>-0.1539168678366628</v>
+        <v>-0.2386427588026835</v>
       </c>
       <c r="X58" t="n">
         <v>1</v>
       </c>
       <c r="Y58" t="n">
-        <v>-0.1539168678366628</v>
+        <v>-0.2386427588026835</v>
       </c>
       <c r="Z58" t="n">
-        <v>0.5762191378898942</v>
+        <v>0.4914932469238735</v>
       </c>
       <c r="AA58" t="n">
         <v>1.3</v>
@@ -6181,26 +6181,26 @@
         </is>
       </c>
       <c r="AC58" t="n">
-        <v>2.060433618838304</v>
+        <v>3.497918963086481</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="1" t="inlineStr">
         <is>
-          <t>x4MK4Mzp</t>
+          <t>bJAT205d</t>
         </is>
       </c>
       <c r="B59" s="2" t="n">
-        <v>45684.69791666666</v>
+        <v>45683.69791666666</v>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>genoa</t>
+          <t>lazio</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>monza</t>
+          <t>fiorentina</t>
         </is>
       </c>
       <c r="E59" t="n">
@@ -6220,37 +6220,37 @@
         </is>
       </c>
       <c r="I59" t="n">
-        <v>2.2</v>
+        <v>2.05</v>
       </c>
       <c r="J59" t="n">
-        <v>3</v>
+        <v>3.5</v>
       </c>
       <c r="K59" t="n">
         <v>3.7</v>
       </c>
       <c r="L59" t="n">
-        <v>0.4295665634674923</v>
+        <v>0.4673403103572718</v>
       </c>
       <c r="M59" t="n">
-        <v>0.315015479876161</v>
+        <v>0.273727896066402</v>
       </c>
       <c r="N59" t="n">
-        <v>0.2554179566563468</v>
+        <v>0.2589317935763262</v>
       </c>
       <c r="O59" t="n">
-        <v>0.05814905814905802</v>
+        <v>0.04378943403333646</v>
       </c>
       <c r="P59" t="n">
         <v>1</v>
       </c>
       <c r="Q59" t="n">
-        <v>0.3712725810893399</v>
+        <v>0.1251587896203653</v>
       </c>
       <c r="R59" t="n">
-        <v>0.4069114597785847</v>
+        <v>0.7879557560083729</v>
       </c>
       <c r="S59" t="n">
-        <v>0.2218159591320755</v>
+        <v>0.08688545437126195</v>
       </c>
       <c r="T59" t="n">
         <v>1</v>
@@ -6258,19 +6258,19 @@
       <c r="U59" t="inlineStr"/>
       <c r="V59" t="inlineStr"/>
       <c r="W59" t="n">
-        <v>-0.02265510368890761</v>
+        <v>0.3206154456511011</v>
       </c>
       <c r="X59" t="n">
         <v>1</v>
       </c>
       <c r="Y59" t="n">
-        <v>-0.02265510368890761</v>
+        <v>0.3206154456511011</v>
       </c>
       <c r="Z59" t="n">
-        <v>0.4069114597785847</v>
+        <v>0.7879557560083729</v>
       </c>
       <c r="AA59" t="n">
-        <v>2.2</v>
+        <v>2.05</v>
       </c>
       <c r="AB59" t="inlineStr">
         <is>
@@ -6278,26 +6278,26 @@
         </is>
       </c>
       <c r="AC59" t="n">
-        <v>6.101030676813513</v>
+        <v>7.055469072100474</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="1" t="inlineStr">
         <is>
-          <t>EB0Jrczn</t>
+          <t>naF5yLBL</t>
         </is>
       </c>
       <c r="B60" s="2" t="n">
-        <v>45688.69791666666</v>
+        <v>45684.60416666666</v>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>parma</t>
+          <t>venezia</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>lecce</t>
+          <t>verona</t>
         </is>
       </c>
       <c r="E60" t="n">
@@ -6317,37 +6317,37 @@
         </is>
       </c>
       <c r="I60" t="n">
-        <v>2.1</v>
+        <v>2.15</v>
       </c>
       <c r="J60" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="K60" t="n">
         <v>3.3</v>
       </c>
-      <c r="K60" t="n">
-        <v>3.6</v>
-      </c>
       <c r="L60" t="n">
-        <v>0.4505119453924914</v>
+        <v>0.4413450515857852</v>
       </c>
       <c r="M60" t="n">
-        <v>0.2866894197952218</v>
+        <v>0.2711119602598395</v>
       </c>
       <c r="N60" t="n">
-        <v>0.2627986348122867</v>
+        <v>0.2875429881543752</v>
       </c>
       <c r="O60" t="n">
-        <v>0.05699855699855716</v>
+        <v>0.05386086781435617</v>
       </c>
       <c r="P60" t="n">
         <v>1</v>
       </c>
       <c r="Q60" t="n">
-        <v>0.3481695085688084</v>
+        <v>0.1792033425000428</v>
       </c>
       <c r="R60" t="n">
-        <v>0.4590804575053478</v>
+        <v>0.6967411898110234</v>
       </c>
       <c r="S60" t="n">
-        <v>0.1927500339258439</v>
+        <v>0.1240554676889338</v>
       </c>
       <c r="T60" t="n">
         <v>1</v>
@@ -6355,19 +6355,19 @@
       <c r="U60" t="inlineStr"/>
       <c r="V60" t="inlineStr"/>
       <c r="W60" t="n">
-        <v>0.008568512112856419</v>
+        <v>0.2553961382252382</v>
       </c>
       <c r="X60" t="n">
         <v>1</v>
       </c>
       <c r="Y60" t="n">
-        <v>0.008568512112856419</v>
+        <v>0.2553961382252382</v>
       </c>
       <c r="Z60" t="n">
-        <v>0.4590804575053478</v>
+        <v>0.6967411898110234</v>
       </c>
       <c r="AA60" t="n">
-        <v>2.1</v>
+        <v>2.15</v>
       </c>
       <c r="AB60" t="inlineStr">
         <is>
@@ -6375,26 +6375,26 @@
         </is>
       </c>
       <c r="AC60" t="n">
-        <v>8.263448235096261</v>
+        <v>5.96089427773228</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="1" t="inlineStr">
         <is>
-          <t>bDkKtGm1</t>
+          <t>Ork8ytTI</t>
         </is>
       </c>
       <c r="B61" s="2" t="n">
-        <v>45689.58333333334</v>
+        <v>45689.45833333334</v>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>atalanta</t>
+          <t>monza</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>torino</t>
+          <t>verona</t>
         </is>
       </c>
       <c r="E61" t="n">
@@ -6414,37 +6414,37 @@
         </is>
       </c>
       <c r="I61" t="n">
-        <v>1.4</v>
+        <v>2.15</v>
       </c>
       <c r="J61" t="n">
-        <v>4.33</v>
+        <v>3.1</v>
       </c>
       <c r="K61" t="n">
-        <v>8.5</v>
+        <v>3.6</v>
       </c>
       <c r="L61" t="n">
-        <v>0.6720287764529735</v>
+        <v>0.4365343242714649</v>
       </c>
       <c r="M61" t="n">
-        <v>0.217284130954772</v>
+        <v>0.3027576765108547</v>
       </c>
       <c r="N61" t="n">
-        <v>0.1106870925922545</v>
+        <v>0.2607079992176805</v>
       </c>
       <c r="O61" t="n">
-        <v>0.06287965532633377</v>
+        <v>0.06547470200883554</v>
       </c>
       <c r="P61" t="n">
         <v>1</v>
       </c>
       <c r="Q61" t="n">
-        <v>0.3428032563429664</v>
+        <v>0.2143806883522005</v>
       </c>
       <c r="R61" t="n">
-        <v>0.4232348701910985</v>
+        <v>0.5485352370676453</v>
       </c>
       <c r="S61" t="n">
-        <v>0.233961873465935</v>
+        <v>0.2370840745801543</v>
       </c>
       <c r="T61" t="n">
         <v>1</v>
@@ -6452,19 +6452,19 @@
       <c r="U61" t="inlineStr"/>
       <c r="V61" t="inlineStr"/>
       <c r="W61" t="n">
-        <v>-0.2487939062618751</v>
+        <v>0.1120009127961804</v>
       </c>
       <c r="X61" t="n">
         <v>1</v>
       </c>
       <c r="Y61" t="n">
-        <v>-0.2487939062618751</v>
+        <v>0.1120009127961804</v>
       </c>
       <c r="Z61" t="n">
-        <v>0.4232348701910985</v>
+        <v>0.5485352370676453</v>
       </c>
       <c r="AA61" t="n">
-        <v>1.4</v>
+        <v>2.15</v>
       </c>
       <c r="AB61" t="inlineStr">
         <is>
@@ -6472,26 +6472,26 @@
         </is>
       </c>
       <c r="AC61" t="n">
-        <v>0</v>
+        <v>4.182422844811743</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="1" t="inlineStr">
         <is>
-          <t>t0ciuOTg</t>
+          <t>bDkKtGm1</t>
         </is>
       </c>
       <c r="B62" s="2" t="n">
-        <v>45690.35416666666</v>
+        <v>45689.58333333334</v>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>juventus</t>
+          <t>atalanta</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>empoli</t>
+          <t>torino</t>
         </is>
       </c>
       <c r="E62" t="n">
@@ -6514,34 +6514,34 @@
         <v>1.4</v>
       </c>
       <c r="J62" t="n">
-        <v>4.5</v>
+        <v>4.33</v>
       </c>
       <c r="K62" t="n">
         <v>8.5</v>
       </c>
       <c r="L62" t="n">
-        <v>0.6775907883082374</v>
+        <v>0.6720287764529735</v>
       </c>
       <c r="M62" t="n">
-        <v>0.2108060230292294</v>
+        <v>0.217284130954772</v>
       </c>
       <c r="N62" t="n">
-        <v>0.1116031886625332</v>
+        <v>0.1106870925922545</v>
       </c>
       <c r="O62" t="n">
-        <v>0.05415499533146595</v>
+        <v>0.06287965532633377</v>
       </c>
       <c r="P62" t="n">
         <v>1</v>
       </c>
       <c r="Q62" t="n">
-        <v>0.4316929992687961</v>
+        <v>0.1211341992920172</v>
       </c>
       <c r="R62" t="n">
-        <v>0.5039815631596912</v>
+        <v>0.8473607986958672</v>
       </c>
       <c r="S62" t="n">
-        <v>0.06432543757151267</v>
+        <v>0.03150500201211553</v>
       </c>
       <c r="T62" t="n">
         <v>1</v>
@@ -6549,16 +6549,16 @@
       <c r="U62" t="inlineStr"/>
       <c r="V62" t="inlineStr"/>
       <c r="W62" t="n">
-        <v>-0.1736092251485462</v>
+        <v>0.1753320222428937</v>
       </c>
       <c r="X62" t="n">
         <v>1</v>
       </c>
       <c r="Y62" t="n">
-        <v>-0.1736092251485462</v>
+        <v>0.1753320222428937</v>
       </c>
       <c r="Z62" t="n">
-        <v>0.5039815631596912</v>
+        <v>0.8473607986958672</v>
       </c>
       <c r="AA62" t="n">
         <v>1.4</v>
@@ -6569,26 +6569,26 @@
         </is>
       </c>
       <c r="AC62" t="n">
-        <v>0</v>
+        <v>7.768329584350407</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="1" t="inlineStr">
         <is>
-          <t>Kp9rspas</t>
+          <t>WQmSvfID</t>
         </is>
       </c>
       <c r="B63" s="2" t="n">
-        <v>45690.45833333334</v>
+        <v>45689.69791666666</v>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>fiorentina</t>
+          <t>bologna</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>genoa</t>
+          <t>como</t>
         </is>
       </c>
       <c r="E63" t="n">
@@ -6608,37 +6608,37 @@
         </is>
       </c>
       <c r="I63" t="n">
-        <v>1.57</v>
+        <v>1.8</v>
       </c>
       <c r="J63" t="n">
-        <v>4</v>
+        <v>3.5</v>
       </c>
       <c r="K63" t="n">
-        <v>5.5</v>
+        <v>4.5</v>
       </c>
       <c r="L63" t="n">
-        <v>0.5959637003927942</v>
+        <v>0.5223880597014926</v>
       </c>
       <c r="M63" t="n">
-        <v>0.2339157524041718</v>
+        <v>0.2686567164179104</v>
       </c>
       <c r="N63" t="n">
-        <v>0.170120547203034</v>
+        <v>0.208955223880597</v>
       </c>
       <c r="O63" t="n">
-        <v>0.06876085697741741</v>
+        <v>0.06349206349206349</v>
       </c>
       <c r="P63" t="n">
         <v>1</v>
       </c>
       <c r="Q63" t="n">
-        <v>0.3791381468792345</v>
+        <v>0.1954453953762109</v>
       </c>
       <c r="R63" t="n">
-        <v>0.4555183053429598</v>
+        <v>0.7631365375243826</v>
       </c>
       <c r="S63" t="n">
-        <v>0.1653435477778056</v>
+        <v>0.0414180670994064</v>
       </c>
       <c r="T63" t="n">
         <v>1</v>
@@ -6646,19 +6646,19 @@
       <c r="U63" t="inlineStr"/>
       <c r="V63" t="inlineStr"/>
       <c r="W63" t="n">
-        <v>-0.1404453950498344</v>
+        <v>0.24074847782289</v>
       </c>
       <c r="X63" t="n">
         <v>1</v>
       </c>
       <c r="Y63" t="n">
-        <v>-0.1404453950498344</v>
+        <v>0.24074847782289</v>
       </c>
       <c r="Z63" t="n">
-        <v>0.4555183053429598</v>
+        <v>0.7631365375243826</v>
       </c>
       <c r="AA63" t="n">
-        <v>1.57</v>
+        <v>1.8</v>
       </c>
       <c r="AB63" t="inlineStr">
         <is>
@@ -6666,26 +6666,26 @@
         </is>
       </c>
       <c r="AC63" t="n">
-        <v>0.6152781634822202</v>
+        <v>6.757638450292591</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="1" t="inlineStr">
         <is>
-          <t>AwfSty5b</t>
+          <t>t0ciuOTg</t>
         </is>
       </c>
       <c r="B64" s="2" t="n">
-        <v>45690.69791666666</v>
+        <v>45690.35416666666</v>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>as roma</t>
+          <t>juventus</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>napoli</t>
+          <t>empoli</t>
         </is>
       </c>
       <c r="E64" t="n">
@@ -6705,37 +6705,37 @@
         </is>
       </c>
       <c r="I64" t="n">
-        <v>2.8</v>
+        <v>1.4</v>
       </c>
       <c r="J64" t="n">
-        <v>3.2</v>
+        <v>4.5</v>
       </c>
       <c r="K64" t="n">
-        <v>2.55</v>
+        <v>8.5</v>
       </c>
       <c r="L64" t="n">
-        <v>0.336356141797197</v>
+        <v>0.6775907883082374</v>
       </c>
       <c r="M64" t="n">
-        <v>0.2943116240725474</v>
+        <v>0.2108060230292294</v>
       </c>
       <c r="N64" t="n">
-        <v>0.3693322341302556</v>
+        <v>0.1116031886625332</v>
       </c>
       <c r="O64" t="n">
-        <v>0.06179971988795518</v>
+        <v>0.05415499533146595</v>
       </c>
       <c r="P64" t="n">
         <v>1</v>
       </c>
       <c r="Q64" t="n">
-        <v>0.280331341758519</v>
+        <v>0.1188207267383211</v>
       </c>
       <c r="R64" t="n">
-        <v>0.3675835417936063</v>
+        <v>0.8637231193125966</v>
       </c>
       <c r="S64" t="n">
-        <v>0.3520851164478746</v>
+        <v>0.01745615394908234</v>
       </c>
       <c r="T64" t="n">
         <v>1</v>
@@ -6743,19 +6743,19 @@
       <c r="U64" t="inlineStr"/>
       <c r="V64" t="inlineStr"/>
       <c r="W64" t="n">
-        <v>0.03122739999640928</v>
+        <v>0.1861323310043592</v>
       </c>
       <c r="X64" t="n">
         <v>1</v>
       </c>
       <c r="Y64" t="n">
-        <v>0.03122739999640928</v>
+        <v>0.1861323310043592</v>
       </c>
       <c r="Z64" t="n">
-        <v>0.3675835417936063</v>
+        <v>0.8637231193125966</v>
       </c>
       <c r="AA64" t="n">
-        <v>2.8</v>
+        <v>1.4</v>
       </c>
       <c r="AB64" t="inlineStr">
         <is>
@@ -6763,26 +6763,26 @@
         </is>
       </c>
       <c r="AC64" t="n">
-        <v>6.616503752284913</v>
+        <v>7.964677431751159</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="1" t="inlineStr">
         <is>
-          <t>bwZAFwk2</t>
+          <t>Kp9rspas</t>
         </is>
       </c>
       <c r="B65" s="2" t="n">
-        <v>45681.69791666666</v>
+        <v>45690.45833333334</v>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>torino</t>
+          <t>fiorentina</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>cagliari</t>
+          <t>genoa</t>
         </is>
       </c>
       <c r="E65" t="n">
@@ -6802,37 +6802,37 @@
         </is>
       </c>
       <c r="I65" t="n">
-        <v>2.15</v>
+        <v>1.57</v>
       </c>
       <c r="J65" t="n">
-        <v>3.2</v>
+        <v>4</v>
       </c>
       <c r="K65" t="n">
-        <v>3.7</v>
+        <v>5.5</v>
       </c>
       <c r="L65" t="n">
-        <v>0.4438612933458295</v>
+        <v>0.5959637003927942</v>
       </c>
       <c r="M65" t="n">
-        <v>0.2982193064667292</v>
+        <v>0.2339157524041718</v>
       </c>
       <c r="N65" t="n">
-        <v>0.2579194001874414</v>
+        <v>0.170120547203034</v>
       </c>
       <c r="O65" t="n">
-        <v>0.04788654934003755</v>
+        <v>0.06876085697741741</v>
       </c>
       <c r="P65" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q65" t="n">
-        <v>0.4200132863000589</v>
+        <v>0.3781426267486833</v>
       </c>
       <c r="R65" t="n">
-        <v>0.3763696478844424</v>
+        <v>0.4586722903685529</v>
       </c>
       <c r="S65" t="n">
-        <v>0.2036170658154987</v>
+        <v>0.1631850828827637</v>
       </c>
       <c r="T65" t="n">
         <v>1</v>
@@ -6840,19 +6840,19 @@
       <c r="U65" t="inlineStr"/>
       <c r="V65" t="inlineStr"/>
       <c r="W65" t="n">
-        <v>0.1217939798333297</v>
+        <v>-0.1372914100242413</v>
       </c>
       <c r="X65" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Y65" t="n">
-        <v>0.1217939798333297</v>
+        <v>-0.1372914100242413</v>
       </c>
       <c r="Z65" t="n">
-        <v>0.4200132863000589</v>
+        <v>0.4586722903685529</v>
       </c>
       <c r="AA65" t="n">
-        <v>3.2</v>
+        <v>1.57</v>
       </c>
       <c r="AB65" t="inlineStr">
         <is>
@@ -6860,26 +6860,26 @@
         </is>
       </c>
       <c r="AC65" t="n">
-        <v>9.360239153401059</v>
+        <v>3.104067484422635</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="1" t="inlineStr">
         <is>
-          <t>bJAT205d</t>
+          <t>bwZAFwk2</t>
         </is>
       </c>
       <c r="B66" s="2" t="n">
-        <v>45683.69791666666</v>
+        <v>45681.69791666666</v>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>lazio</t>
+          <t>torino</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>fiorentina</t>
+          <t>cagliari</t>
         </is>
       </c>
       <c r="E66" t="n">
@@ -6899,37 +6899,37 @@
         </is>
       </c>
       <c r="I66" t="n">
-        <v>2.05</v>
+        <v>2.15</v>
       </c>
       <c r="J66" t="n">
-        <v>3.5</v>
+        <v>3.2</v>
       </c>
       <c r="K66" t="n">
         <v>3.7</v>
       </c>
       <c r="L66" t="n">
-        <v>0.4673403103572718</v>
+        <v>0.4438612933458295</v>
       </c>
       <c r="M66" t="n">
-        <v>0.273727896066402</v>
+        <v>0.2982193064667292</v>
       </c>
       <c r="N66" t="n">
-        <v>0.2589317935763262</v>
+        <v>0.2579194001874414</v>
       </c>
       <c r="O66" t="n">
-        <v>0.04378943403333646</v>
+        <v>0.04788654934003755</v>
       </c>
       <c r="P66" t="n">
         <v>0</v>
       </c>
       <c r="Q66" t="n">
-        <v>0.3424911013630586</v>
+        <v>0.6421911165971865</v>
       </c>
       <c r="R66" t="n">
-        <v>0.331065240750304</v>
+        <v>0.1892937149364486</v>
       </c>
       <c r="S66" t="n">
-        <v>0.3264436578866374</v>
+        <v>0.1685151684663648</v>
       </c>
       <c r="T66" t="n">
         <v>1</v>
@@ -6937,19 +6937,19 @@
       <c r="U66" t="inlineStr"/>
       <c r="V66" t="inlineStr"/>
       <c r="W66" t="n">
-        <v>0.06876320529665658</v>
+        <v>0.3439718101304574</v>
       </c>
       <c r="X66" t="n">
         <v>0</v>
       </c>
       <c r="Y66" t="n">
-        <v>0.06876320529665658</v>
+        <v>0.3439718101304574</v>
       </c>
       <c r="Z66" t="n">
-        <v>0.3424911013630586</v>
+        <v>0.6421911165971865</v>
       </c>
       <c r="AA66" t="n">
-        <v>3.5</v>
+        <v>3.2</v>
       </c>
       <c r="AB66" t="inlineStr">
         <is>
@@ -6957,26 +6957,26 @@
         </is>
       </c>
       <c r="AC66" t="n">
-        <v>7.964839824535055</v>
+        <v>8.906293399166238</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="1" t="inlineStr">
         <is>
-          <t>naF5yLBL</t>
+          <t>htW2HaKk</t>
         </is>
       </c>
       <c r="B67" s="2" t="n">
-        <v>45684.60416666666</v>
+        <v>45682.58333333334</v>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>venezia</t>
+          <t>napoli</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>verona</t>
+          <t>juventus</t>
         </is>
       </c>
       <c r="E67" t="n">
@@ -6999,34 +6999,34 @@
         <v>2.15</v>
       </c>
       <c r="J67" t="n">
-        <v>3.5</v>
+        <v>3.1</v>
       </c>
       <c r="K67" t="n">
-        <v>3.3</v>
+        <v>3.8</v>
       </c>
       <c r="L67" t="n">
-        <v>0.4413450515857852</v>
+        <v>0.4426075521322562</v>
       </c>
       <c r="M67" t="n">
-        <v>0.2711119602598395</v>
+        <v>0.3069697538981777</v>
       </c>
       <c r="N67" t="n">
-        <v>0.2875429881543752</v>
+        <v>0.250422693969566</v>
       </c>
       <c r="O67" t="n">
-        <v>0.05386086781435617</v>
+        <v>0.0508548189678999</v>
       </c>
       <c r="P67" t="n">
         <v>0</v>
       </c>
       <c r="Q67" t="n">
-        <v>0.455841654097045</v>
+        <v>0.5691260196730433</v>
       </c>
       <c r="R67" t="n">
-        <v>0.3818418559316768</v>
+        <v>0.3135269573844757</v>
       </c>
       <c r="S67" t="n">
-        <v>0.1623164899712781</v>
+        <v>0.1173470229424811</v>
       </c>
       <c r="T67" t="n">
         <v>1</v>
@@ -7034,19 +7034,19 @@
       <c r="U67" t="inlineStr"/>
       <c r="V67" t="inlineStr"/>
       <c r="W67" t="n">
-        <v>0.1847296938372055</v>
+        <v>0.2621562657748656</v>
       </c>
       <c r="X67" t="n">
         <v>0</v>
       </c>
       <c r="Y67" t="n">
-        <v>0.1847296938372055</v>
+        <v>0.2621562657748656</v>
       </c>
       <c r="Z67" t="n">
-        <v>0.455841654097045</v>
+        <v>0.5691260196730433</v>
       </c>
       <c r="AA67" t="n">
-        <v>3.5</v>
+        <v>3.1</v>
       </c>
       <c r="AB67" t="inlineStr">
         <is>
@@ -7054,26 +7054,26 @@
         </is>
       </c>
       <c r="AC67" t="n">
-        <v>10.00514977374681</v>
+        <v>8.029512236076521</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="1" t="inlineStr">
         <is>
-          <t>Ork8ytTI</t>
+          <t>x4MK4Mzp</t>
         </is>
       </c>
       <c r="B68" s="2" t="n">
-        <v>45689.45833333334</v>
+        <v>45684.69791666666</v>
       </c>
       <c r="C68" t="inlineStr">
         <is>
+          <t>genoa</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
           <t>monza</t>
-        </is>
-      </c>
-      <c r="D68" t="inlineStr">
-        <is>
-          <t>verona</t>
         </is>
       </c>
       <c r="E68" t="n">
@@ -7093,37 +7093,37 @@
         </is>
       </c>
       <c r="I68" t="n">
-        <v>2.15</v>
+        <v>2.2</v>
       </c>
       <c r="J68" t="n">
-        <v>3.1</v>
+        <v>3</v>
       </c>
       <c r="K68" t="n">
-        <v>3.6</v>
+        <v>3.7</v>
       </c>
       <c r="L68" t="n">
-        <v>0.4365343242714649</v>
+        <v>0.4295665634674923</v>
       </c>
       <c r="M68" t="n">
-        <v>0.3027576765108547</v>
+        <v>0.315015479876161</v>
       </c>
       <c r="N68" t="n">
-        <v>0.2607079992176805</v>
+        <v>0.2554179566563468</v>
       </c>
       <c r="O68" t="n">
-        <v>0.06547470200883554</v>
+        <v>0.05814905814905802</v>
       </c>
       <c r="P68" t="n">
         <v>0</v>
       </c>
       <c r="Q68" t="n">
-        <v>0.4280969800506781</v>
+        <v>0.5494671942343683</v>
       </c>
       <c r="R68" t="n">
-        <v>0.3807428730716954</v>
+        <v>0.3832345330033678</v>
       </c>
       <c r="S68" t="n">
-        <v>0.1911601468776264</v>
+        <v>0.06729827276226394</v>
       </c>
       <c r="T68" t="n">
         <v>1</v>
@@ -7131,19 +7131,19 @@
       <c r="U68" t="inlineStr"/>
       <c r="V68" t="inlineStr"/>
       <c r="W68" t="n">
-        <v>0.1253393035398235</v>
+        <v>0.2344517143582073</v>
       </c>
       <c r="X68" t="n">
         <v>0</v>
       </c>
       <c r="Y68" t="n">
-        <v>0.1253393035398235</v>
+        <v>0.2344517143582073</v>
       </c>
       <c r="Z68" t="n">
-        <v>0.4280969800506781</v>
+        <v>0.5494671942343683</v>
       </c>
       <c r="AA68" t="n">
-        <v>3.1</v>
+        <v>3</v>
       </c>
       <c r="AB68" t="inlineStr">
         <is>
@@ -7151,26 +7151,26 @@
         </is>
       </c>
       <c r="AC68" t="n">
-        <v>9.505745640912206</v>
+        <v>7.793606330812419</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="1" t="inlineStr">
         <is>
-          <t>2oCZvFZA</t>
+          <t>EB0Jrczn</t>
         </is>
       </c>
       <c r="B69" s="2" t="n">
-        <v>45689.45833333334</v>
+        <v>45688.69791666666</v>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>udinese</t>
+          <t>parma</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>venezia</t>
+          <t>lecce</t>
         </is>
       </c>
       <c r="E69" t="n">
@@ -7190,58 +7190,54 @@
         </is>
       </c>
       <c r="I69" t="n">
-        <v>1.8</v>
+        <v>2.1</v>
       </c>
       <c r="J69" t="n">
         <v>3.3</v>
       </c>
       <c r="K69" t="n">
-        <v>4.75</v>
+        <v>3.6</v>
       </c>
       <c r="L69" t="n">
-        <v>0.5196419691695674</v>
+        <v>0.4505119453924914</v>
       </c>
       <c r="M69" t="n">
-        <v>0.2834410740924913</v>
+        <v>0.2866894197952218</v>
       </c>
       <c r="N69" t="n">
-        <v>0.1969169567379413</v>
+        <v>0.2627986348122867</v>
       </c>
       <c r="O69" t="n">
-        <v>0.06911217437533224</v>
+        <v>0.05699855699855716</v>
       </c>
       <c r="P69" t="n">
         <v>0</v>
       </c>
       <c r="Q69" t="n">
-        <v>0.4561494420175064</v>
+        <v>0.4038945963810401</v>
       </c>
       <c r="R69" t="n">
-        <v>0.3895656086433587</v>
+        <v>0.3062718022668496</v>
       </c>
       <c r="S69" t="n">
-        <v>0.1542849493391349</v>
+        <v>0.2898336013521101</v>
       </c>
       <c r="T69" t="n">
         <v>1</v>
       </c>
-      <c r="U69" t="n">
-        <v>1</v>
-      </c>
-      <c r="V69" t="n">
-        <v>1</v>
-      </c>
+      <c r="U69" t="inlineStr"/>
+      <c r="V69" t="inlineStr"/>
       <c r="W69" t="n">
-        <v>0.1727083679250151</v>
+        <v>0.1172051765858183</v>
       </c>
       <c r="X69" t="n">
         <v>0</v>
       </c>
       <c r="Y69" t="n">
-        <v>0.1727083679250151</v>
+        <v>0.1172051765858183</v>
       </c>
       <c r="Z69" t="n">
-        <v>0.4561494420175064</v>
+        <v>0.4038945963810401</v>
       </c>
       <c r="AA69" t="n">
         <v>3.3</v>
@@ -7252,26 +7248,26 @@
         </is>
       </c>
       <c r="AC69" t="n">
-        <v>5.005344978157557</v>
+        <v>6.046735156572481</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="1" t="inlineStr">
         <is>
-          <t>WQmSvfID</t>
+          <t>2oCZvFZA</t>
         </is>
       </c>
       <c r="B70" s="2" t="n">
-        <v>45689.69791666666</v>
+        <v>45689.45833333334</v>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>bologna</t>
+          <t>udinese</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>como</t>
+          <t>venezia</t>
         </is>
       </c>
       <c r="E70" t="n">
@@ -7294,54 +7290,58 @@
         <v>1.8</v>
       </c>
       <c r="J70" t="n">
-        <v>3.5</v>
+        <v>3.3</v>
       </c>
       <c r="K70" t="n">
-        <v>4.5</v>
+        <v>4.75</v>
       </c>
       <c r="L70" t="n">
-        <v>0.5223880597014926</v>
+        <v>0.5196419691695674</v>
       </c>
       <c r="M70" t="n">
-        <v>0.2686567164179104</v>
+        <v>0.2834410740924913</v>
       </c>
       <c r="N70" t="n">
-        <v>0.208955223880597</v>
+        <v>0.1969169567379413</v>
       </c>
       <c r="O70" t="n">
-        <v>0.06349206349206349</v>
+        <v>0.06911217437533224</v>
       </c>
       <c r="P70" t="n">
         <v>0</v>
       </c>
       <c r="Q70" t="n">
-        <v>0.4831459241902815</v>
+        <v>0.5355202294277688</v>
       </c>
       <c r="R70" t="n">
-        <v>0.3138087438468286</v>
+        <v>0.2550516099873402</v>
       </c>
       <c r="S70" t="n">
-        <v>0.20304533196289</v>
+        <v>0.2094281605848909</v>
       </c>
       <c r="T70" t="n">
         <v>1</v>
       </c>
-      <c r="U70" t="inlineStr"/>
-      <c r="V70" t="inlineStr"/>
+      <c r="U70" t="n">
+        <v>1</v>
+      </c>
+      <c r="V70" t="n">
+        <v>1</v>
+      </c>
       <c r="W70" t="n">
-        <v>0.2144892077723711</v>
+        <v>0.2520791553352775</v>
       </c>
       <c r="X70" t="n">
         <v>0</v>
       </c>
       <c r="Y70" t="n">
-        <v>0.2144892077723711</v>
+        <v>0.2520791553352775</v>
       </c>
       <c r="Z70" t="n">
-        <v>0.4831459241902815</v>
+        <v>0.5355202294277688</v>
       </c>
       <c r="AA70" t="n">
-        <v>3.5</v>
+        <v>3.3</v>
       </c>
       <c r="AB70" t="inlineStr">
         <is>
@@ -7349,7 +7349,7 @@
         </is>
       </c>
       <c r="AC70" t="n">
-        <v>10.49662663542507</v>
+        <v>3.813121376566612</v>
       </c>
     </row>
     <row r="71">
@@ -7412,13 +7412,13 @@
         <v>2</v>
       </c>
       <c r="Q71" t="n">
-        <v>0.3270315055055304</v>
+        <v>0.1416082615275219</v>
       </c>
       <c r="R71" t="n">
-        <v>0.332296588602205</v>
+        <v>0.06116305433511001</v>
       </c>
       <c r="S71" t="n">
-        <v>0.3406719058922646</v>
+        <v>0.7972286841373681</v>
       </c>
       <c r="T71" t="n">
         <v>1</v>
@@ -7426,16 +7426,16 @@
       <c r="U71" t="inlineStr"/>
       <c r="V71" t="inlineStr"/>
       <c r="W71" t="n">
-        <v>-0.1710032210112887</v>
+        <v>0.2855535572338148</v>
       </c>
       <c r="X71" t="n">
         <v>2</v>
       </c>
       <c r="Y71" t="n">
-        <v>-0.1710032210112887</v>
+        <v>0.2855535572338148</v>
       </c>
       <c r="Z71" t="n">
-        <v>0.3406719058922646</v>
+        <v>0.7972286841373681</v>
       </c>
       <c r="AA71" t="n">
         <v>1.85</v>
@@ -7446,26 +7446,26 @@
         </is>
       </c>
       <c r="AC71" t="n">
-        <v>0</v>
+        <v>10.76674420964842</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="1" t="inlineStr">
         <is>
-          <t>htW2HaKk</t>
+          <t>W4fmNUjB</t>
         </is>
       </c>
       <c r="B72" s="2" t="n">
-        <v>45682.58333333334</v>
+        <v>45682.69791666666</v>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>napoli</t>
+          <t>empoli</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>juventus</t>
+          <t>bologna</t>
         </is>
       </c>
       <c r="E72" t="n">
@@ -7485,37 +7485,37 @@
         </is>
       </c>
       <c r="I72" t="n">
-        <v>2.15</v>
+        <v>3.75</v>
       </c>
       <c r="J72" t="n">
-        <v>3.1</v>
+        <v>3.25</v>
       </c>
       <c r="K72" t="n">
-        <v>3.8</v>
+        <v>2.05</v>
       </c>
       <c r="L72" t="n">
-        <v>0.4426075521322562</v>
+        <v>0.2510598210080076</v>
       </c>
       <c r="M72" t="n">
-        <v>0.3069697538981777</v>
+        <v>0.2896844088553933</v>
       </c>
       <c r="N72" t="n">
-        <v>0.250422693969566</v>
+        <v>0.4592557701365992</v>
       </c>
       <c r="O72" t="n">
-        <v>0.0508548189678999</v>
+        <v>0.06216385240775479</v>
       </c>
       <c r="P72" t="n">
         <v>2</v>
       </c>
       <c r="Q72" t="n">
-        <v>0.3833815806681548</v>
+        <v>0.313345721568263</v>
       </c>
       <c r="R72" t="n">
-        <v>0.2204611011125606</v>
+        <v>0.1055673374383774</v>
       </c>
       <c r="S72" t="n">
-        <v>0.3961573182192846</v>
+        <v>0.5810869409933597</v>
       </c>
       <c r="T72" t="n">
         <v>1</v>
@@ -7523,19 +7523,19 @@
       <c r="U72" t="inlineStr"/>
       <c r="V72" t="inlineStr"/>
       <c r="W72" t="n">
-        <v>0.1457346242497186</v>
+        <v>0.1218311708567604</v>
       </c>
       <c r="X72" t="n">
         <v>2</v>
       </c>
       <c r="Y72" t="n">
-        <v>0.1457346242497186</v>
+        <v>0.1218311708567604</v>
       </c>
       <c r="Z72" t="n">
-        <v>0.3961573182192846</v>
+        <v>0.5810869409933597</v>
       </c>
       <c r="AA72" t="n">
-        <v>3.8</v>
+        <v>2.05</v>
       </c>
       <c r="AB72" t="inlineStr">
         <is>
@@ -7543,26 +7543,26 @@
         </is>
       </c>
       <c r="AC72" t="n">
-        <v>7.130831727947123</v>
+        <v>8.173043291920315</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="1" t="inlineStr">
         <is>
-          <t>W4fmNUjB</t>
+          <t>vZBcwss9</t>
         </is>
       </c>
       <c r="B73" s="2" t="n">
-        <v>45682.69791666666</v>
+        <v>45683.45833333334</v>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>empoli</t>
+          <t>udinese</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>bologna</t>
+          <t>as roma</t>
         </is>
       </c>
       <c r="E73" t="n">
@@ -7582,57 +7582,61 @@
         </is>
       </c>
       <c r="I73" t="n">
-        <v>3.75</v>
+        <v>3.3</v>
       </c>
       <c r="J73" t="n">
-        <v>3.25</v>
+        <v>3.3</v>
       </c>
       <c r="K73" t="n">
-        <v>2.05</v>
+        <v>2.25</v>
       </c>
       <c r="L73" t="n">
-        <v>0.2510598210080076</v>
+        <v>0.2884615384615384</v>
       </c>
       <c r="M73" t="n">
-        <v>0.2896844088553933</v>
+        <v>0.2884615384615384</v>
       </c>
       <c r="N73" t="n">
-        <v>0.4592557701365992</v>
+        <v>0.423076923076923</v>
       </c>
       <c r="O73" t="n">
-        <v>0.06216385240775479</v>
+        <v>0.05050505050505061</v>
       </c>
       <c r="P73" t="n">
         <v>2</v>
       </c>
       <c r="Q73" t="n">
-        <v>0.3910787539425644</v>
+        <v>0.3782050025390681</v>
       </c>
       <c r="R73" t="n">
-        <v>0.1979401462465879</v>
+        <v>0.1155314689342525</v>
       </c>
       <c r="S73" t="n">
-        <v>0.4109810998108477</v>
+        <v>0.5062635285266793</v>
       </c>
       <c r="T73" t="n">
         <v>1</v>
       </c>
-      <c r="U73" t="inlineStr"/>
-      <c r="V73" t="inlineStr"/>
+      <c r="U73" t="n">
+        <v>1</v>
+      </c>
+      <c r="V73" t="n">
+        <v>1</v>
+      </c>
       <c r="W73" t="n">
-        <v>-0.0482746703257515</v>
+        <v>0.08318660544975631</v>
       </c>
       <c r="X73" t="n">
         <v>2</v>
       </c>
       <c r="Y73" t="n">
-        <v>-0.0482746703257515</v>
+        <v>0.08318660544975631</v>
       </c>
       <c r="Z73" t="n">
-        <v>0.4109810998108477</v>
+        <v>0.5062635285266793</v>
       </c>
       <c r="AA73" t="n">
-        <v>2.05</v>
+        <v>2.25</v>
       </c>
       <c r="AB73" t="inlineStr">
         <is>
@@ -7640,26 +7644,26 @@
         </is>
       </c>
       <c r="AC73" t="n">
-        <v>5.659771664868205</v>
+        <v>3.637581171160076</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="1" t="inlineStr">
         <is>
-          <t>vZBcwss9</t>
+          <t>4GcFQ3c3</t>
         </is>
       </c>
       <c r="B74" s="2" t="n">
-        <v>45683.45833333334</v>
+        <v>45683.58333333334</v>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>udinese</t>
+          <t>lecce</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>as roma</t>
+          <t>inter</t>
         </is>
       </c>
       <c r="E74" t="n">
@@ -7679,61 +7683,57 @@
         </is>
       </c>
       <c r="I74" t="n">
-        <v>3.3</v>
+        <v>9</v>
       </c>
       <c r="J74" t="n">
-        <v>3.3</v>
+        <v>5.25</v>
       </c>
       <c r="K74" t="n">
-        <v>2.25</v>
+        <v>1.33</v>
       </c>
       <c r="L74" t="n">
-        <v>0.2884615384615384</v>
+        <v>0.105471847739889</v>
       </c>
       <c r="M74" t="n">
-        <v>0.2884615384615384</v>
+        <v>0.1808088818398097</v>
       </c>
       <c r="N74" t="n">
-        <v>0.423076923076923</v>
+        <v>0.7137192704203014</v>
       </c>
       <c r="O74" t="n">
-        <v>0.05050505050505061</v>
+        <v>0.05346700083542189</v>
       </c>
       <c r="P74" t="n">
         <v>2</v>
       </c>
       <c r="Q74" t="n">
-        <v>0.3533253075257501</v>
+        <v>0.1215871283657537</v>
       </c>
       <c r="R74" t="n">
-        <v>0.2481608913953272</v>
+        <v>0.02568209101000827</v>
       </c>
       <c r="S74" t="n">
-        <v>0.3985138010789226</v>
+        <v>0.8527307806242381</v>
       </c>
       <c r="T74" t="n">
         <v>1</v>
       </c>
-      <c r="U74" t="n">
-        <v>1</v>
-      </c>
-      <c r="V74" t="n">
-        <v>1</v>
-      </c>
+      <c r="U74" t="inlineStr"/>
+      <c r="V74" t="inlineStr"/>
       <c r="W74" t="n">
-        <v>-0.02456312199800043</v>
+        <v>0.1390115102039368</v>
       </c>
       <c r="X74" t="n">
         <v>2</v>
       </c>
       <c r="Y74" t="n">
-        <v>-0.02456312199800043</v>
+        <v>0.1390115102039368</v>
       </c>
       <c r="Z74" t="n">
-        <v>0.3985138010789226</v>
+        <v>0.8527307806242381</v>
       </c>
       <c r="AA74" t="n">
-        <v>2.25</v>
+        <v>1.33</v>
       </c>
       <c r="AB74" t="inlineStr">
         <is>
@@ -7741,21 +7741,21 @@
         </is>
       </c>
       <c r="AC74" t="n">
-        <v>3.144488013746295</v>
+        <v>11.43276936749086</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="1" t="inlineStr">
         <is>
-          <t>4GcFQ3c3</t>
+          <t>SGeaw2b6</t>
         </is>
       </c>
       <c r="B75" s="2" t="n">
-        <v>45683.58333333334</v>
+        <v>45690.58333333334</v>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>lecce</t>
+          <t>ac milan</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -7780,37 +7780,37 @@
         </is>
       </c>
       <c r="I75" t="n">
-        <v>9</v>
+        <v>3.1</v>
       </c>
       <c r="J75" t="n">
-        <v>5.25</v>
+        <v>3.3</v>
       </c>
       <c r="K75" t="n">
-        <v>1.33</v>
+        <v>2.25</v>
       </c>
       <c r="L75" t="n">
-        <v>0.105471847739889</v>
+        <v>0.3014616321559074</v>
       </c>
       <c r="M75" t="n">
-        <v>0.1808088818398097</v>
+        <v>0.2831912302070645</v>
       </c>
       <c r="N75" t="n">
-        <v>0.7137192704203014</v>
+        <v>0.415347137637028</v>
       </c>
       <c r="O75" t="n">
-        <v>0.05346700083542189</v>
+        <v>0.07005539263603788</v>
       </c>
       <c r="P75" t="n">
         <v>2</v>
       </c>
       <c r="Q75" t="n">
-        <v>0.2351474832077743</v>
+        <v>0.2431778023155322</v>
       </c>
       <c r="R75" t="n">
-        <v>0.1159383563722011</v>
+        <v>0.1583692637022357</v>
       </c>
       <c r="S75" t="n">
-        <v>0.6489141604200246</v>
+        <v>0.598452933982232</v>
       </c>
       <c r="T75" t="n">
         <v>1</v>
@@ -7818,19 +7818,19 @@
       <c r="U75" t="inlineStr"/>
       <c r="V75" t="inlineStr"/>
       <c r="W75" t="n">
-        <v>-0.06480511000027678</v>
+        <v>0.183105796345204</v>
       </c>
       <c r="X75" t="n">
         <v>2</v>
       </c>
       <c r="Y75" t="n">
-        <v>-0.06480511000027678</v>
+        <v>0.183105796345204</v>
       </c>
       <c r="Z75" t="n">
-        <v>0.6489141604200246</v>
+        <v>0.598452933982232</v>
       </c>
       <c r="AA75" t="n">
-        <v>1.33</v>
+        <v>2.25</v>
       </c>
       <c r="AB75" t="inlineStr">
         <is>
@@ -7838,26 +7838,26 @@
         </is>
       </c>
       <c r="AC75" t="n">
-        <v>9.347470927550479</v>
+        <v>8.381435207786783</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="1" t="inlineStr">
         <is>
-          <t>SGeaw2b6</t>
+          <t>AwfSty5b</t>
         </is>
       </c>
       <c r="B76" s="2" t="n">
-        <v>45690.58333333334</v>
+        <v>45690.69791666666</v>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>ac milan</t>
+          <t>as roma</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>inter</t>
+          <t>napoli</t>
         </is>
       </c>
       <c r="E76" t="n">
@@ -7877,37 +7877,37 @@
         </is>
       </c>
       <c r="I76" t="n">
-        <v>3.1</v>
+        <v>2.8</v>
       </c>
       <c r="J76" t="n">
-        <v>3.3</v>
+        <v>3.2</v>
       </c>
       <c r="K76" t="n">
-        <v>2.25</v>
+        <v>2.55</v>
       </c>
       <c r="L76" t="n">
-        <v>0.3014616321559074</v>
+        <v>0.336356141797197</v>
       </c>
       <c r="M76" t="n">
-        <v>0.2831912302070645</v>
+        <v>0.2943116240725474</v>
       </c>
       <c r="N76" t="n">
-        <v>0.415347137637028</v>
+        <v>0.3693322341302556</v>
       </c>
       <c r="O76" t="n">
-        <v>0.07005539263603788</v>
+        <v>0.06179971988795518</v>
       </c>
       <c r="P76" t="n">
         <v>2</v>
       </c>
       <c r="Q76" t="n">
-        <v>0.2968647600909247</v>
+        <v>0.2603878572162487</v>
       </c>
       <c r="R76" t="n">
-        <v>0.3255662605986677</v>
+        <v>0.2415646209635194</v>
       </c>
       <c r="S76" t="n">
-        <v>0.3775689793104076</v>
+        <v>0.498047521820232</v>
       </c>
       <c r="T76" t="n">
         <v>1</v>
@@ -7915,19 +7915,19 @@
       <c r="U76" t="inlineStr"/>
       <c r="V76" t="inlineStr"/>
       <c r="W76" t="n">
-        <v>-0.03777815832662035</v>
+        <v>0.1287152876899764</v>
       </c>
       <c r="X76" t="n">
         <v>2</v>
       </c>
       <c r="Y76" t="n">
-        <v>-0.03777815832662035</v>
+        <v>0.1287152876899764</v>
       </c>
       <c r="Z76" t="n">
-        <v>0.3775689793104076</v>
+        <v>0.498047521820232</v>
       </c>
       <c r="AA76" t="n">
-        <v>2.25</v>
+        <v>2.55</v>
       </c>
       <c r="AB76" t="inlineStr">
         <is>
@@ -7935,7 +7935,7 @@
         </is>
       </c>
       <c r="AC76" t="n">
-        <v>5.436227927829004</v>
+        <v>7.176570261842783</v>
       </c>
     </row>
     <row r="77">
@@ -7998,13 +7998,13 @@
         <v>2</v>
       </c>
       <c r="Q77" t="n">
-        <v>0.250949664344346</v>
+        <v>0.2987208499111965</v>
       </c>
       <c r="R77" t="n">
-        <v>0.2113235469434867</v>
+        <v>0.04107558803168093</v>
       </c>
       <c r="S77" t="n">
-        <v>0.5377267887121672</v>
+        <v>0.6602035620571226</v>
       </c>
       <c r="T77" t="n">
         <v>1</v>
@@ -8012,16 +8012,16 @@
       <c r="U77" t="inlineStr"/>
       <c r="V77" t="inlineStr"/>
       <c r="W77" t="n">
-        <v>0.08082527210629264</v>
+        <v>0.2033020454512481</v>
       </c>
       <c r="X77" t="n">
         <v>2</v>
       </c>
       <c r="Y77" t="n">
-        <v>0.08082527210629264</v>
+        <v>0.2033020454512481</v>
       </c>
       <c r="Z77" t="n">
-        <v>0.5377267887121672</v>
+        <v>0.6602035620571226</v>
       </c>
       <c r="AA77" t="n">
         <v>2.05</v>
@@ -8032,7 +8032,7 @@
         </is>
       </c>
       <c r="AC77" t="n">
-        <v>9.679082196819008</v>
+        <v>9.122442744685472</v>
       </c>
     </row>
     <row r="78">
@@ -8131,7 +8131,7 @@
         </is>
       </c>
       <c r="AC78" t="n">
-        <v>9.007369754750586</v>
+        <v>7.807369754750587</v>
       </c>
     </row>
     <row r="79">
@@ -8230,7 +8230,7 @@
         </is>
       </c>
       <c r="AC79" t="n">
-        <v>8.628441652758612</v>
+        <v>7.428441652758613</v>
       </c>
     </row>
     <row r="80">
@@ -8329,7 +8329,7 @@
         </is>
       </c>
       <c r="AC80" t="n">
-        <v>8.17340575228066</v>
+        <v>6.97340575228066</v>
       </c>
     </row>
     <row r="81">
@@ -8428,7 +8428,7 @@
         </is>
       </c>
       <c r="AC81" t="n">
-        <v>6.139332770947562</v>
+        <v>4.939332770947563</v>
       </c>
     </row>
     <row r="82">
@@ -8527,7 +8527,7 @@
         </is>
       </c>
       <c r="AC82" t="n">
-        <v>11.00344070707258</v>
+        <v>9.803440707072578</v>
       </c>
     </row>
     <row r="83">
@@ -8626,7 +8626,7 @@
         </is>
       </c>
       <c r="AC83" t="n">
-        <v>2.223248807950946</v>
+        <v>1.023248807950946</v>
       </c>
     </row>
     <row r="84">
@@ -8725,7 +8725,7 @@
         </is>
       </c>
       <c r="AC84" t="n">
-        <v>7.607256571793</v>
+        <v>6.407256571793</v>
       </c>
     </row>
     <row r="85">
@@ -8824,7 +8824,7 @@
         </is>
       </c>
       <c r="AC85" t="n">
-        <v>9.144784207282601</v>
+        <v>7.944784207282601</v>
       </c>
     </row>
     <row r="86">
@@ -8923,7 +8923,7 @@
         </is>
       </c>
       <c r="AC86" t="n">
-        <v>8.710186867687165</v>
+        <v>7.510186867687164</v>
       </c>
     </row>
     <row r="87">
@@ -9022,7 +9022,7 @@
         </is>
       </c>
       <c r="AC87" t="n">
-        <v>4.891903448897097</v>
+        <v>3.691903448897098</v>
       </c>
     </row>
     <row r="88">
@@ -9121,7 +9121,7 @@
         </is>
       </c>
       <c r="AC88" t="n">
-        <v>7.244670723941416</v>
+        <v>6.044670723941417</v>
       </c>
     </row>
     <row r="89">
@@ -9220,7 +9220,7 @@
         </is>
       </c>
       <c r="AC89" t="n">
-        <v>6.671312172315509</v>
+        <v>5.47131217231551</v>
       </c>
     </row>
     <row r="90">
@@ -9319,7 +9319,7 @@
         </is>
       </c>
       <c r="AC90" t="n">
-        <v>7.173252247230842</v>
+        <v>5.973252247230842</v>
       </c>
     </row>
     <row r="91">
@@ -9418,7 +9418,7 @@
         </is>
       </c>
       <c r="AC91" t="n">
-        <v>7.538237559360721</v>
+        <v>6.338237559360721</v>
       </c>
     </row>
     <row r="92">
@@ -9517,7 +9517,7 @@
         </is>
       </c>
       <c r="AC92" t="n">
-        <v>7.838395862765243</v>
+        <v>6.638395862765242</v>
       </c>
     </row>
     <row r="93">
@@ -9616,7 +9616,7 @@
         </is>
       </c>
       <c r="AC93" t="n">
-        <v>4.821174493855509</v>
+        <v>7.22117449385551</v>
       </c>
     </row>
     <row r="94">
@@ -9715,7 +9715,7 @@
         </is>
       </c>
       <c r="AC94" t="n">
-        <v>0.2117159540940882</v>
+        <v>2.611715954094088</v>
       </c>
     </row>
     <row r="95">
@@ -9814,7 +9814,7 @@
         </is>
       </c>
       <c r="AC95" t="n">
-        <v>0</v>
+        <v>2.17279433130474</v>
       </c>
     </row>
     <row r="96">
@@ -9913,7 +9913,7 @@
         </is>
       </c>
       <c r="AC96" t="n">
-        <v>3.820815622552447</v>
+        <v>6.220815622552448</v>
       </c>
     </row>
     <row r="97">
@@ -10012,7 +10012,7 @@
         </is>
       </c>
       <c r="AC97" t="n">
-        <v>1.208436384012615</v>
+        <v>3.608436384012615</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualizo predicciones por uso de kelly
</commit_message>
<xml_diff>
--- a/data/predicciones.xlsx
+++ b/data/predicciones.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC97"/>
+  <dimension ref="A1:AD97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -575,6 +575,11 @@
       </c>
       <c r="AC1" s="1" t="inlineStr">
         <is>
+          <t>stake_to_bet_norm</t>
+        </is>
+      </c>
+      <c r="AD1" s="1" t="inlineStr">
+        <is>
           <t>stake_to_bet</t>
         </is>
       </c>
@@ -673,7 +678,10 @@
         </is>
       </c>
       <c r="AC2" t="n">
-        <v>0</v>
+        <v>-11.60346812365947</v>
+      </c>
+      <c r="AD2" t="n">
+        <v>1.141783779436085e-05</v>
       </c>
     </row>
     <row r="3">
@@ -774,7 +782,10 @@
         </is>
       </c>
       <c r="AC3" t="n">
-        <v>4.349248910009321</v>
+        <v>-17.58632303569895</v>
+      </c>
+      <c r="AD3" t="n">
+        <v>2.879167634379533e-08</v>
       </c>
     </row>
     <row r="4">
@@ -871,7 +882,10 @@
         </is>
       </c>
       <c r="AC4" t="n">
-        <v>2.272120876050594</v>
+        <v>-0.9055268007475179</v>
+      </c>
+      <c r="AD4" t="n">
+        <v>0.3598950795241962</v>
       </c>
     </row>
     <row r="5">
@@ -968,7 +982,10 @@
         </is>
       </c>
       <c r="AC5" t="n">
-        <v>2.041319084593269</v>
+        <v>-1.372182854086922</v>
+      </c>
+      <c r="AD5" t="n">
+        <v>0.2528342530481353</v>
       </c>
     </row>
     <row r="6">
@@ -1065,7 +1082,10 @@
         </is>
       </c>
       <c r="AC6" t="n">
-        <v>2.426940437882931</v>
+        <v>0.1698974713976842</v>
+      </c>
+      <c r="AD6" t="n">
+        <v>0.677965616021361</v>
       </c>
     </row>
     <row r="7">
@@ -1162,7 +1182,10 @@
         </is>
       </c>
       <c r="AC7" t="n">
-        <v>0</v>
+        <v>-14.05972538998856</v>
+      </c>
+      <c r="AD7" t="n">
+        <v>9.791484006480864e-07</v>
       </c>
     </row>
     <row r="8">
@@ -1263,7 +1286,10 @@
         </is>
       </c>
       <c r="AC8" t="n">
-        <v>7.41812177849396</v>
+        <v>1.098916746714305</v>
+      </c>
+      <c r="AD8" t="n">
+        <v>11.25085622307731</v>
       </c>
     </row>
     <row r="9">
@@ -1360,7 +1386,10 @@
         </is>
       </c>
       <c r="AC9" t="n">
-        <v>5.596352487988231</v>
+        <v>0.6206412297193616</v>
+      </c>
+      <c r="AD9" t="n">
+        <v>9.755465583165039</v>
       </c>
     </row>
     <row r="10">
@@ -1457,7 +1486,10 @@
         </is>
       </c>
       <c r="AC10" t="n">
-        <v>6.614926808304434</v>
+        <v>0.8149810243752235</v>
+      </c>
+      <c r="AD10" t="n">
+        <v>10.39754870254037</v>
       </c>
     </row>
     <row r="11">
@@ -1558,7 +1590,10 @@
         </is>
       </c>
       <c r="AC11" t="n">
-        <v>7.080301790843282</v>
+        <v>0.9580123548415658</v>
+      </c>
+      <c r="AD11" t="n">
+        <v>10.84085503518367</v>
       </c>
     </row>
     <row r="12">
@@ -1659,7 +1694,10 @@
         </is>
       </c>
       <c r="AC12" t="n">
-        <v>4.438504608877666</v>
+        <v>0.2338669498598813</v>
+      </c>
+      <c r="AD12" t="n">
+        <v>8.373025597445988</v>
       </c>
     </row>
     <row r="13">
@@ -1756,7 +1794,10 @@
         </is>
       </c>
       <c r="AC13" t="n">
-        <v>6.296243262041672</v>
+        <v>0.760960608185076</v>
+      </c>
+      <c r="AD13" t="n">
+        <v>10.22343383820384</v>
       </c>
     </row>
     <row r="14">
@@ -1853,7 +1894,10 @@
         </is>
       </c>
       <c r="AC14" t="n">
-        <v>4.815164668902383</v>
+        <v>0.3483760252709882</v>
+      </c>
+      <c r="AD14" t="n">
+        <v>8.793355709394065</v>
       </c>
     </row>
     <row r="15">
@@ -1950,7 +1994,10 @@
         </is>
       </c>
       <c r="AC15" t="n">
-        <v>5.399296513317783</v>
+        <v>0.9718531088395775</v>
+      </c>
+      <c r="AD15" t="n">
+        <v>5.441165306699458</v>
       </c>
     </row>
     <row r="16">
@@ -2051,7 +2098,10 @@
         </is>
       </c>
       <c r="AC16" t="n">
-        <v>7.045917684876547</v>
+        <v>-0.240561629166934</v>
+      </c>
+      <c r="AD16" t="n">
+        <v>3.301109630238939</v>
       </c>
     </row>
     <row r="17">
@@ -2148,7 +2198,10 @@
         </is>
       </c>
       <c r="AC17" t="n">
-        <v>5.342469816592597</v>
+        <v>-2.10569445756439</v>
+      </c>
+      <c r="AD17" t="n">
+        <v>0.8140843563207754</v>
       </c>
     </row>
     <row r="18">
@@ -2245,7 +2298,10 @@
         </is>
       </c>
       <c r="AC18" t="n">
-        <v>7.359717942280147</v>
+        <v>1.922065523488971</v>
+      </c>
+      <c r="AD18" t="n">
+        <v>6.542764420347981</v>
       </c>
     </row>
     <row r="19">
@@ -2342,7 +2398,10 @@
         </is>
       </c>
       <c r="AC19" t="n">
-        <v>6.055301553451765</v>
+        <v>0.01075442890893329</v>
+      </c>
+      <c r="AD19" t="n">
+        <v>3.770164359857599</v>
       </c>
     </row>
     <row r="20">
@@ -2439,7 +2498,10 @@
         </is>
       </c>
       <c r="AC20" t="n">
-        <v>7.987967390488346</v>
+        <v>1.981391084183679</v>
+      </c>
+      <c r="AD20" t="n">
+        <v>6.59122030790077</v>
       </c>
     </row>
     <row r="21">
@@ -2536,7 +2598,10 @@
         </is>
       </c>
       <c r="AC21" t="n">
-        <v>5.079104056506274</v>
+        <v>0.5558624193863311</v>
+      </c>
+      <c r="AD21" t="n">
+        <v>4.766209833898598</v>
       </c>
     </row>
     <row r="22">
@@ -2635,7 +2700,10 @@
         </is>
       </c>
       <c r="AC22" t="n">
-        <v>7.412335051052183</v>
+        <v>0.4807086874011383</v>
+      </c>
+      <c r="AD22" t="n">
+        <v>6.951546078849344</v>
       </c>
     </row>
     <row r="23">
@@ -2734,7 +2802,10 @@
         </is>
       </c>
       <c r="AC23" t="n">
-        <v>4.347897732132791</v>
+        <v>-0.5535403624998688</v>
+      </c>
+      <c r="AD23" t="n">
+        <v>4.106738346420874</v>
       </c>
     </row>
     <row r="24">
@@ -2833,7 +2904,10 @@
         </is>
       </c>
       <c r="AC24" t="n">
-        <v>6.782281312629124</v>
+        <v>-0.6993611033200786</v>
+      </c>
+      <c r="AD24" t="n">
+        <v>3.734481315019639</v>
       </c>
     </row>
     <row r="25">
@@ -2932,7 +3006,10 @@
         </is>
       </c>
       <c r="AC25" t="n">
-        <v>5.545209869220241</v>
+        <v>-0.2936598988178432</v>
+      </c>
+      <c r="AD25" t="n">
+        <v>4.804966128089863</v>
       </c>
     </row>
     <row r="26">
@@ -3031,7 +3108,10 @@
         </is>
       </c>
       <c r="AC26" t="n">
-        <v>7.289730408427765</v>
+        <v>-0.1876762277557319</v>
+      </c>
+      <c r="AD26" t="n">
+        <v>5.098704484475767</v>
       </c>
     </row>
     <row r="27">
@@ -3130,7 +3210,10 @@
         </is>
       </c>
       <c r="AC27" t="n">
-        <v>7.479253464493518</v>
+        <v>-0.09337556761078179</v>
+      </c>
+      <c r="AD27" t="n">
+        <v>5.362571864227939</v>
       </c>
     </row>
     <row r="28">
@@ -3229,7 +3312,10 @@
         </is>
       </c>
       <c r="AC28" t="n">
-        <v>3.311763958273665</v>
+        <v>0.3563522148365012</v>
+      </c>
+      <c r="AD28" t="n">
+        <v>3.675982013834711</v>
       </c>
     </row>
     <row r="29">
@@ -3328,7 +3414,10 @@
         </is>
       </c>
       <c r="AC29" t="n">
-        <v>3.836492269590202</v>
+        <v>0.393575372761396</v>
+      </c>
+      <c r="AD29" t="n">
+        <v>3.732144377464585</v>
       </c>
     </row>
     <row r="30">
@@ -3427,7 +3516,10 @@
         </is>
       </c>
       <c r="AC30" t="n">
-        <v>3.527907313980382</v>
+        <v>0.2773041544012314</v>
+      </c>
+      <c r="AD30" t="n">
+        <v>3.555532362113815</v>
       </c>
     </row>
     <row r="31">
@@ -3526,7 +3618,10 @@
         </is>
       </c>
       <c r="AC31" t="n">
-        <v>3.411138030674357</v>
+        <v>0.2180440097802296</v>
+      </c>
+      <c r="AD31" t="n">
+        <v>3.464350346256</v>
       </c>
     </row>
     <row r="32">
@@ -3625,7 +3720,10 @@
         </is>
       </c>
       <c r="AC32" t="n">
-        <v>3.825213272379562</v>
+        <v>0.350067999889136</v>
+      </c>
+      <c r="AD32" t="n">
+        <v>3.666462928851106</v>
       </c>
     </row>
     <row r="33">
@@ -3724,7 +3822,10 @@
         </is>
       </c>
       <c r="AC33" t="n">
-        <v>3.533287664551292</v>
+        <v>0.2992450511937354</v>
+      </c>
+      <c r="AD33" t="n">
+        <v>3.589112205858059</v>
       </c>
     </row>
     <row r="34">
@@ -3823,7 +3924,10 @@
         </is>
       </c>
       <c r="AC34" t="n">
-        <v>3.284029013211557</v>
+        <v>0.2761357341431679</v>
+      </c>
+      <c r="AD34" t="n">
+        <v>3.553741213688711</v>
       </c>
     </row>
     <row r="35">
@@ -3922,7 +4026,10 @@
         </is>
       </c>
       <c r="AC35" t="n">
-        <v>2.636750299733584</v>
+        <v>0.003353631598680729</v>
+      </c>
+      <c r="AD35" t="n">
+        <v>2.50419203556942</v>
       </c>
     </row>
     <row r="36">
@@ -4021,7 +4128,10 @@
         </is>
       </c>
       <c r="AC36" t="n">
-        <v>3.316272611280524</v>
+        <v>0.1868807894051916</v>
+      </c>
+      <c r="AD36" t="n">
+        <v>2.732923487686572</v>
       </c>
     </row>
     <row r="37">
@@ -4120,7 +4230,10 @@
         </is>
       </c>
       <c r="AC37" t="n">
-        <v>3.568645367616315</v>
+        <v>0.1467602754529171</v>
+      </c>
+      <c r="AD37" t="n">
+        <v>2.683121780342022</v>
       </c>
     </row>
     <row r="38">
@@ -4219,7 +4332,10 @@
         </is>
       </c>
       <c r="AC38" t="n">
-        <v>1.817401626623792</v>
+        <v>-0.4947642173165425</v>
+      </c>
+      <c r="AD38" t="n">
+        <v>1.893859418855209</v>
       </c>
     </row>
     <row r="39">
@@ -4318,7 +4434,10 @@
         </is>
       </c>
       <c r="AC39" t="n">
-        <v>5.001648861700169</v>
+        <v>-0.01575519776481952</v>
+      </c>
+      <c r="AD39" t="n">
+        <v>2.480306410164463</v>
       </c>
     </row>
     <row r="40">
@@ -4419,7 +4538,10 @@
         </is>
       </c>
       <c r="AC40" t="n">
-        <v>4.788613734363567</v>
+        <v>-0.7004636893665617</v>
+      </c>
+      <c r="AD40" t="n">
+        <v>3.317094299487862</v>
       </c>
     </row>
     <row r="41">
@@ -4516,7 +4638,10 @@
         </is>
       </c>
       <c r="AC41" t="n">
-        <v>5.106908984155707</v>
+        <v>-0.1187654423838049</v>
+      </c>
+      <c r="AD41" t="n">
+        <v>4.703434905364877</v>
       </c>
     </row>
     <row r="42">
@@ -4613,7 +4738,10 @@
         </is>
       </c>
       <c r="AC42" t="n">
-        <v>3.903893097618444</v>
+        <v>-0.4666130002557288</v>
+      </c>
+      <c r="AD42" t="n">
+        <v>3.854182136714689</v>
       </c>
     </row>
     <row r="43">
@@ -4710,7 +4838,10 @@
         </is>
       </c>
       <c r="AC43" t="n">
-        <v>3.626663323298775</v>
+        <v>-0.1370010030103673</v>
+      </c>
+      <c r="AD43" t="n">
+        <v>4.658032199198447</v>
       </c>
     </row>
     <row r="44">
@@ -4811,7 +4942,10 @@
         </is>
       </c>
       <c r="AC44" t="n">
-        <v>6.966891144661663</v>
+        <v>-3.240880993684173</v>
+      </c>
+      <c r="AD44" t="n">
+        <v>0.3765595206874657</v>
       </c>
     </row>
     <row r="45">
@@ -4908,7 +5042,10 @@
         </is>
       </c>
       <c r="AC45" t="n">
-        <v>4.739417599027191</v>
+        <v>-0.6353127708928049</v>
+      </c>
+      <c r="AD45" t="n">
+        <v>3.463068611170398</v>
       </c>
     </row>
     <row r="46">
@@ -5005,7 +5142,10 @@
         </is>
       </c>
       <c r="AC46" t="n">
-        <v>4.273076236464505</v>
+        <v>-0.2965814635971371</v>
+      </c>
+      <c r="AD46" t="n">
+        <v>4.263933847357309</v>
       </c>
     </row>
     <row r="47">
@@ -5102,7 +5242,10 @@
         </is>
       </c>
       <c r="AC47" t="n">
-        <v>5.708715265211424</v>
+        <v>-0.8677372789904794</v>
+      </c>
+      <c r="AD47" t="n">
+        <v>2.957253452025189</v>
       </c>
     </row>
     <row r="48">
@@ -5199,7 +5342,10 @@
         </is>
       </c>
       <c r="AC48" t="n">
-        <v>3.759014213855417</v>
+        <v>0.1685585387103963</v>
+      </c>
+      <c r="AD48" t="n">
+        <v>6.097951628965663</v>
       </c>
     </row>
     <row r="49">
@@ -5300,7 +5446,10 @@
         </is>
       </c>
       <c r="AC49" t="n">
-        <v>3.643205169327538</v>
+        <v>0.1318890214995732</v>
+      </c>
+      <c r="AD49" t="n">
+        <v>5.995401110114424</v>
       </c>
     </row>
     <row r="50">
@@ -5397,7 +5546,10 @@
         </is>
       </c>
       <c r="AC50" t="n">
-        <v>4.367977433131697</v>
+        <v>0.2859468939990081</v>
+      </c>
+      <c r="AD50" t="n">
+        <v>6.42379024348825</v>
       </c>
     </row>
     <row r="51">
@@ -5494,7 +5646,10 @@
         </is>
       </c>
       <c r="AC51" t="n">
-        <v>1.560808688369159</v>
+        <v>4.216208669757011</v>
+      </c>
+      <c r="AD51" t="n">
+        <v>0.6159125322807046</v>
       </c>
     </row>
     <row r="52">
@@ -5595,7 +5750,10 @@
         </is>
       </c>
       <c r="AC52" t="n">
-        <v>3.875828127940919</v>
+        <v>-2.829483554251136</v>
+      </c>
+      <c r="AD52" t="n">
+        <v>0.03484473695081625</v>
       </c>
     </row>
     <row r="53">
@@ -5692,7 +5850,10 @@
         </is>
       </c>
       <c r="AC53" t="n">
-        <v>1.891854791576428</v>
+        <v>1.48973653216046</v>
+      </c>
+      <c r="AD53" t="n">
+        <v>0.5100242026293054</v>
       </c>
     </row>
     <row r="54">
@@ -5789,7 +5950,10 @@
         </is>
       </c>
       <c r="AC54" t="n">
-        <v>2.545649912643785</v>
+        <v>0.5532883971057532</v>
+      </c>
+      <c r="AD54" t="n">
+        <v>0.3968113670073156</v>
       </c>
     </row>
     <row r="55">
@@ -5886,7 +6050,10 @@
         </is>
       </c>
       <c r="AC55" t="n">
-        <v>2.46955423690292</v>
+        <v>2.740042935969835</v>
+      </c>
+      <c r="AD55" t="n">
+        <v>0.587092839322124</v>
       </c>
     </row>
     <row r="56">
@@ -5987,7 +6154,10 @@
         </is>
       </c>
       <c r="AC56" t="n">
-        <v>1.862730836864006</v>
+        <v>3.450923347456024</v>
+      </c>
+      <c r="AD56" t="n">
+        <v>0.605786665568531</v>
       </c>
     </row>
     <row r="57">
@@ -6084,7 +6254,10 @@
         </is>
       </c>
       <c r="AC57" t="n">
-        <v>3.325349049484263</v>
+        <v>3.35772741901319</v>
+      </c>
+      <c r="AD57" t="n">
+        <v>0.603973106682649</v>
       </c>
     </row>
     <row r="58">
@@ -6181,7 +6354,10 @@
         </is>
       </c>
       <c r="AC58" t="n">
-        <v>3.497918963086481</v>
+        <v>-12.03529263329881</v>
+      </c>
+      <c r="AD58" t="n">
+        <v>1.482778410766954e-05</v>
       </c>
     </row>
     <row r="59">
@@ -6278,7 +6454,10 @@
         </is>
       </c>
       <c r="AC59" t="n">
-        <v>7.055469072100474</v>
+        <v>5.860088569687279</v>
+      </c>
+      <c r="AD59" t="n">
+        <v>2.492892784707718</v>
       </c>
     </row>
     <row r="60">
@@ -6375,7 +6554,10 @@
         </is>
       </c>
       <c r="AC60" t="n">
-        <v>5.96089427773228</v>
+        <v>4.330378766032177</v>
+      </c>
+      <c r="AD60" t="n">
+        <v>2.467521102927468</v>
       </c>
     </row>
     <row r="61">
@@ -6472,7 +6654,10 @@
         </is>
       </c>
       <c r="AC61" t="n">
-        <v>4.182422844811743</v>
+        <v>1.559571823438586</v>
+      </c>
+      <c r="AD61" t="n">
+        <v>2.065729759616301</v>
       </c>
     </row>
     <row r="62">
@@ -6569,7 +6754,10 @@
         </is>
       </c>
       <c r="AC62" t="n">
-        <v>7.768329584350407</v>
+        <v>4.657627954355352</v>
+      </c>
+      <c r="AD62" t="n">
+        <v>2.47650062441819</v>
       </c>
     </row>
     <row r="63">
@@ -6666,7 +6854,10 @@
         </is>
       </c>
       <c r="AC63" t="n">
-        <v>6.757638450292591</v>
+        <v>4.670572094298608</v>
+      </c>
+      <c r="AD63" t="n">
+        <v>2.47680003883436</v>
       </c>
     </row>
     <row r="64">
@@ -6763,7 +6954,10 @@
         </is>
       </c>
       <c r="AC64" t="n">
-        <v>7.964677431751159</v>
+        <v>5.230309175940881</v>
+      </c>
+      <c r="AD64" t="n">
+        <v>2.486691549160609</v>
       </c>
     </row>
     <row r="65">
@@ -6860,7 +7054,10 @@
         </is>
       </c>
       <c r="AC65" t="n">
-        <v>3.104067484422635</v>
+        <v>-4.910254458269682</v>
+      </c>
+      <c r="AD65" t="n">
+        <v>0.01829171033819345</v>
       </c>
     </row>
     <row r="66">
@@ -6957,7 +7154,10 @@
         </is>
       </c>
       <c r="AC66" t="n">
-        <v>8.906293399166238</v>
+        <v>1.198876787626133</v>
+      </c>
+      <c r="AD66" t="n">
+        <v>7.683249099991364</v>
       </c>
     </row>
     <row r="67">
@@ -7054,7 +7254,10 @@
         </is>
       </c>
       <c r="AC67" t="n">
-        <v>8.029512236076521</v>
+        <v>0.9098698345076599</v>
+      </c>
+      <c r="AD67" t="n">
+        <v>7.129735261279732</v>
       </c>
     </row>
     <row r="68">
@@ -7151,7 +7354,10 @@
         </is>
       </c>
       <c r="AC68" t="n">
-        <v>7.793606330812419</v>
+        <v>0.810501978378881</v>
+      </c>
+      <c r="AD68" t="n">
+        <v>6.922164625347704</v>
       </c>
     </row>
     <row r="69">
@@ -7248,7 +7454,10 @@
         </is>
       </c>
       <c r="AC69" t="n">
-        <v>6.046735156572481</v>
+        <v>0.3617958348450351</v>
+      </c>
+      <c r="AD69" t="n">
+        <v>5.894750854156883</v>
       </c>
     </row>
     <row r="70">
@@ -7349,7 +7558,10 @@
         </is>
       </c>
       <c r="AC70" t="n">
-        <v>3.813121376566612</v>
+        <v>0.8339312577300401</v>
+      </c>
+      <c r="AD70" t="n">
+        <v>3.485927656846326</v>
       </c>
     </row>
     <row r="71">
@@ -7446,7 +7658,10 @@
         </is>
       </c>
       <c r="AC71" t="n">
-        <v>10.76674420964842</v>
+        <v>1.117348389774426</v>
+      </c>
+      <c r="AD71" t="n">
+        <v>9.418706734951048</v>
       </c>
     </row>
     <row r="72">
@@ -7543,7 +7758,10 @@
         </is>
       </c>
       <c r="AC72" t="n">
-        <v>8.173043291920315</v>
+        <v>0.3642442457835948</v>
+      </c>
+      <c r="AD72" t="n">
+        <v>7.375843207706938</v>
       </c>
     </row>
     <row r="73">
@@ -7644,7 +7862,10 @@
         </is>
       </c>
       <c r="AC73" t="n">
-        <v>3.637581171160076</v>
+        <v>0.2225487026960456</v>
+      </c>
+      <c r="AD73" t="n">
+        <v>3.471304215649196</v>
       </c>
     </row>
     <row r="74">
@@ -7741,7 +7962,10 @@
         </is>
       </c>
       <c r="AC74" t="n">
-        <v>11.43276936749086</v>
+        <v>0.8129208377590106</v>
+      </c>
+      <c r="AD74" t="n">
+        <v>8.659144595353769</v>
       </c>
     </row>
     <row r="75">
@@ -7838,7 +8062,10 @@
         </is>
       </c>
       <c r="AC75" t="n">
-        <v>8.381435207786783</v>
+        <v>0.5544305623360352</v>
+      </c>
+      <c r="AD75" t="n">
+        <v>7.939536289105735</v>
       </c>
     </row>
     <row r="76">
@@ -7935,7 +8162,10 @@
         </is>
       </c>
       <c r="AC76" t="n">
-        <v>7.176570261842783</v>
+        <v>0.3484144266343117</v>
+      </c>
+      <c r="AD76" t="n">
+        <v>7.327912859669353</v>
       </c>
     </row>
     <row r="77">
@@ -8032,7 +8262,10 @@
         </is>
       </c>
       <c r="AC77" t="n">
-        <v>9.122442744685472</v>
+        <v>0.6731758137468595</v>
+      </c>
+      <c r="AD77" t="n">
+        <v>8.27767389857036</v>
       </c>
     </row>
     <row r="78">
@@ -8131,7 +8364,10 @@
         </is>
       </c>
       <c r="AC78" t="n">
-        <v>7.807369754750587</v>
+        <v>0.2927610289309844</v>
+      </c>
+      <c r="AD78" t="n">
+        <v>10.02175901577276</v>
       </c>
     </row>
     <row r="79">
@@ -8230,7 +8466,10 @@
         </is>
       </c>
       <c r="AC79" t="n">
-        <v>7.428441652758613</v>
+        <v>-0.1311840955917405</v>
+      </c>
+      <c r="AD79" t="n">
+        <v>8.176891244607772</v>
       </c>
     </row>
     <row r="80">
@@ -8329,7 +8568,10 @@
         </is>
       </c>
       <c r="AC80" t="n">
-        <v>6.97340575228066</v>
+        <v>-0.1821571252361549</v>
+      </c>
+      <c r="AD80" t="n">
+        <v>7.955258902585734</v>
       </c>
     </row>
     <row r="81">
@@ -8428,7 +8670,10 @@
         </is>
       </c>
       <c r="AC81" t="n">
-        <v>4.939332770947563</v>
+        <v>-0.3242676136015173</v>
+      </c>
+      <c r="AD81" t="n">
+        <v>7.343630896967114</v>
       </c>
     </row>
     <row r="82">
@@ -8527,7 +8772,10 @@
         </is>
       </c>
       <c r="AC82" t="n">
-        <v>9.803440707072578</v>
+        <v>-0.03986585972426113</v>
+      </c>
+      <c r="AD82" t="n">
+        <v>8.575609959409986</v>
       </c>
     </row>
     <row r="83">
@@ -8626,7 +8874,10 @@
         </is>
       </c>
       <c r="AC83" t="n">
-        <v>1.023248807950946</v>
+        <v>-1.897697467818602</v>
+      </c>
+      <c r="AD83" t="n">
+        <v>2.281462707593858</v>
       </c>
     </row>
     <row r="84">
@@ -8725,7 +8976,10 @@
         </is>
       </c>
       <c r="AC84" t="n">
-        <v>6.407256571793</v>
+        <v>-0.8361453704046218</v>
+      </c>
+      <c r="AD84" t="n">
+        <v>5.291076596200213</v>
       </c>
     </row>
     <row r="85">
@@ -8824,7 +9078,10 @@
         </is>
       </c>
       <c r="AC85" t="n">
-        <v>7.944784207282601</v>
+        <v>-0.6857805344317106</v>
+      </c>
+      <c r="AD85" t="n">
+        <v>5.862016488338512</v>
       </c>
     </row>
     <row r="86">
@@ -8923,7 +9180,10 @@
         </is>
       </c>
       <c r="AC86" t="n">
-        <v>7.510186867687164</v>
+        <v>0.3142071054226014</v>
+      </c>
+      <c r="AD86" t="n">
+        <v>10.11345709970532</v>
       </c>
     </row>
     <row r="87">
@@ -9022,7 +9282,10 @@
         </is>
       </c>
       <c r="AC87" t="n">
-        <v>3.691903448897098</v>
+        <v>-0.5378657229781926</v>
+      </c>
+      <c r="AD87" t="n">
+        <v>6.451973657834287</v>
       </c>
     </row>
     <row r="88">
@@ -9121,7 +9384,10 @@
         </is>
       </c>
       <c r="AC88" t="n">
-        <v>6.044670723941417</v>
+        <v>0.1711156034137412</v>
+      </c>
+      <c r="AD88" t="n">
+        <v>9.496809404431019</v>
       </c>
     </row>
     <row r="89">
@@ -9220,7 +9486,10 @@
         </is>
       </c>
       <c r="AC89" t="n">
-        <v>5.47131217231551</v>
+        <v>-0.002667058036810479</v>
+      </c>
+      <c r="AD89" t="n">
+        <v>8.738331628005573</v>
       </c>
     </row>
     <row r="90">
@@ -9319,7 +9588,10 @@
         </is>
       </c>
       <c r="AC90" t="n">
-        <v>5.973252247230842</v>
+        <v>0.1380807584340789</v>
+      </c>
+      <c r="AD90" t="n">
+        <v>9.353145310291467</v>
       </c>
     </row>
     <row r="91">
@@ -9418,7 +9690,10 @@
         </is>
       </c>
       <c r="AC91" t="n">
-        <v>6.338237559360721</v>
+        <v>0.3783016672490899</v>
+      </c>
+      <c r="AD91" t="n">
+        <v>10.38560985890997</v>
       </c>
     </row>
     <row r="92">
@@ -9517,7 +9792,10 @@
         </is>
       </c>
       <c r="AC92" t="n">
-        <v>6.638395862765242</v>
+        <v>0.256856404065222</v>
+      </c>
+      <c r="AD92" t="n">
+        <v>9.867608972873876</v>
       </c>
     </row>
     <row r="93">
@@ -9616,7 +9894,10 @@
         </is>
       </c>
       <c r="AC93" t="n">
-        <v>7.22117449385551</v>
+        <v>0.675591380236109</v>
+      </c>
+      <c r="AD93" t="n">
+        <v>1.656885074880077</v>
       </c>
     </row>
     <row r="94">
@@ -9715,7 +9996,10 @@
         </is>
       </c>
       <c r="AC94" t="n">
-        <v>2.611715954094088</v>
+        <v>0.9411132738256699</v>
+      </c>
+      <c r="AD94" t="n">
+        <v>1.798311196700733</v>
       </c>
     </row>
     <row r="95">
@@ -9814,7 +10098,10 @@
         </is>
       </c>
       <c r="AC95" t="n">
-        <v>2.17279433130474</v>
+        <v>0.9973264621875639</v>
+      </c>
+      <c r="AD95" t="n">
+        <v>1.826331511470441</v>
       </c>
     </row>
     <row r="96">
@@ -9913,7 +10200,10 @@
         </is>
       </c>
       <c r="AC96" t="n">
-        <v>6.220815622552448</v>
+        <v>-0.6381730401126611</v>
+      </c>
+      <c r="AD96" t="n">
+        <v>0.8641491071344722</v>
       </c>
     </row>
     <row r="97">
@@ -10012,7 +10302,10 @@
         </is>
       </c>
       <c r="AC97" t="n">
-        <v>3.608436384012615</v>
+        <v>1.166284412326291</v>
+      </c>
+      <c r="AD97" t="n">
+        <v>1.906181873154184</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
DATA. Actualizo predicciones en proximos partidos
</commit_message>
<xml_diff>
--- a/data/predicciones.xlsx
+++ b/data/predicciones.xlsx
@@ -510,57 +510,57 @@
       </c>
       <c r="P1" s="1" t="inlineStr">
         <is>
+          <t>result_to_bet</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>prob_result_to_bet</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>odd_to_bet</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>strategy</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>stake_to_bet_norm</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>stake_to_bet</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
           <t>emergency_fill</t>
-        </is>
-      </c>
-      <c r="Q1" s="1" t="inlineStr">
-        <is>
-          <t>result_to_bet</t>
-        </is>
-      </c>
-      <c r="R1" s="1" t="inlineStr">
-        <is>
-          <t>prob_result_to_bet</t>
-        </is>
-      </c>
-      <c r="S1" s="1" t="inlineStr">
-        <is>
-          <t>odd_to_bet</t>
-        </is>
-      </c>
-      <c r="T1" s="1" t="inlineStr">
-        <is>
-          <t>strategy</t>
-        </is>
-      </c>
-      <c r="U1" s="1" t="inlineStr">
-        <is>
-          <t>stake_to_bet_norm</t>
-        </is>
-      </c>
-      <c r="V1" s="1" t="inlineStr">
-        <is>
-          <t>stake_to_bet</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>SU438zoI</t>
+          <t>v9YLQH0n</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>45690.45833333334</v>
+        <v>45689.39583333334</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>manchester utd</t>
+          <t>nottingham</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>crystal palace</t>
+          <t>brighton</t>
         </is>
       </c>
       <c r="E2" t="n">
@@ -570,69 +570,71 @@
         <v>481</v>
       </c>
       <c r="G2" t="n">
-        <v>2.1</v>
+        <v>2.4</v>
       </c>
       <c r="H2" t="n">
-        <v>3.4</v>
+        <v>3.5</v>
       </c>
       <c r="I2" t="n">
-        <v>3.5</v>
+        <v>2.8</v>
       </c>
       <c r="J2" t="n">
         <v>1</v>
       </c>
       <c r="K2" t="n">
-        <v>0.3855688483309294</v>
+        <v>0.4007298004809222</v>
       </c>
       <c r="L2" t="n">
-        <v>0.5219890033464289</v>
+        <v>0.4797272200188482</v>
       </c>
       <c r="M2" t="n">
-        <v>0.0924421483226416</v>
+        <v>0.1195429795002296</v>
       </c>
       <c r="N2" t="n">
         <v>1</v>
       </c>
-      <c r="O2" t="inlineStr"/>
-      <c r="P2" t="inlineStr"/>
+      <c r="O2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P2" t="n">
+        <v>1</v>
+      </c>
       <c r="Q2" t="n">
-        <v>1</v>
+        <v>0.4797272200188482</v>
       </c>
       <c r="R2" t="n">
-        <v>0.5219890033464289</v>
-      </c>
-      <c r="S2" t="n">
-        <v>2.1</v>
-      </c>
-      <c r="T2" t="inlineStr">
-        <is>
-          <t>dif_prob_mod_bm &gt; 0</t>
-        </is>
+        <v>2.4</v>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>dif_prob_mod_bm &gt; 0</t>
+        </is>
+      </c>
+      <c r="T2" t="n">
+        <v>1.081038057465969</v>
       </c>
       <c r="U2" t="n">
-        <v>0.8743355184318256</v>
-      </c>
-      <c r="V2" t="n">
-        <v>2.116941083094706</v>
-      </c>
+        <v>2.240071127419242</v>
+      </c>
+      <c r="V2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>4jKwEvHt</t>
+          <t>Q58nCIog</t>
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>45691.70833333334</v>
+        <v>45689.5</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>chelsea</t>
+          <t>everton</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>west ham</t>
+          <t>leicester</t>
         </is>
       </c>
       <c r="E3" t="n">
@@ -642,69 +644,71 @@
         <v>481</v>
       </c>
       <c r="G3" t="n">
-        <v>1.36</v>
+        <v>1.8</v>
       </c>
       <c r="H3" t="n">
-        <v>4.75</v>
+        <v>3.7</v>
       </c>
       <c r="I3" t="n">
-        <v>7.5</v>
+        <v>4.5</v>
       </c>
       <c r="J3" t="n">
         <v>1</v>
       </c>
       <c r="K3" t="n">
-        <v>0.1781810059241761</v>
+        <v>0.382768911166384</v>
       </c>
       <c r="L3" t="n">
-        <v>0.6030643920239229</v>
+        <v>0.4343438231667807</v>
       </c>
       <c r="M3" t="n">
-        <v>0.2187546020519011</v>
+        <v>0.1828872656668354</v>
       </c>
       <c r="N3" t="n">
         <v>1</v>
       </c>
-      <c r="O3" t="inlineStr"/>
-      <c r="P3" t="inlineStr"/>
+      <c r="O3" t="n">
+        <v>0</v>
+      </c>
+      <c r="P3" t="n">
+        <v>1</v>
+      </c>
       <c r="Q3" t="n">
-        <v>1</v>
+        <v>0.4343438231667807</v>
       </c>
       <c r="R3" t="n">
-        <v>0.6030643920239229</v>
-      </c>
-      <c r="S3" t="n">
-        <v>1.36</v>
-      </c>
-      <c r="T3" t="inlineStr">
-        <is>
-          <t>dif_prob_mod_bm &gt; 0</t>
-        </is>
+        <v>1.8</v>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>dif_prob_mod_bm &gt; 0</t>
+        </is>
+      </c>
+      <c r="T3" t="n">
+        <v>-2.727263978747435</v>
       </c>
       <c r="U3" t="n">
-        <v>-4.995345190207353</v>
-      </c>
-      <c r="V3" t="n">
-        <v>0.02017160258845055</v>
-      </c>
+        <v>0.1841508343609474</v>
+      </c>
+      <c r="V3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>v9YLQH0n</t>
+          <t>YVBfAdG5</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>45689.39583333334</v>
+        <v>45689.5</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>nottingham</t>
+          <t>ipswich</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>brighton</t>
+          <t>southampton</t>
         </is>
       </c>
       <c r="E4" t="n">
@@ -714,69 +718,71 @@
         <v>481</v>
       </c>
       <c r="G4" t="n">
-        <v>2.4</v>
+        <v>1.95</v>
       </c>
       <c r="H4" t="n">
-        <v>3.5</v>
+        <v>3.6</v>
       </c>
       <c r="I4" t="n">
-        <v>2.8</v>
+        <v>3.9</v>
       </c>
       <c r="J4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K4" t="n">
-        <v>0.6870106834703122</v>
+        <v>0.3162648442246361</v>
       </c>
       <c r="L4" t="n">
-        <v>0.2436294888743391</v>
+        <v>0.3574261690253308</v>
       </c>
       <c r="M4" t="n">
-        <v>0.0693598276553485</v>
+        <v>0.3263089867500332</v>
       </c>
       <c r="N4" t="n">
         <v>1</v>
       </c>
-      <c r="O4" t="inlineStr"/>
-      <c r="P4" t="inlineStr"/>
+      <c r="O4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P4" t="n">
+        <v>1</v>
+      </c>
       <c r="Q4" t="n">
-        <v>0</v>
+        <v>0.3574261690253308</v>
       </c>
       <c r="R4" t="n">
-        <v>0.6870106834703122</v>
-      </c>
-      <c r="S4" t="n">
-        <v>3.5</v>
-      </c>
-      <c r="T4" t="inlineStr">
-        <is>
-          <t>dif_prob_mod_bm &gt; 0</t>
-        </is>
+        <v>1.95</v>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>dif_prob_mod_bm &gt; 0</t>
+        </is>
+      </c>
+      <c r="T4" t="n">
+        <v>-3.189673372637948</v>
       </c>
       <c r="U4" t="n">
-        <v>1.248477681907638</v>
-      </c>
-      <c r="V4" t="n">
-        <v>10.48998909672907</v>
-      </c>
+        <v>0.1186685602398582</v>
+      </c>
+      <c r="V4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>z1BLcJWa</t>
+          <t>SU438zoI</t>
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>45689.5</v>
+        <v>45690.45833333334</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>bournemouth</t>
+          <t>manchester utd</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>liverpool</t>
+          <t>crystal palace</t>
         </is>
       </c>
       <c r="E5" t="n">
@@ -786,69 +792,71 @@
         <v>481</v>
       </c>
       <c r="G5" t="n">
-        <v>4.5</v>
+        <v>2.1</v>
       </c>
       <c r="H5" t="n">
-        <v>4.33</v>
+        <v>3.4</v>
       </c>
       <c r="I5" t="n">
-        <v>1.67</v>
+        <v>3.5</v>
       </c>
       <c r="J5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K5" t="n">
-        <v>0.6517210031182497</v>
+        <v>0.3054182768078471</v>
       </c>
       <c r="L5" t="n">
-        <v>0.03012596203921332</v>
+        <v>0.4310210291497264</v>
       </c>
       <c r="M5" t="n">
-        <v>0.318153034842537</v>
+        <v>0.2635606940424265</v>
       </c>
       <c r="N5" t="n">
         <v>1</v>
       </c>
-      <c r="O5" t="inlineStr"/>
-      <c r="P5" t="inlineStr"/>
+      <c r="O5" t="n">
+        <v>0</v>
+      </c>
+      <c r="P5" t="n">
+        <v>1</v>
+      </c>
       <c r="Q5" t="n">
-        <v>0</v>
+        <v>0.4310210291497264</v>
       </c>
       <c r="R5" t="n">
-        <v>0.6517210031182497</v>
-      </c>
-      <c r="S5" t="n">
-        <v>4.33</v>
-      </c>
-      <c r="T5" t="inlineStr">
-        <is>
-          <t>dif_prob_mod_bm &gt; 0</t>
-        </is>
+        <v>2.1</v>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>dif_prob_mod_bm &gt; 0</t>
+        </is>
+      </c>
+      <c r="T5" t="n">
+        <v>-0.8623258071415865</v>
       </c>
       <c r="U5" t="n">
-        <v>1.215850479480828</v>
-      </c>
-      <c r="V5" t="n">
-        <v>10.41298856937406</v>
-      </c>
+        <v>0.890560941121364</v>
+      </c>
+      <c r="V5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>Q58nCIog</t>
+          <t>8E9Tec1C</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>45689.5</v>
+        <v>45690.5625</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>everton</t>
+          <t>arsenal</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>leicester</t>
+          <t>manchester city</t>
         </is>
       </c>
       <c r="E6" t="n">
@@ -858,25 +866,25 @@
         <v>481</v>
       </c>
       <c r="G6" t="n">
-        <v>1.8</v>
+        <v>2.1</v>
       </c>
       <c r="H6" t="n">
-        <v>3.7</v>
+        <v>3.6</v>
       </c>
       <c r="I6" t="n">
-        <v>4.5</v>
+        <v>3.4</v>
       </c>
       <c r="J6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K6" t="n">
-        <v>0.7014517156229618</v>
+        <v>0.2436263154199827</v>
       </c>
       <c r="L6" t="n">
-        <v>0.2581059952927857</v>
+        <v>0.3920959031187042</v>
       </c>
       <c r="M6" t="n">
-        <v>0.04044228908425249</v>
+        <v>0.3642777814613132</v>
       </c>
       <c r="N6" t="n">
         <v>1</v>
@@ -888,30 +896,28 @@
         <v>1</v>
       </c>
       <c r="Q6" t="n">
-        <v>0</v>
+        <v>0.3920959031187042</v>
       </c>
       <c r="R6" t="n">
-        <v>0.7014517156229618</v>
-      </c>
-      <c r="S6" t="n">
-        <v>3.7</v>
-      </c>
-      <c r="T6" t="inlineStr">
-        <is>
-          <t>dif_prob_mod_bm &gt; 0</t>
-        </is>
+        <v>2.1</v>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>dif_prob_mod_bm &gt; 0</t>
+        </is>
+      </c>
+      <c r="T6" t="n">
+        <v>-1.60544184955201</v>
       </c>
       <c r="U6" t="n">
-        <v>1.313062837699555</v>
-      </c>
-      <c r="V6" t="n">
-        <v>10.63834057961615</v>
-      </c>
+        <v>0.5016672447872559</v>
+      </c>
+      <c r="V6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>YVBfAdG5</t>
+          <t>z1BLcJWa</t>
         </is>
       </c>
       <c r="B7" s="2" t="n">
@@ -919,12 +925,12 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>ipswich</t>
+          <t>bournemouth</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>southampton</t>
+          <t>liverpool</t>
         </is>
       </c>
       <c r="E7" t="n">
@@ -934,25 +940,25 @@
         <v>481</v>
       </c>
       <c r="G7" t="n">
-        <v>1.95</v>
+        <v>4.5</v>
       </c>
       <c r="H7" t="n">
-        <v>3.6</v>
+        <v>4.33</v>
       </c>
       <c r="I7" t="n">
-        <v>3.9</v>
+        <v>1.67</v>
       </c>
       <c r="J7" t="n">
         <v>0</v>
       </c>
       <c r="K7" t="n">
-        <v>0.4515434829071772</v>
+        <v>0.4666425754327391</v>
       </c>
       <c r="L7" t="n">
-        <v>0.3704483985587467</v>
+        <v>0.1583077177151531</v>
       </c>
       <c r="M7" t="n">
-        <v>0.1780081185340762</v>
+        <v>0.3750497068521079</v>
       </c>
       <c r="N7" t="n">
         <v>1</v>
@@ -961,28 +967,26 @@
         <v>0</v>
       </c>
       <c r="P7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q7" t="n">
-        <v>0</v>
+        <v>0.4666425754327391</v>
       </c>
       <c r="R7" t="n">
-        <v>0.4515434829071772</v>
-      </c>
-      <c r="S7" t="n">
-        <v>3.6</v>
-      </c>
-      <c r="T7" t="inlineStr">
-        <is>
-          <t>dif_prob_mod_bm &gt; 0</t>
-        </is>
+        <v>4.33</v>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>dif_prob_mod_bm &gt; 0</t>
+        </is>
+      </c>
+      <c r="T7" t="n">
+        <v>0.6810559570395464</v>
       </c>
       <c r="U7" t="n">
-        <v>0.5346637080904597</v>
-      </c>
-      <c r="V7" t="n">
-        <v>8.512697557058972</v>
-      </c>
+        <v>8.963653526696433</v>
+      </c>
+      <c r="V7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
@@ -1022,57 +1026,59 @@
         <v>0</v>
       </c>
       <c r="K8" t="n">
-        <v>0.6279858131214231</v>
+        <v>0.5015742967920402</v>
       </c>
       <c r="L8" t="n">
-        <v>0.2988826978812361</v>
+        <v>0.3728496360988793</v>
       </c>
       <c r="M8" t="n">
-        <v>0.07313148899734068</v>
+        <v>0.1255760671090804</v>
       </c>
       <c r="N8" t="n">
         <v>1</v>
       </c>
-      <c r="O8" t="inlineStr"/>
-      <c r="P8" t="inlineStr"/>
+      <c r="O8" t="n">
+        <v>0</v>
+      </c>
+      <c r="P8" t="n">
+        <v>0</v>
+      </c>
       <c r="Q8" t="n">
-        <v>0</v>
+        <v>0.5015742967920402</v>
       </c>
       <c r="R8" t="n">
-        <v>0.6279858131214231</v>
-      </c>
-      <c r="S8" t="n">
         <v>4</v>
       </c>
-      <c r="T8" t="inlineStr">
-        <is>
-          <t>dif_prob_mod_bm &gt; 0</t>
-        </is>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>dif_prob_mod_bm &gt; 0</t>
+        </is>
+      </c>
+      <c r="T8" t="n">
+        <v>0.7454053238282674</v>
       </c>
       <c r="U8" t="n">
-        <v>1.119957964804217</v>
-      </c>
-      <c r="V8" t="n">
-        <v>10.17874241012483</v>
-      </c>
+        <v>9.155385707905669</v>
+      </c>
+      <c r="V8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
         <is>
-          <t>8E9Tec1C</t>
+          <t>4jKwEvHt</t>
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>45690.5625</v>
+        <v>45691.70833333334</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>arsenal</t>
+          <t>chelsea</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>manchester city</t>
+          <t>west ham</t>
         </is>
       </c>
       <c r="E9" t="n">
@@ -1082,51 +1088,53 @@
         <v>481</v>
       </c>
       <c r="G9" t="n">
-        <v>2.1</v>
+        <v>1.36</v>
       </c>
       <c r="H9" t="n">
-        <v>3.6</v>
+        <v>4.75</v>
       </c>
       <c r="I9" t="n">
-        <v>3.4</v>
+        <v>7.5</v>
       </c>
       <c r="J9" t="n">
         <v>0</v>
       </c>
       <c r="K9" t="n">
-        <v>0.4069721805251957</v>
+        <v>0.5600320277661145</v>
       </c>
       <c r="L9" t="n">
-        <v>0.3203857990483977</v>
+        <v>0.3565634023979357</v>
       </c>
       <c r="M9" t="n">
-        <v>0.2726420204264066</v>
+        <v>0.08340456983595002</v>
       </c>
       <c r="N9" t="n">
         <v>1</v>
       </c>
-      <c r="O9" t="inlineStr"/>
-      <c r="P9" t="inlineStr"/>
+      <c r="O9" t="n">
+        <v>0</v>
+      </c>
+      <c r="P9" t="n">
+        <v>0</v>
+      </c>
       <c r="Q9" t="n">
-        <v>0</v>
+        <v>0.5600320277661145</v>
       </c>
       <c r="R9" t="n">
-        <v>0.4069721805251957</v>
-      </c>
-      <c r="S9" t="n">
-        <v>3.6</v>
-      </c>
-      <c r="T9" t="inlineStr">
-        <is>
-          <t>dif_prob_mod_bm &gt; 0</t>
-        </is>
+        <v>4.75</v>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>dif_prob_mod_bm &gt; 0</t>
+        </is>
+      </c>
+      <c r="T9" t="n">
+        <v>0.9837938559342481</v>
       </c>
       <c r="U9" t="n">
-        <v>0.3975212392228247</v>
-      </c>
-      <c r="V9" t="n">
-        <v>8.074241538084367</v>
-      </c>
+        <v>9.82611474297225</v>
+      </c>
+      <c r="V9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
@@ -1166,39 +1174,41 @@
         <v>2</v>
       </c>
       <c r="K10" t="n">
-        <v>0.1377749428442042</v>
+        <v>0.1073010420078463</v>
       </c>
       <c r="L10" t="n">
-        <v>0.09156788799933628</v>
+        <v>0.1400103827836477</v>
       </c>
       <c r="M10" t="n">
-        <v>0.7706571691564597</v>
+        <v>0.7526885752085061</v>
       </c>
       <c r="N10" t="n">
         <v>1</v>
       </c>
-      <c r="O10" t="inlineStr"/>
-      <c r="P10" t="inlineStr"/>
+      <c r="O10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P10" t="n">
+        <v>2</v>
+      </c>
       <c r="Q10" t="n">
-        <v>2</v>
+        <v>0.7526885752085061</v>
       </c>
       <c r="R10" t="n">
-        <v>0.7706571691564597</v>
-      </c>
-      <c r="S10" t="n">
         <v>2.1</v>
       </c>
-      <c r="T10" t="inlineStr">
-        <is>
-          <t>dif_prob_mod_bm &gt; 0</t>
-        </is>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>dif_prob_mod_bm &gt; 0</t>
+        </is>
+      </c>
+      <c r="T10" t="n">
+        <v>1.173022238258309</v>
       </c>
       <c r="U10" t="n">
-        <v>1.249252636825384</v>
-      </c>
-      <c r="V10" t="n">
-        <v>10.49180123997604</v>
-      </c>
+        <v>10.30982667718166</v>
+      </c>
+      <c r="V10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
@@ -1238,39 +1248,41 @@
         <v>2</v>
       </c>
       <c r="K11" t="n">
-        <v>0.2950206827866058</v>
+        <v>0.3516142955747229</v>
       </c>
       <c r="L11" t="n">
-        <v>0.308258499992397</v>
+        <v>0.1950248443985114</v>
       </c>
       <c r="M11" t="n">
-        <v>0.3967208172209972</v>
+        <v>0.4533608600267658</v>
       </c>
       <c r="N11" t="n">
         <v>1</v>
       </c>
-      <c r="O11" t="inlineStr"/>
-      <c r="P11" t="inlineStr"/>
+      <c r="O11" t="n">
+        <v>0</v>
+      </c>
+      <c r="P11" t="n">
+        <v>2</v>
+      </c>
       <c r="Q11" t="n">
-        <v>2</v>
+        <v>0.4533608600267658</v>
       </c>
       <c r="R11" t="n">
-        <v>0.3967208172209972</v>
-      </c>
-      <c r="S11" t="n">
         <v>3.2</v>
       </c>
-      <c r="T11" t="inlineStr">
-        <is>
-          <t>dif_prob_mod_bm &gt; 0</t>
-        </is>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>dif_prob_mod_bm &gt; 0</t>
+        </is>
+      </c>
+      <c r="T11" t="n">
+        <v>0.4553078303895461</v>
       </c>
       <c r="U11" t="n">
-        <v>0.2722289041486777</v>
-      </c>
-      <c r="V11" t="n">
-        <v>7.663140211153616</v>
-      </c>
+        <v>8.260656406451861</v>
+      </c>
+      <c r="V11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
@@ -1324,27 +1336,27 @@
       <c r="O12" t="n">
         <v>0</v>
       </c>
-      <c r="P12" t="inlineStr"/>
+      <c r="P12" t="n">
+        <v>1</v>
+      </c>
       <c r="Q12" t="n">
-        <v>1</v>
+        <v>0.7043898552446455</v>
       </c>
       <c r="R12" t="n">
-        <v>0.7043898552446455</v>
-      </c>
-      <c r="S12" t="n">
         <v>1.33</v>
       </c>
-      <c r="T12" t="inlineStr">
-        <is>
-          <t>dif_prob_mod_bm &gt; 0</t>
-        </is>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>dif_prob_mod_bm &gt; 0</t>
+        </is>
+      </c>
+      <c r="T12" t="n">
+        <v>-0.2734263745654609</v>
       </c>
       <c r="U12" t="n">
-        <v>-0.2734263745654609</v>
-      </c>
-      <c r="V12" t="n">
         <v>9.073388503722112</v>
       </c>
+      <c r="V12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
@@ -1398,27 +1410,27 @@
       <c r="O13" t="n">
         <v>0</v>
       </c>
-      <c r="P13" t="inlineStr"/>
+      <c r="P13" t="n">
+        <v>1</v>
+      </c>
       <c r="Q13" t="n">
-        <v>1</v>
+        <v>0.6806535796964873</v>
       </c>
       <c r="R13" t="n">
-        <v>0.6806535796964873</v>
-      </c>
-      <c r="S13" t="n">
         <v>1.4</v>
       </c>
-      <c r="T13" t="inlineStr">
-        <is>
-          <t>dif_prob_mod_bm &gt; 0</t>
-        </is>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>dif_prob_mod_bm &gt; 0</t>
+        </is>
+      </c>
+      <c r="T13" t="n">
+        <v>-0.1681606729461351</v>
       </c>
       <c r="U13" t="n">
-        <v>-0.1681606729461351</v>
-      </c>
-      <c r="V13" t="n">
         <v>9.619231022462712</v>
       </c>
+      <c r="V13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="1" t="inlineStr">
@@ -1472,27 +1484,27 @@
       <c r="O14" t="n">
         <v>0</v>
       </c>
-      <c r="P14" t="inlineStr"/>
+      <c r="P14" t="n">
+        <v>0</v>
+      </c>
       <c r="Q14" t="n">
-        <v>0</v>
+        <v>0.3846574048803889</v>
       </c>
       <c r="R14" t="n">
-        <v>0.3846574048803889</v>
-      </c>
-      <c r="S14" t="n">
         <v>3.4</v>
       </c>
-      <c r="T14" t="inlineStr">
-        <is>
-          <t>dif_prob_mod_bm &gt; 0</t>
-        </is>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>dif_prob_mod_bm &gt; 0</t>
+        </is>
+      </c>
+      <c r="T14" t="n">
+        <v>0.2850325709197428</v>
       </c>
       <c r="U14" t="n">
-        <v>0.2850325709197428</v>
-      </c>
-      <c r="V14" t="n">
         <v>7.705524484853624</v>
       </c>
+      <c r="V14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="1" t="inlineStr">
@@ -1546,27 +1558,27 @@
       <c r="O15" t="n">
         <v>0</v>
       </c>
-      <c r="P15" t="inlineStr"/>
+      <c r="P15" t="n">
+        <v>0</v>
+      </c>
       <c r="Q15" t="n">
-        <v>0</v>
+        <v>0.3763125641141917</v>
       </c>
       <c r="R15" t="n">
-        <v>0.3763125641141917</v>
-      </c>
-      <c r="S15" t="n">
         <v>3.4</v>
       </c>
-      <c r="T15" t="inlineStr">
-        <is>
-          <t>dif_prob_mod_bm &gt; 0</t>
-        </is>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t>dif_prob_mod_bm &gt; 0</t>
+        </is>
+      </c>
+      <c r="T15" t="n">
+        <v>0.258761775915048</v>
       </c>
       <c r="U15" t="n">
-        <v>0.258761775915048</v>
-      </c>
-      <c r="V15" t="n">
         <v>7.618480441728133</v>
       </c>
+      <c r="V15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="1" t="inlineStr">
@@ -1620,27 +1632,27 @@
       <c r="O16" t="n">
         <v>0</v>
       </c>
-      <c r="P16" t="inlineStr"/>
+      <c r="P16" t="n">
+        <v>0</v>
+      </c>
       <c r="Q16" t="n">
-        <v>0</v>
+        <v>0.4256999551742678</v>
       </c>
       <c r="R16" t="n">
-        <v>0.4256999551742678</v>
-      </c>
-      <c r="S16" t="n">
         <v>3.4</v>
       </c>
-      <c r="T16" t="inlineStr">
-        <is>
-          <t>dif_prob_mod_bm &gt; 0</t>
-        </is>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>dif_prob_mod_bm &gt; 0</t>
+        </is>
+      </c>
+      <c r="T16" t="n">
+        <v>0.4142405996226951</v>
       </c>
       <c r="U16" t="n">
-        <v>0.4142405996226951</v>
-      </c>
-      <c r="V16" t="n">
         <v>8.128407481243014</v>
       </c>
+      <c r="V16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="1" t="inlineStr">
@@ -1694,27 +1706,27 @@
       <c r="O17" t="n">
         <v>0</v>
       </c>
-      <c r="P17" t="inlineStr"/>
+      <c r="P17" t="n">
+        <v>0</v>
+      </c>
       <c r="Q17" t="n">
-        <v>0</v>
+        <v>0.3798323858239034</v>
       </c>
       <c r="R17" t="n">
-        <v>0.3798323858239034</v>
-      </c>
-      <c r="S17" t="n">
         <v>3.5</v>
       </c>
-      <c r="T17" t="inlineStr">
-        <is>
-          <t>dif_prob_mod_bm &gt; 0</t>
-        </is>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>dif_prob_mod_bm &gt; 0</t>
+        </is>
+      </c>
+      <c r="T17" t="n">
+        <v>0.2928118670076996</v>
       </c>
       <c r="U17" t="n">
-        <v>0.2928118670076996</v>
-      </c>
-      <c r="V17" t="n">
         <v>7.731239194057843</v>
       </c>
+      <c r="V17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="1" t="inlineStr">
@@ -1768,27 +1780,27 @@
       <c r="O18" t="n">
         <v>0</v>
       </c>
-      <c r="P18" t="inlineStr"/>
+      <c r="P18" t="n">
+        <v>0</v>
+      </c>
       <c r="Q18" t="n">
-        <v>0</v>
+        <v>0.3610444616466352</v>
       </c>
       <c r="R18" t="n">
-        <v>0.3610444616466352</v>
-      </c>
-      <c r="S18" t="n">
         <v>3.9</v>
       </c>
-      <c r="T18" t="inlineStr">
-        <is>
-          <t>dif_prob_mod_bm &gt; 0</t>
-        </is>
+      <c r="S18" t="inlineStr">
+        <is>
+          <t>dif_prob_mod_bm &gt; 0</t>
+        </is>
+      </c>
+      <c r="T18" t="n">
+        <v>0.3126999236949251</v>
       </c>
       <c r="U18" t="n">
-        <v>0.3126999236949251</v>
-      </c>
-      <c r="V18" t="n">
         <v>7.796845953525049</v>
       </c>
+      <c r="V18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="1" t="inlineStr">
@@ -1842,27 +1854,27 @@
       <c r="O19" t="n">
         <v>0</v>
       </c>
-      <c r="P19" t="inlineStr"/>
+      <c r="P19" t="n">
+        <v>2</v>
+      </c>
       <c r="Q19" t="n">
-        <v>2</v>
+        <v>0.4674731409717773</v>
       </c>
       <c r="R19" t="n">
-        <v>0.4674731409717773</v>
-      </c>
-      <c r="S19" t="n">
         <v>1.83</v>
       </c>
-      <c r="T19" t="inlineStr">
-        <is>
-          <t>dif_prob_mod_bm &gt; 0</t>
-        </is>
+      <c r="S19" t="inlineStr">
+        <is>
+          <t>dif_prob_mod_bm &gt; 0</t>
+        </is>
+      </c>
+      <c r="T19" t="n">
+        <v>-0.6965019374537222</v>
       </c>
       <c r="U19" t="n">
-        <v>-0.6965019374537222</v>
-      </c>
-      <c r="V19" t="n">
         <v>2.494411868221891</v>
       </c>
+      <c r="V19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="1" t="inlineStr">
@@ -1916,27 +1928,27 @@
       <c r="O20" t="n">
         <v>0</v>
       </c>
-      <c r="P20" t="inlineStr"/>
+      <c r="P20" t="n">
+        <v>2</v>
+      </c>
       <c r="Q20" t="n">
-        <v>2</v>
+        <v>0.6431285815455916</v>
       </c>
       <c r="R20" t="n">
-        <v>0.6431285815455916</v>
-      </c>
-      <c r="S20" t="n">
         <v>1.44</v>
       </c>
-      <c r="T20" t="inlineStr">
-        <is>
-          <t>dif_prob_mod_bm &gt; 0</t>
-        </is>
+      <c r="S20" t="inlineStr">
+        <is>
+          <t>dif_prob_mod_bm &gt; 0</t>
+        </is>
+      </c>
+      <c r="T20" t="n">
+        <v>-0.6717712961304377</v>
       </c>
       <c r="U20" t="n">
-        <v>-0.6717712961304377</v>
-      </c>
-      <c r="V20" t="n">
         <v>2.535752486201099</v>
       </c>
+      <c r="V20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="1" t="inlineStr">
@@ -1994,24 +2006,24 @@
         <v>1</v>
       </c>
       <c r="Q21" t="n">
-        <v>1</v>
+        <v>0.5137547849844676</v>
       </c>
       <c r="R21" t="n">
-        <v>0.5137547849844676</v>
-      </c>
-      <c r="S21" t="n">
         <v>2.4</v>
       </c>
-      <c r="T21" t="inlineStr">
-        <is>
-          <t>dif_prob_mod_bm &gt; 0</t>
-        </is>
+      <c r="S21" t="inlineStr">
+        <is>
+          <t>dif_prob_mod_bm &gt; 0</t>
+        </is>
+      </c>
+      <c r="T21" t="n">
+        <v>0.2377668203701247</v>
       </c>
       <c r="U21" t="n">
-        <v>0.2377668203701247</v>
+        <v>11.74242812576997</v>
       </c>
       <c r="V21" t="n">
-        <v>11.74242812576997</v>
+        <v>1</v>
       </c>
     </row>
     <row r="22">
@@ -2070,24 +2082,24 @@
         <v>1</v>
       </c>
       <c r="Q22" t="n">
-        <v>1</v>
+        <v>0.5550865364079309</v>
       </c>
       <c r="R22" t="n">
-        <v>0.5550865364079309</v>
-      </c>
-      <c r="S22" t="n">
         <v>1.05</v>
       </c>
-      <c r="T22" t="inlineStr">
-        <is>
-          <t>dif_prob_mod_bm &gt; 0</t>
-        </is>
+      <c r="S22" t="inlineStr">
+        <is>
+          <t>dif_prob_mod_bm &gt; 0</t>
+        </is>
+      </c>
+      <c r="T22" t="n">
+        <v>-11.91883247919063</v>
       </c>
       <c r="U22" t="n">
-        <v>-11.91883247919063</v>
+        <v>0.0001399372143093516</v>
       </c>
       <c r="V22" t="n">
-        <v>0.0001399372143093516</v>
+        <v>1</v>
       </c>
     </row>
     <row r="23">
@@ -2140,27 +2152,27 @@
         <v>1</v>
       </c>
       <c r="O23" t="inlineStr"/>
-      <c r="P23" t="inlineStr"/>
+      <c r="P23" t="n">
+        <v>1</v>
+      </c>
       <c r="Q23" t="n">
-        <v>1</v>
+        <v>0.6294145786811493</v>
       </c>
       <c r="R23" t="n">
-        <v>0.6294145786811493</v>
-      </c>
-      <c r="S23" t="n">
         <v>1.57</v>
       </c>
-      <c r="T23" t="inlineStr">
-        <is>
-          <t>dif_prob_mod_bm &gt; 0</t>
-        </is>
+      <c r="S23" t="inlineStr">
+        <is>
+          <t>dif_prob_mod_bm &gt; 0</t>
+        </is>
+      </c>
+      <c r="T23" t="n">
+        <v>-0.02962183325963812</v>
       </c>
       <c r="U23" t="n">
-        <v>-0.02962183325963812</v>
-      </c>
-      <c r="V23" t="n">
         <v>10.3444967457871</v>
       </c>
+      <c r="V23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="1" t="inlineStr">
@@ -2212,27 +2224,27 @@
         <v>1</v>
       </c>
       <c r="O24" t="inlineStr"/>
-      <c r="P24" t="inlineStr"/>
+      <c r="P24" t="n">
+        <v>1</v>
+      </c>
       <c r="Q24" t="n">
-        <v>1</v>
+        <v>0.5397630416864644</v>
       </c>
       <c r="R24" t="n">
-        <v>0.5397630416864644</v>
-      </c>
-      <c r="S24" t="n">
         <v>1.91</v>
       </c>
-      <c r="T24" t="inlineStr">
-        <is>
-          <t>dif_prob_mod_bm &gt; 0</t>
-        </is>
+      <c r="S24" t="inlineStr">
+        <is>
+          <t>dif_prob_mod_bm &gt; 0</t>
+        </is>
+      </c>
+      <c r="T24" t="n">
+        <v>0.04858306062974404</v>
       </c>
       <c r="U24" t="n">
-        <v>0.04858306062974404</v>
-      </c>
-      <c r="V24" t="n">
         <v>10.75501091146519</v>
       </c>
+      <c r="V24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="1" t="inlineStr">
@@ -2284,27 +2296,27 @@
         <v>1</v>
       </c>
       <c r="O25" t="inlineStr"/>
-      <c r="P25" t="inlineStr"/>
+      <c r="P25" t="n">
+        <v>1</v>
+      </c>
       <c r="Q25" t="n">
-        <v>1</v>
+        <v>0.4747572903219309</v>
       </c>
       <c r="R25" t="n">
-        <v>0.4747572903219309</v>
-      </c>
-      <c r="S25" t="n">
         <v>1.25</v>
       </c>
-      <c r="T25" t="inlineStr">
-        <is>
-          <t>dif_prob_mod_bm &gt; 0</t>
-        </is>
+      <c r="S25" t="inlineStr">
+        <is>
+          <t>dif_prob_mod_bm &gt; 0</t>
+        </is>
+      </c>
+      <c r="T25" t="n">
+        <v>-2.323162211986208</v>
       </c>
       <c r="U25" t="n">
-        <v>-2.323162211986208</v>
-      </c>
-      <c r="V25" t="n">
         <v>1.873677906895099</v>
       </c>
+      <c r="V25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="1" t="inlineStr">
@@ -2356,27 +2368,27 @@
         <v>1</v>
       </c>
       <c r="O26" t="inlineStr"/>
-      <c r="P26" t="inlineStr"/>
+      <c r="P26" t="n">
+        <v>0</v>
+      </c>
       <c r="Q26" t="n">
-        <v>0</v>
+        <v>0.6247526875470442</v>
       </c>
       <c r="R26" t="n">
-        <v>0.6247526875470442</v>
-      </c>
-      <c r="S26" t="n">
         <v>3.4</v>
       </c>
-      <c r="T26" t="inlineStr">
-        <is>
-          <t>dif_prob_mod_bm &gt; 0</t>
-        </is>
+      <c r="S26" t="inlineStr">
+        <is>
+          <t>dif_prob_mod_bm &gt; 0</t>
+        </is>
+      </c>
+      <c r="T26" t="n">
+        <v>0.6691423438452084</v>
       </c>
       <c r="U26" t="n">
-        <v>0.6691423438452084</v>
-      </c>
-      <c r="V26" t="n">
         <v>13.88753287002925</v>
       </c>
+      <c r="V26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="1" t="inlineStr">
@@ -2428,27 +2440,27 @@
         <v>1</v>
       </c>
       <c r="O27" t="inlineStr"/>
-      <c r="P27" t="inlineStr"/>
+      <c r="P27" t="n">
+        <v>2</v>
+      </c>
       <c r="Q27" t="n">
-        <v>2</v>
+        <v>0.6000949845606875</v>
       </c>
       <c r="R27" t="n">
-        <v>0.6000949845606875</v>
-      </c>
-      <c r="S27" t="n">
         <v>1.75</v>
       </c>
-      <c r="T27" t="inlineStr">
-        <is>
-          <t>dif_prob_mod_bm &gt; 0</t>
-        </is>
+      <c r="S27" t="inlineStr">
+        <is>
+          <t>dif_prob_mod_bm &gt; 0</t>
+        </is>
+      </c>
+      <c r="T27" t="n">
+        <v>0.6688829730827095</v>
       </c>
       <c r="U27" t="n">
-        <v>0.6688829730827095</v>
-      </c>
-      <c r="V27" t="n">
         <v>1.98375897925198</v>
       </c>
+      <c r="V27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="1" t="inlineStr">
@@ -2503,27 +2515,27 @@
         <v>0</v>
       </c>
       <c r="P28" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q28" t="n">
-        <v>2</v>
+        <v>0.424590258371411</v>
       </c>
       <c r="R28" t="n">
-        <v>0.424590258371411</v>
-      </c>
-      <c r="S28" t="n">
         <v>3.1</v>
       </c>
-      <c r="T28" t="inlineStr">
-        <is>
-          <t>dif_prob_mod_bm &gt; 0</t>
-        </is>
+      <c r="S28" t="inlineStr">
+        <is>
+          <t>dif_prob_mod_bm &gt; 0</t>
+        </is>
+      </c>
+      <c r="T28" t="n">
+        <v>1.505856195006543</v>
       </c>
       <c r="U28" t="n">
-        <v>1.505856195006543</v>
+        <v>2.455338849128095</v>
       </c>
       <c r="V28" t="n">
-        <v>2.455338849128095</v>
+        <v>1</v>
       </c>
     </row>
     <row r="29">
@@ -2576,27 +2588,27 @@
         <v>1</v>
       </c>
       <c r="O29" t="inlineStr"/>
-      <c r="P29" t="inlineStr"/>
+      <c r="P29" t="n">
+        <v>2</v>
+      </c>
       <c r="Q29" t="n">
-        <v>2</v>
+        <v>0.5080384244550153</v>
       </c>
       <c r="R29" t="n">
-        <v>0.5080384244550153</v>
-      </c>
-      <c r="S29" t="n">
         <v>2.25</v>
       </c>
-      <c r="T29" t="inlineStr">
-        <is>
-          <t>dif_prob_mod_bm &gt; 0</t>
-        </is>
+      <c r="S29" t="inlineStr">
+        <is>
+          <t>dif_prob_mod_bm &gt; 0</t>
+        </is>
+      </c>
+      <c r="T29" t="n">
+        <v>1.144691640190276</v>
       </c>
       <c r="U29" t="n">
-        <v>1.144691640190276</v>
-      </c>
-      <c r="V29" t="n">
         <v>2.275619964303006</v>
       </c>
+      <c r="V29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="1" t="inlineStr">
@@ -2636,59 +2648,57 @@
         <v>1</v>
       </c>
       <c r="K30" t="n">
-        <v>0.3765153042428285</v>
+        <v>0.3502484008320507</v>
       </c>
       <c r="L30" t="n">
-        <v>0.382597831588973</v>
+        <v>0.4633213069580707</v>
       </c>
       <c r="M30" t="n">
-        <v>0.2408868641681985</v>
+        <v>0.1864302922098786</v>
       </c>
       <c r="N30" t="n">
         <v>1</v>
       </c>
-      <c r="O30" t="n">
-        <v>0</v>
-      </c>
-      <c r="P30" t="inlineStr"/>
+      <c r="O30" t="inlineStr"/>
+      <c r="P30" t="n">
+        <v>1</v>
+      </c>
       <c r="Q30" t="n">
-        <v>1</v>
+        <v>0.4633213069580707</v>
       </c>
       <c r="R30" t="n">
-        <v>0.382597831588973</v>
-      </c>
-      <c r="S30" t="n">
         <v>2.15</v>
       </c>
-      <c r="T30" t="inlineStr">
-        <is>
-          <t>dif_prob_mod_bm &gt; 0</t>
-        </is>
+      <c r="S30" t="inlineStr">
+        <is>
+          <t>dif_prob_mod_bm &gt; 0</t>
+        </is>
+      </c>
+      <c r="T30" t="n">
+        <v>-0.007457372058257236</v>
       </c>
       <c r="U30" t="n">
-        <v>-1.542736192032245</v>
-      </c>
-      <c r="V30" t="n">
-        <v>0.5284135948789995</v>
-      </c>
+        <v>6.724831485943391</v>
+      </c>
+      <c r="V30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="1" t="inlineStr">
         <is>
-          <t>2oCZvFZA</t>
+          <t>bDkKtGm1</t>
         </is>
       </c>
       <c r="B31" s="2" t="n">
-        <v>45689.45833333334</v>
+        <v>45689.58333333334</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>udinese</t>
+          <t>atalanta</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>venezia</t>
+          <t>torino</t>
         </is>
       </c>
       <c r="E31" t="n">
@@ -2698,71 +2708,69 @@
         <v>771</v>
       </c>
       <c r="G31" t="n">
-        <v>1.83</v>
+        <v>1.42</v>
       </c>
       <c r="H31" t="n">
-        <v>3.4</v>
+        <v>4.75</v>
       </c>
       <c r="I31" t="n">
-        <v>4.5</v>
+        <v>7</v>
       </c>
       <c r="J31" t="n">
         <v>1</v>
       </c>
       <c r="K31" t="n">
-        <v>0.3987487653879336</v>
+        <v>0.333903165440996</v>
       </c>
       <c r="L31" t="n">
-        <v>0.429542536684309</v>
+        <v>0.3950406132023191</v>
       </c>
       <c r="M31" t="n">
-        <v>0.1717086979277573</v>
+        <v>0.2710562213566848</v>
       </c>
       <c r="N31" t="n">
         <v>1</v>
       </c>
-      <c r="O31" t="n">
-        <v>0</v>
-      </c>
-      <c r="P31" t="inlineStr"/>
+      <c r="O31" t="inlineStr"/>
+      <c r="P31" t="n">
+        <v>1</v>
+      </c>
       <c r="Q31" t="n">
-        <v>1</v>
+        <v>0.3950406132023191</v>
       </c>
       <c r="R31" t="n">
-        <v>0.429542536684309</v>
-      </c>
-      <c r="S31" t="n">
-        <v>1.83</v>
-      </c>
-      <c r="T31" t="inlineStr">
-        <is>
-          <t>dif_prob_mod_bm &gt; 0</t>
-        </is>
+        <v>1.42</v>
+      </c>
+      <c r="S31" t="inlineStr">
+        <is>
+          <t>dif_prob_mod_bm &gt; 0</t>
+        </is>
+      </c>
+      <c r="T31" t="n">
+        <v>-2.322975287051359</v>
       </c>
       <c r="U31" t="n">
-        <v>-2.577556118888125</v>
-      </c>
-      <c r="V31" t="n">
-        <v>0.2117907391819226</v>
-      </c>
+        <v>1.204712305321105</v>
+      </c>
+      <c r="V31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="1" t="inlineStr">
         <is>
-          <t>WQmSvfID</t>
+          <t>t0ciuOTg</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
-        <v>45689.69791666666</v>
+        <v>45690.35416666666</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>bologna</t>
+          <t>juventus</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>como</t>
+          <t>empoli</t>
         </is>
       </c>
       <c r="E32" t="n">
@@ -2772,71 +2780,69 @@
         <v>771</v>
       </c>
       <c r="G32" t="n">
-        <v>1.83</v>
+        <v>1.36</v>
       </c>
       <c r="H32" t="n">
-        <v>3.6</v>
+        <v>4.75</v>
       </c>
       <c r="I32" t="n">
-        <v>4.33</v>
+        <v>9</v>
       </c>
       <c r="J32" t="n">
         <v>1</v>
       </c>
       <c r="K32" t="n">
-        <v>0.2936067140337434</v>
+        <v>0.4418693848503056</v>
       </c>
       <c r="L32" t="n">
-        <v>0.5590669710855019</v>
+        <v>0.4863281215162752</v>
       </c>
       <c r="M32" t="n">
-        <v>0.1473263148807547</v>
+        <v>0.07180249363341915</v>
       </c>
       <c r="N32" t="n">
         <v>1</v>
       </c>
-      <c r="O32" t="n">
-        <v>0</v>
-      </c>
-      <c r="P32" t="inlineStr"/>
+      <c r="O32" t="inlineStr"/>
+      <c r="P32" t="n">
+        <v>1</v>
+      </c>
       <c r="Q32" t="n">
-        <v>1</v>
+        <v>0.4863281215162752</v>
       </c>
       <c r="R32" t="n">
-        <v>0.5590669710855019</v>
-      </c>
-      <c r="S32" t="n">
-        <v>1.83</v>
-      </c>
-      <c r="T32" t="inlineStr">
-        <is>
-          <t>dif_prob_mod_bm &gt; 0</t>
-        </is>
+        <v>1.36</v>
+      </c>
+      <c r="S32" t="inlineStr">
+        <is>
+          <t>dif_prob_mod_bm &gt; 0</t>
+        </is>
+      </c>
+      <c r="T32" t="n">
+        <v>-2.090084905789294</v>
       </c>
       <c r="U32" t="n">
-        <v>0.2782235793550409</v>
-      </c>
-      <c r="V32" t="n">
-        <v>1.707331971163456</v>
-      </c>
+        <v>1.485867476994951</v>
+      </c>
+      <c r="V32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="1" t="inlineStr">
         <is>
-          <t>t0ciuOTg</t>
+          <t>Kp9rspas</t>
         </is>
       </c>
       <c r="B33" s="2" t="n">
-        <v>45690.35416666666</v>
+        <v>45690.45833333334</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>juventus</t>
+          <t>fiorentina</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>empoli</t>
+          <t>genoa</t>
         </is>
       </c>
       <c r="E33" t="n">
@@ -2846,71 +2852,69 @@
         <v>771</v>
       </c>
       <c r="G33" t="n">
-        <v>1.36</v>
+        <v>1.65</v>
       </c>
       <c r="H33" t="n">
-        <v>4.75</v>
+        <v>3.9</v>
       </c>
       <c r="I33" t="n">
-        <v>9</v>
+        <v>5.25</v>
       </c>
       <c r="J33" t="n">
         <v>1</v>
       </c>
       <c r="K33" t="n">
-        <v>0.4068786957616737</v>
+        <v>0.3684394886642793</v>
       </c>
       <c r="L33" t="n">
-        <v>0.5306028453310299</v>
+        <v>0.4560463569929265</v>
       </c>
       <c r="M33" t="n">
-        <v>0.06251845890729642</v>
+        <v>0.1755141543427943</v>
       </c>
       <c r="N33" t="n">
         <v>1</v>
       </c>
-      <c r="O33" t="n">
-        <v>0</v>
-      </c>
-      <c r="P33" t="inlineStr"/>
+      <c r="O33" t="inlineStr"/>
+      <c r="P33" t="n">
+        <v>1</v>
+      </c>
       <c r="Q33" t="n">
-        <v>1</v>
+        <v>0.4560463569929265</v>
       </c>
       <c r="R33" t="n">
-        <v>0.5306028453310299</v>
-      </c>
-      <c r="S33" t="n">
-        <v>1.36</v>
-      </c>
-      <c r="T33" t="inlineStr">
-        <is>
-          <t>dif_prob_mod_bm &gt; 0</t>
-        </is>
+        <v>1.65</v>
+      </c>
+      <c r="S33" t="inlineStr">
+        <is>
+          <t>dif_prob_mod_bm &gt; 0</t>
+        </is>
+      </c>
+      <c r="T33" t="n">
+        <v>-0.8462342255099874</v>
       </c>
       <c r="U33" t="n">
-        <v>-7.732781398605536</v>
-      </c>
-      <c r="V33" t="n">
-        <v>0.001314094770973998</v>
-      </c>
+        <v>4.053016046186949</v>
+      </c>
+      <c r="V33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="1" t="inlineStr">
         <is>
-          <t>Kp9rspas</t>
+          <t>Ork8ytTI</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
-        <v>45690.45833333334</v>
+        <v>45689.45833333334</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>fiorentina</t>
+          <t>monza</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>genoa</t>
+          <t>verona</t>
         </is>
       </c>
       <c r="E34" t="n">
@@ -2920,71 +2924,69 @@
         <v>771</v>
       </c>
       <c r="G34" t="n">
-        <v>1.65</v>
+        <v>2.3</v>
       </c>
       <c r="H34" t="n">
-        <v>3.9</v>
+        <v>3</v>
       </c>
       <c r="I34" t="n">
-        <v>5.25</v>
+        <v>3.5</v>
       </c>
       <c r="J34" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K34" t="n">
-        <v>0.3661407560077807</v>
+        <v>0.4248389337355024</v>
       </c>
       <c r="L34" t="n">
-        <v>0.524976143099398</v>
+        <v>0.3476780598573965</v>
       </c>
       <c r="M34" t="n">
-        <v>0.1088831008928214</v>
+        <v>0.2274830064071011</v>
       </c>
       <c r="N34" t="n">
         <v>1</v>
       </c>
-      <c r="O34" t="n">
-        <v>0</v>
-      </c>
-      <c r="P34" t="inlineStr"/>
+      <c r="O34" t="inlineStr"/>
+      <c r="P34" t="n">
+        <v>0</v>
+      </c>
       <c r="Q34" t="n">
-        <v>1</v>
+        <v>0.4248389337355024</v>
       </c>
       <c r="R34" t="n">
-        <v>0.524976143099398</v>
-      </c>
-      <c r="S34" t="n">
-        <v>1.65</v>
-      </c>
-      <c r="T34" t="inlineStr">
-        <is>
-          <t>dif_prob_mod_bm &gt; 0</t>
-        </is>
+        <v>3</v>
+      </c>
+      <c r="S34" t="inlineStr">
+        <is>
+          <t>dif_prob_mod_bm &gt; 0</t>
+        </is>
+      </c>
+      <c r="T34" t="n">
+        <v>0.30501866800723</v>
       </c>
       <c r="U34" t="n">
-        <v>-2.058297905938359</v>
-      </c>
-      <c r="V34" t="n">
-        <v>0.3396498164186039</v>
-      </c>
+        <v>7.771530300684557</v>
+      </c>
+      <c r="V34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="1" t="inlineStr">
         <is>
-          <t>SGeaw2b6</t>
+          <t>2oCZvFZA</t>
         </is>
       </c>
       <c r="B35" s="2" t="n">
-        <v>45690.58333333334</v>
+        <v>45689.45833333334</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>ac milan</t>
+          <t>udinese</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>inter</t>
+          <t>venezia</t>
         </is>
       </c>
       <c r="E35" t="n">
@@ -2994,71 +2996,69 @@
         <v>771</v>
       </c>
       <c r="G35" t="n">
-        <v>3.9</v>
+        <v>1.83</v>
       </c>
       <c r="H35" t="n">
-        <v>3.5</v>
+        <v>3.4</v>
       </c>
       <c r="I35" t="n">
-        <v>1.95</v>
+        <v>4.5</v>
       </c>
       <c r="J35" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K35" t="n">
-        <v>0.2971092600079664</v>
+        <v>0.4482982387825182</v>
       </c>
       <c r="L35" t="n">
-        <v>0.422216628167053</v>
+        <v>0.4051844851813466</v>
       </c>
       <c r="M35" t="n">
-        <v>0.2806741118249805</v>
+        <v>0.1465172760361353</v>
       </c>
       <c r="N35" t="n">
         <v>1</v>
       </c>
-      <c r="O35" t="n">
-        <v>0</v>
-      </c>
-      <c r="P35" t="inlineStr"/>
+      <c r="O35" t="inlineStr"/>
+      <c r="P35" t="n">
+        <v>0</v>
+      </c>
       <c r="Q35" t="n">
-        <v>1</v>
+        <v>0.4482982387825182</v>
       </c>
       <c r="R35" t="n">
-        <v>0.422216628167053</v>
-      </c>
-      <c r="S35" t="n">
-        <v>3.9</v>
-      </c>
-      <c r="T35" t="inlineStr">
-        <is>
-          <t>dif_prob_mod_bm &gt; 0</t>
-        </is>
+        <v>3.4</v>
+      </c>
+      <c r="S35" t="inlineStr">
+        <is>
+          <t>dif_prob_mod_bm &gt; 0</t>
+        </is>
+      </c>
+      <c r="T35" t="n">
+        <v>0.4853833443153349</v>
       </c>
       <c r="U35" t="n">
-        <v>2.229809827074161</v>
-      </c>
-      <c r="V35" t="n">
-        <v>2.708684060141953</v>
-      </c>
+        <v>8.356746574766078</v>
+      </c>
+      <c r="V35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="1" t="inlineStr">
         <is>
-          <t>AwfSty5b</t>
+          <t>WQmSvfID</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
-        <v>45690.69791666666</v>
+        <v>45689.69791666666</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>as roma</t>
+          <t>bologna</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>napoli</t>
+          <t>como</t>
         </is>
       </c>
       <c r="E36" t="n">
@@ -3068,71 +3068,73 @@
         <v>771</v>
       </c>
       <c r="G36" t="n">
-        <v>3.1</v>
+        <v>1.83</v>
       </c>
       <c r="H36" t="n">
-        <v>3.2</v>
+        <v>3.6</v>
       </c>
       <c r="I36" t="n">
-        <v>2.38</v>
+        <v>4.33</v>
       </c>
       <c r="J36" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K36" t="n">
-        <v>0.2896090100947376</v>
+        <v>0.447459622808495</v>
       </c>
       <c r="L36" t="n">
-        <v>0.420938584309217</v>
+        <v>0.3296072609297592</v>
       </c>
       <c r="M36" t="n">
-        <v>0.2894524055960452</v>
+        <v>0.2229331162617458</v>
       </c>
       <c r="N36" t="n">
         <v>1</v>
       </c>
       <c r="O36" t="n">
-        <v>0</v>
-      </c>
-      <c r="P36" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="P36" t="n">
+        <v>0</v>
+      </c>
       <c r="Q36" t="n">
-        <v>1</v>
+        <v>0.447459622808495</v>
       </c>
       <c r="R36" t="n">
-        <v>0.420938584309217</v>
-      </c>
-      <c r="S36" t="n">
-        <v>3.1</v>
-      </c>
-      <c r="T36" t="inlineStr">
-        <is>
-          <t>dif_prob_mod_bm &gt; 0</t>
-        </is>
+        <v>3.6</v>
+      </c>
+      <c r="S36" t="inlineStr">
+        <is>
+          <t>dif_prob_mod_bm &gt; 0</t>
+        </is>
+      </c>
+      <c r="T36" t="n">
+        <v>0.5220979847098991</v>
       </c>
       <c r="U36" t="n">
-        <v>1.451950530278918</v>
+        <v>4.236557946509294</v>
       </c>
       <c r="V36" t="n">
-        <v>2.430895322972049</v>
+        <v>1</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="1" t="inlineStr">
         <is>
-          <t>Ork8ytTI</t>
+          <t>SGeaw2b6</t>
         </is>
       </c>
       <c r="B37" s="2" t="n">
-        <v>45689.45833333334</v>
+        <v>45690.58333333334</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>monza</t>
+          <t>ac milan</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>verona</t>
+          <t>inter</t>
         </is>
       </c>
       <c r="E37" t="n">
@@ -3142,71 +3144,69 @@
         <v>771</v>
       </c>
       <c r="G37" t="n">
-        <v>2.3</v>
+        <v>3.9</v>
       </c>
       <c r="H37" t="n">
-        <v>3</v>
+        <v>3.5</v>
       </c>
       <c r="I37" t="n">
-        <v>3.5</v>
+        <v>1.95</v>
       </c>
       <c r="J37" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K37" t="n">
-        <v>0.5459499984102366</v>
+        <v>0.314137944084132</v>
       </c>
       <c r="L37" t="n">
-        <v>0.1719851359999892</v>
+        <v>0.300390716864111</v>
       </c>
       <c r="M37" t="n">
-        <v>0.2820648655897742</v>
+        <v>0.3854713390517569</v>
       </c>
       <c r="N37" t="n">
         <v>1</v>
       </c>
-      <c r="O37" t="n">
-        <v>0</v>
-      </c>
-      <c r="P37" t="inlineStr"/>
+      <c r="O37" t="inlineStr"/>
+      <c r="P37" t="n">
+        <v>2</v>
+      </c>
       <c r="Q37" t="n">
-        <v>0</v>
+        <v>0.3854713390517569</v>
       </c>
       <c r="R37" t="n">
-        <v>0.5459499984102366</v>
-      </c>
-      <c r="S37" t="n">
-        <v>3</v>
-      </c>
-      <c r="T37" t="inlineStr">
-        <is>
-          <t>dif_prob_mod_bm &gt; 0</t>
-        </is>
+        <v>1.95</v>
+      </c>
+      <c r="S37" t="inlineStr">
+        <is>
+          <t>dif_prob_mod_bm &gt; 0</t>
+        </is>
+      </c>
+      <c r="T37" t="n">
+        <v>-0.5808909680680094</v>
       </c>
       <c r="U37" t="n">
-        <v>0.4556071394505071</v>
-      </c>
-      <c r="V37" t="n">
-        <v>12.85140258303321</v>
-      </c>
+        <v>4.842822703976623</v>
+      </c>
+      <c r="V37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="1" t="inlineStr">
         <is>
-          <t>bDkKtGm1</t>
+          <t>AwfSty5b</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
-        <v>45689.58333333334</v>
+        <v>45690.69791666666</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>atalanta</t>
+          <t>as roma</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>torino</t>
+          <t>napoli</t>
         </is>
       </c>
       <c r="E38" t="n">
@@ -3216,53 +3216,51 @@
         <v>771</v>
       </c>
       <c r="G38" t="n">
-        <v>1.42</v>
+        <v>3.1</v>
       </c>
       <c r="H38" t="n">
-        <v>4.75</v>
+        <v>3.2</v>
       </c>
       <c r="I38" t="n">
-        <v>7</v>
+        <v>2.38</v>
       </c>
       <c r="J38" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K38" t="n">
-        <v>0.4358423391718592</v>
+        <v>0.2816194307644775</v>
       </c>
       <c r="L38" t="n">
-        <v>0.4312154184592805</v>
+        <v>0.3449465664776952</v>
       </c>
       <c r="M38" t="n">
-        <v>0.1329422423688603</v>
+        <v>0.3734340027578272</v>
       </c>
       <c r="N38" t="n">
         <v>1</v>
       </c>
-      <c r="O38" t="n">
-        <v>0</v>
-      </c>
-      <c r="P38" t="inlineStr"/>
+      <c r="O38" t="inlineStr"/>
+      <c r="P38" t="n">
+        <v>2</v>
+      </c>
       <c r="Q38" t="n">
-        <v>0</v>
+        <v>0.3734340027578272</v>
       </c>
       <c r="R38" t="n">
-        <v>0.4358423391718592</v>
-      </c>
-      <c r="S38" t="n">
-        <v>4.75</v>
-      </c>
-      <c r="T38" t="inlineStr">
-        <is>
-          <t>dif_prob_mod_bm &gt; 0</t>
-        </is>
+        <v>2.38</v>
+      </c>
+      <c r="S38" t="inlineStr">
+        <is>
+          <t>dif_prob_mod_bm &gt; 0</t>
+        </is>
+      </c>
+      <c r="T38" t="n">
+        <v>-0.1791096190601794</v>
       </c>
       <c r="U38" t="n">
-        <v>0.4077147089776499</v>
-      </c>
-      <c r="V38" t="n">
-        <v>12.61133543358164</v>
-      </c>
+        <v>6.147115897598663</v>
+      </c>
+      <c r="V38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="1" t="inlineStr">
@@ -3302,41 +3300,39 @@
         <v>2</v>
       </c>
       <c r="K39" t="n">
-        <v>0.1791399910294647</v>
+        <v>0.2424454198980837</v>
       </c>
       <c r="L39" t="n">
-        <v>0.1449255665442812</v>
+        <v>0.1993746310629123</v>
       </c>
       <c r="M39" t="n">
-        <v>0.6759344424262541</v>
+        <v>0.5581799490390039</v>
       </c>
       <c r="N39" t="n">
         <v>1</v>
       </c>
-      <c r="O39" t="n">
-        <v>0</v>
-      </c>
-      <c r="P39" t="inlineStr"/>
+      <c r="O39" t="inlineStr"/>
+      <c r="P39" t="n">
+        <v>2</v>
+      </c>
       <c r="Q39" t="n">
+        <v>0.5581799490390039</v>
+      </c>
+      <c r="R39" t="n">
         <v>2</v>
       </c>
-      <c r="R39" t="n">
-        <v>0.6759344424262541</v>
-      </c>
-      <c r="S39" t="n">
-        <v>2</v>
-      </c>
-      <c r="T39" t="inlineStr">
-        <is>
-          <t>dif_prob_mod_bm &gt; 0</t>
-        </is>
+      <c r="S39" t="inlineStr">
+        <is>
+          <t>dif_prob_mod_bm &gt; 0</t>
+        </is>
+      </c>
+      <c r="T39" t="n">
+        <v>0.2585775512844619</v>
       </c>
       <c r="U39" t="n">
-        <v>0.7819308552277959</v>
-      </c>
-      <c r="V39" t="n">
-        <v>9.262297460365788</v>
-      </c>
+        <v>7.617868969166058</v>
+      </c>
+      <c r="V39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="1" t="inlineStr">
@@ -3376,41 +3372,39 @@
         <v>1</v>
       </c>
       <c r="K40" t="n">
-        <v>0.275123380112129</v>
+        <v>0.09436274384855614</v>
       </c>
       <c r="L40" t="n">
-        <v>0.6316609991223364</v>
+        <v>0.9018149227882214</v>
       </c>
       <c r="M40" t="n">
-        <v>0.09321562076553459</v>
+        <v>0.00382233336322238</v>
       </c>
       <c r="N40" t="n">
         <v>1</v>
       </c>
-      <c r="O40" t="n">
-        <v>0</v>
-      </c>
-      <c r="P40" t="inlineStr"/>
+      <c r="O40" t="inlineStr"/>
+      <c r="P40" t="n">
+        <v>1</v>
+      </c>
       <c r="Q40" t="n">
-        <v>1</v>
+        <v>0.9018149227882214</v>
       </c>
       <c r="R40" t="n">
-        <v>0.6316609991223364</v>
-      </c>
-      <c r="S40" t="n">
         <v>1.19</v>
       </c>
-      <c r="T40" t="inlineStr">
-        <is>
-          <t>dif_prob_mod_bm &gt; 0</t>
-        </is>
+      <c r="S40" t="inlineStr">
+        <is>
+          <t>dif_prob_mod_bm &gt; 0</t>
+        </is>
+      </c>
+      <c r="T40" t="n">
+        <v>0.8556696855904495</v>
       </c>
       <c r="U40" t="n">
-        <v>-2.904367380636489</v>
-      </c>
-      <c r="V40" t="n">
-        <v>0.7011642103698786</v>
-      </c>
+        <v>9.473694313132279</v>
+      </c>
+      <c r="V40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="1" t="inlineStr">
@@ -3450,41 +3444,39 @@
         <v>1</v>
       </c>
       <c r="K41" t="n">
-        <v>0.4104610450080212</v>
+        <v>0.06862380360619014</v>
       </c>
       <c r="L41" t="n">
-        <v>0.4467829269955551</v>
+        <v>0.8979888737660324</v>
       </c>
       <c r="M41" t="n">
-        <v>0.1427560279964238</v>
+        <v>0.03338732262777758</v>
       </c>
       <c r="N41" t="n">
         <v>1</v>
       </c>
-      <c r="O41" t="n">
-        <v>0</v>
-      </c>
-      <c r="P41" t="inlineStr"/>
+      <c r="O41" t="inlineStr"/>
+      <c r="P41" t="n">
+        <v>1</v>
+      </c>
       <c r="Q41" t="n">
-        <v>1</v>
+        <v>0.8979888737660324</v>
       </c>
       <c r="R41" t="n">
-        <v>0.4467829269955551</v>
-      </c>
-      <c r="S41" t="n">
         <v>1.44</v>
       </c>
-      <c r="T41" t="inlineStr">
-        <is>
-          <t>dif_prob_mod_bm &gt; 0</t>
-        </is>
+      <c r="S41" t="inlineStr">
+        <is>
+          <t>dif_prob_mod_bm &gt; 0</t>
+        </is>
+      </c>
+      <c r="T41" t="n">
+        <v>1.480323122338822</v>
       </c>
       <c r="U41" t="n">
-        <v>-1.80117467235556</v>
-      </c>
-      <c r="V41" t="n">
-        <v>1.913059794940955</v>
-      </c>
+        <v>10.99738864979531</v>
+      </c>
+      <c r="V41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="1" t="inlineStr">
@@ -3524,41 +3516,39 @@
         <v>1</v>
       </c>
       <c r="K42" t="n">
-        <v>0.2338018814832161</v>
+        <v>0.03093977925509008</v>
       </c>
       <c r="L42" t="n">
-        <v>0.6772173737986642</v>
+        <v>0.9046471123945106</v>
       </c>
       <c r="M42" t="n">
-        <v>0.08898074471811962</v>
+        <v>0.06441310835039929</v>
       </c>
       <c r="N42" t="n">
         <v>1</v>
       </c>
-      <c r="O42" t="n">
-        <v>0</v>
-      </c>
-      <c r="P42" t="inlineStr"/>
+      <c r="O42" t="inlineStr"/>
+      <c r="P42" t="n">
+        <v>1</v>
+      </c>
       <c r="Q42" t="n">
-        <v>1</v>
+        <v>0.9046471123945106</v>
       </c>
       <c r="R42" t="n">
-        <v>0.6772173737986642</v>
-      </c>
-      <c r="S42" t="n">
         <v>1.2</v>
       </c>
-      <c r="T42" t="inlineStr">
-        <is>
-          <t>dif_prob_mod_bm &gt; 0</t>
-        </is>
+      <c r="S42" t="inlineStr">
+        <is>
+          <t>dif_prob_mod_bm &gt; 0</t>
+        </is>
+      </c>
+      <c r="T42" t="n">
+        <v>0.9508503874823627</v>
       </c>
       <c r="U42" t="n">
-        <v>-2.081546127128923</v>
-      </c>
-      <c r="V42" t="n">
-        <v>1.497196181887437</v>
-      </c>
+        <v>9.737363236319773</v>
+      </c>
+      <c r="V42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="1" t="inlineStr">
@@ -3598,59 +3588,57 @@
         <v>1</v>
       </c>
       <c r="K43" t="n">
-        <v>0.2547024519653249</v>
+        <v>0.1024846729058405</v>
       </c>
       <c r="L43" t="n">
-        <v>0.5526450881035055</v>
+        <v>0.7083262245436563</v>
       </c>
       <c r="M43" t="n">
-        <v>0.1926524599311696</v>
+        <v>0.189189102550503</v>
       </c>
       <c r="N43" t="n">
         <v>1</v>
       </c>
-      <c r="O43" t="n">
-        <v>0</v>
-      </c>
-      <c r="P43" t="inlineStr"/>
+      <c r="O43" t="inlineStr"/>
+      <c r="P43" t="n">
+        <v>1</v>
+      </c>
       <c r="Q43" t="n">
-        <v>1</v>
+        <v>0.7083262245436563</v>
       </c>
       <c r="R43" t="n">
-        <v>0.5526450881035055</v>
-      </c>
-      <c r="S43" t="n">
         <v>2.3</v>
       </c>
-      <c r="T43" t="inlineStr">
-        <is>
-          <t>dif_prob_mod_bm &gt; 0</t>
-        </is>
+      <c r="S43" t="inlineStr">
+        <is>
+          <t>dif_prob_mod_bm &gt; 0</t>
+        </is>
+      </c>
+      <c r="T43" t="n">
+        <v>1.075470626410956</v>
       </c>
       <c r="U43" t="n">
-        <v>0.4633909446804491</v>
-      </c>
-      <c r="V43" t="n">
-        <v>8.286546962843302</v>
-      </c>
+        <v>10.06608444570931</v>
+      </c>
+      <c r="V43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="1" t="inlineStr">
         <is>
-          <t>SM0qnskQ</t>
+          <t>CfxGtLCm</t>
         </is>
       </c>
       <c r="B44" s="2" t="n">
-        <v>45691.70833333334</v>
+        <v>45690.60416666666</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>girona</t>
+          <t>osasuna</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>las palmas</t>
+          <t>real sociedad</t>
         </is>
       </c>
       <c r="E44" t="n">
@@ -3660,71 +3648,69 @@
         <v>1481</v>
       </c>
       <c r="G44" t="n">
-        <v>1.6</v>
+        <v>3</v>
       </c>
       <c r="H44" t="n">
-        <v>4.2</v>
+        <v>3</v>
       </c>
       <c r="I44" t="n">
-        <v>5</v>
+        <v>2.55</v>
       </c>
       <c r="J44" t="n">
         <v>1</v>
       </c>
       <c r="K44" t="n">
-        <v>0.3411175600501996</v>
+        <v>0.1988526796869084</v>
       </c>
       <c r="L44" t="n">
-        <v>0.4790574004960153</v>
+        <v>0.5828390554652776</v>
       </c>
       <c r="M44" t="n">
-        <v>0.1798250394537851</v>
+        <v>0.2183082648478141</v>
       </c>
       <c r="N44" t="n">
         <v>1</v>
       </c>
-      <c r="O44" t="n">
-        <v>0</v>
-      </c>
-      <c r="P44" t="inlineStr"/>
+      <c r="O44" t="inlineStr"/>
+      <c r="P44" t="n">
+        <v>1</v>
+      </c>
       <c r="Q44" t="n">
-        <v>1</v>
+        <v>0.5828390554652776</v>
       </c>
       <c r="R44" t="n">
-        <v>0.4790574004960153</v>
-      </c>
-      <c r="S44" t="n">
-        <v>1.6</v>
-      </c>
-      <c r="T44" t="inlineStr">
-        <is>
-          <t>dif_prob_mod_bm &gt; 0</t>
-        </is>
+        <v>3</v>
+      </c>
+      <c r="S44" t="inlineStr">
+        <is>
+          <t>dif_prob_mod_bm &gt; 0</t>
+        </is>
+      </c>
+      <c r="T44" t="n">
+        <v>0.8316857404398141</v>
       </c>
       <c r="U44" t="n">
-        <v>-0.864845034097687</v>
-      </c>
-      <c r="V44" t="n">
-        <v>4.000429000634505</v>
-      </c>
+        <v>9.405601912083522</v>
+      </c>
+      <c r="V44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="1" t="inlineStr">
         <is>
-          <t>GnZWxwCC</t>
+          <t>SM0qnskQ</t>
         </is>
       </c>
       <c r="B45" s="2" t="n">
-        <v>45688.70833333334</v>
+        <v>45691.70833333334</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>leganes</t>
+          <t>girona</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>rayo vallecano</t>
+          <t>las palmas</t>
         </is>
       </c>
       <c r="E45" t="n">
@@ -3734,71 +3720,69 @@
         <v>1481</v>
       </c>
       <c r="G45" t="n">
-        <v>3</v>
+        <v>1.6</v>
       </c>
       <c r="H45" t="n">
-        <v>3</v>
+        <v>4.2</v>
       </c>
       <c r="I45" t="n">
-        <v>2.55</v>
+        <v>5</v>
       </c>
       <c r="J45" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K45" t="n">
-        <v>0.3948484091996389</v>
+        <v>0.2943302908759011</v>
       </c>
       <c r="L45" t="n">
-        <v>0.2115027417183989</v>
+        <v>0.6094539255988166</v>
       </c>
       <c r="M45" t="n">
-        <v>0.3936488490819622</v>
+        <v>0.09621578352528226</v>
       </c>
       <c r="N45" t="n">
         <v>1</v>
       </c>
-      <c r="O45" t="n">
-        <v>0</v>
-      </c>
-      <c r="P45" t="inlineStr"/>
+      <c r="O45" t="inlineStr"/>
+      <c r="P45" t="n">
+        <v>1</v>
+      </c>
       <c r="Q45" t="n">
-        <v>0</v>
+        <v>0.6094539255988166</v>
       </c>
       <c r="R45" t="n">
-        <v>0.3948484091996389</v>
-      </c>
-      <c r="S45" t="n">
-        <v>3</v>
-      </c>
-      <c r="T45" t="inlineStr">
-        <is>
-          <t>dif_prob_mod_bm &gt; 0</t>
-        </is>
+        <v>1.6</v>
+      </c>
+      <c r="S45" t="inlineStr">
+        <is>
+          <t>dif_prob_mod_bm &gt; 0</t>
+        </is>
+      </c>
+      <c r="T45" t="n">
+        <v>-0.09212488534034569</v>
       </c>
       <c r="U45" t="n">
-        <v>0.1318180197135119</v>
-      </c>
-      <c r="V45" t="n">
-        <v>11.19104426162537</v>
-      </c>
+        <v>6.439298224588118</v>
+      </c>
+      <c r="V45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="1" t="inlineStr">
         <is>
-          <t>CfxGtLCm</t>
+          <t>GnZWxwCC</t>
         </is>
       </c>
       <c r="B46" s="2" t="n">
-        <v>45690.60416666666</v>
+        <v>45688.70833333334</v>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>osasuna</t>
+          <t>leganes</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>real sociedad</t>
+          <t>rayo vallecano</t>
         </is>
       </c>
       <c r="E46" t="n">
@@ -3820,13 +3804,13 @@
         <v>0</v>
       </c>
       <c r="K46" t="n">
-        <v>0.4514627464770786</v>
+        <v>0.4627520454560675</v>
       </c>
       <c r="L46" t="n">
-        <v>0.1976583500773928</v>
+        <v>0.08552068206809124</v>
       </c>
       <c r="M46" t="n">
-        <v>0.3508789034455286</v>
+        <v>0.4517272724758413</v>
       </c>
       <c r="N46" t="n">
         <v>1</v>
@@ -3834,45 +3818,47 @@
       <c r="O46" t="n">
         <v>0</v>
       </c>
-      <c r="P46" t="inlineStr"/>
+      <c r="P46" t="n">
+        <v>0</v>
+      </c>
       <c r="Q46" t="n">
-        <v>0</v>
+        <v>0.4627520454560675</v>
       </c>
       <c r="R46" t="n">
-        <v>0.4514627464770786</v>
-      </c>
-      <c r="S46" t="n">
         <v>3</v>
       </c>
-      <c r="T46" t="inlineStr">
-        <is>
-          <t>dif_prob_mod_bm &gt; 0</t>
-        </is>
+      <c r="S46" t="inlineStr">
+        <is>
+          <t>dif_prob_mod_bm &gt; 0</t>
+        </is>
+      </c>
+      <c r="T46" t="n">
+        <v>1.941280681841012</v>
       </c>
       <c r="U46" t="n">
-        <v>0.253134456736597</v>
+        <v>2.623478317070065</v>
       </c>
       <c r="V46" t="n">
-        <v>11.82190477777681</v>
+        <v>1</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="1" t="inlineStr">
         <is>
-          <t>2q9cOwcJ</t>
+          <t>YLnW8uHi</t>
         </is>
       </c>
       <c r="B47" s="2" t="n">
-        <v>45689.41666666666</v>
+        <v>45689.70833333334</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>getafe</t>
+          <t>espanyol</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>sevilla</t>
+          <t>real madrid</t>
         </is>
       </c>
       <c r="E47" t="n">
@@ -3882,25 +3868,25 @@
         <v>1481</v>
       </c>
       <c r="G47" t="n">
-        <v>2.45</v>
+        <v>9</v>
       </c>
       <c r="H47" t="n">
-        <v>2.9</v>
+        <v>5.75</v>
       </c>
       <c r="I47" t="n">
-        <v>3.25</v>
+        <v>1.3</v>
       </c>
       <c r="J47" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K47" t="n">
-        <v>0.3516009058273227</v>
+        <v>0.5949375372985796</v>
       </c>
       <c r="L47" t="n">
-        <v>0.2800807916890317</v>
+        <v>0.01413365164766524</v>
       </c>
       <c r="M47" t="n">
-        <v>0.3683183024836457</v>
+        <v>0.3909288110537553</v>
       </c>
       <c r="N47" t="n">
         <v>1</v>
@@ -3908,45 +3894,47 @@
       <c r="O47" t="n">
         <v>0</v>
       </c>
-      <c r="P47" t="inlineStr"/>
+      <c r="P47" t="n">
+        <v>0</v>
+      </c>
       <c r="Q47" t="n">
-        <v>2</v>
+        <v>0.5949375372985796</v>
       </c>
       <c r="R47" t="n">
-        <v>0.3683183024836457</v>
-      </c>
-      <c r="S47" t="n">
-        <v>3.25</v>
-      </c>
-      <c r="T47" t="inlineStr">
-        <is>
-          <t>dif_prob_mod_bm &gt; 0</t>
-        </is>
+        <v>5.75</v>
+      </c>
+      <c r="S47" t="inlineStr">
+        <is>
+          <t>dif_prob_mod_bm &gt; 0</t>
+        </is>
+      </c>
+      <c r="T47" t="n">
+        <v>5.096612293614384</v>
       </c>
       <c r="U47" t="n">
-        <v>0.8757088136526594</v>
+        <v>2.98175927969987</v>
       </c>
       <c r="V47" t="n">
-        <v>2.117796579922938</v>
+        <v>1</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="1" t="inlineStr">
         <is>
-          <t>YLnW8uHi</t>
+          <t>l0XvyHtP</t>
         </is>
       </c>
       <c r="B48" s="2" t="n">
-        <v>45689.70833333334</v>
+        <v>45690.70833333334</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>espanyol</t>
+          <t>betis</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>real madrid</t>
+          <t>ath bilbao</t>
         </is>
       </c>
       <c r="E48" t="n">
@@ -3956,71 +3944,69 @@
         <v>1481</v>
       </c>
       <c r="G48" t="n">
-        <v>9</v>
+        <v>2.9</v>
       </c>
       <c r="H48" t="n">
-        <v>5.75</v>
+        <v>3.3</v>
       </c>
       <c r="I48" t="n">
-        <v>1.3</v>
+        <v>2.45</v>
       </c>
       <c r="J48" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K48" t="n">
-        <v>0.2424942757502738</v>
+        <v>0.7983658857644801</v>
       </c>
       <c r="L48" t="n">
-        <v>0.03781277809655703</v>
+        <v>0.02813877324986954</v>
       </c>
       <c r="M48" t="n">
-        <v>0.7196929461531691</v>
+        <v>0.1734953409856504</v>
       </c>
       <c r="N48" t="n">
         <v>1</v>
       </c>
-      <c r="O48" t="n">
-        <v>0</v>
-      </c>
-      <c r="P48" t="inlineStr"/>
+      <c r="O48" t="inlineStr"/>
+      <c r="P48" t="n">
+        <v>0</v>
+      </c>
       <c r="Q48" t="n">
-        <v>2</v>
+        <v>0.7983658857644801</v>
       </c>
       <c r="R48" t="n">
-        <v>0.7196929461531691</v>
-      </c>
-      <c r="S48" t="n">
-        <v>1.3</v>
-      </c>
-      <c r="T48" t="inlineStr">
-        <is>
-          <t>dif_prob_mod_bm &gt; 0</t>
-        </is>
+        <v>3.3</v>
+      </c>
+      <c r="S48" t="inlineStr">
+        <is>
+          <t>dif_prob_mod_bm &gt; 0</t>
+        </is>
+      </c>
+      <c r="T48" t="n">
+        <v>7.106988795751237</v>
       </c>
       <c r="U48" t="n">
-        <v>-2.146639000029336</v>
-      </c>
-      <c r="V48" t="n">
-        <v>0.3139371413562208</v>
-      </c>
+        <v>2.997543936785263</v>
+      </c>
+      <c r="V48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="1" t="inlineStr">
         <is>
-          <t>l0XvyHtP</t>
+          <t>2q9cOwcJ</t>
         </is>
       </c>
       <c r="B49" s="2" t="n">
-        <v>45690.70833333334</v>
+        <v>45689.41666666666</v>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>betis</t>
+          <t>getafe</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>ath bilbao</t>
+          <t>sevilla</t>
         </is>
       </c>
       <c r="E49" t="n">
@@ -4030,53 +4016,51 @@
         <v>1481</v>
       </c>
       <c r="G49" t="n">
+        <v>2.45</v>
+      </c>
+      <c r="H49" t="n">
         <v>2.9</v>
       </c>
-      <c r="H49" t="n">
-        <v>3.3</v>
-      </c>
       <c r="I49" t="n">
-        <v>2.45</v>
+        <v>3.25</v>
       </c>
       <c r="J49" t="n">
         <v>2</v>
       </c>
       <c r="K49" t="n">
-        <v>0.3467714232705138</v>
+        <v>0.06699193152706948</v>
       </c>
       <c r="L49" t="n">
-        <v>0.1464005137506659</v>
+        <v>0.1480935332655854</v>
       </c>
       <c r="M49" t="n">
-        <v>0.5068280629788203</v>
+        <v>0.7849145352073451</v>
       </c>
       <c r="N49" t="n">
         <v>1</v>
       </c>
-      <c r="O49" t="n">
-        <v>0</v>
-      </c>
-      <c r="P49" t="inlineStr"/>
+      <c r="O49" t="inlineStr"/>
+      <c r="P49" t="n">
+        <v>2</v>
+      </c>
       <c r="Q49" t="n">
-        <v>2</v>
+        <v>0.7849145352073451</v>
       </c>
       <c r="R49" t="n">
-        <v>0.5068280629788203</v>
-      </c>
-      <c r="S49" t="n">
-        <v>2.45</v>
-      </c>
-      <c r="T49" t="inlineStr">
-        <is>
-          <t>dif_prob_mod_bm &gt; 0</t>
-        </is>
+        <v>3.25</v>
+      </c>
+      <c r="S49" t="inlineStr">
+        <is>
+          <t>dif_prob_mod_bm &gt; 0</t>
+        </is>
+      </c>
+      <c r="T49" t="n">
+        <v>2.757283981197994</v>
       </c>
       <c r="U49" t="n">
-        <v>1.667094857228344</v>
-      </c>
-      <c r="V49" t="n">
-        <v>2.523564317229353</v>
-      </c>
+        <v>7.052425544743421</v>
+      </c>
+      <c r="V49" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
DATA. Actualizo predicciones tras implementar Expected ROI para seleccionar estrategia.
</commit_message>
<xml_diff>
--- a/data/predicciones.xlsx
+++ b/data/predicciones.xlsx
@@ -1203,10 +1203,10 @@
         </is>
       </c>
       <c r="T10" t="n">
-        <v>1.173022238258309</v>
+        <v>2.111440028864956</v>
       </c>
       <c r="U10" t="n">
-        <v>10.30982667718166</v>
+        <v>6.690075950635718</v>
       </c>
       <c r="V10" t="inlineStr"/>
     </row>
@@ -1277,10 +1277,10 @@
         </is>
       </c>
       <c r="T11" t="n">
-        <v>0.4553078303895461</v>
+        <v>0.819554094701183</v>
       </c>
       <c r="U11" t="n">
-        <v>8.260656406451861</v>
+        <v>5.206062589442977</v>
       </c>
       <c r="V11" t="inlineStr"/>
     </row>
@@ -3399,10 +3399,10 @@
         </is>
       </c>
       <c r="T40" t="n">
-        <v>0.8556696855904495</v>
+        <v>1.540205434062809</v>
       </c>
       <c r="U40" t="n">
-        <v>9.473694313132279</v>
+        <v>6.176209404776601</v>
       </c>
       <c r="V40" t="inlineStr"/>
     </row>
@@ -3471,10 +3471,10 @@
         </is>
       </c>
       <c r="T41" t="n">
-        <v>1.480323122338822</v>
+        <v>2.664581620209879</v>
       </c>
       <c r="U41" t="n">
-        <v>10.99738864979531</v>
+        <v>7.011780398646064</v>
       </c>
       <c r="V41" t="inlineStr"/>
     </row>
@@ -3543,10 +3543,10 @@
         </is>
       </c>
       <c r="T42" t="n">
-        <v>0.9508503874823627</v>
+        <v>1.711530697468253</v>
       </c>
       <c r="U42" t="n">
-        <v>9.737363236319773</v>
+        <v>6.352760380036897</v>
       </c>
       <c r="V42" t="inlineStr"/>
     </row>
@@ -3615,10 +3615,10 @@
         </is>
       </c>
       <c r="T43" t="n">
-        <v>1.075470626410956</v>
+        <v>1.935847127539722</v>
       </c>
       <c r="U43" t="n">
-        <v>10.06608444570931</v>
+        <v>6.554213979183962</v>
       </c>
       <c r="V43" t="inlineStr"/>
     </row>
@@ -3687,10 +3687,10 @@
         </is>
       </c>
       <c r="T44" t="n">
-        <v>0.8316857404398141</v>
+        <v>1.497034332791666</v>
       </c>
       <c r="U44" t="n">
-        <v>9.405601912083522</v>
+        <v>6.128488055991386</v>
       </c>
       <c r="V44" t="inlineStr"/>
     </row>
@@ -3759,10 +3759,10 @@
         </is>
       </c>
       <c r="T45" t="n">
-        <v>-0.09212488534034569</v>
+        <v>-0.1658247936126222</v>
       </c>
       <c r="U45" t="n">
-        <v>6.439298224588118</v>
+        <v>3.439789031282862</v>
       </c>
       <c r="V45" t="inlineStr"/>
     </row>
@@ -4055,10 +4055,10 @@
         </is>
       </c>
       <c r="T49" t="n">
-        <v>2.757283981197994</v>
+        <v>6.893209952994985</v>
       </c>
       <c r="U49" t="n">
-        <v>7.052425544743421</v>
+        <v>2.996959130551137</v>
       </c>
       <c r="V49" t="inlineStr"/>
     </row>

</xml_diff>

<commit_message>
DATA. Actualizo predicciones de hoy
</commit_message>
<xml_diff>
--- a/data/predicciones.xlsx
+++ b/data/predicciones.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AJ4"/>
+  <dimension ref="A1:AA4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -465,288 +465,222 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>competition</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
           <t>odds_home</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>odds_draw</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>odds_away</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>prob_home_bm</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>prob_draw_bm</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>prob_away_bm</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>overround</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>predicted_result</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>prob_class_0</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>prob_class_1</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
-        <is>
-          <t>prob_class_0</t>
-        </is>
-      </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>prob_class_2</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
-        <is>
-          <t>copiado_formaciones</t>
-        </is>
-      </c>
-      <c r="S1" s="1" t="inlineStr">
-        <is>
-          <t>dif_prob_mod_bm</t>
-        </is>
-      </c>
       <c r="T1" s="1" t="inlineStr">
         <is>
+          <t>emergency_fill</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>player_emergency_fill</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
           <t>result_to_bet</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
-        <is>
-          <t>dif_prob_result_to_bet</t>
-        </is>
-      </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>prob_result_to_bet</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>odd_to_bet</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>strategy</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
-        <is>
-          <t>multiplier</t>
-        </is>
-      </c>
       <c r="Z1" s="1" t="inlineStr">
         <is>
+          <t>stake_to_bet_norm</t>
+        </is>
+      </c>
+      <c r="AA1" s="1" t="inlineStr">
+        <is>
           <t>stake_to_bet</t>
-        </is>
-      </c>
-      <c r="AA1" s="1" t="inlineStr">
-        <is>
-          <t>country</t>
-        </is>
-      </c>
-      <c r="AB1" s="1" t="inlineStr">
-        <is>
-          <t>competition</t>
-        </is>
-      </c>
-      <c r="AC1" s="1" t="inlineStr">
-        <is>
-          <t>emergency_fill</t>
-        </is>
-      </c>
-      <c r="AD1" s="1" t="inlineStr">
-        <is>
-          <t>stake_to_bet_raw</t>
-        </is>
-      </c>
-      <c r="AE1" s="1" t="inlineStr">
-        <is>
-          <t>stake_to_bet_norm</t>
-        </is>
-      </c>
-      <c r="AF1" s="1" t="inlineStr">
-        <is>
-          <t>player_emergency_fill</t>
-        </is>
-      </c>
-      <c r="AG1" s="1" t="inlineStr">
-        <is>
-          <t>goals_home</t>
-        </is>
-      </c>
-      <c r="AH1" s="1" t="inlineStr">
-        <is>
-          <t>goals_away</t>
-        </is>
-      </c>
-      <c r="AI1" s="1" t="inlineStr">
-        <is>
-          <t>result</t>
-        </is>
-      </c>
-      <c r="AJ1" s="1" t="inlineStr">
-        <is>
-          <t>acerte</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>naF5yLBL</t>
+          <t>4jKwEvHt</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>45684.60416666666</v>
+        <v>45691.70833333334</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>venezia</t>
+          <t>chelsea</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>verona</t>
+          <t>west ham</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>77</v>
+        <v>48</v>
       </c>
       <c r="F2" t="n">
-        <v>771</v>
-      </c>
-      <c r="G2" t="n">
-        <v>2.25</v>
-      </c>
-      <c r="H2" t="n">
-        <v>3.3</v>
+        <v>481</v>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>premier league</t>
+        </is>
       </c>
       <c r="I2" t="n">
-        <v>3.25</v>
+        <v>1.27</v>
       </c>
       <c r="J2" t="n">
-        <v>0.4212076583210604</v>
+        <v>6</v>
       </c>
       <c r="K2" t="n">
-        <v>0.2871870397643594</v>
+        <v>9.5</v>
       </c>
       <c r="L2" t="n">
-        <v>0.2916053019145803</v>
+        <v>0.7433005150942166</v>
       </c>
       <c r="M2" t="n">
-        <v>0.05516705516705511</v>
+        <v>0.1573319423616092</v>
       </c>
       <c r="N2" t="n">
+        <v>0.09936754254417422</v>
+      </c>
+      <c r="O2" t="n">
+        <v>0.05933139936455301</v>
+      </c>
+      <c r="P2" t="n">
         <v>1</v>
       </c>
-      <c r="O2" t="n">
-        <v>0.6092537396176542</v>
-      </c>
-      <c r="P2" t="n">
-        <v>0.05161499313746432</v>
-      </c>
       <c r="Q2" t="n">
-        <v>0.3391312672448816</v>
+        <v>0.3962971088735305</v>
       </c>
       <c r="R2" t="n">
+        <v>0.5248593512890527</v>
+      </c>
+      <c r="S2" t="n">
+        <v>0.07884353983741681</v>
+      </c>
+      <c r="T2" t="n">
+        <v>0</v>
+      </c>
+      <c r="U2" t="n">
+        <v>0</v>
+      </c>
+      <c r="V2" t="n">
         <v>1</v>
       </c>
-      <c r="S2" t="n">
-        <v>0.1880460812965938</v>
-      </c>
-      <c r="T2" t="n">
-        <v>1</v>
-      </c>
-      <c r="U2" t="n">
-        <v>0.1880460812965938</v>
-      </c>
-      <c r="V2" t="n">
-        <v>0.6092537396176542</v>
-      </c>
       <c r="W2" t="n">
-        <v>2.25</v>
-      </c>
-      <c r="X2" t="inlineStr">
-        <is>
-          <t>dif_prob_mod_bm &gt; -1</t>
-        </is>
-      </c>
-      <c r="Y2" t="inlineStr"/>
+        <v>0.5248593512890527</v>
+      </c>
+      <c r="X2" t="n">
+        <v>1.27</v>
+      </c>
+      <c r="Y2" t="inlineStr">
+        <is>
+          <t>dif_prob_mod_bm &gt; 0</t>
+        </is>
+      </c>
       <c r="Z2" t="n">
-        <v>1.246696053880533</v>
-      </c>
-      <c r="AA2" t="inlineStr">
-        <is>
-          <t>italy</t>
-        </is>
-      </c>
-      <c r="AB2" t="inlineStr">
-        <is>
-          <t>serie a</t>
-        </is>
-      </c>
-      <c r="AC2" t="inlineStr"/>
-      <c r="AD2" t="inlineStr"/>
-      <c r="AE2" t="n">
-        <v>5.93313462623555</v>
-      </c>
-      <c r="AF2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG2" t="n">
-        <v>1</v>
-      </c>
-      <c r="AH2" t="n">
-        <v>1</v>
-      </c>
-      <c r="AI2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ2" t="n">
-        <v>0</v>
+        <v>-12.34920829121863</v>
+      </c>
+      <c r="AA2" t="n">
+        <v>6.499745626041516e-06</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>x4MK4Mzp</t>
+          <t>l2ICn6yK</t>
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>45684.69791666666</v>
+        <v>45691.69791666666</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>genoa</t>
+          <t>cagliari</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>monza</t>
+          <t>lazio</t>
         </is>
       </c>
       <c r="E3" t="n">
@@ -755,114 +689,93 @@
       <c r="F3" t="n">
         <v>771</v>
       </c>
-      <c r="G3" t="n">
-        <v>2.25</v>
-      </c>
-      <c r="H3" t="n">
-        <v>3</v>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>italy</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>serie a</t>
+        </is>
       </c>
       <c r="I3" t="n">
-        <v>3.6</v>
+        <v>3.9</v>
       </c>
       <c r="J3" t="n">
-        <v>0.4210526315789474</v>
+        <v>3.4</v>
       </c>
       <c r="K3" t="n">
-        <v>0.3157894736842106</v>
+        <v>1.95</v>
       </c>
       <c r="L3" t="n">
-        <v>0.2631578947368421</v>
+        <v>0.2411347517730496</v>
       </c>
       <c r="M3" t="n">
-        <v>0.05555555555555536</v>
+        <v>0.276595744680851</v>
       </c>
       <c r="N3" t="n">
-        <v>0</v>
+        <v>0.4822695035460993</v>
       </c>
       <c r="O3" t="n">
-        <v>0.3533479698795551</v>
+        <v>0.06334841628959298</v>
       </c>
       <c r="P3" t="n">
-        <v>0.5659316602521656</v>
+        <v>2</v>
       </c>
       <c r="Q3" t="n">
-        <v>0.08072036986827937</v>
+        <v>0.2512422669571432</v>
       </c>
       <c r="R3" t="n">
-        <v>1</v>
+        <v>0.1671251957957098</v>
       </c>
       <c r="S3" t="n">
-        <v>0.250142186567955</v>
+        <v>0.581632537247147</v>
       </c>
       <c r="T3" t="n">
         <v>0</v>
       </c>
       <c r="U3" t="n">
-        <v>0.250142186567955</v>
+        <v>0</v>
       </c>
       <c r="V3" t="n">
-        <v>0.5659316602521656</v>
+        <v>2</v>
       </c>
       <c r="W3" t="n">
-        <v>3</v>
-      </c>
-      <c r="X3" t="inlineStr">
-        <is>
-          <t>dif_prob_mod_bm &gt; -1</t>
-        </is>
-      </c>
-      <c r="Y3" t="inlineStr"/>
+        <v>0.581632537247147</v>
+      </c>
+      <c r="X3" t="n">
+        <v>1.95</v>
+      </c>
+      <c r="Y3" t="inlineStr">
+        <is>
+          <t>dif_prob_mod_bm &gt; 0</t>
+        </is>
+      </c>
       <c r="Z3" t="n">
-        <v>5.009269683463181</v>
-      </c>
-      <c r="AA3" t="inlineStr">
-        <is>
-          <t>italy</t>
-        </is>
-      </c>
-      <c r="AB3" t="inlineStr">
-        <is>
-          <t>serie a</t>
-        </is>
-      </c>
-      <c r="AC3" t="inlineStr"/>
-      <c r="AD3" t="inlineStr"/>
-      <c r="AE3" t="n">
-        <v>1.395589961512993</v>
-      </c>
-      <c r="AF3" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG3" t="n">
-        <v>2</v>
-      </c>
-      <c r="AH3" t="n">
-        <v>0</v>
-      </c>
-      <c r="AI3" t="n">
-        <v>1</v>
-      </c>
-      <c r="AJ3" t="n">
-        <v>0</v>
+        <v>0.2017796204991529</v>
+      </c>
+      <c r="AA3" t="n">
+        <v>5.777881658867424</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>4QK5Q8Mk</t>
+          <t>SM0qnskQ</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>45684.70833333334</v>
+        <v>45691.70833333334</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>alaves</t>
+          <t>girona</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>celta vigo</t>
+          <t>las palmas</t>
         </is>
       </c>
       <c r="E4" t="n">
@@ -871,93 +784,74 @@
       <c r="F4" t="n">
         <v>1481</v>
       </c>
-      <c r="G4" t="n">
-        <v>2.45</v>
-      </c>
-      <c r="H4" t="n">
-        <v>3.1</v>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>spain</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>laliga</t>
+        </is>
       </c>
       <c r="I4" t="n">
-        <v>3.1</v>
+        <v>1.48</v>
       </c>
       <c r="J4" t="n">
-        <v>0.3875</v>
+        <v>4.5</v>
       </c>
       <c r="K4" t="n">
-        <v>0.30625</v>
+        <v>6.25</v>
       </c>
       <c r="L4" t="n">
-        <v>0.30625</v>
+        <v>0.6386964914272737</v>
       </c>
       <c r="M4" t="n">
-        <v>0.05332455562870297</v>
+        <v>0.2100601794027478</v>
       </c>
       <c r="N4" t="n">
+        <v>0.1512433291699784</v>
+      </c>
+      <c r="O4" t="n">
+        <v>0.0578978978978979</v>
+      </c>
+      <c r="P4" t="n">
         <v>1</v>
       </c>
-      <c r="O4" t="n">
-        <v>0.6643119815334537</v>
-      </c>
-      <c r="P4" t="n">
-        <v>0.07538113895966174</v>
-      </c>
       <c r="Q4" t="n">
-        <v>0.2603068795068844</v>
+        <v>0.1594260529204714</v>
       </c>
       <c r="R4" t="n">
+        <v>0.799605481879446</v>
+      </c>
+      <c r="S4" t="n">
+        <v>0.04096846520008246</v>
+      </c>
+      <c r="T4" t="n">
+        <v>0</v>
+      </c>
+      <c r="U4" t="n">
+        <v>0</v>
+      </c>
+      <c r="V4" t="n">
         <v>1</v>
       </c>
-      <c r="S4" t="n">
-        <v>0.2768119815334537</v>
-      </c>
-      <c r="T4" t="n">
-        <v>1</v>
-      </c>
-      <c r="U4" t="n">
-        <v>0.2768119815334537</v>
-      </c>
-      <c r="V4" t="n">
-        <v>0.6643119815334537</v>
-      </c>
       <c r="W4" t="n">
-        <v>2.45</v>
-      </c>
-      <c r="X4" t="inlineStr">
-        <is>
-          <t>dif_prob_mod_bm &gt; -1</t>
-        </is>
-      </c>
-      <c r="Y4" t="inlineStr"/>
+        <v>0.799605481879446</v>
+      </c>
+      <c r="X4" t="n">
+        <v>1.48</v>
+      </c>
+      <c r="Y4" t="inlineStr">
+        <is>
+          <t>dif_prob_mod_bm &gt; 0</t>
+        </is>
+      </c>
       <c r="Z4" t="n">
-        <v>8.797882219317488</v>
-      </c>
-      <c r="AA4" t="inlineStr">
-        <is>
-          <t>spain</t>
-        </is>
-      </c>
-      <c r="AB4" t="inlineStr">
-        <is>
-          <t>laliga</t>
-        </is>
-      </c>
-      <c r="AC4" t="inlineStr"/>
-      <c r="AD4" t="inlineStr"/>
-      <c r="AE4" t="n">
-        <v>0.8656060065613264</v>
-      </c>
-      <c r="AF4" t="inlineStr"/>
-      <c r="AG4" t="n">
-        <v>1</v>
-      </c>
-      <c r="AH4" t="n">
-        <v>1</v>
-      </c>
-      <c r="AI4" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ4" t="n">
-        <v>0</v>
+        <v>1.528467609846501</v>
+      </c>
+      <c r="AA4" t="n">
+        <v>3.081682487265471</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Implemento confidence margin para reducir stake
</commit_message>
<xml_diff>
--- a/data/predicciones.xlsx
+++ b/data/predicciones.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB89"/>
+  <dimension ref="A1:AC89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -570,6 +570,11 @@
       </c>
       <c r="AB1" s="1" t="inlineStr">
         <is>
+          <t>confidence_margin</t>
+        </is>
+      </c>
+      <c r="AC1" s="1" t="inlineStr">
+        <is>
           <t>emergency_fill</t>
         </is>
       </c>
@@ -668,7 +673,10 @@
       <c r="AA2" t="n">
         <v>0.001153815536812339</v>
       </c>
-      <c r="AB2" t="inlineStr"/>
+      <c r="AB2" t="n">
+        <v>0.04739399106741832</v>
+      </c>
+      <c r="AC2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
@@ -764,7 +772,10 @@
       <c r="AA3" t="n">
         <v>1.893781670897427</v>
       </c>
-      <c r="AB3" t="inlineStr"/>
+      <c r="AB3" t="n">
+        <v>0.3840986447075839</v>
+      </c>
+      <c r="AC3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
@@ -860,7 +871,10 @@
       <c r="AA4" t="n">
         <v>0.322222202459801</v>
       </c>
-      <c r="AB4" t="inlineStr"/>
+      <c r="AB4" t="n">
+        <v>0.1398580131832268</v>
+      </c>
+      <c r="AC4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
@@ -956,7 +970,10 @@
       <c r="AA5" t="n">
         <v>1.693046095251164e-08</v>
       </c>
-      <c r="AB5" t="inlineStr"/>
+      <c r="AB5" t="n">
+        <v>0.1836421670714946</v>
+      </c>
+      <c r="AC5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
@@ -1052,7 +1069,10 @@
       <c r="AA6" t="n">
         <v>4.456486113343987</v>
       </c>
-      <c r="AB6" t="inlineStr"/>
+      <c r="AB6" t="n">
+        <v>0.344333265187366</v>
+      </c>
+      <c r="AC6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
@@ -1148,7 +1168,10 @@
       <c r="AA7" t="n">
         <v>4.203783139294571</v>
       </c>
-      <c r="AB7" t="inlineStr"/>
+      <c r="AB7" t="n">
+        <v>0.3287829378998133</v>
+      </c>
+      <c r="AC7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
@@ -1244,7 +1267,10 @@
       <c r="AA8" t="n">
         <v>4.214080334861166</v>
       </c>
-      <c r="AB8" t="inlineStr"/>
+      <c r="AB8" t="n">
+        <v>0.6864390532340492</v>
+      </c>
+      <c r="AC8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
@@ -1340,7 +1366,10 @@
       <c r="AA9" t="n">
         <v>3.67479008397232</v>
       </c>
-      <c r="AB9" t="inlineStr"/>
+      <c r="AB9" t="n">
+        <v>0.3759548073306545</v>
+      </c>
+      <c r="AC9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
@@ -1436,7 +1465,10 @@
       <c r="AA10" t="n">
         <v>4.709663371809698</v>
       </c>
-      <c r="AB10" t="inlineStr"/>
+      <c r="AB10" t="n">
+        <v>0.8967353439609921</v>
+      </c>
+      <c r="AC10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
@@ -1532,7 +1564,10 @@
       <c r="AA11" t="n">
         <v>3.075449472421982</v>
       </c>
-      <c r="AB11" t="inlineStr"/>
+      <c r="AB11" t="n">
+        <v>0.0727872966680122</v>
+      </c>
+      <c r="AC11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
@@ -1628,7 +1663,10 @@
       <c r="AA12" t="n">
         <v>4.185215740740377</v>
       </c>
-      <c r="AB12" t="inlineStr"/>
+      <c r="AB12" t="n">
+        <v>0.6588596547270916</v>
+      </c>
+      <c r="AC12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
@@ -1722,7 +1760,10 @@
       <c r="AA13" t="n">
         <v>4.024464115468177</v>
       </c>
-      <c r="AB13" t="inlineStr"/>
+      <c r="AB13" t="n">
+        <v>0.2065276283160786</v>
+      </c>
+      <c r="AC13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="1" t="inlineStr">
@@ -1816,7 +1857,10 @@
       <c r="AA14" t="n">
         <v>4.308776551846192</v>
       </c>
-      <c r="AB14" t="inlineStr"/>
+      <c r="AB14" t="n">
+        <v>0.3022503153312382</v>
+      </c>
+      <c r="AC14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="1" t="inlineStr">
@@ -1910,7 +1954,10 @@
       <c r="AA15" t="n">
         <v>6.058131467828698</v>
       </c>
-      <c r="AB15" t="inlineStr"/>
+      <c r="AB15" t="n">
+        <v>0.2088091826260769</v>
+      </c>
+      <c r="AC15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="1" t="inlineStr">
@@ -2004,7 +2051,10 @@
       <c r="AA16" t="n">
         <v>5.938045786257184</v>
       </c>
-      <c r="AB16" t="inlineStr"/>
+      <c r="AB16" t="n">
+        <v>0.5316578045577145</v>
+      </c>
+      <c r="AC16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="1" t="inlineStr">
@@ -2098,7 +2148,10 @@
       <c r="AA17" t="n">
         <v>3.654077475858244</v>
       </c>
-      <c r="AB17" t="inlineStr"/>
+      <c r="AB17" t="n">
+        <v>0.07276222977905428</v>
+      </c>
+      <c r="AC17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="1" t="inlineStr">
@@ -2193,6 +2246,9 @@
         <v>1.907621972554927</v>
       </c>
       <c r="AB18" t="n">
+        <v>0.1175577117584464</v>
+      </c>
+      <c r="AC18" t="n">
         <v>1</v>
       </c>
     </row>
@@ -2286,7 +2342,10 @@
       <c r="AA19" t="n">
         <v>3.745819582914672</v>
       </c>
-      <c r="AB19" t="inlineStr"/>
+      <c r="AB19" t="n">
+        <v>0.09944157160786871</v>
+      </c>
+      <c r="AC19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="1" t="inlineStr">
@@ -2376,9 +2435,12 @@
       </c>
       <c r="Z20" t="inlineStr"/>
       <c r="AA20" t="n">
-        <v>3.260203952854438</v>
-      </c>
-      <c r="AB20" t="inlineStr"/>
+        <v>1.630101976427219</v>
+      </c>
+      <c r="AB20" t="n">
+        <v>0.03275822224089703</v>
+      </c>
+      <c r="AC20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="1" t="inlineStr">
@@ -2468,9 +2530,12 @@
       </c>
       <c r="Z21" t="inlineStr"/>
       <c r="AA21" t="n">
-        <v>3.335525123858694</v>
-      </c>
-      <c r="AB21" t="inlineStr"/>
+        <v>1.667762561929347</v>
+      </c>
+      <c r="AB21" t="n">
+        <v>0.02988649267859894</v>
+      </c>
+      <c r="AC21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="1" t="inlineStr">
@@ -2560,9 +2625,12 @@
       </c>
       <c r="Z22" t="inlineStr"/>
       <c r="AA22" t="n">
-        <v>3.745116632097411</v>
-      </c>
-      <c r="AB22" t="inlineStr"/>
+        <v>1.872558316048706</v>
+      </c>
+      <c r="AB22" t="n">
+        <v>0.01991824472635378</v>
+      </c>
+      <c r="AC22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="1" t="inlineStr">
@@ -2652,9 +2720,12 @@
       </c>
       <c r="Z23" t="inlineStr"/>
       <c r="AA23" t="n">
-        <v>3.414565772954691</v>
-      </c>
-      <c r="AB23" t="inlineStr"/>
+        <v>1.707282886477346</v>
+      </c>
+      <c r="AB23" t="n">
+        <v>0.02568562588552958</v>
+      </c>
+      <c r="AC23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="1" t="inlineStr">
@@ -2746,7 +2817,10 @@
       <c r="AA24" t="n">
         <v>3.525033506130931</v>
       </c>
-      <c r="AB24" t="inlineStr"/>
+      <c r="AB24" t="n">
+        <v>0.05514727402796771</v>
+      </c>
+      <c r="AC24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="1" t="inlineStr">
@@ -2838,7 +2912,10 @@
       <c r="AA25" t="n">
         <v>3.529352481517327</v>
       </c>
-      <c r="AB25" t="inlineStr"/>
+      <c r="AB25" t="n">
+        <v>0.05495969570996473</v>
+      </c>
+      <c r="AC25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="1" t="inlineStr">
@@ -2930,9 +3007,12 @@
         <v>0.1468910992396839</v>
       </c>
       <c r="AA26" t="n">
-        <v>4.829911977416</v>
-      </c>
-      <c r="AB26" t="inlineStr"/>
+        <v>2.414955988708</v>
+      </c>
+      <c r="AB26" t="n">
+        <v>0.02618277786977469</v>
+      </c>
+      <c r="AC26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="1" t="inlineStr">
@@ -3026,7 +3106,10 @@
       <c r="AA27" t="n">
         <v>4.377883209287183</v>
       </c>
-      <c r="AB27" t="inlineStr"/>
+      <c r="AB27" t="n">
+        <v>0.3046702214957177</v>
+      </c>
+      <c r="AC27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="1" t="inlineStr">
@@ -3120,7 +3203,10 @@
       <c r="AA28" t="n">
         <v>5.128625940817812</v>
       </c>
-      <c r="AB28" t="inlineStr"/>
+      <c r="AB28" t="n">
+        <v>0.4481904272743403</v>
+      </c>
+      <c r="AC28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="1" t="inlineStr">
@@ -3214,7 +3300,10 @@
       <c r="AA29" t="n">
         <v>3.757712423739184</v>
       </c>
-      <c r="AB29" t="inlineStr"/>
+      <c r="AB29" t="n">
+        <v>0.1167194917476921</v>
+      </c>
+      <c r="AC29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="1" t="inlineStr">
@@ -3311,6 +3400,9 @@
         <v>1.446245488850359</v>
       </c>
       <c r="AB30" t="n">
+        <v>0.1203795706039189</v>
+      </c>
+      <c r="AC30" t="n">
         <v>1</v>
       </c>
     </row>
@@ -3404,7 +3496,10 @@
       <c r="AA31" t="n">
         <v>6.14309299853371</v>
       </c>
-      <c r="AB31" t="inlineStr"/>
+      <c r="AB31" t="n">
+        <v>0.04286165855675528</v>
+      </c>
+      <c r="AC31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="1" t="inlineStr">
@@ -3496,7 +3591,10 @@
       <c r="AA32" t="n">
         <v>8.071509901586692</v>
       </c>
-      <c r="AB32" t="inlineStr"/>
+      <c r="AB32" t="n">
+        <v>0.3523654310567055</v>
+      </c>
+      <c r="AC32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="1" t="inlineStr">
@@ -3586,9 +3684,12 @@
       </c>
       <c r="Z33" t="inlineStr"/>
       <c r="AA33" t="n">
-        <v>4.791599181696074</v>
-      </c>
-      <c r="AB33" t="inlineStr"/>
+        <v>2.395799590848037</v>
+      </c>
+      <c r="AB33" t="n">
+        <v>0.01102603632254179</v>
+      </c>
+      <c r="AC33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="1" t="inlineStr">
@@ -3680,7 +3781,10 @@
       <c r="AA34" t="n">
         <v>6.663040937112079</v>
       </c>
-      <c r="AB34" t="inlineStr"/>
+      <c r="AB34" t="n">
+        <v>0.1725023485304856</v>
+      </c>
+      <c r="AC34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="1" t="inlineStr">
@@ -3772,7 +3876,10 @@
       <c r="AA35" t="n">
         <v>7.806381476950278</v>
       </c>
-      <c r="AB35" t="inlineStr"/>
+      <c r="AB35" t="n">
+        <v>0.1857830188687544</v>
+      </c>
+      <c r="AC35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="1" t="inlineStr">
@@ -3864,7 +3971,10 @@
       <c r="AA36" t="n">
         <v>7.092999455326837</v>
       </c>
-      <c r="AB36" t="inlineStr"/>
+      <c r="AB36" t="n">
+        <v>0.2498012752252686</v>
+      </c>
+      <c r="AC36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="1" t="inlineStr">
@@ -3959,6 +4069,9 @@
         <v>6.98729004271098</v>
       </c>
       <c r="AB37" t="n">
+        <v>0.1019598298993324</v>
+      </c>
+      <c r="AC37" t="n">
         <v>1</v>
       </c>
     </row>
@@ -4054,9 +4167,12 @@
         <v>0.6041089623766995</v>
       </c>
       <c r="AA38" t="n">
-        <v>9.052341318324899</v>
+        <v>4.52617065916245</v>
       </c>
       <c r="AB38" t="n">
+        <v>0.003079309257606078</v>
+      </c>
+      <c r="AC38" t="n">
         <v>1</v>
       </c>
     </row>
@@ -4152,7 +4268,10 @@
       <c r="AA39" t="n">
         <v>8.434124899354602</v>
       </c>
-      <c r="AB39" t="inlineStr"/>
+      <c r="AB39" t="n">
+        <v>0.1338894598759931</v>
+      </c>
+      <c r="AC39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="1" t="inlineStr">
@@ -4249,6 +4368,9 @@
         <v>8.213699756746221</v>
       </c>
       <c r="AB40" t="n">
+        <v>0.1286204132324692</v>
+      </c>
+      <c r="AC40" t="n">
         <v>1</v>
       </c>
     </row>
@@ -4342,7 +4464,10 @@
       <c r="AA41" t="n">
         <v>0.9857115367123752</v>
       </c>
-      <c r="AB41" t="inlineStr"/>
+      <c r="AB41" t="n">
+        <v>0.1888285091574472</v>
+      </c>
+      <c r="AC41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="1" t="inlineStr">
@@ -4437,6 +4562,9 @@
         <v>0.9497774713863081</v>
       </c>
       <c r="AB42" t="n">
+        <v>0.1916241544298661</v>
+      </c>
+      <c r="AC42" t="n">
         <v>1</v>
       </c>
     </row>
@@ -4530,7 +4658,10 @@
       <c r="AA43" t="n">
         <v>1.055695608931322</v>
       </c>
-      <c r="AB43" t="inlineStr"/>
+      <c r="AB43" t="n">
+        <v>0.2406531231595041</v>
+      </c>
+      <c r="AC43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="1" t="inlineStr">
@@ -4622,7 +4753,10 @@
       <c r="AA44" t="n">
         <v>1.26783054470622</v>
       </c>
-      <c r="AB44" t="inlineStr"/>
+      <c r="AB44" t="n">
+        <v>0.4157541526964347</v>
+      </c>
+      <c r="AC44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="1" t="inlineStr">
@@ -4717,6 +4851,9 @@
         <v>0.8433126929150305</v>
       </c>
       <c r="AB45" t="n">
+        <v>0.09986882768076272</v>
+      </c>
+      <c r="AC45" t="n">
         <v>1</v>
       </c>
     </row>
@@ -4808,9 +4945,12 @@
       </c>
       <c r="Z46" t="inlineStr"/>
       <c r="AA46" t="n">
-        <v>0.7880650016377873</v>
-      </c>
-      <c r="AB46" t="inlineStr"/>
+        <v>0.3940325008188936</v>
+      </c>
+      <c r="AB46" t="n">
+        <v>0.007030051479937627</v>
+      </c>
+      <c r="AC46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="1" t="inlineStr">
@@ -4905,6 +5045,9 @@
         <v>1.343606420523692</v>
       </c>
       <c r="AB47" t="n">
+        <v>0.4786781698874154</v>
+      </c>
+      <c r="AC47" t="n">
         <v>1</v>
       </c>
     </row>
@@ -4998,7 +5141,10 @@
       <c r="AA48" t="n">
         <v>1.175419958348716</v>
       </c>
-      <c r="AB48" t="inlineStr"/>
+      <c r="AB48" t="n">
+        <v>0.3304115501055636</v>
+      </c>
+      <c r="AC48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="1" t="inlineStr">
@@ -5090,7 +5236,10 @@
       <c r="AA49" t="n">
         <v>1.009369660159489</v>
       </c>
-      <c r="AB49" t="inlineStr"/>
+      <c r="AB49" t="n">
+        <v>0.2284610346034467</v>
+      </c>
+      <c r="AC49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" s="1" t="inlineStr">
@@ -5182,9 +5331,12 @@
       </c>
       <c r="Z50" t="inlineStr"/>
       <c r="AA50" t="n">
-        <v>0.7329301112951311</v>
+        <v>0.3664650556475655</v>
       </c>
       <c r="AB50" t="n">
+        <v>0.03858349265106414</v>
+      </c>
+      <c r="AC50" t="n">
         <v>1</v>
       </c>
     </row>
@@ -5278,7 +5430,10 @@
       <c r="AA51" t="n">
         <v>1.100214238098028</v>
       </c>
-      <c r="AB51" t="inlineStr"/>
+      <c r="AB51" t="n">
+        <v>0.1841797636677216</v>
+      </c>
+      <c r="AC51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" s="1" t="inlineStr">
@@ -5370,7 +5525,10 @@
       <c r="AA52" t="n">
         <v>1.136273333920035</v>
       </c>
-      <c r="AB52" t="inlineStr"/>
+      <c r="AB52" t="n">
+        <v>0.2173559887379316</v>
+      </c>
+      <c r="AC52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" s="1" t="inlineStr">
@@ -5462,7 +5620,10 @@
       <c r="AA53" t="n">
         <v>1.19585549085631</v>
       </c>
-      <c r="AB53" t="inlineStr"/>
+      <c r="AB53" t="n">
+        <v>0.3082577304308737</v>
+      </c>
+      <c r="AC53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" s="1" t="inlineStr">
@@ -5552,9 +5713,12 @@
       </c>
       <c r="Z54" t="inlineStr"/>
       <c r="AA54" t="n">
-        <v>0.8176190933636504</v>
-      </c>
-      <c r="AB54" t="inlineStr"/>
+        <v>0.4088095466818252</v>
+      </c>
+      <c r="AB54" t="n">
+        <v>0.004211885545910954</v>
+      </c>
+      <c r="AC54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" s="1" t="inlineStr">
@@ -5649,6 +5813,9 @@
         <v>1.316681699296524</v>
       </c>
       <c r="AB55" t="n">
+        <v>0.4188949621484066</v>
+      </c>
+      <c r="AC55" t="n">
         <v>1</v>
       </c>
     </row>
@@ -5742,7 +5909,10 @@
       <c r="AA56" t="n">
         <v>1.467509396340491</v>
       </c>
-      <c r="AB56" t="inlineStr"/>
+      <c r="AB56" t="n">
+        <v>0.5167217662095852</v>
+      </c>
+      <c r="AC56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" s="1" t="inlineStr">
@@ -5834,7 +6004,10 @@
       <c r="AA57" t="n">
         <v>0.7554969442250973</v>
       </c>
-      <c r="AB57" t="inlineStr"/>
+      <c r="AB57" t="n">
+        <v>0.06289816886392008</v>
+      </c>
+      <c r="AC57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" s="1" t="inlineStr">
@@ -5929,6 +6102,9 @@
         <v>0.8217981355669157</v>
       </c>
       <c r="AB58" t="n">
+        <v>0.1149948504934717</v>
+      </c>
+      <c r="AC58" t="n">
         <v>1</v>
       </c>
     </row>
@@ -6022,7 +6198,10 @@
       <c r="AA59" t="n">
         <v>7.126122852967393</v>
       </c>
-      <c r="AB59" t="inlineStr"/>
+      <c r="AB59" t="n">
+        <v>0.1436601204833214</v>
+      </c>
+      <c r="AC59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" s="1" t="inlineStr">
@@ -6114,9 +6293,12 @@
       </c>
       <c r="Z60" t="inlineStr"/>
       <c r="AA60" t="n">
-        <v>5.988241527132366</v>
+        <v>2.994120763566183</v>
       </c>
       <c r="AB60" t="n">
+        <v>0.03515639146839616</v>
+      </c>
+      <c r="AC60" t="n">
         <v>1</v>
       </c>
     </row>
@@ -6210,7 +6392,10 @@
       <c r="AA61" t="n">
         <v>5.722526903863123</v>
       </c>
-      <c r="AB61" t="inlineStr"/>
+      <c r="AB61" t="n">
+        <v>0.07949695818623725</v>
+      </c>
+      <c r="AC61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" s="1" t="inlineStr">
@@ -6300,7 +6485,10 @@
       <c r="AA62" t="n">
         <v>7.29254395462817</v>
       </c>
-      <c r="AB62" t="inlineStr"/>
+      <c r="AB62" t="n">
+        <v>0.1598932690320206</v>
+      </c>
+      <c r="AC62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" s="1" t="inlineStr">
@@ -6395,6 +6583,9 @@
         <v>7.191938260573733</v>
       </c>
       <c r="AB63" t="n">
+        <v>0.1780484937096538</v>
+      </c>
+      <c r="AC63" t="n">
         <v>1</v>
       </c>
     </row>
@@ -6488,7 +6679,10 @@
       <c r="AA64" t="n">
         <v>8.645145336236181</v>
       </c>
-      <c r="AB64" t="inlineStr"/>
+      <c r="AB64" t="n">
+        <v>0.3343877386775617</v>
+      </c>
+      <c r="AC64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" s="1" t="inlineStr">
@@ -6580,7 +6774,10 @@
       <c r="AA65" t="n">
         <v>10.8569910490829</v>
       </c>
-      <c r="AB65" t="inlineStr"/>
+      <c r="AB65" t="n">
+        <v>0.5855163992448831</v>
+      </c>
+      <c r="AC65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" s="1" t="inlineStr">
@@ -6675,6 +6872,9 @@
         <v>10.38265882314563</v>
       </c>
       <c r="AB66" t="n">
+        <v>0.5411081969932081</v>
+      </c>
+      <c r="AC66" t="n">
         <v>1</v>
       </c>
     </row>
@@ -6768,9 +6968,12 @@
       </c>
       <c r="Z67" t="inlineStr"/>
       <c r="AA67" t="n">
-        <v>5.432198824584218</v>
+        <v>2.716099412292109</v>
       </c>
       <c r="AB67" t="n">
+        <v>0.02872480205979389</v>
+      </c>
+      <c r="AC67" t="n">
         <v>1</v>
       </c>
     </row>
@@ -6867,6 +7070,9 @@
         <v>9.495637944807504</v>
       </c>
       <c r="AB68" t="n">
+        <v>0.4294602774798805</v>
+      </c>
+      <c r="AC68" t="n">
         <v>1</v>
       </c>
     </row>
@@ -6960,7 +7166,10 @@
       <c r="AA69" t="n">
         <v>8.365756091331638</v>
       </c>
-      <c r="AB69" t="inlineStr"/>
+      <c r="AB69" t="n">
+        <v>0.3126353600010882</v>
+      </c>
+      <c r="AC69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" s="1" t="inlineStr">
@@ -7054,7 +7263,10 @@
       <c r="AA70" t="n">
         <v>6.850604237393622</v>
       </c>
-      <c r="AB70" t="inlineStr"/>
+      <c r="AB70" t="n">
+        <v>0.7499592604555554</v>
+      </c>
+      <c r="AC70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" s="1" t="inlineStr">
@@ -7148,7 +7360,10 @@
       <c r="AA71" t="n">
         <v>6.294073634614914</v>
       </c>
-      <c r="AB71" t="inlineStr"/>
+      <c r="AB71" t="n">
+        <v>0.6114511325746249</v>
+      </c>
+      <c r="AC71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" s="1" t="inlineStr">
@@ -7242,7 +7457,10 @@
       <c r="AA72" t="n">
         <v>6.662802745980152</v>
       </c>
-      <c r="AB72" t="inlineStr"/>
+      <c r="AB72" t="n">
+        <v>0.4513350771617413</v>
+      </c>
+      <c r="AC72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" s="1" t="inlineStr">
@@ -7339,6 +7557,9 @@
         <v>3.009501009952456</v>
       </c>
       <c r="AB73" t="n">
+        <v>0.07208482282580314</v>
+      </c>
+      <c r="AC73" t="n">
         <v>1</v>
       </c>
     </row>
@@ -7437,6 +7658,9 @@
         <v>5.837388040175599</v>
       </c>
       <c r="AB74" t="n">
+        <v>0.5141998880313108</v>
+      </c>
+      <c r="AC74" t="n">
         <v>1</v>
       </c>
     </row>
@@ -7532,7 +7756,10 @@
       <c r="AA75" t="n">
         <v>5.326103616586976</v>
       </c>
-      <c r="AB75" t="inlineStr"/>
+      <c r="AB75" t="n">
+        <v>0.2128397358289605</v>
+      </c>
+      <c r="AC75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" s="1" t="inlineStr">
@@ -7626,7 +7853,10 @@
       <c r="AA76" t="n">
         <v>6.097866413832848</v>
       </c>
-      <c r="AB76" t="inlineStr"/>
+      <c r="AB76" t="n">
+        <v>0.1482782385130523</v>
+      </c>
+      <c r="AC76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" s="1" t="inlineStr">
@@ -7720,7 +7950,10 @@
       <c r="AA77" t="n">
         <v>7.440718745357945</v>
       </c>
-      <c r="AB77" t="inlineStr"/>
+      <c r="AB77" t="n">
+        <v>0.8193217102436385</v>
+      </c>
+      <c r="AC77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" s="1" t="inlineStr">
@@ -7814,7 +8047,10 @@
       <c r="AA78" t="n">
         <v>6.775917695853008</v>
       </c>
-      <c r="AB78" t="inlineStr"/>
+      <c r="AB78" t="n">
+        <v>0.7293911906558673</v>
+      </c>
+      <c r="AC78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" s="1" t="inlineStr">
@@ -7906,9 +8142,12 @@
         <v>-0.2579277336858381</v>
       </c>
       <c r="AA79" t="n">
-        <v>3.922858666944991</v>
-      </c>
-      <c r="AB79" t="inlineStr"/>
+        <v>1.961429333472495</v>
+      </c>
+      <c r="AB79" t="n">
+        <v>0.004796223392691923</v>
+      </c>
+      <c r="AC79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" s="1" t="inlineStr">
@@ -8002,7 +8241,10 @@
       <c r="AA80" t="n">
         <v>0.2736069009720922</v>
       </c>
-      <c r="AB80" t="inlineStr"/>
+      <c r="AB80" t="n">
+        <v>0.2225271996294316</v>
+      </c>
+      <c r="AC80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" s="1" t="inlineStr">
@@ -8096,7 +8338,10 @@
       <c r="AA81" t="n">
         <v>1.987482302703113</v>
       </c>
-      <c r="AB81" t="inlineStr"/>
+      <c r="AB81" t="n">
+        <v>0.376386018697578</v>
+      </c>
+      <c r="AC81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" s="1" t="inlineStr">
@@ -8190,7 +8435,10 @@
       <c r="AA82" t="n">
         <v>1.99952410403066</v>
       </c>
-      <c r="AB82" t="inlineStr"/>
+      <c r="AB82" t="n">
+        <v>0.7764778193761898</v>
+      </c>
+      <c r="AC82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" s="1" t="inlineStr">
@@ -8284,7 +8532,10 @@
       <c r="AA83" t="n">
         <v>1.984223740197021</v>
       </c>
-      <c r="AB83" t="inlineStr"/>
+      <c r="AB83" t="n">
+        <v>0.3223482974988242</v>
+      </c>
+      <c r="AC83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" s="1" t="inlineStr">
@@ -8381,6 +8632,9 @@
         <v>1.996622685433186</v>
       </c>
       <c r="AB84" t="n">
+        <v>0.5905600426431091</v>
+      </c>
+      <c r="AC84" t="n">
         <v>1</v>
       </c>
     </row>
@@ -8476,7 +8730,10 @@
       <c r="AA85" t="n">
         <v>3.844871118644643</v>
       </c>
-      <c r="AB85" t="inlineStr"/>
+      <c r="AB85" t="n">
+        <v>0.3663856409331741</v>
+      </c>
+      <c r="AC85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" s="1" t="inlineStr">
@@ -8570,7 +8827,10 @@
       <c r="AA86" t="n">
         <v>4.226548707450942</v>
       </c>
-      <c r="AB86" t="inlineStr"/>
+      <c r="AB86" t="n">
+        <v>0.1389396854958488</v>
+      </c>
+      <c r="AC86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" s="1" t="inlineStr">
@@ -8664,7 +8924,10 @@
       <c r="AA87" t="n">
         <v>2.787472602744611</v>
       </c>
-      <c r="AB87" t="inlineStr"/>
+      <c r="AB87" t="n">
+        <v>0.2034832354800955</v>
+      </c>
+      <c r="AC87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" s="1" t="inlineStr">
@@ -8758,7 +9021,10 @@
       <c r="AA88" t="n">
         <v>3.213745823654924</v>
       </c>
-      <c r="AB88" t="inlineStr"/>
+      <c r="AB88" t="n">
+        <v>0.2298610697222075</v>
+      </c>
+      <c r="AC88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" s="1" t="inlineStr">
@@ -8852,7 +9118,10 @@
       <c r="AA89" t="n">
         <v>4.210771241798088</v>
       </c>
-      <c r="AB89" t="inlineStr"/>
+      <c r="AB89" t="n">
+        <v>0.3660938584573002</v>
+      </c>
+      <c r="AC89" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
DATA. Actualizo data desde compu vieja
</commit_message>
<xml_diff>
--- a/data/predicciones.xlsx
+++ b/data/predicciones.xlsx
@@ -433,6 +433,11 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>id_match</t>
+        </is>
+      </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
           <t>date</t>

</xml_diff>

<commit_message>
DATA. Actualizo predicciones para el finde
</commit_message>
<xml_diff>
--- a/data/predicciones.xlsx
+++ b/data/predicciones.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB41"/>
+  <dimension ref="A1:AB39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -530,163 +530,161 @@
       </c>
       <c r="T1" s="1" t="inlineStr">
         <is>
+          <t>copiado_formaciones</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
           <t>emergency_fill</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>player_emergency_fill</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>result_to_bet</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>prob_result_to_bet</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>odd_to_bet</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>strategy</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>stake_to_bet</t>
         </is>
       </c>
-      <c r="AA1" s="1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>confidence_margin</t>
-        </is>
-      </c>
-      <c r="AB1" s="1" t="inlineStr">
-        <is>
-          <t>copiado_formaciones</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>W4vHttEb</t>
+          <t>bHDVry2M</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>45715.70833333334</v>
+        <v>45716.69791666666</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>west ham</t>
+          <t>monaco</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>leicester</t>
+          <t>reims</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>48</v>
+        <v>55</v>
       </c>
       <c r="F2" t="n">
-        <v>481</v>
+        <v>551</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>england</t>
+          <t>france</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>premier league</t>
+          <t>ligue 1</t>
         </is>
       </c>
       <c r="I2" t="n">
-        <v>1.75</v>
+        <v>1.33</v>
       </c>
       <c r="J2" t="n">
-        <v>3.7</v>
+        <v>5</v>
       </c>
       <c r="K2" t="n">
-        <v>4.75</v>
+        <v>8.5</v>
       </c>
       <c r="L2" t="n">
-        <v>0.5430668211664735</v>
+        <v>0.7030022330659168</v>
       </c>
       <c r="M2" t="n">
-        <v>0.2568559289300889</v>
+        <v>0.1869985939955339</v>
       </c>
       <c r="N2" t="n">
-        <v>0.2000772499034376</v>
+        <v>0.1099991729385493</v>
       </c>
       <c r="O2" t="n">
-        <v>0.05222515748831524</v>
+        <v>0.06952675807164965</v>
       </c>
       <c r="P2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q2" t="n">
-        <v>0.4500015250536773</v>
+        <v>0.2906914973789296</v>
       </c>
       <c r="R2" t="n">
-        <v>0.2974169185465333</v>
+        <v>0.5083760831869562</v>
       </c>
       <c r="S2" t="n">
-        <v>0.2525815563997894</v>
+        <v>0.2009324194341142</v>
       </c>
       <c r="T2" t="n">
-        <v>0</v>
-      </c>
-      <c r="U2" t="n">
-        <v>0</v>
-      </c>
-      <c r="V2" t="n">
-        <v>0</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="U2" t="inlineStr"/>
+      <c r="V2" t="inlineStr"/>
       <c r="W2" t="n">
-        <v>0.4500015250536773</v>
+        <v>1</v>
       </c>
       <c r="X2" t="n">
-        <v>3.7</v>
-      </c>
-      <c r="Y2" t="inlineStr">
+        <v>0.5083760831869562</v>
+      </c>
+      <c r="Y2" t="n">
+        <v>1.33</v>
+      </c>
+      <c r="Z2" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0.0</t>
         </is>
       </c>
-      <c r="Z2" t="n">
-        <v>3.150010675375741</v>
-      </c>
       <c r="AA2" t="n">
-        <v>0.152584606507144</v>
-      </c>
-      <c r="AB2" t="inlineStr"/>
+        <v>8.006923310194558</v>
+      </c>
+      <c r="AB2" t="n">
+        <v>0.2176845858080265</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>bHDVry2M</t>
+          <t>UyMEnJ2c</t>
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>45716.69791666666</v>
+        <v>45717.625</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>monaco</t>
+          <t>lens</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>reims</t>
+          <t>le havre</t>
         </is>
       </c>
       <c r="E3" t="n">
@@ -706,81 +704,81 @@
         </is>
       </c>
       <c r="I3" t="n">
-        <v>1.38</v>
+        <v>1.36</v>
       </c>
       <c r="J3" t="n">
         <v>5</v>
       </c>
       <c r="K3" t="n">
-        <v>7.5</v>
+        <v>8</v>
       </c>
       <c r="L3" t="n">
-        <v>0.6849315068493151</v>
+        <v>0.6934812760055478</v>
       </c>
       <c r="M3" t="n">
-        <v>0.189041095890411</v>
+        <v>0.188626907073509</v>
       </c>
       <c r="N3" t="n">
-        <v>0.126027397260274</v>
+        <v>0.1178918169209431</v>
       </c>
       <c r="O3" t="n">
-        <v>0.05797101449275366</v>
+        <v>0.06029411764705883</v>
       </c>
       <c r="P3" t="n">
         <v>1</v>
       </c>
       <c r="Q3" t="n">
-        <v>0.2239099725162628</v>
+        <v>0.4569032670263181</v>
       </c>
       <c r="R3" t="n">
-        <v>0.6134609830555158</v>
+        <v>0.5016828662862088</v>
       </c>
       <c r="S3" t="n">
-        <v>0.1626290444282215</v>
-      </c>
-      <c r="T3" t="inlineStr"/>
+        <v>0.04141386668747317</v>
+      </c>
+      <c r="T3" t="n">
+        <v>1</v>
+      </c>
       <c r="U3" t="inlineStr"/>
-      <c r="V3" t="n">
-        <v>1</v>
-      </c>
+      <c r="V3" t="inlineStr"/>
       <c r="W3" t="n">
-        <v>0.6134609830555158</v>
+        <v>1</v>
       </c>
       <c r="X3" t="n">
-        <v>1.38</v>
-      </c>
-      <c r="Y3" t="inlineStr">
+        <v>0.5016828662862088</v>
+      </c>
+      <c r="Y3" t="n">
+        <v>1.36</v>
+      </c>
+      <c r="Z3" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0.0</t>
         </is>
       </c>
-      <c r="Z3" t="n">
-        <v>8.58845376277722</v>
-      </c>
       <c r="AA3" t="n">
-        <v>0.389551010539253</v>
+        <v>7.901505144007788</v>
       </c>
       <c r="AB3" t="n">
-        <v>1</v>
+        <v>0.04477959925989078</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>UyMEnJ2c</t>
+          <t>f1MVnSdt</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>45717.625</v>
+        <v>45717.71180555555</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>lens</t>
+          <t>psg</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>le havre</t>
+          <t>lille</t>
         </is>
       </c>
       <c r="E4" t="n">
@@ -800,81 +798,81 @@
         </is>
       </c>
       <c r="I4" t="n">
-        <v>1.36</v>
+        <v>1.4</v>
       </c>
       <c r="J4" t="n">
-        <v>5</v>
+        <v>4.75</v>
       </c>
       <c r="K4" t="n">
-        <v>8</v>
+        <v>7.5</v>
       </c>
       <c r="L4" t="n">
-        <v>0.6934812760055478</v>
+        <v>0.6750355281856939</v>
       </c>
       <c r="M4" t="n">
-        <v>0.188626907073509</v>
+        <v>0.1989578398863098</v>
       </c>
       <c r="N4" t="n">
-        <v>0.1178918169209431</v>
+        <v>0.1260066319279962</v>
       </c>
       <c r="O4" t="n">
-        <v>0.06029411764705883</v>
+        <v>0.05814536340852139</v>
       </c>
       <c r="P4" t="n">
         <v>1</v>
       </c>
       <c r="Q4" t="n">
-        <v>0.4232707252818798</v>
+        <v>0.3644716380756057</v>
       </c>
       <c r="R4" t="n">
-        <v>0.5322113504869838</v>
+        <v>0.5652620572771029</v>
       </c>
       <c r="S4" t="n">
-        <v>0.04451792423113646</v>
-      </c>
-      <c r="T4" t="inlineStr"/>
+        <v>0.07026630464729137</v>
+      </c>
+      <c r="T4" t="n">
+        <v>1</v>
+      </c>
       <c r="U4" t="inlineStr"/>
-      <c r="V4" t="n">
-        <v>1</v>
-      </c>
+      <c r="V4" t="inlineStr"/>
       <c r="W4" t="n">
-        <v>0.5322113504869838</v>
+        <v>1</v>
       </c>
       <c r="X4" t="n">
-        <v>1.36</v>
-      </c>
-      <c r="Y4" t="inlineStr">
+        <v>0.5652620572771029</v>
+      </c>
+      <c r="Y4" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="Z4" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0.0</t>
         </is>
       </c>
-      <c r="Z4" t="n">
-        <v>7.450958906817772</v>
-      </c>
       <c r="AA4" t="n">
-        <v>0.1089406252051039</v>
+        <v>8.902877402114369</v>
       </c>
       <c r="AB4" t="n">
-        <v>1</v>
+        <v>0.2007904192014972</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>f1MVnSdt</t>
+          <t>xpEnqpd5</t>
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>45717.71180555555</v>
+        <v>45718.45833333334</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>psg</t>
+          <t>lyon</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>lille</t>
+          <t>brest</t>
         </is>
       </c>
       <c r="E5" t="n">
@@ -894,81 +892,81 @@
         </is>
       </c>
       <c r="I5" t="n">
-        <v>1.42</v>
+        <v>1.67</v>
       </c>
       <c r="J5" t="n">
-        <v>4.75</v>
+        <v>3.8</v>
       </c>
       <c r="K5" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="L5" t="n">
-        <v>0.6658656253129068</v>
+        <v>0.5638651471984806</v>
       </c>
       <c r="M5" t="n">
-        <v>0.1990587764093321</v>
+        <v>0.247803893637227</v>
       </c>
       <c r="N5" t="n">
-        <v>0.1350755982777611</v>
+        <v>0.1883309591642925</v>
       </c>
       <c r="O5" t="n">
-        <v>0.05760881075929269</v>
+        <v>0.06196028994642289</v>
       </c>
       <c r="P5" t="n">
         <v>1</v>
       </c>
       <c r="Q5" t="n">
-        <v>0.3966321488520033</v>
+        <v>0.3164289687332383</v>
       </c>
       <c r="R5" t="n">
-        <v>0.5252338051799619</v>
+        <v>0.4183670538003988</v>
       </c>
       <c r="S5" t="n">
-        <v>0.07813404596803503</v>
-      </c>
-      <c r="T5" t="inlineStr"/>
+        <v>0.2652039774663629</v>
+      </c>
+      <c r="T5" t="n">
+        <v>1</v>
+      </c>
       <c r="U5" t="inlineStr"/>
-      <c r="V5" t="n">
-        <v>1</v>
-      </c>
+      <c r="V5" t="inlineStr"/>
       <c r="W5" t="n">
-        <v>0.5252338051799619</v>
+        <v>1</v>
       </c>
       <c r="X5" t="n">
-        <v>1.42</v>
-      </c>
-      <c r="Y5" t="inlineStr">
+        <v>0.4183670538003988</v>
+      </c>
+      <c r="Y5" t="n">
+        <v>1.67</v>
+      </c>
+      <c r="Z5" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0.0</t>
         </is>
       </c>
-      <c r="Z5" t="n">
-        <v>7.353273272519465</v>
-      </c>
       <c r="AA5" t="n">
-        <v>0.1286016563279586</v>
+        <v>6.589281097356281</v>
       </c>
       <c r="AB5" t="n">
-        <v>1</v>
+        <v>0.1019380850671605</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>xpEnqpd5</t>
+          <t>tIKwo6Rh</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>45718.45833333334</v>
+        <v>45718.69791666666</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>lyon</t>
+          <t>marseille</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>brest</t>
+          <t>nantes</t>
         </is>
       </c>
       <c r="E6" t="n">
@@ -988,81 +986,81 @@
         </is>
       </c>
       <c r="I6" t="n">
-        <v>1.65</v>
+        <v>1.4</v>
       </c>
       <c r="J6" t="n">
-        <v>3.9</v>
+        <v>5</v>
       </c>
       <c r="K6" t="n">
-        <v>5.25</v>
+        <v>7</v>
       </c>
       <c r="L6" t="n">
-        <v>0.5755850727387729</v>
+        <v>0.6756756756756757</v>
       </c>
       <c r="M6" t="n">
-        <v>0.243516761543327</v>
+        <v>0.1891891891891892</v>
       </c>
       <c r="N6" t="n">
-        <v>0.1808981657179</v>
+        <v>0.1351351351351351</v>
       </c>
       <c r="O6" t="n">
-        <v>0.05294705294705304</v>
+        <v>0.05714285714285716</v>
       </c>
       <c r="P6" t="n">
         <v>1</v>
       </c>
       <c r="Q6" t="n">
-        <v>0.2976500269377471</v>
+        <v>0.131558701916953</v>
       </c>
       <c r="R6" t="n">
-        <v>0.4075107758295754</v>
+        <v>0.8176375438600945</v>
       </c>
       <c r="S6" t="n">
-        <v>0.2948391972326774</v>
-      </c>
-      <c r="T6" t="inlineStr"/>
+        <v>0.05080375422295247</v>
+      </c>
+      <c r="T6" t="n">
+        <v>1</v>
+      </c>
       <c r="U6" t="inlineStr"/>
-      <c r="V6" t="n">
-        <v>1</v>
-      </c>
+      <c r="V6" t="inlineStr"/>
       <c r="W6" t="n">
-        <v>0.4075107758295754</v>
+        <v>1</v>
       </c>
       <c r="X6" t="n">
-        <v>1.65</v>
-      </c>
-      <c r="Y6" t="inlineStr">
+        <v>0.8176375438600945</v>
+      </c>
+      <c r="Y6" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="Z6" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0.0</t>
         </is>
       </c>
-      <c r="Z6" t="n">
-        <v>5.705150861614055</v>
-      </c>
       <c r="AA6" t="n">
-        <v>0.1098607488918283</v>
+        <v>12.87779131579649</v>
       </c>
       <c r="AB6" t="n">
-        <v>1</v>
+        <v>0.6860788419431414</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>tIKwo6Rh</t>
+          <t>I1f2wFPq</t>
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>45718.69791666666</v>
+        <v>45718.55208333334</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>marseille</t>
+          <t>angers</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>nantes</t>
+          <t>toulouse</t>
         </is>
       </c>
       <c r="E7" t="n">
@@ -1082,68 +1080,68 @@
         </is>
       </c>
       <c r="I7" t="n">
-        <v>1.42</v>
+        <v>3.4</v>
       </c>
       <c r="J7" t="n">
-        <v>5</v>
+        <v>3.1</v>
       </c>
       <c r="K7" t="n">
-        <v>6.5</v>
+        <v>2.3</v>
       </c>
       <c r="L7" t="n">
-        <v>0.6655744419414295</v>
+        <v>0.2797175362887406</v>
       </c>
       <c r="M7" t="n">
-        <v>0.189023141511366</v>
+        <v>0.3067869752844252</v>
       </c>
       <c r="N7" t="n">
-        <v>0.1454024165472046</v>
+        <v>0.413495488426834</v>
       </c>
       <c r="O7" t="n">
-        <v>0.05807150595882993</v>
+        <v>0.05148090091576618</v>
       </c>
       <c r="P7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q7" t="n">
-        <v>0.1398326210133467</v>
+        <v>0.4860726432991681</v>
       </c>
       <c r="R7" t="n">
-        <v>0.804257069816722</v>
+        <v>0.2851291579616363</v>
       </c>
       <c r="S7" t="n">
-        <v>0.05591030916993133</v>
-      </c>
-      <c r="T7" t="inlineStr"/>
+        <v>0.2287981987391956</v>
+      </c>
+      <c r="T7" t="n">
+        <v>1</v>
+      </c>
       <c r="U7" t="inlineStr"/>
-      <c r="V7" t="n">
-        <v>1</v>
-      </c>
+      <c r="V7" t="inlineStr"/>
       <c r="W7" t="n">
-        <v>0.804257069816722</v>
+        <v>0</v>
       </c>
       <c r="X7" t="n">
-        <v>1.42</v>
-      </c>
-      <c r="Y7" t="inlineStr">
+        <v>0.4860726432991681</v>
+      </c>
+      <c r="Y7" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="Z7" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0.0</t>
         </is>
       </c>
-      <c r="Z7" t="n">
-        <v>11.25959897743411</v>
-      </c>
       <c r="AA7" t="n">
-        <v>0.6644244488033753</v>
+        <v>7.655644131961896</v>
       </c>
       <c r="AB7" t="n">
-        <v>1</v>
+        <v>0.2009434853375318</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
         <is>
-          <t>I1f2wFPq</t>
+          <t>jiANpcX9</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
@@ -1151,12 +1149,12 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>angers</t>
+          <t>auxerre</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>toulouse</t>
+          <t>strasbourg</t>
         </is>
       </c>
       <c r="E8" t="n">
@@ -1176,68 +1174,68 @@
         </is>
       </c>
       <c r="I8" t="n">
-        <v>3.3</v>
+        <v>2.8</v>
       </c>
       <c r="J8" t="n">
-        <v>3.1</v>
+        <v>3.4</v>
       </c>
       <c r="K8" t="n">
-        <v>2.35</v>
+        <v>2.5</v>
       </c>
       <c r="L8" t="n">
-        <v>0.2882865057380293</v>
+        <v>0.3397282174260591</v>
       </c>
       <c r="M8" t="n">
-        <v>0.3068856351404828</v>
+        <v>0.2797761790567546</v>
       </c>
       <c r="N8" t="n">
-        <v>0.4048278591214879</v>
+        <v>0.3804956035171863</v>
       </c>
       <c r="O8" t="n">
-        <v>0.05114286308521043</v>
+        <v>0.05126050420168071</v>
       </c>
       <c r="P8" t="n">
         <v>0</v>
       </c>
       <c r="Q8" t="n">
-        <v>0.4885618620604572</v>
+        <v>0.4889012503729694</v>
       </c>
       <c r="R8" t="n">
-        <v>0.2364006528448594</v>
+        <v>0.3149152661526948</v>
       </c>
       <c r="S8" t="n">
-        <v>0.2750374850946833</v>
-      </c>
-      <c r="T8" t="inlineStr"/>
+        <v>0.1961834834743358</v>
+      </c>
+      <c r="T8" t="n">
+        <v>1</v>
+      </c>
       <c r="U8" t="inlineStr"/>
-      <c r="V8" t="n">
-        <v>0</v>
-      </c>
+      <c r="V8" t="inlineStr"/>
       <c r="W8" t="n">
-        <v>0.4885618620604572</v>
+        <v>0</v>
       </c>
       <c r="X8" t="n">
-        <v>3.1</v>
-      </c>
-      <c r="Y8" t="inlineStr">
+        <v>0.4889012503729694</v>
+      </c>
+      <c r="Y8" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="Z8" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0.0</t>
         </is>
       </c>
-      <c r="Z8" t="n">
-        <v>6.8398660688464</v>
-      </c>
       <c r="AA8" t="n">
-        <v>0.2135243769657739</v>
+        <v>7.700194693374267</v>
       </c>
       <c r="AB8" t="n">
-        <v>1</v>
+        <v>0.1739859842202746</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
         <is>
-          <t>jiANpcX9</t>
+          <t>AcCfsOQH</t>
         </is>
       </c>
       <c r="B9" s="2" t="n">
@@ -1245,12 +1243,12 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>auxerre</t>
+          <t>montpellier</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>strasbourg</t>
+          <t>rennes</t>
         </is>
       </c>
       <c r="E9" t="n">
@@ -1270,81 +1268,81 @@
         </is>
       </c>
       <c r="I9" t="n">
-        <v>2.8</v>
+        <v>3.7</v>
       </c>
       <c r="J9" t="n">
         <v>3.4</v>
       </c>
       <c r="K9" t="n">
-        <v>2.5</v>
+        <v>2.05</v>
       </c>
       <c r="L9" t="n">
-        <v>0.3397282174260591</v>
+        <v>0.2568638290031325</v>
       </c>
       <c r="M9" t="n">
-        <v>0.2797761790567546</v>
+        <v>0.2795282845034089</v>
       </c>
       <c r="N9" t="n">
-        <v>0.3804956035171863</v>
+        <v>0.4636078864934587</v>
       </c>
       <c r="O9" t="n">
-        <v>0.05126050420168071</v>
+        <v>0.05219279537787425</v>
       </c>
       <c r="P9" t="n">
         <v>0</v>
       </c>
       <c r="Q9" t="n">
-        <v>0.4889012503729694</v>
+        <v>0.524797358985422</v>
       </c>
       <c r="R9" t="n">
-        <v>0.3149152661526948</v>
+        <v>0.08618041359164652</v>
       </c>
       <c r="S9" t="n">
-        <v>0.1961834834743358</v>
-      </c>
-      <c r="T9" t="inlineStr"/>
+        <v>0.3890222274229315</v>
+      </c>
+      <c r="T9" t="n">
+        <v>1</v>
+      </c>
       <c r="U9" t="inlineStr"/>
-      <c r="V9" t="n">
-        <v>0</v>
-      </c>
+      <c r="V9" t="inlineStr"/>
       <c r="W9" t="n">
-        <v>0.4889012503729694</v>
+        <v>0</v>
       </c>
       <c r="X9" t="n">
+        <v>0.524797358985422</v>
+      </c>
+      <c r="Y9" t="n">
         <v>3.4</v>
       </c>
-      <c r="Y9" t="inlineStr">
+      <c r="Z9" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0.0</t>
         </is>
       </c>
-      <c r="Z9" t="n">
-        <v>6.844617505221571</v>
-      </c>
       <c r="AA9" t="n">
-        <v>0.1739859842202746</v>
+        <v>8.265558404020396</v>
       </c>
       <c r="AB9" t="n">
-        <v>1</v>
+        <v>0.1357751315624905</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
         <is>
-          <t>AcCfsOQH</t>
+          <t>4bUSOFAj</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
-        <v>45718.55208333334</v>
+        <v>45717.54166666666</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>montpellier</t>
+          <t>st etienne</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>rennes</t>
+          <t>nice</t>
         </is>
       </c>
       <c r="E10" t="n">
@@ -1364,179 +1362,183 @@
         </is>
       </c>
       <c r="I10" t="n">
-        <v>3.5</v>
+        <v>5</v>
       </c>
       <c r="J10" t="n">
-        <v>3.4</v>
+        <v>4</v>
       </c>
       <c r="K10" t="n">
-        <v>2.1</v>
+        <v>1.67</v>
       </c>
       <c r="L10" t="n">
-        <v>0.2705570291777188</v>
+        <v>0.1906936911218955</v>
       </c>
       <c r="M10" t="n">
-        <v>0.2785145888594165</v>
+        <v>0.2383671139023694</v>
       </c>
       <c r="N10" t="n">
-        <v>0.4509283819628648</v>
+        <v>0.5709391949757351</v>
       </c>
       <c r="O10" t="n">
-        <v>0.05602240896358524</v>
+        <v>0.04880239520958085</v>
       </c>
       <c r="P10" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="Q10" t="n">
-        <v>0.524797358985422</v>
+        <v>0.3452601331485691</v>
       </c>
       <c r="R10" t="n">
-        <v>0.08618041359164652</v>
+        <v>0.1280862898256316</v>
       </c>
       <c r="S10" t="n">
-        <v>0.3890222274229315</v>
-      </c>
-      <c r="T10" t="inlineStr"/>
-      <c r="U10" t="inlineStr"/>
+        <v>0.5266535770257993</v>
+      </c>
+      <c r="T10" t="n">
+        <v>1</v>
+      </c>
+      <c r="U10" t="n">
+        <v>1</v>
+      </c>
       <c r="V10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W10" t="n">
-        <v>0.524797358985422</v>
+        <v>2</v>
       </c>
       <c r="X10" t="n">
-        <v>3.4</v>
-      </c>
-      <c r="Y10" t="inlineStr">
-        <is>
-          <t>dif_prob_mod_bm &gt; 0.0</t>
-        </is>
-      </c>
-      <c r="Z10" t="n">
-        <v>7.347163025795909</v>
+        <v>0.5266535770257993</v>
+      </c>
+      <c r="Y10" t="n">
+        <v>1.67</v>
+      </c>
+      <c r="Z10" t="inlineStr">
+        <is>
+          <t>dif_prob_mod_bm &gt; 0.45</t>
+        </is>
       </c>
       <c r="AA10" t="n">
-        <v>0.1357751315624905</v>
+        <v>4.14739691907817</v>
       </c>
       <c r="AB10" t="n">
-        <v>1</v>
+        <v>0.1813934438772302</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
         <is>
-          <t>4bUSOFAj</t>
+          <t>nsQlSolf</t>
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>45717.54166666666</v>
+        <v>45717.47916666666</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>st etienne</t>
+          <t>rb leipzig</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>nice</t>
+          <t>mainz</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="F11" t="n">
-        <v>551</v>
+        <v>591</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>france</t>
+          <t>germany</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>ligue 1</t>
+          <t>bundesliga</t>
         </is>
       </c>
       <c r="I11" t="n">
-        <v>5</v>
+        <v>1.95</v>
       </c>
       <c r="J11" t="n">
-        <v>4</v>
+        <v>3.7</v>
       </c>
       <c r="K11" t="n">
-        <v>1.67</v>
+        <v>3.75</v>
       </c>
       <c r="L11" t="n">
-        <v>0.1906936911218955</v>
+        <v>0.4885133350937418</v>
       </c>
       <c r="M11" t="n">
-        <v>0.2383671139023694</v>
+        <v>0.2574597306575125</v>
       </c>
       <c r="N11" t="n">
-        <v>0.5709391949757351</v>
+        <v>0.2540269342487457</v>
       </c>
       <c r="O11" t="n">
-        <v>0.04880239520958085</v>
+        <v>0.04975744975744978</v>
       </c>
       <c r="P11" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q11" t="n">
-        <v>0.334805150679232</v>
+        <v>0.4424491233830961</v>
       </c>
       <c r="R11" t="n">
-        <v>0.1750314193057714</v>
+        <v>0.4541626549621784</v>
       </c>
       <c r="S11" t="n">
-        <v>0.4901634300149967</v>
+        <v>0.1033882216547256</v>
       </c>
       <c r="T11" t="n">
         <v>1</v>
       </c>
       <c r="U11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V11" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="W11" t="n">
-        <v>0.4901634300149967</v>
+        <v>1</v>
       </c>
       <c r="X11" t="n">
-        <v>1.67</v>
-      </c>
-      <c r="Y11" t="inlineStr">
-        <is>
-          <t>dif_prob_mod_bm &gt; 0.45</t>
-        </is>
-      </c>
-      <c r="Z11" t="n">
-        <v>3.431144010104977</v>
+        <v>0.4541626549621784</v>
+      </c>
+      <c r="Y11" t="n">
+        <v>1.95</v>
+      </c>
+      <c r="Z11" t="inlineStr">
+        <is>
+          <t>dif_prob_mod_bm &gt; 0.0</t>
+        </is>
       </c>
       <c r="AA11" t="n">
-        <v>0.1553582793357647</v>
+        <v>1.589569292367624</v>
       </c>
       <c r="AB11" t="n">
-        <v>1</v>
+        <v>0.01171353157908228</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
         <is>
-          <t>nsQlSolf</t>
+          <t>K83VvPXa</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
-        <v>45717.47916666666</v>
+        <v>45718.47916666666</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>rb leipzig</t>
+          <t>union berlin</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>mainz</t>
+          <t>holstein kiel</t>
         </is>
       </c>
       <c r="E12" t="n">
@@ -1556,85 +1558,85 @@
         </is>
       </c>
       <c r="I12" t="n">
-        <v>1.95</v>
+        <v>1.57</v>
       </c>
       <c r="J12" t="n">
-        <v>3.6</v>
+        <v>4.33</v>
       </c>
       <c r="K12" t="n">
-        <v>3.8</v>
+        <v>5.25</v>
       </c>
       <c r="L12" t="n">
-        <v>0.4866595517609392</v>
+        <v>0.6018171661844011</v>
       </c>
       <c r="M12" t="n">
-        <v>0.263607257203842</v>
+        <v>0.2182108431661685</v>
       </c>
       <c r="N12" t="n">
-        <v>0.2497331910352188</v>
+        <v>0.1799719906494304</v>
       </c>
       <c r="O12" t="n">
-        <v>0.05375618533513271</v>
+        <v>0.05836574785251614</v>
       </c>
       <c r="P12" t="n">
         <v>1</v>
       </c>
       <c r="Q12" t="n">
-        <v>0.4195727486937567</v>
+        <v>0.3161999600728732</v>
       </c>
       <c r="R12" t="n">
-        <v>0.4634312599002793</v>
+        <v>0.5596727902332074</v>
       </c>
       <c r="S12" t="n">
-        <v>0.116995991405964</v>
+        <v>0.1241272496939193</v>
       </c>
       <c r="T12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U12" t="n">
         <v>0</v>
       </c>
       <c r="V12" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="W12" t="n">
-        <v>0.4634312599002793</v>
+        <v>1</v>
       </c>
       <c r="X12" t="n">
-        <v>1.95</v>
-      </c>
-      <c r="Y12" t="inlineStr">
+        <v>0.5596727902332074</v>
+      </c>
+      <c r="Y12" t="n">
+        <v>1.57</v>
+      </c>
+      <c r="Z12" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0.0</t>
         </is>
       </c>
-      <c r="Z12" t="n">
-        <v>12.97607527720782</v>
-      </c>
       <c r="AA12" t="n">
-        <v>0.04385851120652262</v>
+        <v>9.794273829081128</v>
       </c>
       <c r="AB12" t="n">
-        <v>1</v>
+        <v>0.2434728301603342</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
-          <t>K83VvPXa</t>
+          <t>ne5Nto3m</t>
         </is>
       </c>
       <c r="B13" s="2" t="n">
-        <v>45718.47916666666</v>
+        <v>45718.5625</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>union berlin</t>
+          <t>augsburg</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>holstein kiel</t>
+          <t>freiburg</t>
         </is>
       </c>
       <c r="E13" t="n">
@@ -1654,85 +1656,85 @@
         </is>
       </c>
       <c r="I13" t="n">
-        <v>1.57</v>
+        <v>2.7</v>
       </c>
       <c r="J13" t="n">
-        <v>4.33</v>
+        <v>3.25</v>
       </c>
       <c r="K13" t="n">
-        <v>5.25</v>
+        <v>2.7</v>
       </c>
       <c r="L13" t="n">
-        <v>0.6018171661844011</v>
+        <v>0.3532608695652174</v>
       </c>
       <c r="M13" t="n">
-        <v>0.2182108431661685</v>
+        <v>0.2934782608695652</v>
       </c>
       <c r="N13" t="n">
-        <v>0.1799719906494304</v>
+        <v>0.3532608695652174</v>
       </c>
       <c r="O13" t="n">
-        <v>0.05836574785251614</v>
+        <v>0.04843304843304841</v>
       </c>
       <c r="P13" t="n">
         <v>1</v>
       </c>
       <c r="Q13" t="n">
-        <v>0.3454618222341859</v>
+        <v>0.346639216313311</v>
       </c>
       <c r="R13" t="n">
-        <v>0.5370230577812855</v>
+        <v>0.4091294352020944</v>
       </c>
       <c r="S13" t="n">
-        <v>0.1175151199845285</v>
+        <v>0.2442313484845947</v>
       </c>
       <c r="T13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U13" t="n">
         <v>0</v>
       </c>
       <c r="V13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="W13" t="n">
-        <v>0.5370230577812855</v>
+        <v>1</v>
       </c>
       <c r="X13" t="n">
-        <v>1.57</v>
-      </c>
-      <c r="Y13" t="inlineStr">
+        <v>0.4091294352020944</v>
+      </c>
+      <c r="Y13" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="Z13" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0.0</t>
         </is>
       </c>
-      <c r="Z13" t="n">
-        <v>15.03664561787599</v>
-      </c>
       <c r="AA13" t="n">
-        <v>0.1915612355470995</v>
+        <v>7.159765116036652</v>
       </c>
       <c r="AB13" t="n">
-        <v>1</v>
+        <v>0.06249021888878342</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="inlineStr">
         <is>
-          <t>ne5Nto3m</t>
+          <t>rT9in7uQ</t>
         </is>
       </c>
       <c r="B14" s="2" t="n">
-        <v>45718.5625</v>
+        <v>45717.47916666666</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>augsburg</t>
+          <t>werder bremen</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>freiburg</t>
+          <t>wolfsburg</t>
         </is>
       </c>
       <c r="E14" t="n">
@@ -1752,66 +1754,66 @@
         </is>
       </c>
       <c r="I14" t="n">
-        <v>2.6</v>
+        <v>2.75</v>
       </c>
       <c r="J14" t="n">
-        <v>3.25</v>
+        <v>3.4</v>
       </c>
       <c r="K14" t="n">
-        <v>2.75</v>
+        <v>2.5</v>
       </c>
       <c r="L14" t="n">
-        <v>0.3642384105960265</v>
+        <v>0.3437815975733064</v>
       </c>
       <c r="M14" t="n">
-        <v>0.2913907284768212</v>
+        <v>0.2780586450960567</v>
       </c>
       <c r="N14" t="n">
-        <v>0.3443708609271524</v>
+        <v>0.3781597573306371</v>
       </c>
       <c r="O14" t="n">
-        <v>0.05594405594405583</v>
+        <v>0.05775401069518704</v>
       </c>
       <c r="P14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q14" t="n">
-        <v>0.346639216313311</v>
+        <v>0.3557161122323404</v>
       </c>
       <c r="R14" t="n">
-        <v>0.4091294352020944</v>
+        <v>0.3351855200624196</v>
       </c>
       <c r="S14" t="n">
-        <v>0.2442313484845947</v>
+        <v>0.30909836770524</v>
       </c>
       <c r="T14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U14" t="n">
         <v>0</v>
       </c>
       <c r="V14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="W14" t="n">
-        <v>0.4091294352020944</v>
+        <v>0</v>
       </c>
       <c r="X14" t="n">
-        <v>2.6</v>
-      </c>
-      <c r="Y14" t="inlineStr">
+        <v>0.3557161122323404</v>
+      </c>
+      <c r="Y14" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="Z14" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0.0</t>
         </is>
       </c>
-      <c r="Z14" t="n">
-        <v>11.45562418565864</v>
-      </c>
       <c r="AA14" t="n">
-        <v>0.06249021888878342</v>
+        <v>6.225031964065956</v>
       </c>
       <c r="AB14" t="n">
-        <v>1</v>
+        <v>0.02053059216992081</v>
       </c>
     </row>
     <row r="15">
@@ -1850,66 +1852,64 @@
         </is>
       </c>
       <c r="I15" t="n">
-        <v>5</v>
+        <v>4.33</v>
       </c>
       <c r="J15" t="n">
-        <v>4</v>
+        <v>4.1</v>
       </c>
       <c r="K15" t="n">
-        <v>1.67</v>
+        <v>1.7</v>
       </c>
       <c r="L15" t="n">
-        <v>0.1906936911218955</v>
+        <v>0.2172422391223039</v>
       </c>
       <c r="M15" t="n">
-        <v>0.2383671139023694</v>
+        <v>0.2294289988779454</v>
       </c>
       <c r="N15" t="n">
-        <v>0.5709391949757351</v>
+        <v>0.5533287619997507</v>
       </c>
       <c r="O15" t="n">
-        <v>0.04880239520958085</v>
+        <v>0.06308461535912735</v>
       </c>
       <c r="P15" t="n">
         <v>2</v>
       </c>
       <c r="Q15" t="n">
-        <v>0.2121439927061113</v>
+        <v>0.2835602971242944</v>
       </c>
       <c r="R15" t="n">
-        <v>0.07122113460161757</v>
+        <v>0.1140244205133608</v>
       </c>
       <c r="S15" t="n">
-        <v>0.7166348726922712</v>
-      </c>
-      <c r="T15" t="n">
-        <v>0</v>
-      </c>
+        <v>0.6024152823623448</v>
+      </c>
+      <c r="T15" t="inlineStr"/>
       <c r="U15" t="n">
         <v>0</v>
       </c>
       <c r="V15" t="n">
+        <v>0</v>
+      </c>
+      <c r="W15" t="n">
         <v>2</v>
       </c>
-      <c r="W15" t="n">
-        <v>0.7166348726922712</v>
-      </c>
       <c r="X15" t="n">
-        <v>1.67</v>
-      </c>
-      <c r="Y15" t="inlineStr">
+        <v>0.6024152823623448</v>
+      </c>
+      <c r="Y15" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="Z15" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0.55</t>
         </is>
       </c>
-      <c r="Z15" t="n">
-        <v>10.0328882176918</v>
-      </c>
       <c r="AA15" t="n">
-        <v>0.5044908799861599</v>
+        <v>10.54226744134103</v>
       </c>
       <c r="AB15" t="n">
-        <v>1</v>
+        <v>0.3188549852380503</v>
       </c>
     </row>
     <row r="16">
@@ -1948,25 +1948,25 @@
         </is>
       </c>
       <c r="I16" t="n">
-        <v>2.4</v>
+        <v>2.35</v>
       </c>
       <c r="J16" t="n">
         <v>3.6</v>
       </c>
       <c r="K16" t="n">
-        <v>2.8</v>
+        <v>2.88</v>
       </c>
       <c r="L16" t="n">
-        <v>0.3962264150943396</v>
+        <v>0.4050632911392404</v>
       </c>
       <c r="M16" t="n">
-        <v>0.2641509433962264</v>
+        <v>0.2644163150492264</v>
       </c>
       <c r="N16" t="n">
-        <v>0.3396226415094339</v>
+        <v>0.330520393811533</v>
       </c>
       <c r="O16" t="n">
-        <v>0.05158730158730163</v>
+        <v>0.05053191489361719</v>
       </c>
       <c r="P16" t="n">
         <v>2</v>
@@ -1981,33 +1981,33 @@
         <v>0.4094100046031812</v>
       </c>
       <c r="T16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U16" t="n">
         <v>0</v>
       </c>
       <c r="V16" t="n">
+        <v>0</v>
+      </c>
+      <c r="W16" t="n">
         <v>-2</v>
       </c>
-      <c r="W16" t="n">
+      <c r="X16" t="n">
         <v>0.5905899953968188</v>
       </c>
-      <c r="X16" t="n">
-        <v>1.44</v>
-      </c>
-      <c r="Y16" t="inlineStr">
+      <c r="Y16" t="n">
+        <v>1.421848739495798</v>
+      </c>
+      <c r="Z16" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &lt; 0.55</t>
         </is>
       </c>
-      <c r="Z16" t="n">
-        <v>8.268259935555463</v>
-      </c>
       <c r="AA16" t="n">
+        <v>10.33532491944433</v>
+      </c>
+      <c r="AB16" t="n">
         <v>0.06329515771105931</v>
-      </c>
-      <c r="AB16" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="17">
@@ -2046,25 +2046,25 @@
         </is>
       </c>
       <c r="I17" t="n">
-        <v>3.1</v>
+        <v>3.2</v>
       </c>
       <c r="J17" t="n">
         <v>3.5</v>
       </c>
       <c r="K17" t="n">
-        <v>2.25</v>
+        <v>2.2</v>
       </c>
       <c r="L17" t="n">
-        <v>0.306420233463035</v>
+        <v>0.2968388589051658</v>
       </c>
       <c r="M17" t="n">
-        <v>0.2714007782101167</v>
+        <v>0.2713955281418658</v>
       </c>
       <c r="N17" t="n">
-        <v>0.4221789883268482</v>
+        <v>0.4317656129529684</v>
       </c>
       <c r="O17" t="n">
-        <v>0.05273937532002049</v>
+        <v>0.05275974025974017</v>
       </c>
       <c r="P17" t="n">
         <v>2</v>
@@ -2079,33 +2079,33 @@
         <v>0.5907218267173234</v>
       </c>
       <c r="T17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U17" t="n">
         <v>0</v>
       </c>
       <c r="V17" t="n">
+        <v>0</v>
+      </c>
+      <c r="W17" t="n">
         <v>2</v>
       </c>
-      <c r="W17" t="n">
+      <c r="X17" t="n">
         <v>0.5907218267173234</v>
       </c>
-      <c r="X17" t="n">
-        <v>2.25</v>
-      </c>
-      <c r="Y17" t="inlineStr">
+      <c r="Y17" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="Z17" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0.55</t>
         </is>
       </c>
-      <c r="Z17" t="n">
-        <v>8.270105574042526</v>
-      </c>
       <c r="AA17" t="n">
+        <v>10.33763196755316</v>
+      </c>
+      <c r="AB17" t="n">
         <v>0.3044063634508237</v>
-      </c>
-      <c r="AB17" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="18">
@@ -2144,25 +2144,25 @@
         </is>
       </c>
       <c r="I18" t="n">
-        <v>4</v>
+        <v>3.9</v>
       </c>
       <c r="J18" t="n">
-        <v>3.75</v>
+        <v>3.7</v>
       </c>
       <c r="K18" t="n">
-        <v>1.85</v>
+        <v>1.9</v>
       </c>
       <c r="L18" t="n">
-        <v>0.2364720920323818</v>
+        <v>0.2435053688950468</v>
       </c>
       <c r="M18" t="n">
-        <v>0.2522368981678739</v>
+        <v>0.2566678212677519</v>
       </c>
       <c r="N18" t="n">
-        <v>0.5112910097997444</v>
+        <v>0.4998268098372012</v>
       </c>
       <c r="O18" t="n">
-        <v>0.05720720720720696</v>
+        <v>0.05299631615421085</v>
       </c>
       <c r="P18" t="n">
         <v>2</v>
@@ -2177,52 +2177,52 @@
         <v>0.7951561832391476</v>
       </c>
       <c r="T18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U18" t="n">
         <v>0</v>
       </c>
       <c r="V18" t="n">
+        <v>0</v>
+      </c>
+      <c r="W18" t="n">
         <v>2</v>
       </c>
-      <c r="W18" t="n">
+      <c r="X18" t="n">
         <v>0.7951561832391476</v>
       </c>
-      <c r="X18" t="n">
-        <v>1.85</v>
-      </c>
-      <c r="Y18" t="inlineStr">
+      <c r="Y18" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="Z18" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0.55</t>
         </is>
       </c>
-      <c r="Z18" t="n">
-        <v>11.13218656534807</v>
-      </c>
       <c r="AA18" t="n">
+        <v>13.91523320668508</v>
+      </c>
+      <c r="AB18" t="n">
         <v>0.6367702539556789</v>
-      </c>
-      <c r="AB18" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="inlineStr">
         <is>
-          <t>rT9in7uQ</t>
+          <t>f7TdQPI6</t>
         </is>
       </c>
       <c r="B19" s="2" t="n">
-        <v>45717.47916666666</v>
+        <v>45717.60416666666</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>werder bremen</t>
+          <t>eintracht frankfurt</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>wolfsburg</t>
+          <t>bayer leverkusen</t>
         </is>
       </c>
       <c r="E19" t="n">
@@ -2242,183 +2242,177 @@
         </is>
       </c>
       <c r="I19" t="n">
-        <v>2.63</v>
+        <v>4.75</v>
       </c>
       <c r="J19" t="n">
-        <v>3.4</v>
+        <v>3.7</v>
       </c>
       <c r="K19" t="n">
-        <v>2.6</v>
+        <v>1.75</v>
       </c>
       <c r="L19" t="n">
-        <v>0.3590576766856215</v>
+        <v>0.2000772499034376</v>
       </c>
       <c r="M19" t="n">
-        <v>0.2777416734362307</v>
+        <v>0.2568559289300889</v>
       </c>
       <c r="N19" t="n">
-        <v>0.3632006498781478</v>
+        <v>0.5430668211664735</v>
       </c>
       <c r="O19" t="n">
-        <v>0.05896116855633737</v>
+        <v>0.05222515748831524</v>
       </c>
       <c r="P19" t="n">
         <v>2</v>
       </c>
       <c r="Q19" t="n">
-        <v>0.328937956734344</v>
+        <v>0.1841554618162599</v>
       </c>
       <c r="R19" t="n">
-        <v>0.3094056642015054</v>
+        <v>0.03013727897147922</v>
       </c>
       <c r="S19" t="n">
-        <v>0.3616563790641504</v>
+        <v>0.7857072592122608</v>
       </c>
       <c r="T19" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U19" t="n">
         <v>0</v>
       </c>
       <c r="V19" t="n">
-        <v>-2</v>
+        <v>0</v>
       </c>
       <c r="W19" t="n">
-        <v>0.6383436209358495</v>
+        <v>2</v>
       </c>
       <c r="X19" t="n">
-        <v>1.482918739635158</v>
-      </c>
-      <c r="Y19" t="inlineStr">
-        <is>
-          <t>dif_prob_mod_bm &lt; 0.55</t>
-        </is>
-      </c>
-      <c r="Z19" t="n">
-        <v>1.787362138620378</v>
+        <v>0.7857072592122608</v>
+      </c>
+      <c r="Y19" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="Z19" t="inlineStr">
+        <is>
+          <t>dif_prob_mod_bm &gt; 0.55</t>
+        </is>
       </c>
       <c r="AA19" t="n">
-        <v>0.03271842232980643</v>
+        <v>13.74987703621456</v>
       </c>
       <c r="AB19" t="n">
-        <v>1</v>
+        <v>0.601551797396001</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="inlineStr">
         <is>
-          <t>f7TdQPI6</t>
+          <t>46UzYFuA</t>
         </is>
       </c>
       <c r="B20" s="2" t="n">
-        <v>45717.60416666666</v>
+        <v>45716.69791666666</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>eintracht frankfurt</t>
+          <t>fiorentina</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>bayer leverkusen</t>
+          <t>lecce</t>
         </is>
       </c>
       <c r="E20" t="n">
-        <v>59</v>
+        <v>77</v>
       </c>
       <c r="F20" t="n">
-        <v>591</v>
+        <v>771</v>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>germany</t>
+          <t>italy</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>bundesliga</t>
+          <t>serie a</t>
         </is>
       </c>
       <c r="I20" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="J20" t="n">
+        <v>3.25</v>
+      </c>
+      <c r="K20" t="n">
         <v>4.75</v>
       </c>
-      <c r="J20" t="n">
-        <v>3.75</v>
-      </c>
-      <c r="K20" t="n">
-        <v>1.73</v>
-      </c>
       <c r="L20" t="n">
-        <v>0.1995079572537864</v>
+        <v>0.5038759689922481</v>
       </c>
       <c r="M20" t="n">
-        <v>0.2527100791881294</v>
+        <v>0.2945736434108528</v>
       </c>
       <c r="N20" t="n">
-        <v>0.5477819635580841</v>
+        <v>0.2015503875968992</v>
       </c>
       <c r="O20" t="n">
-        <v>0.05522766453706529</v>
+        <v>0.04453441295546545</v>
       </c>
       <c r="P20" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q20" t="n">
-        <v>0.1841554618162599</v>
+        <v>0.3834413522524662</v>
       </c>
       <c r="R20" t="n">
-        <v>0.03013727897147922</v>
+        <v>0.4083367091799716</v>
       </c>
       <c r="S20" t="n">
-        <v>0.7857072592122608</v>
-      </c>
-      <c r="T20" t="n">
-        <v>0</v>
-      </c>
-      <c r="U20" t="n">
-        <v>0</v>
-      </c>
-      <c r="V20" t="n">
-        <v>2</v>
-      </c>
+        <v>0.2082219385675623</v>
+      </c>
+      <c r="T20" t="inlineStr"/>
+      <c r="U20" t="inlineStr"/>
+      <c r="V20" t="inlineStr"/>
       <c r="W20" t="n">
-        <v>0.7857072592122608</v>
+        <v>-1</v>
       </c>
       <c r="X20" t="n">
-        <v>1.73</v>
-      </c>
-      <c r="Y20" t="inlineStr">
-        <is>
-          <t>dif_prob_mod_bm &gt; 0.55</t>
-        </is>
-      </c>
-      <c r="Z20" t="n">
-        <v>10.99990162897165</v>
+        <v>0.5916632908200284</v>
+      </c>
+      <c r="Y20" t="n">
+        <v>1.9296875</v>
+      </c>
+      <c r="Z20" t="inlineStr">
+        <is>
+          <t>dif_prob_mod_bm &lt; 0.55</t>
+        </is>
       </c>
       <c r="AA20" t="n">
-        <v>0.601551797396001</v>
+        <v>2.0708215178701</v>
       </c>
       <c r="AB20" t="n">
-        <v>1</v>
+        <v>0.02489535692750539</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="inlineStr">
         <is>
-          <t>46UzYFuA</t>
+          <t>GWYtCYIj</t>
         </is>
       </c>
       <c r="B21" s="2" t="n">
-        <v>45716.69791666666</v>
+        <v>45717.45833333334</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>fiorentina</t>
+          <t>atalanta</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>lecce</t>
+          <t>venezia</t>
         </is>
       </c>
       <c r="E21" t="n">
@@ -2438,81 +2432,85 @@
         </is>
       </c>
       <c r="I21" t="n">
-        <v>1.73</v>
+        <v>1.2</v>
       </c>
       <c r="J21" t="n">
-        <v>3.5</v>
+        <v>6.5</v>
       </c>
       <c r="K21" t="n">
-        <v>5.25</v>
+        <v>15</v>
       </c>
       <c r="L21" t="n">
-        <v>0.5483028720626633</v>
+        <v>0.7907542579075426</v>
       </c>
       <c r="M21" t="n">
-        <v>0.2710182767624021</v>
+        <v>0.145985401459854</v>
       </c>
       <c r="N21" t="n">
-        <v>0.1806788511749347</v>
+        <v>0.0632603406326034</v>
       </c>
       <c r="O21" t="n">
-        <v>0.05422515827140106</v>
+        <v>0.05384615384615388</v>
       </c>
       <c r="P21" t="n">
         <v>1</v>
       </c>
       <c r="Q21" t="n">
-        <v>0.3266640769591456</v>
+        <v>0.1553851889122539</v>
       </c>
       <c r="R21" t="n">
-        <v>0.5343209767680094</v>
+        <v>0.8109988871388439</v>
       </c>
       <c r="S21" t="n">
-        <v>0.139014946272845</v>
-      </c>
-      <c r="T21" t="inlineStr"/>
-      <c r="U21" t="inlineStr"/>
+        <v>0.03361592394890208</v>
+      </c>
+      <c r="T21" t="n">
+        <v>1</v>
+      </c>
+      <c r="U21" t="n">
+        <v>1</v>
+      </c>
       <c r="V21" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="W21" t="n">
-        <v>0.4656790232319906</v>
+        <v>1</v>
       </c>
       <c r="X21" t="n">
-        <v>2.1</v>
-      </c>
-      <c r="Y21" t="inlineStr">
-        <is>
-          <t>dif_prob_mod_bm &lt; 0.55</t>
-        </is>
-      </c>
-      <c r="Z21" t="n">
-        <v>1.629876581311967</v>
+        <v>0.8109988871388439</v>
+      </c>
+      <c r="Y21" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="Z21" t="inlineStr">
+        <is>
+          <t>dif_prob_mod_bm &gt; 0.55</t>
+        </is>
       </c>
       <c r="AA21" t="n">
-        <v>0.2076568998088638</v>
+        <v>14.19248052492977</v>
       </c>
       <c r="AB21" t="n">
-        <v>1</v>
+        <v>0.6556136982265901</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="inlineStr">
         <is>
-          <t>GWYtCYIj</t>
+          <t>rckAnFf3</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
-        <v>45717.45833333334</v>
+        <v>45718.35416666666</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>atalanta</t>
+          <t>monza</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>venezia</t>
+          <t>torino</t>
         </is>
       </c>
       <c r="E22" t="n">
@@ -2532,85 +2530,81 @@
         </is>
       </c>
       <c r="I22" t="n">
-        <v>1.22</v>
+        <v>4.1</v>
       </c>
       <c r="J22" t="n">
-        <v>6</v>
+        <v>3.3</v>
       </c>
       <c r="K22" t="n">
-        <v>15</v>
+        <v>1.95</v>
       </c>
       <c r="L22" t="n">
-        <v>0.7784120394395433</v>
+        <v>0.2301502145922747</v>
       </c>
       <c r="M22" t="n">
-        <v>0.1582771146860404</v>
+        <v>0.2859442060085837</v>
       </c>
       <c r="N22" t="n">
-        <v>0.06331084587441618</v>
+        <v>0.4839055793991416</v>
       </c>
       <c r="O22" t="n">
-        <v>0.0530054644808744</v>
+        <v>0.05975325487520622</v>
       </c>
       <c r="P22" t="n">
         <v>1</v>
       </c>
       <c r="Q22" t="n">
-        <v>0.1553851889122539</v>
+        <v>0.32865332702087</v>
       </c>
       <c r="R22" t="n">
-        <v>0.8109988871388439</v>
+        <v>0.3756522111610109</v>
       </c>
       <c r="S22" t="n">
-        <v>0.03361592394890208</v>
+        <v>0.2956944618181191</v>
       </c>
       <c r="T22" t="n">
         <v>1</v>
       </c>
-      <c r="U22" t="n">
-        <v>0</v>
-      </c>
-      <c r="V22" t="n">
-        <v>1</v>
-      </c>
+      <c r="U22" t="inlineStr"/>
+      <c r="V22" t="inlineStr"/>
       <c r="W22" t="n">
-        <v>0.8109988871388439</v>
+        <v>-1</v>
       </c>
       <c r="X22" t="n">
-        <v>1.22</v>
-      </c>
-      <c r="Y22" t="inlineStr">
-        <is>
-          <t>dif_prob_mod_bm &gt; 0.55</t>
-        </is>
-      </c>
-      <c r="Z22" t="n">
-        <v>2.838496104985954</v>
+        <v>0.624347788838989</v>
+      </c>
+      <c r="Y22" t="n">
+        <v>1.225714285714286</v>
+      </c>
+      <c r="Z22" t="inlineStr">
+        <is>
+          <t>dif_prob_mod_bm &lt; 0.55</t>
+        </is>
       </c>
       <c r="AA22" t="n">
-        <v>0.6556136982265901</v>
+        <v>10.92608630468231</v>
       </c>
       <c r="AB22" t="n">
-        <v>1</v>
+        <v>0.04699888414014097</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="1" t="inlineStr">
         <is>
-          <t>rckAnFf3</t>
+          <t>8vySZyBc</t>
         </is>
       </c>
       <c r="B23" s="2" t="n">
-        <v>45718.35416666666</v>
+        <v>45718.45833333334</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>monza</t>
+          <t>bologna</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>torino</t>
+          <t>cagliari</t>
         </is>
       </c>
       <c r="E23" t="n">
@@ -2630,68 +2624,68 @@
         </is>
       </c>
       <c r="I23" t="n">
-        <v>3.9</v>
+        <v>1.57</v>
       </c>
       <c r="J23" t="n">
-        <v>3.3</v>
+        <v>3.75</v>
       </c>
       <c r="K23" t="n">
-        <v>2</v>
+        <v>6.5</v>
       </c>
       <c r="L23" t="n">
-        <v>0.242024202420242</v>
+        <v>0.6023352072650892</v>
       </c>
       <c r="M23" t="n">
-        <v>0.286028602860286</v>
+        <v>0.2521776734416507</v>
       </c>
       <c r="N23" t="n">
-        <v>0.4719471947194719</v>
+        <v>0.14548711929326</v>
       </c>
       <c r="O23" t="n">
-        <v>0.05944055944055959</v>
+        <v>0.05745549567205632</v>
       </c>
       <c r="P23" t="n">
         <v>1</v>
       </c>
       <c r="Q23" t="n">
-        <v>0.32865332702087</v>
+        <v>0.3042708315683902</v>
       </c>
       <c r="R23" t="n">
-        <v>0.3756522111610109</v>
+        <v>0.6632096993075507</v>
       </c>
       <c r="S23" t="n">
-        <v>0.2956944618181191</v>
-      </c>
-      <c r="T23" t="inlineStr"/>
+        <v>0.0325194691240591</v>
+      </c>
+      <c r="T23" t="n">
+        <v>1</v>
+      </c>
       <c r="U23" t="inlineStr"/>
-      <c r="V23" t="n">
-        <v>-1</v>
-      </c>
+      <c r="V23" t="inlineStr"/>
       <c r="W23" t="n">
-        <v>0.624347788838989</v>
+        <v>1</v>
       </c>
       <c r="X23" t="n">
-        <v>1.245283018867924</v>
-      </c>
-      <c r="Y23" t="inlineStr">
-        <is>
-          <t>dif_prob_mod_bm &lt; 0.55</t>
-        </is>
-      </c>
-      <c r="Z23" t="n">
-        <v>2.185217260936462</v>
+        <v>0.6632096993075507</v>
+      </c>
+      <c r="Y23" t="n">
+        <v>1.57</v>
+      </c>
+      <c r="Z23" t="inlineStr">
+        <is>
+          <t>dif_prob_mod_bm &gt; 0.55</t>
+        </is>
       </c>
       <c r="AA23" t="n">
-        <v>0.04699888414014097</v>
+        <v>11.60616973788214</v>
       </c>
       <c r="AB23" t="n">
-        <v>1</v>
+        <v>0.3589388677391604</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="1" t="inlineStr">
         <is>
-          <t>8vySZyBc</t>
+          <t>xKSrWgAM</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
@@ -2699,12 +2693,12 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>bologna</t>
+          <t>genoa</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>cagliari</t>
+          <t>empoli</t>
         </is>
       </c>
       <c r="E24" t="n">
@@ -2724,81 +2718,81 @@
         </is>
       </c>
       <c r="I24" t="n">
-        <v>1.6</v>
+        <v>1.91</v>
       </c>
       <c r="J24" t="n">
-        <v>3.7</v>
+        <v>3.1</v>
       </c>
       <c r="K24" t="n">
-        <v>6.25</v>
+        <v>4.75</v>
       </c>
       <c r="L24" t="n">
-        <v>0.5922653348700219</v>
+        <v>0.495482611841109</v>
       </c>
       <c r="M24" t="n">
-        <v>0.2561147394032527</v>
+        <v>0.3052812221343607</v>
       </c>
       <c r="N24" t="n">
-        <v>0.1516199257267256</v>
+        <v>0.1992361660245301</v>
       </c>
       <c r="O24" t="n">
-        <v>0.05527027027027009</v>
+        <v>0.05666717037484781</v>
       </c>
       <c r="P24" t="n">
         <v>1</v>
       </c>
       <c r="Q24" t="n">
-        <v>0.3373978982021756</v>
+        <v>0.3691240865138111</v>
       </c>
       <c r="R24" t="n">
-        <v>0.6313533565364448</v>
+        <v>0.5480822182653053</v>
       </c>
       <c r="S24" t="n">
-        <v>0.03124874526137956</v>
-      </c>
-      <c r="T24" t="inlineStr"/>
+        <v>0.0827936952208836</v>
+      </c>
+      <c r="T24" t="n">
+        <v>1</v>
+      </c>
       <c r="U24" t="inlineStr"/>
-      <c r="V24" t="n">
-        <v>1</v>
-      </c>
+      <c r="V24" t="inlineStr"/>
       <c r="W24" t="n">
-        <v>0.6313533565364448</v>
+        <v>-1</v>
       </c>
       <c r="X24" t="n">
-        <v>1.6</v>
-      </c>
-      <c r="Y24" t="inlineStr">
-        <is>
-          <t>dif_prob_mod_bm &gt; 0.55</t>
-        </is>
-      </c>
-      <c r="Z24" t="n">
-        <v>2.209736747877556</v>
+        <v>0.4519177817346947</v>
+      </c>
+      <c r="Y24" t="n">
+        <v>1.875796178343949</v>
+      </c>
+      <c r="Z24" t="inlineStr">
+        <is>
+          <t>dif_prob_mod_bm &lt; 0.55</t>
+        </is>
       </c>
       <c r="AA24" t="n">
-        <v>0.2939554583342691</v>
+        <v>7.908561180357156</v>
       </c>
       <c r="AB24" t="n">
-        <v>1</v>
+        <v>0.1789581317514942</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="1" t="inlineStr">
         <is>
-          <t>xKSrWgAM</t>
+          <t>nknRrXgS</t>
         </is>
       </c>
       <c r="B25" s="2" t="n">
-        <v>45718.45833333334</v>
+        <v>45718.58333333334</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>genoa</t>
+          <t>as roma</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>empoli</t>
+          <t>como</t>
         </is>
       </c>
       <c r="E25" t="n">
@@ -2821,78 +2815,82 @@
         <v>1.9</v>
       </c>
       <c r="J25" t="n">
-        <v>3.1</v>
+        <v>3.6</v>
       </c>
       <c r="K25" t="n">
-        <v>4.75</v>
+        <v>4</v>
       </c>
       <c r="L25" t="n">
-        <v>0.4967948717948718</v>
+        <v>0.4993065187239945</v>
       </c>
       <c r="M25" t="n">
-        <v>0.3044871794871795</v>
+        <v>0.2635228848821082</v>
       </c>
       <c r="N25" t="n">
-        <v>0.1987179487179487</v>
+        <v>0.2371705963938974</v>
       </c>
       <c r="O25" t="n">
-        <v>0.05942275042444822</v>
+        <v>0.05409356725146197</v>
       </c>
       <c r="P25" t="n">
         <v>1</v>
       </c>
       <c r="Q25" t="n">
-        <v>0.3874007531720057</v>
+        <v>0.3955215073339148</v>
       </c>
       <c r="R25" t="n">
-        <v>0.5210969799689896</v>
+        <v>0.5198622818673595</v>
       </c>
       <c r="S25" t="n">
-        <v>0.0915022668590047</v>
-      </c>
-      <c r="T25" t="inlineStr"/>
-      <c r="U25" t="inlineStr"/>
+        <v>0.08461621079872572</v>
+      </c>
+      <c r="T25" t="n">
+        <v>1</v>
+      </c>
+      <c r="U25" t="n">
+        <v>1</v>
+      </c>
       <c r="V25" t="n">
+        <v>1</v>
+      </c>
+      <c r="W25" t="n">
         <v>-1</v>
       </c>
-      <c r="W25" t="n">
-        <v>0.4789030200310104</v>
-      </c>
       <c r="X25" t="n">
-        <v>1.875796178343949</v>
-      </c>
-      <c r="Y25" t="inlineStr">
+        <v>0.4801377181326405</v>
+      </c>
+      <c r="Y25" t="n">
+        <v>1.894736842105263</v>
+      </c>
+      <c r="Z25" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &lt; 0.55</t>
         </is>
       </c>
-      <c r="Z25" t="n">
-        <v>1.676160570108536</v>
-      </c>
       <c r="AA25" t="n">
-        <v>0.133696226796984</v>
+        <v>4.201205033660604</v>
       </c>
       <c r="AB25" t="n">
-        <v>1</v>
+        <v>0.1243407745334447</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="1" t="inlineStr">
         <is>
-          <t>nknRrXgS</t>
+          <t>21CNOB2d</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
-        <v>45718.58333333334</v>
+        <v>45718.69791666666</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>as roma</t>
+          <t>ac milan</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>como</t>
+          <t>lazio</t>
         </is>
       </c>
       <c r="E26" t="n">
@@ -2912,85 +2910,81 @@
         </is>
       </c>
       <c r="I26" t="n">
-        <v>1.91</v>
+        <v>2.1</v>
       </c>
       <c r="J26" t="n">
         <v>3.6</v>
       </c>
       <c r="K26" t="n">
-        <v>4</v>
+        <v>3.4</v>
       </c>
       <c r="L26" t="n">
-        <v>0.4979941900677826</v>
+        <v>0.4543429844097995</v>
       </c>
       <c r="M26" t="n">
-        <v>0.2642135841748513</v>
+        <v>0.2650334075723831</v>
       </c>
       <c r="N26" t="n">
-        <v>0.2377922257573662</v>
+        <v>0.2806236080178174</v>
       </c>
       <c r="O26" t="n">
-        <v>0.05133798720186156</v>
+        <v>0.04808590102707755</v>
       </c>
       <c r="P26" t="n">
         <v>1</v>
       </c>
       <c r="Q26" t="n">
-        <v>0.3955215073339148</v>
+        <v>0.1988063294680857</v>
       </c>
       <c r="R26" t="n">
-        <v>0.5198622818673595</v>
+        <v>0.7156499500987038</v>
       </c>
       <c r="S26" t="n">
-        <v>0.08461621079872572</v>
+        <v>0.08554372043321062</v>
       </c>
       <c r="T26" t="n">
         <v>1</v>
       </c>
-      <c r="U26" t="n">
-        <v>1</v>
-      </c>
-      <c r="V26" t="n">
-        <v>-1</v>
-      </c>
+      <c r="U26" t="inlineStr"/>
+      <c r="V26" t="inlineStr"/>
       <c r="W26" t="n">
-        <v>0.4801377181326405</v>
+        <v>1</v>
       </c>
       <c r="X26" t="n">
-        <v>1.894736842105263</v>
-      </c>
-      <c r="Y26" t="inlineStr">
-        <is>
-          <t>dif_prob_mod_bm &lt; 0.55</t>
-        </is>
-      </c>
-      <c r="Z26" t="n">
-        <v>0.8402410067321209</v>
+        <v>0.7156499500987038</v>
+      </c>
+      <c r="Y26" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="Z26" t="inlineStr">
+        <is>
+          <t>dif_prob_mod_bm &gt; 0.55</t>
+        </is>
       </c>
       <c r="AA26" t="n">
-        <v>0.1243407745334447</v>
+        <v>12.52387412672732</v>
       </c>
       <c r="AB26" t="n">
-        <v>1</v>
+        <v>0.5168436206306181</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="1" t="inlineStr">
         <is>
-          <t>21CNOB2d</t>
+          <t>d49FQXXq</t>
         </is>
       </c>
       <c r="B27" s="2" t="n">
-        <v>45718.69791666666</v>
+        <v>45719.69791666666</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>ac milan</t>
+          <t>juventus</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>lazio</t>
+          <t>verona</t>
         </is>
       </c>
       <c r="E27" t="n">
@@ -3010,81 +3004,81 @@
         </is>
       </c>
       <c r="I27" t="n">
-        <v>2</v>
+        <v>1.3</v>
       </c>
       <c r="J27" t="n">
-        <v>3.8</v>
+        <v>5</v>
       </c>
       <c r="K27" t="n">
-        <v>3.4</v>
+        <v>12</v>
       </c>
       <c r="L27" t="n">
-        <v>0.472913616398243</v>
+        <v>0.7308160779537151</v>
       </c>
       <c r="M27" t="n">
-        <v>0.2489019033674963</v>
+        <v>0.1900121802679659</v>
       </c>
       <c r="N27" t="n">
-        <v>0.2781844802342606</v>
+        <v>0.07917174177831914</v>
       </c>
       <c r="O27" t="n">
-        <v>0.05727554179566563</v>
+        <v>0.05256410256410238</v>
       </c>
       <c r="P27" t="n">
         <v>1</v>
       </c>
       <c r="Q27" t="n">
-        <v>0.2100166957912785</v>
+        <v>0.146833214268016</v>
       </c>
       <c r="R27" t="n">
-        <v>0.7199825062254618</v>
+        <v>0.8387063304138811</v>
       </c>
       <c r="S27" t="n">
-        <v>0.07000079798325978</v>
-      </c>
-      <c r="T27" t="inlineStr"/>
+        <v>0.01446045531810282</v>
+      </c>
+      <c r="T27" t="n">
+        <v>1</v>
+      </c>
       <c r="U27" t="inlineStr"/>
-      <c r="V27" t="n">
-        <v>1</v>
-      </c>
+      <c r="V27" t="inlineStr"/>
       <c r="W27" t="n">
-        <v>0.7199825062254618</v>
+        <v>1</v>
       </c>
       <c r="X27" t="n">
-        <v>2</v>
-      </c>
-      <c r="Y27" t="inlineStr">
+        <v>0.8387063304138811</v>
+      </c>
+      <c r="Y27" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="Z27" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0.55</t>
         </is>
       </c>
-      <c r="Z27" t="n">
-        <v>2.519938771789116</v>
-      </c>
       <c r="AA27" t="n">
-        <v>0.5099658104341833</v>
+        <v>14.67736078224292</v>
       </c>
       <c r="AB27" t="n">
-        <v>1</v>
+        <v>0.6918731161458651</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="1" t="inlineStr">
         <is>
-          <t>d49FQXXq</t>
+          <t>rLXdwBHk</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
-        <v>45719.69791666666</v>
+        <v>45717.69791666666</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>juventus</t>
+          <t>udinese</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>verona</t>
+          <t>parma</t>
         </is>
       </c>
       <c r="E28" t="n">
@@ -3104,81 +3098,85 @@
         </is>
       </c>
       <c r="I28" t="n">
-        <v>1.3</v>
+        <v>1.8</v>
       </c>
       <c r="J28" t="n">
-        <v>5</v>
+        <v>3.6</v>
       </c>
       <c r="K28" t="n">
-        <v>13</v>
+        <v>4.5</v>
       </c>
       <c r="L28" t="n">
-        <v>0.7352941176470589</v>
+        <v>0.5263157894736842</v>
       </c>
       <c r="M28" t="n">
-        <v>0.1911764705882353</v>
+        <v>0.2631578947368421</v>
       </c>
       <c r="N28" t="n">
-        <v>0.0735294117647059</v>
+        <v>0.2105263157894737</v>
       </c>
       <c r="O28" t="n">
-        <v>0.04615384615384599</v>
+        <v>0.05555555555555558</v>
       </c>
       <c r="P28" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q28" t="n">
-        <v>0.146833214268016</v>
+        <v>0.4222589831496589</v>
       </c>
       <c r="R28" t="n">
-        <v>0.8387063304138811</v>
+        <v>0.4027905333599394</v>
       </c>
       <c r="S28" t="n">
-        <v>0.01446045531810282</v>
-      </c>
-      <c r="T28" t="inlineStr"/>
-      <c r="U28" t="inlineStr"/>
+        <v>0.1749504834904017</v>
+      </c>
+      <c r="T28" t="n">
+        <v>1</v>
+      </c>
+      <c r="U28" t="n">
+        <v>1</v>
+      </c>
       <c r="V28" t="n">
         <v>1</v>
       </c>
       <c r="W28" t="n">
-        <v>0.8387063304138811</v>
+        <v>0</v>
       </c>
       <c r="X28" t="n">
-        <v>1.3</v>
-      </c>
-      <c r="Y28" t="inlineStr">
-        <is>
-          <t>dif_prob_mod_bm &gt; 0.55</t>
-        </is>
-      </c>
-      <c r="Z28" t="n">
-        <v>2.935472156448584</v>
+        <v>0.4222589831496589</v>
+      </c>
+      <c r="Y28" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="Z28" t="inlineStr">
+        <is>
+          <t>dif_prob_mod_bm &gt; 0.0</t>
+        </is>
       </c>
       <c r="AA28" t="n">
-        <v>0.6918731161458651</v>
+        <v>3.694766102559515</v>
       </c>
       <c r="AB28" t="n">
-        <v>1</v>
+        <v>0.01946844978971951</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="1" t="inlineStr">
         <is>
-          <t>8f71RSPs</t>
+          <t>jNhIpgPF</t>
         </is>
       </c>
       <c r="B29" s="2" t="n">
-        <v>45715.69791666666</v>
+        <v>45717.58333333334</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>bologna</t>
+          <t>napoli</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>ac milan</t>
+          <t>inter</t>
         </is>
       </c>
       <c r="E29" t="n">
@@ -3198,227 +3196,233 @@
         </is>
       </c>
       <c r="I29" t="n">
-        <v>3</v>
+        <v>3.1</v>
       </c>
       <c r="J29" t="n">
-        <v>3.3</v>
+        <v>3.2</v>
       </c>
       <c r="K29" t="n">
-        <v>2.4</v>
+        <v>2.38</v>
       </c>
       <c r="L29" t="n">
-        <v>0.316546762589928</v>
+        <v>0.3056915790318696</v>
       </c>
       <c r="M29" t="n">
-        <v>0.2877697841726619</v>
+        <v>0.2961387171871237</v>
       </c>
       <c r="N29" t="n">
-        <v>0.3956834532374101</v>
+        <v>0.3981697037810067</v>
       </c>
       <c r="O29" t="n">
-        <v>0.05303030303030298</v>
+        <v>0.05524871238818108</v>
       </c>
       <c r="P29" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="Q29" t="n">
-        <v>0.5289455394213708</v>
+        <v>0.3273911279773877</v>
       </c>
       <c r="R29" t="n">
-        <v>0.2678496434537633</v>
+        <v>0.2276337143313177</v>
       </c>
       <c r="S29" t="n">
-        <v>0.203204817124866</v>
-      </c>
-      <c r="T29" t="inlineStr"/>
-      <c r="U29" t="inlineStr"/>
+        <v>0.4449751576912945</v>
+      </c>
+      <c r="T29" t="n">
+        <v>1</v>
+      </c>
+      <c r="U29" t="n">
+        <v>1</v>
+      </c>
       <c r="V29" t="n">
         <v>0</v>
       </c>
       <c r="W29" t="n">
-        <v>0.5289455394213708</v>
+        <v>2</v>
       </c>
       <c r="X29" t="n">
-        <v>3.3</v>
-      </c>
-      <c r="Y29" t="inlineStr">
+        <v>0.4449751576912945</v>
+      </c>
+      <c r="Y29" t="n">
+        <v>2.38</v>
+      </c>
+      <c r="Z29" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0.0</t>
         </is>
       </c>
-      <c r="Z29" t="n">
-        <v>7.405237551899191</v>
-      </c>
       <c r="AA29" t="n">
-        <v>0.2610958959676075</v>
-      </c>
-      <c r="AB29" t="inlineStr"/>
+        <v>7.787065259597653</v>
+      </c>
+      <c r="AB29" t="n">
+        <v>0.1175840297139067</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="1" t="inlineStr">
         <is>
-          <t>rLXdwBHk</t>
+          <t>Y3cJ6mro</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
-        <v>45717.69791666666</v>
+        <v>45717.41666666666</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>udinese</t>
+          <t>girona</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>parma</t>
+          <t>celta vigo</t>
         </is>
       </c>
       <c r="E30" t="n">
-        <v>77</v>
+        <v>148</v>
       </c>
       <c r="F30" t="n">
-        <v>771</v>
+        <v>1481</v>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>italy</t>
+          <t>spain</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>serie a</t>
+          <t>laliga</t>
         </is>
       </c>
       <c r="I30" t="n">
-        <v>1.8</v>
+        <v>2.15</v>
       </c>
       <c r="J30" t="n">
-        <v>3.6</v>
+        <v>3.4</v>
       </c>
       <c r="K30" t="n">
-        <v>4.5</v>
+        <v>3.3</v>
       </c>
       <c r="L30" t="n">
-        <v>0.5263157894736842</v>
+        <v>0.4378536585365854</v>
       </c>
       <c r="M30" t="n">
-        <v>0.2631578947368421</v>
+        <v>0.2768780487804878</v>
       </c>
       <c r="N30" t="n">
-        <v>0.2105263157894737</v>
+        <v>0.2852682926829269</v>
       </c>
       <c r="O30" t="n">
-        <v>0.05555555555555558</v>
+        <v>0.06226422915889396</v>
       </c>
       <c r="P30" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q30" t="n">
-        <v>0.4222589831496589</v>
+        <v>0.06991849441036169</v>
       </c>
       <c r="R30" t="n">
-        <v>0.4027905333599394</v>
+        <v>0.8649714814212883</v>
       </c>
       <c r="S30" t="n">
-        <v>0.1749504834904017</v>
+        <v>0.06511002416835003</v>
       </c>
       <c r="T30" t="n">
         <v>1</v>
       </c>
       <c r="U30" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V30" t="n">
         <v>0</v>
       </c>
       <c r="W30" t="n">
-        <v>0.4222589831496589</v>
+        <v>1</v>
       </c>
       <c r="X30" t="n">
-        <v>3.6</v>
-      </c>
-      <c r="Y30" t="inlineStr">
-        <is>
-          <t>dif_prob_mod_bm &gt; 0.0</t>
-        </is>
-      </c>
-      <c r="Z30" t="n">
-        <v>2.955812882047612</v>
+        <v>0.8649714814212883</v>
+      </c>
+      <c r="Y30" t="n">
+        <v>2.15</v>
+      </c>
+      <c r="Z30" t="inlineStr">
+        <is>
+          <t>dif_prob_mod_bm &gt; 0</t>
+        </is>
       </c>
       <c r="AA30" t="n">
-        <v>0.01946844978971951</v>
+        <v>12.10960073989804</v>
       </c>
       <c r="AB30" t="n">
-        <v>1</v>
+        <v>0.7950529870109266</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="1" t="inlineStr">
         <is>
-          <t>jNhIpgPF</t>
+          <t>WxxwRHTa</t>
         </is>
       </c>
       <c r="B31" s="2" t="n">
-        <v>45717.58333333334</v>
+        <v>45717.51041666666</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>napoli</t>
+          <t>rayo vallecano</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>inter</t>
+          <t>sevilla</t>
         </is>
       </c>
       <c r="E31" t="n">
-        <v>77</v>
+        <v>148</v>
       </c>
       <c r="F31" t="n">
-        <v>771</v>
+        <v>1481</v>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>italy</t>
+          <t>spain</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>serie a</t>
+          <t>laliga</t>
         </is>
       </c>
       <c r="I31" t="n">
-        <v>3.1</v>
+        <v>2.4</v>
       </c>
       <c r="J31" t="n">
         <v>3.2</v>
       </c>
       <c r="K31" t="n">
-        <v>2.38</v>
+        <v>3.1</v>
       </c>
       <c r="L31" t="n">
-        <v>0.3056915790318696</v>
+        <v>0.3961661341853036</v>
       </c>
       <c r="M31" t="n">
-        <v>0.2961387171871237</v>
+        <v>0.2971246006389776</v>
       </c>
       <c r="N31" t="n">
-        <v>0.3981697037810067</v>
+        <v>0.3067092651757188</v>
       </c>
       <c r="O31" t="n">
-        <v>0.05524871238818108</v>
+        <v>0.051747311827957</v>
       </c>
       <c r="P31" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q31" t="n">
-        <v>0.3273911279773877</v>
+        <v>0.1242133111955828</v>
       </c>
       <c r="R31" t="n">
-        <v>0.2276337143313177</v>
+        <v>0.5571672878661983</v>
       </c>
       <c r="S31" t="n">
-        <v>0.4449751576912945</v>
+        <v>0.3186194009382191</v>
       </c>
       <c r="T31" t="n">
         <v>1</v>
@@ -3427,46 +3431,46 @@
         <v>0</v>
       </c>
       <c r="V31" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="W31" t="n">
-        <v>0.4449751576912945</v>
+        <v>1</v>
       </c>
       <c r="X31" t="n">
-        <v>2.38</v>
-      </c>
-      <c r="Y31" t="inlineStr">
-        <is>
-          <t>dif_prob_mod_bm &gt; 0.0</t>
-        </is>
-      </c>
-      <c r="Z31" t="n">
-        <v>12.45930441535624</v>
+        <v>0.5571672878661983</v>
+      </c>
+      <c r="Y31" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="Z31" t="inlineStr">
+        <is>
+          <t>dif_prob_mod_bm &gt; 0</t>
+        </is>
       </c>
       <c r="AA31" t="n">
-        <v>0.1175840297139067</v>
+        <v>7.800342030126775</v>
       </c>
       <c r="AB31" t="n">
-        <v>1</v>
+        <v>0.2385478869279792</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="1" t="inlineStr">
         <is>
-          <t>Y3cJ6mro</t>
+          <t>QaFBAdqJ</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
-        <v>45717.41666666666</v>
+        <v>45718.51041666666</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>girona</t>
+          <t>barcelona</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>celta vigo</t>
+          <t>real sociedad</t>
         </is>
       </c>
       <c r="E32" t="n">
@@ -3486,85 +3490,85 @@
         </is>
       </c>
       <c r="I32" t="n">
-        <v>2.15</v>
+        <v>1.27</v>
       </c>
       <c r="J32" t="n">
-        <v>3.5</v>
+        <v>5.5</v>
       </c>
       <c r="K32" t="n">
-        <v>3.3</v>
+        <v>11</v>
       </c>
       <c r="L32" t="n">
-        <v>0.4413450515857852</v>
+        <v>0.7427413909520594</v>
       </c>
       <c r="M32" t="n">
-        <v>0.2711119602598395</v>
+        <v>0.1715057393652937</v>
       </c>
       <c r="N32" t="n">
-        <v>0.2875429881543752</v>
+        <v>0.08575286968264687</v>
       </c>
       <c r="O32" t="n">
-        <v>0.05386086781435617</v>
+        <v>0.06012884753042225</v>
       </c>
       <c r="P32" t="n">
         <v>1</v>
       </c>
       <c r="Q32" t="n">
-        <v>0.1206315164881251</v>
+        <v>0.05914193834811012</v>
       </c>
       <c r="R32" t="n">
-        <v>0.8086880351200572</v>
+        <v>0.8269075540317835</v>
       </c>
       <c r="S32" t="n">
-        <v>0.07068044839181768</v>
+        <v>0.1139505076201063</v>
       </c>
       <c r="T32" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U32" t="n">
         <v>0</v>
       </c>
       <c r="V32" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="W32" t="n">
-        <v>0.8086880351200572</v>
+        <v>1</v>
       </c>
       <c r="X32" t="n">
-        <v>2.15</v>
-      </c>
-      <c r="Y32" t="inlineStr">
+        <v>0.8269075540317835</v>
+      </c>
+      <c r="Y32" t="n">
+        <v>1.27</v>
+      </c>
+      <c r="Z32" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
-      <c r="Z32" t="n">
-        <v>11.3216324916808</v>
-      </c>
       <c r="AA32" t="n">
-        <v>0.6880565186319321</v>
+        <v>11.57670575644497</v>
       </c>
       <c r="AB32" t="n">
-        <v>1</v>
+        <v>0.7129570464116772</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="1" t="inlineStr">
         <is>
-          <t>WxxwRHTa</t>
+          <t>ANmUSwam</t>
         </is>
       </c>
       <c r="B33" s="2" t="n">
-        <v>45717.51041666666</v>
+        <v>45718.70833333334</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>rayo vallecano</t>
+          <t>osasuna</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>sevilla</t>
+          <t>valencia</t>
         </is>
       </c>
       <c r="E33" t="n">
@@ -3608,61 +3612,61 @@
         <v>1</v>
       </c>
       <c r="Q33" t="n">
-        <v>0.1247424261044102</v>
+        <v>0.09814446133160062</v>
       </c>
       <c r="R33" t="n">
-        <v>0.5565674914569678</v>
+        <v>0.4869639418876485</v>
       </c>
       <c r="S33" t="n">
-        <v>0.318690082438622</v>
+        <v>0.4148915967807507</v>
       </c>
       <c r="T33" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U33" t="n">
         <v>0</v>
       </c>
       <c r="V33" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="W33" t="n">
-        <v>0.5565674914569678</v>
+        <v>1</v>
       </c>
       <c r="X33" t="n">
+        <v>0.4869639418876485</v>
+      </c>
+      <c r="Y33" t="n">
         <v>2.3</v>
       </c>
-      <c r="Y33" t="inlineStr">
+      <c r="Z33" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
-      <c r="Z33" t="n">
-        <v>7.791944880397549</v>
-      </c>
       <c r="AA33" t="n">
-        <v>0.2378774090183458</v>
+        <v>6.817495186427078</v>
       </c>
       <c r="AB33" t="n">
-        <v>1</v>
+        <v>0.07207234510689781</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="1" t="inlineStr">
         <is>
-          <t>QaFBAdqJ</t>
+          <t>EgwRcF8j</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
-        <v>45718.51041666666</v>
+        <v>45719.70833333334</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>barcelona</t>
+          <t>villarreal</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>real sociedad</t>
+          <t>espanyol</t>
         </is>
       </c>
       <c r="E34" t="n">
@@ -3682,85 +3686,85 @@
         </is>
       </c>
       <c r="I34" t="n">
-        <v>1.25</v>
+        <v>1.4</v>
       </c>
       <c r="J34" t="n">
-        <v>6</v>
+        <v>4.75</v>
       </c>
       <c r="K34" t="n">
-        <v>12</v>
+        <v>7.5</v>
       </c>
       <c r="L34" t="n">
-        <v>0.7619047619047619</v>
+        <v>0.6750355281856939</v>
       </c>
       <c r="M34" t="n">
-        <v>0.1587301587301587</v>
+        <v>0.1989578398863098</v>
       </c>
       <c r="N34" t="n">
-        <v>0.07936507936507936</v>
+        <v>0.1260066319279962</v>
       </c>
       <c r="O34" t="n">
-        <v>0.05000000000000004</v>
+        <v>0.05814536340852139</v>
       </c>
       <c r="P34" t="n">
         <v>1</v>
       </c>
       <c r="Q34" t="n">
-        <v>0.1064855452361175</v>
+        <v>0.1941039315789558</v>
       </c>
       <c r="R34" t="n">
-        <v>0.7690209626279376</v>
+        <v>0.752120484889328</v>
       </c>
       <c r="S34" t="n">
-        <v>0.1244934921359449</v>
+        <v>0.05377558353171623</v>
       </c>
       <c r="T34" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U34" t="n">
         <v>0</v>
       </c>
       <c r="V34" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="W34" t="n">
-        <v>0.7690209626279376</v>
+        <v>1</v>
       </c>
       <c r="X34" t="n">
-        <v>1.25</v>
-      </c>
-      <c r="Y34" t="inlineStr">
+        <v>0.752120484889328</v>
+      </c>
+      <c r="Y34" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="Z34" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
-      <c r="Z34" t="n">
-        <v>10.76629347679113</v>
-      </c>
       <c r="AA34" t="n">
-        <v>0.6445274704919928</v>
+        <v>10.52968678845059</v>
       </c>
       <c r="AB34" t="n">
-        <v>1</v>
+        <v>0.5580165533103723</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="1" t="inlineStr">
         <is>
-          <t>ANmUSwam</t>
+          <t>p006SU44</t>
         </is>
       </c>
       <c r="B35" s="2" t="n">
-        <v>45718.70833333334</v>
+        <v>45716.70833333334</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>osasuna</t>
+          <t>valladolid</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>valencia</t>
+          <t>las palmas</t>
         </is>
       </c>
       <c r="E35" t="n">
@@ -3780,85 +3784,85 @@
         </is>
       </c>
       <c r="I35" t="n">
-        <v>2.3</v>
+        <v>3</v>
       </c>
       <c r="J35" t="n">
         <v>3.2</v>
       </c>
       <c r="K35" t="n">
-        <v>3.3</v>
+        <v>2.45</v>
       </c>
       <c r="L35" t="n">
-        <v>0.4139553116424932</v>
+        <v>0.3162565550625252</v>
       </c>
       <c r="M35" t="n">
-        <v>0.2975303802430419</v>
+        <v>0.2964905203711174</v>
       </c>
       <c r="N35" t="n">
-        <v>0.2885143081144649</v>
+        <v>0.3872529245663574</v>
       </c>
       <c r="O35" t="n">
-        <v>0.05031291172595531</v>
+        <v>0.05399659863945572</v>
       </c>
       <c r="P35" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q35" t="n">
-        <v>0.1369401144496862</v>
+        <v>0.4663988146932137</v>
       </c>
       <c r="R35" t="n">
-        <v>0.4436658101481742</v>
+        <v>0.1538348973214209</v>
       </c>
       <c r="S35" t="n">
-        <v>0.4193940754021395</v>
+        <v>0.3797662879853653</v>
       </c>
       <c r="T35" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U35" t="n">
         <v>0</v>
       </c>
       <c r="V35" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="W35" t="n">
-        <v>0.4436658101481742</v>
+        <v>0</v>
       </c>
       <c r="X35" t="n">
-        <v>2.3</v>
-      </c>
-      <c r="Y35" t="inlineStr">
+        <v>0.4663988146932137</v>
+      </c>
+      <c r="Y35" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="Z35" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
-      <c r="Z35" t="n">
-        <v>1.242264268414888</v>
-      </c>
       <c r="AA35" t="n">
-        <v>0.02427173474603467</v>
+        <v>6.529583405704992</v>
       </c>
       <c r="AB35" t="n">
-        <v>1</v>
+        <v>0.08663252670784838</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="1" t="inlineStr">
         <is>
-          <t>EgwRcF8j</t>
+          <t>v3uoPebC</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
-        <v>45719.70833333334</v>
+        <v>45717.70833333334</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>villarreal</t>
+          <t>atl  madrid</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>espanyol</t>
+          <t>ath bilbao</t>
         </is>
       </c>
       <c r="E36" t="n">
@@ -3878,85 +3882,85 @@
         </is>
       </c>
       <c r="I36" t="n">
-        <v>1.42</v>
+        <v>1.95</v>
       </c>
       <c r="J36" t="n">
-        <v>4.75</v>
+        <v>3.5</v>
       </c>
       <c r="K36" t="n">
-        <v>7</v>
+        <v>3.75</v>
       </c>
       <c r="L36" t="n">
-        <v>0.6658656253129068</v>
+        <v>0.4814305364511692</v>
       </c>
       <c r="M36" t="n">
-        <v>0.1990587764093321</v>
+        <v>0.2682255845942228</v>
       </c>
       <c r="N36" t="n">
-        <v>0.1350755982777611</v>
+        <v>0.250343878954608</v>
       </c>
       <c r="O36" t="n">
-        <v>0.05760881075929269</v>
+        <v>0.06520146520146519</v>
       </c>
       <c r="P36" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q36" t="n">
-        <v>0.1949250904077869</v>
+        <v>0.5426421990993135</v>
       </c>
       <c r="R36" t="n">
-        <v>0.7512889614946694</v>
+        <v>0.3260870079060489</v>
       </c>
       <c r="S36" t="n">
-        <v>0.05378594809754361</v>
+        <v>0.1312707929946376</v>
       </c>
       <c r="T36" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U36" t="n">
         <v>0</v>
       </c>
       <c r="V36" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="W36" t="n">
-        <v>0.7512889614946694</v>
+        <v>0</v>
       </c>
       <c r="X36" t="n">
-        <v>1.42</v>
-      </c>
-      <c r="Y36" t="inlineStr">
+        <v>0.5426421990993135</v>
+      </c>
+      <c r="Y36" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="Z36" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
-      <c r="Z36" t="n">
-        <v>10.51804546092537</v>
-      </c>
       <c r="AA36" t="n">
-        <v>0.5563638710868825</v>
+        <v>7.59699078739039</v>
       </c>
       <c r="AB36" t="n">
-        <v>1</v>
+        <v>0.2165551911932647</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="1" t="inlineStr">
         <is>
-          <t>p006SU44</t>
+          <t>Qcp5Ujzh</t>
         </is>
       </c>
       <c r="B37" s="2" t="n">
-        <v>45716.70833333334</v>
+        <v>45718.41666666666</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>valladolid</t>
+          <t>leganes</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>las palmas</t>
+          <t>getafe</t>
         </is>
       </c>
       <c r="E37" t="n">
@@ -3976,40 +3980,40 @@
         </is>
       </c>
       <c r="I37" t="n">
-        <v>2.9</v>
+        <v>3.2</v>
       </c>
       <c r="J37" t="n">
-        <v>3.3</v>
+        <v>2.88</v>
       </c>
       <c r="K37" t="n">
-        <v>2.45</v>
+        <v>2.6</v>
       </c>
       <c r="L37" t="n">
-        <v>0.326534733441034</v>
+        <v>0.29923273657289</v>
       </c>
       <c r="M37" t="n">
-        <v>0.2869547657512116</v>
+        <v>0.3324808184143222</v>
       </c>
       <c r="N37" t="n">
-        <v>0.3865105008077544</v>
+        <v>0.3682864450127877</v>
       </c>
       <c r="O37" t="n">
-        <v>0.05602115454332202</v>
+        <v>0.0443376068376069</v>
       </c>
       <c r="P37" t="n">
         <v>0</v>
       </c>
       <c r="Q37" t="n">
-        <v>0.4047643545463909</v>
+        <v>0.4518147571778194</v>
       </c>
       <c r="R37" t="n">
-        <v>0.2195735225449612</v>
+        <v>0.2021522271739266</v>
       </c>
       <c r="S37" t="n">
-        <v>0.3756621229086478</v>
+        <v>0.346033015648254</v>
       </c>
       <c r="T37" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U37" t="n">
         <v>0</v>
@@ -4018,43 +4022,43 @@
         <v>0</v>
       </c>
       <c r="W37" t="n">
-        <v>0.4047643545463909</v>
+        <v>0</v>
       </c>
       <c r="X37" t="n">
-        <v>3.3</v>
-      </c>
-      <c r="Y37" t="inlineStr">
+        <v>0.4518147571778194</v>
+      </c>
+      <c r="Y37" t="n">
+        <v>2.88</v>
+      </c>
+      <c r="Z37" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
-      <c r="Z37" t="n">
-        <v>2.833350481824736</v>
-      </c>
       <c r="AA37" t="n">
-        <v>0.02910223163774311</v>
+        <v>6.325406600489471</v>
       </c>
       <c r="AB37" t="n">
-        <v>1</v>
+        <v>0.1057817415295654</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="1" t="inlineStr">
         <is>
-          <t>v3uoPebC</t>
+          <t>hQ3EQ8ZG</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
-        <v>45717.70833333334</v>
+        <v>45718.60416666666</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>atl  madrid</t>
+          <t>mallorca</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>ath bilbao</t>
+          <t>alaves</t>
         </is>
       </c>
       <c r="E38" t="n">
@@ -4074,40 +4078,40 @@
         </is>
       </c>
       <c r="I38" t="n">
-        <v>2</v>
+        <v>2.25</v>
       </c>
       <c r="J38" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="K38" t="n">
         <v>3.5</v>
       </c>
-      <c r="K38" t="n">
-        <v>3.7</v>
-      </c>
       <c r="L38" t="n">
-        <v>0.473491773308958</v>
+        <v>0.4221789883268483</v>
       </c>
       <c r="M38" t="n">
-        <v>0.2705667276051188</v>
+        <v>0.3064202334630351</v>
       </c>
       <c r="N38" t="n">
-        <v>0.2559414990859232</v>
+        <v>0.2714007782101168</v>
       </c>
       <c r="O38" t="n">
-        <v>0.05598455598455598</v>
+        <v>0.05273937532002027</v>
       </c>
       <c r="P38" t="n">
         <v>0</v>
       </c>
       <c r="Q38" t="n">
-        <v>0.674507948394747</v>
+        <v>0.4506753940269728</v>
       </c>
       <c r="R38" t="n">
-        <v>0.2219960034469786</v>
+        <v>0.4288717829133488</v>
       </c>
       <c r="S38" t="n">
-        <v>0.1034960481582744</v>
+        <v>0.1204528230596784</v>
       </c>
       <c r="T38" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U38" t="n">
         <v>0</v>
@@ -4116,43 +4120,43 @@
         <v>0</v>
       </c>
       <c r="W38" t="n">
-        <v>0.674507948394747</v>
+        <v>0</v>
       </c>
       <c r="X38" t="n">
-        <v>3.5</v>
-      </c>
-      <c r="Y38" t="inlineStr">
+        <v>0.4506753940269728</v>
+      </c>
+      <c r="Y38" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="Z38" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
-      <c r="Z38" t="n">
-        <v>4.721555638763228</v>
-      </c>
       <c r="AA38" t="n">
-        <v>0.4525119449477685</v>
+        <v>6.30945551637762</v>
       </c>
       <c r="AB38" t="n">
-        <v>1</v>
+        <v>0.021803611113624</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="1" t="inlineStr">
         <is>
-          <t>Qcp5Ujzh</t>
+          <t>t8cbYayQ</t>
         </is>
       </c>
       <c r="B39" s="2" t="n">
-        <v>45718.41666666666</v>
+        <v>45717.60416666666</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>leganes</t>
+          <t>betis</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>getafe</t>
+          <t>real madrid</t>
         </is>
       </c>
       <c r="E39" t="n">
@@ -4172,40 +4176,40 @@
         </is>
       </c>
       <c r="I39" t="n">
-        <v>3.1</v>
+        <v>4</v>
       </c>
       <c r="J39" t="n">
-        <v>2.88</v>
+        <v>3.9</v>
       </c>
       <c r="K39" t="n">
-        <v>2.6</v>
+        <v>1.8</v>
       </c>
       <c r="L39" t="n">
-        <v>0.305932341885929</v>
+        <v>0.2354124748490946</v>
       </c>
       <c r="M39" t="n">
-        <v>0.3293021735577709</v>
+        <v>0.2414486921529175</v>
       </c>
       <c r="N39" t="n">
-        <v>0.3647654845563</v>
+        <v>0.5231388329979879</v>
       </c>
       <c r="O39" t="n">
-        <v>0.05441825199889716</v>
+        <v>0.06196581196581197</v>
       </c>
       <c r="P39" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="Q39" t="n">
-        <v>0.504524134212745</v>
+        <v>0.03757050589060448</v>
       </c>
       <c r="R39" t="n">
-        <v>0.1757318360304019</v>
+        <v>0.01442418376344927</v>
       </c>
       <c r="S39" t="n">
-        <v>0.3197440297568531</v>
+        <v>0.9480053103459463</v>
       </c>
       <c r="T39" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U39" t="n">
         <v>0</v>
@@ -4214,220 +4218,24 @@
         <v>0</v>
       </c>
       <c r="W39" t="n">
-        <v>0.504524134212745</v>
+        <v>2</v>
       </c>
       <c r="X39" t="n">
-        <v>2.88</v>
-      </c>
-      <c r="Y39" t="inlineStr">
+        <v>0.9480053103459463</v>
+      </c>
+      <c r="Y39" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="Z39" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
-      <c r="Z39" t="n">
-        <v>3.531668939489215</v>
-      </c>
       <c r="AA39" t="n">
-        <v>0.1847801044558919</v>
+        <v>13.27207434484325</v>
       </c>
       <c r="AB39" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="1" t="inlineStr">
-        <is>
-          <t>hQ3EQ8ZG</t>
-        </is>
-      </c>
-      <c r="B40" s="2" t="n">
-        <v>45718.60416666666</v>
-      </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>mallorca</t>
-        </is>
-      </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>alaves</t>
-        </is>
-      </c>
-      <c r="E40" t="n">
-        <v>148</v>
-      </c>
-      <c r="F40" t="n">
-        <v>1481</v>
-      </c>
-      <c r="G40" t="inlineStr">
-        <is>
-          <t>spain</t>
-        </is>
-      </c>
-      <c r="H40" t="inlineStr">
-        <is>
-          <t>laliga</t>
-        </is>
-      </c>
-      <c r="I40" t="n">
-        <v>2.25</v>
-      </c>
-      <c r="J40" t="n">
-        <v>3.1</v>
-      </c>
-      <c r="K40" t="n">
-        <v>3.5</v>
-      </c>
-      <c r="L40" t="n">
-        <v>0.4221789883268483</v>
-      </c>
-      <c r="M40" t="n">
-        <v>0.3064202334630351</v>
-      </c>
-      <c r="N40" t="n">
-        <v>0.2714007782101168</v>
-      </c>
-      <c r="O40" t="n">
-        <v>0.05273937532002027</v>
-      </c>
-      <c r="P40" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q40" t="n">
-        <v>0.519734155495743</v>
-      </c>
-      <c r="R40" t="n">
-        <v>0.3689645942241222</v>
-      </c>
-      <c r="S40" t="n">
-        <v>0.1113012502801348</v>
-      </c>
-      <c r="T40" t="n">
-        <v>0</v>
-      </c>
-      <c r="U40" t="n">
-        <v>0</v>
-      </c>
-      <c r="V40" t="n">
-        <v>0</v>
-      </c>
-      <c r="W40" t="n">
-        <v>0.519734155495743</v>
-      </c>
-      <c r="X40" t="n">
-        <v>3.1</v>
-      </c>
-      <c r="Y40" t="inlineStr">
-        <is>
-          <t>dif_prob_mod_bm &gt; 0</t>
-        </is>
-      </c>
-      <c r="Z40" t="n">
-        <v>3.638139088470201</v>
-      </c>
-      <c r="AA40" t="n">
-        <v>0.1507695612716208</v>
-      </c>
-      <c r="AB40" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="1" t="inlineStr">
-        <is>
-          <t>t8cbYayQ</t>
-        </is>
-      </c>
-      <c r="B41" s="2" t="n">
-        <v>45717.60416666666</v>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>betis</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>real madrid</t>
-        </is>
-      </c>
-      <c r="E41" t="n">
-        <v>148</v>
-      </c>
-      <c r="F41" t="n">
-        <v>1481</v>
-      </c>
-      <c r="G41" t="inlineStr">
-        <is>
-          <t>spain</t>
-        </is>
-      </c>
-      <c r="H41" t="inlineStr">
-        <is>
-          <t>laliga</t>
-        </is>
-      </c>
-      <c r="I41" t="n">
-        <v>4.33</v>
-      </c>
-      <c r="J41" t="n">
-        <v>4</v>
-      </c>
-      <c r="K41" t="n">
-        <v>1.73</v>
-      </c>
-      <c r="L41" t="n">
-        <v>0.2180839497146315</v>
-      </c>
-      <c r="M41" t="n">
-        <v>0.2360758755660886</v>
-      </c>
-      <c r="N41" t="n">
-        <v>0.54584017471928</v>
-      </c>
-      <c r="O41" t="n">
-        <v>0.05898156429801493</v>
-      </c>
-      <c r="P41" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q41" t="n">
-        <v>0.03921424796109968</v>
-      </c>
-      <c r="R41" t="n">
-        <v>0.01419829044905897</v>
-      </c>
-      <c r="S41" t="n">
-        <v>0.9465874615898413</v>
-      </c>
-      <c r="T41" t="n">
-        <v>0</v>
-      </c>
-      <c r="U41" t="n">
-        <v>0</v>
-      </c>
-      <c r="V41" t="n">
-        <v>2</v>
-      </c>
-      <c r="W41" t="n">
-        <v>0.9465874615898413</v>
-      </c>
-      <c r="X41" t="n">
-        <v>1.73</v>
-      </c>
-      <c r="Y41" t="inlineStr">
-        <is>
-          <t>dif_prob_mod_bm &gt; 0</t>
-        </is>
-      </c>
-      <c r="Z41" t="n">
-        <v>6.626112231128888</v>
-      </c>
-      <c r="AA41" t="n">
-        <v>0.9073732136287416</v>
-      </c>
-      <c r="AB41" t="n">
-        <v>1</v>
+        <v>0.9104348044553418</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
DATA. Bajo el porc_m de 0.2 a 0.15
</commit_message>
<xml_diff>
--- a/data/predicciones.xlsx
+++ b/data/predicciones.xlsx
@@ -663,7 +663,7 @@
         </is>
       </c>
       <c r="Z2" t="n">
-        <v>8.822540812720957</v>
+        <v>6.616905609540717</v>
       </c>
       <c r="AA2" t="n">
         <v>0.2892377163418371</v>
@@ -759,7 +759,7 @@
         </is>
       </c>
       <c r="Z3" t="n">
-        <v>9.324639201324164</v>
+        <v>6.993479400993122</v>
       </c>
       <c r="AA3" t="n">
         <v>0.3667368386383034</v>
@@ -855,7 +855,7 @@
         </is>
       </c>
       <c r="Z4" t="n">
-        <v>10.07555795546843</v>
+        <v>7.55666846660132</v>
       </c>
       <c r="AA4" t="n">
         <v>0.4349996050600681</v>
@@ -951,7 +951,7 @@
         </is>
       </c>
       <c r="Z5" t="n">
-        <v>12.20136924542783</v>
+        <v>9.151026934070874</v>
       </c>
       <c r="AA5" t="n">
         <v>0.5330200483517167</v>
@@ -1047,7 +1047,7 @@
         </is>
       </c>
       <c r="Z6" t="n">
-        <v>8.919897070957587</v>
+        <v>6.689922803218189</v>
       </c>
       <c r="AA6" t="n">
         <v>0.324778443845452</v>
@@ -1143,7 +1143,7 @@
         </is>
       </c>
       <c r="Z7" t="n">
-        <v>9.158385644508057</v>
+        <v>6.868789233381041</v>
       </c>
       <c r="AA7" t="n">
         <v>0.242663481813102</v>
@@ -1239,7 +1239,7 @@
         </is>
       </c>
       <c r="Z8" t="n">
-        <v>11.83151579129375</v>
+        <v>8.873636843470308</v>
       </c>
       <c r="AA8" t="n">
         <v>0.5430988102032794</v>
@@ -1335,7 +1335,7 @@
         </is>
       </c>
       <c r="Z9" t="n">
-        <v>1.358599946585974</v>
+        <v>1.01894995993948</v>
       </c>
       <c r="AA9" t="n">
         <v>0.01714376271259382</v>
@@ -1431,7 +1431,7 @@
         </is>
       </c>
       <c r="Z10" t="n">
-        <v>5.93415980953279</v>
+        <v>4.450619857149593</v>
       </c>
       <c r="AA10" t="n">
         <v>0.01270489629260907</v>
@@ -1527,7 +1527,7 @@
         </is>
       </c>
       <c r="Z11" t="n">
-        <v>8.535138220113934</v>
+        <v>6.401353665085449</v>
       </c>
       <c r="AA11" t="n">
         <v>0.268927327405422</v>
@@ -1623,7 +1623,7 @@
         </is>
       </c>
       <c r="Z12" t="n">
-        <v>8.932671872126457</v>
+        <v>6.699503904094843</v>
       </c>
       <c r="AA12" t="n">
         <v>0.14747760149254</v>
@@ -1721,7 +1721,7 @@
         </is>
       </c>
       <c r="Z13" t="n">
-        <v>13.2729188069881</v>
+        <v>9.954689105241076</v>
       </c>
       <c r="AA13" t="n">
         <v>0.4242182057246524</v>
@@ -1819,7 +1819,7 @@
         </is>
       </c>
       <c r="Z14" t="n">
-        <v>10.07275046555262</v>
+        <v>7.554562849164462</v>
       </c>
       <c r="AA14" t="n">
         <v>0.2396676846426827</v>
@@ -1915,7 +1915,7 @@
         </is>
       </c>
       <c r="Z15" t="n">
-        <v>10.16545360326666</v>
+        <v>7.624090202449995</v>
       </c>
       <c r="AA15" t="n">
         <v>0.2449830286679799</v>
@@ -2011,7 +2011,7 @@
         </is>
       </c>
       <c r="Z16" t="n">
-        <v>8.184295872058451</v>
+        <v>6.138221904043838</v>
       </c>
       <c r="AA16" t="n">
         <v>0.07024781883686648</v>
@@ -2107,7 +2107,7 @@
         </is>
       </c>
       <c r="Z17" t="n">
-        <v>1.457783710246368</v>
+        <v>1.093337782684775</v>
       </c>
       <c r="AA17" t="n">
         <v>0.02548366643753203</v>
@@ -2201,7 +2201,7 @@
         </is>
       </c>
       <c r="Z18" t="n">
-        <v>8.460877322127605</v>
+        <v>6.345657991595703</v>
       </c>
       <c r="AA18" t="n">
         <v>0.1264299463715549</v>
@@ -2295,7 +2295,7 @@
         </is>
       </c>
       <c r="Z19" t="n">
-        <v>8.095770820527013</v>
+        <v>6.071828115395259</v>
       </c>
       <c r="AA19" t="n">
         <v>0.09385969203103028</v>
@@ -2391,7 +2391,7 @@
         </is>
       </c>
       <c r="Z20" t="n">
-        <v>3.926323393639496</v>
+        <v>2.944742545229622</v>
       </c>
       <c r="AA20" t="n">
         <v>0.06737441718291154</v>
@@ -2489,7 +2489,7 @@
         </is>
       </c>
       <c r="Z21" t="n">
-        <v>11.38822183149708</v>
+        <v>8.541166373622811</v>
       </c>
       <c r="AA21" t="n">
         <v>0.2271805668511316</v>
@@ -2587,7 +2587,7 @@
         </is>
       </c>
       <c r="Z22" t="n">
-        <v>11.77300325512901</v>
+        <v>8.829752441346756</v>
       </c>
       <c r="AA22" t="n">
         <v>0.2195835643651847</v>
@@ -2685,7 +2685,7 @@
         </is>
       </c>
       <c r="Z23" t="n">
-        <v>11.10634950999402</v>
+        <v>8.329762132495517</v>
       </c>
       <c r="AA23" t="n">
         <v>0.1784313727751914</v>
@@ -2783,7 +2783,7 @@
         </is>
       </c>
       <c r="Z24" t="n">
-        <v>10.77821968647749</v>
+        <v>8.083664764858113</v>
       </c>
       <c r="AA24" t="n">
         <v>0.1937175918370535</v>
@@ -2881,7 +2881,7 @@
         </is>
       </c>
       <c r="Z25" t="n">
-        <v>12.25442614087445</v>
+        <v>9.19081960565584</v>
       </c>
       <c r="AA25" t="n">
         <v>0.2380084083818134</v>
@@ -2979,7 +2979,7 @@
         </is>
       </c>
       <c r="Z26" t="n">
-        <v>8.649586271085136</v>
+        <v>6.487189703313851</v>
       </c>
       <c r="AA26" t="n">
         <v>0.05409556623689876</v>
@@ -3077,7 +3077,7 @@
         </is>
       </c>
       <c r="Z27" t="n">
-        <v>1.726553577636412</v>
+        <v>1.294915183227309</v>
       </c>
       <c r="AA27" t="n">
         <v>0.004874845939002781</v>
@@ -3175,7 +3175,7 @@
         </is>
       </c>
       <c r="Z28" t="n">
-        <v>8.509486188406107</v>
+        <v>6.382114641304581</v>
       </c>
       <c r="AA28" t="n">
         <v>0.06603995883164865</v>
@@ -3273,7 +3273,7 @@
         </is>
       </c>
       <c r="Z29" t="n">
-        <v>8.040857407615745</v>
+        <v>6.030643055711809</v>
       </c>
       <c r="AA29" t="n">
         <v>0.003189790487149791</v>
@@ -3371,7 +3371,7 @@
         </is>
       </c>
       <c r="Z30" t="n">
-        <v>2.964589203103712</v>
+        <v>2.223441902327784</v>
       </c>
       <c r="AA30" t="n">
         <v>0.01759834784251979</v>
@@ -3469,7 +3469,7 @@
         </is>
       </c>
       <c r="Z31" t="n">
-        <v>4.929435593648229</v>
+        <v>3.697076695236171</v>
       </c>
       <c r="AA31" t="n">
         <v>0.4076436874120243</v>
@@ -3565,7 +3565,7 @@
         </is>
       </c>
       <c r="Z32" t="n">
-        <v>0.6696346567812709</v>
+        <v>0.502225992585953</v>
       </c>
       <c r="AA32" t="n">
         <v>0.002268490124341938</v>
@@ -3659,7 +3659,7 @@
         </is>
       </c>
       <c r="Z33" t="n">
-        <v>6.418660582534651</v>
+        <v>4.813995436900988</v>
       </c>
       <c r="AA33" t="n">
         <v>0.65314611304167</v>
@@ -3755,7 +3755,7 @@
         </is>
       </c>
       <c r="Z34" t="n">
-        <v>5.984005395132096</v>
+        <v>4.488004046349071</v>
       </c>
       <c r="AA34" t="n">
         <v>0.5129523227565529</v>
@@ -3851,7 +3851,7 @@
         </is>
       </c>
       <c r="Z35" t="n">
-        <v>6.232804265560657</v>
+        <v>4.674603199170492</v>
       </c>
       <c r="AA35" t="n">
         <v>0.6503964625767549</v>
@@ -3947,7 +3947,7 @@
         </is>
       </c>
       <c r="Z36" t="n">
-        <v>4.380238626858884</v>
+        <v>3.285178970144163</v>
       </c>
       <c r="AA36" t="n">
         <v>0.2723084567893851</v>
@@ -4043,7 +4043,7 @@
         </is>
       </c>
       <c r="Z37" t="n">
-        <v>6.868457015460186</v>
+        <v>5.151342761595139</v>
       </c>
       <c r="AA37" t="n">
         <v>0.7687039407454913</v>
@@ -4139,7 +4139,7 @@
         </is>
       </c>
       <c r="Z38" t="n">
-        <v>3.815358544120448</v>
+        <v>2.861518908090336</v>
       </c>
       <c r="AA38" t="n">
         <v>0.06576960305185331</v>
@@ -4235,7 +4235,7 @@
         </is>
       </c>
       <c r="Z39" t="n">
-        <v>4.748144313029468</v>
+        <v>3.561108234772101</v>
       </c>
       <c r="AA39" t="n">
         <v>0.2576680670387645</v>
@@ -4331,7 +4331,7 @@
         </is>
       </c>
       <c r="Z40" t="n">
-        <v>10.74850444638411</v>
+        <v>8.061378334788085</v>
       </c>
       <c r="AA40" t="n">
         <v>0.2659946325921776</v>
@@ -4427,7 +4427,7 @@
         </is>
       </c>
       <c r="Z41" t="n">
-        <v>7.538440119117458</v>
+        <v>5.653830089338093</v>
       </c>
       <c r="AA41" t="n">
         <v>0.03367945598509514</v>
@@ -4523,7 +4523,7 @@
         </is>
       </c>
       <c r="Z42" t="n">
-        <v>12.20715845564484</v>
+        <v>9.155368841733628</v>
       </c>
       <c r="AA42" t="n">
         <v>0.4057672136872293</v>
@@ -4619,7 +4619,7 @@
         </is>
       </c>
       <c r="Z43" t="n">
-        <v>15.0883877988357</v>
+        <v>11.31629084912677</v>
       </c>
       <c r="AA43" t="n">
         <v>0.6428508882537345</v>
@@ -4715,7 +4715,7 @@
         </is>
       </c>
       <c r="Z44" t="n">
-        <v>10.14637794469211</v>
+        <v>7.60978345851908</v>
       </c>
       <c r="AA44" t="n">
         <v>0.1577477966534874</v>
@@ -4811,7 +4811,7 @@
         </is>
       </c>
       <c r="Z45" t="n">
-        <v>14.00491356911671</v>
+        <v>10.50368517683753</v>
       </c>
       <c r="AA45" t="n">
         <v>0.5447074706177735</v>
@@ -4907,7 +4907,7 @@
         </is>
       </c>
       <c r="Z46" t="n">
-        <v>12.89582890813189</v>
+        <v>9.671871681098917</v>
       </c>
       <c r="AA46" t="n">
         <v>0.4397563214272065</v>
@@ -5003,7 +5003,7 @@
         </is>
       </c>
       <c r="Z47" t="n">
-        <v>12.60983777587895</v>
+        <v>9.457378331909212</v>
       </c>
       <c r="AA47" t="n">
         <v>0.4242933439703247</v>
@@ -5099,7 +5099,7 @@
         </is>
       </c>
       <c r="Z48" t="n">
-        <v>7.856774538765855</v>
+        <v>5.892580904074391</v>
       </c>
       <c r="AA48" t="n">
         <v>0.09870931369954694</v>
@@ -5195,7 +5195,7 @@
         </is>
       </c>
       <c r="Z49" t="n">
-        <v>7.185418932187327</v>
+        <v>5.389064199140495</v>
       </c>
       <c r="AA49" t="n">
         <v>0.06461254905152419</v>

</xml_diff>

<commit_message>
DATA. Actualizo predicciones tras implementar kelly + linear
</commit_message>
<xml_diff>
--- a/data/predicciones.xlsx
+++ b/data/predicciones.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB49"/>
+  <dimension ref="A1:AC49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -560,15 +560,20 @@
       </c>
       <c r="Z1" s="1" t="inlineStr">
         <is>
+          <t>kelly_criterion</t>
+        </is>
+      </c>
+      <c r="AA1" s="1" t="inlineStr">
+        <is>
           <t>stake_to_bet</t>
         </is>
       </c>
-      <c r="AA1" s="1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>confidence_margin</t>
         </is>
       </c>
-      <c r="AB1" s="1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>emergency_fill</t>
         </is>
@@ -663,12 +668,15 @@
         </is>
       </c>
       <c r="Z2" t="n">
-        <v>6.616905609540717</v>
+        <v>0.3852639122006374</v>
       </c>
       <c r="AA2" t="n">
+        <v>5.376235807751832</v>
+      </c>
+      <c r="AB2" t="n">
         <v>0.2892377163418371</v>
       </c>
-      <c r="AB2" t="inlineStr"/>
+      <c r="AC2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
@@ -759,12 +767,15 @@
         </is>
       </c>
       <c r="Z3" t="n">
-        <v>6.993479400993122</v>
+        <v>0.4223245462684373</v>
       </c>
       <c r="AA3" t="n">
+        <v>5.682202013306912</v>
+      </c>
+      <c r="AB3" t="n">
         <v>0.3667368386383034</v>
       </c>
-      <c r="AB3" t="inlineStr"/>
+      <c r="AC3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
@@ -855,12 +866,15 @@
         </is>
       </c>
       <c r="Z4" t="n">
-        <v>7.55666846660132</v>
+        <v>-0.193116800634831</v>
       </c>
       <c r="AA4" t="n">
+        <v>5.256686853194107</v>
+      </c>
+      <c r="AB4" t="n">
         <v>0.4349996050600681</v>
       </c>
-      <c r="AB4" t="inlineStr"/>
+      <c r="AC4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
@@ -951,12 +965,15 @@
         </is>
       </c>
       <c r="Z5" t="n">
-        <v>9.151026934070874</v>
+        <v>-1.395727350894945</v>
       </c>
       <c r="AA5" t="n">
+        <v>1.631601706485402</v>
+      </c>
+      <c r="AB5" t="n">
         <v>0.5330200483517167</v>
       </c>
-      <c r="AB5" t="inlineStr"/>
+      <c r="AC5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
@@ -1047,12 +1064,15 @@
         </is>
       </c>
       <c r="Z6" t="n">
-        <v>6.689922803218189</v>
+        <v>0.2034884204827284</v>
       </c>
       <c r="AA6" t="n">
+        <v>5.435562277614779</v>
+      </c>
+      <c r="AB6" t="n">
         <v>0.324778443845452</v>
       </c>
-      <c r="AB6" t="inlineStr"/>
+      <c r="AC6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
@@ -1143,12 +1163,15 @@
         </is>
       </c>
       <c r="Z7" t="n">
-        <v>6.868789233381041</v>
+        <v>0.2965275561893362</v>
       </c>
       <c r="AA7" t="n">
+        <v>5.580891252122096</v>
+      </c>
+      <c r="AB7" t="n">
         <v>0.242663481813102</v>
       </c>
-      <c r="AB7" t="inlineStr"/>
+      <c r="AC7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
@@ -1239,12 +1262,15 @@
         </is>
       </c>
       <c r="Z8" t="n">
-        <v>8.873636843470308</v>
+        <v>-0.5631815782648459</v>
       </c>
       <c r="AA8" t="n">
+        <v>4.333549339308669</v>
+      </c>
+      <c r="AB8" t="n">
         <v>0.5430988102032794</v>
       </c>
-      <c r="AB8" t="inlineStr"/>
+      <c r="AC8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
@@ -1335,12 +1361,15 @@
         </is>
       </c>
       <c r="Z9" t="n">
-        <v>1.01894995993948</v>
+        <v>0.0277090235206111</v>
       </c>
       <c r="AA9" t="n">
+        <v>0.8278968424508277</v>
+      </c>
+      <c r="AB9" t="n">
         <v>0.01714376271259382</v>
       </c>
-      <c r="AB9" t="inlineStr"/>
+      <c r="AC9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
@@ -1431,12 +1460,15 @@
         </is>
       </c>
       <c r="Z10" t="n">
-        <v>4.450619857149593</v>
+        <v>0.1087537331357158</v>
       </c>
       <c r="AA10" t="n">
+        <v>3.616128633934044</v>
+      </c>
+      <c r="AB10" t="n">
         <v>0.01270489629260907</v>
       </c>
-      <c r="AB10" t="inlineStr"/>
+      <c r="AC10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
@@ -1527,12 +1559,15 @@
         </is>
       </c>
       <c r="Z11" t="n">
-        <v>6.401353665085449</v>
+        <v>0.1446512543880548</v>
       </c>
       <c r="AA11" t="n">
+        <v>5.201099852881927</v>
+      </c>
+      <c r="AB11" t="n">
         <v>0.268927327405422</v>
       </c>
-      <c r="AB11" t="inlineStr"/>
+      <c r="AC11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
@@ -1623,12 +1658,15 @@
         </is>
       </c>
       <c r="Z12" t="n">
-        <v>6.699503904094843</v>
+        <v>-0.03455458586643988</v>
       </c>
       <c r="AA12" t="n">
+        <v>5.220735061726474</v>
+      </c>
+      <c r="AB12" t="n">
         <v>0.14747760149254</v>
       </c>
-      <c r="AB12" t="n">
+      <c r="AC12" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1721,12 +1759,15 @@
         </is>
       </c>
       <c r="Z13" t="n">
-        <v>9.954689105241076</v>
+        <v>0.05209310462105093</v>
       </c>
       <c r="AA13" t="n">
+        <v>7.963751284192861</v>
+      </c>
+      <c r="AB13" t="n">
         <v>0.4242182057246524</v>
       </c>
-      <c r="AB13" t="n">
+      <c r="AC13" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1819,12 +1860,15 @@
         </is>
       </c>
       <c r="Z14" t="n">
-        <v>7.554562849164462</v>
+        <v>-0.7372686685282925</v>
       </c>
       <c r="AA14" t="n">
+        <v>3.005331827309629</v>
+      </c>
+      <c r="AB14" t="n">
         <v>0.2396676846426827</v>
       </c>
-      <c r="AB14" t="n">
+      <c r="AC14" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1915,12 +1959,15 @@
         </is>
       </c>
       <c r="Z15" t="n">
-        <v>7.624090202449995</v>
+        <v>-0.3857769922669705</v>
       </c>
       <c r="AA15" t="n">
+        <v>4.382201678317105</v>
+      </c>
+      <c r="AB15" t="n">
         <v>0.2449830286679799</v>
       </c>
-      <c r="AB15" t="inlineStr"/>
+      <c r="AC15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="1" t="inlineStr">
@@ -2011,12 +2058,15 @@
         </is>
       </c>
       <c r="Z16" t="n">
-        <v>6.138221904043838</v>
+        <v>-0.3784988149265142</v>
       </c>
       <c r="AA16" t="n">
+        <v>3.552867392179301</v>
+      </c>
+      <c r="AB16" t="n">
         <v>0.07024781883686648</v>
       </c>
-      <c r="AB16" t="n">
+      <c r="AC16" t="n">
         <v>1</v>
       </c>
     </row>
@@ -2107,12 +2157,15 @@
         </is>
       </c>
       <c r="Z17" t="n">
-        <v>1.093337782684775</v>
+        <v>-0.106334866837229</v>
       </c>
       <c r="AA17" t="n">
+        <v>0.8050617827000505</v>
+      </c>
+      <c r="AB17" t="n">
         <v>0.02548366643753203</v>
       </c>
-      <c r="AB17" t="inlineStr"/>
+      <c r="AC17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="1" t="inlineStr">
@@ -2201,12 +2254,15 @@
         </is>
       </c>
       <c r="Z18" t="n">
-        <v>6.345657991595703</v>
+        <v>0.1025126806099247</v>
       </c>
       <c r="AA18" t="n">
+        <v>5.076526393276562</v>
+      </c>
+      <c r="AB18" t="n">
         <v>0.1264299463715549</v>
       </c>
-      <c r="AB18" t="inlineStr"/>
+      <c r="AC18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="1" t="inlineStr">
@@ -2295,12 +2351,15 @@
         </is>
       </c>
       <c r="Z19" t="n">
-        <v>6.071828115395259</v>
+        <v>-0.005702120334786958</v>
       </c>
       <c r="AA19" t="n">
+        <v>4.836689242218585</v>
+      </c>
+      <c r="AB19" t="n">
         <v>0.09385969203103028</v>
       </c>
-      <c r="AB19" t="inlineStr"/>
+      <c r="AC19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="1" t="inlineStr">
@@ -2391,12 +2450,15 @@
         </is>
       </c>
       <c r="Z20" t="n">
-        <v>2.944742545229622</v>
+        <v>0.1676813539431903</v>
       </c>
       <c r="AA20" t="n">
+        <v>2.355794036183698</v>
+      </c>
+      <c r="AB20" t="n">
         <v>0.06737441718291154</v>
       </c>
-      <c r="AB20" t="n">
+      <c r="AC20" t="n">
         <v>1</v>
       </c>
     </row>
@@ -2489,12 +2551,15 @@
         </is>
       </c>
       <c r="Z21" t="n">
-        <v>8.541166373622811</v>
+        <v>0.233909062701661</v>
       </c>
       <c r="AA21" t="n">
+        <v>10.87057538461085</v>
+      </c>
+      <c r="AB21" t="n">
         <v>0.2271805668511316</v>
       </c>
-      <c r="AB21" t="n">
+      <c r="AC21" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2587,12 +2652,15 @@
         </is>
       </c>
       <c r="Z22" t="n">
-        <v>8.829752441346756</v>
+        <v>-1.324317442016135</v>
       </c>
       <c r="AA22" t="n">
+        <v>2.711251472281507</v>
+      </c>
+      <c r="AB22" t="n">
         <v>0.2195835643651847</v>
       </c>
-      <c r="AB22" t="n">
+      <c r="AC22" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2685,12 +2753,15 @@
         </is>
       </c>
       <c r="Z23" t="n">
-        <v>8.329762132495517</v>
+        <v>-3.304134634163204</v>
       </c>
       <c r="AA23" t="n">
+        <v>0.1482177555699337</v>
+      </c>
+      <c r="AB23" t="n">
         <v>0.1784313727751914</v>
       </c>
-      <c r="AB23" t="n">
+      <c r="AC23" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2783,12 +2854,15 @@
         </is>
       </c>
       <c r="Z24" t="n">
-        <v>8.083664764858113</v>
+        <v>-0.4724977598361445</v>
       </c>
       <c r="AA24" t="n">
+        <v>6.787723737469378</v>
+      </c>
+      <c r="AB24" t="n">
         <v>0.1937175918370535</v>
       </c>
-      <c r="AB24" t="n">
+      <c r="AC24" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2881,12 +2955,15 @@
         </is>
       </c>
       <c r="Z25" t="n">
-        <v>9.19081960565584</v>
+        <v>-0.2787931393192183</v>
       </c>
       <c r="AA25" t="n">
+        <v>9.286571654709743</v>
+      </c>
+      <c r="AB25" t="n">
         <v>0.2380084083818134</v>
       </c>
-      <c r="AB25" t="n">
+      <c r="AC25" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2979,12 +3056,15 @@
         </is>
       </c>
       <c r="Z26" t="n">
-        <v>6.487189703313851</v>
+        <v>0.1597641709074561</v>
       </c>
       <c r="AA26" t="n">
+        <v>8.256423258763084</v>
+      </c>
+      <c r="AB26" t="n">
         <v>0.05409556623689876</v>
       </c>
-      <c r="AB26" t="n">
+      <c r="AC26" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3077,12 +3157,15 @@
         </is>
       </c>
       <c r="Z27" t="n">
-        <v>1.294915183227309</v>
+        <v>0.04519770629871843</v>
       </c>
       <c r="AA27" t="n">
+        <v>1.648073869562029</v>
+      </c>
+      <c r="AB27" t="n">
         <v>0.004874845939002781</v>
       </c>
-      <c r="AB27" t="n">
+      <c r="AC27" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3175,12 +3258,15 @@
         </is>
       </c>
       <c r="Z28" t="n">
-        <v>6.382114641304581</v>
+        <v>0.1889867063411296</v>
       </c>
       <c r="AA28" t="n">
+        <v>8.122691361660376</v>
+      </c>
+      <c r="AB28" t="n">
         <v>0.06603995883164865</v>
       </c>
-      <c r="AB28" t="n">
+      <c r="AC28" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3273,12 +3359,15 @@
         </is>
       </c>
       <c r="Z29" t="n">
-        <v>6.030643055711809</v>
+        <v>0.1539913580373179</v>
       </c>
       <c r="AA29" t="n">
+        <v>7.675363889087756</v>
+      </c>
+      <c r="AB29" t="n">
         <v>0.003189790487149791</v>
       </c>
-      <c r="AB29" t="n">
+      <c r="AC29" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3371,12 +3460,15 @@
         </is>
       </c>
       <c r="Z30" t="n">
+        <v>0.07084681723937544</v>
+      </c>
+      <c r="AA30" t="n">
         <v>2.223441902327784</v>
       </c>
-      <c r="AA30" t="n">
+      <c r="AB30" t="n">
         <v>0.01759834784251979</v>
       </c>
-      <c r="AB30" t="n">
+      <c r="AC30" t="n">
         <v>1</v>
       </c>
     </row>
@@ -3469,12 +3561,15 @@
         </is>
       </c>
       <c r="Z31" t="n">
+        <v>0.4791006810653244</v>
+      </c>
+      <c r="AA31" t="n">
         <v>3.697076695236171</v>
       </c>
-      <c r="AA31" t="n">
+      <c r="AB31" t="n">
         <v>0.4076436874120243</v>
       </c>
-      <c r="AB31" t="n">
+      <c r="AC31" t="n">
         <v>1</v>
       </c>
     </row>
@@ -3565,12 +3660,15 @@
         </is>
       </c>
       <c r="Z32" t="n">
+        <v>0.030869434147157</v>
+      </c>
+      <c r="AA32" t="n">
         <v>0.502225992585953</v>
       </c>
-      <c r="AA32" t="n">
+      <c r="AB32" t="n">
         <v>0.002268490124341938</v>
       </c>
-      <c r="AB32" t="inlineStr"/>
+      <c r="AC32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="1" t="inlineStr">
@@ -3659,12 +3757,15 @@
         </is>
       </c>
       <c r="Z33" t="n">
+        <v>0.5315552753056412</v>
+      </c>
+      <c r="AA33" t="n">
         <v>4.813995436900988</v>
       </c>
-      <c r="AA33" t="n">
+      <c r="AB33" t="n">
         <v>0.65314611304167</v>
       </c>
-      <c r="AB33" t="inlineStr"/>
+      <c r="AC33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="1" t="inlineStr">
@@ -3755,12 +3856,15 @@
         </is>
       </c>
       <c r="Z34" t="n">
-        <v>4.488004046349071</v>
+        <v>-1.051994508526261</v>
       </c>
       <c r="AA34" t="n">
+        <v>1.535616231449598</v>
+      </c>
+      <c r="AB34" t="n">
         <v>0.5129523227565529</v>
       </c>
-      <c r="AB34" t="n">
+      <c r="AC34" t="n">
         <v>1</v>
       </c>
     </row>
@@ -3851,12 +3955,15 @@
         </is>
       </c>
       <c r="Z35" t="n">
+        <v>0.484567910788525</v>
+      </c>
+      <c r="AA35" t="n">
         <v>4.674603199170492</v>
       </c>
-      <c r="AA35" t="n">
+      <c r="AB35" t="n">
         <v>0.6503964625767549</v>
       </c>
-      <c r="AB35" t="inlineStr"/>
+      <c r="AC35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="1" t="inlineStr">
@@ -3947,12 +4054,15 @@
         </is>
       </c>
       <c r="Z36" t="n">
-        <v>3.285178970144163</v>
+        <v>-0.2462774903139367</v>
       </c>
       <c r="AA36" t="n">
+        <v>2.685187596594701</v>
+      </c>
+      <c r="AB36" t="n">
         <v>0.2723084567893851</v>
       </c>
-      <c r="AB36" t="n">
+      <c r="AC36" t="n">
         <v>1</v>
       </c>
     </row>
@@ -4043,12 +4153,15 @@
         </is>
       </c>
       <c r="Z37" t="n">
+        <v>0.7171142538650463</v>
+      </c>
+      <c r="AA37" t="n">
         <v>5.151342761595139</v>
       </c>
-      <c r="AA37" t="n">
+      <c r="AB37" t="n">
         <v>0.7687039407454913</v>
       </c>
-      <c r="AB37" t="inlineStr"/>
+      <c r="AC37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="1" t="inlineStr">
@@ -4139,12 +4252,15 @@
         </is>
       </c>
       <c r="Z38" t="n">
+        <v>0.215379727022584</v>
+      </c>
+      <c r="AA38" t="n">
         <v>2.861518908090336</v>
       </c>
-      <c r="AA38" t="n">
+      <c r="AB38" t="n">
         <v>0.06576960305185331</v>
       </c>
-      <c r="AB38" t="n">
+      <c r="AC38" t="n">
         <v>1</v>
       </c>
     </row>
@@ -4235,12 +4351,15 @@
         </is>
       </c>
       <c r="Z39" t="n">
+        <v>0.4309252547801569</v>
+      </c>
+      <c r="AA39" t="n">
         <v>3.561108234772101</v>
       </c>
-      <c r="AA39" t="n">
+      <c r="AB39" t="n">
         <v>0.2576680670387645</v>
       </c>
-      <c r="AB39" t="inlineStr"/>
+      <c r="AC39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="1" t="inlineStr">
@@ -4331,12 +4450,15 @@
         </is>
       </c>
       <c r="Z40" t="n">
-        <v>8.061378334788085</v>
+        <v>-0.1962001864429308</v>
       </c>
       <c r="AA40" t="n">
+        <v>6.883633771717943</v>
+      </c>
+      <c r="AB40" t="n">
         <v>0.2659946325921776</v>
       </c>
-      <c r="AB40" t="inlineStr"/>
+      <c r="AC40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="1" t="inlineStr">
@@ -4427,12 +4549,15 @@
         </is>
       </c>
       <c r="Z41" t="n">
+        <v>0.1225600091190399</v>
+      </c>
+      <c r="AA41" t="n">
         <v>5.653830089338093</v>
       </c>
-      <c r="AA41" t="n">
+      <c r="AB41" t="n">
         <v>0.03367945598509514</v>
       </c>
-      <c r="AB41" t="inlineStr"/>
+      <c r="AC41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="1" t="inlineStr">
@@ -4523,12 +4648,15 @@
         </is>
       </c>
       <c r="Z42" t="n">
-        <v>9.155368841733628</v>
+        <v>-0.2983547550152528</v>
       </c>
       <c r="AA42" t="n">
+        <v>7.140229744879822</v>
+      </c>
+      <c r="AB42" t="n">
         <v>0.4057672136872293</v>
       </c>
-      <c r="AB42" t="inlineStr"/>
+      <c r="AC42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="1" t="inlineStr">
@@ -4619,12 +4747,15 @@
         </is>
       </c>
       <c r="Z43" t="n">
-        <v>11.31629084912677</v>
+        <v>-0.2352459582624117</v>
       </c>
       <c r="AA43" t="n">
+        <v>9.340169630520823</v>
+      </c>
+      <c r="AB43" t="n">
         <v>0.6428508882537345</v>
       </c>
-      <c r="AB43" t="inlineStr"/>
+      <c r="AC43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="1" t="inlineStr">
@@ -4715,12 +4846,15 @@
         </is>
       </c>
       <c r="Z44" t="n">
+        <v>0.06803978365180074</v>
+      </c>
+      <c r="AA44" t="n">
         <v>7.60978345851908</v>
       </c>
-      <c r="AA44" t="n">
+      <c r="AB44" t="n">
         <v>0.1577477966534874</v>
       </c>
-      <c r="AB44" t="inlineStr"/>
+      <c r="AC44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="1" t="inlineStr">
@@ -4811,12 +4945,15 @@
         </is>
       </c>
       <c r="Z45" t="n">
-        <v>10.50368517683753</v>
+        <v>-0.1694485473392826</v>
       </c>
       <c r="AA45" t="n">
+        <v>9.175949910430854</v>
+      </c>
+      <c r="AB45" t="n">
         <v>0.5447074706177735</v>
       </c>
-      <c r="AB45" t="inlineStr"/>
+      <c r="AC45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="1" t="inlineStr">
@@ -4907,12 +5044,15 @@
         </is>
       </c>
       <c r="Z46" t="n">
+        <v>0.1432742327202653</v>
+      </c>
+      <c r="AA46" t="n">
         <v>9.671871681098917</v>
       </c>
-      <c r="AA46" t="n">
+      <c r="AB46" t="n">
         <v>0.4397563214272065</v>
       </c>
-      <c r="AB46" t="inlineStr"/>
+      <c r="AC46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="1" t="inlineStr">
@@ -5003,12 +5143,15 @@
         </is>
       </c>
       <c r="Z47" t="n">
-        <v>9.457378331909212</v>
+        <v>-0.1370965361217912</v>
       </c>
       <c r="AA47" t="n">
+        <v>8.488360532694404</v>
+      </c>
+      <c r="AB47" t="n">
         <v>0.4242933439703247</v>
       </c>
-      <c r="AB47" t="inlineStr"/>
+      <c r="AC47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="1" t="inlineStr">
@@ -5099,12 +5242,15 @@
         </is>
       </c>
       <c r="Z48" t="n">
+        <v>0.1469301082308789</v>
+      </c>
+      <c r="AA48" t="n">
         <v>5.892580904074391</v>
       </c>
-      <c r="AA48" t="n">
+      <c r="AB48" t="n">
         <v>0.09870931369954694</v>
       </c>
-      <c r="AB48" t="inlineStr"/>
+      <c r="AC48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="1" t="inlineStr">
@@ -5195,12 +5341,15 @@
         </is>
       </c>
       <c r="Z49" t="n">
-        <v>5.389064199140495</v>
+        <v>-0.08242750523819817</v>
       </c>
       <c r="AA49" t="n">
+        <v>5.056332629800196</v>
+      </c>
+      <c r="AB49" t="n">
         <v>0.06461254905152419</v>
       </c>
-      <c r="AB49" t="inlineStr"/>
+      <c r="AC49" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
DATA. Actualizo predicciones tras cambio de modelos (x nuevas metricas "expected")
</commit_message>
<xml_diff>
--- a/data/predicciones.xlsx
+++ b/data/predicciones.xlsx
@@ -639,13 +639,13 @@
         <v>0</v>
       </c>
       <c r="Q2" t="n">
-        <v>0.4982005786910595</v>
+        <v>0.5514088007950597</v>
       </c>
       <c r="R2" t="n">
-        <v>0.1094502552755841</v>
+        <v>0.1864201147517175</v>
       </c>
       <c r="S2" t="n">
-        <v>0.3923491660333565</v>
+        <v>0.2621710844532226</v>
       </c>
       <c r="T2" t="n">
         <v>1</v>
@@ -657,7 +657,7 @@
         <v>0</v>
       </c>
       <c r="W2" t="n">
-        <v>0.4982005786910595</v>
+        <v>0.5514088007950597</v>
       </c>
       <c r="X2" t="n">
         <v>3.7</v>
@@ -668,13 +668,13 @@
         </is>
       </c>
       <c r="Z2" t="n">
-        <v>0.3123489411692298</v>
+        <v>0.3852639122006374</v>
       </c>
       <c r="AA2" t="n">
-        <v>5.978406944292715</v>
+        <v>6.616905609540717</v>
       </c>
       <c r="AB2" t="n">
-        <v>0.1058514126577031</v>
+        <v>0.2892377163418371</v>
       </c>
       <c r="AC2" t="inlineStr"/>
     </row>
@@ -738,13 +738,13 @@
         <v>0</v>
       </c>
       <c r="Q3" t="n">
-        <v>0.4850447658361123</v>
+        <v>0.5827899500827602</v>
       </c>
       <c r="R3" t="n">
-        <v>0.3014918331327296</v>
+        <v>0.2160531114444568</v>
       </c>
       <c r="S3" t="n">
-        <v>0.2134634010311582</v>
+        <v>0.2011569384727831</v>
       </c>
       <c r="T3" t="n">
         <v>1</v>
@@ -756,7 +756,7 @@
         <v>0</v>
       </c>
       <c r="W3" t="n">
-        <v>0.4850447658361123</v>
+        <v>0.5827899500827602</v>
       </c>
       <c r="X3" t="n">
         <v>3.6</v>
@@ -767,13 +767,13 @@
         </is>
       </c>
       <c r="Z3" t="n">
-        <v>0.2869850603884632</v>
+        <v>0.4223245462684373</v>
       </c>
       <c r="AA3" t="n">
-        <v>5.820537190033348</v>
+        <v>6.993479400993123</v>
       </c>
       <c r="AB3" t="n">
-        <v>0.1835529327033827</v>
+        <v>0.3667368386383034</v>
       </c>
       <c r="AC3" t="inlineStr"/>
     </row>
@@ -834,16 +834,16 @@
         <v>0.0578978978978979</v>
       </c>
       <c r="P4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q4" t="n">
-        <v>0.4077449006273495</v>
+        <v>0.1947227671567085</v>
       </c>
       <c r="R4" t="n">
-        <v>0.3906415946053324</v>
+        <v>0.6297223722167766</v>
       </c>
       <c r="S4" t="n">
-        <v>0.2016135047673183</v>
+        <v>0.1755548606265148</v>
       </c>
       <c r="T4" t="n">
         <v>1</v>
@@ -852,13 +852,13 @@
         <v>0</v>
       </c>
       <c r="V4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W4" t="n">
-        <v>0.4077449006273495</v>
+        <v>0.6297223722167766</v>
       </c>
       <c r="X4" t="n">
-        <v>4.5</v>
+        <v>1.48</v>
       </c>
       <c r="Y4" t="inlineStr">
         <is>
@@ -866,13 +866,13 @@
         </is>
       </c>
       <c r="Z4" t="n">
-        <v>0.2385291579494493</v>
+        <v>-0.1416893523316054</v>
       </c>
       <c r="AA4" t="n">
-        <v>4.892938807528194</v>
+        <v>6.756653045210631</v>
       </c>
       <c r="AB4" t="n">
-        <v>0.0171033060220171</v>
+        <v>0.4349996050600681</v>
       </c>
       <c r="AC4" t="inlineStr"/>
     </row>
@@ -936,13 +936,13 @@
         <v>1</v>
       </c>
       <c r="Q5" t="n">
-        <v>0.1363746778628798</v>
+        <v>0.2295655294875229</v>
       </c>
       <c r="R5" t="n">
-        <v>0.8517863362561515</v>
+        <v>0.7625855778392395</v>
       </c>
       <c r="S5" t="n">
-        <v>0.0118389858809687</v>
+        <v>0.007848892673237635</v>
       </c>
       <c r="T5" t="n">
         <v>1</v>
@@ -954,7 +954,7 @@
         <v>1</v>
       </c>
       <c r="W5" t="n">
-        <v>0.8517863362561515</v>
+        <v>0.7625855778392395</v>
       </c>
       <c r="X5" t="n">
         <v>1.13</v>
@@ -965,13 +965,13 @@
         </is>
       </c>
       <c r="Z5" t="n">
-        <v>-0.2883187694657608</v>
+        <v>-1.063679208012766</v>
       </c>
       <c r="AA5" t="n">
-        <v>8.044980074129807</v>
+        <v>3.085888344508815</v>
       </c>
       <c r="AB5" t="n">
-        <v>0.7154116583932717</v>
+        <v>0.5330200483517167</v>
       </c>
       <c r="AC5" t="inlineStr"/>
     </row>
@@ -1035,13 +1035,13 @@
         <v>1</v>
       </c>
       <c r="Q6" t="n">
-        <v>0.1596133327429995</v>
+        <v>0.2097913099757538</v>
       </c>
       <c r="R6" t="n">
-        <v>0.7016126321125952</v>
+        <v>0.5574935669348491</v>
       </c>
       <c r="S6" t="n">
-        <v>0.1387740351444053</v>
+        <v>0.2327151230893972</v>
       </c>
       <c r="T6" t="n">
         <v>1</v>
@@ -1053,7 +1053,7 @@
         <v>1</v>
       </c>
       <c r="W6" t="n">
-        <v>0.7016126321125952</v>
+        <v>0.5574935669348491</v>
       </c>
       <c r="X6" t="n">
         <v>2.25</v>
@@ -1064,13 +1064,13 @@
         </is>
       </c>
       <c r="Z6" t="n">
-        <v>0.4629027378026713</v>
+        <v>0.2034884204827284</v>
       </c>
       <c r="AA6" t="n">
-        <v>8.419351585351142</v>
+        <v>6.68992280321819</v>
       </c>
       <c r="AB6" t="n">
-        <v>0.5419992993695957</v>
+        <v>0.324778443845452</v>
       </c>
       <c r="AC6" t="inlineStr"/>
     </row>
@@ -1131,16 +1131,16 @@
         <v>0.05441825199889694</v>
       </c>
       <c r="P7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q7" t="n">
-        <v>0.2838230181993255</v>
+        <v>0.09786527624959518</v>
       </c>
       <c r="R7" t="n">
-        <v>0.2714583995516209</v>
+        <v>0.5723991027817534</v>
       </c>
       <c r="S7" t="n">
-        <v>0.4447185822490536</v>
+        <v>0.3297356209686514</v>
       </c>
       <c r="T7" t="n">
         <v>1</v>
@@ -1149,13 +1149,13 @@
         <v>0</v>
       </c>
       <c r="V7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="W7" t="n">
-        <v>0.4447185822490536</v>
+        <v>0.5723991027817534</v>
       </c>
       <c r="X7" t="n">
-        <v>2.88</v>
+        <v>2.6</v>
       </c>
       <c r="Y7" t="inlineStr">
         <is>
@@ -1163,13 +1163,13 @@
         </is>
       </c>
       <c r="Z7" t="n">
-        <v>0.1493561259985502</v>
+        <v>0.3051485420203494</v>
       </c>
       <c r="AA7" t="n">
-        <v>5.336622986988644</v>
+        <v>6.868789233381041</v>
       </c>
       <c r="AB7" t="n">
-        <v>0.160895564049728</v>
+        <v>0.242663481813102</v>
       </c>
       <c r="AC7" t="inlineStr"/>
     </row>
@@ -1233,13 +1233,13 @@
         <v>1</v>
       </c>
       <c r="Q8" t="n">
-        <v>0.1953066937510947</v>
+        <v>0.1963709267525796</v>
       </c>
       <c r="R8" t="n">
-        <v>0.7845141642092379</v>
+        <v>0.739469736955859</v>
       </c>
       <c r="S8" t="n">
-        <v>0.02017914203966726</v>
+        <v>0.06415933629156136</v>
       </c>
       <c r="T8" t="n">
         <v>1</v>
@@ -1251,7 +1251,7 @@
         <v>1</v>
       </c>
       <c r="W8" t="n">
-        <v>0.7845141642092379</v>
+        <v>0.739469736955859</v>
       </c>
       <c r="X8" t="n">
         <v>1.2</v>
@@ -1262,13 +1262,13 @@
         </is>
       </c>
       <c r="Z8" t="n">
-        <v>-0.2929150147445727</v>
+        <v>-0.5631815782648459</v>
       </c>
       <c r="AA8" t="n">
-        <v>7.37864745621538</v>
+        <v>5.333599186841439</v>
       </c>
       <c r="AB8" t="n">
-        <v>0.5892074704581431</v>
+        <v>0.5430988102032794</v>
       </c>
       <c r="AC8" t="inlineStr"/>
     </row>
@@ -1329,16 +1329,16 @@
         <v>0.04918890633176343</v>
       </c>
       <c r="P9" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="Q9" t="n">
-        <v>0.662901904210674</v>
+        <v>0.1680187960963603</v>
       </c>
       <c r="R9" t="n">
-        <v>0.2207364295117329</v>
+        <v>0.4074187205955229</v>
       </c>
       <c r="S9" t="n">
-        <v>0.1163616662775931</v>
+        <v>0.4245624833081167</v>
       </c>
       <c r="T9" t="n">
         <v>1</v>
@@ -1347,13 +1347,13 @@
         <v>0</v>
       </c>
       <c r="V9" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="W9" t="n">
-        <v>0.662901904210674</v>
+        <v>0.4245624833081167</v>
       </c>
       <c r="X9" t="n">
-        <v>3.9</v>
+        <v>2.45</v>
       </c>
       <c r="Y9" t="inlineStr">
         <is>
@@ -1361,13 +1361,13 @@
         </is>
       </c>
       <c r="Z9" t="n">
-        <v>0.5466611815246996</v>
+        <v>0.0277090235206111</v>
       </c>
       <c r="AA9" t="n">
-        <v>7.954822850528088</v>
+        <v>1.01894995993948</v>
       </c>
       <c r="AB9" t="n">
-        <v>0.4421654746989411</v>
+        <v>0.01714376271259382</v>
       </c>
       <c r="AC9" t="inlineStr"/>
     </row>
@@ -1428,16 +1428,16 @@
         <v>0.06554621848739495</v>
       </c>
       <c r="P10" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="Q10" t="n">
-        <v>0.3369429364671985</v>
+        <v>0.3708849880957994</v>
       </c>
       <c r="R10" t="n">
-        <v>0.125943683291328</v>
+        <v>0.2709349201010102</v>
       </c>
       <c r="S10" t="n">
-        <v>0.5371133802414736</v>
+        <v>0.3581800918031903</v>
       </c>
       <c r="T10" t="n">
         <v>1</v>
@@ -1446,13 +1446,13 @@
         <v>0</v>
       </c>
       <c r="V10" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="W10" t="n">
-        <v>0.5371133802414736</v>
+        <v>0.3708849880957994</v>
       </c>
       <c r="X10" t="n">
-        <v>1.75</v>
+        <v>3.4</v>
       </c>
       <c r="Y10" t="inlineStr">
         <is>
@@ -1460,13 +1460,13 @@
         </is>
       </c>
       <c r="Z10" t="n">
-        <v>-0.08006877943656161</v>
+        <v>0.1087537331357158</v>
       </c>
       <c r="AA10" t="n">
-        <v>6.058771041690684</v>
+        <v>4.450619857149593</v>
       </c>
       <c r="AB10" t="n">
-        <v>0.2001704437742751</v>
+        <v>0.01270489629260907</v>
       </c>
       <c r="AC10" t="inlineStr"/>
     </row>
@@ -1530,13 +1530,13 @@
         <v>2</v>
       </c>
       <c r="Q11" t="n">
-        <v>0.338151969697943</v>
+        <v>0.2645188113516988</v>
       </c>
       <c r="R11" t="n">
-        <v>0.2846664091585874</v>
+        <v>0.2020350498911804</v>
       </c>
       <c r="S11" t="n">
-        <v>0.3771816211434696</v>
+        <v>0.5334461387571208</v>
       </c>
       <c r="T11" t="n">
         <v>1</v>
@@ -1548,7 +1548,7 @@
         <v>2</v>
       </c>
       <c r="W11" t="n">
-        <v>0.3771816211434696</v>
+        <v>0.5334461387571208</v>
       </c>
       <c r="X11" t="n">
         <v>2.25</v>
@@ -1559,13 +1559,13 @@
         </is>
       </c>
       <c r="Z11" t="n">
-        <v>-0.1210730819417546</v>
+        <v>0.1602030497628174</v>
       </c>
       <c r="AA11" t="n">
-        <v>0.823261300146111</v>
+        <v>6.401353665085449</v>
       </c>
       <c r="AB11" t="n">
-        <v>0.03902965144552667</v>
+        <v>0.268927327405422</v>
       </c>
       <c r="AC11" t="inlineStr"/>
     </row>
@@ -1629,23 +1629,25 @@
         <v>2</v>
       </c>
       <c r="Q12" t="n">
-        <v>0.3750407534589282</v>
+        <v>0.2991559921137829</v>
       </c>
       <c r="R12" t="n">
-        <v>0.1980487800083202</v>
+        <v>0.2542104142798942</v>
       </c>
       <c r="S12" t="n">
-        <v>0.4269104665327516</v>
+        <v>0.4466335936063229</v>
       </c>
       <c r="T12" t="n">
         <v>1</v>
       </c>
-      <c r="U12" t="inlineStr"/>
+      <c r="U12" t="n">
+        <v>0</v>
+      </c>
       <c r="V12" t="n">
         <v>2</v>
       </c>
       <c r="W12" t="n">
-        <v>0.4269104665327516</v>
+        <v>0.4466335936063229</v>
       </c>
       <c r="X12" t="n">
         <v>2.15</v>
@@ -1656,15 +1658,17 @@
         </is>
       </c>
       <c r="Z12" t="n">
-        <v>-0.07142825822137742</v>
+        <v>-0.03455458586643988</v>
       </c>
       <c r="AA12" t="n">
-        <v>6.464995460191645</v>
+        <v>6.960980082301965</v>
       </c>
       <c r="AB12" t="n">
-        <v>0.05186971307382343</v>
-      </c>
-      <c r="AC12" t="inlineStr"/>
+        <v>0.14747760149254</v>
+      </c>
+      <c r="AC12" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
@@ -1726,13 +1730,13 @@
         <v>2</v>
       </c>
       <c r="Q13" t="n">
-        <v>0.2669596712453156</v>
+        <v>0.2394277346247528</v>
       </c>
       <c r="R13" t="n">
-        <v>0.09232304218936477</v>
+        <v>0.09692632502584211</v>
       </c>
       <c r="S13" t="n">
-        <v>0.6407172865653196</v>
+        <v>0.6636459403494052</v>
       </c>
       <c r="T13" t="n">
         <v>1</v>
@@ -1744,7 +1748,7 @@
         <v>2</v>
       </c>
       <c r="W13" t="n">
-        <v>0.6407172865653196</v>
+        <v>0.6636459403494052</v>
       </c>
       <c r="X13" t="n">
         <v>1.65</v>
@@ -1755,13 +1759,13 @@
         </is>
       </c>
       <c r="Z13" t="n">
-        <v>0.08797465051196497</v>
+        <v>0.1461781562715669</v>
       </c>
       <c r="AA13" t="n">
-        <v>10.25147658504511</v>
+        <v>10.61833504559048</v>
       </c>
       <c r="AB13" t="n">
-        <v>0.373757615320004</v>
+        <v>0.4242182057246524</v>
       </c>
       <c r="AC13" t="n">
         <v>1</v>
@@ -1827,23 +1831,25 @@
         <v>1</v>
       </c>
       <c r="Q14" t="n">
-        <v>0.2953553308409347</v>
+        <v>0.2639698386349481</v>
       </c>
       <c r="R14" t="n">
-        <v>0.5450609350201607</v>
+        <v>0.5036375232776308</v>
       </c>
       <c r="S14" t="n">
-        <v>0.1595837341389047</v>
+        <v>0.2323926380874211</v>
       </c>
       <c r="T14" t="n">
         <v>1</v>
       </c>
-      <c r="U14" t="inlineStr"/>
+      <c r="U14" t="n">
+        <v>0</v>
+      </c>
       <c r="V14" t="n">
         <v>1</v>
       </c>
       <c r="W14" t="n">
-        <v>0.5450609350201607</v>
+        <v>0.5036375232776308</v>
       </c>
       <c r="X14" t="n">
         <v>1.4</v>
@@ -1854,15 +1860,17 @@
         </is>
       </c>
       <c r="Z14" t="n">
-        <v>-0.5922867274294377</v>
+        <v>-0.7372686685282925</v>
       </c>
       <c r="AA14" t="n">
-        <v>5.083175623685854</v>
+        <v>4.007109103079506</v>
       </c>
       <c r="AB14" t="n">
-        <v>0.249705604179226</v>
-      </c>
-      <c r="AC14" t="inlineStr"/>
+        <v>0.2396676846426827</v>
+      </c>
+      <c r="AC14" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="inlineStr">
@@ -1924,13 +1932,13 @@
         <v>1</v>
       </c>
       <c r="Q15" t="n">
-        <v>0.2817916266045167</v>
+        <v>0.2632896514953531</v>
       </c>
       <c r="R15" t="n">
-        <v>0.5405911151090551</v>
+        <v>0.508272680163333</v>
       </c>
       <c r="S15" t="n">
-        <v>0.1776172582864282</v>
+        <v>0.2284376683413138</v>
       </c>
       <c r="T15" t="n">
         <v>1</v>
@@ -1940,7 +1948,7 @@
         <v>1</v>
       </c>
       <c r="W15" t="n">
-        <v>0.5405911151090551</v>
+        <v>0.508272680163333</v>
       </c>
       <c r="X15" t="n">
         <v>1.55</v>
@@ -1951,13 +1959,13 @@
         </is>
       </c>
       <c r="Z15" t="n">
-        <v>-0.2946977665108446</v>
+        <v>-0.3857769922669705</v>
       </c>
       <c r="AA15" t="n">
-        <v>6.768259608325794</v>
+        <v>5.842935571089474</v>
       </c>
       <c r="AB15" t="n">
-        <v>0.2587994885045384</v>
+        <v>0.2449830286679799</v>
       </c>
       <c r="AC15" t="inlineStr"/>
     </row>
@@ -2021,13 +2029,13 @@
         <v>1</v>
       </c>
       <c r="Q16" t="n">
-        <v>0.355622758643497</v>
+        <v>0.338966974766056</v>
       </c>
       <c r="R16" t="n">
-        <v>0.4551879783290751</v>
+        <v>0.4092147936029225</v>
       </c>
       <c r="S16" t="n">
-        <v>0.1891892630274278</v>
+        <v>0.2518182316310215</v>
       </c>
       <c r="T16" t="n">
         <v>1</v>
@@ -2039,7 +2047,7 @@
         <v>1</v>
       </c>
       <c r="W16" t="n">
-        <v>0.4551879783290751</v>
+        <v>0.4092147936029225</v>
       </c>
       <c r="X16" t="n">
         <v>1.73</v>
@@ -2050,13 +2058,13 @@
         </is>
       </c>
       <c r="Z16" t="n">
-        <v>-0.2911298595763015</v>
+        <v>-0.4000800096807454</v>
       </c>
       <c r="AA16" t="n">
-        <v>5.717580741736086</v>
+        <v>4.639726263096001</v>
       </c>
       <c r="AB16" t="n">
-        <v>0.09956521968557819</v>
+        <v>0.07024781883686648</v>
       </c>
       <c r="AC16" t="n">
         <v>1</v>
@@ -2122,13 +2130,13 @@
         <v>1</v>
       </c>
       <c r="Q17" t="n">
-        <v>0.27462468521776</v>
+        <v>0.2965918113143484</v>
       </c>
       <c r="R17" t="n">
-        <v>0.366948622755483</v>
+        <v>0.3644459275615918</v>
       </c>
       <c r="S17" t="n">
-        <v>0.3584266920267571</v>
+        <v>0.3389622611240598</v>
       </c>
       <c r="T17" t="n">
         <v>1</v>
@@ -2138,7 +2146,7 @@
         <v>1</v>
       </c>
       <c r="W17" t="n">
-        <v>0.366948622755483</v>
+        <v>0.3644459275615918</v>
       </c>
       <c r="X17" t="n">
         <v>2.35</v>
@@ -2149,13 +2157,13 @@
         </is>
       </c>
       <c r="Z17" t="n">
-        <v>-0.1019783233515666</v>
+        <v>-0.106334866837229</v>
       </c>
       <c r="AA17" t="n">
-        <v>1.084600373554454</v>
+        <v>1.073415710266734</v>
       </c>
       <c r="AB17" t="n">
-        <v>0.008521930728725813</v>
+        <v>0.02548366643753203</v>
       </c>
       <c r="AC17" t="inlineStr"/>
     </row>
@@ -2219,13 +2227,13 @@
         <v>2</v>
       </c>
       <c r="Q18" t="n">
-        <v>0.270480231315141</v>
+        <v>0.2966139197348253</v>
       </c>
       <c r="R18" t="n">
-        <v>0.2035954667252323</v>
+        <v>0.2803422141587946</v>
       </c>
       <c r="S18" t="n">
-        <v>0.5259243019596266</v>
+        <v>0.4230438661063802</v>
       </c>
       <c r="T18" t="n">
         <v>1</v>
@@ -2235,7 +2243,7 @@
         <v>2</v>
       </c>
       <c r="W18" t="n">
-        <v>0.5259243019596266</v>
+        <v>0.4230438661063802</v>
       </c>
       <c r="X18" t="n">
         <v>2.75</v>
@@ -2246,13 +2254,13 @@
         </is>
       </c>
       <c r="Z18" t="n">
-        <v>0.2550239030794132</v>
+        <v>0.09335464673859743</v>
       </c>
       <c r="AA18" t="n">
-        <v>8.414788831354025</v>
+        <v>6.768701857702083</v>
       </c>
       <c r="AB18" t="n">
-        <v>0.2554440706444855</v>
+        <v>0.1264299463715549</v>
       </c>
       <c r="AC18" t="inlineStr"/>
     </row>
@@ -2313,29 +2321,29 @@
         <v>0.05303030303030298</v>
       </c>
       <c r="P19" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q19" t="n">
-        <v>0.4275852402369614</v>
+        <v>0.2842826099783292</v>
       </c>
       <c r="R19" t="n">
-        <v>0.3710925465319584</v>
+        <v>0.4047885410263506</v>
       </c>
       <c r="S19" t="n">
-        <v>0.2013222132310802</v>
+        <v>0.3109288489953203</v>
       </c>
       <c r="T19" t="n">
         <v>1</v>
       </c>
       <c r="U19" t="inlineStr"/>
       <c r="V19" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W19" t="n">
-        <v>0.4275852402369614</v>
+        <v>0.4047885410263506</v>
       </c>
       <c r="X19" t="n">
-        <v>3.3</v>
+        <v>2.4</v>
       </c>
       <c r="Y19" t="inlineStr">
         <is>
@@ -2343,13 +2351,13 @@
         </is>
       </c>
       <c r="Z19" t="n">
-        <v>0.1787092577312923</v>
+        <v>-0.02036250109768474</v>
       </c>
       <c r="AA19" t="n">
-        <v>6.841363843791382</v>
+        <v>6.377714259978583</v>
       </c>
       <c r="AB19" t="n">
-        <v>0.05649269370500298</v>
+        <v>0.09385969203103028</v>
       </c>
       <c r="AC19" t="inlineStr"/>
     </row>
@@ -2410,31 +2418,31 @@
         <v>0.05598455598455576</v>
       </c>
       <c r="P20" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q20" t="n">
-        <v>0.3102330412558623</v>
+        <v>0.3926323393639496</v>
       </c>
       <c r="R20" t="n">
-        <v>0.4086656689504178</v>
+        <v>0.2821097384550122</v>
       </c>
       <c r="S20" t="n">
-        <v>0.28110128979372</v>
+        <v>0.3252579221810381</v>
       </c>
       <c r="T20" t="n">
         <v>1</v>
       </c>
       <c r="U20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V20" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="W20" t="n">
-        <v>0.4086656689504178</v>
+        <v>0.3926323393639496</v>
       </c>
       <c r="X20" t="n">
-        <v>2</v>
+        <v>3.7</v>
       </c>
       <c r="Y20" t="inlineStr">
         <is>
@@ -2442,13 +2450,13 @@
         </is>
       </c>
       <c r="Z20" t="n">
-        <v>-0.1826686620991644</v>
+        <v>0.1676813539431903</v>
       </c>
       <c r="AA20" t="n">
-        <v>5.648408587410632</v>
+        <v>3.141058714911598</v>
       </c>
       <c r="AB20" t="n">
-        <v>0.09843262769455552</v>
+        <v>0.06737441718291154</v>
       </c>
       <c r="AC20" t="n">
         <v>1</v>
@@ -2514,13 +2522,13 @@
         <v>2</v>
       </c>
       <c r="Q21" t="n">
-        <v>0.2453179425501339</v>
+        <v>0.09321833817535242</v>
       </c>
       <c r="R21" t="n">
-        <v>0.3070471961346672</v>
+        <v>0.2517790682380885</v>
       </c>
       <c r="S21" t="n">
-        <v>0.447634861315199</v>
+        <v>0.6550025935865591</v>
       </c>
       <c r="T21" t="n">
         <v>1</v>
@@ -2532,7 +2540,7 @@
         <v>2</v>
       </c>
       <c r="W21" t="n">
-        <v>0.447634861315199</v>
+        <v>0.6550025935865591</v>
       </c>
       <c r="X21" t="n">
         <v>2.7</v>
@@ -2543,13 +2551,13 @@
         </is>
       </c>
       <c r="Z21" t="n">
-        <v>0.1227141915006102</v>
+        <v>0.4520629427551233</v>
       </c>
       <c r="AA21" t="n">
-        <v>7.162157781043184</v>
+        <v>10.48004149738495</v>
       </c>
       <c r="AB21" t="n">
-        <v>0.1405876651805318</v>
+        <v>0.4032235253484706</v>
       </c>
       <c r="AC21" t="n">
         <v>0</v>
@@ -2615,13 +2623,13 @@
         <v>1</v>
       </c>
       <c r="Q22" t="n">
-        <v>0.1706621496857801</v>
+        <v>0.4327495622772096</v>
       </c>
       <c r="R22" t="n">
-        <v>0.7911210300153418</v>
+        <v>0.5296491031343392</v>
       </c>
       <c r="S22" t="n">
-        <v>0.03821682029887809</v>
+        <v>0.03760133458845114</v>
       </c>
       <c r="T22" t="n">
         <v>1</v>
@@ -2633,7 +2641,7 @@
         <v>1</v>
       </c>
       <c r="W22" t="n">
-        <v>0.7911210300153418</v>
+        <v>0.5296491031343392</v>
       </c>
       <c r="X22" t="n">
         <v>1.27</v>
@@ -2644,13 +2652,13 @@
         </is>
       </c>
       <c r="Z22" t="n">
-        <v>0.01749521525734876</v>
+        <v>-1.212391255627367</v>
       </c>
       <c r="AA22" t="n">
-        <v>12.65793648024547</v>
+        <v>2.366108169665149</v>
       </c>
       <c r="AB22" t="n">
-        <v>0.6204588803295618</v>
+        <v>0.09689954085712965</v>
       </c>
       <c r="AC22" t="n">
         <v>0</v>
@@ -2716,13 +2724,13 @@
         <v>1</v>
       </c>
       <c r="Q23" t="n">
-        <v>0.123409782677124</v>
+        <v>0.2084222312718251</v>
       </c>
       <c r="R23" t="n">
-        <v>0.8557987879198172</v>
+        <v>0.7496278091023392</v>
       </c>
       <c r="S23" t="n">
-        <v>0.02079142940305879</v>
+        <v>0.04194995962583581</v>
       </c>
       <c r="T23" t="n">
         <v>1</v>
@@ -2734,7 +2742,7 @@
         <v>1</v>
       </c>
       <c r="W23" t="n">
-        <v>0.8557987879198172</v>
+        <v>0.7496278091023392</v>
       </c>
       <c r="X23" t="n">
         <v>1.11</v>
@@ -2745,13 +2753,13 @@
         </is>
       </c>
       <c r="Z23" t="n">
-        <v>-0.455121321900025</v>
+        <v>-1.52648301724003</v>
       </c>
       <c r="AA23" t="n">
-        <v>9.192318946823553</v>
+        <v>2.20636584070299</v>
       </c>
       <c r="AB23" t="n">
-        <v>0.7323890052426932</v>
+        <v>0.541205577830514</v>
       </c>
       <c r="AC23" t="n">
         <v>0</v>
@@ -2817,13 +2825,13 @@
         <v>1</v>
       </c>
       <c r="Q24" t="n">
-        <v>0.1231974161779005</v>
+        <v>0.2535609101968603</v>
       </c>
       <c r="R24" t="n">
-        <v>0.8099379305971018</v>
+        <v>0.7026090506388647</v>
       </c>
       <c r="S24" t="n">
-        <v>0.06686465322499768</v>
+        <v>0.04383003916427512</v>
       </c>
       <c r="T24" t="n">
         <v>1</v>
@@ -2835,7 +2843,7 @@
         <v>1</v>
       </c>
       <c r="W24" t="n">
-        <v>0.8099379305971018</v>
+        <v>0.7026090506388647</v>
       </c>
       <c r="X24" t="n">
         <v>1.53</v>
@@ -2846,13 +2854,13 @@
         </is>
       </c>
       <c r="Z24" t="n">
-        <v>0.4513302524784261</v>
+        <v>0.1414940518442698</v>
       </c>
       <c r="AA24" t="n">
-        <v>12.95900688955363</v>
+        <v>11.24174481022184</v>
       </c>
       <c r="AB24" t="n">
-        <v>0.6867405144192014</v>
+        <v>0.4490481404420044</v>
       </c>
       <c r="AC24" t="n">
         <v>0</v>
@@ -2918,13 +2926,13 @@
         <v>2</v>
       </c>
       <c r="Q25" t="n">
-        <v>0.2284380018054831</v>
+        <v>0.139561601889736</v>
       </c>
       <c r="R25" t="n">
-        <v>0.02772674879869746</v>
+        <v>0.05548625024637604</v>
       </c>
       <c r="S25" t="n">
-        <v>0.7438352493958195</v>
+        <v>0.8049521478638879</v>
       </c>
       <c r="T25" t="n">
         <v>1</v>
@@ -2936,7 +2944,7 @@
         <v>2</v>
       </c>
       <c r="W25" t="n">
-        <v>0.7438352493958195</v>
+        <v>0.8049521478638879</v>
       </c>
       <c r="X25" t="n">
         <v>1.53</v>
@@ -2947,13 +2955,13 @@
         </is>
       </c>
       <c r="Z25" t="n">
-        <v>0.2605055312747242</v>
+        <v>0.4369373325127331</v>
       </c>
       <c r="AA25" t="n">
-        <v>11.90136399033311</v>
+        <v>12.87923436582221</v>
       </c>
       <c r="AB25" t="n">
-        <v>0.5153972475903363</v>
+        <v>0.6653905459741519</v>
       </c>
       <c r="AC25" t="n">
         <v>0</v>
@@ -3016,16 +3024,16 @@
         <v>0.04920634920634925</v>
       </c>
       <c r="P26" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q26" t="n">
-        <v>0.319589530900913</v>
+        <v>0.4242969450579085</v>
       </c>
       <c r="R26" t="n">
-        <v>0.5256827584459104</v>
+        <v>0.3535073925059247</v>
       </c>
       <c r="S26" t="n">
-        <v>0.1547277106531766</v>
+        <v>0.2221956624361668</v>
       </c>
       <c r="T26" t="n">
         <v>1</v>
@@ -3034,13 +3042,13 @@
         <v>0</v>
       </c>
       <c r="V26" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="W26" t="n">
-        <v>0.5256827584459104</v>
+        <v>0.4242969450579085</v>
       </c>
       <c r="X26" t="n">
-        <v>1.75</v>
+        <v>3.6</v>
       </c>
       <c r="Y26" t="inlineStr">
         <is>
@@ -3048,13 +3056,13 @@
         </is>
       </c>
       <c r="Z26" t="n">
-        <v>-0.1067402302928757</v>
+        <v>0.2028726931571041</v>
       </c>
       <c r="AA26" t="n">
-        <v>7.739020909204321</v>
+        <v>6.788751120926536</v>
       </c>
       <c r="AB26" t="n">
-        <v>0.2060932275449974</v>
+        <v>0.07078955255198377</v>
       </c>
       <c r="AC26" t="n">
         <v>0</v>
@@ -3120,13 +3128,13 @@
         <v>0</v>
       </c>
       <c r="Q27" t="n">
-        <v>0.4849126475946745</v>
+        <v>0.4597566215738206</v>
       </c>
       <c r="R27" t="n">
-        <v>0.1309767282088347</v>
+        <v>0.1805992005806551</v>
       </c>
       <c r="S27" t="n">
-        <v>0.3841106241964908</v>
+        <v>0.3596441778455242</v>
       </c>
       <c r="T27" t="n">
         <v>1</v>
@@ -3138,7 +3146,7 @@
         <v>0</v>
       </c>
       <c r="W27" t="n">
-        <v>0.4849126475946745</v>
+        <v>0.4597566215738206</v>
       </c>
       <c r="X27" t="n">
         <v>3.3</v>
@@ -3149,13 +3157,13 @@
         </is>
       </c>
       <c r="Z27" t="n">
-        <v>0.2609616248097504</v>
+        <v>0.2248681961711339</v>
       </c>
       <c r="AA27" t="n">
-        <v>7.758602361514793</v>
+        <v>7.356105945181131</v>
       </c>
       <c r="AB27" t="n">
-        <v>0.1008020233981837</v>
+        <v>0.1001124437282964</v>
       </c>
       <c r="AC27" t="n">
         <v>0</v>
@@ -3218,16 +3226,16 @@
         <v>0.05435995536425953</v>
       </c>
       <c r="P28" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q28" t="n">
-        <v>0.3427253486924999</v>
+        <v>0.4528735071835181</v>
       </c>
       <c r="R28" t="n">
-        <v>0.367914072116755</v>
+        <v>0.3563125760751009</v>
       </c>
       <c r="S28" t="n">
-        <v>0.289360579190745</v>
+        <v>0.190813916741381</v>
       </c>
       <c r="T28" t="n">
         <v>1</v>
@@ -3236,13 +3244,13 @@
         <v>0</v>
       </c>
       <c r="V28" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="W28" t="n">
-        <v>0.367914072116755</v>
+        <v>0.4528735071835181</v>
       </c>
       <c r="X28" t="n">
-        <v>1.7</v>
+        <v>4.1</v>
       </c>
       <c r="Y28" t="inlineStr">
         <is>
@@ -3250,13 +3258,13 @@
         </is>
       </c>
       <c r="Z28" t="n">
-        <v>-0.5350658248593092</v>
+        <v>0.2763810901459433</v>
       </c>
       <c r="AA28" t="n">
-        <v>0.7286933152831084</v>
+        <v>7.24597611493629</v>
       </c>
       <c r="AB28" t="n">
-        <v>0.02518872342425515</v>
+        <v>0.09656093110841724</v>
       </c>
       <c r="AC28" t="n">
         <v>0</v>
@@ -3322,13 +3330,13 @@
         <v>1</v>
       </c>
       <c r="Q29" t="n">
-        <v>0.2851320838158716</v>
+        <v>0.2284959652192129</v>
       </c>
       <c r="R29" t="n">
-        <v>0.5192348997289669</v>
+        <v>0.5748996455129791</v>
       </c>
       <c r="S29" t="n">
-        <v>0.1956330164551615</v>
+        <v>0.1966043892678079</v>
       </c>
       <c r="T29" t="n">
         <v>1</v>
@@ -3340,7 +3348,7 @@
         <v>1</v>
       </c>
       <c r="W29" t="n">
-        <v>0.5192348997289669</v>
+        <v>0.5748996455129791</v>
       </c>
       <c r="X29" t="n">
         <v>1.75</v>
@@ -3351,13 +3359,13 @@
         </is>
       </c>
       <c r="Z29" t="n">
-        <v>-0.121785233965744</v>
+        <v>0.008099172863617943</v>
       </c>
       <c r="AA29" t="n">
-        <v>7.551039884758696</v>
+        <v>9.198394328207668</v>
       </c>
       <c r="AB29" t="n">
-        <v>0.2341028159130952</v>
+        <v>0.3464036802937662</v>
       </c>
       <c r="AC29" t="n">
         <v>0</v>
@@ -4410,29 +4418,31 @@
         <v>0.05394672374223175</v>
       </c>
       <c r="P40" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q40" t="n">
-        <v>0.3779810576962759</v>
+        <v>0.2997161277438283</v>
       </c>
       <c r="R40" t="n">
-        <v>0.3217823704459913</v>
+        <v>0.565710760336006</v>
       </c>
       <c r="S40" t="n">
-        <v>0.3002365718577329</v>
+        <v>0.1345731119201658</v>
       </c>
       <c r="T40" t="n">
         <v>1</v>
       </c>
-      <c r="U40" t="inlineStr"/>
+      <c r="U40" t="n">
+        <v>0</v>
+      </c>
       <c r="V40" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W40" t="n">
-        <v>0.3779810576962759</v>
+        <v>0.565710760336006</v>
       </c>
       <c r="X40" t="n">
-        <v>3.8</v>
+        <v>1.57</v>
       </c>
       <c r="Y40" t="inlineStr">
         <is>
@@ -4440,13 +4450,13 @@
         </is>
       </c>
       <c r="Z40" t="n">
-        <v>0.1558314354449458</v>
+        <v>-0.1962001864429308</v>
       </c>
       <c r="AA40" t="n">
-        <v>4.535772692355311</v>
+        <v>7.728992305086814</v>
       </c>
       <c r="AB40" t="n">
-        <v>0.0561986872502846</v>
+        <v>0.2659946325921776</v>
       </c>
       <c r="AC40" t="inlineStr"/>
     </row>
@@ -4510,13 +4520,13 @@
         <v>0</v>
       </c>
       <c r="Q41" t="n">
-        <v>0.4066633931485054</v>
+        <v>0.3967600062693399</v>
       </c>
       <c r="R41" t="n">
-        <v>0.2326300789147079</v>
+        <v>0.2401594434464154</v>
       </c>
       <c r="S41" t="n">
-        <v>0.3607065279367867</v>
+        <v>0.3630805502842447</v>
       </c>
       <c r="T41" t="n">
         <v>1</v>
@@ -4528,7 +4538,7 @@
         <v>0</v>
       </c>
       <c r="W41" t="n">
-        <v>0.4066633931485054</v>
+        <v>0.3967600062693399</v>
       </c>
       <c r="X41" t="n">
         <v>3.25</v>
@@ -4539,17 +4549,15 @@
         </is>
       </c>
       <c r="Z41" t="n">
-        <v>0.1429582345478412</v>
+        <v>0.1286533423890465</v>
       </c>
       <c r="AA41" t="n">
-        <v>4.879960717782065</v>
+        <v>6.348160100309439</v>
       </c>
       <c r="AB41" t="n">
-        <v>0.04595686521171871</v>
-      </c>
-      <c r="AC41" t="n">
-        <v>1</v>
-      </c>
+        <v>0.03367945598509514</v>
+      </c>
+      <c r="AC41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="1" t="inlineStr">
@@ -4611,23 +4619,25 @@
         <v>1</v>
       </c>
       <c r="Q42" t="n">
-        <v>0.3353229852335383</v>
+        <v>0.2367148102940779</v>
       </c>
       <c r="R42" t="n">
-        <v>0.4809804463300263</v>
+        <v>0.6424820239813073</v>
       </c>
       <c r="S42" t="n">
-        <v>0.1836965684364354</v>
+        <v>0.1208031657246147</v>
       </c>
       <c r="T42" t="n">
         <v>1</v>
       </c>
-      <c r="U42" t="inlineStr"/>
+      <c r="U42" t="n">
+        <v>0</v>
+      </c>
       <c r="V42" t="n">
         <v>1</v>
       </c>
       <c r="W42" t="n">
-        <v>0.4809804463300263</v>
+        <v>0.6424820239813073</v>
       </c>
       <c r="X42" t="n">
         <v>1.38</v>
@@ -4638,13 +4648,13 @@
         </is>
       </c>
       <c r="Z42" t="n">
-        <v>-0.884860484380431</v>
+        <v>-0.2983547550152528</v>
       </c>
       <c r="AA42" t="n">
-        <v>2.419614814767192</v>
+        <v>8.017100064426467</v>
       </c>
       <c r="AB42" t="n">
-        <v>0.145657461096488</v>
+        <v>0.4057672136872293</v>
       </c>
       <c r="AC42" t="inlineStr"/>
     </row>
@@ -4708,23 +4718,25 @@
         <v>1</v>
       </c>
       <c r="Q43" t="n">
-        <v>0.3817286210780497</v>
+        <v>0.1512747853691969</v>
       </c>
       <c r="R43" t="n">
-        <v>0.494098164389982</v>
+        <v>0.7941256736229314</v>
       </c>
       <c r="S43" t="n">
-        <v>0.1241732145319683</v>
+        <v>0.0545995410078718</v>
       </c>
       <c r="T43" t="n">
         <v>1</v>
       </c>
-      <c r="U43" t="inlineStr"/>
+      <c r="U43" t="n">
+        <v>0</v>
+      </c>
       <c r="V43" t="n">
         <v>1</v>
       </c>
       <c r="W43" t="n">
-        <v>0.494098164389982</v>
+        <v>0.7941256736229314</v>
       </c>
       <c r="X43" t="n">
         <v>1.22</v>
@@ -4735,13 +4747,13 @@
         </is>
       </c>
       <c r="Z43" t="n">
-        <v>-1.805455633837373</v>
+        <v>-0.1416667190001077</v>
       </c>
       <c r="AA43" t="n">
-        <v>0.7410546667190326</v>
+        <v>11.36105393354034</v>
       </c>
       <c r="AB43" t="n">
-        <v>0.1123695433119323</v>
+        <v>0.6428508882537345</v>
       </c>
       <c r="AC43" t="inlineStr"/>
     </row>
@@ -4805,23 +4817,25 @@
         <v>2</v>
       </c>
       <c r="Q44" t="n">
-        <v>0.2732857195484897</v>
+        <v>0.3762720951724129</v>
       </c>
       <c r="R44" t="n">
-        <v>0.1284467278002551</v>
+        <v>0.08970801300168672</v>
       </c>
       <c r="S44" t="n">
-        <v>0.5982675526512553</v>
+        <v>0.5340198918259004</v>
       </c>
       <c r="T44" t="n">
         <v>1</v>
       </c>
-      <c r="U44" t="inlineStr"/>
+      <c r="U44" t="n">
+        <v>0</v>
+      </c>
       <c r="V44" t="n">
         <v>2</v>
       </c>
       <c r="W44" t="n">
-        <v>0.5982675526512553</v>
+        <v>0.5340198918259004</v>
       </c>
       <c r="X44" t="n">
         <v>2</v>
@@ -4832,13 +4846,13 @@
         </is>
       </c>
       <c r="Z44" t="n">
-        <v>0.1965351053025106</v>
+        <v>0.06803978365180074</v>
       </c>
       <c r="AA44" t="n">
-        <v>7.179210631815065</v>
+        <v>8.544318269214406</v>
       </c>
       <c r="AB44" t="n">
-        <v>0.3249818331027656</v>
+        <v>0.1577477966534874</v>
       </c>
       <c r="AC44" t="inlineStr"/>
     </row>
@@ -4902,23 +4916,25 @@
         <v>1</v>
       </c>
       <c r="Q45" t="n">
-        <v>0.2147983482586515</v>
+        <v>0.1923932435462637</v>
       </c>
       <c r="R45" t="n">
-        <v>0.713517096362164</v>
+        <v>0.7371007141640372</v>
       </c>
       <c r="S45" t="n">
-        <v>0.07168455537918467</v>
+        <v>0.07050604228969912</v>
       </c>
       <c r="T45" t="n">
         <v>1</v>
       </c>
-      <c r="U45" t="inlineStr"/>
+      <c r="U45" t="n">
+        <v>0</v>
+      </c>
       <c r="V45" t="n">
         <v>1</v>
       </c>
       <c r="W45" t="n">
-        <v>0.713517096362164</v>
+        <v>0.7371007141640372</v>
       </c>
       <c r="X45" t="n">
         <v>1.29</v>
@@ -4929,13 +4945,13 @@
         </is>
       </c>
       <c r="Z45" t="n">
-        <v>-0.2743549851476153</v>
+        <v>-0.1694485473392826</v>
       </c>
       <c r="AA45" t="n">
-        <v>6.824843291492115</v>
+        <v>10.30282095206271</v>
       </c>
       <c r="AB45" t="n">
-        <v>0.4987187481035125</v>
+        <v>0.5447074706177735</v>
       </c>
       <c r="AC45" t="inlineStr"/>
     </row>
@@ -4999,23 +5015,25 @@
         <v>1</v>
       </c>
       <c r="Q46" t="n">
-        <v>0.3408476098704054</v>
+        <v>0.2389715158428929</v>
       </c>
       <c r="R46" t="n">
-        <v>0.4235261514218358</v>
+        <v>0.6787278372700994</v>
       </c>
       <c r="S46" t="n">
-        <v>0.235626238707759</v>
+        <v>0.08230064688700764</v>
       </c>
       <c r="T46" t="n">
         <v>1</v>
       </c>
-      <c r="U46" t="inlineStr"/>
+      <c r="U46" t="n">
+        <v>0</v>
+      </c>
       <c r="V46" t="n">
         <v>1</v>
       </c>
       <c r="W46" t="n">
-        <v>0.4235261514218358</v>
+        <v>0.6787278372700994</v>
       </c>
       <c r="X46" t="n">
         <v>1.62</v>
@@ -5026,13 +5044,13 @@
         </is>
       </c>
       <c r="Z46" t="n">
-        <v>-0.506270378542945</v>
+        <v>0.1605469296412277</v>
       </c>
       <c r="AA46" t="n">
-        <v>3.240232607502086</v>
+        <v>10.85964539632159</v>
       </c>
       <c r="AB46" t="n">
-        <v>0.08267854155143045</v>
+        <v>0.4397563214272065</v>
       </c>
       <c r="AC46" t="inlineStr"/>
     </row>
@@ -5096,23 +5114,25 @@
         <v>1</v>
       </c>
       <c r="Q47" t="n">
-        <v>0.425843910799397</v>
+        <v>0.2393823284443568</v>
       </c>
       <c r="R47" t="n">
-        <v>0.4359897826404358</v>
+        <v>0.6636756724146815</v>
       </c>
       <c r="S47" t="n">
-        <v>0.1381663065601672</v>
+        <v>0.09694199914096159</v>
       </c>
       <c r="T47" t="n">
         <v>1</v>
       </c>
-      <c r="U47" t="inlineStr"/>
+      <c r="U47" t="n">
+        <v>0</v>
+      </c>
       <c r="V47" t="n">
         <v>1</v>
       </c>
       <c r="W47" t="n">
-        <v>0.4359897826404358</v>
+        <v>0.6636756724146815</v>
       </c>
       <c r="X47" t="n">
         <v>1.42</v>
@@ -5123,13 +5143,13 @@
         </is>
       </c>
       <c r="Z47" t="n">
-        <v>-0.9068916872632889</v>
+        <v>-0.1370965361217912</v>
       </c>
       <c r="AA47" t="n">
-        <v>0.4273092961324951</v>
+        <v>9.530790773551614</v>
       </c>
       <c r="AB47" t="n">
-        <v>0.01014587184103871</v>
+        <v>0.4242933439703247</v>
       </c>
       <c r="AC47" t="inlineStr"/>
     </row>
@@ -5193,13 +5213,13 @@
         <v>0</v>
       </c>
       <c r="Q48" t="n">
-        <v>0.361961678664959</v>
+        <v>0.4135144494087292</v>
       </c>
       <c r="R48" t="n">
-        <v>0.3219924559592394</v>
+        <v>0.3148051357091823</v>
       </c>
       <c r="S48" t="n">
-        <v>0.3160458653758016</v>
+        <v>0.2716804148820885</v>
       </c>
       <c r="T48" t="n">
         <v>1</v>
@@ -5211,7 +5231,7 @@
         <v>0</v>
       </c>
       <c r="W48" t="n">
-        <v>0.361961678664959</v>
+        <v>0.4135144494087292</v>
       </c>
       <c r="X48" t="n">
         <v>3.2</v>
@@ -5222,17 +5242,15 @@
         </is>
       </c>
       <c r="Z48" t="n">
-        <v>0.07194425987630411</v>
+        <v>0.1469301082308789</v>
       </c>
       <c r="AA48" t="n">
-        <v>4.343540143979509</v>
+        <v>6.616231190539668</v>
       </c>
       <c r="AB48" t="n">
-        <v>0.03996922270571968</v>
-      </c>
-      <c r="AC48" t="n">
-        <v>1</v>
-      </c>
+        <v>0.09870931369954694</v>
+      </c>
+      <c r="AC48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="1" t="inlineStr">
@@ -5291,29 +5309,31 @@
         <v>0.06061256005490723</v>
       </c>
       <c r="P49" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="Q49" t="n">
-        <v>0.4297456015563137</v>
+        <v>0.3082526614528583</v>
       </c>
       <c r="R49" t="n">
-        <v>0.3165019017323719</v>
+        <v>0.3135673947478088</v>
       </c>
       <c r="S49" t="n">
-        <v>0.2537524967113144</v>
+        <v>0.378179943799333</v>
       </c>
       <c r="T49" t="n">
         <v>1</v>
       </c>
-      <c r="U49" t="inlineStr"/>
+      <c r="U49" t="n">
+        <v>0</v>
+      </c>
       <c r="V49" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="W49" t="n">
-        <v>0.4297456015563137</v>
+        <v>0.378179943799333</v>
       </c>
       <c r="X49" t="n">
-        <v>3.2</v>
+        <v>2.35</v>
       </c>
       <c r="Y49" t="inlineStr">
         <is>
@@ -5321,13 +5341,13 @@
         </is>
       </c>
       <c r="Z49" t="n">
-        <v>0.1705390568091836</v>
+        <v>-0.08242750523819817</v>
       </c>
       <c r="AA49" t="n">
-        <v>5.156947218675764</v>
+        <v>5.677285759775658</v>
       </c>
       <c r="AB49" t="n">
-        <v>0.1132436998239418</v>
+        <v>0.06461254905152419</v>
       </c>
       <c r="AC49" t="inlineStr"/>
     </row>

</xml_diff>

<commit_message>
Actualizo results (faltan dos)
</commit_message>
<xml_diff>
--- a/data/predicciones.xlsx
+++ b/data/predicciones.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL3"/>
+  <dimension ref="A1:AL5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -848,6 +848,242 @@
         <v>0</v>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>2PzWBZV8</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>45724.625</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>lille</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>montpellier</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>55</v>
+      </c>
+      <c r="F4" t="n">
+        <v>551</v>
+      </c>
+      <c r="G4" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="H4" t="n">
+        <v>4.75</v>
+      </c>
+      <c r="I4" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0.675035528</v>
+      </c>
+      <c r="K4" t="n">
+        <v>0.19895784</v>
+      </c>
+      <c r="L4" t="n">
+        <v>0.126006632</v>
+      </c>
+      <c r="M4" t="n">
+        <v>0.058145363</v>
+      </c>
+      <c r="N4" t="n">
+        <v>1</v>
+      </c>
+      <c r="O4" t="n">
+        <v>0.503637523</v>
+      </c>
+      <c r="P4" t="n">
+        <v>0.263969839</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>0.232392638</v>
+      </c>
+      <c r="R4" t="n">
+        <v>1</v>
+      </c>
+      <c r="S4" t="inlineStr"/>
+      <c r="T4" t="n">
+        <v>1</v>
+      </c>
+      <c r="U4" t="inlineStr"/>
+      <c r="V4" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="W4" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="X4" t="inlineStr">
+        <is>
+          <t>dif_prob_mod_bm &gt; 0</t>
+        </is>
+      </c>
+      <c r="Y4" t="inlineStr"/>
+      <c r="Z4" t="n">
+        <v>4</v>
+      </c>
+      <c r="AA4" t="inlineStr">
+        <is>
+          <t>france</t>
+        </is>
+      </c>
+      <c r="AB4" t="inlineStr">
+        <is>
+          <t>ligue 1</t>
+        </is>
+      </c>
+      <c r="AC4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD4" t="inlineStr"/>
+      <c r="AE4" t="inlineStr"/>
+      <c r="AF4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG4" t="n">
+        <v>0.239667685</v>
+      </c>
+      <c r="AH4" t="n">
+        <v>-0.7</v>
+      </c>
+      <c r="AI4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AJ4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AL4" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>2yTWkl1e</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>45724.69791666666</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>inter</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>monza</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>77</v>
+      </c>
+      <c r="F5" t="n">
+        <v>771</v>
+      </c>
+      <c r="G5" t="n">
+        <v>1.14</v>
+      </c>
+      <c r="H5" t="n">
+        <v>8</v>
+      </c>
+      <c r="I5" t="n">
+        <v>21</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0.835571471</v>
+      </c>
+      <c r="K5" t="n">
+        <v>0.119068935</v>
+      </c>
+      <c r="L5" t="n">
+        <v>0.045359594</v>
+      </c>
+      <c r="M5" t="n">
+        <v>0.04981203</v>
+      </c>
+      <c r="N5" t="n">
+        <v>1</v>
+      </c>
+      <c r="O5" t="n">
+        <v>0.748000674</v>
+      </c>
+      <c r="P5" t="n">
+        <v>0.235048352</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>0.016950974</v>
+      </c>
+      <c r="R5" t="n">
+        <v>1</v>
+      </c>
+      <c r="S5" t="inlineStr"/>
+      <c r="T5" t="n">
+        <v>1</v>
+      </c>
+      <c r="U5" t="inlineStr"/>
+      <c r="V5" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="W5" t="n">
+        <v>1.14</v>
+      </c>
+      <c r="X5" t="inlineStr">
+        <is>
+          <t>dif_prob_mod_bm &gt; 0</t>
+        </is>
+      </c>
+      <c r="Y5" t="inlineStr"/>
+      <c r="Z5" t="n">
+        <v>2</v>
+      </c>
+      <c r="AA5" t="inlineStr">
+        <is>
+          <t>italy</t>
+        </is>
+      </c>
+      <c r="AB5" t="inlineStr">
+        <is>
+          <t>serie a</t>
+        </is>
+      </c>
+      <c r="AC5" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD5" t="inlineStr"/>
+      <c r="AE5" t="inlineStr"/>
+      <c r="AF5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG5" t="n">
+        <v>0.512952323</v>
+      </c>
+      <c r="AH5" t="n">
+        <v>-1.1</v>
+      </c>
+      <c r="AI5" t="n">
+        <v>3</v>
+      </c>
+      <c r="AJ5" t="n">
+        <v>2</v>
+      </c>
+      <c r="AK5" t="n">
+        <v>1</v>
+      </c>
+      <c r="AL5" t="n">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
DATA. Actualizo predicciones por cuotas y missing y cambio de mod en SPA
</commit_message>
<xml_diff>
--- a/data/predicciones.xlsx
+++ b/data/predicciones.xlsx
@@ -621,19 +621,19 @@
         <v>4.33</v>
       </c>
       <c r="K2" t="n">
-        <v>4.33</v>
+        <v>4.5</v>
       </c>
       <c r="L2" t="n">
-        <v>0.5645371577574968</v>
+        <v>0.5692192187805826</v>
       </c>
       <c r="M2" t="n">
-        <v>0.2177314211212516</v>
+        <v>0.2195372044719568</v>
       </c>
       <c r="N2" t="n">
-        <v>0.2177314211212516</v>
+        <v>0.2112435767474606</v>
       </c>
       <c r="O2" t="n">
-        <v>0.06069615964376096</v>
+        <v>0.05197149964889314</v>
       </c>
       <c r="P2" t="n">
         <v>1</v>
@@ -716,25 +716,25 @@
         </is>
       </c>
       <c r="I3" t="n">
-        <v>2.1</v>
+        <v>2.05</v>
       </c>
       <c r="J3" t="n">
         <v>3.2</v>
       </c>
       <c r="K3" t="n">
-        <v>3.7</v>
+        <v>3.9</v>
       </c>
       <c r="L3" t="n">
-        <v>0.449677174325864</v>
+        <v>0.4616238209728131</v>
       </c>
       <c r="M3" t="n">
-        <v>0.2951006456513482</v>
+        <v>0.2957277603107084</v>
       </c>
       <c r="N3" t="n">
-        <v>0.2552221800227877</v>
+        <v>0.2426484187164787</v>
       </c>
       <c r="O3" t="n">
-        <v>0.05896074646074645</v>
+        <v>0.05671513445903686</v>
       </c>
       <c r="P3" t="n">
         <v>0</v>
@@ -921,22 +921,22 @@
         <v>3.75</v>
       </c>
       <c r="J5" t="n">
-        <v>3.3</v>
+        <v>3.5</v>
       </c>
       <c r="K5" t="n">
         <v>2</v>
       </c>
       <c r="L5" t="n">
-        <v>0.2492917847025495</v>
+        <v>0.253393665158371</v>
       </c>
       <c r="M5" t="n">
-        <v>0.28328611898017</v>
+        <v>0.2714932126696832</v>
       </c>
       <c r="N5" t="n">
-        <v>0.4674220963172804</v>
+        <v>0.4751131221719457</v>
       </c>
       <c r="O5" t="n">
-        <v>0.06969696969696981</v>
+        <v>0.05238095238095242</v>
       </c>
       <c r="P5" t="n">
         <v>2</v>
@@ -1019,25 +1019,25 @@
         </is>
       </c>
       <c r="I6" t="n">
-        <v>3.7</v>
+        <v>3.75</v>
       </c>
       <c r="J6" t="n">
-        <v>3.3</v>
+        <v>3.4</v>
       </c>
       <c r="K6" t="n">
-        <v>2.1</v>
+        <v>2</v>
       </c>
       <c r="L6" t="n">
-        <v>0.2575250836120401</v>
+        <v>0.2513863216266174</v>
       </c>
       <c r="M6" t="n">
-        <v>0.2887402452619844</v>
+        <v>0.2772643253234751</v>
       </c>
       <c r="N6" t="n">
-        <v>0.4537346711259755</v>
+        <v>0.4713493530499075</v>
       </c>
       <c r="O6" t="n">
-        <v>0.04949104949104943</v>
+        <v>0.0607843137254902</v>
       </c>
       <c r="P6" t="n">
         <v>2</v>
@@ -1067,7 +1067,7 @@
         <v>0.639140890746701</v>
       </c>
       <c r="Y6" t="n">
-        <v>2.1</v>
+        <v>2</v>
       </c>
       <c r="Z6" t="inlineStr">
         <is>
@@ -1075,7 +1075,7 @@
         </is>
       </c>
       <c r="AA6" t="n">
-        <v>0.3110871550618837</v>
+        <v>0.278281781493402</v>
       </c>
       <c r="AB6" t="n">
         <v>6.710979352840361</v>
@@ -1123,22 +1123,22 @@
         <v>1.7</v>
       </c>
       <c r="J7" t="n">
-        <v>3.9</v>
+        <v>4.2</v>
       </c>
       <c r="K7" t="n">
-        <v>4.75</v>
+        <v>4.33</v>
       </c>
       <c r="L7" t="n">
-        <v>0.5574781823653325</v>
+        <v>0.556367975035947</v>
       </c>
       <c r="M7" t="n">
-        <v>0.2430033102618116</v>
+        <v>0.2251965613240738</v>
       </c>
       <c r="N7" t="n">
-        <v>0.1995185073728558</v>
+        <v>0.2184354636399792</v>
       </c>
       <c r="O7" t="n">
-        <v>0.05517186631737725</v>
+        <v>0.05727741442997525</v>
       </c>
       <c r="P7" t="n">
         <v>2</v>
@@ -1168,7 +1168,7 @@
         <v>0.8859181646348711</v>
       </c>
       <c r="Y7" t="n">
-        <v>4.75</v>
+        <v>4.33</v>
       </c>
       <c r="Z7" t="inlineStr">
         <is>
@@ -1176,7 +1176,7 @@
         </is>
       </c>
       <c r="AA7" t="n">
-        <v>0.8554963418708366</v>
+        <v>0.8516593552159135</v>
       </c>
       <c r="AB7" t="n">
         <v>9.302140728666146</v>
@@ -1221,25 +1221,25 @@
         </is>
       </c>
       <c r="I8" t="n">
-        <v>1.95</v>
+        <v>2</v>
       </c>
       <c r="J8" t="n">
-        <v>3.7</v>
+        <v>3.75</v>
       </c>
       <c r="K8" t="n">
-        <v>3.7</v>
+        <v>3.6</v>
       </c>
       <c r="L8" t="n">
-        <v>0.486842105263158</v>
+        <v>0.4787234042553192</v>
       </c>
       <c r="M8" t="n">
-        <v>0.256578947368421</v>
+        <v>0.2553191489361702</v>
       </c>
       <c r="N8" t="n">
-        <v>0.256578947368421</v>
+        <v>0.2659574468085107</v>
       </c>
       <c r="O8" t="n">
-        <v>0.05336105336105335</v>
+        <v>0.04444444444444429</v>
       </c>
       <c r="P8" t="n">
         <v>2</v>
@@ -1269,7 +1269,7 @@
         <v>0.902090554457058</v>
       </c>
       <c r="Y8" t="n">
-        <v>3.7</v>
+        <v>3.6</v>
       </c>
       <c r="Z8" t="inlineStr">
         <is>
@@ -1277,7 +1277,7 @@
         </is>
       </c>
       <c r="AA8" t="n">
-        <v>0.865827796848561</v>
+        <v>0.8644330754020803</v>
       </c>
       <c r="AB8" t="n">
         <v>9.471950821799108</v>
@@ -1429,19 +1429,19 @@
         <v>4</v>
       </c>
       <c r="K10" t="n">
-        <v>5.5</v>
+        <v>6</v>
       </c>
       <c r="L10" t="n">
-        <v>0.5959637003927942</v>
+        <v>0.6045340050377834</v>
       </c>
       <c r="M10" t="n">
-        <v>0.2339157524041718</v>
+        <v>0.23727959697733</v>
       </c>
       <c r="N10" t="n">
-        <v>0.170120547203034</v>
+        <v>0.1581863979848867</v>
       </c>
       <c r="O10" t="n">
-        <v>0.06876085697741741</v>
+        <v>0.05360934182590227</v>
       </c>
       <c r="P10" t="n">
         <v>1</v>
@@ -1527,22 +1527,22 @@
         <v>1.36</v>
       </c>
       <c r="J11" t="n">
-        <v>5.25</v>
+        <v>5.5</v>
       </c>
       <c r="K11" t="n">
         <v>7</v>
       </c>
       <c r="L11" t="n">
-        <v>0.6880733944954128</v>
+        <v>0.6936936936936937</v>
       </c>
       <c r="M11" t="n">
-        <v>0.1782437745740498</v>
+        <v>0.1715315315315316</v>
       </c>
       <c r="N11" t="n">
-        <v>0.1336828309305373</v>
+        <v>0.1347747747747748</v>
       </c>
       <c r="O11" t="n">
-        <v>0.06862745098039214</v>
+        <v>0.05996944232238333</v>
       </c>
       <c r="P11" t="n">
         <v>1</v>
@@ -1624,22 +1624,22 @@
         <v>1.67</v>
       </c>
       <c r="J12" t="n">
-        <v>3.7</v>
+        <v>3.9</v>
       </c>
       <c r="K12" t="n">
         <v>5</v>
       </c>
       <c r="L12" t="n">
-        <v>0.5601138393532957</v>
+        <v>0.5674708261793209</v>
       </c>
       <c r="M12" t="n">
-        <v>0.2528081383027037</v>
+        <v>0.2429939178767861</v>
       </c>
       <c r="N12" t="n">
-        <v>0.1870780223440008</v>
+        <v>0.1895352559438931</v>
       </c>
       <c r="O12" t="n">
-        <v>0.06907266547985103</v>
+        <v>0.05521265161983724</v>
       </c>
       <c r="P12" t="n">
         <v>1</v>
@@ -1721,22 +1721,22 @@
         <v>2.2</v>
       </c>
       <c r="J13" t="n">
-        <v>3.4</v>
+        <v>3.5</v>
       </c>
       <c r="K13" t="n">
         <v>3.2</v>
       </c>
       <c r="L13" t="n">
-        <v>0.4283464566929134</v>
+        <v>0.4317656129529684</v>
       </c>
       <c r="M13" t="n">
-        <v>0.2771653543307087</v>
+        <v>0.2713955281418658</v>
       </c>
       <c r="N13" t="n">
-        <v>0.294488188976378</v>
+        <v>0.2968388589051658</v>
       </c>
       <c r="O13" t="n">
-        <v>0.06116310160427796</v>
+        <v>0.05275974025974017</v>
       </c>
       <c r="P13" t="n">
         <v>1</v>
@@ -1912,25 +1912,25 @@
         </is>
       </c>
       <c r="I15" t="n">
-        <v>1.48</v>
+        <v>1.45</v>
       </c>
       <c r="J15" t="n">
         <v>5</v>
       </c>
       <c r="K15" t="n">
-        <v>5.5</v>
+        <v>6</v>
       </c>
       <c r="L15" t="n">
-        <v>0.6389405204460966</v>
+        <v>0.6528835690968444</v>
       </c>
       <c r="M15" t="n">
-        <v>0.1891263940520446</v>
+        <v>0.1893362350380849</v>
       </c>
       <c r="N15" t="n">
-        <v>0.1719330855018587</v>
+        <v>0.1577801958650707</v>
       </c>
       <c r="O15" t="n">
-        <v>0.05749385749385749</v>
+        <v>0.05632183908045985</v>
       </c>
       <c r="P15" t="n">
         <v>1</v>
@@ -1956,7 +1956,7 @@
         <v>0.4234568083806666</v>
       </c>
       <c r="Y15" t="n">
-        <v>1.48</v>
+        <v>1.45</v>
       </c>
       <c r="Z15" t="inlineStr">
         <is>
@@ -1964,10 +1964,10 @@
         </is>
       </c>
       <c r="AA15" t="n">
-        <v>-0.7776748408262778</v>
+        <v>-0.8577502841067409</v>
       </c>
       <c r="AB15" t="n">
-        <v>0.7039554093951731</v>
+        <v>0.6415251151323692</v>
       </c>
       <c r="AC15" t="n">
         <v>0.08955931114154431</v>
@@ -2015,19 +2015,19 @@
         <v>3.5</v>
       </c>
       <c r="K16" t="n">
-        <v>3.5</v>
+        <v>3.6</v>
       </c>
       <c r="L16" t="n">
-        <v>0.4605263157894737</v>
+        <v>0.4640029460504511</v>
       </c>
       <c r="M16" t="n">
-        <v>0.2697368421052631</v>
+        <v>0.2717731541152641</v>
       </c>
       <c r="N16" t="n">
-        <v>0.2697368421052631</v>
+        <v>0.2642238998342846</v>
       </c>
       <c r="O16" t="n">
-        <v>0.0592334494773521</v>
+        <v>0.05129694154084419</v>
       </c>
       <c r="P16" t="n">
         <v>0</v>
@@ -2112,19 +2112,19 @@
         <v>3.2</v>
       </c>
       <c r="K17" t="n">
-        <v>2.1</v>
+        <v>2.15</v>
       </c>
       <c r="L17" t="n">
-        <v>0.2604651162790698</v>
+        <v>0.2631981637337414</v>
       </c>
       <c r="M17" t="n">
-        <v>0.2930232558139535</v>
+        <v>0.296097934200459</v>
       </c>
       <c r="N17" t="n">
-        <v>0.4465116279069767</v>
+        <v>0.4407039020657995</v>
       </c>
       <c r="O17" t="n">
-        <v>0.06646825396825395</v>
+        <v>0.05539405684754528</v>
       </c>
       <c r="P17" t="n">
         <v>2</v>
@@ -2150,7 +2150,7 @@
         <v>0.4465970382995856</v>
       </c>
       <c r="Y17" t="n">
-        <v>2.1</v>
+        <v>2.15</v>
       </c>
       <c r="Z17" t="inlineStr">
         <is>
@@ -2158,10 +2158,10 @@
         </is>
       </c>
       <c r="AA17" t="n">
-        <v>-0.05649656324624562</v>
+        <v>-0.03462292839642699</v>
       </c>
       <c r="AB17" t="n">
-        <v>7.484486746979738</v>
+        <v>7.612548496169001</v>
       </c>
       <c r="AC17" t="n">
         <v>0.1057077269288484</v>
@@ -2209,19 +2209,19 @@
         <v>4.75</v>
       </c>
       <c r="K18" t="n">
-        <v>1.44</v>
+        <v>1.42</v>
       </c>
       <c r="L18" t="n">
-        <v>0.1453000531067446</v>
+        <v>0.1439701173959445</v>
       </c>
       <c r="M18" t="n">
-        <v>0.1988316516197557</v>
+        <v>0.1970117395944503</v>
       </c>
       <c r="N18" t="n">
-        <v>0.6558682952734998</v>
+        <v>0.6590181430096052</v>
       </c>
       <c r="O18" t="n">
-        <v>0.05881691408007184</v>
+        <v>0.06859782174830364</v>
       </c>
       <c r="P18" t="n">
         <v>2</v>
@@ -2247,7 +2247,7 @@
         <v>0.5179024413655883</v>
       </c>
       <c r="Y18" t="n">
-        <v>1.44</v>
+        <v>1.42</v>
       </c>
       <c r="Z18" t="inlineStr">
         <is>
@@ -2255,10 +2255,10 @@
         </is>
       </c>
       <c r="AA18" t="n">
-        <v>-0.5777738282580749</v>
+        <v>-0.6299488887163446</v>
       </c>
       <c r="AB18" t="n">
-        <v>5.36455583562247</v>
+        <v>5.073756808859895</v>
       </c>
       <c r="AC18" t="n">
         <v>0.1934758779774503</v>
@@ -2300,25 +2300,25 @@
         </is>
       </c>
       <c r="I19" t="n">
-        <v>1.95</v>
+        <v>2</v>
       </c>
       <c r="J19" t="n">
-        <v>3.3</v>
+        <v>3.25</v>
       </c>
       <c r="K19" t="n">
         <v>4</v>
       </c>
       <c r="L19" t="n">
-        <v>0.4811372334609076</v>
+        <v>0.4727272727272727</v>
       </c>
       <c r="M19" t="n">
-        <v>0.2843083652268999</v>
+        <v>0.2909090909090909</v>
       </c>
       <c r="N19" t="n">
-        <v>0.2345544013121924</v>
+        <v>0.2363636363636364</v>
       </c>
       <c r="O19" t="n">
-        <v>0.06585081585081598</v>
+        <v>0.05769230769230771</v>
       </c>
       <c r="P19" t="n">
         <v>0</v>
@@ -2348,7 +2348,7 @@
         <v>0.3640266688230058</v>
       </c>
       <c r="Y19" t="n">
-        <v>3.3</v>
+        <v>3.25</v>
       </c>
       <c r="Z19" t="inlineStr">
         <is>
@@ -2356,7 +2356,7 @@
         </is>
       </c>
       <c r="AA19" t="n">
-        <v>0.08751652483300826</v>
+        <v>0.08137185496656392</v>
       </c>
       <c r="AB19" t="n">
         <v>7.644560045283121</v>
@@ -2401,25 +2401,25 @@
         </is>
       </c>
       <c r="I20" t="n">
-        <v>2.25</v>
+        <v>2.4</v>
       </c>
       <c r="J20" t="n">
-        <v>3.5</v>
+        <v>3.6</v>
       </c>
       <c r="K20" t="n">
-        <v>3</v>
+        <v>2.75</v>
       </c>
       <c r="L20" t="n">
-        <v>0.417910447761194</v>
+        <v>0.3937947494033414</v>
       </c>
       <c r="M20" t="n">
-        <v>0.2686567164179104</v>
+        <v>0.2625298329355609</v>
       </c>
       <c r="N20" t="n">
-        <v>0.3134328358208955</v>
+        <v>0.3436754176610979</v>
       </c>
       <c r="O20" t="n">
-        <v>0.06349206349206349</v>
+        <v>0.05808080808080796</v>
       </c>
       <c r="P20" t="n">
         <v>0</v>
@@ -2449,7 +2449,7 @@
         <v>0.3621597653085013</v>
       </c>
       <c r="Y20" t="n">
-        <v>3.5</v>
+        <v>3.6</v>
       </c>
       <c r="Z20" t="inlineStr">
         <is>
@@ -2457,7 +2457,7 @@
         </is>
       </c>
       <c r="AA20" t="n">
-        <v>0.1070236714319019</v>
+        <v>0.1168365981194634</v>
       </c>
       <c r="AB20" t="n">
         <v>7.605355071478527</v>
@@ -2502,25 +2502,25 @@
         </is>
       </c>
       <c r="I21" t="n">
-        <v>2.4</v>
+        <v>2.38</v>
       </c>
       <c r="J21" t="n">
         <v>3.6</v>
       </c>
       <c r="K21" t="n">
-        <v>2.7</v>
+        <v>2.88</v>
       </c>
       <c r="L21" t="n">
-        <v>0.391304347826087</v>
+        <v>0.4020100502512564</v>
       </c>
       <c r="M21" t="n">
-        <v>0.2608695652173913</v>
+        <v>0.2657733109994417</v>
       </c>
       <c r="N21" t="n">
-        <v>0.3478260869565217</v>
+        <v>0.3322166387493021</v>
       </c>
       <c r="O21" t="n">
-        <v>0.06481481481481488</v>
+        <v>0.0451680672268906</v>
       </c>
       <c r="P21" t="n">
         <v>0</v>
@@ -2606,22 +2606,22 @@
         <v>3.1</v>
       </c>
       <c r="J22" t="n">
-        <v>3.5</v>
+        <v>3.6</v>
       </c>
       <c r="K22" t="n">
         <v>2.2</v>
       </c>
       <c r="L22" t="n">
-        <v>0.303508080409933</v>
+        <v>0.3057915057915058</v>
       </c>
       <c r="M22" t="n">
-        <v>0.2688214426487978</v>
+        <v>0.2633204633204633</v>
       </c>
       <c r="N22" t="n">
-        <v>0.4276704769412692</v>
+        <v>0.4308880308880308</v>
       </c>
       <c r="O22" t="n">
-        <v>0.06284038542103065</v>
+        <v>0.05490387748452275</v>
       </c>
       <c r="P22" t="n">
         <v>0</v>
@@ -2651,7 +2651,7 @@
         <v>0.3796238743895269</v>
       </c>
       <c r="Y22" t="n">
-        <v>3.5</v>
+        <v>3.6</v>
       </c>
       <c r="Z22" t="inlineStr">
         <is>
@@ -2659,7 +2659,7 @@
         </is>
       </c>
       <c r="AA22" t="n">
-        <v>0.1314734241453377</v>
+        <v>0.1410176722316527</v>
       </c>
       <c r="AB22" t="n">
         <v>7.972101362180066</v>
@@ -2704,25 +2704,25 @@
         </is>
       </c>
       <c r="I23" t="n">
-        <v>1.92</v>
+        <v>2</v>
       </c>
       <c r="J23" t="n">
         <v>3.5</v>
       </c>
       <c r="K23" t="n">
-        <v>3.7</v>
+        <v>3.75</v>
       </c>
       <c r="L23" t="n">
-        <v>0.4836781952640622</v>
+        <v>0.4751131221719457</v>
       </c>
       <c r="M23" t="n">
-        <v>0.2653320385448569</v>
+        <v>0.2714932126696832</v>
       </c>
       <c r="N23" t="n">
-        <v>0.2509897661910809</v>
+        <v>0.253393665158371</v>
       </c>
       <c r="O23" t="n">
-        <v>0.07681788931788924</v>
+        <v>0.05238095238095242</v>
       </c>
       <c r="P23" t="n">
         <v>0</v>
@@ -2808,22 +2808,22 @@
         <v>2.25</v>
       </c>
       <c r="J24" t="n">
-        <v>3.2</v>
+        <v>3.25</v>
       </c>
       <c r="K24" t="n">
         <v>3.3</v>
       </c>
       <c r="L24" t="n">
-        <v>0.4192972007147112</v>
+        <v>0.4212076583210604</v>
       </c>
       <c r="M24" t="n">
-        <v>0.2948183442525313</v>
+        <v>0.2916053019145803</v>
       </c>
       <c r="N24" t="n">
-        <v>0.2858844550327576</v>
+        <v>0.2871870397643594</v>
       </c>
       <c r="O24" t="n">
-        <v>0.0599747474747474</v>
+        <v>0.05516705516705511</v>
       </c>
       <c r="P24" t="n">
         <v>2</v>
@@ -2906,25 +2906,25 @@
         </is>
       </c>
       <c r="I25" t="n">
-        <v>2.6</v>
+        <v>2.55</v>
       </c>
       <c r="J25" t="n">
         <v>3.3</v>
       </c>
       <c r="K25" t="n">
-        <v>2.7</v>
+        <v>2.75</v>
       </c>
       <c r="L25" t="n">
-        <v>0.3635250917992656</v>
+        <v>0.3703703703703703</v>
       </c>
       <c r="M25" t="n">
-        <v>0.2864137086903305</v>
+        <v>0.2861952861952861</v>
       </c>
       <c r="N25" t="n">
-        <v>0.3500611995104039</v>
+        <v>0.3434343434343434</v>
       </c>
       <c r="O25" t="n">
-        <v>0.05801605801605803</v>
+        <v>0.05882352941176494</v>
       </c>
       <c r="P25" t="n">
         <v>2</v>
@@ -2954,7 +2954,7 @@
         <v>0.4435846554593713</v>
       </c>
       <c r="Y25" t="n">
-        <v>2.7</v>
+        <v>2.75</v>
       </c>
       <c r="Z25" t="inlineStr">
         <is>
@@ -2962,7 +2962,7 @@
         </is>
       </c>
       <c r="AA25" t="n">
-        <v>0.1162815116119427</v>
+        <v>0.1256330300075835</v>
       </c>
       <c r="AB25" t="n">
         <v>9.315277764646796</v>
@@ -3007,7 +3007,7 @@
         </is>
       </c>
       <c r="I26" t="n">
-        <v>7.5</v>
+        <v>8.5</v>
       </c>
       <c r="J26" t="n">
         <v>5</v>
@@ -3016,16 +3016,16 @@
         <v>1.36</v>
       </c>
       <c r="L26" t="n">
-        <v>0.1247706422018349</v>
+        <v>0.111731843575419</v>
       </c>
       <c r="M26" t="n">
-        <v>0.1871559633027523</v>
+        <v>0.1899441340782123</v>
       </c>
       <c r="N26" t="n">
-        <v>0.6880733944954128</v>
+        <v>0.6983240223463688</v>
       </c>
       <c r="O26" t="n">
-        <v>0.06862745098039214</v>
+        <v>0.05294117647058805</v>
       </c>
       <c r="P26" t="n">
         <v>2</v>
@@ -3209,25 +3209,25 @@
         </is>
       </c>
       <c r="I28" t="n">
-        <v>1.8</v>
+        <v>1.73</v>
       </c>
       <c r="J28" t="n">
         <v>3.5</v>
       </c>
       <c r="K28" t="n">
-        <v>4.75</v>
+        <v>5</v>
       </c>
       <c r="L28" t="n">
-        <v>0.5281969817315331</v>
+        <v>0.5433938829374321</v>
       </c>
       <c r="M28" t="n">
-        <v>0.2716441620333598</v>
+        <v>0.2685918335662164</v>
       </c>
       <c r="N28" t="n">
-        <v>0.2001588562351072</v>
+        <v>0.1880142834963515</v>
       </c>
       <c r="O28" t="n">
-        <v>0.05179615705931484</v>
+        <v>0.06374896779521055</v>
       </c>
       <c r="P28" t="n">
         <v>1</v>
@@ -3257,7 +3257,7 @@
         <v>0.6340129587479735</v>
       </c>
       <c r="Y28" t="n">
-        <v>1.8</v>
+        <v>1.73</v>
       </c>
       <c r="Z28" t="inlineStr">
         <is>
@@ -3265,7 +3265,7 @@
         </is>
       </c>
       <c r="AA28" t="n">
-        <v>0.1765291571829404</v>
+        <v>0.1326608474438276</v>
       </c>
       <c r="AB28" t="n">
         <v>4.438090711235814</v>
@@ -3316,19 +3316,19 @@
         <v>3.6</v>
       </c>
       <c r="K29" t="n">
-        <v>4.33</v>
+        <v>4.5</v>
       </c>
       <c r="L29" t="n">
-        <v>0.5220012055455093</v>
+        <v>0.5263157894736842</v>
       </c>
       <c r="M29" t="n">
-        <v>0.2610006027727547</v>
+        <v>0.2631578947368421</v>
       </c>
       <c r="N29" t="n">
-        <v>0.216998191681736</v>
+        <v>0.2105263157894737</v>
       </c>
       <c r="O29" t="n">
-        <v>0.0642802155504234</v>
+        <v>0.05555555555555558</v>
       </c>
       <c r="P29" t="n">
         <v>1</v>
@@ -3410,22 +3410,22 @@
         <v>1.8</v>
       </c>
       <c r="J30" t="n">
-        <v>3.2</v>
+        <v>3.3</v>
       </c>
       <c r="K30" t="n">
         <v>5</v>
       </c>
       <c r="L30" t="n">
-        <v>0.5201560468140443</v>
+        <v>0.5248091603053435</v>
       </c>
       <c r="M30" t="n">
-        <v>0.2925877763328999</v>
+        <v>0.2862595419847329</v>
       </c>
       <c r="N30" t="n">
-        <v>0.1872561768530559</v>
+        <v>0.1889312977099237</v>
       </c>
       <c r="O30" t="n">
-        <v>0.06805555555555554</v>
+        <v>0.05858585858585852</v>
       </c>
       <c r="P30" t="n">
         <v>1</v>
@@ -3508,25 +3508,25 @@
         </is>
       </c>
       <c r="I31" t="n">
-        <v>1.57</v>
+        <v>1.53</v>
       </c>
       <c r="J31" t="n">
         <v>4.2</v>
       </c>
       <c r="K31" t="n">
-        <v>5.5</v>
+        <v>6</v>
       </c>
       <c r="L31" t="n">
-        <v>0.6026768243366641</v>
+        <v>0.6175562417291575</v>
       </c>
       <c r="M31" t="n">
-        <v>0.2252863367163244</v>
+        <v>0.2249669166299073</v>
       </c>
       <c r="N31" t="n">
-        <v>0.1720368389470114</v>
+        <v>0.1574768416409351</v>
       </c>
       <c r="O31" t="n">
-        <v>0.05685609507265554</v>
+        <v>0.05835667600373484</v>
       </c>
       <c r="P31" t="n">
         <v>1</v>
@@ -3552,7 +3552,7 @@
         <v>0.606766940296952</v>
       </c>
       <c r="Y31" t="n">
-        <v>1.57</v>
+        <v>1.53</v>
       </c>
       <c r="Z31" t="inlineStr">
         <is>
@@ -3560,10 +3560,10 @@
         </is>
       </c>
       <c r="AA31" t="n">
-        <v>-0.08311562058558825</v>
+        <v>-0.1351822289540819</v>
       </c>
       <c r="AB31" t="n">
-        <v>3.982943992897853</v>
+        <v>3.818211483353144</v>
       </c>
       <c r="AC31" t="n">
         <v>0.2420316919435578</v>
@@ -3712,19 +3712,19 @@
         <v>3.1</v>
       </c>
       <c r="K33" t="n">
-        <v>3.3</v>
+        <v>3.4</v>
       </c>
       <c r="L33" t="n">
-        <v>0.4100200400801604</v>
+        <v>0.413495488426834</v>
       </c>
       <c r="M33" t="n">
-        <v>0.3042084168336673</v>
+        <v>0.3067869752844252</v>
       </c>
       <c r="N33" t="n">
-        <v>0.2857715430861724</v>
+        <v>0.2797175362887406</v>
       </c>
       <c r="O33" t="n">
-        <v>0.06039355688724557</v>
+        <v>0.05148090091576618</v>
       </c>
       <c r="P33" t="n">
         <v>0</v>
@@ -3806,22 +3806,22 @@
         <v>2.55</v>
       </c>
       <c r="J34" t="n">
-        <v>3.5</v>
+        <v>3.3</v>
       </c>
       <c r="K34" t="n">
-        <v>2.63</v>
+        <v>2.8</v>
       </c>
       <c r="L34" t="n">
-        <v>0.3706238801763534</v>
+        <v>0.3726557773744706</v>
       </c>
       <c r="M34" t="n">
-        <v>0.2700259698427717</v>
+        <v>0.2879612825166364</v>
       </c>
       <c r="N34" t="n">
-        <v>0.3593501499808749</v>
+        <v>0.3393829401088929</v>
       </c>
       <c r="O34" t="n">
-        <v>0.05809928534151299</v>
+        <v>0.05233002291825839</v>
       </c>
       <c r="P34" t="n">
         <v>0</v>
@@ -3851,7 +3851,7 @@
         <v>0.429456815035675</v>
       </c>
       <c r="Y34" t="n">
-        <v>3.5</v>
+        <v>3.3</v>
       </c>
       <c r="Z34" t="inlineStr">
         <is>
@@ -3859,7 +3859,7 @@
         </is>
       </c>
       <c r="AA34" t="n">
-        <v>0.2012395410499449</v>
+        <v>0.1813945607033597</v>
       </c>
       <c r="AB34" t="n">
         <v>6.012395410499448</v>
@@ -3904,25 +3904,25 @@
         </is>
       </c>
       <c r="I35" t="n">
-        <v>3</v>
+        <v>3.1</v>
       </c>
       <c r="J35" t="n">
         <v>3</v>
       </c>
       <c r="K35" t="n">
-        <v>2.55</v>
+        <v>2.45</v>
       </c>
       <c r="L35" t="n">
-        <v>0.3148148148148148</v>
+        <v>0.303155289750464</v>
       </c>
       <c r="M35" t="n">
-        <v>0.3148148148148148</v>
+        <v>0.3132604660754795</v>
       </c>
       <c r="N35" t="n">
-        <v>0.3703703703703704</v>
+        <v>0.3835842441740565</v>
       </c>
       <c r="O35" t="n">
-        <v>0.05882352941176472</v>
+        <v>0.06407724380074598</v>
       </c>
       <c r="P35" t="n">
         <v>2</v>
@@ -3952,7 +3952,7 @@
         <v>0.4127240740935605</v>
       </c>
       <c r="Y35" t="n">
-        <v>2.55</v>
+        <v>2.45</v>
       </c>
       <c r="Z35" t="inlineStr">
         <is>
@@ -3960,7 +3960,7 @@
         </is>
       </c>
       <c r="AA35" t="n">
-        <v>0.0338363799603737</v>
+        <v>0.007706194158085055</v>
       </c>
       <c r="AB35" t="n">
         <v>2.889068518654924</v>
@@ -4005,25 +4005,25 @@
         </is>
       </c>
       <c r="I36" t="n">
-        <v>6.25</v>
+        <v>5.75</v>
       </c>
       <c r="J36" t="n">
         <v>4.33</v>
       </c>
       <c r="K36" t="n">
-        <v>1.5</v>
+        <v>1.53</v>
       </c>
       <c r="L36" t="n">
-        <v>0.1512839923135154</v>
+        <v>0.1643084432253056</v>
       </c>
       <c r="M36" t="n">
-        <v>0.2183660397135038</v>
+        <v>0.2181925054377615</v>
       </c>
       <c r="N36" t="n">
-        <v>0.6303499679729809</v>
+        <v>0.6174990513369328</v>
       </c>
       <c r="O36" t="n">
-        <v>0.05761354888375658</v>
+        <v>0.05845469693718108</v>
       </c>
       <c r="P36" t="n">
         <v>2</v>
@@ -4053,7 +4053,7 @@
         <v>0.5884681010357674</v>
       </c>
       <c r="Y36" t="n">
-        <v>1.5</v>
+        <v>1.53</v>
       </c>
       <c r="Z36" t="inlineStr">
         <is>
@@ -4061,10 +4061,10 @@
         </is>
       </c>
       <c r="AA36" t="n">
-        <v>-0.2345956968926978</v>
+        <v>-0.1880071800288223</v>
       </c>
       <c r="AB36" t="n">
-        <v>3.401890800787216</v>
+        <v>3.542255660284848</v>
       </c>
       <c r="AC36" t="n">
         <v>0.2710465709203975</v>
@@ -4106,25 +4106,25 @@
         </is>
       </c>
       <c r="I37" t="n">
-        <v>3.25</v>
+        <v>3.4</v>
       </c>
       <c r="J37" t="n">
-        <v>3.3</v>
+        <v>3.2</v>
       </c>
       <c r="K37" t="n">
-        <v>2.2</v>
+        <v>2.25</v>
       </c>
       <c r="L37" t="n">
-        <v>0.2888402625820569</v>
+        <v>0.2798289933929266</v>
       </c>
       <c r="M37" t="n">
-        <v>0.2844638949671772</v>
+        <v>0.2973183054799844</v>
       </c>
       <c r="N37" t="n">
-        <v>0.4266958424507659</v>
+        <v>0.4228527011270889</v>
       </c>
       <c r="O37" t="n">
-        <v>0.06526806526806528</v>
+        <v>0.05106209150326801</v>
       </c>
       <c r="P37" t="n">
         <v>2</v>
@@ -4154,7 +4154,7 @@
         <v>0.4738684654047624</v>
       </c>
       <c r="Y37" t="n">
-        <v>2.2</v>
+        <v>2.25</v>
       </c>
       <c r="Z37" t="inlineStr">
         <is>
@@ -4162,7 +4162,7 @@
         </is>
       </c>
       <c r="AA37" t="n">
-        <v>0.0354255199087312</v>
+        <v>0.05296323772857239</v>
       </c>
       <c r="AB37" t="n">
         <v>3.317079257833337</v>
@@ -4174,20 +4174,20 @@
     <row r="38">
       <c r="A38" s="1" t="inlineStr">
         <is>
-          <t>2FJLJdV9</t>
+          <t>MH5y3WcE</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
-        <v>45731.51041666666</v>
+        <v>45730.70833333334</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>mallorca</t>
+          <t>las palmas</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>espanyol</t>
+          <t>alaves</t>
         </is>
       </c>
       <c r="E38" t="n">
@@ -4207,42 +4207,44 @@
         </is>
       </c>
       <c r="I38" t="n">
-        <v>1.8</v>
+        <v>3</v>
       </c>
       <c r="J38" t="n">
-        <v>3.3</v>
+        <v>3.1</v>
       </c>
       <c r="K38" t="n">
-        <v>5</v>
+        <v>2.5</v>
       </c>
       <c r="L38" t="n">
-        <v>0.5248091603053435</v>
+        <v>0.3156822810590631</v>
       </c>
       <c r="M38" t="n">
-        <v>0.2862595419847329</v>
+        <v>0.3054989816700611</v>
       </c>
       <c r="N38" t="n">
-        <v>0.1889312977099237</v>
+        <v>0.3788187372708758</v>
       </c>
       <c r="O38" t="n">
-        <v>0.05858585858585852</v>
+        <v>0.05591397849462365</v>
       </c>
       <c r="P38" t="n">
         <v>1</v>
       </c>
       <c r="Q38" t="n">
-        <v>0.3752511765064035</v>
+        <v>0.2087588667813048</v>
       </c>
       <c r="R38" t="n">
-        <v>0.4643650265337161</v>
+        <v>0.6968926909618604</v>
       </c>
       <c r="S38" t="n">
-        <v>0.1603837969598803</v>
+        <v>0.09434844225683475</v>
       </c>
       <c r="T38" t="n">
         <v>1</v>
       </c>
-      <c r="U38" t="inlineStr"/>
+      <c r="U38" t="n">
+        <v>0</v>
+      </c>
       <c r="V38" t="n">
         <v>0</v>
       </c>
@@ -4250,10 +4252,10 @@
         <v>1</v>
       </c>
       <c r="X38" t="n">
-        <v>0.4643650265337161</v>
+        <v>0.6968926909618604</v>
       </c>
       <c r="Y38" t="n">
-        <v>1.8</v>
+        <v>3</v>
       </c>
       <c r="Z38" t="inlineStr">
         <is>
@@ -4261,32 +4263,32 @@
         </is>
       </c>
       <c r="AA38" t="n">
-        <v>-0.2051786902991386</v>
+        <v>0.5453390364427906</v>
       </c>
       <c r="AB38" t="n">
-        <v>4.131387015772588</v>
+        <v>7.317373255099533</v>
       </c>
       <c r="AC38" t="n">
-        <v>0.08911385002731265</v>
+        <v>0.4881338241805555</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="1" t="inlineStr">
         <is>
-          <t>6BzIrse2</t>
+          <t>2FJLJdV9</t>
         </is>
       </c>
       <c r="B39" s="2" t="n">
-        <v>45732.60416666666</v>
+        <v>45731.51041666666</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>rayo vallecano</t>
+          <t>mallorca</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>real sociedad</t>
+          <t>espanyol</t>
         </is>
       </c>
       <c r="E39" t="n">
@@ -4306,42 +4308,44 @@
         </is>
       </c>
       <c r="I39" t="n">
-        <v>2.6</v>
+        <v>1.8</v>
       </c>
       <c r="J39" t="n">
-        <v>3</v>
+        <v>3.3</v>
       </c>
       <c r="K39" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L39" t="n">
-        <v>0.3658536585365854</v>
+        <v>0.5248091603053435</v>
       </c>
       <c r="M39" t="n">
-        <v>0.3170731707317074</v>
+        <v>0.2862595419847329</v>
       </c>
       <c r="N39" t="n">
-        <v>0.3170731707317074</v>
+        <v>0.1889312977099237</v>
       </c>
       <c r="O39" t="n">
-        <v>0.0512820512820511</v>
+        <v>0.05858585858585852</v>
       </c>
       <c r="P39" t="n">
         <v>1</v>
       </c>
       <c r="Q39" t="n">
-        <v>0.3205217897764424</v>
+        <v>0.04496947414383049</v>
       </c>
       <c r="R39" t="n">
-        <v>0.5120408796450534</v>
+        <v>0.6653099071716773</v>
       </c>
       <c r="S39" t="n">
-        <v>0.1674373305785044</v>
+        <v>0.2897206186844923</v>
       </c>
       <c r="T39" t="n">
         <v>1</v>
       </c>
-      <c r="U39" t="inlineStr"/>
+      <c r="U39" t="n">
+        <v>0</v>
+      </c>
       <c r="V39" t="n">
         <v>0</v>
       </c>
@@ -4349,10 +4353,10 @@
         <v>1</v>
       </c>
       <c r="X39" t="n">
-        <v>0.5120408796450534</v>
+        <v>0.6653099071716773</v>
       </c>
       <c r="Y39" t="n">
-        <v>2.6</v>
+        <v>1.8</v>
       </c>
       <c r="Z39" t="inlineStr">
         <is>
@@ -4360,32 +4364,32 @@
         </is>
       </c>
       <c r="AA39" t="n">
-        <v>0.2070664294232118</v>
+        <v>0.2469472911362738</v>
       </c>
       <c r="AB39" t="n">
-        <v>5.376429236273061</v>
+        <v>6.985754025302611</v>
       </c>
       <c r="AC39" t="n">
-        <v>0.191519089868611</v>
+        <v>0.375589288487185</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="1" t="inlineStr">
         <is>
-          <t>GppsqB6r</t>
+          <t>lz02jgE8</t>
         </is>
       </c>
       <c r="B40" s="2" t="n">
-        <v>45731.41666666666</v>
+        <v>45732.51041666666</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>valladolid</t>
+          <t>sevilla</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>celta vigo</t>
+          <t>ath bilbao</t>
         </is>
       </c>
       <c r="E40" t="n">
@@ -4405,53 +4409,55 @@
         </is>
       </c>
       <c r="I40" t="n">
-        <v>5</v>
+        <v>2.9</v>
       </c>
       <c r="J40" t="n">
-        <v>3.75</v>
+        <v>3.2</v>
       </c>
       <c r="K40" t="n">
-        <v>1.7</v>
+        <v>2.5</v>
       </c>
       <c r="L40" t="n">
-        <v>0.1895910780669145</v>
+        <v>0.3261312678353037</v>
       </c>
       <c r="M40" t="n">
-        <v>0.2527881040892193</v>
+        <v>0.2955564614757439</v>
       </c>
       <c r="N40" t="n">
-        <v>0.5576208178438662</v>
+        <v>0.3783122706889523</v>
       </c>
       <c r="O40" t="n">
-        <v>0.05490196078431375</v>
+        <v>0.05732758620689671</v>
       </c>
       <c r="P40" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q40" t="n">
-        <v>0.4310033402051662</v>
+        <v>0.3966344202737069</v>
       </c>
       <c r="R40" t="n">
-        <v>0.1501830644963013</v>
+        <v>0.4133547303000261</v>
       </c>
       <c r="S40" t="n">
-        <v>0.4188135952985325</v>
+        <v>0.1900108494262671</v>
       </c>
       <c r="T40" t="n">
         <v>1</v>
       </c>
-      <c r="U40" t="inlineStr"/>
+      <c r="U40" t="n">
+        <v>0</v>
+      </c>
       <c r="V40" t="n">
         <v>0</v>
       </c>
       <c r="W40" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X40" t="n">
-        <v>0.4310033402051662</v>
+        <v>0.4133547303000261</v>
       </c>
       <c r="Y40" t="n">
-        <v>3.75</v>
+        <v>2.9</v>
       </c>
       <c r="Z40" t="inlineStr">
         <is>
@@ -4459,32 +4465,32 @@
         </is>
       </c>
       <c r="AA40" t="n">
-        <v>0.2240954639161357</v>
+        <v>0.1045940620368818</v>
       </c>
       <c r="AB40" t="n">
-        <v>7.542558453590408</v>
+        <v>0.8680449336300549</v>
       </c>
       <c r="AC40" t="n">
-        <v>0.01218974490663366</v>
+        <v>0.01672031002631919</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="1" t="inlineStr">
         <is>
-          <t>fBDkuT57</t>
+          <t>tUjwjP2S</t>
         </is>
       </c>
       <c r="B41" s="2" t="n">
-        <v>45731.60416666666</v>
+        <v>45732.70833333334</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>villarreal</t>
+          <t>atl  madrid</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>real madrid</t>
+          <t>barcelona</t>
         </is>
       </c>
       <c r="E41" t="n">
@@ -4504,53 +4510,55 @@
         </is>
       </c>
       <c r="I41" t="n">
-        <v>3.4</v>
+        <v>3.1</v>
       </c>
       <c r="J41" t="n">
-        <v>3.7</v>
+        <v>3.6</v>
       </c>
       <c r="K41" t="n">
-        <v>2</v>
+        <v>2.2</v>
       </c>
       <c r="L41" t="n">
-        <v>0.2763256161314414</v>
+        <v>0.3057915057915058</v>
       </c>
       <c r="M41" t="n">
-        <v>0.2539208364451083</v>
+        <v>0.2633204633204633</v>
       </c>
       <c r="N41" t="n">
-        <v>0.4697535474234503</v>
+        <v>0.4308880308880308</v>
       </c>
       <c r="O41" t="n">
-        <v>0.06438791732909377</v>
+        <v>0.05490387748452275</v>
       </c>
       <c r="P41" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q41" t="n">
-        <v>0.4486650993731827</v>
+        <v>0.2611919148649668</v>
       </c>
       <c r="R41" t="n">
-        <v>0.18134740625014</v>
+        <v>0.6867098866618981</v>
       </c>
       <c r="S41" t="n">
-        <v>0.3699874943766774</v>
+        <v>0.05209819847313505</v>
       </c>
       <c r="T41" t="n">
         <v>1</v>
       </c>
-      <c r="U41" t="inlineStr"/>
+      <c r="U41" t="n">
+        <v>0</v>
+      </c>
       <c r="V41" t="n">
         <v>0</v>
       </c>
       <c r="W41" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X41" t="n">
-        <v>0.4486650993731827</v>
+        <v>0.6867098866618981</v>
       </c>
       <c r="Y41" t="n">
-        <v>3.7</v>
+        <v>3.1</v>
       </c>
       <c r="Z41" t="inlineStr">
         <is>
@@ -4558,32 +4566,32 @@
         </is>
       </c>
       <c r="AA41" t="n">
-        <v>0.244466988029917</v>
+        <v>0.5375241184056592</v>
       </c>
       <c r="AB41" t="n">
-        <v>7.851639239030697</v>
+        <v>7.21045380994993</v>
       </c>
       <c r="AC41" t="n">
-        <v>0.07867760499650528</v>
+        <v>0.4255179717969313</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="1" t="inlineStr">
         <is>
-          <t>0EX9p3Qk</t>
+          <t>GppsqB6r</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
-        <v>45731.70833333334</v>
+        <v>45731.41666666666</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>girona</t>
+          <t>valladolid</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>valencia</t>
+          <t>celta vigo</t>
         </is>
       </c>
       <c r="E42" t="n">
@@ -4603,86 +4611,88 @@
         </is>
       </c>
       <c r="I42" t="n">
-        <v>1.95</v>
+        <v>5</v>
       </c>
       <c r="J42" t="n">
-        <v>3.4</v>
+        <v>3.8</v>
       </c>
       <c r="K42" t="n">
+        <v>1.67</v>
+      </c>
+      <c r="L42" t="n">
+        <v>0.1883309591642925</v>
+      </c>
+      <c r="M42" t="n">
+        <v>0.247803893637227</v>
+      </c>
+      <c r="N42" t="n">
+        <v>0.5638651471984806</v>
+      </c>
+      <c r="O42" t="n">
+        <v>0.06196028994642289</v>
+      </c>
+      <c r="P42" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q42" t="n">
+        <v>0.6340235742826343</v>
+      </c>
+      <c r="R42" t="n">
+        <v>0.1029612389095809</v>
+      </c>
+      <c r="S42" t="n">
+        <v>0.2630151868077849</v>
+      </c>
+      <c r="T42" t="n">
+        <v>1</v>
+      </c>
+      <c r="U42" t="n">
+        <v>0</v>
+      </c>
+      <c r="V42" t="n">
+        <v>0</v>
+      </c>
+      <c r="W42" t="n">
+        <v>0</v>
+      </c>
+      <c r="X42" t="n">
+        <v>0.6340235742826343</v>
+      </c>
+      <c r="Y42" t="n">
         <v>3.8</v>
       </c>
-      <c r="L42" t="n">
-        <v>0.4792284866468843</v>
-      </c>
-      <c r="M42" t="n">
-        <v>0.2748516320474778</v>
-      </c>
-      <c r="N42" t="n">
-        <v>0.245919881305638</v>
-      </c>
-      <c r="O42" t="n">
-        <v>0.0700960546161784</v>
-      </c>
-      <c r="P42" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q42" t="n">
-        <v>0.3550037211677838</v>
-      </c>
-      <c r="R42" t="n">
-        <v>0.3546354326490165</v>
-      </c>
-      <c r="S42" t="n">
-        <v>0.2903608461831997</v>
-      </c>
-      <c r="T42" t="n">
-        <v>1</v>
-      </c>
-      <c r="U42" t="inlineStr"/>
-      <c r="V42" t="n">
-        <v>0</v>
-      </c>
-      <c r="W42" t="n">
-        <v>0</v>
-      </c>
-      <c r="X42" t="n">
-        <v>0.3550037211677838</v>
-      </c>
-      <c r="Y42" t="n">
-        <v>3.4</v>
-      </c>
       <c r="Z42" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
       <c r="AA42" t="n">
-        <v>0.08625527165436044</v>
+        <v>0.5033177079550037</v>
       </c>
       <c r="AB42" t="n">
-        <v>6.212565120436217</v>
+        <v>13.31449505993532</v>
       </c>
       <c r="AC42" t="n">
-        <v>0.0003682885187673013</v>
+        <v>0.3710083874748495</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="1" t="inlineStr">
         <is>
-          <t>lbrkskye</t>
+          <t>fBDkuT57</t>
         </is>
       </c>
       <c r="B43" s="2" t="n">
-        <v>45732.60416666666</v>
+        <v>45731.60416666666</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>osasuna</t>
+          <t>villarreal</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>getafe</t>
+          <t>real madrid</t>
         </is>
       </c>
       <c r="E43" t="n">
@@ -4702,42 +4712,44 @@
         </is>
       </c>
       <c r="I43" t="n">
-        <v>2.25</v>
+        <v>3.1</v>
       </c>
       <c r="J43" t="n">
-        <v>2.8</v>
+        <v>3.75</v>
       </c>
       <c r="K43" t="n">
-        <v>3.7</v>
+        <v>2.15</v>
       </c>
       <c r="L43" t="n">
-        <v>0.4146487892735641</v>
+        <v>0.3059482022578503</v>
       </c>
       <c r="M43" t="n">
-        <v>0.3331999199519712</v>
+        <v>0.2529171805331563</v>
       </c>
       <c r="N43" t="n">
-        <v>0.2521512907744646</v>
+        <v>0.4411346172089934</v>
       </c>
       <c r="O43" t="n">
-        <v>0.0718575718575718</v>
+        <v>0.05436359089772447</v>
       </c>
       <c r="P43" t="n">
         <v>0</v>
       </c>
       <c r="Q43" t="n">
-        <v>0.3824428931437525</v>
+        <v>0.6492552146555224</v>
       </c>
       <c r="R43" t="n">
-        <v>0.3126194927723244</v>
+        <v>0.01639529249356981</v>
       </c>
       <c r="S43" t="n">
-        <v>0.304937614083923</v>
+        <v>0.3343494928509079</v>
       </c>
       <c r="T43" t="n">
         <v>1</v>
       </c>
-      <c r="U43" t="inlineStr"/>
+      <c r="U43" t="n">
+        <v>0</v>
+      </c>
       <c r="V43" t="n">
         <v>0</v>
       </c>
@@ -4745,10 +4757,10 @@
         <v>0</v>
       </c>
       <c r="X43" t="n">
-        <v>0.3824428931437525</v>
+        <v>0.6492552146555224</v>
       </c>
       <c r="Y43" t="n">
-        <v>2.8</v>
+        <v>3.75</v>
       </c>
       <c r="Z43" t="inlineStr">
         <is>
@@ -4756,32 +4768,32 @@
         </is>
       </c>
       <c r="AA43" t="n">
-        <v>0.03935561155694828</v>
+        <v>0.5217116563484396</v>
       </c>
       <c r="AB43" t="n">
-        <v>6.692750630015668</v>
+        <v>13.63435950776597</v>
       </c>
       <c r="AC43" t="n">
-        <v>0.06982340037142815</v>
+        <v>0.3149057218046145</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="1" t="inlineStr">
         <is>
-          <t>MH5y3WcE</t>
+          <t>0EX9p3Qk</t>
         </is>
       </c>
       <c r="B44" s="2" t="n">
-        <v>45730.70833333334</v>
+        <v>45731.70833333334</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>las palmas</t>
+          <t>girona</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>alaves</t>
+          <t>valencia</t>
         </is>
       </c>
       <c r="E44" t="n">
@@ -4801,53 +4813,55 @@
         </is>
       </c>
       <c r="I44" t="n">
-        <v>2.9</v>
+        <v>1.95</v>
       </c>
       <c r="J44" t="n">
-        <v>3.1</v>
+        <v>3.5</v>
       </c>
       <c r="K44" t="n">
-        <v>2.6</v>
+        <v>3.9</v>
       </c>
       <c r="L44" t="n">
-        <v>0.3277755185034567</v>
+        <v>0.4861111111111112</v>
       </c>
       <c r="M44" t="n">
-        <v>0.3066287108580724</v>
+        <v>0.2708333333333333</v>
       </c>
       <c r="N44" t="n">
-        <v>0.3655957706384709</v>
+        <v>0.2430555555555556</v>
       </c>
       <c r="O44" t="n">
-        <v>0.05202361598357141</v>
+        <v>0.05494505494505497</v>
       </c>
       <c r="P44" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="Q44" t="n">
-        <v>0.3209011448736794</v>
+        <v>0.4973412181640925</v>
       </c>
       <c r="R44" t="n">
-        <v>0.1706919167788391</v>
+        <v>0.2566072602407481</v>
       </c>
       <c r="S44" t="n">
-        <v>0.5084069383474815</v>
+        <v>0.2460515215951593</v>
       </c>
       <c r="T44" t="n">
         <v>1</v>
       </c>
-      <c r="U44" t="inlineStr"/>
+      <c r="U44" t="n">
+        <v>0</v>
+      </c>
       <c r="V44" t="n">
         <v>0</v>
       </c>
       <c r="W44" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="X44" t="n">
-        <v>0.5084069383474815</v>
+        <v>0.4973412181640925</v>
       </c>
       <c r="Y44" t="n">
-        <v>2.6</v>
+        <v>3.5</v>
       </c>
       <c r="Z44" t="inlineStr">
         <is>
@@ -4855,13 +4869,13 @@
         </is>
       </c>
       <c r="AA44" t="n">
-        <v>0.2011612748146575</v>
+        <v>0.2962777054297295</v>
       </c>
       <c r="AB44" t="n">
-        <v>0.8897121421080926</v>
+        <v>10.44416558144594</v>
       </c>
       <c r="AC44" t="n">
-        <v>0.1875057934738021</v>
+        <v>0.2407339579233444</v>
       </c>
     </row>
     <row r="45">
@@ -4900,42 +4914,44 @@
         </is>
       </c>
       <c r="I45" t="n">
-        <v>3.9</v>
+        <v>3.75</v>
       </c>
       <c r="J45" t="n">
         <v>3.25</v>
       </c>
       <c r="K45" t="n">
-        <v>2</v>
+        <v>2.1</v>
       </c>
       <c r="L45" t="n">
-        <v>0.2409638554216868</v>
+        <v>0.2538354253835426</v>
       </c>
       <c r="M45" t="n">
-        <v>0.2891566265060241</v>
+        <v>0.292887029288703</v>
       </c>
       <c r="N45" t="n">
-        <v>0.4698795180722892</v>
+        <v>0.4532775453277546</v>
       </c>
       <c r="O45" t="n">
-        <v>0.0641025641025641</v>
+        <v>0.05054945054945037</v>
       </c>
       <c r="P45" t="n">
         <v>2</v>
       </c>
       <c r="Q45" t="n">
-        <v>0.3385544934499816</v>
+        <v>0.109408675453246</v>
       </c>
       <c r="R45" t="n">
-        <v>0.1509115135418081</v>
+        <v>0.4370665462495993</v>
       </c>
       <c r="S45" t="n">
-        <v>0.5105339930082103</v>
+        <v>0.4535247782971546</v>
       </c>
       <c r="T45" t="n">
         <v>1</v>
       </c>
-      <c r="U45" t="inlineStr"/>
+      <c r="U45" t="n">
+        <v>0</v>
+      </c>
       <c r="V45" t="n">
         <v>0</v>
       </c>
@@ -4943,10 +4959,10 @@
         <v>2</v>
       </c>
       <c r="X45" t="n">
-        <v>0.5105339930082103</v>
+        <v>0.4535247782971546</v>
       </c>
       <c r="Y45" t="n">
-        <v>2</v>
+        <v>2.1</v>
       </c>
       <c r="Z45" t="inlineStr">
         <is>
@@ -4954,32 +4970,32 @@
         </is>
       </c>
       <c r="AA45" t="n">
-        <v>0.02106798601642068</v>
+        <v>-0.04327087779634121</v>
       </c>
       <c r="AB45" t="n">
-        <v>0.8934344877643681</v>
+        <v>0.1535840711377134</v>
       </c>
       <c r="AC45" t="n">
-        <v>0.1719794995582288</v>
+        <v>0.01645823204755531</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="1" t="inlineStr">
         <is>
-          <t>lz02jgE8</t>
+          <t>lbrkskye</t>
         </is>
       </c>
       <c r="B46" s="2" t="n">
-        <v>45732.51041666666</v>
+        <v>45732.60416666666</v>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>sevilla</t>
+          <t>osasuna</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>ath bilbao</t>
+          <t>getafe</t>
         </is>
       </c>
       <c r="E46" t="n">
@@ -4999,42 +5015,44 @@
         </is>
       </c>
       <c r="I46" t="n">
-        <v>3</v>
+        <v>2.25</v>
       </c>
       <c r="J46" t="n">
-        <v>3.2</v>
+        <v>2.88</v>
       </c>
       <c r="K46" t="n">
-        <v>2.4</v>
+        <v>3.8</v>
       </c>
       <c r="L46" t="n">
-        <v>0.3137254901960784</v>
+        <v>0.4213444213444213</v>
       </c>
       <c r="M46" t="n">
-        <v>0.2941176470588235</v>
+        <v>0.3291753291753292</v>
       </c>
       <c r="N46" t="n">
-        <v>0.392156862745098</v>
+        <v>0.2494802494802495</v>
       </c>
       <c r="O46" t="n">
-        <v>0.0625</v>
+        <v>0.05482456140350878</v>
       </c>
       <c r="P46" t="n">
         <v>2</v>
       </c>
       <c r="Q46" t="n">
-        <v>0.3285199202798995</v>
+        <v>0.1519711439684714</v>
       </c>
       <c r="R46" t="n">
-        <v>0.1393138671147877</v>
+        <v>0.3630337446325912</v>
       </c>
       <c r="S46" t="n">
-        <v>0.5321662126053129</v>
+        <v>0.4849951113989375</v>
       </c>
       <c r="T46" t="n">
         <v>1</v>
       </c>
-      <c r="U46" t="inlineStr"/>
+      <c r="U46" t="n">
+        <v>0</v>
+      </c>
       <c r="V46" t="n">
         <v>0</v>
       </c>
@@ -5042,10 +5060,10 @@
         <v>2</v>
       </c>
       <c r="X46" t="n">
-        <v>0.5321662126053129</v>
+        <v>0.4849951113989375</v>
       </c>
       <c r="Y46" t="n">
-        <v>2.4</v>
+        <v>3.8</v>
       </c>
       <c r="Z46" t="inlineStr">
         <is>
@@ -5053,32 +5071,32 @@
         </is>
       </c>
       <c r="AA46" t="n">
-        <v>0.1979992216091079</v>
+        <v>0.3010647940414151</v>
       </c>
       <c r="AB46" t="n">
-        <v>0.9312908720592976</v>
+        <v>0.8487414449481406</v>
       </c>
       <c r="AC46" t="n">
-        <v>0.2036462923254135</v>
+        <v>0.1219613667663463</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="1" t="inlineStr">
         <is>
-          <t>tUjwjP2S</t>
+          <t>6BzIrse2</t>
         </is>
       </c>
       <c r="B47" s="2" t="n">
-        <v>45732.70833333334</v>
+        <v>45732.60416666666</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>atl  madrid</t>
+          <t>rayo vallecano</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>barcelona</t>
+          <t>real sociedad</t>
         </is>
       </c>
       <c r="E47" t="n">
@@ -5098,42 +5116,44 @@
         </is>
       </c>
       <c r="I47" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="J47" t="n">
         <v>3</v>
       </c>
-      <c r="J47" t="n">
-        <v>3.5</v>
-      </c>
       <c r="K47" t="n">
-        <v>2.25</v>
+        <v>3.1</v>
       </c>
       <c r="L47" t="n">
-        <v>0.3134328358208955</v>
+        <v>0.3788187372708758</v>
       </c>
       <c r="M47" t="n">
-        <v>0.2686567164179104</v>
+        <v>0.3156822810590631</v>
       </c>
       <c r="N47" t="n">
-        <v>0.417910447761194</v>
+        <v>0.3054989816700611</v>
       </c>
       <c r="O47" t="n">
-        <v>0.06349206349206349</v>
+        <v>0.05591397849462365</v>
       </c>
       <c r="P47" t="n">
         <v>2</v>
       </c>
       <c r="Q47" t="n">
-        <v>0.360158691714796</v>
+        <v>0.2514995349394125</v>
       </c>
       <c r="R47" t="n">
-        <v>0.1265732302446819</v>
+        <v>0.017494109000573</v>
       </c>
       <c r="S47" t="n">
-        <v>0.5132680780405221</v>
+        <v>0.7310063560600145</v>
       </c>
       <c r="T47" t="n">
         <v>1</v>
       </c>
-      <c r="U47" t="inlineStr"/>
+      <c r="U47" t="n">
+        <v>0</v>
+      </c>
       <c r="V47" t="n">
         <v>0</v>
       </c>
@@ -5141,10 +5161,10 @@
         <v>2</v>
       </c>
       <c r="X47" t="n">
-        <v>0.5132680780405221</v>
+        <v>0.7310063560600145</v>
       </c>
       <c r="Y47" t="n">
-        <v>2.25</v>
+        <v>3.1</v>
       </c>
       <c r="Z47" t="inlineStr">
         <is>
@@ -5152,13 +5172,13 @@
         </is>
       </c>
       <c r="AA47" t="n">
-        <v>0.1238825404729398</v>
+        <v>0.6029141446600215</v>
       </c>
       <c r="AB47" t="n">
-        <v>0.8982191365709136</v>
+        <v>1.279261123105025</v>
       </c>
       <c r="AC47" t="n">
-        <v>0.1531093863257261</v>
+        <v>0.479506821120602</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
DATA. Actualizo predicciones tras reduccion de espacio m para la ea + cambio modelo en eng y fra
</commit_message>
<xml_diff>
--- a/data/predicciones.xlsx
+++ b/data/predicciones.xlsx
@@ -621,31 +621,31 @@
         <v>4.33</v>
       </c>
       <c r="K2" t="n">
-        <v>4.33</v>
+        <v>4.5</v>
       </c>
       <c r="L2" t="n">
-        <v>0.5645371577574968</v>
+        <v>0.5692192187805826</v>
       </c>
       <c r="M2" t="n">
-        <v>0.2177314211212516</v>
+        <v>0.2195372044719568</v>
       </c>
       <c r="N2" t="n">
-        <v>0.2177314211212516</v>
+        <v>0.2112435767474606</v>
       </c>
       <c r="O2" t="n">
-        <v>0.06069615964376096</v>
+        <v>0.05197149964889314</v>
       </c>
       <c r="P2" t="n">
         <v>1</v>
       </c>
       <c r="Q2" t="n">
-        <v>0.003748854788823625</v>
+        <v>0.1819318047806384</v>
       </c>
       <c r="R2" t="n">
-        <v>0.9584938014830882</v>
+        <v>0.6053335771930102</v>
       </c>
       <c r="S2" t="n">
-        <v>0.03775734372808835</v>
+        <v>0.2127346180263514</v>
       </c>
       <c r="T2" t="n">
         <v>1</v>
@@ -660,7 +660,7 @@
         <v>1</v>
       </c>
       <c r="X2" t="n">
-        <v>0.9584938014830882</v>
+        <v>0.6053335771930102</v>
       </c>
       <c r="Y2" t="n">
         <v>1.67</v>
@@ -671,32 +671,32 @@
         </is>
       </c>
       <c r="AA2" t="n">
-        <v>0.8965442514578467</v>
+        <v>0.0162792147945178</v>
       </c>
       <c r="AB2" t="n">
-        <v>1.677364152595404</v>
+        <v>9.080003657895153</v>
       </c>
       <c r="AC2" t="n">
-        <v>0.9207364577549998</v>
+        <v>0.3925989591666588</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>KrrkXYu9</t>
+          <t>WM1fBiJk</t>
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>45731.5</v>
+        <v>45732.4375</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>everton</t>
+          <t>arsenal</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>west ham</t>
+          <t>chelsea</t>
         </is>
       </c>
       <c r="E3" t="n">
@@ -716,37 +716,37 @@
         </is>
       </c>
       <c r="I3" t="n">
-        <v>2.1</v>
+        <v>1.8</v>
       </c>
       <c r="J3" t="n">
-        <v>3.2</v>
+        <v>3.6</v>
       </c>
       <c r="K3" t="n">
-        <v>3.7</v>
+        <v>4.5</v>
       </c>
       <c r="L3" t="n">
-        <v>0.449677174325864</v>
+        <v>0.5263157894736842</v>
       </c>
       <c r="M3" t="n">
-        <v>0.2951006456513482</v>
+        <v>0.2631578947368421</v>
       </c>
       <c r="N3" t="n">
-        <v>0.2552221800227877</v>
+        <v>0.2105263157894737</v>
       </c>
       <c r="O3" t="n">
-        <v>0.05896074646074645</v>
+        <v>0.05555555555555558</v>
       </c>
       <c r="P3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q3" t="n">
-        <v>0.9601086049693609</v>
+        <v>0.3345539039645855</v>
       </c>
       <c r="R3" t="n">
-        <v>0.02214276141821787</v>
+        <v>0.3493164095189908</v>
       </c>
       <c r="S3" t="n">
-        <v>0.01774863361242142</v>
+        <v>0.3161296865164237</v>
       </c>
       <c r="T3" t="n">
         <v>1</v>
@@ -758,13 +758,13 @@
         <v>0</v>
       </c>
       <c r="W3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X3" t="n">
-        <v>0.9601086049693609</v>
+        <v>0.3493164095189908</v>
       </c>
       <c r="Y3" t="n">
-        <v>3.2</v>
+        <v>1.8</v>
       </c>
       <c r="Z3" t="inlineStr">
         <is>
@@ -772,32 +772,32 @@
         </is>
       </c>
       <c r="AA3" t="n">
-        <v>0.9419761526827067</v>
+        <v>-0.4640380785822707</v>
       </c>
       <c r="AB3" t="n">
-        <v>10.08114035217829</v>
+        <v>0.5937998558844142</v>
       </c>
       <c r="AC3" t="n">
-        <v>0.937965843551143</v>
+        <v>0.01476250555440528</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>WM1fBiJk</t>
+          <t>KrrkXYu9</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>45732.4375</v>
+        <v>45731.5</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>arsenal</t>
+          <t>everton</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>chelsea</t>
+          <t>west ham</t>
         </is>
       </c>
       <c r="E4" t="n">
@@ -817,37 +817,37 @@
         </is>
       </c>
       <c r="I4" t="n">
-        <v>1.8</v>
+        <v>2.05</v>
       </c>
       <c r="J4" t="n">
-        <v>3.6</v>
+        <v>3.2</v>
       </c>
       <c r="K4" t="n">
-        <v>4.5</v>
+        <v>3.9</v>
       </c>
       <c r="L4" t="n">
-        <v>0.5263157894736842</v>
+        <v>0.4616238209728131</v>
       </c>
       <c r="M4" t="n">
-        <v>0.2631578947368421</v>
+        <v>0.2957277603107084</v>
       </c>
       <c r="N4" t="n">
-        <v>0.2105263157894737</v>
+        <v>0.2426484187164787</v>
       </c>
       <c r="O4" t="n">
-        <v>0.05555555555555558</v>
+        <v>0.05671513445903686</v>
       </c>
       <c r="P4" t="n">
         <v>0</v>
       </c>
       <c r="Q4" t="n">
-        <v>0.4948661281438991</v>
+        <v>0.3903159329531108</v>
       </c>
       <c r="R4" t="n">
-        <v>0.02183399383424048</v>
+        <v>0.2962311001079771</v>
       </c>
       <c r="S4" t="n">
-        <v>0.4832998780218604</v>
+        <v>0.3134529669389122</v>
       </c>
       <c r="T4" t="n">
         <v>1</v>
@@ -862,10 +862,10 @@
         <v>0</v>
       </c>
       <c r="X4" t="n">
-        <v>0.4948661281438991</v>
+        <v>0.3903159329531108</v>
       </c>
       <c r="Y4" t="n">
-        <v>3.6</v>
+        <v>3.2</v>
       </c>
       <c r="Z4" t="inlineStr">
         <is>
@@ -873,13 +873,13 @@
         </is>
       </c>
       <c r="AA4" t="n">
-        <v>0.3005838697377065</v>
+        <v>0.1131868115681612</v>
       </c>
       <c r="AB4" t="n">
-        <v>5.19609434551094</v>
+        <v>3.903159329531108</v>
       </c>
       <c r="AC4" t="n">
-        <v>0.01156625012203877</v>
+        <v>0.07686296601419862</v>
       </c>
     </row>
     <row r="5">
@@ -921,34 +921,34 @@
         <v>3.75</v>
       </c>
       <c r="J5" t="n">
-        <v>3.3</v>
+        <v>3.5</v>
       </c>
       <c r="K5" t="n">
         <v>2</v>
       </c>
       <c r="L5" t="n">
-        <v>0.2492917847025495</v>
+        <v>0.253393665158371</v>
       </c>
       <c r="M5" t="n">
-        <v>0.28328611898017</v>
+        <v>0.2714932126696832</v>
       </c>
       <c r="N5" t="n">
-        <v>0.4674220963172804</v>
+        <v>0.4751131221719457</v>
       </c>
       <c r="O5" t="n">
-        <v>0.06969696969696981</v>
+        <v>0.05238095238095242</v>
       </c>
       <c r="P5" t="n">
         <v>2</v>
       </c>
       <c r="Q5" t="n">
-        <v>0.04618457941927705</v>
+        <v>0.2029766535425652</v>
       </c>
       <c r="R5" t="n">
-        <v>0.0152417736073448</v>
+        <v>0.1845772805013731</v>
       </c>
       <c r="S5" t="n">
-        <v>0.9385736469733781</v>
+        <v>0.6124460659560617</v>
       </c>
       <c r="T5" t="n">
         <v>1</v>
@@ -963,7 +963,7 @@
         <v>2</v>
       </c>
       <c r="X5" t="n">
-        <v>0.9385736469733781</v>
+        <v>0.6124460659560617</v>
       </c>
       <c r="Y5" t="n">
         <v>2</v>
@@ -974,13 +974,13 @@
         </is>
       </c>
       <c r="AA5" t="n">
-        <v>0.8771472939467562</v>
+        <v>0.2248921319121233</v>
       </c>
       <c r="AB5" t="n">
-        <v>9.855023293220469</v>
+        <v>7.655575824450771</v>
       </c>
       <c r="AC5" t="n">
-        <v>0.8923890675541011</v>
+        <v>0.4094694124134964</v>
       </c>
     </row>
     <row r="6">
@@ -1019,37 +1019,37 @@
         </is>
       </c>
       <c r="I6" t="n">
-        <v>3.7</v>
+        <v>3.75</v>
       </c>
       <c r="J6" t="n">
-        <v>3.3</v>
+        <v>3.4</v>
       </c>
       <c r="K6" t="n">
-        <v>2.1</v>
+        <v>2</v>
       </c>
       <c r="L6" t="n">
-        <v>0.2575250836120401</v>
+        <v>0.2513863216266174</v>
       </c>
       <c r="M6" t="n">
-        <v>0.2887402452619844</v>
+        <v>0.2772643253234751</v>
       </c>
       <c r="N6" t="n">
-        <v>0.4537346711259755</v>
+        <v>0.4713493530499075</v>
       </c>
       <c r="O6" t="n">
-        <v>0.04949104949104943</v>
+        <v>0.0607843137254902</v>
       </c>
       <c r="P6" t="n">
         <v>2</v>
       </c>
       <c r="Q6" t="n">
-        <v>0.3531501780959142</v>
+        <v>0.3409728869479181</v>
       </c>
       <c r="R6" t="n">
-        <v>0.007708931157384713</v>
+        <v>0.1496814042073696</v>
       </c>
       <c r="S6" t="n">
-        <v>0.639140890746701</v>
+        <v>0.5093457088447123</v>
       </c>
       <c r="T6" t="n">
         <v>1</v>
@@ -1064,10 +1064,10 @@
         <v>2</v>
       </c>
       <c r="X6" t="n">
-        <v>0.639140890746701</v>
+        <v>0.5093457088447123</v>
       </c>
       <c r="Y6" t="n">
-        <v>2.1</v>
+        <v>2</v>
       </c>
       <c r="Z6" t="inlineStr">
         <is>
@@ -1075,13 +1075,13 @@
         </is>
       </c>
       <c r="AA6" t="n">
-        <v>0.3110871550618837</v>
+        <v>0.01869141768942462</v>
       </c>
       <c r="AB6" t="n">
-        <v>6.710979352840361</v>
+        <v>6.366821360558903</v>
       </c>
       <c r="AC6" t="n">
-        <v>0.2859907126507868</v>
+        <v>0.1683728218967942</v>
       </c>
     </row>
     <row r="7">
@@ -1123,34 +1123,34 @@
         <v>1.7</v>
       </c>
       <c r="J7" t="n">
-        <v>3.9</v>
+        <v>4.2</v>
       </c>
       <c r="K7" t="n">
-        <v>4.75</v>
+        <v>4.33</v>
       </c>
       <c r="L7" t="n">
-        <v>0.5574781823653325</v>
+        <v>0.556367975035947</v>
       </c>
       <c r="M7" t="n">
-        <v>0.2430033102618116</v>
+        <v>0.2251965613240738</v>
       </c>
       <c r="N7" t="n">
-        <v>0.1995185073728558</v>
+        <v>0.2184354636399792</v>
       </c>
       <c r="O7" t="n">
-        <v>0.05517186631737725</v>
+        <v>0.05727741442997525</v>
       </c>
       <c r="P7" t="n">
         <v>2</v>
       </c>
       <c r="Q7" t="n">
-        <v>0.1137302364813753</v>
+        <v>0.3288440897264435</v>
       </c>
       <c r="R7" t="n">
-        <v>0.0003515988837535767</v>
+        <v>0.2289601394870671</v>
       </c>
       <c r="S7" t="n">
-        <v>0.8859181646348711</v>
+        <v>0.4421957707864893</v>
       </c>
       <c r="T7" t="n">
         <v>1</v>
@@ -1165,10 +1165,10 @@
         <v>2</v>
       </c>
       <c r="X7" t="n">
-        <v>0.8859181646348711</v>
+        <v>0.4421957707864893</v>
       </c>
       <c r="Y7" t="n">
-        <v>4.75</v>
+        <v>4.33</v>
       </c>
       <c r="Z7" t="inlineStr">
         <is>
@@ -1176,13 +1176,13 @@
         </is>
       </c>
       <c r="AA7" t="n">
-        <v>0.8554963418708366</v>
+        <v>0.2746869932448945</v>
       </c>
       <c r="AB7" t="n">
-        <v>9.302140728666146</v>
+        <v>5.527447134831116</v>
       </c>
       <c r="AC7" t="n">
-        <v>0.7721879281534958</v>
+        <v>0.1133516810600458</v>
       </c>
     </row>
     <row r="8">
@@ -1221,37 +1221,37 @@
         </is>
       </c>
       <c r="I8" t="n">
-        <v>1.95</v>
+        <v>2</v>
       </c>
       <c r="J8" t="n">
-        <v>3.7</v>
+        <v>3.75</v>
       </c>
       <c r="K8" t="n">
-        <v>3.7</v>
+        <v>3.6</v>
       </c>
       <c r="L8" t="n">
-        <v>0.486842105263158</v>
+        <v>0.4787234042553192</v>
       </c>
       <c r="M8" t="n">
-        <v>0.256578947368421</v>
+        <v>0.2553191489361702</v>
       </c>
       <c r="N8" t="n">
-        <v>0.256578947368421</v>
+        <v>0.2659574468085107</v>
       </c>
       <c r="O8" t="n">
-        <v>0.05336105336105335</v>
+        <v>0.04444444444444429</v>
       </c>
       <c r="P8" t="n">
         <v>2</v>
       </c>
       <c r="Q8" t="n">
-        <v>0.09538689467432719</v>
+        <v>0.2028438277875327</v>
       </c>
       <c r="R8" t="n">
-        <v>0.00252255086861485</v>
+        <v>0.2040858139837192</v>
       </c>
       <c r="S8" t="n">
-        <v>0.902090554457058</v>
+        <v>0.5930703582287481</v>
       </c>
       <c r="T8" t="n">
         <v>1</v>
@@ -1266,10 +1266,10 @@
         <v>2</v>
       </c>
       <c r="X8" t="n">
-        <v>0.902090554457058</v>
+        <v>0.5930703582287481</v>
       </c>
       <c r="Y8" t="n">
-        <v>3.7</v>
+        <v>3.6</v>
       </c>
       <c r="Z8" t="inlineStr">
         <is>
@@ -1277,13 +1277,13 @@
         </is>
       </c>
       <c r="AA8" t="n">
-        <v>0.865827796848561</v>
+        <v>0.4365589575474974</v>
       </c>
       <c r="AB8" t="n">
-        <v>9.471950821799108</v>
+        <v>7.413379477859351</v>
       </c>
       <c r="AC8" t="n">
-        <v>0.8067036597827308</v>
+        <v>0.3889845442450289</v>
       </c>
     </row>
     <row r="9">
@@ -1346,13 +1346,13 @@
         <v>2</v>
       </c>
       <c r="Q9" t="n">
-        <v>0.02514691498385857</v>
+        <v>0.1766210291085296</v>
       </c>
       <c r="R9" t="n">
-        <v>0.1024152536126395</v>
+        <v>0.1996884664169913</v>
       </c>
       <c r="S9" t="n">
-        <v>0.872437831403502</v>
+        <v>0.623690504474479</v>
       </c>
       <c r="T9" t="n">
         <v>1</v>
@@ -1367,7 +1367,7 @@
         <v>2</v>
       </c>
       <c r="X9" t="n">
-        <v>0.872437831403502</v>
+        <v>0.623690504474479</v>
       </c>
       <c r="Y9" t="n">
         <v>1.83</v>
@@ -1378,13 +1378,13 @@
         </is>
       </c>
       <c r="AA9" t="n">
-        <v>0.7187484716486851</v>
+        <v>0.1703055701063816</v>
       </c>
       <c r="AB9" t="n">
-        <v>9.160597229736769</v>
+        <v>7.796131305930988</v>
       </c>
       <c r="AC9" t="n">
-        <v>0.7700225777908625</v>
+        <v>0.4240020380574877</v>
       </c>
     </row>
     <row r="10">
@@ -1429,31 +1429,31 @@
         <v>4</v>
       </c>
       <c r="K10" t="n">
-        <v>5.5</v>
+        <v>6</v>
       </c>
       <c r="L10" t="n">
-        <v>0.5959637003927942</v>
+        <v>0.6045340050377834</v>
       </c>
       <c r="M10" t="n">
-        <v>0.2339157524041718</v>
+        <v>0.23727959697733</v>
       </c>
       <c r="N10" t="n">
-        <v>0.170120547203034</v>
+        <v>0.1581863979848867</v>
       </c>
       <c r="O10" t="n">
-        <v>0.06876085697741741</v>
+        <v>0.05360934182590227</v>
       </c>
       <c r="P10" t="n">
         <v>1</v>
       </c>
       <c r="Q10" t="n">
-        <v>0.324477770545987</v>
+        <v>0.2867448725048787</v>
       </c>
       <c r="R10" t="n">
-        <v>0.4637522384700204</v>
+        <v>0.4656366345949217</v>
       </c>
       <c r="S10" t="n">
-        <v>0.2117699909839925</v>
+        <v>0.2476184929001998</v>
       </c>
       <c r="T10" t="n">
         <v>1</v>
@@ -1468,7 +1468,7 @@
         <v>1</v>
       </c>
       <c r="X10" t="n">
-        <v>0.4637522384700204</v>
+        <v>0.4656366345949217</v>
       </c>
       <c r="Y10" t="n">
         <v>1.57</v>
@@ -1479,13 +1479,13 @@
         </is>
       </c>
       <c r="AA10" t="n">
-        <v>-0.4770333080738035</v>
+        <v>-0.4718429538350402</v>
       </c>
       <c r="AB10" t="n">
-        <v>0.53299407487669</v>
+        <v>1.304510869998926</v>
       </c>
       <c r="AC10" t="n">
-        <v>0.1392744679240334</v>
+        <v>0.178891762090043</v>
       </c>
     </row>
     <row r="11">
@@ -1527,45 +1527,49 @@
         <v>1.36</v>
       </c>
       <c r="J11" t="n">
-        <v>5.25</v>
+        <v>5.5</v>
       </c>
       <c r="K11" t="n">
         <v>7</v>
       </c>
       <c r="L11" t="n">
-        <v>0.6880733944954128</v>
+        <v>0.6936936936936937</v>
       </c>
       <c r="M11" t="n">
-        <v>0.1782437745740498</v>
+        <v>0.1715315315315316</v>
       </c>
       <c r="N11" t="n">
-        <v>0.1336828309305373</v>
+        <v>0.1347747747747748</v>
       </c>
       <c r="O11" t="n">
-        <v>0.06862745098039214</v>
+        <v>0.05996944232238333</v>
       </c>
       <c r="P11" t="n">
         <v>1</v>
       </c>
       <c r="Q11" t="n">
-        <v>0.3151703740088735</v>
+        <v>0.2701672091768437</v>
       </c>
       <c r="R11" t="n">
-        <v>0.502145549994072</v>
+        <v>0.5196998489974072</v>
       </c>
       <c r="S11" t="n">
-        <v>0.1826840759970546</v>
+        <v>0.2101329418257492</v>
       </c>
       <c r="T11" t="n">
         <v>1</v>
       </c>
-      <c r="U11" t="inlineStr"/>
-      <c r="V11" t="inlineStr"/>
+      <c r="U11" t="n">
+        <v>1</v>
+      </c>
+      <c r="V11" t="n">
+        <v>0</v>
+      </c>
       <c r="W11" t="n">
         <v>1</v>
       </c>
       <c r="X11" t="n">
-        <v>0.502145549994072</v>
+        <v>0.5196998489974072</v>
       </c>
       <c r="Y11" t="n">
         <v>1.36</v>
@@ -1576,13 +1580,13 @@
         </is>
       </c>
       <c r="AA11" t="n">
-        <v>-0.880783477800172</v>
+        <v>-0.814467237120906</v>
       </c>
       <c r="AB11" t="n">
-        <v>0.7403432334770879</v>
+        <v>1.704369997036379</v>
       </c>
       <c r="AC11" t="n">
-        <v>0.1869751759851985</v>
+        <v>0.2495326398205635</v>
       </c>
     </row>
     <row r="12">
@@ -1624,45 +1628,49 @@
         <v>1.67</v>
       </c>
       <c r="J12" t="n">
-        <v>3.7</v>
+        <v>3.9</v>
       </c>
       <c r="K12" t="n">
         <v>5</v>
       </c>
       <c r="L12" t="n">
-        <v>0.5601138393532957</v>
+        <v>0.5674708261793209</v>
       </c>
       <c r="M12" t="n">
-        <v>0.2528081383027037</v>
+        <v>0.2429939178767861</v>
       </c>
       <c r="N12" t="n">
-        <v>0.1870780223440008</v>
+        <v>0.1895352559438931</v>
       </c>
       <c r="O12" t="n">
-        <v>0.06907266547985103</v>
+        <v>0.05521265161983724</v>
       </c>
       <c r="P12" t="n">
         <v>1</v>
       </c>
       <c r="Q12" t="n">
-        <v>0.3324608718279879</v>
+        <v>0.290347959509236</v>
       </c>
       <c r="R12" t="n">
-        <v>0.3885275719693547</v>
+        <v>0.3872018922687704</v>
       </c>
       <c r="S12" t="n">
-        <v>0.2790115562026576</v>
+        <v>0.3224501482219935</v>
       </c>
       <c r="T12" t="n">
         <v>1</v>
       </c>
-      <c r="U12" t="inlineStr"/>
-      <c r="V12" t="inlineStr"/>
+      <c r="U12" t="n">
+        <v>1</v>
+      </c>
+      <c r="V12" t="n">
+        <v>0</v>
+      </c>
       <c r="W12" t="n">
         <v>1</v>
       </c>
       <c r="X12" t="n">
-        <v>0.3885275719693547</v>
+        <v>0.3872018922687704</v>
       </c>
       <c r="Y12" t="n">
         <v>1.67</v>
@@ -1673,19 +1681,19 @@
         </is>
       </c>
       <c r="AA12" t="n">
-        <v>-0.524117843001758</v>
+        <v>-0.5274221491211247</v>
       </c>
       <c r="AB12" t="n">
-        <v>0.8512372059595756</v>
+        <v>2.000253597831641</v>
       </c>
       <c r="AC12" t="n">
-        <v>0.05606670014136678</v>
+        <v>0.06475174404677692</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
-          <t>hEkEOCFE</t>
+          <t>bZz9Dn7D</t>
         </is>
       </c>
       <c r="B13" s="2" t="n">
@@ -1693,12 +1701,12 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>montpellier</t>
+          <t>strasbourg</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>st etienne</t>
+          <t>toulouse</t>
         </is>
       </c>
       <c r="E13" t="n">
@@ -1718,51 +1726,55 @@
         </is>
       </c>
       <c r="I13" t="n">
-        <v>2.2</v>
+        <v>2.25</v>
       </c>
       <c r="J13" t="n">
-        <v>3.4</v>
+        <v>3.25</v>
       </c>
       <c r="K13" t="n">
-        <v>3.2</v>
+        <v>3.25</v>
       </c>
       <c r="L13" t="n">
-        <v>0.4283464566929134</v>
+        <v>0.4193548387096774</v>
       </c>
       <c r="M13" t="n">
-        <v>0.2771653543307087</v>
+        <v>0.2903225806451613</v>
       </c>
       <c r="N13" t="n">
-        <v>0.294488188976378</v>
+        <v>0.2903225806451613</v>
       </c>
       <c r="O13" t="n">
-        <v>0.06116310160427796</v>
+        <v>0.05982905982905984</v>
       </c>
       <c r="P13" t="n">
         <v>1</v>
       </c>
       <c r="Q13" t="n">
-        <v>0.346093611067589</v>
+        <v>0.3171570327596602</v>
       </c>
       <c r="R13" t="n">
-        <v>0.3633121028727284</v>
+        <v>0.4041497819598617</v>
       </c>
       <c r="S13" t="n">
-        <v>0.2905942860596827</v>
+        <v>0.2786931852804782</v>
       </c>
       <c r="T13" t="n">
         <v>1</v>
       </c>
-      <c r="U13" t="inlineStr"/>
-      <c r="V13" t="inlineStr"/>
+      <c r="U13" t="n">
+        <v>1</v>
+      </c>
+      <c r="V13" t="n">
+        <v>0</v>
+      </c>
       <c r="W13" t="n">
         <v>1</v>
       </c>
       <c r="X13" t="n">
-        <v>0.3633121028727284</v>
+        <v>0.4041497819598617</v>
       </c>
       <c r="Y13" t="n">
-        <v>2.2</v>
+        <v>2.25</v>
       </c>
       <c r="Z13" t="inlineStr">
         <is>
@@ -1770,32 +1782,32 @@
         </is>
       </c>
       <c r="AA13" t="n">
-        <v>-0.1672611447333311</v>
+        <v>-0.07253039247224899</v>
       </c>
       <c r="AB13" t="n">
-        <v>0.2225815761682787</v>
+        <v>3.748879338601554</v>
       </c>
       <c r="AC13" t="n">
-        <v>0.01721849180513946</v>
+        <v>0.08699274920020145</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="inlineStr">
         <is>
-          <t>bZz9Dn7D</t>
+          <t>jk9J2Vhe</t>
         </is>
       </c>
       <c r="B14" s="2" t="n">
-        <v>45732.55208333334</v>
+        <v>45732.69791666666</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>strasbourg</t>
+          <t>psg</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>toulouse</t>
+          <t>marseille</t>
         </is>
       </c>
       <c r="E14" t="n">
@@ -1815,51 +1827,55 @@
         </is>
       </c>
       <c r="I14" t="n">
-        <v>2.25</v>
+        <v>1.45</v>
       </c>
       <c r="J14" t="n">
-        <v>3.25</v>
+        <v>5</v>
       </c>
       <c r="K14" t="n">
-        <v>3.25</v>
+        <v>6</v>
       </c>
       <c r="L14" t="n">
-        <v>0.4193548387096774</v>
+        <v>0.6528835690968444</v>
       </c>
       <c r="M14" t="n">
-        <v>0.2903225806451613</v>
+        <v>0.1893362350380849</v>
       </c>
       <c r="N14" t="n">
-        <v>0.2903225806451613</v>
+        <v>0.1577801958650707</v>
       </c>
       <c r="O14" t="n">
-        <v>0.05982905982905984</v>
+        <v>0.05632183908045985</v>
       </c>
       <c r="P14" t="n">
         <v>1</v>
       </c>
       <c r="Q14" t="n">
-        <v>0.3444739169138507</v>
+        <v>0.3851244220539524</v>
       </c>
       <c r="R14" t="n">
-        <v>0.3885043726616377</v>
+        <v>0.3880416997331687</v>
       </c>
       <c r="S14" t="n">
-        <v>0.2670217104245117</v>
+        <v>0.2268338782128791</v>
       </c>
       <c r="T14" t="n">
         <v>1</v>
       </c>
-      <c r="U14" t="inlineStr"/>
-      <c r="V14" t="inlineStr"/>
+      <c r="U14" t="n">
+        <v>1</v>
+      </c>
+      <c r="V14" t="n">
+        <v>0</v>
+      </c>
       <c r="W14" t="n">
         <v>1</v>
       </c>
       <c r="X14" t="n">
-        <v>0.3885043726616377</v>
+        <v>0.3880416997331687</v>
       </c>
       <c r="Y14" t="n">
-        <v>2.25</v>
+        <v>1.45</v>
       </c>
       <c r="Z14" t="inlineStr">
         <is>
@@ -1867,32 +1883,32 @@
         </is>
       </c>
       <c r="AA14" t="n">
-        <v>-0.1006921292090521</v>
+        <v>-0.9718656341931234</v>
       </c>
       <c r="AB14" t="n">
-        <v>1.257271827165174</v>
+        <v>0.1943910569532937</v>
       </c>
       <c r="AC14" t="n">
-        <v>0.04403045574778702</v>
+        <v>0.002917277679216235</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="inlineStr">
         <is>
-          <t>jk9J2Vhe</t>
+          <t>OEiKK3Et</t>
         </is>
       </c>
       <c r="B15" s="2" t="n">
-        <v>45732.69791666666</v>
+        <v>45731.54166666666</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>psg</t>
+          <t>nantes</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>marseille</t>
+          <t>lille</t>
         </is>
       </c>
       <c r="E15" t="n">
@@ -1912,37 +1928,37 @@
         </is>
       </c>
       <c r="I15" t="n">
-        <v>1.48</v>
+        <v>3.6</v>
       </c>
       <c r="J15" t="n">
-        <v>5</v>
+        <v>3.2</v>
       </c>
       <c r="K15" t="n">
-        <v>5.5</v>
+        <v>2.15</v>
       </c>
       <c r="L15" t="n">
-        <v>0.6389405204460966</v>
+        <v>0.2631981637337414</v>
       </c>
       <c r="M15" t="n">
-        <v>0.1891263940520446</v>
+        <v>0.296097934200459</v>
       </c>
       <c r="N15" t="n">
-        <v>0.1719330855018587</v>
+        <v>0.4407039020657995</v>
       </c>
       <c r="O15" t="n">
-        <v>0.05749385749385749</v>
+        <v>0.05539405684754528</v>
       </c>
       <c r="P15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q15" t="n">
-        <v>0.3338974972391223</v>
+        <v>0.3599593831083472</v>
       </c>
       <c r="R15" t="n">
-        <v>0.4234568083806666</v>
+        <v>0.2179311917455568</v>
       </c>
       <c r="S15" t="n">
-        <v>0.242645694380211</v>
+        <v>0.422109425146096</v>
       </c>
       <c r="T15" t="n">
         <v>1</v>
@@ -1950,13 +1966,13 @@
       <c r="U15" t="inlineStr"/>
       <c r="V15" t="inlineStr"/>
       <c r="W15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="X15" t="n">
-        <v>0.4234568083806666</v>
+        <v>0.422109425146096</v>
       </c>
       <c r="Y15" t="n">
-        <v>1.48</v>
+        <v>2.15</v>
       </c>
       <c r="Z15" t="inlineStr">
         <is>
@@ -1964,32 +1980,32 @@
         </is>
       </c>
       <c r="AA15" t="n">
-        <v>-0.7776748408262778</v>
+        <v>-0.08040411820512493</v>
       </c>
       <c r="AB15" t="n">
-        <v>0.7039554093951731</v>
+        <v>5.823645564827026</v>
       </c>
       <c r="AC15" t="n">
-        <v>0.08955931114154431</v>
+        <v>0.06215004203774877</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="inlineStr">
         <is>
-          <t>xKn0F8x1</t>
+          <t>KtoTIsqg</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
-        <v>45731.71180555555</v>
+        <v>45731.625</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>lens</t>
+          <t>angers</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>rennes</t>
+          <t>monaco</t>
         </is>
       </c>
       <c r="E16" t="n">
@@ -2009,51 +2025,55 @@
         </is>
       </c>
       <c r="I16" t="n">
-        <v>2.05</v>
+        <v>6.5</v>
       </c>
       <c r="J16" t="n">
-        <v>3.5</v>
+        <v>4.75</v>
       </c>
       <c r="K16" t="n">
-        <v>3.5</v>
+        <v>1.42</v>
       </c>
       <c r="L16" t="n">
-        <v>0.4605263157894737</v>
+        <v>0.1439701173959445</v>
       </c>
       <c r="M16" t="n">
-        <v>0.2697368421052631</v>
+        <v>0.1970117395944503</v>
       </c>
       <c r="N16" t="n">
-        <v>0.2697368421052631</v>
+        <v>0.6590181430096052</v>
       </c>
       <c r="O16" t="n">
-        <v>0.0592334494773521</v>
+        <v>0.06859782174830364</v>
       </c>
       <c r="P16" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="Q16" t="n">
-        <v>0.3489445586821911</v>
+        <v>0.3309016977987642</v>
       </c>
       <c r="R16" t="n">
-        <v>0.337074904645411</v>
+        <v>0.1698830794120545</v>
       </c>
       <c r="S16" t="n">
-        <v>0.3139805366723979</v>
+        <v>0.4992152227891813</v>
       </c>
       <c r="T16" t="n">
         <v>1</v>
       </c>
-      <c r="U16" t="inlineStr"/>
-      <c r="V16" t="inlineStr"/>
+      <c r="U16" t="n">
+        <v>1</v>
+      </c>
+      <c r="V16" t="n">
+        <v>0</v>
+      </c>
       <c r="W16" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="X16" t="n">
-        <v>0.3489445586821911</v>
+        <v>0.4992152227891813</v>
       </c>
       <c r="Y16" t="n">
-        <v>3.5</v>
+        <v>1.42</v>
       </c>
       <c r="Z16" t="inlineStr">
         <is>
@@ -2061,32 +2081,32 @@
         </is>
       </c>
       <c r="AA16" t="n">
-        <v>0.08852238215506754</v>
+        <v>-0.6931294848556253</v>
       </c>
       <c r="AB16" t="n">
-        <v>7.327835732326012</v>
+        <v>2.995376143699266</v>
       </c>
       <c r="AC16" t="n">
-        <v>0.01186965403678014</v>
+        <v>0.1683135249904171</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="inlineStr">
         <is>
-          <t>OEiKK3Et</t>
+          <t>xKn0F8x1</t>
         </is>
       </c>
       <c r="B17" s="2" t="n">
-        <v>45731.54166666666</v>
+        <v>45731.71180555555</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>nantes</t>
+          <t>lens</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>lille</t>
+          <t>rennes</t>
         </is>
       </c>
       <c r="E17" t="n">
@@ -2106,37 +2126,37 @@
         </is>
       </c>
       <c r="I17" t="n">
+        <v>2.05</v>
+      </c>
+      <c r="J17" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="K17" t="n">
         <v>3.6</v>
       </c>
-      <c r="J17" t="n">
-        <v>3.2</v>
-      </c>
-      <c r="K17" t="n">
-        <v>2.1</v>
-      </c>
       <c r="L17" t="n">
-        <v>0.2604651162790698</v>
+        <v>0.4640029460504511</v>
       </c>
       <c r="M17" t="n">
-        <v>0.2930232558139535</v>
+        <v>0.2717731541152641</v>
       </c>
       <c r="N17" t="n">
-        <v>0.4465116279069767</v>
+        <v>0.2642238998342846</v>
       </c>
       <c r="O17" t="n">
-        <v>0.06646825396825395</v>
+        <v>0.05129694154084419</v>
       </c>
       <c r="P17" t="n">
         <v>2</v>
       </c>
       <c r="Q17" t="n">
-        <v>0.3408893113707371</v>
+        <v>0.3075905795670333</v>
       </c>
       <c r="R17" t="n">
-        <v>0.2125136503296773</v>
+        <v>0.2811150809950221</v>
       </c>
       <c r="S17" t="n">
-        <v>0.4465970382995856</v>
+        <v>0.4112943394379447</v>
       </c>
       <c r="T17" t="n">
         <v>1</v>
@@ -2147,10 +2167,10 @@
         <v>2</v>
       </c>
       <c r="X17" t="n">
-        <v>0.4465970382995856</v>
+        <v>0.4112943394379447</v>
       </c>
       <c r="Y17" t="n">
-        <v>2.1</v>
+        <v>3.6</v>
       </c>
       <c r="Z17" t="inlineStr">
         <is>
@@ -2158,32 +2178,32 @@
         </is>
       </c>
       <c r="AA17" t="n">
-        <v>-0.05649656324624562</v>
+        <v>0.1848690853756157</v>
       </c>
       <c r="AB17" t="n">
-        <v>7.484486746979738</v>
+        <v>6.169415091569171</v>
       </c>
       <c r="AC17" t="n">
-        <v>0.1057077269288484</v>
+        <v>0.1037037598709113</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="inlineStr">
         <is>
-          <t>KtoTIsqg</t>
+          <t>hEkEOCFE</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
-        <v>45731.625</v>
+        <v>45732.55208333334</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>angers</t>
+          <t>montpellier</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>monaco</t>
+          <t>st etienne</t>
         </is>
       </c>
       <c r="E18" t="n">
@@ -2203,37 +2223,37 @@
         </is>
       </c>
       <c r="I18" t="n">
-        <v>6.5</v>
+        <v>2.2</v>
       </c>
       <c r="J18" t="n">
-        <v>4.75</v>
+        <v>3.5</v>
       </c>
       <c r="K18" t="n">
-        <v>1.44</v>
+        <v>3.2</v>
       </c>
       <c r="L18" t="n">
-        <v>0.1453000531067446</v>
+        <v>0.4317656129529684</v>
       </c>
       <c r="M18" t="n">
-        <v>0.1988316516197557</v>
+        <v>0.2713955281418658</v>
       </c>
       <c r="N18" t="n">
-        <v>0.6558682952734998</v>
+        <v>0.2968388589051658</v>
       </c>
       <c r="O18" t="n">
-        <v>0.05881691408007184</v>
+        <v>0.05275974025974017</v>
       </c>
       <c r="P18" t="n">
         <v>2</v>
       </c>
       <c r="Q18" t="n">
-        <v>0.324426563388138</v>
+        <v>0.3158253888592285</v>
       </c>
       <c r="R18" t="n">
-        <v>0.1576709952462738</v>
+        <v>0.3400063945749346</v>
       </c>
       <c r="S18" t="n">
-        <v>0.5179024413655883</v>
+        <v>0.3441682165658369</v>
       </c>
       <c r="T18" t="n">
         <v>1</v>
@@ -2244,10 +2264,10 @@
         <v>2</v>
       </c>
       <c r="X18" t="n">
-        <v>0.5179024413655883</v>
+        <v>0.3441682165658369</v>
       </c>
       <c r="Y18" t="n">
-        <v>1.44</v>
+        <v>3.2</v>
       </c>
       <c r="Z18" t="inlineStr">
         <is>
@@ -2255,13 +2275,13 @@
         </is>
       </c>
       <c r="AA18" t="n">
-        <v>-0.5777738282580749</v>
+        <v>0.04606286045939913</v>
       </c>
       <c r="AB18" t="n">
-        <v>5.36455583562247</v>
+        <v>1.032504649697511</v>
       </c>
       <c r="AC18" t="n">
-        <v>0.1934758779774503</v>
+        <v>0.004161821990902259</v>
       </c>
     </row>
     <row r="19">
@@ -2300,25 +2320,25 @@
         </is>
       </c>
       <c r="I19" t="n">
-        <v>1.95</v>
+        <v>2</v>
       </c>
       <c r="J19" t="n">
-        <v>3.3</v>
+        <v>3.25</v>
       </c>
       <c r="K19" t="n">
         <v>4</v>
       </c>
       <c r="L19" t="n">
-        <v>0.4811372334609076</v>
+        <v>0.4727272727272727</v>
       </c>
       <c r="M19" t="n">
-        <v>0.2843083652268999</v>
+        <v>0.2909090909090909</v>
       </c>
       <c r="N19" t="n">
-        <v>0.2345544013121924</v>
+        <v>0.2363636363636364</v>
       </c>
       <c r="O19" t="n">
-        <v>0.06585081585081598</v>
+        <v>0.05769230769230771</v>
       </c>
       <c r="P19" t="n">
         <v>0</v>
@@ -2348,7 +2368,7 @@
         <v>0.3640266688230058</v>
       </c>
       <c r="Y19" t="n">
-        <v>3.3</v>
+        <v>3.25</v>
       </c>
       <c r="Z19" t="inlineStr">
         <is>
@@ -2356,10 +2376,10 @@
         </is>
       </c>
       <c r="AA19" t="n">
-        <v>0.08751652483300826</v>
+        <v>0.08137185496656392</v>
       </c>
       <c r="AB19" t="n">
-        <v>7.644560045283121</v>
+        <v>5.460400032345087</v>
       </c>
       <c r="AC19" t="n">
         <v>0.02894922060545724</v>
@@ -2401,25 +2421,25 @@
         </is>
       </c>
       <c r="I20" t="n">
-        <v>2.25</v>
+        <v>2.4</v>
       </c>
       <c r="J20" t="n">
-        <v>3.5</v>
+        <v>3.6</v>
       </c>
       <c r="K20" t="n">
-        <v>3</v>
+        <v>2.75</v>
       </c>
       <c r="L20" t="n">
-        <v>0.417910447761194</v>
+        <v>0.3937947494033414</v>
       </c>
       <c r="M20" t="n">
-        <v>0.2686567164179104</v>
+        <v>0.2625298329355609</v>
       </c>
       <c r="N20" t="n">
-        <v>0.3134328358208955</v>
+        <v>0.3436754176610979</v>
       </c>
       <c r="O20" t="n">
-        <v>0.06349206349206349</v>
+        <v>0.05808080808080796</v>
       </c>
       <c r="P20" t="n">
         <v>0</v>
@@ -2449,7 +2469,7 @@
         <v>0.3621597653085013</v>
       </c>
       <c r="Y20" t="n">
-        <v>3.5</v>
+        <v>3.6</v>
       </c>
       <c r="Z20" t="inlineStr">
         <is>
@@ -2457,10 +2477,10 @@
         </is>
       </c>
       <c r="AA20" t="n">
-        <v>0.1070236714319019</v>
+        <v>0.1168365981194634</v>
       </c>
       <c r="AB20" t="n">
-        <v>7.605355071478527</v>
+        <v>5.43239647962752</v>
       </c>
       <c r="AC20" t="n">
         <v>0.04289543686923009</v>
@@ -2502,25 +2522,25 @@
         </is>
       </c>
       <c r="I21" t="n">
-        <v>2.4</v>
+        <v>2.38</v>
       </c>
       <c r="J21" t="n">
         <v>3.6</v>
       </c>
       <c r="K21" t="n">
-        <v>2.7</v>
+        <v>2.88</v>
       </c>
       <c r="L21" t="n">
-        <v>0.391304347826087</v>
+        <v>0.4020100502512564</v>
       </c>
       <c r="M21" t="n">
-        <v>0.2608695652173913</v>
+        <v>0.2657733109994417</v>
       </c>
       <c r="N21" t="n">
-        <v>0.3478260869565217</v>
+        <v>0.3322166387493021</v>
       </c>
       <c r="O21" t="n">
-        <v>0.06481481481481488</v>
+        <v>0.0451680672268906</v>
       </c>
       <c r="P21" t="n">
         <v>0</v>
@@ -2561,7 +2581,7 @@
         <v>0.1590623990001787</v>
       </c>
       <c r="AB21" t="n">
-        <v>8.245779718169375</v>
+        <v>5.889842655835269</v>
       </c>
       <c r="AC21" t="n">
         <v>0.0263440014354237</v>
@@ -2606,22 +2626,22 @@
         <v>3.1</v>
       </c>
       <c r="J22" t="n">
-        <v>3.5</v>
+        <v>3.6</v>
       </c>
       <c r="K22" t="n">
         <v>2.2</v>
       </c>
       <c r="L22" t="n">
-        <v>0.303508080409933</v>
+        <v>0.3057915057915058</v>
       </c>
       <c r="M22" t="n">
-        <v>0.2688214426487978</v>
+        <v>0.2633204633204633</v>
       </c>
       <c r="N22" t="n">
-        <v>0.4276704769412692</v>
+        <v>0.4308880308880308</v>
       </c>
       <c r="O22" t="n">
-        <v>0.06284038542103065</v>
+        <v>0.05490387748452275</v>
       </c>
       <c r="P22" t="n">
         <v>0</v>
@@ -2651,7 +2671,7 @@
         <v>0.3796238743895269</v>
       </c>
       <c r="Y22" t="n">
-        <v>3.5</v>
+        <v>3.6</v>
       </c>
       <c r="Z22" t="inlineStr">
         <is>
@@ -2659,10 +2679,10 @@
         </is>
       </c>
       <c r="AA22" t="n">
-        <v>0.1314734241453377</v>
+        <v>0.1410176722316527</v>
       </c>
       <c r="AB22" t="n">
-        <v>7.972101362180066</v>
+        <v>5.694358115842904</v>
       </c>
       <c r="AC22" t="n">
         <v>0.0493065230196385</v>
@@ -2704,25 +2724,25 @@
         </is>
       </c>
       <c r="I23" t="n">
-        <v>1.92</v>
+        <v>2</v>
       </c>
       <c r="J23" t="n">
         <v>3.5</v>
       </c>
       <c r="K23" t="n">
-        <v>3.7</v>
+        <v>3.75</v>
       </c>
       <c r="L23" t="n">
-        <v>0.4836781952640622</v>
+        <v>0.4751131221719457</v>
       </c>
       <c r="M23" t="n">
-        <v>0.2653320385448569</v>
+        <v>0.2714932126696832</v>
       </c>
       <c r="N23" t="n">
-        <v>0.2509897661910809</v>
+        <v>0.253393665158371</v>
       </c>
       <c r="O23" t="n">
-        <v>0.07681788931788924</v>
+        <v>0.05238095238095242</v>
       </c>
       <c r="P23" t="n">
         <v>0</v>
@@ -2763,7 +2783,7 @@
         <v>0.1443881393418322</v>
       </c>
       <c r="AB23" t="n">
-        <v>8.165822090127483</v>
+        <v>5.832730064376774</v>
       </c>
       <c r="AC23" t="n">
         <v>0.05453877501989568</v>
@@ -2808,22 +2828,22 @@
         <v>2.25</v>
       </c>
       <c r="J24" t="n">
-        <v>3.2</v>
+        <v>3.25</v>
       </c>
       <c r="K24" t="n">
         <v>3.3</v>
       </c>
       <c r="L24" t="n">
-        <v>0.4192972007147112</v>
+        <v>0.4212076583210604</v>
       </c>
       <c r="M24" t="n">
-        <v>0.2948183442525313</v>
+        <v>0.2916053019145803</v>
       </c>
       <c r="N24" t="n">
-        <v>0.2858844550327576</v>
+        <v>0.2871870397643594</v>
       </c>
       <c r="O24" t="n">
-        <v>0.0599747474747474</v>
+        <v>0.05516705516705511</v>
       </c>
       <c r="P24" t="n">
         <v>2</v>
@@ -2864,7 +2884,7 @@
         <v>0.09582982254863967</v>
       </c>
       <c r="AB24" t="n">
-        <v>1.553247298733291</v>
+        <v>1.109462356238065</v>
       </c>
       <c r="AC24" t="n">
         <v>0.006039438668831443</v>
@@ -2906,25 +2926,25 @@
         </is>
       </c>
       <c r="I25" t="n">
-        <v>2.6</v>
+        <v>2.55</v>
       </c>
       <c r="J25" t="n">
         <v>3.3</v>
       </c>
       <c r="K25" t="n">
-        <v>2.7</v>
+        <v>2.75</v>
       </c>
       <c r="L25" t="n">
-        <v>0.3635250917992656</v>
+        <v>0.3703703703703703</v>
       </c>
       <c r="M25" t="n">
-        <v>0.2864137086903305</v>
+        <v>0.2861952861952861</v>
       </c>
       <c r="N25" t="n">
-        <v>0.3500611995104039</v>
+        <v>0.3434343434343434</v>
       </c>
       <c r="O25" t="n">
-        <v>0.05801605801605803</v>
+        <v>0.05882352941176494</v>
       </c>
       <c r="P25" t="n">
         <v>2</v>
@@ -2954,7 +2974,7 @@
         <v>0.4435846554593713</v>
       </c>
       <c r="Y25" t="n">
-        <v>2.7</v>
+        <v>2.75</v>
       </c>
       <c r="Z25" t="inlineStr">
         <is>
@@ -2962,10 +2982,10 @@
         </is>
       </c>
       <c r="AA25" t="n">
-        <v>0.1162815116119427</v>
+        <v>0.1256330300075835</v>
       </c>
       <c r="AB25" t="n">
-        <v>9.315277764646796</v>
+        <v>6.653769831890569</v>
       </c>
       <c r="AC25" t="n">
         <v>0.1046588725540835</v>
@@ -3007,7 +3027,7 @@
         </is>
       </c>
       <c r="I26" t="n">
-        <v>7.5</v>
+        <v>8.5</v>
       </c>
       <c r="J26" t="n">
         <v>5</v>
@@ -3016,16 +3036,16 @@
         <v>1.36</v>
       </c>
       <c r="L26" t="n">
-        <v>0.1247706422018349</v>
+        <v>0.111731843575419</v>
       </c>
       <c r="M26" t="n">
-        <v>0.1871559633027523</v>
+        <v>0.1899441340782123</v>
       </c>
       <c r="N26" t="n">
-        <v>0.6880733944954128</v>
+        <v>0.6983240223463688</v>
       </c>
       <c r="O26" t="n">
-        <v>0.06862745098039214</v>
+        <v>0.05294117647058805</v>
       </c>
       <c r="P26" t="n">
         <v>2</v>
@@ -3066,7 +3086,7 @@
         <v>-0.8164620768923989</v>
       </c>
       <c r="AB26" t="n">
-        <v>4.952217523975561</v>
+        <v>2.545450161703948</v>
       </c>
       <c r="AC26" t="n">
         <v>0.1774672067631947</v>
@@ -3167,7 +3187,7 @@
         <v>0.1697650924292819</v>
       </c>
       <c r="AB27" t="n">
-        <v>11.14547261883452</v>
+        <v>7.961051870596086</v>
       </c>
       <c r="AC27" t="n">
         <v>0.1892974227324384</v>
@@ -3176,7 +3196,7 @@
     <row r="28">
       <c r="A28" s="1" t="inlineStr">
         <is>
-          <t>6VQM0QWA</t>
+          <t>nBu60dLU</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
@@ -3184,12 +3204,12 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>udinese</t>
+          <t>monza</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>verona</t>
+          <t>parma</t>
         </is>
       </c>
       <c r="E28" t="n">
@@ -3209,55 +3229,51 @@
         </is>
       </c>
       <c r="I28" t="n">
-        <v>1.8</v>
+        <v>3.1</v>
       </c>
       <c r="J28" t="n">
-        <v>3.5</v>
+        <v>3</v>
       </c>
       <c r="K28" t="n">
-        <v>4.75</v>
+        <v>2.45</v>
       </c>
       <c r="L28" t="n">
-        <v>0.5281969817315331</v>
+        <v>0.303155289750464</v>
       </c>
       <c r="M28" t="n">
-        <v>0.2716441620333598</v>
+        <v>0.3132604660754795</v>
       </c>
       <c r="N28" t="n">
-        <v>0.2001588562351072</v>
+        <v>0.3835842441740565</v>
       </c>
       <c r="O28" t="n">
-        <v>0.05179615705931484</v>
+        <v>0.06407724380074598</v>
       </c>
       <c r="P28" t="n">
         <v>1</v>
       </c>
       <c r="Q28" t="n">
-        <v>0.301111571970371</v>
+        <v>0.1035450147498123</v>
       </c>
       <c r="R28" t="n">
-        <v>0.6340129587479735</v>
+        <v>0.4729387563576554</v>
       </c>
       <c r="S28" t="n">
-        <v>0.0648754692816555</v>
+        <v>0.4235162288925323</v>
       </c>
       <c r="T28" t="n">
         <v>1</v>
       </c>
-      <c r="U28" t="n">
-        <v>1</v>
-      </c>
-      <c r="V28" t="n">
-        <v>0</v>
-      </c>
+      <c r="U28" t="inlineStr"/>
+      <c r="V28" t="inlineStr"/>
       <c r="W28" t="n">
         <v>1</v>
       </c>
       <c r="X28" t="n">
-        <v>0.6340129587479735</v>
+        <v>0.4729387563576554</v>
       </c>
       <c r="Y28" t="n">
-        <v>1.8</v>
+        <v>3.1</v>
       </c>
       <c r="Z28" t="inlineStr">
         <is>
@@ -3265,32 +3281,32 @@
         </is>
       </c>
       <c r="AA28" t="n">
-        <v>0.1765291571829404</v>
+        <v>0.2219572117660627</v>
       </c>
       <c r="AB28" t="n">
-        <v>4.438090711235814</v>
+        <v>7.09408134536483</v>
       </c>
       <c r="AC28" t="n">
-        <v>0.3329013867776025</v>
+        <v>0.04942252746512305</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="1" t="inlineStr">
         <is>
-          <t>voxb2IjI</t>
+          <t>6VQM0QWA</t>
         </is>
       </c>
       <c r="B29" s="2" t="n">
-        <v>45731.58333333334</v>
+        <v>45731.45833333334</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>ac milan</t>
+          <t>udinese</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>como</t>
+          <t>verona</t>
         </is>
       </c>
       <c r="E29" t="n">
@@ -3310,37 +3326,37 @@
         </is>
       </c>
       <c r="I29" t="n">
-        <v>1.8</v>
+        <v>1.73</v>
       </c>
       <c r="J29" t="n">
-        <v>3.6</v>
+        <v>3.5</v>
       </c>
       <c r="K29" t="n">
-        <v>4.33</v>
+        <v>5</v>
       </c>
       <c r="L29" t="n">
-        <v>0.5220012055455093</v>
+        <v>0.5433938829374321</v>
       </c>
       <c r="M29" t="n">
-        <v>0.2610006027727547</v>
+        <v>0.2685918335662164</v>
       </c>
       <c r="N29" t="n">
-        <v>0.216998191681736</v>
+        <v>0.1880142834963515</v>
       </c>
       <c r="O29" t="n">
-        <v>0.0642802155504234</v>
+        <v>0.06374896779521055</v>
       </c>
       <c r="P29" t="n">
         <v>1</v>
       </c>
       <c r="Q29" t="n">
-        <v>0.314160208802293</v>
+        <v>0.3699671422892812</v>
       </c>
       <c r="R29" t="n">
-        <v>0.6134281217498372</v>
+        <v>0.556180457262347</v>
       </c>
       <c r="S29" t="n">
-        <v>0.07241166944786993</v>
+        <v>0.07385240044837173</v>
       </c>
       <c r="T29" t="n">
         <v>1</v>
@@ -3351,10 +3367,10 @@
         <v>1</v>
       </c>
       <c r="X29" t="n">
-        <v>0.6134281217498372</v>
+        <v>0.556180457262347</v>
       </c>
       <c r="Y29" t="n">
-        <v>1.8</v>
+        <v>1.73</v>
       </c>
       <c r="Z29" t="inlineStr">
         <is>
@@ -3362,32 +3378,32 @@
         </is>
       </c>
       <c r="AA29" t="n">
-        <v>0.1302132739371337</v>
+        <v>-0.05179151909060236</v>
       </c>
       <c r="AB29" t="n">
-        <v>4.29399685224886</v>
+        <v>7.911011316204345</v>
       </c>
       <c r="AC29" t="n">
-        <v>0.2992679129475442</v>
+        <v>0.1862133149730658</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="1" t="inlineStr">
         <is>
-          <t>0IeM2n2b</t>
+          <t>voxb2IjI</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
-        <v>45731.69791666666</v>
+        <v>45731.58333333334</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>torino</t>
+          <t>ac milan</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>empoli</t>
+          <t>como</t>
         </is>
       </c>
       <c r="E30" t="n">
@@ -3410,49 +3426,45 @@
         <v>1.8</v>
       </c>
       <c r="J30" t="n">
-        <v>3.2</v>
+        <v>3.6</v>
       </c>
       <c r="K30" t="n">
-        <v>5</v>
+        <v>4.5</v>
       </c>
       <c r="L30" t="n">
-        <v>0.5201560468140443</v>
+        <v>0.5263157894736842</v>
       </c>
       <c r="M30" t="n">
-        <v>0.2925877763328999</v>
+        <v>0.2631578947368421</v>
       </c>
       <c r="N30" t="n">
-        <v>0.1872561768530559</v>
+        <v>0.2105263157894737</v>
       </c>
       <c r="O30" t="n">
-        <v>0.06805555555555554</v>
+        <v>0.05555555555555558</v>
       </c>
       <c r="P30" t="n">
         <v>1</v>
       </c>
       <c r="Q30" t="n">
-        <v>0.3491448275110267</v>
+        <v>0.2891631517166968</v>
       </c>
       <c r="R30" t="n">
-        <v>0.577922651881169</v>
+        <v>0.5562367657474598</v>
       </c>
       <c r="S30" t="n">
-        <v>0.07293252060780452</v>
+        <v>0.1546000825358435</v>
       </c>
       <c r="T30" t="n">
         <v>1</v>
       </c>
-      <c r="U30" t="n">
-        <v>1</v>
-      </c>
-      <c r="V30" t="n">
-        <v>0</v>
-      </c>
+      <c r="U30" t="inlineStr"/>
+      <c r="V30" t="inlineStr"/>
       <c r="W30" t="n">
         <v>1</v>
       </c>
       <c r="X30" t="n">
-        <v>0.577922651881169</v>
+        <v>0.5562367657474598</v>
       </c>
       <c r="Y30" t="n">
         <v>1.8</v>
@@ -3463,32 +3475,32 @@
         </is>
       </c>
       <c r="AA30" t="n">
-        <v>0.05032596673263022</v>
+        <v>0.001532722931784636</v>
       </c>
       <c r="AB30" t="n">
-        <v>4.045458563168183</v>
+        <v>8.343551486211897</v>
       </c>
       <c r="AC30" t="n">
-        <v>0.2287778243701423</v>
+        <v>0.2670736140307631</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="1" t="inlineStr">
         <is>
-          <t>S4cE48Xo</t>
+          <t>CYps60ig</t>
         </is>
       </c>
       <c r="B31" s="2" t="n">
-        <v>45732.5</v>
+        <v>45732.58333333334</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>as roma</t>
+          <t>fiorentina</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>cagliari</t>
+          <t>juventus</t>
         </is>
       </c>
       <c r="E31" t="n">
@@ -3508,37 +3520,37 @@
         </is>
       </c>
       <c r="I31" t="n">
-        <v>1.57</v>
+        <v>3.4</v>
       </c>
       <c r="J31" t="n">
-        <v>4.2</v>
+        <v>3.2</v>
       </c>
       <c r="K31" t="n">
-        <v>5.5</v>
+        <v>2.25</v>
       </c>
       <c r="L31" t="n">
-        <v>0.6026768243366641</v>
+        <v>0.2798289933929266</v>
       </c>
       <c r="M31" t="n">
-        <v>0.2252863367163244</v>
+        <v>0.2973183054799844</v>
       </c>
       <c r="N31" t="n">
-        <v>0.1720368389470114</v>
+        <v>0.4228527011270889</v>
       </c>
       <c r="O31" t="n">
-        <v>0.05685609507265554</v>
+        <v>0.05106209150326801</v>
       </c>
       <c r="P31" t="n">
         <v>1</v>
       </c>
       <c r="Q31" t="n">
-        <v>0.3647352483533942</v>
+        <v>0.2532324986954283</v>
       </c>
       <c r="R31" t="n">
-        <v>0.606766940296952</v>
+        <v>0.4098687406457967</v>
       </c>
       <c r="S31" t="n">
-        <v>0.02849781134965387</v>
+        <v>0.3368987606587751</v>
       </c>
       <c r="T31" t="n">
         <v>1</v>
@@ -3549,10 +3561,10 @@
         <v>1</v>
       </c>
       <c r="X31" t="n">
-        <v>0.606766940296952</v>
+        <v>0.4098687406457967</v>
       </c>
       <c r="Y31" t="n">
-        <v>1.57</v>
+        <v>3.4</v>
       </c>
       <c r="Z31" t="inlineStr">
         <is>
@@ -3560,32 +3572,32 @@
         </is>
       </c>
       <c r="AA31" t="n">
-        <v>-0.08311562058558825</v>
+        <v>0.1639807159148786</v>
       </c>
       <c r="AB31" t="n">
-        <v>3.982943992897853</v>
+        <v>6.148031109686951</v>
       </c>
       <c r="AC31" t="n">
-        <v>0.2420316919435578</v>
+        <v>0.07296997998702159</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="1" t="inlineStr">
         <is>
-          <t>IVmk4vM5</t>
+          <t>0fHOmJyP</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
-        <v>45730.69791666666</v>
+        <v>45732.69791666666</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>genoa</t>
+          <t>atalanta</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>lecce</t>
+          <t>inter</t>
         </is>
       </c>
       <c r="E32" t="n">
@@ -3605,37 +3617,37 @@
         </is>
       </c>
       <c r="I32" t="n">
-        <v>2.05</v>
+        <v>2.55</v>
       </c>
       <c r="J32" t="n">
-        <v>2.9</v>
+        <v>3.3</v>
       </c>
       <c r="K32" t="n">
-        <v>4.5</v>
+        <v>2.8</v>
       </c>
       <c r="L32" t="n">
-        <v>0.4624379872430901</v>
+        <v>0.3726557773744706</v>
       </c>
       <c r="M32" t="n">
-        <v>0.3268958185683913</v>
+        <v>0.2879612825166364</v>
       </c>
       <c r="N32" t="n">
-        <v>0.2106661941885188</v>
+        <v>0.3393829401088929</v>
       </c>
       <c r="O32" t="n">
-        <v>0.05485468647789915</v>
+        <v>0.05233002291825839</v>
       </c>
       <c r="P32" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q32" t="n">
-        <v>0.4729976683176806</v>
+        <v>0.2406013581651952</v>
       </c>
       <c r="R32" t="n">
-        <v>0.4336338722563537</v>
+        <v>0.5148666709604525</v>
       </c>
       <c r="S32" t="n">
-        <v>0.09336845942596554</v>
+        <v>0.2445319708743524</v>
       </c>
       <c r="T32" t="n">
         <v>1</v>
@@ -3647,13 +3659,13 @@
         <v>0</v>
       </c>
       <c r="W32" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X32" t="n">
-        <v>0.4729976683176806</v>
+        <v>0.5148666709604525</v>
       </c>
       <c r="Y32" t="n">
-        <v>2.9</v>
+        <v>2.55</v>
       </c>
       <c r="Z32" t="inlineStr">
         <is>
@@ -3661,32 +3673,32 @@
         </is>
       </c>
       <c r="AA32" t="n">
-        <v>0.1956280200638283</v>
+        <v>0.2018774264188089</v>
       </c>
       <c r="AB32" t="n">
-        <v>6.621967356447529</v>
+        <v>7.723000064406787</v>
       </c>
       <c r="AC32" t="n">
-        <v>0.03936379606132689</v>
+        <v>0.2703347000861001</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="1" t="inlineStr">
         <is>
-          <t>G6iY7MMt</t>
+          <t>IVmk4vM5</t>
         </is>
       </c>
       <c r="B33" s="2" t="n">
-        <v>45732.45833333334</v>
+        <v>45730.69791666666</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>bologna</t>
+          <t>genoa</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>lazio</t>
+          <t>lecce</t>
         </is>
       </c>
       <c r="E33" t="n">
@@ -3706,51 +3718,55 @@
         </is>
       </c>
       <c r="I33" t="n">
-        <v>2.3</v>
+        <v>2.05</v>
       </c>
       <c r="J33" t="n">
-        <v>3.1</v>
+        <v>2.9</v>
       </c>
       <c r="K33" t="n">
-        <v>3.3</v>
+        <v>4.5</v>
       </c>
       <c r="L33" t="n">
-        <v>0.4100200400801604</v>
+        <v>0.4624379872430901</v>
       </c>
       <c r="M33" t="n">
-        <v>0.3042084168336673</v>
+        <v>0.3268958185683913</v>
       </c>
       <c r="N33" t="n">
-        <v>0.2857715430861724</v>
+        <v>0.2106661941885188</v>
       </c>
       <c r="O33" t="n">
-        <v>0.06039355688724557</v>
+        <v>0.05485468647789915</v>
       </c>
       <c r="P33" t="n">
         <v>0</v>
       </c>
       <c r="Q33" t="n">
-        <v>0.4436385729161679</v>
+        <v>0.6614556258167381</v>
       </c>
       <c r="R33" t="n">
-        <v>0.2107995768712494</v>
+        <v>0.1394727746837952</v>
       </c>
       <c r="S33" t="n">
-        <v>0.3455618502125827</v>
+        <v>0.1990715994994667</v>
       </c>
       <c r="T33" t="n">
         <v>1</v>
       </c>
-      <c r="U33" t="inlineStr"/>
-      <c r="V33" t="inlineStr"/>
+      <c r="U33" t="n">
+        <v>1</v>
+      </c>
+      <c r="V33" t="n">
+        <v>0</v>
+      </c>
       <c r="W33" t="n">
         <v>0</v>
       </c>
       <c r="X33" t="n">
-        <v>0.4436385729161679</v>
+        <v>0.6614556258167381</v>
       </c>
       <c r="Y33" t="n">
-        <v>3.1</v>
+        <v>2.9</v>
       </c>
       <c r="Z33" t="inlineStr">
         <is>
@@ -3758,32 +3774,32 @@
         </is>
       </c>
       <c r="AA33" t="n">
-        <v>0.1787045600191051</v>
+        <v>0.4832743762466003</v>
       </c>
       <c r="AB33" t="n">
-        <v>6.21094002082635</v>
+        <v>6.614556258167381</v>
       </c>
       <c r="AC33" t="n">
-        <v>0.0980767227035852</v>
+        <v>0.4623840263172714</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="1" t="inlineStr">
         <is>
-          <t>0fHOmJyP</t>
+          <t>0IeM2n2b</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
-        <v>45732.69791666666</v>
+        <v>45731.69791666666</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>atalanta</t>
+          <t>torino</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>inter</t>
+          <t>empoli</t>
         </is>
       </c>
       <c r="E34" t="n">
@@ -3803,55 +3819,51 @@
         </is>
       </c>
       <c r="I34" t="n">
-        <v>2.55</v>
+        <v>1.8</v>
       </c>
       <c r="J34" t="n">
-        <v>3.5</v>
+        <v>3.3</v>
       </c>
       <c r="K34" t="n">
-        <v>2.63</v>
+        <v>5</v>
       </c>
       <c r="L34" t="n">
-        <v>0.3706238801763534</v>
+        <v>0.5248091603053435</v>
       </c>
       <c r="M34" t="n">
-        <v>0.2700259698427717</v>
+        <v>0.2862595419847329</v>
       </c>
       <c r="N34" t="n">
-        <v>0.3593501499808749</v>
+        <v>0.1889312977099237</v>
       </c>
       <c r="O34" t="n">
-        <v>0.05809928534151299</v>
+        <v>0.05858585858585852</v>
       </c>
       <c r="P34" t="n">
         <v>0</v>
       </c>
       <c r="Q34" t="n">
-        <v>0.429456815035675</v>
+        <v>0.7106253049137264</v>
       </c>
       <c r="R34" t="n">
-        <v>0.3714772468898676</v>
+        <v>0.2027533659066978</v>
       </c>
       <c r="S34" t="n">
-        <v>0.1990659380744574</v>
+        <v>0.08662132917957568</v>
       </c>
       <c r="T34" t="n">
         <v>1</v>
       </c>
-      <c r="U34" t="n">
-        <v>1</v>
-      </c>
-      <c r="V34" t="n">
-        <v>0</v>
-      </c>
+      <c r="U34" t="inlineStr"/>
+      <c r="V34" t="inlineStr"/>
       <c r="W34" t="n">
         <v>0</v>
       </c>
       <c r="X34" t="n">
-        <v>0.429456815035675</v>
+        <v>0.7106253049137264</v>
       </c>
       <c r="Y34" t="n">
-        <v>3.5</v>
+        <v>3.3</v>
       </c>
       <c r="Z34" t="inlineStr">
         <is>
@@ -3859,32 +3871,32 @@
         </is>
       </c>
       <c r="AA34" t="n">
-        <v>0.2012395410499449</v>
+        <v>0.5848102200936074</v>
       </c>
       <c r="AB34" t="n">
-        <v>6.012395410499448</v>
+        <v>7.106253049137265</v>
       </c>
       <c r="AC34" t="n">
-        <v>0.05797956814580735</v>
+        <v>0.5078719390070286</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="1" t="inlineStr">
         <is>
-          <t>nBu60dLU</t>
+          <t>S4cE48Xo</t>
         </is>
       </c>
       <c r="B35" s="2" t="n">
-        <v>45731.45833333334</v>
+        <v>45732.5</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>monza</t>
+          <t>as roma</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>parma</t>
+          <t>cagliari</t>
         </is>
       </c>
       <c r="E35" t="n">
@@ -3904,55 +3916,51 @@
         </is>
       </c>
       <c r="I35" t="n">
-        <v>3</v>
+        <v>1.53</v>
       </c>
       <c r="J35" t="n">
-        <v>3</v>
+        <v>4.2</v>
       </c>
       <c r="K35" t="n">
-        <v>2.55</v>
+        <v>6</v>
       </c>
       <c r="L35" t="n">
-        <v>0.3148148148148148</v>
+        <v>0.6175562417291575</v>
       </c>
       <c r="M35" t="n">
-        <v>0.3148148148148148</v>
+        <v>0.2249669166299073</v>
       </c>
       <c r="N35" t="n">
-        <v>0.3703703703703704</v>
+        <v>0.1574768416409351</v>
       </c>
       <c r="O35" t="n">
-        <v>0.05882352941176472</v>
+        <v>0.05835667600373484</v>
       </c>
       <c r="P35" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="Q35" t="n">
-        <v>0.3177127885493949</v>
+        <v>0.4746091355359102</v>
       </c>
       <c r="R35" t="n">
-        <v>0.2695631373570447</v>
+        <v>0.4535711787054781</v>
       </c>
       <c r="S35" t="n">
-        <v>0.4127240740935605</v>
+        <v>0.0718196857586115</v>
       </c>
       <c r="T35" t="n">
         <v>1</v>
       </c>
-      <c r="U35" t="n">
-        <v>1</v>
-      </c>
-      <c r="V35" t="n">
-        <v>0</v>
-      </c>
+      <c r="U35" t="inlineStr"/>
+      <c r="V35" t="inlineStr"/>
       <c r="W35" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="X35" t="n">
-        <v>0.4127240740935605</v>
+        <v>0.4746091355359102</v>
       </c>
       <c r="Y35" t="n">
-        <v>2.55</v>
+        <v>4.2</v>
       </c>
       <c r="Z35" t="inlineStr">
         <is>
@@ -3960,13 +3968,13 @@
         </is>
       </c>
       <c r="AA35" t="n">
-        <v>0.0338363799603737</v>
+        <v>0.3104244903908822</v>
       </c>
       <c r="AB35" t="n">
-        <v>2.889068518654924</v>
+        <v>4.746091355359102</v>
       </c>
       <c r="AC35" t="n">
-        <v>0.09501128554416566</v>
+        <v>0.02103795683043208</v>
       </c>
     </row>
     <row r="36">
@@ -4005,37 +4013,37 @@
         </is>
       </c>
       <c r="I36" t="n">
-        <v>6.25</v>
+        <v>5.75</v>
       </c>
       <c r="J36" t="n">
         <v>4.33</v>
       </c>
       <c r="K36" t="n">
-        <v>1.5</v>
+        <v>1.53</v>
       </c>
       <c r="L36" t="n">
-        <v>0.1512839923135154</v>
+        <v>0.1643084432253056</v>
       </c>
       <c r="M36" t="n">
-        <v>0.2183660397135038</v>
+        <v>0.2181925054377615</v>
       </c>
       <c r="N36" t="n">
-        <v>0.6303499679729809</v>
+        <v>0.6174990513369328</v>
       </c>
       <c r="O36" t="n">
-        <v>0.05761354888375658</v>
+        <v>0.05845469693718108</v>
       </c>
       <c r="P36" t="n">
         <v>2</v>
       </c>
       <c r="Q36" t="n">
-        <v>0.3174215301153699</v>
+        <v>0.2467260532398944</v>
       </c>
       <c r="R36" t="n">
-        <v>0.09411036884886266</v>
+        <v>0.1123909277918655</v>
       </c>
       <c r="S36" t="n">
-        <v>0.5884681010357674</v>
+        <v>0.6408830189682402</v>
       </c>
       <c r="T36" t="n">
         <v>1</v>
@@ -4050,10 +4058,10 @@
         <v>2</v>
       </c>
       <c r="X36" t="n">
-        <v>0.5884681010357674</v>
+        <v>0.6408830189682402</v>
       </c>
       <c r="Y36" t="n">
-        <v>1.5</v>
+        <v>1.53</v>
       </c>
       <c r="Z36" t="inlineStr">
         <is>
@@ -4061,32 +4069,32 @@
         </is>
       </c>
       <c r="AA36" t="n">
-        <v>-0.2345956968926978</v>
+        <v>-0.0366961905256462</v>
       </c>
       <c r="AB36" t="n">
-        <v>3.401890800787216</v>
+        <v>6.173756044286679</v>
       </c>
       <c r="AC36" t="n">
-        <v>0.2710465709203975</v>
+        <v>0.3941569657283458</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="1" t="inlineStr">
         <is>
-          <t>CYps60ig</t>
+          <t>G6iY7MMt</t>
         </is>
       </c>
       <c r="B37" s="2" t="n">
-        <v>45732.58333333334</v>
+        <v>45732.45833333334</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>fiorentina</t>
+          <t>bologna</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>juventus</t>
+          <t>lazio</t>
         </is>
       </c>
       <c r="E37" t="n">
@@ -4106,55 +4114,51 @@
         </is>
       </c>
       <c r="I37" t="n">
-        <v>3.25</v>
+        <v>2.3</v>
       </c>
       <c r="J37" t="n">
-        <v>3.3</v>
+        <v>3.1</v>
       </c>
       <c r="K37" t="n">
-        <v>2.2</v>
+        <v>3.4</v>
       </c>
       <c r="L37" t="n">
-        <v>0.2888402625820569</v>
+        <v>0.413495488426834</v>
       </c>
       <c r="M37" t="n">
-        <v>0.2844638949671772</v>
+        <v>0.3067869752844252</v>
       </c>
       <c r="N37" t="n">
-        <v>0.4266958424507659</v>
+        <v>0.2797175362887406</v>
       </c>
       <c r="O37" t="n">
-        <v>0.06526806526806528</v>
+        <v>0.05148090091576618</v>
       </c>
       <c r="P37" t="n">
         <v>2</v>
       </c>
       <c r="Q37" t="n">
-        <v>0.3280468890685433</v>
+        <v>0.3260635955815022</v>
       </c>
       <c r="R37" t="n">
-        <v>0.1980846455266942</v>
+        <v>0.2833968875176439</v>
       </c>
       <c r="S37" t="n">
-        <v>0.4738684654047624</v>
+        <v>0.3905395169008538</v>
       </c>
       <c r="T37" t="n">
         <v>1</v>
       </c>
-      <c r="U37" t="n">
-        <v>1</v>
-      </c>
-      <c r="V37" t="n">
-        <v>0</v>
-      </c>
+      <c r="U37" t="inlineStr"/>
+      <c r="V37" t="inlineStr"/>
       <c r="W37" t="n">
         <v>2</v>
       </c>
       <c r="X37" t="n">
-        <v>0.4738684654047624</v>
+        <v>0.3905395169008538</v>
       </c>
       <c r="Y37" t="n">
-        <v>2.2</v>
+        <v>3.4</v>
       </c>
       <c r="Z37" t="inlineStr">
         <is>
@@ -4162,32 +4166,32 @@
         </is>
       </c>
       <c r="AA37" t="n">
-        <v>0.0354255199087312</v>
+        <v>0.1365976489428761</v>
       </c>
       <c r="AB37" t="n">
-        <v>3.317079257833337</v>
+        <v>3.905395169008537</v>
       </c>
       <c r="AC37" t="n">
-        <v>0.1458215763362191</v>
+        <v>0.06447592131935154</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="1" t="inlineStr">
         <is>
-          <t>2FJLJdV9</t>
+          <t>MH5y3WcE</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
-        <v>45731.51041666666</v>
+        <v>45730.70833333334</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>mallorca</t>
+          <t>las palmas</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>espanyol</t>
+          <t>alaves</t>
         </is>
       </c>
       <c r="E38" t="n">
@@ -4207,42 +4211,44 @@
         </is>
       </c>
       <c r="I38" t="n">
-        <v>1.8</v>
+        <v>3</v>
       </c>
       <c r="J38" t="n">
-        <v>3.3</v>
+        <v>3.1</v>
       </c>
       <c r="K38" t="n">
-        <v>5</v>
+        <v>2.5</v>
       </c>
       <c r="L38" t="n">
-        <v>0.5248091603053435</v>
+        <v>0.3156822810590631</v>
       </c>
       <c r="M38" t="n">
-        <v>0.2862595419847329</v>
+        <v>0.3054989816700611</v>
       </c>
       <c r="N38" t="n">
-        <v>0.1889312977099237</v>
+        <v>0.3788187372708758</v>
       </c>
       <c r="O38" t="n">
-        <v>0.05858585858585852</v>
+        <v>0.05591397849462365</v>
       </c>
       <c r="P38" t="n">
         <v>1</v>
       </c>
       <c r="Q38" t="n">
-        <v>0.3752511765064035</v>
+        <v>0.2655474608194406</v>
       </c>
       <c r="R38" t="n">
-        <v>0.4643650265337161</v>
+        <v>0.4144767249509805</v>
       </c>
       <c r="S38" t="n">
-        <v>0.1603837969598803</v>
+        <v>0.3199758142295789</v>
       </c>
       <c r="T38" t="n">
         <v>1</v>
       </c>
-      <c r="U38" t="inlineStr"/>
+      <c r="U38" t="n">
+        <v>0</v>
+      </c>
       <c r="V38" t="n">
         <v>0</v>
       </c>
@@ -4250,10 +4256,10 @@
         <v>1</v>
       </c>
       <c r="X38" t="n">
-        <v>0.4643650265337161</v>
+        <v>0.4144767249509805</v>
       </c>
       <c r="Y38" t="n">
-        <v>1.8</v>
+        <v>3</v>
       </c>
       <c r="Z38" t="inlineStr">
         <is>
@@ -4261,32 +4267,32 @@
         </is>
       </c>
       <c r="AA38" t="n">
-        <v>-0.2051786902991386</v>
+        <v>0.1217150874264707</v>
       </c>
       <c r="AB38" t="n">
-        <v>4.131387015772588</v>
+        <v>6.217150874264707</v>
       </c>
       <c r="AC38" t="n">
-        <v>0.08911385002731265</v>
+        <v>0.0945009107214016</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="1" t="inlineStr">
         <is>
-          <t>6BzIrse2</t>
+          <t>2FJLJdV9</t>
         </is>
       </c>
       <c r="B39" s="2" t="n">
-        <v>45732.60416666666</v>
+        <v>45731.51041666666</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>rayo vallecano</t>
+          <t>mallorca</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>real sociedad</t>
+          <t>espanyol</t>
         </is>
       </c>
       <c r="E39" t="n">
@@ -4306,42 +4312,44 @@
         </is>
       </c>
       <c r="I39" t="n">
-        <v>2.6</v>
+        <v>1.8</v>
       </c>
       <c r="J39" t="n">
-        <v>3</v>
+        <v>3.3</v>
       </c>
       <c r="K39" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L39" t="n">
-        <v>0.3658536585365854</v>
+        <v>0.5248091603053435</v>
       </c>
       <c r="M39" t="n">
-        <v>0.3170731707317074</v>
+        <v>0.2862595419847329</v>
       </c>
       <c r="N39" t="n">
-        <v>0.3170731707317074</v>
+        <v>0.1889312977099237</v>
       </c>
       <c r="O39" t="n">
-        <v>0.0512820512820511</v>
+        <v>0.05858585858585852</v>
       </c>
       <c r="P39" t="n">
         <v>1</v>
       </c>
       <c r="Q39" t="n">
-        <v>0.3205217897764424</v>
+        <v>0.06410954081048939</v>
       </c>
       <c r="R39" t="n">
-        <v>0.5120408796450534</v>
+        <v>0.5419457153633681</v>
       </c>
       <c r="S39" t="n">
-        <v>0.1674373305785044</v>
+        <v>0.3939447438261424</v>
       </c>
       <c r="T39" t="n">
         <v>1</v>
       </c>
-      <c r="U39" t="inlineStr"/>
+      <c r="U39" t="n">
+        <v>0</v>
+      </c>
       <c r="V39" t="n">
         <v>0</v>
       </c>
@@ -4349,10 +4357,10 @@
         <v>1</v>
       </c>
       <c r="X39" t="n">
-        <v>0.5120408796450534</v>
+        <v>0.5419457153633681</v>
       </c>
       <c r="Y39" t="n">
-        <v>2.6</v>
+        <v>1.8</v>
       </c>
       <c r="Z39" t="inlineStr">
         <is>
@@ -4360,32 +4368,32 @@
         </is>
       </c>
       <c r="AA39" t="n">
-        <v>0.2070664294232118</v>
+        <v>-0.03062214043242174</v>
       </c>
       <c r="AB39" t="n">
-        <v>5.376429236273061</v>
+        <v>7.880330443701112</v>
       </c>
       <c r="AC39" t="n">
-        <v>0.191519089868611</v>
+        <v>0.1480009715372257</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="1" t="inlineStr">
         <is>
-          <t>GppsqB6r</t>
+          <t>lz02jgE8</t>
         </is>
       </c>
       <c r="B40" s="2" t="n">
-        <v>45731.41666666666</v>
+        <v>45732.51041666666</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>valladolid</t>
+          <t>sevilla</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>celta vigo</t>
+          <t>ath bilbao</t>
         </is>
       </c>
       <c r="E40" t="n">
@@ -4405,53 +4413,55 @@
         </is>
       </c>
       <c r="I40" t="n">
-        <v>5</v>
+        <v>2.9</v>
       </c>
       <c r="J40" t="n">
-        <v>3.75</v>
+        <v>3.2</v>
       </c>
       <c r="K40" t="n">
-        <v>1.7</v>
+        <v>2.5</v>
       </c>
       <c r="L40" t="n">
-        <v>0.1895910780669145</v>
+        <v>0.3261312678353037</v>
       </c>
       <c r="M40" t="n">
-        <v>0.2527881040892193</v>
+        <v>0.2955564614757439</v>
       </c>
       <c r="N40" t="n">
-        <v>0.5576208178438662</v>
+        <v>0.3783122706889523</v>
       </c>
       <c r="O40" t="n">
-        <v>0.05490196078431375</v>
+        <v>0.05732758620689671</v>
       </c>
       <c r="P40" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q40" t="n">
-        <v>0.4310033402051662</v>
+        <v>0.2742914879005598</v>
       </c>
       <c r="R40" t="n">
-        <v>0.1501830644963013</v>
+        <v>0.4027392557450454</v>
       </c>
       <c r="S40" t="n">
-        <v>0.4188135952985325</v>
+        <v>0.3229692563543948</v>
       </c>
       <c r="T40" t="n">
         <v>1</v>
       </c>
-      <c r="U40" t="inlineStr"/>
+      <c r="U40" t="n">
+        <v>0</v>
+      </c>
       <c r="V40" t="n">
         <v>0</v>
       </c>
       <c r="W40" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X40" t="n">
-        <v>0.4310033402051662</v>
+        <v>0.4027392557450454</v>
       </c>
       <c r="Y40" t="n">
-        <v>3.75</v>
+        <v>2.9</v>
       </c>
       <c r="Z40" t="inlineStr">
         <is>
@@ -4459,32 +4469,32 @@
         </is>
       </c>
       <c r="AA40" t="n">
-        <v>0.2240954639161357</v>
+        <v>0.08839149561085879</v>
       </c>
       <c r="AB40" t="n">
-        <v>7.542558453590408</v>
+        <v>6.041088836175682</v>
       </c>
       <c r="AC40" t="n">
-        <v>0.01218974490663366</v>
+        <v>0.0797699993906506</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="1" t="inlineStr">
         <is>
-          <t>fBDkuT57</t>
+          <t>lbrkskye</t>
         </is>
       </c>
       <c r="B41" s="2" t="n">
-        <v>45731.60416666666</v>
+        <v>45732.60416666666</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>villarreal</t>
+          <t>osasuna</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>real madrid</t>
+          <t>getafe</t>
         </is>
       </c>
       <c r="E41" t="n">
@@ -4504,53 +4514,55 @@
         </is>
       </c>
       <c r="I41" t="n">
-        <v>3.4</v>
+        <v>2.25</v>
       </c>
       <c r="J41" t="n">
-        <v>3.7</v>
+        <v>2.88</v>
       </c>
       <c r="K41" t="n">
-        <v>2</v>
+        <v>3.8</v>
       </c>
       <c r="L41" t="n">
-        <v>0.2763256161314414</v>
+        <v>0.4213444213444213</v>
       </c>
       <c r="M41" t="n">
-        <v>0.2539208364451083</v>
+        <v>0.3291753291753292</v>
       </c>
       <c r="N41" t="n">
-        <v>0.4697535474234503</v>
+        <v>0.2494802494802495</v>
       </c>
       <c r="O41" t="n">
-        <v>0.06438791732909377</v>
+        <v>0.05482456140350878</v>
       </c>
       <c r="P41" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q41" t="n">
-        <v>0.4486650993731827</v>
+        <v>0.1393064091929172</v>
       </c>
       <c r="R41" t="n">
-        <v>0.18134740625014</v>
+        <v>0.4639527036901374</v>
       </c>
       <c r="S41" t="n">
-        <v>0.3699874943766774</v>
+        <v>0.3967408871169454</v>
       </c>
       <c r="T41" t="n">
         <v>1</v>
       </c>
-      <c r="U41" t="inlineStr"/>
+      <c r="U41" t="n">
+        <v>0</v>
+      </c>
       <c r="V41" t="n">
         <v>0</v>
       </c>
       <c r="W41" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X41" t="n">
-        <v>0.4486650993731827</v>
+        <v>0.4639527036901374</v>
       </c>
       <c r="Y41" t="n">
-        <v>3.7</v>
+        <v>2.25</v>
       </c>
       <c r="Z41" t="inlineStr">
         <is>
@@ -4558,32 +4570,32 @@
         </is>
       </c>
       <c r="AA41" t="n">
-        <v>0.244466988029917</v>
+        <v>0.0351148666422473</v>
       </c>
       <c r="AB41" t="n">
-        <v>7.851639239030697</v>
+        <v>6.959290555352061</v>
       </c>
       <c r="AC41" t="n">
-        <v>0.07867760499650528</v>
+        <v>0.06721181657319203</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="1" t="inlineStr">
         <is>
-          <t>0EX9p3Qk</t>
+          <t>6BzIrse2</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
-        <v>45731.70833333334</v>
+        <v>45732.60416666666</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>girona</t>
+          <t>rayo vallecano</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>valencia</t>
+          <t>real sociedad</t>
         </is>
       </c>
       <c r="E42" t="n">
@@ -4603,53 +4615,55 @@
         </is>
       </c>
       <c r="I42" t="n">
-        <v>1.95</v>
+        <v>2.5</v>
       </c>
       <c r="J42" t="n">
-        <v>3.4</v>
+        <v>3</v>
       </c>
       <c r="K42" t="n">
-        <v>3.8</v>
+        <v>3.1</v>
       </c>
       <c r="L42" t="n">
-        <v>0.4792284866468843</v>
+        <v>0.3788187372708758</v>
       </c>
       <c r="M42" t="n">
-        <v>0.2748516320474778</v>
+        <v>0.3156822810590631</v>
       </c>
       <c r="N42" t="n">
-        <v>0.245919881305638</v>
+        <v>0.3054989816700611</v>
       </c>
       <c r="O42" t="n">
-        <v>0.0700960546161784</v>
+        <v>0.05591397849462365</v>
       </c>
       <c r="P42" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q42" t="n">
-        <v>0.3550037211677838</v>
+        <v>0.1784299249024006</v>
       </c>
       <c r="R42" t="n">
-        <v>0.3546354326490165</v>
+        <v>0.4863827909499324</v>
       </c>
       <c r="S42" t="n">
-        <v>0.2903608461831997</v>
+        <v>0.335187284147667</v>
       </c>
       <c r="T42" t="n">
         <v>1</v>
       </c>
-      <c r="U42" t="inlineStr"/>
+      <c r="U42" t="n">
+        <v>0</v>
+      </c>
       <c r="V42" t="n">
         <v>0</v>
       </c>
       <c r="W42" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X42" t="n">
-        <v>0.3550037211677838</v>
+        <v>0.4863827909499324</v>
       </c>
       <c r="Y42" t="n">
-        <v>3.4</v>
+        <v>2.5</v>
       </c>
       <c r="Z42" t="inlineStr">
         <is>
@@ -4657,32 +4671,32 @@
         </is>
       </c>
       <c r="AA42" t="n">
-        <v>0.08625527165436044</v>
+        <v>0.1439713182498873</v>
       </c>
       <c r="AB42" t="n">
-        <v>6.212565120436217</v>
+        <v>7.295741864248986</v>
       </c>
       <c r="AC42" t="n">
-        <v>0.0003682885187673013</v>
+        <v>0.1511955068022653</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="1" t="inlineStr">
         <is>
-          <t>lbrkskye</t>
+          <t>GppsqB6r</t>
         </is>
       </c>
       <c r="B43" s="2" t="n">
-        <v>45732.60416666666</v>
+        <v>45731.41666666666</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>osasuna</t>
+          <t>valladolid</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>getafe</t>
+          <t>celta vigo</t>
         </is>
       </c>
       <c r="E43" t="n">
@@ -4702,42 +4716,44 @@
         </is>
       </c>
       <c r="I43" t="n">
-        <v>2.25</v>
+        <v>5</v>
       </c>
       <c r="J43" t="n">
-        <v>2.8</v>
+        <v>3.8</v>
       </c>
       <c r="K43" t="n">
-        <v>3.7</v>
+        <v>1.67</v>
       </c>
       <c r="L43" t="n">
-        <v>0.4146487892735641</v>
+        <v>0.1883309591642925</v>
       </c>
       <c r="M43" t="n">
-        <v>0.3331999199519712</v>
+        <v>0.247803893637227</v>
       </c>
       <c r="N43" t="n">
-        <v>0.2521512907744646</v>
+        <v>0.5638651471984806</v>
       </c>
       <c r="O43" t="n">
-        <v>0.0718575718575718</v>
+        <v>0.06196028994642289</v>
       </c>
       <c r="P43" t="n">
         <v>0</v>
       </c>
       <c r="Q43" t="n">
-        <v>0.3824428931437525</v>
+        <v>0.6299576099454309</v>
       </c>
       <c r="R43" t="n">
-        <v>0.3126194927723244</v>
+        <v>0.06051569283369836</v>
       </c>
       <c r="S43" t="n">
-        <v>0.304937614083923</v>
+        <v>0.3095266972208707</v>
       </c>
       <c r="T43" t="n">
         <v>1</v>
       </c>
-      <c r="U43" t="inlineStr"/>
+      <c r="U43" t="n">
+        <v>0</v>
+      </c>
       <c r="V43" t="n">
         <v>0</v>
       </c>
@@ -4745,10 +4761,10 @@
         <v>0</v>
       </c>
       <c r="X43" t="n">
-        <v>0.3824428931437525</v>
+        <v>0.6299576099454309</v>
       </c>
       <c r="Y43" t="n">
-        <v>2.8</v>
+        <v>3.8</v>
       </c>
       <c r="Z43" t="inlineStr">
         <is>
@@ -4756,32 +4772,32 @@
         </is>
       </c>
       <c r="AA43" t="n">
-        <v>0.03935561155694828</v>
+        <v>0.4977996134973705</v>
       </c>
       <c r="AB43" t="n">
-        <v>6.692750630015668</v>
+        <v>9.449364149181465</v>
       </c>
       <c r="AC43" t="n">
-        <v>0.06982340037142815</v>
+        <v>0.3204309127245602</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="1" t="inlineStr">
         <is>
-          <t>MH5y3WcE</t>
+          <t>0EX9p3Qk</t>
         </is>
       </c>
       <c r="B44" s="2" t="n">
-        <v>45730.70833333334</v>
+        <v>45731.70833333334</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>las palmas</t>
+          <t>girona</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>alaves</t>
+          <t>valencia</t>
         </is>
       </c>
       <c r="E44" t="n">
@@ -4801,53 +4817,55 @@
         </is>
       </c>
       <c r="I44" t="n">
-        <v>2.9</v>
+        <v>1.95</v>
       </c>
       <c r="J44" t="n">
-        <v>3.1</v>
+        <v>3.5</v>
       </c>
       <c r="K44" t="n">
-        <v>2.6</v>
+        <v>3.9</v>
       </c>
       <c r="L44" t="n">
-        <v>0.3277755185034567</v>
+        <v>0.4861111111111112</v>
       </c>
       <c r="M44" t="n">
-        <v>0.3066287108580724</v>
+        <v>0.2708333333333333</v>
       </c>
       <c r="N44" t="n">
-        <v>0.3655957706384709</v>
+        <v>0.2430555555555556</v>
       </c>
       <c r="O44" t="n">
-        <v>0.05202361598357141</v>
+        <v>0.05494505494505497</v>
       </c>
       <c r="P44" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="Q44" t="n">
-        <v>0.3209011448736794</v>
+        <v>0.6153624267756741</v>
       </c>
       <c r="R44" t="n">
-        <v>0.1706919167788391</v>
+        <v>0.1146847408456869</v>
       </c>
       <c r="S44" t="n">
-        <v>0.5084069383474815</v>
+        <v>0.269952832378639</v>
       </c>
       <c r="T44" t="n">
         <v>1</v>
       </c>
-      <c r="U44" t="inlineStr"/>
+      <c r="U44" t="n">
+        <v>0</v>
+      </c>
       <c r="V44" t="n">
         <v>0</v>
       </c>
       <c r="W44" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="X44" t="n">
-        <v>0.5084069383474815</v>
+        <v>0.6153624267756741</v>
       </c>
       <c r="Y44" t="n">
-        <v>2.6</v>
+        <v>3.5</v>
       </c>
       <c r="Z44" t="inlineStr">
         <is>
@@ -4855,32 +4873,32 @@
         </is>
       </c>
       <c r="AA44" t="n">
-        <v>0.2011612748146575</v>
+        <v>0.4615073974859437</v>
       </c>
       <c r="AB44" t="n">
-        <v>0.8897121421080926</v>
+        <v>9.230436401635112</v>
       </c>
       <c r="AC44" t="n">
-        <v>0.1875057934738021</v>
+        <v>0.3454095943970351</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="1" t="inlineStr">
         <is>
-          <t>d03AlXrL</t>
+          <t>fBDkuT57</t>
         </is>
       </c>
       <c r="B45" s="2" t="n">
-        <v>45732.41666666666</v>
+        <v>45731.60416666666</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>leganes</t>
+          <t>villarreal</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>betis</t>
+          <t>real madrid</t>
         </is>
       </c>
       <c r="E45" t="n">
@@ -4900,42 +4918,44 @@
         </is>
       </c>
       <c r="I45" t="n">
-        <v>3.9</v>
+        <v>3.1</v>
       </c>
       <c r="J45" t="n">
-        <v>3.25</v>
+        <v>3.75</v>
       </c>
       <c r="K45" t="n">
-        <v>2</v>
+        <v>2.15</v>
       </c>
       <c r="L45" t="n">
-        <v>0.2409638554216868</v>
+        <v>0.3059482022578503</v>
       </c>
       <c r="M45" t="n">
-        <v>0.2891566265060241</v>
+        <v>0.2529171805331563</v>
       </c>
       <c r="N45" t="n">
-        <v>0.4698795180722892</v>
+        <v>0.4411346172089934</v>
       </c>
       <c r="O45" t="n">
-        <v>0.0641025641025641</v>
+        <v>0.05436359089772447</v>
       </c>
       <c r="P45" t="n">
         <v>2</v>
       </c>
       <c r="Q45" t="n">
-        <v>0.3385544934499816</v>
+        <v>0.4740318563340223</v>
       </c>
       <c r="R45" t="n">
-        <v>0.1509115135418081</v>
+        <v>0.0422186367089571</v>
       </c>
       <c r="S45" t="n">
-        <v>0.5105339930082103</v>
+        <v>0.4837495069570206</v>
       </c>
       <c r="T45" t="n">
         <v>1</v>
       </c>
-      <c r="U45" t="inlineStr"/>
+      <c r="U45" t="n">
+        <v>0</v>
+      </c>
       <c r="V45" t="n">
         <v>0</v>
       </c>
@@ -4943,10 +4963,10 @@
         <v>2</v>
       </c>
       <c r="X45" t="n">
-        <v>0.5105339930082103</v>
+        <v>0.4837495069570206</v>
       </c>
       <c r="Y45" t="n">
-        <v>2</v>
+        <v>2.15</v>
       </c>
       <c r="Z45" t="inlineStr">
         <is>
@@ -4954,32 +4974,32 @@
         </is>
       </c>
       <c r="AA45" t="n">
-        <v>0.02106798601642068</v>
+        <v>0.03483603474573414</v>
       </c>
       <c r="AB45" t="n">
-        <v>0.8934344877643681</v>
+        <v>0.9674990139140413</v>
       </c>
       <c r="AC45" t="n">
-        <v>0.1719794995582288</v>
+        <v>0.009717650622998342</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="1" t="inlineStr">
         <is>
-          <t>lz02jgE8</t>
+          <t>d03AlXrL</t>
         </is>
       </c>
       <c r="B46" s="2" t="n">
-        <v>45732.51041666666</v>
+        <v>45732.41666666666</v>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>sevilla</t>
+          <t>leganes</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>ath bilbao</t>
+          <t>betis</t>
         </is>
       </c>
       <c r="E46" t="n">
@@ -4999,42 +5019,44 @@
         </is>
       </c>
       <c r="I46" t="n">
-        <v>3</v>
+        <v>3.75</v>
       </c>
       <c r="J46" t="n">
-        <v>3.2</v>
+        <v>3.25</v>
       </c>
       <c r="K46" t="n">
-        <v>2.4</v>
+        <v>2.1</v>
       </c>
       <c r="L46" t="n">
-        <v>0.3137254901960784</v>
+        <v>0.2538354253835426</v>
       </c>
       <c r="M46" t="n">
-        <v>0.2941176470588235</v>
+        <v>0.292887029288703</v>
       </c>
       <c r="N46" t="n">
-        <v>0.392156862745098</v>
+        <v>0.4532775453277546</v>
       </c>
       <c r="O46" t="n">
-        <v>0.0625</v>
+        <v>0.05054945054945037</v>
       </c>
       <c r="P46" t="n">
         <v>2</v>
       </c>
       <c r="Q46" t="n">
-        <v>0.3285199202798995</v>
+        <v>0.1817550803098659</v>
       </c>
       <c r="R46" t="n">
-        <v>0.1393138671147877</v>
+        <v>0.2118499037001081</v>
       </c>
       <c r="S46" t="n">
-        <v>0.5321662126053129</v>
+        <v>0.6063950159900261</v>
       </c>
       <c r="T46" t="n">
         <v>1</v>
       </c>
-      <c r="U46" t="inlineStr"/>
+      <c r="U46" t="n">
+        <v>0</v>
+      </c>
       <c r="V46" t="n">
         <v>0</v>
       </c>
@@ -5042,10 +5064,10 @@
         <v>2</v>
       </c>
       <c r="X46" t="n">
-        <v>0.5321662126053129</v>
+        <v>0.6063950159900261</v>
       </c>
       <c r="Y46" t="n">
-        <v>2.4</v>
+        <v>2.1</v>
       </c>
       <c r="Z46" t="inlineStr">
         <is>
@@ -5053,13 +5075,13 @@
         </is>
       </c>
       <c r="AA46" t="n">
-        <v>0.1979992216091079</v>
+        <v>0.2485723032536862</v>
       </c>
       <c r="AB46" t="n">
-        <v>0.9312908720592976</v>
+        <v>6.063950159900261</v>
       </c>
       <c r="AC46" t="n">
-        <v>0.2036462923254135</v>
+        <v>0.394545112289918</v>
       </c>
     </row>
     <row r="47">
@@ -5098,42 +5120,44 @@
         </is>
       </c>
       <c r="I47" t="n">
-        <v>3</v>
+        <v>3.1</v>
       </c>
       <c r="J47" t="n">
-        <v>3.5</v>
+        <v>3.6</v>
       </c>
       <c r="K47" t="n">
-        <v>2.25</v>
+        <v>2.2</v>
       </c>
       <c r="L47" t="n">
-        <v>0.3134328358208955</v>
+        <v>0.3057915057915058</v>
       </c>
       <c r="M47" t="n">
-        <v>0.2686567164179104</v>
+        <v>0.2633204633204633</v>
       </c>
       <c r="N47" t="n">
-        <v>0.417910447761194</v>
+        <v>0.4308880308880308</v>
       </c>
       <c r="O47" t="n">
-        <v>0.06349206349206349</v>
+        <v>0.05490387748452275</v>
       </c>
       <c r="P47" t="n">
         <v>2</v>
       </c>
       <c r="Q47" t="n">
-        <v>0.360158691714796</v>
+        <v>0.1500320611963141</v>
       </c>
       <c r="R47" t="n">
-        <v>0.1265732302446819</v>
+        <v>0.4005985816376548</v>
       </c>
       <c r="S47" t="n">
-        <v>0.5132680780405221</v>
+        <v>0.4493693571660312</v>
       </c>
       <c r="T47" t="n">
         <v>1</v>
       </c>
-      <c r="U47" t="inlineStr"/>
+      <c r="U47" t="n">
+        <v>0</v>
+      </c>
       <c r="V47" t="n">
         <v>0</v>
       </c>
@@ -5141,10 +5165,10 @@
         <v>2</v>
       </c>
       <c r="X47" t="n">
-        <v>0.5132680780405221</v>
+        <v>0.4493693571660312</v>
       </c>
       <c r="Y47" t="n">
-        <v>2.25</v>
+        <v>2.2</v>
       </c>
       <c r="Z47" t="inlineStr">
         <is>
@@ -5152,13 +5176,13 @@
         </is>
       </c>
       <c r="AA47" t="n">
-        <v>0.1238825404729398</v>
+        <v>-0.009489511862276199</v>
       </c>
       <c r="AB47" t="n">
-        <v>0.8982191365709136</v>
+        <v>4.451051893171845</v>
       </c>
       <c r="AC47" t="n">
-        <v>0.1531093863257261</v>
+        <v>0.04877077552837639</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
DATA. Cambio de modelos en ENG y FRA y de stakes por reduccion de espacio m para evitar overfitting en ea
</commit_message>
<xml_diff>
--- a/data/predicciones.xlsx
+++ b/data/predicciones.xlsx
@@ -639,13 +639,13 @@
         <v>1</v>
       </c>
       <c r="Q2" t="n">
-        <v>0.003748854788823625</v>
+        <v>0.1819318047806384</v>
       </c>
       <c r="R2" t="n">
-        <v>0.9584938014830882</v>
+        <v>0.6053335771930102</v>
       </c>
       <c r="S2" t="n">
-        <v>0.03775734372808835</v>
+        <v>0.2127346180263514</v>
       </c>
       <c r="T2" t="n">
         <v>1</v>
@@ -660,7 +660,7 @@
         <v>1</v>
       </c>
       <c r="X2" t="n">
-        <v>0.9584938014830882</v>
+        <v>0.6053335771930102</v>
       </c>
       <c r="Y2" t="n">
         <v>1.67</v>
@@ -671,32 +671,32 @@
         </is>
       </c>
       <c r="AA2" t="n">
-        <v>0.8965442514578467</v>
+        <v>0.0162792147945178</v>
       </c>
       <c r="AB2" t="n">
-        <v>1.677364152595404</v>
+        <v>8.716803511579347</v>
       </c>
       <c r="AC2" t="n">
-        <v>0.9207364577549998</v>
+        <v>0.3925989591666588</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>KrrkXYu9</t>
+          <t>WM1fBiJk</t>
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>45731.5</v>
+        <v>45732.4375</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>everton</t>
+          <t>arsenal</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>west ham</t>
+          <t>chelsea</t>
         </is>
       </c>
       <c r="E3" t="n">
@@ -716,37 +716,37 @@
         </is>
       </c>
       <c r="I3" t="n">
-        <v>2.05</v>
+        <v>1.8</v>
       </c>
       <c r="J3" t="n">
-        <v>3.2</v>
+        <v>3.6</v>
       </c>
       <c r="K3" t="n">
-        <v>3.9</v>
+        <v>4.5</v>
       </c>
       <c r="L3" t="n">
-        <v>0.4616238209728131</v>
+        <v>0.5263157894736842</v>
       </c>
       <c r="M3" t="n">
-        <v>0.2957277603107084</v>
+        <v>0.2631578947368421</v>
       </c>
       <c r="N3" t="n">
-        <v>0.2426484187164787</v>
+        <v>0.2105263157894737</v>
       </c>
       <c r="O3" t="n">
-        <v>0.05671513445903686</v>
+        <v>0.05555555555555558</v>
       </c>
       <c r="P3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q3" t="n">
-        <v>0.9601086049693609</v>
+        <v>0.3345539039645855</v>
       </c>
       <c r="R3" t="n">
-        <v>0.02214276141821787</v>
+        <v>0.3493164095189908</v>
       </c>
       <c r="S3" t="n">
-        <v>0.01774863361242142</v>
+        <v>0.3161296865164237</v>
       </c>
       <c r="T3" t="n">
         <v>1</v>
@@ -758,13 +758,13 @@
         <v>0</v>
       </c>
       <c r="W3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X3" t="n">
-        <v>0.9601086049693609</v>
+        <v>0.3493164095189908</v>
       </c>
       <c r="Y3" t="n">
-        <v>3.2</v>
+        <v>1.8</v>
       </c>
       <c r="Z3" t="inlineStr">
         <is>
@@ -772,32 +772,32 @@
         </is>
       </c>
       <c r="AA3" t="n">
-        <v>0.9419761526827067</v>
+        <v>-0.4640380785822707</v>
       </c>
       <c r="AB3" t="n">
-        <v>10.08114035217829</v>
+        <v>0.6693870321770287</v>
       </c>
       <c r="AC3" t="n">
-        <v>0.937965843551143</v>
+        <v>0.01476250555440528</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>WM1fBiJk</t>
+          <t>KrrkXYu9</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>45732.4375</v>
+        <v>45731.5</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>arsenal</t>
+          <t>everton</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>chelsea</t>
+          <t>west ham</t>
         </is>
       </c>
       <c r="E4" t="n">
@@ -817,37 +817,37 @@
         </is>
       </c>
       <c r="I4" t="n">
-        <v>1.8</v>
+        <v>2.05</v>
       </c>
       <c r="J4" t="n">
-        <v>3.6</v>
+        <v>3.2</v>
       </c>
       <c r="K4" t="n">
-        <v>4.5</v>
+        <v>3.9</v>
       </c>
       <c r="L4" t="n">
-        <v>0.5263157894736842</v>
+        <v>0.4616238209728131</v>
       </c>
       <c r="M4" t="n">
-        <v>0.2631578947368421</v>
+        <v>0.2957277603107084</v>
       </c>
       <c r="N4" t="n">
-        <v>0.2105263157894737</v>
+        <v>0.2426484187164787</v>
       </c>
       <c r="O4" t="n">
-        <v>0.05555555555555558</v>
+        <v>0.05671513445903686</v>
       </c>
       <c r="P4" t="n">
         <v>0</v>
       </c>
       <c r="Q4" t="n">
-        <v>0.4948661281438991</v>
+        <v>0.3903159329531108</v>
       </c>
       <c r="R4" t="n">
-        <v>0.02183399383424048</v>
+        <v>0.2962311001079771</v>
       </c>
       <c r="S4" t="n">
-        <v>0.4832998780218604</v>
+        <v>0.3134529669389122</v>
       </c>
       <c r="T4" t="n">
         <v>1</v>
@@ -862,10 +862,10 @@
         <v>0</v>
       </c>
       <c r="X4" t="n">
-        <v>0.4948661281438991</v>
+        <v>0.3903159329531108</v>
       </c>
       <c r="Y4" t="n">
-        <v>3.6</v>
+        <v>3.2</v>
       </c>
       <c r="Z4" t="inlineStr">
         <is>
@@ -873,13 +873,13 @@
         </is>
       </c>
       <c r="AA4" t="n">
-        <v>0.3005838697377065</v>
+        <v>0.1131868115681612</v>
       </c>
       <c r="AB4" t="n">
-        <v>5.19609434551094</v>
+        <v>3.747032956349863</v>
       </c>
       <c r="AC4" t="n">
-        <v>0.01156625012203877</v>
+        <v>0.07686296601419862</v>
       </c>
     </row>
     <row r="5">
@@ -942,13 +942,13 @@
         <v>2</v>
       </c>
       <c r="Q5" t="n">
-        <v>0.04618457941927705</v>
+        <v>0.2029766535425652</v>
       </c>
       <c r="R5" t="n">
-        <v>0.0152417736073448</v>
+        <v>0.1845772805013731</v>
       </c>
       <c r="S5" t="n">
-        <v>0.9385736469733781</v>
+        <v>0.6124460659560617</v>
       </c>
       <c r="T5" t="n">
         <v>1</v>
@@ -963,7 +963,7 @@
         <v>2</v>
       </c>
       <c r="X5" t="n">
-        <v>0.9385736469733781</v>
+        <v>0.6124460659560617</v>
       </c>
       <c r="Y5" t="n">
         <v>2</v>
@@ -974,13 +974,13 @@
         </is>
       </c>
       <c r="AA5" t="n">
-        <v>0.8771472939467562</v>
+        <v>0.2248921319121233</v>
       </c>
       <c r="AB5" t="n">
-        <v>9.855023293220469</v>
+        <v>7.349352791472739</v>
       </c>
       <c r="AC5" t="n">
-        <v>0.8923890675541011</v>
+        <v>0.4094694124134964</v>
       </c>
     </row>
     <row r="6">
@@ -1043,13 +1043,13 @@
         <v>2</v>
       </c>
       <c r="Q6" t="n">
-        <v>0.3531501780959142</v>
+        <v>0.3409728869479181</v>
       </c>
       <c r="R6" t="n">
-        <v>0.007708931157384713</v>
+        <v>0.1496814042073696</v>
       </c>
       <c r="S6" t="n">
-        <v>0.639140890746701</v>
+        <v>0.5093457088447123</v>
       </c>
       <c r="T6" t="n">
         <v>1</v>
@@ -1064,7 +1064,7 @@
         <v>2</v>
       </c>
       <c r="X6" t="n">
-        <v>0.639140890746701</v>
+        <v>0.5093457088447123</v>
       </c>
       <c r="Y6" t="n">
         <v>2</v>
@@ -1075,13 +1075,13 @@
         </is>
       </c>
       <c r="AA6" t="n">
-        <v>0.278281781493402</v>
+        <v>0.01869141768942462</v>
       </c>
       <c r="AB6" t="n">
-        <v>6.710979352840361</v>
+        <v>6.112148506136547</v>
       </c>
       <c r="AC6" t="n">
-        <v>0.2859907126507868</v>
+        <v>0.1683728218967942</v>
       </c>
     </row>
     <row r="7">
@@ -1144,13 +1144,13 @@
         <v>2</v>
       </c>
       <c r="Q7" t="n">
-        <v>0.1137302364813753</v>
+        <v>0.3288440897264435</v>
       </c>
       <c r="R7" t="n">
-        <v>0.0003515988837535767</v>
+        <v>0.2289601394870671</v>
       </c>
       <c r="S7" t="n">
-        <v>0.8859181646348711</v>
+        <v>0.4421957707864893</v>
       </c>
       <c r="T7" t="n">
         <v>1</v>
@@ -1165,7 +1165,7 @@
         <v>2</v>
       </c>
       <c r="X7" t="n">
-        <v>0.8859181646348711</v>
+        <v>0.4421957707864893</v>
       </c>
       <c r="Y7" t="n">
         <v>4.33</v>
@@ -1176,13 +1176,13 @@
         </is>
       </c>
       <c r="AA7" t="n">
-        <v>0.8516593552159135</v>
+        <v>0.2746869932448945</v>
       </c>
       <c r="AB7" t="n">
-        <v>9.302140728666146</v>
+        <v>5.306349249437871</v>
       </c>
       <c r="AC7" t="n">
-        <v>0.7721879281534958</v>
+        <v>0.1133516810600458</v>
       </c>
     </row>
     <row r="8">
@@ -1245,13 +1245,13 @@
         <v>2</v>
       </c>
       <c r="Q8" t="n">
-        <v>0.09538689467432719</v>
+        <v>0.2028438277875327</v>
       </c>
       <c r="R8" t="n">
-        <v>0.00252255086861485</v>
+        <v>0.2040858139837192</v>
       </c>
       <c r="S8" t="n">
-        <v>0.902090554457058</v>
+        <v>0.5930703582287481</v>
       </c>
       <c r="T8" t="n">
         <v>1</v>
@@ -1266,7 +1266,7 @@
         <v>2</v>
       </c>
       <c r="X8" t="n">
-        <v>0.902090554457058</v>
+        <v>0.5930703582287481</v>
       </c>
       <c r="Y8" t="n">
         <v>3.6</v>
@@ -1277,13 +1277,13 @@
         </is>
       </c>
       <c r="AA8" t="n">
-        <v>0.8644330754020803</v>
+        <v>0.4365589575474974</v>
       </c>
       <c r="AB8" t="n">
-        <v>9.471950821799108</v>
+        <v>7.116844298744977</v>
       </c>
       <c r="AC8" t="n">
-        <v>0.8067036597827308</v>
+        <v>0.3889845442450289</v>
       </c>
     </row>
     <row r="9">
@@ -1346,13 +1346,13 @@
         <v>2</v>
       </c>
       <c r="Q9" t="n">
-        <v>0.02514691498385857</v>
+        <v>0.1766210291085296</v>
       </c>
       <c r="R9" t="n">
-        <v>0.1024152536126395</v>
+        <v>0.1996884664169913</v>
       </c>
       <c r="S9" t="n">
-        <v>0.872437831403502</v>
+        <v>0.623690504474479</v>
       </c>
       <c r="T9" t="n">
         <v>1</v>
@@ -1367,7 +1367,7 @@
         <v>2</v>
       </c>
       <c r="X9" t="n">
-        <v>0.872437831403502</v>
+        <v>0.623690504474479</v>
       </c>
       <c r="Y9" t="n">
         <v>1.83</v>
@@ -1378,13 +1378,13 @@
         </is>
       </c>
       <c r="AA9" t="n">
-        <v>0.7187484716486851</v>
+        <v>0.1703055701063816</v>
       </c>
       <c r="AB9" t="n">
-        <v>9.160597229736769</v>
+        <v>7.484286053693748</v>
       </c>
       <c r="AC9" t="n">
-        <v>0.7700225777908625</v>
+        <v>0.4240020380574877</v>
       </c>
     </row>
     <row r="10">
@@ -1447,13 +1447,13 @@
         <v>1</v>
       </c>
       <c r="Q10" t="n">
-        <v>0.324477770545987</v>
+        <v>0.2867448725048787</v>
       </c>
       <c r="R10" t="n">
-        <v>0.4637522384700204</v>
+        <v>0.4656366345949217</v>
       </c>
       <c r="S10" t="n">
-        <v>0.2117699909839925</v>
+        <v>0.2476184929001998</v>
       </c>
       <c r="T10" t="n">
         <v>1</v>
@@ -1468,7 +1468,7 @@
         <v>1</v>
       </c>
       <c r="X10" t="n">
-        <v>0.4637522384700204</v>
+        <v>0.4656366345949217</v>
       </c>
       <c r="Y10" t="n">
         <v>1.57</v>
@@ -1479,13 +1479,13 @@
         </is>
       </c>
       <c r="AA10" t="n">
-        <v>-0.4770333080738035</v>
+        <v>-0.4718429538350402</v>
       </c>
       <c r="AB10" t="n">
-        <v>0.53299407487669</v>
+        <v>1.475552611491797</v>
       </c>
       <c r="AC10" t="n">
-        <v>0.1392744679240334</v>
+        <v>0.178891762090043</v>
       </c>
     </row>
     <row r="11">
@@ -1548,24 +1548,28 @@
         <v>1</v>
       </c>
       <c r="Q11" t="n">
-        <v>0.3151703740088735</v>
+        <v>0.2701672091768437</v>
       </c>
       <c r="R11" t="n">
-        <v>0.502145549994072</v>
+        <v>0.5196998489974072</v>
       </c>
       <c r="S11" t="n">
-        <v>0.1826840759970546</v>
+        <v>0.2101329418257492</v>
       </c>
       <c r="T11" t="n">
         <v>1</v>
       </c>
-      <c r="U11" t="inlineStr"/>
-      <c r="V11" t="inlineStr"/>
+      <c r="U11" t="n">
+        <v>1</v>
+      </c>
+      <c r="V11" t="n">
+        <v>0</v>
+      </c>
       <c r="W11" t="n">
         <v>1</v>
       </c>
       <c r="X11" t="n">
-        <v>0.502145549994072</v>
+        <v>0.5196998489974072</v>
       </c>
       <c r="Y11" t="n">
         <v>1.36</v>
@@ -1576,13 +1580,13 @@
         </is>
       </c>
       <c r="AA11" t="n">
-        <v>-0.880783477800172</v>
+        <v>-0.814467237120906</v>
       </c>
       <c r="AB11" t="n">
-        <v>0.7403432334770879</v>
+        <v>2.271418653842935</v>
       </c>
       <c r="AC11" t="n">
-        <v>0.1869751759851985</v>
+        <v>0.2495326398205635</v>
       </c>
     </row>
     <row r="12">
@@ -1645,24 +1649,28 @@
         <v>1</v>
       </c>
       <c r="Q12" t="n">
-        <v>0.3324608718279879</v>
+        <v>0.290347959509236</v>
       </c>
       <c r="R12" t="n">
-        <v>0.3885275719693547</v>
+        <v>0.3872018922687704</v>
       </c>
       <c r="S12" t="n">
-        <v>0.2790115562026576</v>
+        <v>0.3224501482219935</v>
       </c>
       <c r="T12" t="n">
         <v>1</v>
       </c>
-      <c r="U12" t="inlineStr"/>
-      <c r="V12" t="inlineStr"/>
+      <c r="U12" t="n">
+        <v>1</v>
+      </c>
+      <c r="V12" t="n">
+        <v>0</v>
+      </c>
       <c r="W12" t="n">
         <v>1</v>
       </c>
       <c r="X12" t="n">
-        <v>0.3885275719693547</v>
+        <v>0.3872018922687704</v>
       </c>
       <c r="Y12" t="n">
         <v>1.67</v>
@@ -1673,19 +1681,19 @@
         </is>
       </c>
       <c r="AA12" t="n">
-        <v>-0.524117843001758</v>
+        <v>-0.5274221491211247</v>
       </c>
       <c r="AB12" t="n">
-        <v>0.8512372059595756</v>
+        <v>2.318939589632308</v>
       </c>
       <c r="AC12" t="n">
-        <v>0.05606670014136678</v>
+        <v>0.06475174404677692</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
-          <t>hEkEOCFE</t>
+          <t>bZz9Dn7D</t>
         </is>
       </c>
       <c r="B13" s="2" t="n">
@@ -1693,12 +1701,12 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>montpellier</t>
+          <t>strasbourg</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>st etienne</t>
+          <t>toulouse</t>
         </is>
       </c>
       <c r="E13" t="n">
@@ -1718,51 +1726,55 @@
         </is>
       </c>
       <c r="I13" t="n">
-        <v>2.2</v>
+        <v>2.25</v>
       </c>
       <c r="J13" t="n">
-        <v>3.5</v>
+        <v>3.25</v>
       </c>
       <c r="K13" t="n">
-        <v>3.2</v>
+        <v>3.25</v>
       </c>
       <c r="L13" t="n">
-        <v>0.4317656129529684</v>
+        <v>0.4193548387096774</v>
       </c>
       <c r="M13" t="n">
-        <v>0.2713955281418658</v>
+        <v>0.2903225806451613</v>
       </c>
       <c r="N13" t="n">
-        <v>0.2968388589051658</v>
+        <v>0.2903225806451613</v>
       </c>
       <c r="O13" t="n">
-        <v>0.05275974025974017</v>
+        <v>0.05982905982905984</v>
       </c>
       <c r="P13" t="n">
         <v>1</v>
       </c>
       <c r="Q13" t="n">
-        <v>0.346093611067589</v>
+        <v>0.3171570327596602</v>
       </c>
       <c r="R13" t="n">
-        <v>0.3633121028727284</v>
+        <v>0.4041497819598617</v>
       </c>
       <c r="S13" t="n">
-        <v>0.2905942860596827</v>
+        <v>0.2786931852804782</v>
       </c>
       <c r="T13" t="n">
         <v>1</v>
       </c>
-      <c r="U13" t="inlineStr"/>
-      <c r="V13" t="inlineStr"/>
+      <c r="U13" t="n">
+        <v>1</v>
+      </c>
+      <c r="V13" t="n">
+        <v>0</v>
+      </c>
       <c r="W13" t="n">
         <v>1</v>
       </c>
       <c r="X13" t="n">
-        <v>0.3633121028727284</v>
+        <v>0.4041497819598617</v>
       </c>
       <c r="Y13" t="n">
-        <v>2.2</v>
+        <v>2.25</v>
       </c>
       <c r="Z13" t="inlineStr">
         <is>
@@ -1770,32 +1782,32 @@
         </is>
       </c>
       <c r="AA13" t="n">
-        <v>-0.1672611447333311</v>
+        <v>-0.07253039247224899</v>
       </c>
       <c r="AB13" t="n">
-        <v>0.2225815761682787</v>
+        <v>3.668991214772437</v>
       </c>
       <c r="AC13" t="n">
-        <v>0.01721849180513946</v>
+        <v>0.08699274920020145</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="inlineStr">
         <is>
-          <t>bZz9Dn7D</t>
+          <t>jk9J2Vhe</t>
         </is>
       </c>
       <c r="B14" s="2" t="n">
-        <v>45732.55208333334</v>
+        <v>45732.69791666666</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>strasbourg</t>
+          <t>psg</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>toulouse</t>
+          <t>marseille</t>
         </is>
       </c>
       <c r="E14" t="n">
@@ -1815,51 +1827,55 @@
         </is>
       </c>
       <c r="I14" t="n">
-        <v>2.25</v>
+        <v>1.45</v>
       </c>
       <c r="J14" t="n">
-        <v>3.25</v>
+        <v>5</v>
       </c>
       <c r="K14" t="n">
-        <v>3.25</v>
+        <v>6</v>
       </c>
       <c r="L14" t="n">
-        <v>0.4193548387096774</v>
+        <v>0.6528835690968444</v>
       </c>
       <c r="M14" t="n">
-        <v>0.2903225806451613</v>
+        <v>0.1893362350380849</v>
       </c>
       <c r="N14" t="n">
-        <v>0.2903225806451613</v>
+        <v>0.1577801958650707</v>
       </c>
       <c r="O14" t="n">
-        <v>0.05982905982905984</v>
+        <v>0.05632183908045985</v>
       </c>
       <c r="P14" t="n">
         <v>1</v>
       </c>
       <c r="Q14" t="n">
-        <v>0.3444739169138507</v>
+        <v>0.3851244220539524</v>
       </c>
       <c r="R14" t="n">
-        <v>0.3885043726616377</v>
+        <v>0.3880416997331687</v>
       </c>
       <c r="S14" t="n">
-        <v>0.2670217104245117</v>
+        <v>0.2268338782128791</v>
       </c>
       <c r="T14" t="n">
         <v>1</v>
       </c>
-      <c r="U14" t="inlineStr"/>
-      <c r="V14" t="inlineStr"/>
+      <c r="U14" t="n">
+        <v>1</v>
+      </c>
+      <c r="V14" t="n">
+        <v>0</v>
+      </c>
       <c r="W14" t="n">
         <v>1</v>
       </c>
       <c r="X14" t="n">
-        <v>0.3885043726616377</v>
+        <v>0.3880416997331687</v>
       </c>
       <c r="Y14" t="n">
-        <v>2.25</v>
+        <v>1.45</v>
       </c>
       <c r="Z14" t="inlineStr">
         <is>
@@ -1867,32 +1883,32 @@
         </is>
       </c>
       <c r="AA14" t="n">
-        <v>-0.1006921292090521</v>
+        <v>-0.9718656341931234</v>
       </c>
       <c r="AB14" t="n">
-        <v>1.257271827165174</v>
+        <v>0.2813335015114266</v>
       </c>
       <c r="AC14" t="n">
-        <v>0.04403045574778702</v>
+        <v>0.002917277679216235</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="inlineStr">
         <is>
-          <t>jk9J2Vhe</t>
+          <t>OEiKK3Et</t>
         </is>
       </c>
       <c r="B15" s="2" t="n">
-        <v>45732.69791666666</v>
+        <v>45731.54166666666</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>psg</t>
+          <t>nantes</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>marseille</t>
+          <t>lille</t>
         </is>
       </c>
       <c r="E15" t="n">
@@ -1912,37 +1928,37 @@
         </is>
       </c>
       <c r="I15" t="n">
-        <v>1.45</v>
+        <v>3.6</v>
       </c>
       <c r="J15" t="n">
-        <v>5</v>
+        <v>3.2</v>
       </c>
       <c r="K15" t="n">
-        <v>6</v>
+        <v>2.15</v>
       </c>
       <c r="L15" t="n">
-        <v>0.6528835690968444</v>
+        <v>0.2631981637337414</v>
       </c>
       <c r="M15" t="n">
-        <v>0.1893362350380849</v>
+        <v>0.296097934200459</v>
       </c>
       <c r="N15" t="n">
-        <v>0.1577801958650707</v>
+        <v>0.4407039020657995</v>
       </c>
       <c r="O15" t="n">
-        <v>0.05632183908045985</v>
+        <v>0.05539405684754528</v>
       </c>
       <c r="P15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q15" t="n">
-        <v>0.3338974972391223</v>
+        <v>0.3599593831083472</v>
       </c>
       <c r="R15" t="n">
-        <v>0.4234568083806666</v>
+        <v>0.2179311917455568</v>
       </c>
       <c r="S15" t="n">
-        <v>0.242645694380211</v>
+        <v>0.422109425146096</v>
       </c>
       <c r="T15" t="n">
         <v>1</v>
@@ -1950,13 +1966,13 @@
       <c r="U15" t="inlineStr"/>
       <c r="V15" t="inlineStr"/>
       <c r="W15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="X15" t="n">
-        <v>0.4234568083806666</v>
+        <v>0.422109425146096</v>
       </c>
       <c r="Y15" t="n">
-        <v>1.45</v>
+        <v>2.15</v>
       </c>
       <c r="Z15" t="inlineStr">
         <is>
@@ -1964,32 +1980,32 @@
         </is>
       </c>
       <c r="AA15" t="n">
-        <v>-0.8577502841067409</v>
+        <v>-0.08040411820512493</v>
       </c>
       <c r="AB15" t="n">
-        <v>0.6415251151323692</v>
+        <v>5.712274555570427</v>
       </c>
       <c r="AC15" t="n">
-        <v>0.08955931114154431</v>
+        <v>0.06215004203774877</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="inlineStr">
         <is>
-          <t>xKn0F8x1</t>
+          <t>KtoTIsqg</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
-        <v>45731.71180555555</v>
+        <v>45731.625</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>lens</t>
+          <t>angers</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>rennes</t>
+          <t>monaco</t>
         </is>
       </c>
       <c r="E16" t="n">
@@ -2009,51 +2025,55 @@
         </is>
       </c>
       <c r="I16" t="n">
-        <v>2.05</v>
+        <v>6.5</v>
       </c>
       <c r="J16" t="n">
-        <v>3.5</v>
+        <v>4.75</v>
       </c>
       <c r="K16" t="n">
-        <v>3.6</v>
+        <v>1.42</v>
       </c>
       <c r="L16" t="n">
-        <v>0.4640029460504511</v>
+        <v>0.1439701173959445</v>
       </c>
       <c r="M16" t="n">
-        <v>0.2717731541152641</v>
+        <v>0.1970117395944503</v>
       </c>
       <c r="N16" t="n">
-        <v>0.2642238998342846</v>
+        <v>0.6590181430096052</v>
       </c>
       <c r="O16" t="n">
-        <v>0.05129694154084419</v>
+        <v>0.06859782174830364</v>
       </c>
       <c r="P16" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="Q16" t="n">
-        <v>0.3489445586821911</v>
+        <v>0.3309016977987642</v>
       </c>
       <c r="R16" t="n">
-        <v>0.337074904645411</v>
+        <v>0.1698830794120545</v>
       </c>
       <c r="S16" t="n">
-        <v>0.3139805366723979</v>
+        <v>0.4992152227891813</v>
       </c>
       <c r="T16" t="n">
         <v>1</v>
       </c>
-      <c r="U16" t="inlineStr"/>
-      <c r="V16" t="inlineStr"/>
+      <c r="U16" t="n">
+        <v>1</v>
+      </c>
+      <c r="V16" t="n">
+        <v>0</v>
+      </c>
       <c r="W16" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="X16" t="n">
-        <v>0.3489445586821911</v>
+        <v>0.4992152227891813</v>
       </c>
       <c r="Y16" t="n">
-        <v>3.5</v>
+        <v>1.42</v>
       </c>
       <c r="Z16" t="inlineStr">
         <is>
@@ -2061,32 +2081,32 @@
         </is>
       </c>
       <c r="AA16" t="n">
-        <v>0.08852238215506754</v>
+        <v>-0.6931294848556253</v>
       </c>
       <c r="AB16" t="n">
-        <v>7.327835732326012</v>
+        <v>3.75550582377338</v>
       </c>
       <c r="AC16" t="n">
-        <v>0.01186965403678014</v>
+        <v>0.1683135249904171</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="inlineStr">
         <is>
-          <t>OEiKK3Et</t>
+          <t>xKn0F8x1</t>
         </is>
       </c>
       <c r="B17" s="2" t="n">
-        <v>45731.54166666666</v>
+        <v>45731.71180555555</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>nantes</t>
+          <t>lens</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>lille</t>
+          <t>rennes</t>
         </is>
       </c>
       <c r="E17" t="n">
@@ -2106,37 +2126,37 @@
         </is>
       </c>
       <c r="I17" t="n">
+        <v>2.05</v>
+      </c>
+      <c r="J17" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="K17" t="n">
         <v>3.6</v>
       </c>
-      <c r="J17" t="n">
-        <v>3.2</v>
-      </c>
-      <c r="K17" t="n">
-        <v>2.15</v>
-      </c>
       <c r="L17" t="n">
-        <v>0.2631981637337414</v>
+        <v>0.4640029460504511</v>
       </c>
       <c r="M17" t="n">
-        <v>0.296097934200459</v>
+        <v>0.2717731541152641</v>
       </c>
       <c r="N17" t="n">
-        <v>0.4407039020657995</v>
+        <v>0.2642238998342846</v>
       </c>
       <c r="O17" t="n">
-        <v>0.05539405684754528</v>
+        <v>0.05129694154084419</v>
       </c>
       <c r="P17" t="n">
         <v>2</v>
       </c>
       <c r="Q17" t="n">
-        <v>0.3408893113707371</v>
+        <v>0.3075905795670333</v>
       </c>
       <c r="R17" t="n">
-        <v>0.2125136503296773</v>
+        <v>0.2811150809950221</v>
       </c>
       <c r="S17" t="n">
-        <v>0.4465970382995856</v>
+        <v>0.4112943394379447</v>
       </c>
       <c r="T17" t="n">
         <v>1</v>
@@ -2147,10 +2167,10 @@
         <v>2</v>
       </c>
       <c r="X17" t="n">
-        <v>0.4465970382995856</v>
+        <v>0.4112943394379447</v>
       </c>
       <c r="Y17" t="n">
-        <v>2.15</v>
+        <v>3.6</v>
       </c>
       <c r="Z17" t="inlineStr">
         <is>
@@ -2158,32 +2178,32 @@
         </is>
       </c>
       <c r="AA17" t="n">
-        <v>-0.03462292839642699</v>
+        <v>0.1848690853756157</v>
       </c>
       <c r="AB17" t="n">
-        <v>7.612548496169001</v>
+        <v>5.922638487906403</v>
       </c>
       <c r="AC17" t="n">
-        <v>0.1057077269288484</v>
+        <v>0.1037037598709113</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="inlineStr">
         <is>
-          <t>KtoTIsqg</t>
+          <t>hEkEOCFE</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
-        <v>45731.625</v>
+        <v>45732.55208333334</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>angers</t>
+          <t>montpellier</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>monaco</t>
+          <t>st etienne</t>
         </is>
       </c>
       <c r="E18" t="n">
@@ -2203,37 +2223,37 @@
         </is>
       </c>
       <c r="I18" t="n">
-        <v>6.5</v>
+        <v>2.2</v>
       </c>
       <c r="J18" t="n">
-        <v>4.75</v>
+        <v>3.5</v>
       </c>
       <c r="K18" t="n">
-        <v>1.42</v>
+        <v>3.2</v>
       </c>
       <c r="L18" t="n">
-        <v>0.1439701173959445</v>
+        <v>0.4317656129529684</v>
       </c>
       <c r="M18" t="n">
-        <v>0.1970117395944503</v>
+        <v>0.2713955281418658</v>
       </c>
       <c r="N18" t="n">
-        <v>0.6590181430096052</v>
+        <v>0.2968388589051658</v>
       </c>
       <c r="O18" t="n">
-        <v>0.06859782174830364</v>
+        <v>0.05275974025974017</v>
       </c>
       <c r="P18" t="n">
         <v>2</v>
       </c>
       <c r="Q18" t="n">
-        <v>0.324426563388138</v>
+        <v>0.3158253888592285</v>
       </c>
       <c r="R18" t="n">
-        <v>0.1576709952462738</v>
+        <v>0.3400063945749346</v>
       </c>
       <c r="S18" t="n">
-        <v>0.5179024413655883</v>
+        <v>0.3441682165658369</v>
       </c>
       <c r="T18" t="n">
         <v>1</v>
@@ -2244,10 +2264,10 @@
         <v>2</v>
       </c>
       <c r="X18" t="n">
-        <v>0.5179024413655883</v>
+        <v>0.3441682165658369</v>
       </c>
       <c r="Y18" t="n">
-        <v>1.42</v>
+        <v>3.2</v>
       </c>
       <c r="Z18" t="inlineStr">
         <is>
@@ -2255,13 +2275,13 @@
         </is>
       </c>
       <c r="AA18" t="n">
-        <v>-0.6299488887163446</v>
+        <v>0.04606286045939913</v>
       </c>
       <c r="AB18" t="n">
-        <v>5.073756808859895</v>
+        <v>0.9912044637096102</v>
       </c>
       <c r="AC18" t="n">
-        <v>0.1934758779774503</v>
+        <v>0.004161821990902259</v>
       </c>
     </row>
     <row r="19">
@@ -2359,7 +2379,7 @@
         <v>0.08137185496656392</v>
       </c>
       <c r="AB19" t="n">
-        <v>7.644560045283121</v>
+        <v>5.241984031051283</v>
       </c>
       <c r="AC19" t="n">
         <v>0.02894922060545724</v>
@@ -2460,7 +2480,7 @@
         <v>0.1168365981194634</v>
       </c>
       <c r="AB20" t="n">
-        <v>7.605355071478527</v>
+        <v>5.215100620442419</v>
       </c>
       <c r="AC20" t="n">
         <v>0.04289543686923009</v>
@@ -2561,7 +2581,7 @@
         <v>0.1590623990001787</v>
       </c>
       <c r="AB21" t="n">
-        <v>8.245779718169375</v>
+        <v>5.654248949601858</v>
       </c>
       <c r="AC21" t="n">
         <v>0.0263440014354237</v>
@@ -2662,7 +2682,7 @@
         <v>0.1410176722316527</v>
       </c>
       <c r="AB22" t="n">
-        <v>7.972101362180066</v>
+        <v>5.466583791209188</v>
       </c>
       <c r="AC22" t="n">
         <v>0.0493065230196385</v>
@@ -2763,7 +2783,7 @@
         <v>0.1443881393418322</v>
       </c>
       <c r="AB23" t="n">
-        <v>8.165822090127483</v>
+        <v>5.599420861801702</v>
       </c>
       <c r="AC23" t="n">
         <v>0.05453877501989568</v>
@@ -2864,7 +2884,7 @@
         <v>0.09582982254863967</v>
       </c>
       <c r="AB24" t="n">
-        <v>1.553247298733291</v>
+        <v>1.065083861988542</v>
       </c>
       <c r="AC24" t="n">
         <v>0.006039438668831443</v>
@@ -2965,7 +2985,7 @@
         <v>0.1256330300075835</v>
       </c>
       <c r="AB25" t="n">
-        <v>9.315277764646796</v>
+        <v>6.387619038614947</v>
       </c>
       <c r="AC25" t="n">
         <v>0.1046588725540835</v>
@@ -3066,7 +3086,7 @@
         <v>-0.8164620768923989</v>
       </c>
       <c r="AB26" t="n">
-        <v>4.952217523975561</v>
+        <v>3.39580630215467</v>
       </c>
       <c r="AC26" t="n">
         <v>0.1774672067631947</v>
@@ -3167,7 +3187,7 @@
         <v>0.1697650924292819</v>
       </c>
       <c r="AB27" t="n">
-        <v>11.14547261883452</v>
+        <v>7.642609795772242</v>
       </c>
       <c r="AC27" t="n">
         <v>0.1892974227324384</v>
@@ -3264,7 +3284,7 @@
         <v>0.2219572117660627</v>
       </c>
       <c r="AB28" t="n">
-        <v>4.965856941755381</v>
+        <v>6.810318091550236</v>
       </c>
       <c r="AC28" t="n">
         <v>0.04942252746512305</v>
@@ -3361,7 +3381,7 @@
         <v>-0.05179151909060236</v>
       </c>
       <c r="AB29" t="n">
-        <v>5.61316605405587</v>
+        <v>7.698056302705193</v>
       </c>
       <c r="AC29" t="n">
         <v>0.1862133149730658</v>
@@ -3458,7 +3478,7 @@
         <v>0.001532722931784636</v>
       </c>
       <c r="AB30" t="n">
-        <v>5.840486040348328</v>
+        <v>8.009809426763422</v>
       </c>
       <c r="AC30" t="n">
         <v>0.2670736140307631</v>
@@ -3555,7 +3575,7 @@
         <v>0.1639807159148786</v>
       </c>
       <c r="AB31" t="n">
-        <v>4.303621776780865</v>
+        <v>5.902109865299472</v>
       </c>
       <c r="AC31" t="n">
         <v>0.07296997998702159</v>
@@ -3656,7 +3676,7 @@
         <v>0.2018774264188089</v>
       </c>
       <c r="AB32" t="n">
-        <v>5.406100045084751</v>
+        <v>7.414080061830515</v>
       </c>
       <c r="AC32" t="n">
         <v>0.2703347000861001</v>
@@ -3757,7 +3777,7 @@
         <v>0.4832743762466003</v>
       </c>
       <c r="AB33" t="n">
-        <v>9.260378761434334</v>
+        <v>6.349974007840686</v>
       </c>
       <c r="AC33" t="n">
         <v>0.4623840263172714</v>
@@ -3854,7 +3874,7 @@
         <v>0.5848102200936074</v>
       </c>
       <c r="AB34" t="n">
-        <v>9.94875426879217</v>
+        <v>6.822002927171773</v>
       </c>
       <c r="AC34" t="n">
         <v>0.5078719390070286</v>
@@ -3951,7 +3971,7 @@
         <v>0.3104244903908822</v>
       </c>
       <c r="AB35" t="n">
-        <v>6.644527897502742</v>
+        <v>4.556247701144738</v>
       </c>
       <c r="AC35" t="n">
         <v>0.02103795683043208</v>
@@ -4052,7 +4072,7 @@
         <v>-0.0366961905256462</v>
       </c>
       <c r="AB36" t="n">
-        <v>4.362742979849529</v>
+        <v>5.983190372365069</v>
       </c>
       <c r="AC36" t="n">
         <v>0.3941569657283458</v>
@@ -4149,7 +4169,7 @@
         <v>0.1365976489428761</v>
       </c>
       <c r="AB37" t="n">
-        <v>2.733776618305976</v>
+        <v>3.749179362248196</v>
       </c>
       <c r="AC37" t="n">
         <v>0.06447592131935154</v>
@@ -4250,7 +4270,7 @@
         <v>0.1217150874264707</v>
       </c>
       <c r="AB38" t="n">
-        <v>4.352005611985295</v>
+        <v>5.968464839294119</v>
       </c>
       <c r="AC38" t="n">
         <v>0.0945009107214016</v>
@@ -4351,7 +4371,7 @@
         <v>-0.03062214043242174</v>
       </c>
       <c r="AB39" t="n">
-        <v>5.559763124380114</v>
+        <v>7.624817999149871</v>
       </c>
       <c r="AC39" t="n">
         <v>0.1480009715372257</v>
@@ -4452,7 +4472,7 @@
         <v>0.08839149561085879</v>
       </c>
       <c r="AB40" t="n">
-        <v>4.228762185322977</v>
+        <v>5.799445282728654</v>
       </c>
       <c r="AC40" t="n">
         <v>0.0797699993906506</v>
@@ -4553,7 +4573,7 @@
         <v>0.0351148666422473</v>
       </c>
       <c r="AB41" t="n">
-        <v>4.871503388746443</v>
+        <v>6.680918933137979</v>
       </c>
       <c r="AC41" t="n">
         <v>0.06721181657319203</v>
@@ -4654,7 +4674,7 @@
         <v>0.1439713182498873</v>
       </c>
       <c r="AB42" t="n">
-        <v>5.10701930497429</v>
+        <v>7.003912189679026</v>
       </c>
       <c r="AC42" t="n">
         <v>0.1511955068022653</v>
@@ -4755,7 +4775,7 @@
         <v>0.4977996134973705</v>
       </c>
       <c r="AB43" t="n">
-        <v>13.22910980885405</v>
+        <v>9.071389583214206</v>
       </c>
       <c r="AC43" t="n">
         <v>0.3204309127245602</v>
@@ -4856,7 +4876,7 @@
         <v>0.4615073974859437</v>
       </c>
       <c r="AB44" t="n">
-        <v>12.92261096228916</v>
+        <v>8.861218945569707</v>
       </c>
       <c r="AC44" t="n">
         <v>0.3454095943970351</v>
@@ -4957,7 +4977,7 @@
         <v>0.03483603474573414</v>
       </c>
       <c r="AB45" t="n">
-        <v>0.6772493097398289</v>
+        <v>0.9287990533574796</v>
       </c>
       <c r="AC45" t="n">
         <v>0.009717650622998342</v>
@@ -5058,7 +5078,7 @@
         <v>0.2485723032536862</v>
       </c>
       <c r="AB46" t="n">
-        <v>4.244765111930183</v>
+        <v>5.821392153504251</v>
       </c>
       <c r="AC46" t="n">
         <v>0.394545112289918</v>
@@ -5159,7 +5179,7 @@
         <v>-0.009489511862276199</v>
       </c>
       <c r="AB47" t="n">
-        <v>3.123198324969714</v>
+        <v>4.283243417101322</v>
       </c>
       <c r="AC47" t="n">
         <v>0.04877077552837639</v>

</xml_diff>

<commit_message>
DATA. Actualizo cuotas y pred x jugadores missing
</commit_message>
<xml_diff>
--- a/data/predicciones.xlsx
+++ b/data/predicciones.xlsx
@@ -615,37 +615,37 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>2.05</v>
+        <v>2.1</v>
       </c>
       <c r="J2" t="n">
         <v>3.2</v>
       </c>
       <c r="K2" t="n">
-        <v>3.9</v>
+        <v>3.8</v>
       </c>
       <c r="L2" t="n">
-        <v>0.4616238209728131</v>
+        <v>0.4527177959791511</v>
       </c>
       <c r="M2" t="n">
-        <v>0.2957277603107084</v>
+        <v>0.297096053611318</v>
       </c>
       <c r="N2" t="n">
-        <v>0.2426484187164787</v>
+        <v>0.2501861504095309</v>
       </c>
       <c r="O2" t="n">
-        <v>0.05671513445903686</v>
+        <v>0.05184837092731831</v>
       </c>
       <c r="P2" t="n">
         <v>0</v>
       </c>
       <c r="Q2" t="n">
-        <v>0.3903159329531108</v>
+        <v>0.3873684857574431</v>
       </c>
       <c r="R2" t="n">
-        <v>0.2962311001079771</v>
+        <v>0.2824342167881583</v>
       </c>
       <c r="S2" t="n">
-        <v>0.3134529669389122</v>
+        <v>0.3301972974543986</v>
       </c>
       <c r="T2" t="n">
         <v>1</v>
@@ -660,7 +660,7 @@
         <v>0</v>
       </c>
       <c r="X2" t="n">
-        <v>0.3903159329531108</v>
+        <v>0.3873684857574431</v>
       </c>
       <c r="Y2" t="n">
         <v>3.2</v>
@@ -671,13 +671,13 @@
         </is>
       </c>
       <c r="AA2" t="n">
-        <v>0.1131868115681612</v>
+        <v>0.10889961564719</v>
       </c>
       <c r="AB2" t="n">
-        <v>4.683791195437329</v>
+        <v>4.648421829089317</v>
       </c>
       <c r="AC2" t="n">
-        <v>0.07686296601419862</v>
+        <v>0.05717118830304446</v>
       </c>
     </row>
     <row r="3">
@@ -716,37 +716,37 @@
         </is>
       </c>
       <c r="I3" t="n">
-        <v>3.75</v>
+        <v>4.1</v>
       </c>
       <c r="J3" t="n">
         <v>3.5</v>
       </c>
       <c r="K3" t="n">
-        <v>2</v>
+        <v>1.91</v>
       </c>
       <c r="L3" t="n">
-        <v>0.253393665158371</v>
+        <v>0.2315873345804753</v>
       </c>
       <c r="M3" t="n">
-        <v>0.2714932126696832</v>
+        <v>0.2712880205085568</v>
       </c>
       <c r="N3" t="n">
-        <v>0.4751131221719457</v>
+        <v>0.4971246449109679</v>
       </c>
       <c r="O3" t="n">
-        <v>0.05238095238095242</v>
+        <v>0.0531769341627597</v>
       </c>
       <c r="P3" t="n">
         <v>2</v>
       </c>
       <c r="Q3" t="n">
-        <v>0.2029766535425652</v>
+        <v>0.1877181880191466</v>
       </c>
       <c r="R3" t="n">
-        <v>0.1845772805013731</v>
+        <v>0.1550733915580073</v>
       </c>
       <c r="S3" t="n">
-        <v>0.6124460659560617</v>
+        <v>0.6572084204228461</v>
       </c>
       <c r="T3" t="n">
         <v>1</v>
@@ -761,10 +761,10 @@
         <v>2</v>
       </c>
       <c r="X3" t="n">
-        <v>0.6124460659560617</v>
+        <v>0.6572084204228461</v>
       </c>
       <c r="Y3" t="n">
-        <v>2</v>
+        <v>1.91</v>
       </c>
       <c r="Z3" t="inlineStr">
         <is>
@@ -772,13 +772,13 @@
         </is>
       </c>
       <c r="AA3" t="n">
-        <v>0.2248921319121233</v>
+        <v>0.2805143769314682</v>
       </c>
       <c r="AB3" t="n">
-        <v>7.349352791472739</v>
+        <v>7.886501045074153</v>
       </c>
       <c r="AC3" t="n">
-        <v>0.4094694124134964</v>
+        <v>0.4694902324036995</v>
       </c>
     </row>
     <row r="4">
@@ -841,13 +841,13 @@
         <v>1</v>
       </c>
       <c r="Q4" t="n">
-        <v>0.1819318047806384</v>
+        <v>0.1892970745136956</v>
       </c>
       <c r="R4" t="n">
-        <v>0.6053335771930102</v>
+        <v>0.5605512147577782</v>
       </c>
       <c r="S4" t="n">
-        <v>0.2127346180263514</v>
+        <v>0.250151710728526</v>
       </c>
       <c r="T4" t="n">
         <v>1</v>
@@ -862,7 +862,7 @@
         <v>1</v>
       </c>
       <c r="X4" t="n">
-        <v>0.6053335771930102</v>
+        <v>0.5605512147577782</v>
       </c>
       <c r="Y4" t="n">
         <v>1.67</v>
@@ -873,13 +873,13 @@
         </is>
       </c>
       <c r="AA4" t="n">
-        <v>0.0162792147945178</v>
+        <v>-0.09534249455897073</v>
       </c>
       <c r="AB4" t="n">
-        <v>7.264002926316122</v>
+        <v>6.24643356369017</v>
       </c>
       <c r="AC4" t="n">
-        <v>0.3925989591666588</v>
+        <v>0.3103995040292522</v>
       </c>
     </row>
     <row r="5">
@@ -942,13 +942,13 @@
         <v>2</v>
       </c>
       <c r="Q5" t="n">
-        <v>0.3409728869479181</v>
+        <v>0.3437754425068115</v>
       </c>
       <c r="R5" t="n">
-        <v>0.1496814042073696</v>
+        <v>0.1591890481050512</v>
       </c>
       <c r="S5" t="n">
-        <v>0.5093457088447123</v>
+        <v>0.4970355093881372</v>
       </c>
       <c r="T5" t="n">
         <v>1</v>
@@ -963,7 +963,7 @@
         <v>2</v>
       </c>
       <c r="X5" t="n">
-        <v>0.5093457088447123</v>
+        <v>0.4970355093881372</v>
       </c>
       <c r="Y5" t="n">
         <v>2</v>
@@ -974,13 +974,13 @@
         </is>
       </c>
       <c r="AA5" t="n">
-        <v>0.01869141768942462</v>
+        <v>-0.005928981223725538</v>
       </c>
       <c r="AB5" t="n">
-        <v>6.112148506136548</v>
+        <v>5.937904059644152</v>
       </c>
       <c r="AC5" t="n">
-        <v>0.1683728218967942</v>
+        <v>0.1532600668813257</v>
       </c>
     </row>
     <row r="6">
@@ -1019,37 +1019,37 @@
         </is>
       </c>
       <c r="I6" t="n">
-        <v>1.7</v>
+        <v>1.73</v>
       </c>
       <c r="J6" t="n">
         <v>4.2</v>
       </c>
       <c r="K6" t="n">
-        <v>4.33</v>
+        <v>4.2</v>
       </c>
       <c r="L6" t="n">
-        <v>0.556367975035947</v>
+        <v>0.5483028720626633</v>
       </c>
       <c r="M6" t="n">
-        <v>0.2251965613240738</v>
+        <v>0.2258485639686684</v>
       </c>
       <c r="N6" t="n">
-        <v>0.2184354636399792</v>
+        <v>0.2258485639686684</v>
       </c>
       <c r="O6" t="n">
-        <v>0.05727741442997525</v>
+        <v>0.05422515827140106</v>
       </c>
       <c r="P6" t="n">
         <v>2</v>
       </c>
       <c r="Q6" t="n">
-        <v>0.3288440897264435</v>
+        <v>0.3207615041367547</v>
       </c>
       <c r="R6" t="n">
-        <v>0.2289601394870671</v>
+        <v>0.2228997044055763</v>
       </c>
       <c r="S6" t="n">
-        <v>0.4421957707864893</v>
+        <v>0.4563387914576688</v>
       </c>
       <c r="T6" t="n">
         <v>1</v>
@@ -1064,10 +1064,10 @@
         <v>2</v>
       </c>
       <c r="X6" t="n">
-        <v>0.4421957707864893</v>
+        <v>0.4563387914576688</v>
       </c>
       <c r="Y6" t="n">
-        <v>4.33</v>
+        <v>4.2</v>
       </c>
       <c r="Z6" t="inlineStr">
         <is>
@@ -1075,13 +1075,13 @@
         </is>
       </c>
       <c r="AA6" t="n">
-        <v>0.2746869932448945</v>
+        <v>0.2864446637881904</v>
       </c>
       <c r="AB6" t="n">
-        <v>5.306349249437871</v>
+        <v>5.476065497492026</v>
       </c>
       <c r="AC6" t="n">
-        <v>0.1133516810600458</v>
+        <v>0.1355772873209141</v>
       </c>
     </row>
     <row r="7">
@@ -1144,13 +1144,13 @@
         <v>1</v>
       </c>
       <c r="Q7" t="n">
-        <v>0.3345539039645855</v>
+        <v>0.348908771156899</v>
       </c>
       <c r="R7" t="n">
-        <v>0.3493164095189908</v>
+        <v>0.3646369592558916</v>
       </c>
       <c r="S7" t="n">
-        <v>0.3161296865164237</v>
+        <v>0.2864542695872095</v>
       </c>
       <c r="T7" t="n">
         <v>1</v>
@@ -1165,7 +1165,7 @@
         <v>1</v>
       </c>
       <c r="X7" t="n">
-        <v>0.3493164095189908</v>
+        <v>0.3646369592558916</v>
       </c>
       <c r="Y7" t="n">
         <v>1.8</v>
@@ -1176,13 +1176,13 @@
         </is>
       </c>
       <c r="AA7" t="n">
-        <v>-0.4640380785822707</v>
+        <v>-0.4295668416742439</v>
       </c>
       <c r="AB7" t="n">
-        <v>0.5578225268141906</v>
+        <v>0.6025502995823002</v>
       </c>
       <c r="AC7" t="n">
-        <v>0.01476250555440528</v>
+        <v>0.01572818809899257</v>
       </c>
     </row>
     <row r="8">
@@ -1221,7 +1221,7 @@
         </is>
       </c>
       <c r="I8" t="n">
-        <v>2</v>
+        <v>1.95</v>
       </c>
       <c r="J8" t="n">
         <v>3.75</v>
@@ -1230,28 +1230,28 @@
         <v>3.6</v>
       </c>
       <c r="L8" t="n">
-        <v>0.4787234042553192</v>
+        <v>0.4850444624090541</v>
       </c>
       <c r="M8" t="n">
-        <v>0.2553191489361702</v>
+        <v>0.2522231204527081</v>
       </c>
       <c r="N8" t="n">
-        <v>0.2659574468085107</v>
+        <v>0.2627324171382376</v>
       </c>
       <c r="O8" t="n">
-        <v>0.04444444444444429</v>
+        <v>0.05726495726495751</v>
       </c>
       <c r="P8" t="n">
         <v>2</v>
       </c>
       <c r="Q8" t="n">
-        <v>0.2028438277875327</v>
+        <v>0.2044074454010578</v>
       </c>
       <c r="R8" t="n">
-        <v>0.2040858139837192</v>
+        <v>0.2172107729919482</v>
       </c>
       <c r="S8" t="n">
-        <v>0.5930703582287481</v>
+        <v>0.578381781606994</v>
       </c>
       <c r="T8" t="n">
         <v>1</v>
@@ -1266,7 +1266,7 @@
         <v>2</v>
       </c>
       <c r="X8" t="n">
-        <v>0.5930703582287481</v>
+        <v>0.578381781606994</v>
       </c>
       <c r="Y8" t="n">
         <v>3.6</v>
@@ -1277,13 +1277,13 @@
         </is>
       </c>
       <c r="AA8" t="n">
-        <v>0.4365589575474974</v>
+        <v>0.4162209283789148</v>
       </c>
       <c r="AB8" t="n">
-        <v>7.116844298744977</v>
+        <v>6.940581379283929</v>
       </c>
       <c r="AC8" t="n">
-        <v>0.3889845442450289</v>
+        <v>0.3611710086150459</v>
       </c>
     </row>
     <row r="9">
@@ -1346,13 +1346,13 @@
         <v>2</v>
       </c>
       <c r="Q9" t="n">
-        <v>0.1766210291085296</v>
+        <v>0.204294056336087</v>
       </c>
       <c r="R9" t="n">
-        <v>0.1996884664169913</v>
+        <v>0.2163115749810206</v>
       </c>
       <c r="S9" t="n">
-        <v>0.623690504474479</v>
+        <v>0.5793943686828924</v>
       </c>
       <c r="T9" t="n">
         <v>1</v>
@@ -1367,7 +1367,7 @@
         <v>2</v>
       </c>
       <c r="X9" t="n">
-        <v>0.623690504474479</v>
+        <v>0.5793943686828924</v>
       </c>
       <c r="Y9" t="n">
         <v>1.83</v>
@@ -1378,13 +1378,13 @@
         </is>
       </c>
       <c r="AA9" t="n">
-        <v>0.1703055701063816</v>
+        <v>0.07264059601167848</v>
       </c>
       <c r="AB9" t="n">
-        <v>7.484286053693748</v>
+        <v>6.952732424194709</v>
       </c>
       <c r="AC9" t="n">
-        <v>0.4240020380574877</v>
+        <v>0.3630827937018718</v>
       </c>
     </row>
     <row r="10">
@@ -1423,37 +1423,37 @@
         </is>
       </c>
       <c r="I10" t="n">
-        <v>1.57</v>
+        <v>1.55</v>
       </c>
       <c r="J10" t="n">
-        <v>4</v>
+        <v>4.2</v>
       </c>
       <c r="K10" t="n">
-        <v>6</v>
+        <v>5.75</v>
       </c>
       <c r="L10" t="n">
-        <v>0.6045340050377834</v>
+        <v>0.6102722850464338</v>
       </c>
       <c r="M10" t="n">
-        <v>0.23727959697733</v>
+        <v>0.2252195337671363</v>
       </c>
       <c r="N10" t="n">
-        <v>0.1581863979848867</v>
+        <v>0.16450818118643</v>
       </c>
       <c r="O10" t="n">
-        <v>0.05360934182590227</v>
+        <v>0.05716957189607941</v>
       </c>
       <c r="P10" t="n">
         <v>1</v>
       </c>
       <c r="Q10" t="n">
-        <v>0.3248197856387997</v>
+        <v>0.3201969587926571</v>
       </c>
       <c r="R10" t="n">
-        <v>0.4644140102321041</v>
+        <v>0.4659406439909705</v>
       </c>
       <c r="S10" t="n">
-        <v>0.2107662041290962</v>
+        <v>0.2138623972163723</v>
       </c>
       <c r="T10" t="n">
         <v>1</v>
@@ -1468,10 +1468,10 @@
         <v>1</v>
       </c>
       <c r="X10" t="n">
-        <v>0.4644140102321041</v>
+        <v>0.4659406439909705</v>
       </c>
       <c r="Y10" t="n">
-        <v>1.57</v>
+        <v>1.55</v>
       </c>
       <c r="Z10" t="inlineStr">
         <is>
@@ -1479,13 +1479,13 @@
         </is>
       </c>
       <c r="AA10" t="n">
-        <v>-0.4752105332203446</v>
+        <v>-0.5050763669345374</v>
       </c>
       <c r="AB10" t="n">
-        <v>2.291722570495967</v>
+        <v>2.23067497043724</v>
       </c>
       <c r="AC10" t="n">
-        <v>0.1395942245933045</v>
+        <v>0.1457436851983134</v>
       </c>
     </row>
     <row r="11">
@@ -1548,13 +1548,13 @@
         <v>2</v>
       </c>
       <c r="Q11" t="n">
-        <v>0.3443898841786099</v>
+        <v>0.336057806688228</v>
       </c>
       <c r="R11" t="n">
-        <v>0.2147726570526692</v>
+        <v>0.1952001512444045</v>
       </c>
       <c r="S11" t="n">
-        <v>0.4408374587687209</v>
+        <v>0.4687420420673675</v>
       </c>
       <c r="T11" t="n">
         <v>1</v>
@@ -1565,7 +1565,7 @@
         <v>2</v>
       </c>
       <c r="X11" t="n">
-        <v>0.4408374587687209</v>
+        <v>0.4687420420673675</v>
       </c>
       <c r="Y11" t="n">
         <v>2.15</v>
@@ -1576,13 +1576,13 @@
         </is>
       </c>
       <c r="AA11" t="n">
-        <v>-0.04539083795413056</v>
+        <v>0.006778600386817402</v>
       </c>
       <c r="AB11" t="n">
-        <v>6.387536511091053</v>
+        <v>7.031130631010512</v>
       </c>
       <c r="AC11" t="n">
-        <v>0.09644757459011094</v>
+        <v>0.1326842353791394</v>
       </c>
     </row>
     <row r="12">
@@ -1645,13 +1645,13 @@
         <v>2</v>
       </c>
       <c r="Q12" t="n">
-        <v>0.3302362221979781</v>
+        <v>0.3421684445777872</v>
       </c>
       <c r="R12" t="n">
-        <v>0.1408865092056547</v>
+        <v>0.146188964553715</v>
       </c>
       <c r="S12" t="n">
-        <v>0.5288772685963673</v>
+        <v>0.5116425908684978</v>
       </c>
       <c r="T12" t="n">
         <v>1</v>
@@ -1662,7 +1662,7 @@
         <v>2</v>
       </c>
       <c r="X12" t="n">
-        <v>0.5288772685963673</v>
+        <v>0.5116425908684978</v>
       </c>
       <c r="Y12" t="n">
         <v>1.42</v>
@@ -1673,13 +1673,13 @@
         </is>
       </c>
       <c r="AA12" t="n">
-        <v>-0.5928435204599013</v>
+        <v>-0.6511131451588884</v>
       </c>
       <c r="AB12" t="n">
-        <v>4.621247136491139</v>
+        <v>4.198842259229671</v>
       </c>
       <c r="AC12" t="n">
-        <v>0.1986410463983892</v>
+        <v>0.1694741462907107</v>
       </c>
     </row>
     <row r="13">
@@ -1742,13 +1742,13 @@
         <v>0</v>
       </c>
       <c r="Q13" t="n">
-        <v>0.407221353405305</v>
+        <v>0.3911655750385049</v>
       </c>
       <c r="R13" t="n">
-        <v>0.2400915631419464</v>
+        <v>0.2515745587632219</v>
       </c>
       <c r="S13" t="n">
-        <v>0.3526870834527485</v>
+        <v>0.3572598661982733</v>
       </c>
       <c r="T13" t="n">
         <v>1</v>
@@ -1759,7 +1759,7 @@
         <v>0</v>
       </c>
       <c r="X13" t="n">
-        <v>0.407221353405305</v>
+        <v>0.3911655750385049</v>
       </c>
       <c r="Y13" t="n">
         <v>3.5</v>
@@ -1770,13 +1770,13 @@
         </is>
       </c>
       <c r="AA13" t="n">
-        <v>0.1701098947674271</v>
+        <v>0.1476318050539068</v>
       </c>
       <c r="AB13" t="n">
-        <v>6.108320301079575</v>
+        <v>5.867483625577573</v>
       </c>
       <c r="AC13" t="n">
-        <v>0.05453426995255656</v>
+        <v>0.03390570884023153</v>
       </c>
     </row>
     <row r="14">
@@ -1839,13 +1839,13 @@
         <v>1</v>
       </c>
       <c r="Q14" t="n">
-        <v>0.3332544758518874</v>
+        <v>0.3330724105053016</v>
       </c>
       <c r="R14" t="n">
-        <v>0.5016207449119162</v>
+        <v>0.5081128952946802</v>
       </c>
       <c r="S14" t="n">
-        <v>0.1651247792361963</v>
+        <v>0.1588146942000182</v>
       </c>
       <c r="T14" t="n">
         <v>1</v>
@@ -1856,7 +1856,7 @@
         <v>1</v>
       </c>
       <c r="X14" t="n">
-        <v>0.5016207449119162</v>
+        <v>0.5081128952946802</v>
       </c>
       <c r="Y14" t="n">
         <v>1.36</v>
@@ -1867,13 +1867,13 @@
         </is>
       </c>
       <c r="AA14" t="n">
-        <v>-0.8827660747772051</v>
+        <v>-0.8582401733312078</v>
       </c>
       <c r="AB14" t="n">
-        <v>3.162149220232763</v>
+        <v>3.297143805225689</v>
       </c>
       <c r="AC14" t="n">
-        <v>0.1683662690600288</v>
+        <v>0.1750404847893786</v>
       </c>
     </row>
     <row r="15">
@@ -1912,7 +1912,7 @@
         </is>
       </c>
       <c r="I15" t="n">
-        <v>1.67</v>
+        <v>1.65</v>
       </c>
       <c r="J15" t="n">
         <v>3.9</v>
@@ -1921,28 +1921,28 @@
         <v>5</v>
       </c>
       <c r="L15" t="n">
-        <v>0.5674708261793209</v>
+        <v>0.5704256252742431</v>
       </c>
       <c r="M15" t="n">
-        <v>0.2429939178767861</v>
+        <v>0.2413339183852567</v>
       </c>
       <c r="N15" t="n">
-        <v>0.1895352559438931</v>
+        <v>0.1882404563405002</v>
       </c>
       <c r="O15" t="n">
-        <v>0.05521265161983724</v>
+        <v>0.06247086247086253</v>
       </c>
       <c r="P15" t="n">
         <v>1</v>
       </c>
       <c r="Q15" t="n">
-        <v>0.3213346859363072</v>
+        <v>0.3313516500422912</v>
       </c>
       <c r="R15" t="n">
-        <v>0.3654876547596708</v>
+        <v>0.3730617582062941</v>
       </c>
       <c r="S15" t="n">
-        <v>0.313177659304022</v>
+        <v>0.2955865917514148</v>
       </c>
       <c r="T15" t="n">
         <v>1</v>
@@ -1953,10 +1953,10 @@
         <v>1</v>
       </c>
       <c r="X15" t="n">
-        <v>0.3654876547596708</v>
+        <v>0.3730617582062941</v>
       </c>
       <c r="Y15" t="n">
-        <v>1.67</v>
+        <v>1.65</v>
       </c>
       <c r="Z15" t="inlineStr">
         <is>
@@ -1964,13 +1964,13 @@
         </is>
       </c>
       <c r="AA15" t="n">
-        <v>-0.5815456963452982</v>
+        <v>-0.5914586137840229</v>
       </c>
       <c r="AB15" t="n">
-        <v>3.232066798547255</v>
+        <v>3.264556928655713</v>
       </c>
       <c r="AC15" t="n">
-        <v>0.04415296882336367</v>
+        <v>0.04171010816400283</v>
       </c>
     </row>
     <row r="16">
@@ -2009,37 +2009,37 @@
         </is>
       </c>
       <c r="I16" t="n">
-        <v>2.2</v>
+        <v>2.25</v>
       </c>
       <c r="J16" t="n">
         <v>3.5</v>
       </c>
       <c r="K16" t="n">
-        <v>3.2</v>
+        <v>3.1</v>
       </c>
       <c r="L16" t="n">
-        <v>0.4317656129529684</v>
+        <v>0.4221789883268482</v>
       </c>
       <c r="M16" t="n">
-        <v>0.2713955281418658</v>
+        <v>0.2714007782101167</v>
       </c>
       <c r="N16" t="n">
-        <v>0.2968388589051658</v>
+        <v>0.306420233463035</v>
       </c>
       <c r="O16" t="n">
-        <v>0.05275974025974017</v>
+        <v>0.05273937532002049</v>
       </c>
       <c r="P16" t="n">
         <v>0</v>
       </c>
       <c r="Q16" t="n">
-        <v>0.3527479548252427</v>
+        <v>0.3733086998300114</v>
       </c>
       <c r="R16" t="n">
-        <v>0.315978228305919</v>
+        <v>0.3040606145977652</v>
       </c>
       <c r="S16" t="n">
-        <v>0.3312738168688383</v>
+        <v>0.3226306855722235</v>
       </c>
       <c r="T16" t="n">
         <v>1</v>
@@ -2050,7 +2050,7 @@
         <v>0</v>
       </c>
       <c r="X16" t="n">
-        <v>0.3527479548252427</v>
+        <v>0.3733086998300114</v>
       </c>
       <c r="Y16" t="n">
         <v>3.5</v>
@@ -2061,13 +2061,13 @@
         </is>
       </c>
       <c r="AA16" t="n">
-        <v>0.09384713675533987</v>
+        <v>0.1226321797620159</v>
       </c>
       <c r="AB16" t="n">
-        <v>5.291219322378641</v>
+        <v>5.59963049745017</v>
       </c>
       <c r="AC16" t="n">
-        <v>0.0214741379564044</v>
+        <v>0.0506780142577879</v>
       </c>
     </row>
     <row r="17">
@@ -2130,13 +2130,13 @@
         <v>0</v>
       </c>
       <c r="Q17" t="n">
-        <v>0.4049999809642356</v>
+        <v>0.3892989469816718</v>
       </c>
       <c r="R17" t="n">
-        <v>0.3550746912305567</v>
+        <v>0.3641781385631898</v>
       </c>
       <c r="S17" t="n">
-        <v>0.2399253278052076</v>
+        <v>0.2465229144551384</v>
       </c>
       <c r="T17" t="n">
         <v>1</v>
@@ -2147,7 +2147,7 @@
         <v>0</v>
       </c>
       <c r="X17" t="n">
-        <v>0.4049999809642356</v>
+        <v>0.3892989469816718</v>
       </c>
       <c r="Y17" t="n">
         <v>3.25</v>
@@ -2158,13 +2158,13 @@
         </is>
       </c>
       <c r="AA17" t="n">
-        <v>0.1405555280594515</v>
+        <v>0.1178762567513038</v>
       </c>
       <c r="AB17" t="n">
-        <v>6.074999714463534</v>
+        <v>5.839484204725077</v>
       </c>
       <c r="AC17" t="n">
-        <v>0.04992528973367888</v>
+        <v>0.02512080841848202</v>
       </c>
     </row>
     <row r="18">
@@ -2203,37 +2203,37 @@
         </is>
       </c>
       <c r="I18" t="n">
-        <v>1.45</v>
+        <v>1.42</v>
       </c>
       <c r="J18" t="n">
         <v>5</v>
       </c>
       <c r="K18" t="n">
-        <v>6</v>
+        <v>6.25</v>
       </c>
       <c r="L18" t="n">
-        <v>0.6528835690968444</v>
+        <v>0.6617257808364214</v>
       </c>
       <c r="M18" t="n">
-        <v>0.1893362350380849</v>
+        <v>0.1879301217575437</v>
       </c>
       <c r="N18" t="n">
-        <v>0.1577801958650707</v>
+        <v>0.1503440974060349</v>
       </c>
       <c r="O18" t="n">
-        <v>0.05632183908045985</v>
+        <v>0.0642253521126761</v>
       </c>
       <c r="P18" t="n">
         <v>1</v>
       </c>
       <c r="Q18" t="n">
-        <v>0.3616558399073921</v>
+        <v>0.3506693272537604</v>
       </c>
       <c r="R18" t="n">
-        <v>0.4885489283257208</v>
+        <v>0.4766000226331849</v>
       </c>
       <c r="S18" t="n">
-        <v>0.1497952317668871</v>
+        <v>0.1727306501130548</v>
       </c>
       <c r="T18" t="n">
         <v>1</v>
@@ -2244,10 +2244,10 @@
         <v>1</v>
       </c>
       <c r="X18" t="n">
-        <v>0.4885489283257208</v>
+        <v>0.4766000226331849</v>
       </c>
       <c r="Y18" t="n">
-        <v>1.45</v>
+        <v>1.42</v>
       </c>
       <c r="Z18" t="inlineStr">
         <is>
@@ -2255,13 +2255,13 @@
         </is>
       </c>
       <c r="AA18" t="n">
-        <v>-0.648009008728233</v>
+        <v>-0.7695903996687561</v>
       </c>
       <c r="AB18" t="n">
-        <v>4.022897743958161</v>
+        <v>3.427072731480631</v>
       </c>
       <c r="AC18" t="n">
-        <v>0.1268930884183287</v>
+        <v>0.1259306953794245</v>
       </c>
     </row>
     <row r="19">
@@ -2300,37 +2300,37 @@
         </is>
       </c>
       <c r="I19" t="n">
-        <v>2.25</v>
+        <v>2.3</v>
       </c>
       <c r="J19" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="K19" t="n">
         <v>3.25</v>
       </c>
-      <c r="K19" t="n">
-        <v>3.3</v>
-      </c>
       <c r="L19" t="n">
-        <v>0.4212076583210604</v>
+        <v>0.4121260154547257</v>
       </c>
       <c r="M19" t="n">
-        <v>0.2916053019145803</v>
+        <v>0.296215573608084</v>
       </c>
       <c r="N19" t="n">
-        <v>0.2871870397643594</v>
+        <v>0.2916584109371904</v>
       </c>
       <c r="O19" t="n">
-        <v>0.05516705516705511</v>
+        <v>0.05497491638795982</v>
       </c>
       <c r="P19" t="n">
         <v>2</v>
       </c>
       <c r="Q19" t="n">
-        <v>0.3637813467438568</v>
+        <v>0.3675230895684603</v>
       </c>
       <c r="R19" t="n">
-        <v>0.2663978678434548</v>
+        <v>0.2398525266719508</v>
       </c>
       <c r="S19" t="n">
-        <v>0.3698207854126883</v>
+        <v>0.3926243837595889</v>
       </c>
       <c r="T19" t="n">
         <v>1</v>
@@ -2345,10 +2345,10 @@
         <v>2</v>
       </c>
       <c r="X19" t="n">
-        <v>0.3698207854126883</v>
+        <v>0.3926243837595889</v>
       </c>
       <c r="Y19" t="n">
-        <v>3.3</v>
+        <v>3.25</v>
       </c>
       <c r="Z19" t="inlineStr">
         <is>
@@ -2356,13 +2356,13 @@
         </is>
       </c>
       <c r="AA19" t="n">
-        <v>0.09582982254863967</v>
+        <v>0.1226796654305173</v>
       </c>
       <c r="AB19" t="n">
-        <v>1.553247298733291</v>
+        <v>1.649022411790273</v>
       </c>
       <c r="AC19" t="n">
-        <v>0.006039438668831443</v>
+        <v>0.02510129419112855</v>
       </c>
     </row>
     <row r="20">
@@ -2425,13 +2425,13 @@
         <v>2</v>
       </c>
       <c r="Q20" t="n">
-        <v>0.3389257829052878</v>
+        <v>0.3393261966365683</v>
       </c>
       <c r="R20" t="n">
-        <v>0.217489561635341</v>
+        <v>0.2006951479748571</v>
       </c>
       <c r="S20" t="n">
-        <v>0.4435846554593713</v>
+        <v>0.4599786553885745</v>
       </c>
       <c r="T20" t="n">
         <v>1</v>
@@ -2446,7 +2446,7 @@
         <v>2</v>
       </c>
       <c r="X20" t="n">
-        <v>0.4435846554593713</v>
+        <v>0.4599786553885745</v>
       </c>
       <c r="Y20" t="n">
         <v>2.75</v>
@@ -2457,13 +2457,13 @@
         </is>
       </c>
       <c r="AA20" t="n">
-        <v>0.1256330300075835</v>
+        <v>0.1513950298963313</v>
       </c>
       <c r="AB20" t="n">
-        <v>9.315277764646797</v>
+        <v>9.659551763160064</v>
       </c>
       <c r="AC20" t="n">
-        <v>0.1046588725540835</v>
+        <v>0.1206524587520061</v>
       </c>
     </row>
     <row r="21">
@@ -2502,37 +2502,37 @@
         </is>
       </c>
       <c r="I21" t="n">
-        <v>2</v>
+        <v>1.95</v>
       </c>
       <c r="J21" t="n">
-        <v>3.25</v>
+        <v>3.3</v>
       </c>
       <c r="K21" t="n">
-        <v>4</v>
+        <v>4.1</v>
       </c>
       <c r="L21" t="n">
-        <v>0.4727272727272727</v>
+        <v>0.4839055793991416</v>
       </c>
       <c r="M21" t="n">
-        <v>0.2909090909090909</v>
+        <v>0.2859442060085837</v>
       </c>
       <c r="N21" t="n">
-        <v>0.2363636363636364</v>
+        <v>0.2301502145922747</v>
       </c>
       <c r="O21" t="n">
-        <v>0.05769230769230771</v>
+        <v>0.05975325487520622</v>
       </c>
       <c r="P21" t="n">
         <v>0</v>
       </c>
       <c r="Q21" t="n">
-        <v>0.3640266688230058</v>
+        <v>0.3629139113737304</v>
       </c>
       <c r="R21" t="n">
-        <v>0.3008958829594457</v>
+        <v>0.3057759885076025</v>
       </c>
       <c r="S21" t="n">
-        <v>0.3350774482175485</v>
+        <v>0.3313101001186672</v>
       </c>
       <c r="T21" t="n">
         <v>1</v>
@@ -2547,10 +2547,10 @@
         <v>0</v>
       </c>
       <c r="X21" t="n">
-        <v>0.3640266688230058</v>
+        <v>0.3629139113737304</v>
       </c>
       <c r="Y21" t="n">
-        <v>3.25</v>
+        <v>3.3</v>
       </c>
       <c r="Z21" t="inlineStr">
         <is>
@@ -2558,13 +2558,13 @@
         </is>
       </c>
       <c r="AA21" t="n">
-        <v>0.08137185496656392</v>
+        <v>0.08591995979709133</v>
       </c>
       <c r="AB21" t="n">
-        <v>7.644560045283121</v>
+        <v>7.621192138848337</v>
       </c>
       <c r="AC21" t="n">
-        <v>0.02894922060545724</v>
+        <v>0.03160381125506312</v>
       </c>
     </row>
     <row r="22">
@@ -2606,34 +2606,34 @@
         <v>8.5</v>
       </c>
       <c r="J22" t="n">
-        <v>5</v>
+        <v>5.25</v>
       </c>
       <c r="K22" t="n">
-        <v>1.36</v>
+        <v>1.33</v>
       </c>
       <c r="L22" t="n">
-        <v>0.111731843575419</v>
+        <v>0.1109874826147427</v>
       </c>
       <c r="M22" t="n">
-        <v>0.1899441340782123</v>
+        <v>0.1796940194714882</v>
       </c>
       <c r="N22" t="n">
-        <v>0.6983240223463688</v>
+        <v>0.7093184979137691</v>
       </c>
       <c r="O22" t="n">
-        <v>0.05294117647058805</v>
+        <v>0.06000294854784016</v>
       </c>
       <c r="P22" t="n">
         <v>2</v>
       </c>
       <c r="Q22" t="n">
-        <v>0.3417045964123467</v>
+        <v>0.3402745657403572</v>
       </c>
       <c r="R22" t="n">
-        <v>0.139123600412112</v>
+        <v>0.1322129073788614</v>
       </c>
       <c r="S22" t="n">
-        <v>0.5191718031755413</v>
+        <v>0.5275125268807814</v>
       </c>
       <c r="T22" t="n">
         <v>1</v>
@@ -2648,10 +2648,10 @@
         <v>2</v>
       </c>
       <c r="X22" t="n">
-        <v>0.5191718031755413</v>
+        <v>0.5275125268807814</v>
       </c>
       <c r="Y22" t="n">
-        <v>1.36</v>
+        <v>1.33</v>
       </c>
       <c r="Z22" t="inlineStr">
         <is>
@@ -2659,13 +2659,13 @@
         </is>
       </c>
       <c r="AA22" t="n">
-        <v>-0.8164620768923989</v>
+        <v>-0.9042676946926079</v>
       </c>
       <c r="AB22" t="n">
-        <v>4.952217523975561</v>
+        <v>4.538022664878159</v>
       </c>
       <c r="AC22" t="n">
-        <v>0.1774672067631947</v>
+        <v>0.1872379611404242</v>
       </c>
     </row>
     <row r="23">
@@ -2704,37 +2704,37 @@
         </is>
       </c>
       <c r="I23" t="n">
-        <v>2.4</v>
+        <v>2.35</v>
       </c>
       <c r="J23" t="n">
         <v>3.6</v>
       </c>
       <c r="K23" t="n">
-        <v>2.75</v>
+        <v>2.8</v>
       </c>
       <c r="L23" t="n">
-        <v>0.3937947494033414</v>
+        <v>0.4012738853503184</v>
       </c>
       <c r="M23" t="n">
-        <v>0.2625298329355609</v>
+        <v>0.2619426751592356</v>
       </c>
       <c r="N23" t="n">
-        <v>0.3436754176610979</v>
+        <v>0.3367834394904458</v>
       </c>
       <c r="O23" t="n">
-        <v>0.05808080808080796</v>
+        <v>0.06045254981425208</v>
       </c>
       <c r="P23" t="n">
         <v>0</v>
       </c>
       <c r="Q23" t="n">
-        <v>0.3621597653085013</v>
+        <v>0.3655965076499988</v>
       </c>
       <c r="R23" t="n">
-        <v>0.3192643284392712</v>
+        <v>0.305142011037885</v>
       </c>
       <c r="S23" t="n">
-        <v>0.3185759062522274</v>
+        <v>0.3292614813121161</v>
       </c>
       <c r="T23" t="n">
         <v>1</v>
@@ -2749,7 +2749,7 @@
         <v>0</v>
       </c>
       <c r="X23" t="n">
-        <v>0.3621597653085013</v>
+        <v>0.3655965076499988</v>
       </c>
       <c r="Y23" t="n">
         <v>3.6</v>
@@ -2760,13 +2760,13 @@
         </is>
       </c>
       <c r="AA23" t="n">
-        <v>0.1168365981194634</v>
+        <v>0.12159516443846</v>
       </c>
       <c r="AB23" t="n">
-        <v>7.605355071478527</v>
+        <v>7.677526660649976</v>
       </c>
       <c r="AC23" t="n">
-        <v>0.04289543686923009</v>
+        <v>0.03633502633788271</v>
       </c>
     </row>
     <row r="24">
@@ -2805,37 +2805,37 @@
         </is>
       </c>
       <c r="I24" t="n">
-        <v>2.38</v>
+        <v>2.45</v>
       </c>
       <c r="J24" t="n">
         <v>3.6</v>
       </c>
       <c r="K24" t="n">
-        <v>2.88</v>
+        <v>2.75</v>
       </c>
       <c r="L24" t="n">
-        <v>0.4020100502512564</v>
+        <v>0.3888834331729352</v>
       </c>
       <c r="M24" t="n">
-        <v>0.2657733109994417</v>
+        <v>0.2646567809093587</v>
       </c>
       <c r="N24" t="n">
-        <v>0.3322166387493021</v>
+        <v>0.346459785917706</v>
       </c>
       <c r="O24" t="n">
-        <v>0.0451680672268906</v>
+        <v>0.04957740672026389</v>
       </c>
       <c r="P24" t="n">
         <v>0</v>
       </c>
       <c r="Q24" t="n">
-        <v>0.3926561770556846</v>
+        <v>0.3909760751745404</v>
       </c>
       <c r="R24" t="n">
-        <v>0.2410316473240546</v>
+        <v>0.2516438881041319</v>
       </c>
       <c r="S24" t="n">
-        <v>0.3663121756202609</v>
+        <v>0.3573800367213278</v>
       </c>
       <c r="T24" t="n">
         <v>1</v>
@@ -2850,7 +2850,7 @@
         <v>0</v>
       </c>
       <c r="X24" t="n">
-        <v>0.3926561770556846</v>
+        <v>0.3909760751745404</v>
       </c>
       <c r="Y24" t="n">
         <v>3.6</v>
@@ -2861,13 +2861,13 @@
         </is>
       </c>
       <c r="AA24" t="n">
-        <v>0.1590623990001787</v>
+        <v>0.1567361040878252</v>
       </c>
       <c r="AB24" t="n">
-        <v>8.245779718169375</v>
+        <v>8.210497578665349</v>
       </c>
       <c r="AC24" t="n">
-        <v>0.0263440014354237</v>
+        <v>0.03359603845321263</v>
       </c>
     </row>
     <row r="25">
@@ -2930,13 +2930,13 @@
         <v>0</v>
       </c>
       <c r="Q25" t="n">
-        <v>0.3796238743895269</v>
+        <v>0.3796452533383949</v>
       </c>
       <c r="R25" t="n">
-        <v>0.2900587742405846</v>
+        <v>0.2899645845277158</v>
       </c>
       <c r="S25" t="n">
-        <v>0.3303173513698884</v>
+        <v>0.3303901621338893</v>
       </c>
       <c r="T25" t="n">
         <v>1</v>
@@ -2951,7 +2951,7 @@
         <v>0</v>
       </c>
       <c r="X25" t="n">
-        <v>0.3796238743895269</v>
+        <v>0.3796452533383949</v>
       </c>
       <c r="Y25" t="n">
         <v>3.6</v>
@@ -2962,13 +2962,13 @@
         </is>
       </c>
       <c r="AA25" t="n">
-        <v>0.1410176722316527</v>
+        <v>0.1410472738531622</v>
       </c>
       <c r="AB25" t="n">
-        <v>7.972101362180066</v>
+        <v>7.972550320106293</v>
       </c>
       <c r="AC25" t="n">
-        <v>0.0493065230196385</v>
+        <v>0.04925509120450561</v>
       </c>
     </row>
     <row r="26">
@@ -3007,37 +3007,37 @@
         </is>
       </c>
       <c r="I26" t="n">
-        <v>2</v>
+        <v>1.95</v>
       </c>
       <c r="J26" t="n">
         <v>3.5</v>
       </c>
       <c r="K26" t="n">
-        <v>3.75</v>
+        <v>3.9</v>
       </c>
       <c r="L26" t="n">
-        <v>0.4751131221719457</v>
+        <v>0.4861111111111112</v>
       </c>
       <c r="M26" t="n">
-        <v>0.2714932126696832</v>
+        <v>0.2708333333333333</v>
       </c>
       <c r="N26" t="n">
-        <v>0.253393665158371</v>
+        <v>0.2430555555555556</v>
       </c>
       <c r="O26" t="n">
-        <v>0.05238095238095242</v>
+        <v>0.05494505494505497</v>
       </c>
       <c r="P26" t="n">
         <v>0</v>
       </c>
       <c r="Q26" t="n">
-        <v>0.3888486709584516</v>
+        <v>0.3911658779575489</v>
       </c>
       <c r="R26" t="n">
-        <v>0.3343098959385559</v>
+        <v>0.3269349744065203</v>
       </c>
       <c r="S26" t="n">
-        <v>0.2768414331029924</v>
+        <v>0.2818991476359308</v>
       </c>
       <c r="T26" t="n">
         <v>1</v>
@@ -3052,7 +3052,7 @@
         <v>0</v>
       </c>
       <c r="X26" t="n">
-        <v>0.3888486709584516</v>
+        <v>0.3911658779575489</v>
       </c>
       <c r="Y26" t="n">
         <v>3.5</v>
@@ -3063,13 +3063,13 @@
         </is>
       </c>
       <c r="AA26" t="n">
-        <v>0.1443881393418322</v>
+        <v>0.1476322291405684</v>
       </c>
       <c r="AB26" t="n">
-        <v>8.165822090127483</v>
+        <v>8.214483437108527</v>
       </c>
       <c r="AC26" t="n">
-        <v>0.05453877501989568</v>
+        <v>0.06423090355102862</v>
       </c>
     </row>
     <row r="27">
@@ -3132,13 +3132,13 @@
         <v>2</v>
       </c>
       <c r="Q27" t="n">
-        <v>0.341439368640634</v>
+        <v>0.3371372534871282</v>
       </c>
       <c r="R27" t="n">
-        <v>0.1278238399862936</v>
+        <v>0.1127657077920824</v>
       </c>
       <c r="S27" t="n">
-        <v>0.5307367913730724</v>
+        <v>0.5500970387207894</v>
       </c>
       <c r="T27" t="n">
         <v>1</v>
@@ -3153,7 +3153,7 @@
         <v>2</v>
       </c>
       <c r="X27" t="n">
-        <v>0.5307367913730724</v>
+        <v>0.5500970387207894</v>
       </c>
       <c r="Y27" t="n">
         <v>2.3</v>
@@ -3164,13 +3164,13 @@
         </is>
       </c>
       <c r="AA27" t="n">
-        <v>0.1697650924292819</v>
+        <v>0.2040178377367812</v>
       </c>
       <c r="AB27" t="n">
-        <v>11.14547261883452</v>
+        <v>11.55203781313658</v>
       </c>
       <c r="AC27" t="n">
-        <v>0.1892974227324384</v>
+        <v>0.2129597852336612</v>
       </c>
     </row>
     <row r="28">
@@ -3209,37 +3209,37 @@
         </is>
       </c>
       <c r="I28" t="n">
-        <v>2.05</v>
+        <v>2.1</v>
       </c>
       <c r="J28" t="n">
-        <v>2.9</v>
+        <v>3</v>
       </c>
       <c r="K28" t="n">
-        <v>4.5</v>
+        <v>4.1</v>
       </c>
       <c r="L28" t="n">
-        <v>0.4624379872430901</v>
+        <v>0.4520396912899669</v>
       </c>
       <c r="M28" t="n">
-        <v>0.3268958185683913</v>
+        <v>0.3164277839029768</v>
       </c>
       <c r="N28" t="n">
-        <v>0.2106661941885188</v>
+        <v>0.2315325248070562</v>
       </c>
       <c r="O28" t="n">
-        <v>0.05485468647789915</v>
+        <v>0.05342624854819977</v>
       </c>
       <c r="P28" t="n">
         <v>0</v>
       </c>
       <c r="Q28" t="n">
-        <v>0.6614556258167381</v>
+        <v>0.7167158389919541</v>
       </c>
       <c r="R28" t="n">
-        <v>0.1394727746837952</v>
+        <v>0.1384400058289361</v>
       </c>
       <c r="S28" t="n">
-        <v>0.1990715994994667</v>
+        <v>0.1448441551791098</v>
       </c>
       <c r="T28" t="n">
         <v>1</v>
@@ -3254,10 +3254,10 @@
         <v>0</v>
       </c>
       <c r="X28" t="n">
-        <v>0.6614556258167381</v>
+        <v>0.7167158389919541</v>
       </c>
       <c r="Y28" t="n">
-        <v>2.9</v>
+        <v>3</v>
       </c>
       <c r="Z28" t="inlineStr">
         <is>
@@ -3265,13 +3265,13 @@
         </is>
       </c>
       <c r="AA28" t="n">
-        <v>0.4832743762466003</v>
+        <v>0.5750737584879312</v>
       </c>
       <c r="AB28" t="n">
-        <v>5.953100632350642</v>
+        <v>6.450442550927587</v>
       </c>
       <c r="AC28" t="n">
-        <v>0.4623840263172714</v>
+        <v>0.5718716838128444</v>
       </c>
     </row>
     <row r="29">
@@ -3310,7 +3310,7 @@
         </is>
       </c>
       <c r="I29" t="n">
-        <v>3.1</v>
+        <v>3.2</v>
       </c>
       <c r="J29" t="n">
         <v>3</v>
@@ -3319,28 +3319,28 @@
         <v>2.45</v>
       </c>
       <c r="L29" t="n">
-        <v>0.303155289750464</v>
+        <v>0.2964905203711174</v>
       </c>
       <c r="M29" t="n">
-        <v>0.3132604660754795</v>
+        <v>0.3162565550625252</v>
       </c>
       <c r="N29" t="n">
-        <v>0.3835842441740565</v>
+        <v>0.3872529245663574</v>
       </c>
       <c r="O29" t="n">
-        <v>0.06407724380074598</v>
+        <v>0.05399659863945572</v>
       </c>
       <c r="P29" t="n">
         <v>1</v>
       </c>
       <c r="Q29" t="n">
-        <v>0.1035450147498123</v>
+        <v>0.1184186316431676</v>
       </c>
       <c r="R29" t="n">
-        <v>0.4729387563576554</v>
+        <v>0.5101677514658699</v>
       </c>
       <c r="S29" t="n">
-        <v>0.4235162288925323</v>
+        <v>0.3714136168909625</v>
       </c>
       <c r="T29" t="n">
         <v>1</v>
@@ -3351,10 +3351,10 @@
         <v>1</v>
       </c>
       <c r="X29" t="n">
-        <v>0.4729387563576554</v>
+        <v>0.5101677514658699</v>
       </c>
       <c r="Y29" t="n">
-        <v>3.1</v>
+        <v>3.2</v>
       </c>
       <c r="Z29" t="inlineStr">
         <is>
@@ -3362,13 +3362,13 @@
         </is>
       </c>
       <c r="AA29" t="n">
-        <v>0.2219572117660627</v>
+        <v>0.2875167294049017</v>
       </c>
       <c r="AB29" t="n">
-        <v>4.256448807218898</v>
+        <v>4.591509763192829</v>
       </c>
       <c r="AC29" t="n">
-        <v>0.04942252746512305</v>
+        <v>0.1387541345749074</v>
       </c>
     </row>
     <row r="30">
@@ -3431,13 +3431,13 @@
         <v>1</v>
       </c>
       <c r="Q30" t="n">
-        <v>0.3699671422892812</v>
+        <v>0.3872030766026331</v>
       </c>
       <c r="R30" t="n">
-        <v>0.556180457262347</v>
+        <v>0.5520427392022073</v>
       </c>
       <c r="S30" t="n">
-        <v>0.07385240044837173</v>
+        <v>0.06075418419515957</v>
       </c>
       <c r="T30" t="n">
         <v>1</v>
@@ -3448,7 +3448,7 @@
         <v>1</v>
       </c>
       <c r="X30" t="n">
-        <v>0.556180457262347</v>
+        <v>0.5520427392022073</v>
       </c>
       <c r="Y30" t="n">
         <v>1.73</v>
@@ -3459,13 +3459,13 @@
         </is>
       </c>
       <c r="AA30" t="n">
-        <v>-0.05179151909060236</v>
+        <v>-0.06159734408244039</v>
       </c>
       <c r="AB30" t="n">
-        <v>4.811285189190746</v>
+        <v>4.739018330841173</v>
       </c>
       <c r="AC30" t="n">
-        <v>0.1862133149730658</v>
+        <v>0.1648396625995742</v>
       </c>
     </row>
     <row r="31">
@@ -3504,37 +3504,37 @@
         </is>
       </c>
       <c r="I31" t="n">
-        <v>1.8</v>
+        <v>1.73</v>
       </c>
       <c r="J31" t="n">
-        <v>3.6</v>
+        <v>3.7</v>
       </c>
       <c r="K31" t="n">
-        <v>4.5</v>
+        <v>4.75</v>
       </c>
       <c r="L31" t="n">
-        <v>0.5263157894736842</v>
+        <v>0.5459176541848509</v>
       </c>
       <c r="M31" t="n">
-        <v>0.2631578947368421</v>
+        <v>0.2552533896594033</v>
       </c>
       <c r="N31" t="n">
-        <v>0.2105263157894737</v>
+        <v>0.1988289561557457</v>
       </c>
       <c r="O31" t="n">
-        <v>0.05555555555555558</v>
+        <v>0.05883126814066886</v>
       </c>
       <c r="P31" t="n">
         <v>1</v>
       </c>
       <c r="Q31" t="n">
-        <v>0.2891631517166968</v>
+        <v>0.2708224838681848</v>
       </c>
       <c r="R31" t="n">
-        <v>0.5562367657474598</v>
+        <v>0.5475848802625712</v>
       </c>
       <c r="S31" t="n">
-        <v>0.1546000825358435</v>
+        <v>0.181592635869244</v>
       </c>
       <c r="T31" t="n">
         <v>1</v>
@@ -3545,10 +3545,10 @@
         <v>1</v>
       </c>
       <c r="X31" t="n">
-        <v>0.5562367657474598</v>
+        <v>0.5475848802625712</v>
       </c>
       <c r="Y31" t="n">
-        <v>1.8</v>
+        <v>1.73</v>
       </c>
       <c r="Z31" t="inlineStr">
         <is>
@@ -3556,13 +3556,13 @@
         </is>
       </c>
       <c r="AA31" t="n">
-        <v>0.001532722931784636</v>
+        <v>-0.07216185910376952</v>
       </c>
       <c r="AB31" t="n">
-        <v>5.006130891727138</v>
+        <v>4.661799525683029</v>
       </c>
       <c r="AC31" t="n">
-        <v>0.2670736140307631</v>
+        <v>0.2767623963943864</v>
       </c>
     </row>
     <row r="32">
@@ -3625,13 +3625,13 @@
         <v>0</v>
       </c>
       <c r="Q32" t="n">
-        <v>0.7106253049137264</v>
+        <v>0.7222840509827422</v>
       </c>
       <c r="R32" t="n">
-        <v>0.2027533659066978</v>
+        <v>0.2003167806485436</v>
       </c>
       <c r="S32" t="n">
-        <v>0.08662132917957568</v>
+        <v>0.07739916836871434</v>
       </c>
       <c r="T32" t="n">
         <v>1</v>
@@ -3642,7 +3642,7 @@
         <v>0</v>
       </c>
       <c r="X32" t="n">
-        <v>0.7106253049137264</v>
+        <v>0.7222840509827422</v>
       </c>
       <c r="Y32" t="n">
         <v>3.3</v>
@@ -3653,13 +3653,13 @@
         </is>
       </c>
       <c r="AA32" t="n">
-        <v>0.5848102200936074</v>
+        <v>0.60153798619263</v>
       </c>
       <c r="AB32" t="n">
-        <v>6.395627744223538</v>
+        <v>6.50055645884468</v>
       </c>
       <c r="AC32" t="n">
-        <v>0.5078719390070286</v>
+        <v>0.5219672703341987</v>
       </c>
     </row>
     <row r="33">
@@ -3698,7 +3698,7 @@
         </is>
       </c>
       <c r="I33" t="n">
-        <v>5.75</v>
+        <v>6</v>
       </c>
       <c r="J33" t="n">
         <v>4.33</v>
@@ -3707,28 +3707,28 @@
         <v>1.53</v>
       </c>
       <c r="L33" t="n">
-        <v>0.1643084432253056</v>
+        <v>0.1585477050322006</v>
       </c>
       <c r="M33" t="n">
-        <v>0.2181925054377615</v>
+        <v>0.2196965889591694</v>
       </c>
       <c r="N33" t="n">
-        <v>0.6174990513369328</v>
+        <v>0.6217557060086298</v>
       </c>
       <c r="O33" t="n">
-        <v>0.05845469693718108</v>
+        <v>0.05120832012558685</v>
       </c>
       <c r="P33" t="n">
         <v>2</v>
       </c>
       <c r="Q33" t="n">
-        <v>0.2467260532398944</v>
+        <v>0.2033176799643781</v>
       </c>
       <c r="R33" t="n">
-        <v>0.1123909277918655</v>
+        <v>0.09848738387910269</v>
       </c>
       <c r="S33" t="n">
-        <v>0.6408830189682402</v>
+        <v>0.6981949361565192</v>
       </c>
       <c r="T33" t="n">
         <v>1</v>
@@ -3743,7 +3743,7 @@
         <v>2</v>
       </c>
       <c r="X33" t="n">
-        <v>0.6408830189682402</v>
+        <v>0.6981949361565192</v>
       </c>
       <c r="Y33" t="n">
         <v>1.53</v>
@@ -3754,13 +3754,13 @@
         </is>
       </c>
       <c r="AA33" t="n">
-        <v>-0.0366961905256462</v>
+        <v>0.1287514194707063</v>
       </c>
       <c r="AB33" t="n">
-        <v>5.609240974092252</v>
+        <v>6.283754425408673</v>
       </c>
       <c r="AC33" t="n">
-        <v>0.3941569657283458</v>
+        <v>0.4948772561921411</v>
       </c>
     </row>
     <row r="34">
@@ -3799,37 +3799,37 @@
         </is>
       </c>
       <c r="I34" t="n">
-        <v>2.3</v>
+        <v>2.4</v>
       </c>
       <c r="J34" t="n">
         <v>3.1</v>
       </c>
       <c r="K34" t="n">
-        <v>3.4</v>
+        <v>3.25</v>
       </c>
       <c r="L34" t="n">
-        <v>0.413495488426834</v>
+        <v>0.3979853841595892</v>
       </c>
       <c r="M34" t="n">
-        <v>0.3067869752844252</v>
+        <v>0.3081177167687142</v>
       </c>
       <c r="N34" t="n">
-        <v>0.2797175362887406</v>
+        <v>0.2938968990716966</v>
       </c>
       <c r="O34" t="n">
-        <v>0.05148090091576618</v>
+        <v>0.04693961952026471</v>
       </c>
       <c r="P34" t="n">
         <v>2</v>
       </c>
       <c r="Q34" t="n">
-        <v>0.3260635955815022</v>
+        <v>0.2802786529544899</v>
       </c>
       <c r="R34" t="n">
-        <v>0.2833968875176439</v>
+        <v>0.2609425121097187</v>
       </c>
       <c r="S34" t="n">
-        <v>0.3905395169008538</v>
+        <v>0.4587788349357912</v>
       </c>
       <c r="T34" t="n">
         <v>1</v>
@@ -3840,10 +3840,10 @@
         <v>2</v>
       </c>
       <c r="X34" t="n">
-        <v>0.3905395169008538</v>
+        <v>0.4587788349357912</v>
       </c>
       <c r="Y34" t="n">
-        <v>3.4</v>
+        <v>3.25</v>
       </c>
       <c r="Z34" t="inlineStr">
         <is>
@@ -3851,13 +3851,13 @@
         </is>
       </c>
       <c r="AA34" t="n">
-        <v>0.1365976489428761</v>
+        <v>0.218236094907254</v>
       </c>
       <c r="AB34" t="n">
-        <v>3.514855652107684</v>
+        <v>4.129009514422121</v>
       </c>
       <c r="AC34" t="n">
-        <v>0.06447592131935154</v>
+        <v>0.1785001819813012</v>
       </c>
     </row>
     <row r="35">
@@ -3896,37 +3896,37 @@
         </is>
       </c>
       <c r="I35" t="n">
-        <v>1.53</v>
+        <v>1.47</v>
       </c>
       <c r="J35" t="n">
-        <v>4.2</v>
+        <v>4.33</v>
       </c>
       <c r="K35" t="n">
         <v>6</v>
       </c>
       <c r="L35" t="n">
-        <v>0.6175562417291575</v>
+        <v>0.6311171356318823</v>
       </c>
       <c r="M35" t="n">
-        <v>0.2249669166299073</v>
+        <v>0.2142591661383065</v>
       </c>
       <c r="N35" t="n">
-        <v>0.1574768416409351</v>
+        <v>0.1546236982298112</v>
       </c>
       <c r="O35" t="n">
-        <v>0.05835667600373484</v>
+        <v>0.07788565772729417</v>
       </c>
       <c r="P35" t="n">
         <v>0</v>
       </c>
       <c r="Q35" t="n">
-        <v>0.4746091355359102</v>
+        <v>0.4910203864839924</v>
       </c>
       <c r="R35" t="n">
-        <v>0.4535711787054781</v>
+        <v>0.4484868303984901</v>
       </c>
       <c r="S35" t="n">
-        <v>0.0718196857586115</v>
+        <v>0.06049278311751746</v>
       </c>
       <c r="T35" t="n">
         <v>1</v>
@@ -3937,10 +3937,10 @@
         <v>0</v>
       </c>
       <c r="X35" t="n">
-        <v>0.4746091355359102</v>
+        <v>0.4910203864839924</v>
       </c>
       <c r="Y35" t="n">
-        <v>4.2</v>
+        <v>4.33</v>
       </c>
       <c r="Z35" t="inlineStr">
         <is>
@@ -3948,13 +3948,13 @@
         </is>
       </c>
       <c r="AA35" t="n">
-        <v>0.3104244903908822</v>
+        <v>0.3381736556984045</v>
       </c>
       <c r="AB35" t="n">
-        <v>4.271482219823191</v>
+        <v>4.419183478355931</v>
       </c>
       <c r="AC35" t="n">
-        <v>0.02103795683043208</v>
+        <v>0.04253355608550224</v>
       </c>
     </row>
     <row r="36">
@@ -3993,37 +3993,37 @@
         </is>
       </c>
       <c r="I36" t="n">
-        <v>3.4</v>
+        <v>3.6</v>
       </c>
       <c r="J36" t="n">
         <v>3.2</v>
       </c>
       <c r="K36" t="n">
-        <v>2.25</v>
+        <v>2.15</v>
       </c>
       <c r="L36" t="n">
-        <v>0.2798289933929266</v>
+        <v>0.2631981637337414</v>
       </c>
       <c r="M36" t="n">
-        <v>0.2973183054799844</v>
+        <v>0.296097934200459</v>
       </c>
       <c r="N36" t="n">
-        <v>0.4228527011270889</v>
+        <v>0.4407039020657995</v>
       </c>
       <c r="O36" t="n">
-        <v>0.05106209150326801</v>
+        <v>0.05539405684754528</v>
       </c>
       <c r="P36" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q36" t="n">
-        <v>0.2532324986954283</v>
+        <v>0.2239799965171629</v>
       </c>
       <c r="R36" t="n">
-        <v>0.4098687406457967</v>
+        <v>0.384892512986541</v>
       </c>
       <c r="S36" t="n">
-        <v>0.3368987606587751</v>
+        <v>0.3911274904962961</v>
       </c>
       <c r="T36" t="n">
         <v>1</v>
@@ -4031,13 +4031,13 @@
       <c r="U36" t="inlineStr"/>
       <c r="V36" t="inlineStr"/>
       <c r="W36" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="X36" t="n">
-        <v>0.4098687406457967</v>
+        <v>0.3911274904962961</v>
       </c>
       <c r="Y36" t="n">
-        <v>3.4</v>
+        <v>2.15</v>
       </c>
       <c r="Z36" t="inlineStr">
         <is>
@@ -4045,13 +4045,13 @@
         </is>
       </c>
       <c r="AA36" t="n">
-        <v>0.1639807159148786</v>
+        <v>-0.1383268655938812</v>
       </c>
       <c r="AB36" t="n">
-        <v>3.68881866581217</v>
+        <v>0.6312507591496797</v>
       </c>
       <c r="AC36" t="n">
-        <v>0.07296997998702159</v>
+        <v>0.006234977509755102</v>
       </c>
     </row>
     <row r="37">
@@ -4090,37 +4090,37 @@
         </is>
       </c>
       <c r="I37" t="n">
-        <v>2.55</v>
+        <v>2.6</v>
       </c>
       <c r="J37" t="n">
         <v>3.3</v>
       </c>
       <c r="K37" t="n">
-        <v>2.8</v>
+        <v>2.75</v>
       </c>
       <c r="L37" t="n">
-        <v>0.3726557773744706</v>
+        <v>0.3658536585365854</v>
       </c>
       <c r="M37" t="n">
-        <v>0.2879612825166364</v>
+        <v>0.2882483370288249</v>
       </c>
       <c r="N37" t="n">
-        <v>0.3393829401088929</v>
+        <v>0.3458980044345898</v>
       </c>
       <c r="O37" t="n">
-        <v>0.05233002291825839</v>
+        <v>0.0512820512820511</v>
       </c>
       <c r="P37" t="n">
         <v>1</v>
       </c>
       <c r="Q37" t="n">
-        <v>0.2406013581651952</v>
+        <v>0.2438487323413399</v>
       </c>
       <c r="R37" t="n">
-        <v>0.5148666709604525</v>
+        <v>0.5174982380748462</v>
       </c>
       <c r="S37" t="n">
-        <v>0.2445319708743524</v>
+        <v>0.238653029583814</v>
       </c>
       <c r="T37" t="n">
         <v>1</v>
@@ -4135,10 +4135,10 @@
         <v>1</v>
       </c>
       <c r="X37" t="n">
-        <v>0.5148666709604525</v>
+        <v>0.5174982380748462</v>
       </c>
       <c r="Y37" t="n">
-        <v>2.55</v>
+        <v>2.6</v>
       </c>
       <c r="Z37" t="inlineStr">
         <is>
@@ -4146,13 +4146,13 @@
         </is>
       </c>
       <c r="AA37" t="n">
-        <v>0.2018774264188089</v>
+        <v>0.2159346368716251</v>
       </c>
       <c r="AB37" t="n">
-        <v>4.633800038644072</v>
+        <v>4.657484142673615</v>
       </c>
       <c r="AC37" t="n">
-        <v>0.2703347000861001</v>
+        <v>0.2736495057335063</v>
       </c>
     </row>
     <row r="38">
@@ -4191,37 +4191,37 @@
         </is>
       </c>
       <c r="I38" t="n">
+        <v>2.9</v>
+      </c>
+      <c r="J38" t="n">
         <v>3</v>
       </c>
-      <c r="J38" t="n">
-        <v>3.1</v>
-      </c>
       <c r="K38" t="n">
-        <v>2.5</v>
+        <v>2.63</v>
       </c>
       <c r="L38" t="n">
-        <v>0.3156822810590631</v>
+        <v>0.3258041871412644</v>
       </c>
       <c r="M38" t="n">
-        <v>0.3054989816700611</v>
+        <v>0.3149440475698889</v>
       </c>
       <c r="N38" t="n">
-        <v>0.3788187372708758</v>
+        <v>0.3592517652888467</v>
       </c>
       <c r="O38" t="n">
-        <v>0.05591397849462365</v>
+        <v>0.05838905642235925</v>
       </c>
       <c r="P38" t="n">
         <v>1</v>
       </c>
       <c r="Q38" t="n">
-        <v>0.2655474608194406</v>
+        <v>0.267936947658205</v>
       </c>
       <c r="R38" t="n">
-        <v>0.4144767249509805</v>
+        <v>0.4116964593526058</v>
       </c>
       <c r="S38" t="n">
-        <v>0.3199758142295789</v>
+        <v>0.3203665929891891</v>
       </c>
       <c r="T38" t="n">
         <v>1</v>
@@ -4236,10 +4236,10 @@
         <v>1</v>
       </c>
       <c r="X38" t="n">
-        <v>0.4144767249509805</v>
+        <v>0.4116964593526058</v>
       </c>
       <c r="Y38" t="n">
-        <v>3</v>
+        <v>2.9</v>
       </c>
       <c r="Z38" t="inlineStr">
         <is>
@@ -4247,13 +4247,13 @@
         </is>
       </c>
       <c r="AA38" t="n">
-        <v>0.1217150874264707</v>
+        <v>0.1020630169066088</v>
       </c>
       <c r="AB38" t="n">
-        <v>4.973720699411765</v>
+        <v>4.94035751223127</v>
       </c>
       <c r="AC38" t="n">
-        <v>0.0945009107214016</v>
+        <v>0.09132986636341672</v>
       </c>
     </row>
     <row r="39">
@@ -4316,13 +4316,13 @@
         <v>0</v>
       </c>
       <c r="Q39" t="n">
-        <v>0.6299576099454309</v>
+        <v>0.6223252482249096</v>
       </c>
       <c r="R39" t="n">
-        <v>0.06051569283369836</v>
+        <v>0.06565688348210923</v>
       </c>
       <c r="S39" t="n">
-        <v>0.3095266972208707</v>
+        <v>0.3120178682929812</v>
       </c>
       <c r="T39" t="n">
         <v>1</v>
@@ -4337,7 +4337,7 @@
         <v>0</v>
       </c>
       <c r="X39" t="n">
-        <v>0.6299576099454309</v>
+        <v>0.6223252482249096</v>
       </c>
       <c r="Y39" t="n">
         <v>3.8</v>
@@ -4348,13 +4348,13 @@
         </is>
       </c>
       <c r="AA39" t="n">
-        <v>0.4977996134973705</v>
+        <v>0.4874414083052345</v>
       </c>
       <c r="AB39" t="n">
-        <v>7.559491319345171</v>
+        <v>7.467902978698915</v>
       </c>
       <c r="AC39" t="n">
-        <v>0.3204309127245602</v>
+        <v>0.3103073799319284</v>
       </c>
     </row>
     <row r="40">
@@ -4417,13 +4417,13 @@
         <v>1</v>
       </c>
       <c r="Q40" t="n">
-        <v>0.06410954081048939</v>
+        <v>0.06305896439045974</v>
       </c>
       <c r="R40" t="n">
-        <v>0.5419457153633681</v>
+        <v>0.5442267033629983</v>
       </c>
       <c r="S40" t="n">
-        <v>0.3939447438261424</v>
+        <v>0.3927143322465419</v>
       </c>
       <c r="T40" t="n">
         <v>1</v>
@@ -4438,7 +4438,7 @@
         <v>1</v>
       </c>
       <c r="X40" t="n">
-        <v>0.5419457153633681</v>
+        <v>0.5442267033629983</v>
       </c>
       <c r="Y40" t="n">
         <v>1.8</v>
@@ -4449,13 +4449,13 @@
         </is>
       </c>
       <c r="AA40" t="n">
-        <v>-0.03062214043242174</v>
+        <v>-0.02548991743325388</v>
       </c>
       <c r="AB40" t="n">
-        <v>6.35401499929156</v>
+        <v>6.405885004519023</v>
       </c>
       <c r="AC40" t="n">
-        <v>0.1480009715372257</v>
+        <v>0.1515123711164564</v>
       </c>
     </row>
     <row r="41">
@@ -4500,31 +4500,31 @@
         <v>3.75</v>
       </c>
       <c r="K41" t="n">
-        <v>2.15</v>
+        <v>2.2</v>
       </c>
       <c r="L41" t="n">
-        <v>0.3059482022578503</v>
+        <v>0.3090466379471811</v>
       </c>
       <c r="M41" t="n">
-        <v>0.2529171805331563</v>
+        <v>0.2554785540363364</v>
       </c>
       <c r="N41" t="n">
-        <v>0.4411346172089934</v>
+        <v>0.4354748080164825</v>
       </c>
       <c r="O41" t="n">
-        <v>0.05436359089772447</v>
+        <v>0.04379276637341145</v>
       </c>
       <c r="P41" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="Q41" t="n">
-        <v>0.4740318563340223</v>
+        <v>0.5407223332703381</v>
       </c>
       <c r="R41" t="n">
-        <v>0.0422186367089571</v>
+        <v>0.02048135744957176</v>
       </c>
       <c r="S41" t="n">
-        <v>0.4837495069570206</v>
+        <v>0.4387963092800902</v>
       </c>
       <c r="T41" t="n">
         <v>1</v>
@@ -4536,13 +4536,13 @@
         <v>0</v>
       </c>
       <c r="W41" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="X41" t="n">
-        <v>0.4837495069570206</v>
+        <v>0.5407223332703381</v>
       </c>
       <c r="Y41" t="n">
-        <v>2.15</v>
+        <v>3.75</v>
       </c>
       <c r="Z41" t="inlineStr">
         <is>
@@ -4550,13 +4550,13 @@
         </is>
       </c>
       <c r="AA41" t="n">
-        <v>0.03483603474573414</v>
+        <v>0.3737122726413702</v>
       </c>
       <c r="AB41" t="n">
-        <v>1.160998816696849</v>
+        <v>6.488667999244058</v>
       </c>
       <c r="AC41" t="n">
-        <v>0.009717650622998342</v>
+        <v>0.1019260239902479</v>
       </c>
     </row>
     <row r="42">
@@ -4619,13 +4619,13 @@
         <v>0</v>
       </c>
       <c r="Q42" t="n">
-        <v>0.6153624267756741</v>
+        <v>0.5940716441516797</v>
       </c>
       <c r="R42" t="n">
-        <v>0.1146847408456869</v>
+        <v>0.1320526964909443</v>
       </c>
       <c r="S42" t="n">
-        <v>0.269952832378639</v>
+        <v>0.273875659357376</v>
       </c>
       <c r="T42" t="n">
         <v>1</v>
@@ -4640,7 +4640,7 @@
         <v>0</v>
       </c>
       <c r="X42" t="n">
-        <v>0.6153624267756741</v>
+        <v>0.5940716441516797</v>
       </c>
       <c r="Y42" t="n">
         <v>3.5</v>
@@ -4651,13 +4651,13 @@
         </is>
       </c>
       <c r="AA42" t="n">
-        <v>0.4615073974859437</v>
+        <v>0.4317003018123515</v>
       </c>
       <c r="AB42" t="n">
-        <v>7.384349121308089</v>
+        <v>7.128859729820156</v>
       </c>
       <c r="AC42" t="n">
-        <v>0.3454095943970351</v>
+        <v>0.3201959847943037</v>
       </c>
     </row>
     <row r="43">
@@ -4696,37 +4696,37 @@
         </is>
       </c>
       <c r="I43" t="n">
-        <v>3.75</v>
+        <v>3.8</v>
       </c>
       <c r="J43" t="n">
-        <v>3.25</v>
+        <v>3.3</v>
       </c>
       <c r="K43" t="n">
-        <v>2.1</v>
+        <v>2.05</v>
       </c>
       <c r="L43" t="n">
-        <v>0.2538354253835426</v>
+        <v>0.2496770621885956</v>
       </c>
       <c r="M43" t="n">
-        <v>0.292887029288703</v>
+        <v>0.2875069200959586</v>
       </c>
       <c r="N43" t="n">
-        <v>0.4532775453277546</v>
+        <v>0.4628160177154457</v>
       </c>
       <c r="O43" t="n">
-        <v>0.05054945054945037</v>
+        <v>0.05399307581592572</v>
       </c>
       <c r="P43" t="n">
         <v>2</v>
       </c>
       <c r="Q43" t="n">
-        <v>0.1817550803098659</v>
+        <v>0.1771779863417773</v>
       </c>
       <c r="R43" t="n">
-        <v>0.2118499037001081</v>
+        <v>0.2176355164598661</v>
       </c>
       <c r="S43" t="n">
-        <v>0.6063950159900261</v>
+        <v>0.6051864971983566</v>
       </c>
       <c r="T43" t="n">
         <v>1</v>
@@ -4741,10 +4741,10 @@
         <v>2</v>
       </c>
       <c r="X43" t="n">
-        <v>0.6063950159900261</v>
+        <v>0.6051864971983566</v>
       </c>
       <c r="Y43" t="n">
-        <v>2.1</v>
+        <v>2.05</v>
       </c>
       <c r="Z43" t="inlineStr">
         <is>
@@ -4752,13 +4752,13 @@
         </is>
       </c>
       <c r="AA43" t="n">
-        <v>0.2485723032536862</v>
+        <v>0.2291736373872675</v>
       </c>
       <c r="AB43" t="n">
-        <v>7.276740191880313</v>
+        <v>7.262237966380279</v>
       </c>
       <c r="AC43" t="n">
-        <v>0.394545112289918</v>
+        <v>0.3875509807384905</v>
       </c>
     </row>
     <row r="44">
@@ -4821,13 +4821,13 @@
         <v>1</v>
       </c>
       <c r="Q44" t="n">
-        <v>0.2742914879005598</v>
+        <v>0.3122676554976557</v>
       </c>
       <c r="R44" t="n">
-        <v>0.4027392557450454</v>
+        <v>0.3598673628301626</v>
       </c>
       <c r="S44" t="n">
-        <v>0.3229692563543948</v>
+        <v>0.3278649816721817</v>
       </c>
       <c r="T44" t="n">
         <v>1</v>
@@ -4842,7 +4842,7 @@
         <v>1</v>
       </c>
       <c r="X44" t="n">
-        <v>0.4027392557450454</v>
+        <v>0.3598673628301626</v>
       </c>
       <c r="Y44" t="n">
         <v>2.9</v>
@@ -4853,13 +4853,13 @@
         </is>
       </c>
       <c r="AA44" t="n">
-        <v>0.08839149561085879</v>
+        <v>0.02295544853024821</v>
       </c>
       <c r="AB44" t="n">
-        <v>4.832871068940546</v>
+        <v>0.8636816707923904</v>
       </c>
       <c r="AC44" t="n">
-        <v>0.0797699993906506</v>
+        <v>0.03200238115798093</v>
       </c>
     </row>
     <row r="45">
@@ -4922,13 +4922,13 @@
         <v>1</v>
       </c>
       <c r="Q45" t="n">
-        <v>0.1393064091929172</v>
+        <v>0.1286747274268642</v>
       </c>
       <c r="R45" t="n">
-        <v>0.4639527036901374</v>
+        <v>0.4804991551076898</v>
       </c>
       <c r="S45" t="n">
-        <v>0.3967408871169454</v>
+        <v>0.3908261174654459</v>
       </c>
       <c r="T45" t="n">
         <v>1</v>
@@ -4943,7 +4943,7 @@
         <v>1</v>
       </c>
       <c r="X45" t="n">
-        <v>0.4639527036901374</v>
+        <v>0.4804991551076898</v>
       </c>
       <c r="Y45" t="n">
         <v>2.25</v>
@@ -4954,13 +4954,13 @@
         </is>
       </c>
       <c r="AA45" t="n">
-        <v>0.0351148666422473</v>
+        <v>0.06489847919384166</v>
       </c>
       <c r="AB45" t="n">
-        <v>5.567432444281648</v>
+        <v>5.765989861292278</v>
       </c>
       <c r="AC45" t="n">
-        <v>0.06721181657319203</v>
+        <v>0.08967303764224388</v>
       </c>
     </row>
     <row r="46">
@@ -5020,16 +5020,16 @@
         <v>0.05591397849462365</v>
       </c>
       <c r="P46" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q46" t="n">
-        <v>0.1784299249024006</v>
+        <v>0.4374837775420963</v>
       </c>
       <c r="R46" t="n">
-        <v>0.4863827909499324</v>
+        <v>0.1987897810781952</v>
       </c>
       <c r="S46" t="n">
-        <v>0.335187284147667</v>
+        <v>0.3637264413797086</v>
       </c>
       <c r="T46" t="n">
         <v>1</v>
@@ -5041,13 +5041,13 @@
         <v>0</v>
       </c>
       <c r="W46" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X46" t="n">
-        <v>0.4863827909499324</v>
+        <v>0.4374837775420963</v>
       </c>
       <c r="Y46" t="n">
-        <v>2.5</v>
+        <v>3</v>
       </c>
       <c r="Z46" t="inlineStr">
         <is>
@@ -5055,13 +5055,13 @@
         </is>
       </c>
       <c r="AA46" t="n">
-        <v>0.1439713182498873</v>
+        <v>0.1562256663131444</v>
       </c>
       <c r="AB46" t="n">
-        <v>5.836593491399188</v>
+        <v>5.249805330505155</v>
       </c>
       <c r="AC46" t="n">
-        <v>0.1511955068022653</v>
+        <v>0.07375733616238767</v>
       </c>
     </row>
     <row r="47">
@@ -5124,13 +5124,13 @@
         <v>2</v>
       </c>
       <c r="Q47" t="n">
-        <v>0.1500320611963141</v>
+        <v>0.1791811289736883</v>
       </c>
       <c r="R47" t="n">
-        <v>0.4005985816376548</v>
+        <v>0.3587487226001629</v>
       </c>
       <c r="S47" t="n">
-        <v>0.4493693571660312</v>
+        <v>0.4620701484261488</v>
       </c>
       <c r="T47" t="n">
         <v>1</v>
@@ -5145,7 +5145,7 @@
         <v>2</v>
       </c>
       <c r="X47" t="n">
-        <v>0.4493693571660312</v>
+        <v>0.4620701484261488</v>
       </c>
       <c r="Y47" t="n">
         <v>2.2</v>
@@ -5156,13 +5156,13 @@
         </is>
       </c>
       <c r="AA47" t="n">
-        <v>-0.009489511862276199</v>
+        <v>0.01379527211460618</v>
       </c>
       <c r="AB47" t="n">
-        <v>5.354054271376652</v>
+        <v>5.544841781113786</v>
       </c>
       <c r="AC47" t="n">
-        <v>0.04877077552837639</v>
+        <v>0.1033214258259859</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualizo predicciones x stake con k mayores en kelly_linear
</commit_message>
<xml_diff>
--- a/data/predicciones.xlsx
+++ b/data/predicciones.xlsx
@@ -644,13 +644,13 @@
         <v>1</v>
       </c>
       <c r="Q2" t="n">
-        <v>0.3025965320267902</v>
+        <v>0.3220982557844255</v>
       </c>
       <c r="R2" t="n">
-        <v>0.5624221891434038</v>
+        <v>0.5574080400394626</v>
       </c>
       <c r="S2" t="n">
-        <v>0.134981278829806</v>
+        <v>0.1204937041761118</v>
       </c>
       <c r="T2" t="n">
         <v>1</v>
@@ -665,7 +665,7 @@
         <v>1</v>
       </c>
       <c r="X2" t="n">
-        <v>0.5624221891434038</v>
+        <v>0.5574080400394626</v>
       </c>
       <c r="Y2" t="n">
         <v>1.44</v>
@@ -676,33 +676,33 @@
         </is>
       </c>
       <c r="AA2" t="n">
-        <v>-0.4320728355306785</v>
+        <v>-0.4484827780526678</v>
       </c>
       <c r="AB2" t="n">
-        <v>3.334870272763151</v>
+        <v>2.303382926642866</v>
       </c>
       <c r="AC2" t="n">
-        <v>0.2598256571166136</v>
+        <v>0.2353097842550371</v>
       </c>
       <c r="AD2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>nXEvvsgg</t>
+          <t>QHQVu3Ot</t>
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>45748.65625</v>
+        <v>45748.66666666666</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>wolves</t>
+          <t>nottingham</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>west ham</t>
+          <t>manchester utd</t>
         </is>
       </c>
       <c r="E3" t="n">
@@ -722,40 +722,40 @@
         </is>
       </c>
       <c r="I3" t="n">
-        <v>2.38</v>
+        <v>2.1</v>
       </c>
       <c r="J3" t="n">
-        <v>3.3</v>
+        <v>3.6</v>
       </c>
       <c r="K3" t="n">
-        <v>3</v>
+        <v>3.2</v>
       </c>
       <c r="L3" t="n">
-        <v>0.3976861894432394</v>
+        <v>0.4465116279069767</v>
       </c>
       <c r="M3" t="n">
-        <v>0.2868161002651242</v>
+        <v>0.2604651162790698</v>
       </c>
       <c r="N3" t="n">
-        <v>0.3154977102916365</v>
+        <v>0.2930232558139535</v>
       </c>
       <c r="O3" t="n">
-        <v>0.05653170359052706</v>
+        <v>0.06646825396825395</v>
       </c>
       <c r="P3" t="n">
         <v>1</v>
       </c>
       <c r="Q3" t="n">
-        <v>0.3461204410077632</v>
+        <v>0.3342487223805388</v>
       </c>
       <c r="R3" t="n">
-        <v>0.2638586657009028</v>
+        <v>0.3653799272175192</v>
       </c>
       <c r="S3" t="n">
-        <v>0.3900208932913339</v>
+        <v>0.300371350401942</v>
       </c>
       <c r="T3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="U3" t="n">
         <v>1</v>
@@ -764,13 +764,13 @@
         <v>0</v>
       </c>
       <c r="W3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="X3" t="n">
-        <v>0.3900208932913339</v>
+        <v>0.3653799272175192</v>
       </c>
       <c r="Y3" t="n">
-        <v>3</v>
+        <v>2.1</v>
       </c>
       <c r="Z3" t="inlineStr">
         <is>
@@ -778,33 +778,33 @@
         </is>
       </c>
       <c r="AA3" t="n">
-        <v>0.0850313399370009</v>
+        <v>-0.2115474116756452</v>
       </c>
       <c r="AB3" t="n">
-        <v>3.90020893291334</v>
+        <v>2.531780884303292</v>
       </c>
       <c r="AC3" t="n">
-        <v>0.0439004522835707</v>
+        <v>0.03113120483698034</v>
       </c>
       <c r="AD3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>QHQVu3Ot</t>
+          <t>6Dg5Psv0</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>45748.66666666666</v>
+        <v>45749.65625</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>nottingham</t>
+          <t>bournemouth</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>manchester utd</t>
+          <t>ipswich</t>
         </is>
       </c>
       <c r="E4" t="n">
@@ -824,37 +824,37 @@
         </is>
       </c>
       <c r="I4" t="n">
-        <v>2.1</v>
+        <v>1.36</v>
       </c>
       <c r="J4" t="n">
-        <v>3.6</v>
+        <v>4.75</v>
       </c>
       <c r="K4" t="n">
-        <v>3.2</v>
+        <v>8</v>
       </c>
       <c r="L4" t="n">
-        <v>0.4465116279069767</v>
+        <v>0.6866642573183954</v>
       </c>
       <c r="M4" t="n">
-        <v>0.2604651162790698</v>
+        <v>0.1966028189374774</v>
       </c>
       <c r="N4" t="n">
-        <v>0.2930232558139535</v>
+        <v>0.1167329237441272</v>
       </c>
       <c r="O4" t="n">
-        <v>0.06646825396825395</v>
+        <v>0.07082043343653233</v>
       </c>
       <c r="P4" t="n">
         <v>1</v>
       </c>
       <c r="Q4" t="n">
-        <v>0.3307108072574522</v>
+        <v>0.2967323091995783</v>
       </c>
       <c r="R4" t="n">
-        <v>0.3763659991830028</v>
+        <v>0.5662795590494977</v>
       </c>
       <c r="S4" t="n">
-        <v>0.2929231935595449</v>
+        <v>0.1369881317509239</v>
       </c>
       <c r="T4" t="n">
         <v>1</v>
@@ -869,10 +869,10 @@
         <v>1</v>
       </c>
       <c r="X4" t="n">
-        <v>0.3763659991830028</v>
+        <v>0.5662795590494977</v>
       </c>
       <c r="Y4" t="n">
-        <v>2.1</v>
+        <v>1.36</v>
       </c>
       <c r="Z4" t="inlineStr">
         <is>
@@ -880,20 +880,20 @@
         </is>
       </c>
       <c r="AA4" t="n">
-        <v>-0.1905740015597218</v>
+        <v>-0.6384994435907863</v>
       </c>
       <c r="AB4" t="n">
-        <v>3.05496313557024</v>
+        <v>1.453802744018047</v>
       </c>
       <c r="AC4" t="n">
-        <v>0.04565519192555056</v>
+        <v>0.2695472498499193</v>
       </c>
       <c r="AD4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>6Dg5Psv0</t>
+          <t>UF6ezahI</t>
         </is>
       </c>
       <c r="B5" s="2" t="n">
@@ -901,12 +901,12 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>bournemouth</t>
+          <t>manchester city</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>ipswich</t>
+          <t>leicester</t>
         </is>
       </c>
       <c r="E5" t="n">
@@ -926,37 +926,37 @@
         </is>
       </c>
       <c r="I5" t="n">
-        <v>1.36</v>
+        <v>1.17</v>
       </c>
       <c r="J5" t="n">
-        <v>4.75</v>
+        <v>7</v>
       </c>
       <c r="K5" t="n">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="L5" t="n">
-        <v>0.6866642573183954</v>
+        <v>0.8031206975676917</v>
       </c>
       <c r="M5" t="n">
-        <v>0.1966028189374774</v>
+        <v>0.1342358880220285</v>
       </c>
       <c r="N5" t="n">
-        <v>0.1167329237441272</v>
+        <v>0.06264341441027994</v>
       </c>
       <c r="O5" t="n">
-        <v>0.07082043343653233</v>
+        <v>0.06422466422466422</v>
       </c>
       <c r="P5" t="n">
         <v>1</v>
       </c>
       <c r="Q5" t="n">
-        <v>0.2938631453750061</v>
+        <v>0.2362524679636548</v>
       </c>
       <c r="R5" t="n">
-        <v>0.5647431655997508</v>
+        <v>0.7102530749933007</v>
       </c>
       <c r="S5" t="n">
-        <v>0.1413936890252431</v>
+        <v>0.05349445704304451</v>
       </c>
       <c r="T5" t="n">
         <v>1</v>
@@ -971,10 +971,10 @@
         <v>1</v>
       </c>
       <c r="X5" t="n">
-        <v>0.5647431655997508</v>
+        <v>0.7102530749933007</v>
       </c>
       <c r="Y5" t="n">
-        <v>1.36</v>
+        <v>1.17</v>
       </c>
       <c r="Z5" t="inlineStr">
         <is>
@@ -982,20 +982,20 @@
         </is>
       </c>
       <c r="AA5" t="n">
-        <v>-0.6443035966231634</v>
+        <v>-0.9941406015166959</v>
       </c>
       <c r="AB5" t="n">
-        <v>2.440691777609503</v>
+        <v>0.6850581941077486</v>
       </c>
       <c r="AC5" t="n">
-        <v>0.2708800202247447</v>
+        <v>0.4740006070296459</v>
       </c>
       <c r="AD5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>zgoMLawP</t>
+          <t>2T43YxNU</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
@@ -1003,12 +1003,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>brighton</t>
+          <t>newcastle</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>aston villa</t>
+          <t>brentford</t>
         </is>
       </c>
       <c r="E6" t="n">
@@ -1028,40 +1028,40 @@
         </is>
       </c>
       <c r="I6" t="n">
-        <v>2</v>
+        <v>1.67</v>
       </c>
       <c r="J6" t="n">
+        <v>4.75</v>
+      </c>
+      <c r="K6" t="n">
         <v>4</v>
       </c>
-      <c r="K6" t="n">
-        <v>3.2</v>
-      </c>
       <c r="L6" t="n">
-        <v>0.4705882352941176</v>
+        <v>0.5652658981033842</v>
       </c>
       <c r="M6" t="n">
-        <v>0.2352941176470588</v>
+        <v>0.1987355894384529</v>
       </c>
       <c r="N6" t="n">
-        <v>0.2941176470588235</v>
+        <v>0.2359985124581629</v>
       </c>
       <c r="O6" t="n">
-        <v>0.0625</v>
+        <v>0.05932871099905457</v>
       </c>
       <c r="P6" t="n">
         <v>1</v>
       </c>
       <c r="Q6" t="n">
-        <v>0.3364123207185839</v>
+        <v>0.3059273246456057</v>
       </c>
       <c r="R6" t="n">
-        <v>0.2864325651263231</v>
+        <v>0.5742505050190818</v>
       </c>
       <c r="S6" t="n">
-        <v>0.3771551141550931</v>
+        <v>0.1198221703353124</v>
       </c>
       <c r="T6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="U6" t="n">
         <v>1</v>
@@ -1070,13 +1070,13 @@
         <v>0</v>
       </c>
       <c r="W6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="X6" t="n">
-        <v>0.3771551141550931</v>
+        <v>0.5742505050190818</v>
       </c>
       <c r="Y6" t="n">
-        <v>3.2</v>
+        <v>1.67</v>
       </c>
       <c r="Z6" t="inlineStr">
         <is>
@@ -1084,33 +1084,33 @@
         </is>
       </c>
       <c r="AA6" t="n">
-        <v>0.0940438024074081</v>
+        <v>-0.06119650241512453</v>
       </c>
       <c r="AB6" t="n">
-        <v>3.771551141550931</v>
+        <v>5.216848826814816</v>
       </c>
       <c r="AC6" t="n">
-        <v>0.04074279343650916</v>
+        <v>0.2683231803734761</v>
       </c>
       <c r="AD6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>UF6ezahI</t>
+          <t>UXkVSb0b</t>
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>45749.65625</v>
+        <v>45749.66666666666</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>manchester city</t>
+          <t>liverpool</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>leicester</t>
+          <t>everton</t>
         </is>
       </c>
       <c r="E7" t="n">
@@ -1130,37 +1130,37 @@
         </is>
       </c>
       <c r="I7" t="n">
-        <v>1.17</v>
+        <v>1.4</v>
       </c>
       <c r="J7" t="n">
-        <v>7</v>
+        <v>4.5</v>
       </c>
       <c r="K7" t="n">
-        <v>15</v>
+        <v>8.5</v>
       </c>
       <c r="L7" t="n">
-        <v>0.8031206975676917</v>
+        <v>0.6775907883082374</v>
       </c>
       <c r="M7" t="n">
-        <v>0.1342358880220285</v>
+        <v>0.2108060230292294</v>
       </c>
       <c r="N7" t="n">
-        <v>0.06264341441027994</v>
+        <v>0.1116031886625332</v>
       </c>
       <c r="O7" t="n">
-        <v>0.06422466422466422</v>
+        <v>0.05415499533146595</v>
       </c>
       <c r="P7" t="n">
         <v>1</v>
       </c>
       <c r="Q7" t="n">
-        <v>0.217407962995375</v>
+        <v>0.2806571112202151</v>
       </c>
       <c r="R7" t="n">
-        <v>0.7235640892666777</v>
+        <v>0.6335197493837517</v>
       </c>
       <c r="S7" t="n">
-        <v>0.05902794773794733</v>
+        <v>0.08582313939603335</v>
       </c>
       <c r="T7" t="n">
         <v>1</v>
@@ -1175,10 +1175,10 @@
         <v>1</v>
       </c>
       <c r="X7" t="n">
-        <v>0.7235640892666777</v>
+        <v>0.6335197493837517</v>
       </c>
       <c r="Y7" t="n">
-        <v>1.17</v>
+        <v>1.4</v>
       </c>
       <c r="Z7" t="inlineStr">
         <is>
@@ -1186,33 +1186,33 @@
         </is>
       </c>
       <c r="AA7" t="n">
-        <v>-0.9025295032822777</v>
+        <v>-0.2826808771568695</v>
       </c>
       <c r="AB7" t="n">
-        <v>2.043871025945572</v>
+        <v>3.7991371173304</v>
       </c>
       <c r="AC7" t="n">
-        <v>0.5061561262713028</v>
+        <v>0.3528626381635366</v>
       </c>
       <c r="AD7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
         <is>
-          <t>2T43YxNU</t>
+          <t>nXEvvsgg</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>45749.65625</v>
+        <v>45748.65625</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>newcastle</t>
+          <t>wolves</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>brentford</t>
+          <t>west ham</t>
         </is>
       </c>
       <c r="E8" t="n">
@@ -1232,40 +1232,40 @@
         </is>
       </c>
       <c r="I8" t="n">
-        <v>1.67</v>
+        <v>2.38</v>
       </c>
       <c r="J8" t="n">
-        <v>4.75</v>
+        <v>3.3</v>
       </c>
       <c r="K8" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L8" t="n">
-        <v>0.5652658981033842</v>
+        <v>0.3976861894432394</v>
       </c>
       <c r="M8" t="n">
-        <v>0.1987355894384529</v>
+        <v>0.2868161002651242</v>
       </c>
       <c r="N8" t="n">
-        <v>0.2359985124581629</v>
+        <v>0.3154977102916365</v>
       </c>
       <c r="O8" t="n">
-        <v>0.05932871099905457</v>
+        <v>0.05653170359052706</v>
       </c>
       <c r="P8" t="n">
         <v>1</v>
       </c>
       <c r="Q8" t="n">
-        <v>0.3012726570292144</v>
+        <v>0.3532584439150531</v>
       </c>
       <c r="R8" t="n">
-        <v>0.563787620538173</v>
+        <v>0.2468355864359062</v>
       </c>
       <c r="S8" t="n">
-        <v>0.1349397224326127</v>
+        <v>0.3999059696490407</v>
       </c>
       <c r="T8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="U8" t="n">
         <v>1</v>
@@ -1274,13 +1274,13 @@
         <v>0</v>
       </c>
       <c r="W8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="X8" t="n">
-        <v>0.563787620538173</v>
+        <v>0.3999059696490407</v>
       </c>
       <c r="Y8" t="n">
-        <v>1.67</v>
+        <v>3</v>
       </c>
       <c r="Z8" t="inlineStr">
         <is>
@@ -1288,20 +1288,20 @@
         </is>
       </c>
       <c r="AA8" t="n">
-        <v>-0.0872756323899271</v>
+        <v>0.09985895447356113</v>
       </c>
       <c r="AB8" t="n">
-        <v>5.147072518330932</v>
+        <v>3.999059696490407</v>
       </c>
       <c r="AC8" t="n">
-        <v>0.2625149635089586</v>
+        <v>0.04664752573398767</v>
       </c>
       <c r="AD8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
         <is>
-          <t>xQXNUKVo</t>
+          <t>zgoMLawP</t>
         </is>
       </c>
       <c r="B9" s="2" t="n">
@@ -1309,12 +1309,12 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>southampton</t>
+          <t>brighton</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>crystal palace</t>
+          <t>aston villa</t>
         </is>
       </c>
       <c r="E9" t="n">
@@ -1334,37 +1334,37 @@
         </is>
       </c>
       <c r="I9" t="n">
-        <v>5.5</v>
+        <v>2</v>
       </c>
       <c r="J9" t="n">
-        <v>3.75</v>
+        <v>4</v>
       </c>
       <c r="K9" t="n">
-        <v>1.62</v>
+        <v>3.2</v>
       </c>
       <c r="L9" t="n">
-        <v>0.1705981465880371</v>
+        <v>0.4705882352941176</v>
       </c>
       <c r="M9" t="n">
-        <v>0.2502106149957877</v>
+        <v>0.2352941176470588</v>
       </c>
       <c r="N9" t="n">
-        <v>0.5791912384161753</v>
+        <v>0.2941176470588235</v>
       </c>
       <c r="O9" t="n">
-        <v>0.06576879910213229</v>
+        <v>0.0625</v>
       </c>
       <c r="P9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q9" t="n">
-        <v>0.3348935851715886</v>
+        <v>0.3030295671751106</v>
       </c>
       <c r="R9" t="n">
-        <v>0.1759394886072132</v>
+        <v>0.3236877257425403</v>
       </c>
       <c r="S9" t="n">
-        <v>0.4891669262211983</v>
+        <v>0.3732827070823491</v>
       </c>
       <c r="T9" t="n">
         <v>2</v>
@@ -1379,10 +1379,10 @@
         <v>2</v>
       </c>
       <c r="X9" t="n">
-        <v>0.4891669262211983</v>
+        <v>0.3732827070823491</v>
       </c>
       <c r="Y9" t="n">
-        <v>1.62</v>
+        <v>3.2</v>
       </c>
       <c r="Z9" t="inlineStr">
         <is>
@@ -1390,33 +1390,33 @@
         </is>
       </c>
       <c r="AA9" t="n">
-        <v>-0.3347573863252558</v>
+        <v>0.08841121030159861</v>
       </c>
       <c r="AB9" t="n">
-        <v>3.312692231080964</v>
+        <v>3.732827070823491</v>
       </c>
       <c r="AC9" t="n">
-        <v>0.1542733410496097</v>
+        <v>0.04959498133980877</v>
       </c>
       <c r="AD9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
         <is>
-          <t>UXkVSb0b</t>
+          <t>xQXNUKVo</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
-        <v>45749.66666666666</v>
+        <v>45749.65625</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>liverpool</t>
+          <t>southampton</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>everton</t>
+          <t>crystal palace</t>
         </is>
       </c>
       <c r="E10" t="n">
@@ -1436,40 +1436,40 @@
         </is>
       </c>
       <c r="I10" t="n">
-        <v>1.4</v>
+        <v>5.5</v>
       </c>
       <c r="J10" t="n">
-        <v>4.5</v>
+        <v>3.75</v>
       </c>
       <c r="K10" t="n">
-        <v>8.5</v>
+        <v>1.62</v>
       </c>
       <c r="L10" t="n">
-        <v>0.6775907883082374</v>
+        <v>0.1705981465880371</v>
       </c>
       <c r="M10" t="n">
-        <v>0.2108060230292294</v>
+        <v>0.2502106149957877</v>
       </c>
       <c r="N10" t="n">
-        <v>0.1116031886625332</v>
+        <v>0.5791912384161753</v>
       </c>
       <c r="O10" t="n">
-        <v>0.05415499533146595</v>
+        <v>0.06576879910213229</v>
       </c>
       <c r="P10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q10" t="n">
-        <v>0.2481192848116009</v>
+        <v>0.3263256215634965</v>
       </c>
       <c r="R10" t="n">
-        <v>0.6736489992324781</v>
+        <v>0.2439163078866845</v>
       </c>
       <c r="S10" t="n">
-        <v>0.07823171595592086</v>
+        <v>0.4297580705498191</v>
       </c>
       <c r="T10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="U10" t="n">
         <v>1</v>
@@ -1478,13 +1478,13 @@
         <v>0</v>
       </c>
       <c r="W10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="X10" t="n">
-        <v>0.6736489992324781</v>
+        <v>0.4297580705498191</v>
       </c>
       <c r="Y10" t="n">
-        <v>1.4</v>
+        <v>1.62</v>
       </c>
       <c r="Z10" t="inlineStr">
         <is>
@@ -1492,33 +1492,33 @@
         </is>
       </c>
       <c r="AA10" t="n">
-        <v>-0.1422285026863267</v>
+        <v>-0.4899869769504726</v>
       </c>
       <c r="AB10" t="n">
-        <v>5.784777847711267</v>
+        <v>3.265272902127269</v>
       </c>
       <c r="AC10" t="n">
-        <v>0.4255297144208772</v>
+        <v>0.1034324489863226</v>
       </c>
       <c r="AD10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
         <is>
-          <t>OzTfXtbn</t>
+          <t>p4dxpKsh</t>
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>45744.69791666666</v>
+        <v>45745.71180555555</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>strasbourg</t>
+          <t>monaco</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>lyon</t>
+          <t>nice</t>
         </is>
       </c>
       <c r="E11" t="n">
@@ -1538,40 +1538,40 @@
         </is>
       </c>
       <c r="I11" t="n">
-        <v>2.7</v>
+        <v>1.85</v>
       </c>
       <c r="J11" t="n">
-        <v>3.6</v>
+        <v>3.8</v>
       </c>
       <c r="K11" t="n">
-        <v>2.45</v>
+        <v>3.8</v>
       </c>
       <c r="L11" t="n">
-        <v>0.3506261180679785</v>
+        <v>0.5066666666666666</v>
       </c>
       <c r="M11" t="n">
-        <v>0.2629695885509839</v>
+        <v>0.2466666666666667</v>
       </c>
       <c r="N11" t="n">
-        <v>0.3864042933810375</v>
+        <v>0.2466666666666667</v>
       </c>
       <c r="O11" t="n">
-        <v>0.0563114134542706</v>
+        <v>0.06685633001422464</v>
       </c>
       <c r="P11" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q11" t="n">
-        <v>0.2728560626043755</v>
+        <v>0.372539595096158</v>
       </c>
       <c r="R11" t="n">
-        <v>0.1930732425601662</v>
+        <v>0.4126774798172897</v>
       </c>
       <c r="S11" t="n">
-        <v>0.5340706948354583</v>
+        <v>0.2147829250865524</v>
       </c>
       <c r="T11" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="U11" t="n">
         <v>1</v>
@@ -1580,13 +1580,13 @@
         <v>0</v>
       </c>
       <c r="W11" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="X11" t="n">
-        <v>0.5340706948354583</v>
+        <v>0.4126774798172897</v>
       </c>
       <c r="Y11" t="n">
-        <v>2.45</v>
+        <v>1.85</v>
       </c>
       <c r="Z11" t="inlineStr">
         <is>
@@ -1594,35 +1594,33 @@
         </is>
       </c>
       <c r="AA11" t="n">
-        <v>0.2127401395495676</v>
+        <v>-0.2782901909858987</v>
       </c>
       <c r="AB11" t="n">
-        <v>5.340706948354583</v>
+        <v>2.497657808276925</v>
       </c>
       <c r="AC11" t="n">
-        <v>0.2612146322310828</v>
-      </c>
-      <c r="AD11" t="n">
-        <v>0</v>
-      </c>
+        <v>0.04013788472113178</v>
+      </c>
+      <c r="AD11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
         <is>
-          <t>bDNJRxSN</t>
+          <t>CdaxFarI</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
-        <v>45745.54166666666</v>
+        <v>45746.51041666666</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>reims</t>
+          <t>auxerre</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>marseille</t>
+          <t>montpellier</t>
         </is>
       </c>
       <c r="E12" t="n">
@@ -1642,40 +1640,40 @@
         </is>
       </c>
       <c r="I12" t="n">
-        <v>5</v>
+        <v>1.75</v>
       </c>
       <c r="J12" t="n">
-        <v>4</v>
+        <v>3.8</v>
       </c>
       <c r="K12" t="n">
-        <v>1.6</v>
+        <v>4.33</v>
       </c>
       <c r="L12" t="n">
-        <v>0.186046511627907</v>
+        <v>0.5362840799830516</v>
       </c>
       <c r="M12" t="n">
-        <v>0.2325581395348837</v>
+        <v>0.2469729315711422</v>
       </c>
       <c r="N12" t="n">
-        <v>0.5813953488372093</v>
+        <v>0.2167429884458061</v>
       </c>
       <c r="O12" t="n">
-        <v>0.07499999999999996</v>
+        <v>0.06553334838250358</v>
       </c>
       <c r="P12" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q12" t="n">
-        <v>0.1492042404924184</v>
+        <v>0.3282873747714532</v>
       </c>
       <c r="R12" t="n">
-        <v>0.09505338820583924</v>
+        <v>0.3743878275043467</v>
       </c>
       <c r="S12" t="n">
-        <v>0.7557423713017424</v>
+        <v>0.2973247977242</v>
       </c>
       <c r="T12" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="U12" t="n">
         <v>1</v>
@@ -1684,13 +1682,13 @@
         <v>0</v>
       </c>
       <c r="W12" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="X12" t="n">
-        <v>0.7557423713017424</v>
+        <v>0.3743878275043467</v>
       </c>
       <c r="Y12" t="n">
-        <v>1.6</v>
+        <v>1.75</v>
       </c>
       <c r="Z12" t="inlineStr">
         <is>
@@ -1698,35 +1696,33 @@
         </is>
       </c>
       <c r="AA12" t="n">
-        <v>0.3486463234713131</v>
+        <v>-0.4597617358231911</v>
       </c>
       <c r="AB12" t="n">
-        <v>7.557423713017424</v>
+        <v>1.505966223778562</v>
       </c>
       <c r="AC12" t="n">
-        <v>0.6065381308093239</v>
-      </c>
-      <c r="AD12" t="n">
-        <v>0</v>
-      </c>
+        <v>0.04610045273289348</v>
+      </c>
+      <c r="AD12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
-          <t>QaPBTbcB</t>
+          <t>Ic4jMGko</t>
         </is>
       </c>
       <c r="B13" s="2" t="n">
-        <v>45745.625</v>
+        <v>45746.65625</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>st etienne</t>
+          <t>lille</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>psg</t>
+          <t>lens</t>
         </is>
       </c>
       <c r="E13" t="n">
@@ -1746,40 +1742,40 @@
         </is>
       </c>
       <c r="I13" t="n">
-        <v>13</v>
+        <v>1.95</v>
       </c>
       <c r="J13" t="n">
-        <v>8.5</v>
+        <v>3.5</v>
       </c>
       <c r="K13" t="n">
-        <v>1.14</v>
+        <v>3.8</v>
       </c>
       <c r="L13" t="n">
-        <v>0.07177246129916302</v>
+        <v>0.4830216088614491</v>
       </c>
       <c r="M13" t="n">
-        <v>0.1097696466928376</v>
+        <v>0.2691120392228074</v>
       </c>
       <c r="N13" t="n">
-        <v>0.8184578920079995</v>
+        <v>0.2478663519157436</v>
       </c>
       <c r="O13" t="n">
-        <v>0.07176311820274672</v>
+        <v>0.06169269327164062</v>
       </c>
       <c r="P13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q13" t="n">
-        <v>0.07846166318460572</v>
+        <v>0.3556020932094947</v>
       </c>
       <c r="R13" t="n">
-        <v>0.03229490435458057</v>
+        <v>0.4807080183371107</v>
       </c>
       <c r="S13" t="n">
-        <v>0.8892434324608138</v>
+        <v>0.1636898884533947</v>
       </c>
       <c r="T13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="U13" t="n">
         <v>1</v>
@@ -1788,13 +1784,13 @@
         <v>0</v>
       </c>
       <c r="W13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="X13" t="n">
-        <v>0.8892434324608138</v>
+        <v>0.4807080183371107</v>
       </c>
       <c r="Y13" t="n">
-        <v>1.14</v>
+        <v>1.95</v>
       </c>
       <c r="Z13" t="inlineStr">
         <is>
@@ -1802,35 +1798,33 @@
         </is>
       </c>
       <c r="AA13" t="n">
-        <v>0.09812509289519775</v>
+        <v>-0.06591512025540448</v>
       </c>
       <c r="AB13" t="n">
-        <v>8.892434324608139</v>
+        <v>4.333334025988994</v>
       </c>
       <c r="AC13" t="n">
-        <v>0.8107817692762082</v>
-      </c>
-      <c r="AD13" t="n">
-        <v>0</v>
-      </c>
+        <v>0.125105925127616</v>
+      </c>
+      <c r="AD13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="1" t="inlineStr">
         <is>
-          <t>p4dxpKsh</t>
+          <t>OzTfXtbn</t>
         </is>
       </c>
       <c r="B14" s="2" t="n">
-        <v>45745.71180555555</v>
+        <v>45744.69791666666</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>monaco</t>
+          <t>strasbourg</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>nice</t>
+          <t>lyon</t>
         </is>
       </c>
       <c r="E14" t="n">
@@ -1850,40 +1844,40 @@
         </is>
       </c>
       <c r="I14" t="n">
-        <v>1.85</v>
+        <v>2.7</v>
       </c>
       <c r="J14" t="n">
-        <v>3.8</v>
+        <v>3.6</v>
       </c>
       <c r="K14" t="n">
-        <v>3.8</v>
+        <v>2.45</v>
       </c>
       <c r="L14" t="n">
-        <v>0.5066666666666666</v>
+        <v>0.3506261180679785</v>
       </c>
       <c r="M14" t="n">
-        <v>0.2466666666666667</v>
+        <v>0.2629695885509839</v>
       </c>
       <c r="N14" t="n">
-        <v>0.2466666666666667</v>
+        <v>0.3864042933810375</v>
       </c>
       <c r="O14" t="n">
-        <v>0.06685633001422464</v>
+        <v>0.0563114134542706</v>
       </c>
       <c r="P14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q14" t="n">
-        <v>0.4023032501307444</v>
+        <v>0.2623915780307486</v>
       </c>
       <c r="R14" t="n">
-        <v>0.3431217900756806</v>
+        <v>0.1757040740903016</v>
       </c>
       <c r="S14" t="n">
-        <v>0.2545749597935749</v>
+        <v>0.5619043478789497</v>
       </c>
       <c r="T14" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="U14" t="n">
         <v>1</v>
@@ -1892,13 +1886,13 @@
         <v>0</v>
       </c>
       <c r="W14" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="X14" t="n">
-        <v>0.4023032501307444</v>
+        <v>0.5619043478789497</v>
       </c>
       <c r="Y14" t="n">
-        <v>3.8</v>
+        <v>2.45</v>
       </c>
       <c r="Z14" t="inlineStr">
         <is>
@@ -1906,35 +1900,33 @@
         </is>
       </c>
       <c r="AA14" t="n">
-        <v>0.1888401251774389</v>
+        <v>0.2597694153816736</v>
       </c>
       <c r="AB14" t="n">
-        <v>4.023032501307444</v>
+        <v>5.619043478789497</v>
       </c>
       <c r="AC14" t="n">
-        <v>0.05918146005506381</v>
-      </c>
-      <c r="AD14" t="n">
-        <v>0</v>
-      </c>
+        <v>0.2995127698482011</v>
+      </c>
+      <c r="AD14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="1" t="inlineStr">
         <is>
-          <t>W0W2VKSb</t>
+          <t>bDNJRxSN</t>
         </is>
       </c>
       <c r="B15" s="2" t="n">
-        <v>45746.41666666666</v>
+        <v>45745.54166666666</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>toulouse</t>
+          <t>reims</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>brest</t>
+          <t>marseille</t>
         </is>
       </c>
       <c r="E15" t="n">
@@ -1954,37 +1946,37 @@
         </is>
       </c>
       <c r="I15" t="n">
+        <v>5</v>
+      </c>
+      <c r="J15" t="n">
+        <v>4</v>
+      </c>
+      <c r="K15" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="L15" t="n">
+        <v>0.186046511627907</v>
+      </c>
+      <c r="M15" t="n">
+        <v>0.2325581395348837</v>
+      </c>
+      <c r="N15" t="n">
+        <v>0.5813953488372093</v>
+      </c>
+      <c r="O15" t="n">
+        <v>0.07499999999999996</v>
+      </c>
+      <c r="P15" t="n">
         <v>2</v>
       </c>
-      <c r="J15" t="n">
-        <v>3.25</v>
-      </c>
-      <c r="K15" t="n">
-        <v>4.1</v>
-      </c>
-      <c r="L15" t="n">
-        <v>0.4754683318465656</v>
-      </c>
-      <c r="M15" t="n">
-        <v>0.2925958965209635</v>
-      </c>
-      <c r="N15" t="n">
-        <v>0.231935771632471</v>
-      </c>
-      <c r="O15" t="n">
-        <v>0.05159474671669795</v>
-      </c>
-      <c r="P15" t="n">
-        <v>1</v>
-      </c>
       <c r="Q15" t="n">
-        <v>0.272714526503825</v>
+        <v>0.1420391041223031</v>
       </c>
       <c r="R15" t="n">
-        <v>0.1925053220516518</v>
+        <v>0.06197535309821289</v>
       </c>
       <c r="S15" t="n">
-        <v>0.5347801514445232</v>
+        <v>0.7959855427794842</v>
       </c>
       <c r="T15" t="n">
         <v>2</v>
@@ -1999,10 +1991,10 @@
         <v>2</v>
       </c>
       <c r="X15" t="n">
-        <v>0.5347801514445232</v>
+        <v>0.7959855427794842</v>
       </c>
       <c r="Y15" t="n">
-        <v>4.1</v>
+        <v>1.6</v>
       </c>
       <c r="Z15" t="inlineStr">
         <is>
@@ -2010,35 +2002,33 @@
         </is>
       </c>
       <c r="AA15" t="n">
-        <v>0.3847092325556596</v>
+        <v>0.4559614474119579</v>
       </c>
       <c r="AB15" t="n">
-        <v>5.347801514445232</v>
+        <v>7.959855427794842</v>
       </c>
       <c r="AC15" t="n">
-        <v>0.2620656249406982</v>
-      </c>
-      <c r="AD15" t="n">
-        <v>0</v>
-      </c>
+        <v>0.6539464386571812</v>
+      </c>
+      <c r="AD15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="1" t="inlineStr">
         <is>
-          <t>hfqyHLD5</t>
+          <t>QaPBTbcB</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
-        <v>45746.51041666666</v>
+        <v>45745.625</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>angers</t>
+          <t>st etienne</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>rennes</t>
+          <t>psg</t>
         </is>
       </c>
       <c r="E16" t="n">
@@ -2058,37 +2048,37 @@
         </is>
       </c>
       <c r="I16" t="n">
-        <v>4.1</v>
+        <v>13</v>
       </c>
       <c r="J16" t="n">
-        <v>3.4</v>
+        <v>8.5</v>
       </c>
       <c r="K16" t="n">
-        <v>1.91</v>
+        <v>1.14</v>
       </c>
       <c r="L16" t="n">
-        <v>0.2297541128604281</v>
+        <v>0.07177246129916302</v>
       </c>
       <c r="M16" t="n">
-        <v>0.2770564302140457</v>
+        <v>0.1097696466928376</v>
       </c>
       <c r="N16" t="n">
-        <v>0.4931894569255263</v>
+        <v>0.8184578920079995</v>
       </c>
       <c r="O16" t="n">
-        <v>0.06158029550729749</v>
+        <v>0.07176311820274672</v>
       </c>
       <c r="P16" t="n">
         <v>2</v>
       </c>
       <c r="Q16" t="n">
-        <v>0.1576342485738712</v>
+        <v>0.06733355751545067</v>
       </c>
       <c r="R16" t="n">
-        <v>0.1169873509764736</v>
+        <v>0.01294178035050755</v>
       </c>
       <c r="S16" t="n">
-        <v>0.7253784004496553</v>
+        <v>0.9197246621340417</v>
       </c>
       <c r="T16" t="n">
         <v>2</v>
@@ -2103,10 +2093,10 @@
         <v>2</v>
       </c>
       <c r="X16" t="n">
-        <v>0.7253784004496553</v>
+        <v>0.9197246621340417</v>
       </c>
       <c r="Y16" t="n">
-        <v>1.91</v>
+        <v>1.14</v>
       </c>
       <c r="Z16" t="inlineStr">
         <is>
@@ -2114,35 +2104,33 @@
         </is>
       </c>
       <c r="AA16" t="n">
-        <v>0.4235964229218039</v>
+        <v>0.3463293916629104</v>
       </c>
       <c r="AB16" t="n">
-        <v>7.253784004496553</v>
+        <v>9.197246621340417</v>
       </c>
       <c r="AC16" t="n">
-        <v>0.5677441518757841</v>
-      </c>
-      <c r="AD16" t="n">
-        <v>0</v>
-      </c>
+        <v>0.852391104618591</v>
+      </c>
+      <c r="AD16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="1" t="inlineStr">
         <is>
-          <t>CdaxFarI</t>
+          <t>W0W2VKSb</t>
         </is>
       </c>
       <c r="B17" s="2" t="n">
-        <v>45746.51041666666</v>
+        <v>45746.41666666666</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>auxerre</t>
+          <t>toulouse</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>montpellier</t>
+          <t>brest</t>
         </is>
       </c>
       <c r="E17" t="n">
@@ -2162,40 +2150,40 @@
         </is>
       </c>
       <c r="I17" t="n">
-        <v>1.75</v>
+        <v>2</v>
       </c>
       <c r="J17" t="n">
-        <v>3.8</v>
+        <v>3.25</v>
       </c>
       <c r="K17" t="n">
-        <v>4.33</v>
+        <v>4.1</v>
       </c>
       <c r="L17" t="n">
-        <v>0.5362840799830516</v>
+        <v>0.4754683318465656</v>
       </c>
       <c r="M17" t="n">
-        <v>0.2469729315711422</v>
+        <v>0.2925958965209635</v>
       </c>
       <c r="N17" t="n">
-        <v>0.2167429884458061</v>
+        <v>0.231935771632471</v>
       </c>
       <c r="O17" t="n">
-        <v>0.06553334838250358</v>
+        <v>0.05159474671669795</v>
       </c>
       <c r="P17" t="n">
         <v>1</v>
       </c>
       <c r="Q17" t="n">
-        <v>0.3420899348958844</v>
+        <v>0.3171660242036293</v>
       </c>
       <c r="R17" t="n">
-        <v>0.3682676181733459</v>
+        <v>0.2031794208021112</v>
       </c>
       <c r="S17" t="n">
-        <v>0.2896424469307697</v>
+        <v>0.4796545549942595</v>
       </c>
       <c r="T17" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="U17" t="n">
         <v>1</v>
@@ -2204,13 +2192,13 @@
         <v>0</v>
       </c>
       <c r="W17" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="X17" t="n">
-        <v>0.3682676181733459</v>
+        <v>0.4796545549942595</v>
       </c>
       <c r="Y17" t="n">
-        <v>1.75</v>
+        <v>4.1</v>
       </c>
       <c r="Z17" t="inlineStr">
         <is>
@@ -2218,22 +2206,20 @@
         </is>
       </c>
       <c r="AA17" t="n">
-        <v>-0.4740422242621929</v>
+        <v>0.3118011856375689</v>
       </c>
       <c r="AB17" t="n">
-        <v>0.41138471199767</v>
+        <v>4.796545549942595</v>
       </c>
       <c r="AC17" t="n">
-        <v>0.02617768327746151</v>
-      </c>
-      <c r="AD17" t="n">
-        <v>0</v>
-      </c>
+        <v>0.1624885307906301</v>
+      </c>
+      <c r="AD17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="1" t="inlineStr">
         <is>
-          <t>KM2pDwDU</t>
+          <t>hfqyHLD5</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
@@ -2241,12 +2227,12 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>le havre</t>
+          <t>angers</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>nantes</t>
+          <t>rennes</t>
         </is>
       </c>
       <c r="E18" t="n">
@@ -2266,37 +2252,37 @@
         </is>
       </c>
       <c r="I18" t="n">
-        <v>2.88</v>
+        <v>4.1</v>
       </c>
       <c r="J18" t="n">
-        <v>3.1</v>
+        <v>3.4</v>
       </c>
       <c r="K18" t="n">
-        <v>2.55</v>
+        <v>1.91</v>
       </c>
       <c r="L18" t="n">
-        <v>0.3269636431319021</v>
+        <v>0.2297541128604281</v>
       </c>
       <c r="M18" t="n">
-        <v>0.3037597716838317</v>
+        <v>0.2770564302140457</v>
       </c>
       <c r="N18" t="n">
-        <v>0.369276585184266</v>
+        <v>0.4931894569255263</v>
       </c>
       <c r="O18" t="n">
-        <v>0.06195973012861078</v>
+        <v>0.06158029550729749</v>
       </c>
       <c r="P18" t="n">
         <v>2</v>
       </c>
       <c r="Q18" t="n">
-        <v>0.3671545241603469</v>
+        <v>0.1201140138900814</v>
       </c>
       <c r="R18" t="n">
-        <v>0.2207875222819361</v>
+        <v>0.06812704576712246</v>
       </c>
       <c r="S18" t="n">
-        <v>0.412057953557717</v>
+        <v>0.8117589403427961</v>
       </c>
       <c r="T18" t="n">
         <v>2</v>
@@ -2311,10 +2297,10 @@
         <v>2</v>
       </c>
       <c r="X18" t="n">
-        <v>0.412057953557717</v>
+        <v>0.8117589403427961</v>
       </c>
       <c r="Y18" t="n">
-        <v>2.55</v>
+        <v>1.91</v>
       </c>
       <c r="Z18" t="inlineStr">
         <is>
@@ -2322,35 +2308,33 @@
         </is>
       </c>
       <c r="AA18" t="n">
-        <v>0.03274050424011489</v>
+        <v>0.6049006330271873</v>
       </c>
       <c r="AB18" t="n">
-        <v>4.120579535577169</v>
+        <v>8.11758940342796</v>
       </c>
       <c r="AC18" t="n">
-        <v>0.04490342939737008</v>
-      </c>
-      <c r="AD18" t="n">
-        <v>0</v>
-      </c>
+        <v>0.6916449264527147</v>
+      </c>
+      <c r="AD18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="1" t="inlineStr">
         <is>
-          <t>Ic4jMGko</t>
+          <t>KM2pDwDU</t>
         </is>
       </c>
       <c r="B19" s="2" t="n">
-        <v>45746.65625</v>
+        <v>45746.51041666666</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>lille</t>
+          <t>le havre</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>lens</t>
+          <t>nantes</t>
         </is>
       </c>
       <c r="E19" t="n">
@@ -2370,40 +2354,40 @@
         </is>
       </c>
       <c r="I19" t="n">
-        <v>1.95</v>
+        <v>2.88</v>
       </c>
       <c r="J19" t="n">
-        <v>3.5</v>
+        <v>3.1</v>
       </c>
       <c r="K19" t="n">
-        <v>3.8</v>
+        <v>2.55</v>
       </c>
       <c r="L19" t="n">
-        <v>0.4830216088614491</v>
+        <v>0.3269636431319021</v>
       </c>
       <c r="M19" t="n">
-        <v>0.2691120392228074</v>
+        <v>0.3037597716838317</v>
       </c>
       <c r="N19" t="n">
-        <v>0.2478663519157436</v>
+        <v>0.369276585184266</v>
       </c>
       <c r="O19" t="n">
-        <v>0.06169269327164062</v>
+        <v>0.06195973012861078</v>
       </c>
       <c r="P19" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q19" t="n">
-        <v>0.4198615155053123</v>
+        <v>0.3768884586530304</v>
       </c>
       <c r="R19" t="n">
-        <v>0.3909942120517967</v>
+        <v>0.2271429792541859</v>
       </c>
       <c r="S19" t="n">
-        <v>0.1891442724428909</v>
+        <v>0.3959685620927837</v>
       </c>
       <c r="T19" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="U19" t="n">
         <v>1</v>
@@ -2412,13 +2396,13 @@
         <v>0</v>
       </c>
       <c r="W19" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="X19" t="n">
-        <v>0.4198615155053123</v>
+        <v>0.3959685620927837</v>
       </c>
       <c r="Y19" t="n">
-        <v>3.5</v>
+        <v>2.55</v>
       </c>
       <c r="Z19" t="inlineStr">
         <is>
@@ -2426,17 +2410,15 @@
         </is>
       </c>
       <c r="AA19" t="n">
-        <v>0.1878061217074372</v>
+        <v>0.006270860217160347</v>
       </c>
       <c r="AB19" t="n">
-        <v>4.198615155053123</v>
+        <v>3.959685620927837</v>
       </c>
       <c r="AC19" t="n">
-        <v>0.02886730345351562</v>
-      </c>
-      <c r="AD19" t="n">
-        <v>0</v>
-      </c>
+        <v>0.01908010343975336</v>
+      </c>
+      <c r="AD19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="1" t="inlineStr">
@@ -2531,7 +2513,7 @@
         <v>-0.1114634192041025</v>
       </c>
       <c r="AB20" t="n">
-        <v>6.789302893753407</v>
+        <v>6.371935816216682</v>
       </c>
       <c r="AC20" t="n">
         <v>0.5955025264223748</v>
@@ -2541,7 +2523,7 @@
     <row r="21">
       <c r="A21" s="1" t="inlineStr">
         <is>
-          <t>0MJJTGoK</t>
+          <t>CnbjgzA7</t>
         </is>
       </c>
       <c r="B21" s="2" t="n">
@@ -2549,12 +2531,12 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>b  monchengladbach</t>
+          <t>bayern munich</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>rb leipzig</t>
+          <t>st  pauli</t>
         </is>
       </c>
       <c r="E21" t="n">
@@ -2574,53 +2556,53 @@
         </is>
       </c>
       <c r="I21" t="n">
-        <v>2.88</v>
+        <v>1.14</v>
       </c>
       <c r="J21" t="n">
-        <v>3.7</v>
+        <v>7.5</v>
       </c>
       <c r="K21" t="n">
-        <v>2.25</v>
+        <v>15</v>
       </c>
       <c r="L21" t="n">
-        <v>0.326970661010958</v>
+        <v>0.8143322475570033</v>
       </c>
       <c r="M21" t="n">
-        <v>0.2545068928950159</v>
+        <v>0.1237785016286645</v>
       </c>
       <c r="N21" t="n">
-        <v>0.4185224460940262</v>
+        <v>0.06188925081433225</v>
       </c>
       <c r="O21" t="n">
-        <v>0.06193693693693691</v>
+        <v>0.07719298245614037</v>
       </c>
       <c r="P21" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q21" t="n">
-        <v>0.3287062980943327</v>
+        <v>0.06362082105579843</v>
       </c>
       <c r="R21" t="n">
-        <v>0.1879560681357793</v>
+        <v>0.8941340175733763</v>
       </c>
       <c r="S21" t="n">
-        <v>0.4833376337698879</v>
+        <v>0.04224516137082535</v>
       </c>
       <c r="T21" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="U21" t="n">
         <v>1</v>
       </c>
       <c r="V21" t="inlineStr"/>
       <c r="W21" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="X21" t="n">
-        <v>0.4833376337698879</v>
+        <v>0.8941340175733763</v>
       </c>
       <c r="Y21" t="n">
-        <v>2.25</v>
+        <v>1.14</v>
       </c>
       <c r="Z21" t="inlineStr">
         <is>
@@ -2628,20 +2610,20 @@
         </is>
       </c>
       <c r="AA21" t="n">
-        <v>0.07000774078579823</v>
+        <v>0.1379484288117779</v>
       </c>
       <c r="AB21" t="n">
-        <v>4.833376337698879</v>
+        <v>8.941340175733764</v>
       </c>
       <c r="AC21" t="n">
-        <v>0.1546313356755552</v>
+        <v>0.8305131965175778</v>
       </c>
       <c r="AD21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="1" t="inlineStr">
         <is>
-          <t>CnbjgzA7</t>
+          <t>KhLH9efl</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
@@ -2649,12 +2631,12 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>bayern munich</t>
+          <t>hoffenheim</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>st  pauli</t>
+          <t>augsburg</t>
         </is>
       </c>
       <c r="E22" t="n">
@@ -2674,37 +2656,37 @@
         </is>
       </c>
       <c r="I22" t="n">
-        <v>1.14</v>
+        <v>2.35</v>
       </c>
       <c r="J22" t="n">
-        <v>7.5</v>
+        <v>3.2</v>
       </c>
       <c r="K22" t="n">
-        <v>15</v>
+        <v>3.1</v>
       </c>
       <c r="L22" t="n">
-        <v>0.8143322475570033</v>
+        <v>0.4012133468149647</v>
       </c>
       <c r="M22" t="n">
-        <v>0.1237785016286645</v>
+        <v>0.2946410515672397</v>
       </c>
       <c r="N22" t="n">
-        <v>0.06188925081433225</v>
+        <v>0.3041456016177958</v>
       </c>
       <c r="O22" t="n">
-        <v>0.07719298245614037</v>
+        <v>0.06061256005490723</v>
       </c>
       <c r="P22" t="n">
         <v>1</v>
       </c>
       <c r="Q22" t="n">
-        <v>0.06362082105579843</v>
+        <v>0.1854312213146095</v>
       </c>
       <c r="R22" t="n">
-        <v>0.8941340175733763</v>
+        <v>0.4188397885288456</v>
       </c>
       <c r="S22" t="n">
-        <v>0.04224516137082535</v>
+        <v>0.3957289901565448</v>
       </c>
       <c r="T22" t="n">
         <v>1</v>
@@ -2717,10 +2699,10 @@
         <v>1</v>
       </c>
       <c r="X22" t="n">
-        <v>0.8941340175733763</v>
+        <v>0.4188397885288456</v>
       </c>
       <c r="Y22" t="n">
-        <v>1.14</v>
+        <v>2.35</v>
       </c>
       <c r="Z22" t="inlineStr">
         <is>
@@ -2728,20 +2710,20 @@
         </is>
       </c>
       <c r="AA22" t="n">
-        <v>0.1379484288117779</v>
+        <v>-0.01164925700534293</v>
       </c>
       <c r="AB22" t="n">
-        <v>8.941340175733764</v>
+        <v>4.115217748220544</v>
       </c>
       <c r="AC22" t="n">
-        <v>0.8305131965175778</v>
+        <v>0.02311079837230079</v>
       </c>
       <c r="AD22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="1" t="inlineStr">
         <is>
-          <t>KhLH9efl</t>
+          <t>YFRX5DgD</t>
         </is>
       </c>
       <c r="B23" s="2" t="n">
@@ -2749,12 +2731,12 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>hoffenheim</t>
+          <t>wolfsburg</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>augsburg</t>
+          <t>heidenheim</t>
         </is>
       </c>
       <c r="E23" t="n">
@@ -2774,37 +2756,37 @@
         </is>
       </c>
       <c r="I23" t="n">
-        <v>2.35</v>
+        <v>1.65</v>
       </c>
       <c r="J23" t="n">
-        <v>3.2</v>
+        <v>3.8</v>
       </c>
       <c r="K23" t="n">
-        <v>3.1</v>
+        <v>5.25</v>
       </c>
       <c r="L23" t="n">
-        <v>0.4012133468149647</v>
+        <v>0.571920017200602</v>
       </c>
       <c r="M23" t="n">
-        <v>0.2946410515672397</v>
+        <v>0.2483336916792087</v>
       </c>
       <c r="N23" t="n">
-        <v>0.3041456016177958</v>
+        <v>0.1797462911201892</v>
       </c>
       <c r="O23" t="n">
-        <v>0.06061256005490723</v>
+        <v>0.05969469127363869</v>
       </c>
       <c r="P23" t="n">
         <v>1</v>
       </c>
       <c r="Q23" t="n">
-        <v>0.1854312213146095</v>
+        <v>0.3117261809962231</v>
       </c>
       <c r="R23" t="n">
-        <v>0.4188397885288456</v>
+        <v>0.4831635946886937</v>
       </c>
       <c r="S23" t="n">
-        <v>0.3957289901565448</v>
+        <v>0.2051102243150832</v>
       </c>
       <c r="T23" t="n">
         <v>1</v>
@@ -2817,10 +2799,10 @@
         <v>1</v>
       </c>
       <c r="X23" t="n">
-        <v>0.4188397885288456</v>
+        <v>0.4831635946886937</v>
       </c>
       <c r="Y23" t="n">
-        <v>2.35</v>
+        <v>1.65</v>
       </c>
       <c r="Z23" t="inlineStr">
         <is>
@@ -2828,33 +2810,33 @@
         </is>
       </c>
       <c r="AA23" t="n">
-        <v>-0.01164925700534293</v>
+        <v>-0.3119693365594698</v>
       </c>
       <c r="AB23" t="n">
-        <v>0.8279216737717952</v>
+        <v>2.722410844528147</v>
       </c>
       <c r="AC23" t="n">
-        <v>0.02311079837230079</v>
+        <v>0.1714374136924707</v>
       </c>
       <c r="AD23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="1" t="inlineStr">
         <is>
-          <t>K60jOf9s</t>
+          <t>C0wP7ZO0</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
-        <v>45745.47916666666</v>
+        <v>45746.4375</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>holstein kiel</t>
+          <t>freiburg</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>werder bremen</t>
+          <t>union berlin</t>
         </is>
       </c>
       <c r="E24" t="n">
@@ -2874,87 +2856,91 @@
         </is>
       </c>
       <c r="I24" t="n">
-        <v>3.1</v>
+        <v>2</v>
       </c>
       <c r="J24" t="n">
-        <v>3.8</v>
+        <v>3.5</v>
       </c>
       <c r="K24" t="n">
-        <v>2.1</v>
+        <v>3.7</v>
       </c>
       <c r="L24" t="n">
-        <v>0.303768557289684</v>
+        <v>0.473491773308958</v>
       </c>
       <c r="M24" t="n">
-        <v>0.2478111914731633</v>
+        <v>0.2705667276051188</v>
       </c>
       <c r="N24" t="n">
-        <v>0.4484202512371526</v>
+        <v>0.2559414990859232</v>
       </c>
       <c r="O24" t="n">
-        <v>0.06192901608860857</v>
+        <v>0.05598455598455598</v>
       </c>
       <c r="P24" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q24" t="n">
+        <v>0.3653185016614392</v>
+      </c>
+      <c r="R24" t="n">
+        <v>0.379537966743028</v>
+      </c>
+      <c r="S24" t="n">
+        <v>0.2551435315955327</v>
+      </c>
+      <c r="T24" t="n">
+        <v>1</v>
+      </c>
+      <c r="U24" t="n">
+        <v>1</v>
+      </c>
+      <c r="V24" t="n">
+        <v>0</v>
+      </c>
+      <c r="W24" t="n">
+        <v>1</v>
+      </c>
+      <c r="X24" t="n">
+        <v>0.379537966743028</v>
+      </c>
+      <c r="Y24" t="n">
         <v>2</v>
       </c>
-      <c r="Q24" t="n">
-        <v>0.4410607374331613</v>
-      </c>
-      <c r="R24" t="n">
-        <v>0.172923409070232</v>
-      </c>
-      <c r="S24" t="n">
-        <v>0.3860158534966067</v>
-      </c>
-      <c r="T24" t="n">
-        <v>0</v>
-      </c>
-      <c r="U24" t="n">
-        <v>1</v>
-      </c>
-      <c r="V24" t="inlineStr"/>
-      <c r="W24" t="n">
-        <v>0</v>
-      </c>
-      <c r="X24" t="n">
-        <v>0.4410607374331613</v>
-      </c>
-      <c r="Y24" t="n">
-        <v>3.8</v>
-      </c>
       <c r="Z24" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
       <c r="AA24" t="n">
-        <v>0.2414395722307188</v>
+        <v>-0.2409240665139439</v>
       </c>
       <c r="AB24" t="n">
-        <v>4.410607374331613</v>
+        <v>0.4961059453148076</v>
       </c>
       <c r="AC24" t="n">
-        <v>0.05504488393655455</v>
-      </c>
-      <c r="AD24" t="inlineStr"/>
+        <v>0.01421946508158883</v>
+      </c>
+      <c r="AD24" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="1" t="inlineStr">
         <is>
-          <t>YFRX5DgD</t>
+          <t>SftwHw2E</t>
         </is>
       </c>
       <c r="B25" s="2" t="n">
-        <v>45745.47916666666</v>
+        <v>45746.52083333334</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>wolfsburg</t>
+          <t>dortmund</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>heidenheim</t>
+          <t>mainz</t>
         </is>
       </c>
       <c r="E25" t="n">
@@ -2974,37 +2960,37 @@
         </is>
       </c>
       <c r="I25" t="n">
-        <v>1.65</v>
+        <v>1.7</v>
       </c>
       <c r="J25" t="n">
         <v>3.8</v>
       </c>
       <c r="K25" t="n">
-        <v>5.25</v>
+        <v>5</v>
       </c>
       <c r="L25" t="n">
-        <v>0.571920017200602</v>
+        <v>0.5594817432273262</v>
       </c>
       <c r="M25" t="n">
-        <v>0.2483336916792087</v>
+        <v>0.2502944640753828</v>
       </c>
       <c r="N25" t="n">
-        <v>0.1797462911201892</v>
+        <v>0.1902237926972909</v>
       </c>
       <c r="O25" t="n">
-        <v>0.05969469127363869</v>
+        <v>0.05139318885448918</v>
       </c>
       <c r="P25" t="n">
         <v>1</v>
       </c>
       <c r="Q25" t="n">
-        <v>0.3117261809962231</v>
+        <v>0.1667556080541772</v>
       </c>
       <c r="R25" t="n">
-        <v>0.4831635946886937</v>
+        <v>0.6659852326856369</v>
       </c>
       <c r="S25" t="n">
-        <v>0.2051102243150832</v>
+        <v>0.1672591592601858</v>
       </c>
       <c r="T25" t="n">
         <v>1</v>
@@ -3017,10 +3003,10 @@
         <v>1</v>
       </c>
       <c r="X25" t="n">
-        <v>0.4831635946886937</v>
+        <v>0.6659852326856369</v>
       </c>
       <c r="Y25" t="n">
-        <v>1.65</v>
+        <v>1.7</v>
       </c>
       <c r="Z25" t="inlineStr">
         <is>
@@ -3028,33 +3014,33 @@
         </is>
       </c>
       <c r="AA25" t="n">
-        <v>-0.3119693365594698</v>
+        <v>0.1888212793794039</v>
       </c>
       <c r="AB25" t="n">
-        <v>3.371382138738623</v>
+        <v>6.659852326856369</v>
       </c>
       <c r="AC25" t="n">
-        <v>0.1714374136924707</v>
+        <v>0.4987260734254511</v>
       </c>
       <c r="AD25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="1" t="inlineStr">
         <is>
-          <t>08voFHWQ</t>
+          <t>K60jOf9s</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
-        <v>45745.60416666666</v>
+        <v>45745.47916666666</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>eintracht frankfurt</t>
+          <t>holstein kiel</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>stuttgart</t>
+          <t>werder bremen</t>
         </is>
       </c>
       <c r="E26" t="n">
@@ -3074,37 +3060,37 @@
         </is>
       </c>
       <c r="I26" t="n">
-        <v>2.3</v>
+        <v>3.1</v>
       </c>
       <c r="J26" t="n">
-        <v>3.75</v>
+        <v>3.8</v>
       </c>
       <c r="K26" t="n">
-        <v>2.75</v>
+        <v>2.1</v>
       </c>
       <c r="L26" t="n">
-        <v>0.4082137555665512</v>
+        <v>0.303768557289684</v>
       </c>
       <c r="M26" t="n">
-        <v>0.2503711034141514</v>
+        <v>0.2478111914731633</v>
       </c>
       <c r="N26" t="n">
-        <v>0.3414151410192973</v>
+        <v>0.4484202512371526</v>
       </c>
       <c r="O26" t="n">
-        <v>0.06508563899868269</v>
+        <v>0.06192901608860857</v>
       </c>
       <c r="P26" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q26" t="n">
-        <v>0.4603478651156637</v>
+        <v>0.4410607374331613</v>
       </c>
       <c r="R26" t="n">
-        <v>0.2297976300253913</v>
+        <v>0.172923409070232</v>
       </c>
       <c r="S26" t="n">
-        <v>0.3098545048589451</v>
+        <v>0.3860158534966067</v>
       </c>
       <c r="T26" t="n">
         <v>0</v>
@@ -3117,10 +3103,10 @@
         <v>0</v>
       </c>
       <c r="X26" t="n">
-        <v>0.4603478651156637</v>
+        <v>0.4410607374331613</v>
       </c>
       <c r="Y26" t="n">
-        <v>3.75</v>
+        <v>3.8</v>
       </c>
       <c r="Z26" t="inlineStr">
         <is>
@@ -3128,33 +3114,33 @@
         </is>
       </c>
       <c r="AA26" t="n">
-        <v>0.2641107251577232</v>
+        <v>0.2414395722307188</v>
       </c>
       <c r="AB26" t="n">
-        <v>4.603478651156637</v>
+        <v>4.410607374331613</v>
       </c>
       <c r="AC26" t="n">
-        <v>0.1504933602567186</v>
+        <v>0.05504488393655455</v>
       </c>
       <c r="AD26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="1" t="inlineStr">
         <is>
-          <t>C0wP7ZO0</t>
+          <t>08voFHWQ</t>
         </is>
       </c>
       <c r="B27" s="2" t="n">
-        <v>45746.4375</v>
+        <v>45745.60416666666</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>freiburg</t>
+          <t>eintracht frankfurt</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>union berlin</t>
+          <t>stuttgart</t>
         </is>
       </c>
       <c r="E27" t="n">
@@ -3174,55 +3160,53 @@
         </is>
       </c>
       <c r="I27" t="n">
-        <v>2</v>
+        <v>2.3</v>
       </c>
       <c r="J27" t="n">
-        <v>3.5</v>
+        <v>3.75</v>
       </c>
       <c r="K27" t="n">
-        <v>3.7</v>
+        <v>2.75</v>
       </c>
       <c r="L27" t="n">
-        <v>0.473491773308958</v>
+        <v>0.4082137555665512</v>
       </c>
       <c r="M27" t="n">
-        <v>0.2705667276051188</v>
+        <v>0.2503711034141514</v>
       </c>
       <c r="N27" t="n">
-        <v>0.2559414990859232</v>
+        <v>0.3414151410192973</v>
       </c>
       <c r="O27" t="n">
-        <v>0.05598455598455598</v>
+        <v>0.06508563899868269</v>
       </c>
       <c r="P27" t="n">
         <v>1</v>
       </c>
       <c r="Q27" t="n">
-        <v>0.3653185016614392</v>
+        <v>0.4603478651156637</v>
       </c>
       <c r="R27" t="n">
-        <v>0.379537966743028</v>
+        <v>0.2297976300253913</v>
       </c>
       <c r="S27" t="n">
-        <v>0.2551435315955327</v>
+        <v>0.3098545048589451</v>
       </c>
       <c r="T27" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U27" t="n">
         <v>1</v>
       </c>
-      <c r="V27" t="n">
+      <c r="V27" t="inlineStr"/>
+      <c r="W27" t="n">
         <v>0</v>
       </c>
-      <c r="W27" t="n">
-        <v>1</v>
-      </c>
       <c r="X27" t="n">
-        <v>0.379537966743028</v>
+        <v>0.4603478651156637</v>
       </c>
       <c r="Y27" t="n">
-        <v>2</v>
+        <v>3.75</v>
       </c>
       <c r="Z27" t="inlineStr">
         <is>
@@ -3230,35 +3214,33 @@
         </is>
       </c>
       <c r="AA27" t="n">
-        <v>-0.2409240665139439</v>
+        <v>0.2641107251577232</v>
       </c>
       <c r="AB27" t="n">
-        <v>0.5796543857033759</v>
+        <v>4.603478651156637</v>
       </c>
       <c r="AC27" t="n">
-        <v>0.01421946508158883</v>
-      </c>
-      <c r="AD27" t="n">
-        <v>1</v>
-      </c>
+        <v>0.1504933602567186</v>
+      </c>
+      <c r="AD27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="1" t="inlineStr">
         <is>
-          <t>SftwHw2E</t>
+          <t>0MJJTGoK</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
-        <v>45746.52083333334</v>
+        <v>45745.47916666666</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>dortmund</t>
+          <t>b  monchengladbach</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>mainz</t>
+          <t>rb leipzig</t>
         </is>
       </c>
       <c r="E28" t="n">
@@ -3278,53 +3260,53 @@
         </is>
       </c>
       <c r="I28" t="n">
-        <v>1.7</v>
+        <v>2.88</v>
       </c>
       <c r="J28" t="n">
-        <v>3.8</v>
+        <v>3.7</v>
       </c>
       <c r="K28" t="n">
-        <v>5</v>
+        <v>2.25</v>
       </c>
       <c r="L28" t="n">
-        <v>0.5594817432273262</v>
+        <v>0.326970661010958</v>
       </c>
       <c r="M28" t="n">
-        <v>0.2502944640753828</v>
+        <v>0.2545068928950159</v>
       </c>
       <c r="N28" t="n">
-        <v>0.1902237926972909</v>
+        <v>0.4185224460940262</v>
       </c>
       <c r="O28" t="n">
-        <v>0.05139318885448918</v>
+        <v>0.06193693693693691</v>
       </c>
       <c r="P28" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q28" t="n">
-        <v>0.1667556080541772</v>
+        <v>0.3287062980943327</v>
       </c>
       <c r="R28" t="n">
-        <v>0.6659852326856369</v>
+        <v>0.1879560681357793</v>
       </c>
       <c r="S28" t="n">
-        <v>0.1672591592601858</v>
+        <v>0.4833376337698879</v>
       </c>
       <c r="T28" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="U28" t="n">
         <v>1</v>
       </c>
       <c r="V28" t="inlineStr"/>
       <c r="W28" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="X28" t="n">
-        <v>0.6659852326856369</v>
+        <v>0.4833376337698879</v>
       </c>
       <c r="Y28" t="n">
-        <v>1.7</v>
+        <v>2.25</v>
       </c>
       <c r="Z28" t="inlineStr">
         <is>
@@ -3332,13 +3314,13 @@
         </is>
       </c>
       <c r="AA28" t="n">
-        <v>0.1888212793794039</v>
+        <v>0.07000774078579823</v>
       </c>
       <c r="AB28" t="n">
-        <v>6.659852326856369</v>
+        <v>4.833376337698879</v>
       </c>
       <c r="AC28" t="n">
-        <v>0.4987260734254511</v>
+        <v>0.1546313356755552</v>
       </c>
       <c r="AD28" t="inlineStr"/>
     </row>
@@ -3402,13 +3384,13 @@
         <v>1</v>
       </c>
       <c r="Q29" t="n">
-        <v>0.3706402711553872</v>
+        <v>0.3461757392734069</v>
       </c>
       <c r="R29" t="n">
-        <v>0.442710024535179</v>
+        <v>0.4841210969628983</v>
       </c>
       <c r="S29" t="n">
-        <v>0.1866497043094338</v>
+        <v>0.1697031637636948</v>
       </c>
       <c r="T29" t="n">
         <v>1</v>
@@ -3416,14 +3398,12 @@
       <c r="U29" t="n">
         <v>1</v>
       </c>
-      <c r="V29" t="n">
-        <v>0</v>
-      </c>
+      <c r="V29" t="inlineStr"/>
       <c r="W29" t="n">
         <v>1</v>
       </c>
       <c r="X29" t="n">
-        <v>0.442710024535179</v>
+        <v>0.4841210969628983</v>
       </c>
       <c r="Y29" t="n">
         <v>1.73</v>
@@ -3434,35 +3414,33 @@
         </is>
       </c>
       <c r="AA29" t="n">
-        <v>-0.3207009007590965</v>
+        <v>-0.2225623318550493</v>
       </c>
       <c r="AB29" t="n">
-        <v>3.054076975980194</v>
+        <v>3.282485833185933</v>
       </c>
       <c r="AC29" t="n">
-        <v>0.07206975337979177</v>
-      </c>
-      <c r="AD29" t="n">
-        <v>0</v>
-      </c>
+        <v>0.1379453576894913</v>
+      </c>
+      <c r="AD29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="1" t="inlineStr">
         <is>
-          <t>ENQJ7Yqe</t>
+          <t>KdZr6L8j</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
-        <v>45745.45833333334</v>
+        <v>45745.58333333334</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>venezia</t>
+          <t>juventus</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>bologna</t>
+          <t>genoa</t>
         </is>
       </c>
       <c r="E30" t="n">
@@ -3482,55 +3460,53 @@
         </is>
       </c>
       <c r="I30" t="n">
-        <v>4.5</v>
+        <v>1.55</v>
       </c>
       <c r="J30" t="n">
-        <v>3.5</v>
+        <v>3.9</v>
       </c>
       <c r="K30" t="n">
-        <v>1.83</v>
+        <v>6.5</v>
       </c>
       <c r="L30" t="n">
-        <v>0.2107601184600197</v>
+        <v>0.6112852664576801</v>
       </c>
       <c r="M30" t="n">
-        <v>0.2709772951628825</v>
+        <v>0.2429467084639498</v>
       </c>
       <c r="N30" t="n">
-        <v>0.5182625863770978</v>
+        <v>0.1457680250783699</v>
       </c>
       <c r="O30" t="n">
-        <v>0.05438459536820184</v>
+        <v>0.05541770057899109</v>
       </c>
       <c r="P30" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q30" t="n">
-        <v>0.2614903955310947</v>
+        <v>0.3070464824226415</v>
       </c>
       <c r="R30" t="n">
-        <v>0.1288206697122698</v>
+        <v>0.5875596764324247</v>
       </c>
       <c r="S30" t="n">
-        <v>0.6096889347566355</v>
+        <v>0.1053938411449338</v>
       </c>
       <c r="T30" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="U30" t="n">
         <v>1</v>
       </c>
-      <c r="V30" t="n">
-        <v>0</v>
-      </c>
+      <c r="V30" t="inlineStr"/>
       <c r="W30" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="X30" t="n">
-        <v>0.6096889347566355</v>
+        <v>0.5875596764324247</v>
       </c>
       <c r="Y30" t="n">
-        <v>1.83</v>
+        <v>1.55</v>
       </c>
       <c r="Z30" t="inlineStr">
         <is>
@@ -3538,35 +3514,33 @@
         </is>
       </c>
       <c r="AA30" t="n">
-        <v>0.1394346392827025</v>
+        <v>-0.1623318209631667</v>
       </c>
       <c r="AB30" t="n">
-        <v>6.096889347566355</v>
+        <v>4.472523232774187</v>
       </c>
       <c r="AC30" t="n">
-        <v>0.3481985392255409</v>
-      </c>
-      <c r="AD30" t="n">
-        <v>0</v>
-      </c>
+        <v>0.2805131940097831</v>
+      </c>
+      <c r="AD30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="1" t="inlineStr">
         <is>
-          <t>KdZr6L8j</t>
+          <t>bT51grPp</t>
         </is>
       </c>
       <c r="B31" s="2" t="n">
-        <v>45745.58333333334</v>
+        <v>45746.3125</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>juventus</t>
+          <t>cagliari</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>genoa</t>
+          <t>monza</t>
         </is>
       </c>
       <c r="E31" t="n">
@@ -3586,37 +3560,37 @@
         </is>
       </c>
       <c r="I31" t="n">
-        <v>1.55</v>
+        <v>1.67</v>
       </c>
       <c r="J31" t="n">
-        <v>3.9</v>
+        <v>3.5</v>
       </c>
       <c r="K31" t="n">
-        <v>6.5</v>
+        <v>5.5</v>
       </c>
       <c r="L31" t="n">
-        <v>0.6112852664576801</v>
+        <v>0.5615519253208868</v>
       </c>
       <c r="M31" t="n">
-        <v>0.2429467084639498</v>
+        <v>0.2679404900816802</v>
       </c>
       <c r="N31" t="n">
-        <v>0.1457680250783699</v>
+        <v>0.1705075845974329</v>
       </c>
       <c r="O31" t="n">
-        <v>0.05541770057899109</v>
+        <v>0.06633486274204836</v>
       </c>
       <c r="P31" t="n">
         <v>1</v>
       </c>
       <c r="Q31" t="n">
-        <v>0.3284696946745644</v>
+        <v>0.3405051692089449</v>
       </c>
       <c r="R31" t="n">
-        <v>0.5570506233081103</v>
+        <v>0.4922092167600164</v>
       </c>
       <c r="S31" t="n">
-        <v>0.1144796820173254</v>
+        <v>0.1672856140310388</v>
       </c>
       <c r="T31" t="n">
         <v>1</v>
@@ -3624,17 +3598,15 @@
       <c r="U31" t="n">
         <v>1</v>
       </c>
-      <c r="V31" t="n">
-        <v>0</v>
-      </c>
+      <c r="V31" t="inlineStr"/>
       <c r="W31" t="n">
         <v>1</v>
       </c>
       <c r="X31" t="n">
-        <v>0.5570506233081103</v>
+        <v>0.4922092167600164</v>
       </c>
       <c r="Y31" t="n">
-        <v>1.55</v>
+        <v>1.67</v>
       </c>
       <c r="Z31" t="inlineStr">
         <is>
@@ -3642,35 +3614,33 @@
         </is>
       </c>
       <c r="AA31" t="n">
-        <v>-0.2483118797680528</v>
+        <v>-0.2656874746429443</v>
       </c>
       <c r="AB31" t="n">
-        <v>4.215028548275302</v>
+        <v>3.058137655206776</v>
       </c>
       <c r="AC31" t="n">
-        <v>0.2285809286335458</v>
-      </c>
-      <c r="AD31" t="n">
-        <v>0</v>
-      </c>
+        <v>0.1517040475510715</v>
+      </c>
+      <c r="AD31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="1" t="inlineStr">
         <is>
-          <t>n9AwS2V9</t>
+          <t>lErDBsoT</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
-        <v>45745.69791666666</v>
+        <v>45746.54166666666</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>lecce</t>
+          <t>inter</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>as roma</t>
+          <t>udinese</t>
         </is>
       </c>
       <c r="E32" t="n">
@@ -3690,55 +3660,53 @@
         </is>
       </c>
       <c r="I32" t="n">
+        <v>1.42</v>
+      </c>
+      <c r="J32" t="n">
         <v>4.33</v>
       </c>
-      <c r="J32" t="n">
-        <v>3.5</v>
-      </c>
       <c r="K32" t="n">
-        <v>1.85</v>
+        <v>8</v>
       </c>
       <c r="L32" t="n">
-        <v>0.2184511057505777</v>
+        <v>0.6642556080124874</v>
       </c>
       <c r="M32" t="n">
-        <v>0.2702552251142862</v>
+        <v>0.2178390215652961</v>
       </c>
       <c r="N32" t="n">
-        <v>0.511293669135136</v>
+        <v>0.1179053704222165</v>
       </c>
       <c r="O32" t="n">
-        <v>0.0572017084719163</v>
+        <v>0.06017223432976615</v>
       </c>
       <c r="P32" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q32" t="n">
-        <v>0.2981172198776336</v>
+        <v>0.2323405532291342</v>
       </c>
       <c r="R32" t="n">
-        <v>0.1233463517403995</v>
+        <v>0.7087880139175735</v>
       </c>
       <c r="S32" t="n">
-        <v>0.5785364283819668</v>
+        <v>0.05887143285329239</v>
       </c>
       <c r="T32" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="U32" t="n">
         <v>1</v>
       </c>
-      <c r="V32" t="n">
-        <v>0</v>
-      </c>
+      <c r="V32" t="inlineStr"/>
       <c r="W32" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="X32" t="n">
-        <v>0.5785364283819668</v>
+        <v>0.7087880139175735</v>
       </c>
       <c r="Y32" t="n">
-        <v>1.85</v>
+        <v>1.42</v>
       </c>
       <c r="Z32" t="inlineStr">
         <is>
@@ -3746,35 +3714,33 @@
         </is>
       </c>
       <c r="AA32" t="n">
-        <v>0.08269693236075142</v>
+        <v>0.01542614229274848</v>
       </c>
       <c r="AB32" t="n">
-        <v>5.785364283819669</v>
+        <v>7.087880139175735</v>
       </c>
       <c r="AC32" t="n">
-        <v>0.2804192085043332</v>
-      </c>
-      <c r="AD32" t="n">
-        <v>0</v>
-      </c>
+        <v>0.4764474606884394</v>
+      </c>
+      <c r="AD32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="1" t="inlineStr">
         <is>
-          <t>bT51grPp</t>
+          <t>tASB9fFr</t>
         </is>
       </c>
       <c r="B33" s="2" t="n">
-        <v>45746.3125</v>
+        <v>45746.65625</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>cagliari</t>
+          <t>napoli</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>monza</t>
+          <t>ac milan</t>
         </is>
       </c>
       <c r="E33" t="n">
@@ -3794,37 +3760,37 @@
         </is>
       </c>
       <c r="I33" t="n">
-        <v>1.67</v>
+        <v>1.9</v>
       </c>
       <c r="J33" t="n">
-        <v>3.5</v>
+        <v>3.7</v>
       </c>
       <c r="K33" t="n">
-        <v>5.5</v>
+        <v>3.8</v>
       </c>
       <c r="L33" t="n">
-        <v>0.5615519253208868</v>
+        <v>0.4966442953020134</v>
       </c>
       <c r="M33" t="n">
-        <v>0.2679404900816802</v>
+        <v>0.2550335570469798</v>
       </c>
       <c r="N33" t="n">
-        <v>0.1705075845974329</v>
+        <v>0.2483221476510067</v>
       </c>
       <c r="O33" t="n">
-        <v>0.06633486274204836</v>
+        <v>0.0597439544807965</v>
       </c>
       <c r="P33" t="n">
         <v>1</v>
       </c>
       <c r="Q33" t="n">
-        <v>0.3486130582070131</v>
+        <v>0.3625456381538017</v>
       </c>
       <c r="R33" t="n">
-        <v>0.4546192737494166</v>
+        <v>0.3642414432082768</v>
       </c>
       <c r="S33" t="n">
-        <v>0.1967676680435703</v>
+        <v>0.2732129186379215</v>
       </c>
       <c r="T33" t="n">
         <v>1</v>
@@ -3839,10 +3805,10 @@
         <v>1</v>
       </c>
       <c r="X33" t="n">
-        <v>0.4546192737494166</v>
+        <v>0.3642414432082768</v>
       </c>
       <c r="Y33" t="n">
-        <v>1.67</v>
+        <v>1.9</v>
       </c>
       <c r="Z33" t="inlineStr">
         <is>
@@ -3850,35 +3816,35 @@
         </is>
       </c>
       <c r="AA33" t="n">
-        <v>-0.3593818102066781</v>
+        <v>-0.3421569532269712</v>
       </c>
       <c r="AB33" t="n">
-        <v>2.979259216435993</v>
+        <v>0.384302220570921</v>
       </c>
       <c r="AC33" t="n">
-        <v>0.1060062155424035</v>
+        <v>0.001695805054475141</v>
       </c>
       <c r="AD33" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="1" t="inlineStr">
         <is>
-          <t>KYjdFPo4</t>
+          <t>hnk4D3GG</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
-        <v>45746.41666666666</v>
+        <v>45747.5625</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>fiorentina</t>
+          <t>verona</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>atalanta</t>
+          <t>parma</t>
         </is>
       </c>
       <c r="E34" t="n">
@@ -3898,55 +3864,53 @@
         </is>
       </c>
       <c r="I34" t="n">
-        <v>4.1</v>
+        <v>2.35</v>
       </c>
       <c r="J34" t="n">
-        <v>3.4</v>
+        <v>3.1</v>
       </c>
       <c r="K34" t="n">
-        <v>1.95</v>
+        <v>3.2</v>
       </c>
       <c r="L34" t="n">
-        <v>0.2321022230001751</v>
+        <v>0.4012133468149647</v>
       </c>
       <c r="M34" t="n">
-        <v>0.2798879747943288</v>
+        <v>0.3041456016177958</v>
       </c>
       <c r="N34" t="n">
-        <v>0.4880098022054963</v>
+        <v>0.2946410515672397</v>
       </c>
       <c r="O34" t="n">
-        <v>0.05084059890372661</v>
+        <v>0.06061256005490723</v>
       </c>
       <c r="P34" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q34" t="n">
-        <v>0.3690805324216265</v>
+        <v>0.3279663294899083</v>
       </c>
       <c r="R34" t="n">
-        <v>0.2330805225571006</v>
+        <v>0.3864384995556649</v>
       </c>
       <c r="S34" t="n">
-        <v>0.397838945021273</v>
+        <v>0.2855951709544269</v>
       </c>
       <c r="T34" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="U34" t="n">
         <v>1</v>
       </c>
-      <c r="V34" t="n">
-        <v>0</v>
-      </c>
+      <c r="V34" t="inlineStr"/>
       <c r="W34" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="X34" t="n">
-        <v>0.397838945021273</v>
+        <v>0.3864384995556649</v>
       </c>
       <c r="Y34" t="n">
-        <v>1.95</v>
+        <v>2.35</v>
       </c>
       <c r="Z34" t="inlineStr">
         <is>
@@ -3954,35 +3918,33 @@
         </is>
       </c>
       <c r="AA34" t="n">
-        <v>-0.2360147970615977</v>
+        <v>-0.06805150077347215</v>
       </c>
       <c r="AB34" t="n">
-        <v>0.6112970097781179</v>
+        <v>3.471283591732988</v>
       </c>
       <c r="AC34" t="n">
-        <v>0.02875841259964651</v>
-      </c>
-      <c r="AD34" t="n">
-        <v>0</v>
-      </c>
+        <v>0.05847217006575661</v>
+      </c>
+      <c r="AD34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="1" t="inlineStr">
         <is>
-          <t>lErDBsoT</t>
+          <t>0hCVTO0c</t>
         </is>
       </c>
       <c r="B35" s="2" t="n">
-        <v>45746.54166666666</v>
+        <v>45747.65625</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>inter</t>
+          <t>lazio</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>udinese</t>
+          <t>torino</t>
         </is>
       </c>
       <c r="E35" t="n">
@@ -4002,37 +3964,37 @@
         </is>
       </c>
       <c r="I35" t="n">
-        <v>1.42</v>
+        <v>1.75</v>
       </c>
       <c r="J35" t="n">
-        <v>4.33</v>
+        <v>3.3</v>
       </c>
       <c r="K35" t="n">
-        <v>8</v>
+        <v>5.25</v>
       </c>
       <c r="L35" t="n">
-        <v>0.6642556080124874</v>
+        <v>0.5365853658536586</v>
       </c>
       <c r="M35" t="n">
-        <v>0.2178390215652961</v>
+        <v>0.2845528455284553</v>
       </c>
       <c r="N35" t="n">
-        <v>0.1179053704222165</v>
+        <v>0.1788617886178862</v>
       </c>
       <c r="O35" t="n">
-        <v>0.06017223432976615</v>
+        <v>0.06493506493506485</v>
       </c>
       <c r="P35" t="n">
         <v>1</v>
       </c>
       <c r="Q35" t="n">
-        <v>0.2385021057602099</v>
+        <v>0.349771137860809</v>
       </c>
       <c r="R35" t="n">
-        <v>0.6991954347288691</v>
+        <v>0.5213215439140768</v>
       </c>
       <c r="S35" t="n">
-        <v>0.06230245951092105</v>
+        <v>0.1289073182251143</v>
       </c>
       <c r="T35" t="n">
         <v>1</v>
@@ -4040,17 +4002,15 @@
       <c r="U35" t="n">
         <v>1</v>
       </c>
-      <c r="V35" t="n">
-        <v>0</v>
-      </c>
+      <c r="V35" t="inlineStr"/>
       <c r="W35" t="n">
         <v>1</v>
       </c>
       <c r="X35" t="n">
-        <v>0.6991954347288691</v>
+        <v>0.5213215439140768</v>
       </c>
       <c r="Y35" t="n">
-        <v>1.42</v>
+        <v>1.75</v>
       </c>
       <c r="Z35" t="inlineStr">
         <is>
@@ -4058,35 +4018,33 @@
         </is>
       </c>
       <c r="AA35" t="n">
-        <v>-0.01700591115477593</v>
+        <v>-0.1169163975338208</v>
       </c>
       <c r="AB35" t="n">
-        <v>6.873061253973872</v>
+        <v>4.308209117386149</v>
       </c>
       <c r="AC35" t="n">
-        <v>0.4606933289686592</v>
-      </c>
-      <c r="AD35" t="n">
-        <v>0</v>
-      </c>
+        <v>0.1715504060532678</v>
+      </c>
+      <c r="AD35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="1" t="inlineStr">
         <is>
-          <t>tASB9fFr</t>
+          <t>ENQJ7Yqe</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
-        <v>45746.65625</v>
+        <v>45745.45833333334</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>napoli</t>
+          <t>venezia</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>ac milan</t>
+          <t>bologna</t>
         </is>
       </c>
       <c r="E36" t="n">
@@ -4106,40 +4064,40 @@
         </is>
       </c>
       <c r="I36" t="n">
-        <v>1.9</v>
+        <v>4.5</v>
       </c>
       <c r="J36" t="n">
-        <v>3.7</v>
+        <v>3.5</v>
       </c>
       <c r="K36" t="n">
-        <v>3.8</v>
+        <v>1.83</v>
       </c>
       <c r="L36" t="n">
-        <v>0.4966442953020134</v>
+        <v>0.2107601184600197</v>
       </c>
       <c r="M36" t="n">
-        <v>0.2550335570469798</v>
+        <v>0.2709772951628825</v>
       </c>
       <c r="N36" t="n">
-        <v>0.2483221476510067</v>
+        <v>0.5182625863770978</v>
       </c>
       <c r="O36" t="n">
-        <v>0.0597439544807965</v>
+        <v>0.05438459536820184</v>
       </c>
       <c r="P36" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q36" t="n">
-        <v>0.3607607548304306</v>
+        <v>0.2462719916224489</v>
       </c>
       <c r="R36" t="n">
-        <v>0.3432335964412306</v>
+        <v>0.09185271032005367</v>
       </c>
       <c r="S36" t="n">
-        <v>0.2960056487283387</v>
+        <v>0.6618752980574975</v>
       </c>
       <c r="T36" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="U36" t="n">
         <v>1</v>
@@ -4148,13 +4106,13 @@
         <v>0</v>
       </c>
       <c r="W36" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="X36" t="n">
-        <v>0.3607607548304306</v>
+        <v>0.6618752980574975</v>
       </c>
       <c r="Y36" t="n">
-        <v>3.7</v>
+        <v>1.83</v>
       </c>
       <c r="Z36" t="inlineStr">
         <is>
@@ -4162,35 +4120,35 @@
         </is>
       </c>
       <c r="AA36" t="n">
-        <v>0.1240054788417012</v>
+        <v>0.254496139090627</v>
       </c>
       <c r="AB36" t="n">
-        <v>3.607607548304306</v>
+        <v>6.618752980574975</v>
       </c>
       <c r="AC36" t="n">
-        <v>0.01752715838919999</v>
+        <v>0.4156033064350485</v>
       </c>
       <c r="AD36" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="1" t="inlineStr">
         <is>
-          <t>hnk4D3GG</t>
+          <t>n9AwS2V9</t>
         </is>
       </c>
       <c r="B37" s="2" t="n">
-        <v>45747.5625</v>
+        <v>45745.69791666666</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>verona</t>
+          <t>lecce</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>parma</t>
+          <t>as roma</t>
         </is>
       </c>
       <c r="E37" t="n">
@@ -4210,55 +4168,53 @@
         </is>
       </c>
       <c r="I37" t="n">
-        <v>2.35</v>
+        <v>4.33</v>
       </c>
       <c r="J37" t="n">
-        <v>3.1</v>
+        <v>3.5</v>
       </c>
       <c r="K37" t="n">
-        <v>3.2</v>
+        <v>1.85</v>
       </c>
       <c r="L37" t="n">
-        <v>0.4012133468149647</v>
+        <v>0.2184511057505777</v>
       </c>
       <c r="M37" t="n">
-        <v>0.3041456016177958</v>
+        <v>0.2702552251142862</v>
       </c>
       <c r="N37" t="n">
-        <v>0.2946410515672397</v>
+        <v>0.511293669135136</v>
       </c>
       <c r="O37" t="n">
-        <v>0.06061256005490723</v>
+        <v>0.0572017084719163</v>
       </c>
       <c r="P37" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q37" t="n">
-        <v>0.3266776596454697</v>
+        <v>0.2902605859317151</v>
       </c>
       <c r="R37" t="n">
-        <v>0.4010833772895466</v>
+        <v>0.1012659112783525</v>
       </c>
       <c r="S37" t="n">
-        <v>0.2722389630649837</v>
+        <v>0.6084735027899324</v>
       </c>
       <c r="T37" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="U37" t="n">
         <v>1</v>
       </c>
-      <c r="V37" t="n">
-        <v>0</v>
-      </c>
+      <c r="V37" t="inlineStr"/>
       <c r="W37" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="X37" t="n">
-        <v>0.4010833772895466</v>
+        <v>0.6084735027899324</v>
       </c>
       <c r="Y37" t="n">
-        <v>2.35</v>
+        <v>1.85</v>
       </c>
       <c r="Z37" t="inlineStr">
         <is>
@@ -4266,35 +4222,33 @@
         </is>
       </c>
       <c r="AA37" t="n">
-        <v>-0.04255856545893739</v>
+        <v>0.1478540943074999</v>
       </c>
       <c r="AB37" t="n">
-        <v>3.84024142287151</v>
+        <v>6.084735027899324</v>
       </c>
       <c r="AC37" t="n">
-        <v>0.07440571764407694</v>
-      </c>
-      <c r="AD37" t="n">
-        <v>0</v>
-      </c>
+        <v>0.3182129168582173</v>
+      </c>
+      <c r="AD37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="1" t="inlineStr">
         <is>
-          <t>0hCVTO0c</t>
+          <t>KYjdFPo4</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
-        <v>45747.65625</v>
+        <v>45746.41666666666</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>lazio</t>
+          <t>fiorentina</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>torino</t>
+          <t>atalanta</t>
         </is>
       </c>
       <c r="E38" t="n">
@@ -4314,55 +4268,53 @@
         </is>
       </c>
       <c r="I38" t="n">
-        <v>1.75</v>
+        <v>4.1</v>
       </c>
       <c r="J38" t="n">
-        <v>3.3</v>
+        <v>3.4</v>
       </c>
       <c r="K38" t="n">
-        <v>5.25</v>
+        <v>1.95</v>
       </c>
       <c r="L38" t="n">
-        <v>0.5365853658536586</v>
+        <v>0.2321022230001751</v>
       </c>
       <c r="M38" t="n">
-        <v>0.2845528455284553</v>
+        <v>0.2798879747943288</v>
       </c>
       <c r="N38" t="n">
-        <v>0.1788617886178862</v>
+        <v>0.4880098022054963</v>
       </c>
       <c r="O38" t="n">
-        <v>0.06493506493506485</v>
+        <v>0.05084059890372661</v>
       </c>
       <c r="P38" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q38" t="n">
-        <v>0.3534311464888651</v>
+        <v>0.369369103700268</v>
       </c>
       <c r="R38" t="n">
-        <v>0.4908873714108951</v>
+        <v>0.1941298377994344</v>
       </c>
       <c r="S38" t="n">
-        <v>0.1556814821002398</v>
+        <v>0.4365010585002975</v>
       </c>
       <c r="T38" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="U38" t="n">
         <v>1</v>
       </c>
-      <c r="V38" t="n">
-        <v>0</v>
-      </c>
+      <c r="V38" t="inlineStr"/>
       <c r="W38" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="X38" t="n">
-        <v>0.4908873714108951</v>
+        <v>0.4365010585002975</v>
       </c>
       <c r="Y38" t="n">
-        <v>1.75</v>
+        <v>1.95</v>
       </c>
       <c r="Z38" t="inlineStr">
         <is>
@@ -4370,17 +4322,15 @@
         </is>
       </c>
       <c r="AA38" t="n">
-        <v>-0.1879294667079114</v>
+        <v>-0.1566557220257051</v>
       </c>
       <c r="AB38" t="n">
-        <v>3.997060818255914</v>
+        <v>3.357775793333232</v>
       </c>
       <c r="AC38" t="n">
-        <v>0.13745622492203</v>
-      </c>
-      <c r="AD38" t="n">
-        <v>0</v>
-      </c>
+        <v>0.06713195480002954</v>
+      </c>
+      <c r="AD38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="1" t="inlineStr">
@@ -4442,13 +4392,13 @@
         <v>1</v>
       </c>
       <c r="Q39" t="n">
-        <v>0.2212390086395661</v>
+        <v>0.2271806093009376</v>
       </c>
       <c r="R39" t="n">
-        <v>0.6421017128507369</v>
+        <v>0.6849720303120109</v>
       </c>
       <c r="S39" t="n">
-        <v>0.1366592785096971</v>
+        <v>0.08784736038705153</v>
       </c>
       <c r="T39" t="n">
         <v>1</v>
@@ -4463,7 +4413,7 @@
         <v>1</v>
       </c>
       <c r="X39" t="n">
-        <v>0.6421017128507369</v>
+        <v>0.6849720303120109</v>
       </c>
       <c r="Y39" t="n">
         <v>1.29</v>
@@ -4474,13 +4424,13 @@
         </is>
       </c>
       <c r="AA39" t="n">
-        <v>-0.5920303118018942</v>
+        <v>-0.4013313134396754</v>
       </c>
       <c r="AB39" t="n">
-        <v>3.009182336005672</v>
+        <v>5.493373205728582</v>
       </c>
       <c r="AC39" t="n">
-        <v>0.4208627042111708</v>
+        <v>0.4577914210110733</v>
       </c>
       <c r="AD39" t="n">
         <v>1</v>
@@ -4546,13 +4496,13 @@
         <v>1</v>
       </c>
       <c r="Q40" t="n">
-        <v>0.2709696900930051</v>
+        <v>0.2438008259195674</v>
       </c>
       <c r="R40" t="n">
-        <v>0.5740893586634623</v>
+        <v>0.5737944283909402</v>
       </c>
       <c r="S40" t="n">
-        <v>0.1549409512435326</v>
+        <v>0.1824047456894923</v>
       </c>
       <c r="T40" t="n">
         <v>1</v>
@@ -4565,7 +4515,7 @@
         <v>1</v>
       </c>
       <c r="X40" t="n">
-        <v>0.5740893586634623</v>
+        <v>0.5737944283909402</v>
       </c>
       <c r="Y40" t="n">
         <v>1.33</v>
@@ -4576,33 +4526,33 @@
         </is>
       </c>
       <c r="AA40" t="n">
-        <v>-0.7165489484169545</v>
+        <v>-0.7177376067880287</v>
       </c>
       <c r="AB40" t="n">
-        <v>2.211581141116763</v>
+        <v>3.762844844580467</v>
       </c>
       <c r="AC40" t="n">
-        <v>0.3031196685704572</v>
+        <v>0.3299936024713728</v>
       </c>
       <c r="AD40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="1" t="inlineStr">
         <is>
-          <t>Kjbn1lFr</t>
+          <t>6XRGiceU</t>
         </is>
       </c>
       <c r="B41" s="2" t="n">
-        <v>45745.51041666666</v>
+        <v>45745.70833333334</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>espanyol</t>
+          <t>real madrid</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>atl  madrid</t>
+          <t>leganes</t>
         </is>
       </c>
       <c r="E41" t="n">
@@ -4622,53 +4572,53 @@
         </is>
       </c>
       <c r="I41" t="n">
+        <v>1.18</v>
+      </c>
+      <c r="J41" t="n">
         <v>7</v>
       </c>
-      <c r="J41" t="n">
-        <v>4</v>
-      </c>
       <c r="K41" t="n">
-        <v>1.5</v>
+        <v>15</v>
       </c>
       <c r="L41" t="n">
-        <v>0.1348314606741573</v>
+        <v>0.8017715332926084</v>
       </c>
       <c r="M41" t="n">
-        <v>0.2359550561797753</v>
+        <v>0.1351557727550397</v>
       </c>
       <c r="N41" t="n">
-        <v>0.6292134831460674</v>
+        <v>0.06307269395235185</v>
       </c>
       <c r="O41" t="n">
-        <v>0.05952380952380953</v>
+        <v>0.0569814366424537</v>
       </c>
       <c r="P41" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q41" t="n">
-        <v>0.3279499036156451</v>
+        <v>0.205466613788591</v>
       </c>
       <c r="R41" t="n">
-        <v>0.08595676360993978</v>
+        <v>0.7095148103432004</v>
       </c>
       <c r="S41" t="n">
-        <v>0.5860933327744151</v>
+        <v>0.08501857586820863</v>
       </c>
       <c r="T41" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="U41" t="n">
         <v>1</v>
       </c>
       <c r="V41" t="inlineStr"/>
       <c r="W41" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="X41" t="n">
-        <v>0.5860933327744151</v>
+        <v>0.7095148103432004</v>
       </c>
       <c r="Y41" t="n">
-        <v>1.5</v>
+        <v>1.18</v>
       </c>
       <c r="Z41" t="inlineStr">
         <is>
@@ -4676,33 +4626,33 @@
         </is>
       </c>
       <c r="AA41" t="n">
-        <v>-0.2417200016767547</v>
+        <v>-0.9042917988612422</v>
       </c>
       <c r="AB41" t="n">
-        <v>4.471190554563081</v>
+        <v>4.089208157662595</v>
       </c>
       <c r="AC41" t="n">
-        <v>0.25814342915877</v>
+        <v>0.5040481965546094</v>
       </c>
       <c r="AD41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="1" t="inlineStr">
         <is>
-          <t>Olz0eud5</t>
+          <t>lWLHr2Ca</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
-        <v>45745.60416666666</v>
+        <v>45746.46875</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>alaves</t>
+          <t>barcelona</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>rayo vallecano</t>
+          <t>girona</t>
         </is>
       </c>
       <c r="E42" t="n">
@@ -4722,53 +4672,55 @@
         </is>
       </c>
       <c r="I42" t="n">
-        <v>2.25</v>
+        <v>1.27</v>
       </c>
       <c r="J42" t="n">
-        <v>2.9</v>
+        <v>6</v>
       </c>
       <c r="K42" t="n">
-        <v>3.6</v>
+        <v>9</v>
       </c>
       <c r="L42" t="n">
-        <v>0.4165170556552962</v>
+        <v>0.7392197125256674</v>
       </c>
       <c r="M42" t="n">
-        <v>0.3231597845601437</v>
+        <v>0.1564681724845996</v>
       </c>
       <c r="N42" t="n">
-        <v>0.2603231597845602</v>
+        <v>0.1043121149897331</v>
       </c>
       <c r="O42" t="n">
-        <v>0.06704980842911867</v>
+        <v>0.06517935258092722</v>
       </c>
       <c r="P42" t="n">
         <v>1</v>
       </c>
       <c r="Q42" t="n">
-        <v>0.4260813451083732</v>
+        <v>0.2224295055004011</v>
       </c>
       <c r="R42" t="n">
-        <v>0.2714713620697216</v>
+        <v>0.5948268904309406</v>
       </c>
       <c r="S42" t="n">
-        <v>0.3024472928219052</v>
+        <v>0.1827436040686583</v>
       </c>
       <c r="T42" t="n">
+        <v>1</v>
+      </c>
+      <c r="U42" t="n">
+        <v>1</v>
+      </c>
+      <c r="V42" t="n">
         <v>0</v>
       </c>
-      <c r="U42" t="n">
-        <v>1</v>
-      </c>
-      <c r="V42" t="inlineStr"/>
       <c r="W42" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X42" t="n">
-        <v>0.4260813451083732</v>
+        <v>0.5948268904309406</v>
       </c>
       <c r="Y42" t="n">
-        <v>2.9</v>
+        <v>1.27</v>
       </c>
       <c r="Z42" t="inlineStr">
         <is>
@@ -4776,33 +4728,35 @@
         </is>
       </c>
       <c r="AA42" t="n">
-        <v>0.1240188951654117</v>
+        <v>-0.9058142561211311</v>
       </c>
       <c r="AB42" t="n">
-        <v>4.260813451083732</v>
+        <v>3.424503266163232</v>
       </c>
       <c r="AC42" t="n">
-        <v>0.123634052286468</v>
-      </c>
-      <c r="AD42" t="inlineStr"/>
+        <v>0.3723973849305395</v>
+      </c>
+      <c r="AD42" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="1" t="inlineStr">
         <is>
-          <t>6XRGiceU</t>
+          <t>t6I9pOsm</t>
         </is>
       </c>
       <c r="B43" s="2" t="n">
-        <v>45745.70833333334</v>
+        <v>45746.5625</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>real madrid</t>
+          <t>ath bilbao</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>leganes</t>
+          <t>osasuna</t>
         </is>
       </c>
       <c r="E43" t="n">
@@ -4822,37 +4776,37 @@
         </is>
       </c>
       <c r="I43" t="n">
-        <v>1.18</v>
+        <v>1.53</v>
       </c>
       <c r="J43" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="K43" t="n">
-        <v>15</v>
+        <v>6.25</v>
       </c>
       <c r="L43" t="n">
-        <v>0.8017715332926084</v>
+        <v>0.6145148405333989</v>
       </c>
       <c r="M43" t="n">
-        <v>0.1351557727550397</v>
+        <v>0.2350519265040251</v>
       </c>
       <c r="N43" t="n">
-        <v>0.06307269395235185</v>
+        <v>0.150433232962576</v>
       </c>
       <c r="O43" t="n">
-        <v>0.0569814366424537</v>
+        <v>0.06359477124183011</v>
       </c>
       <c r="P43" t="n">
         <v>1</v>
       </c>
       <c r="Q43" t="n">
-        <v>0.17407084540444</v>
+        <v>0.3696346691853458</v>
       </c>
       <c r="R43" t="n">
-        <v>0.721558009928736</v>
+        <v>0.4363798225991631</v>
       </c>
       <c r="S43" t="n">
-        <v>0.1043711446668241</v>
+        <v>0.1939855082154911</v>
       </c>
       <c r="T43" t="n">
         <v>1</v>
@@ -4860,15 +4814,17 @@
       <c r="U43" t="n">
         <v>1</v>
       </c>
-      <c r="V43" t="inlineStr"/>
+      <c r="V43" t="n">
+        <v>0</v>
+      </c>
       <c r="W43" t="n">
         <v>1</v>
       </c>
       <c r="X43" t="n">
-        <v>0.721558009928736</v>
+        <v>0.4363798225991631</v>
       </c>
       <c r="Y43" t="n">
-        <v>1.18</v>
+        <v>1.53</v>
       </c>
       <c r="Z43" t="inlineStr">
         <is>
@@ -4876,33 +4832,35 @@
         </is>
       </c>
       <c r="AA43" t="n">
-        <v>-0.8253419349116203</v>
+        <v>-0.627054474383548</v>
       </c>
       <c r="AB43" t="n">
-        <v>2.323655541606495</v>
+        <v>3.038763417529559</v>
       </c>
       <c r="AC43" t="n">
-        <v>0.547487164524296</v>
-      </c>
-      <c r="AD43" t="inlineStr"/>
+        <v>0.06674515341381726</v>
+      </c>
+      <c r="AD43" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="1" t="inlineStr">
         <is>
-          <t>f9rqaNdt</t>
+          <t>GrDYvKBO</t>
         </is>
       </c>
       <c r="B44" s="2" t="n">
-        <v>45746.375</v>
+        <v>45747.66666666666</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>getafe</t>
+          <t>celta vigo</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>villarreal</t>
+          <t>las palmas</t>
         </is>
       </c>
       <c r="E44" t="n">
@@ -4922,53 +4880,53 @@
         </is>
       </c>
       <c r="I44" t="n">
-        <v>3.1</v>
+        <v>1.57</v>
       </c>
       <c r="J44" t="n">
-        <v>3.2</v>
+        <v>4.1</v>
       </c>
       <c r="K44" t="n">
-        <v>2.35</v>
+        <v>5.5</v>
       </c>
       <c r="L44" t="n">
-        <v>0.3041456016177958</v>
+        <v>0.5993833395353783</v>
       </c>
       <c r="M44" t="n">
-        <v>0.2946410515672397</v>
+        <v>0.2295199617245229</v>
       </c>
       <c r="N44" t="n">
-        <v>0.4012133468149647</v>
+        <v>0.1710966987400989</v>
       </c>
       <c r="O44" t="n">
-        <v>0.06061256005490723</v>
+        <v>0.06266329600180764</v>
       </c>
       <c r="P44" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q44" t="n">
-        <v>0.2743335183836801</v>
+        <v>0.3579581139513563</v>
       </c>
       <c r="R44" t="n">
-        <v>0.2231546704463831</v>
+        <v>0.3632940683825504</v>
       </c>
       <c r="S44" t="n">
-        <v>0.5025118111699368</v>
+        <v>0.2787478176660933</v>
       </c>
       <c r="T44" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="U44" t="n">
         <v>1</v>
       </c>
       <c r="V44" t="inlineStr"/>
       <c r="W44" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="X44" t="n">
-        <v>0.5025118111699368</v>
+        <v>0.3632940683825504</v>
       </c>
       <c r="Y44" t="n">
-        <v>2.35</v>
+        <v>1.57</v>
       </c>
       <c r="Z44" t="inlineStr">
         <is>
@@ -4976,33 +4934,33 @@
         </is>
       </c>
       <c r="AA44" t="n">
-        <v>0.1340020416661863</v>
+        <v>-0.7537338818235017</v>
       </c>
       <c r="AB44" t="n">
-        <v>5.025118111699368</v>
+        <v>0.4650283985134143</v>
       </c>
       <c r="AC44" t="n">
-        <v>0.2281782927862567</v>
+        <v>0.005335954431194057</v>
       </c>
       <c r="AD44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="1" t="inlineStr">
         <is>
-          <t>lWLHr2Ca</t>
+          <t>Olz0eud5</t>
         </is>
       </c>
       <c r="B45" s="2" t="n">
-        <v>45746.46875</v>
+        <v>45745.60416666666</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>barcelona</t>
+          <t>alaves</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>girona</t>
+          <t>rayo vallecano</t>
         </is>
       </c>
       <c r="E45" t="n">
@@ -5022,55 +4980,53 @@
         </is>
       </c>
       <c r="I45" t="n">
-        <v>1.27</v>
+        <v>2.25</v>
       </c>
       <c r="J45" t="n">
-        <v>6</v>
+        <v>2.9</v>
       </c>
       <c r="K45" t="n">
-        <v>9</v>
+        <v>3.6</v>
       </c>
       <c r="L45" t="n">
-        <v>0.7392197125256674</v>
+        <v>0.4165170556552962</v>
       </c>
       <c r="M45" t="n">
-        <v>0.1564681724845996</v>
+        <v>0.3231597845601437</v>
       </c>
       <c r="N45" t="n">
-        <v>0.1043121149897331</v>
+        <v>0.2603231597845602</v>
       </c>
       <c r="O45" t="n">
-        <v>0.06517935258092722</v>
+        <v>0.06704980842911867</v>
       </c>
       <c r="P45" t="n">
         <v>1</v>
       </c>
       <c r="Q45" t="n">
-        <v>0.1864685276451138</v>
+        <v>0.4883929281835071</v>
       </c>
       <c r="R45" t="n">
-        <v>0.5270741101073164</v>
+        <v>0.2537286937651811</v>
       </c>
       <c r="S45" t="n">
-        <v>0.2864573622475697</v>
+        <v>0.2578783780513118</v>
       </c>
       <c r="T45" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U45" t="n">
         <v>1</v>
       </c>
-      <c r="V45" t="n">
+      <c r="V45" t="inlineStr"/>
+      <c r="W45" t="n">
         <v>0</v>
       </c>
-      <c r="W45" t="n">
-        <v>1</v>
-      </c>
       <c r="X45" t="n">
-        <v>0.5270741101073164</v>
+        <v>0.4883929281835071</v>
       </c>
       <c r="Y45" t="n">
-        <v>1.27</v>
+        <v>2.9</v>
       </c>
       <c r="Z45" t="inlineStr">
         <is>
@@ -5078,35 +5034,33 @@
         </is>
       </c>
       <c r="AA45" t="n">
-        <v>-1.224503259865586</v>
+        <v>0.2191260482800898</v>
       </c>
       <c r="AB45" t="n">
-        <v>0.838166224734428</v>
+        <v>4.883929281835071</v>
       </c>
       <c r="AC45" t="n">
-        <v>0.2406167478597467</v>
-      </c>
-      <c r="AD45" t="n">
-        <v>1</v>
-      </c>
+        <v>0.2305145501321953</v>
+      </c>
+      <c r="AD45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="1" t="inlineStr">
         <is>
-          <t>t6I9pOsm</t>
+          <t>Kjbn1lFr</t>
         </is>
       </c>
       <c r="B46" s="2" t="n">
-        <v>45746.5625</v>
+        <v>45745.51041666666</v>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>ath bilbao</t>
+          <t>espanyol</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>osasuna</t>
+          <t>atl  madrid</t>
         </is>
       </c>
       <c r="E46" t="n">
@@ -5126,55 +5080,53 @@
         </is>
       </c>
       <c r="I46" t="n">
-        <v>1.53</v>
+        <v>7</v>
       </c>
       <c r="J46" t="n">
         <v>4</v>
       </c>
       <c r="K46" t="n">
-        <v>6.25</v>
+        <v>1.5</v>
       </c>
       <c r="L46" t="n">
-        <v>0.6145148405333989</v>
+        <v>0.1348314606741573</v>
       </c>
       <c r="M46" t="n">
-        <v>0.2350519265040251</v>
+        <v>0.2359550561797753</v>
       </c>
       <c r="N46" t="n">
-        <v>0.150433232962576</v>
+        <v>0.6292134831460674</v>
       </c>
       <c r="O46" t="n">
-        <v>0.06359477124183011</v>
+        <v>0.05952380952380953</v>
       </c>
       <c r="P46" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q46" t="n">
-        <v>0.342018365621624</v>
+        <v>0.3255062547097365</v>
       </c>
       <c r="R46" t="n">
-        <v>0.4186180202669092</v>
+        <v>0.06197795970074563</v>
       </c>
       <c r="S46" t="n">
-        <v>0.2393636141114669</v>
+        <v>0.6125157855895179</v>
       </c>
       <c r="T46" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="U46" t="n">
         <v>1</v>
       </c>
-      <c r="V46" t="n">
-        <v>0</v>
-      </c>
+      <c r="V46" t="inlineStr"/>
       <c r="W46" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="X46" t="n">
-        <v>0.4186180202669092</v>
+        <v>0.6125157855895179</v>
       </c>
       <c r="Y46" t="n">
-        <v>1.53</v>
+        <v>1.5</v>
       </c>
       <c r="Z46" t="inlineStr">
         <is>
@@ -5182,35 +5134,33 @@
         </is>
       </c>
       <c r="AA46" t="n">
-        <v>-0.6783291113049601</v>
+        <v>-0.1624526432314463</v>
       </c>
       <c r="AB46" t="n">
-        <v>1.714525164394315</v>
+        <v>4.661443205042167</v>
       </c>
       <c r="AC46" t="n">
-        <v>0.07659965464528518</v>
-      </c>
-      <c r="AD46" t="n">
-        <v>1</v>
-      </c>
+        <v>0.2870095308797814</v>
+      </c>
+      <c r="AD46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="1" t="inlineStr">
         <is>
-          <t>A5Y7gJQH</t>
+          <t>f9rqaNdt</t>
         </is>
       </c>
       <c r="B47" s="2" t="n">
-        <v>45746.5625</v>
+        <v>45746.375</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>valencia</t>
+          <t>getafe</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>mallorca</t>
+          <t>villarreal</t>
         </is>
       </c>
       <c r="E47" t="n">
@@ -5230,37 +5180,37 @@
         </is>
       </c>
       <c r="I47" t="n">
-        <v>2.05</v>
+        <v>3.1</v>
       </c>
       <c r="J47" t="n">
-        <v>3.1</v>
+        <v>3.2</v>
       </c>
       <c r="K47" t="n">
-        <v>4.1</v>
+        <v>2.35</v>
       </c>
       <c r="L47" t="n">
-        <v>0.4626865671641791</v>
+        <v>0.3041456016177958</v>
       </c>
       <c r="M47" t="n">
-        <v>0.3059701492537313</v>
+        <v>0.2946410515672397</v>
       </c>
       <c r="N47" t="n">
-        <v>0.2313432835820896</v>
+        <v>0.4012133468149647</v>
       </c>
       <c r="O47" t="n">
-        <v>0.0542879622344612</v>
+        <v>0.06061256005490723</v>
       </c>
       <c r="P47" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q47" t="n">
-        <v>0.2780698635604373</v>
+        <v>0.3042088466944337</v>
       </c>
       <c r="R47" t="n">
-        <v>0.3154884226278944</v>
+        <v>0.2284635603262672</v>
       </c>
       <c r="S47" t="n">
-        <v>0.4064417138116683</v>
+        <v>0.4673275929792992</v>
       </c>
       <c r="T47" t="n">
         <v>2</v>
@@ -5273,10 +5223,10 @@
         <v>2</v>
       </c>
       <c r="X47" t="n">
-        <v>0.4064417138116683</v>
+        <v>0.4673275929792992</v>
       </c>
       <c r="Y47" t="n">
-        <v>4.1</v>
+        <v>2.35</v>
       </c>
       <c r="Z47" t="inlineStr">
         <is>
@@ -5284,33 +5234,33 @@
         </is>
       </c>
       <c r="AA47" t="n">
-        <v>0.2149712989122065</v>
+        <v>0.07275543963063189</v>
       </c>
       <c r="AB47" t="n">
-        <v>4.064417138116683</v>
+        <v>4.673275929792991</v>
       </c>
       <c r="AC47" t="n">
-        <v>0.09095329118377393</v>
+        <v>0.1631187462848655</v>
       </c>
       <c r="AD47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="1" t="inlineStr">
         <is>
-          <t>rVEQttsC</t>
+          <t>A5Y7gJQH</t>
         </is>
       </c>
       <c r="B48" s="2" t="n">
-        <v>45746.66666666666</v>
+        <v>45746.5625</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>betis</t>
+          <t>valencia</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>sevilla</t>
+          <t>mallorca</t>
         </is>
       </c>
       <c r="E48" t="n">
@@ -5330,37 +5280,37 @@
         </is>
       </c>
       <c r="I48" t="n">
-        <v>2</v>
+        <v>2.05</v>
       </c>
       <c r="J48" t="n">
-        <v>3.4</v>
+        <v>3.1</v>
       </c>
       <c r="K48" t="n">
-        <v>3.75</v>
+        <v>4.1</v>
       </c>
       <c r="L48" t="n">
-        <v>0.4713493530499075</v>
+        <v>0.4626865671641791</v>
       </c>
       <c r="M48" t="n">
-        <v>0.2772643253234751</v>
+        <v>0.3059701492537313</v>
       </c>
       <c r="N48" t="n">
-        <v>0.2513863216266174</v>
+        <v>0.2313432835820896</v>
       </c>
       <c r="O48" t="n">
-        <v>0.0607843137254902</v>
+        <v>0.0542879622344612</v>
       </c>
       <c r="P48" t="n">
         <v>1</v>
       </c>
       <c r="Q48" t="n">
-        <v>0.3360472356579193</v>
+        <v>0.2670873023564836</v>
       </c>
       <c r="R48" t="n">
-        <v>0.3231171906204028</v>
+        <v>0.2649556724416604</v>
       </c>
       <c r="S48" t="n">
-        <v>0.3408355737216779</v>
+        <v>0.467957025201856</v>
       </c>
       <c r="T48" t="n">
         <v>2</v>
@@ -5373,10 +5323,10 @@
         <v>2</v>
       </c>
       <c r="X48" t="n">
-        <v>0.3408355737216779</v>
+        <v>0.467957025201856</v>
       </c>
       <c r="Y48" t="n">
-        <v>3.75</v>
+        <v>4.1</v>
       </c>
       <c r="Z48" t="inlineStr">
         <is>
@@ -5384,33 +5334,33 @@
         </is>
       </c>
       <c r="AA48" t="n">
-        <v>0.101139418711379</v>
+        <v>0.2963302591379385</v>
       </c>
       <c r="AB48" t="n">
-        <v>0.6816711474433559</v>
+        <v>4.67957025201856</v>
       </c>
       <c r="AC48" t="n">
-        <v>0.004788338063758668</v>
+        <v>0.2008697228453724</v>
       </c>
       <c r="AD48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="1" t="inlineStr">
         <is>
-          <t>GrDYvKBO</t>
+          <t>rVEQttsC</t>
         </is>
       </c>
       <c r="B49" s="2" t="n">
-        <v>45747.66666666666</v>
+        <v>45746.66666666666</v>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>celta vigo</t>
+          <t>betis</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>las palmas</t>
+          <t>sevilla</t>
         </is>
       </c>
       <c r="E49" t="n">
@@ -5430,53 +5380,53 @@
         </is>
       </c>
       <c r="I49" t="n">
-        <v>1.57</v>
+        <v>2</v>
       </c>
       <c r="J49" t="n">
-        <v>4.1</v>
+        <v>3.4</v>
       </c>
       <c r="K49" t="n">
-        <v>5.5</v>
+        <v>3.75</v>
       </c>
       <c r="L49" t="n">
-        <v>0.5993833395353783</v>
+        <v>0.4713493530499075</v>
       </c>
       <c r="M49" t="n">
-        <v>0.2295199617245229</v>
+        <v>0.2772643253234751</v>
       </c>
       <c r="N49" t="n">
-        <v>0.1710966987400989</v>
+        <v>0.2513863216266174</v>
       </c>
       <c r="O49" t="n">
-        <v>0.06266329600180764</v>
+        <v>0.0607843137254902</v>
       </c>
       <c r="P49" t="n">
         <v>1</v>
       </c>
       <c r="Q49" t="n">
-        <v>0.3249297036748182</v>
+        <v>0.3243681162328743</v>
       </c>
       <c r="R49" t="n">
-        <v>0.3471655912238253</v>
+        <v>0.3341215160245838</v>
       </c>
       <c r="S49" t="n">
-        <v>0.3279047051013565</v>
+        <v>0.3415103677425418</v>
       </c>
       <c r="T49" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="U49" t="n">
         <v>1</v>
       </c>
       <c r="V49" t="inlineStr"/>
       <c r="W49" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="X49" t="n">
-        <v>0.3471655912238253</v>
+        <v>0.3415103677425418</v>
       </c>
       <c r="Y49" t="n">
-        <v>1.57</v>
+        <v>3.75</v>
       </c>
       <c r="Z49" t="inlineStr">
         <is>
@@ -5484,13 +5434,13 @@
         </is>
       </c>
       <c r="AA49" t="n">
-        <v>-0.7981579329449021</v>
+        <v>0.1020595923761934</v>
       </c>
       <c r="AB49" t="n">
-        <v>0.2339856555784447</v>
+        <v>0.6830207354850837</v>
       </c>
       <c r="AC49" t="n">
-        <v>0.01926088612246879</v>
+        <v>0.007388851717958056</v>
       </c>
       <c r="AD49" t="inlineStr"/>
     </row>

</xml_diff>

<commit_message>
DATA. Actualizo preds luego de aplicar reduccion de stake del 50% a local en la ea
</commit_message>
<xml_diff>
--- a/data/predicciones.xlsx
+++ b/data/predicciones.xlsx
@@ -679,7 +679,7 @@
         <v>-0.4484827780526678</v>
       </c>
       <c r="AB2" t="n">
-        <v>2.303382926642866</v>
+        <v>1.151691463321433</v>
       </c>
       <c r="AC2" t="n">
         <v>0.2353097842550371</v>
@@ -781,7 +781,7 @@
         <v>-0.2115474116756452</v>
       </c>
       <c r="AB3" t="n">
-        <v>2.531780884303292</v>
+        <v>1.265890442151646</v>
       </c>
       <c r="AC3" t="n">
         <v>0.03113120483698034</v>
@@ -883,7 +883,7 @@
         <v>-0.6384994435907863</v>
       </c>
       <c r="AB4" t="n">
-        <v>1.453802744018047</v>
+        <v>0.7269013720090233</v>
       </c>
       <c r="AC4" t="n">
         <v>0.2695472498499193</v>
@@ -985,7 +985,7 @@
         <v>-0.9941406015166959</v>
       </c>
       <c r="AB5" t="n">
-        <v>0.6850581941077486</v>
+        <v>0.3425290970538743</v>
       </c>
       <c r="AC5" t="n">
         <v>0.4740006070296459</v>
@@ -1087,7 +1087,7 @@
         <v>-0.06119650241512453</v>
       </c>
       <c r="AB6" t="n">
-        <v>5.216848826814816</v>
+        <v>2.608424413407408</v>
       </c>
       <c r="AC6" t="n">
         <v>0.2683231803734761</v>
@@ -1189,7 +1189,7 @@
         <v>-0.2826808771568695</v>
       </c>
       <c r="AB7" t="n">
-        <v>3.7991371173304</v>
+        <v>1.8995685586652</v>
       </c>
       <c r="AC7" t="n">
         <v>0.3528626381635366</v>
@@ -1597,7 +1597,7 @@
         <v>-0.2782901909858987</v>
       </c>
       <c r="AB11" t="n">
-        <v>2.497657808276925</v>
+        <v>1.248828904138463</v>
       </c>
       <c r="AC11" t="n">
         <v>0.04013788472113178</v>
@@ -1699,7 +1699,7 @@
         <v>-0.4597617358231911</v>
       </c>
       <c r="AB12" t="n">
-        <v>1.505966223778562</v>
+        <v>0.7529831118892809</v>
       </c>
       <c r="AC12" t="n">
         <v>0.04610045273289348</v>
@@ -1801,7 +1801,7 @@
         <v>-0.06591512025540448</v>
       </c>
       <c r="AB13" t="n">
-        <v>4.333334025988994</v>
+        <v>2.166667012994497</v>
       </c>
       <c r="AC13" t="n">
         <v>0.125105925127616</v>
@@ -2513,7 +2513,7 @@
         <v>-0.1114634192041025</v>
       </c>
       <c r="AB20" t="n">
-        <v>6.371935816216682</v>
+        <v>3.185967908108341</v>
       </c>
       <c r="AC20" t="n">
         <v>0.5955025264223748</v>
@@ -2613,7 +2613,7 @@
         <v>0.1379484288117779</v>
       </c>
       <c r="AB21" t="n">
-        <v>8.941340175733764</v>
+        <v>4.470670087866882</v>
       </c>
       <c r="AC21" t="n">
         <v>0.8305131965175778</v>
@@ -2713,7 +2713,7 @@
         <v>-0.01164925700534293</v>
       </c>
       <c r="AB22" t="n">
-        <v>4.115217748220544</v>
+        <v>2.057608874110272</v>
       </c>
       <c r="AC22" t="n">
         <v>0.02311079837230079</v>
@@ -2813,7 +2813,7 @@
         <v>-0.3119693365594698</v>
       </c>
       <c r="AB23" t="n">
-        <v>2.722410844528147</v>
+        <v>1.361205422264073</v>
       </c>
       <c r="AC23" t="n">
         <v>0.1714374136924707</v>
@@ -2915,7 +2915,7 @@
         <v>-0.2409240665139439</v>
       </c>
       <c r="AB24" t="n">
-        <v>0.4961059453148076</v>
+        <v>0.2480529726574038</v>
       </c>
       <c r="AC24" t="n">
         <v>0.01421946508158883</v>
@@ -3017,7 +3017,7 @@
         <v>0.1888212793794039</v>
       </c>
       <c r="AB25" t="n">
-        <v>6.659852326856369</v>
+        <v>3.329926163428185</v>
       </c>
       <c r="AC25" t="n">
         <v>0.4987260734254511</v>
@@ -3417,7 +3417,7 @@
         <v>-0.2225623318550493</v>
       </c>
       <c r="AB29" t="n">
-        <v>3.282485833185933</v>
+        <v>1.641242916592966</v>
       </c>
       <c r="AC29" t="n">
         <v>0.1379453576894913</v>
@@ -3517,7 +3517,7 @@
         <v>-0.1623318209631667</v>
       </c>
       <c r="AB30" t="n">
-        <v>4.472523232774187</v>
+        <v>2.236261616387094</v>
       </c>
       <c r="AC30" t="n">
         <v>0.2805131940097831</v>
@@ -3617,7 +3617,7 @@
         <v>-0.2656874746429443</v>
       </c>
       <c r="AB31" t="n">
-        <v>3.058137655206776</v>
+        <v>1.529068827603388</v>
       </c>
       <c r="AC31" t="n">
         <v>0.1517040475510715</v>
@@ -3717,7 +3717,7 @@
         <v>0.01542614229274848</v>
       </c>
       <c r="AB32" t="n">
-        <v>7.087880139175735</v>
+        <v>3.543940069587868</v>
       </c>
       <c r="AC32" t="n">
         <v>0.4764474606884394</v>
@@ -3819,7 +3819,7 @@
         <v>-0.3421569532269712</v>
       </c>
       <c r="AB33" t="n">
-        <v>0.384302220570921</v>
+        <v>0.1921511102854605</v>
       </c>
       <c r="AC33" t="n">
         <v>0.001695805054475141</v>
@@ -3921,7 +3921,7 @@
         <v>-0.06805150077347215</v>
       </c>
       <c r="AB34" t="n">
-        <v>3.471283591732988</v>
+        <v>1.735641795866494</v>
       </c>
       <c r="AC34" t="n">
         <v>0.05847217006575661</v>
@@ -4021,7 +4021,7 @@
         <v>-0.1169163975338208</v>
       </c>
       <c r="AB35" t="n">
-        <v>4.308209117386149</v>
+        <v>2.154104558693074</v>
       </c>
       <c r="AC35" t="n">
         <v>0.1715504060532678</v>
@@ -4427,7 +4427,7 @@
         <v>-0.4013313134396754</v>
       </c>
       <c r="AB39" t="n">
-        <v>5.493373205728582</v>
+        <v>2.746686602864291</v>
       </c>
       <c r="AC39" t="n">
         <v>0.4577914210110733</v>
@@ -4529,7 +4529,7 @@
         <v>-0.7177376067880287</v>
       </c>
       <c r="AB40" t="n">
-        <v>3.762844844580467</v>
+        <v>1.881422422290234</v>
       </c>
       <c r="AC40" t="n">
         <v>0.3299936024713728</v>
@@ -4629,7 +4629,7 @@
         <v>-0.9042917988612422</v>
       </c>
       <c r="AB41" t="n">
-        <v>4.089208157662595</v>
+        <v>2.044604078831298</v>
       </c>
       <c r="AC41" t="n">
         <v>0.5040481965546094</v>
@@ -4731,7 +4731,7 @@
         <v>-0.9058142561211311</v>
       </c>
       <c r="AB42" t="n">
-        <v>3.424503266163232</v>
+        <v>1.712251633081616</v>
       </c>
       <c r="AC42" t="n">
         <v>0.3723973849305395</v>
@@ -4835,7 +4835,7 @@
         <v>-0.627054474383548</v>
       </c>
       <c r="AB43" t="n">
-        <v>3.038763417529559</v>
+        <v>1.519381708764779</v>
       </c>
       <c r="AC43" t="n">
         <v>0.06674515341381726</v>
@@ -4937,7 +4937,7 @@
         <v>-0.7537338818235017</v>
       </c>
       <c r="AB44" t="n">
-        <v>0.4650283985134143</v>
+        <v>0.2325141992567071</v>
       </c>
       <c r="AC44" t="n">
         <v>0.005335954431194057</v>

</xml_diff>

<commit_message>
DATA. Cambio de modelos por metricas x pais + bet strategy con ≠ m por resultado
</commit_message>
<xml_diff>
--- a/data/predicciones.xlsx
+++ b/data/predicciones.xlsx
@@ -540,47 +540,47 @@
       </c>
       <c r="V1" s="1" t="inlineStr">
         <is>
+          <t>player_emergency_fill</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>result_to_bet</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>prob_result_to_bet</t>
+        </is>
+      </c>
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
+          <t>odd_to_bet</t>
+        </is>
+      </c>
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
+          <t>strategy</t>
+        </is>
+      </c>
+      <c r="AA1" s="1" t="inlineStr">
+        <is>
+          <t>kelly_criterion</t>
+        </is>
+      </c>
+      <c r="AB1" s="1" t="inlineStr">
+        <is>
+          <t>stake_to_bet</t>
+        </is>
+      </c>
+      <c r="AC1" s="1" t="inlineStr">
+        <is>
+          <t>confidence_margin</t>
+        </is>
+      </c>
+      <c r="AD1" s="1" t="inlineStr">
+        <is>
           <t>emergency_fill</t>
-        </is>
-      </c>
-      <c r="W1" s="1" t="inlineStr">
-        <is>
-          <t>player_emergency_fill</t>
-        </is>
-      </c>
-      <c r="X1" s="1" t="inlineStr">
-        <is>
-          <t>result_to_bet</t>
-        </is>
-      </c>
-      <c r="Y1" s="1" t="inlineStr">
-        <is>
-          <t>prob_result_to_bet</t>
-        </is>
-      </c>
-      <c r="Z1" s="1" t="inlineStr">
-        <is>
-          <t>odd_to_bet</t>
-        </is>
-      </c>
-      <c r="AA1" s="1" t="inlineStr">
-        <is>
-          <t>strategy</t>
-        </is>
-      </c>
-      <c r="AB1" s="1" t="inlineStr">
-        <is>
-          <t>kelly_criterion</t>
-        </is>
-      </c>
-      <c r="AC1" s="1" t="inlineStr">
-        <is>
-          <t>stake_to_bet</t>
-        </is>
-      </c>
-      <c r="AD1" s="1" t="inlineStr">
-        <is>
-          <t>confidence_margin</t>
         </is>
       </c>
     </row>
@@ -644,13 +644,13 @@
         <v>1</v>
       </c>
       <c r="Q2" t="n">
-        <v>0.3032345923571492</v>
+        <v>0.3220982557844255</v>
       </c>
       <c r="R2" t="n">
-        <v>0.6198245408337395</v>
+        <v>0.5574080400394626</v>
       </c>
       <c r="S2" t="n">
-        <v>0.07694086680911141</v>
+        <v>0.1204937041761118</v>
       </c>
       <c r="T2" t="n">
         <v>1</v>
@@ -658,49 +658,51 @@
       <c r="U2" t="n">
         <v>1</v>
       </c>
-      <c r="V2" t="inlineStr"/>
-      <c r="W2" t="inlineStr"/>
+      <c r="V2" t="n">
+        <v>0</v>
+      </c>
+      <c r="W2" t="n">
+        <v>1</v>
+      </c>
       <c r="X2" t="n">
-        <v>1</v>
+        <v>0.5574080400394626</v>
       </c>
       <c r="Y2" t="n">
-        <v>0.6198245408337395</v>
-      </c>
-      <c r="Z2" t="n">
         <v>1.44</v>
       </c>
-      <c r="AA2" t="inlineStr">
+      <c r="Z2" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
+      <c r="AA2" t="n">
+        <v>-0.4484827780526678</v>
+      </c>
       <c r="AB2" t="n">
-        <v>-0.2442105936350345</v>
+        <v>1.282038492090764</v>
       </c>
       <c r="AC2" t="n">
-        <v>2.515073406262837</v>
-      </c>
-      <c r="AD2" t="n">
-        <v>0.3165899484765903</v>
-      </c>
+        <v>0.2353097842550371</v>
+      </c>
+      <c r="AD2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>6Dg5Psv0</t>
+          <t>QHQVu3Ot</t>
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>45749.65625</v>
+        <v>45748.66666666666</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>bournemouth</t>
+          <t>nottingham</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>ipswich</t>
+          <t>manchester utd</t>
         </is>
       </c>
       <c r="E3" t="n">
@@ -720,37 +722,37 @@
         </is>
       </c>
       <c r="I3" t="n">
-        <v>1.36</v>
+        <v>2.1</v>
       </c>
       <c r="J3" t="n">
-        <v>4.75</v>
+        <v>3.6</v>
       </c>
       <c r="K3" t="n">
-        <v>8</v>
+        <v>3.2</v>
       </c>
       <c r="L3" t="n">
-        <v>0.6866642573183954</v>
+        <v>0.4465116279069767</v>
       </c>
       <c r="M3" t="n">
-        <v>0.1966028189374774</v>
+        <v>0.2604651162790698</v>
       </c>
       <c r="N3" t="n">
-        <v>0.1167329237441272</v>
+        <v>0.2930232558139535</v>
       </c>
       <c r="O3" t="n">
-        <v>0.07082043343653233</v>
+        <v>0.06646825396825395</v>
       </c>
       <c r="P3" t="n">
         <v>1</v>
       </c>
       <c r="Q3" t="n">
-        <v>0.3723502720581635</v>
+        <v>0.3342487223805388</v>
       </c>
       <c r="R3" t="n">
-        <v>0.458384637054023</v>
+        <v>0.3653799272175192</v>
       </c>
       <c r="S3" t="n">
-        <v>0.1692650908878135</v>
+        <v>0.300371350401942</v>
       </c>
       <c r="T3" t="n">
         <v>1</v>
@@ -758,36 +760,38 @@
       <c r="U3" t="n">
         <v>1</v>
       </c>
-      <c r="V3" t="inlineStr"/>
-      <c r="W3" t="inlineStr"/>
+      <c r="V3" t="n">
+        <v>0</v>
+      </c>
+      <c r="W3" t="n">
+        <v>1</v>
+      </c>
       <c r="X3" t="n">
-        <v>1</v>
+        <v>0.3653799272175192</v>
       </c>
       <c r="Y3" t="n">
-        <v>0.458384637054023</v>
-      </c>
-      <c r="Z3" t="n">
-        <v>1.36</v>
-      </c>
-      <c r="AA3" t="inlineStr">
+        <v>2.1</v>
+      </c>
+      <c r="Z3" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
+      <c r="AA3" t="n">
+        <v>-0.2115474116756452</v>
+      </c>
       <c r="AB3" t="n">
-        <v>-1.046102482240357</v>
+        <v>0.8403738326002941</v>
       </c>
       <c r="AC3" t="n">
-        <v>0.2380991762490671</v>
-      </c>
-      <c r="AD3" t="n">
-        <v>0.08603436499585954</v>
-      </c>
+        <v>0.03113120483698034</v>
+      </c>
+      <c r="AD3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>zgoMLawP</t>
+          <t>6Dg5Psv0</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
@@ -795,12 +799,12 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>brighton</t>
+          <t>bournemouth</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>aston villa</t>
+          <t>ipswich</t>
         </is>
       </c>
       <c r="E4" t="n">
@@ -820,37 +824,37 @@
         </is>
       </c>
       <c r="I4" t="n">
-        <v>2</v>
+        <v>1.36</v>
       </c>
       <c r="J4" t="n">
-        <v>4</v>
+        <v>4.75</v>
       </c>
       <c r="K4" t="n">
-        <v>3.2</v>
+        <v>8</v>
       </c>
       <c r="L4" t="n">
-        <v>0.4705882352941176</v>
+        <v>0.6866642573183954</v>
       </c>
       <c r="M4" t="n">
-        <v>0.2352941176470588</v>
+        <v>0.1966028189374774</v>
       </c>
       <c r="N4" t="n">
-        <v>0.2941176470588235</v>
+        <v>0.1167329237441272</v>
       </c>
       <c r="O4" t="n">
-        <v>0.0625</v>
+        <v>0.07082043343653233</v>
       </c>
       <c r="P4" t="n">
         <v>1</v>
       </c>
       <c r="Q4" t="n">
-        <v>0.3283486019175831</v>
+        <v>0.2967323091995783</v>
       </c>
       <c r="R4" t="n">
-        <v>0.3446907717084877</v>
+        <v>0.5662795590494977</v>
       </c>
       <c r="S4" t="n">
-        <v>0.3269606263739293</v>
+        <v>0.1369881317509239</v>
       </c>
       <c r="T4" t="n">
         <v>1</v>
@@ -858,31 +862,33 @@
       <c r="U4" t="n">
         <v>1</v>
       </c>
-      <c r="V4" t="inlineStr"/>
-      <c r="W4" t="inlineStr"/>
+      <c r="V4" t="n">
+        <v>0</v>
+      </c>
+      <c r="W4" t="n">
+        <v>1</v>
+      </c>
       <c r="X4" t="n">
-        <v>1</v>
+        <v>0.5662795590494977</v>
       </c>
       <c r="Y4" t="n">
-        <v>0.3446907717084877</v>
-      </c>
-      <c r="Z4" t="n">
-        <v>2</v>
-      </c>
-      <c r="AA4" t="inlineStr">
+        <v>1.36</v>
+      </c>
+      <c r="Z4" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
+      <c r="AA4" t="n">
+        <v>-0.6384994435907863</v>
+      </c>
       <c r="AB4" t="n">
-        <v>-0.3106184565830246</v>
+        <v>1.302442985813845</v>
       </c>
       <c r="AC4" t="n">
-        <v>1.217398048950223</v>
-      </c>
-      <c r="AD4" t="n">
-        <v>0.01634216979090458</v>
-      </c>
+        <v>0.2695472498499193</v>
+      </c>
+      <c r="AD4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
@@ -944,13 +950,13 @@
         <v>1</v>
       </c>
       <c r="Q5" t="n">
-        <v>0.215689031951903</v>
+        <v>0.2362524679636548</v>
       </c>
       <c r="R5" t="n">
-        <v>0.738571697776745</v>
+        <v>0.7102530749933007</v>
       </c>
       <c r="S5" t="n">
-        <v>0.04573927027135195</v>
+        <v>0.05349445704304451</v>
       </c>
       <c r="T5" t="n">
         <v>1</v>
@@ -958,31 +964,33 @@
       <c r="U5" t="n">
         <v>1</v>
       </c>
-      <c r="V5" t="inlineStr"/>
-      <c r="W5" t="inlineStr"/>
+      <c r="V5" t="n">
+        <v>0</v>
+      </c>
+      <c r="W5" t="n">
+        <v>1</v>
+      </c>
       <c r="X5" t="n">
-        <v>1</v>
+        <v>0.7102530749933007</v>
       </c>
       <c r="Y5" t="n">
-        <v>0.738571697776745</v>
-      </c>
-      <c r="Z5" t="n">
         <v>1.17</v>
       </c>
-      <c r="AA5" t="inlineStr">
+      <c r="Z5" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
+      <c r="AA5" t="n">
+        <v>-0.9941406015166959</v>
+      </c>
       <c r="AB5" t="n">
-        <v>-0.7992418447129908</v>
+        <v>1.633582072484592</v>
       </c>
       <c r="AC5" t="n">
-        <v>0.769465232354366</v>
-      </c>
-      <c r="AD5" t="n">
-        <v>0.522882665824842</v>
-      </c>
+        <v>0.4740006070296459</v>
+      </c>
+      <c r="AD5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
@@ -1044,13 +1052,13 @@
         <v>1</v>
       </c>
       <c r="Q6" t="n">
-        <v>0.382547090208058</v>
+        <v>0.3059273246456057</v>
       </c>
       <c r="R6" t="n">
-        <v>0.4510367435026111</v>
+        <v>0.5742505050190818</v>
       </c>
       <c r="S6" t="n">
-        <v>0.1664161662893308</v>
+        <v>0.1198221703353124</v>
       </c>
       <c r="T6" t="n">
         <v>1</v>
@@ -1059,34 +1067,32 @@
         <v>1</v>
       </c>
       <c r="V6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="W6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X6" t="n">
-        <v>1</v>
+        <v>0.5742505050190818</v>
       </c>
       <c r="Y6" t="n">
-        <v>0.4510367435026111</v>
-      </c>
-      <c r="Z6" t="n">
         <v>1.67</v>
       </c>
-      <c r="AA6" t="inlineStr">
+      <c r="Z6" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
+      <c r="AA6" t="n">
+        <v>-0.06119650241512453</v>
+      </c>
       <c r="AB6" t="n">
-        <v>-0.3683114005233427</v>
+        <v>1.320776161543888</v>
       </c>
       <c r="AC6" t="n">
-        <v>1.402817387383452</v>
-      </c>
-      <c r="AD6" t="n">
-        <v>0.06848965329455309</v>
-      </c>
+        <v>0.2683231803734761</v>
+      </c>
+      <c r="AD6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
@@ -1148,13 +1154,13 @@
         <v>1</v>
       </c>
       <c r="Q7" t="n">
-        <v>0.2831998851258044</v>
+        <v>0.2806571112202151</v>
       </c>
       <c r="R7" t="n">
-        <v>0.6404508131612661</v>
+        <v>0.6335197493837517</v>
       </c>
       <c r="S7" t="n">
-        <v>0.0763493017129296</v>
+        <v>0.08582313939603335</v>
       </c>
       <c r="T7" t="n">
         <v>1</v>
@@ -1162,31 +1168,33 @@
       <c r="U7" t="n">
         <v>1</v>
       </c>
-      <c r="V7" t="inlineStr"/>
-      <c r="W7" t="inlineStr"/>
+      <c r="V7" t="n">
+        <v>0</v>
+      </c>
+      <c r="W7" t="n">
+        <v>1</v>
+      </c>
       <c r="X7" t="n">
-        <v>1</v>
+        <v>0.6335197493837517</v>
       </c>
       <c r="Y7" t="n">
-        <v>0.6404508131612661</v>
-      </c>
-      <c r="Z7" t="n">
         <v>1.4</v>
       </c>
-      <c r="AA7" t="inlineStr">
+      <c r="Z7" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
+      <c r="AA7" t="n">
+        <v>-0.2826808771568695</v>
+      </c>
       <c r="AB7" t="n">
-        <v>-0.2584221539355691</v>
+        <v>1.457095423582629</v>
       </c>
       <c r="AC7" t="n">
-        <v>2.524504737945596</v>
-      </c>
-      <c r="AD7" t="n">
-        <v>0.3572509280354617</v>
-      </c>
+        <v>0.3528626381635366</v>
+      </c>
+      <c r="AD7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
@@ -1248,63 +1256,65 @@
         <v>1</v>
       </c>
       <c r="Q8" t="n">
-        <v>0.3834058669835496</v>
+        <v>0.3532584439150531</v>
       </c>
       <c r="R8" t="n">
-        <v>0.2995446005919141</v>
+        <v>0.2468355864359062</v>
       </c>
       <c r="S8" t="n">
-        <v>0.3170495324245363</v>
+        <v>0.3999059696490407</v>
       </c>
       <c r="T8" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="U8" t="n">
         <v>1</v>
       </c>
-      <c r="V8" t="inlineStr"/>
-      <c r="W8" t="inlineStr"/>
+      <c r="V8" t="n">
+        <v>0</v>
+      </c>
+      <c r="W8" t="n">
+        <v>2</v>
+      </c>
       <c r="X8" t="n">
-        <v>0</v>
+        <v>0.3999059696490407</v>
       </c>
       <c r="Y8" t="n">
-        <v>0.3834058669835496</v>
-      </c>
-      <c r="Z8" t="n">
-        <v>3.3</v>
-      </c>
-      <c r="AA8" t="inlineStr">
+        <v>3</v>
+      </c>
+      <c r="Z8" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
+      <c r="AA8" t="n">
+        <v>0.09985895447356113</v>
+      </c>
       <c r="AB8" t="n">
-        <v>0.1153214613242233</v>
+        <v>4.598918650963968</v>
       </c>
       <c r="AC8" t="n">
-        <v>4.79257333729437</v>
-      </c>
-      <c r="AD8" t="n">
-        <v>0.0663563345590133</v>
-      </c>
+        <v>0.04664752573398767</v>
+      </c>
+      <c r="AD8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
         <is>
-          <t>QHQVu3Ot</t>
+          <t>zgoMLawP</t>
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>45748.66666666666</v>
+        <v>45749.65625</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>nottingham</t>
+          <t>brighton</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>manchester utd</t>
+          <t>aston villa</t>
         </is>
       </c>
       <c r="E9" t="n">
@@ -1324,69 +1334,71 @@
         </is>
       </c>
       <c r="I9" t="n">
-        <v>2.1</v>
+        <v>2</v>
       </c>
       <c r="J9" t="n">
-        <v>3.6</v>
+        <v>4</v>
       </c>
       <c r="K9" t="n">
         <v>3.2</v>
       </c>
       <c r="L9" t="n">
-        <v>0.4465116279069767</v>
+        <v>0.4705882352941176</v>
       </c>
       <c r="M9" t="n">
-        <v>0.2604651162790698</v>
+        <v>0.2352941176470588</v>
       </c>
       <c r="N9" t="n">
-        <v>0.2930232558139535</v>
+        <v>0.2941176470588235</v>
       </c>
       <c r="O9" t="n">
-        <v>0.06646825396825395</v>
+        <v>0.0625</v>
       </c>
       <c r="P9" t="n">
         <v>1</v>
       </c>
       <c r="Q9" t="n">
-        <v>0.3662755710119722</v>
+        <v>0.3030295671751106</v>
       </c>
       <c r="R9" t="n">
-        <v>0.3574092605825145</v>
+        <v>0.3236877257425403</v>
       </c>
       <c r="S9" t="n">
-        <v>0.2763151684055133</v>
+        <v>0.3732827070823491</v>
       </c>
       <c r="T9" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="U9" t="n">
         <v>1</v>
       </c>
-      <c r="V9" t="inlineStr"/>
-      <c r="W9" t="inlineStr"/>
+      <c r="V9" t="n">
+        <v>0</v>
+      </c>
+      <c r="W9" t="n">
+        <v>2</v>
+      </c>
       <c r="X9" t="n">
-        <v>0</v>
+        <v>0.3732827070823491</v>
       </c>
       <c r="Y9" t="n">
-        <v>0.3662755710119722</v>
-      </c>
-      <c r="Z9" t="n">
-        <v>3.6</v>
-      </c>
-      <c r="AA9" t="inlineStr">
+        <v>3.2</v>
+      </c>
+      <c r="Z9" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
+      <c r="AA9" t="n">
+        <v>0.08841121030159861</v>
+      </c>
       <c r="AB9" t="n">
-        <v>0.1225354060165768</v>
+        <v>4.292751131447014</v>
       </c>
       <c r="AC9" t="n">
-        <v>4.578444637649652</v>
-      </c>
-      <c r="AD9" t="n">
-        <v>0.008866310429457624</v>
-      </c>
+        <v>0.04959498133980877</v>
+      </c>
+      <c r="AD9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
@@ -1448,13 +1460,13 @@
         <v>2</v>
       </c>
       <c r="Q10" t="n">
-        <v>0.4055130249341327</v>
+        <v>0.3263256215634965</v>
       </c>
       <c r="R10" t="n">
-        <v>0.180333828207914</v>
+        <v>0.2439163078866845</v>
       </c>
       <c r="S10" t="n">
-        <v>0.4141531468579533</v>
+        <v>0.4297580705498191</v>
       </c>
       <c r="T10" t="n">
         <v>2</v>
@@ -1463,52 +1475,50 @@
         <v>1</v>
       </c>
       <c r="V10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="W10" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="X10" t="n">
-        <v>2</v>
+        <v>0.4297580705498191</v>
       </c>
       <c r="Y10" t="n">
-        <v>0.4141531468579533</v>
-      </c>
-      <c r="Z10" t="n">
         <v>1.62</v>
       </c>
-      <c r="AA10" t="inlineStr">
+      <c r="Z10" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
+      <c r="AA10" t="n">
+        <v>-0.4899869769504726</v>
+      </c>
       <c r="AB10" t="n">
-        <v>-0.5307611324034121</v>
+        <v>4.942217811322919</v>
       </c>
       <c r="AC10" t="n">
-        <v>0.7668861053803498</v>
-      </c>
-      <c r="AD10" t="n">
-        <v>0.008640121923820576</v>
-      </c>
+        <v>0.1034324489863226</v>
+      </c>
+      <c r="AD10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
         <is>
-          <t>p4dxpKsh</t>
+          <t>CdaxFarI</t>
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>45745.71180555555</v>
+        <v>45746.51041666666</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>monaco</t>
+          <t>auxerre</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>nice</t>
+          <t>montpellier</t>
         </is>
       </c>
       <c r="E11" t="n">
@@ -1528,37 +1538,37 @@
         </is>
       </c>
       <c r="I11" t="n">
-        <v>1.85</v>
+        <v>1.75</v>
       </c>
       <c r="J11" t="n">
         <v>3.8</v>
       </c>
       <c r="K11" t="n">
-        <v>3.8</v>
+        <v>4.33</v>
       </c>
       <c r="L11" t="n">
-        <v>0.5066666666666666</v>
+        <v>0.5362840799830516</v>
       </c>
       <c r="M11" t="n">
-        <v>0.2466666666666667</v>
+        <v>0.2469729315711422</v>
       </c>
       <c r="N11" t="n">
-        <v>0.2466666666666667</v>
+        <v>0.2167429884458061</v>
       </c>
       <c r="O11" t="n">
-        <v>0.06685633001422464</v>
+        <v>0.06553334838250358</v>
       </c>
       <c r="P11" t="n">
         <v>1</v>
       </c>
       <c r="Q11" t="n">
-        <v>0.2693994345047954</v>
+        <v>0.2753329667748542</v>
       </c>
       <c r="R11" t="n">
-        <v>0.3941521599506397</v>
+        <v>0.4527139176534847</v>
       </c>
       <c r="S11" t="n">
-        <v>0.336448405544565</v>
+        <v>0.2719531155716611</v>
       </c>
       <c r="T11" t="n">
         <v>1</v>
@@ -1566,32 +1576,34 @@
       <c r="U11" t="n">
         <v>1</v>
       </c>
-      <c r="V11" t="inlineStr"/>
+      <c r="V11" t="n">
+        <v>0</v>
+      </c>
       <c r="W11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X11" t="n">
-        <v>1</v>
+        <v>0.4527139176534847</v>
       </c>
       <c r="Y11" t="n">
-        <v>0.3941521599506397</v>
-      </c>
-      <c r="Z11" t="n">
-        <v>1.85</v>
-      </c>
-      <c r="AA11" t="inlineStr">
+        <v>1.75</v>
+      </c>
+      <c r="Z11" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
+      <c r="AA11" t="n">
+        <v>-0.2770008588085357</v>
+      </c>
       <c r="AB11" t="n">
-        <v>-0.3186100048133136</v>
+        <v>2.603105026507537</v>
       </c>
       <c r="AC11" t="n">
-        <v>1.368269030090563</v>
+        <v>0.1773809508786305</v>
       </c>
       <c r="AD11" t="n">
-        <v>0.05770375440607473</v>
+        <v>1</v>
       </c>
     </row>
     <row r="12">
@@ -1654,13 +1666,13 @@
         <v>1</v>
       </c>
       <c r="Q12" t="n">
-        <v>0.329580189595833</v>
+        <v>0.2625045066910773</v>
       </c>
       <c r="R12" t="n">
-        <v>0.4580071637296902</v>
+        <v>0.4112374006939144</v>
       </c>
       <c r="S12" t="n">
-        <v>0.2124126466744767</v>
+        <v>0.3262580926150082</v>
       </c>
       <c r="T12" t="n">
         <v>1</v>
@@ -1670,49 +1682,47 @@
       </c>
       <c r="V12" t="inlineStr"/>
       <c r="W12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X12" t="n">
-        <v>1</v>
+        <v>0.4112374006939144</v>
       </c>
       <c r="Y12" t="n">
-        <v>0.4580071637296902</v>
-      </c>
-      <c r="Z12" t="n">
         <v>1.95</v>
       </c>
-      <c r="AA12" t="inlineStr">
+      <c r="Z12" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
+      <c r="AA12" t="n">
+        <v>-0.2085127038388074</v>
+      </c>
       <c r="AB12" t="n">
-        <v>-0.1125116112916885</v>
+        <v>2.364615053990008</v>
       </c>
       <c r="AC12" t="n">
-        <v>2.383975488990951</v>
-      </c>
-      <c r="AD12" t="n">
-        <v>0.1284269741338572</v>
-      </c>
+        <v>0.08497930807890619</v>
+      </c>
+      <c r="AD12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
-          <t>KM2pDwDU</t>
+          <t>p4dxpKsh</t>
         </is>
       </c>
       <c r="B13" s="2" t="n">
-        <v>45746.51041666666</v>
+        <v>45745.71180555555</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>le havre</t>
+          <t>monaco</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>nantes</t>
+          <t>nice</t>
         </is>
       </c>
       <c r="E13" t="n">
@@ -1732,37 +1742,37 @@
         </is>
       </c>
       <c r="I13" t="n">
-        <v>2.88</v>
+        <v>1.85</v>
       </c>
       <c r="J13" t="n">
-        <v>3.1</v>
+        <v>3.8</v>
       </c>
       <c r="K13" t="n">
-        <v>2.55</v>
+        <v>3.8</v>
       </c>
       <c r="L13" t="n">
-        <v>0.3269636431319021</v>
+        <v>0.5066666666666666</v>
       </c>
       <c r="M13" t="n">
-        <v>0.3037597716838317</v>
+        <v>0.2466666666666667</v>
       </c>
       <c r="N13" t="n">
-        <v>0.369276585184266</v>
+        <v>0.2466666666666667</v>
       </c>
       <c r="O13" t="n">
-        <v>0.06195973012861078</v>
+        <v>0.06685633001422464</v>
       </c>
       <c r="P13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q13" t="n">
-        <v>0.3619751738984914</v>
+        <v>0.3864521213741127</v>
       </c>
       <c r="R13" t="n">
-        <v>0.2884133533797296</v>
+        <v>0.3207498404333426</v>
       </c>
       <c r="S13" t="n">
-        <v>0.349611472721779</v>
+        <v>0.2927980381925447</v>
       </c>
       <c r="T13" t="n">
         <v>0</v>
@@ -1770,32 +1780,34 @@
       <c r="U13" t="n">
         <v>1</v>
       </c>
-      <c r="V13" t="inlineStr"/>
+      <c r="V13" t="n">
+        <v>0</v>
+      </c>
       <c r="W13" t="n">
         <v>0</v>
       </c>
       <c r="X13" t="n">
-        <v>0</v>
+        <v>0.3864521213741127</v>
       </c>
       <c r="Y13" t="n">
-        <v>0.3619751738984914</v>
-      </c>
-      <c r="Z13" t="n">
-        <v>3.1</v>
-      </c>
-      <c r="AA13" t="inlineStr">
+        <v>3.8</v>
+      </c>
+      <c r="Z13" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
+      <c r="AA13" t="n">
+        <v>0.1673278790077244</v>
+      </c>
       <c r="AB13" t="n">
-        <v>0.05815382813586834</v>
+        <v>0.8888398791604594</v>
       </c>
       <c r="AC13" t="n">
-        <v>4.524689673731142</v>
+        <v>0.06570228094077013</v>
       </c>
       <c r="AD13" t="n">
-        <v>0.01236370117671243</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14">
@@ -1858,13 +1870,13 @@
         <v>2</v>
       </c>
       <c r="Q14" t="n">
-        <v>0.2370764983305499</v>
+        <v>0.2917475912376913</v>
       </c>
       <c r="R14" t="n">
-        <v>0.2045588017900802</v>
+        <v>0.1940946840876043</v>
       </c>
       <c r="S14" t="n">
-        <v>0.5583646998793699</v>
+        <v>0.5141577246747043</v>
       </c>
       <c r="T14" t="n">
         <v>2</v>
@@ -1872,32 +1884,34 @@
       <c r="U14" t="n">
         <v>1</v>
       </c>
-      <c r="V14" t="inlineStr"/>
+      <c r="V14" t="n">
+        <v>0</v>
+      </c>
       <c r="W14" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="X14" t="n">
-        <v>2</v>
+        <v>0.5141577246747043</v>
       </c>
       <c r="Y14" t="n">
-        <v>0.5583646998793699</v>
-      </c>
-      <c r="Z14" t="n">
         <v>2.45</v>
       </c>
-      <c r="AA14" t="inlineStr">
+      <c r="Z14" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
+      <c r="AA14" t="n">
+        <v>0.179094086519328</v>
+      </c>
       <c r="AB14" t="n">
-        <v>0.2537886308306595</v>
+        <v>5.321532450383191</v>
       </c>
       <c r="AC14" t="n">
-        <v>6.979558748492122</v>
+        <v>0.222410133437013</v>
       </c>
       <c r="AD14" t="n">
-        <v>0.32128820154882</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15">
@@ -1960,13 +1974,13 @@
         <v>2</v>
       </c>
       <c r="Q15" t="n">
-        <v>0.3208357479859515</v>
+        <v>0.1004835089647717</v>
       </c>
       <c r="R15" t="n">
-        <v>0.1743907041967845</v>
+        <v>0.1174483317310698</v>
       </c>
       <c r="S15" t="n">
-        <v>0.5047735478172639</v>
+        <v>0.7820681593041585</v>
       </c>
       <c r="T15" t="n">
         <v>2</v>
@@ -1974,32 +1988,34 @@
       <c r="U15" t="n">
         <v>1</v>
       </c>
-      <c r="V15" t="inlineStr"/>
+      <c r="V15" t="n">
+        <v>0</v>
+      </c>
       <c r="W15" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="X15" t="n">
-        <v>2</v>
+        <v>0.7820681593041585</v>
       </c>
       <c r="Y15" t="n">
-        <v>0.5047735478172639</v>
-      </c>
-      <c r="Z15" t="n">
         <v>1.6</v>
       </c>
-      <c r="AA15" t="inlineStr">
+      <c r="Z15" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
+      <c r="AA15" t="n">
+        <v>0.4188484248110894</v>
+      </c>
       <c r="AB15" t="n">
-        <v>-0.3206038724872961</v>
+        <v>8.094405448798042</v>
       </c>
       <c r="AC15" t="n">
-        <v>5.306792664815379</v>
+        <v>0.6646198275730887</v>
       </c>
       <c r="AD15" t="n">
-        <v>0.1839377998313124</v>
+        <v>1</v>
       </c>
     </row>
     <row r="16">
@@ -2062,13 +2078,13 @@
         <v>2</v>
       </c>
       <c r="Q16" t="n">
-        <v>0.2526080232284734</v>
+        <v>0.1038261377896294</v>
       </c>
       <c r="R16" t="n">
-        <v>0.05021279736153268</v>
+        <v>0.02733959788000358</v>
       </c>
       <c r="S16" t="n">
-        <v>0.6971791794099939</v>
+        <v>0.868834264330367</v>
       </c>
       <c r="T16" t="n">
         <v>2</v>
@@ -2076,32 +2092,34 @@
       <c r="U16" t="n">
         <v>1</v>
       </c>
-      <c r="V16" t="inlineStr"/>
+      <c r="V16" t="n">
+        <v>0</v>
+      </c>
       <c r="W16" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="X16" t="n">
-        <v>2</v>
+        <v>0.868834264330367</v>
       </c>
       <c r="Y16" t="n">
-        <v>0.6971791794099939</v>
-      </c>
-      <c r="Z16" t="n">
         <v>1.14</v>
       </c>
-      <c r="AA16" t="inlineStr">
+      <c r="Z16" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
+      <c r="AA16" t="n">
+        <v>-0.0680638475955834</v>
+      </c>
       <c r="AB16" t="n">
-        <v>-1.465826681947194</v>
+        <v>8.992434635819299</v>
       </c>
       <c r="AC16" t="n">
-        <v>3.269382835678178</v>
+        <v>0.7650081265407377</v>
       </c>
       <c r="AD16" t="n">
-        <v>0.4445711561815204</v>
+        <v>1</v>
       </c>
     </row>
     <row r="17">
@@ -2164,13 +2182,13 @@
         <v>1</v>
       </c>
       <c r="Q17" t="n">
-        <v>0.2837191041116699</v>
+        <v>0.249670691980813</v>
       </c>
       <c r="R17" t="n">
-        <v>0.2045368420145746</v>
+        <v>0.1947457207697191</v>
       </c>
       <c r="S17" t="n">
-        <v>0.5117440538737555</v>
+        <v>0.5555835872494679</v>
       </c>
       <c r="T17" t="n">
         <v>2</v>
@@ -2178,32 +2196,34 @@
       <c r="U17" t="n">
         <v>1</v>
       </c>
-      <c r="V17" t="inlineStr"/>
+      <c r="V17" t="n">
+        <v>0</v>
+      </c>
       <c r="W17" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="X17" t="n">
-        <v>2</v>
+        <v>0.5555835872494679</v>
       </c>
       <c r="Y17" t="n">
-        <v>0.5117440538737555</v>
-      </c>
-      <c r="Z17" t="n">
         <v>4.1</v>
       </c>
-      <c r="AA17" t="inlineStr">
+      <c r="Z17" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
+      <c r="AA17" t="n">
+        <v>0.4122234541041349</v>
+      </c>
       <c r="AB17" t="n">
-        <v>0.3542421357685154</v>
+        <v>5.750290128031993</v>
       </c>
       <c r="AC17" t="n">
-        <v>6.396800673421944</v>
+        <v>0.3059128952686548</v>
       </c>
       <c r="AD17" t="n">
-        <v>0.2280249497620856</v>
+        <v>1</v>
       </c>
     </row>
     <row r="18">
@@ -2266,13 +2286,13 @@
         <v>2</v>
       </c>
       <c r="Q18" t="n">
-        <v>0.3574986880508562</v>
+        <v>0.3637247043428444</v>
       </c>
       <c r="R18" t="n">
-        <v>0.1130781316288558</v>
+        <v>0.1868887254677783</v>
       </c>
       <c r="S18" t="n">
-        <v>0.5294231803202881</v>
+        <v>0.4493865701893771</v>
       </c>
       <c r="T18" t="n">
         <v>2</v>
@@ -2282,36 +2302,34 @@
       </c>
       <c r="V18" t="inlineStr"/>
       <c r="W18" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="X18" t="n">
-        <v>2</v>
+        <v>0.4493865701893771</v>
       </c>
       <c r="Y18" t="n">
-        <v>0.5294231803202881</v>
-      </c>
-      <c r="Z18" t="n">
         <v>1.91</v>
       </c>
-      <c r="AA18" t="inlineStr">
+      <c r="Z18" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
+      <c r="AA18" t="n">
+        <v>-0.1556831328992195</v>
+      </c>
       <c r="AB18" t="n">
-        <v>0.01230579605686841</v>
+        <v>4.651151001460053</v>
       </c>
       <c r="AC18" t="n">
-        <v>6.617789754003601</v>
-      </c>
-      <c r="AD18" t="n">
-        <v>0.171924492269432</v>
-      </c>
+        <v>0.08566186584653268</v>
+      </c>
+      <c r="AD18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="1" t="inlineStr">
         <is>
-          <t>CdaxFarI</t>
+          <t>KM2pDwDU</t>
         </is>
       </c>
       <c r="B19" s="2" t="n">
@@ -2319,12 +2337,12 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>auxerre</t>
+          <t>le havre</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>montpellier</t>
+          <t>nantes</t>
         </is>
       </c>
       <c r="E19" t="n">
@@ -2344,37 +2362,37 @@
         </is>
       </c>
       <c r="I19" t="n">
-        <v>1.75</v>
+        <v>2.88</v>
       </c>
       <c r="J19" t="n">
-        <v>3.8</v>
+        <v>3.1</v>
       </c>
       <c r="K19" t="n">
-        <v>4.33</v>
+        <v>2.55</v>
       </c>
       <c r="L19" t="n">
-        <v>0.5362840799830516</v>
+        <v>0.3269636431319021</v>
       </c>
       <c r="M19" t="n">
-        <v>0.2469729315711422</v>
+        <v>0.3037597716838317</v>
       </c>
       <c r="N19" t="n">
-        <v>0.2167429884458061</v>
+        <v>0.369276585184266</v>
       </c>
       <c r="O19" t="n">
-        <v>0.06553334838250358</v>
+        <v>0.06195973012861078</v>
       </c>
       <c r="P19" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q19" t="n">
-        <v>0.234067035635105</v>
+        <v>0.1466450563544316</v>
       </c>
       <c r="R19" t="n">
-        <v>0.3639405226146911</v>
+        <v>0.2802032080537756</v>
       </c>
       <c r="S19" t="n">
-        <v>0.4019924417502039</v>
+        <v>0.5731517355917929</v>
       </c>
       <c r="T19" t="n">
         <v>2</v>
@@ -2382,32 +2400,34 @@
       <c r="U19" t="n">
         <v>1</v>
       </c>
-      <c r="V19" t="inlineStr"/>
+      <c r="V19" t="n">
+        <v>0</v>
+      </c>
       <c r="W19" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="X19" t="n">
-        <v>2</v>
+        <v>0.5731517355917929</v>
       </c>
       <c r="Y19" t="n">
-        <v>0.4019924417502039</v>
-      </c>
-      <c r="Z19" t="n">
-        <v>4.33</v>
-      </c>
-      <c r="AA19" t="inlineStr">
+        <v>2.55</v>
+      </c>
+      <c r="Z19" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
+      <c r="AA19" t="n">
+        <v>0.2977657585542399</v>
+      </c>
       <c r="AB19" t="n">
-        <v>0.2224105924259408</v>
+        <v>5.932120463375057</v>
       </c>
       <c r="AC19" t="n">
-        <v>5.024905521877549</v>
+        <v>0.2929485275380173</v>
       </c>
       <c r="AD19" t="n">
-        <v>0.03805191913551276</v>
+        <v>1</v>
       </c>
     </row>
     <row r="20">
@@ -2485,30 +2505,30 @@
         <v>1</v>
       </c>
       <c r="V20" t="inlineStr"/>
-      <c r="W20" t="inlineStr"/>
+      <c r="W20" t="n">
+        <v>1</v>
+      </c>
       <c r="X20" t="n">
-        <v>1</v>
+        <v>0.7825458264646554</v>
       </c>
       <c r="Y20" t="n">
-        <v>0.7825458264646554</v>
-      </c>
-      <c r="Z20" t="n">
         <v>1.27</v>
       </c>
-      <c r="AA20" t="inlineStr">
+      <c r="Z20" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
+      <c r="AA20" t="n">
+        <v>-0.02284000144402813</v>
+      </c>
       <c r="AB20" t="n">
-        <v>-0.02284000144402813</v>
+        <v>1.799855400868708</v>
       </c>
       <c r="AC20" t="n">
-        <v>4.723414307708723</v>
-      </c>
-      <c r="AD20" t="n">
         <v>0.6113133678474076</v>
       </c>
+      <c r="AD20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="1" t="inlineStr">
@@ -2585,30 +2605,30 @@
         <v>1</v>
       </c>
       <c r="V21" t="inlineStr"/>
-      <c r="W21" t="inlineStr"/>
+      <c r="W21" t="n">
+        <v>1</v>
+      </c>
       <c r="X21" t="n">
-        <v>1</v>
+        <v>0.9006459813523363</v>
       </c>
       <c r="Y21" t="n">
-        <v>0.9006459813523363</v>
-      </c>
-      <c r="Z21" t="n">
         <v>1.14</v>
       </c>
-      <c r="AA21" t="inlineStr">
+      <c r="Z21" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
+      <c r="AA21" t="n">
+        <v>0.1909744195833094</v>
+      </c>
       <c r="AB21" t="n">
-        <v>0.1909744195833094</v>
+        <v>2.071485757110374</v>
       </c>
       <c r="AC21" t="n">
-        <v>5.629037383452102</v>
-      </c>
-      <c r="AD21" t="n">
         <v>0.8256672270830573</v>
       </c>
+      <c r="AD21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="1" t="inlineStr">
@@ -2685,30 +2705,30 @@
         <v>1</v>
       </c>
       <c r="V22" t="inlineStr"/>
-      <c r="W22" t="inlineStr"/>
+      <c r="W22" t="n">
+        <v>1</v>
+      </c>
       <c r="X22" t="n">
-        <v>1</v>
+        <v>0.5091193002336956</v>
       </c>
       <c r="Y22" t="n">
-        <v>0.5091193002336956</v>
-      </c>
-      <c r="Z22" t="n">
         <v>2.35</v>
       </c>
-      <c r="AA22" t="inlineStr">
+      <c r="Z22" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
+      <c r="AA22" t="n">
+        <v>0.1455039670734701</v>
+      </c>
       <c r="AB22" t="n">
-        <v>0.1455039670734701</v>
+        <v>1.1709743905375</v>
       </c>
       <c r="AC22" t="n">
-        <v>3.181995626460598</v>
-      </c>
-      <c r="AD22" t="n">
         <v>0.2049859611591311</v>
       </c>
+      <c r="AD22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="1" t="inlineStr">
@@ -2785,30 +2805,30 @@
         <v>1</v>
       </c>
       <c r="V23" t="inlineStr"/>
-      <c r="W23" t="inlineStr"/>
+      <c r="W23" t="n">
+        <v>1</v>
+      </c>
       <c r="X23" t="n">
-        <v>1</v>
+        <v>0.5373389783576131</v>
       </c>
       <c r="Y23" t="n">
-        <v>0.5373389783576131</v>
-      </c>
-      <c r="Z23" t="n">
         <v>1.65</v>
       </c>
-      <c r="AA23" t="inlineStr">
+      <c r="Z23" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
+      <c r="AA23" t="n">
+        <v>-0.1744472087845206</v>
+      </c>
       <c r="AB23" t="n">
-        <v>-0.1744472087845206</v>
+        <v>1.23587965022251</v>
       </c>
       <c r="AC23" t="n">
-        <v>2.499104361919463</v>
-      </c>
-      <c r="AD23" t="n">
         <v>0.2473442706888411</v>
       </c>
+      <c r="AD23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="1" t="inlineStr">
@@ -2885,33 +2905,33 @@
         <v>1</v>
       </c>
       <c r="V24" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="W24" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X24" t="n">
-        <v>1</v>
+        <v>0.4066937553467808</v>
       </c>
       <c r="Y24" t="n">
-        <v>0.4066937553467808</v>
-      </c>
-      <c r="Z24" t="n">
         <v>2</v>
       </c>
-      <c r="AA24" t="inlineStr">
+      <c r="Z24" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
+      <c r="AA24" t="n">
+        <v>-0.1866124893064383</v>
+      </c>
       <c r="AB24" t="n">
-        <v>-0.1866124893064383</v>
+        <v>0.9353956372975959</v>
       </c>
       <c r="AC24" t="n">
-        <v>1.848347205304943</v>
+        <v>0.03813939040308317</v>
       </c>
       <c r="AD24" t="n">
-        <v>0.03813939040308317</v>
+        <v>1</v>
       </c>
     </row>
     <row r="25">
@@ -2989,30 +3009,30 @@
         <v>1</v>
       </c>
       <c r="V25" t="inlineStr"/>
-      <c r="W25" t="inlineStr"/>
+      <c r="W25" t="n">
+        <v>1</v>
+      </c>
       <c r="X25" t="n">
-        <v>1</v>
+        <v>0.7198839679267474</v>
       </c>
       <c r="Y25" t="n">
-        <v>0.7198839679267474</v>
-      </c>
-      <c r="Z25" t="n">
         <v>1.7</v>
       </c>
-      <c r="AA25" t="inlineStr">
+      <c r="Z25" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
+      <c r="AA25" t="n">
+        <v>0.3197182078221008</v>
+      </c>
       <c r="AB25" t="n">
-        <v>0.3197182078221008</v>
+        <v>1.655733126231519</v>
       </c>
       <c r="AC25" t="n">
-        <v>4.499274799542171</v>
-      </c>
-      <c r="AD25" t="n">
         <v>0.5506784616981166</v>
       </c>
+      <c r="AD25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="1" t="inlineStr">
@@ -3089,30 +3109,30 @@
         <v>1</v>
       </c>
       <c r="V26" t="inlineStr"/>
-      <c r="W26" t="inlineStr"/>
+      <c r="W26" t="n">
+        <v>0</v>
+      </c>
       <c r="X26" t="n">
-        <v>0</v>
+        <v>0.454936820626022</v>
       </c>
       <c r="Y26" t="n">
-        <v>0.454936820626022</v>
-      </c>
-      <c r="Z26" t="n">
         <v>3.8</v>
       </c>
-      <c r="AA26" t="inlineStr">
+      <c r="Z26" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
+      <c r="AA26" t="n">
+        <v>0.2602713994210298</v>
+      </c>
       <c r="AB26" t="n">
-        <v>0.2602713994210298</v>
+        <v>4.708596093479327</v>
       </c>
       <c r="AC26" t="n">
-        <v>5.686710257825275</v>
-      </c>
-      <c r="AD26" t="n">
         <v>0.09499876507328531</v>
       </c>
+      <c r="AD26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="1" t="inlineStr">
@@ -3189,30 +3209,30 @@
         <v>1</v>
       </c>
       <c r="V27" t="inlineStr"/>
-      <c r="W27" t="inlineStr"/>
+      <c r="W27" t="n">
+        <v>0</v>
+      </c>
       <c r="X27" t="n">
-        <v>0</v>
+        <v>0.4125590999147862</v>
       </c>
       <c r="Y27" t="n">
-        <v>0.4125590999147862</v>
-      </c>
-      <c r="Z27" t="n">
         <v>3.75</v>
       </c>
-      <c r="AA27" t="inlineStr">
+      <c r="Z27" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
+      <c r="AA27" t="n">
+        <v>0.1989442271565266</v>
+      </c>
       <c r="AB27" t="n">
-        <v>0.1989442271565266</v>
+        <v>4.269986684118037</v>
       </c>
       <c r="AC27" t="n">
-        <v>5.156988748934827</v>
-      </c>
-      <c r="AD27" t="n">
         <v>0.09581271511068973</v>
       </c>
+      <c r="AD27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="1" t="inlineStr">
@@ -3289,30 +3309,30 @@
         <v>1</v>
       </c>
       <c r="V28" t="inlineStr"/>
-      <c r="W28" t="inlineStr"/>
+      <c r="W28" t="n">
+        <v>2</v>
+      </c>
       <c r="X28" t="n">
-        <v>2</v>
+        <v>0.4142279663281674</v>
       </c>
       <c r="Y28" t="n">
-        <v>0.4142279663281674</v>
-      </c>
-      <c r="Z28" t="n">
         <v>2.25</v>
       </c>
-      <c r="AA28" t="inlineStr">
+      <c r="Z28" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
+      <c r="AA28" t="n">
+        <v>-0.05438966060929866</v>
+      </c>
       <c r="AB28" t="n">
-        <v>-0.05438966060929866</v>
+        <v>3.334535128941748</v>
       </c>
       <c r="AC28" t="n">
-        <v>4.756352108942324</v>
-      </c>
-      <c r="AD28" t="n">
         <v>0.0509843071978795</v>
       </c>
+      <c r="AD28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="1" t="inlineStr">
@@ -3374,13 +3394,13 @@
         <v>1</v>
       </c>
       <c r="Q29" t="n">
-        <v>0.364931601644578</v>
+        <v>0.2813174623013069</v>
       </c>
       <c r="R29" t="n">
-        <v>0.4320284708920021</v>
+        <v>0.6092363933642873</v>
       </c>
       <c r="S29" t="n">
-        <v>0.2030399274634198</v>
+        <v>0.1094461443344058</v>
       </c>
       <c r="T29" t="n">
         <v>1</v>
@@ -3389,30 +3409,30 @@
         <v>1</v>
       </c>
       <c r="V29" t="inlineStr"/>
-      <c r="W29" t="inlineStr"/>
+      <c r="W29" t="n">
+        <v>1</v>
+      </c>
       <c r="X29" t="n">
-        <v>1</v>
+        <v>0.6092363933642873</v>
       </c>
       <c r="Y29" t="n">
-        <v>0.4320284708920021</v>
-      </c>
-      <c r="Z29" t="n">
         <v>1.73</v>
       </c>
-      <c r="AA29" t="inlineStr">
+      <c r="Z29" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
+      <c r="AA29" t="n">
+        <v>0.07394378153454376</v>
+      </c>
       <c r="AB29" t="n">
-        <v>-0.346014719666899</v>
+        <v>1.401243704737861</v>
       </c>
       <c r="AC29" t="n">
-        <v>1.801460256377935</v>
-      </c>
-      <c r="AD29" t="n">
-        <v>0.06709686924742414</v>
-      </c>
+        <v>0.3279189310629804</v>
+      </c>
+      <c r="AD29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="1" t="inlineStr">
@@ -3474,13 +3494,13 @@
         <v>1</v>
       </c>
       <c r="Q30" t="n">
-        <v>0.3008579197261173</v>
+        <v>0.3045880120267472</v>
       </c>
       <c r="R30" t="n">
-        <v>0.5824126876962211</v>
+        <v>0.5936828179907958</v>
       </c>
       <c r="S30" t="n">
-        <v>0.1167293925776615</v>
+        <v>0.1017291699824571</v>
       </c>
       <c r="T30" t="n">
         <v>1</v>
@@ -3489,30 +3509,30 @@
         <v>1</v>
       </c>
       <c r="V30" t="inlineStr"/>
-      <c r="W30" t="inlineStr"/>
+      <c r="W30" t="n">
+        <v>1</v>
+      </c>
       <c r="X30" t="n">
-        <v>1</v>
+        <v>0.5936828179907958</v>
       </c>
       <c r="Y30" t="n">
-        <v>0.5824126876962211</v>
-      </c>
-      <c r="Z30" t="n">
         <v>1.55</v>
       </c>
-      <c r="AA30" t="inlineStr">
+      <c r="Z30" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
+      <c r="AA30" t="n">
+        <v>-0.1450756947532118</v>
+      </c>
       <c r="AB30" t="n">
-        <v>-0.1768369710379222</v>
+        <v>1.36547048137883</v>
       </c>
       <c r="AC30" t="n">
-        <v>3.003005608076717</v>
-      </c>
-      <c r="AD30" t="n">
-        <v>0.2815547679701039</v>
-      </c>
+        <v>0.2890948059640486</v>
+      </c>
+      <c r="AD30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="1" t="inlineStr">
@@ -3574,13 +3594,13 @@
         <v>1</v>
       </c>
       <c r="Q31" t="n">
-        <v>0.3720879986453734</v>
+        <v>0.4231000873308556</v>
       </c>
       <c r="R31" t="n">
-        <v>0.4423339802086751</v>
+        <v>0.4555702555943796</v>
       </c>
       <c r="S31" t="n">
-        <v>0.1855780211459515</v>
+        <v>0.1213296570747649</v>
       </c>
       <c r="T31" t="n">
         <v>1</v>
@@ -3589,30 +3609,30 @@
         <v>1</v>
       </c>
       <c r="V31" t="inlineStr"/>
-      <c r="W31" t="inlineStr"/>
+      <c r="W31" t="n">
+        <v>1</v>
+      </c>
       <c r="X31" t="n">
-        <v>1</v>
+        <v>0.4555702555943796</v>
       </c>
       <c r="Y31" t="n">
-        <v>0.4423339802086751</v>
-      </c>
-      <c r="Z31" t="n">
         <v>1.67</v>
       </c>
-      <c r="AA31" t="inlineStr">
+      <c r="Z31" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
+      <c r="AA31" t="n">
+        <v>-0.3570114524737107</v>
+      </c>
       <c r="AB31" t="n">
-        <v>-0.3900033627634515</v>
+        <v>1.047811587867073</v>
       </c>
       <c r="AC31" t="n">
-        <v>1.737921563698758</v>
-      </c>
-      <c r="AD31" t="n">
-        <v>0.07024598156330175</v>
-      </c>
+        <v>0.032470168263524</v>
+      </c>
+      <c r="AD31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="1" t="inlineStr">
@@ -3674,13 +3694,13 @@
         <v>1</v>
       </c>
       <c r="Q32" t="n">
-        <v>0.2096542956234431</v>
+        <v>0.2738871087375422</v>
       </c>
       <c r="R32" t="n">
-        <v>0.7348204972380483</v>
+        <v>0.6727771930227373</v>
       </c>
       <c r="S32" t="n">
-        <v>0.0555252071385085</v>
+        <v>0.05333569823972047</v>
       </c>
       <c r="T32" t="n">
         <v>1</v>
@@ -3689,30 +3709,30 @@
         <v>1</v>
       </c>
       <c r="V32" t="inlineStr"/>
-      <c r="W32" t="inlineStr"/>
+      <c r="W32" t="n">
+        <v>1</v>
+      </c>
       <c r="X32" t="n">
-        <v>1</v>
+        <v>0.6727771930227373</v>
       </c>
       <c r="Y32" t="n">
-        <v>0.7348204972380483</v>
-      </c>
-      <c r="Z32" t="n">
         <v>1.42</v>
       </c>
-      <c r="AA32" t="inlineStr">
+      <c r="Z32" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
+      <c r="AA32" t="n">
+        <v>-0.1063247283516979</v>
+      </c>
       <c r="AB32" t="n">
-        <v>0.1034407287572108</v>
+        <v>1.547387543952296</v>
       </c>
       <c r="AC32" t="n">
-        <v>4.592628107737802</v>
-      </c>
-      <c r="AD32" t="n">
-        <v>0.5251662016146051</v>
-      </c>
+        <v>0.3988900842851951</v>
+      </c>
+      <c r="AD32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="1" t="inlineStr">
@@ -3774,13 +3794,13 @@
         <v>1</v>
       </c>
       <c r="Q33" t="n">
-        <v>0.3640286613092957</v>
+        <v>0.2899031703513697</v>
       </c>
       <c r="R33" t="n">
-        <v>0.3687228921852588</v>
+        <v>0.3682104980889199</v>
       </c>
       <c r="S33" t="n">
-        <v>0.2672484465054455</v>
+        <v>0.3418863315597104</v>
       </c>
       <c r="T33" t="n">
         <v>1</v>
@@ -3789,52 +3809,52 @@
         <v>1</v>
       </c>
       <c r="V33" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="W33" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X33" t="n">
-        <v>1</v>
+        <v>0.3682104980889199</v>
       </c>
       <c r="Y33" t="n">
-        <v>0.3687228921852588</v>
-      </c>
-      <c r="Z33" t="n">
         <v>1.9</v>
       </c>
-      <c r="AA33" t="inlineStr">
+      <c r="Z33" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
+      <c r="AA33" t="n">
+        <v>-0.333777837367836</v>
+      </c>
       <c r="AB33" t="n">
-        <v>-0.332696116497787</v>
+        <v>0.8468841456045157</v>
       </c>
       <c r="AC33" t="n">
-        <v>0.3129806221917346</v>
+        <v>0.02632416652920944</v>
       </c>
       <c r="AD33" t="n">
-        <v>0.004694230875963157</v>
+        <v>1</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="1" t="inlineStr">
         <is>
-          <t>hnk4D3GG</t>
+          <t>KYjdFPo4</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
-        <v>45747.5625</v>
+        <v>45746.41666666666</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>verona</t>
+          <t>fiorentina</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>parma</t>
+          <t>atalanta</t>
         </is>
       </c>
       <c r="E34" t="n">
@@ -3854,87 +3874,87 @@
         </is>
       </c>
       <c r="I34" t="n">
-        <v>2.35</v>
+        <v>4.1</v>
       </c>
       <c r="J34" t="n">
-        <v>3.1</v>
+        <v>3.4</v>
       </c>
       <c r="K34" t="n">
-        <v>3.2</v>
+        <v>1.95</v>
       </c>
       <c r="L34" t="n">
-        <v>0.4012133468149647</v>
+        <v>0.2321022230001751</v>
       </c>
       <c r="M34" t="n">
-        <v>0.3041456016177958</v>
+        <v>0.2798879747943288</v>
       </c>
       <c r="N34" t="n">
-        <v>0.2946410515672397</v>
+        <v>0.4880098022054963</v>
       </c>
       <c r="O34" t="n">
-        <v>0.06061256005490723</v>
+        <v>0.05084059890372661</v>
       </c>
       <c r="P34" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q34" t="n">
-        <v>0.3311155494418314</v>
+        <v>0.4042434275738219</v>
       </c>
       <c r="R34" t="n">
-        <v>0.3772121193122594</v>
+        <v>0.2269085340852681</v>
       </c>
       <c r="S34" t="n">
-        <v>0.2916723312459092</v>
+        <v>0.36884803834091</v>
       </c>
       <c r="T34" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U34" t="n">
         <v>1</v>
       </c>
       <c r="V34" t="inlineStr"/>
-      <c r="W34" t="inlineStr"/>
+      <c r="W34" t="n">
+        <v>0</v>
+      </c>
       <c r="X34" t="n">
-        <v>1</v>
+        <v>0.4042434275738219</v>
       </c>
       <c r="Y34" t="n">
-        <v>0.3772121193122594</v>
-      </c>
-      <c r="Z34" t="n">
-        <v>2.35</v>
-      </c>
-      <c r="AA34" t="inlineStr">
+        <v>3.4</v>
+      </c>
+      <c r="Z34" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
+      <c r="AA34" t="n">
+        <v>0.1560115223962476</v>
+      </c>
       <c r="AB34" t="n">
-        <v>-0.0841122367527336</v>
+        <v>7.438079067358323</v>
       </c>
       <c r="AC34" t="n">
-        <v>2.159741107852912</v>
-      </c>
-      <c r="AD34" t="n">
-        <v>0.04609656987042804</v>
-      </c>
+        <v>0.03539538923291191</v>
+      </c>
+      <c r="AD34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="1" t="inlineStr">
         <is>
-          <t>0hCVTO0c</t>
+          <t>hnk4D3GG</t>
         </is>
       </c>
       <c r="B35" s="2" t="n">
-        <v>45747.65625</v>
+        <v>45747.5625</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>lazio</t>
+          <t>verona</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>torino</t>
+          <t>parma</t>
         </is>
       </c>
       <c r="E35" t="n">
@@ -3954,87 +3974,87 @@
         </is>
       </c>
       <c r="I35" t="n">
-        <v>1.75</v>
+        <v>2.35</v>
       </c>
       <c r="J35" t="n">
-        <v>3.3</v>
+        <v>3.1</v>
       </c>
       <c r="K35" t="n">
-        <v>5.25</v>
+        <v>3.2</v>
       </c>
       <c r="L35" t="n">
-        <v>0.5365853658536586</v>
+        <v>0.4012133468149647</v>
       </c>
       <c r="M35" t="n">
-        <v>0.2845528455284553</v>
+        <v>0.3041456016177958</v>
       </c>
       <c r="N35" t="n">
-        <v>0.1788617886178862</v>
+        <v>0.2946410515672397</v>
       </c>
       <c r="O35" t="n">
-        <v>0.06493506493506485</v>
+        <v>0.06061256005490723</v>
       </c>
       <c r="P35" t="n">
         <v>1</v>
       </c>
       <c r="Q35" t="n">
-        <v>0.3461474805441065</v>
+        <v>0.3765153835048269</v>
       </c>
       <c r="R35" t="n">
-        <v>0.5232916248960415</v>
+        <v>0.3321190471661191</v>
       </c>
       <c r="S35" t="n">
-        <v>0.1305608945598519</v>
+        <v>0.2913655693290539</v>
       </c>
       <c r="T35" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U35" t="n">
         <v>1</v>
       </c>
       <c r="V35" t="inlineStr"/>
-      <c r="W35" t="inlineStr"/>
+      <c r="W35" t="n">
+        <v>0</v>
+      </c>
       <c r="X35" t="n">
-        <v>1</v>
+        <v>0.3765153835048269</v>
       </c>
       <c r="Y35" t="n">
-        <v>0.5232916248960415</v>
-      </c>
-      <c r="Z35" t="n">
-        <v>1.75</v>
-      </c>
-      <c r="AA35" t="inlineStr">
+        <v>3.1</v>
+      </c>
+      <c r="Z35" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
+      <c r="AA35" t="n">
+        <v>0.07961794707855407</v>
+      </c>
       <c r="AB35" t="n">
-        <v>-0.1123195419092364</v>
+        <v>6.927883056488816</v>
       </c>
       <c r="AC35" t="n">
-        <v>2.904760464016889</v>
-      </c>
-      <c r="AD35" t="n">
-        <v>0.177144144351935</v>
-      </c>
+        <v>0.04439633633870788</v>
+      </c>
+      <c r="AD35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="1" t="inlineStr">
         <is>
-          <t>ENQJ7Yqe</t>
+          <t>0hCVTO0c</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
-        <v>45745.45833333334</v>
+        <v>45747.65625</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>venezia</t>
+          <t>lazio</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>bologna</t>
+          <t>torino</t>
         </is>
       </c>
       <c r="E36" t="n">
@@ -4054,91 +4074,87 @@
         </is>
       </c>
       <c r="I36" t="n">
-        <v>4.5</v>
+        <v>1.75</v>
       </c>
       <c r="J36" t="n">
-        <v>3.5</v>
+        <v>3.3</v>
       </c>
       <c r="K36" t="n">
-        <v>1.83</v>
+        <v>5.25</v>
       </c>
       <c r="L36" t="n">
-        <v>0.2107601184600197</v>
+        <v>0.5365853658536586</v>
       </c>
       <c r="M36" t="n">
-        <v>0.2709772951628825</v>
+        <v>0.2845528455284553</v>
       </c>
       <c r="N36" t="n">
-        <v>0.5182625863770978</v>
+        <v>0.1788617886178862</v>
       </c>
       <c r="O36" t="n">
-        <v>0.05438459536820184</v>
+        <v>0.06493506493506485</v>
       </c>
       <c r="P36" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q36" t="n">
-        <v>0.2699798033727277</v>
+        <v>0.4941601521686576</v>
       </c>
       <c r="R36" t="n">
-        <v>0.09047825404398727</v>
+        <v>0.3800423670951724</v>
       </c>
       <c r="S36" t="n">
-        <v>0.639541942583285</v>
+        <v>0.1257974807361701</v>
       </c>
       <c r="T36" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="U36" t="n">
         <v>1</v>
       </c>
-      <c r="V36" t="n">
-        <v>1</v>
-      </c>
+      <c r="V36" t="inlineStr"/>
       <c r="W36" t="n">
         <v>0</v>
       </c>
       <c r="X36" t="n">
-        <v>2</v>
+        <v>0.4941601521686576</v>
       </c>
       <c r="Y36" t="n">
-        <v>0.639541942583285</v>
-      </c>
-      <c r="Z36" t="n">
-        <v>1.83</v>
-      </c>
-      <c r="AA36" t="inlineStr">
+        <v>3.3</v>
+      </c>
+      <c r="Z36" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
+      <c r="AA36" t="n">
+        <v>0.2742297835463348</v>
+      </c>
       <c r="AB36" t="n">
-        <v>0.2052551264185681</v>
+        <v>9.0925467999033</v>
       </c>
       <c r="AC36" t="n">
-        <v>7.994274282291062</v>
-      </c>
-      <c r="AD36" t="n">
-        <v>0.3695621392105573</v>
-      </c>
+        <v>0.1141177850734852</v>
+      </c>
+      <c r="AD36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="1" t="inlineStr">
         <is>
-          <t>n9AwS2V9</t>
+          <t>ENQJ7Yqe</t>
         </is>
       </c>
       <c r="B37" s="2" t="n">
-        <v>45745.69791666666</v>
+        <v>45745.45833333334</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>lecce</t>
+          <t>venezia</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>as roma</t>
+          <t>bologna</t>
         </is>
       </c>
       <c r="E37" t="n">
@@ -4158,37 +4174,37 @@
         </is>
       </c>
       <c r="I37" t="n">
-        <v>4.33</v>
+        <v>4.5</v>
       </c>
       <c r="J37" t="n">
         <v>3.5</v>
       </c>
       <c r="K37" t="n">
-        <v>1.85</v>
+        <v>1.83</v>
       </c>
       <c r="L37" t="n">
-        <v>0.2184511057505777</v>
+        <v>0.2107601184600197</v>
       </c>
       <c r="M37" t="n">
-        <v>0.2702552251142862</v>
+        <v>0.2709772951628825</v>
       </c>
       <c r="N37" t="n">
-        <v>0.511293669135136</v>
+        <v>0.5182625863770978</v>
       </c>
       <c r="O37" t="n">
-        <v>0.0572017084719163</v>
+        <v>0.05438459536820184</v>
       </c>
       <c r="P37" t="n">
         <v>2</v>
       </c>
       <c r="Q37" t="n">
-        <v>0.2975226964075235</v>
+        <v>0.2387773456842109</v>
       </c>
       <c r="R37" t="n">
-        <v>0.112321853777244</v>
+        <v>0.1019656516095647</v>
       </c>
       <c r="S37" t="n">
-        <v>0.5901554498152325</v>
+        <v>0.6592570027062244</v>
       </c>
       <c r="T37" t="n">
         <v>2</v>
@@ -4196,49 +4212,53 @@
       <c r="U37" t="n">
         <v>1</v>
       </c>
-      <c r="V37" t="inlineStr"/>
-      <c r="W37" t="inlineStr"/>
+      <c r="V37" t="n">
+        <v>0</v>
+      </c>
+      <c r="W37" t="n">
+        <v>2</v>
+      </c>
       <c r="X37" t="n">
-        <v>2</v>
+        <v>0.6592570027062244</v>
       </c>
       <c r="Y37" t="n">
-        <v>0.5901554498152325</v>
-      </c>
-      <c r="Z37" t="n">
-        <v>1.85</v>
-      </c>
-      <c r="AA37" t="inlineStr">
+        <v>1.83</v>
+      </c>
+      <c r="Z37" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
+      <c r="AA37" t="n">
+        <v>0.2487232710269768</v>
+      </c>
       <c r="AB37" t="n">
-        <v>0.1079853907743296</v>
+        <v>6.065164424897265</v>
       </c>
       <c r="AC37" t="n">
-        <v>7.376943122690406</v>
+        <v>0.4204796570220136</v>
       </c>
       <c r="AD37" t="n">
-        <v>0.292632753407709</v>
+        <v>1</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="1" t="inlineStr">
         <is>
-          <t>KYjdFPo4</t>
+          <t>n9AwS2V9</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
-        <v>45746.41666666666</v>
+        <v>45745.69791666666</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>fiorentina</t>
+          <t>lecce</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>atalanta</t>
+          <t>as roma</t>
         </is>
       </c>
       <c r="E38" t="n">
@@ -4258,37 +4278,37 @@
         </is>
       </c>
       <c r="I38" t="n">
-        <v>4.1</v>
+        <v>4.33</v>
       </c>
       <c r="J38" t="n">
-        <v>3.4</v>
+        <v>3.5</v>
       </c>
       <c r="K38" t="n">
-        <v>1.95</v>
+        <v>1.85</v>
       </c>
       <c r="L38" t="n">
-        <v>0.2321022230001751</v>
+        <v>0.2184511057505777</v>
       </c>
       <c r="M38" t="n">
-        <v>0.2798879747943288</v>
+        <v>0.2702552251142862</v>
       </c>
       <c r="N38" t="n">
-        <v>0.4880098022054963</v>
+        <v>0.511293669135136</v>
       </c>
       <c r="O38" t="n">
-        <v>0.05084059890372661</v>
+        <v>0.0572017084719163</v>
       </c>
       <c r="P38" t="n">
         <v>2</v>
       </c>
       <c r="Q38" t="n">
-        <v>0.3848568538551007</v>
+        <v>0.332650425600266</v>
       </c>
       <c r="R38" t="n">
-        <v>0.1835059477908871</v>
+        <v>0.1184493246719731</v>
       </c>
       <c r="S38" t="n">
-        <v>0.4316371983540121</v>
+        <v>0.5489002497277609</v>
       </c>
       <c r="T38" t="n">
         <v>2</v>
@@ -4297,30 +4317,30 @@
         <v>1</v>
       </c>
       <c r="V38" t="inlineStr"/>
-      <c r="W38" t="inlineStr"/>
+      <c r="W38" t="n">
+        <v>2</v>
+      </c>
       <c r="X38" t="n">
-        <v>2</v>
+        <v>0.5489002497277609</v>
       </c>
       <c r="Y38" t="n">
-        <v>0.4316371983540121</v>
-      </c>
-      <c r="Z38" t="n">
-        <v>1.95</v>
-      </c>
-      <c r="AA38" t="inlineStr">
+        <v>1.85</v>
+      </c>
+      <c r="Z38" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
+      <c r="AA38" t="n">
+        <v>0.01819466117218543</v>
+      </c>
       <c r="AB38" t="n">
-        <v>-0.1666394349575541</v>
+        <v>5.0498822974954</v>
       </c>
       <c r="AC38" t="n">
-        <v>4.07422208706667</v>
-      </c>
-      <c r="AD38" t="n">
-        <v>0.04678034449891139</v>
-      </c>
+        <v>0.2162498241274949</v>
+      </c>
+      <c r="AD38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="1" t="inlineStr">
@@ -4382,13 +4402,13 @@
         <v>1</v>
       </c>
       <c r="Q39" t="n">
-        <v>0.3135549653622045</v>
+        <v>0.2305520321597711</v>
       </c>
       <c r="R39" t="n">
-        <v>0.5827362430493911</v>
+        <v>0.683057663326422</v>
       </c>
       <c r="S39" t="n">
-        <v>0.1037087915884045</v>
+        <v>0.0863903045138069</v>
       </c>
       <c r="T39" t="n">
         <v>1</v>
@@ -4400,30 +4420,30 @@
         <v>0</v>
       </c>
       <c r="W39" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X39" t="n">
-        <v>1</v>
+        <v>0.683057663326422</v>
       </c>
       <c r="Y39" t="n">
-        <v>0.5827362430493911</v>
-      </c>
-      <c r="Z39" t="n">
         <v>1.29</v>
       </c>
-      <c r="AA39" t="inlineStr">
+      <c r="Z39" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
+      <c r="AA39" t="n">
+        <v>-0.4098469458928122</v>
+      </c>
       <c r="AB39" t="n">
-        <v>-0.856104298159605</v>
+        <v>1.571032625650771</v>
       </c>
       <c r="AC39" t="n">
-        <v>2.171813627911924</v>
+        <v>0.4525056311666509</v>
       </c>
       <c r="AD39" t="n">
-        <v>0.2691812776871866</v>
+        <v>0</v>
       </c>
     </row>
     <row r="40">
@@ -4486,13 +4506,13 @@
         <v>1</v>
       </c>
       <c r="Q40" t="n">
-        <v>0.2674444806425448</v>
+        <v>0.2859904113328284</v>
       </c>
       <c r="R40" t="n">
-        <v>0.5675271494341588</v>
+        <v>0.58658003307333</v>
       </c>
       <c r="S40" t="n">
-        <v>0.1650283699232963</v>
+        <v>0.1274295555938417</v>
       </c>
       <c r="T40" t="n">
         <v>1</v>
@@ -4504,30 +4524,30 @@
         <v>0</v>
       </c>
       <c r="W40" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X40" t="n">
-        <v>1</v>
+        <v>0.58658003307333</v>
       </c>
       <c r="Y40" t="n">
-        <v>0.5675271494341588</v>
-      </c>
-      <c r="Z40" t="n">
         <v>1.33</v>
       </c>
-      <c r="AA40" t="inlineStr">
+      <c r="Z40" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
+      <c r="AA40" t="n">
+        <v>-0.6662077454923365</v>
+      </c>
       <c r="AB40" t="n">
-        <v>-0.742996640159299</v>
+        <v>1.349134076068659</v>
       </c>
       <c r="AC40" t="n">
-        <v>2.28677409581856</v>
+        <v>0.3005896217405016</v>
       </c>
       <c r="AD40" t="n">
-        <v>0.300082668791614</v>
+        <v>0</v>
       </c>
     </row>
     <row r="41">
@@ -4590,13 +4610,13 @@
         <v>1</v>
       </c>
       <c r="Q41" t="n">
-        <v>0.1933787238858396</v>
+        <v>0.1670022568007548</v>
       </c>
       <c r="R41" t="n">
-        <v>0.7539624552368922</v>
+        <v>0.7906034679051955</v>
       </c>
       <c r="S41" t="n">
-        <v>0.05265882087726823</v>
+        <v>0.04239427529404956</v>
       </c>
       <c r="T41" t="n">
         <v>1</v>
@@ -4608,30 +4628,30 @@
         <v>0</v>
       </c>
       <c r="W41" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X41" t="n">
-        <v>1</v>
+        <v>0.7906034679051955</v>
       </c>
       <c r="Y41" t="n">
-        <v>0.7539624552368922</v>
-      </c>
-      <c r="Z41" t="n">
         <v>1.18</v>
       </c>
-      <c r="AA41" t="inlineStr">
+      <c r="Z41" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
+      <c r="AA41" t="n">
+        <v>-0.3727105992881631</v>
+      </c>
       <c r="AB41" t="n">
-        <v>-0.6129127934470404</v>
+        <v>1.81838797618195</v>
       </c>
       <c r="AC41" t="n">
-        <v>3.311733310929629</v>
+        <v>0.6236012111044408</v>
       </c>
       <c r="AD41" t="n">
-        <v>0.5605837313510527</v>
+        <v>0</v>
       </c>
     </row>
     <row r="42">
@@ -4694,13 +4714,13 @@
         <v>1</v>
       </c>
       <c r="Q42" t="n">
-        <v>0.3206687854850142</v>
+        <v>0.2379869131980451</v>
       </c>
       <c r="R42" t="n">
-        <v>0.5219893944000483</v>
+        <v>0.6507394337021107</v>
       </c>
       <c r="S42" t="n">
-        <v>0.1573418201149376</v>
+        <v>0.1112736530998441</v>
       </c>
       <c r="T42" t="n">
         <v>1</v>
@@ -4712,30 +4732,30 @@
         <v>0</v>
       </c>
       <c r="W42" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X42" t="n">
-        <v>1</v>
+        <v>0.6507394337021107</v>
       </c>
       <c r="Y42" t="n">
-        <v>0.5219893944000483</v>
-      </c>
-      <c r="Z42" t="n">
         <v>1.27</v>
       </c>
-      <c r="AA42" t="inlineStr">
+      <c r="Z42" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
+      <c r="AA42" t="n">
+        <v>-0.6428182192530345</v>
+      </c>
       <c r="AB42" t="n">
-        <v>-1.248420255970143</v>
+        <v>1.496700697514855</v>
       </c>
       <c r="AC42" t="n">
-        <v>1.454873962512022</v>
+        <v>0.4127525205040656</v>
       </c>
       <c r="AD42" t="n">
-        <v>0.2013206089150342</v>
+        <v>0</v>
       </c>
     </row>
     <row r="43">
@@ -4798,13 +4818,13 @@
         <v>1</v>
       </c>
       <c r="Q43" t="n">
-        <v>0.3136577785184732</v>
+        <v>0.3277161333715918</v>
       </c>
       <c r="R43" t="n">
-        <v>0.45199124092024</v>
+        <v>0.4978816535233578</v>
       </c>
       <c r="S43" t="n">
-        <v>0.2343509805612867</v>
+        <v>0.1744022131050505</v>
       </c>
       <c r="T43" t="n">
         <v>1</v>
@@ -4816,49 +4836,49 @@
         <v>0</v>
       </c>
       <c r="W43" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X43" t="n">
-        <v>1</v>
+        <v>0.4978816535233578</v>
       </c>
       <c r="Y43" t="n">
-        <v>0.45199124092024</v>
-      </c>
-      <c r="Z43" t="n">
         <v>1.53</v>
       </c>
-      <c r="AA43" t="inlineStr">
+      <c r="Z43" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
+      <c r="AA43" t="n">
+        <v>-0.4495114530363442</v>
+      </c>
       <c r="AB43" t="n">
-        <v>-0.5819875497962883</v>
+        <v>1.145127803103723</v>
       </c>
       <c r="AC43" t="n">
-        <v>2.025346686627845</v>
+        <v>0.1701655201517661</v>
       </c>
       <c r="AD43" t="n">
-        <v>0.1383334624017668</v>
+        <v>0</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="1" t="inlineStr">
         <is>
-          <t>rVEQttsC</t>
+          <t>A5Y7gJQH</t>
         </is>
       </c>
       <c r="B44" s="2" t="n">
-        <v>45746.66666666666</v>
+        <v>45746.5625</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>betis</t>
+          <t>valencia</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>sevilla</t>
+          <t>mallorca</t>
         </is>
       </c>
       <c r="E44" t="n">
@@ -4878,37 +4898,37 @@
         </is>
       </c>
       <c r="I44" t="n">
-        <v>2</v>
+        <v>2.05</v>
       </c>
       <c r="J44" t="n">
-        <v>3.4</v>
+        <v>3.1</v>
       </c>
       <c r="K44" t="n">
-        <v>3.75</v>
+        <v>4.1</v>
       </c>
       <c r="L44" t="n">
-        <v>0.4713493530499075</v>
+        <v>0.4626865671641791</v>
       </c>
       <c r="M44" t="n">
-        <v>0.2772643253234751</v>
+        <v>0.3059701492537313</v>
       </c>
       <c r="N44" t="n">
-        <v>0.2513863216266174</v>
+        <v>0.2313432835820896</v>
       </c>
       <c r="O44" t="n">
-        <v>0.0607843137254902</v>
+        <v>0.0542879622344612</v>
       </c>
       <c r="P44" t="n">
         <v>1</v>
       </c>
       <c r="Q44" t="n">
-        <v>0.2516224448638245</v>
+        <v>0.3555729649102405</v>
       </c>
       <c r="R44" t="n">
-        <v>0.4060362838686854</v>
+        <v>0.3615364290087321</v>
       </c>
       <c r="S44" t="n">
-        <v>0.34234127126749</v>
+        <v>0.2828906060810275</v>
       </c>
       <c r="T44" t="n">
         <v>1</v>
@@ -4920,49 +4940,49 @@
         <v>0</v>
       </c>
       <c r="W44" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X44" t="n">
-        <v>1</v>
+        <v>0.3615364290087321</v>
       </c>
       <c r="Y44" t="n">
-        <v>0.4060362838686854</v>
-      </c>
-      <c r="Z44" t="n">
-        <v>2</v>
-      </c>
-      <c r="AA44" t="inlineStr">
+        <v>2.05</v>
+      </c>
+      <c r="Z44" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
+      <c r="AA44" t="n">
+        <v>-0.2465241147924754</v>
+      </c>
       <c r="AB44" t="n">
-        <v>-0.1879274322626292</v>
+        <v>0.1663067573440168</v>
       </c>
       <c r="AC44" t="n">
-        <v>2.299971851428707</v>
+        <v>0.005963464098491633</v>
       </c>
       <c r="AD44" t="n">
-        <v>0.06369501260119542</v>
+        <v>0</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="1" t="inlineStr">
         <is>
-          <t>GrDYvKBO</t>
+          <t>rVEQttsC</t>
         </is>
       </c>
       <c r="B45" s="2" t="n">
-        <v>45747.66666666666</v>
+        <v>45746.66666666666</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>celta vigo</t>
+          <t>betis</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>las palmas</t>
+          <t>sevilla</t>
         </is>
       </c>
       <c r="E45" t="n">
@@ -4982,37 +5002,37 @@
         </is>
       </c>
       <c r="I45" t="n">
-        <v>1.57</v>
+        <v>2</v>
       </c>
       <c r="J45" t="n">
-        <v>4.1</v>
+        <v>3.4</v>
       </c>
       <c r="K45" t="n">
-        <v>5.5</v>
+        <v>3.75</v>
       </c>
       <c r="L45" t="n">
-        <v>0.5993833395353783</v>
+        <v>0.4713493530499075</v>
       </c>
       <c r="M45" t="n">
-        <v>0.2295199617245229</v>
+        <v>0.2772643253234751</v>
       </c>
       <c r="N45" t="n">
-        <v>0.1710966987400989</v>
+        <v>0.2513863216266174</v>
       </c>
       <c r="O45" t="n">
-        <v>0.06266329600180764</v>
+        <v>0.0607843137254902</v>
       </c>
       <c r="P45" t="n">
         <v>1</v>
       </c>
       <c r="Q45" t="n">
-        <v>0.3582566924102288</v>
+        <v>0.355699083944977</v>
       </c>
       <c r="R45" t="n">
-        <v>0.3623433319406753</v>
+        <v>0.3657946219569925</v>
       </c>
       <c r="S45" t="n">
-        <v>0.279399975649096</v>
+        <v>0.2785062940980305</v>
       </c>
       <c r="T45" t="n">
         <v>1</v>
@@ -5024,49 +5044,49 @@
         <v>0</v>
       </c>
       <c r="W45" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X45" t="n">
-        <v>1</v>
+        <v>0.3657946219569925</v>
       </c>
       <c r="Y45" t="n">
-        <v>0.3623433319406753</v>
-      </c>
-      <c r="Z45" t="n">
-        <v>1.57</v>
-      </c>
-      <c r="AA45" t="inlineStr">
+        <v>2</v>
+      </c>
+      <c r="Z45" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
+      <c r="AA45" t="n">
+        <v>-0.2684107560860149</v>
+      </c>
       <c r="AB45" t="n">
-        <v>-0.756352576935333</v>
+        <v>0.1682655261002166</v>
       </c>
       <c r="AC45" t="n">
-        <v>0.2893661932499308</v>
+        <v>0.01009553801201551</v>
       </c>
       <c r="AD45" t="n">
-        <v>0.004086639530446412</v>
+        <v>0</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="1" t="inlineStr">
         <is>
-          <t>Olz0eud5</t>
+          <t>GrDYvKBO</t>
         </is>
       </c>
       <c r="B46" s="2" t="n">
-        <v>45745.60416666666</v>
+        <v>45747.66666666666</v>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>alaves</t>
+          <t>celta vigo</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>rayo vallecano</t>
+          <t>las palmas</t>
         </is>
       </c>
       <c r="E46" t="n">
@@ -5086,40 +5106,40 @@
         </is>
       </c>
       <c r="I46" t="n">
-        <v>2.25</v>
+        <v>1.57</v>
       </c>
       <c r="J46" t="n">
-        <v>2.9</v>
+        <v>4.1</v>
       </c>
       <c r="K46" t="n">
-        <v>3.6</v>
+        <v>5.5</v>
       </c>
       <c r="L46" t="n">
-        <v>0.4165170556552962</v>
+        <v>0.5993833395353783</v>
       </c>
       <c r="M46" t="n">
-        <v>0.3231597845601437</v>
+        <v>0.2295199617245229</v>
       </c>
       <c r="N46" t="n">
-        <v>0.2603231597845602</v>
+        <v>0.1710966987400989</v>
       </c>
       <c r="O46" t="n">
-        <v>0.06704980842911867</v>
+        <v>0.06266329600180764</v>
       </c>
       <c r="P46" t="n">
         <v>1</v>
       </c>
       <c r="Q46" t="n">
-        <v>0.3897507468559439</v>
+        <v>0.3583583538094059</v>
       </c>
       <c r="R46" t="n">
-        <v>0.3093667098475331</v>
+        <v>0.3596472087554723</v>
       </c>
       <c r="S46" t="n">
-        <v>0.300882543296523</v>
+        <v>0.2819944374351219</v>
       </c>
       <c r="T46" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U46" t="n">
         <v>1</v>
@@ -5128,49 +5148,49 @@
         <v>0</v>
       </c>
       <c r="W46" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X46" t="n">
-        <v>0</v>
+        <v>0.3596472087554723</v>
       </c>
       <c r="Y46" t="n">
-        <v>0.3897507468559439</v>
-      </c>
-      <c r="Z46" t="n">
-        <v>2.9</v>
-      </c>
-      <c r="AA46" t="inlineStr">
+        <v>1.57</v>
+      </c>
+      <c r="Z46" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
+      <c r="AA46" t="n">
+        <v>-0.7637787407963306</v>
+      </c>
       <c r="AB46" t="n">
-        <v>0.06856692941170382</v>
+        <v>0.1654377160275173</v>
       </c>
       <c r="AC46" t="n">
-        <v>4.871884335699299</v>
+        <v>0.001288854946066398</v>
       </c>
       <c r="AD46" t="n">
-        <v>0.08038403700841079</v>
+        <v>0</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="1" t="inlineStr">
         <is>
-          <t>f9rqaNdt</t>
+          <t>Olz0eud5</t>
         </is>
       </c>
       <c r="B47" s="2" t="n">
-        <v>45746.375</v>
+        <v>45745.60416666666</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>getafe</t>
+          <t>alaves</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>villarreal</t>
+          <t>rayo vallecano</t>
         </is>
       </c>
       <c r="E47" t="n">
@@ -5190,37 +5210,37 @@
         </is>
       </c>
       <c r="I47" t="n">
-        <v>3.1</v>
+        <v>2.25</v>
       </c>
       <c r="J47" t="n">
-        <v>3.2</v>
+        <v>2.9</v>
       </c>
       <c r="K47" t="n">
-        <v>2.35</v>
+        <v>3.6</v>
       </c>
       <c r="L47" t="n">
-        <v>0.3041456016177958</v>
+        <v>0.4165170556552962</v>
       </c>
       <c r="M47" t="n">
-        <v>0.2946410515672397</v>
+        <v>0.3231597845601437</v>
       </c>
       <c r="N47" t="n">
-        <v>0.4012133468149647</v>
+        <v>0.2603231597845602</v>
       </c>
       <c r="O47" t="n">
-        <v>0.06061256005490723</v>
+        <v>0.06704980842911867</v>
       </c>
       <c r="P47" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q47" t="n">
-        <v>0.4011312665607018</v>
+        <v>0.3849332791811567</v>
       </c>
       <c r="R47" t="n">
-        <v>0.2135808587415033</v>
+        <v>0.3289894957515934</v>
       </c>
       <c r="S47" t="n">
-        <v>0.385287874697795</v>
+        <v>0.2860772250672497</v>
       </c>
       <c r="T47" t="n">
         <v>0</v>
@@ -5235,46 +5255,46 @@
         <v>0</v>
       </c>
       <c r="X47" t="n">
-        <v>0</v>
+        <v>0.3849332791811567</v>
       </c>
       <c r="Y47" t="n">
-        <v>0.4011312665607018</v>
-      </c>
-      <c r="Z47" t="n">
-        <v>3.2</v>
-      </c>
-      <c r="AA47" t="inlineStr">
+        <v>2.9</v>
+      </c>
+      <c r="Z47" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
+      <c r="AA47" t="n">
+        <v>0.0612139524343971</v>
+      </c>
       <c r="AB47" t="n">
-        <v>0.1289182059064754</v>
+        <v>7.082772336933283</v>
       </c>
       <c r="AC47" t="n">
-        <v>5.014140832008772</v>
+        <v>0.0559437834295633</v>
       </c>
       <c r="AD47" t="n">
-        <v>0.01584339186290684</v>
+        <v>0</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="1" t="inlineStr">
         <is>
-          <t>Kjbn1lFr</t>
+          <t>f9rqaNdt</t>
         </is>
       </c>
       <c r="B48" s="2" t="n">
-        <v>45745.51041666666</v>
+        <v>45746.375</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>espanyol</t>
+          <t>getafe</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>atl  madrid</t>
+          <t>villarreal</t>
         </is>
       </c>
       <c r="E48" t="n">
@@ -5294,40 +5314,40 @@
         </is>
       </c>
       <c r="I48" t="n">
-        <v>7</v>
+        <v>3.1</v>
       </c>
       <c r="J48" t="n">
-        <v>4</v>
+        <v>3.2</v>
       </c>
       <c r="K48" t="n">
-        <v>1.5</v>
+        <v>2.35</v>
       </c>
       <c r="L48" t="n">
-        <v>0.1348314606741573</v>
+        <v>0.3041456016177958</v>
       </c>
       <c r="M48" t="n">
-        <v>0.2359550561797753</v>
+        <v>0.2946410515672397</v>
       </c>
       <c r="N48" t="n">
-        <v>0.6292134831460674</v>
+        <v>0.4012133468149647</v>
       </c>
       <c r="O48" t="n">
-        <v>0.05952380952380953</v>
+        <v>0.06061256005490723</v>
       </c>
       <c r="P48" t="n">
         <v>2</v>
       </c>
       <c r="Q48" t="n">
-        <v>0.3179232955352041</v>
+        <v>0.3914287759434801</v>
       </c>
       <c r="R48" t="n">
-        <v>0.1032524868291907</v>
+        <v>0.220564522223485</v>
       </c>
       <c r="S48" t="n">
-        <v>0.5788242176356052</v>
+        <v>0.388006701833035</v>
       </c>
       <c r="T48" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="U48" t="n">
         <v>1</v>
@@ -5339,46 +5359,46 @@
         <v>0</v>
       </c>
       <c r="X48" t="n">
-        <v>2</v>
+        <v>0.3914287759434801</v>
       </c>
       <c r="Y48" t="n">
-        <v>0.5788242176356052</v>
-      </c>
-      <c r="Z48" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="AA48" t="inlineStr">
+        <v>3.2</v>
+      </c>
+      <c r="Z48" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
+      <c r="AA48" t="n">
+        <v>0.1148054922814256</v>
+      </c>
       <c r="AB48" t="n">
-        <v>-0.2635273470931844</v>
+        <v>7.202289477360034</v>
       </c>
       <c r="AC48" t="n">
-        <v>4.515461372022413</v>
+        <v>0.003422074110445095</v>
       </c>
       <c r="AD48" t="n">
-        <v>0.2609009221004011</v>
+        <v>0</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="1" t="inlineStr">
         <is>
-          <t>A5Y7gJQH</t>
+          <t>Kjbn1lFr</t>
         </is>
       </c>
       <c r="B49" s="2" t="n">
-        <v>45746.5625</v>
+        <v>45745.51041666666</v>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>valencia</t>
+          <t>espanyol</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>mallorca</t>
+          <t>atl  madrid</t>
         </is>
       </c>
       <c r="E49" t="n">
@@ -5398,37 +5418,37 @@
         </is>
       </c>
       <c r="I49" t="n">
-        <v>2.05</v>
+        <v>7</v>
       </c>
       <c r="J49" t="n">
-        <v>3.1</v>
+        <v>4</v>
       </c>
       <c r="K49" t="n">
-        <v>4.1</v>
+        <v>1.5</v>
       </c>
       <c r="L49" t="n">
-        <v>0.4626865671641791</v>
+        <v>0.1348314606741573</v>
       </c>
       <c r="M49" t="n">
-        <v>0.3059701492537313</v>
+        <v>0.2359550561797753</v>
       </c>
       <c r="N49" t="n">
-        <v>0.2313432835820896</v>
+        <v>0.6292134831460674</v>
       </c>
       <c r="O49" t="n">
-        <v>0.0542879622344612</v>
+        <v>0.05952380952380953</v>
       </c>
       <c r="P49" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q49" t="n">
-        <v>0.3031532864302324</v>
+        <v>0.3544226986660331</v>
       </c>
       <c r="R49" t="n">
-        <v>0.3310874465285998</v>
+        <v>0.1183270127597769</v>
       </c>
       <c r="S49" t="n">
-        <v>0.3657592670411678</v>
+        <v>0.52725028857419</v>
       </c>
       <c r="T49" t="n">
         <v>2</v>
@@ -5440,30 +5460,30 @@
         <v>0</v>
       </c>
       <c r="W49" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="X49" t="n">
-        <v>2</v>
+        <v>0.52725028857419</v>
       </c>
       <c r="Y49" t="n">
-        <v>0.3657592670411678</v>
-      </c>
-      <c r="Z49" t="n">
-        <v>4.1</v>
-      </c>
-      <c r="AA49" t="inlineStr">
+        <v>1.5</v>
+      </c>
+      <c r="Z49" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
+      <c r="AA49" t="n">
+        <v>-0.41824913427743</v>
+      </c>
       <c r="AB49" t="n">
-        <v>0.161165482215738</v>
+        <v>1.212675663720637</v>
       </c>
       <c r="AC49" t="n">
-        <v>4.571990838014598</v>
+        <v>0.1728275899081569</v>
       </c>
       <c r="AD49" t="n">
-        <v>0.03467182051256801</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
DATA. Actualizo predicciones tras cambio de modelos (usando f1_score como metrica gral) y kelly_linear en prod
</commit_message>
<xml_diff>
--- a/data/predicciones.xlsx
+++ b/data/predicciones.xlsx
@@ -540,47 +540,47 @@
       </c>
       <c r="V1" s="1" t="inlineStr">
         <is>
+          <t>emergency_fill</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
           <t>player_emergency_fill</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>result_to_bet</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>prob_result_to_bet</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>odd_to_bet</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>strategy</t>
         </is>
       </c>
-      <c r="AA1" s="1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>kelly_criterion</t>
         </is>
       </c>
-      <c r="AB1" s="1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>stake_to_bet</t>
         </is>
       </c>
-      <c r="AC1" s="1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>confidence_margin</t>
-        </is>
-      </c>
-      <c r="AD1" s="1" t="inlineStr">
-        <is>
-          <t>emergency_fill</t>
         </is>
       </c>
     </row>
@@ -644,13 +644,13 @@
         <v>1</v>
       </c>
       <c r="Q2" t="n">
-        <v>0.3220982557844255</v>
+        <v>0.3032345923571492</v>
       </c>
       <c r="R2" t="n">
-        <v>0.5574080400394626</v>
+        <v>0.6198245408337395</v>
       </c>
       <c r="S2" t="n">
-        <v>0.1204937041761118</v>
+        <v>0.07694086680911141</v>
       </c>
       <c r="T2" t="n">
         <v>1</v>
@@ -658,51 +658,49 @@
       <c r="U2" t="n">
         <v>1</v>
       </c>
-      <c r="V2" t="n">
-        <v>0</v>
-      </c>
-      <c r="W2" t="n">
-        <v>1</v>
-      </c>
+      <c r="V2" t="inlineStr"/>
+      <c r="W2" t="inlineStr"/>
       <c r="X2" t="n">
-        <v>0.5574080400394626</v>
+        <v>1</v>
       </c>
       <c r="Y2" t="n">
+        <v>0.6198245408337395</v>
+      </c>
+      <c r="Z2" t="n">
         <v>1.44</v>
       </c>
-      <c r="Z2" t="inlineStr">
+      <c r="AA2" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
-      <c r="AA2" t="n">
-        <v>-0.4484827780526678</v>
-      </c>
       <c r="AB2" t="n">
-        <v>1.282038492090764</v>
+        <v>-0.2442105936350345</v>
       </c>
       <c r="AC2" t="n">
-        <v>0.2353097842550371</v>
-      </c>
-      <c r="AD2" t="inlineStr"/>
+        <v>1.905801074789221</v>
+      </c>
+      <c r="AD2" t="n">
+        <v>0.3165899484765903</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>QHQVu3Ot</t>
+          <t>6Dg5Psv0</t>
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>45748.66666666666</v>
+        <v>45749.65625</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>nottingham</t>
+          <t>bournemouth</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>manchester utd</t>
+          <t>ipswich</t>
         </is>
       </c>
       <c r="E3" t="n">
@@ -722,37 +720,37 @@
         </is>
       </c>
       <c r="I3" t="n">
-        <v>2.1</v>
+        <v>1.36</v>
       </c>
       <c r="J3" t="n">
-        <v>3.6</v>
+        <v>4.75</v>
       </c>
       <c r="K3" t="n">
-        <v>3.2</v>
+        <v>8</v>
       </c>
       <c r="L3" t="n">
-        <v>0.4465116279069767</v>
+        <v>0.6866642573183954</v>
       </c>
       <c r="M3" t="n">
-        <v>0.2604651162790698</v>
+        <v>0.1966028189374774</v>
       </c>
       <c r="N3" t="n">
-        <v>0.2930232558139535</v>
+        <v>0.1167329237441272</v>
       </c>
       <c r="O3" t="n">
-        <v>0.06646825396825395</v>
+        <v>0.07082043343653233</v>
       </c>
       <c r="P3" t="n">
         <v>1</v>
       </c>
       <c r="Q3" t="n">
-        <v>0.3342487223805388</v>
+        <v>0.3723502720581635</v>
       </c>
       <c r="R3" t="n">
-        <v>0.3653799272175192</v>
+        <v>0.458384637054023</v>
       </c>
       <c r="S3" t="n">
-        <v>0.300371350401942</v>
+        <v>0.1692650908878135</v>
       </c>
       <c r="T3" t="n">
         <v>1</v>
@@ -760,38 +758,36 @@
       <c r="U3" t="n">
         <v>1</v>
       </c>
-      <c r="V3" t="n">
-        <v>0</v>
-      </c>
-      <c r="W3" t="n">
-        <v>1</v>
-      </c>
+      <c r="V3" t="inlineStr"/>
+      <c r="W3" t="inlineStr"/>
       <c r="X3" t="n">
-        <v>0.3653799272175192</v>
+        <v>1</v>
       </c>
       <c r="Y3" t="n">
-        <v>2.1</v>
-      </c>
-      <c r="Z3" t="inlineStr">
+        <v>0.458384637054023</v>
+      </c>
+      <c r="Z3" t="n">
+        <v>1.36</v>
+      </c>
+      <c r="AA3" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
-      <c r="AA3" t="n">
-        <v>-0.2115474116756452</v>
-      </c>
       <c r="AB3" t="n">
-        <v>0.8403738326002941</v>
+        <v>-1.046102482240357</v>
       </c>
       <c r="AC3" t="n">
-        <v>0.03113120483698034</v>
-      </c>
-      <c r="AD3" t="inlineStr"/>
+        <v>0.8341773619015219</v>
+      </c>
+      <c r="AD3" t="n">
+        <v>0.08603436499585954</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>6Dg5Psv0</t>
+          <t>zgoMLawP</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
@@ -799,12 +795,12 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>bournemouth</t>
+          <t>brighton</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>ipswich</t>
+          <t>aston villa</t>
         </is>
       </c>
       <c r="E4" t="n">
@@ -824,37 +820,37 @@
         </is>
       </c>
       <c r="I4" t="n">
-        <v>1.36</v>
+        <v>2</v>
       </c>
       <c r="J4" t="n">
-        <v>4.75</v>
+        <v>4</v>
       </c>
       <c r="K4" t="n">
-        <v>8</v>
+        <v>3.2</v>
       </c>
       <c r="L4" t="n">
-        <v>0.6866642573183954</v>
+        <v>0.4705882352941176</v>
       </c>
       <c r="M4" t="n">
-        <v>0.1966028189374774</v>
+        <v>0.2352941176470588</v>
       </c>
       <c r="N4" t="n">
-        <v>0.1167329237441272</v>
+        <v>0.2941176470588235</v>
       </c>
       <c r="O4" t="n">
-        <v>0.07082043343653233</v>
+        <v>0.0625</v>
       </c>
       <c r="P4" t="n">
         <v>1</v>
       </c>
       <c r="Q4" t="n">
-        <v>0.2967323091995783</v>
+        <v>0.3283486019175831</v>
       </c>
       <c r="R4" t="n">
-        <v>0.5662795590494977</v>
+        <v>0.3446907717084877</v>
       </c>
       <c r="S4" t="n">
-        <v>0.1369881317509239</v>
+        <v>0.3269606263739293</v>
       </c>
       <c r="T4" t="n">
         <v>1</v>
@@ -862,33 +858,31 @@
       <c r="U4" t="n">
         <v>1</v>
       </c>
-      <c r="V4" t="n">
-        <v>0</v>
-      </c>
-      <c r="W4" t="n">
-        <v>1</v>
-      </c>
+      <c r="V4" t="inlineStr"/>
+      <c r="W4" t="inlineStr"/>
       <c r="X4" t="n">
-        <v>0.5662795590494977</v>
+        <v>1</v>
       </c>
       <c r="Y4" t="n">
-        <v>1.36</v>
-      </c>
-      <c r="Z4" t="inlineStr">
+        <v>0.3446907717084877</v>
+      </c>
+      <c r="Z4" t="n">
+        <v>2</v>
+      </c>
+      <c r="AA4" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
-      <c r="AA4" t="n">
-        <v>-0.6384994435907863</v>
-      </c>
       <c r="AB4" t="n">
-        <v>1.302442985813845</v>
+        <v>-0.3106184565830246</v>
       </c>
       <c r="AC4" t="n">
-        <v>0.2695472498499193</v>
-      </c>
-      <c r="AD4" t="inlineStr"/>
+        <v>1.020542000984441</v>
+      </c>
+      <c r="AD4" t="n">
+        <v>0.01634216979090458</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
@@ -950,13 +944,13 @@
         <v>1</v>
       </c>
       <c r="Q5" t="n">
-        <v>0.2362524679636548</v>
+        <v>0.215689031951903</v>
       </c>
       <c r="R5" t="n">
-        <v>0.7102530749933007</v>
+        <v>0.738571697776745</v>
       </c>
       <c r="S5" t="n">
-        <v>0.05349445704304451</v>
+        <v>0.04573927027135195</v>
       </c>
       <c r="T5" t="n">
         <v>1</v>
@@ -964,33 +958,31 @@
       <c r="U5" t="n">
         <v>1</v>
       </c>
-      <c r="V5" t="n">
-        <v>0</v>
-      </c>
-      <c r="W5" t="n">
-        <v>1</v>
-      </c>
+      <c r="V5" t="inlineStr"/>
+      <c r="W5" t="inlineStr"/>
       <c r="X5" t="n">
-        <v>0.7102530749933007</v>
+        <v>1</v>
       </c>
       <c r="Y5" t="n">
+        <v>0.738571697776745</v>
+      </c>
+      <c r="Z5" t="n">
         <v>1.17</v>
       </c>
-      <c r="Z5" t="inlineStr">
+      <c r="AA5" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
-      <c r="AA5" t="n">
-        <v>-0.9941406015166959</v>
-      </c>
       <c r="AB5" t="n">
-        <v>1.633582072484592</v>
+        <v>-0.7992418447129908</v>
       </c>
       <c r="AC5" t="n">
-        <v>0.4740006070296459</v>
-      </c>
-      <c r="AD5" t="inlineStr"/>
+        <v>1.603671091726641</v>
+      </c>
+      <c r="AD5" t="n">
+        <v>0.522882665824842</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
@@ -1052,13 +1044,13 @@
         <v>1</v>
       </c>
       <c r="Q6" t="n">
-        <v>0.3059273246456057</v>
+        <v>0.382547090208058</v>
       </c>
       <c r="R6" t="n">
-        <v>0.5742505050190818</v>
+        <v>0.4510367435026111</v>
       </c>
       <c r="S6" t="n">
-        <v>0.1198221703353124</v>
+        <v>0.1664161662893308</v>
       </c>
       <c r="T6" t="n">
         <v>1</v>
@@ -1067,32 +1059,34 @@
         <v>1</v>
       </c>
       <c r="V6" t="n">
+        <v>1</v>
+      </c>
+      <c r="W6" t="n">
         <v>0</v>
       </c>
-      <c r="W6" t="n">
-        <v>1</v>
-      </c>
       <c r="X6" t="n">
-        <v>0.5742505050190818</v>
+        <v>1</v>
       </c>
       <c r="Y6" t="n">
+        <v>0.4510367435026111</v>
+      </c>
+      <c r="Z6" t="n">
         <v>1.67</v>
       </c>
-      <c r="Z6" t="inlineStr">
+      <c r="AA6" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
-      <c r="AA6" t="n">
-        <v>-0.06119650241512453</v>
-      </c>
       <c r="AB6" t="n">
-        <v>1.320776161543888</v>
+        <v>-0.3683114005233427</v>
       </c>
       <c r="AC6" t="n">
-        <v>0.2683231803734761</v>
-      </c>
-      <c r="AD6" t="inlineStr"/>
+        <v>1.291157522755282</v>
+      </c>
+      <c r="AD6" t="n">
+        <v>0.06848965329455309</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
@@ -1154,13 +1148,13 @@
         <v>1</v>
       </c>
       <c r="Q7" t="n">
-        <v>0.2806571112202151</v>
+        <v>0.2831998851258044</v>
       </c>
       <c r="R7" t="n">
-        <v>0.6335197493837517</v>
+        <v>0.6404508131612661</v>
       </c>
       <c r="S7" t="n">
-        <v>0.08582313939603335</v>
+        <v>0.0763493017129296</v>
       </c>
       <c r="T7" t="n">
         <v>1</v>
@@ -1168,33 +1162,31 @@
       <c r="U7" t="n">
         <v>1</v>
       </c>
-      <c r="V7" t="n">
-        <v>0</v>
-      </c>
-      <c r="W7" t="n">
-        <v>1</v>
-      </c>
+      <c r="V7" t="inlineStr"/>
+      <c r="W7" t="inlineStr"/>
       <c r="X7" t="n">
-        <v>0.6335197493837517</v>
+        <v>1</v>
       </c>
       <c r="Y7" t="n">
+        <v>0.6404508131612661</v>
+      </c>
+      <c r="Z7" t="n">
         <v>1.4</v>
       </c>
-      <c r="Z7" t="inlineStr">
+      <c r="AA7" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
-      <c r="AA7" t="n">
-        <v>-0.2826808771568695</v>
-      </c>
       <c r="AB7" t="n">
-        <v>1.457095423582629</v>
+        <v>-0.2584221539355691</v>
       </c>
       <c r="AC7" t="n">
-        <v>0.3528626381635366</v>
-      </c>
-      <c r="AD7" t="inlineStr"/>
+        <v>1.953542342957054</v>
+      </c>
+      <c r="AD7" t="n">
+        <v>0.3572509280354617</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
@@ -1256,65 +1248,63 @@
         <v>1</v>
       </c>
       <c r="Q8" t="n">
-        <v>0.3532584439150531</v>
+        <v>0.3834058669835496</v>
       </c>
       <c r="R8" t="n">
-        <v>0.2468355864359062</v>
+        <v>0.2995446005919141</v>
       </c>
       <c r="S8" t="n">
-        <v>0.3999059696490407</v>
+        <v>0.3170495324245363</v>
       </c>
       <c r="T8" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="U8" t="n">
         <v>1</v>
       </c>
-      <c r="V8" t="n">
+      <c r="V8" t="inlineStr"/>
+      <c r="W8" t="inlineStr"/>
+      <c r="X8" t="n">
         <v>0</v>
       </c>
-      <c r="W8" t="n">
-        <v>2</v>
-      </c>
-      <c r="X8" t="n">
-        <v>0.3999059696490407</v>
-      </c>
       <c r="Y8" t="n">
-        <v>3</v>
-      </c>
-      <c r="Z8" t="inlineStr">
+        <v>0.3834058669835496</v>
+      </c>
+      <c r="Z8" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="AA8" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
-      <c r="AA8" t="n">
-        <v>0.09985895447356113</v>
-      </c>
       <c r="AB8" t="n">
-        <v>4.598918650963968</v>
+        <v>0.1153214613242233</v>
       </c>
       <c r="AC8" t="n">
-        <v>0.04664752573398767</v>
-      </c>
-      <c r="AD8" t="inlineStr"/>
+        <v>4.025761603327271</v>
+      </c>
+      <c r="AD8" t="n">
+        <v>0.0663563345590133</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
         <is>
-          <t>zgoMLawP</t>
+          <t>QHQVu3Ot</t>
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>45749.65625</v>
+        <v>45748.66666666666</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>brighton</t>
+          <t>nottingham</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>aston villa</t>
+          <t>manchester utd</t>
         </is>
       </c>
       <c r="E9" t="n">
@@ -1334,71 +1324,69 @@
         </is>
       </c>
       <c r="I9" t="n">
-        <v>2</v>
+        <v>2.1</v>
       </c>
       <c r="J9" t="n">
-        <v>4</v>
+        <v>3.6</v>
       </c>
       <c r="K9" t="n">
         <v>3.2</v>
       </c>
       <c r="L9" t="n">
-        <v>0.4705882352941176</v>
+        <v>0.4465116279069767</v>
       </c>
       <c r="M9" t="n">
-        <v>0.2352941176470588</v>
+        <v>0.2604651162790698</v>
       </c>
       <c r="N9" t="n">
-        <v>0.2941176470588235</v>
+        <v>0.2930232558139535</v>
       </c>
       <c r="O9" t="n">
-        <v>0.0625</v>
+        <v>0.06646825396825395</v>
       </c>
       <c r="P9" t="n">
         <v>1</v>
       </c>
       <c r="Q9" t="n">
-        <v>0.3030295671751106</v>
+        <v>0.3662755710119722</v>
       </c>
       <c r="R9" t="n">
-        <v>0.3236877257425403</v>
+        <v>0.3574092605825145</v>
       </c>
       <c r="S9" t="n">
-        <v>0.3732827070823491</v>
+        <v>0.2763151684055133</v>
       </c>
       <c r="T9" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="U9" t="n">
         <v>1</v>
       </c>
-      <c r="V9" t="n">
+      <c r="V9" t="inlineStr"/>
+      <c r="W9" t="inlineStr"/>
+      <c r="X9" t="n">
         <v>0</v>
       </c>
-      <c r="W9" t="n">
-        <v>2</v>
-      </c>
-      <c r="X9" t="n">
-        <v>0.3732827070823491</v>
-      </c>
       <c r="Y9" t="n">
-        <v>3.2</v>
-      </c>
-      <c r="Z9" t="inlineStr">
+        <v>0.3662755710119722</v>
+      </c>
+      <c r="Z9" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="AA9" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
-      <c r="AA9" t="n">
-        <v>0.08841121030159861</v>
-      </c>
       <c r="AB9" t="n">
-        <v>4.292751131447014</v>
+        <v>0.1225354060165768</v>
       </c>
       <c r="AC9" t="n">
-        <v>0.04959498133980877</v>
-      </c>
-      <c r="AD9" t="inlineStr"/>
+        <v>3.845893495625708</v>
+      </c>
+      <c r="AD9" t="n">
+        <v>0.008866310429457624</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
@@ -1460,13 +1448,13 @@
         <v>2</v>
       </c>
       <c r="Q10" t="n">
-        <v>0.3263256215634965</v>
+        <v>0.4055130249341327</v>
       </c>
       <c r="R10" t="n">
-        <v>0.2439163078866845</v>
+        <v>0.180333828207914</v>
       </c>
       <c r="S10" t="n">
-        <v>0.4297580705498191</v>
+        <v>0.4141531468579533</v>
       </c>
       <c r="T10" t="n">
         <v>2</v>
@@ -1475,32 +1463,34 @@
         <v>1</v>
       </c>
       <c r="V10" t="n">
+        <v>1</v>
+      </c>
+      <c r="W10" t="n">
         <v>0</v>
       </c>
-      <c r="W10" t="n">
+      <c r="X10" t="n">
         <v>2</v>
       </c>
-      <c r="X10" t="n">
-        <v>0.4297580705498191</v>
-      </c>
       <c r="Y10" t="n">
+        <v>0.4141531468579533</v>
+      </c>
+      <c r="Z10" t="n">
         <v>1.62</v>
       </c>
-      <c r="Z10" t="inlineStr">
+      <c r="AA10" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
-      <c r="AA10" t="n">
-        <v>-0.4899869769504726</v>
-      </c>
       <c r="AB10" t="n">
-        <v>4.942217811322919</v>
+        <v>-0.5307611324034121</v>
       </c>
       <c r="AC10" t="n">
-        <v>0.1034324489863226</v>
-      </c>
-      <c r="AD10" t="inlineStr"/>
+        <v>1.07364054753249</v>
+      </c>
+      <c r="AD10" t="n">
+        <v>0.008640121923820576</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
@@ -1562,13 +1552,13 @@
         <v>1</v>
       </c>
       <c r="Q11" t="n">
-        <v>0.2753329667748542</v>
+        <v>0.1925364736516477</v>
       </c>
       <c r="R11" t="n">
-        <v>0.4527139176534847</v>
+        <v>0.4269318489910416</v>
       </c>
       <c r="S11" t="n">
-        <v>0.2719531155716611</v>
+        <v>0.3805316773573108</v>
       </c>
       <c r="T11" t="n">
         <v>1</v>
@@ -1577,33 +1567,33 @@
         <v>1</v>
       </c>
       <c r="V11" t="n">
+        <v>1</v>
+      </c>
+      <c r="W11" t="n">
         <v>0</v>
       </c>
-      <c r="W11" t="n">
-        <v>1</v>
-      </c>
       <c r="X11" t="n">
-        <v>0.4527139176534847</v>
+        <v>1</v>
       </c>
       <c r="Y11" t="n">
+        <v>0.4269318489910416</v>
+      </c>
+      <c r="Z11" t="n">
         <v>1.75</v>
       </c>
-      <c r="Z11" t="inlineStr">
+      <c r="AA11" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
-      <c r="AA11" t="n">
-        <v>-0.2770008588085357</v>
-      </c>
       <c r="AB11" t="n">
-        <v>2.603105026507537</v>
+        <v>-0.3371590190209028</v>
       </c>
       <c r="AC11" t="n">
-        <v>0.1773809508786305</v>
+        <v>3.111797646121697</v>
       </c>
       <c r="AD11" t="n">
-        <v>1</v>
+        <v>0.04640017163373084</v>
       </c>
     </row>
     <row r="12">
@@ -1666,13 +1656,13 @@
         <v>1</v>
       </c>
       <c r="Q12" t="n">
-        <v>0.2625045066910773</v>
+        <v>0.3757457166812839</v>
       </c>
       <c r="R12" t="n">
-        <v>0.4112374006939144</v>
+        <v>0.42991455295273</v>
       </c>
       <c r="S12" t="n">
-        <v>0.3262580926150082</v>
+        <v>0.1943397303659861</v>
       </c>
       <c r="T12" t="n">
         <v>1</v>
@@ -1681,30 +1671,30 @@
         <v>1</v>
       </c>
       <c r="V12" t="inlineStr"/>
-      <c r="W12" t="n">
-        <v>1</v>
-      </c>
+      <c r="W12" t="inlineStr"/>
       <c r="X12" t="n">
-        <v>0.4112374006939144</v>
+        <v>1</v>
       </c>
       <c r="Y12" t="n">
+        <v>0.42991455295273</v>
+      </c>
+      <c r="Z12" t="n">
         <v>1.95</v>
       </c>
-      <c r="Z12" t="inlineStr">
+      <c r="AA12" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
-      <c r="AA12" t="n">
-        <v>-0.2085127038388074</v>
-      </c>
       <c r="AB12" t="n">
-        <v>2.364615053990008</v>
+        <v>-0.1701753913075543</v>
       </c>
       <c r="AC12" t="n">
-        <v>0.08497930807890619</v>
-      </c>
-      <c r="AD12" t="inlineStr"/>
+        <v>3.442443717761873</v>
+      </c>
+      <c r="AD12" t="n">
+        <v>0.05416883627144609</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
@@ -1766,13 +1756,13 @@
         <v>1</v>
       </c>
       <c r="Q13" t="n">
-        <v>0.3864521213741127</v>
+        <v>0.4472576318312867</v>
       </c>
       <c r="R13" t="n">
-        <v>0.3207498404333426</v>
+        <v>0.307467370706631</v>
       </c>
       <c r="S13" t="n">
-        <v>0.2927980381925447</v>
+        <v>0.2452749974620823</v>
       </c>
       <c r="T13" t="n">
         <v>0</v>
@@ -1781,33 +1771,33 @@
         <v>1</v>
       </c>
       <c r="V13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W13" t="n">
         <v>0</v>
       </c>
       <c r="X13" t="n">
-        <v>0.3864521213741127</v>
+        <v>0</v>
       </c>
       <c r="Y13" t="n">
+        <v>0.4472576318312867</v>
+      </c>
+      <c r="Z13" t="n">
         <v>3.8</v>
       </c>
-      <c r="Z13" t="inlineStr">
+      <c r="AA13" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
-      <c r="AA13" t="n">
-        <v>0.1673278790077244</v>
-      </c>
       <c r="AB13" t="n">
-        <v>0.8888398791604594</v>
+        <v>0.2498496431996034</v>
       </c>
       <c r="AC13" t="n">
-        <v>0.06570228094077013</v>
+        <v>2.348102567114255</v>
       </c>
       <c r="AD13" t="n">
-        <v>1</v>
+        <v>0.1397902611246557</v>
       </c>
     </row>
     <row r="14">
@@ -1870,13 +1860,13 @@
         <v>2</v>
       </c>
       <c r="Q14" t="n">
-        <v>0.2917475912376913</v>
+        <v>0.3369108966757062</v>
       </c>
       <c r="R14" t="n">
-        <v>0.1940946840876043</v>
+        <v>0.1635641496454571</v>
       </c>
       <c r="S14" t="n">
-        <v>0.5141577246747043</v>
+        <v>0.4995249536788367</v>
       </c>
       <c r="T14" t="n">
         <v>2</v>
@@ -1885,33 +1875,33 @@
         <v>1</v>
       </c>
       <c r="V14" t="n">
+        <v>1</v>
+      </c>
+      <c r="W14" t="n">
         <v>0</v>
       </c>
-      <c r="W14" t="n">
+      <c r="X14" t="n">
         <v>2</v>
       </c>
-      <c r="X14" t="n">
-        <v>0.5141577246747043</v>
-      </c>
       <c r="Y14" t="n">
+        <v>0.4995249536788367</v>
+      </c>
+      <c r="Z14" t="n">
         <v>2.45</v>
       </c>
-      <c r="Z14" t="inlineStr">
+      <c r="AA14" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
-      <c r="AA14" t="n">
-        <v>0.179094086519328</v>
-      </c>
       <c r="AB14" t="n">
-        <v>5.321532450383191</v>
+        <v>0.1543697493194137</v>
       </c>
       <c r="AC14" t="n">
-        <v>0.222410133437013</v>
+        <v>7.867518020441678</v>
       </c>
       <c r="AD14" t="n">
-        <v>1</v>
+        <v>0.1626140570031305</v>
       </c>
     </row>
     <row r="15">
@@ -1974,13 +1964,13 @@
         <v>2</v>
       </c>
       <c r="Q15" t="n">
-        <v>0.1004835089647717</v>
+        <v>0.1967406352454221</v>
       </c>
       <c r="R15" t="n">
-        <v>0.1174483317310698</v>
+        <v>0.1070292013445253</v>
       </c>
       <c r="S15" t="n">
-        <v>0.7820681593041585</v>
+        <v>0.6962301634100526</v>
       </c>
       <c r="T15" t="n">
         <v>2</v>
@@ -1989,33 +1979,33 @@
         <v>1</v>
       </c>
       <c r="V15" t="n">
+        <v>1</v>
+      </c>
+      <c r="W15" t="n">
         <v>0</v>
       </c>
-      <c r="W15" t="n">
+      <c r="X15" t="n">
         <v>2</v>
       </c>
-      <c r="X15" t="n">
-        <v>0.7820681593041585</v>
-      </c>
       <c r="Y15" t="n">
+        <v>0.6962301634100526</v>
+      </c>
+      <c r="Z15" t="n">
         <v>1.6</v>
       </c>
-      <c r="Z15" t="inlineStr">
+      <c r="AA15" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
-      <c r="AA15" t="n">
-        <v>0.4188484248110894</v>
-      </c>
       <c r="AB15" t="n">
-        <v>8.094405448798042</v>
+        <v>0.189947102426807</v>
       </c>
       <c r="AC15" t="n">
-        <v>0.6646198275730887</v>
+        <v>10.96562507370833</v>
       </c>
       <c r="AD15" t="n">
-        <v>1</v>
+        <v>0.4994895281646305</v>
       </c>
     </row>
     <row r="16">
@@ -2078,13 +2068,13 @@
         <v>2</v>
       </c>
       <c r="Q16" t="n">
-        <v>0.1038261377896294</v>
+        <v>0.235459764596706</v>
       </c>
       <c r="R16" t="n">
-        <v>0.02733959788000358</v>
+        <v>0.020806732360019</v>
       </c>
       <c r="S16" t="n">
-        <v>0.868834264330367</v>
+        <v>0.743733503043275</v>
       </c>
       <c r="T16" t="n">
         <v>2</v>
@@ -2092,34 +2082,30 @@
       <c r="U16" t="n">
         <v>1</v>
       </c>
-      <c r="V16" t="n">
-        <v>0</v>
-      </c>
-      <c r="W16" t="n">
+      <c r="V16" t="inlineStr"/>
+      <c r="W16" t="inlineStr"/>
+      <c r="X16" t="n">
         <v>2</v>
       </c>
-      <c r="X16" t="n">
-        <v>0.868834264330367</v>
-      </c>
       <c r="Y16" t="n">
+        <v>0.743733503043275</v>
+      </c>
+      <c r="Z16" t="n">
         <v>1.14</v>
       </c>
-      <c r="Z16" t="inlineStr">
+      <c r="AA16" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
-      <c r="AA16" t="n">
-        <v>-0.0680638475955834</v>
-      </c>
       <c r="AB16" t="n">
-        <v>8.992434635819299</v>
+        <v>-1.086741475219048</v>
       </c>
       <c r="AC16" t="n">
-        <v>0.7650081265407377</v>
+        <v>5.909200568288616</v>
       </c>
       <c r="AD16" t="n">
-        <v>1</v>
+        <v>0.5082737384465691</v>
       </c>
     </row>
     <row r="17">
@@ -2182,13 +2168,13 @@
         <v>1</v>
       </c>
       <c r="Q17" t="n">
-        <v>0.249670691980813</v>
+        <v>0.3058077490559443</v>
       </c>
       <c r="R17" t="n">
-        <v>0.1947457207697191</v>
+        <v>0.2525813459229875</v>
       </c>
       <c r="S17" t="n">
-        <v>0.5555835872494679</v>
+        <v>0.4416109050210683</v>
       </c>
       <c r="T17" t="n">
         <v>2</v>
@@ -2197,33 +2183,33 @@
         <v>1</v>
       </c>
       <c r="V17" t="n">
+        <v>1</v>
+      </c>
+      <c r="W17" t="n">
         <v>0</v>
       </c>
-      <c r="W17" t="n">
+      <c r="X17" t="n">
         <v>2</v>
       </c>
-      <c r="X17" t="n">
-        <v>0.5555835872494679</v>
-      </c>
       <c r="Y17" t="n">
+        <v>0.4416109050210683</v>
+      </c>
+      <c r="Z17" t="n">
         <v>4.1</v>
       </c>
-      <c r="Z17" t="inlineStr">
+      <c r="AA17" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
-      <c r="AA17" t="n">
-        <v>0.4122234541041349</v>
-      </c>
       <c r="AB17" t="n">
-        <v>5.750290128031993</v>
+        <v>0.2614853905117354</v>
       </c>
       <c r="AC17" t="n">
-        <v>0.3059128952686548</v>
+        <v>6.955371754081825</v>
       </c>
       <c r="AD17" t="n">
-        <v>1</v>
+        <v>0.1358031559651239</v>
       </c>
     </row>
     <row r="18">
@@ -2286,13 +2272,13 @@
         <v>2</v>
       </c>
       <c r="Q18" t="n">
-        <v>0.3637247043428444</v>
+        <v>0.3697548099325002</v>
       </c>
       <c r="R18" t="n">
-        <v>0.1868887254677783</v>
+        <v>0.1252853591008778</v>
       </c>
       <c r="S18" t="n">
-        <v>0.4493865701893771</v>
+        <v>0.504959830966622</v>
       </c>
       <c r="T18" t="n">
         <v>2</v>
@@ -2301,30 +2287,30 @@
         <v>1</v>
       </c>
       <c r="V18" t="inlineStr"/>
-      <c r="W18" t="n">
+      <c r="W18" t="inlineStr"/>
+      <c r="X18" t="n">
         <v>2</v>
       </c>
-      <c r="X18" t="n">
-        <v>0.4493865701893771</v>
-      </c>
       <c r="Y18" t="n">
+        <v>0.504959830966622</v>
+      </c>
+      <c r="Z18" t="n">
         <v>1.91</v>
       </c>
-      <c r="Z18" t="inlineStr">
+      <c r="AA18" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
-      <c r="AA18" t="n">
-        <v>-0.1556831328992195</v>
-      </c>
       <c r="AB18" t="n">
-        <v>4.651151001460053</v>
+        <v>-0.03904035478434289</v>
       </c>
       <c r="AC18" t="n">
-        <v>0.08566186584653268</v>
-      </c>
-      <c r="AD18" t="inlineStr"/>
+        <v>7.797890791673002</v>
+      </c>
+      <c r="AD18" t="n">
+        <v>0.1352050210341218</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="inlineStr">
@@ -2386,13 +2372,13 @@
         <v>2</v>
       </c>
       <c r="Q19" t="n">
-        <v>0.1466450563544316</v>
+        <v>0.3276280230264123</v>
       </c>
       <c r="R19" t="n">
-        <v>0.2802032080537756</v>
+        <v>0.3049725845117274</v>
       </c>
       <c r="S19" t="n">
-        <v>0.5731517355917929</v>
+        <v>0.3673993924618603</v>
       </c>
       <c r="T19" t="n">
         <v>2</v>
@@ -2401,33 +2387,33 @@
         <v>1</v>
       </c>
       <c r="V19" t="n">
+        <v>1</v>
+      </c>
+      <c r="W19" t="n">
         <v>0</v>
       </c>
-      <c r="W19" t="n">
+      <c r="X19" t="n">
         <v>2</v>
       </c>
-      <c r="X19" t="n">
-        <v>0.5731517355917929</v>
-      </c>
       <c r="Y19" t="n">
+        <v>0.3673993924618603</v>
+      </c>
+      <c r="Z19" t="n">
         <v>2.55</v>
       </c>
-      <c r="Z19" t="inlineStr">
+      <c r="AA19" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
-      <c r="AA19" t="n">
-        <v>0.2977657585542399</v>
-      </c>
       <c r="AB19" t="n">
-        <v>5.932120463375057</v>
+        <v>-0.0407300317562943</v>
       </c>
       <c r="AC19" t="n">
-        <v>0.2929485275380173</v>
+        <v>5.668713731969236</v>
       </c>
       <c r="AD19" t="n">
-        <v>1</v>
+        <v>0.03977136943544807</v>
       </c>
     </row>
     <row r="20">
@@ -2505,30 +2491,30 @@
         <v>1</v>
       </c>
       <c r="V20" t="inlineStr"/>
-      <c r="W20" t="n">
-        <v>1</v>
-      </c>
+      <c r="W20" t="inlineStr"/>
       <c r="X20" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y20" t="n">
         <v>0.7825458264646554</v>
       </c>
-      <c r="Y20" t="n">
+      <c r="Z20" t="n">
         <v>1.27</v>
       </c>
-      <c r="Z20" t="inlineStr">
+      <c r="AA20" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
-      <c r="AA20" t="n">
+      <c r="AB20" t="n">
         <v>-0.02284000144402813</v>
       </c>
-      <c r="AB20" t="n">
-        <v>1.799855400868708</v>
-      </c>
       <c r="AC20" t="n">
+        <v>2.707633393631191</v>
+      </c>
+      <c r="AD20" t="n">
         <v>0.6113133678474076</v>
       </c>
-      <c r="AD20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="1" t="inlineStr">
@@ -2605,30 +2591,30 @@
         <v>1</v>
       </c>
       <c r="V21" t="inlineStr"/>
-      <c r="W21" t="n">
-        <v>1</v>
-      </c>
+      <c r="W21" t="inlineStr"/>
       <c r="X21" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y21" t="n">
         <v>0.9006459813523363</v>
       </c>
-      <c r="Y21" t="n">
+      <c r="Z21" t="n">
         <v>1.14</v>
       </c>
-      <c r="Z21" t="inlineStr">
+      <c r="AA21" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
-      <c r="AA21" t="n">
+      <c r="AB21" t="n">
         <v>0.1909744195833094</v>
       </c>
-      <c r="AB21" t="n">
-        <v>2.071485757110374</v>
-      </c>
       <c r="AC21" t="n">
+        <v>3.152260934733177</v>
+      </c>
+      <c r="AD21" t="n">
         <v>0.8256672270830573</v>
       </c>
-      <c r="AD21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="1" t="inlineStr">
@@ -2705,30 +2691,30 @@
         <v>1</v>
       </c>
       <c r="V22" t="inlineStr"/>
-      <c r="W22" t="n">
-        <v>1</v>
-      </c>
+      <c r="W22" t="inlineStr"/>
       <c r="X22" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y22" t="n">
         <v>0.5091193002336956</v>
       </c>
-      <c r="Y22" t="n">
+      <c r="Z22" t="n">
         <v>2.35</v>
       </c>
-      <c r="Z22" t="inlineStr">
+      <c r="AA22" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
-      <c r="AA22" t="n">
+      <c r="AB22" t="n">
         <v>0.1455039670734701</v>
       </c>
-      <c r="AB22" t="n">
-        <v>1.1709743905375</v>
-      </c>
       <c r="AC22" t="n">
+        <v>1.781917550817935</v>
+      </c>
+      <c r="AD22" t="n">
         <v>0.2049859611591311</v>
       </c>
-      <c r="AD22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="1" t="inlineStr">
@@ -2805,30 +2791,30 @@
         <v>1</v>
       </c>
       <c r="V23" t="inlineStr"/>
-      <c r="W23" t="n">
-        <v>1</v>
-      </c>
+      <c r="W23" t="inlineStr"/>
       <c r="X23" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y23" t="n">
         <v>0.5373389783576131</v>
       </c>
-      <c r="Y23" t="n">
+      <c r="Z23" t="n">
         <v>1.65</v>
       </c>
-      <c r="Z23" t="inlineStr">
+      <c r="AA23" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
-      <c r="AA23" t="n">
+      <c r="AB23" t="n">
         <v>-0.1744472087845206</v>
       </c>
-      <c r="AB23" t="n">
-        <v>1.23587965022251</v>
-      </c>
       <c r="AC23" t="n">
+        <v>1.717060917236152</v>
+      </c>
+      <c r="AD23" t="n">
         <v>0.2473442706888411</v>
       </c>
-      <c r="AD23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="1" t="inlineStr">
@@ -2905,33 +2891,33 @@
         <v>1</v>
       </c>
       <c r="V24" t="n">
+        <v>1</v>
+      </c>
+      <c r="W24" t="n">
         <v>0</v>
       </c>
-      <c r="W24" t="n">
-        <v>1</v>
-      </c>
       <c r="X24" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y24" t="n">
         <v>0.4066937553467808</v>
       </c>
-      <c r="Y24" t="n">
+      <c r="Z24" t="n">
         <v>2</v>
       </c>
-      <c r="Z24" t="inlineStr">
+      <c r="AA24" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
-      <c r="AA24" t="n">
+      <c r="AB24" t="n">
         <v>-0.1866124893064383</v>
       </c>
-      <c r="AB24" t="n">
-        <v>0.9353956372975959</v>
-      </c>
       <c r="AC24" t="n">
+        <v>1.290997502378281</v>
+      </c>
+      <c r="AD24" t="n">
         <v>0.03813939040308317</v>
-      </c>
-      <c r="AD24" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="25">
@@ -3009,30 +2995,30 @@
         <v>1</v>
       </c>
       <c r="V25" t="inlineStr"/>
-      <c r="W25" t="n">
-        <v>1</v>
-      </c>
+      <c r="W25" t="inlineStr"/>
       <c r="X25" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y25" t="n">
         <v>0.7198839679267474</v>
       </c>
-      <c r="Y25" t="n">
+      <c r="Z25" t="n">
         <v>1.7</v>
       </c>
-      <c r="Z25" t="inlineStr">
+      <c r="AA25" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
-      <c r="AA25" t="n">
+      <c r="AB25" t="n">
         <v>0.3197182078221008</v>
       </c>
-      <c r="AB25" t="n">
-        <v>1.655733126231519</v>
-      </c>
       <c r="AC25" t="n">
+        <v>2.519593887743615</v>
+      </c>
+      <c r="AD25" t="n">
         <v>0.5506784616981166</v>
       </c>
-      <c r="AD25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="1" t="inlineStr">
@@ -3109,30 +3095,30 @@
         <v>1</v>
       </c>
       <c r="V26" t="inlineStr"/>
-      <c r="W26" t="n">
+      <c r="W26" t="inlineStr"/>
+      <c r="X26" t="n">
         <v>0</v>
       </c>
-      <c r="X26" t="n">
+      <c r="Y26" t="n">
         <v>0.454936820626022</v>
       </c>
-      <c r="Y26" t="n">
+      <c r="Z26" t="n">
         <v>3.8</v>
       </c>
-      <c r="Z26" t="inlineStr">
+      <c r="AA26" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
-      <c r="AA26" t="n">
+      <c r="AB26" t="n">
         <v>0.2602713994210298</v>
       </c>
-      <c r="AB26" t="n">
-        <v>4.708596093479327</v>
-      </c>
       <c r="AC26" t="n">
+        <v>7.165254924859846</v>
+      </c>
+      <c r="AD26" t="n">
         <v>0.09499876507328531</v>
       </c>
-      <c r="AD26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="1" t="inlineStr">
@@ -3209,30 +3195,30 @@
         <v>1</v>
       </c>
       <c r="V27" t="inlineStr"/>
-      <c r="W27" t="n">
+      <c r="W27" t="inlineStr"/>
+      <c r="X27" t="n">
         <v>0</v>
       </c>
-      <c r="X27" t="n">
+      <c r="Y27" t="n">
         <v>0.4125590999147862</v>
       </c>
-      <c r="Y27" t="n">
+      <c r="Z27" t="n">
         <v>3.75</v>
       </c>
-      <c r="Z27" t="inlineStr">
+      <c r="AA27" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
-      <c r="AA27" t="n">
+      <c r="AB27" t="n">
         <v>0.1989442271565266</v>
       </c>
-      <c r="AB27" t="n">
-        <v>4.269986684118037</v>
-      </c>
       <c r="AC27" t="n">
+        <v>6.497805823657882</v>
+      </c>
+      <c r="AD27" t="n">
         <v>0.09581271511068973</v>
       </c>
-      <c r="AD27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="1" t="inlineStr">
@@ -3309,30 +3295,30 @@
         <v>1</v>
       </c>
       <c r="V28" t="inlineStr"/>
-      <c r="W28" t="n">
+      <c r="W28" t="inlineStr"/>
+      <c r="X28" t="n">
         <v>2</v>
       </c>
-      <c r="X28" t="n">
+      <c r="Y28" t="n">
         <v>0.4142279663281674</v>
       </c>
-      <c r="Y28" t="n">
+      <c r="Z28" t="n">
         <v>2.25</v>
       </c>
-      <c r="Z28" t="inlineStr">
+      <c r="AA28" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
-      <c r="AA28" t="n">
+      <c r="AB28" t="n">
         <v>-0.05438966060929866</v>
       </c>
-      <c r="AB28" t="n">
-        <v>3.334535128941748</v>
-      </c>
       <c r="AC28" t="n">
+        <v>4.936332069980979</v>
+      </c>
+      <c r="AD28" t="n">
         <v>0.0509843071978795</v>
       </c>
-      <c r="AD28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="1" t="inlineStr">
@@ -3409,30 +3395,30 @@
         <v>1</v>
       </c>
       <c r="V29" t="inlineStr"/>
-      <c r="W29" t="n">
-        <v>1</v>
-      </c>
+      <c r="W29" t="inlineStr"/>
       <c r="X29" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y29" t="n">
         <v>0.6092363933642873</v>
       </c>
-      <c r="Y29" t="n">
+      <c r="Z29" t="n">
         <v>1.73</v>
       </c>
-      <c r="Z29" t="inlineStr">
+      <c r="AA29" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
-      <c r="AA29" t="n">
+      <c r="AB29" t="n">
         <v>0.07394378153454376</v>
       </c>
-      <c r="AB29" t="n">
-        <v>1.401243704737861</v>
-      </c>
       <c r="AC29" t="n">
+        <v>2.132327376775005</v>
+      </c>
+      <c r="AD29" t="n">
         <v>0.3279189310629804</v>
       </c>
-      <c r="AD29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="1" t="inlineStr">
@@ -3509,30 +3495,30 @@
         <v>1</v>
       </c>
       <c r="V30" t="inlineStr"/>
-      <c r="W30" t="n">
-        <v>1</v>
-      </c>
+      <c r="W30" t="inlineStr"/>
       <c r="X30" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y30" t="n">
         <v>0.5936828179907958</v>
       </c>
-      <c r="Y30" t="n">
+      <c r="Z30" t="n">
         <v>1.55</v>
       </c>
-      <c r="Z30" t="inlineStr">
+      <c r="AA30" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
-      <c r="AA30" t="n">
+      <c r="AB30" t="n">
         <v>-0.1450756947532118</v>
       </c>
-      <c r="AB30" t="n">
-        <v>1.36547048137883</v>
-      </c>
       <c r="AC30" t="n">
+        <v>1.927428009713883</v>
+      </c>
+      <c r="AD30" t="n">
         <v>0.2890948059640486</v>
       </c>
-      <c r="AD30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="1" t="inlineStr">
@@ -3609,30 +3595,30 @@
         <v>1</v>
       </c>
       <c r="V31" t="inlineStr"/>
-      <c r="W31" t="n">
-        <v>1</v>
-      </c>
+      <c r="W31" t="inlineStr"/>
       <c r="X31" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y31" t="n">
         <v>0.4555702555943796</v>
       </c>
-      <c r="Y31" t="n">
+      <c r="Z31" t="n">
         <v>1.67</v>
       </c>
-      <c r="Z31" t="inlineStr">
+      <c r="AA31" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
-      <c r="AA31" t="n">
+      <c r="AB31" t="n">
         <v>-0.3570114524737107</v>
       </c>
-      <c r="AB31" t="n">
-        <v>1.047811587867073</v>
-      </c>
       <c r="AC31" t="n">
+        <v>1.312854347869637</v>
+      </c>
+      <c r="AD31" t="n">
         <v>0.032470168263524</v>
       </c>
-      <c r="AD31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="1" t="inlineStr">
@@ -3709,30 +3695,30 @@
         <v>1</v>
       </c>
       <c r="V32" t="inlineStr"/>
-      <c r="W32" t="n">
-        <v>1</v>
-      </c>
+      <c r="W32" t="inlineStr"/>
       <c r="X32" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y32" t="n">
         <v>0.6727771930227373</v>
       </c>
-      <c r="Y32" t="n">
+      <c r="Z32" t="n">
         <v>1.42</v>
       </c>
-      <c r="Z32" t="inlineStr">
+      <c r="AA32" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
-      <c r="AA32" t="n">
+      <c r="AB32" t="n">
         <v>-0.1063247283516979</v>
       </c>
-      <c r="AB32" t="n">
-        <v>1.547387543952296</v>
-      </c>
       <c r="AC32" t="n">
+        <v>2.229655482699205</v>
+      </c>
+      <c r="AD32" t="n">
         <v>0.3988900842851951</v>
       </c>
-      <c r="AD32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="1" t="inlineStr">
@@ -3809,33 +3795,33 @@
         <v>1</v>
       </c>
       <c r="V33" t="n">
+        <v>1</v>
+      </c>
+      <c r="W33" t="n">
         <v>0</v>
       </c>
-      <c r="W33" t="n">
-        <v>1</v>
-      </c>
       <c r="X33" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y33" t="n">
         <v>0.3682104980889199</v>
       </c>
-      <c r="Y33" t="n">
+      <c r="Z33" t="n">
         <v>1.9</v>
       </c>
-      <c r="Z33" t="inlineStr">
+      <c r="AA33" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
-      <c r="AA33" t="n">
+      <c r="AB33" t="n">
         <v>-0.333777837367836</v>
       </c>
-      <c r="AB33" t="n">
-        <v>0.8468841456045157</v>
-      </c>
       <c r="AC33" t="n">
+        <v>1.07563562243901</v>
+      </c>
+      <c r="AD33" t="n">
         <v>0.02632416652920944</v>
-      </c>
-      <c r="AD33" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="34">
@@ -3913,30 +3899,30 @@
         <v>1</v>
       </c>
       <c r="V34" t="inlineStr"/>
-      <c r="W34" t="n">
+      <c r="W34" t="inlineStr"/>
+      <c r="X34" t="n">
         <v>0</v>
       </c>
-      <c r="X34" t="n">
+      <c r="Y34" t="n">
         <v>0.4042434275738219</v>
       </c>
-      <c r="Y34" t="n">
+      <c r="Z34" t="n">
         <v>3.4</v>
       </c>
-      <c r="Z34" t="inlineStr">
+      <c r="AA34" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
-      <c r="AA34" t="n">
+      <c r="AB34" t="n">
         <v>0.1560115223962476</v>
       </c>
-      <c r="AB34" t="n">
-        <v>7.438079067358323</v>
-      </c>
       <c r="AC34" t="n">
+        <v>9.196537977304446</v>
+      </c>
+      <c r="AD34" t="n">
         <v>0.03539538923291191</v>
       </c>
-      <c r="AD34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="1" t="inlineStr">
@@ -4013,30 +3999,30 @@
         <v>1</v>
       </c>
       <c r="V35" t="inlineStr"/>
-      <c r="W35" t="n">
+      <c r="W35" t="inlineStr"/>
+      <c r="X35" t="n">
         <v>0</v>
       </c>
-      <c r="X35" t="n">
+      <c r="Y35" t="n">
         <v>0.3765153835048269</v>
       </c>
-      <c r="Y35" t="n">
+      <c r="Z35" t="n">
         <v>3.1</v>
       </c>
-      <c r="Z35" t="inlineStr">
+      <c r="AA35" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
-      <c r="AA35" t="n">
+      <c r="AB35" t="n">
         <v>0.07961794707855407</v>
       </c>
-      <c r="AB35" t="n">
-        <v>6.927883056488816</v>
-      </c>
       <c r="AC35" t="n">
+        <v>8.565724974734813</v>
+      </c>
+      <c r="AD35" t="n">
         <v>0.04439633633870788</v>
       </c>
-      <c r="AD35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="1" t="inlineStr">
@@ -4113,30 +4099,30 @@
         <v>1</v>
       </c>
       <c r="V36" t="inlineStr"/>
-      <c r="W36" t="n">
+      <c r="W36" t="inlineStr"/>
+      <c r="X36" t="n">
         <v>0</v>
       </c>
-      <c r="X36" t="n">
+      <c r="Y36" t="n">
         <v>0.4941601521686576</v>
       </c>
-      <c r="Y36" t="n">
+      <c r="Z36" t="n">
         <v>3.3</v>
       </c>
-      <c r="Z36" t="inlineStr">
+      <c r="AA36" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
-      <c r="AA36" t="n">
+      <c r="AB36" t="n">
         <v>0.2742297835463348</v>
       </c>
-      <c r="AB36" t="n">
-        <v>9.0925467999033</v>
-      </c>
       <c r="AC36" t="n">
+        <v>11.24214346183696</v>
+      </c>
+      <c r="AD36" t="n">
         <v>0.1141177850734852</v>
       </c>
-      <c r="AD36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="1" t="inlineStr">
@@ -4213,33 +4199,33 @@
         <v>1</v>
       </c>
       <c r="V37" t="n">
+        <v>1</v>
+      </c>
+      <c r="W37" t="n">
         <v>0</v>
       </c>
-      <c r="W37" t="n">
+      <c r="X37" t="n">
         <v>2</v>
       </c>
-      <c r="X37" t="n">
+      <c r="Y37" t="n">
         <v>0.6592570027062244</v>
       </c>
-      <c r="Y37" t="n">
+      <c r="Z37" t="n">
         <v>1.83</v>
       </c>
-      <c r="Z37" t="inlineStr">
+      <c r="AA37" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
-      <c r="AA37" t="n">
+      <c r="AB37" t="n">
         <v>0.2487232710269768</v>
       </c>
-      <c r="AB37" t="n">
-        <v>6.065164424897265</v>
-      </c>
       <c r="AC37" t="n">
+        <v>9.229598037887142</v>
+      </c>
+      <c r="AD37" t="n">
         <v>0.4204796570220136</v>
-      </c>
-      <c r="AD37" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="38">
@@ -4317,30 +4303,30 @@
         <v>1</v>
       </c>
       <c r="V38" t="inlineStr"/>
-      <c r="W38" t="n">
+      <c r="W38" t="inlineStr"/>
+      <c r="X38" t="n">
         <v>2</v>
       </c>
-      <c r="X38" t="n">
+      <c r="Y38" t="n">
         <v>0.5489002497277609</v>
       </c>
-      <c r="Y38" t="n">
+      <c r="Z38" t="n">
         <v>1.85</v>
       </c>
-      <c r="Z38" t="inlineStr">
+      <c r="AA38" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
-      <c r="AA38" t="n">
+      <c r="AB38" t="n">
         <v>0.01819466117218543</v>
       </c>
-      <c r="AB38" t="n">
-        <v>5.0498822974954</v>
-      </c>
       <c r="AC38" t="n">
+        <v>7.684603496188651</v>
+      </c>
+      <c r="AD38" t="n">
         <v>0.2162498241274949</v>
       </c>
-      <c r="AD38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="1" t="inlineStr">
@@ -4402,13 +4388,13 @@
         <v>1</v>
       </c>
       <c r="Q39" t="n">
-        <v>0.2305520321597711</v>
+        <v>0.2566780000413285</v>
       </c>
       <c r="R39" t="n">
-        <v>0.683057663326422</v>
+        <v>0.6324699718345181</v>
       </c>
       <c r="S39" t="n">
-        <v>0.0863903045138069</v>
+        <v>0.1108520281241534</v>
       </c>
       <c r="T39" t="n">
         <v>1</v>
@@ -4420,30 +4406,30 @@
         <v>0</v>
       </c>
       <c r="W39" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X39" t="n">
-        <v>0.683057663326422</v>
+        <v>1</v>
       </c>
       <c r="Y39" t="n">
+        <v>0.6324699718345181</v>
+      </c>
+      <c r="Z39" t="n">
         <v>1.29</v>
       </c>
-      <c r="Z39" t="inlineStr">
+      <c r="AA39" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
-      <c r="AA39" t="n">
-        <v>-0.4098469458928122</v>
-      </c>
       <c r="AB39" t="n">
-        <v>1.571032625650771</v>
+        <v>-0.6348749528740398</v>
       </c>
       <c r="AC39" t="n">
-        <v>0.4525056311666509</v>
+        <v>1.533639664385265</v>
       </c>
       <c r="AD39" t="n">
-        <v>0</v>
+        <v>0.3757919717931897</v>
       </c>
     </row>
     <row r="40">
@@ -4506,13 +4492,13 @@
         <v>1</v>
       </c>
       <c r="Q40" t="n">
-        <v>0.2859904113328284</v>
+        <v>0.2797094974858422</v>
       </c>
       <c r="R40" t="n">
-        <v>0.58658003307333</v>
+        <v>0.5810972348504705</v>
       </c>
       <c r="S40" t="n">
-        <v>0.1274295555938417</v>
+        <v>0.1391932676636874</v>
       </c>
       <c r="T40" t="n">
         <v>1</v>
@@ -4524,30 +4510,30 @@
         <v>0</v>
       </c>
       <c r="W40" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X40" t="n">
-        <v>0.58658003307333</v>
+        <v>1</v>
       </c>
       <c r="Y40" t="n">
+        <v>0.5810972348504705</v>
+      </c>
+      <c r="Z40" t="n">
         <v>1.33</v>
       </c>
-      <c r="Z40" t="inlineStr">
+      <c r="AA40" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
-      <c r="AA40" t="n">
-        <v>-0.6662077454923365</v>
-      </c>
       <c r="AB40" t="n">
-        <v>1.349134076068659</v>
+        <v>-0.6883050837844672</v>
       </c>
       <c r="AC40" t="n">
-        <v>0.3005896217405016</v>
+        <v>1.360273986361305</v>
       </c>
       <c r="AD40" t="n">
-        <v>0</v>
+        <v>0.3013877373646283</v>
       </c>
     </row>
     <row r="41">
@@ -4610,13 +4596,13 @@
         <v>1</v>
       </c>
       <c r="Q41" t="n">
-        <v>0.1670022568007548</v>
+        <v>0.2232539112862876</v>
       </c>
       <c r="R41" t="n">
-        <v>0.7906034679051955</v>
+        <v>0.7164941200412097</v>
       </c>
       <c r="S41" t="n">
-        <v>0.04239427529404956</v>
+        <v>0.06025196867250265</v>
       </c>
       <c r="T41" t="n">
         <v>1</v>
@@ -4628,30 +4614,30 @@
         <v>0</v>
       </c>
       <c r="W41" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X41" t="n">
-        <v>0.7906034679051955</v>
+        <v>1</v>
       </c>
       <c r="Y41" t="n">
+        <v>0.7164941200412097</v>
+      </c>
+      <c r="Z41" t="n">
         <v>1.18</v>
       </c>
-      <c r="Z41" t="inlineStr">
+      <c r="AA41" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
-      <c r="AA41" t="n">
-        <v>-0.3727105992881631</v>
-      </c>
       <c r="AB41" t="n">
-        <v>1.81838797618195</v>
+        <v>-0.8585385463965146</v>
       </c>
       <c r="AC41" t="n">
-        <v>0.6236012111044408</v>
+        <v>1.492825121072358</v>
       </c>
       <c r="AD41" t="n">
-        <v>0</v>
+        <v>0.4932402087549221</v>
       </c>
     </row>
     <row r="42">
@@ -4714,13 +4700,13 @@
         <v>1</v>
       </c>
       <c r="Q42" t="n">
-        <v>0.2379869131980451</v>
+        <v>0.2464777551432784</v>
       </c>
       <c r="R42" t="n">
-        <v>0.6507394337021107</v>
+        <v>0.6394868787076196</v>
       </c>
       <c r="S42" t="n">
-        <v>0.1112736530998441</v>
+        <v>0.1140353661491022</v>
       </c>
       <c r="T42" t="n">
         <v>1</v>
@@ -4732,30 +4718,30 @@
         <v>0</v>
       </c>
       <c r="W42" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X42" t="n">
-        <v>0.6507394337021107</v>
+        <v>1</v>
       </c>
       <c r="Y42" t="n">
+        <v>0.6394868787076196</v>
+      </c>
+      <c r="Z42" t="n">
         <v>1.27</v>
       </c>
-      <c r="Z42" t="inlineStr">
+      <c r="AA42" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
-      <c r="AA42" t="n">
-        <v>-0.6428182192530345</v>
-      </c>
       <c r="AB42" t="n">
-        <v>1.496700697514855</v>
+        <v>-0.6957469038567523</v>
       </c>
       <c r="AC42" t="n">
-        <v>0.4127525205040656</v>
+        <v>1.489551077907825</v>
       </c>
       <c r="AD42" t="n">
-        <v>0</v>
+        <v>0.3930091235643412</v>
       </c>
     </row>
     <row r="43">
@@ -4818,13 +4804,13 @@
         <v>1</v>
       </c>
       <c r="Q43" t="n">
-        <v>0.3277161333715918</v>
+        <v>0.2983724417092606</v>
       </c>
       <c r="R43" t="n">
-        <v>0.4978816535233578</v>
+        <v>0.4712586814761995</v>
       </c>
       <c r="S43" t="n">
-        <v>0.1744022131050505</v>
+        <v>0.2303688768145399</v>
       </c>
       <c r="T43" t="n">
         <v>1</v>
@@ -4836,30 +4822,30 @@
         <v>0</v>
       </c>
       <c r="W43" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X43" t="n">
-        <v>0.4978816535233578</v>
+        <v>1</v>
       </c>
       <c r="Y43" t="n">
+        <v>0.4712586814761995</v>
+      </c>
+      <c r="Z43" t="n">
         <v>1.53</v>
       </c>
-      <c r="Z43" t="inlineStr">
+      <c r="AA43" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
-      <c r="AA43" t="n">
-        <v>-0.4495114530363442</v>
-      </c>
       <c r="AB43" t="n">
-        <v>1.145127803103723</v>
+        <v>-0.52636644781399</v>
       </c>
       <c r="AC43" t="n">
-        <v>0.1701655201517661</v>
+        <v>1.225062051428347</v>
       </c>
       <c r="AD43" t="n">
-        <v>0</v>
+        <v>0.172886239766939</v>
       </c>
     </row>
     <row r="44">
@@ -4922,13 +4908,13 @@
         <v>1</v>
       </c>
       <c r="Q44" t="n">
-        <v>0.3555729649102405</v>
+        <v>0.3509223243843754</v>
       </c>
       <c r="R44" t="n">
-        <v>0.3615364290087321</v>
+        <v>0.408357020404592</v>
       </c>
       <c r="S44" t="n">
-        <v>0.2828906060810275</v>
+        <v>0.2407206552110326</v>
       </c>
       <c r="T44" t="n">
         <v>1</v>
@@ -4940,49 +4926,49 @@
         <v>0</v>
       </c>
       <c r="W44" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X44" t="n">
-        <v>0.3615364290087321</v>
+        <v>1</v>
       </c>
       <c r="Y44" t="n">
+        <v>0.408357020404592</v>
+      </c>
+      <c r="Z44" t="n">
         <v>2.05</v>
       </c>
-      <c r="Z44" t="inlineStr">
+      <c r="AA44" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
-      <c r="AA44" t="n">
-        <v>-0.2465241147924754</v>
-      </c>
       <c r="AB44" t="n">
-        <v>0.1663067573440168</v>
+        <v>-0.1551124839719872</v>
       </c>
       <c r="AC44" t="n">
-        <v>0.005963464098491633</v>
+        <v>1.318624059974202</v>
       </c>
       <c r="AD44" t="n">
-        <v>0</v>
+        <v>0.05743469602021656</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="1" t="inlineStr">
         <is>
-          <t>rVEQttsC</t>
+          <t>GrDYvKBO</t>
         </is>
       </c>
       <c r="B45" s="2" t="n">
-        <v>45746.66666666666</v>
+        <v>45747.66666666666</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>betis</t>
+          <t>celta vigo</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>sevilla</t>
+          <t>las palmas</t>
         </is>
       </c>
       <c r="E45" t="n">
@@ -5002,37 +4988,37 @@
         </is>
       </c>
       <c r="I45" t="n">
-        <v>2</v>
+        <v>1.57</v>
       </c>
       <c r="J45" t="n">
-        <v>3.4</v>
+        <v>4.1</v>
       </c>
       <c r="K45" t="n">
-        <v>3.75</v>
+        <v>5.5</v>
       </c>
       <c r="L45" t="n">
-        <v>0.4713493530499075</v>
+        <v>0.5993833395353783</v>
       </c>
       <c r="M45" t="n">
-        <v>0.2772643253234751</v>
+        <v>0.2295199617245229</v>
       </c>
       <c r="N45" t="n">
-        <v>0.2513863216266174</v>
+        <v>0.1710966987400989</v>
       </c>
       <c r="O45" t="n">
-        <v>0.0607843137254902</v>
+        <v>0.06266329600180764</v>
       </c>
       <c r="P45" t="n">
         <v>1</v>
       </c>
       <c r="Q45" t="n">
-        <v>0.355699083944977</v>
+        <v>0.3238104168751494</v>
       </c>
       <c r="R45" t="n">
-        <v>0.3657946219569925</v>
+        <v>0.4355011995646019</v>
       </c>
       <c r="S45" t="n">
-        <v>0.2785062940980305</v>
+        <v>0.2406883835602487</v>
       </c>
       <c r="T45" t="n">
         <v>1</v>
@@ -5044,49 +5030,49 @@
         <v>0</v>
       </c>
       <c r="W45" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X45" t="n">
-        <v>0.3657946219569925</v>
+        <v>1</v>
       </c>
       <c r="Y45" t="n">
-        <v>2</v>
-      </c>
-      <c r="Z45" t="inlineStr">
+        <v>0.4355011995646019</v>
+      </c>
+      <c r="Z45" t="n">
+        <v>1.57</v>
+      </c>
+      <c r="AA45" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
-      <c r="AA45" t="n">
-        <v>-0.2684107560860149</v>
-      </c>
       <c r="AB45" t="n">
-        <v>0.1682655261002166</v>
+        <v>-0.5548475731290788</v>
       </c>
       <c r="AC45" t="n">
-        <v>0.01009553801201551</v>
+        <v>1.111914379392914</v>
       </c>
       <c r="AD45" t="n">
-        <v>0</v>
+        <v>0.1116907826894525</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="1" t="inlineStr">
         <is>
-          <t>GrDYvKBO</t>
+          <t>rVEQttsC</t>
         </is>
       </c>
       <c r="B46" s="2" t="n">
-        <v>45747.66666666666</v>
+        <v>45746.66666666666</v>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>celta vigo</t>
+          <t>betis</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>las palmas</t>
+          <t>sevilla</t>
         </is>
       </c>
       <c r="E46" t="n">
@@ -5106,40 +5092,40 @@
         </is>
       </c>
       <c r="I46" t="n">
-        <v>1.57</v>
+        <v>2</v>
       </c>
       <c r="J46" t="n">
-        <v>4.1</v>
+        <v>3.4</v>
       </c>
       <c r="K46" t="n">
-        <v>5.5</v>
+        <v>3.75</v>
       </c>
       <c r="L46" t="n">
-        <v>0.5993833395353783</v>
+        <v>0.4713493530499075</v>
       </c>
       <c r="M46" t="n">
-        <v>0.2295199617245229</v>
+        <v>0.2772643253234751</v>
       </c>
       <c r="N46" t="n">
-        <v>0.1710966987400989</v>
+        <v>0.2513863216266174</v>
       </c>
       <c r="O46" t="n">
-        <v>0.06266329600180764</v>
+        <v>0.0607843137254902</v>
       </c>
       <c r="P46" t="n">
         <v>1</v>
       </c>
       <c r="Q46" t="n">
-        <v>0.3583583538094059</v>
+        <v>0.3731435205246508</v>
       </c>
       <c r="R46" t="n">
-        <v>0.3596472087554723</v>
+        <v>0.3529377592733988</v>
       </c>
       <c r="S46" t="n">
-        <v>0.2819944374351219</v>
+        <v>0.2739187202019505</v>
       </c>
       <c r="T46" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U46" t="n">
         <v>1</v>
@@ -5148,49 +5134,49 @@
         <v>0</v>
       </c>
       <c r="W46" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X46" t="n">
-        <v>0.3596472087554723</v>
+        <v>0</v>
       </c>
       <c r="Y46" t="n">
-        <v>1.57</v>
-      </c>
-      <c r="Z46" t="inlineStr">
+        <v>0.3731435205246508</v>
+      </c>
+      <c r="Z46" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="AA46" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
-      <c r="AA46" t="n">
-        <v>-0.7637787407963306</v>
-      </c>
       <c r="AB46" t="n">
-        <v>0.1654377160275173</v>
+        <v>0.1119533207432553</v>
       </c>
       <c r="AC46" t="n">
-        <v>0.001288854946066398</v>
+        <v>8.489015091935805</v>
       </c>
       <c r="AD46" t="n">
-        <v>0</v>
+        <v>0.02020576125125195</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="1" t="inlineStr">
         <is>
-          <t>Olz0eud5</t>
+          <t>Kjbn1lFr</t>
         </is>
       </c>
       <c r="B47" s="2" t="n">
-        <v>45745.60416666666</v>
+        <v>45745.51041666666</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>alaves</t>
+          <t>espanyol</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>rayo vallecano</t>
+          <t>atl  madrid</t>
         </is>
       </c>
       <c r="E47" t="n">
@@ -5210,40 +5196,40 @@
         </is>
       </c>
       <c r="I47" t="n">
-        <v>2.25</v>
+        <v>7</v>
       </c>
       <c r="J47" t="n">
-        <v>2.9</v>
+        <v>4</v>
       </c>
       <c r="K47" t="n">
-        <v>3.6</v>
+        <v>1.5</v>
       </c>
       <c r="L47" t="n">
-        <v>0.4165170556552962</v>
+        <v>0.1348314606741573</v>
       </c>
       <c r="M47" t="n">
-        <v>0.3231597845601437</v>
+        <v>0.2359550561797753</v>
       </c>
       <c r="N47" t="n">
-        <v>0.2603231597845602</v>
+        <v>0.6292134831460674</v>
       </c>
       <c r="O47" t="n">
-        <v>0.06704980842911867</v>
+        <v>0.05952380952380953</v>
       </c>
       <c r="P47" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q47" t="n">
-        <v>0.3849332791811567</v>
+        <v>0.2499405592723154</v>
       </c>
       <c r="R47" t="n">
-        <v>0.3289894957515934</v>
+        <v>0.1194316176183696</v>
       </c>
       <c r="S47" t="n">
-        <v>0.2860772250672497</v>
+        <v>0.630627823109315</v>
       </c>
       <c r="T47" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="U47" t="n">
         <v>1</v>
@@ -5255,46 +5241,46 @@
         <v>0</v>
       </c>
       <c r="X47" t="n">
-        <v>0.3849332791811567</v>
+        <v>2</v>
       </c>
       <c r="Y47" t="n">
-        <v>2.9</v>
-      </c>
-      <c r="Z47" t="inlineStr">
+        <v>0.630627823109315</v>
+      </c>
+      <c r="Z47" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="AA47" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
-      <c r="AA47" t="n">
-        <v>0.0612139524343971</v>
-      </c>
       <c r="AB47" t="n">
-        <v>7.082772336933283</v>
+        <v>-0.1081165306720551</v>
       </c>
       <c r="AC47" t="n">
-        <v>0.0559437834295633</v>
+        <v>2.087996210306274</v>
       </c>
       <c r="AD47" t="n">
-        <v>0</v>
+        <v>0.3806872638369996</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="1" t="inlineStr">
         <is>
-          <t>f9rqaNdt</t>
+          <t>Olz0eud5</t>
         </is>
       </c>
       <c r="B48" s="2" t="n">
-        <v>45746.375</v>
+        <v>45745.60416666666</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>getafe</t>
+          <t>alaves</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>villarreal</t>
+          <t>rayo vallecano</t>
         </is>
       </c>
       <c r="E48" t="n">
@@ -5314,40 +5300,40 @@
         </is>
       </c>
       <c r="I48" t="n">
-        <v>3.1</v>
+        <v>2.25</v>
       </c>
       <c r="J48" t="n">
-        <v>3.2</v>
+        <v>2.9</v>
       </c>
       <c r="K48" t="n">
-        <v>2.35</v>
+        <v>3.6</v>
       </c>
       <c r="L48" t="n">
-        <v>0.3041456016177958</v>
+        <v>0.4165170556552962</v>
       </c>
       <c r="M48" t="n">
-        <v>0.2946410515672397</v>
+        <v>0.3231597845601437</v>
       </c>
       <c r="N48" t="n">
-        <v>0.4012133468149647</v>
+        <v>0.2603231597845602</v>
       </c>
       <c r="O48" t="n">
-        <v>0.06061256005490723</v>
+        <v>0.06704980842911867</v>
       </c>
       <c r="P48" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q48" t="n">
+        <v>0.3459467307060448</v>
+      </c>
+      <c r="R48" t="n">
+        <v>0.2803719958462909</v>
+      </c>
+      <c r="S48" t="n">
+        <v>0.3736812734476644</v>
+      </c>
+      <c r="T48" t="n">
         <v>2</v>
-      </c>
-      <c r="Q48" t="n">
-        <v>0.3914287759434801</v>
-      </c>
-      <c r="R48" t="n">
-        <v>0.220564522223485</v>
-      </c>
-      <c r="S48" t="n">
-        <v>0.388006701833035</v>
-      </c>
-      <c r="T48" t="n">
-        <v>0</v>
       </c>
       <c r="U48" t="n">
         <v>1</v>
@@ -5359,46 +5345,46 @@
         <v>0</v>
       </c>
       <c r="X48" t="n">
-        <v>0.3914287759434801</v>
+        <v>2</v>
       </c>
       <c r="Y48" t="n">
-        <v>3.2</v>
-      </c>
-      <c r="Z48" t="inlineStr">
+        <v>0.3736812734476644</v>
+      </c>
+      <c r="Z48" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="AA48" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
-      <c r="AA48" t="n">
-        <v>0.1148054922814256</v>
-      </c>
       <c r="AB48" t="n">
-        <v>7.202289477360034</v>
+        <v>0.13278945554292</v>
       </c>
       <c r="AC48" t="n">
-        <v>0.003422074110445095</v>
+        <v>1.307884457066825</v>
       </c>
       <c r="AD48" t="n">
-        <v>0</v>
+        <v>0.02773454274161957</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="1" t="inlineStr">
         <is>
-          <t>Kjbn1lFr</t>
+          <t>f9rqaNdt</t>
         </is>
       </c>
       <c r="B49" s="2" t="n">
-        <v>45745.51041666666</v>
+        <v>45746.375</v>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>espanyol</t>
+          <t>getafe</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>atl  madrid</t>
+          <t>villarreal</t>
         </is>
       </c>
       <c r="E49" t="n">
@@ -5418,37 +5404,37 @@
         </is>
       </c>
       <c r="I49" t="n">
-        <v>7</v>
+        <v>3.1</v>
       </c>
       <c r="J49" t="n">
-        <v>4</v>
+        <v>3.2</v>
       </c>
       <c r="K49" t="n">
-        <v>1.5</v>
+        <v>2.35</v>
       </c>
       <c r="L49" t="n">
-        <v>0.1348314606741573</v>
+        <v>0.3041456016177958</v>
       </c>
       <c r="M49" t="n">
-        <v>0.2359550561797753</v>
+        <v>0.2946410515672397</v>
       </c>
       <c r="N49" t="n">
-        <v>0.6292134831460674</v>
+        <v>0.4012133468149647</v>
       </c>
       <c r="O49" t="n">
-        <v>0.05952380952380953</v>
+        <v>0.06061256005490723</v>
       </c>
       <c r="P49" t="n">
         <v>2</v>
       </c>
       <c r="Q49" t="n">
-        <v>0.3544226986660331</v>
+        <v>0.344081963617453</v>
       </c>
       <c r="R49" t="n">
-        <v>0.1183270127597769</v>
+        <v>0.2816581465830766</v>
       </c>
       <c r="S49" t="n">
-        <v>0.52725028857419</v>
+        <v>0.3742598897994704</v>
       </c>
       <c r="T49" t="n">
         <v>2</v>
@@ -5460,30 +5446,30 @@
         <v>0</v>
       </c>
       <c r="W49" t="n">
+        <v>0</v>
+      </c>
+      <c r="X49" t="n">
         <v>2</v>
       </c>
-      <c r="X49" t="n">
-        <v>0.52725028857419</v>
-      </c>
       <c r="Y49" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="Z49" t="inlineStr">
+        <v>0.3742598897994704</v>
+      </c>
+      <c r="Z49" t="n">
+        <v>2.35</v>
+      </c>
+      <c r="AA49" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
-      <c r="AA49" t="n">
-        <v>-0.41824913427743</v>
-      </c>
       <c r="AB49" t="n">
-        <v>1.212675663720637</v>
+        <v>-0.0892513029416626</v>
       </c>
       <c r="AC49" t="n">
-        <v>0.1728275899081569</v>
+        <v>1.251492817264384</v>
       </c>
       <c r="AD49" t="n">
-        <v>0</v>
+        <v>0.03017792618201742</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
DATA. Actualizo preds. Sin kelly_linear.
</commit_message>
<xml_diff>
--- a/data/predicciones.xlsx
+++ b/data/predicciones.xlsx
@@ -678,7 +678,7 @@
         <v>-0.2442105936350345</v>
       </c>
       <c r="AC2" t="n">
-        <v>1.905801074789221</v>
+        <v>1.859473622501219</v>
       </c>
       <c r="AD2" t="n">
         <v>0.3165899484765903</v>
@@ -778,7 +778,7 @@
         <v>-1.046102482240357</v>
       </c>
       <c r="AC3" t="n">
-        <v>0.8341773619015219</v>
+        <v>1.375153911162069</v>
       </c>
       <c r="AD3" t="n">
         <v>0.08603436499585954</v>
@@ -878,7 +878,7 @@
         <v>-0.3106184565830246</v>
       </c>
       <c r="AC4" t="n">
-        <v>1.020542000984441</v>
+        <v>1.034072315125463</v>
       </c>
       <c r="AD4" t="n">
         <v>0.01634216979090458</v>
@@ -978,7 +978,7 @@
         <v>-0.7992418447129908</v>
       </c>
       <c r="AC5" t="n">
-        <v>1.603671091726641</v>
+        <v>2.215715093330235</v>
       </c>
       <c r="AD5" t="n">
         <v>0.522882665824842</v>
@@ -1082,7 +1082,7 @@
         <v>-0.3683114005233427</v>
       </c>
       <c r="AC6" t="n">
-        <v>1.291157522755282</v>
+        <v>1.353110230507833</v>
       </c>
       <c r="AD6" t="n">
         <v>0.06848965329455309</v>
@@ -1182,7 +1182,7 @@
         <v>-0.2584221539355691</v>
       </c>
       <c r="AC7" t="n">
-        <v>1.953542342957054</v>
+        <v>1.921352439483798</v>
       </c>
       <c r="AD7" t="n">
         <v>0.3572509280354617</v>
@@ -1282,7 +1282,7 @@
         <v>0.1153214613242233</v>
       </c>
       <c r="AC8" t="n">
-        <v>4.025761603327271</v>
+        <v>3.450652802851947</v>
       </c>
       <c r="AD8" t="n">
         <v>0.0663563345590133</v>
@@ -1382,7 +1382,7 @@
         <v>0.1225354060165768</v>
       </c>
       <c r="AC9" t="n">
-        <v>3.845893495625708</v>
+        <v>3.29648013910775</v>
       </c>
       <c r="AD9" t="n">
         <v>0.008866310429457624</v>
@@ -1486,7 +1486,7 @@
         <v>-0.5307611324034121</v>
       </c>
       <c r="AC10" t="n">
-        <v>1.07364054753249</v>
+        <v>1.24245944057386</v>
       </c>
       <c r="AD10" t="n">
         <v>0.008640121923820576</v>
@@ -1590,7 +1590,7 @@
         <v>-0.3371590190209028</v>
       </c>
       <c r="AC11" t="n">
-        <v>3.111797646121697</v>
+        <v>3.201988867432812</v>
       </c>
       <c r="AD11" t="n">
         <v>0.04640017163373084</v>
@@ -1690,7 +1690,7 @@
         <v>-0.1701753913075543</v>
       </c>
       <c r="AC12" t="n">
-        <v>3.442443717761873</v>
+        <v>3.224359147145475</v>
       </c>
       <c r="AD12" t="n">
         <v>0.05416883627144609</v>
@@ -1794,7 +1794,7 @@
         <v>0.2498496431996034</v>
       </c>
       <c r="AC13" t="n">
-        <v>2.348102567114255</v>
+        <v>2.01265934324079</v>
       </c>
       <c r="AD13" t="n">
         <v>0.1397902611246557</v>
@@ -1898,7 +1898,7 @@
         <v>0.1543697493194137</v>
       </c>
       <c r="AC14" t="n">
-        <v>7.867518020441678</v>
+        <v>6.743586874664296</v>
       </c>
       <c r="AD14" t="n">
         <v>0.1626140570031305</v>
@@ -2002,7 +2002,7 @@
         <v>0.189947102426807</v>
       </c>
       <c r="AC15" t="n">
-        <v>10.96562507370833</v>
+        <v>9.39910720603571</v>
       </c>
       <c r="AD15" t="n">
         <v>0.4994895281646305</v>
@@ -2102,7 +2102,7 @@
         <v>-1.086741475219048</v>
       </c>
       <c r="AC16" t="n">
-        <v>5.909200568288616</v>
+        <v>10.04040229108421</v>
       </c>
       <c r="AD16" t="n">
         <v>0.5082737384465691</v>
@@ -2206,7 +2206,7 @@
         <v>0.2614853905117354</v>
       </c>
       <c r="AC17" t="n">
-        <v>6.955371754081825</v>
+        <v>5.961747217784422</v>
       </c>
       <c r="AD17" t="n">
         <v>0.1358031559651239</v>
@@ -2306,7 +2306,7 @@
         <v>-0.03904035478434289</v>
       </c>
       <c r="AC18" t="n">
-        <v>7.797890791673002</v>
+        <v>6.816957718049396</v>
       </c>
       <c r="AD18" t="n">
         <v>0.1352050210341218</v>
@@ -2410,7 +2410,7 @@
         <v>-0.0407300317562943</v>
       </c>
       <c r="AC19" t="n">
-        <v>5.668713731969236</v>
+        <v>4.959891798235113</v>
       </c>
       <c r="AD19" t="n">
         <v>0.03977136943544807</v>
@@ -2510,7 +2510,7 @@
         <v>-0.02284000144402813</v>
       </c>
       <c r="AC20" t="n">
-        <v>2.707633393631191</v>
+        <v>2.347637479393966</v>
       </c>
       <c r="AD20" t="n">
         <v>0.6113133678474076</v>
@@ -2610,7 +2610,7 @@
         <v>0.1909744195833094</v>
       </c>
       <c r="AC21" t="n">
-        <v>3.152260934733177</v>
+        <v>2.701937944057009</v>
       </c>
       <c r="AD21" t="n">
         <v>0.8256672270830573</v>
@@ -2710,7 +2710,7 @@
         <v>0.1455039670734701</v>
       </c>
       <c r="AC22" t="n">
-        <v>1.781917550817935</v>
+        <v>1.527357900701087</v>
       </c>
       <c r="AD22" t="n">
         <v>0.2049859611591311</v>
@@ -2810,7 +2810,7 @@
         <v>-0.1744472087845206</v>
       </c>
       <c r="AC23" t="n">
-        <v>1.717060917236152</v>
+        <v>1.612016935072839</v>
       </c>
       <c r="AD23" t="n">
         <v>0.2473442706888411</v>
@@ -2914,7 +2914,7 @@
         <v>-0.1866124893064383</v>
       </c>
       <c r="AC24" t="n">
-        <v>1.290997502378281</v>
+        <v>1.220081266040342</v>
       </c>
       <c r="AD24" t="n">
         <v>0.03813939040308317</v>
@@ -3014,7 +3014,7 @@
         <v>0.3197182078221008</v>
       </c>
       <c r="AC25" t="n">
-        <v>2.519593887743615</v>
+        <v>2.159651903780242</v>
       </c>
       <c r="AD25" t="n">
         <v>0.5506784616981166</v>
@@ -3114,7 +3114,7 @@
         <v>0.2602713994210298</v>
       </c>
       <c r="AC26" t="n">
-        <v>7.165254924859846</v>
+        <v>6.141647078451297</v>
       </c>
       <c r="AD26" t="n">
         <v>0.09499876507328531</v>
@@ -3214,7 +3214,7 @@
         <v>0.1989442271565266</v>
       </c>
       <c r="AC27" t="n">
-        <v>6.497805823657882</v>
+        <v>5.569547848849614</v>
       </c>
       <c r="AD27" t="n">
         <v>0.09581271511068973</v>
@@ -3314,7 +3314,7 @@
         <v>-0.05438966060929866</v>
       </c>
       <c r="AC28" t="n">
-        <v>4.936332069980979</v>
+        <v>4.349393646445758</v>
       </c>
       <c r="AD28" t="n">
         <v>0.0509843071978795</v>
@@ -3414,7 +3414,7 @@
         <v>0.07394378153454376</v>
       </c>
       <c r="AC29" t="n">
-        <v>2.132327376775005</v>
+        <v>1.827709180092862</v>
       </c>
       <c r="AD29" t="n">
         <v>0.3279189310629804</v>
@@ -3514,7 +3514,7 @@
         <v>-0.1450756947532118</v>
       </c>
       <c r="AC30" t="n">
-        <v>1.927428009713883</v>
+        <v>1.781048453972387</v>
       </c>
       <c r="AD30" t="n">
         <v>0.2890948059640486</v>
@@ -3614,7 +3614,7 @@
         <v>-0.3570114524737107</v>
       </c>
       <c r="AC31" t="n">
-        <v>1.312854347869637</v>
+        <v>1.366710766783139</v>
       </c>
       <c r="AD31" t="n">
         <v>0.032470168263524</v>
@@ -3714,7 +3714,7 @@
         <v>-0.1063247283516979</v>
       </c>
       <c r="AC32" t="n">
-        <v>2.229655482699205</v>
+        <v>2.018331579068212</v>
       </c>
       <c r="AD32" t="n">
         <v>0.3988900842851951</v>
@@ -3818,7 +3818,7 @@
         <v>-0.333777837367836</v>
       </c>
       <c r="AC33" t="n">
-        <v>1.07563562243901</v>
+        <v>1.104631494266759</v>
       </c>
       <c r="AD33" t="n">
         <v>0.02632416652920944</v>
@@ -3918,7 +3918,7 @@
         <v>0.1560115223962476</v>
       </c>
       <c r="AC34" t="n">
-        <v>9.196537977304446</v>
+        <v>7.882746837689526</v>
       </c>
       <c r="AD34" t="n">
         <v>0.03539538923291191</v>
@@ -4018,7 +4018,7 @@
         <v>0.07961794707855407</v>
       </c>
       <c r="AC35" t="n">
-        <v>8.565724974734813</v>
+        <v>7.342049978344125</v>
       </c>
       <c r="AD35" t="n">
         <v>0.04439633633870788</v>
@@ -4118,7 +4118,7 @@
         <v>0.2742297835463348</v>
       </c>
       <c r="AC36" t="n">
-        <v>11.24214346183696</v>
+        <v>9.636122967288824</v>
       </c>
       <c r="AD36" t="n">
         <v>0.1141177850734852</v>
@@ -4222,7 +4222,7 @@
         <v>0.2487232710269768</v>
       </c>
       <c r="AC37" t="n">
-        <v>9.229598037887142</v>
+        <v>7.911084032474693</v>
       </c>
       <c r="AD37" t="n">
         <v>0.4204796570220136</v>
@@ -4322,7 +4322,7 @@
         <v>0.01819466117218543</v>
       </c>
       <c r="AC38" t="n">
-        <v>7.684603496188651</v>
+        <v>6.58680299673313</v>
       </c>
       <c r="AD38" t="n">
         <v>0.2162498241274949</v>
@@ -4426,7 +4426,7 @@
         <v>-0.6348749528740398</v>
       </c>
       <c r="AC39" t="n">
-        <v>1.533639664385265</v>
+        <v>1.897409915503554</v>
       </c>
       <c r="AD39" t="n">
         <v>0.3757919717931897</v>
@@ -4530,7 +4530,7 @@
         <v>-0.6883050837844672</v>
       </c>
       <c r="AC40" t="n">
-        <v>1.360273986361305</v>
+        <v>1.743291704551411</v>
       </c>
       <c r="AD40" t="n">
         <v>0.3013877373646283</v>
@@ -4634,7 +4634,7 @@
         <v>-0.8585385463965146</v>
       </c>
       <c r="AC41" t="n">
-        <v>1.492825121072358</v>
+        <v>2.149482360123629</v>
       </c>
       <c r="AD41" t="n">
         <v>0.4932402087549221</v>
@@ -4738,7 +4738,7 @@
         <v>-0.6957469038567523</v>
       </c>
       <c r="AC42" t="n">
-        <v>1.489551077907825</v>
+        <v>1.918460636122858</v>
       </c>
       <c r="AD42" t="n">
         <v>0.3930091235643412</v>
@@ -4842,7 +4842,7 @@
         <v>-0.52636644781399</v>
       </c>
       <c r="AC43" t="n">
-        <v>1.225062051428347</v>
+        <v>1.413776044428599</v>
       </c>
       <c r="AD43" t="n">
         <v>0.172886239766939</v>
@@ -4946,7 +4946,7 @@
         <v>-0.1551124839719872</v>
       </c>
       <c r="AC44" t="n">
-        <v>1.318624059974202</v>
+        <v>1.225071061213776</v>
       </c>
       <c r="AD44" t="n">
         <v>0.05743469602021656</v>
@@ -5050,7 +5050,7 @@
         <v>-0.5548475731290788</v>
       </c>
       <c r="AC45" t="n">
-        <v>1.111914379392914</v>
+        <v>1.306503598693806</v>
       </c>
       <c r="AD45" t="n">
         <v>0.1116907826894525</v>
@@ -5154,7 +5154,7 @@
         <v>0.1119533207432553</v>
       </c>
       <c r="AC46" t="n">
-        <v>8.489015091935805</v>
+        <v>7.276298650230689</v>
       </c>
       <c r="AD46" t="n">
         <v>0.02020576125125195</v>
@@ -5258,7 +5258,7 @@
         <v>-0.1081165306720551</v>
       </c>
       <c r="AC47" t="n">
-        <v>2.087996210306274</v>
+        <v>1.891883469327945</v>
       </c>
       <c r="AD47" t="n">
         <v>0.3806872638369996</v>
@@ -5362,7 +5362,7 @@
         <v>0.13278945554292</v>
       </c>
       <c r="AC48" t="n">
-        <v>1.307884457066825</v>
+        <v>1.121043820342993</v>
       </c>
       <c r="AD48" t="n">
         <v>0.02773454274161957</v>
@@ -5466,7 +5466,7 @@
         <v>-0.0892513029416626</v>
       </c>
       <c r="AC49" t="n">
-        <v>1.251492817264384</v>
+        <v>1.122779669398411</v>
       </c>
       <c r="AD49" t="n">
         <v>0.03017792618201742</v>

</xml_diff>

<commit_message>
DATA. Actualizo preds x cambio de modelos (x cambio en metricas)
</commit_message>
<xml_diff>
--- a/data/predicciones.xlsx
+++ b/data/predicciones.xlsx
@@ -540,47 +540,47 @@
       </c>
       <c r="V1" s="1" t="inlineStr">
         <is>
+          <t>player_emergency_fill</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>result_to_bet</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>prob_result_to_bet</t>
+        </is>
+      </c>
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
+          <t>odd_to_bet</t>
+        </is>
+      </c>
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
+          <t>strategy</t>
+        </is>
+      </c>
+      <c r="AA1" s="1" t="inlineStr">
+        <is>
+          <t>kelly_criterion</t>
+        </is>
+      </c>
+      <c r="AB1" s="1" t="inlineStr">
+        <is>
+          <t>stake_to_bet</t>
+        </is>
+      </c>
+      <c r="AC1" s="1" t="inlineStr">
+        <is>
+          <t>confidence_margin</t>
+        </is>
+      </c>
+      <c r="AD1" s="1" t="inlineStr">
+        <is>
           <t>emergency_fill</t>
-        </is>
-      </c>
-      <c r="W1" s="1" t="inlineStr">
-        <is>
-          <t>player_emergency_fill</t>
-        </is>
-      </c>
-      <c r="X1" s="1" t="inlineStr">
-        <is>
-          <t>result_to_bet</t>
-        </is>
-      </c>
-      <c r="Y1" s="1" t="inlineStr">
-        <is>
-          <t>prob_result_to_bet</t>
-        </is>
-      </c>
-      <c r="Z1" s="1" t="inlineStr">
-        <is>
-          <t>odd_to_bet</t>
-        </is>
-      </c>
-      <c r="AA1" s="1" t="inlineStr">
-        <is>
-          <t>strategy</t>
-        </is>
-      </c>
-      <c r="AB1" s="1" t="inlineStr">
-        <is>
-          <t>kelly_criterion</t>
-        </is>
-      </c>
-      <c r="AC1" s="1" t="inlineStr">
-        <is>
-          <t>stake_to_bet</t>
-        </is>
-      </c>
-      <c r="AD1" s="1" t="inlineStr">
-        <is>
-          <t>confidence_margin</t>
         </is>
       </c>
     </row>
@@ -644,13 +644,13 @@
         <v>1</v>
       </c>
       <c r="Q2" t="n">
-        <v>0.3032345923571492</v>
+        <v>0.3130628854580313</v>
       </c>
       <c r="R2" t="n">
-        <v>0.6198245408337395</v>
+        <v>0.5735642917377995</v>
       </c>
       <c r="S2" t="n">
-        <v>0.07694086680911141</v>
+        <v>0.1133728228041693</v>
       </c>
       <c r="T2" t="n">
         <v>1</v>
@@ -658,49 +658,51 @@
       <c r="U2" t="n">
         <v>1</v>
       </c>
-      <c r="V2" t="inlineStr"/>
-      <c r="W2" t="inlineStr"/>
+      <c r="V2" t="n">
+        <v>0</v>
+      </c>
+      <c r="W2" t="n">
+        <v>1</v>
+      </c>
       <c r="X2" t="n">
-        <v>1</v>
+        <v>0.5735642917377995</v>
       </c>
       <c r="Y2" t="n">
-        <v>0.6198245408337395</v>
-      </c>
-      <c r="Z2" t="n">
         <v>1.44</v>
       </c>
-      <c r="AA2" t="inlineStr">
+      <c r="Z2" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
+      <c r="AA2" t="n">
+        <v>-0.3956077724944743</v>
+      </c>
       <c r="AB2" t="n">
-        <v>-0.2442105936350345</v>
+        <v>1.384703762016951</v>
       </c>
       <c r="AC2" t="n">
-        <v>1.859473622501219</v>
-      </c>
-      <c r="AD2" t="n">
-        <v>0.3165899484765903</v>
-      </c>
+        <v>0.2605014062797683</v>
+      </c>
+      <c r="AD2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>6Dg5Psv0</t>
+          <t>QHQVu3Ot</t>
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>45749.65625</v>
+        <v>45748.66666666666</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>bournemouth</t>
+          <t>nottingham</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>ipswich</t>
+          <t>manchester utd</t>
         </is>
       </c>
       <c r="E3" t="n">
@@ -720,37 +722,37 @@
         </is>
       </c>
       <c r="I3" t="n">
-        <v>1.36</v>
+        <v>2.1</v>
       </c>
       <c r="J3" t="n">
-        <v>4.75</v>
+        <v>3.6</v>
       </c>
       <c r="K3" t="n">
-        <v>8</v>
+        <v>3.2</v>
       </c>
       <c r="L3" t="n">
-        <v>0.6866642573183954</v>
+        <v>0.4465116279069767</v>
       </c>
       <c r="M3" t="n">
-        <v>0.1966028189374774</v>
+        <v>0.2604651162790698</v>
       </c>
       <c r="N3" t="n">
-        <v>0.1167329237441272</v>
+        <v>0.2930232558139535</v>
       </c>
       <c r="O3" t="n">
-        <v>0.07082043343653233</v>
+        <v>0.06646825396825395</v>
       </c>
       <c r="P3" t="n">
         <v>1</v>
       </c>
       <c r="Q3" t="n">
-        <v>0.3723502720581635</v>
+        <v>0.3537118703380377</v>
       </c>
       <c r="R3" t="n">
-        <v>0.458384637054023</v>
+        <v>0.3663571231487831</v>
       </c>
       <c r="S3" t="n">
-        <v>0.1692650908878135</v>
+        <v>0.2799310065131793</v>
       </c>
       <c r="T3" t="n">
         <v>1</v>
@@ -758,36 +760,38 @@
       <c r="U3" t="n">
         <v>1</v>
       </c>
-      <c r="V3" t="inlineStr"/>
-      <c r="W3" t="inlineStr"/>
+      <c r="V3" t="n">
+        <v>0</v>
+      </c>
+      <c r="W3" t="n">
+        <v>1</v>
+      </c>
       <c r="X3" t="n">
-        <v>1</v>
+        <v>0.3663571231487831</v>
       </c>
       <c r="Y3" t="n">
-        <v>0.458384637054023</v>
-      </c>
-      <c r="Z3" t="n">
-        <v>1.36</v>
-      </c>
-      <c r="AA3" t="inlineStr">
+        <v>2.1</v>
+      </c>
+      <c r="Z3" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
+      <c r="AA3" t="n">
+        <v>-0.2096818558068686</v>
+      </c>
       <c r="AB3" t="n">
-        <v>-1.046102482240357</v>
+        <v>0.1968528077706222</v>
       </c>
       <c r="AC3" t="n">
-        <v>1.375153911162069</v>
-      </c>
-      <c r="AD3" t="n">
-        <v>0.08603436499585954</v>
-      </c>
+        <v>0.01264525281074536</v>
+      </c>
+      <c r="AD3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>zgoMLawP</t>
+          <t>6Dg5Psv0</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
@@ -795,12 +799,12 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>brighton</t>
+          <t>bournemouth</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>aston villa</t>
+          <t>ipswich</t>
         </is>
       </c>
       <c r="E4" t="n">
@@ -820,37 +824,37 @@
         </is>
       </c>
       <c r="I4" t="n">
-        <v>2</v>
+        <v>1.36</v>
       </c>
       <c r="J4" t="n">
-        <v>4</v>
+        <v>4.75</v>
       </c>
       <c r="K4" t="n">
-        <v>3.2</v>
+        <v>8</v>
       </c>
       <c r="L4" t="n">
-        <v>0.4705882352941176</v>
+        <v>0.6866642573183954</v>
       </c>
       <c r="M4" t="n">
-        <v>0.2352941176470588</v>
+        <v>0.1966028189374774</v>
       </c>
       <c r="N4" t="n">
-        <v>0.2941176470588235</v>
+        <v>0.1167329237441272</v>
       </c>
       <c r="O4" t="n">
-        <v>0.0625</v>
+        <v>0.07082043343653233</v>
       </c>
       <c r="P4" t="n">
         <v>1</v>
       </c>
       <c r="Q4" t="n">
-        <v>0.3283486019175831</v>
+        <v>0.3018209036334504</v>
       </c>
       <c r="R4" t="n">
-        <v>0.3446907717084877</v>
+        <v>0.5519929205215001</v>
       </c>
       <c r="S4" t="n">
-        <v>0.3269606263739293</v>
+        <v>0.1461861758450495</v>
       </c>
       <c r="T4" t="n">
         <v>1</v>
@@ -858,31 +862,33 @@
       <c r="U4" t="n">
         <v>1</v>
       </c>
-      <c r="V4" t="inlineStr"/>
-      <c r="W4" t="inlineStr"/>
+      <c r="V4" t="n">
+        <v>0</v>
+      </c>
+      <c r="W4" t="n">
+        <v>1</v>
+      </c>
       <c r="X4" t="n">
-        <v>1</v>
+        <v>0.5519929205215001</v>
       </c>
       <c r="Y4" t="n">
-        <v>0.3446907717084877</v>
-      </c>
-      <c r="Z4" t="n">
-        <v>2</v>
-      </c>
-      <c r="AA4" t="inlineStr">
+        <v>1.36</v>
+      </c>
+      <c r="Z4" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
+      <c r="AA4" t="n">
+        <v>-0.6924711891409994</v>
+      </c>
       <c r="AB4" t="n">
-        <v>-0.3106184565830246</v>
+        <v>1.104483420387402</v>
       </c>
       <c r="AC4" t="n">
-        <v>1.034072315125463</v>
-      </c>
-      <c r="AD4" t="n">
-        <v>0.01634216979090458</v>
-      </c>
+        <v>0.2501720168880496</v>
+      </c>
+      <c r="AD4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
@@ -944,13 +950,13 @@
         <v>1</v>
       </c>
       <c r="Q5" t="n">
-        <v>0.215689031951903</v>
+        <v>0.2506041182162601</v>
       </c>
       <c r="R5" t="n">
-        <v>0.738571697776745</v>
+        <v>0.6933896141043031</v>
       </c>
       <c r="S5" t="n">
-        <v>0.04573927027135195</v>
+        <v>0.05600626767943685</v>
       </c>
       <c r="T5" t="n">
         <v>1</v>
@@ -958,31 +964,33 @@
       <c r="U5" t="n">
         <v>1</v>
       </c>
-      <c r="V5" t="inlineStr"/>
-      <c r="W5" t="inlineStr"/>
+      <c r="V5" t="n">
+        <v>0</v>
+      </c>
+      <c r="W5" t="n">
+        <v>1</v>
+      </c>
       <c r="X5" t="n">
-        <v>1</v>
+        <v>0.6933896141043031</v>
       </c>
       <c r="Y5" t="n">
-        <v>0.738571697776745</v>
-      </c>
-      <c r="Z5" t="n">
         <v>1.17</v>
       </c>
-      <c r="AA5" t="inlineStr">
+      <c r="Z5" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
+      <c r="AA5" t="n">
+        <v>-1.110200891164503</v>
+      </c>
       <c r="AB5" t="n">
-        <v>-0.7992418447129908</v>
+        <v>1.03107079218174</v>
       </c>
       <c r="AC5" t="n">
-        <v>2.215715093330235</v>
-      </c>
-      <c r="AD5" t="n">
-        <v>0.522882665824842</v>
-      </c>
+        <v>0.442785495888043</v>
+      </c>
+      <c r="AD5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
@@ -1044,13 +1052,13 @@
         <v>1</v>
       </c>
       <c r="Q6" t="n">
-        <v>0.382547090208058</v>
+        <v>0.2881228350102186</v>
       </c>
       <c r="R6" t="n">
-        <v>0.4510367435026111</v>
+        <v>0.5972965392402477</v>
       </c>
       <c r="S6" t="n">
-        <v>0.1664161662893308</v>
+        <v>0.1145806257495336</v>
       </c>
       <c r="T6" t="n">
         <v>1</v>
@@ -1059,34 +1067,32 @@
         <v>1</v>
       </c>
       <c r="V6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="W6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X6" t="n">
-        <v>1</v>
+        <v>0.5972965392402477</v>
       </c>
       <c r="Y6" t="n">
-        <v>0.4510367435026111</v>
-      </c>
-      <c r="Z6" t="n">
         <v>1.67</v>
       </c>
-      <c r="AA6" t="inlineStr">
+      <c r="Z6" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
+      <c r="AA6" t="n">
+        <v>-0.003753402192218457</v>
+      </c>
       <c r="AB6" t="n">
-        <v>-0.3683114005233427</v>
+        <v>1.788526780459037</v>
       </c>
       <c r="AC6" t="n">
-        <v>1.353110230507833</v>
-      </c>
-      <c r="AD6" t="n">
-        <v>0.06848965329455309</v>
-      </c>
+        <v>0.3091737042300292</v>
+      </c>
+      <c r="AD6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
@@ -1148,13 +1154,13 @@
         <v>1</v>
       </c>
       <c r="Q7" t="n">
-        <v>0.2831998851258044</v>
+        <v>0.3139090504681026</v>
       </c>
       <c r="R7" t="n">
-        <v>0.6404508131612661</v>
+        <v>0.5884761484566114</v>
       </c>
       <c r="S7" t="n">
-        <v>0.0763493017129296</v>
+        <v>0.09761480107528593</v>
       </c>
       <c r="T7" t="n">
         <v>1</v>
@@ -1162,31 +1168,33 @@
       <c r="U7" t="n">
         <v>1</v>
       </c>
-      <c r="V7" t="inlineStr"/>
-      <c r="W7" t="inlineStr"/>
+      <c r="V7" t="n">
+        <v>0</v>
+      </c>
+      <c r="W7" t="n">
+        <v>1</v>
+      </c>
       <c r="X7" t="n">
-        <v>1</v>
+        <v>0.5884761484566114</v>
       </c>
       <c r="Y7" t="n">
-        <v>0.6404508131612661</v>
-      </c>
-      <c r="Z7" t="n">
         <v>1.4</v>
       </c>
-      <c r="AA7" t="inlineStr">
+      <c r="Z7" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
+      <c r="AA7" t="n">
+        <v>-0.4403334804018602</v>
+      </c>
       <c r="AB7" t="n">
-        <v>-0.2584221539355691</v>
+        <v>1.382900742899112</v>
       </c>
       <c r="AC7" t="n">
-        <v>1.921352439483798</v>
-      </c>
-      <c r="AD7" t="n">
-        <v>0.3572509280354617</v>
-      </c>
+        <v>0.2745670979885088</v>
+      </c>
+      <c r="AD7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
@@ -1248,63 +1256,65 @@
         <v>1</v>
       </c>
       <c r="Q8" t="n">
-        <v>0.3834058669835496</v>
+        <v>0.3515991343759853</v>
       </c>
       <c r="R8" t="n">
-        <v>0.2995446005919141</v>
+        <v>0.2858203998914456</v>
       </c>
       <c r="S8" t="n">
-        <v>0.3170495324245363</v>
+        <v>0.3625804657325691</v>
       </c>
       <c r="T8" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="U8" t="n">
         <v>1</v>
       </c>
-      <c r="V8" t="inlineStr"/>
-      <c r="W8" t="inlineStr"/>
+      <c r="V8" t="n">
+        <v>0</v>
+      </c>
+      <c r="W8" t="n">
+        <v>2</v>
+      </c>
       <c r="X8" t="n">
-        <v>0</v>
+        <v>0.3625804657325691</v>
       </c>
       <c r="Y8" t="n">
-        <v>0.3834058669835496</v>
-      </c>
-      <c r="Z8" t="n">
-        <v>3.3</v>
-      </c>
-      <c r="AA8" t="inlineStr">
+        <v>3</v>
+      </c>
+      <c r="Z8" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
+      <c r="AA8" t="n">
+        <v>0.04387069859885367</v>
+      </c>
       <c r="AB8" t="n">
-        <v>0.1153214613242233</v>
+        <v>0.8701931177581659</v>
       </c>
       <c r="AC8" t="n">
-        <v>3.450652802851947</v>
-      </c>
-      <c r="AD8" t="n">
-        <v>0.0663563345590133</v>
-      </c>
+        <v>0.01098133135658386</v>
+      </c>
+      <c r="AD8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
         <is>
-          <t>QHQVu3Ot</t>
+          <t>zgoMLawP</t>
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>45748.66666666666</v>
+        <v>45749.65625</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>nottingham</t>
+          <t>brighton</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>manchester utd</t>
+          <t>aston villa</t>
         </is>
       </c>
       <c r="E9" t="n">
@@ -1324,69 +1334,71 @@
         </is>
       </c>
       <c r="I9" t="n">
-        <v>2.1</v>
+        <v>2</v>
       </c>
       <c r="J9" t="n">
-        <v>3.6</v>
+        <v>4</v>
       </c>
       <c r="K9" t="n">
         <v>3.2</v>
       </c>
       <c r="L9" t="n">
-        <v>0.4465116279069767</v>
+        <v>0.4705882352941176</v>
       </c>
       <c r="M9" t="n">
-        <v>0.2604651162790698</v>
+        <v>0.2352941176470588</v>
       </c>
       <c r="N9" t="n">
-        <v>0.2930232558139535</v>
+        <v>0.2941176470588235</v>
       </c>
       <c r="O9" t="n">
-        <v>0.06646825396825395</v>
+        <v>0.0625</v>
       </c>
       <c r="P9" t="n">
         <v>1</v>
       </c>
       <c r="Q9" t="n">
-        <v>0.3662755710119722</v>
+        <v>0.2942611715749515</v>
       </c>
       <c r="R9" t="n">
-        <v>0.3574092605825145</v>
+        <v>0.2824036729260985</v>
       </c>
       <c r="S9" t="n">
-        <v>0.2763151684055133</v>
+        <v>0.42333515549895</v>
       </c>
       <c r="T9" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="U9" t="n">
         <v>1</v>
       </c>
-      <c r="V9" t="inlineStr"/>
-      <c r="W9" t="inlineStr"/>
+      <c r="V9" t="n">
+        <v>0</v>
+      </c>
+      <c r="W9" t="n">
+        <v>2</v>
+      </c>
       <c r="X9" t="n">
-        <v>0</v>
+        <v>0.42333515549895</v>
       </c>
       <c r="Y9" t="n">
-        <v>0.3662755710119722</v>
-      </c>
-      <c r="Z9" t="n">
-        <v>3.6</v>
-      </c>
-      <c r="AA9" t="inlineStr">
+        <v>3.2</v>
+      </c>
+      <c r="Z9" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
+      <c r="AA9" t="n">
+        <v>0.1612147716348363</v>
+      </c>
       <c r="AB9" t="n">
-        <v>0.1225354060165768</v>
+        <v>5.080021865987399</v>
       </c>
       <c r="AC9" t="n">
-        <v>3.29648013910775</v>
-      </c>
-      <c r="AD9" t="n">
-        <v>0.008866310429457624</v>
-      </c>
+        <v>0.1290739839239984</v>
+      </c>
+      <c r="AD9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
@@ -1448,13 +1460,13 @@
         <v>2</v>
       </c>
       <c r="Q10" t="n">
-        <v>0.4055130249341327</v>
+        <v>0.2884600202373528</v>
       </c>
       <c r="R10" t="n">
-        <v>0.180333828207914</v>
+        <v>0.1758219106223335</v>
       </c>
       <c r="S10" t="n">
-        <v>0.4141531468579533</v>
+        <v>0.5357180691403137</v>
       </c>
       <c r="T10" t="n">
         <v>2</v>
@@ -1463,34 +1475,32 @@
         <v>1</v>
       </c>
       <c r="V10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="W10" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="X10" t="n">
-        <v>2</v>
+        <v>0.5357180691403137</v>
       </c>
       <c r="Y10" t="n">
-        <v>0.4141531468579533</v>
-      </c>
-      <c r="Z10" t="n">
         <v>1.62</v>
       </c>
-      <c r="AA10" t="inlineStr">
+      <c r="Z10" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
+      <c r="AA10" t="n">
+        <v>-0.2131237548269221</v>
+      </c>
       <c r="AB10" t="n">
-        <v>-0.5307611324034121</v>
+        <v>6.428616829683764</v>
       </c>
       <c r="AC10" t="n">
-        <v>1.24245944057386</v>
-      </c>
-      <c r="AD10" t="n">
-        <v>0.008640121923820576</v>
-      </c>
+        <v>0.2472580489029609</v>
+      </c>
+      <c r="AD10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
@@ -1552,13 +1562,13 @@
         <v>1</v>
       </c>
       <c r="Q11" t="n">
-        <v>0.1925364736516477</v>
+        <v>0.2753329667748542</v>
       </c>
       <c r="R11" t="n">
-        <v>0.4269318489910416</v>
+        <v>0.4527139176534847</v>
       </c>
       <c r="S11" t="n">
-        <v>0.3805316773573108</v>
+        <v>0.2719531155716611</v>
       </c>
       <c r="T11" t="n">
         <v>1</v>
@@ -1567,33 +1577,33 @@
         <v>1</v>
       </c>
       <c r="V11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="W11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X11" t="n">
-        <v>1</v>
+        <v>0.4527139176534847</v>
       </c>
       <c r="Y11" t="n">
-        <v>0.4269318489910416</v>
-      </c>
-      <c r="Z11" t="n">
         <v>1.75</v>
       </c>
-      <c r="AA11" t="inlineStr">
+      <c r="Z11" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
+      <c r="AA11" t="n">
+        <v>-0.2770008588085357</v>
+      </c>
       <c r="AB11" t="n">
-        <v>-0.3371590190209028</v>
+        <v>3.513696403513295</v>
       </c>
       <c r="AC11" t="n">
-        <v>3.201988867432812</v>
+        <v>0.1773809508786305</v>
       </c>
       <c r="AD11" t="n">
-        <v>0.04640017163373084</v>
+        <v>1</v>
       </c>
     </row>
     <row r="12">
@@ -1656,13 +1666,13 @@
         <v>1</v>
       </c>
       <c r="Q12" t="n">
-        <v>0.3757457166812839</v>
+        <v>0.2625045066910773</v>
       </c>
       <c r="R12" t="n">
-        <v>0.42991455295273</v>
+        <v>0.4112374006939144</v>
       </c>
       <c r="S12" t="n">
-        <v>0.1943397303659861</v>
+        <v>0.3262580926150082</v>
       </c>
       <c r="T12" t="n">
         <v>1</v>
@@ -1671,30 +1681,30 @@
         <v>1</v>
       </c>
       <c r="V12" t="inlineStr"/>
-      <c r="W12" t="inlineStr"/>
+      <c r="W12" t="n">
+        <v>1</v>
+      </c>
       <c r="X12" t="n">
-        <v>1</v>
+        <v>0.4112374006939144</v>
       </c>
       <c r="Y12" t="n">
-        <v>0.42991455295273</v>
-      </c>
-      <c r="Z12" t="n">
         <v>1.95</v>
       </c>
-      <c r="AA12" t="inlineStr">
+      <c r="Z12" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
+      <c r="AA12" t="n">
+        <v>-0.2085127038388074</v>
+      </c>
       <c r="AB12" t="n">
-        <v>-0.1701753913075543</v>
+        <v>3.31666159989541</v>
       </c>
       <c r="AC12" t="n">
-        <v>3.224359147145475</v>
-      </c>
-      <c r="AD12" t="n">
-        <v>0.05416883627144609</v>
-      </c>
+        <v>0.08497930807890619</v>
+      </c>
+      <c r="AD12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
@@ -1756,13 +1766,13 @@
         <v>1</v>
       </c>
       <c r="Q13" t="n">
-        <v>0.4472576318312867</v>
+        <v>0.3864521213741127</v>
       </c>
       <c r="R13" t="n">
-        <v>0.307467370706631</v>
+        <v>0.3207498404333426</v>
       </c>
       <c r="S13" t="n">
-        <v>0.2452749974620823</v>
+        <v>0.2927980381925447</v>
       </c>
       <c r="T13" t="n">
         <v>0</v>
@@ -1771,33 +1781,33 @@
         <v>1</v>
       </c>
       <c r="V13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="W13" t="n">
         <v>0</v>
       </c>
       <c r="X13" t="n">
-        <v>0</v>
+        <v>0.3864521213741127</v>
       </c>
       <c r="Y13" t="n">
-        <v>0.4472576318312867</v>
-      </c>
-      <c r="Z13" t="n">
         <v>3.8</v>
       </c>
-      <c r="AA13" t="inlineStr">
+      <c r="Z13" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
+      <c r="AA13" t="n">
+        <v>0.1673278790077244</v>
+      </c>
       <c r="AB13" t="n">
-        <v>0.2498496431996034</v>
+        <v>1.159356364122338</v>
       </c>
       <c r="AC13" t="n">
-        <v>2.01265934324079</v>
+        <v>0.06570228094077013</v>
       </c>
       <c r="AD13" t="n">
-        <v>0.1397902611246557</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14">
@@ -1860,13 +1870,13 @@
         <v>2</v>
       </c>
       <c r="Q14" t="n">
-        <v>0.3369108966757062</v>
+        <v>0.2917475912376913</v>
       </c>
       <c r="R14" t="n">
-        <v>0.1635641496454571</v>
+        <v>0.1940946840876043</v>
       </c>
       <c r="S14" t="n">
-        <v>0.4995249536788367</v>
+        <v>0.5141577246747043</v>
       </c>
       <c r="T14" t="n">
         <v>2</v>
@@ -1875,33 +1885,33 @@
         <v>1</v>
       </c>
       <c r="V14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="W14" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="X14" t="n">
-        <v>2</v>
+        <v>0.5141577246747043</v>
       </c>
       <c r="Y14" t="n">
-        <v>0.4995249536788367</v>
-      </c>
-      <c r="Z14" t="n">
         <v>2.45</v>
       </c>
-      <c r="AA14" t="inlineStr">
+      <c r="Z14" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
+      <c r="AA14" t="n">
+        <v>0.179094086519328</v>
+      </c>
       <c r="AB14" t="n">
-        <v>0.1543697493194137</v>
+        <v>6.169892696096452</v>
       </c>
       <c r="AC14" t="n">
-        <v>6.743586874664296</v>
+        <v>0.222410133437013</v>
       </c>
       <c r="AD14" t="n">
-        <v>0.1626140570031305</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15">
@@ -1964,13 +1974,13 @@
         <v>2</v>
       </c>
       <c r="Q15" t="n">
-        <v>0.1967406352454221</v>
+        <v>0.1004835089647717</v>
       </c>
       <c r="R15" t="n">
-        <v>0.1070292013445253</v>
+        <v>0.1174483317310698</v>
       </c>
       <c r="S15" t="n">
-        <v>0.6962301634100526</v>
+        <v>0.7820681593041585</v>
       </c>
       <c r="T15" t="n">
         <v>2</v>
@@ -1979,33 +1989,33 @@
         <v>1</v>
       </c>
       <c r="V15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="W15" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="X15" t="n">
-        <v>2</v>
+        <v>0.7820681593041585</v>
       </c>
       <c r="Y15" t="n">
-        <v>0.6962301634100526</v>
-      </c>
-      <c r="Z15" t="n">
         <v>1.6</v>
       </c>
-      <c r="AA15" t="inlineStr">
+      <c r="Z15" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
+      <c r="AA15" t="n">
+        <v>0.4188484248110894</v>
+      </c>
       <c r="AB15" t="n">
-        <v>0.189947102426807</v>
+        <v>9.384817911649902</v>
       </c>
       <c r="AC15" t="n">
-        <v>9.39910720603571</v>
+        <v>0.6646198275730887</v>
       </c>
       <c r="AD15" t="n">
-        <v>0.4994895281646305</v>
+        <v>1</v>
       </c>
     </row>
     <row r="16">
@@ -2068,13 +2078,13 @@
         <v>2</v>
       </c>
       <c r="Q16" t="n">
-        <v>0.235459764596706</v>
+        <v>0.1038261377896294</v>
       </c>
       <c r="R16" t="n">
-        <v>0.020806732360019</v>
+        <v>0.02733959788000358</v>
       </c>
       <c r="S16" t="n">
-        <v>0.743733503043275</v>
+        <v>0.868834264330367</v>
       </c>
       <c r="T16" t="n">
         <v>2</v>
@@ -2082,30 +2092,34 @@
       <c r="U16" t="n">
         <v>1</v>
       </c>
-      <c r="V16" t="inlineStr"/>
-      <c r="W16" t="inlineStr"/>
+      <c r="V16" t="n">
+        <v>0</v>
+      </c>
+      <c r="W16" t="n">
+        <v>2</v>
+      </c>
       <c r="X16" t="n">
-        <v>2</v>
+        <v>0.868834264330367</v>
       </c>
       <c r="Y16" t="n">
-        <v>0.743733503043275</v>
-      </c>
-      <c r="Z16" t="n">
         <v>1.14</v>
       </c>
-      <c r="AA16" t="inlineStr">
+      <c r="Z16" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
+      <c r="AA16" t="n">
+        <v>-0.0680638475955834</v>
+      </c>
       <c r="AB16" t="n">
-        <v>-1.086741475219048</v>
+        <v>10.07133087058614</v>
       </c>
       <c r="AC16" t="n">
-        <v>10.04040229108421</v>
+        <v>0.7650081265407377</v>
       </c>
       <c r="AD16" t="n">
-        <v>0.5082737384465691</v>
+        <v>1</v>
       </c>
     </row>
     <row r="17">
@@ -2168,13 +2182,13 @@
         <v>1</v>
       </c>
       <c r="Q17" t="n">
-        <v>0.3058077490559443</v>
+        <v>0.249670691980813</v>
       </c>
       <c r="R17" t="n">
-        <v>0.2525813459229875</v>
+        <v>0.1947457207697191</v>
       </c>
       <c r="S17" t="n">
-        <v>0.4416109050210683</v>
+        <v>0.5555835872494679</v>
       </c>
       <c r="T17" t="n">
         <v>2</v>
@@ -2183,33 +2197,33 @@
         <v>1</v>
       </c>
       <c r="V17" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="W17" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="X17" t="n">
-        <v>2</v>
+        <v>0.5555835872494679</v>
       </c>
       <c r="Y17" t="n">
-        <v>0.4416109050210683</v>
-      </c>
-      <c r="Z17" t="n">
         <v>4.1</v>
       </c>
-      <c r="AA17" t="inlineStr">
+      <c r="Z17" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
+      <c r="AA17" t="n">
+        <v>0.4122234541041349</v>
+      </c>
       <c r="AB17" t="n">
-        <v>0.2614853905117354</v>
+        <v>6.667003046993615</v>
       </c>
       <c r="AC17" t="n">
-        <v>5.961747217784422</v>
+        <v>0.3059128952686548</v>
       </c>
       <c r="AD17" t="n">
-        <v>0.1358031559651239</v>
+        <v>1</v>
       </c>
     </row>
     <row r="18">
@@ -2272,13 +2286,13 @@
         <v>2</v>
       </c>
       <c r="Q18" t="n">
-        <v>0.3697548099325002</v>
+        <v>0.3637247043428444</v>
       </c>
       <c r="R18" t="n">
-        <v>0.1252853591008778</v>
+        <v>0.1868887254677783</v>
       </c>
       <c r="S18" t="n">
-        <v>0.504959830966622</v>
+        <v>0.4493865701893771</v>
       </c>
       <c r="T18" t="n">
         <v>2</v>
@@ -2287,30 +2301,30 @@
         <v>1</v>
       </c>
       <c r="V18" t="inlineStr"/>
-      <c r="W18" t="inlineStr"/>
+      <c r="W18" t="n">
+        <v>2</v>
+      </c>
       <c r="X18" t="n">
-        <v>2</v>
+        <v>0.4493865701893771</v>
       </c>
       <c r="Y18" t="n">
-        <v>0.504959830966622</v>
-      </c>
-      <c r="Z18" t="n">
         <v>1.91</v>
       </c>
-      <c r="AA18" t="inlineStr">
+      <c r="Z18" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
+      <c r="AA18" t="n">
+        <v>-0.1556831328992195</v>
+      </c>
       <c r="AB18" t="n">
-        <v>-0.03904035478434289</v>
+        <v>4.973713179303114</v>
       </c>
       <c r="AC18" t="n">
-        <v>6.816957718049396</v>
-      </c>
-      <c r="AD18" t="n">
-        <v>0.1352050210341218</v>
-      </c>
+        <v>0.08566186584653268</v>
+      </c>
+      <c r="AD18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="1" t="inlineStr">
@@ -2372,13 +2386,13 @@
         <v>2</v>
       </c>
       <c r="Q19" t="n">
-        <v>0.3276280230264123</v>
+        <v>0.1466450563544316</v>
       </c>
       <c r="R19" t="n">
-        <v>0.3049725845117274</v>
+        <v>0.2802032080537756</v>
       </c>
       <c r="S19" t="n">
-        <v>0.3673993924618603</v>
+        <v>0.5731517355917929</v>
       </c>
       <c r="T19" t="n">
         <v>2</v>
@@ -2387,33 +2401,33 @@
         <v>1</v>
       </c>
       <c r="V19" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="W19" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="X19" t="n">
-        <v>2</v>
+        <v>0.5731517355917929</v>
       </c>
       <c r="Y19" t="n">
-        <v>0.3673993924618603</v>
-      </c>
-      <c r="Z19" t="n">
         <v>2.55</v>
       </c>
-      <c r="AA19" t="inlineStr">
+      <c r="Z19" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
+      <c r="AA19" t="n">
+        <v>0.2977657585542399</v>
+      </c>
       <c r="AB19" t="n">
-        <v>-0.0407300317562943</v>
+        <v>6.877820827101515</v>
       </c>
       <c r="AC19" t="n">
-        <v>4.959891798235113</v>
+        <v>0.2929485275380173</v>
       </c>
       <c r="AD19" t="n">
-        <v>0.03977136943544807</v>
+        <v>1</v>
       </c>
     </row>
     <row r="20">
@@ -2491,30 +2505,30 @@
         <v>1</v>
       </c>
       <c r="V20" t="inlineStr"/>
-      <c r="W20" t="inlineStr"/>
+      <c r="W20" t="n">
+        <v>1</v>
+      </c>
       <c r="X20" t="n">
-        <v>1</v>
+        <v>0.7825458264646554</v>
       </c>
       <c r="Y20" t="n">
-        <v>0.7825458264646554</v>
-      </c>
-      <c r="Z20" t="n">
         <v>1.27</v>
       </c>
-      <c r="AA20" t="inlineStr">
+      <c r="Z20" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
+      <c r="AA20" t="n">
+        <v>-0.02284000144402813</v>
+      </c>
       <c r="AB20" t="n">
-        <v>-0.02284000144402813</v>
+        <v>2.320828623112449</v>
       </c>
       <c r="AC20" t="n">
-        <v>2.347637479393966</v>
-      </c>
-      <c r="AD20" t="n">
         <v>0.6113133678474076</v>
       </c>
+      <c r="AD20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="1" t="inlineStr">
@@ -2591,30 +2605,30 @@
         <v>1</v>
       </c>
       <c r="V21" t="inlineStr"/>
-      <c r="W21" t="inlineStr"/>
+      <c r="W21" t="n">
+        <v>1</v>
+      </c>
       <c r="X21" t="n">
-        <v>1</v>
+        <v>0.9006459813523363</v>
       </c>
       <c r="Y21" t="n">
-        <v>0.9006459813523363</v>
-      </c>
-      <c r="Z21" t="n">
         <v>1.14</v>
       </c>
-      <c r="AA21" t="inlineStr">
+      <c r="Z21" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
+      <c r="AA21" t="n">
+        <v>0.1909744195833094</v>
+      </c>
       <c r="AB21" t="n">
-        <v>0.1909744195833094</v>
+        <v>2.701937944057009</v>
       </c>
       <c r="AC21" t="n">
-        <v>2.701937944057009</v>
-      </c>
-      <c r="AD21" t="n">
         <v>0.8256672270830573</v>
       </c>
+      <c r="AD21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="1" t="inlineStr">
@@ -2691,30 +2705,30 @@
         <v>1</v>
       </c>
       <c r="V22" t="inlineStr"/>
-      <c r="W22" t="inlineStr"/>
+      <c r="W22" t="n">
+        <v>1</v>
+      </c>
       <c r="X22" t="n">
-        <v>1</v>
+        <v>0.5091193002336956</v>
       </c>
       <c r="Y22" t="n">
-        <v>0.5091193002336956</v>
-      </c>
-      <c r="Z22" t="n">
         <v>2.35</v>
       </c>
-      <c r="AA22" t="inlineStr">
+      <c r="Z22" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
+      <c r="AA22" t="n">
+        <v>0.1455039670734701</v>
+      </c>
       <c r="AB22" t="n">
-        <v>0.1455039670734701</v>
+        <v>1.527357900701087</v>
       </c>
       <c r="AC22" t="n">
-        <v>1.527357900701087</v>
-      </c>
-      <c r="AD22" t="n">
         <v>0.2049859611591311</v>
       </c>
+      <c r="AD22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="1" t="inlineStr">
@@ -2791,30 +2805,30 @@
         <v>1</v>
       </c>
       <c r="V23" t="inlineStr"/>
-      <c r="W23" t="inlineStr"/>
+      <c r="W23" t="n">
+        <v>1</v>
+      </c>
       <c r="X23" t="n">
-        <v>1</v>
+        <v>0.5373389783576131</v>
       </c>
       <c r="Y23" t="n">
-        <v>0.5373389783576131</v>
-      </c>
-      <c r="Z23" t="n">
         <v>1.65</v>
       </c>
-      <c r="AA23" t="inlineStr">
+      <c r="Z23" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
+      <c r="AA23" t="n">
+        <v>-0.1744472087845206</v>
+      </c>
       <c r="AB23" t="n">
-        <v>-0.1744472087845206</v>
+        <v>1.471766500488131</v>
       </c>
       <c r="AC23" t="n">
-        <v>1.612016935072839</v>
-      </c>
-      <c r="AD23" t="n">
         <v>0.2473442706888411</v>
       </c>
+      <c r="AD23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="1" t="inlineStr">
@@ -2891,33 +2905,33 @@
         <v>1</v>
       </c>
       <c r="V24" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="W24" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X24" t="n">
-        <v>1</v>
+        <v>0.4066937553467808</v>
       </c>
       <c r="Y24" t="n">
-        <v>0.4066937553467808</v>
-      </c>
-      <c r="Z24" t="n">
         <v>2</v>
       </c>
-      <c r="AA24" t="inlineStr">
+      <c r="Z24" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
+      <c r="AA24" t="n">
+        <v>-0.1866124893064383</v>
+      </c>
       <c r="AB24" t="n">
-        <v>-0.1866124893064383</v>
+        <v>1.106569287752813</v>
       </c>
       <c r="AC24" t="n">
-        <v>1.220081266040342</v>
+        <v>0.03813939040308317</v>
       </c>
       <c r="AD24" t="n">
-        <v>0.03813939040308317</v>
+        <v>1</v>
       </c>
     </row>
     <row r="25">
@@ -2995,30 +3009,30 @@
         <v>1</v>
       </c>
       <c r="V25" t="inlineStr"/>
-      <c r="W25" t="inlineStr"/>
+      <c r="W25" t="n">
+        <v>1</v>
+      </c>
       <c r="X25" t="n">
-        <v>1</v>
+        <v>0.7198839679267474</v>
       </c>
       <c r="Y25" t="n">
-        <v>0.7198839679267474</v>
-      </c>
-      <c r="Z25" t="n">
         <v>1.7</v>
       </c>
-      <c r="AA25" t="inlineStr">
+      <c r="Z25" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
+      <c r="AA25" t="n">
+        <v>0.3197182078221008</v>
+      </c>
       <c r="AB25" t="n">
-        <v>0.3197182078221008</v>
+        <v>2.159651903780242</v>
       </c>
       <c r="AC25" t="n">
-        <v>2.159651903780242</v>
-      </c>
-      <c r="AD25" t="n">
         <v>0.5506784616981166</v>
       </c>
+      <c r="AD25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="1" t="inlineStr">
@@ -3095,30 +3109,30 @@
         <v>1</v>
       </c>
       <c r="V26" t="inlineStr"/>
-      <c r="W26" t="inlineStr"/>
+      <c r="W26" t="n">
+        <v>0</v>
+      </c>
       <c r="X26" t="n">
-        <v>0</v>
+        <v>0.454936820626022</v>
       </c>
       <c r="Y26" t="n">
-        <v>0.454936820626022</v>
-      </c>
-      <c r="Z26" t="n">
         <v>3.8</v>
       </c>
-      <c r="AA26" t="inlineStr">
+      <c r="Z26" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
+      <c r="AA26" t="n">
+        <v>0.2602713994210298</v>
+      </c>
       <c r="AB26" t="n">
-        <v>0.2602713994210298</v>
+        <v>5.459241847512263</v>
       </c>
       <c r="AC26" t="n">
-        <v>6.141647078451297</v>
-      </c>
-      <c r="AD26" t="n">
         <v>0.09499876507328531</v>
       </c>
+      <c r="AD26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="1" t="inlineStr">
@@ -3195,30 +3209,30 @@
         <v>1</v>
       </c>
       <c r="V27" t="inlineStr"/>
-      <c r="W27" t="inlineStr"/>
+      <c r="W27" t="n">
+        <v>0</v>
+      </c>
       <c r="X27" t="n">
-        <v>0</v>
+        <v>0.4125590999147862</v>
       </c>
       <c r="Y27" t="n">
-        <v>0.4125590999147862</v>
-      </c>
-      <c r="Z27" t="n">
         <v>3.75</v>
       </c>
-      <c r="AA27" t="inlineStr">
+      <c r="Z27" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
+      <c r="AA27" t="n">
+        <v>0.1989442271565266</v>
+      </c>
       <c r="AB27" t="n">
-        <v>0.1989442271565266</v>
+        <v>4.950709198977434</v>
       </c>
       <c r="AC27" t="n">
-        <v>5.569547848849614</v>
-      </c>
-      <c r="AD27" t="n">
         <v>0.09581271511068973</v>
       </c>
+      <c r="AD27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="1" t="inlineStr">
@@ -3295,30 +3309,30 @@
         <v>1</v>
       </c>
       <c r="V28" t="inlineStr"/>
-      <c r="W28" t="inlineStr"/>
+      <c r="W28" t="n">
+        <v>2</v>
+      </c>
       <c r="X28" t="n">
-        <v>2</v>
+        <v>0.4142279663281674</v>
       </c>
       <c r="Y28" t="n">
-        <v>0.4142279663281674</v>
-      </c>
-      <c r="Z28" t="n">
         <v>2.25</v>
       </c>
-      <c r="AA28" t="inlineStr">
+      <c r="Z28" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
+      <c r="AA28" t="n">
+        <v>-0.05438966060929866</v>
+      </c>
       <c r="AB28" t="n">
-        <v>-0.05438966060929866</v>
+        <v>4.835590599165041</v>
       </c>
       <c r="AC28" t="n">
-        <v>4.349393646445758</v>
-      </c>
-      <c r="AD28" t="n">
         <v>0.0509843071978795</v>
       </c>
+      <c r="AD28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="1" t="inlineStr">
@@ -3395,30 +3409,30 @@
         <v>1</v>
       </c>
       <c r="V29" t="inlineStr"/>
-      <c r="W29" t="inlineStr"/>
+      <c r="W29" t="n">
+        <v>1</v>
+      </c>
       <c r="X29" t="n">
-        <v>1</v>
+        <v>0.6092363933642873</v>
       </c>
       <c r="Y29" t="n">
-        <v>0.6092363933642873</v>
-      </c>
-      <c r="Z29" t="n">
         <v>1.73</v>
       </c>
-      <c r="AA29" t="inlineStr">
+      <c r="Z29" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
+      <c r="AA29" t="n">
+        <v>0.07394378153454376</v>
+      </c>
       <c r="AB29" t="n">
-        <v>0.07394378153454376</v>
+        <v>1.827709180092862</v>
       </c>
       <c r="AC29" t="n">
-        <v>1.827709180092862</v>
-      </c>
-      <c r="AD29" t="n">
         <v>0.3279189310629804</v>
       </c>
+      <c r="AD29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="1" t="inlineStr">
@@ -3495,30 +3509,30 @@
         <v>1</v>
       </c>
       <c r="V30" t="inlineStr"/>
-      <c r="W30" t="inlineStr"/>
+      <c r="W30" t="n">
+        <v>1</v>
+      </c>
       <c r="X30" t="n">
-        <v>1</v>
+        <v>0.5936828179907958</v>
       </c>
       <c r="Y30" t="n">
-        <v>0.5936828179907958</v>
-      </c>
-      <c r="Z30" t="n">
         <v>1.55</v>
       </c>
-      <c r="AA30" t="inlineStr">
+      <c r="Z30" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
+      <c r="AA30" t="n">
+        <v>-0.1450756947532118</v>
+      </c>
       <c r="AB30" t="n">
-        <v>-0.1450756947532118</v>
+        <v>1.652081151183328</v>
       </c>
       <c r="AC30" t="n">
-        <v>1.781048453972387</v>
-      </c>
-      <c r="AD30" t="n">
         <v>0.2890948059640486</v>
       </c>
+      <c r="AD30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="1" t="inlineStr">
@@ -3595,30 +3609,30 @@
         <v>1</v>
       </c>
       <c r="V31" t="inlineStr"/>
-      <c r="W31" t="inlineStr"/>
+      <c r="W31" t="n">
+        <v>1</v>
+      </c>
       <c r="X31" t="n">
-        <v>1</v>
+        <v>0.4555702555943796</v>
       </c>
       <c r="Y31" t="n">
-        <v>0.4555702555943796</v>
-      </c>
-      <c r="Z31" t="n">
         <v>1.67</v>
       </c>
-      <c r="AA31" t="inlineStr">
+      <c r="Z31" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
+      <c r="AA31" t="n">
+        <v>-0.3570114524737107</v>
+      </c>
       <c r="AB31" t="n">
-        <v>-0.3570114524737107</v>
+        <v>1.125303726745403</v>
       </c>
       <c r="AC31" t="n">
-        <v>1.366710766783139</v>
-      </c>
-      <c r="AD31" t="n">
         <v>0.032470168263524</v>
       </c>
+      <c r="AD31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="1" t="inlineStr">
@@ -3695,30 +3709,30 @@
         <v>1</v>
       </c>
       <c r="V32" t="inlineStr"/>
-      <c r="W32" t="inlineStr"/>
+      <c r="W32" t="n">
+        <v>1</v>
+      </c>
       <c r="X32" t="n">
-        <v>1</v>
+        <v>0.6727771930227373</v>
       </c>
       <c r="Y32" t="n">
-        <v>0.6727771930227373</v>
-      </c>
-      <c r="Z32" t="n">
         <v>1.42</v>
       </c>
-      <c r="AA32" t="inlineStr">
+      <c r="Z32" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
+      <c r="AA32" t="n">
+        <v>-0.1063247283516979</v>
+      </c>
       <c r="AB32" t="n">
-        <v>-0.1063247283516979</v>
+        <v>1.911133270885033</v>
       </c>
       <c r="AC32" t="n">
-        <v>2.018331579068212</v>
-      </c>
-      <c r="AD32" t="n">
         <v>0.3988900842851951</v>
       </c>
+      <c r="AD32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="1" t="inlineStr">
@@ -3795,33 +3809,33 @@
         <v>1</v>
       </c>
       <c r="V33" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="W33" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X33" t="n">
-        <v>1</v>
+        <v>0.3682104980889199</v>
       </c>
       <c r="Y33" t="n">
-        <v>0.3682104980889199</v>
-      </c>
-      <c r="Z33" t="n">
         <v>1.9</v>
       </c>
-      <c r="AA33" t="inlineStr">
+      <c r="Z33" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
+      <c r="AA33" t="n">
+        <v>-0.333777837367836</v>
+      </c>
       <c r="AB33" t="n">
-        <v>-0.333777837367836</v>
+        <v>0.9219733906620089</v>
       </c>
       <c r="AC33" t="n">
-        <v>1.104631494266759</v>
+        <v>0.02632416652920944</v>
       </c>
       <c r="AD33" t="n">
-        <v>0.02632416652920944</v>
+        <v>1</v>
       </c>
     </row>
     <row r="34">
@@ -3899,30 +3913,30 @@
         <v>1</v>
       </c>
       <c r="V34" t="inlineStr"/>
-      <c r="W34" t="inlineStr"/>
+      <c r="W34" t="n">
+        <v>0</v>
+      </c>
       <c r="X34" t="n">
-        <v>0</v>
+        <v>0.4042434275738219</v>
       </c>
       <c r="Y34" t="n">
-        <v>0.4042434275738219</v>
-      </c>
-      <c r="Z34" t="n">
         <v>3.4</v>
       </c>
-      <c r="AA34" t="inlineStr">
+      <c r="Z34" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
+      <c r="AA34" t="n">
+        <v>0.1560115223962476</v>
+      </c>
       <c r="AB34" t="n">
-        <v>0.1560115223962476</v>
+        <v>4.850921130885863</v>
       </c>
       <c r="AC34" t="n">
-        <v>7.882746837689526</v>
-      </c>
-      <c r="AD34" t="n">
         <v>0.03539538923291191</v>
       </c>
+      <c r="AD34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="1" t="inlineStr">
@@ -3999,30 +4013,30 @@
         <v>1</v>
       </c>
       <c r="V35" t="inlineStr"/>
-      <c r="W35" t="inlineStr"/>
+      <c r="W35" t="n">
+        <v>0</v>
+      </c>
       <c r="X35" t="n">
-        <v>0</v>
+        <v>0.3765153835048269</v>
       </c>
       <c r="Y35" t="n">
-        <v>0.3765153835048269</v>
-      </c>
-      <c r="Z35" t="n">
         <v>3.1</v>
       </c>
-      <c r="AA35" t="inlineStr">
+      <c r="Z35" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
+      <c r="AA35" t="n">
+        <v>0.07961794707855407</v>
+      </c>
       <c r="AB35" t="n">
-        <v>0.07961794707855407</v>
+        <v>4.518184602057923</v>
       </c>
       <c r="AC35" t="n">
-        <v>7.342049978344125</v>
-      </c>
-      <c r="AD35" t="n">
         <v>0.04439633633870788</v>
       </c>
+      <c r="AD35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="1" t="inlineStr">
@@ -4099,30 +4113,30 @@
         <v>1</v>
       </c>
       <c r="V36" t="inlineStr"/>
-      <c r="W36" t="inlineStr"/>
+      <c r="W36" t="n">
+        <v>0</v>
+      </c>
       <c r="X36" t="n">
-        <v>0</v>
+        <v>0.4941601521686576</v>
       </c>
       <c r="Y36" t="n">
-        <v>0.4941601521686576</v>
-      </c>
-      <c r="Z36" t="n">
         <v>3.3</v>
       </c>
-      <c r="AA36" t="inlineStr">
+      <c r="Z36" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
+      <c r="AA36" t="n">
+        <v>0.2742297835463348</v>
+      </c>
       <c r="AB36" t="n">
-        <v>0.2742297835463348</v>
+        <v>5.929921826023891</v>
       </c>
       <c r="AC36" t="n">
-        <v>9.636122967288824</v>
-      </c>
-      <c r="AD36" t="n">
         <v>0.1141177850734852</v>
       </c>
+      <c r="AD36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="1" t="inlineStr">
@@ -4199,33 +4213,33 @@
         <v>1</v>
       </c>
       <c r="V37" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="W37" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="X37" t="n">
-        <v>2</v>
+        <v>0.6592570027062244</v>
       </c>
       <c r="Y37" t="n">
-        <v>0.6592570027062244</v>
-      </c>
-      <c r="Z37" t="n">
         <v>1.83</v>
       </c>
-      <c r="AA37" t="inlineStr">
+      <c r="Z37" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
+      <c r="AA37" t="n">
+        <v>0.2487232710269768</v>
+      </c>
       <c r="AB37" t="n">
-        <v>0.2487232710269768</v>
+        <v>7.911084032474693</v>
       </c>
       <c r="AC37" t="n">
-        <v>7.911084032474693</v>
+        <v>0.4204796570220136</v>
       </c>
       <c r="AD37" t="n">
-        <v>0.4204796570220136</v>
+        <v>1</v>
       </c>
     </row>
     <row r="38">
@@ -4303,30 +4317,30 @@
         <v>1</v>
       </c>
       <c r="V38" t="inlineStr"/>
-      <c r="W38" t="inlineStr"/>
+      <c r="W38" t="n">
+        <v>2</v>
+      </c>
       <c r="X38" t="n">
-        <v>2</v>
+        <v>0.5489002497277609</v>
       </c>
       <c r="Y38" t="n">
-        <v>0.5489002497277609</v>
-      </c>
-      <c r="Z38" t="n">
         <v>1.85</v>
       </c>
-      <c r="AA38" t="inlineStr">
+      <c r="Z38" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
+      <c r="AA38" t="n">
+        <v>0.01819466117218543</v>
+      </c>
       <c r="AB38" t="n">
-        <v>0.01819466117218543</v>
+        <v>6.58680299673313</v>
       </c>
       <c r="AC38" t="n">
-        <v>6.58680299673313</v>
-      </c>
-      <c r="AD38" t="n">
         <v>0.2162498241274949</v>
       </c>
+      <c r="AD38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="1" t="inlineStr">
@@ -4388,13 +4402,13 @@
         <v>1</v>
       </c>
       <c r="Q39" t="n">
-        <v>0.2566780000413285</v>
+        <v>0.2305520321597711</v>
       </c>
       <c r="R39" t="n">
-        <v>0.6324699718345181</v>
+        <v>0.683057663326422</v>
       </c>
       <c r="S39" t="n">
-        <v>0.1108520281241534</v>
+        <v>0.0863903045138069</v>
       </c>
       <c r="T39" t="n">
         <v>1</v>
@@ -4406,30 +4420,30 @@
         <v>0</v>
       </c>
       <c r="W39" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X39" t="n">
-        <v>1</v>
+        <v>0.683057663326422</v>
       </c>
       <c r="Y39" t="n">
-        <v>0.6324699718345181</v>
-      </c>
-      <c r="Z39" t="n">
         <v>1.29</v>
       </c>
-      <c r="AA39" t="inlineStr">
+      <c r="Z39" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
+      <c r="AA39" t="n">
+        <v>-0.4098469458928122</v>
+      </c>
       <c r="AB39" t="n">
-        <v>-0.6348749528740398</v>
+        <v>2.049172989979266</v>
       </c>
       <c r="AC39" t="n">
-        <v>1.897409915503554</v>
+        <v>0.4525056311666509</v>
       </c>
       <c r="AD39" t="n">
-        <v>0.3757919717931897</v>
+        <v>0</v>
       </c>
     </row>
     <row r="40">
@@ -4492,13 +4506,13 @@
         <v>1</v>
       </c>
       <c r="Q40" t="n">
-        <v>0.2797094974858422</v>
+        <v>0.2859904113328284</v>
       </c>
       <c r="R40" t="n">
-        <v>0.5810972348504705</v>
+        <v>0.58658003307333</v>
       </c>
       <c r="S40" t="n">
-        <v>0.1391932676636874</v>
+        <v>0.1274295555938417</v>
       </c>
       <c r="T40" t="n">
         <v>1</v>
@@ -4510,30 +4524,30 @@
         <v>0</v>
       </c>
       <c r="W40" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X40" t="n">
-        <v>1</v>
+        <v>0.58658003307333</v>
       </c>
       <c r="Y40" t="n">
-        <v>0.5810972348504705</v>
-      </c>
-      <c r="Z40" t="n">
         <v>1.33</v>
       </c>
-      <c r="AA40" t="inlineStr">
+      <c r="Z40" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
+      <c r="AA40" t="n">
+        <v>-0.6662077454923365</v>
+      </c>
       <c r="AB40" t="n">
-        <v>-0.6883050837844672</v>
+        <v>1.75974009921999</v>
       </c>
       <c r="AC40" t="n">
-        <v>1.743291704551411</v>
+        <v>0.3005896217405016</v>
       </c>
       <c r="AD40" t="n">
-        <v>0.3013877373646283</v>
+        <v>0</v>
       </c>
     </row>
     <row r="41">
@@ -4596,13 +4610,13 @@
         <v>1</v>
       </c>
       <c r="Q41" t="n">
-        <v>0.2232539112862876</v>
+        <v>0.1670022568007548</v>
       </c>
       <c r="R41" t="n">
-        <v>0.7164941200412097</v>
+        <v>0.7906034679051955</v>
       </c>
       <c r="S41" t="n">
-        <v>0.06025196867250265</v>
+        <v>0.04239427529404956</v>
       </c>
       <c r="T41" t="n">
         <v>1</v>
@@ -4614,30 +4628,30 @@
         <v>0</v>
       </c>
       <c r="W41" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X41" t="n">
-        <v>1</v>
+        <v>0.7906034679051955</v>
       </c>
       <c r="Y41" t="n">
-        <v>0.7164941200412097</v>
-      </c>
-      <c r="Z41" t="n">
         <v>1.18</v>
       </c>
-      <c r="AA41" t="inlineStr">
+      <c r="Z41" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
+      <c r="AA41" t="n">
+        <v>-0.3727105992881631</v>
+      </c>
       <c r="AB41" t="n">
-        <v>-0.8585385463965146</v>
+        <v>2.371810403715586</v>
       </c>
       <c r="AC41" t="n">
-        <v>2.149482360123629</v>
+        <v>0.6236012111044408</v>
       </c>
       <c r="AD41" t="n">
-        <v>0.4932402087549221</v>
+        <v>0</v>
       </c>
     </row>
     <row r="42">
@@ -4700,13 +4714,13 @@
         <v>1</v>
       </c>
       <c r="Q42" t="n">
-        <v>0.2464777551432784</v>
+        <v>0.2379869131980451</v>
       </c>
       <c r="R42" t="n">
-        <v>0.6394868787076196</v>
+        <v>0.6507394337021107</v>
       </c>
       <c r="S42" t="n">
-        <v>0.1140353661491022</v>
+        <v>0.1112736530998441</v>
       </c>
       <c r="T42" t="n">
         <v>1</v>
@@ -4718,30 +4732,30 @@
         <v>0</v>
       </c>
       <c r="W42" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X42" t="n">
-        <v>1</v>
+        <v>0.6507394337021107</v>
       </c>
       <c r="Y42" t="n">
-        <v>0.6394868787076196</v>
-      </c>
-      <c r="Z42" t="n">
         <v>1.27</v>
       </c>
-      <c r="AA42" t="inlineStr">
+      <c r="Z42" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
+      <c r="AA42" t="n">
+        <v>-0.6428182192530345</v>
+      </c>
       <c r="AB42" t="n">
-        <v>-0.6957469038567523</v>
+        <v>1.952218301106332</v>
       </c>
       <c r="AC42" t="n">
-        <v>1.918460636122858</v>
+        <v>0.4127525205040656</v>
       </c>
       <c r="AD42" t="n">
-        <v>0.3930091235643412</v>
+        <v>0</v>
       </c>
     </row>
     <row r="43">
@@ -4804,13 +4818,13 @@
         <v>1</v>
       </c>
       <c r="Q43" t="n">
-        <v>0.2983724417092606</v>
+        <v>0.3277161333715918</v>
       </c>
       <c r="R43" t="n">
-        <v>0.4712586814761995</v>
+        <v>0.4978816535233578</v>
       </c>
       <c r="S43" t="n">
-        <v>0.2303688768145399</v>
+        <v>0.1744022131050505</v>
       </c>
       <c r="T43" t="n">
         <v>1</v>
@@ -4822,30 +4836,30 @@
         <v>0</v>
       </c>
       <c r="W43" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X43" t="n">
-        <v>1</v>
+        <v>0.4978816535233578</v>
       </c>
       <c r="Y43" t="n">
-        <v>0.4712586814761995</v>
-      </c>
-      <c r="Z43" t="n">
         <v>1.53</v>
       </c>
-      <c r="AA43" t="inlineStr">
+      <c r="Z43" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
+      <c r="AA43" t="n">
+        <v>-0.4495114530363442</v>
+      </c>
       <c r="AB43" t="n">
-        <v>-0.52636644781399</v>
+        <v>1.493644960570073</v>
       </c>
       <c r="AC43" t="n">
-        <v>1.413776044428599</v>
+        <v>0.1701655201517661</v>
       </c>
       <c r="AD43" t="n">
-        <v>0.172886239766939</v>
+        <v>0</v>
       </c>
     </row>
     <row r="44">
@@ -4908,13 +4922,13 @@
         <v>1</v>
       </c>
       <c r="Q44" t="n">
-        <v>0.3509223243843754</v>
+        <v>0.3555729649102405</v>
       </c>
       <c r="R44" t="n">
-        <v>0.408357020404592</v>
+        <v>0.3615364290087321</v>
       </c>
       <c r="S44" t="n">
-        <v>0.2407206552110326</v>
+        <v>0.2828906060810275</v>
       </c>
       <c r="T44" t="n">
         <v>1</v>
@@ -4926,49 +4940,49 @@
         <v>0</v>
       </c>
       <c r="W44" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X44" t="n">
-        <v>1</v>
+        <v>0.3615364290087321</v>
       </c>
       <c r="Y44" t="n">
-        <v>0.408357020404592</v>
-      </c>
-      <c r="Z44" t="n">
         <v>2.05</v>
       </c>
-      <c r="AA44" t="inlineStr">
+      <c r="Z44" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
+      <c r="AA44" t="n">
+        <v>-0.2465241147924754</v>
+      </c>
       <c r="AB44" t="n">
-        <v>-0.1551124839719872</v>
+        <v>0.2169218574052393</v>
       </c>
       <c r="AC44" t="n">
-        <v>1.225071061213776</v>
+        <v>0.005963464098491633</v>
       </c>
       <c r="AD44" t="n">
-        <v>0.05743469602021656</v>
+        <v>0</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="1" t="inlineStr">
         <is>
-          <t>GrDYvKBO</t>
+          <t>rVEQttsC</t>
         </is>
       </c>
       <c r="B45" s="2" t="n">
-        <v>45747.66666666666</v>
+        <v>45746.66666666666</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>celta vigo</t>
+          <t>betis</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>las palmas</t>
+          <t>sevilla</t>
         </is>
       </c>
       <c r="E45" t="n">
@@ -4988,37 +5002,37 @@
         </is>
       </c>
       <c r="I45" t="n">
-        <v>1.57</v>
+        <v>2</v>
       </c>
       <c r="J45" t="n">
-        <v>4.1</v>
+        <v>3.4</v>
       </c>
       <c r="K45" t="n">
-        <v>5.5</v>
+        <v>3.75</v>
       </c>
       <c r="L45" t="n">
-        <v>0.5993833395353783</v>
+        <v>0.4713493530499075</v>
       </c>
       <c r="M45" t="n">
-        <v>0.2295199617245229</v>
+        <v>0.2772643253234751</v>
       </c>
       <c r="N45" t="n">
-        <v>0.1710966987400989</v>
+        <v>0.2513863216266174</v>
       </c>
       <c r="O45" t="n">
-        <v>0.06266329600180764</v>
+        <v>0.0607843137254902</v>
       </c>
       <c r="P45" t="n">
         <v>1</v>
       </c>
       <c r="Q45" t="n">
-        <v>0.3238104168751494</v>
+        <v>0.355699083944977</v>
       </c>
       <c r="R45" t="n">
-        <v>0.4355011995646019</v>
+        <v>0.3657946219569925</v>
       </c>
       <c r="S45" t="n">
-        <v>0.2406883835602487</v>
+        <v>0.2785062940980305</v>
       </c>
       <c r="T45" t="n">
         <v>1</v>
@@ -5030,49 +5044,49 @@
         <v>0</v>
       </c>
       <c r="W45" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X45" t="n">
-        <v>1</v>
+        <v>0.3657946219569925</v>
       </c>
       <c r="Y45" t="n">
-        <v>0.4355011995646019</v>
-      </c>
-      <c r="Z45" t="n">
-        <v>1.57</v>
-      </c>
-      <c r="AA45" t="inlineStr">
+        <v>2</v>
+      </c>
+      <c r="Z45" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
+      <c r="AA45" t="n">
+        <v>-0.2684107560860149</v>
+      </c>
       <c r="AB45" t="n">
-        <v>-0.5548475731290788</v>
+        <v>0.2194767731741955</v>
       </c>
       <c r="AC45" t="n">
-        <v>1.306503598693806</v>
+        <v>0.01009553801201551</v>
       </c>
       <c r="AD45" t="n">
-        <v>0.1116907826894525</v>
+        <v>0</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="1" t="inlineStr">
         <is>
-          <t>rVEQttsC</t>
+          <t>GrDYvKBO</t>
         </is>
       </c>
       <c r="B46" s="2" t="n">
-        <v>45746.66666666666</v>
+        <v>45747.66666666666</v>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>betis</t>
+          <t>celta vigo</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>sevilla</t>
+          <t>las palmas</t>
         </is>
       </c>
       <c r="E46" t="n">
@@ -5092,40 +5106,40 @@
         </is>
       </c>
       <c r="I46" t="n">
-        <v>2</v>
+        <v>1.57</v>
       </c>
       <c r="J46" t="n">
-        <v>3.4</v>
+        <v>4.1</v>
       </c>
       <c r="K46" t="n">
-        <v>3.75</v>
+        <v>5.5</v>
       </c>
       <c r="L46" t="n">
-        <v>0.4713493530499075</v>
+        <v>0.5993833395353783</v>
       </c>
       <c r="M46" t="n">
-        <v>0.2772643253234751</v>
+        <v>0.2295199617245229</v>
       </c>
       <c r="N46" t="n">
-        <v>0.2513863216266174</v>
+        <v>0.1710966987400989</v>
       </c>
       <c r="O46" t="n">
-        <v>0.0607843137254902</v>
+        <v>0.06266329600180764</v>
       </c>
       <c r="P46" t="n">
         <v>1</v>
       </c>
       <c r="Q46" t="n">
-        <v>0.3731435205246508</v>
+        <v>0.3583583538094059</v>
       </c>
       <c r="R46" t="n">
-        <v>0.3529377592733988</v>
+        <v>0.3596472087554723</v>
       </c>
       <c r="S46" t="n">
-        <v>0.2739187202019505</v>
+        <v>0.2819944374351219</v>
       </c>
       <c r="T46" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U46" t="n">
         <v>1</v>
@@ -5134,49 +5148,49 @@
         <v>0</v>
       </c>
       <c r="W46" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X46" t="n">
-        <v>0</v>
+        <v>0.3596472087554723</v>
       </c>
       <c r="Y46" t="n">
-        <v>0.3731435205246508</v>
-      </c>
-      <c r="Z46" t="n">
-        <v>3.4</v>
-      </c>
-      <c r="AA46" t="inlineStr">
+        <v>1.57</v>
+      </c>
+      <c r="Z46" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
+      <c r="AA46" t="n">
+        <v>-0.7637787407963306</v>
+      </c>
       <c r="AB46" t="n">
-        <v>0.1119533207432553</v>
+        <v>0.2157883252532834</v>
       </c>
       <c r="AC46" t="n">
-        <v>7.276298650230689</v>
+        <v>0.001288854946066398</v>
       </c>
       <c r="AD46" t="n">
-        <v>0.02020576125125195</v>
+        <v>0</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="1" t="inlineStr">
         <is>
-          <t>Kjbn1lFr</t>
+          <t>Olz0eud5</t>
         </is>
       </c>
       <c r="B47" s="2" t="n">
-        <v>45745.51041666666</v>
+        <v>45745.60416666666</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>espanyol</t>
+          <t>alaves</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>atl  madrid</t>
+          <t>rayo vallecano</t>
         </is>
       </c>
       <c r="E47" t="n">
@@ -5196,40 +5210,40 @@
         </is>
       </c>
       <c r="I47" t="n">
-        <v>7</v>
+        <v>2.25</v>
       </c>
       <c r="J47" t="n">
-        <v>4</v>
+        <v>2.9</v>
       </c>
       <c r="K47" t="n">
-        <v>1.5</v>
+        <v>3.6</v>
       </c>
       <c r="L47" t="n">
-        <v>0.1348314606741573</v>
+        <v>0.4165170556552962</v>
       </c>
       <c r="M47" t="n">
-        <v>0.2359550561797753</v>
+        <v>0.3231597845601437</v>
       </c>
       <c r="N47" t="n">
-        <v>0.6292134831460674</v>
+        <v>0.2603231597845602</v>
       </c>
       <c r="O47" t="n">
-        <v>0.05952380952380953</v>
+        <v>0.06704980842911867</v>
       </c>
       <c r="P47" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q47" t="n">
-        <v>0.2499405592723154</v>
+        <v>0.3849332791811567</v>
       </c>
       <c r="R47" t="n">
-        <v>0.1194316176183696</v>
+        <v>0.3289894957515934</v>
       </c>
       <c r="S47" t="n">
-        <v>0.630627823109315</v>
+        <v>0.2860772250672497</v>
       </c>
       <c r="T47" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="U47" t="n">
         <v>1</v>
@@ -5241,46 +5255,46 @@
         <v>0</v>
       </c>
       <c r="X47" t="n">
-        <v>2</v>
+        <v>0.3849332791811567</v>
       </c>
       <c r="Y47" t="n">
-        <v>0.630627823109315</v>
-      </c>
-      <c r="Z47" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="AA47" t="inlineStr">
+        <v>2.9</v>
+      </c>
+      <c r="Z47" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
+      <c r="AA47" t="n">
+        <v>0.0612139524343971</v>
+      </c>
       <c r="AB47" t="n">
-        <v>-0.1081165306720551</v>
+        <v>4.61919935017388</v>
       </c>
       <c r="AC47" t="n">
-        <v>1.891883469327945</v>
+        <v>0.0559437834295633</v>
       </c>
       <c r="AD47" t="n">
-        <v>0.3806872638369996</v>
+        <v>0</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="1" t="inlineStr">
         <is>
-          <t>Olz0eud5</t>
+          <t>f9rqaNdt</t>
         </is>
       </c>
       <c r="B48" s="2" t="n">
-        <v>45745.60416666666</v>
+        <v>45746.375</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>alaves</t>
+          <t>getafe</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>rayo vallecano</t>
+          <t>villarreal</t>
         </is>
       </c>
       <c r="E48" t="n">
@@ -5300,40 +5314,40 @@
         </is>
       </c>
       <c r="I48" t="n">
-        <v>2.25</v>
+        <v>3.1</v>
       </c>
       <c r="J48" t="n">
-        <v>2.9</v>
+        <v>3.2</v>
       </c>
       <c r="K48" t="n">
-        <v>3.6</v>
+        <v>2.35</v>
       </c>
       <c r="L48" t="n">
-        <v>0.4165170556552962</v>
+        <v>0.3041456016177958</v>
       </c>
       <c r="M48" t="n">
-        <v>0.3231597845601437</v>
+        <v>0.2946410515672397</v>
       </c>
       <c r="N48" t="n">
-        <v>0.2603231597845602</v>
+        <v>0.4012133468149647</v>
       </c>
       <c r="O48" t="n">
-        <v>0.06704980842911867</v>
+        <v>0.06061256005490723</v>
       </c>
       <c r="P48" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q48" t="n">
-        <v>0.3459467307060448</v>
+        <v>0.3914287759434801</v>
       </c>
       <c r="R48" t="n">
-        <v>0.2803719958462909</v>
+        <v>0.220564522223485</v>
       </c>
       <c r="S48" t="n">
-        <v>0.3736812734476644</v>
+        <v>0.388006701833035</v>
       </c>
       <c r="T48" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="U48" t="n">
         <v>1</v>
@@ -5345,46 +5359,46 @@
         <v>0</v>
       </c>
       <c r="X48" t="n">
-        <v>2</v>
+        <v>0.3914287759434801</v>
       </c>
       <c r="Y48" t="n">
-        <v>0.3736812734476644</v>
-      </c>
-      <c r="Z48" t="n">
-        <v>3.6</v>
-      </c>
-      <c r="AA48" t="inlineStr">
+        <v>3.2</v>
+      </c>
+      <c r="Z48" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
+      <c r="AA48" t="n">
+        <v>0.1148054922814256</v>
+      </c>
       <c r="AB48" t="n">
-        <v>0.13278945554292</v>
+        <v>4.69714531132176</v>
       </c>
       <c r="AC48" t="n">
-        <v>1.121043820342993</v>
+        <v>0.003422074110445095</v>
       </c>
       <c r="AD48" t="n">
-        <v>0.02773454274161957</v>
+        <v>0</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="1" t="inlineStr">
         <is>
-          <t>f9rqaNdt</t>
+          <t>Kjbn1lFr</t>
         </is>
       </c>
       <c r="B49" s="2" t="n">
-        <v>45746.375</v>
+        <v>45745.51041666666</v>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>getafe</t>
+          <t>espanyol</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>villarreal</t>
+          <t>atl  madrid</t>
         </is>
       </c>
       <c r="E49" t="n">
@@ -5404,37 +5418,37 @@
         </is>
       </c>
       <c r="I49" t="n">
-        <v>3.1</v>
+        <v>7</v>
       </c>
       <c r="J49" t="n">
-        <v>3.2</v>
+        <v>4</v>
       </c>
       <c r="K49" t="n">
-        <v>2.35</v>
+        <v>1.5</v>
       </c>
       <c r="L49" t="n">
-        <v>0.3041456016177958</v>
+        <v>0.1348314606741573</v>
       </c>
       <c r="M49" t="n">
-        <v>0.2946410515672397</v>
+        <v>0.2359550561797753</v>
       </c>
       <c r="N49" t="n">
-        <v>0.4012133468149647</v>
+        <v>0.6292134831460674</v>
       </c>
       <c r="O49" t="n">
-        <v>0.06061256005490723</v>
+        <v>0.05952380952380953</v>
       </c>
       <c r="P49" t="n">
         <v>2</v>
       </c>
       <c r="Q49" t="n">
-        <v>0.344081963617453</v>
+        <v>0.3544226986660331</v>
       </c>
       <c r="R49" t="n">
-        <v>0.2816581465830766</v>
+        <v>0.1183270127597769</v>
       </c>
       <c r="S49" t="n">
-        <v>0.3742598897994704</v>
+        <v>0.52725028857419</v>
       </c>
       <c r="T49" t="n">
         <v>2</v>
@@ -5446,30 +5460,30 @@
         <v>0</v>
       </c>
       <c r="W49" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="X49" t="n">
-        <v>2</v>
+        <v>0.52725028857419</v>
       </c>
       <c r="Y49" t="n">
-        <v>0.3742598897994704</v>
-      </c>
-      <c r="Z49" t="n">
-        <v>2.35</v>
-      </c>
-      <c r="AA49" t="inlineStr">
+        <v>1.5</v>
+      </c>
+      <c r="Z49" t="inlineStr">
         <is>
           <t>dif_prob_mod_bm &gt; 0</t>
         </is>
       </c>
+      <c r="AA49" t="n">
+        <v>-0.41824913427743</v>
+      </c>
       <c r="AB49" t="n">
-        <v>-0.0892513029416626</v>
+        <v>1.25570706761227</v>
       </c>
       <c r="AC49" t="n">
-        <v>1.122779669398411</v>
+        <v>0.1728275899081569</v>
       </c>
       <c r="AD49" t="n">
-        <v>0.03017792618201742</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Arreglo error en estrategia: mejoro espacio m para optimizar las diferencias entre rdos y ligas
</commit_message>
<xml_diff>
--- a/data/predicciones.xlsx
+++ b/data/predicciones.xlsx
@@ -679,7 +679,7 @@
         <v>-0.3956077724944743</v>
       </c>
       <c r="AB2" t="n">
-        <v>1.384703762016951</v>
+        <v>2.307839603361585</v>
       </c>
       <c r="AC2" t="n">
         <v>0.2605014062797683</v>
@@ -781,7 +781,7 @@
         <v>-0.2096818558068686</v>
       </c>
       <c r="AB3" t="n">
-        <v>0.1968528077706222</v>
+        <v>0.3280880129510371</v>
       </c>
       <c r="AC3" t="n">
         <v>0.01264525281074536</v>
@@ -883,7 +883,7 @@
         <v>-0.6924711891409994</v>
       </c>
       <c r="AB4" t="n">
-        <v>1.104483420387402</v>
+        <v>1.84080570064567</v>
       </c>
       <c r="AC4" t="n">
         <v>0.2501720168880496</v>
@@ -985,7 +985,7 @@
         <v>-1.110200891164503</v>
       </c>
       <c r="AB5" t="n">
-        <v>1.03107079218174</v>
+        <v>1.718451320302901</v>
       </c>
       <c r="AC5" t="n">
         <v>0.442785495888043</v>
@@ -1087,7 +1087,7 @@
         <v>-0.003753402192218457</v>
       </c>
       <c r="AB6" t="n">
-        <v>1.788526780459037</v>
+        <v>2.980877967431729</v>
       </c>
       <c r="AC6" t="n">
         <v>0.3091737042300292</v>
@@ -1189,7 +1189,7 @@
         <v>-0.4403334804018602</v>
       </c>
       <c r="AB7" t="n">
-        <v>1.382900742899112</v>
+        <v>2.30483457149852</v>
       </c>
       <c r="AC7" t="n">
         <v>0.2745670979885088</v>
@@ -1291,7 +1291,7 @@
         <v>0.04387069859885367</v>
       </c>
       <c r="AB8" t="n">
-        <v>0.8701931177581659</v>
+        <v>0.6526448383186246</v>
       </c>
       <c r="AC8" t="n">
         <v>0.01098133135658386</v>
@@ -1393,7 +1393,7 @@
         <v>0.1612147716348363</v>
       </c>
       <c r="AB9" t="n">
-        <v>5.080021865987399</v>
+        <v>3.81001639949055</v>
       </c>
       <c r="AC9" t="n">
         <v>0.1290739839239984</v>
@@ -1495,7 +1495,7 @@
         <v>-0.2131237548269221</v>
       </c>
       <c r="AB10" t="n">
-        <v>6.428616829683764</v>
+        <v>4.821462622262824</v>
       </c>
       <c r="AC10" t="n">
         <v>0.2472580489029609</v>
@@ -1597,7 +1597,7 @@
         <v>-0.2770008588085357</v>
       </c>
       <c r="AB11" t="n">
-        <v>3.513696403513295</v>
+        <v>2.342464269008864</v>
       </c>
       <c r="AC11" t="n">
         <v>0.1773809508786305</v>
@@ -1699,7 +1699,7 @@
         <v>-0.2085127038388074</v>
       </c>
       <c r="AB12" t="n">
-        <v>3.31666159989541</v>
+        <v>2.211107733263607</v>
       </c>
       <c r="AC12" t="n">
         <v>0.08497930807890619</v>
@@ -1801,7 +1801,7 @@
         <v>0.1673278790077244</v>
       </c>
       <c r="AB13" t="n">
-        <v>1.159356364122338</v>
+        <v>1.932260606870564</v>
       </c>
       <c r="AC13" t="n">
         <v>0.06570228094077013</v>
@@ -1905,7 +1905,7 @@
         <v>0.179094086519328</v>
       </c>
       <c r="AB14" t="n">
-        <v>6.169892696096452</v>
+        <v>4.62741952207234</v>
       </c>
       <c r="AC14" t="n">
         <v>0.222410133437013</v>
@@ -2009,7 +2009,7 @@
         <v>0.4188484248110894</v>
       </c>
       <c r="AB15" t="n">
-        <v>9.384817911649902</v>
+        <v>7.038613433737428</v>
       </c>
       <c r="AC15" t="n">
         <v>0.6646198275730887</v>
@@ -2113,7 +2113,7 @@
         <v>-0.0680638475955834</v>
       </c>
       <c r="AB16" t="n">
-        <v>10.07133087058614</v>
+        <v>7.553498152939603</v>
       </c>
       <c r="AC16" t="n">
         <v>0.7650081265407377</v>
@@ -2217,7 +2217,7 @@
         <v>0.4122234541041349</v>
       </c>
       <c r="AB17" t="n">
-        <v>6.667003046993615</v>
+        <v>5.000252285245211</v>
       </c>
       <c r="AC17" t="n">
         <v>0.3059128952686548</v>
@@ -2319,7 +2319,7 @@
         <v>-0.1556831328992195</v>
       </c>
       <c r="AB18" t="n">
-        <v>4.973713179303114</v>
+        <v>3.730284884477335</v>
       </c>
       <c r="AC18" t="n">
         <v>0.08566186584653268</v>
@@ -2421,7 +2421,7 @@
         <v>0.2977657585542399</v>
       </c>
       <c r="AB19" t="n">
-        <v>6.877820827101515</v>
+        <v>5.158365620326137</v>
       </c>
       <c r="AC19" t="n">
         <v>0.2929485275380173</v>
@@ -2523,7 +2523,7 @@
         <v>-0.02284000144402813</v>
       </c>
       <c r="AB20" t="n">
-        <v>2.320828623112449</v>
+        <v>3.868047705187416</v>
       </c>
       <c r="AC20" t="n">
         <v>0.6113133678474076</v>
@@ -2623,7 +2623,7 @@
         <v>0.1909744195833094</v>
       </c>
       <c r="AB21" t="n">
-        <v>2.701937944057009</v>
+        <v>4.503229906761682</v>
       </c>
       <c r="AC21" t="n">
         <v>0.8256672270830573</v>
@@ -2723,7 +2723,7 @@
         <v>0.1455039670734701</v>
       </c>
       <c r="AB22" t="n">
-        <v>1.527357900701087</v>
+        <v>2.545596501168478</v>
       </c>
       <c r="AC22" t="n">
         <v>0.2049859611591311</v>
@@ -2823,7 +2823,7 @@
         <v>-0.1744472087845206</v>
       </c>
       <c r="AB23" t="n">
-        <v>1.471766500488131</v>
+        <v>2.452944167480218</v>
       </c>
       <c r="AC23" t="n">
         <v>0.2473442706888411</v>
@@ -2925,7 +2925,7 @@
         <v>-0.1866124893064383</v>
       </c>
       <c r="AB24" t="n">
-        <v>1.106569287752813</v>
+        <v>1.844282146254688</v>
       </c>
       <c r="AC24" t="n">
         <v>0.03813939040308317</v>
@@ -3027,7 +3027,7 @@
         <v>0.3197182078221008</v>
       </c>
       <c r="AB25" t="n">
-        <v>2.159651903780242</v>
+        <v>3.599419839633737</v>
       </c>
       <c r="AC25" t="n">
         <v>0.5506784616981166</v>
@@ -3127,7 +3127,7 @@
         <v>0.2602713994210298</v>
       </c>
       <c r="AB26" t="n">
-        <v>5.459241847512263</v>
+        <v>4.094431385634198</v>
       </c>
       <c r="AC26" t="n">
         <v>0.09499876507328531</v>
@@ -3227,7 +3227,7 @@
         <v>0.1989442271565266</v>
       </c>
       <c r="AB27" t="n">
-        <v>4.950709198977434</v>
+        <v>3.713031899233076</v>
       </c>
       <c r="AC27" t="n">
         <v>0.09581271511068973</v>
@@ -3327,7 +3327,7 @@
         <v>-0.05438966060929866</v>
       </c>
       <c r="AB28" t="n">
-        <v>4.835590599165041</v>
+        <v>3.223727066110028</v>
       </c>
       <c r="AC28" t="n">
         <v>0.0509843071978795</v>
@@ -3427,7 +3427,7 @@
         <v>0.07394378153454376</v>
       </c>
       <c r="AB29" t="n">
-        <v>1.827709180092862</v>
+        <v>3.046181966821436</v>
       </c>
       <c r="AC29" t="n">
         <v>0.3279189310629804</v>
@@ -3527,7 +3527,7 @@
         <v>-0.1450756947532118</v>
       </c>
       <c r="AB30" t="n">
-        <v>1.652081151183328</v>
+        <v>2.753468585305548</v>
       </c>
       <c r="AC30" t="n">
         <v>0.2890948059640486</v>
@@ -3627,7 +3627,7 @@
         <v>-0.3570114524737107</v>
       </c>
       <c r="AB31" t="n">
-        <v>1.125303726745403</v>
+        <v>1.875506211242339</v>
       </c>
       <c r="AC31" t="n">
         <v>0.032470168263524</v>
@@ -3727,7 +3727,7 @@
         <v>-0.1063247283516979</v>
       </c>
       <c r="AB32" t="n">
-        <v>1.911133270885033</v>
+        <v>3.185222118141722</v>
       </c>
       <c r="AC32" t="n">
         <v>0.3988900842851951</v>
@@ -3829,7 +3829,7 @@
         <v>-0.333777837367836</v>
       </c>
       <c r="AB33" t="n">
-        <v>0.9219733906620089</v>
+        <v>1.536622317770015</v>
       </c>
       <c r="AC33" t="n">
         <v>0.02632416652920944</v>
@@ -3931,7 +3931,7 @@
         <v>0.1560115223962476</v>
       </c>
       <c r="AB34" t="n">
-        <v>4.850921130885863</v>
+        <v>6.063651413607328</v>
       </c>
       <c r="AC34" t="n">
         <v>0.03539538923291191</v>
@@ -4031,7 +4031,7 @@
         <v>0.07961794707855407</v>
       </c>
       <c r="AB35" t="n">
-        <v>4.518184602057923</v>
+        <v>5.647730752572405</v>
       </c>
       <c r="AC35" t="n">
         <v>0.04439633633870788</v>
@@ -4131,7 +4131,7 @@
         <v>0.2742297835463348</v>
       </c>
       <c r="AB36" t="n">
-        <v>5.929921826023891</v>
+        <v>7.412402282529865</v>
       </c>
       <c r="AC36" t="n">
         <v>0.1141177850734852</v>
@@ -4233,7 +4233,7 @@
         <v>0.2487232710269768</v>
       </c>
       <c r="AB37" t="n">
-        <v>7.911084032474693</v>
+        <v>5.274056021649796</v>
       </c>
       <c r="AC37" t="n">
         <v>0.4204796570220136</v>
@@ -4335,7 +4335,7 @@
         <v>0.01819466117218543</v>
       </c>
       <c r="AB38" t="n">
-        <v>6.58680299673313</v>
+        <v>4.391201997822087</v>
       </c>
       <c r="AC38" t="n">
         <v>0.2162498241274949</v>
@@ -4437,7 +4437,7 @@
         <v>-0.4098469458928122</v>
       </c>
       <c r="AB39" t="n">
-        <v>2.049172989979266</v>
+        <v>3.415288316632111</v>
       </c>
       <c r="AC39" t="n">
         <v>0.4525056311666509</v>
@@ -4541,7 +4541,7 @@
         <v>-0.6662077454923365</v>
       </c>
       <c r="AB40" t="n">
-        <v>1.75974009921999</v>
+        <v>2.93290016536665</v>
       </c>
       <c r="AC40" t="n">
         <v>0.3005896217405016</v>
@@ -4645,7 +4645,7 @@
         <v>-0.3727105992881631</v>
       </c>
       <c r="AB41" t="n">
-        <v>2.371810403715586</v>
+        <v>3.953017339525978</v>
       </c>
       <c r="AC41" t="n">
         <v>0.6236012111044408</v>
@@ -4749,7 +4749,7 @@
         <v>-0.6428182192530345</v>
       </c>
       <c r="AB42" t="n">
-        <v>1.952218301106332</v>
+        <v>3.253697168510554</v>
       </c>
       <c r="AC42" t="n">
         <v>0.4127525205040656</v>
@@ -4853,7 +4853,7 @@
         <v>-0.4495114530363442</v>
       </c>
       <c r="AB43" t="n">
-        <v>1.493644960570073</v>
+        <v>2.489408267616789</v>
       </c>
       <c r="AC43" t="n">
         <v>0.1701655201517661</v>
@@ -4957,7 +4957,7 @@
         <v>-0.2465241147924754</v>
       </c>
       <c r="AB44" t="n">
-        <v>0.2169218574052393</v>
+        <v>0.3615364290087321</v>
       </c>
       <c r="AC44" t="n">
         <v>0.005963464098491633</v>
@@ -5061,7 +5061,7 @@
         <v>-0.2684107560860149</v>
       </c>
       <c r="AB45" t="n">
-        <v>0.2194767731741955</v>
+        <v>0.3657946219569925</v>
       </c>
       <c r="AC45" t="n">
         <v>0.01009553801201551</v>
@@ -5165,7 +5165,7 @@
         <v>-0.7637787407963306</v>
       </c>
       <c r="AB46" t="n">
-        <v>0.2157883252532834</v>
+        <v>0.3596472087554723</v>
       </c>
       <c r="AC46" t="n">
         <v>0.001288854946066398</v>
@@ -5269,7 +5269,7 @@
         <v>0.0612139524343971</v>
       </c>
       <c r="AB47" t="n">
-        <v>4.61919935017388</v>
+        <v>5.773999187717351</v>
       </c>
       <c r="AC47" t="n">
         <v>0.0559437834295633</v>
@@ -5373,7 +5373,7 @@
         <v>0.1148054922814256</v>
       </c>
       <c r="AB48" t="n">
-        <v>4.69714531132176</v>
+        <v>5.871431639152202</v>
       </c>
       <c r="AC48" t="n">
         <v>0.003422074110445095</v>
@@ -5477,7 +5477,7 @@
         <v>-0.41824913427743</v>
       </c>
       <c r="AB49" t="n">
-        <v>1.25570706761227</v>
+        <v>2.092845112687117</v>
       </c>
       <c r="AC49" t="n">
         <v>0.1728275899081569</v>

</xml_diff>

<commit_message>
DATA. Actualizo preds al usar k mayores en kelly_linear
</commit_message>
<xml_diff>
--- a/data/predicciones.xlsx
+++ b/data/predicciones.xlsx
@@ -679,7 +679,7 @@
         <v>-0.4522230730949388</v>
       </c>
       <c r="AB2" t="n">
-        <v>2.843721056088348</v>
+        <v>1.497672187291312</v>
       </c>
       <c r="AC2" t="n">
         <v>0.2779934092243338</v>
@@ -781,7 +781,7 @@
         <v>-0.1123184112210562</v>
       </c>
       <c r="AB3" t="n">
-        <v>2.190427287064541</v>
+        <v>1.933300421197954</v>
       </c>
       <c r="AC3" t="n">
         <v>0.01845893504897511</v>
@@ -883,7 +883,7 @@
         <v>-0.8444402950095776</v>
       </c>
       <c r="AB4" t="n">
-        <v>1.922962769693028</v>
+        <v>0.4705368329654742</v>
       </c>
       <c r="AC4" t="n">
         <v>0.1879813249933843</v>
@@ -985,7 +985,7 @@
         <v>-0.6893268898722044</v>
       </c>
       <c r="AB5" t="n">
-        <v>3.001151926665969</v>
+        <v>1.008051842867319</v>
       </c>
       <c r="AC5" t="n">
         <v>0.4860377534518934</v>
@@ -1189,7 +1189,7 @@
         <v>-0.5543004765305417</v>
       </c>
       <c r="AB7" t="n">
-        <v>2.684362603413351</v>
+        <v>1.172521400278644</v>
       </c>
       <c r="AC7" t="n">
         <v>0.2747811998569986</v>
@@ -1291,7 +1291,7 @@
         <v>-0.1653362378229074</v>
       </c>
       <c r="AB8" t="n">
-        <v>3.101951407991768</v>
+        <v>2.559124941453109</v>
       </c>
       <c r="AC8" t="n">
         <v>0.244674603163902</v>
@@ -1495,7 +1495,7 @@
         <v>-0.6126601816550009</v>
       </c>
       <c r="AB10" t="n">
-        <v>2.297691763389917</v>
+        <v>0.8975628318991012</v>
       </c>
       <c r="AC10" t="n">
         <v>0.1795266806861472</v>
@@ -1903,7 +1903,7 @@
         <v>-0.1529594544881459</v>
       </c>
       <c r="AB14" t="n">
-        <v>5.806062589399451</v>
+        <v>6.28586901539826</v>
       </c>
       <c r="AC14" t="n">
         <v>0.268890991494271</v>
@@ -2107,7 +2107,7 @@
         <v>-0.005822433351410325</v>
       </c>
       <c r="AB16" t="n">
-        <v>4.67525999193936</v>
+        <v>4.688910387487124</v>
       </c>
       <c r="AC16" t="n">
         <v>0.1016844416236228</v>
@@ -2209,7 +2209,7 @@
         <v>-0.1446886017637856</v>
       </c>
       <c r="AB17" t="n">
-        <v>0.7841192012788571</v>
+        <v>0.8451548978353538</v>
       </c>
       <c r="AC17" t="n">
         <v>0.008564428326145734</v>
@@ -2515,7 +2515,7 @@
         <v>-0.1672641612117348</v>
       </c>
       <c r="AB20" t="n">
-        <v>4.44761380564777</v>
+        <v>4.852494501051068</v>
       </c>
       <c r="AC20" t="n">
         <v>0.1248986729679319</v>
@@ -2717,7 +2717,7 @@
         <v>-0.4177665923133001</v>
       </c>
       <c r="AB22" t="n">
-        <v>4.041015413341344</v>
+        <v>1.695552684281648</v>
       </c>
       <c r="AC22" t="n">
         <v>0.2415296250760163</v>
@@ -2817,7 +2817,7 @@
         <v>0.1274586518543151</v>
       </c>
       <c r="AB23" t="n">
-        <v>8.73220487876268</v>
+        <v>6.549153659072011</v>
       </c>
       <c r="AC23" t="n">
         <v>0.786593546779856</v>
@@ -2919,7 +2919,7 @@
         <v>-0.1690749038168054</v>
       </c>
       <c r="AB24" t="n">
-        <v>3.43081539632013</v>
+        <v>2.112325255153518</v>
       </c>
       <c r="AC24" t="n">
         <v>0.05910005988735212</v>
@@ -3021,7 +3021,7 @@
         <v>-0.3942435526577809</v>
       </c>
       <c r="AB25" t="n">
-        <v>4.06939313077707</v>
+        <v>1.777748311350294</v>
       </c>
       <c r="AC25" t="n">
         <v>0.1977079044008937</v>
@@ -3121,7 +3121,7 @@
         <v>-0.46218505579608</v>
       </c>
       <c r="AB26" t="n">
-        <v>0.5412710180149227</v>
+        <v>0.2100401555744404</v>
       </c>
       <c r="AC26" t="n">
         <v>0.005330944851409503</v>
@@ -3221,7 +3221,7 @@
         <v>-0.03753817713866209</v>
       </c>
       <c r="AB27" t="n">
-        <v>5.516442267551487</v>
+        <v>3.979294721921052</v>
       </c>
       <c r="AC27" t="n">
         <v>0.2873589778225264</v>
@@ -3423,7 +3423,7 @@
         <v>-0.1461742799462329</v>
       </c>
       <c r="AB29" t="n">
-        <v>4.60562543004037</v>
+        <v>4.968083273371607</v>
       </c>
       <c r="AC29" t="n">
         <v>0.0879547381611579</v>
@@ -3835,7 +3835,7 @@
         <v>-0.0609817196676492</v>
       </c>
       <c r="AB33" t="n">
-        <v>3.916488043301961</v>
+        <v>3.671133993291387</v>
       </c>
       <c r="AC33" t="n">
         <v>0.4392895389443506</v>
@@ -4147,7 +4147,7 @@
         <v>-0.001901181566260279</v>
       </c>
       <c r="AB36" t="n">
-        <v>2.541569685554988</v>
+        <v>2.536733121448104</v>
       </c>
       <c r="AC36" t="n">
         <v>0.07359318607602722</v>
@@ -4251,7 +4251,7 @@
         <v>-0.3720149336203384</v>
       </c>
       <c r="AB37" t="n">
-        <v>8.887011313384896</v>
+        <v>5.373872831346219</v>
       </c>
       <c r="AC37" t="n">
         <v>0.2879200760493381</v>
@@ -4459,7 +4459,7 @@
         <v>-0.01758740211824121</v>
       </c>
       <c r="AB39" t="n">
-        <v>12.99143624405273</v>
+        <v>12.76100084486951</v>
       </c>
       <c r="AC39" t="n">
         <v>0.4970650919578923</v>
@@ -4561,7 +4561,7 @@
         <v>-0.04526671210027725</v>
       </c>
       <c r="AB40" t="n">
-        <v>3.174880104583876</v>
+        <v>3.101445948898677</v>
       </c>
       <c r="AC40" t="n">
         <v>0.194743624708684</v>
@@ -4765,7 +4765,7 @@
         <v>-0.2795864873003509</v>
       </c>
       <c r="AB42" t="n">
-        <v>2.321203013522265</v>
+        <v>1.960983802680679</v>
       </c>
       <c r="AC42" t="n">
         <v>0.06073194702341472</v>
@@ -4865,7 +4865,7 @@
         <v>-0.1075199548117138</v>
       </c>
       <c r="AB43" t="n">
-        <v>0.4302849314061695</v>
+        <v>0.4060039333803053</v>
       </c>
       <c r="AC43" t="n">
         <v>0.005046800677886043</v>
@@ -5369,7 +5369,7 @@
         <v>-0.06924537525887162</v>
       </c>
       <c r="AB48" t="n">
-        <v>6.30610595752344</v>
+        <v>6.532177161322579</v>
       </c>
       <c r="AC48" t="n">
         <v>0.389204583300794</v>
@@ -5575,7 +5575,7 @@
         <v>-0.4405336659979874</v>
       </c>
       <c r="AB50" t="n">
-        <v>1.991547544656338</v>
+        <v>2.542744241916944</v>
       </c>
       <c r="AC50" t="n">
         <v>0.06502561889981995</v>
@@ -5679,7 +5679,7 @@
         <v>-0.5251274822668059</v>
       </c>
       <c r="AB51" t="n">
-        <v>2.88768179434954</v>
+        <v>3.884905690093769</v>
       </c>
       <c r="AC51" t="n">
         <v>0.3611339389394195</v>
@@ -5783,7 +5783,7 @@
         <v>-0.4162602791483861</v>
       </c>
       <c r="AB52" t="n">
-        <v>3.030342264239372</v>
+        <v>3.812595534074336</v>
       </c>
       <c r="AC52" t="n">
         <v>0.3420192677967054</v>
@@ -6095,7 +6095,7 @@
         <v>-0.02349035084089116</v>
       </c>
       <c r="AB55" t="n">
-        <v>2.603468912561273</v>
+        <v>2.541622692379286</v>
       </c>
       <c r="AC55" t="n">
         <v>0.09050191552934528</v>
@@ -6303,7 +6303,7 @@
         <v>-0.05726200646087507</v>
       </c>
       <c r="AB57" t="n">
-        <v>3.030645165917577</v>
+        <v>2.852623365230276</v>
       </c>
       <c r="AC57" t="n">
         <v>0.168988514450316</v>

</xml_diff>

<commit_message>
DATA. Actualizo predicciones de GER tras cambio de modelo (385 --> 766)
</commit_message>
<xml_diff>
--- a/data/predicciones.xlsx
+++ b/data/predicciones.xlsx
@@ -644,13 +644,13 @@
         <v>1</v>
       </c>
       <c r="Q2" t="n">
-        <v>0.2609309121395115</v>
+        <v>0.2973816159856481</v>
       </c>
       <c r="R2" t="n">
-        <v>0.579939152490989</v>
+        <v>0.5342883520978339</v>
       </c>
       <c r="S2" t="n">
-        <v>0.1591299353694995</v>
+        <v>0.168330031916518</v>
       </c>
       <c r="T2" t="n">
         <v>1</v>
@@ -668,7 +668,7 @@
         <v>1</v>
       </c>
       <c r="Y2" t="n">
-        <v>0.579939152490989</v>
+        <v>0.5342883520978339</v>
       </c>
       <c r="Z2" t="n">
         <v>1.44</v>
@@ -679,13 +679,13 @@
         </is>
       </c>
       <c r="AB2" t="n">
-        <v>-0.3747445918476724</v>
+        <v>-0.5241472113161803</v>
       </c>
       <c r="AC2" t="n">
-        <v>1.422166262746738</v>
+        <v>0.918273889523</v>
       </c>
       <c r="AD2" t="n">
-        <v>0.3190082403514775</v>
+        <v>0.2369067361121858</v>
       </c>
     </row>
     <row r="3">
@@ -748,13 +748,13 @@
         <v>1</v>
       </c>
       <c r="Q3" t="n">
-        <v>0.4086776642734851</v>
+        <v>0.3413160817386151</v>
       </c>
       <c r="R3" t="n">
-        <v>0.4463057839247925</v>
+        <v>0.4773221847280554</v>
       </c>
       <c r="S3" t="n">
-        <v>0.1450165518017225</v>
+        <v>0.1813617335333296</v>
       </c>
       <c r="T3" t="n">
         <v>1</v>
@@ -772,7 +772,7 @@
         <v>1</v>
       </c>
       <c r="Y3" t="n">
-        <v>0.4463057839247925</v>
+        <v>0.4773221847280554</v>
       </c>
       <c r="Z3" t="n">
         <v>1.55</v>
@@ -783,32 +783,32 @@
         </is>
       </c>
       <c r="AB3" t="n">
-        <v>-0.5604109725755847</v>
+        <v>-0.4730011157663891</v>
       </c>
       <c r="AC3" t="n">
-        <v>0.7003978392255046</v>
+        <v>0.9299089364327014</v>
       </c>
       <c r="AD3" t="n">
-        <v>0.03762811965130736</v>
+        <v>0.1360061029894403</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>WQoQzYhm</t>
+          <t>t0yAzPb4</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>45751.64583333334</v>
+        <v>45753.4375</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>augsburg</t>
+          <t>st  pauli</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>bayern munich</t>
+          <t>b  monchengladbach</t>
         </is>
       </c>
       <c r="E4" t="n">
@@ -828,37 +828,37 @@
         </is>
       </c>
       <c r="I4" t="n">
-        <v>7.5</v>
+        <v>2.5</v>
       </c>
       <c r="J4" t="n">
-        <v>4.75</v>
+        <v>3.4</v>
       </c>
       <c r="K4" t="n">
-        <v>1.4</v>
+        <v>2.75</v>
       </c>
       <c r="L4" t="n">
-        <v>0.1260066319279962</v>
+        <v>0.3781597573306371</v>
       </c>
       <c r="M4" t="n">
-        <v>0.1989578398863098</v>
+        <v>0.2780586450960567</v>
       </c>
       <c r="N4" t="n">
-        <v>0.6750355281856941</v>
+        <v>0.3437815975733064</v>
       </c>
       <c r="O4" t="n">
-        <v>0.05814536340852117</v>
+        <v>0.05775401069518704</v>
       </c>
       <c r="P4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q4" t="n">
-        <v>0.5524860159046925</v>
+        <v>0.3825182376935461</v>
       </c>
       <c r="R4" t="n">
-        <v>0.03223276688774225</v>
+        <v>0.2662772265261987</v>
       </c>
       <c r="S4" t="n">
-        <v>0.4152812172075652</v>
+        <v>0.3512045357802551</v>
       </c>
       <c r="T4" t="n">
         <v>0</v>
@@ -876,10 +876,10 @@
         <v>0</v>
       </c>
       <c r="Y4" t="n">
-        <v>0.5524860159046925</v>
+        <v>0.3825182376935461</v>
       </c>
       <c r="Z4" t="n">
-        <v>4.75</v>
+        <v>3.4</v>
       </c>
       <c r="AA4" t="inlineStr">
         <is>
@@ -887,32 +887,32 @@
         </is>
       </c>
       <c r="AB4" t="n">
-        <v>0.4331489534792771</v>
+        <v>0.125234170065857</v>
       </c>
       <c r="AC4" t="n">
-        <v>4.507122761327755</v>
+        <v>3.060145901548369</v>
       </c>
       <c r="AD4" t="n">
-        <v>0.1372047986971273</v>
+        <v>0.03131370191329103</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>Kpm1xoUi</t>
+          <t>WQoQzYhm</t>
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>45752.4375</v>
+        <v>45751.64583333334</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>bochum</t>
+          <t>augsburg</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>stuttgart</t>
+          <t>bayern munich</t>
         </is>
       </c>
       <c r="E5" t="n">
@@ -932,37 +932,37 @@
         </is>
       </c>
       <c r="I5" t="n">
-        <v>3.1</v>
+        <v>7.5</v>
       </c>
       <c r="J5" t="n">
-        <v>3.7</v>
+        <v>4.75</v>
       </c>
       <c r="K5" t="n">
-        <v>2.15</v>
+        <v>1.4</v>
       </c>
       <c r="L5" t="n">
-        <v>0.3049060942889996</v>
+        <v>0.1260066319279962</v>
       </c>
       <c r="M5" t="n">
-        <v>0.2554618627826753</v>
+        <v>0.1989578398863098</v>
       </c>
       <c r="N5" t="n">
-        <v>0.439632042928325</v>
+        <v>0.6750355281856941</v>
       </c>
       <c r="O5" t="n">
-        <v>0.05796719450132803</v>
+        <v>0.05814536340852117</v>
       </c>
       <c r="P5" t="n">
         <v>2</v>
       </c>
       <c r="Q5" t="n">
-        <v>0.4075831717551193</v>
+        <v>0.3197492353114755</v>
       </c>
       <c r="R5" t="n">
-        <v>0.1572431887568017</v>
+        <v>0.07953686928066148</v>
       </c>
       <c r="S5" t="n">
-        <v>0.435173639488079</v>
+        <v>0.6007138954078629</v>
       </c>
       <c r="T5" t="n">
         <v>2</v>
@@ -980,10 +980,10 @@
         <v>2</v>
       </c>
       <c r="Y5" t="n">
-        <v>0.435173639488079</v>
+        <v>0.6007138954078629</v>
       </c>
       <c r="Z5" t="n">
-        <v>2.15</v>
+        <v>1.4</v>
       </c>
       <c r="AA5" t="inlineStr">
         <is>
@@ -991,19 +991,19 @@
         </is>
       </c>
       <c r="AB5" t="n">
-        <v>-0.05597971747880885</v>
+        <v>-0.39750136607248</v>
       </c>
       <c r="AC5" t="n">
-        <v>3.882253576348609</v>
+        <v>2.281812600594532</v>
       </c>
       <c r="AD5" t="n">
-        <v>0.02759046773295976</v>
+        <v>0.2809646600963874</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>0reftfVP</t>
+          <t>Kpm1xoUi</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
@@ -1011,12 +1011,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>freiburg</t>
+          <t>bochum</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>dortmund</t>
+          <t>stuttgart</t>
         </is>
       </c>
       <c r="E6" t="n">
@@ -1036,37 +1036,37 @@
         </is>
       </c>
       <c r="I6" t="n">
-        <v>3</v>
+        <v>3.1</v>
       </c>
       <c r="J6" t="n">
-        <v>3.5</v>
+        <v>3.7</v>
       </c>
       <c r="K6" t="n">
-        <v>2.3</v>
+        <v>2.15</v>
       </c>
       <c r="L6" t="n">
-        <v>0.3163064833005893</v>
+        <v>0.3049060942889996</v>
       </c>
       <c r="M6" t="n">
-        <v>0.2711198428290766</v>
+        <v>0.2554618627826753</v>
       </c>
       <c r="N6" t="n">
-        <v>0.4125736738703339</v>
+        <v>0.439632042928325</v>
       </c>
       <c r="O6" t="n">
-        <v>0.0538302277432714</v>
+        <v>0.05796719450132803</v>
       </c>
       <c r="P6" t="n">
         <v>2</v>
       </c>
       <c r="Q6" t="n">
-        <v>0.4062960681576867</v>
+        <v>0.3261352277090944</v>
       </c>
       <c r="R6" t="n">
-        <v>0.1165348707665742</v>
+        <v>0.195921889852938</v>
       </c>
       <c r="S6" t="n">
-        <v>0.4771690610757391</v>
+        <v>0.4779428824379676</v>
       </c>
       <c r="T6" t="n">
         <v>2</v>
@@ -1084,10 +1084,10 @@
         <v>2</v>
       </c>
       <c r="Y6" t="n">
-        <v>0.4771690610757391</v>
+        <v>0.4779428824379676</v>
       </c>
       <c r="Z6" t="n">
-        <v>2.3</v>
+        <v>2.15</v>
       </c>
       <c r="AA6" t="inlineStr">
         <is>
@@ -1095,19 +1095,19 @@
         </is>
       </c>
       <c r="AB6" t="n">
-        <v>0.07499141574938456</v>
+        <v>0.02398017151446125</v>
       </c>
       <c r="AC6" t="n">
-        <v>4.646119805211145</v>
+        <v>3.899007725151841</v>
       </c>
       <c r="AD6" t="n">
-        <v>0.07087299291805249</v>
+        <v>0.1518076547288733</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>CMEaKC86</t>
+          <t>0reftfVP</t>
         </is>
       </c>
       <c r="B7" s="2" t="n">
@@ -1115,12 +1115,12 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>heidenheim</t>
+          <t>freiburg</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>bayer leverkusen</t>
+          <t>dortmund</t>
         </is>
       </c>
       <c r="E7" t="n">
@@ -1140,37 +1140,37 @@
         </is>
       </c>
       <c r="I7" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="J7" t="n">
-        <v>4.75</v>
+        <v>3.5</v>
       </c>
       <c r="K7" t="n">
-        <v>1.42</v>
+        <v>2.3</v>
       </c>
       <c r="L7" t="n">
-        <v>0.1350755982777611</v>
+        <v>0.3163064833005893</v>
       </c>
       <c r="M7" t="n">
-        <v>0.1990587764093321</v>
+        <v>0.2711198428290766</v>
       </c>
       <c r="N7" t="n">
-        <v>0.6658656253129068</v>
+        <v>0.4125736738703339</v>
       </c>
       <c r="O7" t="n">
-        <v>0.05760881075929269</v>
+        <v>0.0538302277432714</v>
       </c>
       <c r="P7" t="n">
         <v>2</v>
       </c>
       <c r="Q7" t="n">
-        <v>0.3683986891075977</v>
+        <v>0.3289785953158937</v>
       </c>
       <c r="R7" t="n">
-        <v>0.05279572358076545</v>
+        <v>0.1879120573865835</v>
       </c>
       <c r="S7" t="n">
-        <v>0.5788055873116369</v>
+        <v>0.4831093472975227</v>
       </c>
       <c r="T7" t="n">
         <v>2</v>
@@ -1188,10 +1188,10 @@
         <v>2</v>
       </c>
       <c r="Y7" t="n">
-        <v>0.5788055873116369</v>
+        <v>0.4831093472975227</v>
       </c>
       <c r="Z7" t="n">
-        <v>1.42</v>
+        <v>2.3</v>
       </c>
       <c r="AA7" t="inlineStr">
         <is>
@@ -1199,32 +1199,32 @@
         </is>
       </c>
       <c r="AB7" t="n">
-        <v>-0.4240382524225612</v>
+        <v>0.0855011529110017</v>
       </c>
       <c r="AC7" t="n">
-        <v>2.467275141127401</v>
+        <v>3.941155201637685</v>
       </c>
       <c r="AD7" t="n">
-        <v>0.2104068982040392</v>
+        <v>0.154130751981629</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
         <is>
-          <t>KnI7IjwJ</t>
+          <t>CMEaKC86</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>45752.5625</v>
+        <v>45752.4375</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>werder bremen</t>
+          <t>heidenheim</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>eintracht frankfurt</t>
+          <t>bayer leverkusen</t>
         </is>
       </c>
       <c r="E8" t="n">
@@ -1244,37 +1244,37 @@
         </is>
       </c>
       <c r="I8" t="n">
-        <v>2.63</v>
+        <v>7</v>
       </c>
       <c r="J8" t="n">
-        <v>3.6</v>
+        <v>4.75</v>
       </c>
       <c r="K8" t="n">
-        <v>2.45</v>
+        <v>1.42</v>
       </c>
       <c r="L8" t="n">
-        <v>0.3566302084386309</v>
+        <v>0.1350755982777611</v>
       </c>
       <c r="M8" t="n">
-        <v>0.2605381800537775</v>
+        <v>0.1990587764093321</v>
       </c>
       <c r="N8" t="n">
-        <v>0.3828316115075915</v>
+        <v>0.6658656253129068</v>
       </c>
       <c r="O8" t="n">
-        <v>0.06616917996602956</v>
+        <v>0.05760881075929269</v>
       </c>
       <c r="P8" t="n">
         <v>2</v>
       </c>
       <c r="Q8" t="n">
-        <v>0.2609138327199742</v>
+        <v>0.2593466547829721</v>
       </c>
       <c r="R8" t="n">
-        <v>0.3401714555840494</v>
+        <v>0.09474647352787516</v>
       </c>
       <c r="S8" t="n">
-        <v>0.3989147116959765</v>
+        <v>0.6459068716891527</v>
       </c>
       <c r="T8" t="n">
         <v>2</v>
@@ -1292,10 +1292,10 @@
         <v>2</v>
       </c>
       <c r="Y8" t="n">
-        <v>0.3989147116959765</v>
+        <v>0.6459068716891527</v>
       </c>
       <c r="Z8" t="n">
-        <v>2.45</v>
+        <v>1.42</v>
       </c>
       <c r="AA8" t="inlineStr">
         <is>
@@ -1303,32 +1303,32 @@
         </is>
       </c>
       <c r="AB8" t="n">
-        <v>-0.01562686644472937</v>
+        <v>-0.1971720052414361</v>
       </c>
       <c r="AC8" t="n">
-        <v>3.79314013413435</v>
+        <v>3.754724517084861</v>
       </c>
       <c r="AD8" t="n">
-        <v>0.0587432561119271</v>
+        <v>0.3865602169061806</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
         <is>
-          <t>t0yAzPb4</t>
+          <t>KnI7IjwJ</t>
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>45753.4375</v>
+        <v>45752.5625</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>st  pauli</t>
+          <t>werder bremen</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>b  monchengladbach</t>
+          <t>eintracht frankfurt</t>
         </is>
       </c>
       <c r="E9" t="n">
@@ -1348,37 +1348,37 @@
         </is>
       </c>
       <c r="I9" t="n">
-        <v>2.5</v>
+        <v>2.63</v>
       </c>
       <c r="J9" t="n">
-        <v>3.4</v>
+        <v>3.6</v>
       </c>
       <c r="K9" t="n">
-        <v>2.75</v>
+        <v>2.45</v>
       </c>
       <c r="L9" t="n">
-        <v>0.3781597573306371</v>
+        <v>0.3566302084386309</v>
       </c>
       <c r="M9" t="n">
-        <v>0.2780586450960567</v>
+        <v>0.2605381800537775</v>
       </c>
       <c r="N9" t="n">
-        <v>0.3437815975733064</v>
+        <v>0.3828316115075915</v>
       </c>
       <c r="O9" t="n">
-        <v>0.05775401069518704</v>
+        <v>0.06616917996602956</v>
       </c>
       <c r="P9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q9" t="n">
-        <v>0.3137310840705893</v>
+        <v>0.2716321796904092</v>
       </c>
       <c r="R9" t="n">
-        <v>0.2748543377004632</v>
+        <v>0.3130600070742627</v>
       </c>
       <c r="S9" t="n">
-        <v>0.4114145782289474</v>
+        <v>0.4153078132353282</v>
       </c>
       <c r="T9" t="n">
         <v>2</v>
@@ -1396,10 +1396,10 @@
         <v>2</v>
       </c>
       <c r="Y9" t="n">
-        <v>0.4114145782289474</v>
+        <v>0.4153078132353282</v>
       </c>
       <c r="Z9" t="n">
-        <v>2.75</v>
+        <v>2.45</v>
       </c>
       <c r="AA9" t="inlineStr">
         <is>
@@ -1407,13 +1407,13 @@
         </is>
       </c>
       <c r="AB9" t="n">
-        <v>0.07508005150263168</v>
+        <v>0.01207182236314074</v>
       </c>
       <c r="AC9" t="n">
-        <v>4.005878788018698</v>
+        <v>3.388037423761888</v>
       </c>
       <c r="AD9" t="n">
-        <v>0.09768349415835814</v>
+        <v>0.1022478061610654</v>
       </c>
     </row>
     <row r="10">
@@ -1476,13 +1476,13 @@
         <v>1</v>
       </c>
       <c r="Q10" t="n">
-        <v>0.3189173343466405</v>
+        <v>0.3140662255919414</v>
       </c>
       <c r="R10" t="n">
-        <v>0.3379507824606586</v>
+        <v>0.221667807517742</v>
       </c>
       <c r="S10" t="n">
-        <v>0.3431318831927009</v>
+        <v>0.4642659668903166</v>
       </c>
       <c r="T10" t="n">
         <v>2</v>
@@ -1500,7 +1500,7 @@
         <v>2</v>
       </c>
       <c r="Y10" t="n">
-        <v>0.3431318831927009</v>
+        <v>0.4642659668903166</v>
       </c>
       <c r="Z10" t="n">
         <v>2.9</v>
@@ -1511,13 +1511,13 @@
         </is>
       </c>
       <c r="AB10" t="n">
-        <v>-0.002588178284824891</v>
+        <v>0.1823006863062727</v>
       </c>
       <c r="AC10" t="n">
-        <v>0.6656100592432027</v>
+        <v>3.787432887789425</v>
       </c>
       <c r="AD10" t="n">
-        <v>0.005181100732042365</v>
+        <v>0.1501997412983753</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
DATA. Cambio modelo de GER (habia quedado mal en df_best)
</commit_message>
<xml_diff>
--- a/data/predicciones.xlsx
+++ b/data/predicciones.xlsx
@@ -1410,7 +1410,7 @@
         <v>0.2181414715230612</v>
       </c>
       <c r="AC9" t="n">
-        <v>2.870574502439178</v>
+        <v>2.152930876829384</v>
       </c>
       <c r="AD9" t="n">
         <v>0.02039203374120091</v>
@@ -1514,7 +1514,7 @@
         <v>0.1294561590032969</v>
       </c>
       <c r="AC10" t="n">
-        <v>2.836372280374805</v>
+        <v>2.127279210281103</v>
       </c>
       <c r="AD10" t="n">
         <v>0.01065953608682491</v>
@@ -1618,7 +1618,7 @@
         <v>0.04477680918768312</v>
       </c>
       <c r="AC11" t="n">
-        <v>10.22388404593842</v>
+        <v>7.667913034453812</v>
       </c>
       <c r="AD11" t="n">
         <v>0.4296933336337196</v>
@@ -1722,7 +1722,7 @@
         <v>-0.3565116701014128</v>
       </c>
       <c r="AC12" t="n">
-        <v>7.612627529065554</v>
+        <v>5.709470646799165</v>
       </c>
       <c r="AD12" t="n">
         <v>0.1579405226803096</v>
@@ -1826,7 +1826,7 @@
         <v>0.128867082352362</v>
       </c>
       <c r="AC13" t="n">
-        <v>5.953619701351452</v>
+        <v>4.465214776013589</v>
       </c>
       <c r="AD13" t="n">
         <v>0.02279886174872864</v>
@@ -1928,7 +1928,7 @@
         <v>-0.6768180167150881</v>
       </c>
       <c r="AC14" t="n">
-        <v>0.1074764499327121</v>
+        <v>0.08060733744953405</v>
       </c>
       <c r="AD14" t="n">
         <v>0.01451845683041503</v>
@@ -2030,7 +2030,7 @@
         <v>0.1775989859127432</v>
       </c>
       <c r="AC15" t="n">
-        <v>1.773091374342254</v>
+        <v>1.32981853075669</v>
       </c>
       <c r="AD15" t="n">
         <v>0.06646728404152824</v>
@@ -2132,7 +2132,7 @@
         <v>0.1300939305302405</v>
       </c>
       <c r="AC16" t="n">
-        <v>1.771658236663027</v>
+        <v>1.32874367749727</v>
       </c>
       <c r="AD16" t="n">
         <v>0.04752470408725545</v>
@@ -2234,7 +2234,7 @@
         <v>0.1230533596581917</v>
       </c>
       <c r="AC17" t="n">
-        <v>1.649923418889123</v>
+        <v>1.237442564166842</v>
       </c>
       <c r="AD17" t="n">
         <v>0.01377646883827305</v>
@@ -2336,7 +2336,7 @@
         <v>0.09525034668864966</v>
       </c>
       <c r="AC18" t="n">
-        <v>5.271139460543722</v>
+        <v>3.953354595407792</v>
       </c>
       <c r="AD18" t="n">
         <v>0.09588935809318022</v>
@@ -2438,7 +2438,7 @@
         <v>-0.05783094195888888</v>
       </c>
       <c r="AC19" t="n">
-        <v>5.210201395798761</v>
+        <v>3.90765104684907</v>
       </c>
       <c r="AD19" t="n">
         <v>0.05599627264749391</v>
@@ -2540,7 +2540,7 @@
         <v>-0.0024521523977028</v>
       </c>
       <c r="AC20" t="n">
-        <v>5.985287085613783</v>
+        <v>4.488965314210337</v>
       </c>
       <c r="AD20" t="n">
         <v>0.1717157879412299</v>
@@ -2642,7 +2642,7 @@
         <v>-0.2064455292174335</v>
       </c>
       <c r="AC21" t="n">
-        <v>4.761326824695399</v>
+        <v>3.570995118521549</v>
       </c>
       <c r="AD21" t="n">
         <v>0.04203889064596927</v>
@@ -2651,20 +2651,20 @@
     <row r="22">
       <c r="A22" s="1" t="inlineStr">
         <is>
-          <t>KSgVuKzp</t>
+          <t>ERlHY2TG</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
-        <v>45758.64583333334</v>
+        <v>45759.4375</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>wolfsburg</t>
+          <t>bayer leverkusen</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>rb leipzig</t>
+          <t>union berlin</t>
         </is>
       </c>
       <c r="E22" t="n">
@@ -2684,37 +2684,37 @@
         </is>
       </c>
       <c r="I22" t="n">
-        <v>2.55</v>
+        <v>1.33</v>
       </c>
       <c r="J22" t="n">
-        <v>3.7</v>
+        <v>4.75</v>
       </c>
       <c r="K22" t="n">
-        <v>2.55</v>
+        <v>10</v>
       </c>
       <c r="L22" t="n">
-        <v>0.371859296482412</v>
+        <v>0.7077140835102618</v>
       </c>
       <c r="M22" t="n">
-        <v>0.2562814070351758</v>
+        <v>0.1981599433828733</v>
       </c>
       <c r="N22" t="n">
-        <v>0.371859296482412</v>
+        <v>0.09412597310686482</v>
       </c>
       <c r="O22" t="n">
-        <v>0.05458399576046657</v>
+        <v>0.06240601503759402</v>
       </c>
       <c r="P22" t="n">
         <v>1</v>
       </c>
       <c r="Q22" t="n">
-        <v>0.3244657578962132</v>
+        <v>0.1077393480138757</v>
       </c>
       <c r="R22" t="n">
-        <v>0.3658542789384599</v>
+        <v>0.8337157833209778</v>
       </c>
       <c r="S22" t="n">
-        <v>0.309679963165327</v>
+        <v>0.05854486866514639</v>
       </c>
       <c r="T22" t="n">
         <v>1</v>
@@ -2722,7 +2722,9 @@
       <c r="U22" t="n">
         <v>1</v>
       </c>
-      <c r="V22" t="inlineStr"/>
+      <c r="V22" t="n">
+        <v>0</v>
+      </c>
       <c r="W22" t="n">
         <v>0</v>
       </c>
@@ -2730,10 +2732,10 @@
         <v>1</v>
       </c>
       <c r="Y22" t="n">
-        <v>0.3658542789384599</v>
+        <v>0.8337157833209778</v>
       </c>
       <c r="Z22" t="n">
-        <v>2.55</v>
+        <v>1.33</v>
       </c>
       <c r="AA22" t="inlineStr">
         <is>
@@ -2741,32 +2743,32 @@
         </is>
       </c>
       <c r="AB22" t="n">
-        <v>-0.04327199271414665</v>
+        <v>0.3298242176269713</v>
       </c>
       <c r="AC22" t="n">
         <v>0</v>
       </c>
       <c r="AD22" t="n">
-        <v>0.04138852104224666</v>
+        <v>0.7259764353071021</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="1" t="inlineStr">
         <is>
-          <t>ERlHY2TG</t>
+          <t>6PTeRKLj</t>
         </is>
       </c>
       <c r="B23" s="2" t="n">
-        <v>45759.4375</v>
+        <v>45759.5625</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>bayer leverkusen</t>
+          <t>bayern munich</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>union berlin</t>
+          <t>dortmund</t>
         </is>
       </c>
       <c r="E23" t="n">
@@ -2786,37 +2788,37 @@
         </is>
       </c>
       <c r="I23" t="n">
-        <v>1.33</v>
+        <v>1.4</v>
       </c>
       <c r="J23" t="n">
         <v>4.75</v>
       </c>
       <c r="K23" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="L23" t="n">
-        <v>0.7077140835102618</v>
+        <v>0.6690140845070423</v>
       </c>
       <c r="M23" t="n">
-        <v>0.1981599433828733</v>
+        <v>0.1971830985915493</v>
       </c>
       <c r="N23" t="n">
-        <v>0.09412597310686482</v>
+        <v>0.1338028169014084</v>
       </c>
       <c r="O23" t="n">
-        <v>0.06240601503759402</v>
+        <v>0.06766917293233088</v>
       </c>
       <c r="P23" t="n">
         <v>1</v>
       </c>
       <c r="Q23" t="n">
-        <v>0.2817867924331423</v>
+        <v>0.2840145162213724</v>
       </c>
       <c r="R23" t="n">
-        <v>0.5940953964676391</v>
+        <v>0.4981692703980502</v>
       </c>
       <c r="S23" t="n">
-        <v>0.1241178110992186</v>
+        <v>0.2178162133805774</v>
       </c>
       <c r="T23" t="n">
         <v>1</v>
@@ -2824,7 +2826,9 @@
       <c r="U23" t="n">
         <v>1</v>
       </c>
-      <c r="V23" t="inlineStr"/>
+      <c r="V23" t="n">
+        <v>0</v>
+      </c>
       <c r="W23" t="n">
         <v>0</v>
       </c>
@@ -2832,10 +2836,10 @@
         <v>1</v>
       </c>
       <c r="Y23" t="n">
-        <v>0.5940953964676391</v>
+        <v>0.4981692703980502</v>
       </c>
       <c r="Z23" t="n">
-        <v>1.33</v>
+        <v>1.4</v>
       </c>
       <c r="AA23" t="inlineStr">
         <is>
@@ -2843,32 +2847,32 @@
         </is>
       </c>
       <c r="AB23" t="n">
-        <v>-0.635918553630424</v>
+        <v>-0.7564075536068245</v>
       </c>
       <c r="AC23" t="n">
         <v>0</v>
       </c>
       <c r="AD23" t="n">
-        <v>0.3123086040344968</v>
+        <v>0.2141547541766778</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="1" t="inlineStr">
         <is>
-          <t>6PTeRKLj</t>
+          <t>MXBrkODc</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
-        <v>45759.5625</v>
+        <v>45760.52083333334</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>bayern munich</t>
+          <t>eintracht frankfurt</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>dortmund</t>
+          <t>heidenheim</t>
         </is>
       </c>
       <c r="E24" t="n">
@@ -2888,37 +2892,37 @@
         </is>
       </c>
       <c r="I24" t="n">
-        <v>1.4</v>
+        <v>1.67</v>
       </c>
       <c r="J24" t="n">
-        <v>4.75</v>
+        <v>4.5</v>
       </c>
       <c r="K24" t="n">
-        <v>7</v>
+        <v>4.33</v>
       </c>
       <c r="L24" t="n">
-        <v>0.6690140845070423</v>
+        <v>0.5692192187805826</v>
       </c>
       <c r="M24" t="n">
-        <v>0.1971830985915493</v>
+        <v>0.2112435767474606</v>
       </c>
       <c r="N24" t="n">
-        <v>0.1338028169014084</v>
+        <v>0.2195372044719568</v>
       </c>
       <c r="O24" t="n">
-        <v>0.06766917293233088</v>
+        <v>0.05197149964889314</v>
       </c>
       <c r="P24" t="n">
         <v>1</v>
       </c>
       <c r="Q24" t="n">
-        <v>0.3126252589816379</v>
+        <v>0.3040510831780539</v>
       </c>
       <c r="R24" t="n">
-        <v>0.5320924578982763</v>
+        <v>0.5242934950491377</v>
       </c>
       <c r="S24" t="n">
-        <v>0.1552822831200859</v>
+        <v>0.1716554217728083</v>
       </c>
       <c r="T24" t="n">
         <v>1</v>
@@ -2926,7 +2930,9 @@
       <c r="U24" t="n">
         <v>1</v>
       </c>
-      <c r="V24" t="inlineStr"/>
+      <c r="V24" t="n">
+        <v>0</v>
+      </c>
       <c r="W24" t="n">
         <v>0</v>
       </c>
@@ -2934,10 +2940,10 @@
         <v>1</v>
       </c>
       <c r="Y24" t="n">
-        <v>0.5320924578982763</v>
+        <v>0.5242934950491377</v>
       </c>
       <c r="Z24" t="n">
-        <v>1.4</v>
+        <v>1.67</v>
       </c>
       <c r="AA24" t="inlineStr">
         <is>
@@ -2945,32 +2951,32 @@
         </is>
       </c>
       <c r="AB24" t="n">
-        <v>-0.6376763973560333</v>
+        <v>-0.1857162138327464</v>
       </c>
       <c r="AC24" t="n">
         <v>0</v>
       </c>
       <c r="AD24" t="n">
-        <v>0.2194671989166384</v>
+        <v>0.2202424118710838</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="1" t="inlineStr">
         <is>
-          <t>AgrQWtbT</t>
+          <t>Gfmvvb5d</t>
         </is>
       </c>
       <c r="B25" s="2" t="n">
-        <v>45760.4375</v>
+        <v>45759.4375</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>stuttgart</t>
+          <t>b  monchengladbach</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>werder bremen</t>
+          <t>freiburg</t>
         </is>
       </c>
       <c r="E25" t="n">
@@ -2990,56 +2996,58 @@
         </is>
       </c>
       <c r="I25" t="n">
-        <v>1.57</v>
+        <v>2.25</v>
       </c>
       <c r="J25" t="n">
-        <v>4.33</v>
+        <v>3.4</v>
       </c>
       <c r="K25" t="n">
-        <v>4.75</v>
+        <v>3.2</v>
       </c>
       <c r="L25" t="n">
-        <v>0.5906280601095251</v>
+        <v>0.4228527011270889</v>
       </c>
       <c r="M25" t="n">
-        <v>0.2141538231805899</v>
+        <v>0.2798289933929266</v>
       </c>
       <c r="N25" t="n">
-        <v>0.1952181167098851</v>
+        <v>0.2973183054799844</v>
       </c>
       <c r="O25" t="n">
-        <v>0.07841587316579934</v>
+        <v>0.05106209150326801</v>
       </c>
       <c r="P25" t="n">
         <v>1</v>
       </c>
       <c r="Q25" t="n">
-        <v>0.3103203458863102</v>
+        <v>0.5553696717151836</v>
       </c>
       <c r="R25" t="n">
-        <v>0.3843362142104569</v>
+        <v>0.2008292572892841</v>
       </c>
       <c r="S25" t="n">
-        <v>0.3053434399032329</v>
+        <v>0.2438010709955324</v>
       </c>
       <c r="T25" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U25" t="n">
         <v>1</v>
       </c>
-      <c r="V25" t="inlineStr"/>
+      <c r="V25" t="n">
+        <v>0</v>
+      </c>
       <c r="W25" t="n">
         <v>0</v>
       </c>
       <c r="X25" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Y25" t="n">
-        <v>0.3843362142104569</v>
+        <v>0.5553696717151836</v>
       </c>
       <c r="Z25" t="n">
-        <v>1.57</v>
+        <v>3.4</v>
       </c>
       <c r="AA25" t="inlineStr">
         <is>
@@ -3047,32 +3055,32 @@
         </is>
       </c>
       <c r="AB25" t="n">
-        <v>-0.6957756906834782</v>
+        <v>0.3701070349298434</v>
       </c>
       <c r="AC25" t="n">
-        <v>0</v>
+        <v>5.623117926116233</v>
       </c>
       <c r="AD25" t="n">
-        <v>0.07401586832414669</v>
+        <v>0.3115686007196512</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="1" t="inlineStr">
         <is>
-          <t>MXBrkODc</t>
+          <t>SjjRauSF</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
-        <v>45760.52083333334</v>
+        <v>45759.4375</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>eintracht frankfurt</t>
+          <t>holstein kiel</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>heidenheim</t>
+          <t>st  pauli</t>
         </is>
       </c>
       <c r="E26" t="n">
@@ -3092,56 +3100,58 @@
         </is>
       </c>
       <c r="I26" t="n">
-        <v>1.67</v>
+        <v>2.88</v>
       </c>
       <c r="J26" t="n">
-        <v>4.5</v>
+        <v>3.2</v>
       </c>
       <c r="K26" t="n">
-        <v>4.33</v>
+        <v>2.5</v>
       </c>
       <c r="L26" t="n">
-        <v>0.5692192187805826</v>
+        <v>0.327653997378768</v>
       </c>
       <c r="M26" t="n">
-        <v>0.2112435767474606</v>
+        <v>0.2948885976408912</v>
       </c>
       <c r="N26" t="n">
-        <v>0.2195372044719568</v>
+        <v>0.3774574049803408</v>
       </c>
       <c r="O26" t="n">
-        <v>0.05197149964889314</v>
+        <v>0.05972222222222223</v>
       </c>
       <c r="P26" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q26" t="n">
-        <v>0.3084216734147087</v>
+        <v>0.5144391395222441</v>
       </c>
       <c r="R26" t="n">
-        <v>0.5375571137836863</v>
+        <v>0.14681301239331</v>
       </c>
       <c r="S26" t="n">
-        <v>0.1540212128016051</v>
+        <v>0.3387478480844459</v>
       </c>
       <c r="T26" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U26" t="n">
         <v>1</v>
       </c>
-      <c r="V26" t="inlineStr"/>
+      <c r="V26" t="n">
+        <v>0</v>
+      </c>
       <c r="W26" t="n">
         <v>0</v>
       </c>
       <c r="X26" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Y26" t="n">
-        <v>0.5375571137836863</v>
+        <v>0.5144391395222441</v>
       </c>
       <c r="Z26" t="n">
-        <v>1.67</v>
+        <v>3.2</v>
       </c>
       <c r="AA26" t="inlineStr">
         <is>
@@ -3149,32 +3159,32 @@
         </is>
       </c>
       <c r="AB26" t="n">
-        <v>-0.1526561492257372</v>
+        <v>0.2937296574869005</v>
       </c>
       <c r="AC26" t="n">
-        <v>0</v>
+        <v>5.208696287662721</v>
       </c>
       <c r="AD26" t="n">
-        <v>0.2291354403689776</v>
+        <v>0.1756912914377982</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="1" t="inlineStr">
         <is>
-          <t>Gfmvvb5d</t>
+          <t>AgrQWtbT</t>
         </is>
       </c>
       <c r="B27" s="2" t="n">
-        <v>45759.4375</v>
+        <v>45760.4375</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>b  monchengladbach</t>
+          <t>stuttgart</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>freiburg</t>
+          <t>werder bremen</t>
         </is>
       </c>
       <c r="E27" t="n">
@@ -3194,56 +3204,58 @@
         </is>
       </c>
       <c r="I27" t="n">
-        <v>2.25</v>
+        <v>1.57</v>
       </c>
       <c r="J27" t="n">
-        <v>3.4</v>
+        <v>4.33</v>
       </c>
       <c r="K27" t="n">
-        <v>3.2</v>
+        <v>4.75</v>
       </c>
       <c r="L27" t="n">
-        <v>0.4228527011270889</v>
+        <v>0.5906280601095251</v>
       </c>
       <c r="M27" t="n">
-        <v>0.2798289933929266</v>
+        <v>0.2141538231805899</v>
       </c>
       <c r="N27" t="n">
-        <v>0.2973183054799844</v>
+        <v>0.1952181167098851</v>
       </c>
       <c r="O27" t="n">
-        <v>0.05106209150326801</v>
+        <v>0.07841587316579934</v>
       </c>
       <c r="P27" t="n">
         <v>1</v>
       </c>
       <c r="Q27" t="n">
-        <v>0.3091678711339827</v>
+        <v>0.4398897496396375</v>
       </c>
       <c r="R27" t="n">
-        <v>0.2480491122936091</v>
+        <v>0.327722820107536</v>
       </c>
       <c r="S27" t="n">
-        <v>0.4427830165724082</v>
+        <v>0.2323874302528265</v>
       </c>
       <c r="T27" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="U27" t="n">
         <v>1</v>
       </c>
-      <c r="V27" t="inlineStr"/>
+      <c r="V27" t="n">
+        <v>0</v>
+      </c>
       <c r="W27" t="n">
         <v>0</v>
       </c>
       <c r="X27" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="Y27" t="n">
-        <v>0.4427830165724082</v>
+        <v>0.4398897496396375</v>
       </c>
       <c r="Z27" t="n">
-        <v>3.2</v>
+        <v>4.33</v>
       </c>
       <c r="AA27" t="inlineStr">
         <is>
@@ -3251,32 +3263,32 @@
         </is>
       </c>
       <c r="AB27" t="n">
-        <v>0.1895025695598664</v>
+        <v>0.2716884732551442</v>
       </c>
       <c r="AC27" t="n">
-        <v>2.656698099434449</v>
+        <v>4.45388371510133</v>
       </c>
       <c r="AD27" t="n">
-        <v>0.1336151454384255</v>
+        <v>0.1121669295321015</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="1" t="inlineStr">
         <is>
-          <t>8lzQ11c3</t>
+          <t>KSgVuKzp</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
-        <v>45759.4375</v>
+        <v>45758.64583333334</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>bochum</t>
+          <t>wolfsburg</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>augsburg</t>
+          <t>rb leipzig</t>
         </is>
       </c>
       <c r="E28" t="n">
@@ -3296,37 +3308,37 @@
         </is>
       </c>
       <c r="I28" t="n">
-        <v>2.3</v>
+        <v>2.55</v>
       </c>
       <c r="J28" t="n">
-        <v>3.4</v>
+        <v>3.7</v>
       </c>
       <c r="K28" t="n">
-        <v>3</v>
+        <v>2.55</v>
       </c>
       <c r="L28" t="n">
-        <v>0.4093097913322633</v>
+        <v>0.371859296482412</v>
       </c>
       <c r="M28" t="n">
-        <v>0.2768860353130017</v>
+        <v>0.2562814070351758</v>
       </c>
       <c r="N28" t="n">
-        <v>0.3138041733547351</v>
+        <v>0.371859296482412</v>
       </c>
       <c r="O28" t="n">
-        <v>0.06223358908780896</v>
+        <v>0.05458399576046657</v>
       </c>
       <c r="P28" t="n">
         <v>1</v>
       </c>
       <c r="Q28" t="n">
-        <v>0.2763259567436151</v>
+        <v>0.3550807128992463</v>
       </c>
       <c r="R28" t="n">
-        <v>0.3525104859662375</v>
+        <v>0.2697446889071599</v>
       </c>
       <c r="S28" t="n">
-        <v>0.3711635572901475</v>
+        <v>0.3751745981935939</v>
       </c>
       <c r="T28" t="n">
         <v>2</v>
@@ -3334,7 +3346,9 @@
       <c r="U28" t="n">
         <v>1</v>
       </c>
-      <c r="V28" t="inlineStr"/>
+      <c r="V28" t="n">
+        <v>0</v>
+      </c>
       <c r="W28" t="n">
         <v>0</v>
       </c>
@@ -3342,10 +3356,10 @@
         <v>2</v>
       </c>
       <c r="Y28" t="n">
-        <v>0.3711635572901475</v>
+        <v>0.3751745981935939</v>
       </c>
       <c r="Z28" t="n">
-        <v>3</v>
+        <v>2.55</v>
       </c>
       <c r="AA28" t="inlineStr">
         <is>
@@ -3353,19 +3367,19 @@
         </is>
       </c>
       <c r="AB28" t="n">
-        <v>0.05674533593522124</v>
+        <v>-0.02793856426215203</v>
       </c>
       <c r="AC28" t="n">
-        <v>2.226981343740885</v>
+        <v>2.954499960774552</v>
       </c>
       <c r="AD28" t="n">
-        <v>0.01865307132390998</v>
+        <v>0.02009388529434764</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="1" t="inlineStr">
         <is>
-          <t>SUEjm2rA</t>
+          <t>8lzQ11c3</t>
         </is>
       </c>
       <c r="B29" s="2" t="n">
@@ -3373,12 +3387,12 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>hoffenheim</t>
+          <t>bochum</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>mainz</t>
+          <t>augsburg</t>
         </is>
       </c>
       <c r="E29" t="n">
@@ -3398,37 +3412,37 @@
         </is>
       </c>
       <c r="I29" t="n">
-        <v>2.8</v>
+        <v>2.3</v>
       </c>
       <c r="J29" t="n">
-        <v>3.5</v>
+        <v>3.4</v>
       </c>
       <c r="K29" t="n">
-        <v>2.35</v>
+        <v>3</v>
       </c>
       <c r="L29" t="n">
-        <v>0.3342816500711238</v>
+        <v>0.4093097913322633</v>
       </c>
       <c r="M29" t="n">
-        <v>0.267425320056899</v>
+        <v>0.2768860353130017</v>
       </c>
       <c r="N29" t="n">
-        <v>0.3982930298719773</v>
+        <v>0.3138041733547351</v>
       </c>
       <c r="O29" t="n">
-        <v>0.06838905775075976</v>
+        <v>0.06223358908780896</v>
       </c>
       <c r="P29" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q29" t="n">
-        <v>0.334498826908409</v>
+        <v>0.2677148166739484</v>
       </c>
       <c r="R29" t="n">
-        <v>0.3241042659744032</v>
+        <v>0.3311005310580269</v>
       </c>
       <c r="S29" t="n">
-        <v>0.3413969071171877</v>
+        <v>0.4011846522680246</v>
       </c>
       <c r="T29" t="n">
         <v>2</v>
@@ -3436,7 +3450,9 @@
       <c r="U29" t="n">
         <v>1</v>
       </c>
-      <c r="V29" t="inlineStr"/>
+      <c r="V29" t="n">
+        <v>0</v>
+      </c>
       <c r="W29" t="n">
         <v>0</v>
       </c>
@@ -3444,10 +3460,10 @@
         <v>2</v>
       </c>
       <c r="Y29" t="n">
-        <v>0.3413969071171877</v>
+        <v>0.4011846522680246</v>
       </c>
       <c r="Z29" t="n">
-        <v>2.35</v>
+        <v>3</v>
       </c>
       <c r="AA29" t="inlineStr">
         <is>
@@ -3455,19 +3471,19 @@
         </is>
       </c>
       <c r="AB29" t="n">
-        <v>-0.1464572357589696</v>
+        <v>0.101776978402037</v>
       </c>
       <c r="AC29" t="n">
-        <v>0.4096762885406253</v>
+        <v>3.159329136610694</v>
       </c>
       <c r="AD29" t="n">
-        <v>0.00689808020877869</v>
+        <v>0.07008412120999774</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="1" t="inlineStr">
         <is>
-          <t>SjjRauSF</t>
+          <t>SUEjm2rA</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
@@ -3475,12 +3491,12 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>holstein kiel</t>
+          <t>hoffenheim</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>st  pauli</t>
+          <t>mainz</t>
         </is>
       </c>
       <c r="E30" t="n">
@@ -3500,37 +3516,37 @@
         </is>
       </c>
       <c r="I30" t="n">
-        <v>2.88</v>
+        <v>2.8</v>
       </c>
       <c r="J30" t="n">
-        <v>3.2</v>
+        <v>3.5</v>
       </c>
       <c r="K30" t="n">
-        <v>2.5</v>
+        <v>2.35</v>
       </c>
       <c r="L30" t="n">
-        <v>0.327653997378768</v>
+        <v>0.3342816500711238</v>
       </c>
       <c r="M30" t="n">
-        <v>0.2948885976408912</v>
+        <v>0.267425320056899</v>
       </c>
       <c r="N30" t="n">
-        <v>0.3774574049803408</v>
+        <v>0.3982930298719773</v>
       </c>
       <c r="O30" t="n">
-        <v>0.05972222222222223</v>
+        <v>0.06838905775075976</v>
       </c>
       <c r="P30" t="n">
         <v>2</v>
       </c>
       <c r="Q30" t="n">
-        <v>0.2978764403928997</v>
+        <v>0.3135121246913471</v>
       </c>
       <c r="R30" t="n">
-        <v>0.321954935455852</v>
+        <v>0.2641882119921293</v>
       </c>
       <c r="S30" t="n">
-        <v>0.3801686241512484</v>
+        <v>0.4222996633165235</v>
       </c>
       <c r="T30" t="n">
         <v>2</v>
@@ -3538,7 +3554,9 @@
       <c r="U30" t="n">
         <v>1</v>
       </c>
-      <c r="V30" t="inlineStr"/>
+      <c r="V30" t="n">
+        <v>0</v>
+      </c>
       <c r="W30" t="n">
         <v>0</v>
       </c>
@@ -3546,10 +3564,10 @@
         <v>2</v>
       </c>
       <c r="Y30" t="n">
-        <v>0.3801686241512484</v>
+        <v>0.4222996633165235</v>
       </c>
       <c r="Z30" t="n">
-        <v>2.5</v>
+        <v>2.35</v>
       </c>
       <c r="AA30" t="inlineStr">
         <is>
@@ -3557,13 +3575,13 @@
         </is>
       </c>
       <c r="AB30" t="n">
-        <v>-0.03305229308125276</v>
+        <v>-0.005626512004570156</v>
       </c>
       <c r="AC30" t="n">
-        <v>2.28101174490749</v>
+        <v>3.325609848617623</v>
       </c>
       <c r="AD30" t="n">
-        <v>0.05821368869539634</v>
+        <v>0.1087875386251764</v>
       </c>
     </row>
     <row r="31">
@@ -3660,7 +3678,7 @@
         <v>-0.5148012962208931</v>
       </c>
       <c r="AC31" t="n">
-        <v>1.978389823478933</v>
+        <v>1.483792367609199</v>
       </c>
       <c r="AD31" t="n">
         <v>0.3778304605270781</v>
@@ -3760,7 +3778,7 @@
         <v>-0.6989768078344432</v>
       </c>
       <c r="AC32" t="n">
-        <v>1.650812534955001</v>
+        <v>1.238109401216251</v>
       </c>
       <c r="AD32" t="n">
         <v>0.2142387686565616</v>
@@ -3860,7 +3878,7 @@
         <v>-0.1615693222821422</v>
       </c>
       <c r="AC33" t="n">
-        <v>1.565120248945589</v>
+        <v>1.173840186709192</v>
       </c>
       <c r="AD33" t="n">
         <v>0.1797566407972458</v>
@@ -3964,7 +3982,7 @@
         <v>-0.2737132441018397</v>
       </c>
       <c r="AC34" t="n">
-        <v>2.140984091187131</v>
+        <v>1.605738068390348</v>
       </c>
       <c r="AD34" t="n">
         <v>0.4768780936312302</v>
@@ -4064,7 +4082,7 @@
         <v>0.1994573667586717</v>
       </c>
       <c r="AC35" t="n">
-        <v>10.27641200157723</v>
+        <v>7.707309001182923</v>
       </c>
       <c r="AD35" t="n">
         <v>0.1030514615287572</v>
@@ -4168,7 +4186,7 @@
         <v>-0.004214088975192055</v>
       </c>
       <c r="AC36" t="n">
-        <v>8.209599152665945</v>
+        <v>6.157199364499458</v>
       </c>
       <c r="AD36" t="n">
         <v>0.009836279572028983</v>
@@ -4268,7 +4286,7 @@
         <v>0.1503542647536552</v>
       </c>
       <c r="AC37" t="n">
-        <v>9.606001661708982</v>
+        <v>7.204501246281737</v>
       </c>
       <c r="AD37" t="n">
         <v>0.06458095492846644</v>
@@ -4368,7 +4386,7 @@
         <v>0.1288779609397273</v>
       </c>
       <c r="AC38" t="n">
-        <v>9.525972274075468</v>
+        <v>7.144479205556601</v>
       </c>
       <c r="AD38" t="n">
         <v>0.07995529364887377</v>
@@ -4472,7 +4490,7 @@
         <v>-0.01625400419552559</v>
       </c>
       <c r="AC39" t="n">
-        <v>4.441852349024913</v>
+        <v>3.331389261768685</v>
       </c>
       <c r="AD39" t="n">
         <v>0.04916817577938215</v>
@@ -4572,7 +4590,7 @@
         <v>0.3177124351282909</v>
       </c>
       <c r="AC40" t="n">
-        <v>7.906274610769746</v>
+        <v>5.929705958077309</v>
       </c>
       <c r="AD40" t="n">
         <v>0.4413732827563627</v>
@@ -4676,7 +4694,7 @@
         <v>0.162496595677248</v>
       </c>
       <c r="AC41" t="n">
-        <v>0.8366603119308629</v>
+        <v>0.6274952339481472</v>
       </c>
       <c r="AD41" t="n">
         <v>0.008318002111439904</v>
@@ -5300,7 +5318,7 @@
         <v>0.08730536773096151</v>
       </c>
       <c r="AC47" t="n">
-        <v>11.45168973130664</v>
+        <v>8.588767298479977</v>
       </c>
       <c r="AD47" t="n">
         <v>0.02730518135570681</v>
@@ -5404,7 +5422,7 @@
         <v>0.05343903800903104</v>
       </c>
       <c r="AC48" t="n">
-        <v>10.47718015893626</v>
+        <v>7.857885119202198</v>
       </c>
       <c r="AD48" t="n">
         <v>0.005192909543936086</v>
@@ -5508,7 +5526,7 @@
         <v>0.1055059381115614</v>
       </c>
       <c r="AC49" t="n">
-        <v>11.29694234233265</v>
+        <v>8.472706756749485</v>
       </c>
       <c r="AD49" t="n">
         <v>0.06454786518341771</v>

</xml_diff>

<commit_message>
DATA. Actualizo preds de SPA (x cambio de modelo)
</commit_message>
<xml_diff>
--- a/data/predicciones.xlsx
+++ b/data/predicciones.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD31"/>
+  <dimension ref="A1:AD30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -620,37 +620,37 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>1.75</v>
+        <v>1.85</v>
       </c>
       <c r="J2" t="n">
-        <v>3.4</v>
+        <v>3.2</v>
       </c>
       <c r="K2" t="n">
-        <v>5.5</v>
+        <v>5.25</v>
       </c>
       <c r="L2" t="n">
-        <v>0.5455871626549963</v>
+        <v>0.5179989208355815</v>
       </c>
       <c r="M2" t="n">
-        <v>0.2808169219547775</v>
+        <v>0.2994681261080706</v>
       </c>
       <c r="N2" t="n">
-        <v>0.1735959153902261</v>
+        <v>0.1825329530563478</v>
       </c>
       <c r="O2" t="n">
-        <v>0.04736440030557687</v>
+        <v>0.04351673101673104</v>
       </c>
       <c r="P2" t="n">
         <v>1</v>
       </c>
       <c r="Q2" t="n">
-        <v>0.3179719443453715</v>
+        <v>0.3181473390293549</v>
       </c>
       <c r="R2" t="n">
-        <v>0.4298873204860497</v>
+        <v>0.4027904760337619</v>
       </c>
       <c r="S2" t="n">
-        <v>0.2521407351685786</v>
+        <v>0.2790621849368829</v>
       </c>
       <c r="T2" t="n">
         <v>1</v>
@@ -664,10 +664,10 @@
         <v>1</v>
       </c>
       <c r="Y2" t="n">
-        <v>0.4298873204860497</v>
+        <v>0.4027904760337619</v>
       </c>
       <c r="Z2" t="n">
-        <v>1.75</v>
+        <v>1.85</v>
       </c>
       <c r="AA2" t="inlineStr">
         <is>
@@ -675,13 +675,13 @@
         </is>
       </c>
       <c r="AB2" t="n">
-        <v>-0.3302629188658839</v>
+        <v>-0.2998089639265181</v>
       </c>
       <c r="AC2" t="n">
-        <v>2.516763767800488</v>
+        <v>2.40001036742933</v>
       </c>
       <c r="AD2" t="n">
-        <v>0.1119153761406782</v>
+        <v>0.08464313700440701</v>
       </c>
     </row>
     <row r="3">
@@ -744,13 +744,13 @@
         <v>1</v>
       </c>
       <c r="Q3" t="n">
-        <v>0.2834637712803722</v>
+        <v>0.2907069872995475</v>
       </c>
       <c r="R3" t="n">
-        <v>0.5191851535220207</v>
+        <v>0.4902386198548464</v>
       </c>
       <c r="S3" t="n">
-        <v>0.1973510751976073</v>
+        <v>0.2190543928456061</v>
       </c>
       <c r="T3" t="n">
         <v>1</v>
@@ -764,7 +764,7 @@
         <v>1</v>
       </c>
       <c r="Y3" t="n">
-        <v>0.5191851535220207</v>
+        <v>0.4902386198548464</v>
       </c>
       <c r="Z3" t="n">
         <v>1.75</v>
@@ -775,13 +775,13 @@
         </is>
       </c>
       <c r="AB3" t="n">
-        <v>-0.1219013084486185</v>
+        <v>-0.1894432203386917</v>
       </c>
       <c r="AC3" t="n">
-        <v>3.413057249533991</v>
+        <v>3.107585668684514</v>
       </c>
       <c r="AD3" t="n">
-        <v>0.2357213822416485</v>
+        <v>0.1995316325552989</v>
       </c>
     </row>
     <row r="4">
@@ -844,13 +844,13 @@
         <v>1</v>
       </c>
       <c r="Q4" t="n">
-        <v>0.3347631790871167</v>
+        <v>0.2610053715453801</v>
       </c>
       <c r="R4" t="n">
-        <v>0.4803685854616074</v>
+        <v>0.5774668242796189</v>
       </c>
       <c r="S4" t="n">
-        <v>0.184868235451276</v>
+        <v>0.1615278041750014</v>
       </c>
       <c r="T4" t="n">
         <v>1</v>
@@ -864,7 +864,7 @@
         <v>1</v>
       </c>
       <c r="Y4" t="n">
-        <v>0.4803685854616074</v>
+        <v>0.5774668242796189</v>
       </c>
       <c r="Z4" t="n">
         <v>1.62</v>
@@ -875,13 +875,13 @@
         </is>
       </c>
       <c r="AB4" t="n">
-        <v>-0.3577465992777356</v>
+        <v>-0.1040382978500278</v>
       </c>
       <c r="AC4" t="n">
-        <v>2.76743812234782</v>
+        <v>3.832181903541927</v>
       </c>
       <c r="AD4" t="n">
-        <v>0.1456054063744907</v>
+        <v>0.3164614527342389</v>
       </c>
     </row>
     <row r="5">
@@ -920,37 +920,37 @@
         </is>
       </c>
       <c r="I5" t="n">
-        <v>1.67</v>
+        <v>1.75</v>
       </c>
       <c r="J5" t="n">
-        <v>3.5</v>
+        <v>3.4</v>
       </c>
       <c r="K5" t="n">
-        <v>6</v>
+        <v>5.5</v>
       </c>
       <c r="L5" t="n">
-        <v>0.5696460056964601</v>
+        <v>0.5455871626549963</v>
       </c>
       <c r="M5" t="n">
-        <v>0.2718025227180252</v>
+        <v>0.2808169219547775</v>
       </c>
       <c r="N5" t="n">
-        <v>0.1585514715855147</v>
+        <v>0.1735959153902261</v>
       </c>
       <c r="O5" t="n">
-        <v>0.05118334759053322</v>
+        <v>0.04736440030557687</v>
       </c>
       <c r="P5" t="n">
         <v>1</v>
       </c>
       <c r="Q5" t="n">
-        <v>0.2552782423305258</v>
+        <v>0.2561603499527556</v>
       </c>
       <c r="R5" t="n">
-        <v>0.6030071214634144</v>
+        <v>0.6060498394845099</v>
       </c>
       <c r="S5" t="n">
-        <v>0.1417146362060599</v>
+        <v>0.1377898105627346</v>
       </c>
       <c r="T5" t="n">
         <v>1</v>
@@ -964,10 +964,10 @@
         <v>1</v>
       </c>
       <c r="Y5" t="n">
-        <v>0.6030071214634144</v>
+        <v>0.6060498394845099</v>
       </c>
       <c r="Z5" t="n">
-        <v>1.67</v>
+        <v>1.75</v>
       </c>
       <c r="AA5" t="inlineStr">
         <is>
@@ -975,13 +975,13 @@
         </is>
       </c>
       <c r="AB5" t="n">
-        <v>0.01048043708045071</v>
+        <v>0.08078295879718962</v>
       </c>
       <c r="AC5" t="n">
-        <v>4.2210498502439</v>
+        <v>4.242348876391569</v>
       </c>
       <c r="AD5" t="n">
-        <v>0.3477288791328886</v>
+        <v>0.3498894895317543</v>
       </c>
     </row>
     <row r="6">
@@ -1020,37 +1020,37 @@
         </is>
       </c>
       <c r="I6" t="n">
-        <v>1.14</v>
+        <v>1.13</v>
       </c>
       <c r="J6" t="n">
         <v>8</v>
       </c>
       <c r="K6" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="L6" t="n">
-        <v>0.8316008316008316</v>
+        <v>0.8367784031478807</v>
       </c>
       <c r="M6" t="n">
-        <v>0.1185031185031185</v>
+        <v>0.1181949494446381</v>
       </c>
       <c r="N6" t="n">
-        <v>0.04989604989604989</v>
+        <v>0.04502664740748119</v>
       </c>
       <c r="O6" t="n">
-        <v>0.05482456140350878</v>
+        <v>0.0575747998314371</v>
       </c>
       <c r="P6" t="n">
         <v>1</v>
       </c>
       <c r="Q6" t="n">
-        <v>0.1438117262423627</v>
+        <v>0.1810536352158293</v>
       </c>
       <c r="R6" t="n">
-        <v>0.8166810361777346</v>
+        <v>0.7563707669441232</v>
       </c>
       <c r="S6" t="n">
-        <v>0.03950723757990281</v>
+        <v>0.06257559784004721</v>
       </c>
       <c r="T6" t="n">
         <v>1</v>
@@ -1064,10 +1064,10 @@
         <v>1</v>
       </c>
       <c r="Y6" t="n">
-        <v>0.8166810361777346</v>
+        <v>0.7563707669441232</v>
       </c>
       <c r="Z6" t="n">
-        <v>1.14</v>
+        <v>1.13</v>
       </c>
       <c r="AA6" t="inlineStr">
         <is>
@@ -1075,13 +1075,13 @@
         </is>
       </c>
       <c r="AB6" t="n">
-        <v>-0.4927401339813051</v>
+        <v>-1.117700256562623</v>
       </c>
       <c r="AC6" t="n">
-        <v>4.33614823747949</v>
+        <v>2.609580167281797</v>
       </c>
       <c r="AD6" t="n">
-        <v>0.6728693099353719</v>
+        <v>0.5753171317282939</v>
       </c>
     </row>
     <row r="7">
@@ -1144,13 +1144,13 @@
         <v>1</v>
       </c>
       <c r="Q7" t="n">
-        <v>0.203515586338626</v>
+        <v>0.2244312594932545</v>
       </c>
       <c r="R7" t="n">
-        <v>0.7107762539947464</v>
+        <v>0.6685096144269871</v>
       </c>
       <c r="S7" t="n">
-        <v>0.08570815966662755</v>
+        <v>0.1070591260797583</v>
       </c>
       <c r="T7" t="n">
         <v>1</v>
@@ -1164,7 +1164,7 @@
         <v>1</v>
       </c>
       <c r="Y7" t="n">
-        <v>0.7107762539947464</v>
+        <v>0.6685096144269871</v>
       </c>
       <c r="Z7" t="n">
         <v>1.36</v>
@@ -1175,13 +1175,13 @@
         </is>
       </c>
       <c r="AB7" t="n">
-        <v>-0.09262304046429101</v>
+        <v>-0.2522970121647152</v>
       </c>
       <c r="AC7" t="n">
-        <v>4.745178466249066</v>
+        <v>4.092358416214952</v>
       </c>
       <c r="AD7" t="n">
-        <v>0.5072606676561204</v>
+        <v>0.4440783549337326</v>
       </c>
     </row>
     <row r="8">
@@ -1244,13 +1244,13 @@
         <v>1</v>
       </c>
       <c r="Q8" t="n">
-        <v>0.3717953532710502</v>
+        <v>0.3270554379968321</v>
       </c>
       <c r="R8" t="n">
-        <v>0.3867451220641476</v>
+        <v>0.4581458209646962</v>
       </c>
       <c r="S8" t="n">
-        <v>0.2414595246648019</v>
+        <v>0.2147987410384717</v>
       </c>
       <c r="T8" t="n">
         <v>1</v>
@@ -1264,7 +1264,7 @@
         <v>1</v>
       </c>
       <c r="Y8" t="n">
-        <v>0.3867451220641476</v>
+        <v>0.4581458209646962</v>
       </c>
       <c r="Z8" t="n">
         <v>1.75</v>
@@ -1275,13 +1275,13 @@
         </is>
       </c>
       <c r="AB8" t="n">
-        <v>-0.4309280485169889</v>
+        <v>-0.2643264177490421</v>
       </c>
       <c r="AC8" t="n">
-        <v>0.4265540671746808</v>
+        <v>2.785621285701493</v>
       </c>
       <c r="AD8" t="n">
-        <v>0.0149497687930974</v>
+        <v>0.1310903829678642</v>
       </c>
     </row>
     <row r="9">
@@ -1344,13 +1344,13 @@
         <v>1</v>
       </c>
       <c r="Q9" t="n">
-        <v>0.3283518632105101</v>
+        <v>0.309847632515598</v>
       </c>
       <c r="R9" t="n">
-        <v>0.4502703751254281</v>
+        <v>0.4743995346947421</v>
       </c>
       <c r="S9" t="n">
-        <v>0.2213777616640616</v>
+        <v>0.2157528327896598</v>
       </c>
       <c r="T9" t="n">
         <v>1</v>
@@ -1364,7 +1364,7 @@
         <v>1</v>
       </c>
       <c r="Y9" t="n">
-        <v>0.4502703751254281</v>
+        <v>0.4743995346947421</v>
       </c>
       <c r="Z9" t="n">
         <v>1.9</v>
@@ -1375,32 +1375,32 @@
         </is>
       </c>
       <c r="AB9" t="n">
-        <v>-0.160540319179652</v>
+        <v>-0.1096009823111002</v>
       </c>
       <c r="AC9" t="n">
-        <v>2.899431696061425</v>
+        <v>3.138997400729663</v>
       </c>
       <c r="AD9" t="n">
-        <v>0.1219185119149179</v>
+        <v>0.1645519021791441</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
         <is>
-          <t>dhHEf26m</t>
+          <t>Qmk8moaK</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
-        <v>45767.5625</v>
+        <v>45767.66666666666</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>sevilla</t>
+          <t>real madrid</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>alaves</t>
+          <t>ath bilbao</t>
         </is>
       </c>
       <c r="E10" t="n">
@@ -1420,37 +1420,37 @@
         </is>
       </c>
       <c r="I10" t="n">
-        <v>2.05</v>
+        <v>1.62</v>
       </c>
       <c r="J10" t="n">
-        <v>3.1</v>
+        <v>4</v>
       </c>
       <c r="K10" t="n">
-        <v>3.9</v>
+        <v>5</v>
       </c>
       <c r="L10" t="n">
-        <v>0.4572617246596066</v>
+        <v>0.578368999421631</v>
       </c>
       <c r="M10" t="n">
-        <v>0.3023827534039334</v>
+        <v>0.2342394447657606</v>
       </c>
       <c r="N10" t="n">
-        <v>0.2403555219364599</v>
+        <v>0.1873915558126084</v>
       </c>
       <c r="O10" t="n">
-        <v>0.06679577962032734</v>
+        <v>0.06728395061728398</v>
       </c>
       <c r="P10" t="n">
         <v>1</v>
       </c>
       <c r="Q10" t="n">
-        <v>0.348376628264328</v>
+        <v>0.2872811982947548</v>
       </c>
       <c r="R10" t="n">
-        <v>0.3643057815857971</v>
+        <v>0.5224501643459624</v>
       </c>
       <c r="S10" t="n">
-        <v>0.2873175901498746</v>
+        <v>0.1902686373592828</v>
       </c>
       <c r="T10" t="n">
         <v>1</v>
@@ -1464,10 +1464,10 @@
         <v>1</v>
       </c>
       <c r="Y10" t="n">
-        <v>0.3643057815857971</v>
+        <v>0.5224501643459624</v>
       </c>
       <c r="Z10" t="n">
-        <v>2.05</v>
+        <v>1.62</v>
       </c>
       <c r="AA10" t="inlineStr">
         <is>
@@ -1475,32 +1475,32 @@
         </is>
       </c>
       <c r="AB10" t="n">
-        <v>-0.2411172835705867</v>
+        <v>-0.2477915060637756</v>
       </c>
       <c r="AC10" t="n">
-        <v>2.244179881671279</v>
+        <v>3.206349920974572</v>
       </c>
       <c r="AD10" t="n">
-        <v>0.0159291533214691</v>
+        <v>0.2351689660512076</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
         <is>
-          <t>Qmk8moaK</t>
+          <t>AyybJmyR</t>
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>45767.66666666666</v>
+        <v>45769.58333333334</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>real madrid</t>
+          <t>valencia</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>ath bilbao</t>
+          <t>espanyol</t>
         </is>
       </c>
       <c r="E11" t="n">
@@ -1519,38 +1519,22 @@
           <t>laliga</t>
         </is>
       </c>
-      <c r="I11" t="n">
-        <v>1.62</v>
-      </c>
-      <c r="J11" t="n">
-        <v>4</v>
-      </c>
-      <c r="K11" t="n">
-        <v>5</v>
-      </c>
-      <c r="L11" t="n">
-        <v>0.578368999421631</v>
-      </c>
-      <c r="M11" t="n">
-        <v>0.2342394447657606</v>
-      </c>
-      <c r="N11" t="n">
-        <v>0.1873915558126084</v>
-      </c>
-      <c r="O11" t="n">
-        <v>0.06728395061728398</v>
-      </c>
-      <c r="P11" t="n">
-        <v>1</v>
-      </c>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr"/>
+      <c r="L11" t="inlineStr"/>
+      <c r="M11" t="inlineStr"/>
+      <c r="N11" t="inlineStr"/>
+      <c r="O11" t="inlineStr"/>
+      <c r="P11" t="inlineStr"/>
       <c r="Q11" t="n">
-        <v>0.3052617221803428</v>
+        <v>0.3297638019409445</v>
       </c>
       <c r="R11" t="n">
-        <v>0.5129600362386417</v>
+        <v>0.4414310562212034</v>
       </c>
       <c r="S11" t="n">
-        <v>0.1817782415810155</v>
+        <v>0.2288051418378521</v>
       </c>
       <c r="T11" t="n">
         <v>1</v>
@@ -1564,24 +1548,18 @@
         <v>1</v>
       </c>
       <c r="Y11" t="n">
-        <v>0.5129600362386417</v>
-      </c>
-      <c r="Z11" t="n">
-        <v>1.62</v>
-      </c>
+        <v>0.4414310562212034</v>
+      </c>
+      <c r="Z11" t="inlineStr"/>
       <c r="AA11" t="inlineStr">
         <is>
           <t>prob_result_to_bet &gt; 0</t>
         </is>
       </c>
-      <c r="AB11" t="n">
-        <v>-0.2725882924087102</v>
-      </c>
-      <c r="AC11" t="n">
-        <v>3.104334097658135</v>
-      </c>
+      <c r="AB11" t="inlineStr"/>
+      <c r="AC11" t="inlineStr"/>
       <c r="AD11" t="n">
-        <v>0.207698314058299</v>
+        <v>0.111667254280259</v>
       </c>
     </row>
     <row r="12">
@@ -1628,13 +1606,13 @@
       <c r="O12" t="inlineStr"/>
       <c r="P12" t="inlineStr"/>
       <c r="Q12" t="n">
-        <v>0.1333796738456912</v>
+        <v>0.1654655713278333</v>
       </c>
       <c r="R12" t="n">
-        <v>0.8152878886422639</v>
+        <v>0.7703625184520414</v>
       </c>
       <c r="S12" t="n">
-        <v>0.05133243751204479</v>
+        <v>0.0641719102201256</v>
       </c>
       <c r="T12" t="n">
         <v>1</v>
@@ -1648,7 +1626,7 @@
         <v>1</v>
       </c>
       <c r="Y12" t="n">
-        <v>0.8152878886422639</v>
+        <v>0.7703625184520414</v>
       </c>
       <c r="Z12" t="inlineStr"/>
       <c r="AA12" t="inlineStr">
@@ -1659,7 +1637,7 @@
       <c r="AB12" t="inlineStr"/>
       <c r="AC12" t="inlineStr"/>
       <c r="AD12" t="n">
-        <v>0.6819082147965727</v>
+        <v>0.6048969471242081</v>
       </c>
     </row>
     <row r="13">
@@ -1706,13 +1684,13 @@
       <c r="O13" t="inlineStr"/>
       <c r="P13" t="inlineStr"/>
       <c r="Q13" t="n">
-        <v>0.2136886767148132</v>
+        <v>0.2010826142103263</v>
       </c>
       <c r="R13" t="n">
-        <v>0.6905403330880756</v>
+        <v>0.7206576667722052</v>
       </c>
       <c r="S13" t="n">
-        <v>0.09577099019711131</v>
+        <v>0.07825971901746873</v>
       </c>
       <c r="T13" t="n">
         <v>1</v>
@@ -1726,7 +1704,7 @@
         <v>1</v>
       </c>
       <c r="Y13" t="n">
-        <v>0.6905403330880756</v>
+        <v>0.7206576667722052</v>
       </c>
       <c r="Z13" t="inlineStr"/>
       <c r="AA13" t="inlineStr">
@@ -1737,7 +1715,7 @@
       <c r="AB13" t="inlineStr"/>
       <c r="AC13" t="inlineStr"/>
       <c r="AD13" t="n">
-        <v>0.4768516563732624</v>
+        <v>0.519575052561879</v>
       </c>
     </row>
     <row r="14">
@@ -1784,13 +1762,13 @@
       <c r="O14" t="inlineStr"/>
       <c r="P14" t="inlineStr"/>
       <c r="Q14" t="n">
-        <v>0.2470990010688819</v>
+        <v>0.2756547705654286</v>
       </c>
       <c r="R14" t="n">
-        <v>0.6206389343734249</v>
+        <v>0.5600930963520144</v>
       </c>
       <c r="S14" t="n">
-        <v>0.1322620645576934</v>
+        <v>0.1642521330825568</v>
       </c>
       <c r="T14" t="n">
         <v>1</v>
@@ -1808,7 +1786,7 @@
         <v>1</v>
       </c>
       <c r="Y14" t="n">
-        <v>0.6206389343734249</v>
+        <v>0.5600930963520144</v>
       </c>
       <c r="Z14" t="inlineStr"/>
       <c r="AA14" t="inlineStr">
@@ -1819,7 +1797,7 @@
       <c r="AB14" t="inlineStr"/>
       <c r="AC14" t="inlineStr"/>
       <c r="AD14" t="n">
-        <v>0.373539933304543</v>
+        <v>0.2844383257865858</v>
       </c>
     </row>
     <row r="15">
@@ -1866,13 +1844,13 @@
       <c r="O15" t="inlineStr"/>
       <c r="P15" t="inlineStr"/>
       <c r="Q15" t="n">
-        <v>0.1833615126479962</v>
+        <v>0.2204396329435235</v>
       </c>
       <c r="R15" t="n">
-        <v>0.748530122034116</v>
+        <v>0.6898810755218332</v>
       </c>
       <c r="S15" t="n">
-        <v>0.06810836531788761</v>
+        <v>0.08967929153464337</v>
       </c>
       <c r="T15" t="n">
         <v>1</v>
@@ -1886,7 +1864,7 @@
         <v>1</v>
       </c>
       <c r="Y15" t="n">
-        <v>0.748530122034116</v>
+        <v>0.6898810755218332</v>
       </c>
       <c r="Z15" t="inlineStr"/>
       <c r="AA15" t="inlineStr">
@@ -1897,26 +1875,26 @@
       <c r="AB15" t="inlineStr"/>
       <c r="AC15" t="inlineStr"/>
       <c r="AD15" t="n">
-        <v>0.5651686093861197</v>
+        <v>0.4694414425783097</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="inlineStr">
         <is>
-          <t>WU55TP7l</t>
+          <t>vJBRz8FE</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
-        <v>45758.66666666666</v>
+        <v>45760.375</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>valencia</t>
+          <t>osasuna</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>sevilla</t>
+          <t>girona</t>
         </is>
       </c>
       <c r="E16" t="n">
@@ -1936,37 +1914,37 @@
         </is>
       </c>
       <c r="I16" t="n">
-        <v>2.25</v>
+        <v>2.45</v>
       </c>
       <c r="J16" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="K16" t="n">
         <v>3.1</v>
       </c>
-      <c r="K16" t="n">
-        <v>3.5</v>
-      </c>
       <c r="L16" t="n">
-        <v>0.4221789883268483</v>
+        <v>0.3912443305068034</v>
       </c>
       <c r="M16" t="n">
-        <v>0.3064202334630351</v>
+        <v>0.2995464405442714</v>
       </c>
       <c r="N16" t="n">
-        <v>0.2714007782101168</v>
+        <v>0.3092092289489253</v>
       </c>
       <c r="O16" t="n">
-        <v>0.05273937532002027</v>
+        <v>0.04324391046741272</v>
       </c>
       <c r="P16" t="n">
         <v>1</v>
       </c>
       <c r="Q16" t="n">
-        <v>0.3576931131472717</v>
+        <v>0.3550221298742434</v>
       </c>
       <c r="R16" t="n">
-        <v>0.3576362478022997</v>
+        <v>0.3289484957910336</v>
       </c>
       <c r="S16" t="n">
-        <v>0.2846706390504286</v>
+        <v>0.3160293743347231</v>
       </c>
       <c r="T16" t="n">
         <v>0</v>
@@ -1980,10 +1958,10 @@
         <v>0</v>
       </c>
       <c r="Y16" t="n">
-        <v>0.3576931131472717</v>
+        <v>0.3550221298742434</v>
       </c>
       <c r="Z16" t="n">
-        <v>3.1</v>
+        <v>3.2</v>
       </c>
       <c r="AA16" t="inlineStr">
         <is>
@@ -1991,32 +1969,32 @@
         </is>
       </c>
       <c r="AB16" t="n">
-        <v>0.0518326908364487</v>
+        <v>0.06185037072617229</v>
       </c>
       <c r="AC16" t="n">
-        <v>4.387295208658508</v>
+        <v>4.549147145942115</v>
       </c>
       <c r="AD16" t="n">
-        <v>5.686534497201245e-05</v>
+        <v>0.02607363408320984</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="inlineStr">
         <is>
-          <t>vJBRz8FE</t>
+          <t>OrFjZfvA</t>
         </is>
       </c>
       <c r="B17" s="2" t="n">
-        <v>45760.375</v>
+        <v>45760.5625</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>osasuna</t>
+          <t>betis</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>girona</t>
+          <t>villarreal</t>
         </is>
       </c>
       <c r="E17" t="n">
@@ -2036,37 +2014,37 @@
         </is>
       </c>
       <c r="I17" t="n">
-        <v>2.45</v>
+        <v>2.3</v>
       </c>
       <c r="J17" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="K17" t="n">
         <v>3.2</v>
       </c>
-      <c r="K17" t="n">
-        <v>3.1</v>
-      </c>
       <c r="L17" t="n">
-        <v>0.3912443305068034</v>
+        <v>0.4139553116424932</v>
       </c>
       <c r="M17" t="n">
-        <v>0.2995464405442714</v>
+        <v>0.2885143081144649</v>
       </c>
       <c r="N17" t="n">
-        <v>0.3092092289489253</v>
+        <v>0.2975303802430419</v>
       </c>
       <c r="O17" t="n">
-        <v>0.04324391046741272</v>
+        <v>0.05031291172595531</v>
       </c>
       <c r="P17" t="n">
         <v>1</v>
       </c>
       <c r="Q17" t="n">
-        <v>0.3438891884092764</v>
+        <v>0.3549331654895776</v>
       </c>
       <c r="R17" t="n">
-        <v>0.3296816090142561</v>
+        <v>0.2966901149671875</v>
       </c>
       <c r="S17" t="n">
-        <v>0.3264292025764675</v>
+        <v>0.3483767195432348</v>
       </c>
       <c r="T17" t="n">
         <v>0</v>
@@ -2080,10 +2058,10 @@
         <v>0</v>
       </c>
       <c r="Y17" t="n">
-        <v>0.3438891884092764</v>
+        <v>0.3549331654895776</v>
       </c>
       <c r="Z17" t="n">
-        <v>3.2</v>
+        <v>3.3</v>
       </c>
       <c r="AA17" t="inlineStr">
         <is>
@@ -2091,32 +2069,32 @@
         </is>
       </c>
       <c r="AB17" t="n">
-        <v>0.04565700132258387</v>
+        <v>0.07446932439808956</v>
       </c>
       <c r="AC17" t="n">
-        <v>4.285401212378342</v>
+        <v>4.746149000506011</v>
       </c>
       <c r="AD17" t="n">
-        <v>0.01420757939502032</v>
+        <v>0.006556445946342804</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="inlineStr">
         <is>
-          <t>OrFjZfvA</t>
+          <t>0AcMPs7D</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
-        <v>45760.5625</v>
+        <v>45766.375</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>betis</t>
+          <t>rayo vallecano</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>villarreal</t>
+          <t>valencia</t>
         </is>
       </c>
       <c r="E18" t="n">
@@ -2139,34 +2117,34 @@
         <v>2.35</v>
       </c>
       <c r="J18" t="n">
-        <v>3.3</v>
+        <v>3</v>
       </c>
       <c r="K18" t="n">
-        <v>3.1</v>
+        <v>3.25</v>
       </c>
       <c r="L18" t="n">
-        <v>0.4048278591214879</v>
+        <v>0.3989769820971867</v>
       </c>
       <c r="M18" t="n">
-        <v>0.2882865057380293</v>
+        <v>0.3125319693094629</v>
       </c>
       <c r="N18" t="n">
-        <v>0.3068856351404828</v>
+        <v>0.2884910485933504</v>
       </c>
       <c r="O18" t="n">
-        <v>0.05114286308521043</v>
+        <v>0.06655755591925816</v>
       </c>
       <c r="P18" t="n">
         <v>1</v>
       </c>
       <c r="Q18" t="n">
-        <v>0.3642908902735112</v>
+        <v>0.3599689560794718</v>
       </c>
       <c r="R18" t="n">
-        <v>0.3021382462135215</v>
+        <v>0.2965898005702781</v>
       </c>
       <c r="S18" t="n">
-        <v>0.3335708635129672</v>
+        <v>0.3434412433502503</v>
       </c>
       <c r="T18" t="n">
         <v>0</v>
@@ -2180,10 +2158,10 @@
         <v>0</v>
       </c>
       <c r="Y18" t="n">
-        <v>0.3642908902735112</v>
+        <v>0.3599689560794718</v>
       </c>
       <c r="Z18" t="n">
-        <v>3.3</v>
+        <v>3</v>
       </c>
       <c r="AA18" t="inlineStr">
         <is>
@@ -2191,32 +2169,32 @@
         </is>
       </c>
       <c r="AB18" t="n">
-        <v>0.08789562517503774</v>
+        <v>0.03995343411920765</v>
       </c>
       <c r="AC18" t="n">
-        <v>4.946241188920132</v>
+        <v>4.190030428082699</v>
       </c>
       <c r="AD18" t="n">
-        <v>0.03072002676054403</v>
+        <v>0.01652771272922143</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="inlineStr">
         <is>
-          <t>0AcMPs7D</t>
+          <t>dhHEf26m</t>
         </is>
       </c>
       <c r="B19" s="2" t="n">
-        <v>45766.375</v>
+        <v>45767.5625</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>rayo vallecano</t>
+          <t>sevilla</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>valencia</t>
+          <t>alaves</t>
         </is>
       </c>
       <c r="E19" t="n">
@@ -2236,37 +2214,37 @@
         </is>
       </c>
       <c r="I19" t="n">
-        <v>2.35</v>
+        <v>2.05</v>
       </c>
       <c r="J19" t="n">
-        <v>3</v>
+        <v>3.1</v>
       </c>
       <c r="K19" t="n">
-        <v>3.25</v>
+        <v>3.9</v>
       </c>
       <c r="L19" t="n">
-        <v>0.3989769820971867</v>
+        <v>0.4572617246596066</v>
       </c>
       <c r="M19" t="n">
-        <v>0.3125319693094629</v>
+        <v>0.3023827534039334</v>
       </c>
       <c r="N19" t="n">
-        <v>0.2884910485933504</v>
+        <v>0.2403555219364599</v>
       </c>
       <c r="O19" t="n">
-        <v>0.06655755591925816</v>
+        <v>0.06679577962032734</v>
       </c>
       <c r="P19" t="n">
         <v>1</v>
       </c>
       <c r="Q19" t="n">
-        <v>0.3751337896262188</v>
+        <v>0.3714838451302532</v>
       </c>
       <c r="R19" t="n">
-        <v>0.2720037785984763</v>
+        <v>0.2820061117644747</v>
       </c>
       <c r="S19" t="n">
-        <v>0.3528624317753047</v>
+        <v>0.3465100431052724</v>
       </c>
       <c r="T19" t="n">
         <v>0</v>
@@ -2280,10 +2258,10 @@
         <v>0</v>
       </c>
       <c r="Y19" t="n">
-        <v>0.3751337896262188</v>
+        <v>0.3714838451302532</v>
       </c>
       <c r="Z19" t="n">
-        <v>3</v>
+        <v>3.1</v>
       </c>
       <c r="AA19" t="inlineStr">
         <is>
@@ -2291,13 +2269,13 @@
         </is>
       </c>
       <c r="AB19" t="n">
-        <v>0.06270068443932825</v>
+        <v>0.07219043804942146</v>
       </c>
       <c r="AC19" t="n">
-        <v>4.56267324689188</v>
+        <v>4.711183656954979</v>
       </c>
       <c r="AD19" t="n">
-        <v>0.02227135785091411</v>
+        <v>0.02497380202498084</v>
       </c>
     </row>
     <row r="20">
@@ -2336,37 +2314,37 @@
         </is>
       </c>
       <c r="I20" t="n">
-        <v>2.8</v>
+        <v>2.9</v>
       </c>
       <c r="J20" t="n">
         <v>3.3</v>
       </c>
       <c r="K20" t="n">
-        <v>2.4</v>
+        <v>2.35</v>
       </c>
       <c r="L20" t="n">
-        <v>0.3316582914572864</v>
+        <v>0.3212510356255179</v>
       </c>
       <c r="M20" t="n">
-        <v>0.2814070351758794</v>
+        <v>0.2823115161557581</v>
       </c>
       <c r="N20" t="n">
-        <v>0.3869346733668342</v>
+        <v>0.3964374482187241</v>
       </c>
       <c r="O20" t="n">
-        <v>0.07683982683982693</v>
+        <v>0.07338980413081653</v>
       </c>
       <c r="P20" t="n">
         <v>2</v>
       </c>
       <c r="Q20" t="n">
-        <v>0.3752180247284038</v>
+        <v>0.3720594705094771</v>
       </c>
       <c r="R20" t="n">
-        <v>0.2641048309818871</v>
+        <v>0.2827914568512272</v>
       </c>
       <c r="S20" t="n">
-        <v>0.3606771442897091</v>
+        <v>0.3451490726392958</v>
       </c>
       <c r="T20" t="n">
         <v>0</v>
@@ -2380,7 +2358,7 @@
         <v>0</v>
       </c>
       <c r="Y20" t="n">
-        <v>0.3752180247284038</v>
+        <v>0.3720594705094771</v>
       </c>
       <c r="Z20" t="n">
         <v>3.3</v>
@@ -2391,32 +2369,32 @@
         </is>
       </c>
       <c r="AB20" t="n">
-        <v>0.1035736876537968</v>
+        <v>0.09904184899185837</v>
       </c>
       <c r="AC20" t="n">
-        <v>5.166186174442277</v>
+        <v>5.104194018132013</v>
       </c>
       <c r="AD20" t="n">
-        <v>0.01454088043869473</v>
+        <v>0.02691039787018129</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="inlineStr">
         <is>
-          <t>AyybJmyR</t>
+          <t>lSTUh1hc</t>
         </is>
       </c>
       <c r="B21" s="2" t="n">
-        <v>45769.58333333334</v>
+        <v>45770.6875</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>valencia</t>
+          <t>alaves</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>espanyol</t>
+          <t>real sociedad</t>
         </is>
       </c>
       <c r="E21" t="n">
@@ -2444,13 +2422,13 @@
       <c r="O21" t="inlineStr"/>
       <c r="P21" t="inlineStr"/>
       <c r="Q21" t="n">
-        <v>0.3932220341732839</v>
+        <v>0.3548793674667227</v>
       </c>
       <c r="R21" t="n">
-        <v>0.3313137725789825</v>
+        <v>0.3260098339277983</v>
       </c>
       <c r="S21" t="n">
-        <v>0.2754641932477332</v>
+        <v>0.3191107986054789</v>
       </c>
       <c r="T21" t="n">
         <v>0</v>
@@ -2464,7 +2442,7 @@
         <v>0</v>
       </c>
       <c r="Y21" t="n">
-        <v>0.3932220341732839</v>
+        <v>0.3548793674667227</v>
       </c>
       <c r="Z21" t="inlineStr"/>
       <c r="AA21" t="inlineStr">
@@ -2475,26 +2453,26 @@
       <c r="AB21" t="inlineStr"/>
       <c r="AC21" t="inlineStr"/>
       <c r="AD21" t="n">
-        <v>0.06190826159430141</v>
+        <v>0.02886953353892446</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="inlineStr">
         <is>
-          <t>bNYvD4N7</t>
+          <t>WjapokZj</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
-        <v>45759.66666666666</v>
+        <v>45771.58333333334</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>leganes</t>
+          <t>osasuna</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>barcelona</t>
+          <t>sevilla</t>
         </is>
       </c>
       <c r="E22" t="n">
@@ -2513,88 +2491,70 @@
           <t>laliga</t>
         </is>
       </c>
-      <c r="I22" t="n">
-        <v>8.5</v>
-      </c>
-      <c r="J22" t="n">
-        <v>6</v>
-      </c>
-      <c r="K22" t="n">
-        <v>1.3</v>
-      </c>
-      <c r="L22" t="n">
-        <v>0.1116678596993558</v>
-      </c>
-      <c r="M22" t="n">
-        <v>0.1581961345740873</v>
-      </c>
-      <c r="N22" t="n">
-        <v>0.730136005726557</v>
-      </c>
-      <c r="O22" t="n">
-        <v>0.05354449472096512</v>
-      </c>
-      <c r="P22" t="n">
-        <v>2</v>
-      </c>
+      <c r="I22" t="inlineStr"/>
+      <c r="J22" t="inlineStr"/>
+      <c r="K22" t="inlineStr"/>
+      <c r="L22" t="inlineStr"/>
+      <c r="M22" t="inlineStr"/>
+      <c r="N22" t="inlineStr"/>
+      <c r="O22" t="inlineStr"/>
+      <c r="P22" t="inlineStr"/>
       <c r="Q22" t="n">
-        <v>0.2982654134769249</v>
+        <v>0.3482839322655607</v>
       </c>
       <c r="R22" t="n">
-        <v>0.03826011183752158</v>
+        <v>0.3065424038690709</v>
       </c>
       <c r="S22" t="n">
-        <v>0.6634744746855533</v>
+        <v>0.3451736638653682</v>
       </c>
       <c r="T22" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="U22" t="n">
         <v>1</v>
       </c>
-      <c r="V22" t="inlineStr"/>
-      <c r="W22" t="inlineStr"/>
+      <c r="V22" t="n">
+        <v>1</v>
+      </c>
+      <c r="W22" t="n">
+        <v>0</v>
+      </c>
       <c r="X22" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="Y22" t="n">
-        <v>0.6634744746855533</v>
-      </c>
-      <c r="Z22" t="n">
-        <v>1.3</v>
-      </c>
+        <v>0.3482839322655607</v>
+      </c>
+      <c r="Z22" t="inlineStr"/>
       <c r="AA22" t="inlineStr">
         <is>
           <t>prob_result_to_bet &gt; 0</t>
         </is>
       </c>
-      <c r="AB22" t="n">
-        <v>-0.4582772763626022</v>
-      </c>
-      <c r="AC22" t="n">
-        <v>0.9650781466885616</v>
-      </c>
+      <c r="AB22" t="inlineStr"/>
+      <c r="AC22" t="inlineStr"/>
       <c r="AD22" t="n">
-        <v>0.3652090612086284</v>
+        <v>0.003110268400192462</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="1" t="inlineStr">
         <is>
-          <t>jcVWEQhe</t>
+          <t>bNYvD4N7</t>
         </is>
       </c>
       <c r="B23" s="2" t="n">
-        <v>45760.46875</v>
+        <v>45759.66666666666</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>alaves</t>
+          <t>leganes</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>real madrid</t>
+          <t>barcelona</t>
         </is>
       </c>
       <c r="E23" t="n">
@@ -2614,37 +2574,37 @@
         </is>
       </c>
       <c r="I23" t="n">
-        <v>5.25</v>
+        <v>8</v>
       </c>
       <c r="J23" t="n">
-        <v>4.1</v>
+        <v>6</v>
       </c>
       <c r="K23" t="n">
-        <v>1.62</v>
+        <v>1.3</v>
       </c>
       <c r="L23" t="n">
-        <v>0.181119109947644</v>
+        <v>0.1178247734138973</v>
       </c>
       <c r="M23" t="n">
-        <v>0.2319208115183246</v>
+        <v>0.1570996978851964</v>
       </c>
       <c r="N23" t="n">
-        <v>0.5869600785340313</v>
+        <v>0.7250755287009064</v>
       </c>
       <c r="O23" t="n">
-        <v>0.05166258011786473</v>
+        <v>0.06089743589743568</v>
       </c>
       <c r="P23" t="n">
         <v>2</v>
       </c>
       <c r="Q23" t="n">
-        <v>0.2968459955176405</v>
+        <v>0.2869362565013873</v>
       </c>
       <c r="R23" t="n">
-        <v>0.07435258105103498</v>
+        <v>0.0436511846747126</v>
       </c>
       <c r="S23" t="n">
-        <v>0.6288014234313244</v>
+        <v>0.6694125588239001</v>
       </c>
       <c r="T23" t="n">
         <v>2</v>
@@ -2658,10 +2618,10 @@
         <v>2</v>
       </c>
       <c r="Y23" t="n">
-        <v>0.6288014234313244</v>
+        <v>0.6694125588239001</v>
       </c>
       <c r="Z23" t="n">
-        <v>1.62</v>
+        <v>1.3</v>
       </c>
       <c r="AA23" t="inlineStr">
         <is>
@@ -2669,32 +2629,32 @@
         </is>
       </c>
       <c r="AB23" t="n">
-        <v>0.03009404186894446</v>
+        <v>-0.4325455784297663</v>
       </c>
       <c r="AC23" t="n">
-        <v>3.710404283854632</v>
+        <v>3.687968430095464</v>
       </c>
       <c r="AD23" t="n">
-        <v>0.3319554279136839</v>
+        <v>0.3824763023225127</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="1" t="inlineStr">
         <is>
-          <t>GxrkL96E</t>
+          <t>jcVWEQhe</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
-        <v>45765.66666666666</v>
+        <v>45760.46875</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>espanyol</t>
+          <t>alaves</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>getafe</t>
+          <t>real madrid</t>
         </is>
       </c>
       <c r="E24" t="n">
@@ -2714,37 +2674,37 @@
         </is>
       </c>
       <c r="I24" t="n">
-        <v>2.75</v>
+        <v>5.25</v>
       </c>
       <c r="J24" t="n">
-        <v>2.75</v>
+        <v>4.1</v>
       </c>
       <c r="K24" t="n">
-        <v>3</v>
+        <v>1.62</v>
       </c>
       <c r="L24" t="n">
-        <v>0.3428571428571429</v>
+        <v>0.181119109947644</v>
       </c>
       <c r="M24" t="n">
-        <v>0.3428571428571429</v>
+        <v>0.2319208115183246</v>
       </c>
       <c r="N24" t="n">
-        <v>0.3142857142857143</v>
+        <v>0.5869600785340313</v>
       </c>
       <c r="O24" t="n">
-        <v>0.06060606060606055</v>
+        <v>0.05166258011786473</v>
       </c>
       <c r="P24" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q24" t="n">
-        <v>0.3297723665591055</v>
+        <v>0.3101152636366888</v>
       </c>
       <c r="R24" t="n">
-        <v>0.2473193269609033</v>
+        <v>0.1017224283883242</v>
       </c>
       <c r="S24" t="n">
-        <v>0.4229083064799914</v>
+        <v>0.5881623079749867</v>
       </c>
       <c r="T24" t="n">
         <v>2</v>
@@ -2758,10 +2718,10 @@
         <v>2</v>
       </c>
       <c r="Y24" t="n">
-        <v>0.4229083064799914</v>
+        <v>0.5881623079749867</v>
       </c>
       <c r="Z24" t="n">
-        <v>3</v>
+        <v>1.62</v>
       </c>
       <c r="AA24" t="inlineStr">
         <is>
@@ -2769,32 +2729,32 @@
         </is>
       </c>
       <c r="AB24" t="n">
-        <v>0.1343624597199871</v>
+        <v>-0.07609203400084111</v>
       </c>
       <c r="AC24" t="n">
-        <v>4.418532902760163</v>
+        <v>3.960571058986902</v>
       </c>
       <c r="AD24" t="n">
-        <v>0.09313593992088592</v>
+        <v>0.2780470443382979</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="1" t="inlineStr">
         <is>
-          <t>ALQvrPMs</t>
+          <t>GxrkL96E</t>
         </is>
       </c>
       <c r="B25" s="2" t="n">
-        <v>45766.66666666666</v>
+        <v>45765.66666666666</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>las palmas</t>
+          <t>espanyol</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>atl  madrid</t>
+          <t>getafe</t>
         </is>
       </c>
       <c r="E25" t="n">
@@ -2814,37 +2774,37 @@
         </is>
       </c>
       <c r="I25" t="n">
-        <v>5.25</v>
+        <v>2.75</v>
       </c>
       <c r="J25" t="n">
-        <v>3.8</v>
+        <v>2.63</v>
       </c>
       <c r="K25" t="n">
-        <v>1.65</v>
+        <v>3</v>
       </c>
       <c r="L25" t="n">
-        <v>0.1797462911201892</v>
+        <v>0.3375762113595037</v>
       </c>
       <c r="M25" t="n">
-        <v>0.2483336916792087</v>
+        <v>0.3529789282276179</v>
       </c>
       <c r="N25" t="n">
-        <v>0.571920017200602</v>
+        <v>0.3094448604128784</v>
       </c>
       <c r="O25" t="n">
-        <v>0.05969469127363869</v>
+        <v>0.07719783385182621</v>
       </c>
       <c r="P25" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="Q25" t="n">
-        <v>0.3063019934052796</v>
+        <v>0.3377059988813639</v>
       </c>
       <c r="R25" t="n">
-        <v>0.07857009567203983</v>
+        <v>0.2621414616554315</v>
       </c>
       <c r="S25" t="n">
-        <v>0.6151279109226808</v>
+        <v>0.4001525394632046</v>
       </c>
       <c r="T25" t="n">
         <v>2</v>
@@ -2858,10 +2818,10 @@
         <v>2</v>
       </c>
       <c r="Y25" t="n">
-        <v>0.6151279109226808</v>
+        <v>0.4001525394632046</v>
       </c>
       <c r="Z25" t="n">
-        <v>1.65</v>
+        <v>3</v>
       </c>
       <c r="AA25" t="inlineStr">
         <is>
@@ -2869,32 +2829,32 @@
         </is>
       </c>
       <c r="AB25" t="n">
-        <v>0.02301700464988198</v>
+        <v>0.1002288091948069</v>
       </c>
       <c r="AC25" t="n">
-        <v>3.661005318212581</v>
+        <v>2.801067776242432</v>
       </c>
       <c r="AD25" t="n">
-        <v>0.3088259175174012</v>
+        <v>0.06244654058184068</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="1" t="inlineStr">
         <is>
-          <t>nRL3xLjJ</t>
+          <t>ALQvrPMs</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
-        <v>45767.375</v>
+        <v>45766.66666666666</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>valladolid</t>
+          <t>las palmas</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>osasuna</t>
+          <t>atl  madrid</t>
         </is>
       </c>
       <c r="E26" t="n">
@@ -2914,37 +2874,37 @@
         </is>
       </c>
       <c r="I26" t="n">
-        <v>4.2</v>
+        <v>5.25</v>
       </c>
       <c r="J26" t="n">
-        <v>3.3</v>
+        <v>3.8</v>
       </c>
       <c r="K26" t="n">
-        <v>1.9</v>
+        <v>1.65</v>
       </c>
       <c r="L26" t="n">
-        <v>0.2230522945570971</v>
+        <v>0.1797462911201892</v>
       </c>
       <c r="M26" t="n">
-        <v>0.2838847385272145</v>
+        <v>0.2483336916792087</v>
       </c>
       <c r="N26" t="n">
-        <v>0.4930629669156883</v>
+        <v>0.571920017200602</v>
       </c>
       <c r="O26" t="n">
-        <v>0.06744133059922541</v>
+        <v>0.05969469127363869</v>
       </c>
       <c r="P26" t="n">
         <v>2</v>
       </c>
       <c r="Q26" t="n">
-        <v>0.3620687286741617</v>
+        <v>0.325304741156451</v>
       </c>
       <c r="R26" t="n">
-        <v>0.1346341640319651</v>
+        <v>0.08957654024901197</v>
       </c>
       <c r="S26" t="n">
-        <v>0.5032971072938731</v>
+        <v>0.5851187185945369</v>
       </c>
       <c r="T26" t="n">
         <v>2</v>
@@ -2958,10 +2918,10 @@
         <v>2</v>
       </c>
       <c r="Y26" t="n">
-        <v>0.5032971072938731</v>
+        <v>0.5851187185945369</v>
       </c>
       <c r="Z26" t="n">
-        <v>1.9</v>
+        <v>1.65</v>
       </c>
       <c r="AA26" t="inlineStr">
         <is>
@@ -2969,32 +2929,32 @@
         </is>
       </c>
       <c r="AB26" t="n">
-        <v>-0.04859499571293459</v>
+        <v>-0.05316017587540642</v>
       </c>
       <c r="AC26" t="n">
-        <v>3.160902052729289</v>
+        <v>3.986989112305531</v>
       </c>
       <c r="AD26" t="n">
-        <v>0.1412283786197114</v>
+        <v>0.2598139774380859</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="1" t="inlineStr">
         <is>
-          <t>Qol45JK5</t>
+          <t>nRL3xLjJ</t>
         </is>
       </c>
       <c r="B27" s="2" t="n">
-        <v>45770.58333333334</v>
+        <v>45767.375</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>celta vigo</t>
+          <t>valladolid</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>villarreal</t>
+          <t>osasuna</t>
         </is>
       </c>
       <c r="E27" t="n">
@@ -3013,22 +2973,38 @@
           <t>laliga</t>
         </is>
       </c>
-      <c r="I27" t="inlineStr"/>
-      <c r="J27" t="inlineStr"/>
-      <c r="K27" t="inlineStr"/>
-      <c r="L27" t="inlineStr"/>
-      <c r="M27" t="inlineStr"/>
-      <c r="N27" t="inlineStr"/>
-      <c r="O27" t="inlineStr"/>
-      <c r="P27" t="inlineStr"/>
+      <c r="I27" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="J27" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="K27" t="n">
+        <v>1.91</v>
+      </c>
+      <c r="L27" t="n">
+        <v>0.2278412377096588</v>
+      </c>
+      <c r="M27" t="n">
+        <v>0.2830754771544245</v>
+      </c>
+      <c r="N27" t="n">
+        <v>0.4890832851359167</v>
+      </c>
+      <c r="O27" t="n">
+        <v>0.0704929514787771</v>
+      </c>
+      <c r="P27" t="n">
+        <v>2</v>
+      </c>
       <c r="Q27" t="n">
-        <v>0.3773032002371716</v>
+        <v>0.3496130796082662</v>
       </c>
       <c r="R27" t="n">
-        <v>0.2345219295288117</v>
+        <v>0.1812277115441845</v>
       </c>
       <c r="S27" t="n">
-        <v>0.388174870234017</v>
+        <v>0.4691592088475491</v>
       </c>
       <c r="T27" t="n">
         <v>2</v>
@@ -3042,37 +3018,43 @@
         <v>2</v>
       </c>
       <c r="Y27" t="n">
-        <v>0.388174870234017</v>
-      </c>
-      <c r="Z27" t="inlineStr"/>
+        <v>0.4691592088475491</v>
+      </c>
+      <c r="Z27" t="n">
+        <v>1.91</v>
+      </c>
       <c r="AA27" t="inlineStr">
         <is>
           <t>prob_result_to_bet &gt; 0</t>
         </is>
       </c>
-      <c r="AB27" t="inlineStr"/>
-      <c r="AC27" t="inlineStr"/>
+      <c r="AB27" t="n">
+        <v>-0.1141823198914079</v>
+      </c>
+      <c r="AC27" t="n">
+        <v>3.096823998583814</v>
+      </c>
       <c r="AD27" t="n">
-        <v>0.01087166999684541</v>
+        <v>0.1195461292392829</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="1" t="inlineStr">
         <is>
-          <t>lSTUh1hc</t>
+          <t>Qol45JK5</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
-        <v>45770.6875</v>
+        <v>45770.58333333334</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>alaves</t>
+          <t>celta vigo</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>real sociedad</t>
+          <t>villarreal</t>
         </is>
       </c>
       <c r="E28" t="n">
@@ -3100,13 +3082,13 @@
       <c r="O28" t="inlineStr"/>
       <c r="P28" t="inlineStr"/>
       <c r="Q28" t="n">
-        <v>0.358521886396156</v>
+        <v>0.3469380462582169</v>
       </c>
       <c r="R28" t="n">
-        <v>0.2820131371895885</v>
+        <v>0.2392715227075504</v>
       </c>
       <c r="S28" t="n">
-        <v>0.3594649764142555</v>
+        <v>0.4137904310342326</v>
       </c>
       <c r="T28" t="n">
         <v>2</v>
@@ -3120,7 +3102,7 @@
         <v>2</v>
       </c>
       <c r="Y28" t="n">
-        <v>0.3594649764142555</v>
+        <v>0.4137904310342326</v>
       </c>
       <c r="Z28" t="inlineStr"/>
       <c r="AA28" t="inlineStr">
@@ -3131,7 +3113,7 @@
       <c r="AB28" t="inlineStr"/>
       <c r="AC28" t="inlineStr"/>
       <c r="AD28" t="n">
-        <v>0.0009430900180995017</v>
+        <v>0.06685238477601563</v>
       </c>
     </row>
     <row r="29">
@@ -3178,13 +3160,13 @@
       <c r="O29" t="inlineStr"/>
       <c r="P29" t="inlineStr"/>
       <c r="Q29" t="n">
-        <v>0.2931368593895033</v>
+        <v>0.3005253950237924</v>
       </c>
       <c r="R29" t="n">
-        <v>0.1004172894302447</v>
+        <v>0.08751076568414738</v>
       </c>
       <c r="S29" t="n">
-        <v>0.6064458511802521</v>
+        <v>0.6119638392920603</v>
       </c>
       <c r="T29" t="n">
         <v>2</v>
@@ -3202,7 +3184,7 @@
         <v>2</v>
       </c>
       <c r="Y29" t="n">
-        <v>0.6064458511802521</v>
+        <v>0.6119638392920603</v>
       </c>
       <c r="Z29" t="inlineStr"/>
       <c r="AA29" t="inlineStr">
@@ -3213,7 +3195,7 @@
       <c r="AB29" t="inlineStr"/>
       <c r="AC29" t="inlineStr"/>
       <c r="AD29" t="n">
-        <v>0.3133089917907488</v>
+        <v>0.3114384442682679</v>
       </c>
     </row>
     <row r="30">
@@ -3260,13 +3242,13 @@
       <c r="O30" t="inlineStr"/>
       <c r="P30" t="inlineStr"/>
       <c r="Q30" t="n">
-        <v>0.3351951465895876</v>
+        <v>0.3450242752479069</v>
       </c>
       <c r="R30" t="n">
-        <v>0.2441799611463608</v>
+        <v>0.218675290418827</v>
       </c>
       <c r="S30" t="n">
-        <v>0.4206248922640514</v>
+        <v>0.4363004343332665</v>
       </c>
       <c r="T30" t="n">
         <v>2</v>
@@ -3280,7 +3262,7 @@
         <v>2</v>
       </c>
       <c r="Y30" t="n">
-        <v>0.4206248922640514</v>
+        <v>0.4363004343332665</v>
       </c>
       <c r="Z30" t="inlineStr"/>
       <c r="AA30" t="inlineStr">
@@ -3291,89 +3273,7 @@
       <c r="AB30" t="inlineStr"/>
       <c r="AC30" t="inlineStr"/>
       <c r="AD30" t="n">
-        <v>0.08542974567446376</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="1" t="inlineStr">
-        <is>
-          <t>WjapokZj</t>
-        </is>
-      </c>
-      <c r="B31" s="2" t="n">
-        <v>45771.58333333334</v>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>osasuna</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>sevilla</t>
-        </is>
-      </c>
-      <c r="E31" t="n">
-        <v>148</v>
-      </c>
-      <c r="F31" t="n">
-        <v>1481</v>
-      </c>
-      <c r="G31" t="inlineStr">
-        <is>
-          <t>spain</t>
-        </is>
-      </c>
-      <c r="H31" t="inlineStr">
-        <is>
-          <t>laliga</t>
-        </is>
-      </c>
-      <c r="I31" t="inlineStr"/>
-      <c r="J31" t="inlineStr"/>
-      <c r="K31" t="inlineStr"/>
-      <c r="L31" t="inlineStr"/>
-      <c r="M31" t="inlineStr"/>
-      <c r="N31" t="inlineStr"/>
-      <c r="O31" t="inlineStr"/>
-      <c r="P31" t="inlineStr"/>
-      <c r="Q31" t="n">
-        <v>0.3556859569841113</v>
-      </c>
-      <c r="R31" t="n">
-        <v>0.2581087572074921</v>
-      </c>
-      <c r="S31" t="n">
-        <v>0.3862052858083966</v>
-      </c>
-      <c r="T31" t="n">
-        <v>2</v>
-      </c>
-      <c r="U31" t="n">
-        <v>1</v>
-      </c>
-      <c r="V31" t="n">
-        <v>1</v>
-      </c>
-      <c r="W31" t="n">
-        <v>0</v>
-      </c>
-      <c r="X31" t="n">
-        <v>2</v>
-      </c>
-      <c r="Y31" t="n">
-        <v>0.3862052858083966</v>
-      </c>
-      <c r="Z31" t="inlineStr"/>
-      <c r="AA31" t="inlineStr">
-        <is>
-          <t>prob_result_to_bet &gt; 0</t>
-        </is>
-      </c>
-      <c r="AB31" t="inlineStr"/>
-      <c r="AC31" t="inlineStr"/>
-      <c r="AD31" t="n">
-        <v>0.03051932882428532</v>
+        <v>0.09127615908535963</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
DATA. Actualizo predicciones tras cambio de modelos y en bs
</commit_message>
<xml_diff>
--- a/data/predicciones.xlsx
+++ b/data/predicciones.xlsx
@@ -671,14 +671,14 @@
       </c>
       <c r="AA2" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; -10</t>
+          <t>kelly_crit &gt; nan</t>
         </is>
       </c>
       <c r="AB2" t="n">
         <v>-0.3431683915042654</v>
       </c>
       <c r="AC2" t="n">
-        <v>3.683333158279915</v>
+        <v>4.632200549310965</v>
       </c>
       <c r="AD2" t="n">
         <v>0.1237960596356306</v>
@@ -771,14 +771,14 @@
       </c>
       <c r="AA3" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; -10</t>
+          <t>kelly_crit &gt; nan</t>
         </is>
       </c>
       <c r="AB3" t="n">
         <v>-0.04310902503243516</v>
       </c>
       <c r="AC3" t="n">
-        <v>5.26304712760076</v>
+        <v>5.619782233047594</v>
       </c>
       <c r="AD3" t="n">
         <v>0.03655818749549206</v>
@@ -875,14 +875,14 @@
       </c>
       <c r="AA4" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; -10</t>
+          <t>kelly_crit &gt; nan</t>
         </is>
       </c>
       <c r="AB4" t="n">
         <v>-0.5741422837557426</v>
       </c>
       <c r="AC4" t="n">
-        <v>2.648828085997137</v>
+        <v>3.433501786748659</v>
       </c>
       <c r="AD4" t="n">
         <v>0.1497370464228457</v>
@@ -975,14 +975,14 @@
       </c>
       <c r="AA5" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; -10</t>
+          <t>kelly_crit &gt; nan</t>
         </is>
       </c>
       <c r="AB5" t="n">
         <v>-0.1588154682300212</v>
       </c>
       <c r="AC5" t="n">
-        <v>4.633785365441027</v>
+        <v>5.503027150455367</v>
       </c>
       <c r="AD5" t="n">
         <v>0.09711917534485237</v>
@@ -1075,14 +1075,14 @@
       </c>
       <c r="AA6" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; -10</t>
+          <t>kelly_crit &gt; nan</t>
         </is>
       </c>
       <c r="AB6" t="n">
         <v>-0.09703341599720818</v>
       </c>
       <c r="AC6" t="n">
-        <v>4.967984891417715</v>
+        <v>4.752130354390779</v>
       </c>
       <c r="AD6" t="n">
         <v>0.01608021976647306</v>
@@ -1179,14 +1179,14 @@
       </c>
       <c r="AA7" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; -10</t>
+          <t>kelly_crit &gt; nan</t>
         </is>
       </c>
       <c r="AB7" t="n">
         <v>-0.4984026231322618</v>
       </c>
       <c r="AC7" t="n">
-        <v>2.965270127085621</v>
+        <v>3.097445840119211</v>
       </c>
       <c r="AD7" t="n">
         <v>0.03964386541199916</v>
@@ -1279,14 +1279,14 @@
       </c>
       <c r="AA8" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; -10</t>
+          <t>kelly_crit &gt; nan</t>
         </is>
       </c>
       <c r="AB8" t="n">
         <v>-0.542075954382832</v>
       </c>
       <c r="AC8" t="n">
-        <v>2.779932219792611</v>
+        <v>3.684481844019597</v>
       </c>
       <c r="AD8" t="n">
         <v>0.1916649793803577</v>
@@ -1383,14 +1383,14 @@
       </c>
       <c r="AA9" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; -10</t>
+          <t>kelly_crit &gt; nan</t>
         </is>
       </c>
       <c r="AB9" t="n">
         <v>-0.2789858709756171</v>
       </c>
       <c r="AC9" t="n">
-        <v>4.004185781782999</v>
+        <v>5.026843768047388</v>
       </c>
       <c r="AD9" t="n">
         <v>0.1614383030026024</v>
@@ -1487,14 +1487,14 @@
       </c>
       <c r="AA10" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; -10</t>
+          <t>kelly_crit &gt; nan</t>
         </is>
       </c>
       <c r="AB10" t="n">
         <v>-1.028270809099173</v>
       </c>
       <c r="AC10" t="n">
-        <v>1.247323595429342</v>
+        <v>1.934914651193073</v>
       </c>
       <c r="AD10" t="n">
         <v>0.2423069859744025</v>
@@ -1591,14 +1591,14 @@
       </c>
       <c r="AA11" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; -10</t>
+          <t>kelly_crit &gt; nan</t>
         </is>
       </c>
       <c r="AB11" t="n">
         <v>-0.363041385425679</v>
       </c>
       <c r="AC11" t="n">
-        <v>3.586604167439265</v>
+        <v>4.781851227079884</v>
       </c>
       <c r="AD11" t="n">
         <v>0.1327939036371711</v>
@@ -1695,14 +1695,14 @@
       </c>
       <c r="AA12" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; -10</t>
+          <t>kelly_crit &gt; nan</t>
         </is>
       </c>
       <c r="AB12" t="n">
         <v>-0.9232560831056776</v>
       </c>
       <c r="AC12" t="n">
-        <v>1.499112218698352</v>
+        <v>2.137466046258008</v>
       </c>
       <c r="AD12" t="n">
         <v>0.1792139082532195</v>
@@ -1799,14 +1799,14 @@
       </c>
       <c r="AA13" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; -10</t>
+          <t>kelly_crit &gt; nan</t>
         </is>
       </c>
       <c r="AB13" t="n">
         <v>0.149826256215659</v>
       </c>
       <c r="AC13" t="n">
-        <v>7.100470198541713</v>
+        <v>5.603342831857283</v>
       </c>
       <c r="AD13" t="n">
         <v>0.01041717464356479</v>
@@ -1903,14 +1903,14 @@
       </c>
       <c r="AA14" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; -10</t>
+          <t>kelly_crit &gt; nan</t>
         </is>
       </c>
       <c r="AB14" t="n">
         <v>0.1881889731925057</v>
       </c>
       <c r="AC14" t="n">
-        <v>7.477567874227813</v>
+        <v>6.113960382242293</v>
       </c>
       <c r="AD14" t="n">
         <v>0.1006231435415206</v>
@@ -2003,14 +2003,14 @@
       </c>
       <c r="AA15" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; -10</t>
+          <t>kelly_crit &gt; nan</t>
         </is>
       </c>
       <c r="AB15" t="n">
         <v>0.1277504488064317</v>
       </c>
       <c r="AC15" t="n">
-        <v>6.875454182041719</v>
+        <v>5.45240356125959</v>
       </c>
       <c r="AD15" t="n">
         <v>0.02447410732311933</v>
@@ -2107,14 +2107,14 @@
       </c>
       <c r="AA16" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; -10</t>
+          <t>kelly_crit &gt; nan</t>
         </is>
       </c>
       <c r="AB16" t="n">
         <v>-0.1621154150812483</v>
       </c>
       <c r="AC16" t="n">
-        <v>3.395435870406929</v>
+        <v>1.026950822369062</v>
       </c>
       <c r="AD16" t="n">
         <v>0.08912129085429416</v>
@@ -2207,14 +2207,14 @@
       </c>
       <c r="AA17" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; -10</t>
+          <t>kelly_crit &gt; nan</t>
         </is>
       </c>
       <c r="AB17" t="n">
         <v>0.1118942042191997</v>
       </c>
       <c r="AC17" t="n">
-        <v>4.719823301264342</v>
+        <v>1.287224536708457</v>
       </c>
       <c r="AD17" t="n">
         <v>0.1092083414533798</v>
@@ -2307,14 +2307,14 @@
       </c>
       <c r="AA18" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; -10</t>
+          <t>kelly_crit &gt; nan</t>
         </is>
       </c>
       <c r="AB18" t="n">
         <v>-0.7469870012290095</v>
       </c>
       <c r="AC18" t="n">
-        <v>0.510065870891194</v>
+        <v>0.2787552507059921</v>
       </c>
       <c r="AD18" t="n">
         <v>0.1436275199902656</v>
@@ -2411,14 +2411,14 @@
       </c>
       <c r="AA19" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; -10</t>
+          <t>kelly_crit &gt; nan</t>
         </is>
       </c>
       <c r="AB19" t="n">
         <v>-0.7674303717791368</v>
       </c>
       <c r="AC19" t="n">
-        <v>0.6311398239094296</v>
+        <v>0.3527382157270356</v>
       </c>
       <c r="AD19" t="n">
         <v>0.4018907282909164</v>
@@ -2511,14 +2511,14 @@
       </c>
       <c r="AA20" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; -10</t>
+          <t>kelly_crit &gt; nan</t>
         </is>
       </c>
       <c r="AB20" t="n">
         <v>0.2204089136009099</v>
       </c>
       <c r="AC20" t="n">
-        <v>4.139598439688007</v>
+        <v>1.128981392642184</v>
       </c>
       <c r="AD20" t="n">
         <v>0.05616946011402418</v>
@@ -2615,14 +2615,14 @@
       </c>
       <c r="AA21" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; -10</t>
+          <t>kelly_crit &gt; nan</t>
         </is>
       </c>
       <c r="AB21" t="n">
         <v>-0.3293461645491026</v>
       </c>
       <c r="AC21" t="n">
-        <v>2.2830685806431</v>
+        <v>0.7996361078124642</v>
       </c>
       <c r="AD21" t="n">
         <v>0.1718138070598556</v>
@@ -2715,14 +2715,14 @@
       </c>
       <c r="AA22" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; -10</t>
+          <t>kelly_crit &gt; nan</t>
         </is>
       </c>
       <c r="AB22" t="n">
         <v>-0.2220536622623122</v>
       </c>
       <c r="AC22" t="n">
-        <v>3.206262384101221</v>
+        <v>4.848692487570276</v>
       </c>
       <c r="AD22" t="n">
         <v>0.2019496636869704</v>
@@ -2815,14 +2815,14 @@
       </c>
       <c r="AA23" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; -10</t>
+          <t>kelly_crit &gt; nan</t>
         </is>
       </c>
       <c r="AB23" t="n">
         <v>-0.8397769593655313</v>
       </c>
       <c r="AC23" t="n">
-        <v>0.3695799707706902</v>
+        <v>1.730356507079985</v>
       </c>
       <c r="AD23" t="n">
         <v>0.6103579675175075</v>
@@ -2915,14 +2915,14 @@
       </c>
       <c r="AA24" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; -10</t>
+          <t>kelly_crit &gt; nan</t>
         </is>
       </c>
       <c r="AB24" t="n">
         <v>-0.514687636472877</v>
       </c>
       <c r="AC24" t="n">
-        <v>1.244882859089998</v>
+        <v>2.375693711307424</v>
       </c>
       <c r="AD24" t="n">
         <v>0.1751134522683858</v>
@@ -3015,14 +3015,14 @@
       </c>
       <c r="AA25" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; -10</t>
+          <t>kelly_crit &gt; nan</t>
         </is>
       </c>
       <c r="AB25" t="n">
         <v>-1.046956319975492</v>
       </c>
       <c r="AC25" t="n">
-        <v>0.16447524367289</v>
+        <v>0.7845440058707277</v>
       </c>
       <c r="AD25" t="n">
         <v>0.3824399215584676</v>
@@ -3115,14 +3115,14 @@
       </c>
       <c r="AA26" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; -10</t>
+          <t>kelly_crit &gt; nan</t>
         </is>
       </c>
       <c r="AB26" t="n">
         <v>-0.3669185779058267</v>
       </c>
       <c r="AC26" t="n">
-        <v>2.060260009938618</v>
+        <v>3.942347478998544</v>
       </c>
       <c r="AD26" t="n">
         <v>0.2070563719858555</v>
@@ -3215,14 +3215,14 @@
       </c>
       <c r="AA27" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; -10</t>
+          <t>kelly_crit &gt; nan</t>
         </is>
       </c>
       <c r="AB27" t="n">
         <v>-0.1874671134080337</v>
       </c>
       <c r="AC27" t="n">
-        <v>3.529349612747087</v>
+        <v>7.328986373359086</v>
       </c>
       <c r="AD27" t="n">
         <v>0.4615877137351533</v>
@@ -3315,14 +3315,14 @@
       </c>
       <c r="AA28" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; -10</t>
+          <t>kelly_crit &gt; nan</t>
         </is>
       </c>
       <c r="AB28" t="n">
         <v>-0.4864140480297029</v>
       </c>
       <c r="AC28" t="n">
-        <v>1.375305571038293</v>
+        <v>3.570958949883455</v>
       </c>
       <c r="AD28" t="n">
         <v>0.3879417939777161</v>
@@ -3415,14 +3415,14 @@
       </c>
       <c r="AA29" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; -10</t>
+          <t>kelly_crit &gt; nan</t>
         </is>
       </c>
       <c r="AB29" t="n">
         <v>-0.4829447296605331</v>
       </c>
       <c r="AC29" t="n">
-        <v>1.392091925894163</v>
+        <v>2.532616664092473</v>
       </c>
       <c r="AD29" t="n">
         <v>0.07702642532127657</v>
@@ -3515,14 +3515,14 @@
       </c>
       <c r="AA30" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; -10</t>
+          <t>kelly_crit &gt; nan</t>
         </is>
       </c>
       <c r="AB30" t="n">
         <v>-0.4074011344866009</v>
       </c>
       <c r="AC30" t="n">
-        <v>1.802729970383093</v>
+        <v>2.87040603233396</v>
       </c>
       <c r="AD30" t="n">
         <v>0.1300301580715786</v>
@@ -3619,14 +3619,14 @@
       </c>
       <c r="AA31" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; -10</t>
+          <t>kelly_crit &gt; nan</t>
         </is>
       </c>
       <c r="AB31" t="n">
         <v>0.1701628009049046</v>
       </c>
       <c r="AC31" t="n">
-        <v>7.302724261846478</v>
+        <v>6.442303884331828</v>
       </c>
       <c r="AD31" t="n">
         <v>0.1054887282930089</v>
@@ -3719,14 +3719,14 @@
       </c>
       <c r="AA32" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; -10</t>
+          <t>kelly_crit &gt; nan</t>
         </is>
       </c>
       <c r="AB32" t="n">
         <v>0.07016476519401811</v>
       </c>
       <c r="AC32" t="n">
-        <v>3.871263199820806</v>
+        <v>1.055799054496583</v>
       </c>
       <c r="AD32" t="n">
         <v>0.0006064692166009023</v>
@@ -3819,14 +3819,14 @@
       </c>
       <c r="AA33" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; -10</t>
+          <t>kelly_crit &gt; nan</t>
         </is>
       </c>
       <c r="AB33" t="n">
         <v>0.2784434307635032</v>
       </c>
       <c r="AC33" t="n">
-        <v>5.047158303798901</v>
+        <v>1.376497719217882</v>
       </c>
       <c r="AD33" t="n">
         <v>0.1701159480146994</v>
@@ -3919,14 +3919,14 @@
       </c>
       <c r="AA34" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; -10</t>
+          <t>kelly_crit &gt; nan</t>
         </is>
       </c>
       <c r="AB34" t="n">
         <v>-0.1454757510383939</v>
       </c>
       <c r="AC34" t="n">
-        <v>1.020129147466237</v>
+        <v>1.043856548932646</v>
       </c>
       <c r="AD34" t="n">
         <v>0.002936265720946296</v>
@@ -4019,14 +4019,14 @@
       </c>
       <c r="AA35" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; -10</t>
+          <t>kelly_crit &gt; nan</t>
         </is>
       </c>
       <c r="AB35" t="n">
         <v>-0.2235507367507809</v>
       </c>
       <c r="AC35" t="n">
-        <v>4.887782978167782</v>
+        <v>7.213947420442127</v>
       </c>
       <c r="AD35" t="n">
         <v>0.1549829660246578</v>
@@ -4123,14 +4123,14 @@
       </c>
       <c r="AA36" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; -10</t>
+          <t>kelly_crit &gt; nan</t>
         </is>
       </c>
       <c r="AB36" t="n">
         <v>-0.7150768138279497</v>
       </c>
       <c r="AC36" t="n">
-        <v>3.613258241350813</v>
+        <v>5.954121155500691</v>
       </c>
       <c r="AD36" t="n">
         <v>0.2991513135729987</v>
@@ -4223,14 +4223,14 @@
       </c>
       <c r="AA37" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; -10</t>
+          <t>kelly_crit &gt; nan</t>
         </is>
       </c>
       <c r="AB37" t="n">
         <v>-0.5601814383906134</v>
       </c>
       <c r="AC37" t="n">
-        <v>3.998560273568164</v>
+        <v>5.706431449869343</v>
       </c>
       <c r="AD37" t="n">
         <v>0.1732475316508266</v>
@@ -4323,14 +4323,14 @@
       </c>
       <c r="AA38" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; -10</t>
+          <t>kelly_crit &gt; nan</t>
         </is>
       </c>
       <c r="AB38" t="n">
         <v>0.04526611147022155</v>
       </c>
       <c r="AC38" t="n">
-        <v>5.624460555412771</v>
+        <v>9.103114217904309</v>
       </c>
       <c r="AD38" t="n">
         <v>0.2834144579195952</v>
@@ -4423,14 +4423,14 @@
       </c>
       <c r="AA39" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; -10</t>
+          <t>kelly_crit &gt; nan</t>
         </is>
       </c>
       <c r="AB39" t="n">
         <v>-0.09432957462287642</v>
       </c>
       <c r="AC39" t="n">
-        <v>5.240785850063413</v>
+        <v>5.603435727461605</v>
       </c>
       <c r="AD39" t="n">
         <v>0.08122242239616234</v>
@@ -4525,14 +4525,14 @@
       </c>
       <c r="AA40" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; -0.5</t>
+          <t>kelly_crit &gt; nan</t>
         </is>
       </c>
       <c r="AB40" t="n">
         <v>-0.1361905974892645</v>
       </c>
       <c r="AC40" t="n">
-        <v>4.037884686926533</v>
+        <v>0</v>
       </c>
       <c r="AD40" t="n">
         <v>0.1535068558278012</v>
@@ -4627,14 +4627,14 @@
       </c>
       <c r="AA41" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; -0.5</t>
+          <t>kelly_crit &gt; nan</t>
         </is>
       </c>
       <c r="AB41" t="n">
         <v>-0.06615271180432153</v>
       </c>
       <c r="AC41" t="n">
-        <v>4.776536594801058</v>
+        <v>0</v>
       </c>
       <c r="AD41" t="n">
         <v>0.1134391129166815</v>
@@ -4719,24 +4719,24 @@
         <v>0</v>
       </c>
       <c r="X42" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="Y42" t="n">
-        <v>0.4012137771393897</v>
+        <v>0.5987862228606103</v>
       </c>
       <c r="Z42" t="n">
-        <v>3.254716981132076</v>
+        <v>1.33</v>
       </c>
       <c r="AA42" t="inlineStr">
         <is>
-          <t>kelly_crit &lt; -0.5</t>
+          <t>kelly_crit &gt; nan</t>
         </is>
       </c>
       <c r="AB42" t="n">
-        <v>0.1356433184648094</v>
+        <v>-0.6170131018042065</v>
       </c>
       <c r="AC42" t="n">
-        <v>6.956519058680942</v>
+        <v>0</v>
       </c>
       <c r="AD42" t="n">
         <v>0.3042787295266122</v>
@@ -4831,14 +4831,14 @@
       </c>
       <c r="AA43" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; -0.5</t>
+          <t>kelly_crit &gt; nan</t>
         </is>
       </c>
       <c r="AB43" t="n">
         <v>-0.2611306018436721</v>
       </c>
       <c r="AC43" t="n">
-        <v>2.863061689324537</v>
+        <v>0</v>
       </c>
       <c r="AD43" t="n">
         <v>0.1632939770453267</v>
@@ -4923,24 +4923,24 @@
         <v>0</v>
       </c>
       <c r="X44" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="Y44" t="n">
-        <v>0.4706236147382553</v>
+        <v>0.5293763852617447</v>
       </c>
       <c r="Z44" t="n">
-        <v>2.853260869565217</v>
+        <v>1.4</v>
       </c>
       <c r="AA44" t="inlineStr">
         <is>
-          <t>kelly_crit &lt; -0.5</t>
+          <t>kelly_crit &gt; nan</t>
         </is>
       </c>
       <c r="AB44" t="n">
-        <v>0.1849777059753197</v>
+        <v>-0.6471826515838939</v>
       </c>
       <c r="AC44" t="n">
-        <v>7.446739911305725</v>
+        <v>0</v>
       </c>
       <c r="AD44" t="n">
         <v>0.2138669516926589</v>
@@ -5025,24 +5025,24 @@
         <v>0</v>
       </c>
       <c r="X45" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="Y45" t="n">
-        <v>0.5996563888016579</v>
+        <v>0.4003436111983421</v>
       </c>
       <c r="Z45" t="n">
-        <v>2.422685656154629</v>
+        <v>1.55</v>
       </c>
       <c r="AA45" t="inlineStr">
         <is>
-          <t>kelly_crit &lt; -0.5</t>
+          <t>kelly_crit &gt; nan</t>
         </is>
       </c>
       <c r="AB45" t="n">
-        <v>0.3182564818957086</v>
+        <v>-0.6899407320773997</v>
       </c>
       <c r="AC45" t="n">
-        <v>8.593863264347357</v>
+        <v>0</v>
       </c>
       <c r="AD45" t="n">
         <v>0.09144392883377045</v>
@@ -5127,24 +5127,24 @@
         <v>0</v>
       </c>
       <c r="X46" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="Y46" t="n">
-        <v>0.5504900490601686</v>
+        <v>0.4495099509398314</v>
       </c>
       <c r="Z46" t="n">
-        <v>3.148148148148148</v>
+        <v>1.33</v>
       </c>
       <c r="AA46" t="inlineStr">
         <is>
-          <t>kelly_crit &lt; -0.5</t>
+          <t>kelly_crit &gt; nan</t>
         </is>
       </c>
       <c r="AB46" t="n">
-        <v>0.3412354167261092</v>
+        <v>-1.218641712878861</v>
       </c>
       <c r="AC46" t="n">
-        <v>8.762178417386707</v>
+        <v>0</v>
       </c>
       <c r="AD46" t="n">
         <v>0.1493394923066809</v>
@@ -5229,24 +5229,24 @@
         <v>0</v>
       </c>
       <c r="X47" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="Y47" t="n">
-        <v>0.5036290605279977</v>
+        <v>0.4963709394720023</v>
       </c>
       <c r="Z47" t="n">
-        <v>4.085714285714285</v>
+        <v>1.22</v>
       </c>
       <c r="AA47" t="inlineStr">
         <is>
-          <t>kelly_crit &lt; -0.5</t>
+          <t>kelly_crit &gt; nan</t>
         </is>
       </c>
       <c r="AB47" t="n">
-        <v>0.3427681079213304</v>
+        <v>-1.792852062927988</v>
       </c>
       <c r="AC47" t="n">
-        <v>8.773087023625701</v>
+        <v>0</v>
       </c>
       <c r="AD47" t="n">
         <v>0.1907095766246527</v>
@@ -5341,14 +5341,14 @@
       </c>
       <c r="AA48" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; -0.5</t>
+          <t>kelly_crit &gt; nan</t>
         </is>
       </c>
       <c r="AB48" t="n">
         <v>-0.1423162105782112</v>
       </c>
       <c r="AC48" t="n">
-        <v>3.975471235447694</v>
+        <v>0</v>
       </c>
       <c r="AD48" t="n">
         <v>0.06045094485912922</v>
@@ -5443,14 +5443,14 @@
       </c>
       <c r="AA49" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; -10.0</t>
+          <t>kelly_crit &gt; nan</t>
         </is>
       </c>
       <c r="AB49" t="n">
         <v>0.09094787948197122</v>
       </c>
       <c r="AC49" t="n">
-        <v>6.489537370621322</v>
+        <v>5.26015585159255</v>
       </c>
       <c r="AD49" t="n">
         <v>0.01610800388827704</v>
@@ -5545,14 +5545,14 @@
       </c>
       <c r="AA50" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; -10.0</t>
+          <t>kelly_crit &gt; nan</t>
         </is>
       </c>
       <c r="AB50" t="n">
         <v>-1.12803788162436</v>
       </c>
       <c r="AC50" t="n">
-        <v>0.1307764035761723</v>
+        <v>0.5387498574106805</v>
       </c>
       <c r="AD50" t="n">
         <v>0.2849717873985828</v>
@@ -5647,14 +5647,14 @@
       </c>
       <c r="AA51" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; -10.0</t>
+          <t>kelly_crit &gt; nan</t>
         </is>
       </c>
       <c r="AB51" t="n">
         <v>0.00552387703070727</v>
       </c>
       <c r="AC51" t="n">
-        <v>4.715757265491916</v>
+        <v>6.430578089307159</v>
       </c>
       <c r="AD51" t="n">
         <v>0.1426523200520525</v>
@@ -5749,14 +5749,14 @@
       </c>
       <c r="AA52" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; -10.0</t>
+          <t>kelly_crit &gt; nan</t>
         </is>
       </c>
       <c r="AB52" t="n">
         <v>0.216334504420764</v>
       </c>
       <c r="AC52" t="n">
-        <v>5.572390826914181</v>
+        <v>7.598714763973883</v>
       </c>
       <c r="AD52" t="n">
         <v>0.2151014884798638</v>
@@ -5851,14 +5851,14 @@
       </c>
       <c r="AA53" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; -10.0</t>
+          <t>kelly_crit &gt; nan</t>
         </is>
       </c>
       <c r="AB53" t="n">
         <v>-0.1054936766237659</v>
       </c>
       <c r="AC53" t="n">
-        <v>4.746800198307363</v>
+        <v>6.889503474946152</v>
       </c>
       <c r="AD53" t="n">
         <v>0.2742636402449553</v>
@@ -5953,14 +5953,14 @@
       </c>
       <c r="AA54" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; -10.0</t>
+          <t>kelly_crit &gt; nan</t>
         </is>
       </c>
       <c r="AB54" t="n">
         <v>-0.007947123111376218</v>
       </c>
       <c r="AC54" t="n">
-        <v>5.656711522503302</v>
+        <v>7.744837316446358</v>
       </c>
       <c r="AD54" t="n">
         <v>0.2361229540488352</v>
@@ -6055,14 +6055,14 @@
       </c>
       <c r="AA55" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; -10.0</t>
+          <t>kelly_crit &gt; nan</t>
         </is>
       </c>
       <c r="AB55" t="n">
         <v>-0.1437069679327543</v>
       </c>
       <c r="AC55" t="n">
-        <v>3.07599355337678</v>
+        <v>4.587466410177922</v>
       </c>
       <c r="AD55" t="n">
         <v>0.0533468453555867</v>
@@ -6157,14 +6157,14 @@
       </c>
       <c r="AA56" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; -10.0</t>
+          <t>kelly_crit &gt; nan</t>
         </is>
       </c>
       <c r="AB56" t="n">
         <v>0.2275322714196271</v>
       </c>
       <c r="AC56" t="n">
-        <v>5.770987683455938</v>
+        <v>7.869528659258096</v>
       </c>
       <c r="AD56" t="n">
         <v>0.2448557819703636</v>
@@ -6259,14 +6259,14 @@
       </c>
       <c r="AA57" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; -10.0</t>
+          <t>kelly_crit &gt; nan</t>
         </is>
       </c>
       <c r="AB57" t="n">
         <v>0.1142294874243656</v>
       </c>
       <c r="AC57" t="n">
-        <v>4.504349574445349</v>
+        <v>6.142294874243656</v>
       </c>
       <c r="AD57" t="n">
         <v>0.1044685684304161</v>
@@ -6359,14 +6359,14 @@
       </c>
       <c r="AA58" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; -1</t>
+          <t>kelly_crit &gt; nan</t>
         </is>
       </c>
       <c r="AB58" t="n">
         <v>-0.1732770884572202</v>
       </c>
       <c r="AC58" t="n">
-        <v>6.680588811871746</v>
+        <v>0</v>
       </c>
       <c r="AD58" t="n">
         <v>0.4031282028609658</v>
@@ -6459,14 +6459,14 @@
       </c>
       <c r="AA59" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; -1</t>
+          <t>kelly_crit &gt; nan</t>
         </is>
       </c>
       <c r="AB59" t="n">
         <v>-0.05075108991396968</v>
       </c>
       <c r="AC59" t="n">
-        <v>4.149662727162155</v>
+        <v>0</v>
       </c>
       <c r="AD59" t="n">
         <v>0.05648088413622426</v>
@@ -6559,14 +6559,14 @@
       </c>
       <c r="AA60" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; -1</t>
+          <t>kelly_crit &gt; nan</t>
         </is>
       </c>
       <c r="AB60" t="n">
         <v>-0.8548140236693231</v>
       </c>
       <c r="AC60" t="n">
-        <v>3.755144135654018</v>
+        <v>0</v>
       </c>
       <c r="AD60" t="n">
         <v>0.249281062708837</v>
@@ -6663,14 +6663,14 @@
       </c>
       <c r="AA61" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; -1</t>
+          <t>kelly_crit &gt; nan</t>
         </is>
       </c>
       <c r="AB61" t="n">
         <v>-0.1489006481020879</v>
       </c>
       <c r="AC61" t="n">
-        <v>4.807456954409762</v>
+        <v>0</v>
       </c>
       <c r="AD61" t="n">
         <v>0.15564445901889</v>
@@ -6763,14 +6763,14 @@
       </c>
       <c r="AA62" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; -1</t>
+          <t>kelly_crit &gt; nan</t>
         </is>
       </c>
       <c r="AB62" t="n">
         <v>0.02971966905715935</v>
       </c>
       <c r="AC62" t="n">
-        <v>6.795451899247691</v>
+        <v>0</v>
       </c>
       <c r="AD62" t="n">
         <v>0.3354350532459212</v>
@@ -6863,14 +6863,14 @@
       </c>
       <c r="AA63" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; -1</t>
+          <t>kelly_crit &gt; nan</t>
         </is>
       </c>
       <c r="AB63" t="n">
         <v>-0.4268340307264248</v>
       </c>
       <c r="AC63" t="n">
-        <v>3.583386655863098</v>
+        <v>0</v>
       </c>
       <c r="AD63" t="n">
         <v>0.05862154007349846</v>
@@ -6963,14 +6963,14 @@
       </c>
       <c r="AA64" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; -1</t>
+          <t>kelly_crit &gt; nan</t>
         </is>
       </c>
       <c r="AB64" t="n">
         <v>-0.7291453354479848</v>
       </c>
       <c r="AC64" t="n">
-        <v>5.095421972633045</v>
+        <v>0</v>
       </c>
       <c r="AD64" t="n">
         <v>0.4718017330083224</v>
@@ -7063,14 +7063,14 @@
       </c>
       <c r="AA65" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; -1</t>
+          <t>kelly_crit &gt; nan</t>
         </is>
       </c>
       <c r="AB65" t="n">
         <v>-0.3984114256965124</v>
       </c>
       <c r="AC65" t="n">
-        <v>4.452123569682885</v>
+        <v>0</v>
       </c>
       <c r="AD65" t="n">
         <v>0.1481979428017515</v>
@@ -7167,14 +7167,14 @@
       </c>
       <c r="AA66" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; -1</t>
+          <t>kelly_crit &gt; nan</t>
         </is>
       </c>
       <c r="AB66" t="n">
         <v>-0.6696897002852222</v>
       </c>
       <c r="AC66" t="n">
-        <v>3.302920647035783</v>
+        <v>0</v>
       </c>
       <c r="AD66" t="n">
         <v>0.06987525583056364</v>
@@ -7267,14 +7267,14 @@
       </c>
       <c r="AA67" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; -10</t>
+          <t>kelly_crit &gt; nan</t>
         </is>
       </c>
       <c r="AB67" t="n">
         <v>0.2246592528594413</v>
       </c>
       <c r="AC67" t="n">
-        <v>6.115227483947542</v>
+        <v>6.790509736158789</v>
       </c>
       <c r="AD67" t="n">
         <v>0.1019585891065535</v>
@@ -7367,14 +7367,14 @@
       </c>
       <c r="AA68" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; -10</t>
+          <t>kelly_crit &gt; nan</t>
         </is>
       </c>
       <c r="AB68" t="n">
         <v>0.1458628476140506</v>
       </c>
       <c r="AC68" t="n">
-        <v>5.900413151026333</v>
+        <v>6.605893502413946</v>
       </c>
       <c r="AD68" t="n">
         <v>0.08263077214756703</v>
@@ -7467,14 +7467,14 @@
       </c>
       <c r="AA69" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; -10</t>
+          <t>kelly_crit &gt; nan</t>
         </is>
       </c>
       <c r="AB69" t="n">
         <v>0.1964016469855505</v>
       </c>
       <c r="AC69" t="n">
-        <v>6.038375051804252</v>
+        <v>6.491311556317593</v>
       </c>
       <c r="AD69" t="n">
         <v>0.07906431845824791</v>
@@ -7567,14 +7567,14 @@
       </c>
       <c r="AA70" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; -10</t>
+          <t>kelly_crit &gt; nan</t>
         </is>
       </c>
       <c r="AB70" t="n">
         <v>0.09850647071705937</v>
       </c>
       <c r="AC70" t="n">
-        <v>5.770673955575158</v>
+        <v>5.985064707170593</v>
       </c>
       <c r="AD70" t="n">
         <v>0.04941763182404901</v>
@@ -7671,14 +7671,14 @@
       </c>
       <c r="AA71" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; -10</t>
+          <t>kelly_crit &gt; nan</t>
         </is>
       </c>
       <c r="AB71" t="n">
         <v>-0.7684580421175504</v>
       </c>
       <c r="AC71" t="n">
-        <v>4.198932566860261</v>
+        <v>1.145163427325526</v>
       </c>
       <c r="AD71" t="n">
         <v>0.3235055588655411</v>
@@ -7771,14 +7771,14 @@
       </c>
       <c r="AA72" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; -10</t>
+          <t>kelly_crit &gt; nan</t>
         </is>
       </c>
       <c r="AB72" t="n">
         <v>0.07873112310110565</v>
       </c>
       <c r="AC72" t="n">
-        <v>5.272110895802528</v>
+        <v>1.437848426127962</v>
       </c>
       <c r="AD72" t="n">
         <v>0.1281733984414477</v>
@@ -7871,14 +7871,14 @@
       </c>
       <c r="AA73" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; -10</t>
+          <t>kelly_crit &gt; nan</t>
         </is>
       </c>
       <c r="AB73" t="n">
         <v>-0.05650137524077496</v>
       </c>
       <c r="AC73" t="n">
-        <v>4.306163062621609</v>
+        <v>1.174408107987711</v>
       </c>
       <c r="AD73" t="n">
         <v>0.04202552682753125</v>
@@ -7975,14 +7975,14 @@
       </c>
       <c r="AA74" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; -10</t>
+          <t>kelly_crit &gt; nan</t>
         </is>
       </c>
       <c r="AB74" t="n">
         <v>0.02978651465120086</v>
       </c>
       <c r="AC74" t="n">
-        <v>5.070917589535116</v>
+        <v>1.382977524418668</v>
       </c>
       <c r="AD74" t="n">
         <v>0.1244837321597994</v>
@@ -8075,14 +8075,14 @@
       </c>
       <c r="AA75" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; -10</t>
+          <t>kelly_crit &gt; nan</t>
         </is>
       </c>
       <c r="AB75" t="n">
         <v>-0.04882106249928279</v>
       </c>
       <c r="AC75" t="n">
-        <v>5.907767817711003</v>
+        <v>1.611209404830273</v>
       </c>
       <c r="AD75" t="n">
         <v>0.2161693090529785</v>
@@ -8175,14 +8175,14 @@
       </c>
       <c r="AA76" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; -10</t>
+          <t>kelly_crit &gt; nan</t>
         </is>
       </c>
       <c r="AB76" t="n">
         <v>0.04164717077363733</v>
       </c>
       <c r="AC76" t="n">
-        <v>5.977428366201106</v>
+        <v>1.630207736236665</v>
       </c>
       <c r="AD76" t="n">
         <v>0.2734880442224538</v>
@@ -8275,14 +8275,14 @@
       </c>
       <c r="AA77" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; -10</t>
+          <t>kelly_crit &gt; nan</t>
         </is>
       </c>
       <c r="AB77" t="n">
         <v>0.4063246228423841</v>
       </c>
       <c r="AC77" t="n">
-        <v>8.500699955422878</v>
+        <v>2.31837271511533</v>
       </c>
       <c r="AD77" t="n">
         <v>0.6038834255794184</v>
@@ -8379,14 +8379,14 @@
       </c>
       <c r="AA78" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; -0.75</t>
+          <t>kelly_crit &gt; nan</t>
         </is>
       </c>
       <c r="AB78" t="n">
         <v>-0.3445833281411935</v>
       </c>
       <c r="AC78" t="n">
-        <v>6.292462112920918</v>
+        <v>0</v>
       </c>
       <c r="AD78" t="n">
         <v>0.4717928283636509</v>
@@ -8483,14 +8483,14 @@
       </c>
       <c r="AA79" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; -0.75</t>
+          <t>kelly_crit &gt; nan</t>
         </is>
       </c>
       <c r="AB79" t="n">
         <v>-0.1944500805536382</v>
       </c>
       <c r="AC79" t="n">
-        <v>4.482153620907308</v>
+        <v>0</v>
       </c>
       <c r="AD79" t="n">
         <v>0.1425384656259607</v>
@@ -8587,14 +8587,14 @@
       </c>
       <c r="AA80" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; -0.75</t>
+          <t>kelly_crit &gt; nan</t>
         </is>
       </c>
       <c r="AB80" t="n">
         <v>-0.2308696183587648</v>
       </c>
       <c r="AC80" t="n">
-        <v>3.744060257832759</v>
+        <v>0</v>
       </c>
       <c r="AD80" t="n">
         <v>0.0571204317362829</v>
@@ -8691,14 +8691,14 @@
       </c>
       <c r="AA81" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; -0.75</t>
+          <t>kelly_crit &gt; nan</t>
         </is>
       </c>
       <c r="AB81" t="n">
         <v>-0.2002271675107855</v>
       </c>
       <c r="AC81" t="n">
-        <v>5.134122320398446</v>
+        <v>0</v>
       </c>
       <c r="AD81" t="n">
         <v>0.2373325519000442</v>
@@ -8795,14 +8795,14 @@
       </c>
       <c r="AA82" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; -0.75</t>
+          <t>kelly_crit &gt; nan</t>
         </is>
       </c>
       <c r="AB82" t="n">
         <v>-0.3948120660624269</v>
       </c>
       <c r="AC82" t="n">
-        <v>3.990019648698029</v>
+        <v>0</v>
       </c>
       <c r="AD82" t="n">
         <v>0.1398045665264039</v>
@@ -8899,14 +8899,14 @@
       </c>
       <c r="AA83" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; -0.75</t>
+          <t>kelly_crit &gt; nan</t>
         </is>
       </c>
       <c r="AB83" t="n">
         <v>-0.1508111444323127</v>
       </c>
       <c r="AC83" t="n">
-        <v>7.830872368220967</v>
+        <v>0</v>
       </c>
       <c r="AD83" t="n">
         <v>0.5954910923273432</v>
@@ -8993,24 +8993,24 @@
         <v>0</v>
       </c>
       <c r="X84" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="Y84" t="n">
-        <v>0.4452489738677701</v>
+        <v>0.5547510261322299</v>
       </c>
       <c r="Z84" t="n">
-        <v>3.275862068965517</v>
+        <v>1.3</v>
       </c>
       <c r="AA84" t="inlineStr">
         <is>
-          <t>kelly_crit &lt; -0.75</t>
+          <t>kelly_crit &gt; nan</t>
         </is>
       </c>
       <c r="AB84" t="n">
-        <v>0.2014947351126994</v>
+        <v>-0.92941222009367</v>
       </c>
       <c r="AC84" t="n">
-        <v>4.897738712545471</v>
+        <v>0</v>
       </c>
       <c r="AD84" t="n">
         <v>0.2567405293640926</v>
@@ -9107,14 +9107,14 @@
       </c>
       <c r="AA85" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; -0.75</t>
+          <t>kelly_crit &gt; nan</t>
         </is>
       </c>
       <c r="AB85" t="n">
         <v>-0.44699101676891</v>
       </c>
       <c r="AC85" t="n">
-        <v>4.554346389292879</v>
+        <v>0</v>
       </c>
       <c r="AD85" t="n">
         <v>0.2272563783116517</v>
@@ -9211,14 +9211,14 @@
       </c>
       <c r="AA86" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; -0.75</t>
+          <t>kelly_crit &gt; nan</t>
         </is>
       </c>
       <c r="AB86" t="n">
         <v>-0.6070556264472319</v>
       </c>
       <c r="AC86" t="n">
-        <v>5.265907425092557</v>
+        <v>0</v>
       </c>
       <c r="AD86" t="n">
         <v>0.4439893801718107</v>
@@ -9297,7 +9297,7 @@
       <c r="Z87" t="inlineStr"/>
       <c r="AA87" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; -0.75</t>
+          <t>kelly_crit &gt; nan</t>
         </is>
       </c>
       <c r="AB87" t="inlineStr"/>
@@ -9397,14 +9397,14 @@
       </c>
       <c r="AA88" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; -10.0</t>
+          <t>kelly_crit &gt; nan</t>
         </is>
       </c>
       <c r="AB88" t="n">
         <v>-0.01558971840228222</v>
       </c>
       <c r="AC88" t="n">
-        <v>5.457129142665542</v>
+        <v>5.515164243563603</v>
       </c>
       <c r="AD88" t="n">
         <v>0.01249233269740341</v>
@@ -9501,14 +9501,14 @@
       </c>
       <c r="AA89" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; -10.0</t>
+          <t>kelly_crit &gt; nan</t>
         </is>
       </c>
       <c r="AB89" t="n">
         <v>0.109683765186285</v>
       </c>
       <c r="AC89" t="n">
-        <v>5.801328319909799</v>
+        <v>5.254646618930956</v>
       </c>
       <c r="AD89" t="n">
         <v>0.00339082772239685</v>
@@ -9605,14 +9605,14 @@
       </c>
       <c r="AA90" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; -10.0</t>
+          <t>kelly_crit &gt; nan</t>
         </is>
       </c>
       <c r="AB90" t="n">
         <v>0.08573453563001551</v>
       </c>
       <c r="AC90" t="n">
-        <v>5.735625661880492</v>
+        <v>5.204298596035881</v>
       </c>
       <c r="AD90" t="n">
         <v>0.003568674968657148</v>
@@ -9709,14 +9709,14 @@
       </c>
       <c r="AA91" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; -10.0</t>
+          <t>kelly_crit &gt; nan</t>
         </is>
       </c>
       <c r="AB91" t="n">
         <v>0.05326736353348965</v>
       </c>
       <c r="AC91" t="n">
-        <v>5.646450622958104</v>
+        <v>5.532673635334896</v>
       </c>
       <c r="AD91" t="n">
         <v>0.02067249192923304</v>
@@ -9813,14 +9813,14 @@
       </c>
       <c r="AA92" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; -10.0</t>
+          <t>kelly_crit &gt; nan</t>
         </is>
       </c>
       <c r="AB92" t="n">
         <v>0.056627088530569</v>
       </c>
       <c r="AC92" t="n">
-        <v>5.655682894265867</v>
+        <v>5.414113964100943</v>
       </c>
       <c r="AD92" t="n">
         <v>0.01988380471222434</v>
@@ -9917,14 +9917,14 @@
       </c>
       <c r="AA93" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; -10.0</t>
+          <t>kelly_crit &gt; nan</t>
         </is>
       </c>
       <c r="AB93" t="n">
         <v>0.06088777782115085</v>
       </c>
       <c r="AC93" t="n">
-        <v>1.133477935651459</v>
+        <v>0.2022583529595462</v>
       </c>
       <c r="AD93" t="n">
         <v>0.004674757767190174</v>
@@ -10021,14 +10021,14 @@
       </c>
       <c r="AA94" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; -10.0</t>
+          <t>kelly_crit &gt; nan</t>
         </is>
       </c>
       <c r="AB94" t="n">
         <v>-0.2403382945052021</v>
       </c>
       <c r="AC94" t="n">
-        <v>4.842232835602879</v>
+        <v>1.451840764189412</v>
       </c>
       <c r="AD94" t="n">
         <v>0.2322647259665827</v>
@@ -10125,14 +10125,14 @@
       </c>
       <c r="AA95" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; -10.0</t>
+          <t>kelly_crit &gt; nan</t>
         </is>
       </c>
       <c r="AB95" t="n">
         <v>-0.2965086191668617</v>
       </c>
       <c r="AC95" t="n">
-        <v>4.690523213997715</v>
+        <v>1.054001594061126</v>
       </c>
       <c r="AD95" t="n">
         <v>0.07733861005289627</v>
@@ -10229,14 +10229,14 @@
       </c>
       <c r="AA96" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; -10.0</t>
+          <t>kelly_crit &gt; nan</t>
         </is>
       </c>
       <c r="AB96" t="n">
         <v>-0.07072898023423942</v>
       </c>
       <c r="AC96" t="n">
-        <v>1.061115269878881</v>
+        <v>0.2020931098197082</v>
       </c>
       <c r="AD96" t="n">
         <v>0.01020478379222362</v>
@@ -10333,14 +10333,14 @@
       </c>
       <c r="AA97" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; -10.0</t>
+          <t>kelly_crit &gt; nan</t>
         </is>
       </c>
       <c r="AB97" t="n">
         <v>-0.05546513437865862</v>
       </c>
       <c r="AC97" t="n">
-        <v>5.347509971574931</v>
+        <v>1.649162477056587</v>
       </c>
       <c r="AD97" t="n">
         <v>0.2283401038933406</v>
@@ -10437,14 +10437,14 @@
       </c>
       <c r="AA98" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; -10.0</t>
+          <t>kelly_crit &gt; nan</t>
         </is>
       </c>
       <c r="AB98" t="n">
         <v>0.03448727426994453</v>
       </c>
       <c r="AC98" t="n">
-        <v>1.118966121071149</v>
+        <v>0.2418021490803</v>
       </c>
       <c r="AD98" t="n">
         <v>0.001548808688201675</v>

</xml_diff>

<commit_message>
DATA. Actualizo preds tras cambio en bs
</commit_message>
<xml_diff>
--- a/data/predicciones.xlsx
+++ b/data/predicciones.xlsx
@@ -678,7 +678,7 @@
         <v>0.05610182298167751</v>
       </c>
       <c r="AC2" t="n">
-        <v>6.224977023536887</v>
+        <v>4.97998161882951</v>
       </c>
       <c r="AD2" t="n">
         <v>0.0475203353546983</v>
@@ -782,7 +782,7 @@
         <v>-0.5890497207890028</v>
       </c>
       <c r="AC3" t="n">
-        <v>3.422389006621919</v>
+        <v>1.696956870514444</v>
       </c>
       <c r="AD3" t="n">
         <v>0.1597783632506189</v>
@@ -882,7 +882,7 @@
         <v>-0.01828865791221341</v>
       </c>
       <c r="AC4" t="n">
-        <v>6.395137370735387</v>
+        <v>5.068480286786428</v>
       </c>
       <c r="AD4" t="n">
         <v>0.1066625259595653</v>
@@ -982,7 +982,7 @@
         <v>-0.0821077912897632</v>
       </c>
       <c r="AC5" t="n">
-        <v>4.83002646384587</v>
+        <v>3.693063241113356</v>
       </c>
       <c r="AD5" t="n">
         <v>0.01608021976647306</v>
@@ -1086,7 +1086,7 @@
         <v>-0.4396417359506044</v>
       </c>
       <c r="AC6" t="n">
-        <v>3.370413015362987</v>
+        <v>1.939540060160874</v>
       </c>
       <c r="AD6" t="n">
         <v>0.03964386541199916</v>
@@ -1186,7 +1186,7 @@
         <v>-0.6084545318772012</v>
       </c>
       <c r="AC7" t="n">
-        <v>3.278739600371491</v>
+        <v>1.593345850673302</v>
       </c>
       <c r="AD7" t="n">
         <v>0.1882890201682544</v>
@@ -1290,7 +1290,7 @@
         <v>-0.3106700791748478</v>
       </c>
       <c r="AC8" t="n">
-        <v>4.82605312381721</v>
+        <v>3.121105990265458</v>
       </c>
       <c r="AD8" t="n">
         <v>0.1614383030026024</v>
@@ -1394,7 +1394,7 @@
         <v>-1.200524279737471</v>
       </c>
       <c r="AC9" t="n">
-        <v>1.395697212180289</v>
+        <v>0.3568498918498898</v>
       </c>
       <c r="AD9" t="n">
         <v>0.226703371026734</v>
@@ -1498,7 +1498,7 @@
         <v>-0.363041385425679</v>
       </c>
       <c r="AC10" t="n">
-        <v>4.781851227079884</v>
+        <v>2.954078989383769</v>
       </c>
       <c r="AD10" t="n">
         <v>0.1327939036371711</v>
@@ -1602,7 +1602,7 @@
         <v>-0.9232560831056776</v>
       </c>
       <c r="AC11" t="n">
-        <v>2.137466046258008</v>
+        <v>0.7400338711591888</v>
       </c>
       <c r="AD11" t="n">
         <v>0.1792139082532195</v>
@@ -1706,7 +1706,7 @@
         <v>0.18561103342571</v>
       </c>
       <c r="AC12" t="n">
-        <v>6.04172136768281</v>
+        <v>4.833377094146248</v>
       </c>
       <c r="AD12" t="n">
         <v>0.03327718529956053</v>
@@ -1810,7 +1810,7 @@
         <v>0.1928382849474048</v>
       </c>
       <c r="AC13" t="n">
-        <v>6.351838767293624</v>
+        <v>5.081471013834898</v>
       </c>
       <c r="AD13" t="n">
         <v>0.1262998150582524</v>
@@ -1910,7 +1910,7 @@
         <v>0.1440085951474115</v>
       </c>
       <c r="AC14" t="n">
-        <v>5.45240356125959</v>
+        <v>4.361922849007672</v>
       </c>
       <c r="AD14" t="n">
         <v>0.02447410732311933</v>
@@ -2014,7 +2014,7 @@
         <v>-0.1658733795403367</v>
       </c>
       <c r="AC15" t="n">
-        <v>1.008464519323882</v>
+        <v>4.033858077295529</v>
       </c>
       <c r="AD15" t="n">
         <v>0.08513451733849159</v>
@@ -2114,7 +2114,7 @@
         <v>0.1156426371261935</v>
       </c>
       <c r="AC16" t="n">
-        <v>1.311681398150006</v>
+        <v>5.246725592600022</v>
       </c>
       <c r="AD16" t="n">
         <v>0.132421614048361</v>
@@ -2214,7 +2214,7 @@
         <v>-0.7009078098752155</v>
       </c>
       <c r="AC17" t="n">
-        <v>0.3244824452616725</v>
+        <v>1.29792978104669</v>
       </c>
       <c r="AD17" t="n">
         <v>0.1493386406208241</v>
@@ -2318,7 +2318,7 @@
         <v>-0.9123744201373019</v>
       </c>
       <c r="AC18" t="n">
-        <v>0.2390679198979126</v>
+        <v>0.9562716795916505</v>
       </c>
       <c r="AD18" t="n">
         <v>0.4139988942118152</v>
@@ -2418,7 +2418,7 @@
         <v>0.2204089136009099</v>
       </c>
       <c r="AC19" t="n">
-        <v>1.128981392642184</v>
+        <v>4.515925570568735</v>
       </c>
       <c r="AD19" t="n">
         <v>0.05616946011402418</v>
@@ -2522,7 +2522,7 @@
         <v>-0.3566989662887962</v>
       </c>
       <c r="AC20" t="n">
-        <v>0.7527277170109504</v>
+        <v>3.010910868043802</v>
       </c>
       <c r="AD20" t="n">
         <v>0.1718138070598556</v>
@@ -2615,14 +2615,14 @@
       </c>
       <c r="AA21" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; nan</t>
+          <t>kelly_crit &gt; -0.75</t>
         </is>
       </c>
       <c r="AB21" t="n">
         <v>-0.199253804795107</v>
       </c>
       <c r="AC21" t="n">
-        <v>5.174163523765907</v>
+        <v>4.139330819012725</v>
       </c>
       <c r="AD21" t="n">
         <v>0.2215758231191805</v>
@@ -2705,24 +2705,24 @@
       <c r="V22" t="inlineStr"/>
       <c r="W22" t="inlineStr"/>
       <c r="X22" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="Y22" t="n">
-        <v>0.7812963887462138</v>
+        <v>0.2187036112537862</v>
       </c>
       <c r="Z22" t="n">
-        <v>1.13</v>
+        <v>5.884615384615384</v>
       </c>
       <c r="AA22" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; nan</t>
+          <t>kelly_crit &lt; -0.75</t>
         </is>
       </c>
       <c r="AB22" t="n">
-        <v>-0.9010390824367587</v>
+        <v>0.05875316946322277</v>
       </c>
       <c r="AC22" t="n">
-        <v>1.471720151209845</v>
+        <v>2.624443335045435</v>
       </c>
       <c r="AD22" t="n">
         <v>0.6206085104737893</v>
@@ -2815,14 +2815,14 @@
       </c>
       <c r="AA23" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; nan</t>
+          <t>kelly_crit &gt; -0.75</t>
         </is>
       </c>
       <c r="AB23" t="n">
         <v>-0.488636850769212</v>
       </c>
       <c r="AC23" t="n">
-        <v>2.585805522047464</v>
+        <v>2.068644417637971</v>
       </c>
       <c r="AD23" t="n">
         <v>0.1843457787476404</v>
@@ -2905,24 +2905,24 @@
       <c r="V24" t="inlineStr"/>
       <c r="W24" t="inlineStr"/>
       <c r="X24" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="Y24" t="n">
-        <v>0.6283394597796286</v>
+        <v>0.3716605402203714</v>
       </c>
       <c r="Z24" t="n">
-        <v>1.2</v>
+        <v>4.421052631578947</v>
       </c>
       <c r="AA24" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; nan</t>
+          <t>kelly_crit &lt; -0.75</t>
         </is>
       </c>
       <c r="AB24" t="n">
-        <v>-1.229963241322229</v>
+        <v>0.1879920827463261</v>
       </c>
       <c r="AC24" t="n">
-        <v>0.459307644579751</v>
+        <v>4.459926482644457</v>
       </c>
       <c r="AD24" t="n">
         <v>0.3792207413399871</v>
@@ -3015,14 +3015,14 @@
       </c>
       <c r="AA25" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; nan</t>
+          <t>kelly_crit &gt; -0.75</t>
         </is>
       </c>
       <c r="AB25" t="n">
         <v>-0.4599822065758858</v>
       </c>
       <c r="AC25" t="n">
-        <v>3.175025873022762</v>
+        <v>2.540020698418209</v>
       </c>
       <c r="AD25" t="n">
         <v>0.2070563719858555</v>
@@ -3115,14 +3115,14 @@
       </c>
       <c r="AA26" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; nan</t>
+          <t>kelly_crit &gt; -0.75</t>
         </is>
       </c>
       <c r="AB26" t="n">
         <v>-0.1874671134080337</v>
       </c>
       <c r="AC26" t="n">
-        <v>7.328986373359086</v>
+        <v>5.863189098687268</v>
       </c>
       <c r="AD26" t="n">
         <v>0.4615877137351533</v>
@@ -3215,14 +3215,14 @@
       </c>
       <c r="AA27" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; nan</t>
+          <t>kelly_crit &gt; -0.75</t>
         </is>
       </c>
       <c r="AB27" t="n">
         <v>-0.3932803357471401</v>
       </c>
       <c r="AC27" t="n">
-        <v>4.451422737715436</v>
+        <v>3.56113819017235</v>
       </c>
       <c r="AD27" t="n">
         <v>0.3879417939777161</v>
@@ -3315,14 +3315,14 @@
       </c>
       <c r="AA28" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; nan</t>
+          <t>kelly_crit &gt; -0.75</t>
         </is>
       </c>
       <c r="AB28" t="n">
         <v>-0.4829447296605331</v>
       </c>
       <c r="AC28" t="n">
-        <v>2.532616664092473</v>
+        <v>2.026093331273979</v>
       </c>
       <c r="AD28" t="n">
         <v>0.07702642532127657</v>
@@ -3415,14 +3415,14 @@
       </c>
       <c r="AA29" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; nan</t>
+          <t>kelly_crit &gt; -0.75</t>
         </is>
       </c>
       <c r="AB29" t="n">
         <v>-0.4074011344866009</v>
       </c>
       <c r="AC29" t="n">
-        <v>2.87040603233396</v>
+        <v>2.296324825867168</v>
       </c>
       <c r="AD29" t="n">
         <v>0.1300301580715786</v>
@@ -3519,14 +3519,14 @@
       </c>
       <c r="AA30" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; nan</t>
+          <t>kelly_crit &gt; -0.75</t>
         </is>
       </c>
       <c r="AB30" t="n">
         <v>0.1701628009049046</v>
       </c>
       <c r="AC30" t="n">
-        <v>6.442303884331828</v>
+        <v>5.153843107465462</v>
       </c>
       <c r="AD30" t="n">
         <v>0.1054887282930089</v>
@@ -3619,14 +3619,14 @@
       </c>
       <c r="AA31" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; nan</t>
+          <t>kelly_crit &gt; -0.75</t>
         </is>
       </c>
       <c r="AB31" t="n">
         <v>-0.4249924191366971</v>
       </c>
       <c r="AC31" t="n">
-        <v>2.978839882460748</v>
+        <v>2.383071905968598</v>
       </c>
       <c r="AD31" t="n">
         <v>0.1374116151274458</v>
@@ -3726,7 +3726,7 @@
         <v>0.06777345912781428</v>
       </c>
       <c r="AC32" t="n">
-        <v>1.050799050903612</v>
+        <v>4.203196203614447</v>
       </c>
       <c r="AD32" t="n">
         <v>0.008343623630123309</v>
@@ -3826,7 +3826,7 @@
         <v>0.2722231155114644</v>
       </c>
       <c r="AC33" t="n">
-        <v>1.376497719217882</v>
+        <v>5.505990876871528</v>
       </c>
       <c r="AD33" t="n">
         <v>0.1701159480146994</v>
@@ -3926,7 +3926,7 @@
         <v>-0.1055793011504492</v>
       </c>
       <c r="AC34" t="n">
-        <v>5.481637394105801</v>
+        <v>3.902375363045672</v>
       </c>
       <c r="AD34" t="n">
         <v>0.01689370889332192</v>
@@ -4026,7 +4026,7 @@
         <v>-0.1605570311430063</v>
       </c>
       <c r="AC35" t="n">
-        <v>7.4899227882905</v>
+        <v>4.974634895254</v>
       </c>
       <c r="AD35" t="n">
         <v>0.1578070449665375</v>
@@ -4130,7 +4130,7 @@
         <v>-0.4951951710294946</v>
       </c>
       <c r="AC36" t="n">
-        <v>6.863929363405502</v>
+        <v>2.676691465059648</v>
       </c>
       <c r="AD36" t="n">
         <v>0.2991513135729987</v>
@@ -4230,7 +4230,7 @@
         <v>-0.5601814383906134</v>
       </c>
       <c r="AC37" t="n">
-        <v>5.706431449869343</v>
+        <v>1.972005052617056</v>
       </c>
       <c r="AD37" t="n">
         <v>0.1732475316508266</v>
@@ -4330,7 +4330,7 @@
         <v>0.04526611147022155</v>
       </c>
       <c r="AC38" t="n">
-        <v>9.103114217904309</v>
+        <v>7.282491374323447</v>
       </c>
       <c r="AD38" t="n">
         <v>0.2834144579195952</v>
@@ -4430,7 +4430,7 @@
         <v>-0.1145949371158925</v>
       </c>
       <c r="AC39" t="n">
-        <v>5.544012380482322</v>
+        <v>3.903678421228969</v>
       </c>
       <c r="AD39" t="n">
         <v>0.08122242239616234</v>
@@ -4496,13 +4496,13 @@
         <v>1</v>
       </c>
       <c r="Q40" t="n">
-        <v>0.307188243518748</v>
+        <v>0.3387318943245072</v>
       </c>
       <c r="R40" t="n">
-        <v>0.4746644912944168</v>
+        <v>0.4038356490092653</v>
       </c>
       <c r="S40" t="n">
-        <v>0.2181472651868351</v>
+        <v>0.2574324566662274</v>
       </c>
       <c r="T40" t="n">
         <v>1</v>
@@ -4511,37 +4511,35 @@
         <v>1</v>
       </c>
       <c r="V40" t="inlineStr"/>
-      <c r="W40" t="n">
-        <v>0</v>
-      </c>
+      <c r="W40" t="inlineStr"/>
       <c r="X40" t="n">
         <v>1</v>
       </c>
       <c r="Y40" t="n">
-        <v>0.4746644912944168</v>
+        <v>0.4038356490092653</v>
       </c>
       <c r="Z40" t="n">
         <v>1.91</v>
       </c>
       <c r="AA40" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; nan</t>
+          <t>kelly_crit &gt; -0.5</t>
         </is>
       </c>
       <c r="AB40" t="n">
-        <v>-0.1026272765139165</v>
+        <v>-0.2512900114201136</v>
       </c>
       <c r="AC40" t="n">
-        <v>0</v>
+        <v>3.101250617866383</v>
       </c>
       <c r="AD40" t="n">
-        <v>0.1674762477756688</v>
+        <v>0.06510375468475804</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="1" t="inlineStr">
         <is>
-          <t>SSDn5z4e</t>
+          <t>zHgZcJdS</t>
         </is>
       </c>
       <c r="B41" s="2" t="n">
@@ -4549,12 +4547,12 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>mainz</t>
+          <t>rb leipzig</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>wolfsburg</t>
+          <t>holstein kiel</t>
         </is>
       </c>
       <c r="E41" t="n">
@@ -4574,37 +4572,37 @@
         </is>
       </c>
       <c r="I41" t="n">
-        <v>2</v>
+        <v>1.33</v>
       </c>
       <c r="J41" t="n">
-        <v>3.6</v>
+        <v>5.75</v>
       </c>
       <c r="K41" t="n">
-        <v>3.6</v>
+        <v>7.5</v>
       </c>
       <c r="L41" t="n">
-        <v>0.4736842105263158</v>
+        <v>0.7099057574385776</v>
       </c>
       <c r="M41" t="n">
-        <v>0.2631578947368421</v>
+        <v>0.1642042882423145</v>
       </c>
       <c r="N41" t="n">
-        <v>0.2631578947368421</v>
+        <v>0.1258899543191078</v>
       </c>
       <c r="O41" t="n">
-        <v>0.05555555555555558</v>
+        <v>0.05912607605971454</v>
       </c>
       <c r="P41" t="n">
         <v>1</v>
       </c>
       <c r="Q41" t="n">
-        <v>0.3507135728089528</v>
+        <v>0.3140270563745143</v>
       </c>
       <c r="R41" t="n">
-        <v>0.4112468979270829</v>
+        <v>0.5636542385534805</v>
       </c>
       <c r="S41" t="n">
-        <v>0.2380395292639642</v>
+        <v>0.1223187050720052</v>
       </c>
       <c r="T41" t="n">
         <v>1</v>
@@ -4613,37 +4611,35 @@
         <v>1</v>
       </c>
       <c r="V41" t="inlineStr"/>
-      <c r="W41" t="n">
-        <v>0</v>
-      </c>
+      <c r="W41" t="inlineStr"/>
       <c r="X41" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="Y41" t="n">
-        <v>0.4112468979270829</v>
+        <v>0.4363457614465195</v>
       </c>
       <c r="Z41" t="n">
-        <v>2</v>
+        <v>3.254716981132076</v>
       </c>
       <c r="AA41" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; nan</t>
+          <t>kelly_crit &lt; -0.5</t>
         </is>
       </c>
       <c r="AB41" t="n">
-        <v>-0.1775062041458342</v>
+        <v>0.1863568522972771</v>
       </c>
       <c r="AC41" t="n">
-        <v>0</v>
+        <v>5.236149137358233</v>
       </c>
       <c r="AD41" t="n">
-        <v>0.06053332511813003</v>
+        <v>0.2496271821789662</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="1" t="inlineStr">
         <is>
-          <t>zHgZcJdS</t>
+          <t>S4VaEvs9</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
@@ -4651,12 +4647,12 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>rb leipzig</t>
+          <t>werder bremen</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>holstein kiel</t>
+          <t>bochum</t>
         </is>
       </c>
       <c r="E42" t="n">
@@ -4676,37 +4672,37 @@
         </is>
       </c>
       <c r="I42" t="n">
-        <v>1.33</v>
+        <v>1.7</v>
       </c>
       <c r="J42" t="n">
-        <v>5.75</v>
+        <v>4.1</v>
       </c>
       <c r="K42" t="n">
-        <v>7.5</v>
+        <v>4.5</v>
       </c>
       <c r="L42" t="n">
-        <v>0.7099057574385776</v>
+        <v>0.5579074690051407</v>
       </c>
       <c r="M42" t="n">
-        <v>0.1642042882423145</v>
+        <v>0.231327487148473</v>
       </c>
       <c r="N42" t="n">
-        <v>0.1258899543191078</v>
+        <v>0.2107650438463864</v>
       </c>
       <c r="O42" t="n">
-        <v>0.05912607605971454</v>
+        <v>0.05435995536425953</v>
       </c>
       <c r="P42" t="n">
         <v>1</v>
       </c>
       <c r="Q42" t="n">
-        <v>0.2983426582597553</v>
+        <v>0.3274521183422588</v>
       </c>
       <c r="R42" t="n">
-        <v>0.5923875656591518</v>
+        <v>0.4452668197440856</v>
       </c>
       <c r="S42" t="n">
-        <v>0.1092697760810929</v>
+        <v>0.2272810619136556</v>
       </c>
       <c r="T42" t="n">
         <v>1</v>
@@ -4715,50 +4711,48 @@
         <v>1</v>
       </c>
       <c r="V42" t="inlineStr"/>
-      <c r="W42" t="n">
-        <v>0</v>
-      </c>
+      <c r="W42" t="inlineStr"/>
       <c r="X42" t="n">
         <v>1</v>
       </c>
       <c r="Y42" t="n">
-        <v>0.5923875656591518</v>
+        <v>0.4452668197440856</v>
       </c>
       <c r="Z42" t="n">
-        <v>1.33</v>
+        <v>1.7</v>
       </c>
       <c r="AA42" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; nan</t>
+          <t>kelly_crit &gt; -0.5</t>
         </is>
       </c>
       <c r="AB42" t="n">
-        <v>-0.642801629313115</v>
+        <v>-0.3472091520500778</v>
       </c>
       <c r="AC42" t="n">
-        <v>0</v>
+        <v>2.787399827822841</v>
       </c>
       <c r="AD42" t="n">
-        <v>0.2940449073993965</v>
+        <v>0.1178147014018268</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="1" t="inlineStr">
         <is>
-          <t>S4VaEvs9</t>
+          <t>KlV5hcKk</t>
         </is>
       </c>
       <c r="B43" s="2" t="n">
-        <v>45766.4375</v>
+        <v>45767.52083333334</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>werder bremen</t>
+          <t>dortmund</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>bochum</t>
+          <t>b  monchengladbach</t>
         </is>
       </c>
       <c r="E43" t="n">
@@ -4778,37 +4772,37 @@
         </is>
       </c>
       <c r="I43" t="n">
-        <v>1.7</v>
+        <v>1.4</v>
       </c>
       <c r="J43" t="n">
-        <v>4.1</v>
+        <v>5.25</v>
       </c>
       <c r="K43" t="n">
-        <v>4.5</v>
+        <v>6.25</v>
       </c>
       <c r="L43" t="n">
-        <v>0.5579074690051407</v>
+        <v>0.6708407871198568</v>
       </c>
       <c r="M43" t="n">
-        <v>0.231327487148473</v>
+        <v>0.1788908765652951</v>
       </c>
       <c r="N43" t="n">
-        <v>0.2107650438463864</v>
+        <v>0.1502683363148479</v>
       </c>
       <c r="O43" t="n">
-        <v>0.05435995536425953</v>
+        <v>0.0647619047619048</v>
       </c>
       <c r="P43" t="n">
         <v>1</v>
       </c>
       <c r="Q43" t="n">
-        <v>0.3048045284282245</v>
+        <v>0.2607888107299002</v>
       </c>
       <c r="R43" t="n">
-        <v>0.465210475109153</v>
+        <v>0.6311863698871139</v>
       </c>
       <c r="S43" t="n">
-        <v>0.2299849964626226</v>
+        <v>0.1080248193829858</v>
       </c>
       <c r="T43" t="n">
         <v>1</v>
@@ -4817,50 +4811,48 @@
         <v>1</v>
       </c>
       <c r="V43" t="inlineStr"/>
-      <c r="W43" t="n">
-        <v>0</v>
-      </c>
+      <c r="W43" t="inlineStr"/>
       <c r="X43" t="n">
         <v>1</v>
       </c>
       <c r="Y43" t="n">
-        <v>0.465210475109153</v>
+        <v>0.6311863698871139</v>
       </c>
       <c r="Z43" t="n">
-        <v>1.7</v>
+        <v>1.4</v>
       </c>
       <c r="AA43" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; nan</t>
+          <t>kelly_crit &gt; -0.5</t>
         </is>
       </c>
       <c r="AB43" t="n">
-        <v>-0.2987745604491998</v>
+        <v>-0.2908477053951017</v>
       </c>
       <c r="AC43" t="n">
-        <v>0</v>
+        <v>4.464639850830803</v>
       </c>
       <c r="AD43" t="n">
-        <v>0.1604059466809285</v>
+        <v>0.3703975591572136</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="1" t="inlineStr">
         <is>
-          <t>KlV5hcKk</t>
+          <t>Mg5N6mu0</t>
         </is>
       </c>
       <c r="B44" s="2" t="n">
-        <v>45767.52083333334</v>
+        <v>45772.64583333334</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>dortmund</t>
+          <t>stuttgart</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>b  monchengladbach</t>
+          <t>heidenheim</t>
         </is>
       </c>
       <c r="E44" t="n">
@@ -4880,37 +4872,37 @@
         </is>
       </c>
       <c r="I44" t="n">
-        <v>1.4</v>
+        <v>1.53</v>
       </c>
       <c r="J44" t="n">
-        <v>5.25</v>
+        <v>4.33</v>
       </c>
       <c r="K44" t="n">
-        <v>6.25</v>
+        <v>5.75</v>
       </c>
       <c r="L44" t="n">
-        <v>0.6708407871198568</v>
+        <v>0.6174990513369328</v>
       </c>
       <c r="M44" t="n">
-        <v>0.1788908765652951</v>
+        <v>0.2181925054377615</v>
       </c>
       <c r="N44" t="n">
-        <v>0.1502683363148479</v>
+        <v>0.1643084432253056</v>
       </c>
       <c r="O44" t="n">
-        <v>0.0647619047619048</v>
+        <v>0.05845469693718108</v>
       </c>
       <c r="P44" t="n">
         <v>1</v>
       </c>
       <c r="Q44" t="n">
-        <v>0.3114290895736069</v>
+        <v>0.3460539559940009</v>
       </c>
       <c r="R44" t="n">
-        <v>0.53803674203723</v>
+        <v>0.4072697597688347</v>
       </c>
       <c r="S44" t="n">
-        <v>0.1505341683891631</v>
+        <v>0.2466762842371645</v>
       </c>
       <c r="T44" t="n">
         <v>1</v>
@@ -4919,50 +4911,48 @@
         <v>1</v>
       </c>
       <c r="V44" t="inlineStr"/>
-      <c r="W44" t="n">
-        <v>0</v>
-      </c>
+      <c r="W44" t="inlineStr"/>
       <c r="X44" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="Y44" t="n">
-        <v>0.53803674203723</v>
+        <v>0.5927302402311654</v>
       </c>
       <c r="Z44" t="n">
-        <v>1.4</v>
+        <v>2.46999007936508</v>
       </c>
       <c r="AA44" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; nan</t>
+          <t>kelly_crit &lt; -0.5</t>
         </is>
       </c>
       <c r="AB44" t="n">
-        <v>-0.6168714028696954</v>
+        <v>0.3156741121076727</v>
       </c>
       <c r="AC44" t="n">
-        <v>0</v>
+        <v>7.112762882773984</v>
       </c>
       <c r="AD44" t="n">
-        <v>0.2266076524636231</v>
+        <v>0.06121580377483377</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="1" t="inlineStr">
         <is>
-          <t>Mg5N6mu0</t>
+          <t>lt7F89Am</t>
         </is>
       </c>
       <c r="B45" s="2" t="n">
-        <v>45772.64583333334</v>
+        <v>45773.4375</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>stuttgart</t>
+          <t>bayer leverkusen</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>heidenheim</t>
+          <t>augsburg</t>
         </is>
       </c>
       <c r="E45" t="n">
@@ -4982,37 +4972,37 @@
         </is>
       </c>
       <c r="I45" t="n">
-        <v>1.53</v>
+        <v>1.33</v>
       </c>
       <c r="J45" t="n">
-        <v>4.33</v>
+        <v>5</v>
       </c>
       <c r="K45" t="n">
-        <v>5.75</v>
+        <v>8.5</v>
       </c>
       <c r="L45" t="n">
-        <v>0.6174990513369328</v>
+        <v>0.7030022330659168</v>
       </c>
       <c r="M45" t="n">
-        <v>0.2181925054377615</v>
+        <v>0.1869985939955339</v>
       </c>
       <c r="N45" t="n">
-        <v>0.1643084432253056</v>
+        <v>0.1099991729385493</v>
       </c>
       <c r="O45" t="n">
-        <v>0.05845469693718108</v>
+        <v>0.06952675807164965</v>
       </c>
       <c r="P45" t="n">
         <v>1</v>
       </c>
       <c r="Q45" t="n">
-        <v>0.3088996823645716</v>
+        <v>0.3010280537153352</v>
       </c>
       <c r="R45" t="n">
-        <v>0.4003436111983421</v>
+        <v>0.5923250640256479</v>
       </c>
       <c r="S45" t="n">
-        <v>0.2907567064370864</v>
+        <v>0.106646882259017</v>
       </c>
       <c r="T45" t="n">
         <v>1</v>
@@ -5021,37 +5011,35 @@
         <v>1</v>
       </c>
       <c r="V45" t="inlineStr"/>
-      <c r="W45" t="n">
-        <v>0</v>
-      </c>
+      <c r="W45" t="inlineStr"/>
       <c r="X45" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="Y45" t="n">
-        <v>0.4003436111983421</v>
+        <v>0.4076749359743521</v>
       </c>
       <c r="Z45" t="n">
-        <v>1.53</v>
+        <v>3.148148148148148</v>
       </c>
       <c r="AA45" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; nan</t>
+          <t>kelly_crit &lt; -0.5</t>
         </is>
       </c>
       <c r="AB45" t="n">
-        <v>-0.7310835374840313</v>
+        <v>0.1319374061693091</v>
       </c>
       <c r="AC45" t="n">
-        <v>0</v>
+        <v>4.892099231692225</v>
       </c>
       <c r="AD45" t="n">
-        <v>0.09144392883377045</v>
+        <v>0.2912970103103127</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="1" t="inlineStr">
         <is>
-          <t>lt7F89Am</t>
+          <t>ILbW4R9C</t>
         </is>
       </c>
       <c r="B46" s="2" t="n">
@@ -5059,12 +5047,12 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>bayer leverkusen</t>
+          <t>bayern munich</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>augsburg</t>
+          <t>mainz</t>
         </is>
       </c>
       <c r="E46" t="n">
@@ -5084,37 +5072,37 @@
         </is>
       </c>
       <c r="I46" t="n">
-        <v>1.33</v>
+        <v>1.22</v>
       </c>
       <c r="J46" t="n">
-        <v>5</v>
+        <v>6.5</v>
       </c>
       <c r="K46" t="n">
-        <v>8.5</v>
+        <v>11</v>
       </c>
       <c r="L46" t="n">
-        <v>0.7030022330659168</v>
+        <v>0.7700592353257942</v>
       </c>
       <c r="M46" t="n">
-        <v>0.1869985939955339</v>
+        <v>0.1445341949380722</v>
       </c>
       <c r="N46" t="n">
-        <v>0.1099991729385493</v>
+        <v>0.08540656973613354</v>
       </c>
       <c r="O46" t="n">
-        <v>0.06952675807164965</v>
+        <v>0.0644273759027858</v>
       </c>
       <c r="P46" t="n">
         <v>1</v>
       </c>
       <c r="Q46" t="n">
-        <v>0.3001704586331505</v>
+        <v>0.344678627424805</v>
       </c>
       <c r="R46" t="n">
-        <v>0.4495099509398314</v>
+        <v>0.4790770910139683</v>
       </c>
       <c r="S46" t="n">
-        <v>0.2503195904270181</v>
+        <v>0.1762442815612265</v>
       </c>
       <c r="T46" t="n">
         <v>1</v>
@@ -5123,50 +5111,48 @@
         <v>1</v>
       </c>
       <c r="V46" t="inlineStr"/>
-      <c r="W46" t="n">
-        <v>0</v>
-      </c>
+      <c r="W46" t="inlineStr"/>
       <c r="X46" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="Y46" t="n">
-        <v>0.4495099509398314</v>
+        <v>0.5209229089860317</v>
       </c>
       <c r="Z46" t="n">
-        <v>1.33</v>
+        <v>4.085714285714285</v>
       </c>
       <c r="AA46" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; nan</t>
+          <t>kelly_crit &lt; -0.5</t>
         </is>
       </c>
       <c r="AB46" t="n">
-        <v>-1.218641712878861</v>
+        <v>0.3656664443055789</v>
       </c>
       <c r="AC46" t="n">
-        <v>0</v>
+        <v>6.25107490783238</v>
       </c>
       <c r="AD46" t="n">
-        <v>0.1493394923066809</v>
+        <v>0.1343984635891633</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="1" t="inlineStr">
         <is>
-          <t>ILbW4R9C</t>
+          <t>xQHf5eLh</t>
         </is>
       </c>
       <c r="B47" s="2" t="n">
-        <v>45773.4375</v>
+        <v>45774.52083333334</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>bayern munich</t>
+          <t>werder bremen</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>mainz</t>
+          <t>st  pauli</t>
         </is>
       </c>
       <c r="E47" t="n">
@@ -5186,37 +5172,37 @@
         </is>
       </c>
       <c r="I47" t="n">
-        <v>1.22</v>
+        <v>2</v>
       </c>
       <c r="J47" t="n">
-        <v>6.5</v>
+        <v>3.5</v>
       </c>
       <c r="K47" t="n">
-        <v>11</v>
+        <v>3.6</v>
       </c>
       <c r="L47" t="n">
-        <v>0.7700592353257942</v>
+        <v>0.4701492537313433</v>
       </c>
       <c r="M47" t="n">
-        <v>0.1445341949380722</v>
+        <v>0.2686567164179104</v>
       </c>
       <c r="N47" t="n">
-        <v>0.08540656973613354</v>
+        <v>0.2611940298507463</v>
       </c>
       <c r="O47" t="n">
-        <v>0.0644273759027858</v>
+        <v>0.06349206349206349</v>
       </c>
       <c r="P47" t="n">
         <v>1</v>
       </c>
       <c r="Q47" t="n">
-        <v>0.3056613628473496</v>
+        <v>0.3406608067235813</v>
       </c>
       <c r="R47" t="n">
-        <v>0.4963709394720023</v>
+        <v>0.4127995200963983</v>
       </c>
       <c r="S47" t="n">
-        <v>0.1979676976806481</v>
+        <v>0.2465396731800205</v>
       </c>
       <c r="T47" t="n">
         <v>1</v>
@@ -5225,50 +5211,48 @@
         <v>1</v>
       </c>
       <c r="V47" t="inlineStr"/>
-      <c r="W47" t="n">
-        <v>0</v>
-      </c>
+      <c r="W47" t="inlineStr"/>
       <c r="X47" t="n">
         <v>1</v>
       </c>
       <c r="Y47" t="n">
-        <v>0.4963709394720023</v>
+        <v>0.4127995200963983</v>
       </c>
       <c r="Z47" t="n">
-        <v>1.22</v>
+        <v>2</v>
       </c>
       <c r="AA47" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; nan</t>
+          <t>kelly_crit &gt; -0.5</t>
         </is>
       </c>
       <c r="AB47" t="n">
-        <v>-1.792852062927988</v>
+        <v>-0.1744009598072034</v>
       </c>
       <c r="AC47" t="n">
-        <v>0</v>
+        <v>3.686500488945471</v>
       </c>
       <c r="AD47" t="n">
-        <v>0.1907095766246527</v>
+        <v>0.07213871337281691</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="1" t="inlineStr">
         <is>
-          <t>YiB33Zk5</t>
+          <t>SSDn5z4e</t>
         </is>
       </c>
       <c r="B48" s="2" t="n">
-        <v>45773.4375</v>
+        <v>45766.4375</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
+          <t>mainz</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
           <t>wolfsburg</t>
-        </is>
-      </c>
-      <c r="D48" t="inlineStr">
-        <is>
-          <t>freiburg</t>
         </is>
       </c>
       <c r="E48" t="n">
@@ -5288,56 +5272,54 @@
         </is>
       </c>
       <c r="I48" t="n">
-        <v>2.2</v>
+        <v>2</v>
       </c>
       <c r="J48" t="n">
-        <v>3.5</v>
+        <v>3.6</v>
       </c>
       <c r="K48" t="n">
-        <v>3.1</v>
+        <v>3.6</v>
       </c>
       <c r="L48" t="n">
-        <v>0.4276704769412693</v>
+        <v>0.4736842105263158</v>
       </c>
       <c r="M48" t="n">
-        <v>0.2688214426487978</v>
+        <v>0.2631578947368421</v>
       </c>
       <c r="N48" t="n">
-        <v>0.303508080409933</v>
+        <v>0.2631578947368421</v>
       </c>
       <c r="O48" t="n">
-        <v>0.06284038542103043</v>
+        <v>0.05555555555555558</v>
       </c>
       <c r="P48" t="n">
         <v>1</v>
       </c>
       <c r="Q48" t="n">
-        <v>0.3066140836717234</v>
+        <v>0.3877324588810543</v>
       </c>
       <c r="R48" t="n">
-        <v>0.3769184305937029</v>
+        <v>0.3140988573326658</v>
       </c>
       <c r="S48" t="n">
-        <v>0.3164674857345737</v>
+        <v>0.2981686837862798</v>
       </c>
       <c r="T48" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U48" t="n">
         <v>1</v>
       </c>
       <c r="V48" t="inlineStr"/>
-      <c r="W48" t="n">
+      <c r="W48" t="inlineStr"/>
+      <c r="X48" t="n">
         <v>0</v>
       </c>
-      <c r="X48" t="n">
-        <v>1</v>
-      </c>
       <c r="Y48" t="n">
-        <v>0.3769184305937029</v>
+        <v>0.3877324588810543</v>
       </c>
       <c r="Z48" t="n">
-        <v>2.2</v>
+        <v>3.6</v>
       </c>
       <c r="AA48" t="inlineStr">
         <is>
@@ -5345,32 +5327,32 @@
         </is>
       </c>
       <c r="AB48" t="n">
-        <v>-0.1423162105782112</v>
+        <v>0.1522449430660753</v>
       </c>
       <c r="AC48" t="n">
-        <v>0</v>
+        <v>4.652789506572652</v>
       </c>
       <c r="AD48" t="n">
-        <v>0.06045094485912922</v>
+        <v>0.07363360154838849</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="1" t="inlineStr">
         <is>
-          <t>xQHf5eLh</t>
+          <t>YiB33Zk5</t>
         </is>
       </c>
       <c r="B49" s="2" t="n">
-        <v>45774.52083333334</v>
+        <v>45773.4375</v>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>werder bremen</t>
+          <t>wolfsburg</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>st  pauli</t>
+          <t>freiburg</t>
         </is>
       </c>
       <c r="E49" t="n">
@@ -5390,37 +5372,37 @@
         </is>
       </c>
       <c r="I49" t="n">
-        <v>2</v>
+        <v>2.2</v>
       </c>
       <c r="J49" t="n">
         <v>3.5</v>
       </c>
       <c r="K49" t="n">
-        <v>3.6</v>
+        <v>3.1</v>
       </c>
       <c r="L49" t="n">
-        <v>0.4701492537313433</v>
+        <v>0.4276704769412693</v>
       </c>
       <c r="M49" t="n">
-        <v>0.2686567164179104</v>
+        <v>0.2688214426487978</v>
       </c>
       <c r="N49" t="n">
-        <v>0.2611940298507463</v>
+        <v>0.303508080409933</v>
       </c>
       <c r="O49" t="n">
-        <v>0.06349206349206349</v>
+        <v>0.06284038542103043</v>
       </c>
       <c r="P49" t="n">
         <v>1</v>
       </c>
       <c r="Q49" t="n">
-        <v>0.3506770567728366</v>
+        <v>0.3781433755138855</v>
       </c>
       <c r="R49" t="n">
-        <v>0.3147538903426039</v>
+        <v>0.259472351437267</v>
       </c>
       <c r="S49" t="n">
-        <v>0.3345690528845596</v>
+        <v>0.3623842730488475</v>
       </c>
       <c r="T49" t="n">
         <v>0</v>
@@ -5428,7 +5410,9 @@
       <c r="U49" t="n">
         <v>1</v>
       </c>
-      <c r="V49" t="inlineStr"/>
+      <c r="V49" t="n">
+        <v>1</v>
+      </c>
       <c r="W49" t="n">
         <v>0</v>
       </c>
@@ -5436,7 +5420,7 @@
         <v>0</v>
       </c>
       <c r="Y49" t="n">
-        <v>0.3506770567728366</v>
+        <v>0.3781433755138855</v>
       </c>
       <c r="Z49" t="n">
         <v>3.5</v>
@@ -5447,13 +5431,13 @@
         </is>
       </c>
       <c r="AB49" t="n">
-        <v>0.09094787948197122</v>
+        <v>0.1294007257194397</v>
       </c>
       <c r="AC49" t="n">
-        <v>5.26015585159255</v>
+        <v>4.537720506166625</v>
       </c>
       <c r="AD49" t="n">
-        <v>0.01610800388827704</v>
+        <v>0.01575910246503803</v>
       </c>
     </row>
     <row r="50">
@@ -5516,13 +5500,13 @@
         <v>2</v>
       </c>
       <c r="Q50" t="n">
-        <v>0.2632222380849683</v>
+        <v>0.2581203002874567</v>
       </c>
       <c r="R50" t="n">
-        <v>0.1900881843041213</v>
+        <v>0.08630053215225547</v>
       </c>
       <c r="S50" t="n">
-        <v>0.5466895776109104</v>
+        <v>0.6555791675602877</v>
       </c>
       <c r="T50" t="n">
         <v>2</v>
@@ -5531,31 +5515,29 @@
         <v>1</v>
       </c>
       <c r="V50" t="inlineStr"/>
-      <c r="W50" t="n">
-        <v>0</v>
-      </c>
+      <c r="W50" t="inlineStr"/>
       <c r="X50" t="n">
         <v>2</v>
       </c>
       <c r="Y50" t="n">
-        <v>0.5466895776109104</v>
+        <v>0.6555791675602877</v>
       </c>
       <c r="Z50" t="n">
         <v>1.3</v>
       </c>
       <c r="AA50" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; nan</t>
+          <t>kelly_crit &gt; -0.5</t>
         </is>
       </c>
       <c r="AB50" t="n">
-        <v>-0.9643451636860547</v>
+        <v>-0.4924902739054199</v>
       </c>
       <c r="AC50" t="n">
-        <v>0.8610183620272677</v>
+        <v>2.923511883247693</v>
       </c>
       <c r="AD50" t="n">
-        <v>0.2834673395259421</v>
+        <v>0.3974588672728309</v>
       </c>
     </row>
     <row r="51">
@@ -5618,13 +5600,13 @@
         <v>2</v>
       </c>
       <c r="Q51" t="n">
-        <v>0.2839612209862037</v>
+        <v>0.3894309156287546</v>
       </c>
       <c r="R51" t="n">
-        <v>0.2805913538979676</v>
+        <v>0.2143250278630489</v>
       </c>
       <c r="S51" t="n">
-        <v>0.4354474251158287</v>
+        <v>0.3962440565081966</v>
       </c>
       <c r="T51" t="n">
         <v>2</v>
@@ -5633,31 +5615,29 @@
         <v>1</v>
       </c>
       <c r="V51" t="inlineStr"/>
-      <c r="W51" t="n">
-        <v>0</v>
-      </c>
+      <c r="W51" t="inlineStr"/>
       <c r="X51" t="n">
         <v>2</v>
       </c>
       <c r="Y51" t="n">
-        <v>0.4354474251158287</v>
+        <v>0.3962440565081966</v>
       </c>
       <c r="Z51" t="n">
         <v>2.45</v>
       </c>
       <c r="AA51" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; nan</t>
+          <t>kelly_crit &gt; -0.5</t>
         </is>
       </c>
       <c r="AB51" t="n">
-        <v>0.04610082174743479</v>
+        <v>-0.0201393527964954</v>
       </c>
       <c r="AC51" t="n">
-        <v>6.531711376737431</v>
+        <v>0.9222661156061558</v>
       </c>
       <c r="AD51" t="n">
-        <v>0.151486204129625</v>
+        <v>0.006813140879441959</v>
       </c>
     </row>
     <row r="52">
@@ -5720,13 +5700,13 @@
         <v>1</v>
       </c>
       <c r="Q52" t="n">
-        <v>0.2871118423922772</v>
+        <v>0.3404501951035566</v>
       </c>
       <c r="R52" t="n">
-        <v>0.1913211259956003</v>
+        <v>0.2828049370707059</v>
       </c>
       <c r="S52" t="n">
-        <v>0.5215670316121221</v>
+        <v>0.3767448678257376</v>
       </c>
       <c r="T52" t="n">
         <v>2</v>
@@ -5735,31 +5715,29 @@
         <v>1</v>
       </c>
       <c r="V52" t="inlineStr"/>
-      <c r="W52" t="n">
-        <v>0</v>
-      </c>
+      <c r="W52" t="inlineStr"/>
       <c r="X52" t="n">
         <v>2</v>
       </c>
       <c r="Y52" t="n">
-        <v>0.5215670316121221</v>
+        <v>0.3767448678257376</v>
       </c>
       <c r="Z52" t="n">
         <v>2.75</v>
       </c>
       <c r="AA52" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; nan</t>
+          <t>kelly_crit &gt; -0.5</t>
         </is>
       </c>
       <c r="AB52" t="n">
-        <v>0.2481767639619063</v>
+        <v>0.02059907801187347</v>
       </c>
       <c r="AC52" t="n">
-        <v>7.823505474181832</v>
+        <v>4.520938413908851</v>
       </c>
       <c r="AD52" t="n">
-        <v>0.234455189219845</v>
+        <v>0.03629467272218106</v>
       </c>
     </row>
     <row r="53">
@@ -5822,13 +5800,13 @@
         <v>2</v>
       </c>
       <c r="Q53" t="n">
-        <v>0.2700677582342167</v>
+        <v>0.2204653809622818</v>
       </c>
       <c r="R53" t="n">
-        <v>0.1842993317068892</v>
+        <v>0.06859920483198191</v>
       </c>
       <c r="S53" t="n">
-        <v>0.5456329100588942</v>
+        <v>0.7109354142057362</v>
       </c>
       <c r="T53" t="n">
         <v>2</v>
@@ -5837,31 +5815,29 @@
         <v>1</v>
       </c>
       <c r="V53" t="inlineStr"/>
-      <c r="W53" t="n">
-        <v>0</v>
-      </c>
+      <c r="W53" t="inlineStr"/>
       <c r="X53" t="n">
         <v>2</v>
       </c>
       <c r="Y53" t="n">
-        <v>0.5456329100588942</v>
+        <v>0.7109354142057362</v>
       </c>
       <c r="Z53" t="n">
         <v>1.67</v>
       </c>
       <c r="AA53" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; nan</t>
+          <t>kelly_crit &gt; -0.5</t>
         </is>
       </c>
       <c r="AB53" t="n">
-        <v>-0.1325269256740995</v>
+        <v>0.2794957339157903</v>
       </c>
       <c r="AC53" t="n">
-        <v>6.578593243935606</v>
+        <v>8.531224970468836</v>
       </c>
       <c r="AD53" t="n">
-        <v>0.2755651518246776</v>
+        <v>0.4904700332434545</v>
       </c>
     </row>
     <row r="54">
@@ -5924,13 +5900,13 @@
         <v>2</v>
       </c>
       <c r="Q54" t="n">
-        <v>0.2864284086878813</v>
+        <v>0.3430213725602039</v>
       </c>
       <c r="R54" t="n">
-        <v>0.191020228575402</v>
+        <v>0.0984932446908233</v>
       </c>
       <c r="S54" t="n">
-        <v>0.5225513627367165</v>
+        <v>0.5584853827489729</v>
       </c>
       <c r="T54" t="n">
         <v>2</v>
@@ -5939,31 +5915,29 @@
         <v>1</v>
       </c>
       <c r="V54" t="inlineStr"/>
-      <c r="W54" t="n">
-        <v>0</v>
-      </c>
+      <c r="W54" t="inlineStr"/>
       <c r="X54" t="n">
         <v>2</v>
       </c>
       <c r="Y54" t="n">
-        <v>0.5225513627367165</v>
+        <v>0.5584853827489729</v>
       </c>
       <c r="Z54" t="n">
         <v>1.9</v>
       </c>
       <c r="AA54" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; nan</t>
+          <t>kelly_crit &gt; -0.5</t>
         </is>
       </c>
       <c r="AB54" t="n">
-        <v>-0.007947123111376218</v>
+        <v>0.06791358580338711</v>
       </c>
       <c r="AC54" t="n">
-        <v>7.744837316446358</v>
+        <v>6.701824592987674</v>
       </c>
       <c r="AD54" t="n">
-        <v>0.2361229540488352</v>
+        <v>0.215464010188769</v>
       </c>
     </row>
     <row r="55">
@@ -6026,13 +6000,13 @@
         <v>2</v>
       </c>
       <c r="Q55" t="n">
-        <v>0.3349029159827075</v>
+        <v>0.3047114956541098</v>
       </c>
       <c r="R55" t="n">
-        <v>0.2768473226789981</v>
+        <v>0.1819951953488748</v>
       </c>
       <c r="S55" t="n">
-        <v>0.3882497613382943</v>
+        <v>0.5132933089970154</v>
       </c>
       <c r="T55" t="n">
         <v>2</v>
@@ -6041,31 +6015,29 @@
         <v>1</v>
       </c>
       <c r="V55" t="inlineStr"/>
-      <c r="W55" t="n">
-        <v>0</v>
-      </c>
+      <c r="W55" t="inlineStr"/>
       <c r="X55" t="n">
         <v>2</v>
       </c>
       <c r="Y55" t="n">
-        <v>0.3882497613382943</v>
+        <v>0.5132933089970154</v>
       </c>
       <c r="Z55" t="n">
         <v>2.15</v>
       </c>
       <c r="AA55" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; nan</t>
+          <t>kelly_crit &gt; -0.5</t>
         </is>
       </c>
       <c r="AB55" t="n">
-        <v>-0.1437069679327543</v>
+        <v>0.09007009942920272</v>
       </c>
       <c r="AC55" t="n">
-        <v>4.587466410177922</v>
+        <v>6.159519707964185</v>
       </c>
       <c r="AD55" t="n">
-        <v>0.0533468453555867</v>
+        <v>0.2085818133429056</v>
       </c>
     </row>
     <row r="56">
@@ -6128,13 +6100,13 @@
         <v>1</v>
       </c>
       <c r="Q56" t="n">
-        <v>0.2797794619801762</v>
+        <v>0.3548048232869056</v>
       </c>
       <c r="R56" t="n">
-        <v>0.195585294069284</v>
+        <v>0.1763077266753668</v>
       </c>
       <c r="S56" t="n">
-        <v>0.5246352439505397</v>
+        <v>0.4688874500377275</v>
       </c>
       <c r="T56" t="n">
         <v>2</v>
@@ -6143,31 +6115,29 @@
         <v>1</v>
       </c>
       <c r="V56" t="inlineStr"/>
-      <c r="W56" t="n">
-        <v>0</v>
-      </c>
+      <c r="W56" t="inlineStr"/>
       <c r="X56" t="n">
         <v>2</v>
       </c>
       <c r="Y56" t="n">
-        <v>0.5246352439505397</v>
+        <v>0.4688874500377275</v>
       </c>
       <c r="Z56" t="n">
         <v>2.6</v>
       </c>
       <c r="AA56" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; nan</t>
+          <t>kelly_crit &gt; -0.5</t>
         </is>
       </c>
       <c r="AB56" t="n">
-        <v>0.2275322714196271</v>
+        <v>0.1369421063113073</v>
       </c>
       <c r="AC56" t="n">
-        <v>7.869528659258096</v>
+        <v>5.62664940045273</v>
       </c>
       <c r="AD56" t="n">
-        <v>0.2448557819703636</v>
+        <v>0.1140826267508219</v>
       </c>
     </row>
     <row r="57">
@@ -6230,13 +6200,13 @@
         <v>1</v>
       </c>
       <c r="Q57" t="n">
-        <v>0.2854959185312617</v>
+        <v>0.3422458158620744</v>
       </c>
       <c r="R57" t="n">
-        <v>0.305017756519161</v>
+        <v>0.2446956891123296</v>
       </c>
       <c r="S57" t="n">
-        <v>0.4094863249495771</v>
+        <v>0.413058495025596</v>
       </c>
       <c r="T57" t="n">
         <v>2</v>
@@ -6245,31 +6215,29 @@
         <v>1</v>
       </c>
       <c r="V57" t="inlineStr"/>
-      <c r="W57" t="n">
-        <v>0</v>
-      </c>
+      <c r="W57" t="inlineStr"/>
       <c r="X57" t="n">
         <v>2</v>
       </c>
       <c r="Y57" t="n">
-        <v>0.4094863249495771</v>
+        <v>0.413058495025596</v>
       </c>
       <c r="Z57" t="n">
         <v>3</v>
       </c>
       <c r="AA57" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; nan</t>
+          <t>kelly_crit &gt; -0.5</t>
         </is>
       </c>
       <c r="AB57" t="n">
-        <v>0.1142294874243656</v>
+        <v>0.119587742538394</v>
       </c>
       <c r="AC57" t="n">
-        <v>6.142294874243656</v>
+        <v>4.956701940307152</v>
       </c>
       <c r="AD57" t="n">
-        <v>0.1044685684304161</v>
+        <v>0.07081267916352157</v>
       </c>
     </row>
     <row r="58">
@@ -6359,14 +6327,14 @@
       </c>
       <c r="AA58" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; nan</t>
+          <t>kelly_crit &gt; -1.0</t>
         </is>
       </c>
       <c r="AB58" t="n">
         <v>-0.1420874953669795</v>
       </c>
       <c r="AC58" t="n">
-        <v>0</v>
+        <v>6.38688435386694</v>
       </c>
       <c r="AD58" t="n">
         <v>0.4147550257510424</v>
@@ -6459,14 +6427,14 @@
       </c>
       <c r="AA59" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; nan</t>
+          <t>kelly_crit &gt; -1.0</t>
         </is>
       </c>
       <c r="AB59" t="n">
         <v>-0.05075108991396968</v>
       </c>
       <c r="AC59" t="n">
-        <v>0</v>
+        <v>4.29183523092106</v>
       </c>
       <c r="AD59" t="n">
         <v>0.05648088413622426</v>
@@ -6559,14 +6527,14 @@
       </c>
       <c r="AA60" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; nan</t>
+          <t>kelly_crit &gt; -1.0</t>
         </is>
       </c>
       <c r="AB60" t="n">
         <v>-0.8548140236693231</v>
       </c>
       <c r="AC60" t="n">
-        <v>0</v>
+        <v>0.9809751063055085</v>
       </c>
       <c r="AD60" t="n">
         <v>0.249281062708837</v>
@@ -6663,14 +6631,14 @@
       </c>
       <c r="AA61" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; nan</t>
+          <t>kelly_crit &gt; -1.0</t>
         </is>
       </c>
       <c r="AB61" t="n">
         <v>-0.05574654149921598</v>
       </c>
       <c r="AC61" t="n">
-        <v>0</v>
+        <v>5.192872085829408</v>
       </c>
       <c r="AD61" t="n">
         <v>0.15564445901889</v>
@@ -6763,14 +6731,14 @@
       </c>
       <c r="AA62" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; nan</t>
+          <t>kelly_crit &gt; -1.0</t>
         </is>
       </c>
       <c r="AB62" t="n">
         <v>-0.4268340307264248</v>
       </c>
       <c r="AC62" t="n">
-        <v>0</v>
+        <v>2.152797373050863</v>
       </c>
       <c r="AD62" t="n">
         <v>0.05862154007349846</v>
@@ -6863,14 +6831,14 @@
       </c>
       <c r="AA63" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; nan</t>
+          <t>kelly_crit &gt; -1.0</t>
         </is>
       </c>
       <c r="AB63" t="n">
         <v>-0.3984114256965124</v>
       </c>
       <c r="AC63" t="n">
-        <v>0</v>
+        <v>2.809018541069217</v>
       </c>
       <c r="AD63" t="n">
         <v>0.1481979428017515</v>
@@ -6963,14 +6931,14 @@
       </c>
       <c r="AA64" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; nan</t>
+          <t>kelly_crit &gt; -1.0</t>
         </is>
       </c>
       <c r="AB64" t="n">
         <v>0.07172314658715247</v>
       </c>
       <c r="AC64" t="n">
-        <v>0</v>
+        <v>7.413220253724753</v>
       </c>
       <c r="AD64" t="n">
         <v>0.3354350532459212</v>
@@ -7063,14 +7031,14 @@
       </c>
       <c r="AA65" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; nan</t>
+          <t>kelly_crit &gt; -1.0</t>
         </is>
       </c>
       <c r="AB65" t="n">
         <v>-0.7626750181849787</v>
       </c>
       <c r="AC65" t="n">
-        <v>0</v>
+        <v>1.56136253754415</v>
       </c>
       <c r="AD65" t="n">
         <v>0.4624206523364852</v>
@@ -7167,14 +7135,14 @@
       </c>
       <c r="AA66" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; nan</t>
+          <t>kelly_crit &gt; -1.0</t>
         </is>
       </c>
       <c r="AB66" t="n">
         <v>-0.6696897002852222</v>
       </c>
       <c r="AC66" t="n">
-        <v>0</v>
+        <v>1.258516200435803</v>
       </c>
       <c r="AD66" t="n">
         <v>0.06987525583056364</v>
@@ -7274,7 +7242,7 @@
         <v>0.2136972114827007</v>
       </c>
       <c r="AC67" t="n">
-        <v>6.779561756410053</v>
+        <v>5.423649405128042</v>
       </c>
       <c r="AD67" t="n">
         <v>0.09984935434991021</v>
@@ -7374,7 +7342,7 @@
         <v>0.1642790273075228</v>
       </c>
       <c r="AC68" t="n">
-        <v>6.642790273075227</v>
+        <v>5.314232218460182</v>
       </c>
       <c r="AD68" t="n">
         <v>0.07579233952576409</v>
@@ -7474,7 +7442,7 @@
         <v>0.1900059851665848</v>
       </c>
       <c r="AC69" t="n">
-        <v>6.423592784116781</v>
+        <v>5.138874227293424</v>
       </c>
       <c r="AD69" t="n">
         <v>0.08779358491339201</v>
@@ -7574,7 +7542,7 @@
         <v>0.08084554458358401</v>
       </c>
       <c r="AC70" t="n">
-        <v>5.80845544583584</v>
+        <v>4.646764356668672</v>
       </c>
       <c r="AD70" t="n">
         <v>0.01899571727374888</v>
@@ -7678,7 +7646,7 @@
         <v>-0.8700060204188741</v>
       </c>
       <c r="AC71" t="n">
-        <v>1.067232888501066</v>
+        <v>7.229275979403817</v>
       </c>
       <c r="AD71" t="n">
         <v>0.3235055588655411</v>
@@ -7778,7 +7746,7 @@
         <v>0.1127190181399645</v>
       </c>
       <c r="AC72" t="n">
-        <v>1.495480074237331</v>
+        <v>5.981920296949324</v>
       </c>
       <c r="AD72" t="n">
         <v>0.1579860303398773</v>
@@ -7878,7 +7846,7 @@
         <v>0.01758708024595539</v>
       </c>
       <c r="AC73" t="n">
-        <v>1.20854114633086</v>
+        <v>4.83416458532344</v>
       </c>
       <c r="AD73" t="n">
         <v>0.04202552682753125</v>
@@ -7982,7 +7950,7 @@
         <v>0.02978651465120086</v>
       </c>
       <c r="AC74" t="n">
-        <v>1.382977524418668</v>
+        <v>5.531910097674672</v>
       </c>
       <c r="AD74" t="n">
         <v>0.1244837321597994</v>
@@ -8082,7 +8050,7 @@
         <v>-0.04882106249928279</v>
       </c>
       <c r="AC75" t="n">
-        <v>1.611209404830273</v>
+        <v>6.606063107146545</v>
       </c>
       <c r="AD75" t="n">
         <v>0.2161693090529785</v>
@@ -8182,7 +8150,7 @@
         <v>0.4336728528570153</v>
       </c>
       <c r="AC76" t="n">
-        <v>2.31837271511533</v>
+        <v>9.273490860461319</v>
       </c>
       <c r="AD76" t="n">
         <v>0.6038834255794184</v>
@@ -8282,7 +8250,7 @@
         <v>0.01368451163050348</v>
       </c>
       <c r="AC77" t="n">
-        <v>1.590240165838364</v>
+        <v>6.360960663353455</v>
       </c>
       <c r="AD77" t="n">
         <v>0.2517387598920544</v>
@@ -8348,13 +8316,13 @@
         <v>1</v>
       </c>
       <c r="Q78" t="n">
-        <v>0.2246459390421605</v>
+        <v>0.2002956064500629</v>
       </c>
       <c r="R78" t="n">
-        <v>0.6761607629301088</v>
+        <v>0.6552718807772617</v>
       </c>
       <c r="S78" t="n">
-        <v>0.09919329802773057</v>
+        <v>0.1444325127726751</v>
       </c>
       <c r="T78" t="n">
         <v>1</v>
@@ -8362,34 +8330,32 @@
       <c r="U78" t="n">
         <v>1</v>
       </c>
-      <c r="V78" t="n">
-        <v>0</v>
-      </c>
+      <c r="V78" t="inlineStr"/>
       <c r="W78" t="n">
         <v>0</v>
       </c>
       <c r="X78" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="Y78" t="n">
-        <v>0.6761607629301088</v>
+        <v>0.3447281192227383</v>
       </c>
       <c r="Z78" t="n">
-        <v>1.29</v>
+        <v>3.6</v>
       </c>
       <c r="AA78" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; nan</t>
+          <t>kelly_crit &lt; -0.25</t>
         </is>
       </c>
       <c r="AB78" t="n">
-        <v>-0.440526261448826</v>
+        <v>0.09270047276994529</v>
       </c>
       <c r="AC78" t="n">
-        <v>0</v>
+        <v>4.136737430672859</v>
       </c>
       <c r="AD78" t="n">
-        <v>0.4515148238879484</v>
+        <v>0.4549762743271988</v>
       </c>
     </row>
     <row r="79">
@@ -8452,13 +8418,13 @@
         <v>1</v>
       </c>
       <c r="Q79" t="n">
-        <v>0.3074355709566868</v>
+        <v>0.2224602001857862</v>
       </c>
       <c r="R79" t="n">
-        <v>0.4555848450702866</v>
+        <v>0.570987891147317</v>
       </c>
       <c r="S79" t="n">
-        <v>0.2369795839730266</v>
+        <v>0.2065519086668968</v>
       </c>
       <c r="T79" t="n">
         <v>1</v>
@@ -8466,9 +8432,7 @@
       <c r="U79" t="n">
         <v>1</v>
       </c>
-      <c r="V79" t="n">
-        <v>0</v>
-      </c>
+      <c r="V79" t="inlineStr"/>
       <c r="W79" t="n">
         <v>0</v>
       </c>
@@ -8476,24 +8440,24 @@
         <v>1</v>
       </c>
       <c r="Y79" t="n">
-        <v>0.4555848450702866</v>
+        <v>0.570987891147317</v>
       </c>
       <c r="Z79" t="n">
         <v>1.85</v>
       </c>
       <c r="AA79" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; nan</t>
+          <t>kelly_crit &gt; -0.25</t>
         </is>
       </c>
       <c r="AB79" t="n">
-        <v>-0.184903572494082</v>
+        <v>0.06626776308533699</v>
       </c>
       <c r="AC79" t="n">
-        <v>0</v>
+        <v>6.851854693767804</v>
       </c>
       <c r="AD79" t="n">
-        <v>0.1481492741135998</v>
+        <v>0.3485276909615307</v>
       </c>
     </row>
     <row r="80">
@@ -8556,13 +8520,13 @@
         <v>1</v>
       </c>
       <c r="Q80" t="n">
-        <v>0.3482094247689674</v>
+        <v>0.3223288397441358</v>
       </c>
       <c r="R80" t="n">
-        <v>0.3593156712942029</v>
+        <v>0.4956953179689862</v>
       </c>
       <c r="S80" t="n">
-        <v>0.2924749039368294</v>
+        <v>0.1819758422868781</v>
       </c>
       <c r="T80" t="n">
         <v>1</v>
@@ -8570,9 +8534,7 @@
       <c r="U80" t="n">
         <v>1</v>
       </c>
-      <c r="V80" t="n">
-        <v>0</v>
-      </c>
+      <c r="V80" t="inlineStr"/>
       <c r="W80" t="n">
         <v>0</v>
       </c>
@@ -8580,24 +8542,24 @@
         <v>1</v>
       </c>
       <c r="Y80" t="n">
-        <v>0.3593156712942029</v>
+        <v>0.4956953179689862</v>
       </c>
       <c r="Z80" t="n">
         <v>1.7</v>
       </c>
       <c r="AA80" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; nan</t>
+          <t>kelly_crit &gt; -0.25</t>
         </is>
       </c>
       <c r="AB80" t="n">
-        <v>-0.5559476554283643</v>
+        <v>-0.2247399420753192</v>
       </c>
       <c r="AC80" t="n">
-        <v>0</v>
+        <v>4.015757794059659</v>
       </c>
       <c r="AD80" t="n">
-        <v>0.01110624652523551</v>
+        <v>0.1733664782248504</v>
       </c>
     </row>
     <row r="81">
@@ -8660,13 +8622,13 @@
         <v>1</v>
       </c>
       <c r="Q81" t="n">
-        <v>0.3219364733830948</v>
+        <v>0.3084000926552674</v>
       </c>
       <c r="R81" t="n">
-        <v>0.4033734926664592</v>
+        <v>0.5394913456421024</v>
       </c>
       <c r="S81" t="n">
-        <v>0.2746900339504462</v>
+        <v>0.1521085617026303</v>
       </c>
       <c r="T81" t="n">
         <v>1</v>
@@ -8674,9 +8636,7 @@
       <c r="U81" t="n">
         <v>1</v>
       </c>
-      <c r="V81" t="n">
-        <v>0</v>
-      </c>
+      <c r="V81" t="inlineStr"/>
       <c r="W81" t="n">
         <v>0</v>
       </c>
@@ -8684,24 +8644,24 @@
         <v>1</v>
       </c>
       <c r="Y81" t="n">
-        <v>0.4033734926664592</v>
+        <v>0.5394913456421024</v>
       </c>
       <c r="Z81" t="n">
         <v>2.05</v>
       </c>
       <c r="AA81" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; nan</t>
+          <t>kelly_crit &gt; -0.25</t>
         </is>
       </c>
       <c r="AB81" t="n">
-        <v>-0.1648422286035798</v>
+        <v>0.1009116748250571</v>
       </c>
       <c r="AC81" t="n">
-        <v>0</v>
+        <v>6.473896147705229</v>
       </c>
       <c r="AD81" t="n">
-        <v>0.08143701928336439</v>
+        <v>0.231091252986835</v>
       </c>
     </row>
     <row r="82">
@@ -8764,13 +8724,13 @@
         <v>1</v>
       </c>
       <c r="Q82" t="n">
-        <v>0.2758782836971369</v>
+        <v>0.3012394946813111</v>
       </c>
       <c r="R82" t="n">
-        <v>0.534053591192615</v>
+        <v>0.5045751244294299</v>
       </c>
       <c r="S82" t="n">
-        <v>0.190068125110248</v>
+        <v>0.1941853808892587</v>
       </c>
       <c r="T82" t="n">
         <v>1</v>
@@ -8778,9 +8738,7 @@
       <c r="U82" t="n">
         <v>1</v>
       </c>
-      <c r="V82" t="n">
-        <v>0</v>
-      </c>
+      <c r="V82" t="inlineStr"/>
       <c r="W82" t="n">
         <v>0</v>
       </c>
@@ -8788,24 +8746,24 @@
         <v>1</v>
       </c>
       <c r="Y82" t="n">
-        <v>0.534053591192615</v>
+        <v>0.5045751244294299</v>
       </c>
       <c r="Z82" t="n">
         <v>1.67</v>
       </c>
       <c r="AA82" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; nan</t>
+          <t>kelly_crit &gt; -0.25</t>
         </is>
       </c>
       <c r="AB82" t="n">
-        <v>-0.1613888100124374</v>
+        <v>-0.2348649883624659</v>
       </c>
       <c r="AC82" t="n">
-        <v>0</v>
+        <v>4.005853237901506</v>
       </c>
       <c r="AD82" t="n">
-        <v>0.2581753074954781</v>
+        <v>0.2033356297481188</v>
       </c>
     </row>
     <row r="83">
@@ -8868,13 +8826,13 @@
         <v>1</v>
       </c>
       <c r="Q83" t="n">
-        <v>0.3107240135096098</v>
+        <v>0.3330112939461005</v>
       </c>
       <c r="R83" t="n">
-        <v>0.4505285800360137</v>
+        <v>0.4612112887789009</v>
       </c>
       <c r="S83" t="n">
-        <v>0.2387474064543763</v>
+        <v>0.2057774172749982</v>
       </c>
       <c r="T83" t="n">
         <v>1</v>
@@ -8882,34 +8840,32 @@
       <c r="U83" t="n">
         <v>1</v>
       </c>
-      <c r="V83" t="n">
-        <v>0</v>
-      </c>
+      <c r="V83" t="inlineStr"/>
       <c r="W83" t="n">
         <v>0</v>
       </c>
       <c r="X83" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="Y83" t="n">
-        <v>0.4505285800360137</v>
+        <v>0.5387887112210992</v>
       </c>
       <c r="Z83" t="n">
-        <v>1.7</v>
+        <v>2.1</v>
       </c>
       <c r="AA83" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; nan</t>
+          <t>kelly_crit &lt; -0.25</t>
         </is>
       </c>
       <c r="AB83" t="n">
-        <v>-0.3344305913411096</v>
+        <v>0.1195057214220985</v>
       </c>
       <c r="AC83" t="n">
-        <v>0</v>
+        <v>6.46546453465319</v>
       </c>
       <c r="AD83" t="n">
-        <v>0.1398045665264039</v>
+        <v>0.1281999948328004</v>
       </c>
     </row>
     <row r="84">
@@ -8972,13 +8928,13 @@
         <v>1</v>
       </c>
       <c r="Q84" t="n">
-        <v>0.1743466787861942</v>
+        <v>0.2647317529359469</v>
       </c>
       <c r="R84" t="n">
-        <v>0.7698377711135375</v>
+        <v>0.6001761667043215</v>
       </c>
       <c r="S84" t="n">
-        <v>0.0558155501002684</v>
+        <v>0.1350920803597314</v>
       </c>
       <c r="T84" t="n">
         <v>1</v>
@@ -8986,34 +8942,32 @@
       <c r="U84" t="n">
         <v>1</v>
       </c>
-      <c r="V84" t="n">
-        <v>0</v>
-      </c>
+      <c r="V84" t="inlineStr"/>
       <c r="W84" t="n">
         <v>0</v>
       </c>
       <c r="X84" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="Y84" t="n">
-        <v>0.7698377711135375</v>
+        <v>0.3998238332956785</v>
       </c>
       <c r="Z84" t="n">
-        <v>1.2</v>
+        <v>4.333333333333333</v>
       </c>
       <c r="AA84" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; nan</t>
+          <t>kelly_crit &lt; -0.25</t>
         </is>
       </c>
       <c r="AB84" t="n">
-        <v>-0.3809733733187755</v>
+        <v>0.219770983284382</v>
       </c>
       <c r="AC84" t="n">
-        <v>0</v>
+        <v>4.797885999548142</v>
       </c>
       <c r="AD84" t="n">
-        <v>0.5954910923273432</v>
+        <v>0.3354444137683746</v>
       </c>
     </row>
     <row r="85">
@@ -9076,13 +9030,13 @@
         <v>1</v>
       </c>
       <c r="Q85" t="n">
-        <v>0.2980104967681373</v>
+        <v>0.2563850506016223</v>
       </c>
       <c r="R85" t="n">
-        <v>0.5547510261322299</v>
+        <v>0.5553108472221264</v>
       </c>
       <c r="S85" t="n">
-        <v>0.1472384770996327</v>
+        <v>0.1883041021762514</v>
       </c>
       <c r="T85" t="n">
         <v>1</v>
@@ -9090,34 +9044,32 @@
       <c r="U85" t="n">
         <v>1</v>
       </c>
-      <c r="V85" t="n">
-        <v>0</v>
-      </c>
+      <c r="V85" t="inlineStr"/>
       <c r="W85" t="n">
         <v>0</v>
       </c>
       <c r="X85" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="Y85" t="n">
-        <v>0.5547510261322299</v>
+        <v>0.4446891527778736</v>
       </c>
       <c r="Z85" t="n">
-        <v>1.3</v>
+        <v>3.275862068965517</v>
       </c>
       <c r="AA85" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; nan</t>
+          <t>kelly_crit &lt; -0.25</t>
         </is>
       </c>
       <c r="AB85" t="n">
-        <v>-0.92941222009367</v>
+        <v>0.2006889320287575</v>
       </c>
       <c r="AC85" t="n">
-        <v>0</v>
+        <v>5.336269833334482</v>
       </c>
       <c r="AD85" t="n">
-        <v>0.2567405293640926</v>
+        <v>0.2989257966205041</v>
       </c>
     </row>
     <row r="86">
@@ -9180,13 +9132,13 @@
         <v>1</v>
       </c>
       <c r="Q86" t="n">
-        <v>0.3034492378714045</v>
+        <v>0.2178790120684078</v>
       </c>
       <c r="R86" t="n">
-        <v>0.5307056161830562</v>
+        <v>0.5973856507462741</v>
       </c>
       <c r="S86" t="n">
-        <v>0.1658451459455393</v>
+        <v>0.184735337185318</v>
       </c>
       <c r="T86" t="n">
         <v>1</v>
@@ -9194,9 +9146,7 @@
       <c r="U86" t="n">
         <v>1</v>
       </c>
-      <c r="V86" t="n">
-        <v>0</v>
-      </c>
+      <c r="V86" t="inlineStr"/>
       <c r="W86" t="n">
         <v>0</v>
       </c>
@@ -9204,24 +9154,24 @@
         <v>1</v>
       </c>
       <c r="Y86" t="n">
-        <v>0.5307056161830562</v>
+        <v>0.5973856507462741</v>
       </c>
       <c r="Z86" t="n">
         <v>1.53</v>
       </c>
       <c r="AA86" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; nan</t>
+          <t>kelly_crit &gt; -0.25</t>
         </is>
       </c>
       <c r="AB86" t="n">
-        <v>-0.3547554853583471</v>
+        <v>-0.1622640648267935</v>
       </c>
       <c r="AC86" t="n">
-        <v>0</v>
+        <v>5.457469688020315</v>
       </c>
       <c r="AD86" t="n">
-        <v>0.2272563783116517</v>
+        <v>0.3795066386778663</v>
       </c>
     </row>
     <row r="87">
@@ -9284,13 +9234,13 @@
         <v>1</v>
       </c>
       <c r="Q87" t="n">
-        <v>0.234599494538743</v>
+        <v>0.2774930654895853</v>
       </c>
       <c r="R87" t="n">
-        <v>0.6785888747105536</v>
+        <v>0.5351348332317637</v>
       </c>
       <c r="S87" t="n">
-        <v>0.08681163075070339</v>
+        <v>0.1873721012786508</v>
       </c>
       <c r="T87" t="n">
         <v>1</v>
@@ -9298,34 +9248,32 @@
       <c r="U87" t="n">
         <v>1</v>
       </c>
-      <c r="V87" t="n">
-        <v>0</v>
-      </c>
+      <c r="V87" t="inlineStr"/>
       <c r="W87" t="n">
         <v>0</v>
       </c>
       <c r="X87" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="Y87" t="n">
-        <v>0.6785888747105536</v>
+        <v>0.4648651667682363</v>
       </c>
       <c r="Z87" t="n">
-        <v>1.25</v>
+        <v>3.771428571428571</v>
       </c>
       <c r="AA87" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; nan</t>
+          <t>kelly_crit &lt; -0.25</t>
         </is>
       </c>
       <c r="AB87" t="n">
-        <v>-0.6070556264472319</v>
+        <v>0.2717752784887339</v>
       </c>
       <c r="AC87" t="n">
-        <v>0</v>
+        <v>5.578382001218835</v>
       </c>
       <c r="AD87" t="n">
-        <v>0.4439893801718107</v>
+        <v>0.2576417677421784</v>
       </c>
     </row>
     <row r="88">
@@ -9388,13 +9336,13 @@
         <v>1</v>
       </c>
       <c r="Q88" t="n">
-        <v>0.2830101168027956</v>
+        <v>0.3242055335780573</v>
       </c>
       <c r="R88" t="n">
-        <v>0.4969307686874934</v>
+        <v>0.4204115773666476</v>
       </c>
       <c r="S88" t="n">
-        <v>0.220059114509711</v>
+        <v>0.2553828890552952</v>
       </c>
       <c r="T88" t="n">
         <v>1</v>
@@ -9402,53 +9350,51 @@
       <c r="U88" t="n">
         <v>1</v>
       </c>
-      <c r="V88" t="n">
-        <v>0</v>
-      </c>
+      <c r="V88" t="inlineStr"/>
       <c r="W88" t="n">
         <v>0</v>
       </c>
       <c r="X88" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="Y88" t="n">
-        <v>0.4969307686874934</v>
+        <v>0.5795884226333523</v>
       </c>
       <c r="Z88" t="n">
-        <v>1.5</v>
+        <v>2.857824956672444</v>
       </c>
       <c r="AA88" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; nan</t>
+          <t>kelly_crit &lt; -0.25</t>
         </is>
       </c>
       <c r="AB88" t="n">
-        <v>-0.5092076939375197</v>
+        <v>0.3532960715392814</v>
       </c>
       <c r="AC88" t="n">
-        <v>0</v>
+        <v>6.955061071600228</v>
       </c>
       <c r="AD88" t="n">
-        <v>0.2139206518846978</v>
+        <v>0.09620604378859038</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="1" t="inlineStr">
         <is>
-          <t>GxrkL96E</t>
+          <t>EDNevsM6</t>
         </is>
       </c>
       <c r="B89" s="2" t="n">
-        <v>45765.66666666666</v>
+        <v>45768.66666666666</v>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>espanyol</t>
+          <t>girona</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>getafe</t>
+          <t>betis</t>
         </is>
       </c>
       <c r="E89" t="n">
@@ -9468,37 +9414,37 @@
         </is>
       </c>
       <c r="I89" t="n">
-        <v>2.9</v>
+        <v>2.88</v>
       </c>
       <c r="J89" t="n">
-        <v>2.63</v>
+        <v>3.3</v>
       </c>
       <c r="K89" t="n">
-        <v>3</v>
+        <v>2.45</v>
       </c>
       <c r="L89" t="n">
-        <v>0.3258041871412644</v>
+        <v>0.328058429701765</v>
       </c>
       <c r="M89" t="n">
-        <v>0.3592517652888467</v>
+        <v>0.2863055386488131</v>
       </c>
       <c r="N89" t="n">
-        <v>0.3149440475698889</v>
+        <v>0.3856360316494217</v>
       </c>
       <c r="O89" t="n">
-        <v>0.05838905642235925</v>
+        <v>0.05841579055864776</v>
       </c>
       <c r="P89" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="Q89" t="n">
-        <v>0.3708606139538387</v>
+        <v>0.365802189358198</v>
       </c>
       <c r="R89" t="n">
-        <v>0.2675596903211992</v>
+        <v>0.3508979587066263</v>
       </c>
       <c r="S89" t="n">
-        <v>0.3615796957249618</v>
+        <v>0.2832998519351756</v>
       </c>
       <c r="T89" t="n">
         <v>0</v>
@@ -9506,9 +9452,7 @@
       <c r="U89" t="n">
         <v>1</v>
       </c>
-      <c r="V89" t="n">
-        <v>0</v>
-      </c>
+      <c r="V89" t="inlineStr"/>
       <c r="W89" t="n">
         <v>0</v>
       </c>
@@ -9516,10 +9460,10 @@
         <v>0</v>
       </c>
       <c r="Y89" t="n">
-        <v>0.3708606139538387</v>
+        <v>0.365802189358198</v>
       </c>
       <c r="Z89" t="n">
-        <v>2.63</v>
+        <v>3.3</v>
       </c>
       <c r="AA89" t="inlineStr">
         <is>
@@ -9527,32 +9471,32 @@
         </is>
       </c>
       <c r="AB89" t="n">
-        <v>-0.01511446951006387</v>
+        <v>0.09006401081828404</v>
       </c>
       <c r="AC89" t="n">
-        <v>5.520869798804294</v>
+        <v>4.389626272298376</v>
       </c>
       <c r="AD89" t="n">
-        <v>0.009280918228876889</v>
+        <v>0.01490423065157165</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="1" t="inlineStr">
         <is>
-          <t>0AcMPs7D</t>
+          <t>GxrkL96E</t>
         </is>
       </c>
       <c r="B90" s="2" t="n">
-        <v>45766.375</v>
+        <v>45765.66666666666</v>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>rayo vallecano</t>
+          <t>espanyol</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>valencia</t>
+          <t>getafe</t>
         </is>
       </c>
       <c r="E90" t="n">
@@ -9572,58 +9516,56 @@
         </is>
       </c>
       <c r="I90" t="n">
-        <v>2.3</v>
+        <v>2.9</v>
       </c>
       <c r="J90" t="n">
-        <v>3.1</v>
+        <v>2.63</v>
       </c>
       <c r="K90" t="n">
-        <v>3.4</v>
+        <v>3</v>
       </c>
       <c r="L90" t="n">
-        <v>0.413495488426834</v>
+        <v>0.3258041871412644</v>
       </c>
       <c r="M90" t="n">
-        <v>0.3067869752844252</v>
+        <v>0.3592517652888467</v>
       </c>
       <c r="N90" t="n">
-        <v>0.2797175362887406</v>
+        <v>0.3149440475698889</v>
       </c>
       <c r="O90" t="n">
-        <v>0.05148090091576618</v>
+        <v>0.05838905642235925</v>
       </c>
       <c r="P90" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q90" t="n">
-        <v>0.3333333333333333</v>
+        <v>0.273948032872772</v>
       </c>
       <c r="R90" t="n">
-        <v>0.3333333333333333</v>
+        <v>0.262177856656036</v>
       </c>
       <c r="S90" t="n">
-        <v>0.3333333333333333</v>
+        <v>0.4638741104711918</v>
       </c>
       <c r="T90" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="U90" t="n">
         <v>1</v>
       </c>
-      <c r="V90" t="n">
-        <v>0</v>
-      </c>
+      <c r="V90" t="inlineStr"/>
       <c r="W90" t="n">
         <v>0</v>
       </c>
       <c r="X90" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="Y90" t="n">
-        <v>0.3333333333333333</v>
+        <v>0.4638741104711918</v>
       </c>
       <c r="Z90" t="n">
-        <v>3.1</v>
+        <v>3</v>
       </c>
       <c r="AA90" t="inlineStr">
         <is>
@@ -9631,32 +9573,32 @@
         </is>
       </c>
       <c r="AB90" t="n">
-        <v>0.01587301587301582</v>
+        <v>0.1958111657067877</v>
       </c>
       <c r="AC90" t="n">
-        <v>4.999999999999999</v>
+        <v>5.566489325654302</v>
       </c>
       <c r="AD90" t="n">
-        <v>0</v>
+        <v>0.1899260775984198</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="1" t="inlineStr">
         <is>
-          <t>Qol45JK5</t>
+          <t>0AcMPs7D</t>
         </is>
       </c>
       <c r="B91" s="2" t="n">
-        <v>45770.58333333334</v>
+        <v>45766.375</v>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>celta vigo</t>
+          <t>rayo vallecano</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>villarreal</t>
+          <t>valencia</t>
         </is>
       </c>
       <c r="E91" t="n">
@@ -9676,58 +9618,56 @@
         </is>
       </c>
       <c r="I91" t="n">
-        <v>2.4</v>
+        <v>2.3</v>
       </c>
       <c r="J91" t="n">
-        <v>3.5</v>
+        <v>3.1</v>
       </c>
       <c r="K91" t="n">
-        <v>2.75</v>
+        <v>3.4</v>
       </c>
       <c r="L91" t="n">
-        <v>0.3908629441624366</v>
+        <v>0.413495488426834</v>
       </c>
       <c r="M91" t="n">
-        <v>0.2680203045685279</v>
+        <v>0.3067869752844252</v>
       </c>
       <c r="N91" t="n">
-        <v>0.3411167512690356</v>
+        <v>0.2797175362887406</v>
       </c>
       <c r="O91" t="n">
-        <v>0.06601731601731586</v>
+        <v>0.05148090091576618</v>
       </c>
       <c r="P91" t="n">
         <v>1</v>
       </c>
       <c r="Q91" t="n">
-        <v>0.3469532397357254</v>
+        <v>0.3693334958608548</v>
       </c>
       <c r="R91" t="n">
-        <v>0.3096621954972063</v>
+        <v>0.1481250940986206</v>
       </c>
       <c r="S91" t="n">
-        <v>0.3433845647670682</v>
+        <v>0.4825414100405245</v>
       </c>
       <c r="T91" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="U91" t="n">
         <v>1</v>
       </c>
-      <c r="V91" t="n">
-        <v>0</v>
-      </c>
+      <c r="V91" t="inlineStr"/>
       <c r="W91" t="n">
         <v>0</v>
       </c>
       <c r="X91" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="Y91" t="n">
-        <v>0.3469532397357254</v>
+        <v>0.4825414100405245</v>
       </c>
       <c r="Z91" t="n">
-        <v>3.5</v>
+        <v>3.4</v>
       </c>
       <c r="AA91" t="inlineStr">
         <is>
@@ -9735,32 +9675,32 @@
         </is>
       </c>
       <c r="AB91" t="n">
-        <v>0.08573453563001551</v>
+        <v>0.2669336642240764</v>
       </c>
       <c r="AC91" t="n">
-        <v>5.204298596035881</v>
+        <v>5.790496920486294</v>
       </c>
       <c r="AD91" t="n">
-        <v>0.003568674968657148</v>
+        <v>0.1132079141796697</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="1" t="inlineStr">
         <is>
-          <t>lSTUh1hc</t>
+          <t>ALQvrPMs</t>
         </is>
       </c>
       <c r="B92" s="2" t="n">
-        <v>45770.6875</v>
+        <v>45766.66666666666</v>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>alaves</t>
+          <t>las palmas</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>real sociedad</t>
+          <t>atl  madrid</t>
         </is>
       </c>
       <c r="E92" t="n">
@@ -9780,58 +9720,56 @@
         </is>
       </c>
       <c r="I92" t="n">
-        <v>2.35</v>
+        <v>5.75</v>
       </c>
       <c r="J92" t="n">
-        <v>3.1</v>
+        <v>4.2</v>
       </c>
       <c r="K92" t="n">
-        <v>3.25</v>
+        <v>1.55</v>
       </c>
       <c r="L92" t="n">
-        <v>0.403040304030403</v>
+        <v>0.16450818118643</v>
       </c>
       <c r="M92" t="n">
-        <v>0.3055305530553055</v>
+        <v>0.2252195337671362</v>
       </c>
       <c r="N92" t="n">
-        <v>0.2914291429142914</v>
+        <v>0.6102722850464337</v>
       </c>
       <c r="O92" t="n">
-        <v>0.05580486774721516</v>
+        <v>0.05716957189607963</v>
       </c>
       <c r="P92" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q92" t="n">
-        <v>0.3688449090223264</v>
+        <v>0.2938553720649227</v>
       </c>
       <c r="R92" t="n">
-        <v>0.2829826738845801</v>
+        <v>0.14431271791708</v>
       </c>
       <c r="S92" t="n">
-        <v>0.3481724170930934</v>
+        <v>0.561831910017997</v>
       </c>
       <c r="T92" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="U92" t="n">
         <v>1</v>
       </c>
-      <c r="V92" t="n">
-        <v>0</v>
-      </c>
+      <c r="V92" t="inlineStr"/>
       <c r="W92" t="n">
         <v>0</v>
       </c>
       <c r="X92" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="Y92" t="n">
-        <v>0.3688449090223264</v>
+        <v>0.561831910017997</v>
       </c>
       <c r="Z92" t="n">
-        <v>3.1</v>
+        <v>1.55</v>
       </c>
       <c r="AA92" t="inlineStr">
         <is>
@@ -9839,32 +9777,32 @@
         </is>
       </c>
       <c r="AB92" t="n">
-        <v>0.06829486569962474</v>
+        <v>-0.2348373444947355</v>
       </c>
       <c r="AC92" t="n">
-        <v>5.532673635334896</v>
+        <v>6.741982920215965</v>
       </c>
       <c r="AD92" t="n">
-        <v>0.02067249192923304</v>
+        <v>0.2679765379530743</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="1" t="inlineStr">
         <is>
-          <t>WjapokZj</t>
+          <t>nRL3xLjJ</t>
         </is>
       </c>
       <c r="B93" s="2" t="n">
-        <v>45771.58333333334</v>
+        <v>45767.375</v>
       </c>
       <c r="C93" t="inlineStr">
         <is>
+          <t>valladolid</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
           <t>osasuna</t>
-        </is>
-      </c>
-      <c r="D93" t="inlineStr">
-        <is>
-          <t>sevilla</t>
         </is>
       </c>
       <c r="E93" t="n">
@@ -9884,58 +9822,56 @@
         </is>
       </c>
       <c r="I93" t="n">
-        <v>2.5</v>
+        <v>4.75</v>
       </c>
       <c r="J93" t="n">
-        <v>3.2</v>
+        <v>3.4</v>
       </c>
       <c r="K93" t="n">
-        <v>2.88</v>
+        <v>1.83</v>
       </c>
       <c r="L93" t="n">
-        <v>0.3774574049803408</v>
+        <v>0.2002929388852227</v>
       </c>
       <c r="M93" t="n">
-        <v>0.2948885976408912</v>
+        <v>0.2798210175602376</v>
       </c>
       <c r="N93" t="n">
-        <v>0.327653997378768</v>
+        <v>0.5198860435545397</v>
       </c>
       <c r="O93" t="n">
-        <v>0.05972222222222223</v>
+        <v>0.0510920502799912</v>
       </c>
       <c r="P93" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q93" t="n">
-        <v>0.3609409309400629</v>
+        <v>0.3096408429607286</v>
       </c>
       <c r="R93" t="n">
-        <v>0.2980019428320985</v>
+        <v>0.1597578200109194</v>
       </c>
       <c r="S93" t="n">
-        <v>0.3410571262278385</v>
+        <v>0.5306013370283519</v>
       </c>
       <c r="T93" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="U93" t="n">
         <v>1</v>
       </c>
-      <c r="V93" t="n">
-        <v>0</v>
-      </c>
+      <c r="V93" t="inlineStr"/>
       <c r="W93" t="n">
         <v>0</v>
       </c>
       <c r="X93" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="Y93" t="n">
-        <v>0.3609409309400629</v>
+        <v>0.5306013370283519</v>
       </c>
       <c r="Z93" t="n">
-        <v>3.2</v>
+        <v>1.83</v>
       </c>
       <c r="AA93" t="inlineStr">
         <is>
@@ -9943,32 +9879,32 @@
         </is>
       </c>
       <c r="AB93" t="n">
-        <v>0.0704595359128187</v>
+        <v>-0.0349392207688145</v>
       </c>
       <c r="AC93" t="n">
-        <v>5.414113964100943</v>
+        <v>6.367216044340222</v>
       </c>
       <c r="AD93" t="n">
-        <v>0.01988380471222434</v>
+        <v>0.2209604940676232</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="1" t="inlineStr">
         <is>
-          <t>ALQvrPMs</t>
+          <t>Qol45JK5</t>
         </is>
       </c>
       <c r="B94" s="2" t="n">
-        <v>45766.66666666666</v>
+        <v>45770.58333333334</v>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>las palmas</t>
+          <t>celta vigo</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>atl  madrid</t>
+          <t>villarreal</t>
         </is>
       </c>
       <c r="E94" t="n">
@@ -9988,37 +9924,37 @@
         </is>
       </c>
       <c r="I94" t="n">
-        <v>5.75</v>
+        <v>2.4</v>
       </c>
       <c r="J94" t="n">
-        <v>4.2</v>
+        <v>3.5</v>
       </c>
       <c r="K94" t="n">
-        <v>1.55</v>
+        <v>2.75</v>
       </c>
       <c r="L94" t="n">
-        <v>0.16450818118643</v>
+        <v>0.3908629441624366</v>
       </c>
       <c r="M94" t="n">
-        <v>0.2252195337671362</v>
+        <v>0.2680203045685279</v>
       </c>
       <c r="N94" t="n">
-        <v>0.6102722850464337</v>
+        <v>0.3411167512690356</v>
       </c>
       <c r="O94" t="n">
-        <v>0.05716957189607963</v>
+        <v>0.06601731601731586</v>
       </c>
       <c r="P94" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q94" t="n">
-        <v>0.3171448641791066</v>
+        <v>0.3604385744537616</v>
       </c>
       <c r="R94" t="n">
-        <v>0.1321056276013278</v>
+        <v>0.1900255345135736</v>
       </c>
       <c r="S94" t="n">
-        <v>0.5507495082195656</v>
+        <v>0.4495358910326646</v>
       </c>
       <c r="T94" t="n">
         <v>2</v>
@@ -10026,9 +9962,7 @@
       <c r="U94" t="n">
         <v>1</v>
       </c>
-      <c r="V94" t="n">
-        <v>0</v>
-      </c>
+      <c r="V94" t="inlineStr"/>
       <c r="W94" t="n">
         <v>0</v>
       </c>
@@ -10036,10 +9970,10 @@
         <v>2</v>
       </c>
       <c r="Y94" t="n">
-        <v>0.5507495082195656</v>
+        <v>0.4495358910326646</v>
       </c>
       <c r="Z94" t="n">
-        <v>1.55</v>
+        <v>2.75</v>
       </c>
       <c r="AA94" t="inlineStr">
         <is>
@@ -10047,32 +9981,32 @@
         </is>
       </c>
       <c r="AB94" t="n">
-        <v>-0.2660695677448606</v>
+        <v>0.1349849716227587</v>
       </c>
       <c r="AC94" t="n">
-        <v>1.433729615175497</v>
+        <v>5.394430692391976</v>
       </c>
       <c r="AD94" t="n">
-        <v>0.233604644040459</v>
+        <v>0.08909731657890302</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="1" t="inlineStr">
         <is>
-          <t>nRL3xLjJ</t>
+          <t>lSTUh1hc</t>
         </is>
       </c>
       <c r="B95" s="2" t="n">
-        <v>45767.375</v>
+        <v>45770.6875</v>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>valladolid</t>
+          <t>alaves</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>osasuna</t>
+          <t>real sociedad</t>
         </is>
       </c>
       <c r="E95" t="n">
@@ -10092,37 +10026,37 @@
         </is>
       </c>
       <c r="I95" t="n">
-        <v>4.75</v>
+        <v>2.35</v>
       </c>
       <c r="J95" t="n">
-        <v>3.4</v>
+        <v>3.1</v>
       </c>
       <c r="K95" t="n">
-        <v>1.83</v>
+        <v>3.25</v>
       </c>
       <c r="L95" t="n">
-        <v>0.2002929388852227</v>
+        <v>0.403040304030403</v>
       </c>
       <c r="M95" t="n">
-        <v>0.2798210175602376</v>
+        <v>0.3055305530553055</v>
       </c>
       <c r="N95" t="n">
-        <v>0.5198860435545397</v>
+        <v>0.2914291429142914</v>
       </c>
       <c r="O95" t="n">
-        <v>0.0510920502799912</v>
+        <v>0.05580486774721516</v>
       </c>
       <c r="P95" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q95" t="n">
-        <v>0.3347586034399208</v>
+        <v>0.3926474934027478</v>
       </c>
       <c r="R95" t="n">
-        <v>0.2508547173151877</v>
+        <v>0.164560534039235</v>
       </c>
       <c r="S95" t="n">
-        <v>0.4143866792448915</v>
+        <v>0.4427919725580169</v>
       </c>
       <c r="T95" t="n">
         <v>2</v>
@@ -10130,9 +10064,7 @@
       <c r="U95" t="n">
         <v>1</v>
       </c>
-      <c r="V95" t="n">
-        <v>0</v>
-      </c>
+      <c r="V95" t="inlineStr"/>
       <c r="W95" t="n">
         <v>0</v>
       </c>
@@ -10140,10 +10072,10 @@
         <v>2</v>
       </c>
       <c r="Y95" t="n">
-        <v>0.4143866792448915</v>
+        <v>0.4427919725580169</v>
       </c>
       <c r="Z95" t="n">
-        <v>1.83</v>
+        <v>3.25</v>
       </c>
       <c r="AA95" t="inlineStr">
         <is>
@@ -10151,32 +10083,32 @@
         </is>
       </c>
       <c r="AB95" t="n">
-        <v>-0.2911715385323477</v>
+        <v>0.19514396036158</v>
       </c>
       <c r="AC95" t="n">
-        <v>1.063441560787886</v>
+        <v>5.313503670696202</v>
       </c>
       <c r="AD95" t="n">
-        <v>0.07962807580497072</v>
+        <v>0.05014447915526904</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="1" t="inlineStr">
         <is>
-          <t>EDNevsM6</t>
+          <t>n1xD3ckI</t>
         </is>
       </c>
       <c r="B96" s="2" t="n">
-        <v>45768.66666666666</v>
+        <v>45770.6875</v>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>girona</t>
+          <t>getafe</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>betis</t>
+          <t>real madrid</t>
         </is>
       </c>
       <c r="E96" t="n">
@@ -10196,37 +10128,37 @@
         </is>
       </c>
       <c r="I96" t="n">
-        <v>2.88</v>
+        <v>4.5</v>
       </c>
       <c r="J96" t="n">
-        <v>3.3</v>
+        <v>3.7</v>
       </c>
       <c r="K96" t="n">
-        <v>2.45</v>
+        <v>1.73</v>
       </c>
       <c r="L96" t="n">
-        <v>0.328058429701765</v>
+        <v>0.2075820469581009</v>
       </c>
       <c r="M96" t="n">
-        <v>0.2863055386488131</v>
+        <v>0.2524646517057984</v>
       </c>
       <c r="N96" t="n">
-        <v>0.3856360316494217</v>
+        <v>0.5399533013361008</v>
       </c>
       <c r="O96" t="n">
-        <v>0.05841579055864776</v>
+        <v>0.07052717457341728</v>
       </c>
       <c r="P96" t="n">
         <v>2</v>
       </c>
       <c r="Q96" t="n">
-        <v>0.3389599537124544</v>
+        <v>0.3177552718671804</v>
       </c>
       <c r="R96" t="n">
-        <v>0.3118753087828674</v>
+        <v>0.1318751088976358</v>
       </c>
       <c r="S96" t="n">
-        <v>0.349164737504678</v>
+        <v>0.5503696192351837</v>
       </c>
       <c r="T96" t="n">
         <v>2</v>
@@ -10234,9 +10166,7 @@
       <c r="U96" t="n">
         <v>1</v>
       </c>
-      <c r="V96" t="n">
-        <v>0</v>
-      </c>
+      <c r="V96" t="inlineStr"/>
       <c r="W96" t="n">
         <v>0</v>
       </c>
@@ -10244,10 +10174,10 @@
         <v>2</v>
       </c>
       <c r="Y96" t="n">
-        <v>0.349164737504678</v>
+        <v>0.5503696192351837</v>
       </c>
       <c r="Z96" t="n">
-        <v>2.45</v>
+        <v>1.73</v>
       </c>
       <c r="AA96" t="inlineStr">
         <is>
@@ -10255,32 +10185,32 @@
         </is>
       </c>
       <c r="AB96" t="n">
-        <v>-0.0996871676645095</v>
+        <v>-0.06556240920977016</v>
       </c>
       <c r="AC96" t="n">
-        <v>0.1990653082508933</v>
+        <v>6.604435430822204</v>
       </c>
       <c r="AD96" t="n">
-        <v>0.01020478379222362</v>
+        <v>0.2326143473680032</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="1" t="inlineStr">
         <is>
-          <t>n1xD3ckI</t>
+          <t>MuSxiuN9</t>
         </is>
       </c>
       <c r="B97" s="2" t="n">
-        <v>45770.6875</v>
+        <v>45771.58333333334</v>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>getafe</t>
+          <t>leganes</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>real madrid</t>
+          <t>girona</t>
         </is>
       </c>
       <c r="E97" t="n">
@@ -10300,37 +10230,37 @@
         </is>
       </c>
       <c r="I97" t="n">
-        <v>4.5</v>
+        <v>2.55</v>
       </c>
       <c r="J97" t="n">
-        <v>3.7</v>
+        <v>3.2</v>
       </c>
       <c r="K97" t="n">
-        <v>1.73</v>
+        <v>2.8</v>
       </c>
       <c r="L97" t="n">
-        <v>0.2075820469581009</v>
+        <v>0.3693322341302556</v>
       </c>
       <c r="M97" t="n">
-        <v>0.2524646517057984</v>
+        <v>0.2943116240725474</v>
       </c>
       <c r="N97" t="n">
-        <v>0.5399533013361008</v>
+        <v>0.336356141797197</v>
       </c>
       <c r="O97" t="n">
-        <v>0.07052717457341728</v>
+        <v>0.06179971988795518</v>
       </c>
       <c r="P97" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q97" t="n">
-        <v>0.3370566054801529</v>
+        <v>0.2764709700640772</v>
       </c>
       <c r="R97" t="n">
-        <v>0.09754668514635362</v>
+        <v>0.150069804722545</v>
       </c>
       <c r="S97" t="n">
-        <v>0.5653967093734935</v>
+        <v>0.5734592252133778</v>
       </c>
       <c r="T97" t="n">
         <v>2</v>
@@ -10338,9 +10268,7 @@
       <c r="U97" t="n">
         <v>1</v>
       </c>
-      <c r="V97" t="n">
-        <v>0</v>
-      </c>
+      <c r="V97" t="inlineStr"/>
       <c r="W97" t="n">
         <v>0</v>
       </c>
@@ -10348,10 +10276,10 @@
         <v>2</v>
       </c>
       <c r="Y97" t="n">
-        <v>0.5653967093734935</v>
+        <v>0.5734592252133778</v>
       </c>
       <c r="Z97" t="n">
-        <v>1.73</v>
+        <v>2.8</v>
       </c>
       <c r="AA97" t="inlineStr">
         <is>
@@ -10359,19 +10287,19 @@
         </is>
       </c>
       <c r="AB97" t="n">
-        <v>-0.02995026408747431</v>
+        <v>0.3364921281096987</v>
       </c>
       <c r="AC97" t="n">
-        <v>1.670791355549232</v>
+        <v>6.881510702560534</v>
       </c>
       <c r="AD97" t="n">
-        <v>0.2283401038933406</v>
+        <v>0.2969882551493006</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="1" t="inlineStr">
         <is>
-          <t>MuSxiuN9</t>
+          <t>WjapokZj</t>
         </is>
       </c>
       <c r="B98" s="2" t="n">
@@ -10379,12 +10307,12 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>leganes</t>
+          <t>osasuna</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>girona</t>
+          <t>sevilla</t>
         </is>
       </c>
       <c r="E98" t="n">
@@ -10404,37 +10332,37 @@
         </is>
       </c>
       <c r="I98" t="n">
-        <v>2.55</v>
+        <v>2.5</v>
       </c>
       <c r="J98" t="n">
         <v>3.2</v>
       </c>
       <c r="K98" t="n">
-        <v>2.8</v>
+        <v>2.88</v>
       </c>
       <c r="L98" t="n">
-        <v>0.3693322341302556</v>
+        <v>0.3774574049803408</v>
       </c>
       <c r="M98" t="n">
-        <v>0.2943116240725474</v>
+        <v>0.2948885976408912</v>
       </c>
       <c r="N98" t="n">
-        <v>0.336356141797197</v>
+        <v>0.327653997378768</v>
       </c>
       <c r="O98" t="n">
-        <v>0.06179971988795518</v>
+        <v>0.05972222222222223</v>
       </c>
       <c r="P98" t="n">
         <v>1</v>
       </c>
       <c r="Q98" t="n">
-        <v>0.4014547731122984</v>
+        <v>0.2731863114080319</v>
       </c>
       <c r="R98" t="n">
-        <v>0.1955416450872015</v>
+        <v>0.3165623826298162</v>
       </c>
       <c r="S98" t="n">
-        <v>0.4030035818005001</v>
+        <v>0.410251305962152</v>
       </c>
       <c r="T98" t="n">
         <v>2</v>
@@ -10442,9 +10370,7 @@
       <c r="U98" t="n">
         <v>1</v>
       </c>
-      <c r="V98" t="n">
-        <v>0</v>
-      </c>
+      <c r="V98" t="inlineStr"/>
       <c r="W98" t="n">
         <v>0</v>
       </c>
@@ -10452,10 +10378,10 @@
         <v>2</v>
       </c>
       <c r="Y98" t="n">
-        <v>0.4030035818005001</v>
+        <v>0.410251305962152</v>
       </c>
       <c r="Z98" t="n">
-        <v>2.8</v>
+        <v>2.88</v>
       </c>
       <c r="AA98" t="inlineStr">
         <is>
@@ -10463,13 +10389,13 @@
         </is>
       </c>
       <c r="AB98" t="n">
-        <v>0.071338905023</v>
+        <v>0.0965551921122328</v>
       </c>
       <c r="AC98" t="n">
-        <v>0.2418021490803</v>
+        <v>4.923015671545824</v>
       </c>
       <c r="AD98" t="n">
-        <v>0.001548808688201675</v>
+        <v>0.09368892333233581</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
DATA. Actualizo preds de hoy (de ITA y ENG). Cambio de modelos por train.
</commit_message>
<xml_diff>
--- a/data/predicciones.xlsx
+++ b/data/predicciones.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AM5"/>
+  <dimension ref="A1:AD6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -465,187 +465,142 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>competition</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
           <t>odds_home</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>odds_draw</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>odds_away</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>prob_home_bm</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>prob_draw_bm</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>prob_away_bm</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>overround</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>bookmaker_result</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>prob_class_0</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>prob_class_1</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>prob_class_2</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>predicted_result</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>prob_class_1</t>
-        </is>
-      </c>
-      <c r="P1" s="1" t="inlineStr">
-        <is>
-          <t>prob_class_0</t>
-        </is>
-      </c>
-      <c r="Q1" s="1" t="inlineStr">
-        <is>
-          <t>prob_class_2</t>
-        </is>
-      </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>copiado_formaciones</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
-        <is>
-          <t>dif_prob_mod_bm</t>
-        </is>
-      </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>emergency_fill</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>player_emergency_fill</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>result_to_bet</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
-        <is>
-          <t>dif_prob_result_to_bet</t>
-        </is>
-      </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>prob_result_to_bet</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>odd_to_bet</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>strategy</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
-        <is>
-          <t>multiplier</t>
-        </is>
-      </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
+        <is>
+          <t>kelly_criterion</t>
+        </is>
+      </c>
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>stake_to_bet</t>
         </is>
       </c>
-      <c r="AA1" s="1" t="inlineStr">
-        <is>
-          <t>country</t>
-        </is>
-      </c>
-      <c r="AB1" s="1" t="inlineStr">
-        <is>
-          <t>competition</t>
-        </is>
-      </c>
-      <c r="AC1" s="1" t="inlineStr">
-        <is>
-          <t>emergency_fill</t>
-        </is>
-      </c>
       <c r="AD1" s="1" t="inlineStr">
         <is>
-          <t>stake_to_bet_raw</t>
-        </is>
-      </c>
-      <c r="AE1" s="1" t="inlineStr">
-        <is>
-          <t>stake_to_bet_norm</t>
-        </is>
-      </c>
-      <c r="AF1" s="1" t="inlineStr">
-        <is>
-          <t>player_emergency_fill</t>
-        </is>
-      </c>
-      <c r="AG1" s="1" t="inlineStr">
-        <is>
           <t>confidence_margin</t>
-        </is>
-      </c>
-      <c r="AH1" s="1" t="inlineStr">
-        <is>
-          <t>kelly_criterion</t>
-        </is>
-      </c>
-      <c r="AI1" s="1" t="inlineStr">
-        <is>
-          <t>bookmaker_result</t>
-        </is>
-      </c>
-      <c r="AJ1" s="1" t="inlineStr">
-        <is>
-          <t>goals_home</t>
-        </is>
-      </c>
-      <c r="AK1" s="1" t="inlineStr">
-        <is>
-          <t>goals_away</t>
-        </is>
-      </c>
-      <c r="AL1" s="1" t="inlineStr">
-        <is>
-          <t>result</t>
-        </is>
-      </c>
-      <c r="AM1" s="1" t="inlineStr">
-        <is>
-          <t>acerte</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>tjEpOUFM</t>
+          <t>SnlB9V0T</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>45769.66666666666</v>
+        <v>45770.66666666666</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>manchester city</t>
+          <t>arsenal</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>aston villa</t>
+          <t>crystal palace</t>
         </is>
       </c>
       <c r="E2" t="n">
@@ -654,459 +609,491 @@
       <c r="F2" t="n">
         <v>481</v>
       </c>
-      <c r="G2" t="n">
-        <v>1.8</v>
-      </c>
-      <c r="H2" t="n">
-        <v>4.1</v>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>england</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>premier league</t>
+        </is>
       </c>
       <c r="I2" t="n">
-        <v>3.9</v>
+        <v>1.38</v>
       </c>
       <c r="J2" t="n">
-        <v>0.5261599210266535</v>
+        <v>4.75</v>
       </c>
       <c r="K2" t="n">
-        <v>0.2309970384995065</v>
+        <v>9</v>
       </c>
       <c r="L2" t="n">
-        <v>0.2428430404738401</v>
+        <v>0.692588092345079</v>
       </c>
       <c r="M2" t="n">
-        <v>0.05586825099020221</v>
+        <v>0.2012150668286755</v>
       </c>
       <c r="N2" t="n">
+        <v>0.1061968408262454</v>
+      </c>
+      <c r="O2" t="n">
+        <v>0.04627510806000523</v>
+      </c>
+      <c r="P2" t="n">
         <v>1</v>
       </c>
-      <c r="O2" t="n">
-        <v>0.5082111593461466</v>
-      </c>
-      <c r="P2" t="n">
-        <v>0.3407758685142832</v>
-      </c>
       <c r="Q2" t="n">
-        <v>0.1510129721395701</v>
+        <v>0.2846090376156243</v>
       </c>
       <c r="R2" t="n">
-        <v>1</v>
-      </c>
-      <c r="S2" t="inlineStr"/>
+        <v>0.5202828785872773</v>
+      </c>
+      <c r="S2" t="n">
+        <v>0.195108083797098</v>
+      </c>
       <c r="T2" t="n">
         <v>1</v>
       </c>
-      <c r="U2" t="inlineStr"/>
+      <c r="U2" t="n">
+        <v>1</v>
+      </c>
       <c r="V2" t="n">
-        <v>0.5082111593461466</v>
+        <v>0</v>
       </c>
       <c r="W2" t="n">
-        <v>1.8</v>
-      </c>
-      <c r="X2" t="inlineStr">
-        <is>
-          <t>kelly_crit &gt; -0.25</t>
-        </is>
-      </c>
-      <c r="Y2" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="X2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="Y2" t="n">
+        <v>0.4797171214127227</v>
+      </c>
       <c r="Z2" t="n">
-        <v>1.52463347803844</v>
+        <v>3.109090909090909</v>
       </c>
       <c r="AA2" t="inlineStr">
         <is>
-          <t>england</t>
-        </is>
-      </c>
-      <c r="AB2" t="inlineStr">
-        <is>
-          <t>premier league</t>
-        </is>
-      </c>
-      <c r="AC2" t="inlineStr"/>
-      <c r="AD2" t="inlineStr"/>
-      <c r="AE2" t="inlineStr"/>
-      <c r="AF2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG2" t="n">
-        <v>0.1674352908318634</v>
-      </c>
-      <c r="AH2" t="n">
-        <v>-0.1065248914711701</v>
-      </c>
-      <c r="AI2" t="n">
-        <v>1</v>
-      </c>
-      <c r="AJ2" t="n">
-        <v>2</v>
-      </c>
-      <c r="AK2" t="n">
-        <v>1</v>
-      </c>
-      <c r="AL2" t="n">
-        <v>1</v>
-      </c>
-      <c r="AM2" t="n">
-        <v>1</v>
+          <t>kelly_crit &lt; -0.5</t>
+        </is>
+      </c>
+      <c r="AB2" t="n">
+        <v>0.2330312738066861</v>
+      </c>
+      <c r="AC2" t="n">
+        <v>1.439151364238168</v>
+      </c>
+      <c r="AD2" t="n">
+        <v>0.235673840971653</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>UH5lVWkD</t>
+          <t>EXFt5ZOk</t>
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>45769.65625</v>
+        <v>45770.5625</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>nantes</t>
+          <t>torino</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>psg</t>
+          <t>udinese</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>55</v>
+        <v>77</v>
       </c>
       <c r="F3" t="n">
-        <v>551</v>
-      </c>
-      <c r="G3" t="n">
-        <v>7</v>
-      </c>
-      <c r="H3" t="n">
-        <v>5.75</v>
+        <v>771</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>italy</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>serie a</t>
+        </is>
       </c>
       <c r="I3" t="n">
-        <v>1.36</v>
+        <v>2.35</v>
       </c>
       <c r="J3" t="n">
-        <v>0.1357874631012329</v>
+        <v>3</v>
       </c>
       <c r="K3" t="n">
-        <v>0.1653064768188922</v>
+        <v>3.4</v>
       </c>
       <c r="L3" t="n">
-        <v>0.698906060079875</v>
+        <v>0.4041204437400951</v>
       </c>
       <c r="M3" t="n">
-        <v>0.05206430398246242</v>
+        <v>0.3165610142630745</v>
       </c>
       <c r="N3" t="n">
+        <v>0.2793185419968304</v>
+      </c>
+      <c r="O3" t="n">
+        <v>0.05298289528577382</v>
+      </c>
+      <c r="P3" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>0.3611186126731784</v>
+      </c>
+      <c r="R3" t="n">
+        <v>0.3686566276867528</v>
+      </c>
+      <c r="S3" t="n">
+        <v>0.2702247596400687</v>
+      </c>
+      <c r="T3" t="n">
+        <v>1</v>
+      </c>
+      <c r="U3" t="n">
+        <v>1</v>
+      </c>
+      <c r="V3" t="inlineStr"/>
+      <c r="W3" t="n">
         <v>0</v>
       </c>
-      <c r="O3" t="n">
-        <v>0.2392231549598418</v>
-      </c>
-      <c r="P3" t="n">
-        <v>0.3821643987417085</v>
-      </c>
-      <c r="Q3" t="n">
-        <v>0.3786124462984498</v>
-      </c>
-      <c r="R3" t="n">
+      <c r="X3" t="n">
         <v>1</v>
       </c>
-      <c r="S3" t="inlineStr"/>
-      <c r="T3" t="n">
-        <v>0</v>
-      </c>
-      <c r="U3" t="inlineStr"/>
-      <c r="V3" t="n">
-        <v>0.3821643987417085</v>
-      </c>
-      <c r="W3" t="n">
-        <v>5.75</v>
-      </c>
-      <c r="X3" t="inlineStr">
-        <is>
-          <t>kelly_crit &gt; nan</t>
-        </is>
-      </c>
-      <c r="Y3" t="inlineStr"/>
+      <c r="Y3" t="n">
+        <v>0.3686566276867528</v>
+      </c>
       <c r="Z3" t="n">
-        <v>1.146493196225125</v>
+        <v>2.35</v>
       </c>
       <c r="AA3" t="inlineStr">
         <is>
-          <t>france</t>
-        </is>
-      </c>
-      <c r="AB3" t="inlineStr">
-        <is>
-          <t>ligue 1</t>
-        </is>
-      </c>
-      <c r="AC3" t="inlineStr"/>
-      <c r="AD3" t="inlineStr"/>
-      <c r="AE3" t="inlineStr"/>
-      <c r="AF3" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG3" t="n">
-        <v>0.003551952443258732</v>
-      </c>
-      <c r="AH3" t="n">
-        <v>0.2520937458452261</v>
-      </c>
-      <c r="AI3" t="n">
-        <v>2</v>
-      </c>
-      <c r="AJ3" t="n">
-        <v>1</v>
-      </c>
-      <c r="AK3" t="n">
-        <v>1</v>
-      </c>
-      <c r="AL3" t="n">
-        <v>0</v>
-      </c>
-      <c r="AM3" t="n">
-        <v>1</v>
+          <t>kelly_crit &gt; -1.0</t>
+        </is>
+      </c>
+      <c r="AB3" t="n">
+        <v>-0.09900512958231907</v>
+      </c>
+      <c r="AC3" t="n">
+        <v>0.2211939766120517</v>
+      </c>
+      <c r="AD3" t="n">
+        <v>0.007538015013574484</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>AyybJmyR</t>
+          <t>U5sK10Ic</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>45769.58333333334</v>
+        <v>45770.5625</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>valencia</t>
+          <t>cagliari</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>espanyol</t>
+          <t>fiorentina</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>148</v>
+        <v>77</v>
       </c>
       <c r="F4" t="n">
-        <v>1481</v>
-      </c>
-      <c r="G4" t="n">
-        <v>1.8</v>
-      </c>
-      <c r="H4" t="n">
-        <v>3.5</v>
+        <v>771</v>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>italy</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>serie a</t>
+        </is>
       </c>
       <c r="I4" t="n">
-        <v>4.75</v>
+        <v>2.9</v>
       </c>
       <c r="J4" t="n">
-        <v>0.5281969817315331</v>
+        <v>3.1</v>
       </c>
       <c r="K4" t="n">
-        <v>0.2716441620333598</v>
+        <v>2.6</v>
       </c>
       <c r="L4" t="n">
-        <v>0.2001588562351072</v>
+        <v>0.3277755185034567</v>
       </c>
       <c r="M4" t="n">
-        <v>0.05179615705931484</v>
+        <v>0.3066287108580724</v>
       </c>
       <c r="N4" t="n">
+        <v>0.3655957706384709</v>
+      </c>
+      <c r="O4" t="n">
+        <v>0.05202361598357141</v>
+      </c>
+      <c r="P4" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>0.3328624820903378</v>
+      </c>
+      <c r="R4" t="n">
+        <v>0.2945133354398648</v>
+      </c>
+      <c r="S4" t="n">
+        <v>0.3726241824697973</v>
+      </c>
+      <c r="T4" t="n">
+        <v>2</v>
+      </c>
+      <c r="U4" t="n">
         <v>1</v>
       </c>
-      <c r="O4" t="n">
-        <v>0.5276134071321876</v>
-      </c>
-      <c r="P4" t="n">
-        <v>0.33402159847374</v>
-      </c>
-      <c r="Q4" t="n">
-        <v>0.138364994394072</v>
-      </c>
-      <c r="R4" t="n">
-        <v>1</v>
-      </c>
-      <c r="S4" t="inlineStr"/>
-      <c r="T4" t="n">
-        <v>1</v>
-      </c>
-      <c r="U4" t="inlineStr"/>
-      <c r="V4" t="n">
-        <v>0.5276134071321876</v>
-      </c>
+      <c r="V4" t="inlineStr"/>
       <c r="W4" t="n">
-        <v>1.8</v>
-      </c>
-      <c r="X4" t="inlineStr">
+        <v>0</v>
+      </c>
+      <c r="X4" t="n">
+        <v>2</v>
+      </c>
+      <c r="Y4" t="n">
+        <v>0.3726241824697973</v>
+      </c>
+      <c r="Z4" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="AA4" t="inlineStr">
         <is>
           <t>kelly_crit &gt; nan</t>
         </is>
       </c>
-      <c r="Y4" t="inlineStr"/>
-      <c r="Z4" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA4" t="inlineStr">
-        <is>
-          <t>spain</t>
-        </is>
-      </c>
-      <c r="AB4" t="inlineStr">
-        <is>
-          <t>laliga</t>
-        </is>
+      <c r="AB4" t="n">
+        <v>-0.01948570348657933</v>
       </c>
       <c r="AC4" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD4" t="inlineStr"/>
-      <c r="AE4" t="inlineStr"/>
-      <c r="AF4" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG4" t="n">
-        <v>0.1935918086584476</v>
-      </c>
-      <c r="AH4" t="n">
-        <v>-0.06286983395257781</v>
-      </c>
-      <c r="AI4" t="n">
-        <v>1</v>
-      </c>
-      <c r="AJ4" t="n">
-        <v>1</v>
-      </c>
-      <c r="AK4" t="n">
-        <v>1</v>
-      </c>
-      <c r="AL4" t="n">
-        <v>0</v>
-      </c>
-      <c r="AM4" t="n">
-        <v>0</v>
+        <v>5.58936273704696</v>
+      </c>
+      <c r="AD4" t="n">
+        <v>0.03976170037945953</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>Mgim91Lt</t>
+          <t>boZzbIHM</t>
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>45769.6875</v>
+        <v>45770.5625</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>barcelona</t>
+          <t>genoa</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>mallorca</t>
+          <t>lazio</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>148</v>
+        <v>77</v>
       </c>
       <c r="F5" t="n">
-        <v>1481</v>
-      </c>
-      <c r="G5" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="H5" t="n">
-        <v>7</v>
+        <v>771</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>italy</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>serie a</t>
+        </is>
       </c>
       <c r="I5" t="n">
-        <v>13</v>
+        <v>3.4</v>
       </c>
       <c r="J5" t="n">
-        <v>0.7913043478260869</v>
+        <v>3.2</v>
       </c>
       <c r="K5" t="n">
-        <v>0.1356521739130435</v>
+        <v>2.25</v>
       </c>
       <c r="L5" t="n">
-        <v>0.07304347826086957</v>
+        <v>0.2798289933929266</v>
       </c>
       <c r="M5" t="n">
-        <v>0.05311355311355315</v>
+        <v>0.2973183054799844</v>
       </c>
       <c r="N5" t="n">
+        <v>0.4228527011270889</v>
+      </c>
+      <c r="O5" t="n">
+        <v>0.05106209150326801</v>
+      </c>
+      <c r="P5" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>0.3479151141876893</v>
+      </c>
+      <c r="R5" t="n">
+        <v>0.2679920158913548</v>
+      </c>
+      <c r="S5" t="n">
+        <v>0.3840928699209559</v>
+      </c>
+      <c r="T5" t="n">
+        <v>2</v>
+      </c>
+      <c r="U5" t="n">
         <v>1</v>
       </c>
-      <c r="O5" t="n">
-        <v>0.5856258637708419</v>
-      </c>
-      <c r="P5" t="n">
-        <v>0.2403573216692877</v>
-      </c>
-      <c r="Q5" t="n">
-        <v>0.1740168145598701</v>
-      </c>
-      <c r="R5" t="n">
+      <c r="V5" t="inlineStr"/>
+      <c r="W5" t="n">
+        <v>0</v>
+      </c>
+      <c r="X5" t="n">
+        <v>2</v>
+      </c>
+      <c r="Y5" t="n">
+        <v>0.3840928699209559</v>
+      </c>
+      <c r="Z5" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="AA5" t="inlineStr">
+        <is>
+          <t>kelly_crit &gt; nan</t>
+        </is>
+      </c>
+      <c r="AB5" t="n">
+        <v>-0.1086328341422793</v>
+      </c>
+      <c r="AC5" t="n">
+        <v>5.761393048814339</v>
+      </c>
+      <c r="AD5" t="n">
+        <v>0.03617775573326665</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>xhM2CHWF</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="n">
+        <v>45770.5625</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>parma</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>juventus</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>77</v>
+      </c>
+      <c r="F6" t="n">
+        <v>771</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>italy</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>serie a</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
+        <v>5</v>
+      </c>
+      <c r="J6" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="K6" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="L6" t="n">
+        <v>0.1895910780669145</v>
+      </c>
+      <c r="M6" t="n">
+        <v>0.2527881040892193</v>
+      </c>
+      <c r="N6" t="n">
+        <v>0.5576208178438662</v>
+      </c>
+      <c r="O6" t="n">
+        <v>0.05490196078431375</v>
+      </c>
+      <c r="P6" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>0.3652699756173239</v>
+      </c>
+      <c r="R6" t="n">
+        <v>0.1734073610102015</v>
+      </c>
+      <c r="S6" t="n">
+        <v>0.4613226633724746</v>
+      </c>
+      <c r="T6" t="n">
+        <v>2</v>
+      </c>
+      <c r="U6" t="n">
         <v>1</v>
       </c>
-      <c r="S5" t="inlineStr"/>
-      <c r="T5" t="n">
-        <v>1</v>
-      </c>
-      <c r="U5" t="inlineStr"/>
-      <c r="V5" t="n">
-        <v>0.5856258637708419</v>
-      </c>
-      <c r="W5" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="X5" t="inlineStr">
+      <c r="V6" t="inlineStr"/>
+      <c r="W6" t="n">
+        <v>0</v>
+      </c>
+      <c r="X6" t="n">
+        <v>2</v>
+      </c>
+      <c r="Y6" t="n">
+        <v>0.4613226633724746</v>
+      </c>
+      <c r="Z6" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="AA6" t="inlineStr">
         <is>
           <t>kelly_crit &gt; nan</t>
         </is>
       </c>
-      <c r="Y5" t="inlineStr"/>
-      <c r="Z5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA5" t="inlineStr">
-        <is>
-          <t>spain</t>
-        </is>
-      </c>
-      <c r="AB5" t="inlineStr">
-        <is>
-          <t>laliga</t>
-        </is>
-      </c>
-      <c r="AC5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD5" t="inlineStr"/>
-      <c r="AE5" t="inlineStr"/>
-      <c r="AF5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG5" t="n">
-        <v>0.3452685421015542</v>
-      </c>
-      <c r="AH5" t="n">
-        <v>-1.486244817374949</v>
-      </c>
-      <c r="AI5" t="n">
-        <v>1</v>
-      </c>
-      <c r="AJ5" t="n">
-        <v>1</v>
-      </c>
-      <c r="AK5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AL5" t="n">
-        <v>1</v>
-      </c>
-      <c r="AM5" t="n">
-        <v>1</v>
+      <c r="AB6" t="n">
+        <v>-0.3082163889525616</v>
+      </c>
+      <c r="AC6" t="n">
+        <v>6.91983995058712</v>
+      </c>
+      <c r="AD6" t="n">
+        <v>0.09605268775515069</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
DATA. Actualizo preds de SPA (nuevo train)
</commit_message>
<xml_diff>
--- a/data/predicciones.xlsx
+++ b/data/predicciones.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD6"/>
+  <dimension ref="A1:AC5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -540,45 +540,40 @@
       </c>
       <c r="V1" s="1" t="inlineStr">
         <is>
-          <t>emergency_fill</t>
+          <t>player_emergency_fill</t>
         </is>
       </c>
       <c r="W1" s="1" t="inlineStr">
         <is>
-          <t>player_emergency_fill</t>
+          <t>result_to_bet</t>
         </is>
       </c>
       <c r="X1" s="1" t="inlineStr">
         <is>
-          <t>result_to_bet</t>
+          <t>prob_result_to_bet</t>
         </is>
       </c>
       <c r="Y1" s="1" t="inlineStr">
         <is>
-          <t>prob_result_to_bet</t>
+          <t>odd_to_bet</t>
         </is>
       </c>
       <c r="Z1" s="1" t="inlineStr">
         <is>
-          <t>odd_to_bet</t>
+          <t>strategy</t>
         </is>
       </c>
       <c r="AA1" s="1" t="inlineStr">
         <is>
-          <t>strategy</t>
+          <t>kelly_criterion</t>
         </is>
       </c>
       <c r="AB1" s="1" t="inlineStr">
         <is>
-          <t>kelly_criterion</t>
+          <t>stake_to_bet</t>
         </is>
       </c>
       <c r="AC1" s="1" t="inlineStr">
-        <is>
-          <t>stake_to_bet</t>
-        </is>
-      </c>
-      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>confidence_margin</t>
         </is>
@@ -587,70 +582,70 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>SnlB9V0T</t>
+          <t>QX8VjK5C</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>45770.66666666666</v>
+        <v>45770.58333333334</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>arsenal</t>
+          <t>ath bilbao</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>crystal palace</t>
+          <t>las palmas</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>48</v>
+        <v>148</v>
       </c>
       <c r="F2" t="n">
-        <v>481</v>
+        <v>1481</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>england</t>
+          <t>spain</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>premier league</t>
+          <t>laliga</t>
         </is>
       </c>
       <c r="I2" t="n">
-        <v>1.38</v>
+        <v>1.36</v>
       </c>
       <c r="J2" t="n">
-        <v>4.75</v>
+        <v>5</v>
       </c>
       <c r="K2" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="L2" t="n">
-        <v>0.692588092345079</v>
+        <v>0.6934812760055478</v>
       </c>
       <c r="M2" t="n">
-        <v>0.2012150668286755</v>
+        <v>0.188626907073509</v>
       </c>
       <c r="N2" t="n">
-        <v>0.1061968408262454</v>
+        <v>0.1178918169209431</v>
       </c>
       <c r="O2" t="n">
-        <v>0.04627510806000523</v>
+        <v>0.06029411764705883</v>
       </c>
       <c r="P2" t="n">
         <v>1</v>
       </c>
       <c r="Q2" t="n">
-        <v>0.2846090376156243</v>
+        <v>0.3054629049528139</v>
       </c>
       <c r="R2" t="n">
-        <v>0.5202828785872773</v>
+        <v>0.4729697842881722</v>
       </c>
       <c r="S2" t="n">
-        <v>0.195108083797098</v>
+        <v>0.2215673107590139</v>
       </c>
       <c r="T2" t="n">
         <v>1</v>
@@ -662,201 +657,197 @@
         <v>0</v>
       </c>
       <c r="W2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X2" t="n">
-        <v>-1</v>
+        <v>0.4729697842881722</v>
       </c>
       <c r="Y2" t="n">
-        <v>0.4797171214127227</v>
-      </c>
-      <c r="Z2" t="n">
-        <v>3.109090909090909</v>
-      </c>
-      <c r="AA2" t="inlineStr">
-        <is>
-          <t>kelly_crit &lt; -0.5</t>
-        </is>
+        <v>1.36</v>
+      </c>
+      <c r="Z2" t="inlineStr">
+        <is>
+          <t>kelly_crit &gt; nan</t>
+        </is>
+      </c>
+      <c r="AA2" t="n">
+        <v>-0.9910030371335714</v>
       </c>
       <c r="AB2" t="n">
-        <v>0.2330312738066861</v>
+        <v>1.418909352864516</v>
       </c>
       <c r="AC2" t="n">
-        <v>1.439151364238168</v>
-      </c>
-      <c r="AD2" t="n">
-        <v>0.235673840971653</v>
+        <v>0.1675068793353582</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>EXFt5ZOk</t>
+          <t>Qol45JK5</t>
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>45770.5625</v>
+        <v>45770.58333333334</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>torino</t>
+          <t>celta vigo</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>udinese</t>
+          <t>villarreal</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>77</v>
+        <v>148</v>
       </c>
       <c r="F3" t="n">
-        <v>771</v>
+        <v>1481</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>italy</t>
+          <t>spain</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>serie a</t>
+          <t>laliga</t>
         </is>
       </c>
       <c r="I3" t="n">
-        <v>2.35</v>
+        <v>2.45</v>
       </c>
       <c r="J3" t="n">
-        <v>3</v>
+        <v>3.5</v>
       </c>
       <c r="K3" t="n">
-        <v>3.4</v>
+        <v>2.8</v>
       </c>
       <c r="L3" t="n">
-        <v>0.4041204437400951</v>
+        <v>0.3883495145631068</v>
       </c>
       <c r="M3" t="n">
-        <v>0.3165610142630745</v>
+        <v>0.2718446601941747</v>
       </c>
       <c r="N3" t="n">
-        <v>0.2793185419968304</v>
+        <v>0.3398058252427185</v>
       </c>
       <c r="O3" t="n">
-        <v>0.05298289528577382</v>
+        <v>0.05102040816326525</v>
       </c>
       <c r="P3" t="n">
         <v>1</v>
       </c>
       <c r="Q3" t="n">
-        <v>0.3611186126731784</v>
+        <v>0.3180124304264202</v>
       </c>
       <c r="R3" t="n">
-        <v>0.3686566276867528</v>
+        <v>0.2022855078106537</v>
       </c>
       <c r="S3" t="n">
-        <v>0.2702247596400687</v>
+        <v>0.4797020617629262</v>
       </c>
       <c r="T3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="U3" t="n">
         <v>1</v>
       </c>
-      <c r="V3" t="inlineStr"/>
+      <c r="V3" t="n">
+        <v>0</v>
+      </c>
       <c r="W3" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="X3" t="n">
-        <v>1</v>
+        <v>0.4797020617629262</v>
       </c>
       <c r="Y3" t="n">
-        <v>0.3686566276867528</v>
-      </c>
-      <c r="Z3" t="n">
-        <v>2.35</v>
-      </c>
-      <c r="AA3" t="inlineStr">
-        <is>
-          <t>kelly_crit &gt; -1.0</t>
-        </is>
+        <v>2.8</v>
+      </c>
+      <c r="Z3" t="inlineStr">
+        <is>
+          <t>kelly_crit &gt; nan</t>
+        </is>
+      </c>
+      <c r="AA3" t="n">
+        <v>0.1906476516312185</v>
       </c>
       <c r="AB3" t="n">
-        <v>-0.09900512958231907</v>
+        <v>2.158659277933168</v>
       </c>
       <c r="AC3" t="n">
-        <v>0.2211939766120517</v>
-      </c>
-      <c r="AD3" t="n">
-        <v>0.007538015013574484</v>
+        <v>0.161689631336506</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>U5sK10Ic</t>
+          <t>lSTUh1hc</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>45770.5625</v>
+        <v>45770.6875</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>cagliari</t>
+          <t>alaves</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>fiorentina</t>
+          <t>real sociedad</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>77</v>
+        <v>148</v>
       </c>
       <c r="F4" t="n">
-        <v>771</v>
+        <v>1481</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>italy</t>
+          <t>spain</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>serie a</t>
+          <t>laliga</t>
         </is>
       </c>
       <c r="I4" t="n">
-        <v>2.9</v>
+        <v>2.35</v>
       </c>
       <c r="J4" t="n">
-        <v>3.1</v>
+        <v>3</v>
       </c>
       <c r="K4" t="n">
-        <v>2.6</v>
+        <v>3.3</v>
       </c>
       <c r="L4" t="n">
-        <v>0.3277755185034567</v>
+        <v>0.4007285974499089</v>
       </c>
       <c r="M4" t="n">
-        <v>0.3066287108580724</v>
+        <v>0.3139040680024286</v>
       </c>
       <c r="N4" t="n">
-        <v>0.3655957706384709</v>
+        <v>0.2853673345476624</v>
       </c>
       <c r="O4" t="n">
-        <v>0.05202361598357141</v>
+        <v>0.06189555125725343</v>
       </c>
       <c r="P4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q4" t="n">
-        <v>0.3328624820903378</v>
+        <v>0.3379240865909751</v>
       </c>
       <c r="R4" t="n">
-        <v>0.2945133354398648</v>
+        <v>0.3111728816903065</v>
       </c>
       <c r="S4" t="n">
-        <v>0.3726241824697973</v>
+        <v>0.3509030317187183</v>
       </c>
       <c r="T4" t="n">
         <v>2</v>
@@ -864,101 +855,100 @@
       <c r="U4" t="n">
         <v>1</v>
       </c>
-      <c r="V4" t="inlineStr"/>
+      <c r="V4" t="n">
+        <v>0</v>
+      </c>
       <c r="W4" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="X4" t="n">
-        <v>2</v>
+        <v>0.3509030317187183</v>
       </c>
       <c r="Y4" t="n">
-        <v>0.3726241824697973</v>
-      </c>
-      <c r="Z4" t="n">
-        <v>2.6</v>
-      </c>
-      <c r="AA4" t="inlineStr">
+        <v>3.3</v>
+      </c>
+      <c r="Z4" t="inlineStr">
         <is>
           <t>kelly_crit &gt; nan</t>
         </is>
       </c>
+      <c r="AA4" t="n">
+        <v>0.06868695855294361</v>
+      </c>
       <c r="AB4" t="n">
-        <v>-0.01948570348657933</v>
+        <v>0.3158127285468465</v>
       </c>
       <c r="AC4" t="n">
-        <v>5.58936273704696</v>
-      </c>
-      <c r="AD4" t="n">
-        <v>0.03976170037945953</v>
+        <v>0.01297894512774322</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>boZzbIHM</t>
+          <t>n1xD3ckI</t>
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>45770.5625</v>
+        <v>45770.6875</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>genoa</t>
+          <t>getafe</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>lazio</t>
+          <t>real madrid</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>77</v>
+        <v>148</v>
       </c>
       <c r="F5" t="n">
-        <v>771</v>
+        <v>1481</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>italy</t>
+          <t>spain</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>serie a</t>
+          <t>laliga</t>
         </is>
       </c>
       <c r="I5" t="n">
-        <v>3.4</v>
+        <v>6</v>
       </c>
       <c r="J5" t="n">
-        <v>3.2</v>
+        <v>3.75</v>
       </c>
       <c r="K5" t="n">
-        <v>2.25</v>
+        <v>1.6</v>
       </c>
       <c r="L5" t="n">
-        <v>0.2798289933929266</v>
+        <v>0.1574803149606299</v>
       </c>
       <c r="M5" t="n">
-        <v>0.2973183054799844</v>
+        <v>0.2519685039370079</v>
       </c>
       <c r="N5" t="n">
-        <v>0.4228527011270889</v>
+        <v>0.5905511811023622</v>
       </c>
       <c r="O5" t="n">
-        <v>0.05106209150326801</v>
+        <v>0.05833333333333335</v>
       </c>
       <c r="P5" t="n">
         <v>2</v>
       </c>
       <c r="Q5" t="n">
-        <v>0.3479151141876893</v>
+        <v>0.2621604061382774</v>
       </c>
       <c r="R5" t="n">
-        <v>0.2679920158913548</v>
+        <v>0.2048180685327325</v>
       </c>
       <c r="S5" t="n">
-        <v>0.3840928699209559</v>
+        <v>0.5330215253289899</v>
       </c>
       <c r="T5" t="n">
         <v>2</v>
@@ -966,134 +956,31 @@
       <c r="U5" t="n">
         <v>1</v>
       </c>
-      <c r="V5" t="inlineStr"/>
+      <c r="V5" t="n">
+        <v>0</v>
+      </c>
       <c r="W5" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="X5" t="n">
-        <v>2</v>
+        <v>0.5330215253289899</v>
       </c>
       <c r="Y5" t="n">
-        <v>0.3840928699209559</v>
-      </c>
-      <c r="Z5" t="n">
-        <v>2.25</v>
-      </c>
-      <c r="AA5" t="inlineStr">
+        <v>1.6</v>
+      </c>
+      <c r="Z5" t="inlineStr">
         <is>
           <t>kelly_crit &gt; nan</t>
         </is>
       </c>
+      <c r="AA5" t="n">
+        <v>-0.2452759324560267</v>
+      </c>
       <c r="AB5" t="n">
-        <v>-0.1086328341422793</v>
+        <v>2.105903728745245</v>
       </c>
       <c r="AC5" t="n">
-        <v>5.761393048814339</v>
-      </c>
-      <c r="AD5" t="n">
-        <v>0.03617775573326665</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="1" t="inlineStr">
-        <is>
-          <t>xhM2CHWF</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="n">
-        <v>45770.5625</v>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>parma</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>juventus</t>
-        </is>
-      </c>
-      <c r="E6" t="n">
-        <v>77</v>
-      </c>
-      <c r="F6" t="n">
-        <v>771</v>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>italy</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>serie a</t>
-        </is>
-      </c>
-      <c r="I6" t="n">
-        <v>5</v>
-      </c>
-      <c r="J6" t="n">
-        <v>3.75</v>
-      </c>
-      <c r="K6" t="n">
-        <v>1.7</v>
-      </c>
-      <c r="L6" t="n">
-        <v>0.1895910780669145</v>
-      </c>
-      <c r="M6" t="n">
-        <v>0.2527881040892193</v>
-      </c>
-      <c r="N6" t="n">
-        <v>0.5576208178438662</v>
-      </c>
-      <c r="O6" t="n">
-        <v>0.05490196078431375</v>
-      </c>
-      <c r="P6" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q6" t="n">
-        <v>0.3652699756173239</v>
-      </c>
-      <c r="R6" t="n">
-        <v>0.1734073610102015</v>
-      </c>
-      <c r="S6" t="n">
-        <v>0.4613226633724746</v>
-      </c>
-      <c r="T6" t="n">
-        <v>2</v>
-      </c>
-      <c r="U6" t="n">
-        <v>1</v>
-      </c>
-      <c r="V6" t="inlineStr"/>
-      <c r="W6" t="n">
-        <v>0</v>
-      </c>
-      <c r="X6" t="n">
-        <v>2</v>
-      </c>
-      <c r="Y6" t="n">
-        <v>0.4613226633724746</v>
-      </c>
-      <c r="Z6" t="n">
-        <v>1.7</v>
-      </c>
-      <c r="AA6" t="inlineStr">
-        <is>
-          <t>kelly_crit &gt; nan</t>
-        </is>
-      </c>
-      <c r="AB6" t="n">
-        <v>-0.3082163889525616</v>
-      </c>
-      <c r="AC6" t="n">
-        <v>6.91983995058712</v>
-      </c>
-      <c r="AD6" t="n">
-        <v>0.09605268775515069</v>
+        <v>0.2708611191907125</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
DATA. Actualizo  preds x cambio de modelo
</commit_message>
<xml_diff>
--- a/data/predicciones.xlsx
+++ b/data/predicciones.xlsx
@@ -644,16 +644,16 @@
         <v>1</v>
       </c>
       <c r="Q2" t="n">
-        <v>0.4418827071980649</v>
+        <v>0.3410371919614035</v>
       </c>
       <c r="R2" t="n">
-        <v>0.2592110382176928</v>
+        <v>0.3918031091522433</v>
       </c>
       <c r="S2" t="n">
-        <v>0.2989062545842425</v>
+        <v>0.2671596988863532</v>
       </c>
       <c r="T2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U2" t="n">
         <v>1</v>
@@ -662,27 +662,27 @@
         <v>0</v>
       </c>
       <c r="W2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X2" t="n">
-        <v>0.4418827071980649</v>
+        <v>0.3918031091522433</v>
       </c>
       <c r="Y2" t="n">
-        <v>3.5</v>
+        <v>2.15</v>
       </c>
       <c r="Z2" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; nan</t>
+          <t>kelly_crit &gt; -0.5</t>
         </is>
       </c>
       <c r="AA2" t="n">
-        <v>0.2186357900772909</v>
+        <v>-0.1370637524545018</v>
       </c>
       <c r="AB2" t="n">
-        <v>6.628240607970974</v>
+        <v>3.938505691746077</v>
       </c>
       <c r="AC2" t="n">
-        <v>0.1429764526138225</v>
+        <v>0.05076591719083973</v>
       </c>
       <c r="AD2" t="inlineStr"/>
     </row>
@@ -746,13 +746,13 @@
         <v>1</v>
       </c>
       <c r="Q3" t="n">
-        <v>0.2754983717893369</v>
+        <v>0.2472735901002061</v>
       </c>
       <c r="R3" t="n">
-        <v>0.4943102875154459</v>
+        <v>0.6514314760480413</v>
       </c>
       <c r="S3" t="n">
-        <v>0.2301913406952171</v>
+        <v>0.1012949338517526</v>
       </c>
       <c r="T3" t="n">
         <v>1</v>
@@ -767,24 +767,24 @@
         <v>1</v>
       </c>
       <c r="X3" t="n">
-        <v>0.4943102875154459</v>
+        <v>0.6514314760480413</v>
       </c>
       <c r="Y3" t="n">
         <v>1.36</v>
       </c>
       <c r="Z3" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; nan</t>
+          <t>kelly_crit &gt; -0.5</t>
         </is>
       </c>
       <c r="AA3" t="n">
-        <v>-0.9103833582749817</v>
+        <v>-0.3168144238185104</v>
       </c>
       <c r="AB3" t="n">
-        <v>0.1547718791292825</v>
+        <v>3.326591054913087</v>
       </c>
       <c r="AC3" t="n">
-        <v>0.218811915726109</v>
+        <v>0.4041578859478352</v>
       </c>
       <c r="AD3" t="inlineStr"/>
     </row>
@@ -848,13 +848,13 @@
         <v>1</v>
       </c>
       <c r="Q4" t="n">
-        <v>0.2764949155694316</v>
+        <v>0.3050884139387492</v>
       </c>
       <c r="R4" t="n">
-        <v>0.5219088866221576</v>
+        <v>0.5641088465614079</v>
       </c>
       <c r="S4" t="n">
-        <v>0.201596197808411</v>
+        <v>0.1308027394998429</v>
       </c>
       <c r="T4" t="n">
         <v>1</v>
@@ -869,24 +869,24 @@
         <v>1</v>
       </c>
       <c r="X4" t="n">
-        <v>0.5219088866221576</v>
+        <v>0.5641088465614079</v>
       </c>
       <c r="Y4" t="n">
         <v>1.73</v>
       </c>
       <c r="Z4" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; nan</t>
+          <t>kelly_crit &gt; -0.5</t>
         </is>
       </c>
       <c r="AA4" t="n">
-        <v>-0.133010446772147</v>
+        <v>-0.03300232253255388</v>
       </c>
       <c r="AB4" t="n">
-        <v>5.317295607749852</v>
+        <v>7.765078682331531</v>
       </c>
       <c r="AC4" t="n">
-        <v>0.245413971052726</v>
+        <v>0.2590204326226587</v>
       </c>
       <c r="AD4" t="inlineStr"/>
     </row>
@@ -950,13 +950,13 @@
         <v>1</v>
       </c>
       <c r="Q5" t="n">
-        <v>0.3105987153696069</v>
+        <v>0.2697374579694876</v>
       </c>
       <c r="R5" t="n">
-        <v>0.4884248683018801</v>
+        <v>0.5757639373088004</v>
       </c>
       <c r="S5" t="n">
-        <v>0.2009764163285131</v>
+        <v>0.1544986047217119</v>
       </c>
       <c r="T5" t="n">
         <v>1</v>
@@ -971,24 +971,24 @@
         <v>1</v>
       </c>
       <c r="X5" t="n">
-        <v>0.4884248683018801</v>
+        <v>0.5757639373088004</v>
       </c>
       <c r="Y5" t="n">
         <v>1.62</v>
       </c>
       <c r="Z5" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; nan</t>
+          <t>kelly_crit &gt; -0.5</t>
         </is>
       </c>
       <c r="AA5" t="n">
-        <v>-0.3366963118563776</v>
+        <v>-0.1084877767092634</v>
       </c>
       <c r="AB5" t="n">
-        <v>2.295132924870908</v>
+        <v>6.349877386036933</v>
       </c>
       <c r="AC5" t="n">
-        <v>0.1778261529322732</v>
+        <v>0.3060264793393128</v>
       </c>
       <c r="AD5" t="inlineStr"/>
     </row>
@@ -1052,16 +1052,16 @@
         <v>1</v>
       </c>
       <c r="Q6" t="n">
-        <v>0.2853248757933991</v>
+        <v>0.3740528384882987</v>
       </c>
       <c r="R6" t="n">
-        <v>0.3598382002205582</v>
+        <v>0.3138522824998449</v>
       </c>
       <c r="S6" t="n">
-        <v>0.3548369239860425</v>
+        <v>0.3120948790118564</v>
       </c>
       <c r="T6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U6" t="n">
         <v>1</v>
@@ -1070,27 +1070,27 @@
         <v>0</v>
       </c>
       <c r="W6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X6" t="n">
-        <v>0.3598382002205582</v>
+        <v>0.3740528384882987</v>
       </c>
       <c r="Y6" t="n">
-        <v>2.25</v>
+        <v>3.6</v>
       </c>
       <c r="Z6" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; nan</t>
+          <t>kelly_crit &gt; -0.5</t>
         </is>
       </c>
       <c r="AA6" t="n">
-        <v>-0.1522912396029952</v>
+        <v>0.1333039302145675</v>
       </c>
       <c r="AB6" t="n">
-        <v>0.6872841831869566</v>
+        <v>5.610792577324481</v>
       </c>
       <c r="AC6" t="n">
-        <v>0.005001276234515739</v>
+        <v>0.06020055598845381</v>
       </c>
       <c r="AD6" t="inlineStr"/>
     </row>
@@ -1154,13 +1154,13 @@
         <v>1</v>
       </c>
       <c r="Q7" t="n">
-        <v>0.2562888214394413</v>
+        <v>0.2502015354678649</v>
       </c>
       <c r="R7" t="n">
-        <v>0.4603817144936768</v>
+        <v>0.5750057368861474</v>
       </c>
       <c r="S7" t="n">
-        <v>0.283329464066882</v>
+        <v>0.1747927276459877</v>
       </c>
       <c r="T7" t="n">
         <v>1</v>
@@ -1175,24 +1175,24 @@
         <v>1</v>
       </c>
       <c r="X7" t="n">
-        <v>0.4603817144936768</v>
+        <v>0.5750057368861474</v>
       </c>
       <c r="Y7" t="n">
         <v>1.85</v>
       </c>
       <c r="Z7" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; nan</t>
+          <t>kelly_crit &gt; -0.5</t>
         </is>
       </c>
       <c r="AA7" t="n">
-        <v>-0.1744633272784681</v>
+        <v>0.07501248616396795</v>
       </c>
       <c r="AB7" t="n">
-        <v>4.07123588723883</v>
+        <v>8.625086053292211</v>
       </c>
       <c r="AC7" t="n">
-        <v>0.1770522504267947</v>
+        <v>0.3248042014182825</v>
       </c>
       <c r="AD7" t="inlineStr"/>
     </row>
@@ -1256,13 +1256,13 @@
         <v>1</v>
       </c>
       <c r="Q8" t="n">
-        <v>0.3972589670207061</v>
+        <v>0.3898403843763301</v>
       </c>
       <c r="R8" t="n">
-        <v>0.2301465440904008</v>
+        <v>0.3056733644905494</v>
       </c>
       <c r="S8" t="n">
-        <v>0.3725944888888933</v>
+        <v>0.3044862511331205</v>
       </c>
       <c r="T8" t="n">
         <v>0</v>
@@ -1277,24 +1277,24 @@
         <v>0</v>
       </c>
       <c r="X8" t="n">
-        <v>0.3972589670207061</v>
+        <v>0.3898403843763301</v>
       </c>
       <c r="Y8" t="n">
         <v>4.1</v>
       </c>
       <c r="Z8" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; nan</t>
+          <t>kelly_crit &gt; -0.5</t>
         </is>
       </c>
       <c r="AA8" t="n">
-        <v>0.2028263757370628</v>
+        <v>0.1930147019170817</v>
       </c>
       <c r="AB8" t="n">
-        <v>5.958884505310591</v>
+        <v>5.847605765644952</v>
       </c>
       <c r="AC8" t="n">
-        <v>0.02466447813181277</v>
+        <v>0.08416701988578074</v>
       </c>
       <c r="AD8" t="inlineStr"/>
     </row>
@@ -1358,13 +1358,13 @@
         <v>2</v>
       </c>
       <c r="Q9" t="n">
-        <v>0.3687211509812872</v>
+        <v>0.3772280303043259</v>
       </c>
       <c r="R9" t="n">
-        <v>0.2049391299646834</v>
+        <v>0.1722214590023226</v>
       </c>
       <c r="S9" t="n">
-        <v>0.4263397190540295</v>
+        <v>0.4505505106933513</v>
       </c>
       <c r="T9" t="n">
         <v>2</v>
@@ -1379,24 +1379,24 @@
         <v>2</v>
       </c>
       <c r="X9" t="n">
-        <v>0.4263397190540295</v>
+        <v>0.4505505106933513</v>
       </c>
       <c r="Y9" t="n">
         <v>2.37</v>
       </c>
       <c r="Z9" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; nan</t>
+          <t>kelly_crit &gt; -0.5</t>
         </is>
       </c>
       <c r="AA9" t="n">
-        <v>0.007609586976678684</v>
+        <v>0.04949248930163704</v>
       </c>
       <c r="AB9" t="n">
-        <v>6.395095785810441</v>
+        <v>6.75825766040027</v>
       </c>
       <c r="AC9" t="n">
-        <v>0.05761856807274229</v>
+        <v>0.07332248038902539</v>
       </c>
       <c r="AD9" t="inlineStr"/>
     </row>
@@ -1460,13 +1460,13 @@
         <v>1</v>
       </c>
       <c r="Q10" t="n">
-        <v>0.3348978768403897</v>
+        <v>0.3173543024462517</v>
       </c>
       <c r="R10" t="n">
-        <v>0.3175277054571968</v>
+        <v>0.2132678871645725</v>
       </c>
       <c r="S10" t="n">
-        <v>0.3475744177024135</v>
+        <v>0.4693778103891758</v>
       </c>
       <c r="T10" t="n">
         <v>2</v>
@@ -1481,24 +1481,24 @@
         <v>2</v>
       </c>
       <c r="X10" t="n">
-        <v>0.3475744177024135</v>
+        <v>0.4693778103891758</v>
       </c>
       <c r="Y10" t="n">
         <v>2.9</v>
       </c>
       <c r="Z10" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; nan</t>
+          <t>kelly_crit &gt; -0.5</t>
         </is>
       </c>
       <c r="AA10" t="n">
-        <v>0.004192532282631185</v>
+        <v>0.1901029737518998</v>
       </c>
       <c r="AB10" t="n">
-        <v>1.042723253107241</v>
+        <v>7.040667155837636</v>
       </c>
       <c r="AC10" t="n">
-        <v>0.01267654086202386</v>
+        <v>0.152023507942924</v>
       </c>
       <c r="AD10" t="inlineStr"/>
     </row>
@@ -1562,16 +1562,16 @@
         <v>1</v>
       </c>
       <c r="Q11" t="n">
-        <v>0.2435259745005133</v>
+        <v>0.3452898604920914</v>
       </c>
       <c r="R11" t="n">
-        <v>0.385792762487333</v>
+        <v>0.1670982391722975</v>
       </c>
       <c r="S11" t="n">
-        <v>0.3706812630121534</v>
+        <v>0.4876119003356111</v>
       </c>
       <c r="T11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="U11" t="n">
         <v>1</v>
@@ -1580,27 +1580,27 @@
         <v>0</v>
       </c>
       <c r="W11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="X11" t="n">
-        <v>0.385792762487333</v>
+        <v>0.4876119003356111</v>
       </c>
       <c r="Y11" t="n">
-        <v>2.15</v>
+        <v>3.2</v>
       </c>
       <c r="Z11" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; nan</t>
+          <t>kelly_crit &gt; -0.5</t>
         </is>
       </c>
       <c r="AA11" t="n">
-        <v>-0.1483004875236818</v>
+        <v>0.2547082186699798</v>
       </c>
       <c r="AB11" t="n">
-        <v>3.734578368348904</v>
+        <v>7.314178505034167</v>
       </c>
       <c r="AC11" t="n">
-        <v>0.01511149947517959</v>
+        <v>0.1423220398435197</v>
       </c>
       <c r="AD11" t="inlineStr"/>
     </row>
@@ -1664,13 +1664,13 @@
         <v>1</v>
       </c>
       <c r="Q12" t="n">
-        <v>0.3790545434674459</v>
+        <v>0.4002298398956136</v>
       </c>
       <c r="R12" t="n">
-        <v>0.3687733834848987</v>
+        <v>0.3767208035460751</v>
       </c>
       <c r="S12" t="n">
-        <v>0.2521720730476553</v>
+        <v>0.2230493565583113</v>
       </c>
       <c r="T12" t="n">
         <v>0</v>
@@ -1685,24 +1685,24 @@
         <v>0</v>
       </c>
       <c r="X12" t="n">
-        <v>0.3790545434674459</v>
+        <v>0.4002298398956136</v>
       </c>
       <c r="Y12" t="n">
         <v>3.3</v>
       </c>
       <c r="Z12" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; nan</t>
+          <t>kelly_crit &gt; -0.5</t>
         </is>
       </c>
       <c r="AA12" t="n">
-        <v>0.1090782580185093</v>
+        <v>0.1394602050676196</v>
       </c>
       <c r="AB12" t="n">
-        <v>5.685818152011688</v>
+        <v>6.003447598434205</v>
       </c>
       <c r="AC12" t="n">
-        <v>0.01028115998254714</v>
+        <v>0.02350903634953855</v>
       </c>
       <c r="AD12" t="inlineStr"/>
     </row>
@@ -1766,13 +1766,13 @@
         <v>1</v>
       </c>
       <c r="Q13" t="n">
-        <v>0.3018545041899909</v>
+        <v>0.2273840027973824</v>
       </c>
       <c r="R13" t="n">
-        <v>0.4595812489095583</v>
+        <v>0.5395384762025993</v>
       </c>
       <c r="S13" t="n">
-        <v>0.238564246900451</v>
+        <v>0.2330775210000184</v>
       </c>
       <c r="T13" t="n">
         <v>1</v>
@@ -1787,7 +1787,7 @@
         <v>1</v>
       </c>
       <c r="X13" t="n">
-        <v>0.4595812489095583</v>
+        <v>0.5395384762025993</v>
       </c>
       <c r="Y13" t="n">
         <v>1.45</v>
@@ -1798,13 +1798,13 @@
         </is>
       </c>
       <c r="AA13" t="n">
-        <v>-0.741349309069201</v>
+        <v>-0.4837093544582912</v>
       </c>
       <c r="AB13" t="n">
-        <v>0.3304667259010766</v>
+        <v>1.323530537755693</v>
       </c>
       <c r="AC13" t="n">
-        <v>0.1577267447195674</v>
+        <v>0.3064609552025809</v>
       </c>
       <c r="AD13" t="inlineStr"/>
     </row>
@@ -1868,13 +1868,13 @@
         <v>2</v>
       </c>
       <c r="Q14" t="n">
-        <v>0.3238477032153495</v>
+        <v>0.1850023135742866</v>
       </c>
       <c r="R14" t="n">
-        <v>0.2261639668365977</v>
+        <v>0.07130080240046054</v>
       </c>
       <c r="S14" t="n">
-        <v>0.4499883299480525</v>
+        <v>0.7436968840252528</v>
       </c>
       <c r="T14" t="n">
         <v>2</v>
@@ -1889,7 +1889,7 @@
         <v>2</v>
       </c>
       <c r="X14" t="n">
-        <v>0.4499883299480525</v>
+        <v>0.7436968840252528</v>
       </c>
       <c r="Y14" t="n">
         <v>2.38</v>
@@ -1900,13 +1900,13 @@
         </is>
       </c>
       <c r="AA14" t="n">
-        <v>0.05142914875098908</v>
+        <v>0.5579699883913781</v>
       </c>
       <c r="AB14" t="n">
-        <v>6.749824949220788</v>
+        <v>11.15545326037879</v>
       </c>
       <c r="AC14" t="n">
-        <v>0.126140626732703</v>
+        <v>0.5586945704509663</v>
       </c>
       <c r="AD14" t="inlineStr"/>
     </row>
@@ -1970,13 +1970,13 @@
         <v>1</v>
       </c>
       <c r="Q15" t="n">
-        <v>0.3503851986378667</v>
+        <v>0.3371006856780407</v>
       </c>
       <c r="R15" t="n">
-        <v>0.253382027079209</v>
+        <v>0.238328725755191</v>
       </c>
       <c r="S15" t="n">
-        <v>0.3962327742829242</v>
+        <v>0.4245705885667683</v>
       </c>
       <c r="T15" t="n">
         <v>2</v>
@@ -1991,7 +1991,7 @@
         <v>2</v>
       </c>
       <c r="X15" t="n">
-        <v>0.3962327742829242</v>
+        <v>0.4245705885667683</v>
       </c>
       <c r="Y15" t="n">
         <v>3.4</v>
@@ -2002,13 +2002,13 @@
         </is>
       </c>
       <c r="AA15" t="n">
-        <v>0.1446630969008093</v>
+        <v>0.1848083338029217</v>
       </c>
       <c r="AB15" t="n">
-        <v>5.943491614243865</v>
+        <v>6.368558828501524</v>
       </c>
       <c r="AC15" t="n">
-        <v>0.04584757564505754</v>
+        <v>0.08746990288872752</v>
       </c>
       <c r="AD15" t="inlineStr"/>
     </row>
@@ -2072,13 +2072,13 @@
         <v>2</v>
       </c>
       <c r="Q16" t="n">
-        <v>0.3286445817700294</v>
+        <v>0.2572044771351923</v>
       </c>
       <c r="R16" t="n">
-        <v>0.1914604910260147</v>
+        <v>0.153403785650949</v>
       </c>
       <c r="S16" t="n">
-        <v>0.479894927203956</v>
+        <v>0.5893917372138587</v>
       </c>
       <c r="T16" t="n">
         <v>2</v>
@@ -2093,7 +2093,7 @@
         <v>2</v>
       </c>
       <c r="X16" t="n">
-        <v>0.479894927203956</v>
+        <v>0.5893917372138587</v>
       </c>
       <c r="Y16" t="n">
         <v>1.44</v>
@@ -2104,13 +2104,13 @@
         </is>
       </c>
       <c r="AA16" t="n">
-        <v>-0.7021620564234167</v>
+        <v>-0.3438088600273716</v>
       </c>
       <c r="AB16" t="n">
-        <v>0.4175979285227749</v>
+        <v>2.68752562045967</v>
       </c>
       <c r="AC16" t="n">
-        <v>0.1512503454339267</v>
+        <v>0.3321872600786664</v>
       </c>
       <c r="AD16" t="inlineStr"/>
     </row>
@@ -2174,16 +2174,16 @@
         <v>1</v>
       </c>
       <c r="Q17" t="n">
-        <v>0.3328014730292285</v>
+        <v>0.3712400922927119</v>
       </c>
       <c r="R17" t="n">
-        <v>0.3634586198177375</v>
+        <v>0.2711924855839672</v>
       </c>
       <c r="S17" t="n">
-        <v>0.3037399071530338</v>
+        <v>0.3575674221233209</v>
       </c>
       <c r="T17" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U17" t="n">
         <v>1</v>
@@ -2192,13 +2192,13 @@
         <v>0</v>
       </c>
       <c r="W17" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X17" t="n">
-        <v>0.3634586198177375</v>
+        <v>0.3712400922927119</v>
       </c>
       <c r="Y17" t="n">
-        <v>1.91</v>
+        <v>3.25</v>
       </c>
       <c r="Z17" t="inlineStr">
         <is>
@@ -2206,13 +2206,13 @@
         </is>
       </c>
       <c r="AA17" t="n">
-        <v>-0.3360374023605729</v>
+        <v>0.09179124442280608</v>
       </c>
       <c r="AB17" t="n">
-        <v>1.712661071709111</v>
+        <v>5.568601384390679</v>
       </c>
       <c r="AC17" t="n">
-        <v>0.030657146788509</v>
+        <v>0.013672670169391</v>
       </c>
       <c r="AD17" t="inlineStr"/>
     </row>
@@ -2276,16 +2276,16 @@
         <v>1</v>
       </c>
       <c r="Q18" t="n">
-        <v>0.3615549477408268</v>
+        <v>0.3057711043206808</v>
       </c>
       <c r="R18" t="n">
-        <v>0.2831061812165305</v>
+        <v>0.2889084367192795</v>
       </c>
       <c r="S18" t="n">
-        <v>0.3553388710426425</v>
+        <v>0.4053204589600398</v>
       </c>
       <c r="T18" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="U18" t="n">
         <v>1</v>
@@ -2294,13 +2294,13 @@
         <v>0</v>
       </c>
       <c r="W18" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="X18" t="n">
-        <v>0.3615549477408268</v>
+        <v>0.4053204589600398</v>
       </c>
       <c r="Y18" t="n">
-        <v>3.4</v>
+        <v>3.5</v>
       </c>
       <c r="Z18" t="inlineStr">
         <is>
@@ -2308,13 +2308,13 @@
         </is>
       </c>
       <c r="AA18" t="n">
-        <v>0.09553617596617131</v>
+        <v>0.1674486425440557</v>
       </c>
       <c r="AB18" t="n">
-        <v>5.423324216112402</v>
+        <v>6.079806884400597</v>
       </c>
       <c r="AC18" t="n">
-        <v>0.006216076698184303</v>
+        <v>0.09954935463935899</v>
       </c>
       <c r="AD18" t="inlineStr"/>
     </row>
@@ -2378,13 +2378,13 @@
         <v>1</v>
       </c>
       <c r="Q19" t="n">
-        <v>0.3128678420375234</v>
+        <v>0.2811497506545466</v>
       </c>
       <c r="R19" t="n">
-        <v>0.4389362225727058</v>
+        <v>0.5558212561018836</v>
       </c>
       <c r="S19" t="n">
-        <v>0.2481959353897706</v>
+        <v>0.1630289932435698</v>
       </c>
       <c r="T19" t="n">
         <v>1</v>
@@ -2399,7 +2399,7 @@
         <v>1</v>
       </c>
       <c r="X19" t="n">
-        <v>0.4389362225727058</v>
+        <v>0.5558212561018836</v>
       </c>
       <c r="Y19" t="n">
         <v>1.38</v>
@@ -2410,13 +2410,13 @@
         </is>
       </c>
       <c r="AA19" t="n">
-        <v>-1.037547402235964</v>
+        <v>-0.6130701752089494</v>
       </c>
       <c r="AB19" t="n">
-        <v>0.07313049147866306</v>
+        <v>0.7430108485311158</v>
       </c>
       <c r="AC19" t="n">
-        <v>0.1260683805351824</v>
+        <v>0.274671505447337</v>
       </c>
       <c r="AD19" t="inlineStr"/>
     </row>
@@ -2480,13 +2480,13 @@
         <v>1</v>
       </c>
       <c r="Q20" t="n">
-        <v>0.3033967294454812</v>
+        <v>0.2640887335469377</v>
       </c>
       <c r="R20" t="n">
-        <v>0.4780836549193525</v>
+        <v>0.4891054495064821</v>
       </c>
       <c r="S20" t="n">
-        <v>0.2185196156351661</v>
+        <v>0.2468058169465801</v>
       </c>
       <c r="T20" t="n">
         <v>1</v>
@@ -2501,7 +2501,7 @@
         <v>1</v>
       </c>
       <c r="X20" t="n">
-        <v>0.4780836549193525</v>
+        <v>0.4891054495064821</v>
       </c>
       <c r="Y20" t="n">
         <v>1.7</v>
@@ -2512,13 +2512,13 @@
         </is>
       </c>
       <c r="AA20" t="n">
-        <v>-0.2675111237672867</v>
+        <v>-0.2407439083414005</v>
       </c>
       <c r="AB20" t="n">
-        <v>2.981984506360453</v>
+        <v>3.386774369459146</v>
       </c>
       <c r="AC20" t="n">
-        <v>0.1746869254738713</v>
+        <v>0.2250167159595444</v>
       </c>
       <c r="AD20" t="inlineStr"/>
     </row>
@@ -2582,13 +2582,13 @@
         <v>1</v>
       </c>
       <c r="Q21" t="n">
-        <v>0.3097568272703692</v>
+        <v>0.2574132259545083</v>
       </c>
       <c r="R21" t="n">
-        <v>0.4411844465109625</v>
+        <v>0.3894570294588393</v>
       </c>
       <c r="S21" t="n">
-        <v>0.2490587262186682</v>
+        <v>0.3531297445866524</v>
       </c>
       <c r="T21" t="n">
         <v>1</v>
@@ -2603,7 +2603,7 @@
         <v>1</v>
       </c>
       <c r="X21" t="n">
-        <v>0.4411844465109625</v>
+        <v>0.3894570294588393</v>
       </c>
       <c r="Y21" t="n">
         <v>2.38</v>
@@ -2614,13 +2614,13 @@
         </is>
       </c>
       <c r="AA21" t="n">
-        <v>0.03624563963484827</v>
+        <v>-0.05296541296229165</v>
       </c>
       <c r="AB21" t="n">
-        <v>6.617766697664438</v>
+        <v>5.072804162094552</v>
       </c>
       <c r="AC21" t="n">
-        <v>0.1314276192405933</v>
+        <v>0.03632728487218695</v>
       </c>
       <c r="AD21" t="inlineStr"/>
     </row>
@@ -2684,13 +2684,13 @@
         <v>1</v>
       </c>
       <c r="Q22" t="n">
-        <v>0.4780703057074003</v>
+        <v>0.407005630500086</v>
       </c>
       <c r="R22" t="n">
-        <v>0.2548551223845782</v>
+        <v>0.2383115745882971</v>
       </c>
       <c r="S22" t="n">
-        <v>0.2670745719080215</v>
+        <v>0.354682794911617</v>
       </c>
       <c r="T22" t="n">
         <v>0</v>
@@ -2705,24 +2705,24 @@
         <v>0</v>
       </c>
       <c r="X22" t="n">
-        <v>0.4780703057074003</v>
+        <v>0.407005630500086</v>
       </c>
       <c r="Y22" t="n">
         <v>3.4</v>
       </c>
       <c r="Z22" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; nan</t>
+          <t>kelly_crit &gt; -0.75</t>
         </is>
       </c>
       <c r="AA22" t="n">
-        <v>0.2605995997521504</v>
+        <v>0.1599246432084551</v>
       </c>
       <c r="AB22" t="n">
-        <v>7.171054585611005</v>
+        <v>6.105084457501289</v>
       </c>
       <c r="AC22" t="n">
-        <v>0.2109957337993787</v>
+        <v>0.05232283558846895</v>
       </c>
       <c r="AD22" t="inlineStr"/>
     </row>
@@ -2786,16 +2786,16 @@
         <v>1</v>
       </c>
       <c r="Q23" t="n">
-        <v>0.2301422652651245</v>
+        <v>0.3256386189419139</v>
       </c>
       <c r="R23" t="n">
-        <v>0.464054314351992</v>
+        <v>0.3080363554532359</v>
       </c>
       <c r="S23" t="n">
-        <v>0.3058034203828836</v>
+        <v>0.3663250256048502</v>
       </c>
       <c r="T23" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="U23" t="n">
         <v>1</v>
@@ -2804,27 +2804,27 @@
         <v>0</v>
       </c>
       <c r="W23" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="X23" t="n">
-        <v>0.464054314351992</v>
+        <v>0.3663250256048502</v>
       </c>
       <c r="Y23" t="n">
-        <v>1.95</v>
+        <v>3.4</v>
       </c>
       <c r="Z23" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; nan</t>
+          <t>kelly_crit &gt; -0.75</t>
         </is>
       </c>
       <c r="AA23" t="n">
-        <v>-0.1000990389617008</v>
+        <v>0.1022937862735378</v>
       </c>
       <c r="AB23" t="n">
-        <v>5.254361287777957</v>
+        <v>5.494875384072753</v>
       </c>
       <c r="AC23" t="n">
-        <v>0.1582508939691084</v>
+        <v>0.04068640666293633</v>
       </c>
       <c r="AD23" t="inlineStr"/>
     </row>
@@ -2888,13 +2888,13 @@
         <v>2</v>
       </c>
       <c r="Q24" t="n">
-        <v>0.3273234557781671</v>
+        <v>0.2518869715834346</v>
       </c>
       <c r="R24" t="n">
-        <v>0.1119557302908993</v>
+        <v>0.1666127366531688</v>
       </c>
       <c r="S24" t="n">
-        <v>0.5607208139309335</v>
+        <v>0.5815002917633966</v>
       </c>
       <c r="T24" t="n">
         <v>2</v>
@@ -2909,24 +2909,24 @@
         <v>2</v>
       </c>
       <c r="X24" t="n">
-        <v>0.5607208139309335</v>
+        <v>0.5815002917633966</v>
       </c>
       <c r="Y24" t="n">
         <v>1.67</v>
       </c>
       <c r="Z24" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; nan</t>
+          <t>kelly_crit &gt; -0.75</t>
         </is>
       </c>
       <c r="AA24" t="n">
-        <v>-0.0949197622915538</v>
+        <v>-0.04312613844048922</v>
       </c>
       <c r="AB24" t="n">
-        <v>6.451569786660839</v>
+        <v>7.785711544890959</v>
       </c>
       <c r="AC24" t="n">
-        <v>0.2333973581527664</v>
+        <v>0.329613320179962</v>
       </c>
       <c r="AD24" t="inlineStr"/>
     </row>
@@ -2990,16 +2990,16 @@
         <v>2</v>
       </c>
       <c r="Q25" t="n">
-        <v>0.3301356296377943</v>
+        <v>0.4162156354773337</v>
       </c>
       <c r="R25" t="n">
-        <v>0.1801021015843405</v>
+        <v>0.1677465903449666</v>
       </c>
       <c r="S25" t="n">
-        <v>0.4897622687778653</v>
+        <v>0.4160377741776998</v>
       </c>
       <c r="T25" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="U25" t="n">
         <v>1</v>
@@ -3008,27 +3008,27 @@
         <v>0</v>
       </c>
       <c r="W25" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="X25" t="n">
-        <v>0.4897622687778653</v>
+        <v>0.4162156354773337</v>
       </c>
       <c r="Y25" t="n">
-        <v>2.5</v>
+        <v>3.4</v>
       </c>
       <c r="Z25" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; nan</t>
+          <t>kelly_crit &gt; -0.75</t>
         </is>
       </c>
       <c r="AA25" t="n">
-        <v>0.1496037812964421</v>
+        <v>0.172972150259556</v>
       </c>
       <c r="AB25" t="n">
-        <v>7.346434031667979</v>
+        <v>6.243234532160006</v>
       </c>
       <c r="AC25" t="n">
-        <v>0.159626639140071</v>
+        <v>0.0001778612996339302</v>
       </c>
       <c r="AD25" t="inlineStr"/>
     </row>
@@ -3092,13 +3092,13 @@
         <v>1</v>
       </c>
       <c r="Q26" t="n">
-        <v>0.3749881226838358</v>
+        <v>0.3743186147623027</v>
       </c>
       <c r="R26" t="n">
-        <v>0.306131501864281</v>
+        <v>0.3090751674768587</v>
       </c>
       <c r="S26" t="n">
-        <v>0.3188803754518832</v>
+        <v>0.3166062177608385</v>
       </c>
       <c r="T26" t="n">
         <v>0</v>
@@ -3113,24 +3113,24 @@
         <v>0</v>
       </c>
       <c r="X26" t="n">
-        <v>0.3749881226838358</v>
+        <v>0.3743186147623027</v>
       </c>
       <c r="Y26" t="n">
         <v>3.6</v>
       </c>
       <c r="Z26" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; nan</t>
+          <t>kelly_crit &gt; -0.75</t>
         </is>
       </c>
       <c r="AA26" t="n">
-        <v>0.1345989391006958</v>
+        <v>0.1336719281324192</v>
       </c>
       <c r="AB26" t="n">
-        <v>5.624821840257537</v>
+        <v>5.61477922143454</v>
       </c>
       <c r="AC26" t="n">
-        <v>0.05610774723195255</v>
+        <v>0.05771239700146419</v>
       </c>
       <c r="AD26" t="inlineStr"/>
     </row>
@@ -3194,13 +3194,13 @@
         <v>1</v>
       </c>
       <c r="Q27" t="n">
-        <v>0.3894818193582197</v>
+        <v>0.2919048118571363</v>
       </c>
       <c r="R27" t="n">
-        <v>0.4163641519052846</v>
+        <v>0.5738696155953339</v>
       </c>
       <c r="S27" t="n">
-        <v>0.1941540287364955</v>
+        <v>0.1342255725475298</v>
       </c>
       <c r="T27" t="n">
         <v>1</v>
@@ -3215,24 +3215,24 @@
         <v>1</v>
       </c>
       <c r="X27" t="n">
-        <v>0.4163641519052846</v>
+        <v>0.5738696155953339</v>
       </c>
       <c r="Y27" t="n">
         <v>1.36</v>
       </c>
       <c r="Z27" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; nan</t>
+          <t>kelly_crit &gt; -0.75</t>
         </is>
       </c>
       <c r="AA27" t="n">
-        <v>-1.204846537246702</v>
+        <v>-0.6098258966398494</v>
       </c>
       <c r="AB27" t="n">
-        <v>0.0301476945031463</v>
+        <v>0.779115306988434</v>
       </c>
       <c r="AC27" t="n">
-        <v>0.0268823325470649</v>
+        <v>0.2819648037381975</v>
       </c>
       <c r="AD27" t="inlineStr"/>
     </row>
@@ -3296,16 +3296,16 @@
         <v>1</v>
       </c>
       <c r="Q28" t="n">
-        <v>0.4523591565450458</v>
+        <v>0.4156008091210714</v>
       </c>
       <c r="R28" t="n">
-        <v>0.4163097137439102</v>
+        <v>0.42208182199215</v>
       </c>
       <c r="S28" t="n">
-        <v>0.131331129711044</v>
+        <v>0.1623173688867787</v>
       </c>
       <c r="T28" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U28" t="n">
         <v>1</v>
@@ -3314,27 +3314,27 @@
         <v>0</v>
       </c>
       <c r="W28" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X28" t="n">
-        <v>0.4523591565450458</v>
+        <v>0.42208182199215</v>
       </c>
       <c r="Y28" t="n">
-        <v>3.9</v>
+        <v>1.83</v>
       </c>
       <c r="Z28" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; nan</t>
+          <t>kelly_crit &gt; -0.75</t>
         </is>
       </c>
       <c r="AA28" t="n">
-        <v>0.2635174863881651</v>
+        <v>-0.2742051394630908</v>
       </c>
       <c r="AB28" t="n">
-        <v>6.785387348175687</v>
+        <v>0.5127133753540537</v>
       </c>
       <c r="AC28" t="n">
-        <v>0.03604944280113559</v>
+        <v>0.006481012871078551</v>
       </c>
       <c r="AD28" t="inlineStr"/>
     </row>
@@ -3398,13 +3398,13 @@
         <v>2</v>
       </c>
       <c r="Q29" t="n">
-        <v>0.2380619601848919</v>
+        <v>0.2279070083096867</v>
       </c>
       <c r="R29" t="n">
-        <v>0.0910117339773403</v>
+        <v>0.08584158819728636</v>
       </c>
       <c r="S29" t="n">
-        <v>0.6709263058377678</v>
+        <v>0.6862514034930269</v>
       </c>
       <c r="T29" t="n">
         <v>2</v>
@@ -3419,24 +3419,24 @@
         <v>2</v>
       </c>
       <c r="X29" t="n">
-        <v>0.6709263058377678</v>
+        <v>0.6862514034930269</v>
       </c>
       <c r="Y29" t="n">
         <v>2.2</v>
       </c>
       <c r="Z29" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; nan</t>
+          <t>kelly_crit &gt; -0.75</t>
         </is>
       </c>
       <c r="AA29" t="n">
-        <v>0.396698227369241</v>
+        <v>0.424794239737216</v>
       </c>
       <c r="AB29" t="n">
-        <v>10.06389458756652</v>
+        <v>10.2937710523954</v>
       </c>
       <c r="AC29" t="n">
-        <v>0.4328643456528759</v>
+        <v>0.4583443951833402</v>
       </c>
       <c r="AD29" t="inlineStr"/>
     </row>
@@ -3500,13 +3500,13 @@
         <v>1</v>
       </c>
       <c r="Q30" t="n">
-        <v>0.503356326874797</v>
+        <v>0.4286156586828706</v>
       </c>
       <c r="R30" t="n">
-        <v>0.2207305837363557</v>
+        <v>0.2949589000308416</v>
       </c>
       <c r="S30" t="n">
-        <v>0.2759130893888472</v>
+        <v>0.2764254412862878</v>
       </c>
       <c r="T30" t="n">
         <v>0</v>
@@ -3521,24 +3521,24 @@
         <v>0</v>
       </c>
       <c r="X30" t="n">
-        <v>0.503356326874797</v>
+        <v>0.4286156586828706</v>
       </c>
       <c r="Y30" t="n">
         <v>3.4</v>
       </c>
       <c r="Z30" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; nan</t>
+          <t>kelly_crit &gt; -0.75</t>
         </is>
       </c>
       <c r="AA30" t="n">
-        <v>0.2964214630726291</v>
+        <v>0.1905388498007334</v>
       </c>
       <c r="AB30" t="n">
-        <v>7.550344903121956</v>
+        <v>6.429234880243058</v>
       </c>
       <c r="AC30" t="n">
-        <v>0.2274432374859498</v>
+        <v>0.133656758652029</v>
       </c>
       <c r="AD30" t="inlineStr"/>
     </row>

</xml_diff>

<commit_message>
DATA. Actualizo preds x cambio de modelos
</commit_message>
<xml_diff>
--- a/data/predicciones.xlsx
+++ b/data/predicciones.xlsx
@@ -644,13 +644,13 @@
         <v>1</v>
       </c>
       <c r="Q2" t="n">
-        <v>0.4418053032385619</v>
+        <v>0.3906344728059287</v>
       </c>
       <c r="R2" t="n">
-        <v>0.2594094311749308</v>
+        <v>0.2986591894615606</v>
       </c>
       <c r="S2" t="n">
-        <v>0.2987852655865074</v>
+        <v>0.3107063377325108</v>
       </c>
       <c r="T2" t="n">
         <v>0</v>
@@ -665,7 +665,7 @@
         <v>0</v>
       </c>
       <c r="X2" t="n">
-        <v>0.4418053032385619</v>
+        <v>0.3906344728059287</v>
       </c>
       <c r="Y2" t="n">
         <v>3.5</v>
@@ -676,13 +676,13 @@
         </is>
       </c>
       <c r="AA2" t="n">
-        <v>0.2185274245339866</v>
+        <v>0.1468882619283002</v>
       </c>
       <c r="AB2" t="n">
-        <v>6.627079548578428</v>
+        <v>5.729204360868709</v>
       </c>
       <c r="AC2" t="n">
-        <v>0.1430200376520545</v>
+        <v>0.07992813507341789</v>
       </c>
       <c r="AD2" t="inlineStr"/>
     </row>
@@ -746,13 +746,13 @@
         <v>1</v>
       </c>
       <c r="Q3" t="n">
-        <v>0.2754983717893369</v>
+        <v>0.2533203279340903</v>
       </c>
       <c r="R3" t="n">
-        <v>0.4943102875154459</v>
+        <v>0.610361216208153</v>
       </c>
       <c r="S3" t="n">
-        <v>0.2301913406952171</v>
+        <v>0.1363184558577568</v>
       </c>
       <c r="T3" t="n">
         <v>1</v>
@@ -767,7 +767,7 @@
         <v>1</v>
       </c>
       <c r="X3" t="n">
-        <v>0.4943102875154459</v>
+        <v>0.610361216208153</v>
       </c>
       <c r="Y3" t="n">
         <v>1.36</v>
@@ -778,13 +778,13 @@
         </is>
       </c>
       <c r="AA3" t="n">
-        <v>-0.9103833582749817</v>
+        <v>-0.4719687387691995</v>
       </c>
       <c r="AB3" t="n">
-        <v>0.1547718791292826</v>
+        <v>2.801056770536586</v>
       </c>
       <c r="AC3" t="n">
-        <v>0.218811915726109</v>
+        <v>0.3570408882740627</v>
       </c>
       <c r="AD3" t="inlineStr"/>
     </row>
@@ -848,13 +848,13 @@
         <v>1</v>
       </c>
       <c r="Q4" t="n">
-        <v>0.2764949155694316</v>
+        <v>0.275794663300176</v>
       </c>
       <c r="R4" t="n">
-        <v>0.5219088866221576</v>
+        <v>0.5121688428171068</v>
       </c>
       <c r="S4" t="n">
-        <v>0.201596197808411</v>
+        <v>0.2120364938827172</v>
       </c>
       <c r="T4" t="n">
         <v>1</v>
@@ -869,7 +869,7 @@
         <v>1</v>
       </c>
       <c r="X4" t="n">
-        <v>0.5219088866221576</v>
+        <v>0.5121688428171068</v>
       </c>
       <c r="Y4" t="n">
         <v>1.73</v>
@@ -880,13 +880,13 @@
         </is>
       </c>
       <c r="AA4" t="n">
-        <v>-0.133010446772147</v>
+        <v>-0.1560930163375414</v>
       </c>
       <c r="AB4" t="n">
-        <v>5.317295607749852</v>
+        <v>4.225812429680431</v>
       </c>
       <c r="AC4" t="n">
-        <v>0.245413971052726</v>
+        <v>0.2363741795169308</v>
       </c>
       <c r="AD4" t="inlineStr"/>
     </row>
@@ -950,13 +950,13 @@
         <v>1</v>
       </c>
       <c r="Q5" t="n">
-        <v>0.3105987153696069</v>
+        <v>0.3431741102042224</v>
       </c>
       <c r="R5" t="n">
-        <v>0.4884248683018801</v>
+        <v>0.517782901181053</v>
       </c>
       <c r="S5" t="n">
-        <v>0.2009764163285131</v>
+        <v>0.1390429886147246</v>
       </c>
       <c r="T5" t="n">
         <v>1</v>
@@ -971,7 +971,7 @@
         <v>1</v>
       </c>
       <c r="X5" t="n">
-        <v>0.4884248683018801</v>
+        <v>0.517782901181053</v>
       </c>
       <c r="Y5" t="n">
         <v>1.53</v>
@@ -982,13 +982,13 @@
         </is>
       </c>
       <c r="AA5" t="n">
-        <v>-0.4768112292417423</v>
+        <v>-0.3920606814962055</v>
       </c>
       <c r="AB5" t="n">
-        <v>1.236641991186384</v>
+        <v>3.134323184491004</v>
       </c>
       <c r="AC5" t="n">
-        <v>0.1778261529322732</v>
+        <v>0.1746087909768306</v>
       </c>
       <c r="AD5" t="inlineStr"/>
     </row>
@@ -1052,16 +1052,16 @@
         <v>1</v>
       </c>
       <c r="Q6" t="n">
-        <v>0.2853248757933991</v>
+        <v>0.341149836405289</v>
       </c>
       <c r="R6" t="n">
-        <v>0.3598382002205582</v>
+        <v>0.3334991497571962</v>
       </c>
       <c r="S6" t="n">
-        <v>0.3548369239860425</v>
+        <v>0.3253510138375147</v>
       </c>
       <c r="T6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U6" t="n">
         <v>1</v>
@@ -1070,13 +1070,13 @@
         <v>0</v>
       </c>
       <c r="W6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X6" t="n">
-        <v>0.3598382002205582</v>
+        <v>0.341149836405289</v>
       </c>
       <c r="Y6" t="n">
-        <v>2.25</v>
+        <v>3.6</v>
       </c>
       <c r="Z6" t="inlineStr">
         <is>
@@ -1084,13 +1084,13 @@
         </is>
       </c>
       <c r="AA6" t="n">
-        <v>-0.1522912396029952</v>
+        <v>0.08774592733040017</v>
       </c>
       <c r="AB6" t="n">
-        <v>0.6872841831869565</v>
+        <v>5.437607116246435</v>
       </c>
       <c r="AC6" t="n">
-        <v>0.005001276234515739</v>
+        <v>0.007650686648092764</v>
       </c>
       <c r="AD6" t="inlineStr"/>
     </row>
@@ -1154,13 +1154,13 @@
         <v>1</v>
       </c>
       <c r="Q7" t="n">
-        <v>0.2562888214394413</v>
+        <v>0.2834292059071453</v>
       </c>
       <c r="R7" t="n">
-        <v>0.4603817144936768</v>
+        <v>0.5327326240051714</v>
       </c>
       <c r="S7" t="n">
-        <v>0.283329464066882</v>
+        <v>0.1838381700876834</v>
       </c>
       <c r="T7" t="n">
         <v>1</v>
@@ -1175,7 +1175,7 @@
         <v>1</v>
       </c>
       <c r="X7" t="n">
-        <v>0.4603817144936768</v>
+        <v>0.5327326240051714</v>
       </c>
       <c r="Y7" t="n">
         <v>1.9</v>
@@ -1186,13 +1186,13 @@
         </is>
       </c>
       <c r="AA7" t="n">
-        <v>-0.1391941582911268</v>
+        <v>0.01354665067758406</v>
       </c>
       <c r="AB7" t="n">
-        <v>4.595154968293159</v>
+        <v>5.067729110409536</v>
       </c>
       <c r="AC7" t="n">
-        <v>0.1770522504267947</v>
+        <v>0.2493034180980261</v>
       </c>
       <c r="AD7" t="inlineStr"/>
     </row>
@@ -1256,16 +1256,16 @@
         <v>1</v>
       </c>
       <c r="Q8" t="n">
-        <v>0.3972589670207061</v>
+        <v>0.346414581316054</v>
       </c>
       <c r="R8" t="n">
-        <v>0.2301465440904008</v>
+        <v>0.2766442065397228</v>
       </c>
       <c r="S8" t="n">
-        <v>0.3725944888888933</v>
+        <v>0.3769412121442232</v>
       </c>
       <c r="T8" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="U8" t="n">
         <v>1</v>
@@ -1274,13 +1274,13 @@
         <v>0</v>
       </c>
       <c r="W8" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="X8" t="n">
-        <v>0.3972589670207061</v>
+        <v>0.3769412121442232</v>
       </c>
       <c r="Y8" t="n">
-        <v>4.2</v>
+        <v>4.75</v>
       </c>
       <c r="Z8" t="inlineStr">
         <is>
@@ -1288,13 +1288,13 @@
         </is>
       </c>
       <c r="AA8" t="n">
-        <v>0.2089023942146767</v>
+        <v>0.2107922020493494</v>
       </c>
       <c r="AB8" t="n">
-        <v>5.958884505310591</v>
+        <v>6.038623216180861</v>
       </c>
       <c r="AC8" t="n">
-        <v>0.02466447813181277</v>
+        <v>0.0305266308281692</v>
       </c>
       <c r="AD8" t="inlineStr"/>
     </row>
@@ -1358,13 +1358,13 @@
         <v>2</v>
       </c>
       <c r="Q9" t="n">
-        <v>0.3687211509812872</v>
+        <v>0.3142408971459947</v>
       </c>
       <c r="R9" t="n">
-        <v>0.2049391299646834</v>
+        <v>0.1429211506875118</v>
       </c>
       <c r="S9" t="n">
-        <v>0.4263397190540295</v>
+        <v>0.5428379521664934</v>
       </c>
       <c r="T9" t="n">
         <v>2</v>
@@ -1379,7 +1379,7 @@
         <v>2</v>
       </c>
       <c r="X9" t="n">
-        <v>0.4263397190540295</v>
+        <v>0.5428379521664934</v>
       </c>
       <c r="Y9" t="n">
         <v>2.3</v>
@@ -1390,13 +1390,13 @@
         </is>
       </c>
       <c r="AA9" t="n">
-        <v>-0.0149374201351787</v>
+        <v>0.1911748384484114</v>
       </c>
       <c r="AB9" t="n">
-        <v>6.156391155214096</v>
+        <v>5.944396911969891</v>
       </c>
       <c r="AC9" t="n">
-        <v>0.05761856807274229</v>
+        <v>0.2285970550204987</v>
       </c>
       <c r="AD9" t="inlineStr"/>
     </row>
@@ -1460,13 +1460,13 @@
         <v>1</v>
       </c>
       <c r="Q10" t="n">
-        <v>0.3348978768403897</v>
+        <v>0.3303506166242103</v>
       </c>
       <c r="R10" t="n">
-        <v>0.3175277054571968</v>
+        <v>0.2632295769566436</v>
       </c>
       <c r="S10" t="n">
-        <v>0.3475744177024135</v>
+        <v>0.4064198064191462</v>
       </c>
       <c r="T10" t="n">
         <v>2</v>
@@ -1481,7 +1481,7 @@
         <v>2</v>
       </c>
       <c r="X10" t="n">
-        <v>0.3475744177024135</v>
+        <v>0.4064198064191462</v>
       </c>
       <c r="Y10" t="n">
         <v>3</v>
@@ -1492,13 +1492,13 @@
         </is>
       </c>
       <c r="AA10" t="n">
-        <v>0.02136162655362034</v>
+        <v>0.1096297096287193</v>
       </c>
       <c r="AB10" t="n">
-        <v>1.042723253107241</v>
+        <v>5.545963048172124</v>
       </c>
       <c r="AC10" t="n">
-        <v>0.01267654086202386</v>
+        <v>0.07606918979493582</v>
       </c>
       <c r="AD10" t="inlineStr"/>
     </row>
@@ -1562,16 +1562,16 @@
         <v>1</v>
       </c>
       <c r="Q11" t="n">
-        <v>0.2435259745005133</v>
+        <v>0.2831084227409584</v>
       </c>
       <c r="R11" t="n">
-        <v>0.385792762487333</v>
+        <v>0.2376399343029854</v>
       </c>
       <c r="S11" t="n">
-        <v>0.3706812630121534</v>
+        <v>0.4792516429560561</v>
       </c>
       <c r="T11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="U11" t="n">
         <v>1</v>
@@ -1580,13 +1580,13 @@
         <v>0</v>
       </c>
       <c r="W11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="X11" t="n">
-        <v>0.385792762487333</v>
+        <v>0.4792516429560561</v>
       </c>
       <c r="Y11" t="n">
-        <v>2.1</v>
+        <v>3.1</v>
       </c>
       <c r="Z11" t="inlineStr">
         <is>
@@ -1594,13 +1594,13 @@
         </is>
       </c>
       <c r="AA11" t="n">
-        <v>-0.1725774534332733</v>
+        <v>0.2312762348398923</v>
       </c>
       <c r="AB11" t="n">
-        <v>3.434363428264557</v>
+        <v>6.1361951794707</v>
       </c>
       <c r="AC11" t="n">
-        <v>0.01511149947517959</v>
+        <v>0.1961432202150977</v>
       </c>
       <c r="AD11" t="inlineStr"/>
     </row>
@@ -1664,16 +1664,16 @@
         <v>1</v>
       </c>
       <c r="Q12" t="n">
-        <v>0.3790545434674459</v>
+        <v>0.3635488162286309</v>
       </c>
       <c r="R12" t="n">
-        <v>0.3687733834848987</v>
+        <v>0.3896264519392756</v>
       </c>
       <c r="S12" t="n">
-        <v>0.2521720730476553</v>
+        <v>0.2468247318320934</v>
       </c>
       <c r="T12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U12" t="n">
         <v>1</v>
@@ -1682,13 +1682,13 @@
         <v>0</v>
       </c>
       <c r="W12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X12" t="n">
-        <v>0.3790545434674459</v>
+        <v>0.3896264519392756</v>
       </c>
       <c r="Y12" t="n">
-        <v>3.3</v>
+        <v>2.35</v>
       </c>
       <c r="Z12" t="inlineStr">
         <is>
@@ -1696,13 +1696,13 @@
         </is>
       </c>
       <c r="AA12" t="n">
-        <v>0.1090782580185093</v>
+        <v>-0.06250210217977945</v>
       </c>
       <c r="AB12" t="n">
-        <v>5.685818152011688</v>
+        <v>4.687895796316427</v>
       </c>
       <c r="AC12" t="n">
-        <v>0.01028115998254714</v>
+        <v>0.02607763571064475</v>
       </c>
       <c r="AD12" t="inlineStr"/>
     </row>
@@ -1766,13 +1766,13 @@
         <v>1</v>
       </c>
       <c r="Q13" t="n">
-        <v>0.2943392415000192</v>
+        <v>0.2273840027973824</v>
       </c>
       <c r="R13" t="n">
-        <v>0.521135983248855</v>
+        <v>0.5395384762025993</v>
       </c>
       <c r="S13" t="n">
-        <v>0.1845247752511259</v>
+        <v>0.2330775210000184</v>
       </c>
       <c r="T13" t="n">
         <v>1</v>
@@ -1787,7 +1787,7 @@
         <v>1</v>
       </c>
       <c r="X13" t="n">
-        <v>0.521135983248855</v>
+        <v>0.5395384762025993</v>
       </c>
       <c r="Y13" t="n">
         <v>1.44</v>
@@ -1798,13 +1798,13 @@
         </is>
       </c>
       <c r="AA13" t="n">
-        <v>-0.5671913275492019</v>
+        <v>-0.5069649869733114</v>
       </c>
       <c r="AB13" t="n">
-        <v>0.8663123718287711</v>
+        <v>2.662114531914633</v>
       </c>
       <c r="AC13" t="n">
-        <v>0.2267967417488359</v>
+        <v>0.3064609552025809</v>
       </c>
       <c r="AD13" t="inlineStr"/>
     </row>
@@ -1868,13 +1868,13 @@
         <v>2</v>
       </c>
       <c r="Q14" t="n">
-        <v>0.2983815280474094</v>
+        <v>0.1850023135742866</v>
       </c>
       <c r="R14" t="n">
-        <v>0.2164254205707549</v>
+        <v>0.07130080240046054</v>
       </c>
       <c r="S14" t="n">
-        <v>0.4851930513818353</v>
+        <v>0.7436968840252528</v>
       </c>
       <c r="T14" t="n">
         <v>2</v>
@@ -1889,7 +1889,7 @@
         <v>2</v>
       </c>
       <c r="X14" t="n">
-        <v>0.4851930513818353</v>
+        <v>0.7436968840252528</v>
       </c>
       <c r="Y14" t="n">
         <v>2.45</v>
@@ -1900,13 +1900,13 @@
         </is>
       </c>
       <c r="AA14" t="n">
-        <v>0.1301537764727563</v>
+        <v>0.566936114387496</v>
       </c>
       <c r="AB14" t="n">
-        <v>7.27789577072753</v>
+        <v>7.565527970716536</v>
       </c>
       <c r="AC14" t="n">
-        <v>0.1868115233344259</v>
+        <v>0.5586945704509663</v>
       </c>
       <c r="AD14" t="inlineStr"/>
     </row>
@@ -1970,13 +1970,13 @@
         <v>1</v>
       </c>
       <c r="Q15" t="n">
-        <v>0.3410409826768729</v>
+        <v>0.3371006856780407</v>
       </c>
       <c r="R15" t="n">
-        <v>0.1680633516249223</v>
+        <v>0.238328725755191</v>
       </c>
       <c r="S15" t="n">
-        <v>0.4908956656982048</v>
+        <v>0.4245705885667683</v>
       </c>
       <c r="T15" t="n">
         <v>2</v>
@@ -1991,7 +1991,7 @@
         <v>2</v>
       </c>
       <c r="X15" t="n">
-        <v>0.4908956656982048</v>
+        <v>0.4245705885667683</v>
       </c>
       <c r="Y15" t="n">
         <v>3.4</v>
@@ -2002,13 +2002,13 @@
         </is>
       </c>
       <c r="AA15" t="n">
-        <v>0.2787688597391235</v>
+        <v>0.1848083338029217</v>
       </c>
       <c r="AB15" t="n">
-        <v>7.363434985473072</v>
+        <v>5.913663485654734</v>
       </c>
       <c r="AC15" t="n">
-        <v>0.1498546830213319</v>
+        <v>0.08746990288872752</v>
       </c>
       <c r="AD15" t="inlineStr"/>
     </row>
@@ -2072,13 +2072,13 @@
         <v>2</v>
       </c>
       <c r="Q16" t="n">
-        <v>0.2834375185251546</v>
+        <v>0.2572044771351923</v>
       </c>
       <c r="R16" t="n">
-        <v>0.2269488283511693</v>
+        <v>0.153403785650949</v>
       </c>
       <c r="S16" t="n">
-        <v>0.4896136531236758</v>
+        <v>0.5893917372138587</v>
       </c>
       <c r="T16" t="n">
         <v>2</v>
@@ -2093,7 +2093,7 @@
         <v>2</v>
       </c>
       <c r="X16" t="n">
-        <v>0.4896136531236758</v>
+        <v>0.5893917372138587</v>
       </c>
       <c r="Y16" t="n">
         <v>1.44</v>
@@ -2104,13 +2104,13 @@
         </is>
       </c>
       <c r="AA16" t="n">
-        <v>-0.6703553170497886</v>
+        <v>-0.3438088600273716</v>
       </c>
       <c r="AB16" t="n">
-        <v>0.4970122404974857</v>
+        <v>3.345632326474306</v>
       </c>
       <c r="AC16" t="n">
-        <v>0.2061761345985211</v>
+        <v>0.3321872600786664</v>
       </c>
       <c r="AD16" t="inlineStr"/>
     </row>
@@ -2174,13 +2174,13 @@
         <v>1</v>
       </c>
       <c r="Q17" t="n">
-        <v>0.364389558359006</v>
+        <v>0.3712400922927119</v>
       </c>
       <c r="R17" t="n">
-        <v>0.2961663789950313</v>
+        <v>0.2711924855839672</v>
       </c>
       <c r="S17" t="n">
-        <v>0.3394440626459628</v>
+        <v>0.3575674221233209</v>
       </c>
       <c r="T17" t="n">
         <v>0</v>
@@ -2195,7 +2195,7 @@
         <v>0</v>
       </c>
       <c r="X17" t="n">
-        <v>0.364389558359006</v>
+        <v>0.3712400922927119</v>
       </c>
       <c r="Y17" t="n">
         <v>3.1</v>
@@ -2206,13 +2206,13 @@
         </is>
       </c>
       <c r="AA17" t="n">
-        <v>0.06171791948234219</v>
+        <v>0.0718306124320985</v>
       </c>
       <c r="AB17" t="n">
-        <v>5.46584337538509</v>
+        <v>5.35853663455098</v>
       </c>
       <c r="AC17" t="n">
-        <v>0.02494549571304322</v>
+        <v>0.013672670169391</v>
       </c>
       <c r="AD17" t="inlineStr"/>
     </row>
@@ -2276,13 +2276,13 @@
         <v>1</v>
       </c>
       <c r="Q18" t="n">
-        <v>0.3722843654659693</v>
+        <v>0.3057711043206808</v>
       </c>
       <c r="R18" t="n">
-        <v>0.1913781061069147</v>
+        <v>0.2889084367192795</v>
       </c>
       <c r="S18" t="n">
-        <v>0.4363375284271158</v>
+        <v>0.4053204589600398</v>
       </c>
       <c r="T18" t="n">
         <v>2</v>
@@ -2297,7 +2297,7 @@
         <v>2</v>
       </c>
       <c r="X18" t="n">
-        <v>0.4363375284271158</v>
+        <v>0.4053204589600398</v>
       </c>
       <c r="Y18" t="n">
         <v>3.4</v>
@@ -2308,13 +2308,13 @@
         </is>
       </c>
       <c r="AA18" t="n">
-        <v>0.2014781652717473</v>
+        <v>0.1575373168600563</v>
       </c>
       <c r="AB18" t="n">
-        <v>6.545062926406737</v>
+        <v>5.781234359106269</v>
       </c>
       <c r="AC18" t="n">
-        <v>0.06405316296114644</v>
+        <v>0.09954935463935899</v>
       </c>
       <c r="AD18" t="inlineStr"/>
     </row>
@@ -2378,13 +2378,13 @@
         <v>1</v>
       </c>
       <c r="Q19" t="n">
-        <v>0.3194425593165873</v>
+        <v>0.2843757352196176</v>
       </c>
       <c r="R19" t="n">
-        <v>0.514161236828877</v>
+        <v>0.5459288447769066</v>
       </c>
       <c r="S19" t="n">
-        <v>0.1663962038545355</v>
+        <v>0.1696954200034758</v>
       </c>
       <c r="T19" t="n">
         <v>1</v>
@@ -2399,7 +2399,7 @@
         <v>1</v>
       </c>
       <c r="X19" t="n">
-        <v>0.514161236828877</v>
+        <v>0.5459288447769066</v>
       </c>
       <c r="Y19" t="n">
         <v>1.36</v>
@@ -2410,13 +2410,13 @@
         </is>
       </c>
       <c r="AA19" t="n">
-        <v>-0.8353908830909086</v>
+        <v>-0.7153799197316858</v>
       </c>
       <c r="AB19" t="n">
-        <v>0.2331195116698631</v>
+        <v>1.929803200517899</v>
       </c>
       <c r="AC19" t="n">
-        <v>0.1947186775122897</v>
+        <v>0.261553109557289</v>
       </c>
       <c r="AD19" t="inlineStr"/>
     </row>
@@ -2480,13 +2480,13 @@
         <v>1</v>
       </c>
       <c r="Q20" t="n">
-        <v>0.2925286430661067</v>
+        <v>0.2640887335469377</v>
       </c>
       <c r="R20" t="n">
-        <v>0.5268840344858372</v>
+        <v>0.4891054495064821</v>
       </c>
       <c r="S20" t="n">
-        <v>0.180587322448056</v>
+        <v>0.2468058169465801</v>
       </c>
       <c r="T20" t="n">
         <v>1</v>
@@ -2501,7 +2501,7 @@
         <v>1</v>
       </c>
       <c r="X20" t="n">
-        <v>0.5268840344858372</v>
+        <v>0.4891054495064821</v>
       </c>
       <c r="Y20" t="n">
         <v>1.65</v>
@@ -2512,13 +2512,13 @@
         </is>
       </c>
       <c r="AA20" t="n">
-        <v>-0.200986681689798</v>
+        <v>-0.2968861666373916</v>
       </c>
       <c r="AB20" t="n">
-        <v>4.235713918543629</v>
+        <v>3.55769774763221</v>
       </c>
       <c r="AC20" t="n">
-        <v>0.2343553914197306</v>
+        <v>0.2250167159595444</v>
       </c>
       <c r="AD20" t="inlineStr"/>
     </row>
@@ -2582,13 +2582,13 @@
         <v>1</v>
       </c>
       <c r="Q21" t="n">
-        <v>0.2930913113917836</v>
+        <v>0.2596359731869547</v>
       </c>
       <c r="R21" t="n">
-        <v>0.4862200580418363</v>
+        <v>0.3733801863884679</v>
       </c>
       <c r="S21" t="n">
-        <v>0.2206886305663801</v>
+        <v>0.3669838404245774</v>
       </c>
       <c r="T21" t="n">
         <v>1</v>
@@ -2603,7 +2603,7 @@
         <v>1</v>
       </c>
       <c r="X21" t="n">
-        <v>0.4862200580418363</v>
+        <v>0.3733801863884679</v>
       </c>
       <c r="Y21" t="n">
         <v>2.3</v>
@@ -2614,13 +2614,13 @@
         </is>
       </c>
       <c r="AA21" t="n">
-        <v>0.09100471807401804</v>
+        <v>-0.1086350548511722</v>
       </c>
       <c r="AB21" t="n">
-        <v>7.293300870627545</v>
+        <v>0.8917902922761543</v>
       </c>
       <c r="AC21" t="n">
-        <v>0.1931287466500527</v>
+        <v>0.006396345963890493</v>
       </c>
       <c r="AD21" t="inlineStr"/>
     </row>
@@ -2684,13 +2684,13 @@
         <v>1</v>
       </c>
       <c r="Q22" t="n">
-        <v>0.3756752090953401</v>
+        <v>0.3264364865493029</v>
       </c>
       <c r="R22" t="n">
-        <v>0.1976712533964415</v>
+        <v>0.3167617179253894</v>
       </c>
       <c r="S22" t="n">
-        <v>0.4266535375082184</v>
+        <v>0.3568017955253077</v>
       </c>
       <c r="T22" t="n">
         <v>2</v>
@@ -2705,7 +2705,7 @@
         <v>2</v>
       </c>
       <c r="X22" t="n">
-        <v>0.4266535375082184</v>
+        <v>0.3568017955253077</v>
       </c>
       <c r="Y22" t="n">
         <v>3</v>
@@ -2716,15 +2716,17 @@
         </is>
       </c>
       <c r="AA22" t="n">
-        <v>0.1399803062623275</v>
+        <v>0.0352026932879615</v>
       </c>
       <c r="AB22" t="n">
-        <v>6.399803062623276</v>
+        <v>5.175940795428621</v>
       </c>
       <c r="AC22" t="n">
-        <v>0.05097832841287825</v>
-      </c>
-      <c r="AD22" t="inlineStr"/>
+        <v>0.03036530897600476</v>
+      </c>
+      <c r="AD22" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="1" t="inlineStr">
@@ -2786,13 +2788,13 @@
         <v>1</v>
       </c>
       <c r="Q23" t="n">
-        <v>0.2674023311638205</v>
+        <v>0.2241513331956759</v>
       </c>
       <c r="R23" t="n">
-        <v>0.1921813852603847</v>
+        <v>0.3493469526896319</v>
       </c>
       <c r="S23" t="n">
-        <v>0.5404162835757947</v>
+        <v>0.4265017141146922</v>
       </c>
       <c r="T23" t="n">
         <v>2</v>
@@ -2800,14 +2802,12 @@
       <c r="U23" t="n">
         <v>1</v>
       </c>
-      <c r="V23" t="n">
-        <v>0</v>
-      </c>
+      <c r="V23" t="inlineStr"/>
       <c r="W23" t="n">
         <v>2</v>
       </c>
       <c r="X23" t="n">
-        <v>0.5404162835757947</v>
+        <v>0.4265017141146922</v>
       </c>
       <c r="Y23" t="n">
         <v>3.2</v>
@@ -2818,13 +2818,13 @@
         </is>
       </c>
       <c r="AA23" t="n">
-        <v>0.3315145942920651</v>
+        <v>0.165820675075916</v>
       </c>
       <c r="AB23" t="n">
-        <v>8.106244253636921</v>
+        <v>5.82158688941985</v>
       </c>
       <c r="AC23" t="n">
-        <v>0.2730139524119742</v>
+        <v>0.07715476142506034</v>
       </c>
       <c r="AD23" t="inlineStr"/>
     </row>
@@ -2888,13 +2888,13 @@
         <v>2</v>
       </c>
       <c r="Q24" t="n">
-        <v>0.159508727142733</v>
+        <v>0.1467692902417288</v>
       </c>
       <c r="R24" t="n">
-        <v>0.1137989329454182</v>
+        <v>0.1315693047429575</v>
       </c>
       <c r="S24" t="n">
-        <v>0.7266923399118488</v>
+        <v>0.7216614050153137</v>
       </c>
       <c r="T24" t="n">
         <v>2</v>
@@ -2902,14 +2902,12 @@
       <c r="U24" t="n">
         <v>1</v>
       </c>
-      <c r="V24" t="n">
-        <v>0</v>
-      </c>
+      <c r="V24" t="inlineStr"/>
       <c r="W24" t="n">
         <v>2</v>
       </c>
       <c r="X24" t="n">
-        <v>0.7266923399118488</v>
+        <v>0.7216614050153137</v>
       </c>
       <c r="Y24" t="n">
         <v>1.65</v>
@@ -2920,13 +2918,13 @@
         </is>
       </c>
       <c r="AA24" t="n">
-        <v>0.3062190166993083</v>
+        <v>0.2934481819619502</v>
       </c>
       <c r="AB24" t="n">
-        <v>10.90038509867773</v>
+        <v>6.426527110329742</v>
       </c>
       <c r="AC24" t="n">
-        <v>0.5671836127691158</v>
+        <v>0.5748921147735849</v>
       </c>
       <c r="AD24" t="inlineStr"/>
     </row>
@@ -2990,13 +2988,13 @@
         <v>2</v>
       </c>
       <c r="Q25" t="n">
-        <v>0.207038920528792</v>
+        <v>0.2628343802815696</v>
       </c>
       <c r="R25" t="n">
-        <v>0.199471387948202</v>
+        <v>0.3452111946391885</v>
       </c>
       <c r="S25" t="n">
-        <v>0.593489691523006</v>
+        <v>0.391954425079242</v>
       </c>
       <c r="T25" t="n">
         <v>2</v>
@@ -3004,14 +3002,12 @@
       <c r="U25" t="n">
         <v>1</v>
       </c>
-      <c r="V25" t="n">
-        <v>0</v>
-      </c>
+      <c r="V25" t="inlineStr"/>
       <c r="W25" t="n">
         <v>2</v>
       </c>
       <c r="X25" t="n">
-        <v>0.593489691523006</v>
+        <v>0.391954425079242</v>
       </c>
       <c r="Y25" t="n">
         <v>2.5</v>
@@ -3022,13 +3018,13 @@
         </is>
       </c>
       <c r="AA25" t="n">
-        <v>0.32248281920501</v>
+        <v>-0.01340929153459669</v>
       </c>
       <c r="AB25" t="n">
-        <v>8.90234537284509</v>
+        <v>4.932957560559069</v>
       </c>
       <c r="AC25" t="n">
-        <v>0.386450770994214</v>
+        <v>0.04674323044005352</v>
       </c>
       <c r="AD25" t="inlineStr"/>
     </row>
@@ -3092,13 +3088,13 @@
         <v>2</v>
       </c>
       <c r="Q26" t="n">
-        <v>0.3173458151128735</v>
+        <v>0.2980185458057887</v>
       </c>
       <c r="R26" t="n">
-        <v>0.216914804981591</v>
+        <v>0.2163073649544265</v>
       </c>
       <c r="S26" t="n">
-        <v>0.4657393799055355</v>
+        <v>0.4856740892397848</v>
       </c>
       <c r="T26" t="n">
         <v>2</v>
@@ -3106,14 +3102,12 @@
       <c r="U26" t="n">
         <v>1</v>
       </c>
-      <c r="V26" t="n">
-        <v>0</v>
-      </c>
+      <c r="V26" t="inlineStr"/>
       <c r="W26" t="n">
         <v>2</v>
       </c>
       <c r="X26" t="n">
-        <v>0.4657393799055355</v>
+        <v>0.4856740892397848</v>
       </c>
       <c r="Y26" t="n">
         <v>2.5</v>
@@ -3124,13 +3118,13 @@
         </is>
       </c>
       <c r="AA26" t="n">
-        <v>0.1095656331758926</v>
+        <v>0.1427901487329747</v>
       </c>
       <c r="AB26" t="n">
-        <v>6.986090698583033</v>
+        <v>5.709137739284925</v>
       </c>
       <c r="AC26" t="n">
-        <v>0.148393564792662</v>
+        <v>0.1876555434339961</v>
       </c>
       <c r="AD26" t="inlineStr"/>
     </row>
@@ -3194,13 +3188,13 @@
         <v>1</v>
       </c>
       <c r="Q27" t="n">
-        <v>0.345892390552328</v>
+        <v>0.2780915673052358</v>
       </c>
       <c r="R27" t="n">
-        <v>0.4006060075698742</v>
+        <v>0.4800350930801974</v>
       </c>
       <c r="S27" t="n">
-        <v>0.2535016018777978</v>
+        <v>0.2418733396145669</v>
       </c>
       <c r="T27" t="n">
         <v>1</v>
@@ -3215,7 +3209,7 @@
         <v>1</v>
       </c>
       <c r="X27" t="n">
-        <v>0.4006060075698742</v>
+        <v>0.4800350930801974</v>
       </c>
       <c r="Y27" t="n">
         <v>1.33</v>
@@ -3226,15 +3220,17 @@
         </is>
       </c>
       <c r="AA27" t="n">
-        <v>-1.415739424036567</v>
+        <v>-1.095616140010113</v>
       </c>
       <c r="AB27" t="n">
-        <v>0.01012123979205655</v>
+        <v>1.005406009173694</v>
       </c>
       <c r="AC27" t="n">
-        <v>0.05471361701754629</v>
-      </c>
-      <c r="AD27" t="inlineStr"/>
+        <v>0.2019435257749616</v>
+      </c>
+      <c r="AD27" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="1" t="inlineStr">
@@ -3296,16 +3292,16 @@
         <v>1</v>
       </c>
       <c r="Q28" t="n">
-        <v>0.4315588803422828</v>
+        <v>0.2391541941316752</v>
       </c>
       <c r="R28" t="n">
-        <v>0.2065485153517193</v>
+        <v>0.3854824935478348</v>
       </c>
       <c r="S28" t="n">
-        <v>0.3618926043059978</v>
+        <v>0.37536331232049</v>
       </c>
       <c r="T28" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U28" t="n">
         <v>1</v>
@@ -3314,13 +3310,13 @@
         <v>0</v>
       </c>
       <c r="W28" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X28" t="n">
-        <v>0.4315588803422828</v>
+        <v>0.3854824935478348</v>
       </c>
       <c r="Y28" t="n">
-        <v>3.9</v>
+        <v>1.83</v>
       </c>
       <c r="Z28" t="inlineStr">
         <is>
@@ -3328,15 +3324,17 @@
         </is>
       </c>
       <c r="AA28" t="n">
-        <v>0.2355447011499666</v>
+        <v>-0.35490004434634</v>
       </c>
       <c r="AB28" t="n">
-        <v>6.473383205134243</v>
+        <v>0.6592860295738084</v>
       </c>
       <c r="AC28" t="n">
-        <v>0.06966627603628506</v>
-      </c>
-      <c r="AD28" t="inlineStr"/>
+        <v>0.01011918122734479</v>
+      </c>
+      <c r="AD28" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="1" t="inlineStr">
@@ -3398,13 +3396,13 @@
         <v>2</v>
       </c>
       <c r="Q29" t="n">
-        <v>0.3233844558522494</v>
+        <v>0.3032574772999943</v>
       </c>
       <c r="R29" t="n">
-        <v>0.1162827979533897</v>
+        <v>0.1190968913455669</v>
       </c>
       <c r="S29" t="n">
-        <v>0.5603327461943609</v>
+        <v>0.5776456313544387</v>
       </c>
       <c r="T29" t="n">
         <v>2</v>
@@ -3419,7 +3417,7 @@
         <v>2</v>
       </c>
       <c r="X29" t="n">
-        <v>0.5603327461943609</v>
+        <v>0.5776456313544387</v>
       </c>
       <c r="Y29" t="n">
         <v>2.2</v>
@@ -3430,15 +3428,17 @@
         </is>
       </c>
       <c r="AA29" t="n">
-        <v>0.1939433680229951</v>
+        <v>0.2256836574831377</v>
       </c>
       <c r="AB29" t="n">
-        <v>8.404991192915414</v>
+        <v>6.10964276110885</v>
       </c>
       <c r="AC29" t="n">
-        <v>0.2369482903421115</v>
-      </c>
-      <c r="AD29" t="inlineStr"/>
+        <v>0.2743881540544444</v>
+      </c>
+      <c r="AD29" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="1" t="inlineStr">
@@ -3500,13 +3500,13 @@
         <v>1</v>
       </c>
       <c r="Q30" t="n">
-        <v>0.3101912443453831</v>
+        <v>0.3332557203039493</v>
       </c>
       <c r="R30" t="n">
-        <v>0.301182244058597</v>
+        <v>0.2329169819764269</v>
       </c>
       <c r="S30" t="n">
-        <v>0.3886265115960198</v>
+        <v>0.4338272977196239</v>
       </c>
       <c r="T30" t="n">
         <v>2</v>
@@ -3521,7 +3521,7 @@
         <v>2</v>
       </c>
       <c r="X30" t="n">
-        <v>0.3886265115960198</v>
+        <v>0.4338272977196239</v>
       </c>
       <c r="Y30" t="n">
         <v>2.9</v>
@@ -3532,15 +3532,17 @@
         </is>
       </c>
       <c r="AA30" t="n">
-        <v>0.06685099138339864</v>
+        <v>0.1358416649404786</v>
       </c>
       <c r="AB30" t="n">
-        <v>5.829397673940297</v>
+        <v>5.675061132320044</v>
       </c>
       <c r="AC30" t="n">
-        <v>0.07843526725063671</v>
-      </c>
-      <c r="AD30" t="inlineStr"/>
+        <v>0.1005715774156746</v>
+      </c>
+      <c r="AD30" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="1" t="inlineStr">
@@ -3602,13 +3604,13 @@
         <v>1</v>
       </c>
       <c r="Q31" t="n">
-        <v>0.2647107849572503</v>
+        <v>0.3229623069552767</v>
       </c>
       <c r="R31" t="n">
-        <v>0.2545061857113567</v>
+        <v>0.317325535489806</v>
       </c>
       <c r="S31" t="n">
-        <v>0.4807830293313929</v>
+        <v>0.3597121575549173</v>
       </c>
       <c r="T31" t="n">
         <v>2</v>
@@ -3623,7 +3625,7 @@
         <v>2</v>
       </c>
       <c r="X31" t="n">
-        <v>0.4807830293313929</v>
+        <v>0.3597121575549173</v>
       </c>
       <c r="Y31" t="n">
         <v>3.6</v>
@@ -3634,15 +3636,17 @@
         </is>
       </c>
       <c r="AA31" t="n">
-        <v>0.2810841944588516</v>
+        <v>0.1134476027683471</v>
       </c>
       <c r="AB31" t="n">
-        <v>7.211745439970893</v>
+        <v>5.564816958141988</v>
       </c>
       <c r="AC31" t="n">
-        <v>0.2160722443741426</v>
-      </c>
-      <c r="AD31" t="inlineStr"/>
+        <v>0.03674985059964064</v>
+      </c>
+      <c r="AD31" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="1" t="inlineStr">
@@ -3704,16 +3708,16 @@
         <v>1</v>
       </c>
       <c r="Q32" t="n">
-        <v>0.3883984958291617</v>
+        <v>0.4366963381262134</v>
       </c>
       <c r="R32" t="n">
-        <v>0.4383362249268591</v>
+        <v>0.4144141832066483</v>
       </c>
       <c r="S32" t="n">
-        <v>0.173265279243979</v>
+        <v>0.1488894786671383</v>
       </c>
       <c r="T32" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U32" t="n">
         <v>1</v>
@@ -3722,27 +3726,27 @@
         <v>0</v>
       </c>
       <c r="W32" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X32" t="n">
-        <v>0.4383362249268591</v>
+        <v>0.4366963381262134</v>
       </c>
       <c r="Y32" t="n">
-        <v>2.2</v>
+        <v>3</v>
       </c>
       <c r="Z32" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; -0.75</t>
+          <t>kelly_crit &gt; nan</t>
         </is>
       </c>
       <c r="AA32" t="n">
-        <v>-0.02971692096742482</v>
+        <v>0.1550445071893201</v>
       </c>
       <c r="AB32" t="n">
-        <v>6.087464971257314</v>
+        <v>5.769069883834351</v>
       </c>
       <c r="AC32" t="n">
-        <v>0.04993772909769745</v>
+        <v>0.02228215491956509</v>
       </c>
       <c r="AD32" t="inlineStr"/>
     </row>
@@ -3806,13 +3810,13 @@
         <v>1</v>
       </c>
       <c r="Q33" t="n">
-        <v>0.3726941876957314</v>
+        <v>0.4425093100409055</v>
       </c>
       <c r="R33" t="n">
-        <v>0.3477884910892599</v>
+        <v>0.2995949267724266</v>
       </c>
       <c r="S33" t="n">
-        <v>0.2795173212150085</v>
+        <v>0.2578957631866678</v>
       </c>
       <c r="T33" t="n">
         <v>0</v>
@@ -3827,24 +3831,24 @@
         <v>0</v>
       </c>
       <c r="X33" t="n">
-        <v>0.3726941876957314</v>
+        <v>0.4425093100409055</v>
       </c>
       <c r="Y33" t="n">
         <v>3.2</v>
       </c>
       <c r="Z33" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; -0.75</t>
+          <t>kelly_crit &gt; nan</t>
         </is>
       </c>
       <c r="AA33" t="n">
-        <v>0.08755518210288213</v>
+        <v>0.1891044509685899</v>
       </c>
       <c r="AB33" t="n">
-        <v>5.590412815435972</v>
+        <v>5.934410393302548</v>
       </c>
       <c r="AC33" t="n">
-        <v>0.02490569660647157</v>
+        <v>0.1429143832684789</v>
       </c>
       <c r="AD33" t="inlineStr"/>
     </row>
@@ -3908,13 +3912,13 @@
         <v>2</v>
       </c>
       <c r="Q34" t="n">
-        <v>0.3915323321719533</v>
+        <v>0.4327062245499772</v>
       </c>
       <c r="R34" t="n">
-        <v>0.2422378398140923</v>
+        <v>0.2015156625049229</v>
       </c>
       <c r="S34" t="n">
-        <v>0.3662298280139545</v>
+        <v>0.3657781129450999</v>
       </c>
       <c r="T34" t="n">
         <v>0</v>
@@ -3929,24 +3933,24 @@
         <v>0</v>
       </c>
       <c r="X34" t="n">
-        <v>0.3915323321719533</v>
+        <v>0.4327062245499772</v>
       </c>
       <c r="Y34" t="n">
         <v>3.3</v>
       </c>
       <c r="Z34" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; -0.75</t>
+          <t>kelly_crit &gt; nan</t>
         </is>
       </c>
       <c r="AA34" t="n">
-        <v>0.1269811722467155</v>
+        <v>0.1860567569630107</v>
       </c>
       <c r="AB34" t="n">
-        <v>5.872984982579299</v>
+        <v>5.919695790207257</v>
       </c>
       <c r="AC34" t="n">
-        <v>0.02530250415799878</v>
+        <v>0.06692811160487733</v>
       </c>
       <c r="AD34" t="inlineStr"/>
     </row>
@@ -4010,13 +4014,13 @@
         <v>2</v>
       </c>
       <c r="Q35" t="n">
-        <v>0.2881971055018751</v>
+        <v>0.2875146835929583</v>
       </c>
       <c r="R35" t="n">
-        <v>0.08754446620003138</v>
+        <v>0.08181949214912757</v>
       </c>
       <c r="S35" t="n">
-        <v>0.6242584282980936</v>
+        <v>0.6306658242579142</v>
       </c>
       <c r="T35" t="n">
         <v>2</v>
@@ -4031,24 +4035,24 @@
         <v>2</v>
       </c>
       <c r="X35" t="n">
-        <v>0.6242584282980936</v>
+        <v>0.6306658242579142</v>
       </c>
       <c r="Y35" t="n">
         <v>1.53</v>
       </c>
       <c r="Z35" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; -0.75</t>
+          <t>kelly_crit &gt; nan</t>
         </is>
       </c>
       <c r="AA35" t="n">
-        <v>-0.08468793340361641</v>
+        <v>-0.0661911111045119</v>
       </c>
       <c r="AB35" t="n">
-        <v>7.410458718714607</v>
+        <v>4.669526933394934</v>
       </c>
       <c r="AC35" t="n">
-        <v>0.3360613227962185</v>
+        <v>0.3431511406649559</v>
       </c>
       <c r="AD35" t="inlineStr"/>
     </row>
@@ -4112,13 +4116,13 @@
         <v>1</v>
       </c>
       <c r="Q36" t="n">
-        <v>0.2995201516910434</v>
+        <v>0.1826612458612728</v>
       </c>
       <c r="R36" t="n">
-        <v>0.6215904388534337</v>
+        <v>0.7528138355906638</v>
       </c>
       <c r="S36" t="n">
-        <v>0.0788894094555231</v>
+        <v>0.06452491854806336</v>
       </c>
       <c r="T36" t="n">
         <v>1</v>
@@ -4133,24 +4137,24 @@
         <v>1</v>
       </c>
       <c r="X36" t="n">
-        <v>0.6215904388534337</v>
+        <v>0.7528138355906638</v>
       </c>
       <c r="Y36" t="n">
         <v>1.29</v>
       </c>
       <c r="Z36" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; -0.75</t>
+          <t>kelly_crit &gt; nan</t>
         </is>
       </c>
       <c r="AA36" t="n">
-        <v>-0.683270116824381</v>
+        <v>-0.09955224857946071</v>
       </c>
       <c r="AB36" t="n">
-        <v>0.5927801794415223</v>
+        <v>4.503876643587681</v>
       </c>
       <c r="AC36" t="n">
-        <v>0.3220702871623903</v>
+        <v>0.5701525897293911</v>
       </c>
       <c r="AD36" t="inlineStr"/>
     </row>
@@ -4214,13 +4218,13 @@
         <v>2</v>
       </c>
       <c r="Q37" t="n">
-        <v>0.2600864299081894</v>
+        <v>0.2384064344370778</v>
       </c>
       <c r="R37" t="n">
-        <v>0.07766276810971705</v>
+        <v>0.06859628571736094</v>
       </c>
       <c r="S37" t="n">
-        <v>0.6622508019820933</v>
+        <v>0.6929972798455611</v>
       </c>
       <c r="T37" t="n">
         <v>2</v>
@@ -4235,24 +4239,24 @@
         <v>2</v>
       </c>
       <c r="X37" t="n">
-        <v>0.6622508019820933</v>
+        <v>0.6929972798455611</v>
       </c>
       <c r="Y37" t="n">
         <v>1.83</v>
       </c>
       <c r="Z37" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; -0.75</t>
+          <t>kelly_crit &gt; nan</t>
         </is>
       </c>
       <c r="AA37" t="n">
-        <v>0.2553240573822056</v>
+        <v>0.3231144844787673</v>
       </c>
       <c r="AB37" t="n">
-        <v>9.933762029731399</v>
+        <v>6.561601670013054</v>
       </c>
       <c r="AC37" t="n">
-        <v>0.4021643720739039</v>
+        <v>0.4545908454084833</v>
       </c>
       <c r="AD37" t="inlineStr"/>
     </row>
@@ -4316,13 +4320,13 @@
         <v>2</v>
       </c>
       <c r="Q38" t="n">
-        <v>0.252138555541956</v>
+        <v>0.2508926092721898</v>
       </c>
       <c r="R38" t="n">
-        <v>0.0654175246755673</v>
+        <v>0.06510804873340995</v>
       </c>
       <c r="S38" t="n">
-        <v>0.682443919782477</v>
+        <v>0.6839993419944003</v>
       </c>
       <c r="T38" t="n">
         <v>2</v>
@@ -4337,24 +4341,24 @@
         <v>2</v>
       </c>
       <c r="X38" t="n">
-        <v>0.682443919782477</v>
+        <v>0.6839993419944003</v>
       </c>
       <c r="Y38" t="n">
         <v>1.25</v>
       </c>
       <c r="Z38" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; -0.75</t>
+          <t>kelly_crit &gt; nan</t>
         </is>
       </c>
       <c r="AA38" t="n">
-        <v>-0.5877804010876151</v>
+        <v>-0.5800032900279987</v>
       </c>
       <c r="AB38" t="n">
-        <v>1.02906392639012</v>
+        <v>2.386660895286746</v>
       </c>
       <c r="AC38" t="n">
-        <v>0.430305364240521</v>
+        <v>0.4331067327222105</v>
       </c>
       <c r="AD38" t="inlineStr"/>
     </row>
@@ -4418,13 +4422,13 @@
         <v>1</v>
       </c>
       <c r="Q39" t="n">
-        <v>0.3686601688034257</v>
+        <v>0.3212354611392007</v>
       </c>
       <c r="R39" t="n">
-        <v>0.3765066884570603</v>
+        <v>0.4469678270179713</v>
       </c>
       <c r="S39" t="n">
-        <v>0.2548331427395139</v>
+        <v>0.231796711842828</v>
       </c>
       <c r="T39" t="n">
         <v>1</v>
@@ -4439,24 +4443,24 @@
         <v>1</v>
       </c>
       <c r="X39" t="n">
-        <v>0.3765066884570603</v>
+        <v>0.4469678270179713</v>
       </c>
       <c r="Y39" t="n">
         <v>1.67</v>
       </c>
       <c r="Z39" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; -0.75</t>
+          <t>kelly_crit &gt; nan</t>
         </is>
       </c>
       <c r="AA39" t="n">
-        <v>-0.5540803436965813</v>
+        <v>-0.3784533266865492</v>
       </c>
       <c r="AB39" t="n">
-        <v>0.1331585017406107</v>
+        <v>3.19318241679369</v>
       </c>
       <c r="AC39" t="n">
-        <v>0.007846519653634532</v>
+        <v>0.1257323658787706</v>
       </c>
       <c r="AD39" t="inlineStr"/>
     </row>
@@ -4520,16 +4524,16 @@
         <v>1</v>
       </c>
       <c r="Q40" t="n">
-        <v>0.3611538739125938</v>
+        <v>0.3464749864716173</v>
       </c>
       <c r="R40" t="n">
-        <v>0.3549577018088816</v>
+        <v>0.3684047962059917</v>
       </c>
       <c r="S40" t="n">
-        <v>0.2838884242785244</v>
+        <v>0.2851202173223909</v>
       </c>
       <c r="T40" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U40" t="n">
         <v>1</v>
@@ -4538,27 +4542,27 @@
         <v>0</v>
       </c>
       <c r="W40" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X40" t="n">
-        <v>0.3611538739125938</v>
+        <v>0.3684047962059917</v>
       </c>
       <c r="Y40" t="n">
-        <v>3</v>
+        <v>2.45</v>
       </c>
       <c r="Z40" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; -0.75</t>
+          <t>kelly_crit &gt; nan</t>
         </is>
       </c>
       <c r="AA40" t="n">
-        <v>0.0417308108688908</v>
+        <v>-0.06717810296228979</v>
       </c>
       <c r="AB40" t="n">
-        <v>5.417308108688908</v>
+        <v>4.664613854564685</v>
       </c>
       <c r="AC40" t="n">
-        <v>0.006196172103712205</v>
+        <v>0.02192980973437442</v>
       </c>
       <c r="AD40" t="inlineStr"/>
     </row>
@@ -4622,13 +4626,13 @@
         <v>2</v>
       </c>
       <c r="Q41" t="n">
-        <v>0.255663385333057</v>
+        <v>0.2613119391248026</v>
       </c>
       <c r="R41" t="n">
-        <v>0.0996065168589504</v>
+        <v>0.09932420273722549</v>
       </c>
       <c r="S41" t="n">
-        <v>0.6447300978079923</v>
+        <v>0.6393638581379719</v>
       </c>
       <c r="T41" t="n">
         <v>2</v>
@@ -4643,24 +4647,24 @@
         <v>2</v>
       </c>
       <c r="X41" t="n">
-        <v>0.6447300978079923</v>
+        <v>0.6393638581379719</v>
       </c>
       <c r="Y41" t="n">
         <v>1.8</v>
       </c>
       <c r="Z41" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; -0.75</t>
+          <t>kelly_crit &gt; nan</t>
         </is>
       </c>
       <c r="AA41" t="n">
-        <v>0.2006427200679826</v>
+        <v>0.1885686808104368</v>
       </c>
       <c r="AB41" t="n">
-        <v>9.670951467119885</v>
+        <v>5.931824842505049</v>
       </c>
       <c r="AC41" t="n">
-        <v>0.3890667124749352</v>
+        <v>0.3780519190131693</v>
       </c>
       <c r="AD41" t="inlineStr"/>
     </row>
@@ -4724,13 +4728,13 @@
         <v>1</v>
       </c>
       <c r="Q42" t="n">
-        <v>0.3210922812913544</v>
+        <v>0.3160000573479757</v>
       </c>
       <c r="R42" t="n">
-        <v>0.4252491675793408</v>
+        <v>0.3918329014669735</v>
       </c>
       <c r="S42" t="n">
-        <v>0.2536585511293048</v>
+        <v>0.2921670411850508</v>
       </c>
       <c r="T42" t="n">
         <v>1</v>
@@ -4745,24 +4749,24 @@
         <v>1</v>
       </c>
       <c r="X42" t="n">
-        <v>0.4252491675793408</v>
+        <v>0.3918329014669735</v>
       </c>
       <c r="Y42" t="n">
         <v>2.34</v>
       </c>
       <c r="Z42" t="inlineStr">
         <is>
-          <t>kelly_crit &gt; -0.75</t>
+          <t>kelly_crit &gt; nan</t>
         </is>
       </c>
       <c r="AA42" t="n">
-        <v>-0.003669364077867614</v>
+        <v>-0.06202314221438963</v>
       </c>
       <c r="AB42" t="n">
-        <v>6.320224379265493</v>
+        <v>4.690281336276141</v>
       </c>
       <c r="AC42" t="n">
-        <v>0.1041568862879864</v>
+        <v>0.07583284411899777</v>
       </c>
       <c r="AD42" t="inlineStr"/>
     </row>
@@ -4859,7 +4863,7 @@
         <v>0.1920997245668447</v>
       </c>
       <c r="AB43" t="n">
-        <v>6.920997245668447</v>
+        <v>5.948855583888075</v>
       </c>
       <c r="AC43" t="n">
         <v>0.1215012001421441</v>
@@ -4959,7 +4963,7 @@
         <v>-0.05023849378491772</v>
       </c>
       <c r="AB44" t="n">
-        <v>5.905015427209836</v>
+        <v>4.749018646691638</v>
       </c>
       <c r="AC44" t="n">
         <v>0.1431733128076561</v>
@@ -5059,7 +5063,7 @@
         <v>-0.704564831425524</v>
       </c>
       <c r="AB45" t="n">
-        <v>0.3398692845680747</v>
+        <v>1.963713676753437</v>
       </c>
       <c r="AC45" t="n">
         <v>0.02897141311678697</v>
@@ -5159,7 +5163,7 @@
         <v>0.1128020446634202</v>
       </c>
       <c r="AB46" t="n">
-        <v>5.724748648753939</v>
+        <v>5.561630124618461</v>
       </c>
       <c r="AC46" t="n">
         <v>0.01954769794785133</v>
@@ -5259,7 +5263,7 @@
         <v>-1.535983040224411</v>
       </c>
       <c r="AB47" t="n">
-        <v>0.009812107114135354</v>
+        <v>0.4427855248447259</v>
       </c>
       <c r="AC47" t="n">
         <v>0.509525636868587</v>
@@ -5359,7 +5363,7 @@
         <v>-0.6528052675101883</v>
       </c>
       <c r="AB48" t="n">
-        <v>0.6214328810887345</v>
+        <v>2.132222874171604</v>
       </c>
       <c r="AC48" t="n">
         <v>0.3010323518832672</v>
@@ -5459,7 +5463,7 @@
         <v>0.2175475650556846</v>
       </c>
       <c r="AB49" t="n">
-        <v>6.715209512354307</v>
+        <v>6.070896798596016</v>
       </c>
       <c r="AC49" t="n">
         <v>0.1240923266534085</v>
@@ -5561,7 +5565,7 @@
         <v>0.1095292369353763</v>
       </c>
       <c r="AB50" t="n">
-        <v>7.450356574017321</v>
+        <v>5.545466668954039</v>
       </c>
       <c r="AC50" t="n">
         <v>0.2374235146893771</v>
@@ -5663,7 +5667,7 @@
         <v>0.01123443117046991</v>
       </c>
       <c r="AB51" t="n">
-        <v>5.112344311704699</v>
+        <v>5.056169792763297</v>
       </c>
       <c r="AC51" t="n">
         <v>0.006097776015097367</v>
@@ -5763,7 +5767,7 @@
         <v>0.1009867394327798</v>
       </c>
       <c r="AB52" t="n">
-        <v>5.864865255526633</v>
+        <v>5.503224178447109</v>
       </c>
       <c r="AC52" t="n">
         <v>0.02262335847562269</v>
@@ -5863,7 +5867,7 @@
         <v>0.1227510477841771</v>
       </c>
       <c r="AB53" t="n">
-        <v>6.410270676220068</v>
+        <v>5.610691054726773</v>
       </c>
       <c r="AC53" t="n">
         <v>0.1215295642027948</v>

</xml_diff>

<commit_message>
Data. Actualizo preds por las dudas
</commit_message>
<xml_diff>
--- a/data/predicciones.xlsx
+++ b/data/predicciones.xlsx
@@ -3658,13 +3658,13 @@
         <v>1</v>
       </c>
       <c r="Q31" t="n">
-        <v>0.3636054694652557</v>
+        <v>0.3650935590267181</v>
       </c>
       <c r="R31" t="n">
-        <v>0.4245496094226837</v>
+        <v>0.4057924151420593</v>
       </c>
       <c r="S31" t="n">
-        <v>0.2118449062108994</v>
+        <v>0.2291140109300613</v>
       </c>
       <c r="T31" t="n">
         <v>1</v>
@@ -3682,7 +3682,7 @@
         <v>1</v>
       </c>
       <c r="Y31" t="n">
-        <v>0.4245496094226837</v>
+        <v>0.4057924151420593</v>
       </c>
       <c r="Z31" t="n">
         <v>2.63</v>
@@ -3693,13 +3693,13 @@
         </is>
       </c>
       <c r="AB31" t="n">
-        <v>0.0715125599887473</v>
+        <v>0.04124788455436563</v>
       </c>
       <c r="AC31" t="n">
-        <v>0.06094413995742798</v>
+        <v>0.04069885611534119</v>
       </c>
       <c r="AD31" t="n">
-        <v>1.181378309416593</v>
+        <v>1.129183366877897</v>
       </c>
     </row>
     <row r="32">
@@ -3970,13 +3970,13 @@
         <v>1</v>
       </c>
       <c r="Q34" t="n">
-        <v>0.393835574388504</v>
+        <v>0.3903920352458954</v>
       </c>
       <c r="R34" t="n">
-        <v>0.2840816676616669</v>
+        <v>0.2845852673053741</v>
       </c>
       <c r="S34" t="n">
-        <v>0.3220826983451843</v>
+        <v>0.3250227272510529</v>
       </c>
       <c r="T34" t="n">
         <v>0</v>
@@ -3994,7 +3994,7 @@
         <v>0</v>
       </c>
       <c r="Y34" t="n">
-        <v>0.393835574388504</v>
+        <v>0.3903920352458954</v>
       </c>
       <c r="Z34" t="n">
         <v>3.7</v>
@@ -4005,13 +4005,13 @@
         </is>
       </c>
       <c r="AB34" t="n">
-        <v>0.1693302315694315</v>
+        <v>0.16461130755919</v>
       </c>
       <c r="AC34" t="n">
-        <v>0.0717528760433197</v>
+        <v>0.06536930799484253</v>
       </c>
       <c r="AD34" t="n">
-        <v>5.355912616568705</v>
+        <v>5.309082680577824</v>
       </c>
     </row>
     <row r="35">
@@ -4074,13 +4074,13 @@
         <v>2</v>
       </c>
       <c r="Q35" t="n">
-        <v>0.4367330968379974</v>
+        <v>0.4295808374881744</v>
       </c>
       <c r="R35" t="n">
-        <v>0.2451000213623047</v>
+        <v>0.2653789520263672</v>
       </c>
       <c r="S35" t="n">
-        <v>0.3181668817996979</v>
+        <v>0.305040180683136</v>
       </c>
       <c r="T35" t="n">
         <v>0</v>
@@ -4098,7 +4098,7 @@
         <v>0</v>
       </c>
       <c r="Y35" t="n">
-        <v>0.4367330968379974</v>
+        <v>0.4295808374881744</v>
       </c>
       <c r="Z35" t="n">
         <v>3.2</v>
@@ -4109,13 +4109,13 @@
         </is>
       </c>
       <c r="AB35" t="n">
-        <v>0.1807026863098145</v>
+        <v>0.1702993999827992</v>
       </c>
       <c r="AC35" t="n">
-        <v>0.1185662150382996</v>
+        <v>0.1245406568050385</v>
       </c>
       <c r="AD35" t="n">
-        <v>5.939291561102893</v>
+        <v>5.842025395779544</v>
       </c>
     </row>
     <row r="36">
@@ -4282,13 +4282,13 @@
         <v>2</v>
       </c>
       <c r="Q37" t="n">
-        <v>0.1649738997220993</v>
+        <v>0.1739211231470108</v>
       </c>
       <c r="R37" t="n">
-        <v>0.09969737380743027</v>
+        <v>0.1051043644547462</v>
       </c>
       <c r="S37" t="n">
-        <v>0.735328733921051</v>
+        <v>0.7209745645523071</v>
       </c>
       <c r="T37" t="n">
         <v>2</v>
@@ -4306,7 +4306,7 @@
         <v>2</v>
       </c>
       <c r="Y37" t="n">
-        <v>0.735328733921051</v>
+        <v>0.7209745645523071</v>
       </c>
       <c r="Z37" t="n">
         <v>1.62</v>
@@ -4317,13 +4317,13 @@
         </is>
       </c>
       <c r="AB37" t="n">
-        <v>0.3084395950840366</v>
+        <v>0.2709335396366735</v>
       </c>
       <c r="AC37" t="n">
-        <v>0.5703548341989517</v>
+        <v>0.5470534414052963</v>
       </c>
       <c r="AD37" t="n">
-        <v>9.190727634794211</v>
+        <v>8.867045872346171</v>
       </c>
     </row>
     <row r="38">

</xml_diff>

<commit_message>
DATA. Actualizo preds por cambio en bs
</commit_message>
<xml_diff>
--- a/data/predicciones.xlsx
+++ b/data/predicciones.xlsx
@@ -685,7 +685,7 @@
         <v>0.2616208493709564</v>
       </c>
       <c r="AD2" t="n">
-        <v>8.443230179498428</v>
+        <v>0.3351350472237874</v>
       </c>
     </row>
     <row r="3">
@@ -789,7 +789,7 @@
         <v>0.1471607685089111</v>
       </c>
       <c r="AD3" t="n">
-        <v>9.679674740809185</v>
+        <v>0.3842129353821191</v>
       </c>
     </row>
     <row r="4">
@@ -893,7 +893,7 @@
         <v>0.002228736877441406</v>
       </c>
       <c r="AD4" t="n">
-        <v>2.568255933709205</v>
+        <v>0.2038822951235796</v>
       </c>
     </row>
     <row r="5">
@@ -997,7 +997,7 @@
         <v>0.1249112486839294</v>
       </c>
       <c r="AD5" t="n">
-        <v>4.127341361848764</v>
+        <v>0.3276510796947257</v>
       </c>
     </row>
     <row r="6">
@@ -1101,7 +1101,7 @@
         <v>0.1780906319618225</v>
       </c>
       <c r="AD6" t="n">
-        <v>9.668282507686845</v>
+        <v>0.3837607462904715</v>
       </c>
     </row>
     <row r="7">
@@ -1205,7 +1205,7 @@
         <v>0.1047435700893402</v>
       </c>
       <c r="AD7" t="n">
-        <v>5.609886141581392</v>
+        <v>4.617300430820253</v>
       </c>
     </row>
     <row r="8">
@@ -1309,7 +1309,7 @@
         <v>0.1600898206233978</v>
       </c>
       <c r="AD8" t="n">
-        <v>5.668210773161974</v>
+        <v>4.66530538844824</v>
       </c>
     </row>
     <row r="9">
@@ -1413,7 +1413,7 @@
         <v>0.06004181504249573</v>
       </c>
       <c r="AD9" t="n">
-        <v>5.182866228925698</v>
+        <v>4.265835324949466</v>
       </c>
     </row>
     <row r="10">
@@ -1517,7 +1517,7 @@
         <v>0.004683405160903931</v>
       </c>
       <c r="AD10" t="n">
-        <v>4.237670614413829</v>
+        <v>3.487877981796541</v>
       </c>
     </row>
     <row r="11">
@@ -1621,7 +1621,7 @@
         <v>0.179634302854538</v>
       </c>
       <c r="AD11" t="n">
-        <v>9.630478893985075</v>
+        <v>11.77783013202282</v>
       </c>
     </row>
     <row r="12">
@@ -1725,7 +1725,7 @@
         <v>0.3254745304584503</v>
       </c>
       <c r="AD12" t="n">
-        <v>0.1102382594781421</v>
+        <v>0.9810394032722668</v>
       </c>
     </row>
     <row r="13">
@@ -1829,7 +1829,7 @@
         <v>0.47083680331707</v>
       </c>
       <c r="AD13" t="n">
-        <v>0.08073177767454034</v>
+        <v>0.7184534241548346</v>
       </c>
     </row>
     <row r="14">
@@ -1933,7 +1933,7 @@
         <v>0.3176412284374237</v>
       </c>
       <c r="AD14" t="n">
-        <v>0.3040039907200959</v>
+        <v>2.70541185120548</v>
       </c>
     </row>
     <row r="15">
@@ -2037,7 +2037,7 @@
         <v>0.08063921332359314</v>
       </c>
       <c r="AD15" t="n">
-        <v>0.04679039925368557</v>
+        <v>0.4164001280499937</v>
       </c>
     </row>
     <row r="16">
@@ -2141,7 +2141,7 @@
         <v>0.4000399559736252</v>
       </c>
       <c r="AD16" t="n">
-        <v>0.003185377943433339</v>
+        <v>0.02834752010432548</v>
       </c>
     </row>
     <row r="17">
@@ -2245,7 +2245,7 @@
         <v>0.1436111330986023</v>
       </c>
       <c r="AD17" t="n">
-        <v>0.05894645090908951</v>
+        <v>0.5245800441573313</v>
       </c>
     </row>
     <row r="18">
@@ -2349,7 +2349,7 @@
         <v>0.05546495318412781</v>
       </c>
       <c r="AD18" t="n">
-        <v>0.3161199746044659</v>
+        <v>1.257942899197902</v>
       </c>
     </row>
     <row r="19">
@@ -2453,7 +2453,7 @@
         <v>0.0481448769569397</v>
       </c>
       <c r="AD19" t="n">
-        <v>1.429061530511188</v>
+        <v>2.730901190785898</v>
       </c>
     </row>
     <row r="20">
@@ -2557,7 +2557,7 @@
         <v>0.1573568880558014</v>
       </c>
       <c r="AD20" t="n">
-        <v>2.688443351997603</v>
+        <v>5.137548660136721</v>
       </c>
     </row>
     <row r="21">
@@ -2661,7 +2661,7 @@
         <v>0.5670660883188248</v>
       </c>
       <c r="AD21" t="n">
-        <v>1.109391611043633</v>
+        <v>0.4879604412029059</v>
       </c>
     </row>
     <row r="22">
@@ -2765,7 +2765,7 @@
         <v>0.1060161292552948</v>
       </c>
       <c r="AD22" t="n">
-        <v>0.2853560899796775</v>
+        <v>0.2510249440870219</v>
       </c>
     </row>
     <row r="23">
@@ -2869,7 +2869,7 @@
         <v>0.1002408564090729</v>
       </c>
       <c r="AD23" t="n">
-        <v>5.647967757988735</v>
+        <v>6.81146778936318</v>
       </c>
     </row>
     <row r="24">
@@ -2973,7 +2973,7 @@
         <v>0.08189168572425842</v>
       </c>
       <c r="AD24" t="n">
-        <v>4.377300952044566</v>
+        <v>3.959717933713413</v>
       </c>
     </row>
     <row r="25">
@@ -3077,7 +3077,7 @@
         <v>0.08543038368225098</v>
       </c>
       <c r="AD25" t="n">
-        <v>4.426712640226024</v>
+        <v>4.004415876571509</v>
       </c>
     </row>
     <row r="26">
@@ -3181,7 +3181,7 @@
         <v>0.2960036396980286</v>
       </c>
       <c r="AD26" t="n">
-        <v>5.384164122690718</v>
+        <v>4.870529001373932</v>
       </c>
     </row>
     <row r="27">
@@ -3285,7 +3285,7 @@
         <v>0.3939221799373627</v>
       </c>
       <c r="AD27" t="n">
-        <v>5.345120169971321</v>
+        <v>4.835209739235046</v>
       </c>
     </row>
     <row r="28">
@@ -3389,7 +3389,7 @@
         <v>0.08452656865119934</v>
       </c>
       <c r="AD28" t="n">
-        <v>4.274009221424619</v>
+        <v>3.86627996300476</v>
       </c>
     </row>
     <row r="29">
@@ -3493,7 +3493,7 @@
         <v>0.1581315994262695</v>
       </c>
       <c r="AD29" t="n">
-        <v>4.44698862822966</v>
+        <v>4.022757588553696</v>
       </c>
     </row>
     <row r="30">
@@ -3597,7 +3597,7 @@
         <v>0.1637256443500519</v>
       </c>
       <c r="AD30" t="n">
-        <v>0.1309791489345208</v>
+        <v>0.1152210683157152</v>
       </c>
     </row>
     <row r="31">
@@ -3701,7 +3701,7 @@
         <v>0.2084943056106567</v>
       </c>
       <c r="AD31" t="n">
-        <v>1.255247936693745</v>
+        <v>0.5521146283339134</v>
       </c>
     </row>
     <row r="32">
@@ -3805,7 +3805,7 @@
         <v>0.02219241857528687</v>
       </c>
       <c r="AD32" t="n">
-        <v>5.009975448251422</v>
+        <v>5.305237881026113</v>
       </c>
     </row>
     <row r="33">
@@ -3909,7 +3909,7 @@
         <v>0.09540918469429016</v>
       </c>
       <c r="AD33" t="n">
-        <v>5.835889742456621</v>
+        <v>6.179827356634753</v>
       </c>
     </row>
     <row r="34">
@@ -4013,7 +4013,7 @@
         <v>0.09134882688522339</v>
       </c>
       <c r="AD34" t="n">
-        <v>5.775617575000911</v>
+        <v>6.116003054647568</v>
       </c>
     </row>
     <row r="35">
@@ -4117,7 +4117,7 @@
         <v>0.07457634806632996</v>
       </c>
       <c r="AD35" t="n">
-        <v>5.703926987526105</v>
+        <v>6.040087389129266</v>
       </c>
     </row>
     <row r="36">
@@ -4221,7 +4221,7 @@
         <v>0.1845326125621796</v>
       </c>
       <c r="AD36" t="n">
-        <v>3.099013731480287</v>
+        <v>2.995282395140523</v>
       </c>
     </row>
     <row r="37">
@@ -4325,7 +4325,7 @@
         <v>0.02972429990768433</v>
       </c>
       <c r="AD37" t="n">
-        <v>8.808052234774465</v>
+        <v>8.513225845467963</v>
       </c>
     </row>
     <row r="38">
@@ -4429,7 +4429,7 @@
         <v>0.2150503695011139</v>
       </c>
       <c r="AD38" t="n">
-        <v>1.558424530851833</v>
+        <v>1.506260367289798</v>
       </c>
     </row>
     <row r="39">
@@ -4533,7 +4533,7 @@
         <v>0.1391639113426208</v>
       </c>
       <c r="AD39" t="n">
-        <v>5.549888554911848</v>
+        <v>5.364120628009899</v>
       </c>
     </row>
     <row r="40">
@@ -4637,7 +4637,7 @@
         <v>0.1727591156959534</v>
       </c>
       <c r="AD40" t="n">
-        <v>1.048124535720531</v>
+        <v>1.83839543961497</v>
       </c>
     </row>
     <row r="41">
@@ -4741,7 +4741,7 @@
         <v>0.4866185784339905</v>
       </c>
       <c r="AD41" t="n">
-        <v>1.646438666974894</v>
+        <v>2.887829865457376</v>
       </c>
     </row>
     <row r="42">
@@ -4845,7 +4845,7 @@
         <v>0.03153151273727417</v>
       </c>
       <c r="AD42" t="n">
-        <v>0.6965139479312499</v>
+        <v>1.221675499300065</v>
       </c>
     </row>
     <row r="43">
@@ -4949,7 +4949,7 @@
         <v>0.0444263219833374</v>
       </c>
       <c r="AD43" t="n">
-        <v>0.8302143585519</v>
+        <v>1.456184106610437</v>
       </c>
     </row>
     <row r="44">
@@ -5053,7 +5053,7 @@
         <v>0.07840985059738159</v>
       </c>
       <c r="AD44" t="n">
-        <v>0.9513923911065381</v>
+        <v>1.668728641956913</v>
       </c>
     </row>
     <row r="45">
@@ -5573,7 +5573,7 @@
         <v>0.149784117937088</v>
       </c>
       <c r="AD49" t="n">
-        <v>8.218060455320661</v>
+        <v>0.3371677617932013</v>
       </c>
     </row>
     <row r="50">
@@ -5677,7 +5677,7 @@
         <v>0.1323164999485016</v>
       </c>
       <c r="AD50" t="n">
-        <v>8.409973570988255</v>
+        <v>0.3177869416641564</v>
       </c>
     </row>
     <row r="51">
@@ -5781,7 +5781,7 @@
         <v>0.2649183571338654</v>
       </c>
       <c r="AD51" t="n">
-        <v>5.50660270064092</v>
+        <v>0.2653030415626944</v>
       </c>
     </row>
     <row r="52">
@@ -5885,7 +5885,7 @@
         <v>0.007778525352478027</v>
       </c>
       <c r="AD52" t="n">
-        <v>8.331741731315699</v>
+        <v>0.27438340290434</v>
       </c>
     </row>
     <row r="53">
@@ -5989,7 +5989,7 @@
         <v>0.291805624961853</v>
       </c>
       <c r="AD53" t="n">
-        <v>8.066092572537595</v>
+        <v>0.4002689587076197</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
DATA. Actualizo reduciendo por confidence margin por el partido de ARS-NEW
</commit_message>
<xml_diff>
--- a/data/predicciones.xlsx
+++ b/data/predicciones.xlsx
@@ -789,7 +789,7 @@
         <v>0.002228736877441406</v>
       </c>
       <c r="AD3" t="n">
-        <v>0.2127193725570813</v>
+        <v>0.06381581176712439</v>
       </c>
     </row>
     <row r="4">
@@ -1309,7 +1309,7 @@
         <v>0.01977738738059998</v>
       </c>
       <c r="AD8" t="n">
-        <v>11.11466528631029</v>
+        <v>3.334399585893086</v>
       </c>
     </row>
     <row r="9">

</xml_diff>

<commit_message>
Reduzco stakes de FRA y SPA
</commit_message>
<xml_diff>
--- a/data/predicciones.xlsx
+++ b/data/predicciones.xlsx
@@ -1101,7 +1101,7 @@
         <v>0.05547289834541969</v>
       </c>
       <c r="AD6" t="n">
-        <v>3.882163110260184</v>
+        <v>1.941081555130092</v>
       </c>
     </row>
     <row r="7">
@@ -1205,7 +1205,7 @@
         <v>0.08559803221463225</v>
       </c>
       <c r="AD7" t="n">
-        <v>3.531401704305216</v>
+        <v>1.765700852152608</v>
       </c>
     </row>
     <row r="8">
@@ -1413,7 +1413,7 @@
         <v>0.1783943891027903</v>
       </c>
       <c r="AD9" t="n">
-        <v>4.8034632651171</v>
+        <v>2.40173163255855</v>
       </c>
     </row>
     <row r="10">
@@ -2141,7 +2141,7 @@
         <v>0.569519553156546</v>
       </c>
       <c r="AD16" t="n">
-        <v>6.95574299419891</v>
+        <v>3.477871497099455</v>
       </c>
     </row>
     <row r="17">
@@ -2245,7 +2245,7 @@
         <v>0.02944008057371644</v>
       </c>
       <c r="AD17" t="n">
-        <v>3.530461170717837</v>
+        <v>1.765230585358919</v>
       </c>
     </row>
     <row r="18">
@@ -2453,7 +2453,7 @@
         <v>0.00633547947170876</v>
       </c>
       <c r="AD19" t="n">
-        <v>3.533504733005411</v>
+        <v>1.766752366502705</v>
       </c>
     </row>
   </sheetData>

</xml_diff>